<commit_message>
auto: portfolio snapshot 2026-03-18 (2026-03-18T11:40:53)
</commit_message>
<xml_diff>
--- a/portfolio_auto.xlsx
+++ b/portfolio_auto.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G1"/>
+  <dimension ref="A1:G15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -464,6 +464,384 @@
         <is>
           <t>수익률(%)</t>
         </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>노브</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>185</v>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E2" t="n">
+        <v>5140749</v>
+      </c>
+      <c r="F2" t="n">
+        <v>1830741</v>
+      </c>
+      <c r="G2" t="n">
+        <v>55.3</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>노블</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>99</v>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E3" t="n">
+        <v>7024110</v>
+      </c>
+      <c r="F3" t="n">
+        <v>3116902</v>
+      </c>
+      <c r="G3" t="n">
+        <v>79.77</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>더치 브로스</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>39</v>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>1</v>
+      </c>
+      <c r="E4" t="n">
+        <v>2989154</v>
+      </c>
+      <c r="F4" t="n">
+        <v>-201490</v>
+      </c>
+      <c r="G4" t="n">
+        <v>-6.31</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>발레로 에너지</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>6</v>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>1</v>
+      </c>
+      <c r="E5" t="n">
+        <v>2109459</v>
+      </c>
+      <c r="F5" t="n">
+        <v>45469</v>
+      </c>
+      <c r="G5" t="n">
+        <v>2.2</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>센트러스 에너지</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>21</v>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>1</v>
+      </c>
+      <c r="E6" t="n">
+        <v>6721336</v>
+      </c>
+      <c r="F6" t="n">
+        <v>490117</v>
+      </c>
+      <c r="G6" t="n">
+        <v>7.86</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>스타 벌크 캐리어스</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>50</v>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>1</v>
+      </c>
+      <c r="E7" t="n">
+        <v>1684783</v>
+      </c>
+      <c r="F7" t="n">
+        <v>370430</v>
+      </c>
+      <c r="G7" t="n">
+        <v>28.18</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>시드릴</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>123</v>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>1</v>
+      </c>
+      <c r="E8" t="n">
+        <v>8270679</v>
+      </c>
+      <c r="F8" t="n">
+        <v>1820328</v>
+      </c>
+      <c r="G8" t="n">
+        <v>28.22</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>오케아니스 에코 탱커스</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>65</v>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>1</v>
+      </c>
+      <c r="E9" t="n">
+        <v>4572321</v>
+      </c>
+      <c r="F9" t="n">
+        <v>2315961</v>
+      </c>
+      <c r="G9" t="n">
+        <v>102.64</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>유나이티드헬스 그룹</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>4</v>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>1</v>
+      </c>
+      <c r="E10" t="n">
+        <v>1710222</v>
+      </c>
+      <c r="F10" t="n">
+        <v>15766</v>
+      </c>
+      <c r="G10" t="n">
+        <v>0.93</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>차코스 에너지 내비게이션</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>75</v>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>1</v>
+      </c>
+      <c r="E11" t="n">
+        <v>3892088</v>
+      </c>
+      <c r="F11" t="n">
+        <v>67440</v>
+      </c>
+      <c r="G11" t="n">
+        <v>1.76</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>클리블랜드 클리프스</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>70</v>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>1</v>
+      </c>
+      <c r="E12" t="n">
+        <v>880384</v>
+      </c>
+      <c r="F12" t="n">
+        <v>-135671</v>
+      </c>
+      <c r="G12" t="n">
+        <v>-13.35</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>타이드워터</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>48</v>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>1</v>
+      </c>
+      <c r="E13" t="n">
+        <v>5469451</v>
+      </c>
+      <c r="F13" t="n">
+        <v>1744906</v>
+      </c>
+      <c r="G13" t="n">
+        <v>46.84</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>텍사스 퍼시픽 랜드</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>1</v>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>1</v>
+      </c>
+      <c r="E14" t="n">
+        <v>787419</v>
+      </c>
+      <c r="F14" t="n">
+        <v>8828</v>
+      </c>
+      <c r="G14" t="n">
+        <v>1.13</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>트랜스오션</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>750</v>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>1</v>
+      </c>
+      <c r="E15" t="n">
+        <v>7427805</v>
+      </c>
+      <c r="F15" t="n">
+        <v>3300571</v>
+      </c>
+      <c r="G15" t="n">
+        <v>79.97</v>
       </c>
     </row>
   </sheetData>
@@ -521,7 +899,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2026-03-18T11:40:26</t>
+          <t>2026-03-18T11:40:53</t>
         </is>
       </c>
       <c r="E2" t="n">

</xml_diff>

<commit_message>
auto: portfolio snapshot 2026-03-18 (2026-03-18T11:41:28)
</commit_message>
<xml_diff>
--- a/portfolio_auto.xlsx
+++ b/portfolio_auto.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G15"/>
+  <dimension ref="A1:G29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -490,7 +490,7 @@
         <v>1830741</v>
       </c>
       <c r="G2" t="n">
-        <v>55.3</v>
+        <v>55.3092620924179</v>
       </c>
     </row>
     <row r="3">
@@ -517,7 +517,7 @@
         <v>3116902</v>
       </c>
       <c r="G3" t="n">
-        <v>79.77</v>
+        <v>79.77312700014947</v>
       </c>
     </row>
     <row r="4">
@@ -544,7 +544,7 @@
         <v>-201490</v>
       </c>
       <c r="G4" t="n">
-        <v>-6.31</v>
+        <v>-6.315026057435428</v>
       </c>
     </row>
     <row r="5">
@@ -571,7 +571,7 @@
         <v>45469</v>
       </c>
       <c r="G5" t="n">
-        <v>2.2</v>
+        <v>2.202966099641956</v>
       </c>
     </row>
     <row r="6">
@@ -595,10 +595,10 @@
         <v>6721336</v>
       </c>
       <c r="F6" t="n">
-        <v>490117</v>
+        <v>490117.0000000009</v>
       </c>
       <c r="G6" t="n">
-        <v>7.86</v>
+        <v>7.865507535523965</v>
       </c>
     </row>
     <row r="7">
@@ -622,10 +622,10 @@
         <v>1684783</v>
       </c>
       <c r="F7" t="n">
-        <v>370430</v>
+        <v>370430.0000000002</v>
       </c>
       <c r="G7" t="n">
-        <v>28.18</v>
+        <v>28.18344843432474</v>
       </c>
     </row>
     <row r="8">
@@ -646,13 +646,13 @@
         <v>1</v>
       </c>
       <c r="E8" t="n">
-        <v>8270679</v>
+        <v>8270678.999999999</v>
       </c>
       <c r="F8" t="n">
-        <v>1820328</v>
+        <v>1820327.999999999</v>
       </c>
       <c r="G8" t="n">
-        <v>28.22</v>
+        <v>28.22060380900201</v>
       </c>
     </row>
     <row r="9">
@@ -679,7 +679,7 @@
         <v>2315961</v>
       </c>
       <c r="G9" t="n">
-        <v>102.64</v>
+        <v>102.6414667872148</v>
       </c>
     </row>
     <row r="10">
@@ -706,7 +706,7 @@
         <v>15766</v>
       </c>
       <c r="G10" t="n">
-        <v>0.93</v>
+        <v>0.9304461136789625</v>
       </c>
     </row>
     <row r="11">
@@ -733,7 +733,7 @@
         <v>67440</v>
       </c>
       <c r="G11" t="n">
-        <v>1.76</v>
+        <v>1.763299524557554</v>
       </c>
     </row>
     <row r="12">
@@ -760,7 +760,7 @@
         <v>-135671</v>
       </c>
       <c r="G12" t="n">
-        <v>-13.35</v>
+        <v>-13.35272204752695</v>
       </c>
     </row>
     <row r="13">
@@ -787,7 +787,7 @@
         <v>1744906</v>
       </c>
       <c r="G13" t="n">
-        <v>46.84</v>
+        <v>46.84883656929907</v>
       </c>
     </row>
     <row r="14">
@@ -814,7 +814,7 @@
         <v>8828</v>
       </c>
       <c r="G14" t="n">
-        <v>1.13</v>
+        <v>1.133843057523141</v>
       </c>
     </row>
     <row r="15">
@@ -841,7 +841,385 @@
         <v>3300571</v>
       </c>
       <c r="G15" t="n">
-        <v>79.97</v>
+        <v>79.97053232261607</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>페트로브라스 (ADR)</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>480</v>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>1</v>
+      </c>
+      <c r="E16" t="n">
+        <v>13956818</v>
+      </c>
+      <c r="F16" t="n">
+        <v>1850269</v>
+      </c>
+      <c r="G16" t="n">
+        <v>15.28</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>프론트라인</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>175</v>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>1</v>
+      </c>
+      <c r="E17" t="n">
+        <v>8314144</v>
+      </c>
+      <c r="F17" t="n">
+        <v>3884280</v>
+      </c>
+      <c r="G17" t="n">
+        <v>87.68000000000001</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>피바디 에너지</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>65</v>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>1</v>
+      </c>
+      <c r="E18" t="n">
+        <v>3417602</v>
+      </c>
+      <c r="F18" t="n">
+        <v>1946830</v>
+      </c>
+      <c r="G18" t="n">
+        <v>132.36</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>하프니아</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>80</v>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
+        <v>1</v>
+      </c>
+      <c r="E19" t="n">
+        <v>808815</v>
+      </c>
+      <c r="F19" t="n">
+        <v>183084</v>
+      </c>
+      <c r="G19" t="n">
+        <v>29.25</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>AGNC 인베스트먼트</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>700</v>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="D20" t="n">
+        <v>1</v>
+      </c>
+      <c r="E20" t="n">
+        <v>10972791</v>
+      </c>
+      <c r="F20" t="n">
+        <v>140776</v>
+      </c>
+      <c r="G20" t="n">
+        <v>1.29</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>넥스틸</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>200</v>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
+        <v>1</v>
+      </c>
+      <c r="E21" t="n">
+        <v>2401188</v>
+      </c>
+      <c r="F21" t="n">
+        <v>390188</v>
+      </c>
+      <c r="G21" t="n">
+        <v>19.4</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>대신증권</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>55</v>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="D22" t="n">
+        <v>1</v>
+      </c>
+      <c r="E22" t="n">
+        <v>2239512</v>
+      </c>
+      <c r="F22" t="n">
+        <v>530011</v>
+      </c>
+      <c r="G22" t="n">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>대창단조</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>300</v>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="D23" t="n">
+        <v>1</v>
+      </c>
+      <c r="E23" t="n">
+        <v>1910172</v>
+      </c>
+      <c r="F23" t="n">
+        <v>-147828</v>
+      </c>
+      <c r="G23" t="n">
+        <v>-7.18</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>대한조선</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>100</v>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="D24" t="n">
+        <v>1</v>
+      </c>
+      <c r="E24" t="n">
+        <v>9570820</v>
+      </c>
+      <c r="F24" t="n">
+        <v>2357820</v>
+      </c>
+      <c r="G24" t="n">
+        <v>32.68</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>동방</t>
+        </is>
+      </c>
+      <c r="B25" t="n">
+        <v>681</v>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="D25" t="n">
+        <v>1</v>
+      </c>
+      <c r="E25" t="n">
+        <v>1878981</v>
+      </c>
+      <c r="F25" t="n">
+        <v>-92520</v>
+      </c>
+      <c r="G25" t="n">
+        <v>-4.69</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>동원개발</t>
+        </is>
+      </c>
+      <c r="B26" t="n">
+        <v>1360</v>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="D26" t="n">
+        <v>1</v>
+      </c>
+      <c r="E26" t="n">
+        <v>3970044</v>
+      </c>
+      <c r="F26" t="n">
+        <v>232644</v>
+      </c>
+      <c r="G26" t="n">
+        <v>6.22</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>미창석유</t>
+        </is>
+      </c>
+      <c r="B27" t="n">
+        <v>18</v>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="D27" t="n">
+        <v>1</v>
+      </c>
+      <c r="E27" t="n">
+        <v>2028136</v>
+      </c>
+      <c r="F27" t="n">
+        <v>-364064</v>
+      </c>
+      <c r="G27" t="n">
+        <v>-15.21</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>비에이치아이</t>
+        </is>
+      </c>
+      <c r="B28" t="n">
+        <v>8</v>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="D28" t="n">
+        <v>1</v>
+      </c>
+      <c r="E28" t="n">
+        <v>849498</v>
+      </c>
+      <c r="F28" t="n">
+        <v>184383</v>
+      </c>
+      <c r="G28" t="n">
+        <v>27.72</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>삼성생명</t>
+        </is>
+      </c>
+      <c r="B29" t="n">
+        <v>4</v>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="D29" t="n">
+        <v>1</v>
+      </c>
+      <c r="E29" t="n">
+        <v>952092</v>
+      </c>
+      <c r="F29" t="n">
+        <v>119092</v>
+      </c>
+      <c r="G29" t="n">
+        <v>14.29</v>
       </c>
     </row>
   </sheetData>
@@ -899,7 +1277,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2026-03-18T11:40:53</t>
+          <t>2026-03-18T11:41:28</t>
         </is>
       </c>
       <c r="E2" t="n">

</xml_diff>

<commit_message>
auto: portfolio snapshot 2026-03-18 (2026-03-18T11:41:30)
</commit_message>
<xml_diff>
--- a/portfolio_auto.xlsx
+++ b/portfolio_auto.xlsx
@@ -868,7 +868,7 @@
         <v>1850269</v>
       </c>
       <c r="G16" t="n">
-        <v>15.28</v>
+        <v>15.28320746068925</v>
       </c>
     </row>
     <row r="17">
@@ -889,13 +889,13 @@
         <v>1</v>
       </c>
       <c r="E17" t="n">
-        <v>8314144</v>
+        <v>8314143.999999999</v>
       </c>
       <c r="F17" t="n">
-        <v>3884280</v>
+        <v>3884279.999999999</v>
       </c>
       <c r="G17" t="n">
-        <v>87.68000000000001</v>
+        <v>87.68395598600767</v>
       </c>
     </row>
     <row r="18">
@@ -922,7 +922,7 @@
         <v>1946830</v>
       </c>
       <c r="G18" t="n">
-        <v>132.36</v>
+        <v>132.3678993073025</v>
       </c>
     </row>
     <row r="19">
@@ -949,7 +949,7 @@
         <v>183084</v>
       </c>
       <c r="G19" t="n">
-        <v>29.25</v>
+        <v>29.25921841813814</v>
       </c>
     </row>
     <row r="20">
@@ -976,7 +976,7 @@
         <v>140776</v>
       </c>
       <c r="G20" t="n">
-        <v>1.29</v>
+        <v>1.299628924073683</v>
       </c>
     </row>
     <row r="21">
@@ -1003,7 +1003,7 @@
         <v>390188</v>
       </c>
       <c r="G21" t="n">
-        <v>19.4</v>
+        <v>19.40268523122824</v>
       </c>
     </row>
     <row r="22">
@@ -1030,7 +1030,7 @@
         <v>530011</v>
       </c>
       <c r="G22" t="n">
-        <v>31</v>
+        <v>31.00384264180015</v>
       </c>
     </row>
     <row r="23">
@@ -1057,7 +1057,7 @@
         <v>-147828</v>
       </c>
       <c r="G23" t="n">
-        <v>-7.18</v>
+        <v>-7.183090379008747</v>
       </c>
     </row>
     <row r="24">
@@ -1084,7 +1084,7 @@
         <v>2357820</v>
       </c>
       <c r="G24" t="n">
-        <v>32.68</v>
+        <v>32.68847913489532</v>
       </c>
     </row>
     <row r="25">
@@ -1111,7 +1111,7 @@
         <v>-92520</v>
       </c>
       <c r="G25" t="n">
-        <v>-4.69</v>
+        <v>-4.692871066258652</v>
       </c>
     </row>
     <row r="26">
@@ -1138,7 +1138,7 @@
         <v>232644</v>
       </c>
       <c r="G26" t="n">
-        <v>6.22</v>
+        <v>6.224755177396051</v>
       </c>
     </row>
     <row r="27">
@@ -1165,7 +1165,7 @@
         <v>-364064</v>
       </c>
       <c r="G27" t="n">
-        <v>-15.21</v>
+        <v>-15.21879441518268</v>
       </c>
     </row>
     <row r="28">
@@ -1192,7 +1192,7 @@
         <v>184383</v>
       </c>
       <c r="G28" t="n">
-        <v>27.72</v>
+        <v>27.72197289190591</v>
       </c>
     </row>
     <row r="29">
@@ -1219,7 +1219,7 @@
         <v>119092</v>
       </c>
       <c r="G29" t="n">
-        <v>14.29</v>
+        <v>14.29675870348139</v>
       </c>
     </row>
   </sheetData>
@@ -1277,7 +1277,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2026-03-18T11:41:28</t>
+          <t>2026-03-18T11:41:30</t>
         </is>
       </c>
       <c r="E2" t="n">

</xml_diff>

<commit_message>
auto: portfolio snapshot 2026-03-18 (2026-03-18T11:42:17)
</commit_message>
<xml_diff>
--- a/portfolio_auto.xlsx
+++ b/portfolio_auto.xlsx
@@ -868,7 +868,7 @@
         <v>1850269</v>
       </c>
       <c r="G16" t="n">
-        <v>15.28320746068925</v>
+        <v>15.28</v>
       </c>
     </row>
     <row r="17">
@@ -889,13 +889,13 @@
         <v>1</v>
       </c>
       <c r="E17" t="n">
-        <v>8314143.999999999</v>
+        <v>8314144</v>
       </c>
       <c r="F17" t="n">
-        <v>3884279.999999999</v>
+        <v>3884280</v>
       </c>
       <c r="G17" t="n">
-        <v>87.68395598600767</v>
+        <v>87.68000000000001</v>
       </c>
     </row>
     <row r="18">
@@ -922,7 +922,7 @@
         <v>1946830</v>
       </c>
       <c r="G18" t="n">
-        <v>132.3678993073025</v>
+        <v>132.36</v>
       </c>
     </row>
     <row r="19">
@@ -949,7 +949,7 @@
         <v>183084</v>
       </c>
       <c r="G19" t="n">
-        <v>29.25921841813814</v>
+        <v>29.25</v>
       </c>
     </row>
     <row r="20">
@@ -976,7 +976,7 @@
         <v>140776</v>
       </c>
       <c r="G20" t="n">
-        <v>1.299628924073683</v>
+        <v>1.29</v>
       </c>
     </row>
     <row r="21">
@@ -1003,7 +1003,7 @@
         <v>390188</v>
       </c>
       <c r="G21" t="n">
-        <v>19.40268523122824</v>
+        <v>19.4</v>
       </c>
     </row>
     <row r="22">
@@ -1030,7 +1030,7 @@
         <v>530011</v>
       </c>
       <c r="G22" t="n">
-        <v>31.00384264180015</v>
+        <v>31</v>
       </c>
     </row>
     <row r="23">
@@ -1057,7 +1057,7 @@
         <v>-147828</v>
       </c>
       <c r="G23" t="n">
-        <v>-7.183090379008747</v>
+        <v>-7.18</v>
       </c>
     </row>
     <row r="24">
@@ -1084,7 +1084,7 @@
         <v>2357820</v>
       </c>
       <c r="G24" t="n">
-        <v>32.68847913489532</v>
+        <v>32.68</v>
       </c>
     </row>
     <row r="25">
@@ -1111,7 +1111,7 @@
         <v>-92520</v>
       </c>
       <c r="G25" t="n">
-        <v>-4.692871066258652</v>
+        <v>-4.69</v>
       </c>
     </row>
     <row r="26">
@@ -1138,7 +1138,7 @@
         <v>232644</v>
       </c>
       <c r="G26" t="n">
-        <v>6.224755177396051</v>
+        <v>6.22</v>
       </c>
     </row>
     <row r="27">
@@ -1165,7 +1165,7 @@
         <v>-364064</v>
       </c>
       <c r="G27" t="n">
-        <v>-15.21879441518268</v>
+        <v>-15.21</v>
       </c>
     </row>
     <row r="28">
@@ -1192,7 +1192,7 @@
         <v>184383</v>
       </c>
       <c r="G28" t="n">
-        <v>27.72197289190591</v>
+        <v>27.72</v>
       </c>
     </row>
     <row r="29">
@@ -1219,7 +1219,7 @@
         <v>119092</v>
       </c>
       <c r="G29" t="n">
-        <v>14.29675870348139</v>
+        <v>14.29</v>
       </c>
     </row>
   </sheetData>
@@ -1277,7 +1277,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2026-03-18T11:41:30</t>
+          <t>2026-03-18T11:42:16</t>
         </is>
       </c>
       <c r="E2" t="n">

</xml_diff>

<commit_message>
auto: portfolio snapshot 2026-03-18 (2026-03-18T11:42:49)
</commit_message>
<xml_diff>
--- a/portfolio_auto.xlsx
+++ b/portfolio_auto.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G29"/>
+  <dimension ref="A1:G39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -868,7 +868,7 @@
         <v>1850269</v>
       </c>
       <c r="G16" t="n">
-        <v>15.28</v>
+        <v>15.28320746068925</v>
       </c>
     </row>
     <row r="17">
@@ -889,13 +889,13 @@
         <v>1</v>
       </c>
       <c r="E17" t="n">
-        <v>8314144</v>
+        <v>8314143.999999999</v>
       </c>
       <c r="F17" t="n">
-        <v>3884280</v>
+        <v>3884279.999999999</v>
       </c>
       <c r="G17" t="n">
-        <v>87.68000000000001</v>
+        <v>87.68395598600767</v>
       </c>
     </row>
     <row r="18">
@@ -922,7 +922,7 @@
         <v>1946830</v>
       </c>
       <c r="G18" t="n">
-        <v>132.36</v>
+        <v>132.3678993073025</v>
       </c>
     </row>
     <row r="19">
@@ -949,7 +949,7 @@
         <v>183084</v>
       </c>
       <c r="G19" t="n">
-        <v>29.25</v>
+        <v>29.25921841813814</v>
       </c>
     </row>
     <row r="20">
@@ -976,7 +976,7 @@
         <v>140776</v>
       </c>
       <c r="G20" t="n">
-        <v>1.29</v>
+        <v>1.299628924073683</v>
       </c>
     </row>
     <row r="21">
@@ -1003,7 +1003,7 @@
         <v>390188</v>
       </c>
       <c r="G21" t="n">
-        <v>19.4</v>
+        <v>19.40268523122824</v>
       </c>
     </row>
     <row r="22">
@@ -1030,7 +1030,7 @@
         <v>530011</v>
       </c>
       <c r="G22" t="n">
-        <v>31</v>
+        <v>31.00384264180015</v>
       </c>
     </row>
     <row r="23">
@@ -1057,7 +1057,7 @@
         <v>-147828</v>
       </c>
       <c r="G23" t="n">
-        <v>-7.18</v>
+        <v>-7.183090379008747</v>
       </c>
     </row>
     <row r="24">
@@ -1084,7 +1084,7 @@
         <v>2357820</v>
       </c>
       <c r="G24" t="n">
-        <v>32.68</v>
+        <v>32.68847913489532</v>
       </c>
     </row>
     <row r="25">
@@ -1111,7 +1111,7 @@
         <v>-92520</v>
       </c>
       <c r="G25" t="n">
-        <v>-4.69</v>
+        <v>-4.692871066258652</v>
       </c>
     </row>
     <row r="26">
@@ -1138,7 +1138,7 @@
         <v>232644</v>
       </c>
       <c r="G26" t="n">
-        <v>6.22</v>
+        <v>6.224755177396051</v>
       </c>
     </row>
     <row r="27">
@@ -1165,7 +1165,7 @@
         <v>-364064</v>
       </c>
       <c r="G27" t="n">
-        <v>-15.21</v>
+        <v>-15.21879441518268</v>
       </c>
     </row>
     <row r="28">
@@ -1192,7 +1192,7 @@
         <v>184383</v>
       </c>
       <c r="G28" t="n">
-        <v>27.72</v>
+        <v>27.72197289190591</v>
       </c>
     </row>
     <row r="29">
@@ -1219,7 +1219,277 @@
         <v>119092</v>
       </c>
       <c r="G29" t="n">
-        <v>14.29</v>
+        <v>14.29675870348139</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>삼성화재</t>
+        </is>
+      </c>
+      <c r="B30" t="n">
+        <v>9</v>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="D30" t="n">
+        <v>1</v>
+      </c>
+      <c r="E30" t="n">
+        <v>4459563</v>
+      </c>
+      <c r="F30" t="n">
+        <v>-171437</v>
+      </c>
+      <c r="G30" t="n">
+        <v>-3.7</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>세아제강</t>
+        </is>
+      </c>
+      <c r="B31" t="n">
+        <v>50</v>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="D31" t="n">
+        <v>1</v>
+      </c>
+      <c r="E31" t="n">
+        <v>6866240</v>
+      </c>
+      <c r="F31" t="n">
+        <v>556240</v>
+      </c>
+      <c r="G31" t="n">
+        <v>8.81</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>케이씨</t>
+        </is>
+      </c>
+      <c r="B32" t="n">
+        <v>50</v>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="D32" t="n">
+        <v>1</v>
+      </c>
+      <c r="E32" t="n">
+        <v>1641710</v>
+      </c>
+      <c r="F32" t="n">
+        <v>-7790</v>
+      </c>
+      <c r="G32" t="n">
+        <v>-0.47</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>하나금융지주</t>
+        </is>
+      </c>
+      <c r="B33" t="n">
+        <v>15</v>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="D33" t="n">
+        <v>1</v>
+      </c>
+      <c r="E33" t="n">
+        <v>1724544</v>
+      </c>
+      <c r="F33" t="n">
+        <v>42044</v>
+      </c>
+      <c r="G33" t="n">
+        <v>2.49</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>현대제철</t>
+        </is>
+      </c>
+      <c r="B34" t="n">
+        <v>70</v>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="D34" t="n">
+        <v>1</v>
+      </c>
+      <c r="E34" t="n">
+        <v>2623243</v>
+      </c>
+      <c r="F34" t="n">
+        <v>-184257</v>
+      </c>
+      <c r="G34" t="n">
+        <v>-6.56</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>휴스틸</t>
+        </is>
+      </c>
+      <c r="B35" t="n">
+        <v>500</v>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="D35" t="n">
+        <v>1</v>
+      </c>
+      <c r="E35" t="n">
+        <v>2554880</v>
+      </c>
+      <c r="F35" t="n">
+        <v>276270</v>
+      </c>
+      <c r="G35" t="n">
+        <v>12.12</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>DL이앤씨</t>
+        </is>
+      </c>
+      <c r="B36" t="n">
+        <v>80</v>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="D36" t="n">
+        <v>1</v>
+      </c>
+      <c r="E36" t="n">
+        <v>4143696</v>
+      </c>
+      <c r="F36" t="n">
+        <v>732696</v>
+      </c>
+      <c r="G36" t="n">
+        <v>21.48</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>HD건설기계</t>
+        </is>
+      </c>
+      <c r="B37" t="n">
+        <v>31</v>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="D37" t="n">
+        <v>1</v>
+      </c>
+      <c r="E37" t="n">
+        <v>3947686</v>
+      </c>
+      <c r="F37" t="n">
+        <v>-87410</v>
+      </c>
+      <c r="G37" t="n">
+        <v>-2.16</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>KoAct 코스닥액티브</t>
+        </is>
+      </c>
+      <c r="B38" t="n">
+        <v>200</v>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="D38" t="n">
+        <v>1</v>
+      </c>
+      <c r="E38" t="n">
+        <v>2598000</v>
+      </c>
+      <c r="F38" t="n">
+        <v>-104000</v>
+      </c>
+      <c r="G38" t="n">
+        <v>-3.84</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>TIME 코리아밸류업액티브</t>
+        </is>
+      </c>
+      <c r="B39" t="n">
+        <v>201</v>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="D39" t="n">
+        <v>1</v>
+      </c>
+      <c r="E39" t="n">
+        <v>4904400</v>
+      </c>
+      <c r="F39" t="n">
+        <v>180603</v>
+      </c>
+      <c r="G39" t="n">
+        <v>3.82</v>
       </c>
     </row>
   </sheetData>
@@ -1277,7 +1547,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2026-03-18T11:42:16</t>
+          <t>2026-03-18T11:42:49</t>
         </is>
       </c>
       <c r="E2" t="n">

</xml_diff>

<commit_message>
auto: portfolio snapshot 2026-03-18 (2026-03-18T11:42:51)
</commit_message>
<xml_diff>
--- a/portfolio_auto.xlsx
+++ b/portfolio_auto.xlsx
@@ -1246,7 +1246,7 @@
         <v>-171437</v>
       </c>
       <c r="G30" t="n">
-        <v>-3.7</v>
+        <v>-3.701943424746275</v>
       </c>
     </row>
     <row r="31">
@@ -1267,13 +1267,13 @@
         <v>1</v>
       </c>
       <c r="E31" t="n">
-        <v>6866240</v>
+        <v>6866239.999999999</v>
       </c>
       <c r="F31" t="n">
-        <v>556240</v>
+        <v>556239.9999999991</v>
       </c>
       <c r="G31" t="n">
-        <v>8.81</v>
+        <v>8.815213946117259</v>
       </c>
     </row>
     <row r="32">
@@ -1297,10 +1297,10 @@
         <v>1641710</v>
       </c>
       <c r="F32" t="n">
-        <v>-7790</v>
+        <v>-7790.000000000233</v>
       </c>
       <c r="G32" t="n">
-        <v>-0.47</v>
+        <v>-0.4722643225219905</v>
       </c>
     </row>
     <row r="33">
@@ -1327,7 +1327,7 @@
         <v>42044</v>
       </c>
       <c r="G33" t="n">
-        <v>2.49</v>
+        <v>2.49890044576523</v>
       </c>
     </row>
     <row r="34">
@@ -1354,7 +1354,7 @@
         <v>-184257</v>
       </c>
       <c r="G34" t="n">
-        <v>-6.56</v>
+        <v>-6.563027604630454</v>
       </c>
     </row>
     <row r="35">
@@ -1381,7 +1381,7 @@
         <v>276270</v>
       </c>
       <c r="G35" t="n">
-        <v>12.12</v>
+        <v>12.12449695208921</v>
       </c>
     </row>
     <row r="36">
@@ -1408,7 +1408,7 @@
         <v>732696</v>
       </c>
       <c r="G36" t="n">
-        <v>21.48</v>
+        <v>21.48038698328936</v>
       </c>
     </row>
     <row r="37">
@@ -1435,7 +1435,7 @@
         <v>-87410</v>
       </c>
       <c r="G37" t="n">
-        <v>-2.16</v>
+        <v>-2.166243380578802</v>
       </c>
     </row>
     <row r="38">
@@ -1462,7 +1462,7 @@
         <v>-104000</v>
       </c>
       <c r="G38" t="n">
-        <v>-3.84</v>
+        <v>-3.84900074019245</v>
       </c>
     </row>
     <row r="39">
@@ -1489,7 +1489,7 @@
         <v>180603</v>
       </c>
       <c r="G39" t="n">
-        <v>3.82</v>
+        <v>3.823259128197084</v>
       </c>
     </row>
   </sheetData>
@@ -1547,7 +1547,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2026-03-18T11:42:49</t>
+          <t>2026-03-18T11:42:51</t>
         </is>
       </c>
       <c r="E2" t="n">

</xml_diff>

<commit_message>
auto: portfolio snapshot 2026-03-16 (2026-03-18T11:44:38)
</commit_message>
<xml_diff>
--- a/portfolio_auto.xlsx
+++ b/portfolio_auto.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G1"/>
+  <dimension ref="A1:G15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -464,6 +464,384 @@
         <is>
           <t>수익률(%)</t>
         </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>노브</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>185</v>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E2" t="n">
+        <v>5140749</v>
+      </c>
+      <c r="F2" t="n">
+        <v>1830741</v>
+      </c>
+      <c r="G2" t="n">
+        <v>55.3</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>노블</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>99</v>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E3" t="n">
+        <v>7024110</v>
+      </c>
+      <c r="F3" t="n">
+        <v>3116902</v>
+      </c>
+      <c r="G3" t="n">
+        <v>79.77</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>더치 브로스</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>39</v>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>1</v>
+      </c>
+      <c r="E4" t="n">
+        <v>2989154</v>
+      </c>
+      <c r="F4" t="n">
+        <v>-201490</v>
+      </c>
+      <c r="G4" t="n">
+        <v>-6.31</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>발레로 에너지</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>6</v>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>1</v>
+      </c>
+      <c r="E5" t="n">
+        <v>2109459</v>
+      </c>
+      <c r="F5" t="n">
+        <v>45469</v>
+      </c>
+      <c r="G5" t="n">
+        <v>2.2</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>센트러스 에너지</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>21</v>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>1</v>
+      </c>
+      <c r="E6" t="n">
+        <v>6721336</v>
+      </c>
+      <c r="F6" t="n">
+        <v>490117</v>
+      </c>
+      <c r="G6" t="n">
+        <v>7.86</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>스타 벌크 캐리어스</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>50</v>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>1</v>
+      </c>
+      <c r="E7" t="n">
+        <v>1684783</v>
+      </c>
+      <c r="F7" t="n">
+        <v>370430</v>
+      </c>
+      <c r="G7" t="n">
+        <v>28.18</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>시드릴</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>123</v>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>1</v>
+      </c>
+      <c r="E8" t="n">
+        <v>8270679</v>
+      </c>
+      <c r="F8" t="n">
+        <v>1820328</v>
+      </c>
+      <c r="G8" t="n">
+        <v>28.22</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>오케아니스 에코 탱커스</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>65</v>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>1</v>
+      </c>
+      <c r="E9" t="n">
+        <v>4572321</v>
+      </c>
+      <c r="F9" t="n">
+        <v>2315961</v>
+      </c>
+      <c r="G9" t="n">
+        <v>102.64</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>유나이티드헬스 그룹</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>4</v>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>1</v>
+      </c>
+      <c r="E10" t="n">
+        <v>1710222</v>
+      </c>
+      <c r="F10" t="n">
+        <v>15766</v>
+      </c>
+      <c r="G10" t="n">
+        <v>0.93</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>차코스 에너지 내비게이션</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>75</v>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>1</v>
+      </c>
+      <c r="E11" t="n">
+        <v>3892088</v>
+      </c>
+      <c r="F11" t="n">
+        <v>67440</v>
+      </c>
+      <c r="G11" t="n">
+        <v>1.76</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>클리블랜드 클리프스</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>70</v>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>1</v>
+      </c>
+      <c r="E12" t="n">
+        <v>880384</v>
+      </c>
+      <c r="F12" t="n">
+        <v>-135671</v>
+      </c>
+      <c r="G12" t="n">
+        <v>-13.35</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>타이드워터</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>48</v>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>1</v>
+      </c>
+      <c r="E13" t="n">
+        <v>5469451</v>
+      </c>
+      <c r="F13" t="n">
+        <v>1744906</v>
+      </c>
+      <c r="G13" t="n">
+        <v>46.84</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>텍사스 퍼시픽 랜드</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>1</v>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>1</v>
+      </c>
+      <c r="E14" t="n">
+        <v>787419</v>
+      </c>
+      <c r="F14" t="n">
+        <v>8828</v>
+      </c>
+      <c r="G14" t="n">
+        <v>1.13</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>트랜스오션</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>750</v>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>1</v>
+      </c>
+      <c r="E15" t="n">
+        <v>7427805</v>
+      </c>
+      <c r="F15" t="n">
+        <v>3300571</v>
+      </c>
+      <c r="G15" t="n">
+        <v>79.97</v>
       </c>
     </row>
   </sheetData>
@@ -521,7 +899,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2026-03-18T11:44:09</t>
+          <t>2026-03-18T11:44:38</t>
         </is>
       </c>
       <c r="E2" t="n">

</xml_diff>

<commit_message>
auto: portfolio snapshot 2026-03-16 (2026-03-18T11:44:40)
</commit_message>
<xml_diff>
--- a/portfolio_auto.xlsx
+++ b/portfolio_auto.xlsx
@@ -490,7 +490,7 @@
         <v>1830741</v>
       </c>
       <c r="G2" t="n">
-        <v>55.3</v>
+        <v>55.3092620924179</v>
       </c>
     </row>
     <row r="3">
@@ -517,7 +517,7 @@
         <v>3116902</v>
       </c>
       <c r="G3" t="n">
-        <v>79.77</v>
+        <v>79.77312700014947</v>
       </c>
     </row>
     <row r="4">
@@ -544,7 +544,7 @@
         <v>-201490</v>
       </c>
       <c r="G4" t="n">
-        <v>-6.31</v>
+        <v>-6.315026057435428</v>
       </c>
     </row>
     <row r="5">
@@ -571,7 +571,7 @@
         <v>45469</v>
       </c>
       <c r="G5" t="n">
-        <v>2.2</v>
+        <v>2.202966099641956</v>
       </c>
     </row>
     <row r="6">
@@ -595,10 +595,10 @@
         <v>6721336</v>
       </c>
       <c r="F6" t="n">
-        <v>490117</v>
+        <v>490117.0000000009</v>
       </c>
       <c r="G6" t="n">
-        <v>7.86</v>
+        <v>7.865507535523965</v>
       </c>
     </row>
     <row r="7">
@@ -622,10 +622,10 @@
         <v>1684783</v>
       </c>
       <c r="F7" t="n">
-        <v>370430</v>
+        <v>370430.0000000002</v>
       </c>
       <c r="G7" t="n">
-        <v>28.18</v>
+        <v>28.18344843432474</v>
       </c>
     </row>
     <row r="8">
@@ -646,13 +646,13 @@
         <v>1</v>
       </c>
       <c r="E8" t="n">
-        <v>8270679</v>
+        <v>8270678.999999999</v>
       </c>
       <c r="F8" t="n">
-        <v>1820328</v>
+        <v>1820327.999999999</v>
       </c>
       <c r="G8" t="n">
-        <v>28.22</v>
+        <v>28.22060380900201</v>
       </c>
     </row>
     <row r="9">
@@ -679,7 +679,7 @@
         <v>2315961</v>
       </c>
       <c r="G9" t="n">
-        <v>102.64</v>
+        <v>102.6414667872148</v>
       </c>
     </row>
     <row r="10">
@@ -706,7 +706,7 @@
         <v>15766</v>
       </c>
       <c r="G10" t="n">
-        <v>0.93</v>
+        <v>0.9304461136789625</v>
       </c>
     </row>
     <row r="11">
@@ -733,7 +733,7 @@
         <v>67440</v>
       </c>
       <c r="G11" t="n">
-        <v>1.76</v>
+        <v>1.763299524557554</v>
       </c>
     </row>
     <row r="12">
@@ -760,7 +760,7 @@
         <v>-135671</v>
       </c>
       <c r="G12" t="n">
-        <v>-13.35</v>
+        <v>-13.35272204752695</v>
       </c>
     </row>
     <row r="13">
@@ -787,7 +787,7 @@
         <v>1744906</v>
       </c>
       <c r="G13" t="n">
-        <v>46.84</v>
+        <v>46.84883656929907</v>
       </c>
     </row>
     <row r="14">
@@ -814,7 +814,7 @@
         <v>8828</v>
       </c>
       <c r="G14" t="n">
-        <v>1.13</v>
+        <v>1.133843057523141</v>
       </c>
     </row>
     <row r="15">
@@ -841,7 +841,7 @@
         <v>3300571</v>
       </c>
       <c r="G15" t="n">
-        <v>79.97</v>
+        <v>79.97053232261607</v>
       </c>
     </row>
   </sheetData>
@@ -899,7 +899,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2026-03-18T11:44:38</t>
+          <t>2026-03-18T11:44:40</t>
         </is>
       </c>
       <c r="E2" t="n">

</xml_diff>

<commit_message>
auto: portfolio snapshot 2026-03-16 (2026-03-18T11:45:14)
</commit_message>
<xml_diff>
--- a/portfolio_auto.xlsx
+++ b/portfolio_auto.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G15"/>
+  <dimension ref="A1:G29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -842,6 +842,384 @@
       </c>
       <c r="G15" t="n">
         <v>79.97053232261607</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>페트로브라스 (ADR)</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>480</v>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>1</v>
+      </c>
+      <c r="E16" t="n">
+        <v>13956818</v>
+      </c>
+      <c r="F16" t="n">
+        <v>1850269</v>
+      </c>
+      <c r="G16" t="n">
+        <v>15.28</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>프론트라인</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>175</v>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>1</v>
+      </c>
+      <c r="E17" t="n">
+        <v>8314144</v>
+      </c>
+      <c r="F17" t="n">
+        <v>3884280</v>
+      </c>
+      <c r="G17" t="n">
+        <v>87.68000000000001</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>피바디 에너지</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>65</v>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>1</v>
+      </c>
+      <c r="E18" t="n">
+        <v>3417602</v>
+      </c>
+      <c r="F18" t="n">
+        <v>1946830</v>
+      </c>
+      <c r="G18" t="n">
+        <v>132.36</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>하프니아</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>80</v>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
+        <v>1</v>
+      </c>
+      <c r="E19" t="n">
+        <v>808815</v>
+      </c>
+      <c r="F19" t="n">
+        <v>183084</v>
+      </c>
+      <c r="G19" t="n">
+        <v>29.25</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>AGNC 인베스트먼트</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>700</v>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="D20" t="n">
+        <v>1</v>
+      </c>
+      <c r="E20" t="n">
+        <v>10972791</v>
+      </c>
+      <c r="F20" t="n">
+        <v>140776</v>
+      </c>
+      <c r="G20" t="n">
+        <v>1.29</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>넥스틸</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>200</v>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
+        <v>1</v>
+      </c>
+      <c r="E21" t="n">
+        <v>2401188</v>
+      </c>
+      <c r="F21" t="n">
+        <v>390188</v>
+      </c>
+      <c r="G21" t="n">
+        <v>19.4</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>대신증권</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>55</v>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="D22" t="n">
+        <v>1</v>
+      </c>
+      <c r="E22" t="n">
+        <v>2239512</v>
+      </c>
+      <c r="F22" t="n">
+        <v>530011</v>
+      </c>
+      <c r="G22" t="n">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>대창단조</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>300</v>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="D23" t="n">
+        <v>1</v>
+      </c>
+      <c r="E23" t="n">
+        <v>1910172</v>
+      </c>
+      <c r="F23" t="n">
+        <v>-147828</v>
+      </c>
+      <c r="G23" t="n">
+        <v>-7.18</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>대한조선</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>100</v>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="D24" t="n">
+        <v>1</v>
+      </c>
+      <c r="E24" t="n">
+        <v>9570820</v>
+      </c>
+      <c r="F24" t="n">
+        <v>2357820</v>
+      </c>
+      <c r="G24" t="n">
+        <v>32.68</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>동방</t>
+        </is>
+      </c>
+      <c r="B25" t="n">
+        <v>681</v>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="D25" t="n">
+        <v>1</v>
+      </c>
+      <c r="E25" t="n">
+        <v>1878981</v>
+      </c>
+      <c r="F25" t="n">
+        <v>-92520</v>
+      </c>
+      <c r="G25" t="n">
+        <v>-4.69</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>동원개발</t>
+        </is>
+      </c>
+      <c r="B26" t="n">
+        <v>1360</v>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="D26" t="n">
+        <v>1</v>
+      </c>
+      <c r="E26" t="n">
+        <v>3970044</v>
+      </c>
+      <c r="F26" t="n">
+        <v>232644</v>
+      </c>
+      <c r="G26" t="n">
+        <v>6.22</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>미창석유</t>
+        </is>
+      </c>
+      <c r="B27" t="n">
+        <v>18</v>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="D27" t="n">
+        <v>1</v>
+      </c>
+      <c r="E27" t="n">
+        <v>2028136</v>
+      </c>
+      <c r="F27" t="n">
+        <v>-364064</v>
+      </c>
+      <c r="G27" t="n">
+        <v>-15.21</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>비에이치아이</t>
+        </is>
+      </c>
+      <c r="B28" t="n">
+        <v>8</v>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="D28" t="n">
+        <v>1</v>
+      </c>
+      <c r="E28" t="n">
+        <v>849498</v>
+      </c>
+      <c r="F28" t="n">
+        <v>184383</v>
+      </c>
+      <c r="G28" t="n">
+        <v>27.72</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>삼성생명</t>
+        </is>
+      </c>
+      <c r="B29" t="n">
+        <v>4</v>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="D29" t="n">
+        <v>1</v>
+      </c>
+      <c r="E29" t="n">
+        <v>952092</v>
+      </c>
+      <c r="F29" t="n">
+        <v>119092</v>
+      </c>
+      <c r="G29" t="n">
+        <v>14.29</v>
       </c>
     </row>
   </sheetData>
@@ -899,7 +1277,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2026-03-18T11:44:40</t>
+          <t>2026-03-18T11:45:14</t>
         </is>
       </c>
       <c r="E2" t="n">

</xml_diff>

<commit_message>
auto: portfolio snapshot 2026-03-16 (2026-03-18T11:45:16)
</commit_message>
<xml_diff>
--- a/portfolio_auto.xlsx
+++ b/portfolio_auto.xlsx
@@ -868,7 +868,7 @@
         <v>1850269</v>
       </c>
       <c r="G16" t="n">
-        <v>15.28</v>
+        <v>15.28320746068925</v>
       </c>
     </row>
     <row r="17">
@@ -889,13 +889,13 @@
         <v>1</v>
       </c>
       <c r="E17" t="n">
-        <v>8314144</v>
+        <v>8314143.999999999</v>
       </c>
       <c r="F17" t="n">
-        <v>3884280</v>
+        <v>3884279.999999999</v>
       </c>
       <c r="G17" t="n">
-        <v>87.68000000000001</v>
+        <v>87.68395598600767</v>
       </c>
     </row>
     <row r="18">
@@ -922,7 +922,7 @@
         <v>1946830</v>
       </c>
       <c r="G18" t="n">
-        <v>132.36</v>
+        <v>132.3678993073025</v>
       </c>
     </row>
     <row r="19">
@@ -949,7 +949,7 @@
         <v>183084</v>
       </c>
       <c r="G19" t="n">
-        <v>29.25</v>
+        <v>29.25921841813814</v>
       </c>
     </row>
     <row r="20">
@@ -976,7 +976,7 @@
         <v>140776</v>
       </c>
       <c r="G20" t="n">
-        <v>1.29</v>
+        <v>1.299628924073683</v>
       </c>
     </row>
     <row r="21">
@@ -1003,7 +1003,7 @@
         <v>390188</v>
       </c>
       <c r="G21" t="n">
-        <v>19.4</v>
+        <v>19.40268523122824</v>
       </c>
     </row>
     <row r="22">
@@ -1030,7 +1030,7 @@
         <v>530011</v>
       </c>
       <c r="G22" t="n">
-        <v>31</v>
+        <v>31.00384264180015</v>
       </c>
     </row>
     <row r="23">
@@ -1057,7 +1057,7 @@
         <v>-147828</v>
       </c>
       <c r="G23" t="n">
-        <v>-7.18</v>
+        <v>-7.183090379008747</v>
       </c>
     </row>
     <row r="24">
@@ -1084,7 +1084,7 @@
         <v>2357820</v>
       </c>
       <c r="G24" t="n">
-        <v>32.68</v>
+        <v>32.68847913489532</v>
       </c>
     </row>
     <row r="25">
@@ -1111,7 +1111,7 @@
         <v>-92520</v>
       </c>
       <c r="G25" t="n">
-        <v>-4.69</v>
+        <v>-4.692871066258652</v>
       </c>
     </row>
     <row r="26">
@@ -1138,7 +1138,7 @@
         <v>232644</v>
       </c>
       <c r="G26" t="n">
-        <v>6.22</v>
+        <v>6.224755177396051</v>
       </c>
     </row>
     <row r="27">
@@ -1165,7 +1165,7 @@
         <v>-364064</v>
       </c>
       <c r="G27" t="n">
-        <v>-15.21</v>
+        <v>-15.21879441518268</v>
       </c>
     </row>
     <row r="28">
@@ -1192,7 +1192,7 @@
         <v>184383</v>
       </c>
       <c r="G28" t="n">
-        <v>27.72</v>
+        <v>27.72197289190591</v>
       </c>
     </row>
     <row r="29">
@@ -1219,7 +1219,7 @@
         <v>119092</v>
       </c>
       <c r="G29" t="n">
-        <v>14.29</v>
+        <v>14.29675870348139</v>
       </c>
     </row>
   </sheetData>
@@ -1277,7 +1277,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2026-03-18T11:45:14</t>
+          <t>2026-03-18T11:45:16</t>
         </is>
       </c>
       <c r="E2" t="n">

</xml_diff>

<commit_message>
auto: portfolio snapshot 2026-03-16 (2026-03-18T11:45:47)
</commit_message>
<xml_diff>
--- a/portfolio_auto.xlsx
+++ b/portfolio_auto.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G29"/>
+  <dimension ref="A1:G39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1220,6 +1220,276 @@
       </c>
       <c r="G29" t="n">
         <v>14.29675870348139</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>삼성화재</t>
+        </is>
+      </c>
+      <c r="B30" t="n">
+        <v>9</v>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="D30" t="n">
+        <v>1</v>
+      </c>
+      <c r="E30" t="n">
+        <v>4459563</v>
+      </c>
+      <c r="F30" t="n">
+        <v>-171437</v>
+      </c>
+      <c r="G30" t="n">
+        <v>-3.7</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>세아제강</t>
+        </is>
+      </c>
+      <c r="B31" t="n">
+        <v>50</v>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="D31" t="n">
+        <v>1</v>
+      </c>
+      <c r="E31" t="n">
+        <v>6866240</v>
+      </c>
+      <c r="F31" t="n">
+        <v>556240</v>
+      </c>
+      <c r="G31" t="n">
+        <v>8.81</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>케이씨</t>
+        </is>
+      </c>
+      <c r="B32" t="n">
+        <v>50</v>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="D32" t="n">
+        <v>1</v>
+      </c>
+      <c r="E32" t="n">
+        <v>1641710</v>
+      </c>
+      <c r="F32" t="n">
+        <v>-7790</v>
+      </c>
+      <c r="G32" t="n">
+        <v>-0.47</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>하나금융지주</t>
+        </is>
+      </c>
+      <c r="B33" t="n">
+        <v>15</v>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="D33" t="n">
+        <v>1</v>
+      </c>
+      <c r="E33" t="n">
+        <v>1724544</v>
+      </c>
+      <c r="F33" t="n">
+        <v>42044</v>
+      </c>
+      <c r="G33" t="n">
+        <v>2.49</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>현대제철</t>
+        </is>
+      </c>
+      <c r="B34" t="n">
+        <v>70</v>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="D34" t="n">
+        <v>1</v>
+      </c>
+      <c r="E34" t="n">
+        <v>2623243</v>
+      </c>
+      <c r="F34" t="n">
+        <v>-184257</v>
+      </c>
+      <c r="G34" t="n">
+        <v>-6.56</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>휴스틸</t>
+        </is>
+      </c>
+      <c r="B35" t="n">
+        <v>500</v>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="D35" t="n">
+        <v>1</v>
+      </c>
+      <c r="E35" t="n">
+        <v>2554880</v>
+      </c>
+      <c r="F35" t="n">
+        <v>276270</v>
+      </c>
+      <c r="G35" t="n">
+        <v>12.12</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>DL이앤씨</t>
+        </is>
+      </c>
+      <c r="B36" t="n">
+        <v>80</v>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="D36" t="n">
+        <v>1</v>
+      </c>
+      <c r="E36" t="n">
+        <v>4143696</v>
+      </c>
+      <c r="F36" t="n">
+        <v>732696</v>
+      </c>
+      <c r="G36" t="n">
+        <v>21.48</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>HD건설기계</t>
+        </is>
+      </c>
+      <c r="B37" t="n">
+        <v>31</v>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="D37" t="n">
+        <v>1</v>
+      </c>
+      <c r="E37" t="n">
+        <v>3947686</v>
+      </c>
+      <c r="F37" t="n">
+        <v>-87410</v>
+      </c>
+      <c r="G37" t="n">
+        <v>-2.16</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>KoAct 코스닥액티브</t>
+        </is>
+      </c>
+      <c r="B38" t="n">
+        <v>200</v>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="D38" t="n">
+        <v>1</v>
+      </c>
+      <c r="E38" t="n">
+        <v>2598000</v>
+      </c>
+      <c r="F38" t="n">
+        <v>-104000</v>
+      </c>
+      <c r="G38" t="n">
+        <v>-3.84</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>TIME 코리아밸류업액티브</t>
+        </is>
+      </c>
+      <c r="B39" t="n">
+        <v>201</v>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="D39" t="n">
+        <v>1</v>
+      </c>
+      <c r="E39" t="n">
+        <v>4904400</v>
+      </c>
+      <c r="F39" t="n">
+        <v>180603</v>
+      </c>
+      <c r="G39" t="n">
+        <v>3.82</v>
       </c>
     </row>
   </sheetData>
@@ -1277,7 +1547,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2026-03-18T11:45:16</t>
+          <t>2026-03-18T11:45:47</t>
         </is>
       </c>
       <c r="E2" t="n">

</xml_diff>

<commit_message>
auto: portfolio snapshot 2026-03-16 (2026-03-18T11:45:49)
</commit_message>
<xml_diff>
--- a/portfolio_auto.xlsx
+++ b/portfolio_auto.xlsx
@@ -1246,7 +1246,7 @@
         <v>-171437</v>
       </c>
       <c r="G30" t="n">
-        <v>-3.7</v>
+        <v>-3.701943424746275</v>
       </c>
     </row>
     <row r="31">
@@ -1267,13 +1267,13 @@
         <v>1</v>
       </c>
       <c r="E31" t="n">
-        <v>6866240</v>
+        <v>6866239.999999999</v>
       </c>
       <c r="F31" t="n">
-        <v>556240</v>
+        <v>556239.9999999991</v>
       </c>
       <c r="G31" t="n">
-        <v>8.81</v>
+        <v>8.815213946117259</v>
       </c>
     </row>
     <row r="32">
@@ -1297,10 +1297,10 @@
         <v>1641710</v>
       </c>
       <c r="F32" t="n">
-        <v>-7790</v>
+        <v>-7790.000000000233</v>
       </c>
       <c r="G32" t="n">
-        <v>-0.47</v>
+        <v>-0.4722643225219905</v>
       </c>
     </row>
     <row r="33">
@@ -1327,7 +1327,7 @@
         <v>42044</v>
       </c>
       <c r="G33" t="n">
-        <v>2.49</v>
+        <v>2.49890044576523</v>
       </c>
     </row>
     <row r="34">
@@ -1354,7 +1354,7 @@
         <v>-184257</v>
       </c>
       <c r="G34" t="n">
-        <v>-6.56</v>
+        <v>-6.563027604630454</v>
       </c>
     </row>
     <row r="35">
@@ -1381,7 +1381,7 @@
         <v>276270</v>
       </c>
       <c r="G35" t="n">
-        <v>12.12</v>
+        <v>12.12449695208921</v>
       </c>
     </row>
     <row r="36">
@@ -1408,7 +1408,7 @@
         <v>732696</v>
       </c>
       <c r="G36" t="n">
-        <v>21.48</v>
+        <v>21.48038698328936</v>
       </c>
     </row>
     <row r="37">
@@ -1435,7 +1435,7 @@
         <v>-87410</v>
       </c>
       <c r="G37" t="n">
-        <v>-2.16</v>
+        <v>-2.166243380578802</v>
       </c>
     </row>
     <row r="38">
@@ -1462,7 +1462,7 @@
         <v>-104000</v>
       </c>
       <c r="G38" t="n">
-        <v>-3.84</v>
+        <v>-3.84900074019245</v>
       </c>
     </row>
     <row r="39">
@@ -1489,7 +1489,7 @@
         <v>180603</v>
       </c>
       <c r="G39" t="n">
-        <v>3.82</v>
+        <v>3.823259128197084</v>
       </c>
     </row>
   </sheetData>
@@ -1547,7 +1547,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2026-03-18T11:45:47</t>
+          <t>2026-03-18T11:45:49</t>
         </is>
       </c>
       <c r="E2" t="n">

</xml_diff>

<commit_message>
auto: portfolio snapshot 2026-03-18 (2026-03-18T12:13:57)
</commit_message>
<xml_diff>
--- a/portfolio_auto.xlsx
+++ b/portfolio_auto.xlsx
@@ -469,11 +469,11 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>노브</t>
+          <t>페트로브라스 (ADR)</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>185</v>
+        <v>480</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
@@ -484,23 +484,23 @@
         <v>1</v>
       </c>
       <c r="E2" t="n">
-        <v>5140749</v>
+        <v>13956818</v>
       </c>
       <c r="F2" t="n">
-        <v>1830741</v>
+        <v>1850269</v>
       </c>
       <c r="G2" t="n">
-        <v>55.3092620924179</v>
+        <v>15.28320746068925</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>노블</t>
+          <t>AGNC 인베스트먼트</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>99</v>
+        <v>700</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
@@ -511,23 +511,23 @@
         <v>1</v>
       </c>
       <c r="E3" t="n">
-        <v>7024110</v>
+        <v>10972791</v>
       </c>
       <c r="F3" t="n">
-        <v>3116902</v>
+        <v>140776</v>
       </c>
       <c r="G3" t="n">
-        <v>79.77312700014947</v>
+        <v>1.299628924073683</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>더치 브로스</t>
+          <t>대한조선</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>39</v>
+        <v>100</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
@@ -538,23 +538,23 @@
         <v>1</v>
       </c>
       <c r="E4" t="n">
-        <v>2989154</v>
+        <v>9570820</v>
       </c>
       <c r="F4" t="n">
-        <v>-201490</v>
+        <v>2357820</v>
       </c>
       <c r="G4" t="n">
-        <v>-6.315026057435428</v>
+        <v>32.68847913489532</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>발레로 에너지</t>
+          <t>프론트라인</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>6</v>
+        <v>175</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -565,23 +565,23 @@
         <v>1</v>
       </c>
       <c r="E5" t="n">
-        <v>2109459</v>
+        <v>8314143.999999999</v>
       </c>
       <c r="F5" t="n">
-        <v>45469</v>
+        <v>3884279.999999999</v>
       </c>
       <c r="G5" t="n">
-        <v>2.202966099641956</v>
+        <v>87.68395598600767</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>센트러스 에너지</t>
+          <t>시드릴</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>21</v>
+        <v>123</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
@@ -592,23 +592,23 @@
         <v>1</v>
       </c>
       <c r="E6" t="n">
-        <v>6721336</v>
+        <v>8270678.999999999</v>
       </c>
       <c r="F6" t="n">
-        <v>490117.0000000009</v>
+        <v>1820327.999999999</v>
       </c>
       <c r="G6" t="n">
-        <v>7.865507535523965</v>
+        <v>28.22060380900201</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>스타 벌크 캐리어스</t>
+          <t>트랜스오션</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>50</v>
+        <v>750</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -619,23 +619,23 @@
         <v>1</v>
       </c>
       <c r="E7" t="n">
-        <v>1684783</v>
+        <v>7427805</v>
       </c>
       <c r="F7" t="n">
-        <v>370430.0000000002</v>
+        <v>3300571</v>
       </c>
       <c r="G7" t="n">
-        <v>28.18344843432474</v>
+        <v>79.97053232261607</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>시드릴</t>
+          <t>노블</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>123</v>
+        <v>99</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
@@ -646,23 +646,23 @@
         <v>1</v>
       </c>
       <c r="E8" t="n">
-        <v>8270678.999999999</v>
+        <v>7024110</v>
       </c>
       <c r="F8" t="n">
-        <v>1820327.999999999</v>
+        <v>3116902</v>
       </c>
       <c r="G8" t="n">
-        <v>28.22060380900201</v>
+        <v>79.77312700014947</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>오케아니스 에코 탱커스</t>
+          <t>세아제강</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>65</v>
+        <v>50</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
@@ -673,23 +673,23 @@
         <v>1</v>
       </c>
       <c r="E9" t="n">
-        <v>4572321</v>
+        <v>6866239.999999999</v>
       </c>
       <c r="F9" t="n">
-        <v>2315961</v>
+        <v>556239.9999999991</v>
       </c>
       <c r="G9" t="n">
-        <v>102.6414667872148</v>
+        <v>8.815213946117259</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>유나이티드헬스 그룹</t>
+          <t>센트러스 에너지</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>4</v>
+        <v>21</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
@@ -700,23 +700,23 @@
         <v>1</v>
       </c>
       <c r="E10" t="n">
-        <v>1710222</v>
+        <v>6721336</v>
       </c>
       <c r="F10" t="n">
-        <v>15766</v>
+        <v>490117.0000000009</v>
       </c>
       <c r="G10" t="n">
-        <v>0.9304461136789625</v>
+        <v>7.865507535523965</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>차코스 에너지 내비게이션</t>
+          <t>타이드워터</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>75</v>
+        <v>48</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
@@ -727,23 +727,23 @@
         <v>1</v>
       </c>
       <c r="E11" t="n">
-        <v>3892088</v>
+        <v>5469451</v>
       </c>
       <c r="F11" t="n">
-        <v>67440</v>
+        <v>1744906</v>
       </c>
       <c r="G11" t="n">
-        <v>1.763299524557554</v>
+        <v>46.84883656929907</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>클리블랜드 클리프스</t>
+          <t>노브</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>70</v>
+        <v>185</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
@@ -754,23 +754,23 @@
         <v>1</v>
       </c>
       <c r="E12" t="n">
-        <v>880384</v>
+        <v>5140749</v>
       </c>
       <c r="F12" t="n">
-        <v>-135671</v>
+        <v>1830741</v>
       </c>
       <c r="G12" t="n">
-        <v>-13.35272204752695</v>
+        <v>55.3092620924179</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>타이드워터</t>
+          <t>TIME 코리아밸류업액티브</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>48</v>
+        <v>201</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
@@ -781,23 +781,23 @@
         <v>1</v>
       </c>
       <c r="E13" t="n">
-        <v>5469451</v>
+        <v>4904400</v>
       </c>
       <c r="F13" t="n">
-        <v>1744906</v>
+        <v>180603</v>
       </c>
       <c r="G13" t="n">
-        <v>46.84883656929907</v>
+        <v>3.823259128197084</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>텍사스 퍼시픽 랜드</t>
+          <t>오케아니스 에코 탱커스</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>1</v>
+        <v>65</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
@@ -808,23 +808,23 @@
         <v>1</v>
       </c>
       <c r="E14" t="n">
-        <v>787419</v>
+        <v>4572321</v>
       </c>
       <c r="F14" t="n">
-        <v>8828</v>
+        <v>2315961</v>
       </c>
       <c r="G14" t="n">
-        <v>1.133843057523141</v>
+        <v>102.6414667872148</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>트랜스오션</t>
+          <t>삼성화재</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>750</v>
+        <v>9</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
@@ -835,23 +835,23 @@
         <v>1</v>
       </c>
       <c r="E15" t="n">
-        <v>7427805</v>
+        <v>4459563</v>
       </c>
       <c r="F15" t="n">
-        <v>3300571</v>
+        <v>-171437</v>
       </c>
       <c r="G15" t="n">
-        <v>79.97053232261607</v>
+        <v>-3.701943424746275</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>페트로브라스 (ADR)</t>
+          <t>DL이앤씨</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>480</v>
+        <v>80</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
@@ -862,23 +862,23 @@
         <v>1</v>
       </c>
       <c r="E16" t="n">
-        <v>13956818</v>
+        <v>4143696</v>
       </c>
       <c r="F16" t="n">
-        <v>1850269</v>
+        <v>732696</v>
       </c>
       <c r="G16" t="n">
-        <v>15.28320746068925</v>
+        <v>21.48038698328936</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>프론트라인</t>
+          <t>동원개발</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>175</v>
+        <v>1360</v>
       </c>
       <c r="C17" t="inlineStr">
         <is>
@@ -889,23 +889,23 @@
         <v>1</v>
       </c>
       <c r="E17" t="n">
-        <v>8314143.999999999</v>
+        <v>3970044</v>
       </c>
       <c r="F17" t="n">
-        <v>3884279.999999999</v>
+        <v>232644</v>
       </c>
       <c r="G17" t="n">
-        <v>87.68395598600767</v>
+        <v>6.224755177396051</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>피바디 에너지</t>
+          <t>HD건설기계</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>65</v>
+        <v>31</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
@@ -916,23 +916,23 @@
         <v>1</v>
       </c>
       <c r="E18" t="n">
-        <v>3417602</v>
+        <v>3947686</v>
       </c>
       <c r="F18" t="n">
-        <v>1946830</v>
+        <v>-87410</v>
       </c>
       <c r="G18" t="n">
-        <v>132.3678993073025</v>
+        <v>-2.166243380578802</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>하프니아</t>
+          <t>차코스 에너지 내비게이션</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>80</v>
+        <v>75</v>
       </c>
       <c r="C19" t="inlineStr">
         <is>
@@ -943,23 +943,23 @@
         <v>1</v>
       </c>
       <c r="E19" t="n">
-        <v>808815</v>
+        <v>3892088</v>
       </c>
       <c r="F19" t="n">
-        <v>183084</v>
+        <v>67440</v>
       </c>
       <c r="G19" t="n">
-        <v>29.25921841813814</v>
+        <v>1.763299524557554</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>AGNC 인베스트먼트</t>
+          <t>피바디 에너지</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>700</v>
+        <v>65</v>
       </c>
       <c r="C20" t="inlineStr">
         <is>
@@ -970,23 +970,23 @@
         <v>1</v>
       </c>
       <c r="E20" t="n">
-        <v>10972791</v>
+        <v>3417602</v>
       </c>
       <c r="F20" t="n">
-        <v>140776</v>
+        <v>1946830</v>
       </c>
       <c r="G20" t="n">
-        <v>1.299628924073683</v>
+        <v>132.3678993073025</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>넥스틸</t>
+          <t>더치 브로스</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>200</v>
+        <v>39</v>
       </c>
       <c r="C21" t="inlineStr">
         <is>
@@ -997,23 +997,23 @@
         <v>1</v>
       </c>
       <c r="E21" t="n">
-        <v>2401188</v>
+        <v>2989154</v>
       </c>
       <c r="F21" t="n">
-        <v>390188</v>
+        <v>-201490</v>
       </c>
       <c r="G21" t="n">
-        <v>19.40268523122824</v>
+        <v>-6.315026057435428</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>대신증권</t>
+          <t>현대제철</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>55</v>
+        <v>70</v>
       </c>
       <c r="C22" t="inlineStr">
         <is>
@@ -1024,23 +1024,23 @@
         <v>1</v>
       </c>
       <c r="E22" t="n">
-        <v>2239512</v>
+        <v>2623243</v>
       </c>
       <c r="F22" t="n">
-        <v>530011</v>
+        <v>-184257</v>
       </c>
       <c r="G22" t="n">
-        <v>31.00384264180015</v>
+        <v>-6.563027604630454</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>대창단조</t>
+          <t>KoAct 코스닥액티브</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>300</v>
+        <v>200</v>
       </c>
       <c r="C23" t="inlineStr">
         <is>
@@ -1051,23 +1051,23 @@
         <v>1</v>
       </c>
       <c r="E23" t="n">
-        <v>1910172</v>
+        <v>2598000</v>
       </c>
       <c r="F23" t="n">
-        <v>-147828</v>
+        <v>-104000</v>
       </c>
       <c r="G23" t="n">
-        <v>-7.183090379008747</v>
+        <v>-3.84900074019245</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>대한조선</t>
+          <t>휴스틸</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>100</v>
+        <v>500</v>
       </c>
       <c r="C24" t="inlineStr">
         <is>
@@ -1078,23 +1078,23 @@
         <v>1</v>
       </c>
       <c r="E24" t="n">
-        <v>9570820</v>
+        <v>2554880</v>
       </c>
       <c r="F24" t="n">
-        <v>2357820</v>
+        <v>276270</v>
       </c>
       <c r="G24" t="n">
-        <v>32.68847913489532</v>
+        <v>12.12449695208921</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>동방</t>
+          <t>넥스틸</t>
         </is>
       </c>
       <c r="B25" t="n">
-        <v>681</v>
+        <v>200</v>
       </c>
       <c r="C25" t="inlineStr">
         <is>
@@ -1105,23 +1105,23 @@
         <v>1</v>
       </c>
       <c r="E25" t="n">
-        <v>1878981</v>
+        <v>2401188</v>
       </c>
       <c r="F25" t="n">
-        <v>-92520</v>
+        <v>390188</v>
       </c>
       <c r="G25" t="n">
-        <v>-4.692871066258652</v>
+        <v>19.40268523122824</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>동원개발</t>
+          <t>대신증권</t>
         </is>
       </c>
       <c r="B26" t="n">
-        <v>1360</v>
+        <v>55</v>
       </c>
       <c r="C26" t="inlineStr">
         <is>
@@ -1132,23 +1132,23 @@
         <v>1</v>
       </c>
       <c r="E26" t="n">
-        <v>3970044</v>
+        <v>2239512</v>
       </c>
       <c r="F26" t="n">
-        <v>232644</v>
+        <v>530011</v>
       </c>
       <c r="G26" t="n">
-        <v>6.224755177396051</v>
+        <v>31.00384264180015</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>미창석유</t>
+          <t>발레로 에너지</t>
         </is>
       </c>
       <c r="B27" t="n">
-        <v>18</v>
+        <v>6</v>
       </c>
       <c r="C27" t="inlineStr">
         <is>
@@ -1159,23 +1159,23 @@
         <v>1</v>
       </c>
       <c r="E27" t="n">
-        <v>2028136</v>
+        <v>2109459</v>
       </c>
       <c r="F27" t="n">
-        <v>-364064</v>
+        <v>45469</v>
       </c>
       <c r="G27" t="n">
-        <v>-15.21879441518268</v>
+        <v>2.202966099641956</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>비에이치아이</t>
+          <t>미창석유</t>
         </is>
       </c>
       <c r="B28" t="n">
-        <v>8</v>
+        <v>18</v>
       </c>
       <c r="C28" t="inlineStr">
         <is>
@@ -1186,23 +1186,23 @@
         <v>1</v>
       </c>
       <c r="E28" t="n">
-        <v>849498</v>
+        <v>2028136</v>
       </c>
       <c r="F28" t="n">
-        <v>184383</v>
+        <v>-364064</v>
       </c>
       <c r="G28" t="n">
-        <v>27.72197289190591</v>
+        <v>-15.21879441518268</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>삼성생명</t>
+          <t>대창단조</t>
         </is>
       </c>
       <c r="B29" t="n">
-        <v>4</v>
+        <v>300</v>
       </c>
       <c r="C29" t="inlineStr">
         <is>
@@ -1213,23 +1213,23 @@
         <v>1</v>
       </c>
       <c r="E29" t="n">
-        <v>952092</v>
+        <v>1910172</v>
       </c>
       <c r="F29" t="n">
-        <v>119092</v>
+        <v>-147828</v>
       </c>
       <c r="G29" t="n">
-        <v>14.29675870348139</v>
+        <v>-7.183090379008747</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>삼성화재</t>
+          <t>동방</t>
         </is>
       </c>
       <c r="B30" t="n">
-        <v>9</v>
+        <v>681</v>
       </c>
       <c r="C30" t="inlineStr">
         <is>
@@ -1240,23 +1240,23 @@
         <v>1</v>
       </c>
       <c r="E30" t="n">
-        <v>4459563</v>
+        <v>1878981</v>
       </c>
       <c r="F30" t="n">
-        <v>-171437</v>
+        <v>-92520</v>
       </c>
       <c r="G30" t="n">
-        <v>-3.701943424746275</v>
+        <v>-4.692871066258652</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>세아제강</t>
+          <t>하나금융지주</t>
         </is>
       </c>
       <c r="B31" t="n">
-        <v>50</v>
+        <v>15</v>
       </c>
       <c r="C31" t="inlineStr">
         <is>
@@ -1267,23 +1267,23 @@
         <v>1</v>
       </c>
       <c r="E31" t="n">
-        <v>6866239.999999999</v>
+        <v>1724544</v>
       </c>
       <c r="F31" t="n">
-        <v>556239.9999999991</v>
+        <v>42044</v>
       </c>
       <c r="G31" t="n">
-        <v>8.815213946117259</v>
+        <v>2.49890044576523</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>케이씨</t>
+          <t>유나이티드헬스 그룹</t>
         </is>
       </c>
       <c r="B32" t="n">
-        <v>50</v>
+        <v>4</v>
       </c>
       <c r="C32" t="inlineStr">
         <is>
@@ -1294,23 +1294,23 @@
         <v>1</v>
       </c>
       <c r="E32" t="n">
-        <v>1641710</v>
+        <v>1710222</v>
       </c>
       <c r="F32" t="n">
-        <v>-7790.000000000233</v>
+        <v>15766</v>
       </c>
       <c r="G32" t="n">
-        <v>-0.4722643225219905</v>
+        <v>0.9304461136789625</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>하나금융지주</t>
+          <t>스타 벌크 캐리어스</t>
         </is>
       </c>
       <c r="B33" t="n">
-        <v>15</v>
+        <v>50</v>
       </c>
       <c r="C33" t="inlineStr">
         <is>
@@ -1321,23 +1321,23 @@
         <v>1</v>
       </c>
       <c r="E33" t="n">
-        <v>1724544</v>
+        <v>1684783</v>
       </c>
       <c r="F33" t="n">
-        <v>42044</v>
+        <v>370430.0000000002</v>
       </c>
       <c r="G33" t="n">
-        <v>2.49890044576523</v>
+        <v>28.18344843432474</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>현대제철</t>
+          <t>케이씨</t>
         </is>
       </c>
       <c r="B34" t="n">
-        <v>70</v>
+        <v>50</v>
       </c>
       <c r="C34" t="inlineStr">
         <is>
@@ -1348,23 +1348,23 @@
         <v>1</v>
       </c>
       <c r="E34" t="n">
-        <v>2623243</v>
+        <v>1641710</v>
       </c>
       <c r="F34" t="n">
-        <v>-184257</v>
+        <v>-7790.000000000233</v>
       </c>
       <c r="G34" t="n">
-        <v>-6.563027604630454</v>
+        <v>-0.4722643225219905</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>휴스틸</t>
+          <t>삼성생명</t>
         </is>
       </c>
       <c r="B35" t="n">
-        <v>500</v>
+        <v>4</v>
       </c>
       <c r="C35" t="inlineStr">
         <is>
@@ -1375,23 +1375,23 @@
         <v>1</v>
       </c>
       <c r="E35" t="n">
-        <v>2554880</v>
+        <v>952092</v>
       </c>
       <c r="F35" t="n">
-        <v>276270</v>
+        <v>119092</v>
       </c>
       <c r="G35" t="n">
-        <v>12.12449695208921</v>
+        <v>14.29675870348139</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>DL이앤씨</t>
+          <t>클리블랜드 클리프스</t>
         </is>
       </c>
       <c r="B36" t="n">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="C36" t="inlineStr">
         <is>
@@ -1402,23 +1402,23 @@
         <v>1</v>
       </c>
       <c r="E36" t="n">
-        <v>4143696</v>
+        <v>880384</v>
       </c>
       <c r="F36" t="n">
-        <v>732696</v>
+        <v>-135671</v>
       </c>
       <c r="G36" t="n">
-        <v>21.48038698328936</v>
+        <v>-13.35272204752695</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>HD건설기계</t>
+          <t>비에이치아이</t>
         </is>
       </c>
       <c r="B37" t="n">
-        <v>31</v>
+        <v>8</v>
       </c>
       <c r="C37" t="inlineStr">
         <is>
@@ -1429,23 +1429,23 @@
         <v>1</v>
       </c>
       <c r="E37" t="n">
-        <v>3947686</v>
+        <v>849498</v>
       </c>
       <c r="F37" t="n">
-        <v>-87410</v>
+        <v>184383</v>
       </c>
       <c r="G37" t="n">
-        <v>-2.166243380578802</v>
+        <v>27.72197289190591</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>KoAct 코스닥액티브</t>
+          <t>하프니아</t>
         </is>
       </c>
       <c r="B38" t="n">
-        <v>200</v>
+        <v>80</v>
       </c>
       <c r="C38" t="inlineStr">
         <is>
@@ -1456,23 +1456,23 @@
         <v>1</v>
       </c>
       <c r="E38" t="n">
-        <v>2598000</v>
+        <v>808815</v>
       </c>
       <c r="F38" t="n">
-        <v>-104000</v>
+        <v>183084</v>
       </c>
       <c r="G38" t="n">
-        <v>-3.84900074019245</v>
+        <v>29.25921841813814</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>TIME 코리아밸류업액티브</t>
+          <t>텍사스 퍼시픽 랜드</t>
         </is>
       </c>
       <c r="B39" t="n">
-        <v>201</v>
+        <v>1</v>
       </c>
       <c r="C39" t="inlineStr">
         <is>
@@ -1483,13 +1483,13 @@
         <v>1</v>
       </c>
       <c r="E39" t="n">
-        <v>4904400</v>
+        <v>787419</v>
       </c>
       <c r="F39" t="n">
-        <v>180603</v>
+        <v>8828</v>
       </c>
       <c r="G39" t="n">
-        <v>3.823259128197084</v>
+        <v>1.133843057523141</v>
       </c>
     </row>
   </sheetData>
@@ -1536,7 +1536,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-03-16</t>
+          <t>2026-03-18</t>
         </is>
       </c>
       <c r="B2" t="n">
@@ -1547,11 +1547,11 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2026-03-18T11:45:49</t>
+          <t>2026-03-18T12:13:57</t>
         </is>
       </c>
       <c r="E2" t="n">
-        <v>1501.75</v>
+        <v>1485.880004882812</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
auto: portfolio snapshot 2026-03-18 (2026-03-18T12:21:00)
</commit_message>
<xml_diff>
--- a/portfolio_auto.xlsx
+++ b/portfolio_auto.xlsx
@@ -1300,7 +1300,7 @@
         <v>15766</v>
       </c>
       <c r="G32" t="n">
-        <v>0.9304461136789625</v>
+        <v>0.9304461136789623</v>
       </c>
     </row>
     <row r="33">
@@ -1547,7 +1547,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2026-03-18T12:13:57</t>
+          <t>2026-03-18T12:21:00</t>
         </is>
       </c>
       <c r="E2" t="n">

</xml_diff>

<commit_message>
auto: portfolio snapshot 2026-03-18 (2026-03-18T12:21:28)
</commit_message>
<xml_diff>
--- a/portfolio_auto.xlsx
+++ b/portfolio_auto.xlsx
@@ -1300,7 +1300,7 @@
         <v>15766</v>
       </c>
       <c r="G32" t="n">
-        <v>0.9304461136789623</v>
+        <v>0.9304461136789625</v>
       </c>
     </row>
     <row r="33">
@@ -1324,10 +1324,10 @@
         <v>1684783</v>
       </c>
       <c r="F33" t="n">
-        <v>370430.0000000002</v>
+        <v>370430.0000000005</v>
       </c>
       <c r="G33" t="n">
-        <v>28.18344843432474</v>
+        <v>28.18344843432476</v>
       </c>
     </row>
     <row r="34">
@@ -1351,10 +1351,10 @@
         <v>1641710</v>
       </c>
       <c r="F34" t="n">
-        <v>-7790.000000000233</v>
+        <v>-7790.000000000698</v>
       </c>
       <c r="G34" t="n">
-        <v>-0.4722643225219905</v>
+        <v>-0.4722643225220186</v>
       </c>
     </row>
     <row r="35">
@@ -1547,7 +1547,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2026-03-18T12:21:00</t>
+          <t>2026-03-18T12:21:28</t>
         </is>
       </c>
       <c r="E2" t="n">

</xml_diff>

<commit_message>
auto: portfolio snapshot 2026-03-18 (2026-03-18T13:53:57)
</commit_message>
<xml_diff>
--- a/portfolio_auto.xlsx
+++ b/portfolio_auto.xlsx
@@ -484,13 +484,13 @@
         <v>1</v>
       </c>
       <c r="E2" t="n">
-        <v>13956818</v>
+        <v>14061179.77103613</v>
       </c>
       <c r="F2" t="n">
-        <v>1850269</v>
+        <v>1954630.771036133</v>
       </c>
       <c r="G2" t="n">
-        <v>15.28320746068925</v>
+        <v>16.14523487276294</v>
       </c>
     </row>
     <row r="3">
@@ -511,13 +511,13 @@
         <v>1</v>
       </c>
       <c r="E3" t="n">
-        <v>10972791</v>
+        <v>10796404.23451035</v>
       </c>
       <c r="F3" t="n">
-        <v>140776</v>
+        <v>-35610.76548965462</v>
       </c>
       <c r="G3" t="n">
-        <v>1.299628924073683</v>
+        <v>-0.3287547652920958</v>
       </c>
     </row>
     <row r="4">
@@ -538,13 +538,13 @@
         <v>1</v>
       </c>
       <c r="E4" t="n">
-        <v>9570820</v>
+        <v>9570000</v>
       </c>
       <c r="F4" t="n">
-        <v>2357820</v>
+        <v>2357000</v>
       </c>
       <c r="G4" t="n">
-        <v>32.68847913489532</v>
+        <v>32.67711077221684</v>
       </c>
     </row>
     <row r="5">
@@ -565,13 +565,13 @@
         <v>1</v>
       </c>
       <c r="E5" t="n">
-        <v>8314143.999999999</v>
+        <v>8263721.825703507</v>
       </c>
       <c r="F5" t="n">
-        <v>3884279.999999999</v>
+        <v>3833857.825703507</v>
       </c>
       <c r="G5" t="n">
-        <v>87.68395598600767</v>
+        <v>86.54572297712768</v>
       </c>
     </row>
     <row r="6">
@@ -592,13 +592,13 @@
         <v>1</v>
       </c>
       <c r="E6" t="n">
-        <v>8270678.999999999</v>
+        <v>8129308.858251691</v>
       </c>
       <c r="F6" t="n">
-        <v>1820327.999999999</v>
+        <v>1678957.858251691</v>
       </c>
       <c r="G6" t="n">
-        <v>28.22060380900201</v>
+        <v>26.02893793301622</v>
       </c>
     </row>
     <row r="7">
@@ -619,23 +619,23 @@
         <v>1</v>
       </c>
       <c r="E7" t="n">
-        <v>7427805</v>
+        <v>7210232.489881324</v>
       </c>
       <c r="F7" t="n">
-        <v>3300571</v>
+        <v>3082998.489881324</v>
       </c>
       <c r="G7" t="n">
-        <v>79.97053232261607</v>
+        <v>74.69890221589867</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>노블</t>
+          <t>세아제강</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>99</v>
+        <v>50</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
@@ -646,23 +646,23 @@
         <v>1</v>
       </c>
       <c r="E8" t="n">
-        <v>7024110</v>
+        <v>6915000</v>
       </c>
       <c r="F8" t="n">
-        <v>3116902</v>
+        <v>605000</v>
       </c>
       <c r="G8" t="n">
-        <v>79.77312700014947</v>
+        <v>9.587955625990491</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>세아제강</t>
+          <t>센트러스 에너지</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>50</v>
+        <v>21</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
@@ -673,23 +673,23 @@
         <v>1</v>
       </c>
       <c r="E9" t="n">
-        <v>6866239.999999999</v>
+        <v>6611393.516486719</v>
       </c>
       <c r="F9" t="n">
-        <v>556239.9999999991</v>
+        <v>380174.5164867202</v>
       </c>
       <c r="G9" t="n">
-        <v>8.815213946117259</v>
+        <v>6.101125903081247</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>센트러스 에너지</t>
+          <t>타이드워터</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>21</v>
+        <v>48</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
@@ -700,23 +700,23 @@
         <v>1</v>
       </c>
       <c r="E10" t="n">
-        <v>6721336</v>
+        <v>5478261.098275781</v>
       </c>
       <c r="F10" t="n">
-        <v>490117.0000000009</v>
+        <v>1753716.098275781</v>
       </c>
       <c r="G10" t="n">
-        <v>7.865507535523965</v>
+        <v>47.08537816768976</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>타이드워터</t>
+          <t>노브</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>48</v>
+        <v>185</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
@@ -727,23 +727,23 @@
         <v>1</v>
       </c>
       <c r="E11" t="n">
-        <v>5469451</v>
+        <v>5132155.263837265</v>
       </c>
       <c r="F11" t="n">
-        <v>1744906</v>
+        <v>1822147.263837265</v>
       </c>
       <c r="G11" t="n">
-        <v>46.84883656929907</v>
+        <v>55.04963322859838</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>노브</t>
+          <t>TIME 코리아밸류업액티브</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>185</v>
+        <v>201</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
@@ -754,23 +754,23 @@
         <v>1</v>
       </c>
       <c r="E12" t="n">
-        <v>5140749</v>
+        <v>4904400</v>
       </c>
       <c r="F12" t="n">
-        <v>1830741</v>
+        <v>180603</v>
       </c>
       <c r="G12" t="n">
-        <v>55.3092620924179</v>
+        <v>3.823259128197084</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>TIME 코리아밸류업액티브</t>
+          <t>오케아니스 에코 탱커스</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>201</v>
+        <v>65</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
@@ -781,23 +781,23 @@
         <v>1</v>
       </c>
       <c r="E13" t="n">
-        <v>4904400</v>
+        <v>4535500.038480652</v>
       </c>
       <c r="F13" t="n">
-        <v>180603</v>
+        <v>2279140.038480652</v>
       </c>
       <c r="G13" t="n">
-        <v>3.823259128197084</v>
+        <v>101.0095923735863</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>오케아니스 에코 탱커스</t>
+          <t>삼성화재</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>65</v>
+        <v>9</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
@@ -808,23 +808,23 @@
         <v>1</v>
       </c>
       <c r="E14" t="n">
-        <v>4572321</v>
+        <v>4446000</v>
       </c>
       <c r="F14" t="n">
-        <v>2315961</v>
+        <v>-185000</v>
       </c>
       <c r="G14" t="n">
-        <v>102.6414667872148</v>
+        <v>-3.994817534009933</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>삼성화재</t>
+          <t>DL이앤씨</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>9</v>
+        <v>80</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
@@ -835,23 +835,23 @@
         <v>1</v>
       </c>
       <c r="E15" t="n">
-        <v>4459563</v>
+        <v>4128000</v>
       </c>
       <c r="F15" t="n">
-        <v>-171437</v>
+        <v>717000</v>
       </c>
       <c r="G15" t="n">
-        <v>-3.701943424746275</v>
+        <v>21.02022867194371</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>DL이앤씨</t>
+          <t>동원개발</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>80</v>
+        <v>1360</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
@@ -862,23 +862,23 @@
         <v>1</v>
       </c>
       <c r="E16" t="n">
-        <v>4143696</v>
+        <v>3978000</v>
       </c>
       <c r="F16" t="n">
-        <v>732696</v>
+        <v>240600</v>
       </c>
       <c r="G16" t="n">
-        <v>21.48038698328936</v>
+        <v>6.437630438272596</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>동원개발</t>
+          <t>HD건설기계</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>1360</v>
+        <v>31</v>
       </c>
       <c r="C17" t="inlineStr">
         <is>
@@ -889,23 +889,23 @@
         <v>1</v>
       </c>
       <c r="E17" t="n">
-        <v>3970044</v>
+        <v>3955600</v>
       </c>
       <c r="F17" t="n">
-        <v>232644</v>
+        <v>-79496</v>
       </c>
       <c r="G17" t="n">
-        <v>6.224755177396051</v>
+        <v>-1.970114217852561</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>HD건설기계</t>
+          <t>차코스 에너지 내비게이션</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>31</v>
+        <v>75</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
@@ -916,23 +916,23 @@
         <v>1</v>
       </c>
       <c r="E18" t="n">
-        <v>3947686</v>
+        <v>3915702.545498475</v>
       </c>
       <c r="F18" t="n">
-        <v>-87410</v>
+        <v>91054.5454984745</v>
       </c>
       <c r="G18" t="n">
-        <v>-2.166243380578802</v>
+        <v>2.3807300828331</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>차코스 에너지 내비게이션</t>
+          <t>피바디 에너지</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>75</v>
+        <v>65</v>
       </c>
       <c r="C19" t="inlineStr">
         <is>
@@ -943,23 +943,23 @@
         <v>1</v>
       </c>
       <c r="E19" t="n">
-        <v>3892088</v>
+        <v>3381342.671001556</v>
       </c>
       <c r="F19" t="n">
-        <v>67440</v>
+        <v>1910570.671001556</v>
       </c>
       <c r="G19" t="n">
-        <v>1.763299524557554</v>
+        <v>129.9025730025834</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>피바디 에너지</t>
+          <t>더치 브로스</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>65</v>
+        <v>39</v>
       </c>
       <c r="C20" t="inlineStr">
         <is>
@@ -970,23 +970,23 @@
         <v>1</v>
       </c>
       <c r="E20" t="n">
-        <v>3417602</v>
+        <v>3030170.005811756</v>
       </c>
       <c r="F20" t="n">
-        <v>1946830</v>
+        <v>-160473.9941882445</v>
       </c>
       <c r="G20" t="n">
-        <v>132.3678993073025</v>
+        <v>-5.02951736979257</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>더치 브로스</t>
+          <t>현대제철</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>39</v>
+        <v>70</v>
       </c>
       <c r="C21" t="inlineStr">
         <is>
@@ -997,23 +997,23 @@
         <v>1</v>
       </c>
       <c r="E21" t="n">
-        <v>2989154</v>
+        <v>2607500</v>
       </c>
       <c r="F21" t="n">
-        <v>-201490</v>
+        <v>-200000</v>
       </c>
       <c r="G21" t="n">
-        <v>-6.315026057435428</v>
+        <v>-7.123775601068566</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>현대제철</t>
+          <t>KoAct 코스닥액티브</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>70</v>
+        <v>200</v>
       </c>
       <c r="C22" t="inlineStr">
         <is>
@@ -1024,23 +1024,23 @@
         <v>1</v>
       </c>
       <c r="E22" t="n">
-        <v>2623243</v>
+        <v>2598000</v>
       </c>
       <c r="F22" t="n">
-        <v>-184257</v>
+        <v>-104000</v>
       </c>
       <c r="G22" t="n">
-        <v>-6.563027604630454</v>
+        <v>-3.84900074019245</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>KoAct 코스닥액티브</t>
+          <t>휴스틸</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>200</v>
+        <v>500</v>
       </c>
       <c r="C23" t="inlineStr">
         <is>
@@ -1051,23 +1051,23 @@
         <v>1</v>
       </c>
       <c r="E23" t="n">
-        <v>2598000</v>
+        <v>2560000</v>
       </c>
       <c r="F23" t="n">
-        <v>-104000</v>
+        <v>281390</v>
       </c>
       <c r="G23" t="n">
-        <v>-3.84900074019245</v>
+        <v>12.34919534277476</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>휴스틸</t>
+          <t>넥스틸</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>500</v>
+        <v>200</v>
       </c>
       <c r="C24" t="inlineStr">
         <is>
@@ -1078,23 +1078,23 @@
         <v>1</v>
       </c>
       <c r="E24" t="n">
-        <v>2554880</v>
+        <v>2400000</v>
       </c>
       <c r="F24" t="n">
-        <v>276270</v>
+        <v>389000</v>
       </c>
       <c r="G24" t="n">
-        <v>12.12449695208921</v>
+        <v>19.34361014420686</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>넥스틸</t>
+          <t>대신증권</t>
         </is>
       </c>
       <c r="B25" t="n">
-        <v>200</v>
+        <v>55</v>
       </c>
       <c r="C25" t="inlineStr">
         <is>
@@ -1105,23 +1105,23 @@
         <v>1</v>
       </c>
       <c r="E25" t="n">
-        <v>2401188</v>
+        <v>2238500</v>
       </c>
       <c r="F25" t="n">
-        <v>390188</v>
+        <v>528999</v>
       </c>
       <c r="G25" t="n">
-        <v>19.40268523122824</v>
+        <v>30.94464408034859</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>대신증권</t>
+          <t>발레로 에너지</t>
         </is>
       </c>
       <c r="B26" t="n">
-        <v>55</v>
+        <v>6</v>
       </c>
       <c r="C26" t="inlineStr">
         <is>
@@ -1132,23 +1132,23 @@
         <v>1</v>
       </c>
       <c r="E26" t="n">
-        <v>2239512</v>
+        <v>2145997.115708057</v>
       </c>
       <c r="F26" t="n">
-        <v>530011</v>
+        <v>82007.11570805684</v>
       </c>
       <c r="G26" t="n">
-        <v>31.00384264180015</v>
+        <v>3.973232220507698</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>발레로 에너지</t>
+          <t>미창석유</t>
         </is>
       </c>
       <c r="B27" t="n">
-        <v>6</v>
+        <v>18</v>
       </c>
       <c r="C27" t="inlineStr">
         <is>
@@ -1159,23 +1159,23 @@
         <v>1</v>
       </c>
       <c r="E27" t="n">
-        <v>2109459</v>
+        <v>2032200</v>
       </c>
       <c r="F27" t="n">
-        <v>45469</v>
+        <v>-360000</v>
       </c>
       <c r="G27" t="n">
-        <v>2.202966099641956</v>
+        <v>-15.04890895410083</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>미창석유</t>
+          <t>대창단조</t>
         </is>
       </c>
       <c r="B28" t="n">
-        <v>18</v>
+        <v>300</v>
       </c>
       <c r="C28" t="inlineStr">
         <is>
@@ -1186,23 +1186,23 @@
         <v>1</v>
       </c>
       <c r="E28" t="n">
-        <v>2028136</v>
+        <v>1914000</v>
       </c>
       <c r="F28" t="n">
-        <v>-364064</v>
+        <v>-144000</v>
       </c>
       <c r="G28" t="n">
-        <v>-15.21879441518268</v>
+        <v>-6.997084548104956</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>대창단조</t>
+          <t>동방</t>
         </is>
       </c>
       <c r="B29" t="n">
-        <v>300</v>
+        <v>681</v>
       </c>
       <c r="C29" t="inlineStr">
         <is>
@@ -1213,23 +1213,23 @@
         <v>1</v>
       </c>
       <c r="E29" t="n">
-        <v>1910172</v>
+        <v>1882965</v>
       </c>
       <c r="F29" t="n">
-        <v>-147828</v>
+        <v>-88536</v>
       </c>
       <c r="G29" t="n">
-        <v>-7.183090379008747</v>
+        <v>-4.490791533963209</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>동방</t>
+          <t>하나금융지주</t>
         </is>
       </c>
       <c r="B30" t="n">
-        <v>681</v>
+        <v>15</v>
       </c>
       <c r="C30" t="inlineStr">
         <is>
@@ -1240,23 +1240,23 @@
         <v>1</v>
       </c>
       <c r="E30" t="n">
-        <v>1878981</v>
+        <v>1717500</v>
       </c>
       <c r="F30" t="n">
-        <v>-92520</v>
+        <v>35000</v>
       </c>
       <c r="G30" t="n">
-        <v>-4.692871066258652</v>
+        <v>2.080237741456166</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>하나금융지주</t>
+          <t>유나이티드헬스 그룹</t>
         </is>
       </c>
       <c r="B31" t="n">
-        <v>15</v>
+        <v>4</v>
       </c>
       <c r="C31" t="inlineStr">
         <is>
@@ -1267,23 +1267,23 @@
         <v>1</v>
       </c>
       <c r="E31" t="n">
-        <v>1724544</v>
+        <v>1710129.080517188</v>
       </c>
       <c r="F31" t="n">
-        <v>42044</v>
+        <v>15673.08051718771</v>
       </c>
       <c r="G31" t="n">
-        <v>2.49890044576523</v>
+        <v>0.9249623783201047</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>유나이티드헬스 그룹</t>
+          <t>스타 벌크 캐리어스</t>
         </is>
       </c>
       <c r="B32" t="n">
-        <v>4</v>
+        <v>50</v>
       </c>
       <c r="C32" t="inlineStr">
         <is>
@@ -1294,19 +1294,19 @@
         <v>1</v>
       </c>
       <c r="E32" t="n">
-        <v>1710222</v>
+        <v>1695389.062898559</v>
       </c>
       <c r="F32" t="n">
-        <v>15766</v>
+        <v>381036.06289856</v>
       </c>
       <c r="G32" t="n">
-        <v>0.9304461136789625</v>
+        <v>28.99039016904592</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>스타 벌크 캐리어스</t>
+          <t>케이씨</t>
         </is>
       </c>
       <c r="B33" t="n">
@@ -1321,23 +1321,23 @@
         <v>1</v>
       </c>
       <c r="E33" t="n">
-        <v>1684783</v>
+        <v>1640000</v>
       </c>
       <c r="F33" t="n">
-        <v>370430.0000000005</v>
+        <v>-9500.000000000698</v>
       </c>
       <c r="G33" t="n">
-        <v>28.18344843432476</v>
+        <v>-0.5759321006365986</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>케이씨</t>
+          <t>삼성생명</t>
         </is>
       </c>
       <c r="B34" t="n">
-        <v>50</v>
+        <v>4</v>
       </c>
       <c r="C34" t="inlineStr">
         <is>
@@ -1348,23 +1348,23 @@
         <v>1</v>
       </c>
       <c r="E34" t="n">
-        <v>1641710</v>
+        <v>940000</v>
       </c>
       <c r="F34" t="n">
-        <v>-7790.000000000698</v>
+        <v>107000</v>
       </c>
       <c r="G34" t="n">
-        <v>-0.4722643225220186</v>
+        <v>12.84513805522209</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>삼성생명</t>
+          <t>클리블랜드 클리프스</t>
         </is>
       </c>
       <c r="B35" t="n">
-        <v>4</v>
+        <v>70</v>
       </c>
       <c r="C35" t="inlineStr">
         <is>
@@ -1375,23 +1375,23 @@
         <v>1</v>
       </c>
       <c r="E35" t="n">
-        <v>952092</v>
+        <v>866936.6928166046</v>
       </c>
       <c r="F35" t="n">
-        <v>119092</v>
+        <v>-149118.3071833954</v>
       </c>
       <c r="G35" t="n">
-        <v>14.29675870348139</v>
+        <v>-14.6762042589619</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>클리블랜드 클리프스</t>
+          <t>비에이치아이</t>
         </is>
       </c>
       <c r="B36" t="n">
-        <v>70</v>
+        <v>8</v>
       </c>
       <c r="C36" t="inlineStr">
         <is>
@@ -1402,23 +1402,23 @@
         <v>1</v>
       </c>
       <c r="E36" t="n">
-        <v>880384</v>
+        <v>844800</v>
       </c>
       <c r="F36" t="n">
-        <v>-135671</v>
+        <v>179685</v>
       </c>
       <c r="G36" t="n">
-        <v>-13.35272204752695</v>
+        <v>27.01562887620938</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>비에이치아이</t>
+          <t>하프니아</t>
         </is>
       </c>
       <c r="B37" t="n">
-        <v>8</v>
+        <v>80</v>
       </c>
       <c r="C37" t="inlineStr">
         <is>
@@ -1429,23 +1429,23 @@
         <v>1</v>
       </c>
       <c r="E37" t="n">
-        <v>849498</v>
+        <v>817210.2530013258</v>
       </c>
       <c r="F37" t="n">
-        <v>184383</v>
+        <v>191479.2530013258</v>
       </c>
       <c r="G37" t="n">
-        <v>27.72197289190591</v>
+        <v>30.60088967964281</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>하프니아</t>
+          <t>텍사스 퍼시픽 랜드</t>
         </is>
       </c>
       <c r="B38" t="n">
-        <v>80</v>
+        <v>1</v>
       </c>
       <c r="C38" t="inlineStr">
         <is>
@@ -1456,23 +1456,23 @@
         <v>1</v>
       </c>
       <c r="E38" t="n">
-        <v>808815</v>
+        <v>788827.7025751099</v>
       </c>
       <c r="F38" t="n">
-        <v>183084</v>
+        <v>10236.7025751099</v>
       </c>
       <c r="G38" t="n">
-        <v>29.25921841813814</v>
+        <v>1.314772785083555</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>텍사스 퍼시픽 랜드</t>
+          <t>노블</t>
         </is>
       </c>
       <c r="B39" t="n">
-        <v>1</v>
+        <v>99</v>
       </c>
       <c r="C39" t="inlineStr">
         <is>
@@ -1483,13 +1483,13 @@
         <v>1</v>
       </c>
       <c r="E39" t="n">
-        <v>787419</v>
+        <v>40689</v>
       </c>
       <c r="F39" t="n">
-        <v>8828</v>
+        <v>-3866519</v>
       </c>
       <c r="G39" t="n">
-        <v>1.133843057523141</v>
+        <v>-98.95861699709869</v>
       </c>
     </row>
   </sheetData>
@@ -1547,7 +1547,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2026-03-18T12:21:28</t>
+          <t>2026-03-18T13:53:57</t>
         </is>
       </c>
       <c r="E2" t="n">

</xml_diff>

<commit_message>
auto: portfolio snapshot 2026-03-17 (2026-03-18T14:28:05)
</commit_message>
<xml_diff>
--- a/portfolio_auto.xlsx
+++ b/portfolio_auto.xlsx
@@ -1489,7 +1489,7 @@
         <v>-3866519</v>
       </c>
       <c r="G39" t="n">
-        <v>-98.95861699709869</v>
+        <v>-98.95861699709867</v>
       </c>
     </row>
   </sheetData>
@@ -1536,22 +1536,22 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-03-18</t>
+          <t>2026-03-17</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>31505056</v>
+        <v>33078556</v>
       </c>
       <c r="C2" t="n">
-        <v>6016.63</v>
+        <v>6010.99</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2026-03-18T14:26:54</t>
+          <t>2026-03-18T14:28:05</t>
         </is>
       </c>
       <c r="E2" t="n">
-        <v>1485.880004882812</v>
+        <v>1488.910034179688</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
auto: portfolio snapshot 2026-03-17 (2026-03-18T14:29:29)
</commit_message>
<xml_diff>
--- a/portfolio_auto.xlsx
+++ b/portfolio_auto.xlsx
@@ -487,10 +487,10 @@
         <v>14061179.77103613</v>
       </c>
       <c r="F2" t="n">
-        <v>1954630.771036133</v>
+        <v>1954630.771036137</v>
       </c>
       <c r="G2" t="n">
-        <v>16.14523487276294</v>
+        <v>16.14523487276298</v>
       </c>
     </row>
     <row r="3">
@@ -514,10 +514,10 @@
         <v>10796404.23451035</v>
       </c>
       <c r="F3" t="n">
-        <v>-35610.76548965462</v>
+        <v>-35610.76548965834</v>
       </c>
       <c r="G3" t="n">
-        <v>-0.3287547652920958</v>
+        <v>-0.3287547652921301</v>
       </c>
     </row>
     <row r="4">
@@ -625,7 +625,7 @@
         <v>3082998.489881324</v>
       </c>
       <c r="G7" t="n">
-        <v>74.69890221589867</v>
+        <v>74.6989022158987</v>
       </c>
     </row>
     <row r="8">
@@ -919,10 +919,10 @@
         <v>3915702.545498475</v>
       </c>
       <c r="F18" t="n">
-        <v>91054.5454984745</v>
+        <v>91054.54549847404</v>
       </c>
       <c r="G18" t="n">
-        <v>2.3807300828331</v>
+        <v>2.380730082833088</v>
       </c>
     </row>
     <row r="19">
@@ -973,10 +973,10 @@
         <v>3030170.005811756</v>
       </c>
       <c r="F20" t="n">
-        <v>-160473.9941882445</v>
+        <v>-160473.9941882449</v>
       </c>
       <c r="G20" t="n">
-        <v>-5.02951736979257</v>
+        <v>-5.029517369792584</v>
       </c>
     </row>
     <row r="21">
@@ -1270,10 +1270,10 @@
         <v>1710129.080517188</v>
       </c>
       <c r="F31" t="n">
-        <v>15673.08051718771</v>
+        <v>15673.08051718748</v>
       </c>
       <c r="G31" t="n">
-        <v>0.9249623783201047</v>
+        <v>0.9249623783200909</v>
       </c>
     </row>
     <row r="32">
@@ -1297,10 +1297,10 @@
         <v>1695389.062898559</v>
       </c>
       <c r="F32" t="n">
-        <v>381036.06289856</v>
+        <v>381036.0628985604</v>
       </c>
       <c r="G32" t="n">
-        <v>28.99039016904592</v>
+        <v>28.99039016904597</v>
       </c>
     </row>
     <row r="33">
@@ -1489,7 +1489,7 @@
         <v>-3866519</v>
       </c>
       <c r="G39" t="n">
-        <v>-98.95861699709867</v>
+        <v>-98.95861699709869</v>
       </c>
     </row>
   </sheetData>
@@ -1547,7 +1547,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2026-03-18T14:28:05</t>
+          <t>2026-03-18T14:29:29</t>
         </is>
       </c>
       <c r="E2" t="n">

</xml_diff>

<commit_message>
auto: portfolio snapshot 2026-03-17 (2026-03-18T14:30:27)
</commit_message>
<xml_diff>
--- a/portfolio_auto.xlsx
+++ b/portfolio_auto.xlsx
@@ -631,11 +631,11 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>세아제강</t>
+          <t>센트러스 에너지</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>50</v>
+        <v>21</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
@@ -646,23 +646,23 @@
         <v>1</v>
       </c>
       <c r="E8" t="n">
-        <v>6915000</v>
+        <v>6611393.516486719</v>
       </c>
       <c r="F8" t="n">
-        <v>605000</v>
+        <v>380174.5164867202</v>
       </c>
       <c r="G8" t="n">
-        <v>9.587955625990491</v>
+        <v>6.101125903081247</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>센트러스 에너지</t>
+          <t>타이드워터</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>21</v>
+        <v>48</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
@@ -673,23 +673,23 @@
         <v>1</v>
       </c>
       <c r="E9" t="n">
-        <v>6611393.516486719</v>
+        <v>5478261.098275781</v>
       </c>
       <c r="F9" t="n">
-        <v>380174.5164867202</v>
+        <v>1753716.098275781</v>
       </c>
       <c r="G9" t="n">
-        <v>6.101125903081247</v>
+        <v>47.08537816768976</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>타이드워터</t>
+          <t>노브</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>48</v>
+        <v>185</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
@@ -700,23 +700,23 @@
         <v>1</v>
       </c>
       <c r="E10" t="n">
-        <v>5478261.098275781</v>
+        <v>5132155.263837265</v>
       </c>
       <c r="F10" t="n">
-        <v>1753716.098275781</v>
+        <v>1822147.263837265</v>
       </c>
       <c r="G10" t="n">
-        <v>47.08537816768976</v>
+        <v>55.04963322859838</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>노브</t>
+          <t>오케아니스 에코 탱커스</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>185</v>
+        <v>65</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
@@ -727,23 +727,23 @@
         <v>1</v>
       </c>
       <c r="E11" t="n">
-        <v>5132155.263837265</v>
+        <v>4535500.038480652</v>
       </c>
       <c r="F11" t="n">
-        <v>1822147.263837265</v>
+        <v>2279140.038480652</v>
       </c>
       <c r="G11" t="n">
-        <v>55.04963322859838</v>
+        <v>101.0095923735863</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>TIME 코리아밸류업액티브</t>
+          <t>동원개발</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>201</v>
+        <v>1360</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
@@ -754,23 +754,23 @@
         <v>1</v>
       </c>
       <c r="E12" t="n">
-        <v>4904400</v>
+        <v>3978000</v>
       </c>
       <c r="F12" t="n">
-        <v>180603</v>
+        <v>240600</v>
       </c>
       <c r="G12" t="n">
-        <v>3.823259128197084</v>
+        <v>6.437630438272596</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>오케아니스 에코 탱커스</t>
+          <t>차코스 에너지 내비게이션</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>65</v>
+        <v>75</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
@@ -781,23 +781,23 @@
         <v>1</v>
       </c>
       <c r="E13" t="n">
-        <v>4535500.038480652</v>
+        <v>3915702.545498475</v>
       </c>
       <c r="F13" t="n">
-        <v>2279140.038480652</v>
+        <v>91054.54549847404</v>
       </c>
       <c r="G13" t="n">
-        <v>101.0095923735863</v>
+        <v>2.380730082833088</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>삼성화재</t>
+          <t>피바디 에너지</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>9</v>
+        <v>65</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
@@ -808,23 +808,23 @@
         <v>1</v>
       </c>
       <c r="E14" t="n">
-        <v>4446000</v>
+        <v>3381342.671001556</v>
       </c>
       <c r="F14" t="n">
-        <v>-185000</v>
+        <v>1910570.671001556</v>
       </c>
       <c r="G14" t="n">
-        <v>-3.994817534009933</v>
+        <v>129.9025730025834</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>DL이앤씨</t>
+          <t>더치 브로스</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>80</v>
+        <v>39</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
@@ -835,23 +835,23 @@
         <v>1</v>
       </c>
       <c r="E15" t="n">
-        <v>4128000</v>
+        <v>3030170.005811756</v>
       </c>
       <c r="F15" t="n">
-        <v>717000</v>
+        <v>-160473.9941882449</v>
       </c>
       <c r="G15" t="n">
-        <v>21.02022867194371</v>
+        <v>-5.029517369792584</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>동원개발</t>
+          <t>넥스틸</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>1360</v>
+        <v>200</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
@@ -862,23 +862,23 @@
         <v>1</v>
       </c>
       <c r="E16" t="n">
-        <v>3978000</v>
+        <v>2400000</v>
       </c>
       <c r="F16" t="n">
-        <v>240600</v>
+        <v>389000</v>
       </c>
       <c r="G16" t="n">
-        <v>6.437630438272596</v>
+        <v>19.34361014420686</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>HD건설기계</t>
+          <t>대신증권</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>31</v>
+        <v>55</v>
       </c>
       <c r="C17" t="inlineStr">
         <is>
@@ -889,23 +889,23 @@
         <v>1</v>
       </c>
       <c r="E17" t="n">
-        <v>3955600</v>
+        <v>2238500</v>
       </c>
       <c r="F17" t="n">
-        <v>-79496</v>
+        <v>528999</v>
       </c>
       <c r="G17" t="n">
-        <v>-1.970114217852561</v>
+        <v>30.94464408034859</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>차코스 에너지 내비게이션</t>
+          <t>발레로 에너지</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>75</v>
+        <v>6</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
@@ -916,23 +916,23 @@
         <v>1</v>
       </c>
       <c r="E18" t="n">
-        <v>3915702.545498475</v>
+        <v>2145997.115708057</v>
       </c>
       <c r="F18" t="n">
-        <v>91054.54549847404</v>
+        <v>82007.11570805684</v>
       </c>
       <c r="G18" t="n">
-        <v>2.380730082833088</v>
+        <v>3.973232220507698</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>피바디 에너지</t>
+          <t>미창석유</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>65</v>
+        <v>18</v>
       </c>
       <c r="C19" t="inlineStr">
         <is>
@@ -943,23 +943,23 @@
         <v>1</v>
       </c>
       <c r="E19" t="n">
-        <v>3381342.671001556</v>
+        <v>2032200</v>
       </c>
       <c r="F19" t="n">
-        <v>1910570.671001556</v>
+        <v>-360000</v>
       </c>
       <c r="G19" t="n">
-        <v>129.9025730025834</v>
+        <v>-15.04890895410083</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>더치 브로스</t>
+          <t>대창단조</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>39</v>
+        <v>300</v>
       </c>
       <c r="C20" t="inlineStr">
         <is>
@@ -970,23 +970,23 @@
         <v>1</v>
       </c>
       <c r="E20" t="n">
-        <v>3030170.005811756</v>
+        <v>1914000</v>
       </c>
       <c r="F20" t="n">
-        <v>-160473.9941882449</v>
+        <v>-144000</v>
       </c>
       <c r="G20" t="n">
-        <v>-5.029517369792584</v>
+        <v>-6.997084548104956</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>현대제철</t>
+          <t>동방</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>70</v>
+        <v>681</v>
       </c>
       <c r="C21" t="inlineStr">
         <is>
@@ -997,23 +997,23 @@
         <v>1</v>
       </c>
       <c r="E21" t="n">
-        <v>2607500</v>
+        <v>1882965</v>
       </c>
       <c r="F21" t="n">
-        <v>-200000</v>
+        <v>-88536</v>
       </c>
       <c r="G21" t="n">
-        <v>-7.123775601068566</v>
+        <v>-4.490791533963209</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>KoAct 코스닥액티브</t>
+          <t>유나이티드헬스 그룹</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>200</v>
+        <v>4</v>
       </c>
       <c r="C22" t="inlineStr">
         <is>
@@ -1024,23 +1024,23 @@
         <v>1</v>
       </c>
       <c r="E22" t="n">
-        <v>2598000</v>
+        <v>1710129.080517188</v>
       </c>
       <c r="F22" t="n">
-        <v>-104000</v>
+        <v>15673.08051718748</v>
       </c>
       <c r="G22" t="n">
-        <v>-3.84900074019245</v>
+        <v>0.9249623783200909</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>휴스틸</t>
+          <t>스타 벌크 캐리어스</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>500</v>
+        <v>50</v>
       </c>
       <c r="C23" t="inlineStr">
         <is>
@@ -1051,23 +1051,23 @@
         <v>1</v>
       </c>
       <c r="E23" t="n">
-        <v>2560000</v>
+        <v>1695389.062898559</v>
       </c>
       <c r="F23" t="n">
-        <v>281390</v>
+        <v>381036.0628985604</v>
       </c>
       <c r="G23" t="n">
-        <v>12.34919534277476</v>
+        <v>28.99039016904597</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>넥스틸</t>
+          <t>삼성생명</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>200</v>
+        <v>4</v>
       </c>
       <c r="C24" t="inlineStr">
         <is>
@@ -1078,23 +1078,23 @@
         <v>1</v>
       </c>
       <c r="E24" t="n">
-        <v>2400000</v>
+        <v>940000</v>
       </c>
       <c r="F24" t="n">
-        <v>389000</v>
+        <v>107000</v>
       </c>
       <c r="G24" t="n">
-        <v>19.34361014420686</v>
+        <v>12.84513805522209</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>대신증권</t>
+          <t>클리블랜드 클리프스</t>
         </is>
       </c>
       <c r="B25" t="n">
-        <v>55</v>
+        <v>70</v>
       </c>
       <c r="C25" t="inlineStr">
         <is>
@@ -1105,23 +1105,23 @@
         <v>1</v>
       </c>
       <c r="E25" t="n">
-        <v>2238500</v>
+        <v>866936.6928166046</v>
       </c>
       <c r="F25" t="n">
-        <v>528999</v>
+        <v>-149118.3071833954</v>
       </c>
       <c r="G25" t="n">
-        <v>30.94464408034859</v>
+        <v>-14.6762042589619</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>발레로 에너지</t>
+          <t>비에이치아이</t>
         </is>
       </c>
       <c r="B26" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="C26" t="inlineStr">
         <is>
@@ -1132,23 +1132,23 @@
         <v>1</v>
       </c>
       <c r="E26" t="n">
-        <v>2145997.115708057</v>
+        <v>844800</v>
       </c>
       <c r="F26" t="n">
-        <v>82007.11570805684</v>
+        <v>179685</v>
       </c>
       <c r="G26" t="n">
-        <v>3.973232220507698</v>
+        <v>27.01562887620938</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>미창석유</t>
+          <t>하프니아</t>
         </is>
       </c>
       <c r="B27" t="n">
-        <v>18</v>
+        <v>80</v>
       </c>
       <c r="C27" t="inlineStr">
         <is>
@@ -1159,23 +1159,23 @@
         <v>1</v>
       </c>
       <c r="E27" t="n">
-        <v>2032200</v>
+        <v>817210.2530013258</v>
       </c>
       <c r="F27" t="n">
-        <v>-360000</v>
+        <v>191479.2530013258</v>
       </c>
       <c r="G27" t="n">
-        <v>-15.04890895410083</v>
+        <v>30.60088967964281</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>대창단조</t>
+          <t>텍사스 퍼시픽 랜드</t>
         </is>
       </c>
       <c r="B28" t="n">
-        <v>300</v>
+        <v>1</v>
       </c>
       <c r="C28" t="inlineStr">
         <is>
@@ -1186,23 +1186,23 @@
         <v>1</v>
       </c>
       <c r="E28" t="n">
-        <v>1914000</v>
+        <v>788827.7025751099</v>
       </c>
       <c r="F28" t="n">
-        <v>-144000</v>
+        <v>10236.7025751099</v>
       </c>
       <c r="G28" t="n">
-        <v>-6.997084548104956</v>
+        <v>1.314772785083555</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>동방</t>
+          <t>노블</t>
         </is>
       </c>
       <c r="B29" t="n">
-        <v>681</v>
+        <v>99</v>
       </c>
       <c r="C29" t="inlineStr">
         <is>
@@ -1213,23 +1213,23 @@
         <v>1</v>
       </c>
       <c r="E29" t="n">
-        <v>1882965</v>
+        <v>40689</v>
       </c>
       <c r="F29" t="n">
-        <v>-88536</v>
+        <v>-3866519</v>
       </c>
       <c r="G29" t="n">
-        <v>-4.490791533963209</v>
+        <v>-98.95861699709869</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>하나금융지주</t>
+          <t>삼성화재</t>
         </is>
       </c>
       <c r="B30" t="n">
-        <v>15</v>
+        <v>7</v>
       </c>
       <c r="C30" t="inlineStr">
         <is>
@@ -1240,23 +1240,23 @@
         <v>1</v>
       </c>
       <c r="E30" t="n">
-        <v>1717500</v>
+        <v>3335815</v>
       </c>
       <c r="F30" t="n">
-        <v>35000</v>
+        <v>-295185</v>
       </c>
       <c r="G30" t="n">
-        <v>2.080237741456166</v>
+        <v>-8.119999999999999</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>유나이티드헬스 그룹</t>
+          <t>세아제강</t>
         </is>
       </c>
       <c r="B31" t="n">
-        <v>4</v>
+        <v>50</v>
       </c>
       <c r="C31" t="inlineStr">
         <is>
@@ -1267,19 +1267,19 @@
         <v>1</v>
       </c>
       <c r="E31" t="n">
-        <v>1710129.080517188</v>
+        <v>6896180</v>
       </c>
       <c r="F31" t="n">
-        <v>15673.08051718748</v>
+        <v>586180</v>
       </c>
       <c r="G31" t="n">
-        <v>0.9249623783200909</v>
+        <v>9.279999999999999</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>스타 벌크 캐리어스</t>
+          <t>케이씨</t>
         </is>
       </c>
       <c r="B32" t="n">
@@ -1294,23 +1294,23 @@
         <v>1</v>
       </c>
       <c r="E32" t="n">
-        <v>1695389.062898559</v>
+        <v>1576840</v>
       </c>
       <c r="F32" t="n">
-        <v>381036.0628985604</v>
+        <v>-72660</v>
       </c>
       <c r="G32" t="n">
-        <v>28.99039016904597</v>
+        <v>-4.4</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>케이씨</t>
+          <t>하나금융지주</t>
         </is>
       </c>
       <c r="B33" t="n">
-        <v>50</v>
+        <v>10</v>
       </c>
       <c r="C33" t="inlineStr">
         <is>
@@ -1321,23 +1321,23 @@
         <v>1</v>
       </c>
       <c r="E33" t="n">
-        <v>1640000</v>
+        <v>1107780</v>
       </c>
       <c r="F33" t="n">
-        <v>-9500.000000000698</v>
+        <v>-1220</v>
       </c>
       <c r="G33" t="n">
-        <v>-0.5759321006365986</v>
+        <v>-0.11</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>삼성생명</t>
+          <t>현대제철</t>
         </is>
       </c>
       <c r="B34" t="n">
-        <v>4</v>
+        <v>70</v>
       </c>
       <c r="C34" t="inlineStr">
         <is>
@@ -1348,23 +1348,23 @@
         <v>1</v>
       </c>
       <c r="E34" t="n">
-        <v>940000</v>
+        <v>2494002</v>
       </c>
       <c r="F34" t="n">
-        <v>107000</v>
+        <v>-313498</v>
       </c>
       <c r="G34" t="n">
-        <v>12.84513805522209</v>
+        <v>-11.16</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>클리블랜드 클리프스</t>
+          <t>휴스틸</t>
         </is>
       </c>
       <c r="B35" t="n">
-        <v>70</v>
+        <v>500</v>
       </c>
       <c r="C35" t="inlineStr">
         <is>
@@ -1375,23 +1375,23 @@
         <v>1</v>
       </c>
       <c r="E35" t="n">
-        <v>866936.6928166046</v>
+        <v>2450090</v>
       </c>
       <c r="F35" t="n">
-        <v>-149118.3071833954</v>
+        <v>171480</v>
       </c>
       <c r="G35" t="n">
-        <v>-14.6762042589619</v>
+        <v>7.52</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>비에이치아이</t>
+          <t>DL이앤씨</t>
         </is>
       </c>
       <c r="B36" t="n">
-        <v>8</v>
+        <v>80</v>
       </c>
       <c r="C36" t="inlineStr">
         <is>
@@ -1402,23 +1402,23 @@
         <v>1</v>
       </c>
       <c r="E36" t="n">
-        <v>844800</v>
+        <v>3792400</v>
       </c>
       <c r="F36" t="n">
-        <v>179685</v>
+        <v>381400</v>
       </c>
       <c r="G36" t="n">
-        <v>27.01562887620938</v>
+        <v>11.18</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>하프니아</t>
+          <t>HD건설기계</t>
         </is>
       </c>
       <c r="B37" t="n">
-        <v>80</v>
+        <v>31</v>
       </c>
       <c r="C37" t="inlineStr">
         <is>
@@ -1429,23 +1429,23 @@
         <v>1</v>
       </c>
       <c r="E37" t="n">
-        <v>817210.2530013258</v>
+        <v>3885810</v>
       </c>
       <c r="F37" t="n">
-        <v>191479.2530013258</v>
+        <v>-149286</v>
       </c>
       <c r="G37" t="n">
-        <v>30.60088967964281</v>
+        <v>-3.69</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>텍사스 퍼시픽 랜드</t>
+          <t>KoAct 코스닥액티브</t>
         </is>
       </c>
       <c r="B38" t="n">
-        <v>1</v>
+        <v>200</v>
       </c>
       <c r="C38" t="inlineStr">
         <is>
@@ -1456,23 +1456,23 @@
         <v>1</v>
       </c>
       <c r="E38" t="n">
-        <v>788827.7025751099</v>
+        <v>2580000</v>
       </c>
       <c r="F38" t="n">
-        <v>10236.7025751099</v>
+        <v>-122000</v>
       </c>
       <c r="G38" t="n">
-        <v>1.314772785083555</v>
+        <v>-4.51</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>노블</t>
+          <t>TIME 코리아밸류업액티브</t>
         </is>
       </c>
       <c r="B39" t="n">
-        <v>99</v>
+        <v>201</v>
       </c>
       <c r="C39" t="inlineStr">
         <is>
@@ -1483,13 +1483,13 @@
         <v>1</v>
       </c>
       <c r="E39" t="n">
-        <v>40689</v>
+        <v>4656165</v>
       </c>
       <c r="F39" t="n">
-        <v>-3866519</v>
+        <v>-67632</v>
       </c>
       <c r="G39" t="n">
-        <v>-98.95861699709869</v>
+        <v>-1.43</v>
       </c>
     </row>
   </sheetData>
@@ -1547,7 +1547,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2026-03-18T14:29:29</t>
+          <t>2026-03-18T14:30:27</t>
         </is>
       </c>
       <c r="E2" t="n">

</xml_diff>

<commit_message>
auto: portfolio snapshot 2026-03-17 (2026-03-18T14:30:29)
</commit_message>
<xml_diff>
--- a/portfolio_auto.xlsx
+++ b/portfolio_auto.xlsx
@@ -1240,13 +1240,13 @@
         <v>1</v>
       </c>
       <c r="E30" t="n">
-        <v>3335815</v>
+        <v>3458000</v>
       </c>
       <c r="F30" t="n">
-        <v>-295185</v>
+        <v>-173000</v>
       </c>
       <c r="G30" t="n">
-        <v>-8.119999999999999</v>
+        <v>-4.76452767832553</v>
       </c>
     </row>
     <row r="31">
@@ -1267,13 +1267,13 @@
         <v>1</v>
       </c>
       <c r="E31" t="n">
-        <v>6896180</v>
+        <v>6915000</v>
       </c>
       <c r="F31" t="n">
-        <v>586180</v>
+        <v>605000</v>
       </c>
       <c r="G31" t="n">
-        <v>9.279999999999999</v>
+        <v>9.587955625990491</v>
       </c>
     </row>
     <row r="32">
@@ -1294,13 +1294,13 @@
         <v>1</v>
       </c>
       <c r="E32" t="n">
-        <v>1576840</v>
+        <v>1640000</v>
       </c>
       <c r="F32" t="n">
-        <v>-72660</v>
+        <v>-9500</v>
       </c>
       <c r="G32" t="n">
-        <v>-4.4</v>
+        <v>-0.5759321006365565</v>
       </c>
     </row>
     <row r="33">
@@ -1321,13 +1321,13 @@
         <v>1</v>
       </c>
       <c r="E33" t="n">
-        <v>1107780</v>
+        <v>1145000</v>
       </c>
       <c r="F33" t="n">
-        <v>-1220</v>
+        <v>36000</v>
       </c>
       <c r="G33" t="n">
-        <v>-0.11</v>
+        <v>3.246167718665464</v>
       </c>
     </row>
     <row r="34">
@@ -1348,13 +1348,13 @@
         <v>1</v>
       </c>
       <c r="E34" t="n">
-        <v>2494002</v>
+        <v>2607500</v>
       </c>
       <c r="F34" t="n">
-        <v>-313498</v>
+        <v>-200000</v>
       </c>
       <c r="G34" t="n">
-        <v>-11.16</v>
+        <v>-7.123775601068566</v>
       </c>
     </row>
     <row r="35">
@@ -1375,13 +1375,13 @@
         <v>1</v>
       </c>
       <c r="E35" t="n">
-        <v>2450090</v>
+        <v>2560000</v>
       </c>
       <c r="F35" t="n">
-        <v>171480</v>
+        <v>281390</v>
       </c>
       <c r="G35" t="n">
-        <v>7.52</v>
+        <v>12.34919534277476</v>
       </c>
     </row>
     <row r="36">
@@ -1402,13 +1402,13 @@
         <v>1</v>
       </c>
       <c r="E36" t="n">
-        <v>3792400</v>
+        <v>4128000</v>
       </c>
       <c r="F36" t="n">
-        <v>381400</v>
+        <v>717000</v>
       </c>
       <c r="G36" t="n">
-        <v>11.18</v>
+        <v>21.02022867194371</v>
       </c>
     </row>
     <row r="37">
@@ -1429,13 +1429,13 @@
         <v>1</v>
       </c>
       <c r="E37" t="n">
-        <v>3885810</v>
+        <v>3955600</v>
       </c>
       <c r="F37" t="n">
-        <v>-149286</v>
+        <v>-79496</v>
       </c>
       <c r="G37" t="n">
-        <v>-3.69</v>
+        <v>-1.970114217852561</v>
       </c>
     </row>
     <row r="38">
@@ -1456,13 +1456,13 @@
         <v>1</v>
       </c>
       <c r="E38" t="n">
-        <v>2580000</v>
+        <v>2598000</v>
       </c>
       <c r="F38" t="n">
-        <v>-122000</v>
+        <v>-104000</v>
       </c>
       <c r="G38" t="n">
-        <v>-4.51</v>
+        <v>-3.84900074019245</v>
       </c>
     </row>
     <row r="39">
@@ -1483,13 +1483,13 @@
         <v>1</v>
       </c>
       <c r="E39" t="n">
-        <v>4656165</v>
+        <v>4904400</v>
       </c>
       <c r="F39" t="n">
-        <v>-67632</v>
+        <v>180603</v>
       </c>
       <c r="G39" t="n">
-        <v>-1.43</v>
+        <v>3.823259128197084</v>
       </c>
     </row>
   </sheetData>
@@ -1547,7 +1547,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2026-03-18T14:30:27</t>
+          <t>2026-03-18T14:30:29</t>
         </is>
       </c>
       <c r="E2" t="n">

</xml_diff>

<commit_message>
auto: portfolio snapshot 2026-03-18 (2026-03-18T14:30:48)
</commit_message>
<xml_diff>
--- a/portfolio_auto.xlsx
+++ b/portfolio_auto.xlsx
@@ -487,10 +487,10 @@
         <v>14061179.77103613</v>
       </c>
       <c r="F2" t="n">
-        <v>1954630.771036137</v>
+        <v>1954630.771036133</v>
       </c>
       <c r="G2" t="n">
-        <v>16.14523487276298</v>
+        <v>16.14523487276294</v>
       </c>
     </row>
     <row r="3">
@@ -514,10 +514,10 @@
         <v>10796404.23451035</v>
       </c>
       <c r="F3" t="n">
-        <v>-35610.76548965834</v>
+        <v>-35610.76548965462</v>
       </c>
       <c r="G3" t="n">
-        <v>-0.3287547652921301</v>
+        <v>-0.3287547652920958</v>
       </c>
     </row>
     <row r="4">
@@ -625,17 +625,17 @@
         <v>3082998.489881324</v>
       </c>
       <c r="G7" t="n">
-        <v>74.6989022158987</v>
+        <v>74.69890221589867</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>센트러스 에너지</t>
+          <t>세아제강</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>21</v>
+        <v>50</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
@@ -646,23 +646,23 @@
         <v>1</v>
       </c>
       <c r="E8" t="n">
-        <v>6611393.516486719</v>
+        <v>6915000</v>
       </c>
       <c r="F8" t="n">
-        <v>380174.5164867202</v>
+        <v>605000</v>
       </c>
       <c r="G8" t="n">
-        <v>6.101125903081247</v>
+        <v>9.587955625990491</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>타이드워터</t>
+          <t>센트러스 에너지</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>48</v>
+        <v>21</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
@@ -673,23 +673,23 @@
         <v>1</v>
       </c>
       <c r="E9" t="n">
-        <v>5478261.098275781</v>
+        <v>6611393.516486719</v>
       </c>
       <c r="F9" t="n">
-        <v>1753716.098275781</v>
+        <v>380174.5164867202</v>
       </c>
       <c r="G9" t="n">
-        <v>47.08537816768976</v>
+        <v>6.101125903081247</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>노브</t>
+          <t>타이드워터</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>185</v>
+        <v>48</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
@@ -700,23 +700,23 @@
         <v>1</v>
       </c>
       <c r="E10" t="n">
-        <v>5132155.263837265</v>
+        <v>5478261.098275781</v>
       </c>
       <c r="F10" t="n">
-        <v>1822147.263837265</v>
+        <v>1753716.098275781</v>
       </c>
       <c r="G10" t="n">
-        <v>55.04963322859838</v>
+        <v>47.08537816768976</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>오케아니스 에코 탱커스</t>
+          <t>노브</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>65</v>
+        <v>185</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
@@ -727,23 +727,23 @@
         <v>1</v>
       </c>
       <c r="E11" t="n">
-        <v>4535500.038480652</v>
+        <v>5132155.263837265</v>
       </c>
       <c r="F11" t="n">
-        <v>2279140.038480652</v>
+        <v>1822147.263837265</v>
       </c>
       <c r="G11" t="n">
-        <v>101.0095923735863</v>
+        <v>55.04963322859838</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>동원개발</t>
+          <t>TIME 코리아밸류업액티브</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>1360</v>
+        <v>201</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
@@ -754,23 +754,23 @@
         <v>1</v>
       </c>
       <c r="E12" t="n">
-        <v>3978000</v>
+        <v>4904400</v>
       </c>
       <c r="F12" t="n">
-        <v>240600</v>
+        <v>180603</v>
       </c>
       <c r="G12" t="n">
-        <v>6.437630438272596</v>
+        <v>3.823259128197084</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>차코스 에너지 내비게이션</t>
+          <t>오케아니스 에코 탱커스</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>75</v>
+        <v>65</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
@@ -781,23 +781,23 @@
         <v>1</v>
       </c>
       <c r="E13" t="n">
-        <v>3915702.545498475</v>
+        <v>4535500.038480652</v>
       </c>
       <c r="F13" t="n">
-        <v>91054.54549847404</v>
+        <v>2279140.038480652</v>
       </c>
       <c r="G13" t="n">
-        <v>2.380730082833088</v>
+        <v>101.0095923735863</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>피바디 에너지</t>
+          <t>삼성화재</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>65</v>
+        <v>9</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
@@ -808,23 +808,23 @@
         <v>1</v>
       </c>
       <c r="E14" t="n">
-        <v>3381342.671001556</v>
+        <v>4446000</v>
       </c>
       <c r="F14" t="n">
-        <v>1910570.671001556</v>
+        <v>-185000</v>
       </c>
       <c r="G14" t="n">
-        <v>129.9025730025834</v>
+        <v>-3.994817534009933</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>더치 브로스</t>
+          <t>DL이앤씨</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>39</v>
+        <v>80</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
@@ -835,23 +835,23 @@
         <v>1</v>
       </c>
       <c r="E15" t="n">
-        <v>3030170.005811756</v>
+        <v>4128000</v>
       </c>
       <c r="F15" t="n">
-        <v>-160473.9941882449</v>
+        <v>717000</v>
       </c>
       <c r="G15" t="n">
-        <v>-5.029517369792584</v>
+        <v>21.02022867194371</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>넥스틸</t>
+          <t>동원개발</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>200</v>
+        <v>1360</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
@@ -862,23 +862,23 @@
         <v>1</v>
       </c>
       <c r="E16" t="n">
-        <v>2400000</v>
+        <v>3978000</v>
       </c>
       <c r="F16" t="n">
-        <v>389000</v>
+        <v>240600</v>
       </c>
       <c r="G16" t="n">
-        <v>19.34361014420686</v>
+        <v>6.437630438272596</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>대신증권</t>
+          <t>HD건설기계</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>55</v>
+        <v>31</v>
       </c>
       <c r="C17" t="inlineStr">
         <is>
@@ -889,23 +889,23 @@
         <v>1</v>
       </c>
       <c r="E17" t="n">
-        <v>2238500</v>
+        <v>3955600</v>
       </c>
       <c r="F17" t="n">
-        <v>528999</v>
+        <v>-79496</v>
       </c>
       <c r="G17" t="n">
-        <v>30.94464408034859</v>
+        <v>-1.970114217852561</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>발레로 에너지</t>
+          <t>차코스 에너지 내비게이션</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>6</v>
+        <v>75</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
@@ -916,23 +916,23 @@
         <v>1</v>
       </c>
       <c r="E18" t="n">
-        <v>2145997.115708057</v>
+        <v>3915702.545498475</v>
       </c>
       <c r="F18" t="n">
-        <v>82007.11570805684</v>
+        <v>91054.5454984745</v>
       </c>
       <c r="G18" t="n">
-        <v>3.973232220507698</v>
+        <v>2.3807300828331</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>미창석유</t>
+          <t>피바디 에너지</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>18</v>
+        <v>65</v>
       </c>
       <c r="C19" t="inlineStr">
         <is>
@@ -943,23 +943,23 @@
         <v>1</v>
       </c>
       <c r="E19" t="n">
-        <v>2032200</v>
+        <v>3381342.671001556</v>
       </c>
       <c r="F19" t="n">
-        <v>-360000</v>
+        <v>1910570.671001556</v>
       </c>
       <c r="G19" t="n">
-        <v>-15.04890895410083</v>
+        <v>129.9025730025834</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>대창단조</t>
+          <t>더치 브로스</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>300</v>
+        <v>39</v>
       </c>
       <c r="C20" t="inlineStr">
         <is>
@@ -970,23 +970,23 @@
         <v>1</v>
       </c>
       <c r="E20" t="n">
-        <v>1914000</v>
+        <v>3030170.005811756</v>
       </c>
       <c r="F20" t="n">
-        <v>-144000</v>
+        <v>-160473.9941882445</v>
       </c>
       <c r="G20" t="n">
-        <v>-6.997084548104956</v>
+        <v>-5.02951736979257</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>동방</t>
+          <t>현대제철</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>681</v>
+        <v>70</v>
       </c>
       <c r="C21" t="inlineStr">
         <is>
@@ -997,23 +997,23 @@
         <v>1</v>
       </c>
       <c r="E21" t="n">
-        <v>1882965</v>
+        <v>2607500</v>
       </c>
       <c r="F21" t="n">
-        <v>-88536</v>
+        <v>-200000</v>
       </c>
       <c r="G21" t="n">
-        <v>-4.490791533963209</v>
+        <v>-7.123775601068566</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>유나이티드헬스 그룹</t>
+          <t>KoAct 코스닥액티브</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>4</v>
+        <v>200</v>
       </c>
       <c r="C22" t="inlineStr">
         <is>
@@ -1024,23 +1024,23 @@
         <v>1</v>
       </c>
       <c r="E22" t="n">
-        <v>1710129.080517188</v>
+        <v>2598000</v>
       </c>
       <c r="F22" t="n">
-        <v>15673.08051718748</v>
+        <v>-104000</v>
       </c>
       <c r="G22" t="n">
-        <v>0.9249623783200909</v>
+        <v>-3.84900074019245</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>스타 벌크 캐리어스</t>
+          <t>휴스틸</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>50</v>
+        <v>500</v>
       </c>
       <c r="C23" t="inlineStr">
         <is>
@@ -1051,23 +1051,23 @@
         <v>1</v>
       </c>
       <c r="E23" t="n">
-        <v>1695389.062898559</v>
+        <v>2560000</v>
       </c>
       <c r="F23" t="n">
-        <v>381036.0628985604</v>
+        <v>281390</v>
       </c>
       <c r="G23" t="n">
-        <v>28.99039016904597</v>
+        <v>12.34919534277476</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>삼성생명</t>
+          <t>넥스틸</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>4</v>
+        <v>200</v>
       </c>
       <c r="C24" t="inlineStr">
         <is>
@@ -1078,23 +1078,23 @@
         <v>1</v>
       </c>
       <c r="E24" t="n">
-        <v>940000</v>
+        <v>2400000</v>
       </c>
       <c r="F24" t="n">
-        <v>107000</v>
+        <v>389000</v>
       </c>
       <c r="G24" t="n">
-        <v>12.84513805522209</v>
+        <v>19.34361014420686</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>클리블랜드 클리프스</t>
+          <t>대신증권</t>
         </is>
       </c>
       <c r="B25" t="n">
-        <v>70</v>
+        <v>55</v>
       </c>
       <c r="C25" t="inlineStr">
         <is>
@@ -1105,23 +1105,23 @@
         <v>1</v>
       </c>
       <c r="E25" t="n">
-        <v>866936.6928166046</v>
+        <v>2238500</v>
       </c>
       <c r="F25" t="n">
-        <v>-149118.3071833954</v>
+        <v>528999</v>
       </c>
       <c r="G25" t="n">
-        <v>-14.6762042589619</v>
+        <v>30.94464408034859</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>비에이치아이</t>
+          <t>발레로 에너지</t>
         </is>
       </c>
       <c r="B26" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="C26" t="inlineStr">
         <is>
@@ -1132,23 +1132,23 @@
         <v>1</v>
       </c>
       <c r="E26" t="n">
-        <v>844800</v>
+        <v>2145997.115708057</v>
       </c>
       <c r="F26" t="n">
-        <v>179685</v>
+        <v>82007.11570805684</v>
       </c>
       <c r="G26" t="n">
-        <v>27.01562887620938</v>
+        <v>3.973232220507698</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>하프니아</t>
+          <t>미창석유</t>
         </is>
       </c>
       <c r="B27" t="n">
-        <v>80</v>
+        <v>18</v>
       </c>
       <c r="C27" t="inlineStr">
         <is>
@@ -1159,23 +1159,23 @@
         <v>1</v>
       </c>
       <c r="E27" t="n">
-        <v>817210.2530013258</v>
+        <v>2032200</v>
       </c>
       <c r="F27" t="n">
-        <v>191479.2530013258</v>
+        <v>-360000</v>
       </c>
       <c r="G27" t="n">
-        <v>30.60088967964281</v>
+        <v>-15.04890895410083</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>텍사스 퍼시픽 랜드</t>
+          <t>대창단조</t>
         </is>
       </c>
       <c r="B28" t="n">
-        <v>1</v>
+        <v>300</v>
       </c>
       <c r="C28" t="inlineStr">
         <is>
@@ -1186,23 +1186,23 @@
         <v>1</v>
       </c>
       <c r="E28" t="n">
-        <v>788827.7025751099</v>
+        <v>1914000</v>
       </c>
       <c r="F28" t="n">
-        <v>10236.7025751099</v>
+        <v>-144000</v>
       </c>
       <c r="G28" t="n">
-        <v>1.314772785083555</v>
+        <v>-6.997084548104956</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>노블</t>
+          <t>동방</t>
         </is>
       </c>
       <c r="B29" t="n">
-        <v>99</v>
+        <v>681</v>
       </c>
       <c r="C29" t="inlineStr">
         <is>
@@ -1213,23 +1213,23 @@
         <v>1</v>
       </c>
       <c r="E29" t="n">
-        <v>40689</v>
+        <v>1882965</v>
       </c>
       <c r="F29" t="n">
-        <v>-3866519</v>
+        <v>-88536</v>
       </c>
       <c r="G29" t="n">
-        <v>-98.95861699709869</v>
+        <v>-4.490791533963209</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>삼성화재</t>
+          <t>하나금융지주</t>
         </is>
       </c>
       <c r="B30" t="n">
-        <v>7</v>
+        <v>15</v>
       </c>
       <c r="C30" t="inlineStr">
         <is>
@@ -1240,23 +1240,23 @@
         <v>1</v>
       </c>
       <c r="E30" t="n">
-        <v>3458000</v>
+        <v>1717500</v>
       </c>
       <c r="F30" t="n">
-        <v>-173000</v>
+        <v>35000</v>
       </c>
       <c r="G30" t="n">
-        <v>-4.76452767832553</v>
+        <v>2.080237741456166</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>세아제강</t>
+          <t>유나이티드헬스 그룹</t>
         </is>
       </c>
       <c r="B31" t="n">
-        <v>50</v>
+        <v>4</v>
       </c>
       <c r="C31" t="inlineStr">
         <is>
@@ -1267,19 +1267,19 @@
         <v>1</v>
       </c>
       <c r="E31" t="n">
-        <v>6915000</v>
+        <v>1710129.080517188</v>
       </c>
       <c r="F31" t="n">
-        <v>605000</v>
+        <v>15673.08051718771</v>
       </c>
       <c r="G31" t="n">
-        <v>9.587955625990491</v>
+        <v>0.9249623783201047</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>케이씨</t>
+          <t>스타 벌크 캐리어스</t>
         </is>
       </c>
       <c r="B32" t="n">
@@ -1294,23 +1294,23 @@
         <v>1</v>
       </c>
       <c r="E32" t="n">
-        <v>1640000</v>
+        <v>1695389.062898559</v>
       </c>
       <c r="F32" t="n">
-        <v>-9500</v>
+        <v>381036.06289856</v>
       </c>
       <c r="G32" t="n">
-        <v>-0.5759321006365565</v>
+        <v>28.99039016904592</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>하나금융지주</t>
+          <t>케이씨</t>
         </is>
       </c>
       <c r="B33" t="n">
-        <v>10</v>
+        <v>50</v>
       </c>
       <c r="C33" t="inlineStr">
         <is>
@@ -1321,23 +1321,23 @@
         <v>1</v>
       </c>
       <c r="E33" t="n">
-        <v>1145000</v>
+        <v>1640000</v>
       </c>
       <c r="F33" t="n">
-        <v>36000</v>
+        <v>-9500.000000000698</v>
       </c>
       <c r="G33" t="n">
-        <v>3.246167718665464</v>
+        <v>-0.5759321006365986</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>현대제철</t>
+          <t>삼성생명</t>
         </is>
       </c>
       <c r="B34" t="n">
-        <v>70</v>
+        <v>4</v>
       </c>
       <c r="C34" t="inlineStr">
         <is>
@@ -1348,23 +1348,23 @@
         <v>1</v>
       </c>
       <c r="E34" t="n">
-        <v>2607500</v>
+        <v>940000</v>
       </c>
       <c r="F34" t="n">
-        <v>-200000</v>
+        <v>107000</v>
       </c>
       <c r="G34" t="n">
-        <v>-7.123775601068566</v>
+        <v>12.84513805522209</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>휴스틸</t>
+          <t>클리블랜드 클리프스</t>
         </is>
       </c>
       <c r="B35" t="n">
-        <v>500</v>
+        <v>70</v>
       </c>
       <c r="C35" t="inlineStr">
         <is>
@@ -1375,23 +1375,23 @@
         <v>1</v>
       </c>
       <c r="E35" t="n">
-        <v>2560000</v>
+        <v>866936.6928166046</v>
       </c>
       <c r="F35" t="n">
-        <v>281390</v>
+        <v>-149118.3071833954</v>
       </c>
       <c r="G35" t="n">
-        <v>12.34919534277476</v>
+        <v>-14.6762042589619</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>DL이앤씨</t>
+          <t>비에이치아이</t>
         </is>
       </c>
       <c r="B36" t="n">
-        <v>80</v>
+        <v>8</v>
       </c>
       <c r="C36" t="inlineStr">
         <is>
@@ -1402,23 +1402,23 @@
         <v>1</v>
       </c>
       <c r="E36" t="n">
-        <v>4128000</v>
+        <v>844800</v>
       </c>
       <c r="F36" t="n">
-        <v>717000</v>
+        <v>179685</v>
       </c>
       <c r="G36" t="n">
-        <v>21.02022867194371</v>
+        <v>27.01562887620938</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>HD건설기계</t>
+          <t>하프니아</t>
         </is>
       </c>
       <c r="B37" t="n">
-        <v>31</v>
+        <v>80</v>
       </c>
       <c r="C37" t="inlineStr">
         <is>
@@ -1429,23 +1429,23 @@
         <v>1</v>
       </c>
       <c r="E37" t="n">
-        <v>3955600</v>
+        <v>817210.2530013258</v>
       </c>
       <c r="F37" t="n">
-        <v>-79496</v>
+        <v>191479.2530013258</v>
       </c>
       <c r="G37" t="n">
-        <v>-1.970114217852561</v>
+        <v>30.60088967964281</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>KoAct 코스닥액티브</t>
+          <t>텍사스 퍼시픽 랜드</t>
         </is>
       </c>
       <c r="B38" t="n">
-        <v>200</v>
+        <v>1</v>
       </c>
       <c r="C38" t="inlineStr">
         <is>
@@ -1456,23 +1456,23 @@
         <v>1</v>
       </c>
       <c r="E38" t="n">
-        <v>2598000</v>
+        <v>788827.7025751099</v>
       </c>
       <c r="F38" t="n">
-        <v>-104000</v>
+        <v>10236.7025751099</v>
       </c>
       <c r="G38" t="n">
-        <v>-3.84900074019245</v>
+        <v>1.314772785083555</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>TIME 코리아밸류업액티브</t>
+          <t>노블</t>
         </is>
       </c>
       <c r="B39" t="n">
-        <v>201</v>
+        <v>99</v>
       </c>
       <c r="C39" t="inlineStr">
         <is>
@@ -1483,13 +1483,13 @@
         <v>1</v>
       </c>
       <c r="E39" t="n">
-        <v>4904400</v>
+        <v>40689</v>
       </c>
       <c r="F39" t="n">
-        <v>180603</v>
+        <v>-3866519</v>
       </c>
       <c r="G39" t="n">
-        <v>3.823259128197084</v>
+        <v>-98.95861699709869</v>
       </c>
     </row>
   </sheetData>
@@ -1536,22 +1536,22 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-03-17</t>
+          <t>2026-03-18</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>33078556</v>
+        <v>31505056</v>
       </c>
       <c r="C2" t="n">
-        <v>6010.99</v>
+        <v>6016.63</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2026-03-18T14:30:29</t>
+          <t>2026-03-18T14:30:48</t>
         </is>
       </c>
       <c r="E2" t="n">
-        <v>1488.910034179688</v>
+        <v>1485.880004882812</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
auto: portfolio snapshot 2026-03-17 (2026-03-18T14:31:59)
</commit_message>
<xml_diff>
--- a/portfolio_auto.xlsx
+++ b/portfolio_auto.xlsx
@@ -487,10 +487,10 @@
         <v>14061179.77103613</v>
       </c>
       <c r="F2" t="n">
-        <v>1954630.771036133</v>
+        <v>1954630.771036137</v>
       </c>
       <c r="G2" t="n">
-        <v>16.14523487276294</v>
+        <v>16.14523487276298</v>
       </c>
     </row>
     <row r="3">
@@ -514,10 +514,10 @@
         <v>10796404.23451035</v>
       </c>
       <c r="F3" t="n">
-        <v>-35610.76548965462</v>
+        <v>-35610.76548965834</v>
       </c>
       <c r="G3" t="n">
-        <v>-0.3287547652920958</v>
+        <v>-0.3287547652921301</v>
       </c>
     </row>
     <row r="4">
@@ -625,7 +625,7 @@
         <v>3082998.489881324</v>
       </c>
       <c r="G7" t="n">
-        <v>74.69890221589867</v>
+        <v>74.6989022158987</v>
       </c>
     </row>
     <row r="8">
@@ -919,10 +919,10 @@
         <v>3915702.545498475</v>
       </c>
       <c r="F18" t="n">
-        <v>91054.5454984745</v>
+        <v>91054.54549847404</v>
       </c>
       <c r="G18" t="n">
-        <v>2.3807300828331</v>
+        <v>2.380730082833088</v>
       </c>
     </row>
     <row r="19">
@@ -973,10 +973,10 @@
         <v>3030170.005811756</v>
       </c>
       <c r="F20" t="n">
-        <v>-160473.9941882445</v>
+        <v>-160473.9941882449</v>
       </c>
       <c r="G20" t="n">
-        <v>-5.02951736979257</v>
+        <v>-5.029517369792584</v>
       </c>
     </row>
     <row r="21">
@@ -1270,10 +1270,10 @@
         <v>1710129.080517188</v>
       </c>
       <c r="F31" t="n">
-        <v>15673.08051718771</v>
+        <v>15673.08051718748</v>
       </c>
       <c r="G31" t="n">
-        <v>0.9249623783201047</v>
+        <v>0.9249623783200909</v>
       </c>
     </row>
     <row r="32">
@@ -1297,10 +1297,10 @@
         <v>1695389.062898559</v>
       </c>
       <c r="F32" t="n">
-        <v>381036.06289856</v>
+        <v>381036.0628985604</v>
       </c>
       <c r="G32" t="n">
-        <v>28.99039016904592</v>
+        <v>28.99039016904597</v>
       </c>
     </row>
     <row r="33">
@@ -1536,22 +1536,22 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-03-18</t>
+          <t>2026-03-17</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>31505056</v>
+        <v>0</v>
       </c>
       <c r="C2" t="n">
-        <v>6016.63</v>
+        <v>0</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2026-03-18T14:30:48</t>
+          <t>2026-03-18T14:31:59</t>
         </is>
       </c>
       <c r="E2" t="n">
-        <v>1485.880004882812</v>
+        <v>1488.910034179688</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
auto: portfolio snapshot 2026-03-18 (2026-03-18T14:32:42)
</commit_message>
<xml_diff>
--- a/portfolio_auto.xlsx
+++ b/portfolio_auto.xlsx
@@ -484,13 +484,13 @@
         <v>1</v>
       </c>
       <c r="E2" t="n">
-        <v>14061179.77103613</v>
+        <v>14082576.9328374</v>
       </c>
       <c r="F2" t="n">
-        <v>1954630.771036137</v>
+        <v>1976027.932837404</v>
       </c>
       <c r="G2" t="n">
-        <v>16.14523487276298</v>
+        <v>16.3219752617976</v>
       </c>
     </row>
     <row r="3">
@@ -511,13 +511,13 @@
         <v>1</v>
       </c>
       <c r="E3" t="n">
-        <v>10796404.23451035</v>
+        <v>10822406.73782303</v>
       </c>
       <c r="F3" t="n">
-        <v>-35610.76548965834</v>
+        <v>-9608.262176971883</v>
       </c>
       <c r="G3" t="n">
-        <v>-0.3287547652921301</v>
+        <v>-0.08870244526961865</v>
       </c>
     </row>
     <row r="4">
@@ -565,13 +565,13 @@
         <v>1</v>
       </c>
       <c r="E5" t="n">
-        <v>8263721.825703507</v>
+        <v>8440541.129673157</v>
       </c>
       <c r="F5" t="n">
-        <v>3833857.825703507</v>
+        <v>4010677.129673157</v>
       </c>
       <c r="G5" t="n">
-        <v>86.54572297712768</v>
+        <v>90.53725192631549</v>
       </c>
     </row>
     <row r="6">
@@ -592,13 +592,13 @@
         <v>1</v>
       </c>
       <c r="E6" t="n">
-        <v>8129308.858251691</v>
+        <v>8090014.733635107</v>
       </c>
       <c r="F6" t="n">
-        <v>1678957.858251691</v>
+        <v>1639663.733635107</v>
       </c>
       <c r="G6" t="n">
-        <v>26.02893793301622</v>
+        <v>25.41975984927188</v>
       </c>
     </row>
     <row r="7">
@@ -619,13 +619,13 @@
         <v>1</v>
       </c>
       <c r="E7" t="n">
-        <v>7210232.489881324</v>
+        <v>7093219.418241119</v>
       </c>
       <c r="F7" t="n">
-        <v>3082998.489881324</v>
+        <v>2965985.418241119</v>
       </c>
       <c r="G7" t="n">
-        <v>74.6989022158987</v>
+        <v>71.86375713713153</v>
       </c>
     </row>
     <row r="8">
@@ -673,13 +673,13 @@
         <v>1</v>
       </c>
       <c r="E9" t="n">
-        <v>6611393.516486719</v>
+        <v>6546958.253894605</v>
       </c>
       <c r="F9" t="n">
-        <v>380174.5164867202</v>
+        <v>315739.2538946057</v>
       </c>
       <c r="G9" t="n">
-        <v>6.101125903081247</v>
+        <v>5.067054357977239</v>
       </c>
     </row>
     <row r="10">
@@ -700,13 +700,13 @@
         <v>1</v>
       </c>
       <c r="E10" t="n">
-        <v>5478261.098275781</v>
+        <v>5456864.752692774</v>
       </c>
       <c r="F10" t="n">
-        <v>1753716.098275781</v>
+        <v>1732319.752692774</v>
       </c>
       <c r="G10" t="n">
-        <v>47.08537816768976</v>
+        <v>46.51090945854524</v>
       </c>
     </row>
     <row r="11">
@@ -727,13 +727,13 @@
         <v>1</v>
       </c>
       <c r="E11" t="n">
-        <v>5132155.263837265</v>
+        <v>5041442.310511444</v>
       </c>
       <c r="F11" t="n">
-        <v>1822147.263837265</v>
+        <v>1731434.310511444</v>
       </c>
       <c r="G11" t="n">
-        <v>55.04963322859838</v>
+        <v>52.30906724429197</v>
       </c>
     </row>
     <row r="12">
@@ -781,13 +781,13 @@
         <v>1</v>
       </c>
       <c r="E13" t="n">
-        <v>4535500.038480652</v>
+        <v>4575098.725873504</v>
       </c>
       <c r="F13" t="n">
-        <v>2279140.038480652</v>
+        <v>2318738.725873504</v>
       </c>
       <c r="G13" t="n">
-        <v>101.0095923735863</v>
+        <v>102.7645732894354</v>
       </c>
     </row>
     <row r="14">
@@ -916,13 +916,13 @@
         <v>1</v>
       </c>
       <c r="E18" t="n">
-        <v>3915702.545498475</v>
+        <v>4007418.271141662</v>
       </c>
       <c r="F18" t="n">
-        <v>91054.54549847404</v>
+        <v>182770.2711416623</v>
       </c>
       <c r="G18" t="n">
-        <v>2.380730082833088</v>
+        <v>4.778747511971357</v>
       </c>
     </row>
     <row r="19">
@@ -943,13 +943,13 @@
         <v>1</v>
       </c>
       <c r="E19" t="n">
-        <v>3381342.671001556</v>
+        <v>3423839.074937592</v>
       </c>
       <c r="F19" t="n">
-        <v>1910570.671001556</v>
+        <v>1953067.074937592</v>
       </c>
       <c r="G19" t="n">
-        <v>129.9025730025834</v>
+        <v>132.7919674115085</v>
       </c>
     </row>
     <row r="20">
@@ -970,13 +970,13 @@
         <v>1</v>
       </c>
       <c r="E20" t="n">
-        <v>3030170.005811756</v>
+        <v>2965846.22503092</v>
       </c>
       <c r="F20" t="n">
-        <v>-160473.9941882449</v>
+        <v>-224797.7749690795</v>
       </c>
       <c r="G20" t="n">
-        <v>-5.029517369792584</v>
+        <v>-7.04552983564069</v>
       </c>
     </row>
     <row r="21">
@@ -1132,13 +1132,13 @@
         <v>1</v>
       </c>
       <c r="E26" t="n">
-        <v>2145997.115708057</v>
+        <v>2138731.14071836</v>
       </c>
       <c r="F26" t="n">
-        <v>82007.11570805684</v>
+        <v>74741.1407183595</v>
       </c>
       <c r="G26" t="n">
-        <v>3.973232220507698</v>
+        <v>3.621196842928478</v>
       </c>
     </row>
     <row r="27">
@@ -1267,13 +1267,13 @@
         <v>1</v>
       </c>
       <c r="E31" t="n">
-        <v>1710129.080517188</v>
+        <v>1699490.128895313</v>
       </c>
       <c r="F31" t="n">
-        <v>15673.08051718748</v>
+        <v>5034.128895312548</v>
       </c>
       <c r="G31" t="n">
-        <v>0.9249623783200909</v>
+        <v>0.297094105442251</v>
       </c>
     </row>
     <row r="32">
@@ -1294,13 +1294,13 @@
         <v>1</v>
       </c>
       <c r="E32" t="n">
-        <v>1695389.062898559</v>
+        <v>1712476.648945617</v>
       </c>
       <c r="F32" t="n">
-        <v>381036.0628985604</v>
+        <v>398123.648945618</v>
       </c>
       <c r="G32" t="n">
-        <v>28.99039016904597</v>
+        <v>30.29046602743845</v>
       </c>
     </row>
     <row r="33">
@@ -1375,13 +1375,13 @@
         <v>1</v>
       </c>
       <c r="E35" t="n">
-        <v>866936.6928166046</v>
+        <v>857055.5630100402</v>
       </c>
       <c r="F35" t="n">
-        <v>-149118.3071833954</v>
+        <v>-158999.4369899598</v>
       </c>
       <c r="G35" t="n">
-        <v>-14.6762042589619</v>
+        <v>-15.64870376012714</v>
       </c>
     </row>
     <row r="36">
@@ -1429,13 +1429,13 @@
         <v>1</v>
       </c>
       <c r="E37" t="n">
-        <v>817210.2530013258</v>
+        <v>821489.5606615674</v>
       </c>
       <c r="F37" t="n">
-        <v>191479.2530013258</v>
+        <v>195758.5606615674</v>
       </c>
       <c r="G37" t="n">
-        <v>30.60088967964281</v>
+        <v>31.28477902829928</v>
       </c>
     </row>
     <row r="38">
@@ -1456,13 +1456,13 @@
         <v>1</v>
       </c>
       <c r="E38" t="n">
-        <v>788827.7025751099</v>
+        <v>794737.7576458007</v>
       </c>
       <c r="F38" t="n">
-        <v>10236.7025751099</v>
+        <v>16146.75764580071</v>
       </c>
       <c r="G38" t="n">
-        <v>1.314772785083555</v>
+        <v>2.073843345967358</v>
       </c>
     </row>
     <row r="39">
@@ -1536,22 +1536,22 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-03-17</t>
+          <t>2026-03-18</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0</v>
+        <v>31505056</v>
       </c>
       <c r="C2" t="n">
-        <v>0</v>
+        <v>6016.63</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2026-03-18T14:31:59</t>
+          <t>2026-03-18T14:32:42</t>
         </is>
       </c>
       <c r="E2" t="n">
-        <v>1488.910034179688</v>
+        <v>1485.880004882812</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
auto: portfolio snapshot 2026-03-18 (2026-03-18T21:07:08)
</commit_message>
<xml_diff>
--- a/portfolio_auto.xlsx
+++ b/portfolio_auto.xlsx
@@ -9,6 +9,8 @@
   <sheets>
     <sheet name="보유현황" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="메타" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="스냅샷_보유현황" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="스냅샷_예수금" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -847,11 +849,11 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>동원개발</t>
+          <t>차코스 에너지 내비게이션</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>1360</v>
+        <v>75</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
@@ -862,23 +864,23 @@
         <v>1</v>
       </c>
       <c r="E16" t="n">
-        <v>3978000</v>
+        <v>4007418.271141662</v>
       </c>
       <c r="F16" t="n">
-        <v>240600</v>
+        <v>182770.2711416623</v>
       </c>
       <c r="G16" t="n">
-        <v>6.437630438272596</v>
+        <v>4.778747511971357</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>HD건설기계</t>
+          <t>동원개발</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>31</v>
+        <v>1360</v>
       </c>
       <c r="C17" t="inlineStr">
         <is>
@@ -889,23 +891,23 @@
         <v>1</v>
       </c>
       <c r="E17" t="n">
-        <v>3955600</v>
+        <v>3978000</v>
       </c>
       <c r="F17" t="n">
-        <v>-79496</v>
+        <v>240600</v>
       </c>
       <c r="G17" t="n">
-        <v>-1.970114217852561</v>
+        <v>6.437630438272596</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>차코스 에너지 내비게이션</t>
+          <t>HD건설기계</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>75</v>
+        <v>31</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
@@ -916,13 +918,13 @@
         <v>1</v>
       </c>
       <c r="E18" t="n">
-        <v>4007418.271141662</v>
+        <v>3955600</v>
       </c>
       <c r="F18" t="n">
-        <v>182770.2711416623</v>
+        <v>-79496</v>
       </c>
       <c r="G18" t="n">
-        <v>4.778747511971357</v>
+        <v>-1.970114217852561</v>
       </c>
     </row>
     <row r="19">
@@ -1252,11 +1254,11 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>유나이티드헬스 그룹</t>
+          <t>스타 벌크 캐리어스</t>
         </is>
       </c>
       <c r="B31" t="n">
-        <v>4</v>
+        <v>50</v>
       </c>
       <c r="C31" t="inlineStr">
         <is>
@@ -1267,23 +1269,23 @@
         <v>1</v>
       </c>
       <c r="E31" t="n">
-        <v>1699490.128895313</v>
+        <v>1712476.648945617</v>
       </c>
       <c r="F31" t="n">
-        <v>5034.128895312548</v>
+        <v>398123.648945618</v>
       </c>
       <c r="G31" t="n">
-        <v>0.297094105442251</v>
+        <v>30.29046602743845</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>스타 벌크 캐리어스</t>
+          <t>유나이티드헬스 그룹</t>
         </is>
       </c>
       <c r="B32" t="n">
-        <v>50</v>
+        <v>4</v>
       </c>
       <c r="C32" t="inlineStr">
         <is>
@@ -1294,13 +1296,13 @@
         <v>1</v>
       </c>
       <c r="E32" t="n">
-        <v>1712476.648945617</v>
+        <v>1699490.128895313</v>
       </c>
       <c r="F32" t="n">
-        <v>398123.648945618</v>
+        <v>5034.128895312548</v>
       </c>
       <c r="G32" t="n">
-        <v>30.29046602743845</v>
+        <v>0.297094105442251</v>
       </c>
     </row>
     <row r="33">
@@ -1547,11 +1549,1542 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2026-03-18T14:32:42</t>
+          <t>2026-03-18T21:07:08</t>
         </is>
       </c>
       <c r="E2" t="n">
         <v>1485.880004882812</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I39"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>snapshot_date</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>stock_name</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>quantity</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>currency</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>fx_rate</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>market_value</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>pnl_value</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>pnl_pct</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>created_at</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>2026-03-18</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>페트로브라스 (ADR)</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>480</v>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E2" t="n">
+        <v>1</v>
+      </c>
+      <c r="F2" t="n">
+        <v>14082576.9328374</v>
+      </c>
+      <c r="G2" t="n">
+        <v>1976027.932837404</v>
+      </c>
+      <c r="H2" t="n">
+        <v>16.3219752617976</v>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>2026-03-18T14:32:42</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-03-18</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>AGNC 인베스트먼트</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>700</v>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E3" t="n">
+        <v>1</v>
+      </c>
+      <c r="F3" t="n">
+        <v>10822406.73782303</v>
+      </c>
+      <c r="G3" t="n">
+        <v>-9608.262176971883</v>
+      </c>
+      <c r="H3" t="n">
+        <v>-0.08870244526961865</v>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>2026-03-18T14:32:42</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2026-03-18</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>대한조선</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>100</v>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E4" t="n">
+        <v>1</v>
+      </c>
+      <c r="F4" t="n">
+        <v>9570000</v>
+      </c>
+      <c r="G4" t="n">
+        <v>2357000</v>
+      </c>
+      <c r="H4" t="n">
+        <v>32.67711077221684</v>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>2026-03-18T14:32:42</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2026-03-18</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>프론트라인</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>175</v>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E5" t="n">
+        <v>1</v>
+      </c>
+      <c r="F5" t="n">
+        <v>8440541.129673157</v>
+      </c>
+      <c r="G5" t="n">
+        <v>4010677.129673157</v>
+      </c>
+      <c r="H5" t="n">
+        <v>90.53725192631549</v>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>2026-03-18T14:32:42</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026-03-18</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>시드릴</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>123</v>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E6" t="n">
+        <v>1</v>
+      </c>
+      <c r="F6" t="n">
+        <v>8090014.733635107</v>
+      </c>
+      <c r="G6" t="n">
+        <v>1639663.733635107</v>
+      </c>
+      <c r="H6" t="n">
+        <v>25.41975984927188</v>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>2026-03-18T14:32:42</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2026-03-18</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>트랜스오션</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>750</v>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E7" t="n">
+        <v>1</v>
+      </c>
+      <c r="F7" t="n">
+        <v>7093219.418241119</v>
+      </c>
+      <c r="G7" t="n">
+        <v>2965985.418241119</v>
+      </c>
+      <c r="H7" t="n">
+        <v>71.86375713713153</v>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>2026-03-18T14:32:42</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2026-03-18</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>세아제강</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>50</v>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E8" t="n">
+        <v>1</v>
+      </c>
+      <c r="F8" t="n">
+        <v>6915000</v>
+      </c>
+      <c r="G8" t="n">
+        <v>605000</v>
+      </c>
+      <c r="H8" t="n">
+        <v>9.587955625990491</v>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>2026-03-18T14:32:42</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-03-18</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>센트러스 에너지</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>21</v>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E9" t="n">
+        <v>1</v>
+      </c>
+      <c r="F9" t="n">
+        <v>6546958.253894605</v>
+      </c>
+      <c r="G9" t="n">
+        <v>315739.2538946057</v>
+      </c>
+      <c r="H9" t="n">
+        <v>5.067054357977239</v>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>2026-03-18T14:32:42</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-03-18</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>타이드워터</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>48</v>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E10" t="n">
+        <v>1</v>
+      </c>
+      <c r="F10" t="n">
+        <v>5456864.752692774</v>
+      </c>
+      <c r="G10" t="n">
+        <v>1732319.752692774</v>
+      </c>
+      <c r="H10" t="n">
+        <v>46.51090945854524</v>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>2026-03-18T14:32:42</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2026-03-18</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>노브</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>185</v>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E11" t="n">
+        <v>1</v>
+      </c>
+      <c r="F11" t="n">
+        <v>5041442.310511444</v>
+      </c>
+      <c r="G11" t="n">
+        <v>1731434.310511444</v>
+      </c>
+      <c r="H11" t="n">
+        <v>52.30906724429197</v>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>2026-03-18T14:32:42</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2026-03-18</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>TIME 코리아밸류업액티브</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>201</v>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E12" t="n">
+        <v>1</v>
+      </c>
+      <c r="F12" t="n">
+        <v>4904400</v>
+      </c>
+      <c r="G12" t="n">
+        <v>180603</v>
+      </c>
+      <c r="H12" t="n">
+        <v>3.823259128197084</v>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>2026-03-18T14:32:42</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2026-03-18</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>오케아니스 에코 탱커스</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>65</v>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E13" t="n">
+        <v>1</v>
+      </c>
+      <c r="F13" t="n">
+        <v>4575098.725873504</v>
+      </c>
+      <c r="G13" t="n">
+        <v>2318738.725873504</v>
+      </c>
+      <c r="H13" t="n">
+        <v>102.7645732894354</v>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>2026-03-18T14:32:42</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026-03-18</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>삼성화재</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>9</v>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E14" t="n">
+        <v>1</v>
+      </c>
+      <c r="F14" t="n">
+        <v>4446000</v>
+      </c>
+      <c r="G14" t="n">
+        <v>-185000</v>
+      </c>
+      <c r="H14" t="n">
+        <v>-3.994817534009933</v>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>2026-03-18T14:32:42</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>2026-03-18</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>DL이앤씨</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>80</v>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E15" t="n">
+        <v>1</v>
+      </c>
+      <c r="F15" t="n">
+        <v>4128000</v>
+      </c>
+      <c r="G15" t="n">
+        <v>717000</v>
+      </c>
+      <c r="H15" t="n">
+        <v>21.02022867194371</v>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>2026-03-18T14:32:42</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-03-18</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>차코스 에너지 내비게이션</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>75</v>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E16" t="n">
+        <v>1</v>
+      </c>
+      <c r="F16" t="n">
+        <v>4007418.271141662</v>
+      </c>
+      <c r="G16" t="n">
+        <v>182770.2711416623</v>
+      </c>
+      <c r="H16" t="n">
+        <v>4.778747511971357</v>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>2026-03-18T14:32:42</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2026-03-18</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>동원개발</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
+        <v>1360</v>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E17" t="n">
+        <v>1</v>
+      </c>
+      <c r="F17" t="n">
+        <v>3978000</v>
+      </c>
+      <c r="G17" t="n">
+        <v>240600</v>
+      </c>
+      <c r="H17" t="n">
+        <v>6.437630438272596</v>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>2026-03-18T14:32:42</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>2026-03-18</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>HD건설기계</t>
+        </is>
+      </c>
+      <c r="C18" t="n">
+        <v>31</v>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E18" t="n">
+        <v>1</v>
+      </c>
+      <c r="F18" t="n">
+        <v>3955600</v>
+      </c>
+      <c r="G18" t="n">
+        <v>-79496</v>
+      </c>
+      <c r="H18" t="n">
+        <v>-1.970114217852561</v>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>2026-03-18T14:32:42</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>2026-03-18</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>피바디 에너지</t>
+        </is>
+      </c>
+      <c r="C19" t="n">
+        <v>65</v>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E19" t="n">
+        <v>1</v>
+      </c>
+      <c r="F19" t="n">
+        <v>3423839.074937592</v>
+      </c>
+      <c r="G19" t="n">
+        <v>1953067.074937592</v>
+      </c>
+      <c r="H19" t="n">
+        <v>132.7919674115085</v>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>2026-03-18T14:32:42</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>2026-03-18</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>더치 브로스</t>
+        </is>
+      </c>
+      <c r="C20" t="n">
+        <v>39</v>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E20" t="n">
+        <v>1</v>
+      </c>
+      <c r="F20" t="n">
+        <v>2965846.22503092</v>
+      </c>
+      <c r="G20" t="n">
+        <v>-224797.7749690795</v>
+      </c>
+      <c r="H20" t="n">
+        <v>-7.04552983564069</v>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>2026-03-18T14:32:42</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>2026-03-18</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>현대제철</t>
+        </is>
+      </c>
+      <c r="C21" t="n">
+        <v>70</v>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E21" t="n">
+        <v>1</v>
+      </c>
+      <c r="F21" t="n">
+        <v>2607500</v>
+      </c>
+      <c r="G21" t="n">
+        <v>-200000</v>
+      </c>
+      <c r="H21" t="n">
+        <v>-7.123775601068566</v>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>2026-03-18T14:32:42</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>2026-03-18</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>KoAct 코스닥액티브</t>
+        </is>
+      </c>
+      <c r="C22" t="n">
+        <v>200</v>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E22" t="n">
+        <v>1</v>
+      </c>
+      <c r="F22" t="n">
+        <v>2598000</v>
+      </c>
+      <c r="G22" t="n">
+        <v>-104000</v>
+      </c>
+      <c r="H22" t="n">
+        <v>-3.84900074019245</v>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>2026-03-18T14:32:42</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>2026-03-18</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>휴스틸</t>
+        </is>
+      </c>
+      <c r="C23" t="n">
+        <v>500</v>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E23" t="n">
+        <v>1</v>
+      </c>
+      <c r="F23" t="n">
+        <v>2560000</v>
+      </c>
+      <c r="G23" t="n">
+        <v>281390</v>
+      </c>
+      <c r="H23" t="n">
+        <v>12.34919534277476</v>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>2026-03-18T14:32:42</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>2026-03-18</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>넥스틸</t>
+        </is>
+      </c>
+      <c r="C24" t="n">
+        <v>200</v>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E24" t="n">
+        <v>1</v>
+      </c>
+      <c r="F24" t="n">
+        <v>2400000</v>
+      </c>
+      <c r="G24" t="n">
+        <v>389000</v>
+      </c>
+      <c r="H24" t="n">
+        <v>19.34361014420686</v>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>2026-03-18T14:32:42</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>2026-03-18</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>대신증권</t>
+        </is>
+      </c>
+      <c r="C25" t="n">
+        <v>55</v>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E25" t="n">
+        <v>1</v>
+      </c>
+      <c r="F25" t="n">
+        <v>2238500</v>
+      </c>
+      <c r="G25" t="n">
+        <v>528999</v>
+      </c>
+      <c r="H25" t="n">
+        <v>30.94464408034859</v>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>2026-03-18T14:32:42</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>2026-03-18</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>발레로 에너지</t>
+        </is>
+      </c>
+      <c r="C26" t="n">
+        <v>6</v>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E26" t="n">
+        <v>1</v>
+      </c>
+      <c r="F26" t="n">
+        <v>2138731.14071836</v>
+      </c>
+      <c r="G26" t="n">
+        <v>74741.1407183595</v>
+      </c>
+      <c r="H26" t="n">
+        <v>3.621196842928478</v>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>2026-03-18T14:32:42</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>2026-03-18</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>미창석유</t>
+        </is>
+      </c>
+      <c r="C27" t="n">
+        <v>18</v>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E27" t="n">
+        <v>1</v>
+      </c>
+      <c r="F27" t="n">
+        <v>2032200</v>
+      </c>
+      <c r="G27" t="n">
+        <v>-360000</v>
+      </c>
+      <c r="H27" t="n">
+        <v>-15.04890895410083</v>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>2026-03-18T14:32:42</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>2026-03-18</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>대창단조</t>
+        </is>
+      </c>
+      <c r="C28" t="n">
+        <v>300</v>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E28" t="n">
+        <v>1</v>
+      </c>
+      <c r="F28" t="n">
+        <v>1914000</v>
+      </c>
+      <c r="G28" t="n">
+        <v>-144000</v>
+      </c>
+      <c r="H28" t="n">
+        <v>-6.997084548104956</v>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>2026-03-18T14:32:42</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>2026-03-18</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>동방</t>
+        </is>
+      </c>
+      <c r="C29" t="n">
+        <v>681</v>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E29" t="n">
+        <v>1</v>
+      </c>
+      <c r="F29" t="n">
+        <v>1882965</v>
+      </c>
+      <c r="G29" t="n">
+        <v>-88536</v>
+      </c>
+      <c r="H29" t="n">
+        <v>-4.490791533963209</v>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>2026-03-18T14:32:42</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>2026-03-18</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>하나금융지주</t>
+        </is>
+      </c>
+      <c r="C30" t="n">
+        <v>15</v>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E30" t="n">
+        <v>1</v>
+      </c>
+      <c r="F30" t="n">
+        <v>1717500</v>
+      </c>
+      <c r="G30" t="n">
+        <v>35000</v>
+      </c>
+      <c r="H30" t="n">
+        <v>2.080237741456166</v>
+      </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>2026-03-18T14:32:42</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>2026-03-18</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>스타 벌크 캐리어스</t>
+        </is>
+      </c>
+      <c r="C31" t="n">
+        <v>50</v>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E31" t="n">
+        <v>1</v>
+      </c>
+      <c r="F31" t="n">
+        <v>1712476.648945617</v>
+      </c>
+      <c r="G31" t="n">
+        <v>398123.648945618</v>
+      </c>
+      <c r="H31" t="n">
+        <v>30.29046602743845</v>
+      </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>2026-03-18T14:32:42</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>2026-03-18</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>유나이티드헬스 그룹</t>
+        </is>
+      </c>
+      <c r="C32" t="n">
+        <v>4</v>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E32" t="n">
+        <v>1</v>
+      </c>
+      <c r="F32" t="n">
+        <v>1699490.128895313</v>
+      </c>
+      <c r="G32" t="n">
+        <v>5034.128895312548</v>
+      </c>
+      <c r="H32" t="n">
+        <v>0.297094105442251</v>
+      </c>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>2026-03-18T14:32:42</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>2026-03-18</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>케이씨</t>
+        </is>
+      </c>
+      <c r="C33" t="n">
+        <v>50</v>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E33" t="n">
+        <v>1</v>
+      </c>
+      <c r="F33" t="n">
+        <v>1640000</v>
+      </c>
+      <c r="G33" t="n">
+        <v>-9500.000000000698</v>
+      </c>
+      <c r="H33" t="n">
+        <v>-0.5759321006365986</v>
+      </c>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>2026-03-18T14:32:42</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>2026-03-18</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>삼성생명</t>
+        </is>
+      </c>
+      <c r="C34" t="n">
+        <v>4</v>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E34" t="n">
+        <v>1</v>
+      </c>
+      <c r="F34" t="n">
+        <v>940000</v>
+      </c>
+      <c r="G34" t="n">
+        <v>107000</v>
+      </c>
+      <c r="H34" t="n">
+        <v>12.84513805522209</v>
+      </c>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>2026-03-18T14:32:42</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>2026-03-18</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>클리블랜드 클리프스</t>
+        </is>
+      </c>
+      <c r="C35" t="n">
+        <v>70</v>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E35" t="n">
+        <v>1</v>
+      </c>
+      <c r="F35" t="n">
+        <v>857055.5630100402</v>
+      </c>
+      <c r="G35" t="n">
+        <v>-158999.4369899598</v>
+      </c>
+      <c r="H35" t="n">
+        <v>-15.64870376012714</v>
+      </c>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>2026-03-18T14:32:42</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>2026-03-18</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>비에이치아이</t>
+        </is>
+      </c>
+      <c r="C36" t="n">
+        <v>8</v>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E36" t="n">
+        <v>1</v>
+      </c>
+      <c r="F36" t="n">
+        <v>844800</v>
+      </c>
+      <c r="G36" t="n">
+        <v>179685</v>
+      </c>
+      <c r="H36" t="n">
+        <v>27.01562887620938</v>
+      </c>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>2026-03-18T14:32:42</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>2026-03-18</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>하프니아</t>
+        </is>
+      </c>
+      <c r="C37" t="n">
+        <v>80</v>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E37" t="n">
+        <v>1</v>
+      </c>
+      <c r="F37" t="n">
+        <v>821489.5606615674</v>
+      </c>
+      <c r="G37" t="n">
+        <v>195758.5606615674</v>
+      </c>
+      <c r="H37" t="n">
+        <v>31.28477902829928</v>
+      </c>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>2026-03-18T14:32:42</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>2026-03-18</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>텍사스 퍼시픽 랜드</t>
+        </is>
+      </c>
+      <c r="C38" t="n">
+        <v>1</v>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E38" t="n">
+        <v>1</v>
+      </c>
+      <c r="F38" t="n">
+        <v>794737.7576458007</v>
+      </c>
+      <c r="G38" t="n">
+        <v>16146.75764580071</v>
+      </c>
+      <c r="H38" t="n">
+        <v>2.073843345967358</v>
+      </c>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>2026-03-18T14:32:42</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>2026-03-18</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>노블</t>
+        </is>
+      </c>
+      <c r="C39" t="n">
+        <v>99</v>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E39" t="n">
+        <v>1</v>
+      </c>
+      <c r="F39" t="n">
+        <v>40689</v>
+      </c>
+      <c r="G39" t="n">
+        <v>-3866519</v>
+      </c>
+      <c r="H39" t="n">
+        <v>-98.95861699709869</v>
+      </c>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>2026-03-18T14:32:42</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>snapshot_date</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>cash_krw</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>cash_usd</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>created_at</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>updated_at</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>2026-03-18</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>31505056</v>
+      </c>
+      <c r="C2" t="n">
+        <v>6016.63</v>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>2026-03-18T12:21:00</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>2026-03-18T14:32:42</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
auto: portfolio snapshot 2026-03-17 (2026-03-18T21:07:31)
</commit_message>
<xml_diff>
--- a/portfolio_auto.xlsx
+++ b/portfolio_auto.xlsx
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G39"/>
+  <dimension ref="A1:G1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -466,1032 +466,6 @@
         <is>
           <t>수익률(%)</t>
         </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>페트로브라스 (ADR)</t>
-        </is>
-      </c>
-      <c r="B2" t="n">
-        <v>480</v>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>KRW</t>
-        </is>
-      </c>
-      <c r="D2" t="n">
-        <v>1</v>
-      </c>
-      <c r="E2" t="n">
-        <v>14082576.9328374</v>
-      </c>
-      <c r="F2" t="n">
-        <v>1976027.932837404</v>
-      </c>
-      <c r="G2" t="n">
-        <v>16.3219752617976</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>AGNC 인베스트먼트</t>
-        </is>
-      </c>
-      <c r="B3" t="n">
-        <v>700</v>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>KRW</t>
-        </is>
-      </c>
-      <c r="D3" t="n">
-        <v>1</v>
-      </c>
-      <c r="E3" t="n">
-        <v>10822406.73782303</v>
-      </c>
-      <c r="F3" t="n">
-        <v>-9608.262176971883</v>
-      </c>
-      <c r="G3" t="n">
-        <v>-0.08870244526961865</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>대한조선</t>
-        </is>
-      </c>
-      <c r="B4" t="n">
-        <v>100</v>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>KRW</t>
-        </is>
-      </c>
-      <c r="D4" t="n">
-        <v>1</v>
-      </c>
-      <c r="E4" t="n">
-        <v>9570000</v>
-      </c>
-      <c r="F4" t="n">
-        <v>2357000</v>
-      </c>
-      <c r="G4" t="n">
-        <v>32.67711077221684</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>프론트라인</t>
-        </is>
-      </c>
-      <c r="B5" t="n">
-        <v>175</v>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>KRW</t>
-        </is>
-      </c>
-      <c r="D5" t="n">
-        <v>1</v>
-      </c>
-      <c r="E5" t="n">
-        <v>8440541.129673157</v>
-      </c>
-      <c r="F5" t="n">
-        <v>4010677.129673157</v>
-      </c>
-      <c r="G5" t="n">
-        <v>90.53725192631549</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>시드릴</t>
-        </is>
-      </c>
-      <c r="B6" t="n">
-        <v>123</v>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>KRW</t>
-        </is>
-      </c>
-      <c r="D6" t="n">
-        <v>1</v>
-      </c>
-      <c r="E6" t="n">
-        <v>8090014.733635107</v>
-      </c>
-      <c r="F6" t="n">
-        <v>1639663.733635107</v>
-      </c>
-      <c r="G6" t="n">
-        <v>25.41975984927188</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>트랜스오션</t>
-        </is>
-      </c>
-      <c r="B7" t="n">
-        <v>750</v>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>KRW</t>
-        </is>
-      </c>
-      <c r="D7" t="n">
-        <v>1</v>
-      </c>
-      <c r="E7" t="n">
-        <v>7093219.418241119</v>
-      </c>
-      <c r="F7" t="n">
-        <v>2965985.418241119</v>
-      </c>
-      <c r="G7" t="n">
-        <v>71.86375713713153</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>세아제강</t>
-        </is>
-      </c>
-      <c r="B8" t="n">
-        <v>50</v>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>KRW</t>
-        </is>
-      </c>
-      <c r="D8" t="n">
-        <v>1</v>
-      </c>
-      <c r="E8" t="n">
-        <v>6915000</v>
-      </c>
-      <c r="F8" t="n">
-        <v>605000</v>
-      </c>
-      <c r="G8" t="n">
-        <v>9.587955625990491</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>센트러스 에너지</t>
-        </is>
-      </c>
-      <c r="B9" t="n">
-        <v>21</v>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>KRW</t>
-        </is>
-      </c>
-      <c r="D9" t="n">
-        <v>1</v>
-      </c>
-      <c r="E9" t="n">
-        <v>6546958.253894605</v>
-      </c>
-      <c r="F9" t="n">
-        <v>315739.2538946057</v>
-      </c>
-      <c r="G9" t="n">
-        <v>5.067054357977239</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>타이드워터</t>
-        </is>
-      </c>
-      <c r="B10" t="n">
-        <v>48</v>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>KRW</t>
-        </is>
-      </c>
-      <c r="D10" t="n">
-        <v>1</v>
-      </c>
-      <c r="E10" t="n">
-        <v>5456864.752692774</v>
-      </c>
-      <c r="F10" t="n">
-        <v>1732319.752692774</v>
-      </c>
-      <c r="G10" t="n">
-        <v>46.51090945854524</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>노브</t>
-        </is>
-      </c>
-      <c r="B11" t="n">
-        <v>185</v>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>KRW</t>
-        </is>
-      </c>
-      <c r="D11" t="n">
-        <v>1</v>
-      </c>
-      <c r="E11" t="n">
-        <v>5041442.310511444</v>
-      </c>
-      <c r="F11" t="n">
-        <v>1731434.310511444</v>
-      </c>
-      <c r="G11" t="n">
-        <v>52.30906724429197</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>TIME 코리아밸류업액티브</t>
-        </is>
-      </c>
-      <c r="B12" t="n">
-        <v>201</v>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>KRW</t>
-        </is>
-      </c>
-      <c r="D12" t="n">
-        <v>1</v>
-      </c>
-      <c r="E12" t="n">
-        <v>4904400</v>
-      </c>
-      <c r="F12" t="n">
-        <v>180603</v>
-      </c>
-      <c r="G12" t="n">
-        <v>3.823259128197084</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>오케아니스 에코 탱커스</t>
-        </is>
-      </c>
-      <c r="B13" t="n">
-        <v>65</v>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>KRW</t>
-        </is>
-      </c>
-      <c r="D13" t="n">
-        <v>1</v>
-      </c>
-      <c r="E13" t="n">
-        <v>4575098.725873504</v>
-      </c>
-      <c r="F13" t="n">
-        <v>2318738.725873504</v>
-      </c>
-      <c r="G13" t="n">
-        <v>102.7645732894354</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>삼성화재</t>
-        </is>
-      </c>
-      <c r="B14" t="n">
-        <v>9</v>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>KRW</t>
-        </is>
-      </c>
-      <c r="D14" t="n">
-        <v>1</v>
-      </c>
-      <c r="E14" t="n">
-        <v>4446000</v>
-      </c>
-      <c r="F14" t="n">
-        <v>-185000</v>
-      </c>
-      <c r="G14" t="n">
-        <v>-3.994817534009933</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>DL이앤씨</t>
-        </is>
-      </c>
-      <c r="B15" t="n">
-        <v>80</v>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>KRW</t>
-        </is>
-      </c>
-      <c r="D15" t="n">
-        <v>1</v>
-      </c>
-      <c r="E15" t="n">
-        <v>4128000</v>
-      </c>
-      <c r="F15" t="n">
-        <v>717000</v>
-      </c>
-      <c r="G15" t="n">
-        <v>21.02022867194371</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>차코스 에너지 내비게이션</t>
-        </is>
-      </c>
-      <c r="B16" t="n">
-        <v>75</v>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>KRW</t>
-        </is>
-      </c>
-      <c r="D16" t="n">
-        <v>1</v>
-      </c>
-      <c r="E16" t="n">
-        <v>4007418.271141662</v>
-      </c>
-      <c r="F16" t="n">
-        <v>182770.2711416623</v>
-      </c>
-      <c r="G16" t="n">
-        <v>4.778747511971357</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>동원개발</t>
-        </is>
-      </c>
-      <c r="B17" t="n">
-        <v>1360</v>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>KRW</t>
-        </is>
-      </c>
-      <c r="D17" t="n">
-        <v>1</v>
-      </c>
-      <c r="E17" t="n">
-        <v>3978000</v>
-      </c>
-      <c r="F17" t="n">
-        <v>240600</v>
-      </c>
-      <c r="G17" t="n">
-        <v>6.437630438272596</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>HD건설기계</t>
-        </is>
-      </c>
-      <c r="B18" t="n">
-        <v>31</v>
-      </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>KRW</t>
-        </is>
-      </c>
-      <c r="D18" t="n">
-        <v>1</v>
-      </c>
-      <c r="E18" t="n">
-        <v>3955600</v>
-      </c>
-      <c r="F18" t="n">
-        <v>-79496</v>
-      </c>
-      <c r="G18" t="n">
-        <v>-1.970114217852561</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>피바디 에너지</t>
-        </is>
-      </c>
-      <c r="B19" t="n">
-        <v>65</v>
-      </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>KRW</t>
-        </is>
-      </c>
-      <c r="D19" t="n">
-        <v>1</v>
-      </c>
-      <c r="E19" t="n">
-        <v>3423839.074937592</v>
-      </c>
-      <c r="F19" t="n">
-        <v>1953067.074937592</v>
-      </c>
-      <c r="G19" t="n">
-        <v>132.7919674115085</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>더치 브로스</t>
-        </is>
-      </c>
-      <c r="B20" t="n">
-        <v>39</v>
-      </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>KRW</t>
-        </is>
-      </c>
-      <c r="D20" t="n">
-        <v>1</v>
-      </c>
-      <c r="E20" t="n">
-        <v>2965846.22503092</v>
-      </c>
-      <c r="F20" t="n">
-        <v>-224797.7749690795</v>
-      </c>
-      <c r="G20" t="n">
-        <v>-7.04552983564069</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>현대제철</t>
-        </is>
-      </c>
-      <c r="B21" t="n">
-        <v>70</v>
-      </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>KRW</t>
-        </is>
-      </c>
-      <c r="D21" t="n">
-        <v>1</v>
-      </c>
-      <c r="E21" t="n">
-        <v>2607500</v>
-      </c>
-      <c r="F21" t="n">
-        <v>-200000</v>
-      </c>
-      <c r="G21" t="n">
-        <v>-7.123775601068566</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>KoAct 코스닥액티브</t>
-        </is>
-      </c>
-      <c r="B22" t="n">
-        <v>200</v>
-      </c>
-      <c r="C22" t="inlineStr">
-        <is>
-          <t>KRW</t>
-        </is>
-      </c>
-      <c r="D22" t="n">
-        <v>1</v>
-      </c>
-      <c r="E22" t="n">
-        <v>2598000</v>
-      </c>
-      <c r="F22" t="n">
-        <v>-104000</v>
-      </c>
-      <c r="G22" t="n">
-        <v>-3.84900074019245</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>휴스틸</t>
-        </is>
-      </c>
-      <c r="B23" t="n">
-        <v>500</v>
-      </c>
-      <c r="C23" t="inlineStr">
-        <is>
-          <t>KRW</t>
-        </is>
-      </c>
-      <c r="D23" t="n">
-        <v>1</v>
-      </c>
-      <c r="E23" t="n">
-        <v>2560000</v>
-      </c>
-      <c r="F23" t="n">
-        <v>281390</v>
-      </c>
-      <c r="G23" t="n">
-        <v>12.34919534277476</v>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>넥스틸</t>
-        </is>
-      </c>
-      <c r="B24" t="n">
-        <v>200</v>
-      </c>
-      <c r="C24" t="inlineStr">
-        <is>
-          <t>KRW</t>
-        </is>
-      </c>
-      <c r="D24" t="n">
-        <v>1</v>
-      </c>
-      <c r="E24" t="n">
-        <v>2400000</v>
-      </c>
-      <c r="F24" t="n">
-        <v>389000</v>
-      </c>
-      <c r="G24" t="n">
-        <v>19.34361014420686</v>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>대신증권</t>
-        </is>
-      </c>
-      <c r="B25" t="n">
-        <v>55</v>
-      </c>
-      <c r="C25" t="inlineStr">
-        <is>
-          <t>KRW</t>
-        </is>
-      </c>
-      <c r="D25" t="n">
-        <v>1</v>
-      </c>
-      <c r="E25" t="n">
-        <v>2238500</v>
-      </c>
-      <c r="F25" t="n">
-        <v>528999</v>
-      </c>
-      <c r="G25" t="n">
-        <v>30.94464408034859</v>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>발레로 에너지</t>
-        </is>
-      </c>
-      <c r="B26" t="n">
-        <v>6</v>
-      </c>
-      <c r="C26" t="inlineStr">
-        <is>
-          <t>KRW</t>
-        </is>
-      </c>
-      <c r="D26" t="n">
-        <v>1</v>
-      </c>
-      <c r="E26" t="n">
-        <v>2138731.14071836</v>
-      </c>
-      <c r="F26" t="n">
-        <v>74741.1407183595</v>
-      </c>
-      <c r="G26" t="n">
-        <v>3.621196842928478</v>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>미창석유</t>
-        </is>
-      </c>
-      <c r="B27" t="n">
-        <v>18</v>
-      </c>
-      <c r="C27" t="inlineStr">
-        <is>
-          <t>KRW</t>
-        </is>
-      </c>
-      <c r="D27" t="n">
-        <v>1</v>
-      </c>
-      <c r="E27" t="n">
-        <v>2032200</v>
-      </c>
-      <c r="F27" t="n">
-        <v>-360000</v>
-      </c>
-      <c r="G27" t="n">
-        <v>-15.04890895410083</v>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>대창단조</t>
-        </is>
-      </c>
-      <c r="B28" t="n">
-        <v>300</v>
-      </c>
-      <c r="C28" t="inlineStr">
-        <is>
-          <t>KRW</t>
-        </is>
-      </c>
-      <c r="D28" t="n">
-        <v>1</v>
-      </c>
-      <c r="E28" t="n">
-        <v>1914000</v>
-      </c>
-      <c r="F28" t="n">
-        <v>-144000</v>
-      </c>
-      <c r="G28" t="n">
-        <v>-6.997084548104956</v>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>동방</t>
-        </is>
-      </c>
-      <c r="B29" t="n">
-        <v>681</v>
-      </c>
-      <c r="C29" t="inlineStr">
-        <is>
-          <t>KRW</t>
-        </is>
-      </c>
-      <c r="D29" t="n">
-        <v>1</v>
-      </c>
-      <c r="E29" t="n">
-        <v>1882965</v>
-      </c>
-      <c r="F29" t="n">
-        <v>-88536</v>
-      </c>
-      <c r="G29" t="n">
-        <v>-4.490791533963209</v>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t>하나금융지주</t>
-        </is>
-      </c>
-      <c r="B30" t="n">
-        <v>15</v>
-      </c>
-      <c r="C30" t="inlineStr">
-        <is>
-          <t>KRW</t>
-        </is>
-      </c>
-      <c r="D30" t="n">
-        <v>1</v>
-      </c>
-      <c r="E30" t="n">
-        <v>1717500</v>
-      </c>
-      <c r="F30" t="n">
-        <v>35000</v>
-      </c>
-      <c r="G30" t="n">
-        <v>2.080237741456166</v>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="inlineStr">
-        <is>
-          <t>스타 벌크 캐리어스</t>
-        </is>
-      </c>
-      <c r="B31" t="n">
-        <v>50</v>
-      </c>
-      <c r="C31" t="inlineStr">
-        <is>
-          <t>KRW</t>
-        </is>
-      </c>
-      <c r="D31" t="n">
-        <v>1</v>
-      </c>
-      <c r="E31" t="n">
-        <v>1712476.648945617</v>
-      </c>
-      <c r="F31" t="n">
-        <v>398123.648945618</v>
-      </c>
-      <c r="G31" t="n">
-        <v>30.29046602743845</v>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="inlineStr">
-        <is>
-          <t>유나이티드헬스 그룹</t>
-        </is>
-      </c>
-      <c r="B32" t="n">
-        <v>4</v>
-      </c>
-      <c r="C32" t="inlineStr">
-        <is>
-          <t>KRW</t>
-        </is>
-      </c>
-      <c r="D32" t="n">
-        <v>1</v>
-      </c>
-      <c r="E32" t="n">
-        <v>1699490.128895313</v>
-      </c>
-      <c r="F32" t="n">
-        <v>5034.128895312548</v>
-      </c>
-      <c r="G32" t="n">
-        <v>0.297094105442251</v>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" t="inlineStr">
-        <is>
-          <t>케이씨</t>
-        </is>
-      </c>
-      <c r="B33" t="n">
-        <v>50</v>
-      </c>
-      <c r="C33" t="inlineStr">
-        <is>
-          <t>KRW</t>
-        </is>
-      </c>
-      <c r="D33" t="n">
-        <v>1</v>
-      </c>
-      <c r="E33" t="n">
-        <v>1640000</v>
-      </c>
-      <c r="F33" t="n">
-        <v>-9500.000000000698</v>
-      </c>
-      <c r="G33" t="n">
-        <v>-0.5759321006365986</v>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" t="inlineStr">
-        <is>
-          <t>삼성생명</t>
-        </is>
-      </c>
-      <c r="B34" t="n">
-        <v>4</v>
-      </c>
-      <c r="C34" t="inlineStr">
-        <is>
-          <t>KRW</t>
-        </is>
-      </c>
-      <c r="D34" t="n">
-        <v>1</v>
-      </c>
-      <c r="E34" t="n">
-        <v>940000</v>
-      </c>
-      <c r="F34" t="n">
-        <v>107000</v>
-      </c>
-      <c r="G34" t="n">
-        <v>12.84513805522209</v>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" t="inlineStr">
-        <is>
-          <t>클리블랜드 클리프스</t>
-        </is>
-      </c>
-      <c r="B35" t="n">
-        <v>70</v>
-      </c>
-      <c r="C35" t="inlineStr">
-        <is>
-          <t>KRW</t>
-        </is>
-      </c>
-      <c r="D35" t="n">
-        <v>1</v>
-      </c>
-      <c r="E35" t="n">
-        <v>857055.5630100402</v>
-      </c>
-      <c r="F35" t="n">
-        <v>-158999.4369899598</v>
-      </c>
-      <c r="G35" t="n">
-        <v>-15.64870376012714</v>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" t="inlineStr">
-        <is>
-          <t>비에이치아이</t>
-        </is>
-      </c>
-      <c r="B36" t="n">
-        <v>8</v>
-      </c>
-      <c r="C36" t="inlineStr">
-        <is>
-          <t>KRW</t>
-        </is>
-      </c>
-      <c r="D36" t="n">
-        <v>1</v>
-      </c>
-      <c r="E36" t="n">
-        <v>844800</v>
-      </c>
-      <c r="F36" t="n">
-        <v>179685</v>
-      </c>
-      <c r="G36" t="n">
-        <v>27.01562887620938</v>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" t="inlineStr">
-        <is>
-          <t>하프니아</t>
-        </is>
-      </c>
-      <c r="B37" t="n">
-        <v>80</v>
-      </c>
-      <c r="C37" t="inlineStr">
-        <is>
-          <t>KRW</t>
-        </is>
-      </c>
-      <c r="D37" t="n">
-        <v>1</v>
-      </c>
-      <c r="E37" t="n">
-        <v>821489.5606615674</v>
-      </c>
-      <c r="F37" t="n">
-        <v>195758.5606615674</v>
-      </c>
-      <c r="G37" t="n">
-        <v>31.28477902829928</v>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" t="inlineStr">
-        <is>
-          <t>텍사스 퍼시픽 랜드</t>
-        </is>
-      </c>
-      <c r="B38" t="n">
-        <v>1</v>
-      </c>
-      <c r="C38" t="inlineStr">
-        <is>
-          <t>KRW</t>
-        </is>
-      </c>
-      <c r="D38" t="n">
-        <v>1</v>
-      </c>
-      <c r="E38" t="n">
-        <v>794737.7576458007</v>
-      </c>
-      <c r="F38" t="n">
-        <v>16146.75764580071</v>
-      </c>
-      <c r="G38" t="n">
-        <v>2.073843345967358</v>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" t="inlineStr">
-        <is>
-          <t>노블</t>
-        </is>
-      </c>
-      <c r="B39" t="n">
-        <v>99</v>
-      </c>
-      <c r="C39" t="inlineStr">
-        <is>
-          <t>KRW</t>
-        </is>
-      </c>
-      <c r="D39" t="n">
-        <v>1</v>
-      </c>
-      <c r="E39" t="n">
-        <v>40689</v>
-      </c>
-      <c r="F39" t="n">
-        <v>-3866519</v>
-      </c>
-      <c r="G39" t="n">
-        <v>-98.95861699709869</v>
       </c>
     </row>
   </sheetData>
@@ -1538,22 +512,22 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-03-18</t>
+          <t>2026-03-17</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>31505056</v>
+        <v>33078556</v>
       </c>
       <c r="C2" t="n">
-        <v>6016.63</v>
+        <v>6010.99</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2026-03-18T21:07:08</t>
+          <t>2026-03-18T21:07:31</t>
         </is>
       </c>
       <c r="E2" t="n">
-        <v>1485.880004882812</v>
+        <v>1488.910034179688</v>
       </c>
     </row>
   </sheetData>
@@ -3034,7 +2008,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E2"/>
+  <dimension ref="A1:E3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3067,21 +2041,44 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-03-18</t>
+          <t>2026-03-17</t>
         </is>
       </c>
       <c r="B2" t="n">
+        <v>33078556</v>
+      </c>
+      <c r="C2" t="n">
+        <v>6010.99</v>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>2026-03-18T21:07:31</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>2026-03-18T21:07:31</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-03-18</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
         <v>31505056</v>
       </c>
-      <c r="C2" t="n">
+      <c r="C3" t="n">
         <v>6016.63</v>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="D3" t="inlineStr">
         <is>
           <t>2026-03-18T12:21:00</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="E3" t="inlineStr">
         <is>
           <t>2026-03-18T14:32:42</t>
         </is>

</xml_diff>

<commit_message>
auto: portfolio snapshot 2026-03-17 (2026-03-18T21:08:03)
</commit_message>
<xml_diff>
--- a/portfolio_auto.xlsx
+++ b/portfolio_auto.xlsx
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G1"/>
+  <dimension ref="A1:G15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -466,6 +466,384 @@
         <is>
           <t>수익률(%)</t>
         </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>노브</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>185</v>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E2" t="n">
+        <v>5067449</v>
+      </c>
+      <c r="F2" t="n">
+        <v>1757441</v>
+      </c>
+      <c r="G2" t="n">
+        <v>53.09</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>노블</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>99</v>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E3" t="n">
+        <v>6882090</v>
+      </c>
+      <c r="F3" t="n">
+        <v>2974882</v>
+      </c>
+      <c r="G3" t="n">
+        <v>76.13</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>더치 브로스</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>39</v>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>1</v>
+      </c>
+      <c r="E4" t="n">
+        <v>2926290</v>
+      </c>
+      <c r="F4" t="n">
+        <v>-264354</v>
+      </c>
+      <c r="G4" t="n">
+        <v>-8.279999999999999</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>발레로 에너지</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>6</v>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>1</v>
+      </c>
+      <c r="E5" t="n">
+        <v>2096946</v>
+      </c>
+      <c r="F5" t="n">
+        <v>32956</v>
+      </c>
+      <c r="G5" t="n">
+        <v>1.59</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>센트러스 에너지</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>21</v>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>1</v>
+      </c>
+      <c r="E6" t="n">
+        <v>6691594</v>
+      </c>
+      <c r="F6" t="n">
+        <v>460375</v>
+      </c>
+      <c r="G6" t="n">
+        <v>7.38</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>스타 벌크 캐리어스</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>50</v>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>1</v>
+      </c>
+      <c r="E7" t="n">
+        <v>1661361</v>
+      </c>
+      <c r="F7" t="n">
+        <v>347008</v>
+      </c>
+      <c r="G7" t="n">
+        <v>26.4</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>시드릴</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>123</v>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>1</v>
+      </c>
+      <c r="E8" t="n">
+        <v>7927448</v>
+      </c>
+      <c r="F8" t="n">
+        <v>1477097</v>
+      </c>
+      <c r="G8" t="n">
+        <v>22.89</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>오케아니스 에코 탱커스</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>65</v>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>1</v>
+      </c>
+      <c r="E9" t="n">
+        <v>4451759</v>
+      </c>
+      <c r="F9" t="n">
+        <v>2195399</v>
+      </c>
+      <c r="G9" t="n">
+        <v>97.29000000000001</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>유나이티드헬스 그룹</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>4</v>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>1</v>
+      </c>
+      <c r="E10" t="n">
+        <v>1710490</v>
+      </c>
+      <c r="F10" t="n">
+        <v>16034</v>
+      </c>
+      <c r="G10" t="n">
+        <v>0.9399999999999999</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>차코스 에너지 내비게이션</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>75</v>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>1</v>
+      </c>
+      <c r="E11" t="n">
+        <v>3919272</v>
+      </c>
+      <c r="F11" t="n">
+        <v>94624</v>
+      </c>
+      <c r="G11" t="n">
+        <v>2.47</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>클리블랜드 클리프스</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>70</v>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>1</v>
+      </c>
+      <c r="E12" t="n">
+        <v>908091</v>
+      </c>
+      <c r="F12" t="n">
+        <v>-107964</v>
+      </c>
+      <c r="G12" t="n">
+        <v>-10.62</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>타이드워터</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>48</v>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>1</v>
+      </c>
+      <c r="E13" t="n">
+        <v>5429641</v>
+      </c>
+      <c r="F13" t="n">
+        <v>1705096</v>
+      </c>
+      <c r="G13" t="n">
+        <v>45.78</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>텍사스 퍼시픽 랜드</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>1</v>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>1</v>
+      </c>
+      <c r="E14" t="n">
+        <v>786665</v>
+      </c>
+      <c r="F14" t="n">
+        <v>8074</v>
+      </c>
+      <c r="G14" t="n">
+        <v>1.03</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>트랜스오션</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>750</v>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>1</v>
+      </c>
+      <c r="E15" t="n">
+        <v>6945333</v>
+      </c>
+      <c r="F15" t="n">
+        <v>2818099</v>
+      </c>
+      <c r="G15" t="n">
+        <v>68.28</v>
       </c>
     </row>
   </sheetData>
@@ -523,7 +901,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2026-03-18T21:07:31</t>
+          <t>2026-03-18T21:08:03</t>
         </is>
       </c>
       <c r="E2" t="n">
@@ -541,7 +919,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I39"/>
+  <dimension ref="A1:I53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -594,16 +972,16 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-03-18</t>
+          <t>2026-03-17</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>페트로브라스 (ADR)</t>
+          <t>시드릴</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>480</v>
+        <v>123</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
@@ -614,33 +992,33 @@
         <v>1</v>
       </c>
       <c r="F2" t="n">
-        <v>14082576.9328374</v>
+        <v>7927448</v>
       </c>
       <c r="G2" t="n">
-        <v>1976027.932837404</v>
+        <v>1477097</v>
       </c>
       <c r="H2" t="n">
-        <v>16.3219752617976</v>
+        <v>22.89</v>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>2026-03-18T14:32:42</t>
+          <t>2026-03-18T21:08:03</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-03-18</t>
+          <t>2026-03-17</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>AGNC 인베스트먼트</t>
+          <t>트랜스오션</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>700</v>
+        <v>750</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
@@ -651,33 +1029,33 @@
         <v>1</v>
       </c>
       <c r="F3" t="n">
-        <v>10822406.73782303</v>
+        <v>6945333</v>
       </c>
       <c r="G3" t="n">
-        <v>-9608.262176971883</v>
+        <v>2818099</v>
       </c>
       <c r="H3" t="n">
-        <v>-0.08870244526961865</v>
+        <v>68.28</v>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>2026-03-18T14:32:42</t>
+          <t>2026-03-18T21:08:03</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-03-18</t>
+          <t>2026-03-17</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>대한조선</t>
+          <t>노블</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
@@ -688,33 +1066,33 @@
         <v>1</v>
       </c>
       <c r="F4" t="n">
-        <v>9570000</v>
+        <v>6882090</v>
       </c>
       <c r="G4" t="n">
-        <v>2357000</v>
+        <v>2974882</v>
       </c>
       <c r="H4" t="n">
-        <v>32.67711077221684</v>
+        <v>76.13</v>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>2026-03-18T14:32:42</t>
+          <t>2026-03-18T21:08:03</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-03-18</t>
+          <t>2026-03-17</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>프론트라인</t>
+          <t>센트러스 에너지</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>175</v>
+        <v>21</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
@@ -725,33 +1103,33 @@
         <v>1</v>
       </c>
       <c r="F5" t="n">
-        <v>8440541.129673157</v>
+        <v>6691594</v>
       </c>
       <c r="G5" t="n">
-        <v>4010677.129673157</v>
+        <v>460375</v>
       </c>
       <c r="H5" t="n">
-        <v>90.53725192631549</v>
+        <v>7.38</v>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>2026-03-18T14:32:42</t>
+          <t>2026-03-18T21:08:03</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-03-18</t>
+          <t>2026-03-17</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>시드릴</t>
+          <t>타이드워터</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>123</v>
+        <v>48</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
@@ -762,33 +1140,33 @@
         <v>1</v>
       </c>
       <c r="F6" t="n">
-        <v>8090014.733635107</v>
+        <v>5429641</v>
       </c>
       <c r="G6" t="n">
-        <v>1639663.733635107</v>
+        <v>1705096</v>
       </c>
       <c r="H6" t="n">
-        <v>25.41975984927188</v>
+        <v>45.78</v>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>2026-03-18T14:32:42</t>
+          <t>2026-03-18T21:08:03</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-03-18</t>
+          <t>2026-03-17</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>트랜스오션</t>
+          <t>노브</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>750</v>
+        <v>185</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
@@ -799,33 +1177,33 @@
         <v>1</v>
       </c>
       <c r="F7" t="n">
-        <v>7093219.418241119</v>
+        <v>5067449</v>
       </c>
       <c r="G7" t="n">
-        <v>2965985.418241119</v>
+        <v>1757441</v>
       </c>
       <c r="H7" t="n">
-        <v>71.86375713713153</v>
+        <v>53.09</v>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>2026-03-18T14:32:42</t>
+          <t>2026-03-18T21:08:03</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-03-18</t>
+          <t>2026-03-17</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>세아제강</t>
+          <t>오케아니스 에코 탱커스</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>50</v>
+        <v>65</v>
       </c>
       <c r="D8" t="inlineStr">
         <is>
@@ -836,33 +1214,33 @@
         <v>1</v>
       </c>
       <c r="F8" t="n">
-        <v>6915000</v>
+        <v>4451759</v>
       </c>
       <c r="G8" t="n">
-        <v>605000</v>
+        <v>2195399</v>
       </c>
       <c r="H8" t="n">
-        <v>9.587955625990491</v>
+        <v>97.29000000000001</v>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>2026-03-18T14:32:42</t>
+          <t>2026-03-18T21:08:03</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-03-18</t>
+          <t>2026-03-17</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>센트러스 에너지</t>
+          <t>차코스 에너지 내비게이션</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>21</v>
+        <v>75</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
@@ -873,33 +1251,33 @@
         <v>1</v>
       </c>
       <c r="F9" t="n">
-        <v>6546958.253894605</v>
+        <v>3919272</v>
       </c>
       <c r="G9" t="n">
-        <v>315739.2538946057</v>
+        <v>94624</v>
       </c>
       <c r="H9" t="n">
-        <v>5.067054357977239</v>
+        <v>2.47</v>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>2026-03-18T14:32:42</t>
+          <t>2026-03-18T21:08:03</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-03-18</t>
+          <t>2026-03-17</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>타이드워터</t>
+          <t>더치 브로스</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>48</v>
+        <v>39</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
@@ -910,33 +1288,33 @@
         <v>1</v>
       </c>
       <c r="F10" t="n">
-        <v>5456864.752692774</v>
+        <v>2926290</v>
       </c>
       <c r="G10" t="n">
-        <v>1732319.752692774</v>
+        <v>-264354</v>
       </c>
       <c r="H10" t="n">
-        <v>46.51090945854524</v>
+        <v>-8.279999999999999</v>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>2026-03-18T14:32:42</t>
+          <t>2026-03-18T21:08:03</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-03-18</t>
+          <t>2026-03-17</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>노브</t>
+          <t>발레로 에너지</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>185</v>
+        <v>6</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
@@ -947,33 +1325,33 @@
         <v>1</v>
       </c>
       <c r="F11" t="n">
-        <v>5041442.310511444</v>
+        <v>2096946</v>
       </c>
       <c r="G11" t="n">
-        <v>1731434.310511444</v>
+        <v>32956</v>
       </c>
       <c r="H11" t="n">
-        <v>52.30906724429197</v>
+        <v>1.59</v>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>2026-03-18T14:32:42</t>
+          <t>2026-03-18T21:08:03</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-03-18</t>
+          <t>2026-03-17</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>TIME 코리아밸류업액티브</t>
+          <t>유나이티드헬스 그룹</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>201</v>
+        <v>4</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
@@ -984,33 +1362,33 @@
         <v>1</v>
       </c>
       <c r="F12" t="n">
-        <v>4904400</v>
+        <v>1710490</v>
       </c>
       <c r="G12" t="n">
-        <v>180603</v>
+        <v>16034</v>
       </c>
       <c r="H12" t="n">
-        <v>3.823259128197084</v>
+        <v>0.9399999999999999</v>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>2026-03-18T14:32:42</t>
+          <t>2026-03-18T21:08:03</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-03-18</t>
+          <t>2026-03-17</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>오케아니스 에코 탱커스</t>
+          <t>스타 벌크 캐리어스</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>65</v>
+        <v>50</v>
       </c>
       <c r="D13" t="inlineStr">
         <is>
@@ -1021,33 +1399,33 @@
         <v>1</v>
       </c>
       <c r="F13" t="n">
-        <v>4575098.725873504</v>
+        <v>1661361</v>
       </c>
       <c r="G13" t="n">
-        <v>2318738.725873504</v>
+        <v>347008</v>
       </c>
       <c r="H13" t="n">
-        <v>102.7645732894354</v>
+        <v>26.4</v>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>2026-03-18T14:32:42</t>
+          <t>2026-03-18T21:08:03</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-03-18</t>
+          <t>2026-03-17</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>삼성화재</t>
+          <t>클리블랜드 클리프스</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>9</v>
+        <v>70</v>
       </c>
       <c r="D14" t="inlineStr">
         <is>
@@ -1058,33 +1436,33 @@
         <v>1</v>
       </c>
       <c r="F14" t="n">
-        <v>4446000</v>
+        <v>908091</v>
       </c>
       <c r="G14" t="n">
-        <v>-185000</v>
+        <v>-107964</v>
       </c>
       <c r="H14" t="n">
-        <v>-3.994817534009933</v>
+        <v>-10.62</v>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>2026-03-18T14:32:42</t>
+          <t>2026-03-18T21:08:03</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-03-18</t>
+          <t>2026-03-17</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>DL이앤씨</t>
+          <t>텍사스 퍼시픽 랜드</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>80</v>
+        <v>1</v>
       </c>
       <c r="D15" t="inlineStr">
         <is>
@@ -1095,17 +1473,17 @@
         <v>1</v>
       </c>
       <c r="F15" t="n">
-        <v>4128000</v>
+        <v>786665</v>
       </c>
       <c r="G15" t="n">
-        <v>717000</v>
+        <v>8074</v>
       </c>
       <c r="H15" t="n">
-        <v>21.02022867194371</v>
+        <v>1.03</v>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>2026-03-18T14:32:42</t>
+          <t>2026-03-18T21:08:03</t>
         </is>
       </c>
     </row>
@@ -1117,11 +1495,11 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>차코스 에너지 내비게이션</t>
+          <t>페트로브라스 (ADR)</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>75</v>
+        <v>480</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
@@ -1132,13 +1510,13 @@
         <v>1</v>
       </c>
       <c r="F16" t="n">
-        <v>4007418.271141662</v>
+        <v>14082576.9328374</v>
       </c>
       <c r="G16" t="n">
-        <v>182770.2711416623</v>
+        <v>1976027.932837404</v>
       </c>
       <c r="H16" t="n">
-        <v>4.778747511971357</v>
+        <v>16.3219752617976</v>
       </c>
       <c r="I16" t="inlineStr">
         <is>
@@ -1154,11 +1532,11 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>동원개발</t>
+          <t>AGNC 인베스트먼트</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>1360</v>
+        <v>700</v>
       </c>
       <c r="D17" t="inlineStr">
         <is>
@@ -1169,13 +1547,13 @@
         <v>1</v>
       </c>
       <c r="F17" t="n">
-        <v>3978000</v>
+        <v>10822406.73782303</v>
       </c>
       <c r="G17" t="n">
-        <v>240600</v>
+        <v>-9608.262176971883</v>
       </c>
       <c r="H17" t="n">
-        <v>6.437630438272596</v>
+        <v>-0.08870244526961865</v>
       </c>
       <c r="I17" t="inlineStr">
         <is>
@@ -1191,11 +1569,11 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>HD건설기계</t>
+          <t>대한조선</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>31</v>
+        <v>100</v>
       </c>
       <c r="D18" t="inlineStr">
         <is>
@@ -1206,13 +1584,13 @@
         <v>1</v>
       </c>
       <c r="F18" t="n">
-        <v>3955600</v>
+        <v>9570000</v>
       </c>
       <c r="G18" t="n">
-        <v>-79496</v>
+        <v>2357000</v>
       </c>
       <c r="H18" t="n">
-        <v>-1.970114217852561</v>
+        <v>32.67711077221684</v>
       </c>
       <c r="I18" t="inlineStr">
         <is>
@@ -1228,11 +1606,11 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>피바디 에너지</t>
+          <t>프론트라인</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>65</v>
+        <v>175</v>
       </c>
       <c r="D19" t="inlineStr">
         <is>
@@ -1243,13 +1621,13 @@
         <v>1</v>
       </c>
       <c r="F19" t="n">
-        <v>3423839.074937592</v>
+        <v>8440541.129673157</v>
       </c>
       <c r="G19" t="n">
-        <v>1953067.074937592</v>
+        <v>4010677.129673157</v>
       </c>
       <c r="H19" t="n">
-        <v>132.7919674115085</v>
+        <v>90.53725192631549</v>
       </c>
       <c r="I19" t="inlineStr">
         <is>
@@ -1265,11 +1643,11 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>더치 브로스</t>
+          <t>시드릴</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>39</v>
+        <v>123</v>
       </c>
       <c r="D20" t="inlineStr">
         <is>
@@ -1280,13 +1658,13 @@
         <v>1</v>
       </c>
       <c r="F20" t="n">
-        <v>2965846.22503092</v>
+        <v>8090014.733635107</v>
       </c>
       <c r="G20" t="n">
-        <v>-224797.7749690795</v>
+        <v>1639663.733635107</v>
       </c>
       <c r="H20" t="n">
-        <v>-7.04552983564069</v>
+        <v>25.41975984927188</v>
       </c>
       <c r="I20" t="inlineStr">
         <is>
@@ -1302,11 +1680,11 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>현대제철</t>
+          <t>트랜스오션</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>70</v>
+        <v>750</v>
       </c>
       <c r="D21" t="inlineStr">
         <is>
@@ -1317,13 +1695,13 @@
         <v>1</v>
       </c>
       <c r="F21" t="n">
-        <v>2607500</v>
+        <v>7093219.418241119</v>
       </c>
       <c r="G21" t="n">
-        <v>-200000</v>
+        <v>2965985.418241119</v>
       </c>
       <c r="H21" t="n">
-        <v>-7.123775601068566</v>
+        <v>71.86375713713153</v>
       </c>
       <c r="I21" t="inlineStr">
         <is>
@@ -1339,11 +1717,11 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>KoAct 코스닥액티브</t>
+          <t>세아제강</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>200</v>
+        <v>50</v>
       </c>
       <c r="D22" t="inlineStr">
         <is>
@@ -1354,13 +1732,13 @@
         <v>1</v>
       </c>
       <c r="F22" t="n">
-        <v>2598000</v>
+        <v>6915000</v>
       </c>
       <c r="G22" t="n">
-        <v>-104000</v>
+        <v>605000</v>
       </c>
       <c r="H22" t="n">
-        <v>-3.84900074019245</v>
+        <v>9.587955625990491</v>
       </c>
       <c r="I22" t="inlineStr">
         <is>
@@ -1376,11 +1754,11 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>휴스틸</t>
+          <t>센트러스 에너지</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>500</v>
+        <v>21</v>
       </c>
       <c r="D23" t="inlineStr">
         <is>
@@ -1391,13 +1769,13 @@
         <v>1</v>
       </c>
       <c r="F23" t="n">
-        <v>2560000</v>
+        <v>6546958.253894605</v>
       </c>
       <c r="G23" t="n">
-        <v>281390</v>
+        <v>315739.2538946057</v>
       </c>
       <c r="H23" t="n">
-        <v>12.34919534277476</v>
+        <v>5.067054357977239</v>
       </c>
       <c r="I23" t="inlineStr">
         <is>
@@ -1413,11 +1791,11 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>넥스틸</t>
+          <t>타이드워터</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>200</v>
+        <v>48</v>
       </c>
       <c r="D24" t="inlineStr">
         <is>
@@ -1428,13 +1806,13 @@
         <v>1</v>
       </c>
       <c r="F24" t="n">
-        <v>2400000</v>
+        <v>5456864.752692774</v>
       </c>
       <c r="G24" t="n">
-        <v>389000</v>
+        <v>1732319.752692774</v>
       </c>
       <c r="H24" t="n">
-        <v>19.34361014420686</v>
+        <v>46.51090945854524</v>
       </c>
       <c r="I24" t="inlineStr">
         <is>
@@ -1450,11 +1828,11 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>대신증권</t>
+          <t>노브</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>55</v>
+        <v>185</v>
       </c>
       <c r="D25" t="inlineStr">
         <is>
@@ -1465,13 +1843,13 @@
         <v>1</v>
       </c>
       <c r="F25" t="n">
-        <v>2238500</v>
+        <v>5041442.310511444</v>
       </c>
       <c r="G25" t="n">
-        <v>528999</v>
+        <v>1731434.310511444</v>
       </c>
       <c r="H25" t="n">
-        <v>30.94464408034859</v>
+        <v>52.30906724429197</v>
       </c>
       <c r="I25" t="inlineStr">
         <is>
@@ -1487,11 +1865,11 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>발레로 에너지</t>
+          <t>TIME 코리아밸류업액티브</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>6</v>
+        <v>201</v>
       </c>
       <c r="D26" t="inlineStr">
         <is>
@@ -1502,13 +1880,13 @@
         <v>1</v>
       </c>
       <c r="F26" t="n">
-        <v>2138731.14071836</v>
+        <v>4904400</v>
       </c>
       <c r="G26" t="n">
-        <v>74741.1407183595</v>
+        <v>180603</v>
       </c>
       <c r="H26" t="n">
-        <v>3.621196842928478</v>
+        <v>3.823259128197084</v>
       </c>
       <c r="I26" t="inlineStr">
         <is>
@@ -1524,11 +1902,11 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>미창석유</t>
+          <t>오케아니스 에코 탱커스</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>18</v>
+        <v>65</v>
       </c>
       <c r="D27" t="inlineStr">
         <is>
@@ -1539,13 +1917,13 @@
         <v>1</v>
       </c>
       <c r="F27" t="n">
-        <v>2032200</v>
+        <v>4575098.725873504</v>
       </c>
       <c r="G27" t="n">
-        <v>-360000</v>
+        <v>2318738.725873504</v>
       </c>
       <c r="H27" t="n">
-        <v>-15.04890895410083</v>
+        <v>102.7645732894354</v>
       </c>
       <c r="I27" t="inlineStr">
         <is>
@@ -1561,11 +1939,11 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>대창단조</t>
+          <t>삼성화재</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>300</v>
+        <v>9</v>
       </c>
       <c r="D28" t="inlineStr">
         <is>
@@ -1576,13 +1954,13 @@
         <v>1</v>
       </c>
       <c r="F28" t="n">
-        <v>1914000</v>
+        <v>4446000</v>
       </c>
       <c r="G28" t="n">
-        <v>-144000</v>
+        <v>-185000</v>
       </c>
       <c r="H28" t="n">
-        <v>-6.997084548104956</v>
+        <v>-3.994817534009933</v>
       </c>
       <c r="I28" t="inlineStr">
         <is>
@@ -1598,11 +1976,11 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>동방</t>
+          <t>DL이앤씨</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>681</v>
+        <v>80</v>
       </c>
       <c r="D29" t="inlineStr">
         <is>
@@ -1613,13 +1991,13 @@
         <v>1</v>
       </c>
       <c r="F29" t="n">
-        <v>1882965</v>
+        <v>4128000</v>
       </c>
       <c r="G29" t="n">
-        <v>-88536</v>
+        <v>717000</v>
       </c>
       <c r="H29" t="n">
-        <v>-4.490791533963209</v>
+        <v>21.02022867194371</v>
       </c>
       <c r="I29" t="inlineStr">
         <is>
@@ -1635,11 +2013,11 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>하나금융지주</t>
+          <t>차코스 에너지 내비게이션</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>15</v>
+        <v>75</v>
       </c>
       <c r="D30" t="inlineStr">
         <is>
@@ -1650,13 +2028,13 @@
         <v>1</v>
       </c>
       <c r="F30" t="n">
-        <v>1717500</v>
+        <v>4007418.271141662</v>
       </c>
       <c r="G30" t="n">
-        <v>35000</v>
+        <v>182770.2711416623</v>
       </c>
       <c r="H30" t="n">
-        <v>2.080237741456166</v>
+        <v>4.778747511971357</v>
       </c>
       <c r="I30" t="inlineStr">
         <is>
@@ -1672,11 +2050,11 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>스타 벌크 캐리어스</t>
+          <t>동원개발</t>
         </is>
       </c>
       <c r="C31" t="n">
-        <v>50</v>
+        <v>1360</v>
       </c>
       <c r="D31" t="inlineStr">
         <is>
@@ -1687,13 +2065,13 @@
         <v>1</v>
       </c>
       <c r="F31" t="n">
-        <v>1712476.648945617</v>
+        <v>3978000</v>
       </c>
       <c r="G31" t="n">
-        <v>398123.648945618</v>
+        <v>240600</v>
       </c>
       <c r="H31" t="n">
-        <v>30.29046602743845</v>
+        <v>6.437630438272596</v>
       </c>
       <c r="I31" t="inlineStr">
         <is>
@@ -1709,11 +2087,11 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>유나이티드헬스 그룹</t>
+          <t>HD건설기계</t>
         </is>
       </c>
       <c r="C32" t="n">
-        <v>4</v>
+        <v>31</v>
       </c>
       <c r="D32" t="inlineStr">
         <is>
@@ -1724,13 +2102,13 @@
         <v>1</v>
       </c>
       <c r="F32" t="n">
-        <v>1699490.128895313</v>
+        <v>3955600</v>
       </c>
       <c r="G32" t="n">
-        <v>5034.128895312548</v>
+        <v>-79496</v>
       </c>
       <c r="H32" t="n">
-        <v>0.297094105442251</v>
+        <v>-1.970114217852561</v>
       </c>
       <c r="I32" t="inlineStr">
         <is>
@@ -1746,11 +2124,11 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>케이씨</t>
+          <t>피바디 에너지</t>
         </is>
       </c>
       <c r="C33" t="n">
-        <v>50</v>
+        <v>65</v>
       </c>
       <c r="D33" t="inlineStr">
         <is>
@@ -1761,13 +2139,13 @@
         <v>1</v>
       </c>
       <c r="F33" t="n">
-        <v>1640000</v>
+        <v>3423839.074937592</v>
       </c>
       <c r="G33" t="n">
-        <v>-9500.000000000698</v>
+        <v>1953067.074937592</v>
       </c>
       <c r="H33" t="n">
-        <v>-0.5759321006365986</v>
+        <v>132.7919674115085</v>
       </c>
       <c r="I33" t="inlineStr">
         <is>
@@ -1783,11 +2161,11 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>삼성생명</t>
+          <t>더치 브로스</t>
         </is>
       </c>
       <c r="C34" t="n">
-        <v>4</v>
+        <v>39</v>
       </c>
       <c r="D34" t="inlineStr">
         <is>
@@ -1798,13 +2176,13 @@
         <v>1</v>
       </c>
       <c r="F34" t="n">
-        <v>940000</v>
+        <v>2965846.22503092</v>
       </c>
       <c r="G34" t="n">
-        <v>107000</v>
+        <v>-224797.7749690795</v>
       </c>
       <c r="H34" t="n">
-        <v>12.84513805522209</v>
+        <v>-7.04552983564069</v>
       </c>
       <c r="I34" t="inlineStr">
         <is>
@@ -1820,7 +2198,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>클리블랜드 클리프스</t>
+          <t>현대제철</t>
         </is>
       </c>
       <c r="C35" t="n">
@@ -1835,13 +2213,13 @@
         <v>1</v>
       </c>
       <c r="F35" t="n">
-        <v>857055.5630100402</v>
+        <v>2607500</v>
       </c>
       <c r="G35" t="n">
-        <v>-158999.4369899598</v>
+        <v>-200000</v>
       </c>
       <c r="H35" t="n">
-        <v>-15.64870376012714</v>
+        <v>-7.123775601068566</v>
       </c>
       <c r="I35" t="inlineStr">
         <is>
@@ -1857,11 +2235,11 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>비에이치아이</t>
+          <t>KoAct 코스닥액티브</t>
         </is>
       </c>
       <c r="C36" t="n">
-        <v>8</v>
+        <v>200</v>
       </c>
       <c r="D36" t="inlineStr">
         <is>
@@ -1872,13 +2250,13 @@
         <v>1</v>
       </c>
       <c r="F36" t="n">
-        <v>844800</v>
+        <v>2598000</v>
       </c>
       <c r="G36" t="n">
-        <v>179685</v>
+        <v>-104000</v>
       </c>
       <c r="H36" t="n">
-        <v>27.01562887620938</v>
+        <v>-3.84900074019245</v>
       </c>
       <c r="I36" t="inlineStr">
         <is>
@@ -1894,11 +2272,11 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>하프니아</t>
+          <t>휴스틸</t>
         </is>
       </c>
       <c r="C37" t="n">
-        <v>80</v>
+        <v>500</v>
       </c>
       <c r="D37" t="inlineStr">
         <is>
@@ -1909,13 +2287,13 @@
         <v>1</v>
       </c>
       <c r="F37" t="n">
-        <v>821489.5606615674</v>
+        <v>2560000</v>
       </c>
       <c r="G37" t="n">
-        <v>195758.5606615674</v>
+        <v>281390</v>
       </c>
       <c r="H37" t="n">
-        <v>31.28477902829928</v>
+        <v>12.34919534277476</v>
       </c>
       <c r="I37" t="inlineStr">
         <is>
@@ -1931,11 +2309,11 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>텍사스 퍼시픽 랜드</t>
+          <t>넥스틸</t>
         </is>
       </c>
       <c r="C38" t="n">
-        <v>1</v>
+        <v>200</v>
       </c>
       <c r="D38" t="inlineStr">
         <is>
@@ -1946,13 +2324,13 @@
         <v>1</v>
       </c>
       <c r="F38" t="n">
-        <v>794737.7576458007</v>
+        <v>2400000</v>
       </c>
       <c r="G38" t="n">
-        <v>16146.75764580071</v>
+        <v>389000</v>
       </c>
       <c r="H38" t="n">
-        <v>2.073843345967358</v>
+        <v>19.34361014420686</v>
       </c>
       <c r="I38" t="inlineStr">
         <is>
@@ -1968,30 +2346,548 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
+          <t>대신증권</t>
+        </is>
+      </c>
+      <c r="C39" t="n">
+        <v>55</v>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E39" t="n">
+        <v>1</v>
+      </c>
+      <c r="F39" t="n">
+        <v>2238500</v>
+      </c>
+      <c r="G39" t="n">
+        <v>528999</v>
+      </c>
+      <c r="H39" t="n">
+        <v>30.94464408034859</v>
+      </c>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>2026-03-18T14:32:42</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>2026-03-18</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>발레로 에너지</t>
+        </is>
+      </c>
+      <c r="C40" t="n">
+        <v>6</v>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E40" t="n">
+        <v>1</v>
+      </c>
+      <c r="F40" t="n">
+        <v>2138731.14071836</v>
+      </c>
+      <c r="G40" t="n">
+        <v>74741.1407183595</v>
+      </c>
+      <c r="H40" t="n">
+        <v>3.621196842928478</v>
+      </c>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>2026-03-18T14:32:42</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>2026-03-18</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>미창석유</t>
+        </is>
+      </c>
+      <c r="C41" t="n">
+        <v>18</v>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E41" t="n">
+        <v>1</v>
+      </c>
+      <c r="F41" t="n">
+        <v>2032200</v>
+      </c>
+      <c r="G41" t="n">
+        <v>-360000</v>
+      </c>
+      <c r="H41" t="n">
+        <v>-15.04890895410083</v>
+      </c>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>2026-03-18T14:32:42</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>2026-03-18</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>대창단조</t>
+        </is>
+      </c>
+      <c r="C42" t="n">
+        <v>300</v>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E42" t="n">
+        <v>1</v>
+      </c>
+      <c r="F42" t="n">
+        <v>1914000</v>
+      </c>
+      <c r="G42" t="n">
+        <v>-144000</v>
+      </c>
+      <c r="H42" t="n">
+        <v>-6.997084548104956</v>
+      </c>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>2026-03-18T14:32:42</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>2026-03-18</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>동방</t>
+        </is>
+      </c>
+      <c r="C43" t="n">
+        <v>681</v>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E43" t="n">
+        <v>1</v>
+      </c>
+      <c r="F43" t="n">
+        <v>1882965</v>
+      </c>
+      <c r="G43" t="n">
+        <v>-88536</v>
+      </c>
+      <c r="H43" t="n">
+        <v>-4.490791533963209</v>
+      </c>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>2026-03-18T14:32:42</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>2026-03-18</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>하나금융지주</t>
+        </is>
+      </c>
+      <c r="C44" t="n">
+        <v>15</v>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E44" t="n">
+        <v>1</v>
+      </c>
+      <c r="F44" t="n">
+        <v>1717500</v>
+      </c>
+      <c r="G44" t="n">
+        <v>35000</v>
+      </c>
+      <c r="H44" t="n">
+        <v>2.080237741456166</v>
+      </c>
+      <c r="I44" t="inlineStr">
+        <is>
+          <t>2026-03-18T14:32:42</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>2026-03-18</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>스타 벌크 캐리어스</t>
+        </is>
+      </c>
+      <c r="C45" t="n">
+        <v>50</v>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E45" t="n">
+        <v>1</v>
+      </c>
+      <c r="F45" t="n">
+        <v>1712476.648945617</v>
+      </c>
+      <c r="G45" t="n">
+        <v>398123.648945618</v>
+      </c>
+      <c r="H45" t="n">
+        <v>30.29046602743845</v>
+      </c>
+      <c r="I45" t="inlineStr">
+        <is>
+          <t>2026-03-18T14:32:42</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>2026-03-18</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>유나이티드헬스 그룹</t>
+        </is>
+      </c>
+      <c r="C46" t="n">
+        <v>4</v>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E46" t="n">
+        <v>1</v>
+      </c>
+      <c r="F46" t="n">
+        <v>1699490.128895313</v>
+      </c>
+      <c r="G46" t="n">
+        <v>5034.128895312548</v>
+      </c>
+      <c r="H46" t="n">
+        <v>0.297094105442251</v>
+      </c>
+      <c r="I46" t="inlineStr">
+        <is>
+          <t>2026-03-18T14:32:42</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>2026-03-18</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>케이씨</t>
+        </is>
+      </c>
+      <c r="C47" t="n">
+        <v>50</v>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E47" t="n">
+        <v>1</v>
+      </c>
+      <c r="F47" t="n">
+        <v>1640000</v>
+      </c>
+      <c r="G47" t="n">
+        <v>-9500.000000000698</v>
+      </c>
+      <c r="H47" t="n">
+        <v>-0.5759321006365986</v>
+      </c>
+      <c r="I47" t="inlineStr">
+        <is>
+          <t>2026-03-18T14:32:42</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>2026-03-18</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>삼성생명</t>
+        </is>
+      </c>
+      <c r="C48" t="n">
+        <v>4</v>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E48" t="n">
+        <v>1</v>
+      </c>
+      <c r="F48" t="n">
+        <v>940000</v>
+      </c>
+      <c r="G48" t="n">
+        <v>107000</v>
+      </c>
+      <c r="H48" t="n">
+        <v>12.84513805522209</v>
+      </c>
+      <c r="I48" t="inlineStr">
+        <is>
+          <t>2026-03-18T14:32:42</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>2026-03-18</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>클리블랜드 클리프스</t>
+        </is>
+      </c>
+      <c r="C49" t="n">
+        <v>70</v>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E49" t="n">
+        <v>1</v>
+      </c>
+      <c r="F49" t="n">
+        <v>857055.5630100402</v>
+      </c>
+      <c r="G49" t="n">
+        <v>-158999.4369899598</v>
+      </c>
+      <c r="H49" t="n">
+        <v>-15.64870376012714</v>
+      </c>
+      <c r="I49" t="inlineStr">
+        <is>
+          <t>2026-03-18T14:32:42</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>2026-03-18</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>비에이치아이</t>
+        </is>
+      </c>
+      <c r="C50" t="n">
+        <v>8</v>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E50" t="n">
+        <v>1</v>
+      </c>
+      <c r="F50" t="n">
+        <v>844800</v>
+      </c>
+      <c r="G50" t="n">
+        <v>179685</v>
+      </c>
+      <c r="H50" t="n">
+        <v>27.01562887620938</v>
+      </c>
+      <c r="I50" t="inlineStr">
+        <is>
+          <t>2026-03-18T14:32:42</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>2026-03-18</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>하프니아</t>
+        </is>
+      </c>
+      <c r="C51" t="n">
+        <v>80</v>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E51" t="n">
+        <v>1</v>
+      </c>
+      <c r="F51" t="n">
+        <v>821489.5606615674</v>
+      </c>
+      <c r="G51" t="n">
+        <v>195758.5606615674</v>
+      </c>
+      <c r="H51" t="n">
+        <v>31.28477902829928</v>
+      </c>
+      <c r="I51" t="inlineStr">
+        <is>
+          <t>2026-03-18T14:32:42</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>2026-03-18</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>텍사스 퍼시픽 랜드</t>
+        </is>
+      </c>
+      <c r="C52" t="n">
+        <v>1</v>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E52" t="n">
+        <v>1</v>
+      </c>
+      <c r="F52" t="n">
+        <v>794737.7576458007</v>
+      </c>
+      <c r="G52" t="n">
+        <v>16146.75764580071</v>
+      </c>
+      <c r="H52" t="n">
+        <v>2.073843345967358</v>
+      </c>
+      <c r="I52" t="inlineStr">
+        <is>
+          <t>2026-03-18T14:32:42</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>2026-03-18</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
           <t>노블</t>
         </is>
       </c>
-      <c r="C39" t="n">
+      <c r="C53" t="n">
         <v>99</v>
       </c>
-      <c r="D39" t="inlineStr">
-        <is>
-          <t>KRW</t>
-        </is>
-      </c>
-      <c r="E39" t="n">
-        <v>1</v>
-      </c>
-      <c r="F39" t="n">
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E53" t="n">
+        <v>1</v>
+      </c>
+      <c r="F53" t="n">
         <v>40689</v>
       </c>
-      <c r="G39" t="n">
+      <c r="G53" t="n">
         <v>-3866519</v>
       </c>
-      <c r="H39" t="n">
+      <c r="H53" t="n">
         <v>-98.95861699709869</v>
       </c>
-      <c r="I39" t="inlineStr">
+      <c r="I53" t="inlineStr">
         <is>
           <t>2026-03-18T14:32:42</t>
         </is>
@@ -2057,7 +2953,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>2026-03-18T21:07:31</t>
+          <t>2026-03-18T21:08:03</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: portfolio snapshot 2026-03-17 (2026-03-18T21:08:43)
</commit_message>
<xml_diff>
--- a/portfolio_auto.xlsx
+++ b/portfolio_auto.xlsx
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G15"/>
+  <dimension ref="A1:G29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -486,13 +486,13 @@
         <v>1</v>
       </c>
       <c r="E2" t="n">
-        <v>5067449</v>
+        <v>5041442.310511444</v>
       </c>
       <c r="F2" t="n">
-        <v>1757441</v>
+        <v>1731434.310511444</v>
       </c>
       <c r="G2" t="n">
-        <v>53.09</v>
+        <v>52.30906724429197</v>
       </c>
     </row>
     <row r="3">
@@ -513,13 +513,13 @@
         <v>1</v>
       </c>
       <c r="E3" t="n">
-        <v>6882090</v>
+        <v>40689</v>
       </c>
       <c r="F3" t="n">
-        <v>2974882</v>
+        <v>-3866519</v>
       </c>
       <c r="G3" t="n">
-        <v>76.13</v>
+        <v>-98.95861699709869</v>
       </c>
     </row>
     <row r="4">
@@ -540,13 +540,13 @@
         <v>1</v>
       </c>
       <c r="E4" t="n">
-        <v>2926290</v>
+        <v>2965846.22503092</v>
       </c>
       <c r="F4" t="n">
-        <v>-264354</v>
+        <v>-224797.7749690795</v>
       </c>
       <c r="G4" t="n">
-        <v>-8.279999999999999</v>
+        <v>-7.04552983564069</v>
       </c>
     </row>
     <row r="5">
@@ -567,13 +567,13 @@
         <v>1</v>
       </c>
       <c r="E5" t="n">
-        <v>2096946</v>
+        <v>2138731.14071836</v>
       </c>
       <c r="F5" t="n">
-        <v>32956</v>
+        <v>74741.1407183595</v>
       </c>
       <c r="G5" t="n">
-        <v>1.59</v>
+        <v>3.621196842928478</v>
       </c>
     </row>
     <row r="6">
@@ -594,13 +594,13 @@
         <v>1</v>
       </c>
       <c r="E6" t="n">
-        <v>6691594</v>
+        <v>6546958.253894605</v>
       </c>
       <c r="F6" t="n">
-        <v>460375</v>
+        <v>315739.2538946057</v>
       </c>
       <c r="G6" t="n">
-        <v>7.38</v>
+        <v>5.067054357977239</v>
       </c>
     </row>
     <row r="7">
@@ -621,13 +621,13 @@
         <v>1</v>
       </c>
       <c r="E7" t="n">
-        <v>1661361</v>
+        <v>1712476.648945617</v>
       </c>
       <c r="F7" t="n">
-        <v>347008</v>
+        <v>398123.6489456175</v>
       </c>
       <c r="G7" t="n">
-        <v>26.4</v>
+        <v>30.29046602743841</v>
       </c>
     </row>
     <row r="8">
@@ -648,13 +648,13 @@
         <v>1</v>
       </c>
       <c r="E8" t="n">
-        <v>7927448</v>
+        <v>8090014.733635107</v>
       </c>
       <c r="F8" t="n">
-        <v>1477097</v>
+        <v>1639663.733635107</v>
       </c>
       <c r="G8" t="n">
-        <v>22.89</v>
+        <v>25.41975984927188</v>
       </c>
     </row>
     <row r="9">
@@ -675,13 +675,13 @@
         <v>1</v>
       </c>
       <c r="E9" t="n">
-        <v>4451759</v>
+        <v>4575098.725873504</v>
       </c>
       <c r="F9" t="n">
-        <v>2195399</v>
+        <v>2318738.725873504</v>
       </c>
       <c r="G9" t="n">
-        <v>97.29000000000001</v>
+        <v>102.7645732894354</v>
       </c>
     </row>
     <row r="10">
@@ -702,13 +702,13 @@
         <v>1</v>
       </c>
       <c r="E10" t="n">
-        <v>1710490</v>
+        <v>1699490.128895313</v>
       </c>
       <c r="F10" t="n">
-        <v>16034</v>
+        <v>5034.128895312548</v>
       </c>
       <c r="G10" t="n">
-        <v>0.9399999999999999</v>
+        <v>0.297094105442251</v>
       </c>
     </row>
     <row r="11">
@@ -729,13 +729,13 @@
         <v>1</v>
       </c>
       <c r="E11" t="n">
-        <v>3919272</v>
+        <v>4007418.271141662</v>
       </c>
       <c r="F11" t="n">
-        <v>94624</v>
+        <v>182770.2711416623</v>
       </c>
       <c r="G11" t="n">
-        <v>2.47</v>
+        <v>4.778747511971357</v>
       </c>
     </row>
     <row r="12">
@@ -756,13 +756,13 @@
         <v>1</v>
       </c>
       <c r="E12" t="n">
-        <v>908091</v>
+        <v>857055.5630100402</v>
       </c>
       <c r="F12" t="n">
-        <v>-107964</v>
+        <v>-158999.4369899598</v>
       </c>
       <c r="G12" t="n">
-        <v>-10.62</v>
+        <v>-15.64870376012714</v>
       </c>
     </row>
     <row r="13">
@@ -783,13 +783,13 @@
         <v>1</v>
       </c>
       <c r="E13" t="n">
-        <v>5429641</v>
+        <v>5456864.752692774</v>
       </c>
       <c r="F13" t="n">
-        <v>1705096</v>
+        <v>1732319.752692774</v>
       </c>
       <c r="G13" t="n">
-        <v>45.78</v>
+        <v>46.51090945854524</v>
       </c>
     </row>
     <row r="14">
@@ -810,13 +810,13 @@
         <v>1</v>
       </c>
       <c r="E14" t="n">
-        <v>786665</v>
+        <v>794737.7576458007</v>
       </c>
       <c r="F14" t="n">
-        <v>8074</v>
+        <v>16146.75764580071</v>
       </c>
       <c r="G14" t="n">
-        <v>1.03</v>
+        <v>2.073843345967358</v>
       </c>
     </row>
     <row r="15">
@@ -837,13 +837,391 @@
         <v>1</v>
       </c>
       <c r="E15" t="n">
-        <v>6945333</v>
+        <v>7093219.418241119</v>
       </c>
       <c r="F15" t="n">
-        <v>2818099</v>
+        <v>2965985.418241119</v>
       </c>
       <c r="G15" t="n">
-        <v>68.28</v>
+        <v>71.86375713713153</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>페트로브라스 (ADR)</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>480</v>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>1</v>
+      </c>
+      <c r="E16" t="n">
+        <v>13847377</v>
+      </c>
+      <c r="F16" t="n">
+        <v>1740828</v>
+      </c>
+      <c r="G16" t="n">
+        <v>14.37</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>프론트라인</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>175</v>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>1</v>
+      </c>
+      <c r="E17" t="n">
+        <v>8304682</v>
+      </c>
+      <c r="F17" t="n">
+        <v>3874818</v>
+      </c>
+      <c r="G17" t="n">
+        <v>87.47</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>피바디 에너지</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>65</v>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>1</v>
+      </c>
+      <c r="E18" t="n">
+        <v>3427688</v>
+      </c>
+      <c r="F18" t="n">
+        <v>1956916</v>
+      </c>
+      <c r="G18" t="n">
+        <v>133.05</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>하프니아</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>80</v>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
+        <v>1</v>
+      </c>
+      <c r="E19" t="n">
+        <v>798051</v>
+      </c>
+      <c r="F19" t="n">
+        <v>172320</v>
+      </c>
+      <c r="G19" t="n">
+        <v>27.53</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>AGNC 인베스트먼트</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>700</v>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="D20" t="n">
+        <v>1</v>
+      </c>
+      <c r="E20" t="n">
+        <v>10848269</v>
+      </c>
+      <c r="F20" t="n">
+        <v>16254</v>
+      </c>
+      <c r="G20" t="n">
+        <v>0.15</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>넥스틸</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>200</v>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
+        <v>1</v>
+      </c>
+      <c r="E21" t="n">
+        <v>2391208</v>
+      </c>
+      <c r="F21" t="n">
+        <v>380208</v>
+      </c>
+      <c r="G21" t="n">
+        <v>18.9</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>대신증권</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>55</v>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="D22" t="n">
+        <v>1</v>
+      </c>
+      <c r="E22" t="n">
+        <v>2190111</v>
+      </c>
+      <c r="F22" t="n">
+        <v>480610</v>
+      </c>
+      <c r="G22" t="n">
+        <v>28.11</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>대창단조</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>300</v>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="D23" t="n">
+        <v>1</v>
+      </c>
+      <c r="E23" t="n">
+        <v>1901190</v>
+      </c>
+      <c r="F23" t="n">
+        <v>-156810</v>
+      </c>
+      <c r="G23" t="n">
+        <v>-7.61</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>대한조선</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>100</v>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="D24" t="n">
+        <v>1</v>
+      </c>
+      <c r="E24" t="n">
+        <v>9740480</v>
+      </c>
+      <c r="F24" t="n">
+        <v>2527480</v>
+      </c>
+      <c r="G24" t="n">
+        <v>35.04</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>동방</t>
+        </is>
+      </c>
+      <c r="B25" t="n">
+        <v>681</v>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="D25" t="n">
+        <v>1</v>
+      </c>
+      <c r="E25" t="n">
+        <v>1841600</v>
+      </c>
+      <c r="F25" t="n">
+        <v>-129901</v>
+      </c>
+      <c r="G25" t="n">
+        <v>-6.58</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>동원개발</t>
+        </is>
+      </c>
+      <c r="B26" t="n">
+        <v>1360</v>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="D26" t="n">
+        <v>1</v>
+      </c>
+      <c r="E26" t="n">
+        <v>3881821</v>
+      </c>
+      <c r="F26" t="n">
+        <v>144421</v>
+      </c>
+      <c r="G26" t="n">
+        <v>3.86</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>미창석유</t>
+        </is>
+      </c>
+      <c r="B27" t="n">
+        <v>18</v>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="D27" t="n">
+        <v>1</v>
+      </c>
+      <c r="E27" t="n">
+        <v>2049693</v>
+      </c>
+      <c r="F27" t="n">
+        <v>-342507</v>
+      </c>
+      <c r="G27" t="n">
+        <v>-14.31</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>비에이치아이</t>
+        </is>
+      </c>
+      <c r="B28" t="n">
+        <v>8</v>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="D28" t="n">
+        <v>1</v>
+      </c>
+      <c r="E28" t="n">
+        <v>850296</v>
+      </c>
+      <c r="F28" t="n">
+        <v>185181</v>
+      </c>
+      <c r="G28" t="n">
+        <v>27.84</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>삼성생명</t>
+        </is>
+      </c>
+      <c r="B29" t="n">
+        <v>4</v>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="D29" t="n">
+        <v>1</v>
+      </c>
+      <c r="E29" t="n">
+        <v>872252</v>
+      </c>
+      <c r="F29" t="n">
+        <v>39252</v>
+      </c>
+      <c r="G29" t="n">
+        <v>4.71</v>
       </c>
     </row>
   </sheetData>
@@ -901,7 +1279,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2026-03-18T21:08:03</t>
+          <t>2026-03-18T21:08:43</t>
         </is>
       </c>
       <c r="E2" t="n">
@@ -919,7 +1297,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I53"/>
+  <dimension ref="A1:I67"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -977,11 +1355,11 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>시드릴</t>
+          <t>페트로브라스 (ADR)</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>123</v>
+        <v>480</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
@@ -992,17 +1370,17 @@
         <v>1</v>
       </c>
       <c r="F2" t="n">
-        <v>7927448</v>
+        <v>13847377</v>
       </c>
       <c r="G2" t="n">
-        <v>1477097</v>
+        <v>1740828</v>
       </c>
       <c r="H2" t="n">
-        <v>22.89</v>
+        <v>14.37</v>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>2026-03-18T21:08:03</t>
+          <t>2026-03-18T21:08:43</t>
         </is>
       </c>
     </row>
@@ -1014,11 +1392,11 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>트랜스오션</t>
+          <t>AGNC 인베스트먼트</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>750</v>
+        <v>700</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
@@ -1029,17 +1407,17 @@
         <v>1</v>
       </c>
       <c r="F3" t="n">
-        <v>6945333</v>
+        <v>10848269</v>
       </c>
       <c r="G3" t="n">
-        <v>2818099</v>
+        <v>16254</v>
       </c>
       <c r="H3" t="n">
-        <v>68.28</v>
+        <v>0.15</v>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>2026-03-18T21:08:03</t>
+          <t>2026-03-18T21:08:43</t>
         </is>
       </c>
     </row>
@@ -1051,11 +1429,11 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>노블</t>
+          <t>대한조선</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
@@ -1066,17 +1444,17 @@
         <v>1</v>
       </c>
       <c r="F4" t="n">
-        <v>6882090</v>
+        <v>9740480</v>
       </c>
       <c r="G4" t="n">
-        <v>2974882</v>
+        <v>2527480</v>
       </c>
       <c r="H4" t="n">
-        <v>76.13</v>
+        <v>35.04</v>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>2026-03-18T21:08:03</t>
+          <t>2026-03-18T21:08:43</t>
         </is>
       </c>
     </row>
@@ -1088,11 +1466,11 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>센트러스 에너지</t>
+          <t>프론트라인</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>21</v>
+        <v>175</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
@@ -1103,17 +1481,17 @@
         <v>1</v>
       </c>
       <c r="F5" t="n">
-        <v>6691594</v>
+        <v>8304682</v>
       </c>
       <c r="G5" t="n">
-        <v>460375</v>
+        <v>3874818</v>
       </c>
       <c r="H5" t="n">
-        <v>7.38</v>
+        <v>87.47</v>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>2026-03-18T21:08:03</t>
+          <t>2026-03-18T21:08:43</t>
         </is>
       </c>
     </row>
@@ -1125,11 +1503,11 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>타이드워터</t>
+          <t>시드릴</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>48</v>
+        <v>123</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
@@ -1140,17 +1518,17 @@
         <v>1</v>
       </c>
       <c r="F6" t="n">
-        <v>5429641</v>
+        <v>8090014.733635107</v>
       </c>
       <c r="G6" t="n">
-        <v>1705096</v>
+        <v>1639663.733635107</v>
       </c>
       <c r="H6" t="n">
-        <v>45.78</v>
+        <v>25.41975984927188</v>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>2026-03-18T21:08:03</t>
+          <t>2026-03-18T21:08:43</t>
         </is>
       </c>
     </row>
@@ -1162,11 +1540,11 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>노브</t>
+          <t>트랜스오션</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>185</v>
+        <v>750</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
@@ -1177,17 +1555,17 @@
         <v>1</v>
       </c>
       <c r="F7" t="n">
-        <v>5067449</v>
+        <v>7093219.418241119</v>
       </c>
       <c r="G7" t="n">
-        <v>1757441</v>
+        <v>2965985.418241119</v>
       </c>
       <c r="H7" t="n">
-        <v>53.09</v>
+        <v>71.86375713713153</v>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>2026-03-18T21:08:03</t>
+          <t>2026-03-18T21:08:43</t>
         </is>
       </c>
     </row>
@@ -1199,11 +1577,11 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>오케아니스 에코 탱커스</t>
+          <t>센트러스 에너지</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>65</v>
+        <v>21</v>
       </c>
       <c r="D8" t="inlineStr">
         <is>
@@ -1214,17 +1592,17 @@
         <v>1</v>
       </c>
       <c r="F8" t="n">
-        <v>4451759</v>
+        <v>6546958.253894605</v>
       </c>
       <c r="G8" t="n">
-        <v>2195399</v>
+        <v>315739.2538946057</v>
       </c>
       <c r="H8" t="n">
-        <v>97.29000000000001</v>
+        <v>5.067054357977239</v>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>2026-03-18T21:08:03</t>
+          <t>2026-03-18T21:08:43</t>
         </is>
       </c>
     </row>
@@ -1236,11 +1614,11 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>차코스 에너지 내비게이션</t>
+          <t>타이드워터</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>75</v>
+        <v>48</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
@@ -1251,17 +1629,17 @@
         <v>1</v>
       </c>
       <c r="F9" t="n">
-        <v>3919272</v>
+        <v>5456864.752692774</v>
       </c>
       <c r="G9" t="n">
-        <v>94624</v>
+        <v>1732319.752692774</v>
       </c>
       <c r="H9" t="n">
-        <v>2.47</v>
+        <v>46.51090945854524</v>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>2026-03-18T21:08:03</t>
+          <t>2026-03-18T21:08:43</t>
         </is>
       </c>
     </row>
@@ -1273,11 +1651,11 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>더치 브로스</t>
+          <t>노브</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>39</v>
+        <v>185</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
@@ -1288,17 +1666,17 @@
         <v>1</v>
       </c>
       <c r="F10" t="n">
-        <v>2926290</v>
+        <v>5041442.310511444</v>
       </c>
       <c r="G10" t="n">
-        <v>-264354</v>
+        <v>1731434.310511444</v>
       </c>
       <c r="H10" t="n">
-        <v>-8.279999999999999</v>
+        <v>52.30906724429197</v>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>2026-03-18T21:08:03</t>
+          <t>2026-03-18T21:08:43</t>
         </is>
       </c>
     </row>
@@ -1310,11 +1688,11 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>발레로 에너지</t>
+          <t>오케아니스 에코 탱커스</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>6</v>
+        <v>65</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
@@ -1325,17 +1703,17 @@
         <v>1</v>
       </c>
       <c r="F11" t="n">
-        <v>2096946</v>
+        <v>4575098.725873504</v>
       </c>
       <c r="G11" t="n">
-        <v>32956</v>
+        <v>2318738.725873504</v>
       </c>
       <c r="H11" t="n">
-        <v>1.59</v>
+        <v>102.7645732894354</v>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>2026-03-18T21:08:03</t>
+          <t>2026-03-18T21:08:43</t>
         </is>
       </c>
     </row>
@@ -1347,11 +1725,11 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>유나이티드헬스 그룹</t>
+          <t>차코스 에너지 내비게이션</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>4</v>
+        <v>75</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
@@ -1362,17 +1740,17 @@
         <v>1</v>
       </c>
       <c r="F12" t="n">
-        <v>1710490</v>
+        <v>4007418.271141662</v>
       </c>
       <c r="G12" t="n">
-        <v>16034</v>
+        <v>182770.2711416623</v>
       </c>
       <c r="H12" t="n">
-        <v>0.9399999999999999</v>
+        <v>4.778747511971357</v>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>2026-03-18T21:08:03</t>
+          <t>2026-03-18T21:08:43</t>
         </is>
       </c>
     </row>
@@ -1384,11 +1762,11 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>스타 벌크 캐리어스</t>
+          <t>동원개발</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>50</v>
+        <v>1360</v>
       </c>
       <c r="D13" t="inlineStr">
         <is>
@@ -1399,17 +1777,17 @@
         <v>1</v>
       </c>
       <c r="F13" t="n">
-        <v>1661361</v>
+        <v>3881821</v>
       </c>
       <c r="G13" t="n">
-        <v>347008</v>
+        <v>144421</v>
       </c>
       <c r="H13" t="n">
-        <v>26.4</v>
+        <v>3.86</v>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>2026-03-18T21:08:03</t>
+          <t>2026-03-18T21:08:43</t>
         </is>
       </c>
     </row>
@@ -1421,11 +1799,11 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>클리블랜드 클리프스</t>
+          <t>피바디 에너지</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>70</v>
+        <v>65</v>
       </c>
       <c r="D14" t="inlineStr">
         <is>
@@ -1436,17 +1814,17 @@
         <v>1</v>
       </c>
       <c r="F14" t="n">
-        <v>908091</v>
+        <v>3427688</v>
       </c>
       <c r="G14" t="n">
-        <v>-107964</v>
+        <v>1956916</v>
       </c>
       <c r="H14" t="n">
-        <v>-10.62</v>
+        <v>133.05</v>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>2026-03-18T21:08:03</t>
+          <t>2026-03-18T21:08:43</t>
         </is>
       </c>
     </row>
@@ -1458,11 +1836,11 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>텍사스 퍼시픽 랜드</t>
+          <t>더치 브로스</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>1</v>
+        <v>39</v>
       </c>
       <c r="D15" t="inlineStr">
         <is>
@@ -1473,33 +1851,33 @@
         <v>1</v>
       </c>
       <c r="F15" t="n">
-        <v>786665</v>
+        <v>2965846.22503092</v>
       </c>
       <c r="G15" t="n">
-        <v>8074</v>
+        <v>-224797.7749690795</v>
       </c>
       <c r="H15" t="n">
-        <v>1.03</v>
+        <v>-7.04552983564069</v>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>2026-03-18T21:08:03</t>
+          <t>2026-03-18T21:08:43</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-03-18</t>
+          <t>2026-03-17</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>페트로브라스 (ADR)</t>
+          <t>넥스틸</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>480</v>
+        <v>200</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
@@ -1510,33 +1888,33 @@
         <v>1</v>
       </c>
       <c r="F16" t="n">
-        <v>14082576.9328374</v>
+        <v>2391208</v>
       </c>
       <c r="G16" t="n">
-        <v>1976027.932837404</v>
+        <v>380208</v>
       </c>
       <c r="H16" t="n">
-        <v>16.3219752617976</v>
+        <v>18.9</v>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>2026-03-18T14:32:42</t>
+          <t>2026-03-18T21:08:43</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-03-18</t>
+          <t>2026-03-17</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>AGNC 인베스트먼트</t>
+          <t>대신증권</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>700</v>
+        <v>55</v>
       </c>
       <c r="D17" t="inlineStr">
         <is>
@@ -1547,33 +1925,33 @@
         <v>1</v>
       </c>
       <c r="F17" t="n">
-        <v>10822406.73782303</v>
+        <v>2190111</v>
       </c>
       <c r="G17" t="n">
-        <v>-9608.262176971883</v>
+        <v>480610</v>
       </c>
       <c r="H17" t="n">
-        <v>-0.08870244526961865</v>
+        <v>28.11</v>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>2026-03-18T14:32:42</t>
+          <t>2026-03-18T21:08:43</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-03-18</t>
+          <t>2026-03-17</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>대한조선</t>
+          <t>발레로 에너지</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>100</v>
+        <v>6</v>
       </c>
       <c r="D18" t="inlineStr">
         <is>
@@ -1584,33 +1962,33 @@
         <v>1</v>
       </c>
       <c r="F18" t="n">
-        <v>9570000</v>
+        <v>2138731.14071836</v>
       </c>
       <c r="G18" t="n">
-        <v>2357000</v>
+        <v>74741.1407183595</v>
       </c>
       <c r="H18" t="n">
-        <v>32.67711077221684</v>
+        <v>3.621196842928478</v>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>2026-03-18T14:32:42</t>
+          <t>2026-03-18T21:08:43</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-03-18</t>
+          <t>2026-03-17</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>프론트라인</t>
+          <t>미창석유</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>175</v>
+        <v>18</v>
       </c>
       <c r="D19" t="inlineStr">
         <is>
@@ -1621,33 +1999,33 @@
         <v>1</v>
       </c>
       <c r="F19" t="n">
-        <v>8440541.129673157</v>
+        <v>2049693</v>
       </c>
       <c r="G19" t="n">
-        <v>4010677.129673157</v>
+        <v>-342507</v>
       </c>
       <c r="H19" t="n">
-        <v>90.53725192631549</v>
+        <v>-14.31</v>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>2026-03-18T14:32:42</t>
+          <t>2026-03-18T21:08:43</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-03-18</t>
+          <t>2026-03-17</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>시드릴</t>
+          <t>대창단조</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>123</v>
+        <v>300</v>
       </c>
       <c r="D20" t="inlineStr">
         <is>
@@ -1658,33 +2036,33 @@
         <v>1</v>
       </c>
       <c r="F20" t="n">
-        <v>8090014.733635107</v>
+        <v>1901190</v>
       </c>
       <c r="G20" t="n">
-        <v>1639663.733635107</v>
+        <v>-156810</v>
       </c>
       <c r="H20" t="n">
-        <v>25.41975984927188</v>
+        <v>-7.61</v>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>2026-03-18T14:32:42</t>
+          <t>2026-03-18T21:08:43</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-03-18</t>
+          <t>2026-03-17</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>트랜스오션</t>
+          <t>동방</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>750</v>
+        <v>681</v>
       </c>
       <c r="D21" t="inlineStr">
         <is>
@@ -1695,29 +2073,29 @@
         <v>1</v>
       </c>
       <c r="F21" t="n">
-        <v>7093219.418241119</v>
+        <v>1841600</v>
       </c>
       <c r="G21" t="n">
-        <v>2965985.418241119</v>
+        <v>-129901</v>
       </c>
       <c r="H21" t="n">
-        <v>71.86375713713153</v>
+        <v>-6.58</v>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>2026-03-18T14:32:42</t>
+          <t>2026-03-18T21:08:43</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2026-03-18</t>
+          <t>2026-03-17</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>세아제강</t>
+          <t>스타 벌크 캐리어스</t>
         </is>
       </c>
       <c r="C22" t="n">
@@ -1732,33 +2110,33 @@
         <v>1</v>
       </c>
       <c r="F22" t="n">
-        <v>6915000</v>
+        <v>1712476.648945617</v>
       </c>
       <c r="G22" t="n">
-        <v>605000</v>
+        <v>398123.6489456175</v>
       </c>
       <c r="H22" t="n">
-        <v>9.587955625990491</v>
+        <v>30.29046602743841</v>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>2026-03-18T14:32:42</t>
+          <t>2026-03-18T21:08:43</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-03-18</t>
+          <t>2026-03-17</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>센트러스 에너지</t>
+          <t>유나이티드헬스 그룹</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>21</v>
+        <v>4</v>
       </c>
       <c r="D23" t="inlineStr">
         <is>
@@ -1769,33 +2147,33 @@
         <v>1</v>
       </c>
       <c r="F23" t="n">
-        <v>6546958.253894605</v>
+        <v>1699490.128895313</v>
       </c>
       <c r="G23" t="n">
-        <v>315739.2538946057</v>
+        <v>5034.128895312548</v>
       </c>
       <c r="H23" t="n">
-        <v>5.067054357977239</v>
+        <v>0.297094105442251</v>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>2026-03-18T14:32:42</t>
+          <t>2026-03-18T21:08:43</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>2026-03-18</t>
+          <t>2026-03-17</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>타이드워터</t>
+          <t>삼성생명</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>48</v>
+        <v>4</v>
       </c>
       <c r="D24" t="inlineStr">
         <is>
@@ -1806,33 +2184,33 @@
         <v>1</v>
       </c>
       <c r="F24" t="n">
-        <v>5456864.752692774</v>
+        <v>872252</v>
       </c>
       <c r="G24" t="n">
-        <v>1732319.752692774</v>
+        <v>39252</v>
       </c>
       <c r="H24" t="n">
-        <v>46.51090945854524</v>
+        <v>4.71</v>
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>2026-03-18T14:32:42</t>
+          <t>2026-03-18T21:08:43</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-03-18</t>
+          <t>2026-03-17</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>노브</t>
+          <t>클리블랜드 클리프스</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>185</v>
+        <v>70</v>
       </c>
       <c r="D25" t="inlineStr">
         <is>
@@ -1843,33 +2221,33 @@
         <v>1</v>
       </c>
       <c r="F25" t="n">
-        <v>5041442.310511444</v>
+        <v>857055.5630100402</v>
       </c>
       <c r="G25" t="n">
-        <v>1731434.310511444</v>
+        <v>-158999.4369899598</v>
       </c>
       <c r="H25" t="n">
-        <v>52.30906724429197</v>
+        <v>-15.64870376012714</v>
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>2026-03-18T14:32:42</t>
+          <t>2026-03-18T21:08:43</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>2026-03-18</t>
+          <t>2026-03-17</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>TIME 코리아밸류업액티브</t>
+          <t>비에이치아이</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>201</v>
+        <v>8</v>
       </c>
       <c r="D26" t="inlineStr">
         <is>
@@ -1880,33 +2258,33 @@
         <v>1</v>
       </c>
       <c r="F26" t="n">
-        <v>4904400</v>
+        <v>850296</v>
       </c>
       <c r="G26" t="n">
-        <v>180603</v>
+        <v>185181</v>
       </c>
       <c r="H26" t="n">
-        <v>3.823259128197084</v>
+        <v>27.84</v>
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>2026-03-18T14:32:42</t>
+          <t>2026-03-18T21:08:43</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-03-18</t>
+          <t>2026-03-17</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>오케아니스 에코 탱커스</t>
+          <t>하프니아</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>65</v>
+        <v>80</v>
       </c>
       <c r="D27" t="inlineStr">
         <is>
@@ -1917,33 +2295,33 @@
         <v>1</v>
       </c>
       <c r="F27" t="n">
-        <v>4575098.725873504</v>
+        <v>798051</v>
       </c>
       <c r="G27" t="n">
-        <v>2318738.725873504</v>
+        <v>172320</v>
       </c>
       <c r="H27" t="n">
-        <v>102.7645732894354</v>
+        <v>27.53</v>
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>2026-03-18T14:32:42</t>
+          <t>2026-03-18T21:08:43</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>2026-03-18</t>
+          <t>2026-03-17</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>삼성화재</t>
+          <t>텍사스 퍼시픽 랜드</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="D28" t="inlineStr">
         <is>
@@ -1954,33 +2332,33 @@
         <v>1</v>
       </c>
       <c r="F28" t="n">
-        <v>4446000</v>
+        <v>794737.7576458007</v>
       </c>
       <c r="G28" t="n">
-        <v>-185000</v>
+        <v>16146.75764580071</v>
       </c>
       <c r="H28" t="n">
-        <v>-3.994817534009933</v>
+        <v>2.073843345967358</v>
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>2026-03-18T14:32:42</t>
+          <t>2026-03-18T21:08:43</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-03-18</t>
+          <t>2026-03-17</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>DL이앤씨</t>
+          <t>노블</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>80</v>
+        <v>99</v>
       </c>
       <c r="D29" t="inlineStr">
         <is>
@@ -1991,17 +2369,17 @@
         <v>1</v>
       </c>
       <c r="F29" t="n">
-        <v>4128000</v>
+        <v>40689</v>
       </c>
       <c r="G29" t="n">
-        <v>717000</v>
+        <v>-3866519</v>
       </c>
       <c r="H29" t="n">
-        <v>21.02022867194371</v>
+        <v>-98.95861699709869</v>
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>2026-03-18T14:32:42</t>
+          <t>2026-03-18T21:08:43</t>
         </is>
       </c>
     </row>
@@ -2013,11 +2391,11 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>차코스 에너지 내비게이션</t>
+          <t>페트로브라스 (ADR)</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>75</v>
+        <v>480</v>
       </c>
       <c r="D30" t="inlineStr">
         <is>
@@ -2028,13 +2406,13 @@
         <v>1</v>
       </c>
       <c r="F30" t="n">
-        <v>4007418.271141662</v>
+        <v>14082576.9328374</v>
       </c>
       <c r="G30" t="n">
-        <v>182770.2711416623</v>
+        <v>1976027.932837404</v>
       </c>
       <c r="H30" t="n">
-        <v>4.778747511971357</v>
+        <v>16.3219752617976</v>
       </c>
       <c r="I30" t="inlineStr">
         <is>
@@ -2050,11 +2428,11 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>동원개발</t>
+          <t>AGNC 인베스트먼트</t>
         </is>
       </c>
       <c r="C31" t="n">
-        <v>1360</v>
+        <v>700</v>
       </c>
       <c r="D31" t="inlineStr">
         <is>
@@ -2065,13 +2443,13 @@
         <v>1</v>
       </c>
       <c r="F31" t="n">
-        <v>3978000</v>
+        <v>10822406.73782303</v>
       </c>
       <c r="G31" t="n">
-        <v>240600</v>
+        <v>-9608.262176971883</v>
       </c>
       <c r="H31" t="n">
-        <v>6.437630438272596</v>
+        <v>-0.08870244526961865</v>
       </c>
       <c r="I31" t="inlineStr">
         <is>
@@ -2087,11 +2465,11 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>HD건설기계</t>
+          <t>대한조선</t>
         </is>
       </c>
       <c r="C32" t="n">
-        <v>31</v>
+        <v>100</v>
       </c>
       <c r="D32" t="inlineStr">
         <is>
@@ -2102,13 +2480,13 @@
         <v>1</v>
       </c>
       <c r="F32" t="n">
-        <v>3955600</v>
+        <v>9570000</v>
       </c>
       <c r="G32" t="n">
-        <v>-79496</v>
+        <v>2357000</v>
       </c>
       <c r="H32" t="n">
-        <v>-1.970114217852561</v>
+        <v>32.67711077221684</v>
       </c>
       <c r="I32" t="inlineStr">
         <is>
@@ -2124,11 +2502,11 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>피바디 에너지</t>
+          <t>프론트라인</t>
         </is>
       </c>
       <c r="C33" t="n">
-        <v>65</v>
+        <v>175</v>
       </c>
       <c r="D33" t="inlineStr">
         <is>
@@ -2139,13 +2517,13 @@
         <v>1</v>
       </c>
       <c r="F33" t="n">
-        <v>3423839.074937592</v>
+        <v>8440541.129673157</v>
       </c>
       <c r="G33" t="n">
-        <v>1953067.074937592</v>
+        <v>4010677.129673157</v>
       </c>
       <c r="H33" t="n">
-        <v>132.7919674115085</v>
+        <v>90.53725192631549</v>
       </c>
       <c r="I33" t="inlineStr">
         <is>
@@ -2161,11 +2539,11 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>더치 브로스</t>
+          <t>시드릴</t>
         </is>
       </c>
       <c r="C34" t="n">
-        <v>39</v>
+        <v>123</v>
       </c>
       <c r="D34" t="inlineStr">
         <is>
@@ -2176,13 +2554,13 @@
         <v>1</v>
       </c>
       <c r="F34" t="n">
-        <v>2965846.22503092</v>
+        <v>8090014.733635107</v>
       </c>
       <c r="G34" t="n">
-        <v>-224797.7749690795</v>
+        <v>1639663.733635107</v>
       </c>
       <c r="H34" t="n">
-        <v>-7.04552983564069</v>
+        <v>25.41975984927188</v>
       </c>
       <c r="I34" t="inlineStr">
         <is>
@@ -2198,11 +2576,11 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>현대제철</t>
+          <t>트랜스오션</t>
         </is>
       </c>
       <c r="C35" t="n">
-        <v>70</v>
+        <v>750</v>
       </c>
       <c r="D35" t="inlineStr">
         <is>
@@ -2213,13 +2591,13 @@
         <v>1</v>
       </c>
       <c r="F35" t="n">
-        <v>2607500</v>
+        <v>7093219.418241119</v>
       </c>
       <c r="G35" t="n">
-        <v>-200000</v>
+        <v>2965985.418241119</v>
       </c>
       <c r="H35" t="n">
-        <v>-7.123775601068566</v>
+        <v>71.86375713713153</v>
       </c>
       <c r="I35" t="inlineStr">
         <is>
@@ -2235,11 +2613,11 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>KoAct 코스닥액티브</t>
+          <t>세아제강</t>
         </is>
       </c>
       <c r="C36" t="n">
-        <v>200</v>
+        <v>50</v>
       </c>
       <c r="D36" t="inlineStr">
         <is>
@@ -2250,13 +2628,13 @@
         <v>1</v>
       </c>
       <c r="F36" t="n">
-        <v>2598000</v>
+        <v>6915000</v>
       </c>
       <c r="G36" t="n">
-        <v>-104000</v>
+        <v>605000</v>
       </c>
       <c r="H36" t="n">
-        <v>-3.84900074019245</v>
+        <v>9.587955625990491</v>
       </c>
       <c r="I36" t="inlineStr">
         <is>
@@ -2272,11 +2650,11 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>휴스틸</t>
+          <t>센트러스 에너지</t>
         </is>
       </c>
       <c r="C37" t="n">
-        <v>500</v>
+        <v>21</v>
       </c>
       <c r="D37" t="inlineStr">
         <is>
@@ -2287,13 +2665,13 @@
         <v>1</v>
       </c>
       <c r="F37" t="n">
-        <v>2560000</v>
+        <v>6546958.253894605</v>
       </c>
       <c r="G37" t="n">
-        <v>281390</v>
+        <v>315739.2538946057</v>
       </c>
       <c r="H37" t="n">
-        <v>12.34919534277476</v>
+        <v>5.067054357977239</v>
       </c>
       <c r="I37" t="inlineStr">
         <is>
@@ -2309,11 +2687,11 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>넥스틸</t>
+          <t>타이드워터</t>
         </is>
       </c>
       <c r="C38" t="n">
-        <v>200</v>
+        <v>48</v>
       </c>
       <c r="D38" t="inlineStr">
         <is>
@@ -2324,13 +2702,13 @@
         <v>1</v>
       </c>
       <c r="F38" t="n">
-        <v>2400000</v>
+        <v>5456864.752692774</v>
       </c>
       <c r="G38" t="n">
-        <v>389000</v>
+        <v>1732319.752692774</v>
       </c>
       <c r="H38" t="n">
-        <v>19.34361014420686</v>
+        <v>46.51090945854524</v>
       </c>
       <c r="I38" t="inlineStr">
         <is>
@@ -2346,11 +2724,11 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>대신증권</t>
+          <t>노브</t>
         </is>
       </c>
       <c r="C39" t="n">
-        <v>55</v>
+        <v>185</v>
       </c>
       <c r="D39" t="inlineStr">
         <is>
@@ -2361,13 +2739,13 @@
         <v>1</v>
       </c>
       <c r="F39" t="n">
-        <v>2238500</v>
+        <v>5041442.310511444</v>
       </c>
       <c r="G39" t="n">
-        <v>528999</v>
+        <v>1731434.310511444</v>
       </c>
       <c r="H39" t="n">
-        <v>30.94464408034859</v>
+        <v>52.30906724429197</v>
       </c>
       <c r="I39" t="inlineStr">
         <is>
@@ -2383,11 +2761,11 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>발레로 에너지</t>
+          <t>TIME 코리아밸류업액티브</t>
         </is>
       </c>
       <c r="C40" t="n">
-        <v>6</v>
+        <v>201</v>
       </c>
       <c r="D40" t="inlineStr">
         <is>
@@ -2398,13 +2776,13 @@
         <v>1</v>
       </c>
       <c r="F40" t="n">
-        <v>2138731.14071836</v>
+        <v>4904400</v>
       </c>
       <c r="G40" t="n">
-        <v>74741.1407183595</v>
+        <v>180603</v>
       </c>
       <c r="H40" t="n">
-        <v>3.621196842928478</v>
+        <v>3.823259128197084</v>
       </c>
       <c r="I40" t="inlineStr">
         <is>
@@ -2420,11 +2798,11 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>미창석유</t>
+          <t>오케아니스 에코 탱커스</t>
         </is>
       </c>
       <c r="C41" t="n">
-        <v>18</v>
+        <v>65</v>
       </c>
       <c r="D41" t="inlineStr">
         <is>
@@ -2435,13 +2813,13 @@
         <v>1</v>
       </c>
       <c r="F41" t="n">
-        <v>2032200</v>
+        <v>4575098.725873504</v>
       </c>
       <c r="G41" t="n">
-        <v>-360000</v>
+        <v>2318738.725873504</v>
       </c>
       <c r="H41" t="n">
-        <v>-15.04890895410083</v>
+        <v>102.7645732894354</v>
       </c>
       <c r="I41" t="inlineStr">
         <is>
@@ -2457,11 +2835,11 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>대창단조</t>
+          <t>삼성화재</t>
         </is>
       </c>
       <c r="C42" t="n">
-        <v>300</v>
+        <v>9</v>
       </c>
       <c r="D42" t="inlineStr">
         <is>
@@ -2472,13 +2850,13 @@
         <v>1</v>
       </c>
       <c r="F42" t="n">
-        <v>1914000</v>
+        <v>4446000</v>
       </c>
       <c r="G42" t="n">
-        <v>-144000</v>
+        <v>-185000</v>
       </c>
       <c r="H42" t="n">
-        <v>-6.997084548104956</v>
+        <v>-3.994817534009933</v>
       </c>
       <c r="I42" t="inlineStr">
         <is>
@@ -2494,11 +2872,11 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>동방</t>
+          <t>DL이앤씨</t>
         </is>
       </c>
       <c r="C43" t="n">
-        <v>681</v>
+        <v>80</v>
       </c>
       <c r="D43" t="inlineStr">
         <is>
@@ -2509,13 +2887,13 @@
         <v>1</v>
       </c>
       <c r="F43" t="n">
-        <v>1882965</v>
+        <v>4128000</v>
       </c>
       <c r="G43" t="n">
-        <v>-88536</v>
+        <v>717000</v>
       </c>
       <c r="H43" t="n">
-        <v>-4.490791533963209</v>
+        <v>21.02022867194371</v>
       </c>
       <c r="I43" t="inlineStr">
         <is>
@@ -2531,11 +2909,11 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>하나금융지주</t>
+          <t>차코스 에너지 내비게이션</t>
         </is>
       </c>
       <c r="C44" t="n">
-        <v>15</v>
+        <v>75</v>
       </c>
       <c r="D44" t="inlineStr">
         <is>
@@ -2546,13 +2924,13 @@
         <v>1</v>
       </c>
       <c r="F44" t="n">
-        <v>1717500</v>
+        <v>4007418.271141662</v>
       </c>
       <c r="G44" t="n">
-        <v>35000</v>
+        <v>182770.2711416623</v>
       </c>
       <c r="H44" t="n">
-        <v>2.080237741456166</v>
+        <v>4.778747511971357</v>
       </c>
       <c r="I44" t="inlineStr">
         <is>
@@ -2568,11 +2946,11 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>스타 벌크 캐리어스</t>
+          <t>동원개발</t>
         </is>
       </c>
       <c r="C45" t="n">
-        <v>50</v>
+        <v>1360</v>
       </c>
       <c r="D45" t="inlineStr">
         <is>
@@ -2583,13 +2961,13 @@
         <v>1</v>
       </c>
       <c r="F45" t="n">
-        <v>1712476.648945617</v>
+        <v>3978000</v>
       </c>
       <c r="G45" t="n">
-        <v>398123.648945618</v>
+        <v>240600</v>
       </c>
       <c r="H45" t="n">
-        <v>30.29046602743845</v>
+        <v>6.437630438272596</v>
       </c>
       <c r="I45" t="inlineStr">
         <is>
@@ -2605,11 +2983,11 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>유나이티드헬스 그룹</t>
+          <t>HD건설기계</t>
         </is>
       </c>
       <c r="C46" t="n">
-        <v>4</v>
+        <v>31</v>
       </c>
       <c r="D46" t="inlineStr">
         <is>
@@ -2620,13 +2998,13 @@
         <v>1</v>
       </c>
       <c r="F46" t="n">
-        <v>1699490.128895313</v>
+        <v>3955600</v>
       </c>
       <c r="G46" t="n">
-        <v>5034.128895312548</v>
+        <v>-79496</v>
       </c>
       <c r="H46" t="n">
-        <v>0.297094105442251</v>
+        <v>-1.970114217852561</v>
       </c>
       <c r="I46" t="inlineStr">
         <is>
@@ -2642,11 +3020,11 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>케이씨</t>
+          <t>피바디 에너지</t>
         </is>
       </c>
       <c r="C47" t="n">
-        <v>50</v>
+        <v>65</v>
       </c>
       <c r="D47" t="inlineStr">
         <is>
@@ -2657,13 +3035,13 @@
         <v>1</v>
       </c>
       <c r="F47" t="n">
-        <v>1640000</v>
+        <v>3423839.074937592</v>
       </c>
       <c r="G47" t="n">
-        <v>-9500.000000000698</v>
+        <v>1953067.074937592</v>
       </c>
       <c r="H47" t="n">
-        <v>-0.5759321006365986</v>
+        <v>132.7919674115085</v>
       </c>
       <c r="I47" t="inlineStr">
         <is>
@@ -2679,11 +3057,11 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>삼성생명</t>
+          <t>더치 브로스</t>
         </is>
       </c>
       <c r="C48" t="n">
-        <v>4</v>
+        <v>39</v>
       </c>
       <c r="D48" t="inlineStr">
         <is>
@@ -2694,13 +3072,13 @@
         <v>1</v>
       </c>
       <c r="F48" t="n">
-        <v>940000</v>
+        <v>2965846.22503092</v>
       </c>
       <c r="G48" t="n">
-        <v>107000</v>
+        <v>-224797.7749690795</v>
       </c>
       <c r="H48" t="n">
-        <v>12.84513805522209</v>
+        <v>-7.04552983564069</v>
       </c>
       <c r="I48" t="inlineStr">
         <is>
@@ -2716,7 +3094,7 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>클리블랜드 클리프스</t>
+          <t>현대제철</t>
         </is>
       </c>
       <c r="C49" t="n">
@@ -2731,13 +3109,13 @@
         <v>1</v>
       </c>
       <c r="F49" t="n">
-        <v>857055.5630100402</v>
+        <v>2607500</v>
       </c>
       <c r="G49" t="n">
-        <v>-158999.4369899598</v>
+        <v>-200000</v>
       </c>
       <c r="H49" t="n">
-        <v>-15.64870376012714</v>
+        <v>-7.123775601068566</v>
       </c>
       <c r="I49" t="inlineStr">
         <is>
@@ -2753,11 +3131,11 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>비에이치아이</t>
+          <t>KoAct 코스닥액티브</t>
         </is>
       </c>
       <c r="C50" t="n">
-        <v>8</v>
+        <v>200</v>
       </c>
       <c r="D50" t="inlineStr">
         <is>
@@ -2768,13 +3146,13 @@
         <v>1</v>
       </c>
       <c r="F50" t="n">
-        <v>844800</v>
+        <v>2598000</v>
       </c>
       <c r="G50" t="n">
-        <v>179685</v>
+        <v>-104000</v>
       </c>
       <c r="H50" t="n">
-        <v>27.01562887620938</v>
+        <v>-3.84900074019245</v>
       </c>
       <c r="I50" t="inlineStr">
         <is>
@@ -2790,11 +3168,11 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>하프니아</t>
+          <t>휴스틸</t>
         </is>
       </c>
       <c r="C51" t="n">
-        <v>80</v>
+        <v>500</v>
       </c>
       <c r="D51" t="inlineStr">
         <is>
@@ -2805,13 +3183,13 @@
         <v>1</v>
       </c>
       <c r="F51" t="n">
-        <v>821489.5606615674</v>
+        <v>2560000</v>
       </c>
       <c r="G51" t="n">
-        <v>195758.5606615674</v>
+        <v>281390</v>
       </c>
       <c r="H51" t="n">
-        <v>31.28477902829928</v>
+        <v>12.34919534277476</v>
       </c>
       <c r="I51" t="inlineStr">
         <is>
@@ -2827,11 +3205,11 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>텍사스 퍼시픽 랜드</t>
+          <t>넥스틸</t>
         </is>
       </c>
       <c r="C52" t="n">
-        <v>1</v>
+        <v>200</v>
       </c>
       <c r="D52" t="inlineStr">
         <is>
@@ -2842,13 +3220,13 @@
         <v>1</v>
       </c>
       <c r="F52" t="n">
-        <v>794737.7576458007</v>
+        <v>2400000</v>
       </c>
       <c r="G52" t="n">
-        <v>16146.75764580071</v>
+        <v>389000</v>
       </c>
       <c r="H52" t="n">
-        <v>2.073843345967358</v>
+        <v>19.34361014420686</v>
       </c>
       <c r="I52" t="inlineStr">
         <is>
@@ -2864,30 +3242,548 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
+          <t>대신증권</t>
+        </is>
+      </c>
+      <c r="C53" t="n">
+        <v>55</v>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E53" t="n">
+        <v>1</v>
+      </c>
+      <c r="F53" t="n">
+        <v>2238500</v>
+      </c>
+      <c r="G53" t="n">
+        <v>528999</v>
+      </c>
+      <c r="H53" t="n">
+        <v>30.94464408034859</v>
+      </c>
+      <c r="I53" t="inlineStr">
+        <is>
+          <t>2026-03-18T14:32:42</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>2026-03-18</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>발레로 에너지</t>
+        </is>
+      </c>
+      <c r="C54" t="n">
+        <v>6</v>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E54" t="n">
+        <v>1</v>
+      </c>
+      <c r="F54" t="n">
+        <v>2138731.14071836</v>
+      </c>
+      <c r="G54" t="n">
+        <v>74741.1407183595</v>
+      </c>
+      <c r="H54" t="n">
+        <v>3.621196842928478</v>
+      </c>
+      <c r="I54" t="inlineStr">
+        <is>
+          <t>2026-03-18T14:32:42</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>2026-03-18</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>미창석유</t>
+        </is>
+      </c>
+      <c r="C55" t="n">
+        <v>18</v>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E55" t="n">
+        <v>1</v>
+      </c>
+      <c r="F55" t="n">
+        <v>2032200</v>
+      </c>
+      <c r="G55" t="n">
+        <v>-360000</v>
+      </c>
+      <c r="H55" t="n">
+        <v>-15.04890895410083</v>
+      </c>
+      <c r="I55" t="inlineStr">
+        <is>
+          <t>2026-03-18T14:32:42</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>2026-03-18</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>대창단조</t>
+        </is>
+      </c>
+      <c r="C56" t="n">
+        <v>300</v>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E56" t="n">
+        <v>1</v>
+      </c>
+      <c r="F56" t="n">
+        <v>1914000</v>
+      </c>
+      <c r="G56" t="n">
+        <v>-144000</v>
+      </c>
+      <c r="H56" t="n">
+        <v>-6.997084548104956</v>
+      </c>
+      <c r="I56" t="inlineStr">
+        <is>
+          <t>2026-03-18T14:32:42</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>2026-03-18</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>동방</t>
+        </is>
+      </c>
+      <c r="C57" t="n">
+        <v>681</v>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E57" t="n">
+        <v>1</v>
+      </c>
+      <c r="F57" t="n">
+        <v>1882965</v>
+      </c>
+      <c r="G57" t="n">
+        <v>-88536</v>
+      </c>
+      <c r="H57" t="n">
+        <v>-4.490791533963209</v>
+      </c>
+      <c r="I57" t="inlineStr">
+        <is>
+          <t>2026-03-18T14:32:42</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>2026-03-18</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>하나금융지주</t>
+        </is>
+      </c>
+      <c r="C58" t="n">
+        <v>15</v>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E58" t="n">
+        <v>1</v>
+      </c>
+      <c r="F58" t="n">
+        <v>1717500</v>
+      </c>
+      <c r="G58" t="n">
+        <v>35000</v>
+      </c>
+      <c r="H58" t="n">
+        <v>2.080237741456166</v>
+      </c>
+      <c r="I58" t="inlineStr">
+        <is>
+          <t>2026-03-18T14:32:42</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>2026-03-18</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>스타 벌크 캐리어스</t>
+        </is>
+      </c>
+      <c r="C59" t="n">
+        <v>50</v>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E59" t="n">
+        <v>1</v>
+      </c>
+      <c r="F59" t="n">
+        <v>1712476.648945617</v>
+      </c>
+      <c r="G59" t="n">
+        <v>398123.648945618</v>
+      </c>
+      <c r="H59" t="n">
+        <v>30.29046602743845</v>
+      </c>
+      <c r="I59" t="inlineStr">
+        <is>
+          <t>2026-03-18T14:32:42</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>2026-03-18</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>유나이티드헬스 그룹</t>
+        </is>
+      </c>
+      <c r="C60" t="n">
+        <v>4</v>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E60" t="n">
+        <v>1</v>
+      </c>
+      <c r="F60" t="n">
+        <v>1699490.128895313</v>
+      </c>
+      <c r="G60" t="n">
+        <v>5034.128895312548</v>
+      </c>
+      <c r="H60" t="n">
+        <v>0.297094105442251</v>
+      </c>
+      <c r="I60" t="inlineStr">
+        <is>
+          <t>2026-03-18T14:32:42</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>2026-03-18</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>케이씨</t>
+        </is>
+      </c>
+      <c r="C61" t="n">
+        <v>50</v>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E61" t="n">
+        <v>1</v>
+      </c>
+      <c r="F61" t="n">
+        <v>1640000</v>
+      </c>
+      <c r="G61" t="n">
+        <v>-9500.000000000698</v>
+      </c>
+      <c r="H61" t="n">
+        <v>-0.5759321006365986</v>
+      </c>
+      <c r="I61" t="inlineStr">
+        <is>
+          <t>2026-03-18T14:32:42</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>2026-03-18</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>삼성생명</t>
+        </is>
+      </c>
+      <c r="C62" t="n">
+        <v>4</v>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E62" t="n">
+        <v>1</v>
+      </c>
+      <c r="F62" t="n">
+        <v>940000</v>
+      </c>
+      <c r="G62" t="n">
+        <v>107000</v>
+      </c>
+      <c r="H62" t="n">
+        <v>12.84513805522209</v>
+      </c>
+      <c r="I62" t="inlineStr">
+        <is>
+          <t>2026-03-18T14:32:42</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>2026-03-18</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>클리블랜드 클리프스</t>
+        </is>
+      </c>
+      <c r="C63" t="n">
+        <v>70</v>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E63" t="n">
+        <v>1</v>
+      </c>
+      <c r="F63" t="n">
+        <v>857055.5630100402</v>
+      </c>
+      <c r="G63" t="n">
+        <v>-158999.4369899598</v>
+      </c>
+      <c r="H63" t="n">
+        <v>-15.64870376012714</v>
+      </c>
+      <c r="I63" t="inlineStr">
+        <is>
+          <t>2026-03-18T14:32:42</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>2026-03-18</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>비에이치아이</t>
+        </is>
+      </c>
+      <c r="C64" t="n">
+        <v>8</v>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E64" t="n">
+        <v>1</v>
+      </c>
+      <c r="F64" t="n">
+        <v>844800</v>
+      </c>
+      <c r="G64" t="n">
+        <v>179685</v>
+      </c>
+      <c r="H64" t="n">
+        <v>27.01562887620938</v>
+      </c>
+      <c r="I64" t="inlineStr">
+        <is>
+          <t>2026-03-18T14:32:42</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>2026-03-18</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>하프니아</t>
+        </is>
+      </c>
+      <c r="C65" t="n">
+        <v>80</v>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E65" t="n">
+        <v>1</v>
+      </c>
+      <c r="F65" t="n">
+        <v>821489.5606615674</v>
+      </c>
+      <c r="G65" t="n">
+        <v>195758.5606615674</v>
+      </c>
+      <c r="H65" t="n">
+        <v>31.28477902829928</v>
+      </c>
+      <c r="I65" t="inlineStr">
+        <is>
+          <t>2026-03-18T14:32:42</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>2026-03-18</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>텍사스 퍼시픽 랜드</t>
+        </is>
+      </c>
+      <c r="C66" t="n">
+        <v>1</v>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E66" t="n">
+        <v>1</v>
+      </c>
+      <c r="F66" t="n">
+        <v>794737.7576458007</v>
+      </c>
+      <c r="G66" t="n">
+        <v>16146.75764580071</v>
+      </c>
+      <c r="H66" t="n">
+        <v>2.073843345967358</v>
+      </c>
+      <c r="I66" t="inlineStr">
+        <is>
+          <t>2026-03-18T14:32:42</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>2026-03-18</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
           <t>노블</t>
         </is>
       </c>
-      <c r="C53" t="n">
+      <c r="C67" t="n">
         <v>99</v>
       </c>
-      <c r="D53" t="inlineStr">
-        <is>
-          <t>KRW</t>
-        </is>
-      </c>
-      <c r="E53" t="n">
-        <v>1</v>
-      </c>
-      <c r="F53" t="n">
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E67" t="n">
+        <v>1</v>
+      </c>
+      <c r="F67" t="n">
         <v>40689</v>
       </c>
-      <c r="G53" t="n">
+      <c r="G67" t="n">
         <v>-3866519</v>
       </c>
-      <c r="H53" t="n">
+      <c r="H67" t="n">
         <v>-98.95861699709869</v>
       </c>
-      <c r="I53" t="inlineStr">
+      <c r="I67" t="inlineStr">
         <is>
           <t>2026-03-18T14:32:42</t>
         </is>
@@ -2953,7 +3849,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>2026-03-18T21:08:03</t>
+          <t>2026-03-18T21:08:43</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: portfolio snapshot 2026-03-17 (2026-03-18T21:08:45)
</commit_message>
<xml_diff>
--- a/portfolio_auto.xlsx
+++ b/portfolio_auto.xlsx
@@ -864,13 +864,13 @@
         <v>1</v>
       </c>
       <c r="E16" t="n">
-        <v>13847377</v>
+        <v>14082576.9328374</v>
       </c>
       <c r="F16" t="n">
-        <v>1740828</v>
+        <v>1976027.932837404</v>
       </c>
       <c r="G16" t="n">
-        <v>14.37</v>
+        <v>16.3219752617976</v>
       </c>
     </row>
     <row r="17">
@@ -891,13 +891,13 @@
         <v>1</v>
       </c>
       <c r="E17" t="n">
-        <v>8304682</v>
+        <v>8440541.129673157</v>
       </c>
       <c r="F17" t="n">
-        <v>3874818</v>
+        <v>4010677.129673157</v>
       </c>
       <c r="G17" t="n">
-        <v>87.47</v>
+        <v>90.53725192631549</v>
       </c>
     </row>
     <row r="18">
@@ -918,13 +918,13 @@
         <v>1</v>
       </c>
       <c r="E18" t="n">
-        <v>3427688</v>
+        <v>3423839.074937592</v>
       </c>
       <c r="F18" t="n">
-        <v>1956916</v>
+        <v>1953067.074937592</v>
       </c>
       <c r="G18" t="n">
-        <v>133.05</v>
+        <v>132.7919674115085</v>
       </c>
     </row>
     <row r="19">
@@ -945,13 +945,13 @@
         <v>1</v>
       </c>
       <c r="E19" t="n">
-        <v>798051</v>
+        <v>821489.5606615674</v>
       </c>
       <c r="F19" t="n">
-        <v>172320</v>
+        <v>195758.5606615674</v>
       </c>
       <c r="G19" t="n">
-        <v>27.53</v>
+        <v>31.28477902829928</v>
       </c>
     </row>
     <row r="20">
@@ -972,13 +972,13 @@
         <v>1</v>
       </c>
       <c r="E20" t="n">
-        <v>10848269</v>
+        <v>10822406.73782303</v>
       </c>
       <c r="F20" t="n">
-        <v>16254</v>
+        <v>-9608.262176971883</v>
       </c>
       <c r="G20" t="n">
-        <v>0.15</v>
+        <v>-0.08870244526961865</v>
       </c>
     </row>
     <row r="21">
@@ -999,13 +999,13 @@
         <v>1</v>
       </c>
       <c r="E21" t="n">
-        <v>2391208</v>
+        <v>2400000</v>
       </c>
       <c r="F21" t="n">
-        <v>380208</v>
+        <v>389000</v>
       </c>
       <c r="G21" t="n">
-        <v>18.9</v>
+        <v>19.34361014420686</v>
       </c>
     </row>
     <row r="22">
@@ -1026,13 +1026,13 @@
         <v>1</v>
       </c>
       <c r="E22" t="n">
-        <v>2190111</v>
+        <v>2238500</v>
       </c>
       <c r="F22" t="n">
-        <v>480610</v>
+        <v>528999</v>
       </c>
       <c r="G22" t="n">
-        <v>28.11</v>
+        <v>30.94464408034859</v>
       </c>
     </row>
     <row r="23">
@@ -1053,13 +1053,13 @@
         <v>1</v>
       </c>
       <c r="E23" t="n">
-        <v>1901190</v>
+        <v>1914000</v>
       </c>
       <c r="F23" t="n">
-        <v>-156810</v>
+        <v>-144000</v>
       </c>
       <c r="G23" t="n">
-        <v>-7.61</v>
+        <v>-6.997084548104956</v>
       </c>
     </row>
     <row r="24">
@@ -1080,13 +1080,13 @@
         <v>1</v>
       </c>
       <c r="E24" t="n">
-        <v>9740480</v>
+        <v>9570000</v>
       </c>
       <c r="F24" t="n">
-        <v>2527480</v>
+        <v>2357000</v>
       </c>
       <c r="G24" t="n">
-        <v>35.04</v>
+        <v>32.67711077221684</v>
       </c>
     </row>
     <row r="25">
@@ -1107,13 +1107,13 @@
         <v>1</v>
       </c>
       <c r="E25" t="n">
-        <v>1841600</v>
+        <v>1882965</v>
       </c>
       <c r="F25" t="n">
-        <v>-129901</v>
+        <v>-88536</v>
       </c>
       <c r="G25" t="n">
-        <v>-6.58</v>
+        <v>-4.490791533963209</v>
       </c>
     </row>
     <row r="26">
@@ -1134,13 +1134,13 @@
         <v>1</v>
       </c>
       <c r="E26" t="n">
-        <v>3881821</v>
+        <v>3978000</v>
       </c>
       <c r="F26" t="n">
-        <v>144421</v>
+        <v>240600</v>
       </c>
       <c r="G26" t="n">
-        <v>3.86</v>
+        <v>6.437630438272596</v>
       </c>
     </row>
     <row r="27">
@@ -1161,13 +1161,13 @@
         <v>1</v>
       </c>
       <c r="E27" t="n">
-        <v>2049693</v>
+        <v>2032200</v>
       </c>
       <c r="F27" t="n">
-        <v>-342507</v>
+        <v>-360000</v>
       </c>
       <c r="G27" t="n">
-        <v>-14.31</v>
+        <v>-15.04890895410083</v>
       </c>
     </row>
     <row r="28">
@@ -1188,13 +1188,13 @@
         <v>1</v>
       </c>
       <c r="E28" t="n">
-        <v>850296</v>
+        <v>844800</v>
       </c>
       <c r="F28" t="n">
-        <v>185181</v>
+        <v>179685</v>
       </c>
       <c r="G28" t="n">
-        <v>27.84</v>
+        <v>27.01562887620938</v>
       </c>
     </row>
     <row r="29">
@@ -1215,13 +1215,13 @@
         <v>1</v>
       </c>
       <c r="E29" t="n">
-        <v>872252</v>
+        <v>940000</v>
       </c>
       <c r="F29" t="n">
-        <v>39252</v>
+        <v>107000</v>
       </c>
       <c r="G29" t="n">
-        <v>4.71</v>
+        <v>12.84513805522209</v>
       </c>
     </row>
   </sheetData>
@@ -1279,7 +1279,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2026-03-18T21:08:43</t>
+          <t>2026-03-18T21:08:45</t>
         </is>
       </c>
       <c r="E2" t="n">
@@ -1370,17 +1370,17 @@
         <v>1</v>
       </c>
       <c r="F2" t="n">
-        <v>13847377</v>
+        <v>14082576.9328374</v>
       </c>
       <c r="G2" t="n">
-        <v>1740828</v>
+        <v>1976027.932837404</v>
       </c>
       <c r="H2" t="n">
-        <v>14.37</v>
+        <v>16.3219752617976</v>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>2026-03-18T21:08:43</t>
+          <t>2026-03-18T21:08:45</t>
         </is>
       </c>
     </row>
@@ -1407,17 +1407,17 @@
         <v>1</v>
       </c>
       <c r="F3" t="n">
-        <v>10848269</v>
+        <v>10822406.73782303</v>
       </c>
       <c r="G3" t="n">
-        <v>16254</v>
+        <v>-9608.262176971883</v>
       </c>
       <c r="H3" t="n">
-        <v>0.15</v>
+        <v>-0.08870244526961865</v>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>2026-03-18T21:08:43</t>
+          <t>2026-03-18T21:08:45</t>
         </is>
       </c>
     </row>
@@ -1444,17 +1444,17 @@
         <v>1</v>
       </c>
       <c r="F4" t="n">
-        <v>9740480</v>
+        <v>9570000</v>
       </c>
       <c r="G4" t="n">
-        <v>2527480</v>
+        <v>2357000</v>
       </c>
       <c r="H4" t="n">
-        <v>35.04</v>
+        <v>32.67711077221684</v>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>2026-03-18T21:08:43</t>
+          <t>2026-03-18T21:08:45</t>
         </is>
       </c>
     </row>
@@ -1481,17 +1481,17 @@
         <v>1</v>
       </c>
       <c r="F5" t="n">
-        <v>8304682</v>
+        <v>8440541.129673157</v>
       </c>
       <c r="G5" t="n">
-        <v>3874818</v>
+        <v>4010677.129673157</v>
       </c>
       <c r="H5" t="n">
-        <v>87.47</v>
+        <v>90.53725192631549</v>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>2026-03-18T21:08:43</t>
+          <t>2026-03-18T21:08:45</t>
         </is>
       </c>
     </row>
@@ -1528,7 +1528,7 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>2026-03-18T21:08:43</t>
+          <t>2026-03-18T21:08:45</t>
         </is>
       </c>
     </row>
@@ -1565,7 +1565,7 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>2026-03-18T21:08:43</t>
+          <t>2026-03-18T21:08:45</t>
         </is>
       </c>
     </row>
@@ -1602,7 +1602,7 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>2026-03-18T21:08:43</t>
+          <t>2026-03-18T21:08:45</t>
         </is>
       </c>
     </row>
@@ -1639,7 +1639,7 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>2026-03-18T21:08:43</t>
+          <t>2026-03-18T21:08:45</t>
         </is>
       </c>
     </row>
@@ -1676,7 +1676,7 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>2026-03-18T21:08:43</t>
+          <t>2026-03-18T21:08:45</t>
         </is>
       </c>
     </row>
@@ -1713,7 +1713,7 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>2026-03-18T21:08:43</t>
+          <t>2026-03-18T21:08:45</t>
         </is>
       </c>
     </row>
@@ -1750,7 +1750,7 @@
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>2026-03-18T21:08:43</t>
+          <t>2026-03-18T21:08:45</t>
         </is>
       </c>
     </row>
@@ -1777,17 +1777,17 @@
         <v>1</v>
       </c>
       <c r="F13" t="n">
-        <v>3881821</v>
+        <v>3978000</v>
       </c>
       <c r="G13" t="n">
-        <v>144421</v>
+        <v>240600</v>
       </c>
       <c r="H13" t="n">
-        <v>3.86</v>
+        <v>6.437630438272596</v>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>2026-03-18T21:08:43</t>
+          <t>2026-03-18T21:08:45</t>
         </is>
       </c>
     </row>
@@ -1814,17 +1814,17 @@
         <v>1</v>
       </c>
       <c r="F14" t="n">
-        <v>3427688</v>
+        <v>3423839.074937592</v>
       </c>
       <c r="G14" t="n">
-        <v>1956916</v>
+        <v>1953067.074937592</v>
       </c>
       <c r="H14" t="n">
-        <v>133.05</v>
+        <v>132.7919674115085</v>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>2026-03-18T21:08:43</t>
+          <t>2026-03-18T21:08:45</t>
         </is>
       </c>
     </row>
@@ -1861,7 +1861,7 @@
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>2026-03-18T21:08:43</t>
+          <t>2026-03-18T21:08:45</t>
         </is>
       </c>
     </row>
@@ -1888,17 +1888,17 @@
         <v>1</v>
       </c>
       <c r="F16" t="n">
-        <v>2391208</v>
+        <v>2400000</v>
       </c>
       <c r="G16" t="n">
-        <v>380208</v>
+        <v>389000</v>
       </c>
       <c r="H16" t="n">
-        <v>18.9</v>
+        <v>19.34361014420686</v>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>2026-03-18T21:08:43</t>
+          <t>2026-03-18T21:08:45</t>
         </is>
       </c>
     </row>
@@ -1925,17 +1925,17 @@
         <v>1</v>
       </c>
       <c r="F17" t="n">
-        <v>2190111</v>
+        <v>2238500</v>
       </c>
       <c r="G17" t="n">
-        <v>480610</v>
+        <v>528999</v>
       </c>
       <c r="H17" t="n">
-        <v>28.11</v>
+        <v>30.94464408034859</v>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>2026-03-18T21:08:43</t>
+          <t>2026-03-18T21:08:45</t>
         </is>
       </c>
     </row>
@@ -1972,7 +1972,7 @@
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>2026-03-18T21:08:43</t>
+          <t>2026-03-18T21:08:45</t>
         </is>
       </c>
     </row>
@@ -1999,17 +1999,17 @@
         <v>1</v>
       </c>
       <c r="F19" t="n">
-        <v>2049693</v>
+        <v>2032200</v>
       </c>
       <c r="G19" t="n">
-        <v>-342507</v>
+        <v>-360000</v>
       </c>
       <c r="H19" t="n">
-        <v>-14.31</v>
+        <v>-15.04890895410083</v>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>2026-03-18T21:08:43</t>
+          <t>2026-03-18T21:08:45</t>
         </is>
       </c>
     </row>
@@ -2036,17 +2036,17 @@
         <v>1</v>
       </c>
       <c r="F20" t="n">
-        <v>1901190</v>
+        <v>1914000</v>
       </c>
       <c r="G20" t="n">
-        <v>-156810</v>
+        <v>-144000</v>
       </c>
       <c r="H20" t="n">
-        <v>-7.61</v>
+        <v>-6.997084548104956</v>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>2026-03-18T21:08:43</t>
+          <t>2026-03-18T21:08:45</t>
         </is>
       </c>
     </row>
@@ -2073,17 +2073,17 @@
         <v>1</v>
       </c>
       <c r="F21" t="n">
-        <v>1841600</v>
+        <v>1882965</v>
       </c>
       <c r="G21" t="n">
-        <v>-129901</v>
+        <v>-88536</v>
       </c>
       <c r="H21" t="n">
-        <v>-6.58</v>
+        <v>-4.490791533963209</v>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>2026-03-18T21:08:43</t>
+          <t>2026-03-18T21:08:45</t>
         </is>
       </c>
     </row>
@@ -2120,7 +2120,7 @@
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>2026-03-18T21:08:43</t>
+          <t>2026-03-18T21:08:45</t>
         </is>
       </c>
     </row>
@@ -2157,7 +2157,7 @@
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>2026-03-18T21:08:43</t>
+          <t>2026-03-18T21:08:45</t>
         </is>
       </c>
     </row>
@@ -2184,17 +2184,17 @@
         <v>1</v>
       </c>
       <c r="F24" t="n">
-        <v>872252</v>
+        <v>940000</v>
       </c>
       <c r="G24" t="n">
-        <v>39252</v>
+        <v>107000</v>
       </c>
       <c r="H24" t="n">
-        <v>4.71</v>
+        <v>12.84513805522209</v>
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>2026-03-18T21:08:43</t>
+          <t>2026-03-18T21:08:45</t>
         </is>
       </c>
     </row>
@@ -2231,7 +2231,7 @@
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>2026-03-18T21:08:43</t>
+          <t>2026-03-18T21:08:45</t>
         </is>
       </c>
     </row>
@@ -2258,17 +2258,17 @@
         <v>1</v>
       </c>
       <c r="F26" t="n">
-        <v>850296</v>
+        <v>844800</v>
       </c>
       <c r="G26" t="n">
-        <v>185181</v>
+        <v>179685</v>
       </c>
       <c r="H26" t="n">
-        <v>27.84</v>
+        <v>27.01562887620938</v>
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>2026-03-18T21:08:43</t>
+          <t>2026-03-18T21:08:45</t>
         </is>
       </c>
     </row>
@@ -2295,17 +2295,17 @@
         <v>1</v>
       </c>
       <c r="F27" t="n">
-        <v>798051</v>
+        <v>821489.5606615674</v>
       </c>
       <c r="G27" t="n">
-        <v>172320</v>
+        <v>195758.5606615674</v>
       </c>
       <c r="H27" t="n">
-        <v>27.53</v>
+        <v>31.28477902829928</v>
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>2026-03-18T21:08:43</t>
+          <t>2026-03-18T21:08:45</t>
         </is>
       </c>
     </row>
@@ -2342,7 +2342,7 @@
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>2026-03-18T21:08:43</t>
+          <t>2026-03-18T21:08:45</t>
         </is>
       </c>
     </row>
@@ -2379,7 +2379,7 @@
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>2026-03-18T21:08:43</t>
+          <t>2026-03-18T21:08:45</t>
         </is>
       </c>
     </row>
@@ -3849,7 +3849,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>2026-03-18T21:08:43</t>
+          <t>2026-03-18T21:08:45</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: portfolio snapshot 2026-03-17 (2026-03-18T21:09:27)
</commit_message>
<xml_diff>
--- a/portfolio_auto.xlsx
+++ b/portfolio_auto.xlsx
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G29"/>
+  <dimension ref="A1:G39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1222,6 +1222,276 @@
       </c>
       <c r="G29" t="n">
         <v>12.84513805522209</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>삼성화재</t>
+        </is>
+      </c>
+      <c r="B30" t="n">
+        <v>7</v>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="D30" t="n">
+        <v>1</v>
+      </c>
+      <c r="E30" t="n">
+        <v>3335815</v>
+      </c>
+      <c r="F30" t="n">
+        <v>-295185</v>
+      </c>
+      <c r="G30" t="n">
+        <v>-8.119999999999999</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>세아제강</t>
+        </is>
+      </c>
+      <c r="B31" t="n">
+        <v>50</v>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="D31" t="n">
+        <v>1</v>
+      </c>
+      <c r="E31" t="n">
+        <v>6896180</v>
+      </c>
+      <c r="F31" t="n">
+        <v>586180</v>
+      </c>
+      <c r="G31" t="n">
+        <v>9.279999999999999</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>케이씨</t>
+        </is>
+      </c>
+      <c r="B32" t="n">
+        <v>50</v>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="D32" t="n">
+        <v>1</v>
+      </c>
+      <c r="E32" t="n">
+        <v>1576840</v>
+      </c>
+      <c r="F32" t="n">
+        <v>-72660</v>
+      </c>
+      <c r="G32" t="n">
+        <v>-4.4</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>하나금융지주</t>
+        </is>
+      </c>
+      <c r="B33" t="n">
+        <v>10</v>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="D33" t="n">
+        <v>1</v>
+      </c>
+      <c r="E33" t="n">
+        <v>1107780</v>
+      </c>
+      <c r="F33" t="n">
+        <v>-1220</v>
+      </c>
+      <c r="G33" t="n">
+        <v>-0.11</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>현대제철</t>
+        </is>
+      </c>
+      <c r="B34" t="n">
+        <v>70</v>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="D34" t="n">
+        <v>1</v>
+      </c>
+      <c r="E34" t="n">
+        <v>2494002</v>
+      </c>
+      <c r="F34" t="n">
+        <v>-313498</v>
+      </c>
+      <c r="G34" t="n">
+        <v>-11.16</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>휴스틸</t>
+        </is>
+      </c>
+      <c r="B35" t="n">
+        <v>500</v>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="D35" t="n">
+        <v>1</v>
+      </c>
+      <c r="E35" t="n">
+        <v>2450090</v>
+      </c>
+      <c r="F35" t="n">
+        <v>171480</v>
+      </c>
+      <c r="G35" t="n">
+        <v>7.52</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>DL이앤씨</t>
+        </is>
+      </c>
+      <c r="B36" t="n">
+        <v>80</v>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="D36" t="n">
+        <v>1</v>
+      </c>
+      <c r="E36" t="n">
+        <v>3792400</v>
+      </c>
+      <c r="F36" t="n">
+        <v>381400</v>
+      </c>
+      <c r="G36" t="n">
+        <v>11.18</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>HD건설기계</t>
+        </is>
+      </c>
+      <c r="B37" t="n">
+        <v>31</v>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="D37" t="n">
+        <v>1</v>
+      </c>
+      <c r="E37" t="n">
+        <v>3885810</v>
+      </c>
+      <c r="F37" t="n">
+        <v>-149286</v>
+      </c>
+      <c r="G37" t="n">
+        <v>-3.69</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>KoAct 코스닥액티브</t>
+        </is>
+      </c>
+      <c r="B38" t="n">
+        <v>200</v>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="D38" t="n">
+        <v>1</v>
+      </c>
+      <c r="E38" t="n">
+        <v>2580000</v>
+      </c>
+      <c r="F38" t="n">
+        <v>-122000</v>
+      </c>
+      <c r="G38" t="n">
+        <v>-4.51</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>TIME 코리아밸류업액티브</t>
+        </is>
+      </c>
+      <c r="B39" t="n">
+        <v>201</v>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="D39" t="n">
+        <v>1</v>
+      </c>
+      <c r="E39" t="n">
+        <v>4656165</v>
+      </c>
+      <c r="F39" t="n">
+        <v>-67632</v>
+      </c>
+      <c r="G39" t="n">
+        <v>-1.43</v>
       </c>
     </row>
   </sheetData>
@@ -1279,7 +1549,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2026-03-18T21:08:45</t>
+          <t>2026-03-18T21:09:27</t>
         </is>
       </c>
       <c r="E2" t="n">
@@ -1297,7 +1567,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I67"/>
+  <dimension ref="A1:I77"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1380,7 +1650,7 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>2026-03-18T21:08:45</t>
+          <t>2026-03-18T21:09:27</t>
         </is>
       </c>
     </row>
@@ -1417,7 +1687,7 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>2026-03-18T21:08:45</t>
+          <t>2026-03-18T21:09:27</t>
         </is>
       </c>
     </row>
@@ -1454,7 +1724,7 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>2026-03-18T21:08:45</t>
+          <t>2026-03-18T21:09:27</t>
         </is>
       </c>
     </row>
@@ -1491,7 +1761,7 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>2026-03-18T21:08:45</t>
+          <t>2026-03-18T21:09:27</t>
         </is>
       </c>
     </row>
@@ -1528,7 +1798,7 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>2026-03-18T21:08:45</t>
+          <t>2026-03-18T21:09:27</t>
         </is>
       </c>
     </row>
@@ -1565,7 +1835,7 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>2026-03-18T21:08:45</t>
+          <t>2026-03-18T21:09:27</t>
         </is>
       </c>
     </row>
@@ -1577,11 +1847,11 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>센트러스 에너지</t>
+          <t>세아제강</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>21</v>
+        <v>50</v>
       </c>
       <c r="D8" t="inlineStr">
         <is>
@@ -1592,17 +1862,17 @@
         <v>1</v>
       </c>
       <c r="F8" t="n">
-        <v>6546958.253894605</v>
+        <v>6896180</v>
       </c>
       <c r="G8" t="n">
-        <v>315739.2538946057</v>
+        <v>586180</v>
       </c>
       <c r="H8" t="n">
-        <v>5.067054357977239</v>
+        <v>9.279999999999999</v>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>2026-03-18T21:08:45</t>
+          <t>2026-03-18T21:09:27</t>
         </is>
       </c>
     </row>
@@ -1614,11 +1884,11 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>타이드워터</t>
+          <t>센트러스 에너지</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>48</v>
+        <v>21</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
@@ -1629,17 +1899,17 @@
         <v>1</v>
       </c>
       <c r="F9" t="n">
-        <v>5456864.752692774</v>
+        <v>6546958.253894605</v>
       </c>
       <c r="G9" t="n">
-        <v>1732319.752692774</v>
+        <v>315739.2538946057</v>
       </c>
       <c r="H9" t="n">
-        <v>46.51090945854524</v>
+        <v>5.067054357977239</v>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>2026-03-18T21:08:45</t>
+          <t>2026-03-18T21:09:27</t>
         </is>
       </c>
     </row>
@@ -1651,11 +1921,11 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>노브</t>
+          <t>타이드워터</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>185</v>
+        <v>48</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
@@ -1666,17 +1936,17 @@
         <v>1</v>
       </c>
       <c r="F10" t="n">
-        <v>5041442.310511444</v>
+        <v>5456864.752692774</v>
       </c>
       <c r="G10" t="n">
-        <v>1731434.310511444</v>
+        <v>1732319.752692774</v>
       </c>
       <c r="H10" t="n">
-        <v>52.30906724429197</v>
+        <v>46.51090945854524</v>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>2026-03-18T21:08:45</t>
+          <t>2026-03-18T21:09:27</t>
         </is>
       </c>
     </row>
@@ -1688,11 +1958,11 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>오케아니스 에코 탱커스</t>
+          <t>노브</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>65</v>
+        <v>185</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
@@ -1703,17 +1973,17 @@
         <v>1</v>
       </c>
       <c r="F11" t="n">
-        <v>4575098.725873504</v>
+        <v>5041442.310511444</v>
       </c>
       <c r="G11" t="n">
-        <v>2318738.725873504</v>
+        <v>1731434.310511444</v>
       </c>
       <c r="H11" t="n">
-        <v>102.7645732894354</v>
+        <v>52.30906724429197</v>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>2026-03-18T21:08:45</t>
+          <t>2026-03-18T21:09:27</t>
         </is>
       </c>
     </row>
@@ -1725,11 +1995,11 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>차코스 에너지 내비게이션</t>
+          <t>TIME 코리아밸류업액티브</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>75</v>
+        <v>201</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
@@ -1740,17 +2010,17 @@
         <v>1</v>
       </c>
       <c r="F12" t="n">
-        <v>4007418.271141662</v>
+        <v>4656165</v>
       </c>
       <c r="G12" t="n">
-        <v>182770.2711416623</v>
+        <v>-67632</v>
       </c>
       <c r="H12" t="n">
-        <v>4.778747511971357</v>
+        <v>-1.43</v>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>2026-03-18T21:08:45</t>
+          <t>2026-03-18T21:09:27</t>
         </is>
       </c>
     </row>
@@ -1762,11 +2032,11 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>동원개발</t>
+          <t>오케아니스 에코 탱커스</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>1360</v>
+        <v>65</v>
       </c>
       <c r="D13" t="inlineStr">
         <is>
@@ -1777,17 +2047,17 @@
         <v>1</v>
       </c>
       <c r="F13" t="n">
-        <v>3978000</v>
+        <v>4575098.725873504</v>
       </c>
       <c r="G13" t="n">
-        <v>240600</v>
+        <v>2318738.725873504</v>
       </c>
       <c r="H13" t="n">
-        <v>6.437630438272596</v>
+        <v>102.7645732894354</v>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>2026-03-18T21:08:45</t>
+          <t>2026-03-18T21:09:27</t>
         </is>
       </c>
     </row>
@@ -1799,11 +2069,11 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>피바디 에너지</t>
+          <t>차코스 에너지 내비게이션</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>65</v>
+        <v>75</v>
       </c>
       <c r="D14" t="inlineStr">
         <is>
@@ -1814,17 +2084,17 @@
         <v>1</v>
       </c>
       <c r="F14" t="n">
-        <v>3423839.074937592</v>
+        <v>4007418.271141662</v>
       </c>
       <c r="G14" t="n">
-        <v>1953067.074937592</v>
+        <v>182770.2711416623</v>
       </c>
       <c r="H14" t="n">
-        <v>132.7919674115085</v>
+        <v>4.778747511971357</v>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>2026-03-18T21:08:45</t>
+          <t>2026-03-18T21:09:27</t>
         </is>
       </c>
     </row>
@@ -1836,11 +2106,11 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>더치 브로스</t>
+          <t>동원개발</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>39</v>
+        <v>1360</v>
       </c>
       <c r="D15" t="inlineStr">
         <is>
@@ -1851,17 +2121,17 @@
         <v>1</v>
       </c>
       <c r="F15" t="n">
-        <v>2965846.22503092</v>
+        <v>3978000</v>
       </c>
       <c r="G15" t="n">
-        <v>-224797.7749690795</v>
+        <v>240600</v>
       </c>
       <c r="H15" t="n">
-        <v>-7.04552983564069</v>
+        <v>6.437630438272596</v>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>2026-03-18T21:08:45</t>
+          <t>2026-03-18T21:09:27</t>
         </is>
       </c>
     </row>
@@ -1873,11 +2143,11 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>넥스틸</t>
+          <t>HD건설기계</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>200</v>
+        <v>31</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
@@ -1888,17 +2158,17 @@
         <v>1</v>
       </c>
       <c r="F16" t="n">
-        <v>2400000</v>
+        <v>3885810</v>
       </c>
       <c r="G16" t="n">
-        <v>389000</v>
+        <v>-149286</v>
       </c>
       <c r="H16" t="n">
-        <v>19.34361014420686</v>
+        <v>-3.69</v>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>2026-03-18T21:08:45</t>
+          <t>2026-03-18T21:09:27</t>
         </is>
       </c>
     </row>
@@ -1910,11 +2180,11 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>대신증권</t>
+          <t>DL이앤씨</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>55</v>
+        <v>80</v>
       </c>
       <c r="D17" t="inlineStr">
         <is>
@@ -1925,17 +2195,17 @@
         <v>1</v>
       </c>
       <c r="F17" t="n">
-        <v>2238500</v>
+        <v>3792400</v>
       </c>
       <c r="G17" t="n">
-        <v>528999</v>
+        <v>381400</v>
       </c>
       <c r="H17" t="n">
-        <v>30.94464408034859</v>
+        <v>11.18</v>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>2026-03-18T21:08:45</t>
+          <t>2026-03-18T21:09:27</t>
         </is>
       </c>
     </row>
@@ -1947,11 +2217,11 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>발레로 에너지</t>
+          <t>피바디 에너지</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>6</v>
+        <v>65</v>
       </c>
       <c r="D18" t="inlineStr">
         <is>
@@ -1962,17 +2232,17 @@
         <v>1</v>
       </c>
       <c r="F18" t="n">
-        <v>2138731.14071836</v>
+        <v>3423839.074937592</v>
       </c>
       <c r="G18" t="n">
-        <v>74741.1407183595</v>
+        <v>1953067.074937592</v>
       </c>
       <c r="H18" t="n">
-        <v>3.621196842928478</v>
+        <v>132.7919674115085</v>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>2026-03-18T21:08:45</t>
+          <t>2026-03-18T21:09:27</t>
         </is>
       </c>
     </row>
@@ -1984,11 +2254,11 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>미창석유</t>
+          <t>삼성화재</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>18</v>
+        <v>7</v>
       </c>
       <c r="D19" t="inlineStr">
         <is>
@@ -1999,17 +2269,17 @@
         <v>1</v>
       </c>
       <c r="F19" t="n">
-        <v>2032200</v>
+        <v>3335815</v>
       </c>
       <c r="G19" t="n">
-        <v>-360000</v>
+        <v>-295185</v>
       </c>
       <c r="H19" t="n">
-        <v>-15.04890895410083</v>
+        <v>-8.119999999999999</v>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>2026-03-18T21:08:45</t>
+          <t>2026-03-18T21:09:27</t>
         </is>
       </c>
     </row>
@@ -2021,11 +2291,11 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>대창단조</t>
+          <t>더치 브로스</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>300</v>
+        <v>39</v>
       </c>
       <c r="D20" t="inlineStr">
         <is>
@@ -2036,17 +2306,17 @@
         <v>1</v>
       </c>
       <c r="F20" t="n">
-        <v>1914000</v>
+        <v>2965846.22503092</v>
       </c>
       <c r="G20" t="n">
-        <v>-144000</v>
+        <v>-224797.7749690795</v>
       </c>
       <c r="H20" t="n">
-        <v>-6.997084548104956</v>
+        <v>-7.04552983564069</v>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>2026-03-18T21:08:45</t>
+          <t>2026-03-18T21:09:27</t>
         </is>
       </c>
     </row>
@@ -2058,11 +2328,11 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>동방</t>
+          <t>KoAct 코스닥액티브</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>681</v>
+        <v>200</v>
       </c>
       <c r="D21" t="inlineStr">
         <is>
@@ -2073,17 +2343,17 @@
         <v>1</v>
       </c>
       <c r="F21" t="n">
-        <v>1882965</v>
+        <v>2580000</v>
       </c>
       <c r="G21" t="n">
-        <v>-88536</v>
+        <v>-122000</v>
       </c>
       <c r="H21" t="n">
-        <v>-4.490791533963209</v>
+        <v>-4.51</v>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>2026-03-18T21:08:45</t>
+          <t>2026-03-18T21:09:27</t>
         </is>
       </c>
     </row>
@@ -2095,11 +2365,11 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>스타 벌크 캐리어스</t>
+          <t>현대제철</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>50</v>
+        <v>70</v>
       </c>
       <c r="D22" t="inlineStr">
         <is>
@@ -2110,17 +2380,17 @@
         <v>1</v>
       </c>
       <c r="F22" t="n">
-        <v>1712476.648945617</v>
+        <v>2494002</v>
       </c>
       <c r="G22" t="n">
-        <v>398123.6489456175</v>
+        <v>-313498</v>
       </c>
       <c r="H22" t="n">
-        <v>30.29046602743841</v>
+        <v>-11.16</v>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>2026-03-18T21:08:45</t>
+          <t>2026-03-18T21:09:27</t>
         </is>
       </c>
     </row>
@@ -2132,11 +2402,11 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>유나이티드헬스 그룹</t>
+          <t>휴스틸</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>4</v>
+        <v>500</v>
       </c>
       <c r="D23" t="inlineStr">
         <is>
@@ -2147,17 +2417,17 @@
         <v>1</v>
       </c>
       <c r="F23" t="n">
-        <v>1699490.128895313</v>
+        <v>2450090</v>
       </c>
       <c r="G23" t="n">
-        <v>5034.128895312548</v>
+        <v>171480</v>
       </c>
       <c r="H23" t="n">
-        <v>0.297094105442251</v>
+        <v>7.52</v>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>2026-03-18T21:08:45</t>
+          <t>2026-03-18T21:09:27</t>
         </is>
       </c>
     </row>
@@ -2169,11 +2439,11 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>삼성생명</t>
+          <t>넥스틸</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>4</v>
+        <v>200</v>
       </c>
       <c r="D24" t="inlineStr">
         <is>
@@ -2184,17 +2454,17 @@
         <v>1</v>
       </c>
       <c r="F24" t="n">
-        <v>940000</v>
+        <v>2400000</v>
       </c>
       <c r="G24" t="n">
-        <v>107000</v>
+        <v>389000</v>
       </c>
       <c r="H24" t="n">
-        <v>12.84513805522209</v>
+        <v>19.34361014420686</v>
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>2026-03-18T21:08:45</t>
+          <t>2026-03-18T21:09:27</t>
         </is>
       </c>
     </row>
@@ -2206,11 +2476,11 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>클리블랜드 클리프스</t>
+          <t>대신증권</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>70</v>
+        <v>55</v>
       </c>
       <c r="D25" t="inlineStr">
         <is>
@@ -2221,17 +2491,17 @@
         <v>1</v>
       </c>
       <c r="F25" t="n">
-        <v>857055.5630100402</v>
+        <v>2238500</v>
       </c>
       <c r="G25" t="n">
-        <v>-158999.4369899598</v>
+        <v>528999</v>
       </c>
       <c r="H25" t="n">
-        <v>-15.64870376012714</v>
+        <v>30.94464408034859</v>
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>2026-03-18T21:08:45</t>
+          <t>2026-03-18T21:09:27</t>
         </is>
       </c>
     </row>
@@ -2243,11 +2513,11 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>비에이치아이</t>
+          <t>발레로 에너지</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="D26" t="inlineStr">
         <is>
@@ -2258,17 +2528,17 @@
         <v>1</v>
       </c>
       <c r="F26" t="n">
-        <v>844800</v>
+        <v>2138731.14071836</v>
       </c>
       <c r="G26" t="n">
-        <v>179685</v>
+        <v>74741.1407183595</v>
       </c>
       <c r="H26" t="n">
-        <v>27.01562887620938</v>
+        <v>3.621196842928478</v>
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>2026-03-18T21:08:45</t>
+          <t>2026-03-18T21:09:27</t>
         </is>
       </c>
     </row>
@@ -2280,11 +2550,11 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>하프니아</t>
+          <t>미창석유</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>80</v>
+        <v>18</v>
       </c>
       <c r="D27" t="inlineStr">
         <is>
@@ -2295,17 +2565,17 @@
         <v>1</v>
       </c>
       <c r="F27" t="n">
-        <v>821489.5606615674</v>
+        <v>2032200</v>
       </c>
       <c r="G27" t="n">
-        <v>195758.5606615674</v>
+        <v>-360000</v>
       </c>
       <c r="H27" t="n">
-        <v>31.28477902829928</v>
+        <v>-15.04890895410083</v>
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>2026-03-18T21:08:45</t>
+          <t>2026-03-18T21:09:27</t>
         </is>
       </c>
     </row>
@@ -2317,11 +2587,11 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>텍사스 퍼시픽 랜드</t>
+          <t>대창단조</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>1</v>
+        <v>300</v>
       </c>
       <c r="D28" t="inlineStr">
         <is>
@@ -2332,17 +2602,17 @@
         <v>1</v>
       </c>
       <c r="F28" t="n">
-        <v>794737.7576458007</v>
+        <v>1914000</v>
       </c>
       <c r="G28" t="n">
-        <v>16146.75764580071</v>
+        <v>-144000</v>
       </c>
       <c r="H28" t="n">
-        <v>2.073843345967358</v>
+        <v>-6.997084548104956</v>
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>2026-03-18T21:08:45</t>
+          <t>2026-03-18T21:09:27</t>
         </is>
       </c>
     </row>
@@ -2354,11 +2624,11 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>노블</t>
+          <t>동방</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>99</v>
+        <v>681</v>
       </c>
       <c r="D29" t="inlineStr">
         <is>
@@ -2369,33 +2639,33 @@
         <v>1</v>
       </c>
       <c r="F29" t="n">
-        <v>40689</v>
+        <v>1882965</v>
       </c>
       <c r="G29" t="n">
-        <v>-3866519</v>
+        <v>-88536</v>
       </c>
       <c r="H29" t="n">
-        <v>-98.95861699709869</v>
+        <v>-4.490791533963209</v>
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>2026-03-18T21:08:45</t>
+          <t>2026-03-18T21:09:27</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>2026-03-18</t>
+          <t>2026-03-17</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>페트로브라스 (ADR)</t>
+          <t>스타 벌크 캐리어스</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>480</v>
+        <v>50</v>
       </c>
       <c r="D30" t="inlineStr">
         <is>
@@ -2406,33 +2676,33 @@
         <v>1</v>
       </c>
       <c r="F30" t="n">
-        <v>14082576.9328374</v>
+        <v>1712476.648945617</v>
       </c>
       <c r="G30" t="n">
-        <v>1976027.932837404</v>
+        <v>398123.6489456175</v>
       </c>
       <c r="H30" t="n">
-        <v>16.3219752617976</v>
+        <v>30.29046602743841</v>
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>2026-03-18T14:32:42</t>
+          <t>2026-03-18T21:09:27</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-03-18</t>
+          <t>2026-03-17</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>AGNC 인베스트먼트</t>
+          <t>유나이티드헬스 그룹</t>
         </is>
       </c>
       <c r="C31" t="n">
-        <v>700</v>
+        <v>4</v>
       </c>
       <c r="D31" t="inlineStr">
         <is>
@@ -2443,33 +2713,33 @@
         <v>1</v>
       </c>
       <c r="F31" t="n">
-        <v>10822406.73782303</v>
+        <v>1699490.128895313</v>
       </c>
       <c r="G31" t="n">
-        <v>-9608.262176971883</v>
+        <v>5034.128895312548</v>
       </c>
       <c r="H31" t="n">
-        <v>-0.08870244526961865</v>
+        <v>0.297094105442251</v>
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>2026-03-18T14:32:42</t>
+          <t>2026-03-18T21:09:27</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>2026-03-18</t>
+          <t>2026-03-17</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>대한조선</t>
+          <t>케이씨</t>
         </is>
       </c>
       <c r="C32" t="n">
-        <v>100</v>
+        <v>50</v>
       </c>
       <c r="D32" t="inlineStr">
         <is>
@@ -2480,33 +2750,33 @@
         <v>1</v>
       </c>
       <c r="F32" t="n">
-        <v>9570000</v>
+        <v>1576840</v>
       </c>
       <c r="G32" t="n">
-        <v>2357000</v>
+        <v>-72660</v>
       </c>
       <c r="H32" t="n">
-        <v>32.67711077221684</v>
+        <v>-4.4</v>
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>2026-03-18T14:32:42</t>
+          <t>2026-03-18T21:09:27</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-03-18</t>
+          <t>2026-03-17</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>프론트라인</t>
+          <t>하나금융지주</t>
         </is>
       </c>
       <c r="C33" t="n">
-        <v>175</v>
+        <v>10</v>
       </c>
       <c r="D33" t="inlineStr">
         <is>
@@ -2517,33 +2787,33 @@
         <v>1</v>
       </c>
       <c r="F33" t="n">
-        <v>8440541.129673157</v>
+        <v>1107780</v>
       </c>
       <c r="G33" t="n">
-        <v>4010677.129673157</v>
+        <v>-1220</v>
       </c>
       <c r="H33" t="n">
-        <v>90.53725192631549</v>
+        <v>-0.11</v>
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>2026-03-18T14:32:42</t>
+          <t>2026-03-18T21:09:27</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>2026-03-18</t>
+          <t>2026-03-17</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>시드릴</t>
+          <t>삼성생명</t>
         </is>
       </c>
       <c r="C34" t="n">
-        <v>123</v>
+        <v>4</v>
       </c>
       <c r="D34" t="inlineStr">
         <is>
@@ -2554,33 +2824,33 @@
         <v>1</v>
       </c>
       <c r="F34" t="n">
-        <v>8090014.733635107</v>
+        <v>940000</v>
       </c>
       <c r="G34" t="n">
-        <v>1639663.733635107</v>
+        <v>107000</v>
       </c>
       <c r="H34" t="n">
-        <v>25.41975984927188</v>
+        <v>12.84513805522209</v>
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>2026-03-18T14:32:42</t>
+          <t>2026-03-18T21:09:27</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-03-18</t>
+          <t>2026-03-17</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>트랜스오션</t>
+          <t>클리블랜드 클리프스</t>
         </is>
       </c>
       <c r="C35" t="n">
-        <v>750</v>
+        <v>70</v>
       </c>
       <c r="D35" t="inlineStr">
         <is>
@@ -2591,33 +2861,33 @@
         <v>1</v>
       </c>
       <c r="F35" t="n">
-        <v>7093219.418241119</v>
+        <v>857055.5630100402</v>
       </c>
       <c r="G35" t="n">
-        <v>2965985.418241119</v>
+        <v>-158999.4369899598</v>
       </c>
       <c r="H35" t="n">
-        <v>71.86375713713153</v>
+        <v>-15.64870376012714</v>
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>2026-03-18T14:32:42</t>
+          <t>2026-03-18T21:09:27</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>2026-03-18</t>
+          <t>2026-03-17</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>세아제강</t>
+          <t>비에이치아이</t>
         </is>
       </c>
       <c r="C36" t="n">
-        <v>50</v>
+        <v>8</v>
       </c>
       <c r="D36" t="inlineStr">
         <is>
@@ -2628,33 +2898,33 @@
         <v>1</v>
       </c>
       <c r="F36" t="n">
-        <v>6915000</v>
+        <v>844800</v>
       </c>
       <c r="G36" t="n">
-        <v>605000</v>
+        <v>179685</v>
       </c>
       <c r="H36" t="n">
-        <v>9.587955625990491</v>
+        <v>27.01562887620938</v>
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>2026-03-18T14:32:42</t>
+          <t>2026-03-18T21:09:27</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2026-03-18</t>
+          <t>2026-03-17</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>센트러스 에너지</t>
+          <t>하프니아</t>
         </is>
       </c>
       <c r="C37" t="n">
-        <v>21</v>
+        <v>80</v>
       </c>
       <c r="D37" t="inlineStr">
         <is>
@@ -2665,33 +2935,33 @@
         <v>1</v>
       </c>
       <c r="F37" t="n">
-        <v>6546958.253894605</v>
+        <v>821489.5606615674</v>
       </c>
       <c r="G37" t="n">
-        <v>315739.2538946057</v>
+        <v>195758.5606615674</v>
       </c>
       <c r="H37" t="n">
-        <v>5.067054357977239</v>
+        <v>31.28477902829928</v>
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>2026-03-18T14:32:42</t>
+          <t>2026-03-18T21:09:27</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>2026-03-18</t>
+          <t>2026-03-17</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>타이드워터</t>
+          <t>텍사스 퍼시픽 랜드</t>
         </is>
       </c>
       <c r="C38" t="n">
-        <v>48</v>
+        <v>1</v>
       </c>
       <c r="D38" t="inlineStr">
         <is>
@@ -2702,33 +2972,33 @@
         <v>1</v>
       </c>
       <c r="F38" t="n">
-        <v>5456864.752692774</v>
+        <v>794737.7576458007</v>
       </c>
       <c r="G38" t="n">
-        <v>1732319.752692774</v>
+        <v>16146.75764580071</v>
       </c>
       <c r="H38" t="n">
-        <v>46.51090945854524</v>
+        <v>2.073843345967358</v>
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>2026-03-18T14:32:42</t>
+          <t>2026-03-18T21:09:27</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2026-03-18</t>
+          <t>2026-03-17</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>노브</t>
+          <t>노블</t>
         </is>
       </c>
       <c r="C39" t="n">
-        <v>185</v>
+        <v>99</v>
       </c>
       <c r="D39" t="inlineStr">
         <is>
@@ -2739,17 +3009,17 @@
         <v>1</v>
       </c>
       <c r="F39" t="n">
-        <v>5041442.310511444</v>
+        <v>40689</v>
       </c>
       <c r="G39" t="n">
-        <v>1731434.310511444</v>
+        <v>-3866519</v>
       </c>
       <c r="H39" t="n">
-        <v>52.30906724429197</v>
+        <v>-98.95861699709869</v>
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>2026-03-18T14:32:42</t>
+          <t>2026-03-18T21:09:27</t>
         </is>
       </c>
     </row>
@@ -2761,11 +3031,11 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>TIME 코리아밸류업액티브</t>
+          <t>페트로브라스 (ADR)</t>
         </is>
       </c>
       <c r="C40" t="n">
-        <v>201</v>
+        <v>480</v>
       </c>
       <c r="D40" t="inlineStr">
         <is>
@@ -2776,13 +3046,13 @@
         <v>1</v>
       </c>
       <c r="F40" t="n">
-        <v>4904400</v>
+        <v>14082576.9328374</v>
       </c>
       <c r="G40" t="n">
-        <v>180603</v>
+        <v>1976027.932837404</v>
       </c>
       <c r="H40" t="n">
-        <v>3.823259128197084</v>
+        <v>16.3219752617976</v>
       </c>
       <c r="I40" t="inlineStr">
         <is>
@@ -2798,11 +3068,11 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>오케아니스 에코 탱커스</t>
+          <t>AGNC 인베스트먼트</t>
         </is>
       </c>
       <c r="C41" t="n">
-        <v>65</v>
+        <v>700</v>
       </c>
       <c r="D41" t="inlineStr">
         <is>
@@ -2813,13 +3083,13 @@
         <v>1</v>
       </c>
       <c r="F41" t="n">
-        <v>4575098.725873504</v>
+        <v>10822406.73782303</v>
       </c>
       <c r="G41" t="n">
-        <v>2318738.725873504</v>
+        <v>-9608.262176971883</v>
       </c>
       <c r="H41" t="n">
-        <v>102.7645732894354</v>
+        <v>-0.08870244526961865</v>
       </c>
       <c r="I41" t="inlineStr">
         <is>
@@ -2835,11 +3105,11 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>삼성화재</t>
+          <t>대한조선</t>
         </is>
       </c>
       <c r="C42" t="n">
-        <v>9</v>
+        <v>100</v>
       </c>
       <c r="D42" t="inlineStr">
         <is>
@@ -2850,13 +3120,13 @@
         <v>1</v>
       </c>
       <c r="F42" t="n">
-        <v>4446000</v>
+        <v>9570000</v>
       </c>
       <c r="G42" t="n">
-        <v>-185000</v>
+        <v>2357000</v>
       </c>
       <c r="H42" t="n">
-        <v>-3.994817534009933</v>
+        <v>32.67711077221684</v>
       </c>
       <c r="I42" t="inlineStr">
         <is>
@@ -2872,11 +3142,11 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>DL이앤씨</t>
+          <t>프론트라인</t>
         </is>
       </c>
       <c r="C43" t="n">
-        <v>80</v>
+        <v>175</v>
       </c>
       <c r="D43" t="inlineStr">
         <is>
@@ -2887,13 +3157,13 @@
         <v>1</v>
       </c>
       <c r="F43" t="n">
-        <v>4128000</v>
+        <v>8440541.129673157</v>
       </c>
       <c r="G43" t="n">
-        <v>717000</v>
+        <v>4010677.129673157</v>
       </c>
       <c r="H43" t="n">
-        <v>21.02022867194371</v>
+        <v>90.53725192631549</v>
       </c>
       <c r="I43" t="inlineStr">
         <is>
@@ -2909,11 +3179,11 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>차코스 에너지 내비게이션</t>
+          <t>시드릴</t>
         </is>
       </c>
       <c r="C44" t="n">
-        <v>75</v>
+        <v>123</v>
       </c>
       <c r="D44" t="inlineStr">
         <is>
@@ -2924,13 +3194,13 @@
         <v>1</v>
       </c>
       <c r="F44" t="n">
-        <v>4007418.271141662</v>
+        <v>8090014.733635107</v>
       </c>
       <c r="G44" t="n">
-        <v>182770.2711416623</v>
+        <v>1639663.733635107</v>
       </c>
       <c r="H44" t="n">
-        <v>4.778747511971357</v>
+        <v>25.41975984927188</v>
       </c>
       <c r="I44" t="inlineStr">
         <is>
@@ -2946,11 +3216,11 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>동원개발</t>
+          <t>트랜스오션</t>
         </is>
       </c>
       <c r="C45" t="n">
-        <v>1360</v>
+        <v>750</v>
       </c>
       <c r="D45" t="inlineStr">
         <is>
@@ -2961,13 +3231,13 @@
         <v>1</v>
       </c>
       <c r="F45" t="n">
-        <v>3978000</v>
+        <v>7093219.418241119</v>
       </c>
       <c r="G45" t="n">
-        <v>240600</v>
+        <v>2965985.418241119</v>
       </c>
       <c r="H45" t="n">
-        <v>6.437630438272596</v>
+        <v>71.86375713713153</v>
       </c>
       <c r="I45" t="inlineStr">
         <is>
@@ -2983,11 +3253,11 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>HD건설기계</t>
+          <t>세아제강</t>
         </is>
       </c>
       <c r="C46" t="n">
-        <v>31</v>
+        <v>50</v>
       </c>
       <c r="D46" t="inlineStr">
         <is>
@@ -2998,13 +3268,13 @@
         <v>1</v>
       </c>
       <c r="F46" t="n">
-        <v>3955600</v>
+        <v>6915000</v>
       </c>
       <c r="G46" t="n">
-        <v>-79496</v>
+        <v>605000</v>
       </c>
       <c r="H46" t="n">
-        <v>-1.970114217852561</v>
+        <v>9.587955625990491</v>
       </c>
       <c r="I46" t="inlineStr">
         <is>
@@ -3020,11 +3290,11 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>피바디 에너지</t>
+          <t>센트러스 에너지</t>
         </is>
       </c>
       <c r="C47" t="n">
-        <v>65</v>
+        <v>21</v>
       </c>
       <c r="D47" t="inlineStr">
         <is>
@@ -3035,13 +3305,13 @@
         <v>1</v>
       </c>
       <c r="F47" t="n">
-        <v>3423839.074937592</v>
+        <v>6546958.253894605</v>
       </c>
       <c r="G47" t="n">
-        <v>1953067.074937592</v>
+        <v>315739.2538946057</v>
       </c>
       <c r="H47" t="n">
-        <v>132.7919674115085</v>
+        <v>5.067054357977239</v>
       </c>
       <c r="I47" t="inlineStr">
         <is>
@@ -3057,11 +3327,11 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>더치 브로스</t>
+          <t>타이드워터</t>
         </is>
       </c>
       <c r="C48" t="n">
-        <v>39</v>
+        <v>48</v>
       </c>
       <c r="D48" t="inlineStr">
         <is>
@@ -3072,13 +3342,13 @@
         <v>1</v>
       </c>
       <c r="F48" t="n">
-        <v>2965846.22503092</v>
+        <v>5456864.752692774</v>
       </c>
       <c r="G48" t="n">
-        <v>-224797.7749690795</v>
+        <v>1732319.752692774</v>
       </c>
       <c r="H48" t="n">
-        <v>-7.04552983564069</v>
+        <v>46.51090945854524</v>
       </c>
       <c r="I48" t="inlineStr">
         <is>
@@ -3094,11 +3364,11 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>현대제철</t>
+          <t>노브</t>
         </is>
       </c>
       <c r="C49" t="n">
-        <v>70</v>
+        <v>185</v>
       </c>
       <c r="D49" t="inlineStr">
         <is>
@@ -3109,13 +3379,13 @@
         <v>1</v>
       </c>
       <c r="F49" t="n">
-        <v>2607500</v>
+        <v>5041442.310511444</v>
       </c>
       <c r="G49" t="n">
-        <v>-200000</v>
+        <v>1731434.310511444</v>
       </c>
       <c r="H49" t="n">
-        <v>-7.123775601068566</v>
+        <v>52.30906724429197</v>
       </c>
       <c r="I49" t="inlineStr">
         <is>
@@ -3131,11 +3401,11 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>KoAct 코스닥액티브</t>
+          <t>TIME 코리아밸류업액티브</t>
         </is>
       </c>
       <c r="C50" t="n">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="D50" t="inlineStr">
         <is>
@@ -3146,13 +3416,13 @@
         <v>1</v>
       </c>
       <c r="F50" t="n">
-        <v>2598000</v>
+        <v>4904400</v>
       </c>
       <c r="G50" t="n">
-        <v>-104000</v>
+        <v>180603</v>
       </c>
       <c r="H50" t="n">
-        <v>-3.84900074019245</v>
+        <v>3.823259128197084</v>
       </c>
       <c r="I50" t="inlineStr">
         <is>
@@ -3168,11 +3438,11 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>휴스틸</t>
+          <t>오케아니스 에코 탱커스</t>
         </is>
       </c>
       <c r="C51" t="n">
-        <v>500</v>
+        <v>65</v>
       </c>
       <c r="D51" t="inlineStr">
         <is>
@@ -3183,13 +3453,13 @@
         <v>1</v>
       </c>
       <c r="F51" t="n">
-        <v>2560000</v>
+        <v>4575098.725873504</v>
       </c>
       <c r="G51" t="n">
-        <v>281390</v>
+        <v>2318738.725873504</v>
       </c>
       <c r="H51" t="n">
-        <v>12.34919534277476</v>
+        <v>102.7645732894354</v>
       </c>
       <c r="I51" t="inlineStr">
         <is>
@@ -3205,11 +3475,11 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>넥스틸</t>
+          <t>삼성화재</t>
         </is>
       </c>
       <c r="C52" t="n">
-        <v>200</v>
+        <v>9</v>
       </c>
       <c r="D52" t="inlineStr">
         <is>
@@ -3220,13 +3490,13 @@
         <v>1</v>
       </c>
       <c r="F52" t="n">
-        <v>2400000</v>
+        <v>4446000</v>
       </c>
       <c r="G52" t="n">
-        <v>389000</v>
+        <v>-185000</v>
       </c>
       <c r="H52" t="n">
-        <v>19.34361014420686</v>
+        <v>-3.994817534009933</v>
       </c>
       <c r="I52" t="inlineStr">
         <is>
@@ -3242,11 +3512,11 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>대신증권</t>
+          <t>DL이앤씨</t>
         </is>
       </c>
       <c r="C53" t="n">
-        <v>55</v>
+        <v>80</v>
       </c>
       <c r="D53" t="inlineStr">
         <is>
@@ -3257,13 +3527,13 @@
         <v>1</v>
       </c>
       <c r="F53" t="n">
-        <v>2238500</v>
+        <v>4128000</v>
       </c>
       <c r="G53" t="n">
-        <v>528999</v>
+        <v>717000</v>
       </c>
       <c r="H53" t="n">
-        <v>30.94464408034859</v>
+        <v>21.02022867194371</v>
       </c>
       <c r="I53" t="inlineStr">
         <is>
@@ -3279,11 +3549,11 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>발레로 에너지</t>
+          <t>차코스 에너지 내비게이션</t>
         </is>
       </c>
       <c r="C54" t="n">
-        <v>6</v>
+        <v>75</v>
       </c>
       <c r="D54" t="inlineStr">
         <is>
@@ -3294,13 +3564,13 @@
         <v>1</v>
       </c>
       <c r="F54" t="n">
-        <v>2138731.14071836</v>
+        <v>4007418.271141662</v>
       </c>
       <c r="G54" t="n">
-        <v>74741.1407183595</v>
+        <v>182770.2711416623</v>
       </c>
       <c r="H54" t="n">
-        <v>3.621196842928478</v>
+        <v>4.778747511971357</v>
       </c>
       <c r="I54" t="inlineStr">
         <is>
@@ -3316,11 +3586,11 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>미창석유</t>
+          <t>동원개발</t>
         </is>
       </c>
       <c r="C55" t="n">
-        <v>18</v>
+        <v>1360</v>
       </c>
       <c r="D55" t="inlineStr">
         <is>
@@ -3331,13 +3601,13 @@
         <v>1</v>
       </c>
       <c r="F55" t="n">
-        <v>2032200</v>
+        <v>3978000</v>
       </c>
       <c r="G55" t="n">
-        <v>-360000</v>
+        <v>240600</v>
       </c>
       <c r="H55" t="n">
-        <v>-15.04890895410083</v>
+        <v>6.437630438272596</v>
       </c>
       <c r="I55" t="inlineStr">
         <is>
@@ -3353,11 +3623,11 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>대창단조</t>
+          <t>HD건설기계</t>
         </is>
       </c>
       <c r="C56" t="n">
-        <v>300</v>
+        <v>31</v>
       </c>
       <c r="D56" t="inlineStr">
         <is>
@@ -3368,13 +3638,13 @@
         <v>1</v>
       </c>
       <c r="F56" t="n">
-        <v>1914000</v>
+        <v>3955600</v>
       </c>
       <c r="G56" t="n">
-        <v>-144000</v>
+        <v>-79496</v>
       </c>
       <c r="H56" t="n">
-        <v>-6.997084548104956</v>
+        <v>-1.970114217852561</v>
       </c>
       <c r="I56" t="inlineStr">
         <is>
@@ -3390,11 +3660,11 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>동방</t>
+          <t>피바디 에너지</t>
         </is>
       </c>
       <c r="C57" t="n">
-        <v>681</v>
+        <v>65</v>
       </c>
       <c r="D57" t="inlineStr">
         <is>
@@ -3405,13 +3675,13 @@
         <v>1</v>
       </c>
       <c r="F57" t="n">
-        <v>1882965</v>
+        <v>3423839.074937592</v>
       </c>
       <c r="G57" t="n">
-        <v>-88536</v>
+        <v>1953067.074937592</v>
       </c>
       <c r="H57" t="n">
-        <v>-4.490791533963209</v>
+        <v>132.7919674115085</v>
       </c>
       <c r="I57" t="inlineStr">
         <is>
@@ -3427,11 +3697,11 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>하나금융지주</t>
+          <t>더치 브로스</t>
         </is>
       </c>
       <c r="C58" t="n">
-        <v>15</v>
+        <v>39</v>
       </c>
       <c r="D58" t="inlineStr">
         <is>
@@ -3442,13 +3712,13 @@
         <v>1</v>
       </c>
       <c r="F58" t="n">
-        <v>1717500</v>
+        <v>2965846.22503092</v>
       </c>
       <c r="G58" t="n">
-        <v>35000</v>
+        <v>-224797.7749690795</v>
       </c>
       <c r="H58" t="n">
-        <v>2.080237741456166</v>
+        <v>-7.04552983564069</v>
       </c>
       <c r="I58" t="inlineStr">
         <is>
@@ -3464,11 +3734,11 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>스타 벌크 캐리어스</t>
+          <t>현대제철</t>
         </is>
       </c>
       <c r="C59" t="n">
-        <v>50</v>
+        <v>70</v>
       </c>
       <c r="D59" t="inlineStr">
         <is>
@@ -3479,13 +3749,13 @@
         <v>1</v>
       </c>
       <c r="F59" t="n">
-        <v>1712476.648945617</v>
+        <v>2607500</v>
       </c>
       <c r="G59" t="n">
-        <v>398123.648945618</v>
+        <v>-200000</v>
       </c>
       <c r="H59" t="n">
-        <v>30.29046602743845</v>
+        <v>-7.123775601068566</v>
       </c>
       <c r="I59" t="inlineStr">
         <is>
@@ -3501,11 +3771,11 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>유나이티드헬스 그룹</t>
+          <t>KoAct 코스닥액티브</t>
         </is>
       </c>
       <c r="C60" t="n">
-        <v>4</v>
+        <v>200</v>
       </c>
       <c r="D60" t="inlineStr">
         <is>
@@ -3516,13 +3786,13 @@
         <v>1</v>
       </c>
       <c r="F60" t="n">
-        <v>1699490.128895313</v>
+        <v>2598000</v>
       </c>
       <c r="G60" t="n">
-        <v>5034.128895312548</v>
+        <v>-104000</v>
       </c>
       <c r="H60" t="n">
-        <v>0.297094105442251</v>
+        <v>-3.84900074019245</v>
       </c>
       <c r="I60" t="inlineStr">
         <is>
@@ -3538,11 +3808,11 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>케이씨</t>
+          <t>휴스틸</t>
         </is>
       </c>
       <c r="C61" t="n">
-        <v>50</v>
+        <v>500</v>
       </c>
       <c r="D61" t="inlineStr">
         <is>
@@ -3553,13 +3823,13 @@
         <v>1</v>
       </c>
       <c r="F61" t="n">
-        <v>1640000</v>
+        <v>2560000</v>
       </c>
       <c r="G61" t="n">
-        <v>-9500.000000000698</v>
+        <v>281390</v>
       </c>
       <c r="H61" t="n">
-        <v>-0.5759321006365986</v>
+        <v>12.34919534277476</v>
       </c>
       <c r="I61" t="inlineStr">
         <is>
@@ -3575,11 +3845,11 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>삼성생명</t>
+          <t>넥스틸</t>
         </is>
       </c>
       <c r="C62" t="n">
-        <v>4</v>
+        <v>200</v>
       </c>
       <c r="D62" t="inlineStr">
         <is>
@@ -3590,13 +3860,13 @@
         <v>1</v>
       </c>
       <c r="F62" t="n">
-        <v>940000</v>
+        <v>2400000</v>
       </c>
       <c r="G62" t="n">
-        <v>107000</v>
+        <v>389000</v>
       </c>
       <c r="H62" t="n">
-        <v>12.84513805522209</v>
+        <v>19.34361014420686</v>
       </c>
       <c r="I62" t="inlineStr">
         <is>
@@ -3612,11 +3882,11 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>클리블랜드 클리프스</t>
+          <t>대신증권</t>
         </is>
       </c>
       <c r="C63" t="n">
-        <v>70</v>
+        <v>55</v>
       </c>
       <c r="D63" t="inlineStr">
         <is>
@@ -3627,13 +3897,13 @@
         <v>1</v>
       </c>
       <c r="F63" t="n">
-        <v>857055.5630100402</v>
+        <v>2238500</v>
       </c>
       <c r="G63" t="n">
-        <v>-158999.4369899598</v>
+        <v>528999</v>
       </c>
       <c r="H63" t="n">
-        <v>-15.64870376012714</v>
+        <v>30.94464408034859</v>
       </c>
       <c r="I63" t="inlineStr">
         <is>
@@ -3649,11 +3919,11 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>비에이치아이</t>
+          <t>발레로 에너지</t>
         </is>
       </c>
       <c r="C64" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="D64" t="inlineStr">
         <is>
@@ -3664,13 +3934,13 @@
         <v>1</v>
       </c>
       <c r="F64" t="n">
-        <v>844800</v>
+        <v>2138731.14071836</v>
       </c>
       <c r="G64" t="n">
-        <v>179685</v>
+        <v>74741.1407183595</v>
       </c>
       <c r="H64" t="n">
-        <v>27.01562887620938</v>
+        <v>3.621196842928478</v>
       </c>
       <c r="I64" t="inlineStr">
         <is>
@@ -3686,11 +3956,11 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>하프니아</t>
+          <t>미창석유</t>
         </is>
       </c>
       <c r="C65" t="n">
-        <v>80</v>
+        <v>18</v>
       </c>
       <c r="D65" t="inlineStr">
         <is>
@@ -3701,13 +3971,13 @@
         <v>1</v>
       </c>
       <c r="F65" t="n">
-        <v>821489.5606615674</v>
+        <v>2032200</v>
       </c>
       <c r="G65" t="n">
-        <v>195758.5606615674</v>
+        <v>-360000</v>
       </c>
       <c r="H65" t="n">
-        <v>31.28477902829928</v>
+        <v>-15.04890895410083</v>
       </c>
       <c r="I65" t="inlineStr">
         <is>
@@ -3723,11 +3993,11 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>텍사스 퍼시픽 랜드</t>
+          <t>대창단조</t>
         </is>
       </c>
       <c r="C66" t="n">
-        <v>1</v>
+        <v>300</v>
       </c>
       <c r="D66" t="inlineStr">
         <is>
@@ -3738,13 +4008,13 @@
         <v>1</v>
       </c>
       <c r="F66" t="n">
-        <v>794737.7576458007</v>
+        <v>1914000</v>
       </c>
       <c r="G66" t="n">
-        <v>16146.75764580071</v>
+        <v>-144000</v>
       </c>
       <c r="H66" t="n">
-        <v>2.073843345967358</v>
+        <v>-6.997084548104956</v>
       </c>
       <c r="I66" t="inlineStr">
         <is>
@@ -3760,30 +4030,400 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
+          <t>동방</t>
+        </is>
+      </c>
+      <c r="C67" t="n">
+        <v>681</v>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E67" t="n">
+        <v>1</v>
+      </c>
+      <c r="F67" t="n">
+        <v>1882965</v>
+      </c>
+      <c r="G67" t="n">
+        <v>-88536</v>
+      </c>
+      <c r="H67" t="n">
+        <v>-4.490791533963209</v>
+      </c>
+      <c r="I67" t="inlineStr">
+        <is>
+          <t>2026-03-18T14:32:42</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>2026-03-18</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>하나금융지주</t>
+        </is>
+      </c>
+      <c r="C68" t="n">
+        <v>15</v>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E68" t="n">
+        <v>1</v>
+      </c>
+      <c r="F68" t="n">
+        <v>1717500</v>
+      </c>
+      <c r="G68" t="n">
+        <v>35000</v>
+      </c>
+      <c r="H68" t="n">
+        <v>2.080237741456166</v>
+      </c>
+      <c r="I68" t="inlineStr">
+        <is>
+          <t>2026-03-18T14:32:42</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>2026-03-18</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>스타 벌크 캐리어스</t>
+        </is>
+      </c>
+      <c r="C69" t="n">
+        <v>50</v>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E69" t="n">
+        <v>1</v>
+      </c>
+      <c r="F69" t="n">
+        <v>1712476.648945617</v>
+      </c>
+      <c r="G69" t="n">
+        <v>398123.648945618</v>
+      </c>
+      <c r="H69" t="n">
+        <v>30.29046602743845</v>
+      </c>
+      <c r="I69" t="inlineStr">
+        <is>
+          <t>2026-03-18T14:32:42</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>2026-03-18</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>유나이티드헬스 그룹</t>
+        </is>
+      </c>
+      <c r="C70" t="n">
+        <v>4</v>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E70" t="n">
+        <v>1</v>
+      </c>
+      <c r="F70" t="n">
+        <v>1699490.128895313</v>
+      </c>
+      <c r="G70" t="n">
+        <v>5034.128895312548</v>
+      </c>
+      <c r="H70" t="n">
+        <v>0.297094105442251</v>
+      </c>
+      <c r="I70" t="inlineStr">
+        <is>
+          <t>2026-03-18T14:32:42</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>2026-03-18</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>케이씨</t>
+        </is>
+      </c>
+      <c r="C71" t="n">
+        <v>50</v>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E71" t="n">
+        <v>1</v>
+      </c>
+      <c r="F71" t="n">
+        <v>1640000</v>
+      </c>
+      <c r="G71" t="n">
+        <v>-9500.000000000698</v>
+      </c>
+      <c r="H71" t="n">
+        <v>-0.5759321006365986</v>
+      </c>
+      <c r="I71" t="inlineStr">
+        <is>
+          <t>2026-03-18T14:32:42</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>2026-03-18</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>삼성생명</t>
+        </is>
+      </c>
+      <c r="C72" t="n">
+        <v>4</v>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E72" t="n">
+        <v>1</v>
+      </c>
+      <c r="F72" t="n">
+        <v>940000</v>
+      </c>
+      <c r="G72" t="n">
+        <v>107000</v>
+      </c>
+      <c r="H72" t="n">
+        <v>12.84513805522209</v>
+      </c>
+      <c r="I72" t="inlineStr">
+        <is>
+          <t>2026-03-18T14:32:42</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>2026-03-18</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>클리블랜드 클리프스</t>
+        </is>
+      </c>
+      <c r="C73" t="n">
+        <v>70</v>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E73" t="n">
+        <v>1</v>
+      </c>
+      <c r="F73" t="n">
+        <v>857055.5630100402</v>
+      </c>
+      <c r="G73" t="n">
+        <v>-158999.4369899598</v>
+      </c>
+      <c r="H73" t="n">
+        <v>-15.64870376012714</v>
+      </c>
+      <c r="I73" t="inlineStr">
+        <is>
+          <t>2026-03-18T14:32:42</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>2026-03-18</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>비에이치아이</t>
+        </is>
+      </c>
+      <c r="C74" t="n">
+        <v>8</v>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E74" t="n">
+        <v>1</v>
+      </c>
+      <c r="F74" t="n">
+        <v>844800</v>
+      </c>
+      <c r="G74" t="n">
+        <v>179685</v>
+      </c>
+      <c r="H74" t="n">
+        <v>27.01562887620938</v>
+      </c>
+      <c r="I74" t="inlineStr">
+        <is>
+          <t>2026-03-18T14:32:42</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>2026-03-18</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>하프니아</t>
+        </is>
+      </c>
+      <c r="C75" t="n">
+        <v>80</v>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E75" t="n">
+        <v>1</v>
+      </c>
+      <c r="F75" t="n">
+        <v>821489.5606615674</v>
+      </c>
+      <c r="G75" t="n">
+        <v>195758.5606615674</v>
+      </c>
+      <c r="H75" t="n">
+        <v>31.28477902829928</v>
+      </c>
+      <c r="I75" t="inlineStr">
+        <is>
+          <t>2026-03-18T14:32:42</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>2026-03-18</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>텍사스 퍼시픽 랜드</t>
+        </is>
+      </c>
+      <c r="C76" t="n">
+        <v>1</v>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E76" t="n">
+        <v>1</v>
+      </c>
+      <c r="F76" t="n">
+        <v>794737.7576458007</v>
+      </c>
+      <c r="G76" t="n">
+        <v>16146.75764580071</v>
+      </c>
+      <c r="H76" t="n">
+        <v>2.073843345967358</v>
+      </c>
+      <c r="I76" t="inlineStr">
+        <is>
+          <t>2026-03-18T14:32:42</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>2026-03-18</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
           <t>노블</t>
         </is>
       </c>
-      <c r="C67" t="n">
+      <c r="C77" t="n">
         <v>99</v>
       </c>
-      <c r="D67" t="inlineStr">
-        <is>
-          <t>KRW</t>
-        </is>
-      </c>
-      <c r="E67" t="n">
-        <v>1</v>
-      </c>
-      <c r="F67" t="n">
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E77" t="n">
+        <v>1</v>
+      </c>
+      <c r="F77" t="n">
         <v>40689</v>
       </c>
-      <c r="G67" t="n">
+      <c r="G77" t="n">
         <v>-3866519</v>
       </c>
-      <c r="H67" t="n">
+      <c r="H77" t="n">
         <v>-98.95861699709869</v>
       </c>
-      <c r="I67" t="inlineStr">
+      <c r="I77" t="inlineStr">
         <is>
           <t>2026-03-18T14:32:42</t>
         </is>
@@ -3849,7 +4489,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>2026-03-18T21:08:45</t>
+          <t>2026-03-18T21:09:27</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: portfolio snapshot 2026-03-17 (2026-03-18T21:09:29)
</commit_message>
<xml_diff>
--- a/portfolio_auto.xlsx
+++ b/portfolio_auto.xlsx
@@ -1242,13 +1242,13 @@
         <v>1</v>
       </c>
       <c r="E30" t="n">
-        <v>3335815</v>
+        <v>3458000</v>
       </c>
       <c r="F30" t="n">
-        <v>-295185</v>
+        <v>-173000</v>
       </c>
       <c r="G30" t="n">
-        <v>-8.119999999999999</v>
+        <v>-4.76452767832553</v>
       </c>
     </row>
     <row r="31">
@@ -1269,13 +1269,13 @@
         <v>1</v>
       </c>
       <c r="E31" t="n">
-        <v>6896180</v>
+        <v>6915000</v>
       </c>
       <c r="F31" t="n">
-        <v>586180</v>
+        <v>605000</v>
       </c>
       <c r="G31" t="n">
-        <v>9.279999999999999</v>
+        <v>9.587955625990491</v>
       </c>
     </row>
     <row r="32">
@@ -1296,13 +1296,13 @@
         <v>1</v>
       </c>
       <c r="E32" t="n">
-        <v>1576840</v>
+        <v>1640000</v>
       </c>
       <c r="F32" t="n">
-        <v>-72660</v>
+        <v>-9500</v>
       </c>
       <c r="G32" t="n">
-        <v>-4.4</v>
+        <v>-0.5759321006365565</v>
       </c>
     </row>
     <row r="33">
@@ -1323,13 +1323,13 @@
         <v>1</v>
       </c>
       <c r="E33" t="n">
-        <v>1107780</v>
+        <v>1145000</v>
       </c>
       <c r="F33" t="n">
-        <v>-1220</v>
+        <v>36000</v>
       </c>
       <c r="G33" t="n">
-        <v>-0.11</v>
+        <v>3.246167718665464</v>
       </c>
     </row>
     <row r="34">
@@ -1350,13 +1350,13 @@
         <v>1</v>
       </c>
       <c r="E34" t="n">
-        <v>2494002</v>
+        <v>2607500</v>
       </c>
       <c r="F34" t="n">
-        <v>-313498</v>
+        <v>-200000</v>
       </c>
       <c r="G34" t="n">
-        <v>-11.16</v>
+        <v>-7.123775601068566</v>
       </c>
     </row>
     <row r="35">
@@ -1377,13 +1377,13 @@
         <v>1</v>
       </c>
       <c r="E35" t="n">
-        <v>2450090</v>
+        <v>2560000</v>
       </c>
       <c r="F35" t="n">
-        <v>171480</v>
+        <v>281390</v>
       </c>
       <c r="G35" t="n">
-        <v>7.52</v>
+        <v>12.34919534277476</v>
       </c>
     </row>
     <row r="36">
@@ -1404,13 +1404,13 @@
         <v>1</v>
       </c>
       <c r="E36" t="n">
-        <v>3792400</v>
+        <v>4128000</v>
       </c>
       <c r="F36" t="n">
-        <v>381400</v>
+        <v>717000</v>
       </c>
       <c r="G36" t="n">
-        <v>11.18</v>
+        <v>21.02022867194371</v>
       </c>
     </row>
     <row r="37">
@@ -1431,13 +1431,13 @@
         <v>1</v>
       </c>
       <c r="E37" t="n">
-        <v>3885810</v>
+        <v>3955600</v>
       </c>
       <c r="F37" t="n">
-        <v>-149286</v>
+        <v>-79496</v>
       </c>
       <c r="G37" t="n">
-        <v>-3.69</v>
+        <v>-1.970114217852561</v>
       </c>
     </row>
     <row r="38">
@@ -1458,13 +1458,13 @@
         <v>1</v>
       </c>
       <c r="E38" t="n">
-        <v>2580000</v>
+        <v>2598000</v>
       </c>
       <c r="F38" t="n">
-        <v>-122000</v>
+        <v>-104000</v>
       </c>
       <c r="G38" t="n">
-        <v>-4.51</v>
+        <v>-3.84900074019245</v>
       </c>
     </row>
     <row r="39">
@@ -1485,13 +1485,13 @@
         <v>1</v>
       </c>
       <c r="E39" t="n">
-        <v>4656165</v>
+        <v>4904400</v>
       </c>
       <c r="F39" t="n">
-        <v>-67632</v>
+        <v>180603</v>
       </c>
       <c r="G39" t="n">
-        <v>-1.43</v>
+        <v>3.823259128197084</v>
       </c>
     </row>
   </sheetData>
@@ -1549,7 +1549,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2026-03-18T21:09:27</t>
+          <t>2026-03-18T21:09:28</t>
         </is>
       </c>
       <c r="E2" t="n">
@@ -1650,7 +1650,7 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>2026-03-18T21:09:27</t>
+          <t>2026-03-18T21:09:28</t>
         </is>
       </c>
     </row>
@@ -1687,7 +1687,7 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>2026-03-18T21:09:27</t>
+          <t>2026-03-18T21:09:28</t>
         </is>
       </c>
     </row>
@@ -1724,7 +1724,7 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>2026-03-18T21:09:27</t>
+          <t>2026-03-18T21:09:28</t>
         </is>
       </c>
     </row>
@@ -1761,7 +1761,7 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>2026-03-18T21:09:27</t>
+          <t>2026-03-18T21:09:28</t>
         </is>
       </c>
     </row>
@@ -1798,7 +1798,7 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>2026-03-18T21:09:27</t>
+          <t>2026-03-18T21:09:28</t>
         </is>
       </c>
     </row>
@@ -1835,7 +1835,7 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>2026-03-18T21:09:27</t>
+          <t>2026-03-18T21:09:28</t>
         </is>
       </c>
     </row>
@@ -1862,17 +1862,17 @@
         <v>1</v>
       </c>
       <c r="F8" t="n">
-        <v>6896180</v>
+        <v>6915000</v>
       </c>
       <c r="G8" t="n">
-        <v>586180</v>
+        <v>605000</v>
       </c>
       <c r="H8" t="n">
-        <v>9.279999999999999</v>
+        <v>9.587955625990491</v>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>2026-03-18T21:09:27</t>
+          <t>2026-03-18T21:09:28</t>
         </is>
       </c>
     </row>
@@ -1909,7 +1909,7 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>2026-03-18T21:09:27</t>
+          <t>2026-03-18T21:09:28</t>
         </is>
       </c>
     </row>
@@ -1946,7 +1946,7 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>2026-03-18T21:09:27</t>
+          <t>2026-03-18T21:09:28</t>
         </is>
       </c>
     </row>
@@ -1983,7 +1983,7 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>2026-03-18T21:09:27</t>
+          <t>2026-03-18T21:09:28</t>
         </is>
       </c>
     </row>
@@ -2010,17 +2010,17 @@
         <v>1</v>
       </c>
       <c r="F12" t="n">
-        <v>4656165</v>
+        <v>4904400</v>
       </c>
       <c r="G12" t="n">
-        <v>-67632</v>
+        <v>180603</v>
       </c>
       <c r="H12" t="n">
-        <v>-1.43</v>
+        <v>3.823259128197084</v>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>2026-03-18T21:09:27</t>
+          <t>2026-03-18T21:09:28</t>
         </is>
       </c>
     </row>
@@ -2057,7 +2057,7 @@
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>2026-03-18T21:09:27</t>
+          <t>2026-03-18T21:09:28</t>
         </is>
       </c>
     </row>
@@ -2069,11 +2069,11 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>차코스 에너지 내비게이션</t>
+          <t>DL이앤씨</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>75</v>
+        <v>80</v>
       </c>
       <c r="D14" t="inlineStr">
         <is>
@@ -2084,17 +2084,17 @@
         <v>1</v>
       </c>
       <c r="F14" t="n">
-        <v>4007418.271141662</v>
+        <v>4128000</v>
       </c>
       <c r="G14" t="n">
-        <v>182770.2711416623</v>
+        <v>717000</v>
       </c>
       <c r="H14" t="n">
-        <v>4.778747511971357</v>
+        <v>21.02022867194371</v>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>2026-03-18T21:09:27</t>
+          <t>2026-03-18T21:09:28</t>
         </is>
       </c>
     </row>
@@ -2106,11 +2106,11 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>동원개발</t>
+          <t>차코스 에너지 내비게이션</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>1360</v>
+        <v>75</v>
       </c>
       <c r="D15" t="inlineStr">
         <is>
@@ -2121,17 +2121,17 @@
         <v>1</v>
       </c>
       <c r="F15" t="n">
-        <v>3978000</v>
+        <v>4007418.271141662</v>
       </c>
       <c r="G15" t="n">
-        <v>240600</v>
+        <v>182770.2711416623</v>
       </c>
       <c r="H15" t="n">
-        <v>6.437630438272596</v>
+        <v>4.778747511971357</v>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>2026-03-18T21:09:27</t>
+          <t>2026-03-18T21:09:28</t>
         </is>
       </c>
     </row>
@@ -2143,11 +2143,11 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>HD건설기계</t>
+          <t>동원개발</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>31</v>
+        <v>1360</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
@@ -2158,17 +2158,17 @@
         <v>1</v>
       </c>
       <c r="F16" t="n">
-        <v>3885810</v>
+        <v>3978000</v>
       </c>
       <c r="G16" t="n">
-        <v>-149286</v>
+        <v>240600</v>
       </c>
       <c r="H16" t="n">
-        <v>-3.69</v>
+        <v>6.437630438272596</v>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>2026-03-18T21:09:27</t>
+          <t>2026-03-18T21:09:28</t>
         </is>
       </c>
     </row>
@@ -2180,11 +2180,11 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>DL이앤씨</t>
+          <t>HD건설기계</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>80</v>
+        <v>31</v>
       </c>
       <c r="D17" t="inlineStr">
         <is>
@@ -2195,17 +2195,17 @@
         <v>1</v>
       </c>
       <c r="F17" t="n">
-        <v>3792400</v>
+        <v>3955600</v>
       </c>
       <c r="G17" t="n">
-        <v>381400</v>
+        <v>-79496</v>
       </c>
       <c r="H17" t="n">
-        <v>11.18</v>
+        <v>-1.970114217852561</v>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>2026-03-18T21:09:27</t>
+          <t>2026-03-18T21:09:28</t>
         </is>
       </c>
     </row>
@@ -2217,11 +2217,11 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>피바디 에너지</t>
+          <t>삼성화재</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>65</v>
+        <v>7</v>
       </c>
       <c r="D18" t="inlineStr">
         <is>
@@ -2232,17 +2232,17 @@
         <v>1</v>
       </c>
       <c r="F18" t="n">
-        <v>3423839.074937592</v>
+        <v>3458000</v>
       </c>
       <c r="G18" t="n">
-        <v>1953067.074937592</v>
+        <v>-173000</v>
       </c>
       <c r="H18" t="n">
-        <v>132.7919674115085</v>
+        <v>-4.76452767832553</v>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>2026-03-18T21:09:27</t>
+          <t>2026-03-18T21:09:28</t>
         </is>
       </c>
     </row>
@@ -2254,11 +2254,11 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>삼성화재</t>
+          <t>피바디 에너지</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>7</v>
+        <v>65</v>
       </c>
       <c r="D19" t="inlineStr">
         <is>
@@ -2269,17 +2269,17 @@
         <v>1</v>
       </c>
       <c r="F19" t="n">
-        <v>3335815</v>
+        <v>3423839.074937592</v>
       </c>
       <c r="G19" t="n">
-        <v>-295185</v>
+        <v>1953067.074937592</v>
       </c>
       <c r="H19" t="n">
-        <v>-8.119999999999999</v>
+        <v>132.7919674115085</v>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>2026-03-18T21:09:27</t>
+          <t>2026-03-18T21:09:28</t>
         </is>
       </c>
     </row>
@@ -2316,7 +2316,7 @@
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>2026-03-18T21:09:27</t>
+          <t>2026-03-18T21:09:28</t>
         </is>
       </c>
     </row>
@@ -2328,11 +2328,11 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>KoAct 코스닥액티브</t>
+          <t>현대제철</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>200</v>
+        <v>70</v>
       </c>
       <c r="D21" t="inlineStr">
         <is>
@@ -2343,17 +2343,17 @@
         <v>1</v>
       </c>
       <c r="F21" t="n">
-        <v>2580000</v>
+        <v>2607500</v>
       </c>
       <c r="G21" t="n">
-        <v>-122000</v>
+        <v>-200000</v>
       </c>
       <c r="H21" t="n">
-        <v>-4.51</v>
+        <v>-7.123775601068566</v>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>2026-03-18T21:09:27</t>
+          <t>2026-03-18T21:09:28</t>
         </is>
       </c>
     </row>
@@ -2365,11 +2365,11 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>현대제철</t>
+          <t>KoAct 코스닥액티브</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>70</v>
+        <v>200</v>
       </c>
       <c r="D22" t="inlineStr">
         <is>
@@ -2380,17 +2380,17 @@
         <v>1</v>
       </c>
       <c r="F22" t="n">
-        <v>2494002</v>
+        <v>2598000</v>
       </c>
       <c r="G22" t="n">
-        <v>-313498</v>
+        <v>-104000</v>
       </c>
       <c r="H22" t="n">
-        <v>-11.16</v>
+        <v>-3.84900074019245</v>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>2026-03-18T21:09:27</t>
+          <t>2026-03-18T21:09:28</t>
         </is>
       </c>
     </row>
@@ -2417,17 +2417,17 @@
         <v>1</v>
       </c>
       <c r="F23" t="n">
-        <v>2450090</v>
+        <v>2560000</v>
       </c>
       <c r="G23" t="n">
-        <v>171480</v>
+        <v>281390</v>
       </c>
       <c r="H23" t="n">
-        <v>7.52</v>
+        <v>12.34919534277476</v>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>2026-03-18T21:09:27</t>
+          <t>2026-03-18T21:09:28</t>
         </is>
       </c>
     </row>
@@ -2464,7 +2464,7 @@
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>2026-03-18T21:09:27</t>
+          <t>2026-03-18T21:09:28</t>
         </is>
       </c>
     </row>
@@ -2501,7 +2501,7 @@
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>2026-03-18T21:09:27</t>
+          <t>2026-03-18T21:09:28</t>
         </is>
       </c>
     </row>
@@ -2538,7 +2538,7 @@
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>2026-03-18T21:09:27</t>
+          <t>2026-03-18T21:09:28</t>
         </is>
       </c>
     </row>
@@ -2575,7 +2575,7 @@
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>2026-03-18T21:09:27</t>
+          <t>2026-03-18T21:09:28</t>
         </is>
       </c>
     </row>
@@ -2612,7 +2612,7 @@
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>2026-03-18T21:09:27</t>
+          <t>2026-03-18T21:09:28</t>
         </is>
       </c>
     </row>
@@ -2649,7 +2649,7 @@
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>2026-03-18T21:09:27</t>
+          <t>2026-03-18T21:09:28</t>
         </is>
       </c>
     </row>
@@ -2686,7 +2686,7 @@
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>2026-03-18T21:09:27</t>
+          <t>2026-03-18T21:09:28</t>
         </is>
       </c>
     </row>
@@ -2723,7 +2723,7 @@
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>2026-03-18T21:09:27</t>
+          <t>2026-03-18T21:09:28</t>
         </is>
       </c>
     </row>
@@ -2750,17 +2750,17 @@
         <v>1</v>
       </c>
       <c r="F32" t="n">
-        <v>1576840</v>
+        <v>1640000</v>
       </c>
       <c r="G32" t="n">
-        <v>-72660</v>
+        <v>-9500</v>
       </c>
       <c r="H32" t="n">
-        <v>-4.4</v>
+        <v>-0.5759321006365565</v>
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>2026-03-18T21:09:27</t>
+          <t>2026-03-18T21:09:28</t>
         </is>
       </c>
     </row>
@@ -2787,17 +2787,17 @@
         <v>1</v>
       </c>
       <c r="F33" t="n">
-        <v>1107780</v>
+        <v>1145000</v>
       </c>
       <c r="G33" t="n">
-        <v>-1220</v>
+        <v>36000</v>
       </c>
       <c r="H33" t="n">
-        <v>-0.11</v>
+        <v>3.246167718665464</v>
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>2026-03-18T21:09:27</t>
+          <t>2026-03-18T21:09:28</t>
         </is>
       </c>
     </row>
@@ -2834,7 +2834,7 @@
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>2026-03-18T21:09:27</t>
+          <t>2026-03-18T21:09:28</t>
         </is>
       </c>
     </row>
@@ -2871,7 +2871,7 @@
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>2026-03-18T21:09:27</t>
+          <t>2026-03-18T21:09:28</t>
         </is>
       </c>
     </row>
@@ -2908,7 +2908,7 @@
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>2026-03-18T21:09:27</t>
+          <t>2026-03-18T21:09:28</t>
         </is>
       </c>
     </row>
@@ -2945,7 +2945,7 @@
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>2026-03-18T21:09:27</t>
+          <t>2026-03-18T21:09:28</t>
         </is>
       </c>
     </row>
@@ -2982,7 +2982,7 @@
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>2026-03-18T21:09:27</t>
+          <t>2026-03-18T21:09:28</t>
         </is>
       </c>
     </row>
@@ -3019,7 +3019,7 @@
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>2026-03-18T21:09:27</t>
+          <t>2026-03-18T21:09:28</t>
         </is>
       </c>
     </row>
@@ -4489,7 +4489,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>2026-03-18T21:09:27</t>
+          <t>2026-03-18T21:09:28</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: portfolio snapshot 2026-03-18 (2026-03-18T21:13:42)
</commit_message>
<xml_diff>
--- a/portfolio_auto.xlsx
+++ b/portfolio_auto.xlsx
@@ -471,11 +471,11 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>노브</t>
+          <t>페트로브라스 (ADR)</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>185</v>
+        <v>480</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
@@ -486,23 +486,23 @@
         <v>1</v>
       </c>
       <c r="E2" t="n">
-        <v>5041442.310511444</v>
+        <v>14100407.22082324</v>
       </c>
       <c r="F2" t="n">
-        <v>1731434.310511444</v>
+        <v>1993858.220823243</v>
       </c>
       <c r="G2" t="n">
-        <v>52.30906724429197</v>
+        <v>16.46925330102941</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>노블</t>
+          <t>AGNC 인베스트먼트</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>99</v>
+        <v>700</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
@@ -513,23 +513,23 @@
         <v>1</v>
       </c>
       <c r="E3" t="n">
-        <v>40689</v>
+        <v>10713195.03359146</v>
       </c>
       <c r="F3" t="n">
-        <v>-3866519</v>
+        <v>-118819.9664085377</v>
       </c>
       <c r="G3" t="n">
-        <v>-98.95861699709869</v>
+        <v>-1.09693317825481</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>더치 브로스</t>
+          <t>대한조선</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>39</v>
+        <v>100</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
@@ -540,23 +540,23 @@
         <v>1</v>
       </c>
       <c r="E4" t="n">
-        <v>2965846.22503092</v>
+        <v>9570000</v>
       </c>
       <c r="F4" t="n">
-        <v>-224797.7749690795</v>
+        <v>2357000</v>
       </c>
       <c r="G4" t="n">
-        <v>-7.04552983564069</v>
+        <v>32.67711077221684</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>발레로 에너지</t>
+          <t>프론트라인</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>6</v>
+        <v>175</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -567,23 +567,23 @@
         <v>1</v>
       </c>
       <c r="E5" t="n">
-        <v>2138731.14071836</v>
+        <v>8362532.627803192</v>
       </c>
       <c r="F5" t="n">
-        <v>74741.1407183595</v>
+        <v>3932668.627803192</v>
       </c>
       <c r="G5" t="n">
-        <v>3.621196842928478</v>
+        <v>88.77628360155508</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>센트러스 에너지</t>
+          <t>시드릴</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>21</v>
+        <v>123</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
@@ -594,23 +594,23 @@
         <v>1</v>
       </c>
       <c r="E6" t="n">
-        <v>6546958.253894605</v>
+        <v>8074480.025508801</v>
       </c>
       <c r="F6" t="n">
-        <v>315739.2538946057</v>
+        <v>1624129.025508801</v>
       </c>
       <c r="G6" t="n">
-        <v>5.067054357977239</v>
+        <v>25.17892476717626</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>스타 벌크 캐리어스</t>
+          <t>트랜스오션</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>50</v>
+        <v>750</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -621,23 +621,23 @@
         <v>1</v>
       </c>
       <c r="E7" t="n">
-        <v>1712476.648945617</v>
+        <v>6965062.522888184</v>
       </c>
       <c r="F7" t="n">
-        <v>398123.6489456175</v>
+        <v>2837828.522888184</v>
       </c>
       <c r="G7" t="n">
-        <v>30.29046602743841</v>
+        <v>68.7586049855226</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>시드릴</t>
+          <t>세아제강</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>123</v>
+        <v>50</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
@@ -648,23 +648,23 @@
         <v>1</v>
       </c>
       <c r="E8" t="n">
-        <v>8090014.733635107</v>
+        <v>6915000</v>
       </c>
       <c r="F8" t="n">
-        <v>1639663.733635107</v>
+        <v>605000</v>
       </c>
       <c r="G8" t="n">
-        <v>25.41975984927188</v>
+        <v>9.587955625990491</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>오케아니스 에코 탱커스</t>
+          <t>센트러스 에너지</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>65</v>
+        <v>21</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
@@ -675,23 +675,23 @@
         <v>1</v>
       </c>
       <c r="E9" t="n">
-        <v>4575098.725873504</v>
+        <v>6504677.671671314</v>
       </c>
       <c r="F9" t="n">
-        <v>2318738.725873504</v>
+        <v>273458.6716713151</v>
       </c>
       <c r="G9" t="n">
-        <v>102.7645732894354</v>
+        <v>4.38852609210678</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>유나이티드헬스 그룹</t>
+          <t>타이드워터</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>4</v>
+        <v>48</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
@@ -702,23 +702,23 @@
         <v>1</v>
       </c>
       <c r="E10" t="n">
-        <v>1699490.128895313</v>
+        <v>5368424.783017382</v>
       </c>
       <c r="F10" t="n">
-        <v>5034.128895312548</v>
+        <v>1643879.783017382</v>
       </c>
       <c r="G10" t="n">
-        <v>0.297094105442251</v>
+        <v>44.13639204298463</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>차코스 에너지 내비게이션</t>
+          <t>노브</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>75</v>
+        <v>185</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
@@ -729,23 +729,23 @@
         <v>1</v>
       </c>
       <c r="E11" t="n">
-        <v>4007418.271141662</v>
+        <v>5016702.366485596</v>
       </c>
       <c r="F11" t="n">
-        <v>182770.2711416623</v>
+        <v>1706694.366485596</v>
       </c>
       <c r="G11" t="n">
-        <v>4.778747511971357</v>
+        <v>51.56163871765855</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>클리블랜드 클리프스</t>
+          <t>TIME 코리아밸류업액티브</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>70</v>
+        <v>201</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
@@ -756,23 +756,23 @@
         <v>1</v>
       </c>
       <c r="E12" t="n">
-        <v>857055.5630100402</v>
+        <v>4904400</v>
       </c>
       <c r="F12" t="n">
-        <v>-158999.4369899598</v>
+        <v>180603</v>
       </c>
       <c r="G12" t="n">
-        <v>-15.64870376012714</v>
+        <v>3.823259128197084</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>타이드워터</t>
+          <t>오케아니스 에코 탱커스</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>48</v>
+        <v>65</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
@@ -783,23 +783,23 @@
         <v>1</v>
       </c>
       <c r="E13" t="n">
-        <v>5456864.752692774</v>
+        <v>4584757.166964356</v>
       </c>
       <c r="F13" t="n">
-        <v>1732319.752692774</v>
+        <v>2328397.166964356</v>
       </c>
       <c r="G13" t="n">
-        <v>46.51090945854524</v>
+        <v>103.1926273717118</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>텍사스 퍼시픽 랜드</t>
+          <t>삼성화재</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
@@ -810,23 +810,23 @@
         <v>1</v>
       </c>
       <c r="E14" t="n">
-        <v>794737.7576458007</v>
+        <v>4446000</v>
       </c>
       <c r="F14" t="n">
-        <v>16146.75764580071</v>
+        <v>-185000</v>
       </c>
       <c r="G14" t="n">
-        <v>2.073843345967358</v>
+        <v>-3.994817534009933</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>트랜스오션</t>
+          <t>DL이앤씨</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>750</v>
+        <v>80</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
@@ -837,23 +837,23 @@
         <v>1</v>
       </c>
       <c r="E15" t="n">
-        <v>7093219.418241119</v>
+        <v>4128000</v>
       </c>
       <c r="F15" t="n">
-        <v>2965985.418241119</v>
+        <v>717000</v>
       </c>
       <c r="G15" t="n">
-        <v>71.86375713713153</v>
+        <v>21.02022867194371</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>페트로브라스 (ADR)</t>
+          <t>차코스 에너지 내비게이션</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>480</v>
+        <v>75</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
@@ -864,23 +864,23 @@
         <v>1</v>
       </c>
       <c r="E16" t="n">
-        <v>14082576.9328374</v>
+        <v>3986244.634113007</v>
       </c>
       <c r="F16" t="n">
-        <v>1976027.932837404</v>
+        <v>161596.6341130068</v>
       </c>
       <c r="G16" t="n">
-        <v>16.3219752617976</v>
+        <v>4.225137427366041</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>프론트라인</t>
+          <t>동원개발</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>175</v>
+        <v>1360</v>
       </c>
       <c r="C17" t="inlineStr">
         <is>
@@ -891,23 +891,23 @@
         <v>1</v>
       </c>
       <c r="E17" t="n">
-        <v>8440541.129673157</v>
+        <v>3978000</v>
       </c>
       <c r="F17" t="n">
-        <v>4010677.129673157</v>
+        <v>240600</v>
       </c>
       <c r="G17" t="n">
-        <v>90.53725192631549</v>
+        <v>6.437630438272596</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>피바디 에너지</t>
+          <t>HD건설기계</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>65</v>
+        <v>31</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
@@ -918,23 +918,23 @@
         <v>1</v>
       </c>
       <c r="E18" t="n">
-        <v>3423839.074937592</v>
+        <v>3955600</v>
       </c>
       <c r="F18" t="n">
-        <v>1953067.074937592</v>
+        <v>-79496</v>
       </c>
       <c r="G18" t="n">
-        <v>132.7919674115085</v>
+        <v>-1.970114217852561</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>하프니아</t>
+          <t>피바디 에너지</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>80</v>
+        <v>65</v>
       </c>
       <c r="C19" t="inlineStr">
         <is>
@@ -945,23 +945,23 @@
         <v>1</v>
       </c>
       <c r="E19" t="n">
-        <v>821489.5606615674</v>
+        <v>3502070.421398284</v>
       </c>
       <c r="F19" t="n">
-        <v>195758.5606615674</v>
+        <v>2031298.421398284</v>
       </c>
       <c r="G19" t="n">
-        <v>31.28477902829928</v>
+        <v>138.1110343002372</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>AGNC 인베스트먼트</t>
+          <t>더치 브로스</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>700</v>
+        <v>39</v>
       </c>
       <c r="C20" t="inlineStr">
         <is>
@@ -972,23 +972,23 @@
         <v>1</v>
       </c>
       <c r="E20" t="n">
-        <v>10822406.73782303</v>
+        <v>2965846.22503092</v>
       </c>
       <c r="F20" t="n">
-        <v>-9608.262176971883</v>
+        <v>-224797.7749690795</v>
       </c>
       <c r="G20" t="n">
-        <v>-0.08870244526961865</v>
+        <v>-7.04552983564069</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>넥스틸</t>
+          <t>현대제철</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>200</v>
+        <v>70</v>
       </c>
       <c r="C21" t="inlineStr">
         <is>
@@ -999,23 +999,23 @@
         <v>1</v>
       </c>
       <c r="E21" t="n">
-        <v>2400000</v>
+        <v>2607500</v>
       </c>
       <c r="F21" t="n">
-        <v>389000</v>
+        <v>-200000</v>
       </c>
       <c r="G21" t="n">
-        <v>19.34361014420686</v>
+        <v>-7.123775601068566</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>대신증권</t>
+          <t>KoAct 코스닥액티브</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>55</v>
+        <v>200</v>
       </c>
       <c r="C22" t="inlineStr">
         <is>
@@ -1026,23 +1026,23 @@
         <v>1</v>
       </c>
       <c r="E22" t="n">
-        <v>2238500</v>
+        <v>2598000</v>
       </c>
       <c r="F22" t="n">
-        <v>528999</v>
+        <v>-104000</v>
       </c>
       <c r="G22" t="n">
-        <v>30.94464408034859</v>
+        <v>-3.84900074019245</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>대창단조</t>
+          <t>휴스틸</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>300</v>
+        <v>500</v>
       </c>
       <c r="C23" t="inlineStr">
         <is>
@@ -1053,23 +1053,23 @@
         <v>1</v>
       </c>
       <c r="E23" t="n">
-        <v>1914000</v>
+        <v>2560000</v>
       </c>
       <c r="F23" t="n">
-        <v>-144000</v>
+        <v>281390</v>
       </c>
       <c r="G23" t="n">
-        <v>-6.997084548104956</v>
+        <v>12.34919534277476</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>대한조선</t>
+          <t>넥스틸</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>100</v>
+        <v>200</v>
       </c>
       <c r="C24" t="inlineStr">
         <is>
@@ -1080,23 +1080,23 @@
         <v>1</v>
       </c>
       <c r="E24" t="n">
-        <v>9570000</v>
+        <v>2400000</v>
       </c>
       <c r="F24" t="n">
-        <v>2357000</v>
+        <v>389000</v>
       </c>
       <c r="G24" t="n">
-        <v>32.67711077221684</v>
+        <v>19.34361014420686</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>동방</t>
+          <t>대신증권</t>
         </is>
       </c>
       <c r="B25" t="n">
-        <v>681</v>
+        <v>55</v>
       </c>
       <c r="C25" t="inlineStr">
         <is>
@@ -1107,23 +1107,23 @@
         <v>1</v>
       </c>
       <c r="E25" t="n">
-        <v>1882965</v>
+        <v>2238500</v>
       </c>
       <c r="F25" t="n">
-        <v>-88536</v>
+        <v>528999</v>
       </c>
       <c r="G25" t="n">
-        <v>-4.490791533963209</v>
+        <v>30.94464408034859</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>동원개발</t>
+          <t>발레로 에너지</t>
         </is>
       </c>
       <c r="B26" t="n">
-        <v>1360</v>
+        <v>6</v>
       </c>
       <c r="C26" t="inlineStr">
         <is>
@@ -1134,13 +1134,13 @@
         <v>1</v>
       </c>
       <c r="E26" t="n">
-        <v>3978000</v>
+        <v>2125937.735642139</v>
       </c>
       <c r="F26" t="n">
-        <v>240600</v>
+        <v>61947.73564213887</v>
       </c>
       <c r="G26" t="n">
-        <v>6.437630438272596</v>
+        <v>3.001358322576121</v>
       </c>
     </row>
     <row r="27">
@@ -1173,11 +1173,11 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>비에이치아이</t>
+          <t>대창단조</t>
         </is>
       </c>
       <c r="B28" t="n">
-        <v>8</v>
+        <v>300</v>
       </c>
       <c r="C28" t="inlineStr">
         <is>
@@ -1188,23 +1188,23 @@
         <v>1</v>
       </c>
       <c r="E28" t="n">
-        <v>844800</v>
+        <v>1914000</v>
       </c>
       <c r="F28" t="n">
-        <v>179685</v>
+        <v>-144000</v>
       </c>
       <c r="G28" t="n">
-        <v>27.01562887620938</v>
+        <v>-6.997084548104956</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>삼성생명</t>
+          <t>동방</t>
         </is>
       </c>
       <c r="B29" t="n">
-        <v>4</v>
+        <v>681</v>
       </c>
       <c r="C29" t="inlineStr">
         <is>
@@ -1215,23 +1215,23 @@
         <v>1</v>
       </c>
       <c r="E29" t="n">
-        <v>940000</v>
+        <v>1882965</v>
       </c>
       <c r="F29" t="n">
-        <v>107000</v>
+        <v>-88536</v>
       </c>
       <c r="G29" t="n">
-        <v>12.84513805522209</v>
+        <v>-4.490791533963209</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>삼성화재</t>
+          <t>하나금융지주</t>
         </is>
       </c>
       <c r="B30" t="n">
-        <v>7</v>
+        <v>15</v>
       </c>
       <c r="C30" t="inlineStr">
         <is>
@@ -1242,19 +1242,19 @@
         <v>1</v>
       </c>
       <c r="E30" t="n">
-        <v>3458000</v>
+        <v>1717500</v>
       </c>
       <c r="F30" t="n">
-        <v>-173000</v>
+        <v>35000</v>
       </c>
       <c r="G30" t="n">
-        <v>-4.76452767832553</v>
+        <v>2.080237741456166</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>세아제강</t>
+          <t>스타 벌크 캐리어스</t>
         </is>
       </c>
       <c r="B31" t="n">
@@ -1269,23 +1269,23 @@
         <v>1</v>
       </c>
       <c r="E31" t="n">
-        <v>6915000</v>
+        <v>1693903.148884582</v>
       </c>
       <c r="F31" t="n">
-        <v>605000</v>
+        <v>379550.1488845828</v>
       </c>
       <c r="G31" t="n">
-        <v>9.587955625990491</v>
+        <v>28.87733728188568</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>케이씨</t>
+          <t>유나이티드헬스 그룹</t>
         </is>
       </c>
       <c r="B32" t="n">
-        <v>50</v>
+        <v>4</v>
       </c>
       <c r="C32" t="inlineStr">
         <is>
@@ -1296,23 +1296,23 @@
         <v>1</v>
       </c>
       <c r="E32" t="n">
-        <v>1640000</v>
+        <v>1689920.967345312</v>
       </c>
       <c r="F32" t="n">
-        <v>-9500</v>
+        <v>-4535.032654687762</v>
       </c>
       <c r="G32" t="n">
-        <v>-0.5759321006365565</v>
+        <v>-0.2676394462109233</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>하나금융지주</t>
+          <t>케이씨</t>
         </is>
       </c>
       <c r="B33" t="n">
-        <v>10</v>
+        <v>50</v>
       </c>
       <c r="C33" t="inlineStr">
         <is>
@@ -1323,23 +1323,23 @@
         <v>1</v>
       </c>
       <c r="E33" t="n">
-        <v>1145000</v>
+        <v>1640000</v>
       </c>
       <c r="F33" t="n">
-        <v>36000</v>
+        <v>-9500.000000000698</v>
       </c>
       <c r="G33" t="n">
-        <v>3.246167718665464</v>
+        <v>-0.5759321006365986</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>현대제철</t>
+          <t>삼성생명</t>
         </is>
       </c>
       <c r="B34" t="n">
-        <v>70</v>
+        <v>4</v>
       </c>
       <c r="C34" t="inlineStr">
         <is>
@@ -1350,23 +1350,23 @@
         <v>1</v>
       </c>
       <c r="E34" t="n">
-        <v>2607500</v>
+        <v>940000</v>
       </c>
       <c r="F34" t="n">
-        <v>-200000</v>
+        <v>107000</v>
       </c>
       <c r="G34" t="n">
-        <v>-7.123775601068566</v>
+        <v>12.84513805522209</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>휴스틸</t>
+          <t>클리블랜드 클리프스</t>
         </is>
       </c>
       <c r="B35" t="n">
-        <v>500</v>
+        <v>70</v>
       </c>
       <c r="C35" t="inlineStr">
         <is>
@@ -1377,23 +1377,23 @@
         <v>1</v>
       </c>
       <c r="E35" t="n">
-        <v>2560000</v>
+        <v>850814.9225377198</v>
       </c>
       <c r="F35" t="n">
-        <v>281390</v>
+        <v>-165240.0774622802</v>
       </c>
       <c r="G35" t="n">
-        <v>12.34919534277476</v>
+        <v>-16.26290677790869</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>DL이앤씨</t>
+          <t>비에이치아이</t>
         </is>
       </c>
       <c r="B36" t="n">
-        <v>80</v>
+        <v>8</v>
       </c>
       <c r="C36" t="inlineStr">
         <is>
@@ -1404,23 +1404,23 @@
         <v>1</v>
       </c>
       <c r="E36" t="n">
-        <v>4128000</v>
+        <v>844800</v>
       </c>
       <c r="F36" t="n">
-        <v>717000</v>
+        <v>179685</v>
       </c>
       <c r="G36" t="n">
-        <v>21.02022867194371</v>
+        <v>27.01562887620938</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>HD건설기계</t>
+          <t>하프니아</t>
         </is>
       </c>
       <c r="B37" t="n">
-        <v>31</v>
+        <v>80</v>
       </c>
       <c r="C37" t="inlineStr">
         <is>
@@ -1431,23 +1431,23 @@
         <v>1</v>
       </c>
       <c r="E37" t="n">
-        <v>3955600</v>
+        <v>822583.1797722168</v>
       </c>
       <c r="F37" t="n">
-        <v>-79496</v>
+        <v>196852.1797722168</v>
       </c>
       <c r="G37" t="n">
-        <v>-1.970114217852561</v>
+        <v>31.45955366958275</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>KoAct 코스닥액티브</t>
+          <t>텍사스 퍼시픽 랜드</t>
         </is>
       </c>
       <c r="B38" t="n">
-        <v>200</v>
+        <v>1</v>
       </c>
       <c r="C38" t="inlineStr">
         <is>
@@ -1458,23 +1458,23 @@
         <v>1</v>
       </c>
       <c r="E38" t="n">
-        <v>2598000</v>
+        <v>787635.2983817384</v>
       </c>
       <c r="F38" t="n">
-        <v>-104000</v>
+        <v>9044.298381738365</v>
       </c>
       <c r="G38" t="n">
-        <v>-3.84900074019245</v>
+        <v>1.161623802707502</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>TIME 코리아밸류업액티브</t>
+          <t>노블</t>
         </is>
       </c>
       <c r="B39" t="n">
-        <v>201</v>
+        <v>99</v>
       </c>
       <c r="C39" t="inlineStr">
         <is>
@@ -1485,13 +1485,13 @@
         <v>1</v>
       </c>
       <c r="E39" t="n">
-        <v>4904400</v>
+        <v>6862314.14501056</v>
       </c>
       <c r="F39" t="n">
-        <v>180603</v>
+        <v>2955106.14501056</v>
       </c>
       <c r="G39" t="n">
-        <v>3.823259128197084</v>
+        <v>75.63216867416733</v>
       </c>
     </row>
   </sheetData>
@@ -1538,22 +1538,22 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-03-17</t>
+          <t>2026-03-18</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>33078556</v>
+        <v>31505056</v>
       </c>
       <c r="C2" t="n">
-        <v>6010.99</v>
+        <v>6016.63</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2026-03-18T21:09:28</t>
+          <t>2026-03-18T21:13:42</t>
         </is>
       </c>
       <c r="E2" t="n">
-        <v>1488.910034179688</v>
+        <v>1485.880004882812</v>
       </c>
     </row>
   </sheetData>
@@ -3046,17 +3046,17 @@
         <v>1</v>
       </c>
       <c r="F40" t="n">
-        <v>14082576.9328374</v>
+        <v>14100407.22082324</v>
       </c>
       <c r="G40" t="n">
-        <v>1976027.932837404</v>
+        <v>1993858.220823243</v>
       </c>
       <c r="H40" t="n">
-        <v>16.3219752617976</v>
+        <v>16.46925330102941</v>
       </c>
       <c r="I40" t="inlineStr">
         <is>
-          <t>2026-03-18T14:32:42</t>
+          <t>2026-03-18T21:13:42</t>
         </is>
       </c>
     </row>
@@ -3083,17 +3083,17 @@
         <v>1</v>
       </c>
       <c r="F41" t="n">
-        <v>10822406.73782303</v>
+        <v>10713195.03359146</v>
       </c>
       <c r="G41" t="n">
-        <v>-9608.262176971883</v>
+        <v>-118819.9664085377</v>
       </c>
       <c r="H41" t="n">
-        <v>-0.08870244526961865</v>
+        <v>-1.09693317825481</v>
       </c>
       <c r="I41" t="inlineStr">
         <is>
-          <t>2026-03-18T14:32:42</t>
+          <t>2026-03-18T21:13:42</t>
         </is>
       </c>
     </row>
@@ -3130,7 +3130,7 @@
       </c>
       <c r="I42" t="inlineStr">
         <is>
-          <t>2026-03-18T14:32:42</t>
+          <t>2026-03-18T21:13:42</t>
         </is>
       </c>
     </row>
@@ -3157,17 +3157,17 @@
         <v>1</v>
       </c>
       <c r="F43" t="n">
-        <v>8440541.129673157</v>
+        <v>8362532.627803192</v>
       </c>
       <c r="G43" t="n">
-        <v>4010677.129673157</v>
+        <v>3932668.627803192</v>
       </c>
       <c r="H43" t="n">
-        <v>90.53725192631549</v>
+        <v>88.77628360155508</v>
       </c>
       <c r="I43" t="inlineStr">
         <is>
-          <t>2026-03-18T14:32:42</t>
+          <t>2026-03-18T21:13:42</t>
         </is>
       </c>
     </row>
@@ -3194,17 +3194,17 @@
         <v>1</v>
       </c>
       <c r="F44" t="n">
-        <v>8090014.733635107</v>
+        <v>8074480.025508801</v>
       </c>
       <c r="G44" t="n">
-        <v>1639663.733635107</v>
+        <v>1624129.025508801</v>
       </c>
       <c r="H44" t="n">
-        <v>25.41975984927188</v>
+        <v>25.17892476717626</v>
       </c>
       <c r="I44" t="inlineStr">
         <is>
-          <t>2026-03-18T14:32:42</t>
+          <t>2026-03-18T21:13:42</t>
         </is>
       </c>
     </row>
@@ -3231,17 +3231,17 @@
         <v>1</v>
       </c>
       <c r="F45" t="n">
-        <v>7093219.418241119</v>
+        <v>6965062.522888184</v>
       </c>
       <c r="G45" t="n">
-        <v>2965985.418241119</v>
+        <v>2837828.522888184</v>
       </c>
       <c r="H45" t="n">
-        <v>71.86375713713153</v>
+        <v>68.7586049855226</v>
       </c>
       <c r="I45" t="inlineStr">
         <is>
-          <t>2026-03-18T14:32:42</t>
+          <t>2026-03-18T21:13:42</t>
         </is>
       </c>
     </row>
@@ -3278,7 +3278,7 @@
       </c>
       <c r="I46" t="inlineStr">
         <is>
-          <t>2026-03-18T14:32:42</t>
+          <t>2026-03-18T21:13:42</t>
         </is>
       </c>
     </row>
@@ -3290,11 +3290,11 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>센트러스 에너지</t>
+          <t>노블</t>
         </is>
       </c>
       <c r="C47" t="n">
-        <v>21</v>
+        <v>99</v>
       </c>
       <c r="D47" t="inlineStr">
         <is>
@@ -3305,17 +3305,17 @@
         <v>1</v>
       </c>
       <c r="F47" t="n">
-        <v>6546958.253894605</v>
+        <v>6862314.14501056</v>
       </c>
       <c r="G47" t="n">
-        <v>315739.2538946057</v>
+        <v>2955106.14501056</v>
       </c>
       <c r="H47" t="n">
-        <v>5.067054357977239</v>
+        <v>75.63216867416733</v>
       </c>
       <c r="I47" t="inlineStr">
         <is>
-          <t>2026-03-18T14:32:42</t>
+          <t>2026-03-18T21:13:42</t>
         </is>
       </c>
     </row>
@@ -3327,11 +3327,11 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>타이드워터</t>
+          <t>센트러스 에너지</t>
         </is>
       </c>
       <c r="C48" t="n">
-        <v>48</v>
+        <v>21</v>
       </c>
       <c r="D48" t="inlineStr">
         <is>
@@ -3342,17 +3342,17 @@
         <v>1</v>
       </c>
       <c r="F48" t="n">
-        <v>5456864.752692774</v>
+        <v>6504677.671671314</v>
       </c>
       <c r="G48" t="n">
-        <v>1732319.752692774</v>
+        <v>273458.6716713151</v>
       </c>
       <c r="H48" t="n">
-        <v>46.51090945854524</v>
+        <v>4.38852609210678</v>
       </c>
       <c r="I48" t="inlineStr">
         <is>
-          <t>2026-03-18T14:32:42</t>
+          <t>2026-03-18T21:13:42</t>
         </is>
       </c>
     </row>
@@ -3364,11 +3364,11 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>노브</t>
+          <t>타이드워터</t>
         </is>
       </c>
       <c r="C49" t="n">
-        <v>185</v>
+        <v>48</v>
       </c>
       <c r="D49" t="inlineStr">
         <is>
@@ -3379,17 +3379,17 @@
         <v>1</v>
       </c>
       <c r="F49" t="n">
-        <v>5041442.310511444</v>
+        <v>5368424.783017382</v>
       </c>
       <c r="G49" t="n">
-        <v>1731434.310511444</v>
+        <v>1643879.783017382</v>
       </c>
       <c r="H49" t="n">
-        <v>52.30906724429197</v>
+        <v>44.13639204298463</v>
       </c>
       <c r="I49" t="inlineStr">
         <is>
-          <t>2026-03-18T14:32:42</t>
+          <t>2026-03-18T21:13:42</t>
         </is>
       </c>
     </row>
@@ -3401,11 +3401,11 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>TIME 코리아밸류업액티브</t>
+          <t>노브</t>
         </is>
       </c>
       <c r="C50" t="n">
-        <v>201</v>
+        <v>185</v>
       </c>
       <c r="D50" t="inlineStr">
         <is>
@@ -3416,17 +3416,17 @@
         <v>1</v>
       </c>
       <c r="F50" t="n">
-        <v>4904400</v>
+        <v>5016702.366485596</v>
       </c>
       <c r="G50" t="n">
-        <v>180603</v>
+        <v>1706694.366485596</v>
       </c>
       <c r="H50" t="n">
-        <v>3.823259128197084</v>
+        <v>51.56163871765855</v>
       </c>
       <c r="I50" t="inlineStr">
         <is>
-          <t>2026-03-18T14:32:42</t>
+          <t>2026-03-18T21:13:42</t>
         </is>
       </c>
     </row>
@@ -3438,11 +3438,11 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>오케아니스 에코 탱커스</t>
+          <t>TIME 코리아밸류업액티브</t>
         </is>
       </c>
       <c r="C51" t="n">
-        <v>65</v>
+        <v>201</v>
       </c>
       <c r="D51" t="inlineStr">
         <is>
@@ -3453,17 +3453,17 @@
         <v>1</v>
       </c>
       <c r="F51" t="n">
-        <v>4575098.725873504</v>
+        <v>4904400</v>
       </c>
       <c r="G51" t="n">
-        <v>2318738.725873504</v>
+        <v>180603</v>
       </c>
       <c r="H51" t="n">
-        <v>102.7645732894354</v>
+        <v>3.823259128197084</v>
       </c>
       <c r="I51" t="inlineStr">
         <is>
-          <t>2026-03-18T14:32:42</t>
+          <t>2026-03-18T21:13:42</t>
         </is>
       </c>
     </row>
@@ -3475,11 +3475,11 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>삼성화재</t>
+          <t>오케아니스 에코 탱커스</t>
         </is>
       </c>
       <c r="C52" t="n">
-        <v>9</v>
+        <v>65</v>
       </c>
       <c r="D52" t="inlineStr">
         <is>
@@ -3490,17 +3490,17 @@
         <v>1</v>
       </c>
       <c r="F52" t="n">
-        <v>4446000</v>
+        <v>4584757.166964356</v>
       </c>
       <c r="G52" t="n">
-        <v>-185000</v>
+        <v>2328397.166964356</v>
       </c>
       <c r="H52" t="n">
-        <v>-3.994817534009933</v>
+        <v>103.1926273717118</v>
       </c>
       <c r="I52" t="inlineStr">
         <is>
-          <t>2026-03-18T14:32:42</t>
+          <t>2026-03-18T21:13:42</t>
         </is>
       </c>
     </row>
@@ -3512,11 +3512,11 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>DL이앤씨</t>
+          <t>삼성화재</t>
         </is>
       </c>
       <c r="C53" t="n">
-        <v>80</v>
+        <v>9</v>
       </c>
       <c r="D53" t="inlineStr">
         <is>
@@ -3527,17 +3527,17 @@
         <v>1</v>
       </c>
       <c r="F53" t="n">
-        <v>4128000</v>
+        <v>4446000</v>
       </c>
       <c r="G53" t="n">
-        <v>717000</v>
+        <v>-185000</v>
       </c>
       <c r="H53" t="n">
-        <v>21.02022867194371</v>
+        <v>-3.994817534009933</v>
       </c>
       <c r="I53" t="inlineStr">
         <is>
-          <t>2026-03-18T14:32:42</t>
+          <t>2026-03-18T21:13:42</t>
         </is>
       </c>
     </row>
@@ -3549,11 +3549,11 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>차코스 에너지 내비게이션</t>
+          <t>DL이앤씨</t>
         </is>
       </c>
       <c r="C54" t="n">
-        <v>75</v>
+        <v>80</v>
       </c>
       <c r="D54" t="inlineStr">
         <is>
@@ -3564,17 +3564,17 @@
         <v>1</v>
       </c>
       <c r="F54" t="n">
-        <v>4007418.271141662</v>
+        <v>4128000</v>
       </c>
       <c r="G54" t="n">
-        <v>182770.2711416623</v>
+        <v>717000</v>
       </c>
       <c r="H54" t="n">
-        <v>4.778747511971357</v>
+        <v>21.02022867194371</v>
       </c>
       <c r="I54" t="inlineStr">
         <is>
-          <t>2026-03-18T14:32:42</t>
+          <t>2026-03-18T21:13:42</t>
         </is>
       </c>
     </row>
@@ -3586,11 +3586,11 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>동원개발</t>
+          <t>차코스 에너지 내비게이션</t>
         </is>
       </c>
       <c r="C55" t="n">
-        <v>1360</v>
+        <v>75</v>
       </c>
       <c r="D55" t="inlineStr">
         <is>
@@ -3601,17 +3601,17 @@
         <v>1</v>
       </c>
       <c r="F55" t="n">
-        <v>3978000</v>
+        <v>3986244.634113007</v>
       </c>
       <c r="G55" t="n">
-        <v>240600</v>
+        <v>161596.6341130068</v>
       </c>
       <c r="H55" t="n">
-        <v>6.437630438272596</v>
+        <v>4.225137427366041</v>
       </c>
       <c r="I55" t="inlineStr">
         <is>
-          <t>2026-03-18T14:32:42</t>
+          <t>2026-03-18T21:13:42</t>
         </is>
       </c>
     </row>
@@ -3623,11 +3623,11 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>HD건설기계</t>
+          <t>동원개발</t>
         </is>
       </c>
       <c r="C56" t="n">
-        <v>31</v>
+        <v>1360</v>
       </c>
       <c r="D56" t="inlineStr">
         <is>
@@ -3638,17 +3638,17 @@
         <v>1</v>
       </c>
       <c r="F56" t="n">
-        <v>3955600</v>
+        <v>3978000</v>
       </c>
       <c r="G56" t="n">
-        <v>-79496</v>
+        <v>240600</v>
       </c>
       <c r="H56" t="n">
-        <v>-1.970114217852561</v>
+        <v>6.437630438272596</v>
       </c>
       <c r="I56" t="inlineStr">
         <is>
-          <t>2026-03-18T14:32:42</t>
+          <t>2026-03-18T21:13:42</t>
         </is>
       </c>
     </row>
@@ -3660,11 +3660,11 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>피바디 에너지</t>
+          <t>HD건설기계</t>
         </is>
       </c>
       <c r="C57" t="n">
-        <v>65</v>
+        <v>31</v>
       </c>
       <c r="D57" t="inlineStr">
         <is>
@@ -3675,17 +3675,17 @@
         <v>1</v>
       </c>
       <c r="F57" t="n">
-        <v>3423839.074937592</v>
+        <v>3955600</v>
       </c>
       <c r="G57" t="n">
-        <v>1953067.074937592</v>
+        <v>-79496</v>
       </c>
       <c r="H57" t="n">
-        <v>132.7919674115085</v>
+        <v>-1.970114217852561</v>
       </c>
       <c r="I57" t="inlineStr">
         <is>
-          <t>2026-03-18T14:32:42</t>
+          <t>2026-03-18T21:13:42</t>
         </is>
       </c>
     </row>
@@ -3697,11 +3697,11 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>더치 브로스</t>
+          <t>피바디 에너지</t>
         </is>
       </c>
       <c r="C58" t="n">
-        <v>39</v>
+        <v>65</v>
       </c>
       <c r="D58" t="inlineStr">
         <is>
@@ -3712,17 +3712,17 @@
         <v>1</v>
       </c>
       <c r="F58" t="n">
-        <v>2965846.22503092</v>
+        <v>3502070.421398284</v>
       </c>
       <c r="G58" t="n">
-        <v>-224797.7749690795</v>
+        <v>2031298.421398284</v>
       </c>
       <c r="H58" t="n">
-        <v>-7.04552983564069</v>
+        <v>138.1110343002372</v>
       </c>
       <c r="I58" t="inlineStr">
         <is>
-          <t>2026-03-18T14:32:42</t>
+          <t>2026-03-18T21:13:42</t>
         </is>
       </c>
     </row>
@@ -3734,11 +3734,11 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>현대제철</t>
+          <t>더치 브로스</t>
         </is>
       </c>
       <c r="C59" t="n">
-        <v>70</v>
+        <v>39</v>
       </c>
       <c r="D59" t="inlineStr">
         <is>
@@ -3749,17 +3749,17 @@
         <v>1</v>
       </c>
       <c r="F59" t="n">
-        <v>2607500</v>
+        <v>2965846.22503092</v>
       </c>
       <c r="G59" t="n">
-        <v>-200000</v>
+        <v>-224797.7749690795</v>
       </c>
       <c r="H59" t="n">
-        <v>-7.123775601068566</v>
+        <v>-7.04552983564069</v>
       </c>
       <c r="I59" t="inlineStr">
         <is>
-          <t>2026-03-18T14:32:42</t>
+          <t>2026-03-18T21:13:42</t>
         </is>
       </c>
     </row>
@@ -3771,11 +3771,11 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>KoAct 코스닥액티브</t>
+          <t>현대제철</t>
         </is>
       </c>
       <c r="C60" t="n">
-        <v>200</v>
+        <v>70</v>
       </c>
       <c r="D60" t="inlineStr">
         <is>
@@ -3786,17 +3786,17 @@
         <v>1</v>
       </c>
       <c r="F60" t="n">
-        <v>2598000</v>
+        <v>2607500</v>
       </c>
       <c r="G60" t="n">
-        <v>-104000</v>
+        <v>-200000</v>
       </c>
       <c r="H60" t="n">
-        <v>-3.84900074019245</v>
+        <v>-7.123775601068566</v>
       </c>
       <c r="I60" t="inlineStr">
         <is>
-          <t>2026-03-18T14:32:42</t>
+          <t>2026-03-18T21:13:42</t>
         </is>
       </c>
     </row>
@@ -3808,11 +3808,11 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>휴스틸</t>
+          <t>KoAct 코스닥액티브</t>
         </is>
       </c>
       <c r="C61" t="n">
-        <v>500</v>
+        <v>200</v>
       </c>
       <c r="D61" t="inlineStr">
         <is>
@@ -3823,17 +3823,17 @@
         <v>1</v>
       </c>
       <c r="F61" t="n">
-        <v>2560000</v>
+        <v>2598000</v>
       </c>
       <c r="G61" t="n">
-        <v>281390</v>
+        <v>-104000</v>
       </c>
       <c r="H61" t="n">
-        <v>12.34919534277476</v>
+        <v>-3.84900074019245</v>
       </c>
       <c r="I61" t="inlineStr">
         <is>
-          <t>2026-03-18T14:32:42</t>
+          <t>2026-03-18T21:13:42</t>
         </is>
       </c>
     </row>
@@ -3845,11 +3845,11 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>넥스틸</t>
+          <t>휴스틸</t>
         </is>
       </c>
       <c r="C62" t="n">
-        <v>200</v>
+        <v>500</v>
       </c>
       <c r="D62" t="inlineStr">
         <is>
@@ -3860,17 +3860,17 @@
         <v>1</v>
       </c>
       <c r="F62" t="n">
-        <v>2400000</v>
+        <v>2560000</v>
       </c>
       <c r="G62" t="n">
-        <v>389000</v>
+        <v>281390</v>
       </c>
       <c r="H62" t="n">
-        <v>19.34361014420686</v>
+        <v>12.34919534277476</v>
       </c>
       <c r="I62" t="inlineStr">
         <is>
-          <t>2026-03-18T14:32:42</t>
+          <t>2026-03-18T21:13:42</t>
         </is>
       </c>
     </row>
@@ -3882,11 +3882,11 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>대신증권</t>
+          <t>넥스틸</t>
         </is>
       </c>
       <c r="C63" t="n">
-        <v>55</v>
+        <v>200</v>
       </c>
       <c r="D63" t="inlineStr">
         <is>
@@ -3897,17 +3897,17 @@
         <v>1</v>
       </c>
       <c r="F63" t="n">
-        <v>2238500</v>
+        <v>2400000</v>
       </c>
       <c r="G63" t="n">
-        <v>528999</v>
+        <v>389000</v>
       </c>
       <c r="H63" t="n">
-        <v>30.94464408034859</v>
+        <v>19.34361014420686</v>
       </c>
       <c r="I63" t="inlineStr">
         <is>
-          <t>2026-03-18T14:32:42</t>
+          <t>2026-03-18T21:13:42</t>
         </is>
       </c>
     </row>
@@ -3919,11 +3919,11 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>발레로 에너지</t>
+          <t>대신증권</t>
         </is>
       </c>
       <c r="C64" t="n">
-        <v>6</v>
+        <v>55</v>
       </c>
       <c r="D64" t="inlineStr">
         <is>
@@ -3934,17 +3934,17 @@
         <v>1</v>
       </c>
       <c r="F64" t="n">
-        <v>2138731.14071836</v>
+        <v>2238500</v>
       </c>
       <c r="G64" t="n">
-        <v>74741.1407183595</v>
+        <v>528999</v>
       </c>
       <c r="H64" t="n">
-        <v>3.621196842928478</v>
+        <v>30.94464408034859</v>
       </c>
       <c r="I64" t="inlineStr">
         <is>
-          <t>2026-03-18T14:32:42</t>
+          <t>2026-03-18T21:13:42</t>
         </is>
       </c>
     </row>
@@ -3956,11 +3956,11 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>미창석유</t>
+          <t>발레로 에너지</t>
         </is>
       </c>
       <c r="C65" t="n">
-        <v>18</v>
+        <v>6</v>
       </c>
       <c r="D65" t="inlineStr">
         <is>
@@ -3971,17 +3971,17 @@
         <v>1</v>
       </c>
       <c r="F65" t="n">
-        <v>2032200</v>
+        <v>2125937.735642139</v>
       </c>
       <c r="G65" t="n">
-        <v>-360000</v>
+        <v>61947.73564213887</v>
       </c>
       <c r="H65" t="n">
-        <v>-15.04890895410083</v>
+        <v>3.001358322576121</v>
       </c>
       <c r="I65" t="inlineStr">
         <is>
-          <t>2026-03-18T14:32:42</t>
+          <t>2026-03-18T21:13:42</t>
         </is>
       </c>
     </row>
@@ -3993,11 +3993,11 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>대창단조</t>
+          <t>미창석유</t>
         </is>
       </c>
       <c r="C66" t="n">
-        <v>300</v>
+        <v>18</v>
       </c>
       <c r="D66" t="inlineStr">
         <is>
@@ -4008,17 +4008,17 @@
         <v>1</v>
       </c>
       <c r="F66" t="n">
-        <v>1914000</v>
+        <v>2032200</v>
       </c>
       <c r="G66" t="n">
-        <v>-144000</v>
+        <v>-360000</v>
       </c>
       <c r="H66" t="n">
-        <v>-6.997084548104956</v>
+        <v>-15.04890895410083</v>
       </c>
       <c r="I66" t="inlineStr">
         <is>
-          <t>2026-03-18T14:32:42</t>
+          <t>2026-03-18T21:13:42</t>
         </is>
       </c>
     </row>
@@ -4030,11 +4030,11 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>동방</t>
+          <t>대창단조</t>
         </is>
       </c>
       <c r="C67" t="n">
-        <v>681</v>
+        <v>300</v>
       </c>
       <c r="D67" t="inlineStr">
         <is>
@@ -4045,17 +4045,17 @@
         <v>1</v>
       </c>
       <c r="F67" t="n">
-        <v>1882965</v>
+        <v>1914000</v>
       </c>
       <c r="G67" t="n">
-        <v>-88536</v>
+        <v>-144000</v>
       </c>
       <c r="H67" t="n">
-        <v>-4.490791533963209</v>
+        <v>-6.997084548104956</v>
       </c>
       <c r="I67" t="inlineStr">
         <is>
-          <t>2026-03-18T14:32:42</t>
+          <t>2026-03-18T21:13:42</t>
         </is>
       </c>
     </row>
@@ -4067,11 +4067,11 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>하나금융지주</t>
+          <t>동방</t>
         </is>
       </c>
       <c r="C68" t="n">
-        <v>15</v>
+        <v>681</v>
       </c>
       <c r="D68" t="inlineStr">
         <is>
@@ -4082,17 +4082,17 @@
         <v>1</v>
       </c>
       <c r="F68" t="n">
-        <v>1717500</v>
+        <v>1882965</v>
       </c>
       <c r="G68" t="n">
-        <v>35000</v>
+        <v>-88536</v>
       </c>
       <c r="H68" t="n">
-        <v>2.080237741456166</v>
+        <v>-4.490791533963209</v>
       </c>
       <c r="I68" t="inlineStr">
         <is>
-          <t>2026-03-18T14:32:42</t>
+          <t>2026-03-18T21:13:42</t>
         </is>
       </c>
     </row>
@@ -4104,11 +4104,11 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>스타 벌크 캐리어스</t>
+          <t>하나금융지주</t>
         </is>
       </c>
       <c r="C69" t="n">
-        <v>50</v>
+        <v>15</v>
       </c>
       <c r="D69" t="inlineStr">
         <is>
@@ -4119,17 +4119,17 @@
         <v>1</v>
       </c>
       <c r="F69" t="n">
-        <v>1712476.648945617</v>
+        <v>1717500</v>
       </c>
       <c r="G69" t="n">
-        <v>398123.648945618</v>
+        <v>35000</v>
       </c>
       <c r="H69" t="n">
-        <v>30.29046602743845</v>
+        <v>2.080237741456166</v>
       </c>
       <c r="I69" t="inlineStr">
         <is>
-          <t>2026-03-18T14:32:42</t>
+          <t>2026-03-18T21:13:42</t>
         </is>
       </c>
     </row>
@@ -4141,11 +4141,11 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>유나이티드헬스 그룹</t>
+          <t>스타 벌크 캐리어스</t>
         </is>
       </c>
       <c r="C70" t="n">
-        <v>4</v>
+        <v>50</v>
       </c>
       <c r="D70" t="inlineStr">
         <is>
@@ -4156,17 +4156,17 @@
         <v>1</v>
       </c>
       <c r="F70" t="n">
-        <v>1699490.128895313</v>
+        <v>1693903.148884582</v>
       </c>
       <c r="G70" t="n">
-        <v>5034.128895312548</v>
+        <v>379550.1488845828</v>
       </c>
       <c r="H70" t="n">
-        <v>0.297094105442251</v>
+        <v>28.87733728188568</v>
       </c>
       <c r="I70" t="inlineStr">
         <is>
-          <t>2026-03-18T14:32:42</t>
+          <t>2026-03-18T21:13:42</t>
         </is>
       </c>
     </row>
@@ -4178,11 +4178,11 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>케이씨</t>
+          <t>유나이티드헬스 그룹</t>
         </is>
       </c>
       <c r="C71" t="n">
-        <v>50</v>
+        <v>4</v>
       </c>
       <c r="D71" t="inlineStr">
         <is>
@@ -4193,17 +4193,17 @@
         <v>1</v>
       </c>
       <c r="F71" t="n">
-        <v>1640000</v>
+        <v>1689920.967345312</v>
       </c>
       <c r="G71" t="n">
-        <v>-9500.000000000698</v>
+        <v>-4535.032654687762</v>
       </c>
       <c r="H71" t="n">
-        <v>-0.5759321006365986</v>
+        <v>-0.2676394462109233</v>
       </c>
       <c r="I71" t="inlineStr">
         <is>
-          <t>2026-03-18T14:32:42</t>
+          <t>2026-03-18T21:13:42</t>
         </is>
       </c>
     </row>
@@ -4215,11 +4215,11 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>삼성생명</t>
+          <t>케이씨</t>
         </is>
       </c>
       <c r="C72" t="n">
-        <v>4</v>
+        <v>50</v>
       </c>
       <c r="D72" t="inlineStr">
         <is>
@@ -4230,17 +4230,17 @@
         <v>1</v>
       </c>
       <c r="F72" t="n">
-        <v>940000</v>
+        <v>1640000</v>
       </c>
       <c r="G72" t="n">
-        <v>107000</v>
+        <v>-9500.000000000698</v>
       </c>
       <c r="H72" t="n">
-        <v>12.84513805522209</v>
+        <v>-0.5759321006365986</v>
       </c>
       <c r="I72" t="inlineStr">
         <is>
-          <t>2026-03-18T14:32:42</t>
+          <t>2026-03-18T21:13:42</t>
         </is>
       </c>
     </row>
@@ -4252,11 +4252,11 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>클리블랜드 클리프스</t>
+          <t>삼성생명</t>
         </is>
       </c>
       <c r="C73" t="n">
-        <v>70</v>
+        <v>4</v>
       </c>
       <c r="D73" t="inlineStr">
         <is>
@@ -4267,17 +4267,17 @@
         <v>1</v>
       </c>
       <c r="F73" t="n">
-        <v>857055.5630100402</v>
+        <v>940000</v>
       </c>
       <c r="G73" t="n">
-        <v>-158999.4369899598</v>
+        <v>107000</v>
       </c>
       <c r="H73" t="n">
-        <v>-15.64870376012714</v>
+        <v>12.84513805522209</v>
       </c>
       <c r="I73" t="inlineStr">
         <is>
-          <t>2026-03-18T14:32:42</t>
+          <t>2026-03-18T21:13:42</t>
         </is>
       </c>
     </row>
@@ -4289,11 +4289,11 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>비에이치아이</t>
+          <t>클리블랜드 클리프스</t>
         </is>
       </c>
       <c r="C74" t="n">
-        <v>8</v>
+        <v>70</v>
       </c>
       <c r="D74" t="inlineStr">
         <is>
@@ -4304,17 +4304,17 @@
         <v>1</v>
       </c>
       <c r="F74" t="n">
-        <v>844800</v>
+        <v>850814.9225377198</v>
       </c>
       <c r="G74" t="n">
-        <v>179685</v>
+        <v>-165240.0774622802</v>
       </c>
       <c r="H74" t="n">
-        <v>27.01562887620938</v>
+        <v>-16.26290677790869</v>
       </c>
       <c r="I74" t="inlineStr">
         <is>
-          <t>2026-03-18T14:32:42</t>
+          <t>2026-03-18T21:13:42</t>
         </is>
       </c>
     </row>
@@ -4326,11 +4326,11 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>하프니아</t>
+          <t>비에이치아이</t>
         </is>
       </c>
       <c r="C75" t="n">
-        <v>80</v>
+        <v>8</v>
       </c>
       <c r="D75" t="inlineStr">
         <is>
@@ -4341,17 +4341,17 @@
         <v>1</v>
       </c>
       <c r="F75" t="n">
-        <v>821489.5606615674</v>
+        <v>844800</v>
       </c>
       <c r="G75" t="n">
-        <v>195758.5606615674</v>
+        <v>179685</v>
       </c>
       <c r="H75" t="n">
-        <v>31.28477902829928</v>
+        <v>27.01562887620938</v>
       </c>
       <c r="I75" t="inlineStr">
         <is>
-          <t>2026-03-18T14:32:42</t>
+          <t>2026-03-18T21:13:42</t>
         </is>
       </c>
     </row>
@@ -4363,11 +4363,11 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>텍사스 퍼시픽 랜드</t>
+          <t>하프니아</t>
         </is>
       </c>
       <c r="C76" t="n">
-        <v>1</v>
+        <v>80</v>
       </c>
       <c r="D76" t="inlineStr">
         <is>
@@ -4378,17 +4378,17 @@
         <v>1</v>
       </c>
       <c r="F76" t="n">
-        <v>794737.7576458007</v>
+        <v>822583.1797722168</v>
       </c>
       <c r="G76" t="n">
-        <v>16146.75764580071</v>
+        <v>196852.1797722168</v>
       </c>
       <c r="H76" t="n">
-        <v>2.073843345967358</v>
+        <v>31.45955366958275</v>
       </c>
       <c r="I76" t="inlineStr">
         <is>
-          <t>2026-03-18T14:32:42</t>
+          <t>2026-03-18T21:13:42</t>
         </is>
       </c>
     </row>
@@ -4400,11 +4400,11 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>노블</t>
+          <t>텍사스 퍼시픽 랜드</t>
         </is>
       </c>
       <c r="C77" t="n">
-        <v>99</v>
+        <v>1</v>
       </c>
       <c r="D77" t="inlineStr">
         <is>
@@ -4415,17 +4415,17 @@
         <v>1</v>
       </c>
       <c r="F77" t="n">
-        <v>40689</v>
+        <v>787635.2983817384</v>
       </c>
       <c r="G77" t="n">
-        <v>-3866519</v>
+        <v>9044.298381738365</v>
       </c>
       <c r="H77" t="n">
-        <v>-98.95861699709869</v>
+        <v>1.161623802707502</v>
       </c>
       <c r="I77" t="inlineStr">
         <is>
-          <t>2026-03-18T14:32:42</t>
+          <t>2026-03-18T21:13:42</t>
         </is>
       </c>
     </row>
@@ -4512,7 +4512,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>2026-03-18T14:32:42</t>
+          <t>2026-03-18T21:13:42</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: portfolio snapshot 2026-03-17 (2026-03-18T21:14:04)
</commit_message>
<xml_diff>
--- a/portfolio_auto.xlsx
+++ b/portfolio_auto.xlsx
@@ -795,11 +795,11 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>삼성화재</t>
+          <t>DL이앤씨</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>9</v>
+        <v>80</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
@@ -810,23 +810,23 @@
         <v>1</v>
       </c>
       <c r="E14" t="n">
-        <v>4446000</v>
+        <v>4128000</v>
       </c>
       <c r="F14" t="n">
-        <v>-185000</v>
+        <v>717000</v>
       </c>
       <c r="G14" t="n">
-        <v>-3.994817534009933</v>
+        <v>21.02022867194371</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>DL이앤씨</t>
+          <t>차코스 에너지 내비게이션</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>80</v>
+        <v>75</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
@@ -837,23 +837,23 @@
         <v>1</v>
       </c>
       <c r="E15" t="n">
-        <v>4128000</v>
+        <v>3986244.634113007</v>
       </c>
       <c r="F15" t="n">
-        <v>717000</v>
+        <v>161596.6341130068</v>
       </c>
       <c r="G15" t="n">
-        <v>21.02022867194371</v>
+        <v>4.225137427366041</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>차코스 에너지 내비게이션</t>
+          <t>동원개발</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>75</v>
+        <v>1360</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
@@ -864,23 +864,23 @@
         <v>1</v>
       </c>
       <c r="E16" t="n">
-        <v>3986244.634113007</v>
+        <v>3978000</v>
       </c>
       <c r="F16" t="n">
-        <v>161596.6341130068</v>
+        <v>240600</v>
       </c>
       <c r="G16" t="n">
-        <v>4.225137427366041</v>
+        <v>6.437630438272596</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>동원개발</t>
+          <t>HD건설기계</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>1360</v>
+        <v>31</v>
       </c>
       <c r="C17" t="inlineStr">
         <is>
@@ -891,23 +891,23 @@
         <v>1</v>
       </c>
       <c r="E17" t="n">
-        <v>3978000</v>
+        <v>3955600</v>
       </c>
       <c r="F17" t="n">
-        <v>240600</v>
+        <v>-79496</v>
       </c>
       <c r="G17" t="n">
-        <v>6.437630438272596</v>
+        <v>-1.970114217852561</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>HD건설기계</t>
+          <t>삼성화재</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>31</v>
+        <v>7</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
@@ -918,13 +918,13 @@
         <v>1</v>
       </c>
       <c r="E18" t="n">
-        <v>3955600</v>
+        <v>3458000</v>
       </c>
       <c r="F18" t="n">
-        <v>-79496</v>
+        <v>-173000</v>
       </c>
       <c r="G18" t="n">
-        <v>-1.970114217852561</v>
+        <v>-4.76452767832553</v>
       </c>
     </row>
     <row r="19">
@@ -1227,11 +1227,11 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>하나금융지주</t>
+          <t>스타 벌크 캐리어스</t>
         </is>
       </c>
       <c r="B30" t="n">
-        <v>15</v>
+        <v>50</v>
       </c>
       <c r="C30" t="inlineStr">
         <is>
@@ -1242,23 +1242,23 @@
         <v>1</v>
       </c>
       <c r="E30" t="n">
-        <v>1717500</v>
+        <v>1693903.148884582</v>
       </c>
       <c r="F30" t="n">
-        <v>35000</v>
+        <v>379550.1488845823</v>
       </c>
       <c r="G30" t="n">
-        <v>2.080237741456166</v>
+        <v>28.87733728188564</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>스타 벌크 캐리어스</t>
+          <t>유나이티드헬스 그룹</t>
         </is>
       </c>
       <c r="B31" t="n">
-        <v>50</v>
+        <v>4</v>
       </c>
       <c r="C31" t="inlineStr">
         <is>
@@ -1269,23 +1269,23 @@
         <v>1</v>
       </c>
       <c r="E31" t="n">
-        <v>1693903.148884582</v>
+        <v>1689920.967345312</v>
       </c>
       <c r="F31" t="n">
-        <v>379550.1488845828</v>
+        <v>-4535.032654687762</v>
       </c>
       <c r="G31" t="n">
-        <v>28.87733728188568</v>
+        <v>-0.2676394462109233</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>유나이티드헬스 그룹</t>
+          <t>케이씨</t>
         </is>
       </c>
       <c r="B32" t="n">
-        <v>4</v>
+        <v>50</v>
       </c>
       <c r="C32" t="inlineStr">
         <is>
@@ -1296,23 +1296,23 @@
         <v>1</v>
       </c>
       <c r="E32" t="n">
-        <v>1689920.967345312</v>
+        <v>1640000</v>
       </c>
       <c r="F32" t="n">
-        <v>-4535.032654687762</v>
+        <v>-9500</v>
       </c>
       <c r="G32" t="n">
-        <v>-0.2676394462109233</v>
+        <v>-0.5759321006365565</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>케이씨</t>
+          <t>하나금융지주</t>
         </is>
       </c>
       <c r="B33" t="n">
-        <v>50</v>
+        <v>10</v>
       </c>
       <c r="C33" t="inlineStr">
         <is>
@@ -1323,13 +1323,13 @@
         <v>1</v>
       </c>
       <c r="E33" t="n">
-        <v>1640000</v>
+        <v>1145000</v>
       </c>
       <c r="F33" t="n">
-        <v>-9500.000000000698</v>
+        <v>36000</v>
       </c>
       <c r="G33" t="n">
-        <v>-0.5759321006365986</v>
+        <v>3.246167718665464</v>
       </c>
     </row>
     <row r="34">
@@ -1538,22 +1538,22 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-03-18</t>
+          <t>2026-03-17</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>31505056</v>
+        <v>33078556</v>
       </c>
       <c r="C2" t="n">
-        <v>6016.63</v>
+        <v>6010.99</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2026-03-18T21:13:42</t>
+          <t>2026-03-18T21:14:04</t>
         </is>
       </c>
       <c r="E2" t="n">
-        <v>1485.880004882812</v>
+        <v>1488.910034179688</v>
       </c>
     </row>
   </sheetData>
@@ -1640,17 +1640,17 @@
         <v>1</v>
       </c>
       <c r="F2" t="n">
-        <v>14082576.9328374</v>
+        <v>14100407.22082324</v>
       </c>
       <c r="G2" t="n">
-        <v>1976027.932837404</v>
+        <v>1993858.220823243</v>
       </c>
       <c r="H2" t="n">
-        <v>16.3219752617976</v>
+        <v>16.46925330102941</v>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>2026-03-18T21:09:28</t>
+          <t>2026-03-18T21:14:04</t>
         </is>
       </c>
     </row>
@@ -1677,17 +1677,17 @@
         <v>1</v>
       </c>
       <c r="F3" t="n">
-        <v>10822406.73782303</v>
+        <v>10713195.03359146</v>
       </c>
       <c r="G3" t="n">
-        <v>-9608.262176971883</v>
+        <v>-118819.9664085377</v>
       </c>
       <c r="H3" t="n">
-        <v>-0.08870244526961865</v>
+        <v>-1.09693317825481</v>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>2026-03-18T21:09:28</t>
+          <t>2026-03-18T21:14:04</t>
         </is>
       </c>
     </row>
@@ -1724,7 +1724,7 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>2026-03-18T21:09:28</t>
+          <t>2026-03-18T21:14:04</t>
         </is>
       </c>
     </row>
@@ -1751,17 +1751,17 @@
         <v>1</v>
       </c>
       <c r="F5" t="n">
-        <v>8440541.129673157</v>
+        <v>8362532.627803192</v>
       </c>
       <c r="G5" t="n">
-        <v>4010677.129673157</v>
+        <v>3932668.627803192</v>
       </c>
       <c r="H5" t="n">
-        <v>90.53725192631549</v>
+        <v>88.77628360155508</v>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>2026-03-18T21:09:28</t>
+          <t>2026-03-18T21:14:04</t>
         </is>
       </c>
     </row>
@@ -1788,17 +1788,17 @@
         <v>1</v>
       </c>
       <c r="F6" t="n">
-        <v>8090014.733635107</v>
+        <v>8074480.025508801</v>
       </c>
       <c r="G6" t="n">
-        <v>1639663.733635107</v>
+        <v>1624129.025508801</v>
       </c>
       <c r="H6" t="n">
-        <v>25.41975984927188</v>
+        <v>25.17892476717626</v>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>2026-03-18T21:09:28</t>
+          <t>2026-03-18T21:14:04</t>
         </is>
       </c>
     </row>
@@ -1825,17 +1825,17 @@
         <v>1</v>
       </c>
       <c r="F7" t="n">
-        <v>7093219.418241119</v>
+        <v>6965062.522888184</v>
       </c>
       <c r="G7" t="n">
-        <v>2965985.418241119</v>
+        <v>2837828.522888184</v>
       </c>
       <c r="H7" t="n">
-        <v>71.86375713713153</v>
+        <v>68.7586049855226</v>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>2026-03-18T21:09:28</t>
+          <t>2026-03-18T21:14:04</t>
         </is>
       </c>
     </row>
@@ -1872,7 +1872,7 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>2026-03-18T21:09:28</t>
+          <t>2026-03-18T21:14:04</t>
         </is>
       </c>
     </row>
@@ -1884,11 +1884,11 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>센트러스 에너지</t>
+          <t>노블</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>21</v>
+        <v>99</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
@@ -1899,17 +1899,17 @@
         <v>1</v>
       </c>
       <c r="F9" t="n">
-        <v>6546958.253894605</v>
+        <v>6862314.14501056</v>
       </c>
       <c r="G9" t="n">
-        <v>315739.2538946057</v>
+        <v>2955106.14501056</v>
       </c>
       <c r="H9" t="n">
-        <v>5.067054357977239</v>
+        <v>75.63216867416733</v>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>2026-03-18T21:09:28</t>
+          <t>2026-03-18T21:14:04</t>
         </is>
       </c>
     </row>
@@ -1921,11 +1921,11 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>타이드워터</t>
+          <t>센트러스 에너지</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>48</v>
+        <v>21</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
@@ -1936,17 +1936,17 @@
         <v>1</v>
       </c>
       <c r="F10" t="n">
-        <v>5456864.752692774</v>
+        <v>6504677.671671314</v>
       </c>
       <c r="G10" t="n">
-        <v>1732319.752692774</v>
+        <v>273458.6716713151</v>
       </c>
       <c r="H10" t="n">
-        <v>46.51090945854524</v>
+        <v>4.38852609210678</v>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>2026-03-18T21:09:28</t>
+          <t>2026-03-18T21:14:04</t>
         </is>
       </c>
     </row>
@@ -1958,11 +1958,11 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>노브</t>
+          <t>타이드워터</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>185</v>
+        <v>48</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
@@ -1973,17 +1973,17 @@
         <v>1</v>
       </c>
       <c r="F11" t="n">
-        <v>5041442.310511444</v>
+        <v>5368424.783017382</v>
       </c>
       <c r="G11" t="n">
-        <v>1731434.310511444</v>
+        <v>1643879.783017382</v>
       </c>
       <c r="H11" t="n">
-        <v>52.30906724429197</v>
+        <v>44.13639204298463</v>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>2026-03-18T21:09:28</t>
+          <t>2026-03-18T21:14:04</t>
         </is>
       </c>
     </row>
@@ -1995,11 +1995,11 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>TIME 코리아밸류업액티브</t>
+          <t>노브</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>201</v>
+        <v>185</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
@@ -2010,17 +2010,17 @@
         <v>1</v>
       </c>
       <c r="F12" t="n">
-        <v>4904400</v>
+        <v>5016702.366485596</v>
       </c>
       <c r="G12" t="n">
-        <v>180603</v>
+        <v>1706694.366485596</v>
       </c>
       <c r="H12" t="n">
-        <v>3.823259128197084</v>
+        <v>51.56163871765855</v>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>2026-03-18T21:09:28</t>
+          <t>2026-03-18T21:14:04</t>
         </is>
       </c>
     </row>
@@ -2032,11 +2032,11 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>오케아니스 에코 탱커스</t>
+          <t>TIME 코리아밸류업액티브</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>65</v>
+        <v>201</v>
       </c>
       <c r="D13" t="inlineStr">
         <is>
@@ -2047,17 +2047,17 @@
         <v>1</v>
       </c>
       <c r="F13" t="n">
-        <v>4575098.725873504</v>
+        <v>4904400</v>
       </c>
       <c r="G13" t="n">
-        <v>2318738.725873504</v>
+        <v>180603</v>
       </c>
       <c r="H13" t="n">
-        <v>102.7645732894354</v>
+        <v>3.823259128197084</v>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>2026-03-18T21:09:28</t>
+          <t>2026-03-18T21:14:04</t>
         </is>
       </c>
     </row>
@@ -2069,11 +2069,11 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>DL이앤씨</t>
+          <t>오케아니스 에코 탱커스</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>80</v>
+        <v>65</v>
       </c>
       <c r="D14" t="inlineStr">
         <is>
@@ -2084,17 +2084,17 @@
         <v>1</v>
       </c>
       <c r="F14" t="n">
-        <v>4128000</v>
+        <v>4584757.166964356</v>
       </c>
       <c r="G14" t="n">
-        <v>717000</v>
+        <v>2328397.166964356</v>
       </c>
       <c r="H14" t="n">
-        <v>21.02022867194371</v>
+        <v>103.1926273717118</v>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>2026-03-18T21:09:28</t>
+          <t>2026-03-18T21:14:04</t>
         </is>
       </c>
     </row>
@@ -2106,11 +2106,11 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>차코스 에너지 내비게이션</t>
+          <t>DL이앤씨</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>75</v>
+        <v>80</v>
       </c>
       <c r="D15" t="inlineStr">
         <is>
@@ -2121,17 +2121,17 @@
         <v>1</v>
       </c>
       <c r="F15" t="n">
-        <v>4007418.271141662</v>
+        <v>4128000</v>
       </c>
       <c r="G15" t="n">
-        <v>182770.2711416623</v>
+        <v>717000</v>
       </c>
       <c r="H15" t="n">
-        <v>4.778747511971357</v>
+        <v>21.02022867194371</v>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>2026-03-18T21:09:28</t>
+          <t>2026-03-18T21:14:04</t>
         </is>
       </c>
     </row>
@@ -2143,11 +2143,11 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>동원개발</t>
+          <t>차코스 에너지 내비게이션</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>1360</v>
+        <v>75</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
@@ -2158,17 +2158,17 @@
         <v>1</v>
       </c>
       <c r="F16" t="n">
-        <v>3978000</v>
+        <v>3986244.634113007</v>
       </c>
       <c r="G16" t="n">
-        <v>240600</v>
+        <v>161596.6341130068</v>
       </c>
       <c r="H16" t="n">
-        <v>6.437630438272596</v>
+        <v>4.225137427366041</v>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>2026-03-18T21:09:28</t>
+          <t>2026-03-18T21:14:04</t>
         </is>
       </c>
     </row>
@@ -2180,11 +2180,11 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>HD건설기계</t>
+          <t>동원개발</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>31</v>
+        <v>1360</v>
       </c>
       <c r="D17" t="inlineStr">
         <is>
@@ -2195,17 +2195,17 @@
         <v>1</v>
       </c>
       <c r="F17" t="n">
-        <v>3955600</v>
+        <v>3978000</v>
       </c>
       <c r="G17" t="n">
-        <v>-79496</v>
+        <v>240600</v>
       </c>
       <c r="H17" t="n">
-        <v>-1.970114217852561</v>
+        <v>6.437630438272596</v>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>2026-03-18T21:09:28</t>
+          <t>2026-03-18T21:14:04</t>
         </is>
       </c>
     </row>
@@ -2217,11 +2217,11 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>삼성화재</t>
+          <t>HD건설기계</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>7</v>
+        <v>31</v>
       </c>
       <c r="D18" t="inlineStr">
         <is>
@@ -2232,17 +2232,17 @@
         <v>1</v>
       </c>
       <c r="F18" t="n">
-        <v>3458000</v>
+        <v>3955600</v>
       </c>
       <c r="G18" t="n">
-        <v>-173000</v>
+        <v>-79496</v>
       </c>
       <c r="H18" t="n">
-        <v>-4.76452767832553</v>
+        <v>-1.970114217852561</v>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>2026-03-18T21:09:28</t>
+          <t>2026-03-18T21:14:04</t>
         </is>
       </c>
     </row>
@@ -2269,17 +2269,17 @@
         <v>1</v>
       </c>
       <c r="F19" t="n">
-        <v>3423839.074937592</v>
+        <v>3502070.421398284</v>
       </c>
       <c r="G19" t="n">
-        <v>1953067.074937592</v>
+        <v>2031298.421398284</v>
       </c>
       <c r="H19" t="n">
-        <v>132.7919674115085</v>
+        <v>138.1110343002372</v>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>2026-03-18T21:09:28</t>
+          <t>2026-03-18T21:14:04</t>
         </is>
       </c>
     </row>
@@ -2291,11 +2291,11 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>더치 브로스</t>
+          <t>삼성화재</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>39</v>
+        <v>7</v>
       </c>
       <c r="D20" t="inlineStr">
         <is>
@@ -2306,17 +2306,17 @@
         <v>1</v>
       </c>
       <c r="F20" t="n">
-        <v>2965846.22503092</v>
+        <v>3458000</v>
       </c>
       <c r="G20" t="n">
-        <v>-224797.7749690795</v>
+        <v>-173000</v>
       </c>
       <c r="H20" t="n">
-        <v>-7.04552983564069</v>
+        <v>-4.76452767832553</v>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>2026-03-18T21:09:28</t>
+          <t>2026-03-18T21:14:04</t>
         </is>
       </c>
     </row>
@@ -2328,11 +2328,11 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>현대제철</t>
+          <t>더치 브로스</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>70</v>
+        <v>39</v>
       </c>
       <c r="D21" t="inlineStr">
         <is>
@@ -2343,17 +2343,17 @@
         <v>1</v>
       </c>
       <c r="F21" t="n">
-        <v>2607500</v>
+        <v>2965846.22503092</v>
       </c>
       <c r="G21" t="n">
-        <v>-200000</v>
+        <v>-224797.7749690795</v>
       </c>
       <c r="H21" t="n">
-        <v>-7.123775601068566</v>
+        <v>-7.04552983564069</v>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>2026-03-18T21:09:28</t>
+          <t>2026-03-18T21:14:04</t>
         </is>
       </c>
     </row>
@@ -2365,11 +2365,11 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>KoAct 코스닥액티브</t>
+          <t>현대제철</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>200</v>
+        <v>70</v>
       </c>
       <c r="D22" t="inlineStr">
         <is>
@@ -2380,17 +2380,17 @@
         <v>1</v>
       </c>
       <c r="F22" t="n">
-        <v>2598000</v>
+        <v>2607500</v>
       </c>
       <c r="G22" t="n">
-        <v>-104000</v>
+        <v>-200000</v>
       </c>
       <c r="H22" t="n">
-        <v>-3.84900074019245</v>
+        <v>-7.123775601068566</v>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>2026-03-18T21:09:28</t>
+          <t>2026-03-18T21:14:04</t>
         </is>
       </c>
     </row>
@@ -2402,11 +2402,11 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>휴스틸</t>
+          <t>KoAct 코스닥액티브</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>500</v>
+        <v>200</v>
       </c>
       <c r="D23" t="inlineStr">
         <is>
@@ -2417,17 +2417,17 @@
         <v>1</v>
       </c>
       <c r="F23" t="n">
-        <v>2560000</v>
+        <v>2598000</v>
       </c>
       <c r="G23" t="n">
-        <v>281390</v>
+        <v>-104000</v>
       </c>
       <c r="H23" t="n">
-        <v>12.34919534277476</v>
+        <v>-3.84900074019245</v>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>2026-03-18T21:09:28</t>
+          <t>2026-03-18T21:14:04</t>
         </is>
       </c>
     </row>
@@ -2439,11 +2439,11 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>넥스틸</t>
+          <t>휴스틸</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>200</v>
+        <v>500</v>
       </c>
       <c r="D24" t="inlineStr">
         <is>
@@ -2454,17 +2454,17 @@
         <v>1</v>
       </c>
       <c r="F24" t="n">
-        <v>2400000</v>
+        <v>2560000</v>
       </c>
       <c r="G24" t="n">
-        <v>389000</v>
+        <v>281390</v>
       </c>
       <c r="H24" t="n">
-        <v>19.34361014420686</v>
+        <v>12.34919534277476</v>
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>2026-03-18T21:09:28</t>
+          <t>2026-03-18T21:14:04</t>
         </is>
       </c>
     </row>
@@ -2476,11 +2476,11 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>대신증권</t>
+          <t>넥스틸</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>55</v>
+        <v>200</v>
       </c>
       <c r="D25" t="inlineStr">
         <is>
@@ -2491,17 +2491,17 @@
         <v>1</v>
       </c>
       <c r="F25" t="n">
-        <v>2238500</v>
+        <v>2400000</v>
       </c>
       <c r="G25" t="n">
-        <v>528999</v>
+        <v>389000</v>
       </c>
       <c r="H25" t="n">
-        <v>30.94464408034859</v>
+        <v>19.34361014420686</v>
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>2026-03-18T21:09:28</t>
+          <t>2026-03-18T21:14:04</t>
         </is>
       </c>
     </row>
@@ -2513,11 +2513,11 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>발레로 에너지</t>
+          <t>대신증권</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>6</v>
+        <v>55</v>
       </c>
       <c r="D26" t="inlineStr">
         <is>
@@ -2528,17 +2528,17 @@
         <v>1</v>
       </c>
       <c r="F26" t="n">
-        <v>2138731.14071836</v>
+        <v>2238500</v>
       </c>
       <c r="G26" t="n">
-        <v>74741.1407183595</v>
+        <v>528999</v>
       </c>
       <c r="H26" t="n">
-        <v>3.621196842928478</v>
+        <v>30.94464408034859</v>
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>2026-03-18T21:09:28</t>
+          <t>2026-03-18T21:14:04</t>
         </is>
       </c>
     </row>
@@ -2550,11 +2550,11 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>미창석유</t>
+          <t>발레로 에너지</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>18</v>
+        <v>6</v>
       </c>
       <c r="D27" t="inlineStr">
         <is>
@@ -2565,17 +2565,17 @@
         <v>1</v>
       </c>
       <c r="F27" t="n">
-        <v>2032200</v>
+        <v>2125937.735642139</v>
       </c>
       <c r="G27" t="n">
-        <v>-360000</v>
+        <v>61947.73564213887</v>
       </c>
       <c r="H27" t="n">
-        <v>-15.04890895410083</v>
+        <v>3.001358322576121</v>
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>2026-03-18T21:09:28</t>
+          <t>2026-03-18T21:14:04</t>
         </is>
       </c>
     </row>
@@ -2587,11 +2587,11 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>대창단조</t>
+          <t>미창석유</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>300</v>
+        <v>18</v>
       </c>
       <c r="D28" t="inlineStr">
         <is>
@@ -2602,17 +2602,17 @@
         <v>1</v>
       </c>
       <c r="F28" t="n">
-        <v>1914000</v>
+        <v>2032200</v>
       </c>
       <c r="G28" t="n">
-        <v>-144000</v>
+        <v>-360000</v>
       </c>
       <c r="H28" t="n">
-        <v>-6.997084548104956</v>
+        <v>-15.04890895410083</v>
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>2026-03-18T21:09:28</t>
+          <t>2026-03-18T21:14:04</t>
         </is>
       </c>
     </row>
@@ -2624,11 +2624,11 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>동방</t>
+          <t>대창단조</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>681</v>
+        <v>300</v>
       </c>
       <c r="D29" t="inlineStr">
         <is>
@@ -2639,17 +2639,17 @@
         <v>1</v>
       </c>
       <c r="F29" t="n">
-        <v>1882965</v>
+        <v>1914000</v>
       </c>
       <c r="G29" t="n">
-        <v>-88536</v>
+        <v>-144000</v>
       </c>
       <c r="H29" t="n">
-        <v>-4.490791533963209</v>
+        <v>-6.997084548104956</v>
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>2026-03-18T21:09:28</t>
+          <t>2026-03-18T21:14:04</t>
         </is>
       </c>
     </row>
@@ -2661,11 +2661,11 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>스타 벌크 캐리어스</t>
+          <t>동방</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>50</v>
+        <v>681</v>
       </c>
       <c r="D30" t="inlineStr">
         <is>
@@ -2676,17 +2676,17 @@
         <v>1</v>
       </c>
       <c r="F30" t="n">
-        <v>1712476.648945617</v>
+        <v>1882965</v>
       </c>
       <c r="G30" t="n">
-        <v>398123.6489456175</v>
+        <v>-88536</v>
       </c>
       <c r="H30" t="n">
-        <v>30.29046602743841</v>
+        <v>-4.490791533963209</v>
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>2026-03-18T21:09:28</t>
+          <t>2026-03-18T21:14:04</t>
         </is>
       </c>
     </row>
@@ -2698,11 +2698,11 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>유나이티드헬스 그룹</t>
+          <t>스타 벌크 캐리어스</t>
         </is>
       </c>
       <c r="C31" t="n">
-        <v>4</v>
+        <v>50</v>
       </c>
       <c r="D31" t="inlineStr">
         <is>
@@ -2713,17 +2713,17 @@
         <v>1</v>
       </c>
       <c r="F31" t="n">
-        <v>1699490.128895313</v>
+        <v>1693903.148884582</v>
       </c>
       <c r="G31" t="n">
-        <v>5034.128895312548</v>
+        <v>379550.1488845823</v>
       </c>
       <c r="H31" t="n">
-        <v>0.297094105442251</v>
+        <v>28.87733728188564</v>
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>2026-03-18T21:09:28</t>
+          <t>2026-03-18T21:14:04</t>
         </is>
       </c>
     </row>
@@ -2735,11 +2735,11 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>케이씨</t>
+          <t>유나이티드헬스 그룹</t>
         </is>
       </c>
       <c r="C32" t="n">
-        <v>50</v>
+        <v>4</v>
       </c>
       <c r="D32" t="inlineStr">
         <is>
@@ -2750,17 +2750,17 @@
         <v>1</v>
       </c>
       <c r="F32" t="n">
-        <v>1640000</v>
+        <v>1689920.967345312</v>
       </c>
       <c r="G32" t="n">
-        <v>-9500</v>
+        <v>-4535.032654687762</v>
       </c>
       <c r="H32" t="n">
-        <v>-0.5759321006365565</v>
+        <v>-0.2676394462109233</v>
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>2026-03-18T21:09:28</t>
+          <t>2026-03-18T21:14:04</t>
         </is>
       </c>
     </row>
@@ -2772,11 +2772,11 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>하나금융지주</t>
+          <t>케이씨</t>
         </is>
       </c>
       <c r="C33" t="n">
-        <v>10</v>
+        <v>50</v>
       </c>
       <c r="D33" t="inlineStr">
         <is>
@@ -2787,17 +2787,17 @@
         <v>1</v>
       </c>
       <c r="F33" t="n">
-        <v>1145000</v>
+        <v>1640000</v>
       </c>
       <c r="G33" t="n">
-        <v>36000</v>
+        <v>-9500</v>
       </c>
       <c r="H33" t="n">
-        <v>3.246167718665464</v>
+        <v>-0.5759321006365565</v>
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>2026-03-18T21:09:28</t>
+          <t>2026-03-18T21:14:04</t>
         </is>
       </c>
     </row>
@@ -2809,11 +2809,11 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>삼성생명</t>
+          <t>하나금융지주</t>
         </is>
       </c>
       <c r="C34" t="n">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="D34" t="inlineStr">
         <is>
@@ -2824,17 +2824,17 @@
         <v>1</v>
       </c>
       <c r="F34" t="n">
-        <v>940000</v>
+        <v>1145000</v>
       </c>
       <c r="G34" t="n">
-        <v>107000</v>
+        <v>36000</v>
       </c>
       <c r="H34" t="n">
-        <v>12.84513805522209</v>
+        <v>3.246167718665464</v>
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>2026-03-18T21:09:28</t>
+          <t>2026-03-18T21:14:04</t>
         </is>
       </c>
     </row>
@@ -2846,11 +2846,11 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>클리블랜드 클리프스</t>
+          <t>삼성생명</t>
         </is>
       </c>
       <c r="C35" t="n">
-        <v>70</v>
+        <v>4</v>
       </c>
       <c r="D35" t="inlineStr">
         <is>
@@ -2861,17 +2861,17 @@
         <v>1</v>
       </c>
       <c r="F35" t="n">
-        <v>857055.5630100402</v>
+        <v>940000</v>
       </c>
       <c r="G35" t="n">
-        <v>-158999.4369899598</v>
+        <v>107000</v>
       </c>
       <c r="H35" t="n">
-        <v>-15.64870376012714</v>
+        <v>12.84513805522209</v>
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>2026-03-18T21:09:28</t>
+          <t>2026-03-18T21:14:04</t>
         </is>
       </c>
     </row>
@@ -2883,11 +2883,11 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>비에이치아이</t>
+          <t>클리블랜드 클리프스</t>
         </is>
       </c>
       <c r="C36" t="n">
-        <v>8</v>
+        <v>70</v>
       </c>
       <c r="D36" t="inlineStr">
         <is>
@@ -2898,17 +2898,17 @@
         <v>1</v>
       </c>
       <c r="F36" t="n">
-        <v>844800</v>
+        <v>850814.9225377198</v>
       </c>
       <c r="G36" t="n">
-        <v>179685</v>
+        <v>-165240.0774622802</v>
       </c>
       <c r="H36" t="n">
-        <v>27.01562887620938</v>
+        <v>-16.26290677790869</v>
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>2026-03-18T21:09:28</t>
+          <t>2026-03-18T21:14:04</t>
         </is>
       </c>
     </row>
@@ -2920,11 +2920,11 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>하프니아</t>
+          <t>비에이치아이</t>
         </is>
       </c>
       <c r="C37" t="n">
-        <v>80</v>
+        <v>8</v>
       </c>
       <c r="D37" t="inlineStr">
         <is>
@@ -2935,17 +2935,17 @@
         <v>1</v>
       </c>
       <c r="F37" t="n">
-        <v>821489.5606615674</v>
+        <v>844800</v>
       </c>
       <c r="G37" t="n">
-        <v>195758.5606615674</v>
+        <v>179685</v>
       </c>
       <c r="H37" t="n">
-        <v>31.28477902829928</v>
+        <v>27.01562887620938</v>
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>2026-03-18T21:09:28</t>
+          <t>2026-03-18T21:14:04</t>
         </is>
       </c>
     </row>
@@ -2957,11 +2957,11 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>텍사스 퍼시픽 랜드</t>
+          <t>하프니아</t>
         </is>
       </c>
       <c r="C38" t="n">
-        <v>1</v>
+        <v>80</v>
       </c>
       <c r="D38" t="inlineStr">
         <is>
@@ -2972,17 +2972,17 @@
         <v>1</v>
       </c>
       <c r="F38" t="n">
-        <v>794737.7576458007</v>
+        <v>822583.1797722168</v>
       </c>
       <c r="G38" t="n">
-        <v>16146.75764580071</v>
+        <v>196852.1797722168</v>
       </c>
       <c r="H38" t="n">
-        <v>2.073843345967358</v>
+        <v>31.45955366958275</v>
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>2026-03-18T21:09:28</t>
+          <t>2026-03-18T21:14:04</t>
         </is>
       </c>
     </row>
@@ -2994,11 +2994,11 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>노블</t>
+          <t>텍사스 퍼시픽 랜드</t>
         </is>
       </c>
       <c r="C39" t="n">
-        <v>99</v>
+        <v>1</v>
       </c>
       <c r="D39" t="inlineStr">
         <is>
@@ -3009,17 +3009,17 @@
         <v>1</v>
       </c>
       <c r="F39" t="n">
-        <v>40689</v>
+        <v>787635.2983817384</v>
       </c>
       <c r="G39" t="n">
-        <v>-3866519</v>
+        <v>9044.298381738365</v>
       </c>
       <c r="H39" t="n">
-        <v>-98.95861699709869</v>
+        <v>1.161623802707502</v>
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>2026-03-18T21:09:28</t>
+          <t>2026-03-18T21:14:04</t>
         </is>
       </c>
     </row>
@@ -4489,7 +4489,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>2026-03-18T21:09:28</t>
+          <t>2026-03-18T21:14:04</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: portfolio snapshot 2026-03-18 (2026-03-18T21:14:30)
</commit_message>
<xml_diff>
--- a/portfolio_auto.xlsx
+++ b/portfolio_auto.xlsx
@@ -660,11 +660,11 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>센트러스 에너지</t>
+          <t>노블</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>21</v>
+        <v>99</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
@@ -675,23 +675,23 @@
         <v>1</v>
       </c>
       <c r="E9" t="n">
-        <v>6504677.671671314</v>
+        <v>6862314.14501056</v>
       </c>
       <c r="F9" t="n">
-        <v>273458.6716713151</v>
+        <v>2955106.14501056</v>
       </c>
       <c r="G9" t="n">
-        <v>4.38852609210678</v>
+        <v>75.63216867416733</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>타이드워터</t>
+          <t>센트러스 에너지</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>48</v>
+        <v>21</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
@@ -702,23 +702,23 @@
         <v>1</v>
       </c>
       <c r="E10" t="n">
-        <v>5368424.783017382</v>
+        <v>6504677.671671314</v>
       </c>
       <c r="F10" t="n">
-        <v>1643879.783017382</v>
+        <v>273458.6716713151</v>
       </c>
       <c r="G10" t="n">
-        <v>44.13639204298463</v>
+        <v>4.38852609210678</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>노브</t>
+          <t>타이드워터</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>185</v>
+        <v>48</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
@@ -729,23 +729,23 @@
         <v>1</v>
       </c>
       <c r="E11" t="n">
-        <v>5016702.366485596</v>
+        <v>5368424.783017382</v>
       </c>
       <c r="F11" t="n">
-        <v>1706694.366485596</v>
+        <v>1643879.783017382</v>
       </c>
       <c r="G11" t="n">
-        <v>51.56163871765855</v>
+        <v>44.13639204298463</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>TIME 코리아밸류업액티브</t>
+          <t>노브</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>201</v>
+        <v>185</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
@@ -756,23 +756,23 @@
         <v>1</v>
       </c>
       <c r="E12" t="n">
-        <v>4904400</v>
+        <v>5016702.366485596</v>
       </c>
       <c r="F12" t="n">
-        <v>180603</v>
+        <v>1706694.366485596</v>
       </c>
       <c r="G12" t="n">
-        <v>3.823259128197084</v>
+        <v>51.56163871765855</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>오케아니스 에코 탱커스</t>
+          <t>TIME 코리아밸류업액티브</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>65</v>
+        <v>201</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
@@ -783,23 +783,23 @@
         <v>1</v>
       </c>
       <c r="E13" t="n">
-        <v>4584757.166964356</v>
+        <v>4904400</v>
       </c>
       <c r="F13" t="n">
-        <v>2328397.166964356</v>
+        <v>180603</v>
       </c>
       <c r="G13" t="n">
-        <v>103.1926273717118</v>
+        <v>3.823259128197084</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>DL이앤씨</t>
+          <t>오케아니스 에코 탱커스</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>80</v>
+        <v>65</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
@@ -810,23 +810,23 @@
         <v>1</v>
       </c>
       <c r="E14" t="n">
-        <v>4128000</v>
+        <v>4584757.166964356</v>
       </c>
       <c r="F14" t="n">
-        <v>717000</v>
+        <v>2328397.166964356</v>
       </c>
       <c r="G14" t="n">
-        <v>21.02022867194371</v>
+        <v>103.1926273717118</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>차코스 에너지 내비게이션</t>
+          <t>삼성화재</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>75</v>
+        <v>9</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
@@ -837,23 +837,23 @@
         <v>1</v>
       </c>
       <c r="E15" t="n">
-        <v>3986244.634113007</v>
+        <v>4446000</v>
       </c>
       <c r="F15" t="n">
-        <v>161596.6341130068</v>
+        <v>-185000</v>
       </c>
       <c r="G15" t="n">
-        <v>4.225137427366041</v>
+        <v>-3.994817534009933</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>동원개발</t>
+          <t>DL이앤씨</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>1360</v>
+        <v>80</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
@@ -864,23 +864,23 @@
         <v>1</v>
       </c>
       <c r="E16" t="n">
-        <v>3978000</v>
+        <v>4128000</v>
       </c>
       <c r="F16" t="n">
-        <v>240600</v>
+        <v>717000</v>
       </c>
       <c r="G16" t="n">
-        <v>6.437630438272596</v>
+        <v>21.02022867194371</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>HD건설기계</t>
+          <t>차코스 에너지 내비게이션</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>31</v>
+        <v>75</v>
       </c>
       <c r="C17" t="inlineStr">
         <is>
@@ -891,23 +891,23 @@
         <v>1</v>
       </c>
       <c r="E17" t="n">
-        <v>3955600</v>
+        <v>3986244.634113007</v>
       </c>
       <c r="F17" t="n">
-        <v>-79496</v>
+        <v>161596.6341130068</v>
       </c>
       <c r="G17" t="n">
-        <v>-1.970114217852561</v>
+        <v>4.225137427366041</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>삼성화재</t>
+          <t>동원개발</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>7</v>
+        <v>1360</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
@@ -918,23 +918,23 @@
         <v>1</v>
       </c>
       <c r="E18" t="n">
-        <v>3458000</v>
+        <v>3978000</v>
       </c>
       <c r="F18" t="n">
-        <v>-173000</v>
+        <v>240600</v>
       </c>
       <c r="G18" t="n">
-        <v>-4.76452767832553</v>
+        <v>6.437630438272596</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>피바디 에너지</t>
+          <t>HD건설기계</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>65</v>
+        <v>31</v>
       </c>
       <c r="C19" t="inlineStr">
         <is>
@@ -945,23 +945,23 @@
         <v>1</v>
       </c>
       <c r="E19" t="n">
-        <v>3502070.421398284</v>
+        <v>3955600</v>
       </c>
       <c r="F19" t="n">
-        <v>2031298.421398284</v>
+        <v>-79496</v>
       </c>
       <c r="G19" t="n">
-        <v>138.1110343002372</v>
+        <v>-1.970114217852561</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>더치 브로스</t>
+          <t>피바디 에너지</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>39</v>
+        <v>65</v>
       </c>
       <c r="C20" t="inlineStr">
         <is>
@@ -972,23 +972,23 @@
         <v>1</v>
       </c>
       <c r="E20" t="n">
-        <v>2965846.22503092</v>
+        <v>3502070.421398284</v>
       </c>
       <c r="F20" t="n">
-        <v>-224797.7749690795</v>
+        <v>2031298.421398284</v>
       </c>
       <c r="G20" t="n">
-        <v>-7.04552983564069</v>
+        <v>138.1110343002372</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>현대제철</t>
+          <t>더치 브로스</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>70</v>
+        <v>39</v>
       </c>
       <c r="C21" t="inlineStr">
         <is>
@@ -999,23 +999,23 @@
         <v>1</v>
       </c>
       <c r="E21" t="n">
-        <v>2607500</v>
+        <v>2965846.22503092</v>
       </c>
       <c r="F21" t="n">
-        <v>-200000</v>
+        <v>-224797.7749690795</v>
       </c>
       <c r="G21" t="n">
-        <v>-7.123775601068566</v>
+        <v>-7.04552983564069</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>KoAct 코스닥액티브</t>
+          <t>현대제철</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>200</v>
+        <v>70</v>
       </c>
       <c r="C22" t="inlineStr">
         <is>
@@ -1026,23 +1026,23 @@
         <v>1</v>
       </c>
       <c r="E22" t="n">
-        <v>2598000</v>
+        <v>2607500</v>
       </c>
       <c r="F22" t="n">
-        <v>-104000</v>
+        <v>-200000</v>
       </c>
       <c r="G22" t="n">
-        <v>-3.84900074019245</v>
+        <v>-7.123775601068566</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>휴스틸</t>
+          <t>KoAct 코스닥액티브</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>500</v>
+        <v>200</v>
       </c>
       <c r="C23" t="inlineStr">
         <is>
@@ -1053,23 +1053,23 @@
         <v>1</v>
       </c>
       <c r="E23" t="n">
-        <v>2560000</v>
+        <v>2598000</v>
       </c>
       <c r="F23" t="n">
-        <v>281390</v>
+        <v>-104000</v>
       </c>
       <c r="G23" t="n">
-        <v>12.34919534277476</v>
+        <v>-3.84900074019245</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>넥스틸</t>
+          <t>휴스틸</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>200</v>
+        <v>500</v>
       </c>
       <c r="C24" t="inlineStr">
         <is>
@@ -1080,23 +1080,23 @@
         <v>1</v>
       </c>
       <c r="E24" t="n">
-        <v>2400000</v>
+        <v>2560000</v>
       </c>
       <c r="F24" t="n">
-        <v>389000</v>
+        <v>281390</v>
       </c>
       <c r="G24" t="n">
-        <v>19.34361014420686</v>
+        <v>12.34919534277476</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>대신증권</t>
+          <t>넥스틸</t>
         </is>
       </c>
       <c r="B25" t="n">
-        <v>55</v>
+        <v>200</v>
       </c>
       <c r="C25" t="inlineStr">
         <is>
@@ -1107,23 +1107,23 @@
         <v>1</v>
       </c>
       <c r="E25" t="n">
-        <v>2238500</v>
+        <v>2400000</v>
       </c>
       <c r="F25" t="n">
-        <v>528999</v>
+        <v>389000</v>
       </c>
       <c r="G25" t="n">
-        <v>30.94464408034859</v>
+        <v>19.34361014420686</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>발레로 에너지</t>
+          <t>대신증권</t>
         </is>
       </c>
       <c r="B26" t="n">
-        <v>6</v>
+        <v>55</v>
       </c>
       <c r="C26" t="inlineStr">
         <is>
@@ -1134,23 +1134,23 @@
         <v>1</v>
       </c>
       <c r="E26" t="n">
-        <v>2125937.735642139</v>
+        <v>2238500</v>
       </c>
       <c r="F26" t="n">
-        <v>61947.73564213887</v>
+        <v>528999</v>
       </c>
       <c r="G26" t="n">
-        <v>3.001358322576121</v>
+        <v>30.94464408034859</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>미창석유</t>
+          <t>발레로 에너지</t>
         </is>
       </c>
       <c r="B27" t="n">
-        <v>18</v>
+        <v>6</v>
       </c>
       <c r="C27" t="inlineStr">
         <is>
@@ -1161,23 +1161,23 @@
         <v>1</v>
       </c>
       <c r="E27" t="n">
-        <v>2032200</v>
+        <v>2125937.735642139</v>
       </c>
       <c r="F27" t="n">
-        <v>-360000</v>
+        <v>61947.73564213887</v>
       </c>
       <c r="G27" t="n">
-        <v>-15.04890895410083</v>
+        <v>3.001358322576121</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>대창단조</t>
+          <t>미창석유</t>
         </is>
       </c>
       <c r="B28" t="n">
-        <v>300</v>
+        <v>18</v>
       </c>
       <c r="C28" t="inlineStr">
         <is>
@@ -1188,23 +1188,23 @@
         <v>1</v>
       </c>
       <c r="E28" t="n">
-        <v>1914000</v>
+        <v>2032200</v>
       </c>
       <c r="F28" t="n">
-        <v>-144000</v>
+        <v>-360000</v>
       </c>
       <c r="G28" t="n">
-        <v>-6.997084548104956</v>
+        <v>-15.04890895410083</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>동방</t>
+          <t>대창단조</t>
         </is>
       </c>
       <c r="B29" t="n">
-        <v>681</v>
+        <v>300</v>
       </c>
       <c r="C29" t="inlineStr">
         <is>
@@ -1215,23 +1215,23 @@
         <v>1</v>
       </c>
       <c r="E29" t="n">
-        <v>1882965</v>
+        <v>1914000</v>
       </c>
       <c r="F29" t="n">
-        <v>-88536</v>
+        <v>-144000</v>
       </c>
       <c r="G29" t="n">
-        <v>-4.490791533963209</v>
+        <v>-6.997084548104956</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>스타 벌크 캐리어스</t>
+          <t>동방</t>
         </is>
       </c>
       <c r="B30" t="n">
-        <v>50</v>
+        <v>681</v>
       </c>
       <c r="C30" t="inlineStr">
         <is>
@@ -1242,23 +1242,23 @@
         <v>1</v>
       </c>
       <c r="E30" t="n">
-        <v>1693903.148884582</v>
+        <v>1882965</v>
       </c>
       <c r="F30" t="n">
-        <v>379550.1488845823</v>
+        <v>-88536</v>
       </c>
       <c r="G30" t="n">
-        <v>28.87733728188564</v>
+        <v>-4.490791533963209</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>유나이티드헬스 그룹</t>
+          <t>하나금융지주</t>
         </is>
       </c>
       <c r="B31" t="n">
-        <v>4</v>
+        <v>15</v>
       </c>
       <c r="C31" t="inlineStr">
         <is>
@@ -1269,19 +1269,19 @@
         <v>1</v>
       </c>
       <c r="E31" t="n">
-        <v>1689920.967345312</v>
+        <v>1717500</v>
       </c>
       <c r="F31" t="n">
-        <v>-4535.032654687762</v>
+        <v>35000</v>
       </c>
       <c r="G31" t="n">
-        <v>-0.2676394462109233</v>
+        <v>2.080237741456166</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>케이씨</t>
+          <t>스타 벌크 캐리어스</t>
         </is>
       </c>
       <c r="B32" t="n">
@@ -1296,23 +1296,23 @@
         <v>1</v>
       </c>
       <c r="E32" t="n">
-        <v>1640000</v>
+        <v>1693903.148884582</v>
       </c>
       <c r="F32" t="n">
-        <v>-9500</v>
+        <v>379550.1488845828</v>
       </c>
       <c r="G32" t="n">
-        <v>-0.5759321006365565</v>
+        <v>28.87733728188568</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>하나금융지주</t>
+          <t>유나이티드헬스 그룹</t>
         </is>
       </c>
       <c r="B33" t="n">
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="C33" t="inlineStr">
         <is>
@@ -1323,23 +1323,23 @@
         <v>1</v>
       </c>
       <c r="E33" t="n">
-        <v>1145000</v>
+        <v>1689920.967345312</v>
       </c>
       <c r="F33" t="n">
-        <v>36000</v>
+        <v>-4535.032654687762</v>
       </c>
       <c r="G33" t="n">
-        <v>3.246167718665464</v>
+        <v>-0.2676394462109233</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>삼성생명</t>
+          <t>케이씨</t>
         </is>
       </c>
       <c r="B34" t="n">
-        <v>4</v>
+        <v>50</v>
       </c>
       <c r="C34" t="inlineStr">
         <is>
@@ -1350,23 +1350,23 @@
         <v>1</v>
       </c>
       <c r="E34" t="n">
-        <v>940000</v>
+        <v>1640000</v>
       </c>
       <c r="F34" t="n">
-        <v>107000</v>
+        <v>-9500.000000000698</v>
       </c>
       <c r="G34" t="n">
-        <v>12.84513805522209</v>
+        <v>-0.5759321006365986</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>클리블랜드 클리프스</t>
+          <t>삼성생명</t>
         </is>
       </c>
       <c r="B35" t="n">
-        <v>70</v>
+        <v>4</v>
       </c>
       <c r="C35" t="inlineStr">
         <is>
@@ -1377,23 +1377,23 @@
         <v>1</v>
       </c>
       <c r="E35" t="n">
-        <v>850814.9225377198</v>
+        <v>940000</v>
       </c>
       <c r="F35" t="n">
-        <v>-165240.0774622802</v>
+        <v>107000</v>
       </c>
       <c r="G35" t="n">
-        <v>-16.26290677790869</v>
+        <v>12.84513805522209</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>비에이치아이</t>
+          <t>클리블랜드 클리프스</t>
         </is>
       </c>
       <c r="B36" t="n">
-        <v>8</v>
+        <v>70</v>
       </c>
       <c r="C36" t="inlineStr">
         <is>
@@ -1404,23 +1404,23 @@
         <v>1</v>
       </c>
       <c r="E36" t="n">
-        <v>844800</v>
+        <v>850814.9225377198</v>
       </c>
       <c r="F36" t="n">
-        <v>179685</v>
+        <v>-165240.0774622802</v>
       </c>
       <c r="G36" t="n">
-        <v>27.01562887620938</v>
+        <v>-16.26290677790869</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>하프니아</t>
+          <t>비에이치아이</t>
         </is>
       </c>
       <c r="B37" t="n">
-        <v>80</v>
+        <v>8</v>
       </c>
       <c r="C37" t="inlineStr">
         <is>
@@ -1431,23 +1431,23 @@
         <v>1</v>
       </c>
       <c r="E37" t="n">
-        <v>822583.1797722168</v>
+        <v>844800</v>
       </c>
       <c r="F37" t="n">
-        <v>196852.1797722168</v>
+        <v>179685</v>
       </c>
       <c r="G37" t="n">
-        <v>31.45955366958275</v>
+        <v>27.01562887620938</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>텍사스 퍼시픽 랜드</t>
+          <t>하프니아</t>
         </is>
       </c>
       <c r="B38" t="n">
-        <v>1</v>
+        <v>80</v>
       </c>
       <c r="C38" t="inlineStr">
         <is>
@@ -1458,23 +1458,23 @@
         <v>1</v>
       </c>
       <c r="E38" t="n">
-        <v>787635.2983817384</v>
+        <v>822583.1797722168</v>
       </c>
       <c r="F38" t="n">
-        <v>9044.298381738365</v>
+        <v>196852.1797722168</v>
       </c>
       <c r="G38" t="n">
-        <v>1.161623802707502</v>
+        <v>31.45955366958275</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>노블</t>
+          <t>텍사스 퍼시픽 랜드</t>
         </is>
       </c>
       <c r="B39" t="n">
-        <v>99</v>
+        <v>1</v>
       </c>
       <c r="C39" t="inlineStr">
         <is>
@@ -1485,13 +1485,13 @@
         <v>1</v>
       </c>
       <c r="E39" t="n">
-        <v>6862314.14501056</v>
+        <v>787635.2983817384</v>
       </c>
       <c r="F39" t="n">
-        <v>2955106.14501056</v>
+        <v>9044.298381738365</v>
       </c>
       <c r="G39" t="n">
-        <v>75.63216867416733</v>
+        <v>1.161623802707502</v>
       </c>
     </row>
   </sheetData>
@@ -1538,22 +1538,22 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-03-17</t>
+          <t>2026-03-18</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>33078556</v>
+        <v>31505056</v>
       </c>
       <c r="C2" t="n">
-        <v>6010.99</v>
+        <v>6016.63</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2026-03-18T21:14:04</t>
+          <t>2026-03-18T21:14:30</t>
         </is>
       </c>
       <c r="E2" t="n">
-        <v>1488.910034179688</v>
+        <v>1485.880004882812</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
auto: portfolio snapshot 2026-03-19 (2026-03-19T00:07:11)
</commit_message>
<xml_diff>
--- a/portfolio_auto.xlsx
+++ b/portfolio_auto.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="보유현황" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="메타" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="스냅샷_보유현황" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="스냅샷_예수금" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="보유현황" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="메타" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="스냅샷_보유현황" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="스냅샷_예수금" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -486,13 +486,13 @@
         <v>1</v>
       </c>
       <c r="E2" t="n">
-        <v>14100407.22082324</v>
+        <v>14231364.16721486</v>
       </c>
       <c r="F2" t="n">
-        <v>1993858.220823243</v>
+        <v>2124815.167214859</v>
       </c>
       <c r="G2" t="n">
-        <v>16.46925330102941</v>
+        <v>17.55095665341841</v>
       </c>
     </row>
     <row r="3">
@@ -513,13 +513,13 @@
         <v>1</v>
       </c>
       <c r="E3" t="n">
-        <v>10713195.03359146</v>
+        <v>10812693.38748475</v>
       </c>
       <c r="F3" t="n">
-        <v>-118819.9664085377</v>
+        <v>-19321.61251525022</v>
       </c>
       <c r="G3" t="n">
-        <v>-1.09693317825481</v>
+        <v>-0.178375053166472</v>
       </c>
     </row>
     <row r="4">
@@ -567,13 +567,13 @@
         <v>1</v>
       </c>
       <c r="E5" t="n">
-        <v>8362532.627803192</v>
+        <v>8440199.302239379</v>
       </c>
       <c r="F5" t="n">
-        <v>3932668.627803192</v>
+        <v>4010335.302239379</v>
       </c>
       <c r="G5" t="n">
-        <v>88.77628360155508</v>
+        <v>90.52953549452938</v>
       </c>
     </row>
     <row r="6">
@@ -594,13 +594,13 @@
         <v>1</v>
       </c>
       <c r="E6" t="n">
-        <v>8074480.025508801</v>
+        <v>8149471.423365676</v>
       </c>
       <c r="F6" t="n">
-        <v>1624129.025508801</v>
+        <v>1699120.423365676</v>
       </c>
       <c r="G6" t="n">
-        <v>25.17892476717626</v>
+        <v>26.34151883154383</v>
       </c>
     </row>
     <row r="7">
@@ -621,13 +621,13 @@
         <v>1</v>
       </c>
       <c r="E7" t="n">
-        <v>6965062.522888184</v>
+        <v>7029750.25177002</v>
       </c>
       <c r="F7" t="n">
-        <v>2837828.522888184</v>
+        <v>2902516.25177002</v>
       </c>
       <c r="G7" t="n">
-        <v>68.7586049855226</v>
+        <v>70.32594351980092</v>
       </c>
     </row>
     <row r="8">
@@ -675,13 +675,13 @@
         <v>1</v>
       </c>
       <c r="E9" t="n">
-        <v>6862314.14501056</v>
+        <v>6926047.602600594</v>
       </c>
       <c r="F9" t="n">
-        <v>2955106.14501056</v>
+        <v>3018839.602600594</v>
       </c>
       <c r="G9" t="n">
-        <v>75.63216867416733</v>
+        <v>77.2633451457049</v>
       </c>
     </row>
     <row r="10">
@@ -702,13 +702,13 @@
         <v>1</v>
       </c>
       <c r="E10" t="n">
-        <v>6504677.671671314</v>
+        <v>6565089.595369929</v>
       </c>
       <c r="F10" t="n">
-        <v>273458.6716713151</v>
+        <v>333870.5953699304</v>
       </c>
       <c r="G10" t="n">
-        <v>4.38852609210678</v>
+        <v>5.358030192325618</v>
       </c>
     </row>
     <row r="11">
@@ -729,13 +729,13 @@
         <v>1</v>
       </c>
       <c r="E11" t="n">
-        <v>5368424.783017382</v>
+        <v>5418283.805207804</v>
       </c>
       <c r="F11" t="n">
-        <v>1643879.783017382</v>
+        <v>1693738.805207804</v>
       </c>
       <c r="G11" t="n">
-        <v>44.13639204298463</v>
+        <v>45.47505279726259</v>
       </c>
     </row>
     <row r="12">
@@ -756,13 +756,13 @@
         <v>1</v>
       </c>
       <c r="E12" t="n">
-        <v>5016702.366485596</v>
+        <v>5063294.781341553</v>
       </c>
       <c r="F12" t="n">
-        <v>1706694.366485596</v>
+        <v>1753286.781341553</v>
       </c>
       <c r="G12" t="n">
-        <v>51.56163871765855</v>
+        <v>52.96926114201393</v>
       </c>
     </row>
     <row r="13">
@@ -810,13 +810,13 @@
         <v>1</v>
       </c>
       <c r="E14" t="n">
-        <v>4584757.166964356</v>
+        <v>4627337.908720952</v>
       </c>
       <c r="F14" t="n">
-        <v>2328397.166964356</v>
+        <v>2370977.908720952</v>
       </c>
       <c r="G14" t="n">
-        <v>103.1926273717118</v>
+        <v>105.0797704586569</v>
       </c>
     </row>
     <row r="15">
@@ -891,13 +891,13 @@
         <v>1</v>
       </c>
       <c r="E17" t="n">
-        <v>3986244.634113007</v>
+        <v>4023266.715580446</v>
       </c>
       <c r="F17" t="n">
-        <v>161596.6341130068</v>
+        <v>198618.7155804457</v>
       </c>
       <c r="G17" t="n">
-        <v>4.225137427366041</v>
+        <v>5.193124062147567</v>
       </c>
     </row>
     <row r="18">
@@ -972,13 +972,13 @@
         <v>1</v>
       </c>
       <c r="E20" t="n">
-        <v>3502070.421398284</v>
+        <v>3534595.754975702</v>
       </c>
       <c r="F20" t="n">
-        <v>2031298.421398284</v>
+        <v>2063823.754975702</v>
       </c>
       <c r="G20" t="n">
-        <v>138.1110343002372</v>
+        <v>140.3224806411668</v>
       </c>
     </row>
     <row r="21">
@@ -999,13 +999,13 @@
         <v>1</v>
       </c>
       <c r="E21" t="n">
-        <v>2965846.22503092</v>
+        <v>2993391.398657081</v>
       </c>
       <c r="F21" t="n">
-        <v>-224797.7749690795</v>
+        <v>-197252.6013429193</v>
       </c>
       <c r="G21" t="n">
-        <v>-7.04552983564069</v>
+        <v>-6.182219054928074</v>
       </c>
     </row>
     <row r="22">
@@ -1161,13 +1161,13 @@
         <v>1</v>
       </c>
       <c r="E27" t="n">
-        <v>2125937.735642139</v>
+        <v>2145682.294059377</v>
       </c>
       <c r="F27" t="n">
-        <v>61947.73564213887</v>
+        <v>81692.29405937716</v>
       </c>
       <c r="G27" t="n">
-        <v>3.001358322576121</v>
+        <v>3.957979159752575</v>
       </c>
     </row>
     <row r="28">
@@ -1296,13 +1296,13 @@
         <v>1</v>
       </c>
       <c r="E32" t="n">
-        <v>1693903.148884582</v>
+        <v>1709635.204022215</v>
       </c>
       <c r="F32" t="n">
-        <v>379550.1488845828</v>
+        <v>395282.2040222154</v>
       </c>
       <c r="G32" t="n">
-        <v>28.87733728188568</v>
+        <v>30.0742801988671</v>
       </c>
     </row>
     <row r="33">
@@ -1323,13 +1323,13 @@
         <v>1</v>
       </c>
       <c r="E33" t="n">
-        <v>1689920.967345312</v>
+        <v>1705616.038137302</v>
       </c>
       <c r="F33" t="n">
-        <v>-4535.032654687762</v>
+        <v>11160.03813730204</v>
       </c>
       <c r="G33" t="n">
-        <v>-0.2676394462109233</v>
+        <v>0.6586207099683933</v>
       </c>
     </row>
     <row r="34">
@@ -1404,13 +1404,13 @@
         <v>1</v>
       </c>
       <c r="E36" t="n">
-        <v>850814.9225377198</v>
+        <v>858716.8307915051</v>
       </c>
       <c r="F36" t="n">
-        <v>-165240.0774622802</v>
+        <v>-157338.1692084949</v>
       </c>
       <c r="G36" t="n">
-        <v>-16.26290677790869</v>
+        <v>-15.48520200269621</v>
       </c>
     </row>
     <row r="37">
@@ -1458,13 +1458,13 @@
         <v>1</v>
       </c>
       <c r="E38" t="n">
-        <v>822583.1797722168</v>
+        <v>830222.8868876956</v>
       </c>
       <c r="F38" t="n">
-        <v>196852.1797722168</v>
+        <v>204491.8868876956</v>
       </c>
       <c r="G38" t="n">
-        <v>31.45955366958275</v>
+        <v>32.68047881401044</v>
       </c>
     </row>
     <row r="39">
@@ -1485,13 +1485,13 @@
         <v>1</v>
       </c>
       <c r="E39" t="n">
-        <v>787635.2983817384</v>
+        <v>794950.4285003915</v>
       </c>
       <c r="F39" t="n">
-        <v>9044.298381738365</v>
+        <v>16359.42850039154</v>
       </c>
       <c r="G39" t="n">
-        <v>1.161623802707502</v>
+        <v>2.101158181945533</v>
       </c>
     </row>
   </sheetData>
@@ -1538,7 +1538,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-03-18</t>
+          <t>2026-03-19</t>
         </is>
       </c>
       <c r="B2" t="n">
@@ -1549,11 +1549,11 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2026-03-18T21:14:30</t>
+          <t>2026-03-19T00:07:11</t>
         </is>
       </c>
       <c r="E2" t="n">
-        <v>1485.880004882812</v>
+        <v>1499.680053710938</v>
       </c>
     </row>
   </sheetData>
@@ -1567,7 +1567,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I77"/>
+  <dimension ref="A1:I115"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4426,6 +4426,1412 @@
       <c r="I77" t="inlineStr">
         <is>
           <t>2026-03-18T21:13:42</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>2026-03-19</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>페트로브라스 (ADR)</t>
+        </is>
+      </c>
+      <c r="C78" t="n">
+        <v>480</v>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E78" t="n">
+        <v>1</v>
+      </c>
+      <c r="F78" t="n">
+        <v>14231364.16721486</v>
+      </c>
+      <c r="G78" t="n">
+        <v>2124815.167214859</v>
+      </c>
+      <c r="H78" t="n">
+        <v>17.55095665341841</v>
+      </c>
+      <c r="I78" t="inlineStr">
+        <is>
+          <t>2026-03-19T00:07:11</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>2026-03-19</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>AGNC 인베스트먼트</t>
+        </is>
+      </c>
+      <c r="C79" t="n">
+        <v>700</v>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E79" t="n">
+        <v>1</v>
+      </c>
+      <c r="F79" t="n">
+        <v>10812693.38748475</v>
+      </c>
+      <c r="G79" t="n">
+        <v>-19321.61251525022</v>
+      </c>
+      <c r="H79" t="n">
+        <v>-0.178375053166472</v>
+      </c>
+      <c r="I79" t="inlineStr">
+        <is>
+          <t>2026-03-19T00:07:11</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>2026-03-19</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>대한조선</t>
+        </is>
+      </c>
+      <c r="C80" t="n">
+        <v>100</v>
+      </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E80" t="n">
+        <v>1</v>
+      </c>
+      <c r="F80" t="n">
+        <v>9570000</v>
+      </c>
+      <c r="G80" t="n">
+        <v>2357000</v>
+      </c>
+      <c r="H80" t="n">
+        <v>32.67711077221684</v>
+      </c>
+      <c r="I80" t="inlineStr">
+        <is>
+          <t>2026-03-19T00:07:11</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>2026-03-19</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>프론트라인</t>
+        </is>
+      </c>
+      <c r="C81" t="n">
+        <v>175</v>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E81" t="n">
+        <v>1</v>
+      </c>
+      <c r="F81" t="n">
+        <v>8440199.302239379</v>
+      </c>
+      <c r="G81" t="n">
+        <v>4010335.302239379</v>
+      </c>
+      <c r="H81" t="n">
+        <v>90.52953549452938</v>
+      </c>
+      <c r="I81" t="inlineStr">
+        <is>
+          <t>2026-03-19T00:07:11</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>2026-03-19</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>시드릴</t>
+        </is>
+      </c>
+      <c r="C82" t="n">
+        <v>123</v>
+      </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E82" t="n">
+        <v>1</v>
+      </c>
+      <c r="F82" t="n">
+        <v>8149471.423365676</v>
+      </c>
+      <c r="G82" t="n">
+        <v>1699120.423365676</v>
+      </c>
+      <c r="H82" t="n">
+        <v>26.34151883154383</v>
+      </c>
+      <c r="I82" t="inlineStr">
+        <is>
+          <t>2026-03-19T00:07:11</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>2026-03-19</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>트랜스오션</t>
+        </is>
+      </c>
+      <c r="C83" t="n">
+        <v>750</v>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E83" t="n">
+        <v>1</v>
+      </c>
+      <c r="F83" t="n">
+        <v>7029750.25177002</v>
+      </c>
+      <c r="G83" t="n">
+        <v>2902516.25177002</v>
+      </c>
+      <c r="H83" t="n">
+        <v>70.32594351980092</v>
+      </c>
+      <c r="I83" t="inlineStr">
+        <is>
+          <t>2026-03-19T00:07:11</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>2026-03-19</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>노블</t>
+        </is>
+      </c>
+      <c r="C84" t="n">
+        <v>99</v>
+      </c>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E84" t="n">
+        <v>1</v>
+      </c>
+      <c r="F84" t="n">
+        <v>6926047.602600594</v>
+      </c>
+      <c r="G84" t="n">
+        <v>3018839.602600594</v>
+      </c>
+      <c r="H84" t="n">
+        <v>77.2633451457049</v>
+      </c>
+      <c r="I84" t="inlineStr">
+        <is>
+          <t>2026-03-19T00:07:11</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>2026-03-19</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>세아제강</t>
+        </is>
+      </c>
+      <c r="C85" t="n">
+        <v>50</v>
+      </c>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E85" t="n">
+        <v>1</v>
+      </c>
+      <c r="F85" t="n">
+        <v>6915000</v>
+      </c>
+      <c r="G85" t="n">
+        <v>605000</v>
+      </c>
+      <c r="H85" t="n">
+        <v>9.587955625990491</v>
+      </c>
+      <c r="I85" t="inlineStr">
+        <is>
+          <t>2026-03-19T00:07:11</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>2026-03-19</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>센트러스 에너지</t>
+        </is>
+      </c>
+      <c r="C86" t="n">
+        <v>21</v>
+      </c>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E86" t="n">
+        <v>1</v>
+      </c>
+      <c r="F86" t="n">
+        <v>6565089.595369929</v>
+      </c>
+      <c r="G86" t="n">
+        <v>333870.5953699304</v>
+      </c>
+      <c r="H86" t="n">
+        <v>5.358030192325618</v>
+      </c>
+      <c r="I86" t="inlineStr">
+        <is>
+          <t>2026-03-19T00:07:11</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>2026-03-19</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>타이드워터</t>
+        </is>
+      </c>
+      <c r="C87" t="n">
+        <v>48</v>
+      </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E87" t="n">
+        <v>1</v>
+      </c>
+      <c r="F87" t="n">
+        <v>5418283.805207804</v>
+      </c>
+      <c r="G87" t="n">
+        <v>1693738.805207804</v>
+      </c>
+      <c r="H87" t="n">
+        <v>45.47505279726259</v>
+      </c>
+      <c r="I87" t="inlineStr">
+        <is>
+          <t>2026-03-19T00:07:11</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>2026-03-19</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>노브</t>
+        </is>
+      </c>
+      <c r="C88" t="n">
+        <v>185</v>
+      </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E88" t="n">
+        <v>1</v>
+      </c>
+      <c r="F88" t="n">
+        <v>5063294.781341553</v>
+      </c>
+      <c r="G88" t="n">
+        <v>1753286.781341553</v>
+      </c>
+      <c r="H88" t="n">
+        <v>52.96926114201393</v>
+      </c>
+      <c r="I88" t="inlineStr">
+        <is>
+          <t>2026-03-19T00:07:11</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>2026-03-19</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>TIME 코리아밸류업액티브</t>
+        </is>
+      </c>
+      <c r="C89" t="n">
+        <v>201</v>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E89" t="n">
+        <v>1</v>
+      </c>
+      <c r="F89" t="n">
+        <v>4904400</v>
+      </c>
+      <c r="G89" t="n">
+        <v>180603</v>
+      </c>
+      <c r="H89" t="n">
+        <v>3.823259128197084</v>
+      </c>
+      <c r="I89" t="inlineStr">
+        <is>
+          <t>2026-03-19T00:07:11</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>2026-03-19</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>오케아니스 에코 탱커스</t>
+        </is>
+      </c>
+      <c r="C90" t="n">
+        <v>65</v>
+      </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E90" t="n">
+        <v>1</v>
+      </c>
+      <c r="F90" t="n">
+        <v>4627337.908720952</v>
+      </c>
+      <c r="G90" t="n">
+        <v>2370977.908720952</v>
+      </c>
+      <c r="H90" t="n">
+        <v>105.0797704586569</v>
+      </c>
+      <c r="I90" t="inlineStr">
+        <is>
+          <t>2026-03-19T00:07:11</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>2026-03-19</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>삼성화재</t>
+        </is>
+      </c>
+      <c r="C91" t="n">
+        <v>9</v>
+      </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E91" t="n">
+        <v>1</v>
+      </c>
+      <c r="F91" t="n">
+        <v>4446000</v>
+      </c>
+      <c r="G91" t="n">
+        <v>-185000</v>
+      </c>
+      <c r="H91" t="n">
+        <v>-3.994817534009933</v>
+      </c>
+      <c r="I91" t="inlineStr">
+        <is>
+          <t>2026-03-19T00:07:11</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>2026-03-19</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>DL이앤씨</t>
+        </is>
+      </c>
+      <c r="C92" t="n">
+        <v>80</v>
+      </c>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E92" t="n">
+        <v>1</v>
+      </c>
+      <c r="F92" t="n">
+        <v>4128000</v>
+      </c>
+      <c r="G92" t="n">
+        <v>717000</v>
+      </c>
+      <c r="H92" t="n">
+        <v>21.02022867194371</v>
+      </c>
+      <c r="I92" t="inlineStr">
+        <is>
+          <t>2026-03-19T00:07:11</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>2026-03-19</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>차코스 에너지 내비게이션</t>
+        </is>
+      </c>
+      <c r="C93" t="n">
+        <v>75</v>
+      </c>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E93" t="n">
+        <v>1</v>
+      </c>
+      <c r="F93" t="n">
+        <v>4023266.715580446</v>
+      </c>
+      <c r="G93" t="n">
+        <v>198618.7155804457</v>
+      </c>
+      <c r="H93" t="n">
+        <v>5.193124062147567</v>
+      </c>
+      <c r="I93" t="inlineStr">
+        <is>
+          <t>2026-03-19T00:07:11</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>2026-03-19</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>동원개발</t>
+        </is>
+      </c>
+      <c r="C94" t="n">
+        <v>1360</v>
+      </c>
+      <c r="D94" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E94" t="n">
+        <v>1</v>
+      </c>
+      <c r="F94" t="n">
+        <v>3978000</v>
+      </c>
+      <c r="G94" t="n">
+        <v>240600</v>
+      </c>
+      <c r="H94" t="n">
+        <v>6.437630438272596</v>
+      </c>
+      <c r="I94" t="inlineStr">
+        <is>
+          <t>2026-03-19T00:07:11</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>2026-03-19</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>HD건설기계</t>
+        </is>
+      </c>
+      <c r="C95" t="n">
+        <v>31</v>
+      </c>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E95" t="n">
+        <v>1</v>
+      </c>
+      <c r="F95" t="n">
+        <v>3955600</v>
+      </c>
+      <c r="G95" t="n">
+        <v>-79496</v>
+      </c>
+      <c r="H95" t="n">
+        <v>-1.970114217852561</v>
+      </c>
+      <c r="I95" t="inlineStr">
+        <is>
+          <t>2026-03-19T00:07:11</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>2026-03-19</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>피바디 에너지</t>
+        </is>
+      </c>
+      <c r="C96" t="n">
+        <v>65</v>
+      </c>
+      <c r="D96" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E96" t="n">
+        <v>1</v>
+      </c>
+      <c r="F96" t="n">
+        <v>3534595.754975702</v>
+      </c>
+      <c r="G96" t="n">
+        <v>2063823.754975702</v>
+      </c>
+      <c r="H96" t="n">
+        <v>140.3224806411668</v>
+      </c>
+      <c r="I96" t="inlineStr">
+        <is>
+          <t>2026-03-19T00:07:11</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>2026-03-19</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>더치 브로스</t>
+        </is>
+      </c>
+      <c r="C97" t="n">
+        <v>39</v>
+      </c>
+      <c r="D97" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E97" t="n">
+        <v>1</v>
+      </c>
+      <c r="F97" t="n">
+        <v>2993391.398657081</v>
+      </c>
+      <c r="G97" t="n">
+        <v>-197252.6013429193</v>
+      </c>
+      <c r="H97" t="n">
+        <v>-6.182219054928074</v>
+      </c>
+      <c r="I97" t="inlineStr">
+        <is>
+          <t>2026-03-19T00:07:11</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>2026-03-19</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>현대제철</t>
+        </is>
+      </c>
+      <c r="C98" t="n">
+        <v>70</v>
+      </c>
+      <c r="D98" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E98" t="n">
+        <v>1</v>
+      </c>
+      <c r="F98" t="n">
+        <v>2607500</v>
+      </c>
+      <c r="G98" t="n">
+        <v>-200000</v>
+      </c>
+      <c r="H98" t="n">
+        <v>-7.123775601068566</v>
+      </c>
+      <c r="I98" t="inlineStr">
+        <is>
+          <t>2026-03-19T00:07:11</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>2026-03-19</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>KoAct 코스닥액티브</t>
+        </is>
+      </c>
+      <c r="C99" t="n">
+        <v>200</v>
+      </c>
+      <c r="D99" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E99" t="n">
+        <v>1</v>
+      </c>
+      <c r="F99" t="n">
+        <v>2598000</v>
+      </c>
+      <c r="G99" t="n">
+        <v>-104000</v>
+      </c>
+      <c r="H99" t="n">
+        <v>-3.84900074019245</v>
+      </c>
+      <c r="I99" t="inlineStr">
+        <is>
+          <t>2026-03-19T00:07:11</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>2026-03-19</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>휴스틸</t>
+        </is>
+      </c>
+      <c r="C100" t="n">
+        <v>500</v>
+      </c>
+      <c r="D100" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E100" t="n">
+        <v>1</v>
+      </c>
+      <c r="F100" t="n">
+        <v>2560000</v>
+      </c>
+      <c r="G100" t="n">
+        <v>281390</v>
+      </c>
+      <c r="H100" t="n">
+        <v>12.34919534277476</v>
+      </c>
+      <c r="I100" t="inlineStr">
+        <is>
+          <t>2026-03-19T00:07:11</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>2026-03-19</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>넥스틸</t>
+        </is>
+      </c>
+      <c r="C101" t="n">
+        <v>200</v>
+      </c>
+      <c r="D101" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E101" t="n">
+        <v>1</v>
+      </c>
+      <c r="F101" t="n">
+        <v>2400000</v>
+      </c>
+      <c r="G101" t="n">
+        <v>389000</v>
+      </c>
+      <c r="H101" t="n">
+        <v>19.34361014420686</v>
+      </c>
+      <c r="I101" t="inlineStr">
+        <is>
+          <t>2026-03-19T00:07:11</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>2026-03-19</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>대신증권</t>
+        </is>
+      </c>
+      <c r="C102" t="n">
+        <v>55</v>
+      </c>
+      <c r="D102" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E102" t="n">
+        <v>1</v>
+      </c>
+      <c r="F102" t="n">
+        <v>2238500</v>
+      </c>
+      <c r="G102" t="n">
+        <v>528999</v>
+      </c>
+      <c r="H102" t="n">
+        <v>30.94464408034859</v>
+      </c>
+      <c r="I102" t="inlineStr">
+        <is>
+          <t>2026-03-19T00:07:11</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>2026-03-19</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>발레로 에너지</t>
+        </is>
+      </c>
+      <c r="C103" t="n">
+        <v>6</v>
+      </c>
+      <c r="D103" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E103" t="n">
+        <v>1</v>
+      </c>
+      <c r="F103" t="n">
+        <v>2145682.294059377</v>
+      </c>
+      <c r="G103" t="n">
+        <v>81692.29405937716</v>
+      </c>
+      <c r="H103" t="n">
+        <v>3.957979159752575</v>
+      </c>
+      <c r="I103" t="inlineStr">
+        <is>
+          <t>2026-03-19T00:07:11</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>2026-03-19</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>미창석유</t>
+        </is>
+      </c>
+      <c r="C104" t="n">
+        <v>18</v>
+      </c>
+      <c r="D104" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E104" t="n">
+        <v>1</v>
+      </c>
+      <c r="F104" t="n">
+        <v>2032200</v>
+      </c>
+      <c r="G104" t="n">
+        <v>-360000</v>
+      </c>
+      <c r="H104" t="n">
+        <v>-15.04890895410083</v>
+      </c>
+      <c r="I104" t="inlineStr">
+        <is>
+          <t>2026-03-19T00:07:11</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>2026-03-19</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>대창단조</t>
+        </is>
+      </c>
+      <c r="C105" t="n">
+        <v>300</v>
+      </c>
+      <c r="D105" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E105" t="n">
+        <v>1</v>
+      </c>
+      <c r="F105" t="n">
+        <v>1914000</v>
+      </c>
+      <c r="G105" t="n">
+        <v>-144000</v>
+      </c>
+      <c r="H105" t="n">
+        <v>-6.997084548104956</v>
+      </c>
+      <c r="I105" t="inlineStr">
+        <is>
+          <t>2026-03-19T00:07:11</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>2026-03-19</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>동방</t>
+        </is>
+      </c>
+      <c r="C106" t="n">
+        <v>681</v>
+      </c>
+      <c r="D106" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E106" t="n">
+        <v>1</v>
+      </c>
+      <c r="F106" t="n">
+        <v>1882965</v>
+      </c>
+      <c r="G106" t="n">
+        <v>-88536</v>
+      </c>
+      <c r="H106" t="n">
+        <v>-4.490791533963209</v>
+      </c>
+      <c r="I106" t="inlineStr">
+        <is>
+          <t>2026-03-19T00:07:11</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>2026-03-19</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>하나금융지주</t>
+        </is>
+      </c>
+      <c r="C107" t="n">
+        <v>15</v>
+      </c>
+      <c r="D107" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E107" t="n">
+        <v>1</v>
+      </c>
+      <c r="F107" t="n">
+        <v>1717500</v>
+      </c>
+      <c r="G107" t="n">
+        <v>35000</v>
+      </c>
+      <c r="H107" t="n">
+        <v>2.080237741456166</v>
+      </c>
+      <c r="I107" t="inlineStr">
+        <is>
+          <t>2026-03-19T00:07:11</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>2026-03-19</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>스타 벌크 캐리어스</t>
+        </is>
+      </c>
+      <c r="C108" t="n">
+        <v>50</v>
+      </c>
+      <c r="D108" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E108" t="n">
+        <v>1</v>
+      </c>
+      <c r="F108" t="n">
+        <v>1709635.204022215</v>
+      </c>
+      <c r="G108" t="n">
+        <v>395282.2040222154</v>
+      </c>
+      <c r="H108" t="n">
+        <v>30.0742801988671</v>
+      </c>
+      <c r="I108" t="inlineStr">
+        <is>
+          <t>2026-03-19T00:07:11</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>2026-03-19</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>유나이티드헬스 그룹</t>
+        </is>
+      </c>
+      <c r="C109" t="n">
+        <v>4</v>
+      </c>
+      <c r="D109" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E109" t="n">
+        <v>1</v>
+      </c>
+      <c r="F109" t="n">
+        <v>1705616.038137302</v>
+      </c>
+      <c r="G109" t="n">
+        <v>11160.03813730204</v>
+      </c>
+      <c r="H109" t="n">
+        <v>0.6586207099683933</v>
+      </c>
+      <c r="I109" t="inlineStr">
+        <is>
+          <t>2026-03-19T00:07:11</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>2026-03-19</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>케이씨</t>
+        </is>
+      </c>
+      <c r="C110" t="n">
+        <v>50</v>
+      </c>
+      <c r="D110" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E110" t="n">
+        <v>1</v>
+      </c>
+      <c r="F110" t="n">
+        <v>1640000</v>
+      </c>
+      <c r="G110" t="n">
+        <v>-9500.000000000698</v>
+      </c>
+      <c r="H110" t="n">
+        <v>-0.5759321006365986</v>
+      </c>
+      <c r="I110" t="inlineStr">
+        <is>
+          <t>2026-03-19T00:07:11</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>2026-03-19</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>삼성생명</t>
+        </is>
+      </c>
+      <c r="C111" t="n">
+        <v>4</v>
+      </c>
+      <c r="D111" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E111" t="n">
+        <v>1</v>
+      </c>
+      <c r="F111" t="n">
+        <v>940000</v>
+      </c>
+      <c r="G111" t="n">
+        <v>107000</v>
+      </c>
+      <c r="H111" t="n">
+        <v>12.84513805522209</v>
+      </c>
+      <c r="I111" t="inlineStr">
+        <is>
+          <t>2026-03-19T00:07:11</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>2026-03-19</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>클리블랜드 클리프스</t>
+        </is>
+      </c>
+      <c r="C112" t="n">
+        <v>70</v>
+      </c>
+      <c r="D112" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E112" t="n">
+        <v>1</v>
+      </c>
+      <c r="F112" t="n">
+        <v>858716.8307915051</v>
+      </c>
+      <c r="G112" t="n">
+        <v>-157338.1692084949</v>
+      </c>
+      <c r="H112" t="n">
+        <v>-15.48520200269621</v>
+      </c>
+      <c r="I112" t="inlineStr">
+        <is>
+          <t>2026-03-19T00:07:11</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>2026-03-19</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>비에이치아이</t>
+        </is>
+      </c>
+      <c r="C113" t="n">
+        <v>8</v>
+      </c>
+      <c r="D113" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E113" t="n">
+        <v>1</v>
+      </c>
+      <c r="F113" t="n">
+        <v>844800</v>
+      </c>
+      <c r="G113" t="n">
+        <v>179685</v>
+      </c>
+      <c r="H113" t="n">
+        <v>27.01562887620938</v>
+      </c>
+      <c r="I113" t="inlineStr">
+        <is>
+          <t>2026-03-19T00:07:11</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>2026-03-19</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>하프니아</t>
+        </is>
+      </c>
+      <c r="C114" t="n">
+        <v>80</v>
+      </c>
+      <c r="D114" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E114" t="n">
+        <v>1</v>
+      </c>
+      <c r="F114" t="n">
+        <v>830222.8868876956</v>
+      </c>
+      <c r="G114" t="n">
+        <v>204491.8868876956</v>
+      </c>
+      <c r="H114" t="n">
+        <v>32.68047881401044</v>
+      </c>
+      <c r="I114" t="inlineStr">
+        <is>
+          <t>2026-03-19T00:07:11</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>2026-03-19</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>텍사스 퍼시픽 랜드</t>
+        </is>
+      </c>
+      <c r="C115" t="n">
+        <v>1</v>
+      </c>
+      <c r="D115" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E115" t="n">
+        <v>1</v>
+      </c>
+      <c r="F115" t="n">
+        <v>794950.4285003915</v>
+      </c>
+      <c r="G115" t="n">
+        <v>16359.42850039154</v>
+      </c>
+      <c r="H115" t="n">
+        <v>2.101158181945533</v>
+      </c>
+      <c r="I115" t="inlineStr">
+        <is>
+          <t>2026-03-19T00:07:11</t>
         </is>
       </c>
     </row>
@@ -4440,7 +5846,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E3"/>
+  <dimension ref="A1:E4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4516,6 +5922,29 @@
         </is>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2026-03-19</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>31505056</v>
+      </c>
+      <c r="C4" t="n">
+        <v>6016.63</v>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>2026-03-19T00:07:11</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>2026-03-19T00:07:11</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
auto: portfolio snapshot 2026-03-19 (2026-03-19T00:08:49)
</commit_message>
<xml_diff>
--- a/portfolio_auto.xlsx
+++ b/portfolio_auto.xlsx
@@ -1549,7 +1549,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2026-03-19T00:07:11</t>
+          <t>2026-03-19T00:08:49</t>
         </is>
       </c>
       <c r="E2" t="n">
@@ -4462,7 +4462,7 @@
       </c>
       <c r="I78" t="inlineStr">
         <is>
-          <t>2026-03-19T00:07:11</t>
+          <t>2026-03-19T00:08:49</t>
         </is>
       </c>
     </row>
@@ -4499,7 +4499,7 @@
       </c>
       <c r="I79" t="inlineStr">
         <is>
-          <t>2026-03-19T00:07:11</t>
+          <t>2026-03-19T00:08:49</t>
         </is>
       </c>
     </row>
@@ -4536,7 +4536,7 @@
       </c>
       <c r="I80" t="inlineStr">
         <is>
-          <t>2026-03-19T00:07:11</t>
+          <t>2026-03-19T00:08:49</t>
         </is>
       </c>
     </row>
@@ -4573,7 +4573,7 @@
       </c>
       <c r="I81" t="inlineStr">
         <is>
-          <t>2026-03-19T00:07:11</t>
+          <t>2026-03-19T00:08:49</t>
         </is>
       </c>
     </row>
@@ -4610,7 +4610,7 @@
       </c>
       <c r="I82" t="inlineStr">
         <is>
-          <t>2026-03-19T00:07:11</t>
+          <t>2026-03-19T00:08:49</t>
         </is>
       </c>
     </row>
@@ -4647,7 +4647,7 @@
       </c>
       <c r="I83" t="inlineStr">
         <is>
-          <t>2026-03-19T00:07:11</t>
+          <t>2026-03-19T00:08:49</t>
         </is>
       </c>
     </row>
@@ -4684,7 +4684,7 @@
       </c>
       <c r="I84" t="inlineStr">
         <is>
-          <t>2026-03-19T00:07:11</t>
+          <t>2026-03-19T00:08:49</t>
         </is>
       </c>
     </row>
@@ -4721,7 +4721,7 @@
       </c>
       <c r="I85" t="inlineStr">
         <is>
-          <t>2026-03-19T00:07:11</t>
+          <t>2026-03-19T00:08:49</t>
         </is>
       </c>
     </row>
@@ -4758,7 +4758,7 @@
       </c>
       <c r="I86" t="inlineStr">
         <is>
-          <t>2026-03-19T00:07:11</t>
+          <t>2026-03-19T00:08:49</t>
         </is>
       </c>
     </row>
@@ -4795,7 +4795,7 @@
       </c>
       <c r="I87" t="inlineStr">
         <is>
-          <t>2026-03-19T00:07:11</t>
+          <t>2026-03-19T00:08:49</t>
         </is>
       </c>
     </row>
@@ -4832,7 +4832,7 @@
       </c>
       <c r="I88" t="inlineStr">
         <is>
-          <t>2026-03-19T00:07:11</t>
+          <t>2026-03-19T00:08:49</t>
         </is>
       </c>
     </row>
@@ -4869,7 +4869,7 @@
       </c>
       <c r="I89" t="inlineStr">
         <is>
-          <t>2026-03-19T00:07:11</t>
+          <t>2026-03-19T00:08:49</t>
         </is>
       </c>
     </row>
@@ -4906,7 +4906,7 @@
       </c>
       <c r="I90" t="inlineStr">
         <is>
-          <t>2026-03-19T00:07:11</t>
+          <t>2026-03-19T00:08:49</t>
         </is>
       </c>
     </row>
@@ -4943,7 +4943,7 @@
       </c>
       <c r="I91" t="inlineStr">
         <is>
-          <t>2026-03-19T00:07:11</t>
+          <t>2026-03-19T00:08:49</t>
         </is>
       </c>
     </row>
@@ -4980,7 +4980,7 @@
       </c>
       <c r="I92" t="inlineStr">
         <is>
-          <t>2026-03-19T00:07:11</t>
+          <t>2026-03-19T00:08:49</t>
         </is>
       </c>
     </row>
@@ -5017,7 +5017,7 @@
       </c>
       <c r="I93" t="inlineStr">
         <is>
-          <t>2026-03-19T00:07:11</t>
+          <t>2026-03-19T00:08:49</t>
         </is>
       </c>
     </row>
@@ -5054,7 +5054,7 @@
       </c>
       <c r="I94" t="inlineStr">
         <is>
-          <t>2026-03-19T00:07:11</t>
+          <t>2026-03-19T00:08:49</t>
         </is>
       </c>
     </row>
@@ -5091,7 +5091,7 @@
       </c>
       <c r="I95" t="inlineStr">
         <is>
-          <t>2026-03-19T00:07:11</t>
+          <t>2026-03-19T00:08:49</t>
         </is>
       </c>
     </row>
@@ -5128,7 +5128,7 @@
       </c>
       <c r="I96" t="inlineStr">
         <is>
-          <t>2026-03-19T00:07:11</t>
+          <t>2026-03-19T00:08:49</t>
         </is>
       </c>
     </row>
@@ -5165,7 +5165,7 @@
       </c>
       <c r="I97" t="inlineStr">
         <is>
-          <t>2026-03-19T00:07:11</t>
+          <t>2026-03-19T00:08:49</t>
         </is>
       </c>
     </row>
@@ -5202,7 +5202,7 @@
       </c>
       <c r="I98" t="inlineStr">
         <is>
-          <t>2026-03-19T00:07:11</t>
+          <t>2026-03-19T00:08:49</t>
         </is>
       </c>
     </row>
@@ -5239,7 +5239,7 @@
       </c>
       <c r="I99" t="inlineStr">
         <is>
-          <t>2026-03-19T00:07:11</t>
+          <t>2026-03-19T00:08:49</t>
         </is>
       </c>
     </row>
@@ -5276,7 +5276,7 @@
       </c>
       <c r="I100" t="inlineStr">
         <is>
-          <t>2026-03-19T00:07:11</t>
+          <t>2026-03-19T00:08:49</t>
         </is>
       </c>
     </row>
@@ -5313,7 +5313,7 @@
       </c>
       <c r="I101" t="inlineStr">
         <is>
-          <t>2026-03-19T00:07:11</t>
+          <t>2026-03-19T00:08:49</t>
         </is>
       </c>
     </row>
@@ -5350,7 +5350,7 @@
       </c>
       <c r="I102" t="inlineStr">
         <is>
-          <t>2026-03-19T00:07:11</t>
+          <t>2026-03-19T00:08:49</t>
         </is>
       </c>
     </row>
@@ -5387,7 +5387,7 @@
       </c>
       <c r="I103" t="inlineStr">
         <is>
-          <t>2026-03-19T00:07:11</t>
+          <t>2026-03-19T00:08:49</t>
         </is>
       </c>
     </row>
@@ -5424,7 +5424,7 @@
       </c>
       <c r="I104" t="inlineStr">
         <is>
-          <t>2026-03-19T00:07:11</t>
+          <t>2026-03-19T00:08:49</t>
         </is>
       </c>
     </row>
@@ -5461,7 +5461,7 @@
       </c>
       <c r="I105" t="inlineStr">
         <is>
-          <t>2026-03-19T00:07:11</t>
+          <t>2026-03-19T00:08:49</t>
         </is>
       </c>
     </row>
@@ -5498,7 +5498,7 @@
       </c>
       <c r="I106" t="inlineStr">
         <is>
-          <t>2026-03-19T00:07:11</t>
+          <t>2026-03-19T00:08:49</t>
         </is>
       </c>
     </row>
@@ -5535,7 +5535,7 @@
       </c>
       <c r="I107" t="inlineStr">
         <is>
-          <t>2026-03-19T00:07:11</t>
+          <t>2026-03-19T00:08:49</t>
         </is>
       </c>
     </row>
@@ -5572,7 +5572,7 @@
       </c>
       <c r="I108" t="inlineStr">
         <is>
-          <t>2026-03-19T00:07:11</t>
+          <t>2026-03-19T00:08:49</t>
         </is>
       </c>
     </row>
@@ -5609,7 +5609,7 @@
       </c>
       <c r="I109" t="inlineStr">
         <is>
-          <t>2026-03-19T00:07:11</t>
+          <t>2026-03-19T00:08:49</t>
         </is>
       </c>
     </row>
@@ -5646,7 +5646,7 @@
       </c>
       <c r="I110" t="inlineStr">
         <is>
-          <t>2026-03-19T00:07:11</t>
+          <t>2026-03-19T00:08:49</t>
         </is>
       </c>
     </row>
@@ -5683,7 +5683,7 @@
       </c>
       <c r="I111" t="inlineStr">
         <is>
-          <t>2026-03-19T00:07:11</t>
+          <t>2026-03-19T00:08:49</t>
         </is>
       </c>
     </row>
@@ -5720,7 +5720,7 @@
       </c>
       <c r="I112" t="inlineStr">
         <is>
-          <t>2026-03-19T00:07:11</t>
+          <t>2026-03-19T00:08:49</t>
         </is>
       </c>
     </row>
@@ -5757,7 +5757,7 @@
       </c>
       <c r="I113" t="inlineStr">
         <is>
-          <t>2026-03-19T00:07:11</t>
+          <t>2026-03-19T00:08:49</t>
         </is>
       </c>
     </row>
@@ -5794,7 +5794,7 @@
       </c>
       <c r="I114" t="inlineStr">
         <is>
-          <t>2026-03-19T00:07:11</t>
+          <t>2026-03-19T00:08:49</t>
         </is>
       </c>
     </row>
@@ -5831,7 +5831,7 @@
       </c>
       <c r="I115" t="inlineStr">
         <is>
-          <t>2026-03-19T00:07:11</t>
+          <t>2026-03-19T00:08:49</t>
         </is>
       </c>
     </row>
@@ -5941,7 +5941,7 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>2026-03-19T00:07:11</t>
+          <t>2026-03-19T00:08:49</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: portfolio snapshot 2026-03-19 (2026-03-19T00:21:23)
</commit_message>
<xml_diff>
--- a/portfolio_auto.xlsx
+++ b/portfolio_auto.xlsx
@@ -540,13 +540,13 @@
         <v>1</v>
       </c>
       <c r="E4" t="n">
-        <v>9570000</v>
+        <v>9530000</v>
       </c>
       <c r="F4" t="n">
-        <v>2357000</v>
+        <v>2317000</v>
       </c>
       <c r="G4" t="n">
-        <v>32.67711077221684</v>
+        <v>32.12255649521697</v>
       </c>
     </row>
     <row r="5">
@@ -633,11 +633,11 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>세아제강</t>
+          <t>노블</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>50</v>
+        <v>99</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
@@ -648,23 +648,23 @@
         <v>1</v>
       </c>
       <c r="E8" t="n">
-        <v>6915000</v>
+        <v>6926047.602600594</v>
       </c>
       <c r="F8" t="n">
-        <v>605000</v>
+        <v>3018839.602600594</v>
       </c>
       <c r="G8" t="n">
-        <v>9.587955625990491</v>
+        <v>77.2633451457049</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>노블</t>
+          <t>세아제강</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>99</v>
+        <v>50</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
@@ -675,13 +675,13 @@
         <v>1</v>
       </c>
       <c r="E9" t="n">
-        <v>6926047.602600594</v>
+        <v>6900000</v>
       </c>
       <c r="F9" t="n">
-        <v>3018839.602600594</v>
+        <v>590000</v>
       </c>
       <c r="G9" t="n">
-        <v>77.2633451457049</v>
+        <v>9.350237717908081</v>
       </c>
     </row>
     <row r="10">
@@ -783,13 +783,13 @@
         <v>1</v>
       </c>
       <c r="E13" t="n">
-        <v>4904400</v>
+        <v>4756665</v>
       </c>
       <c r="F13" t="n">
-        <v>180603</v>
+        <v>32868</v>
       </c>
       <c r="G13" t="n">
-        <v>3.823259128197084</v>
+        <v>0.6957961995403275</v>
       </c>
     </row>
     <row r="14">
@@ -837,13 +837,13 @@
         <v>1</v>
       </c>
       <c r="E15" t="n">
-        <v>4446000</v>
+        <v>4356000</v>
       </c>
       <c r="F15" t="n">
-        <v>-185000</v>
+        <v>-275000</v>
       </c>
       <c r="G15" t="n">
-        <v>-3.994817534009933</v>
+        <v>-5.938242280285035</v>
       </c>
     </row>
     <row r="16">
@@ -864,13 +864,13 @@
         <v>1</v>
       </c>
       <c r="E16" t="n">
-        <v>4128000</v>
+        <v>4016000</v>
       </c>
       <c r="F16" t="n">
-        <v>717000</v>
+        <v>605000</v>
       </c>
       <c r="G16" t="n">
-        <v>21.02022867194371</v>
+        <v>17.73673409557314</v>
       </c>
     </row>
     <row r="17">
@@ -918,13 +918,13 @@
         <v>1</v>
       </c>
       <c r="E18" t="n">
-        <v>3978000</v>
+        <v>3971200</v>
       </c>
       <c r="F18" t="n">
-        <v>240600</v>
+        <v>233800</v>
       </c>
       <c r="G18" t="n">
-        <v>6.437630438272596</v>
+        <v>6.255685770856745</v>
       </c>
     </row>
     <row r="19">
@@ -945,13 +945,13 @@
         <v>1</v>
       </c>
       <c r="E19" t="n">
-        <v>3955600</v>
+        <v>3865700</v>
       </c>
       <c r="F19" t="n">
-        <v>-79496</v>
+        <v>-169396</v>
       </c>
       <c r="G19" t="n">
-        <v>-1.970114217852561</v>
+        <v>-4.198066167446822</v>
       </c>
     </row>
     <row r="20">
@@ -1026,13 +1026,13 @@
         <v>1</v>
       </c>
       <c r="E22" t="n">
-        <v>2607500</v>
+        <v>2532250</v>
       </c>
       <c r="F22" t="n">
-        <v>-200000</v>
+        <v>-275250</v>
       </c>
       <c r="G22" t="n">
-        <v>-7.123775601068566</v>
+        <v>-9.804096170970615</v>
       </c>
     </row>
     <row r="23">
@@ -1053,13 +1053,13 @@
         <v>1</v>
       </c>
       <c r="E23" t="n">
-        <v>2598000</v>
+        <v>2526000</v>
       </c>
       <c r="F23" t="n">
-        <v>-104000</v>
+        <v>-176000</v>
       </c>
       <c r="G23" t="n">
-        <v>-3.84900074019245</v>
+        <v>-6.513693560325684</v>
       </c>
     </row>
     <row r="24">
@@ -1080,13 +1080,13 @@
         <v>1</v>
       </c>
       <c r="E24" t="n">
-        <v>2560000</v>
+        <v>2547500</v>
       </c>
       <c r="F24" t="n">
-        <v>281390</v>
+        <v>268890</v>
       </c>
       <c r="G24" t="n">
-        <v>12.34919534277476</v>
+        <v>11.80061528739012</v>
       </c>
     </row>
     <row r="25">
@@ -1107,13 +1107,13 @@
         <v>1</v>
       </c>
       <c r="E25" t="n">
-        <v>2400000</v>
+        <v>2360000</v>
       </c>
       <c r="F25" t="n">
-        <v>389000</v>
+        <v>349000</v>
       </c>
       <c r="G25" t="n">
-        <v>19.34361014420686</v>
+        <v>17.35454997513675</v>
       </c>
     </row>
     <row r="26">
@@ -1134,13 +1134,13 @@
         <v>1</v>
       </c>
       <c r="E26" t="n">
-        <v>2238500</v>
+        <v>2180750</v>
       </c>
       <c r="F26" t="n">
-        <v>528999</v>
+        <v>471249</v>
       </c>
       <c r="G26" t="n">
-        <v>30.94464408034859</v>
+        <v>27.56646530186294</v>
       </c>
     </row>
     <row r="27">
@@ -1188,13 +1188,13 @@
         <v>1</v>
       </c>
       <c r="E28" t="n">
-        <v>2032200</v>
+        <v>2044800</v>
       </c>
       <c r="F28" t="n">
-        <v>-360000</v>
+        <v>-347400</v>
       </c>
       <c r="G28" t="n">
-        <v>-15.04890895410083</v>
+        <v>-14.5221971407073</v>
       </c>
     </row>
     <row r="29">
@@ -1215,13 +1215,13 @@
         <v>1</v>
       </c>
       <c r="E29" t="n">
-        <v>1914000</v>
+        <v>1899000</v>
       </c>
       <c r="F29" t="n">
-        <v>-144000</v>
+        <v>-159000</v>
       </c>
       <c r="G29" t="n">
-        <v>-6.997084548104956</v>
+        <v>-7.725947521865889</v>
       </c>
     </row>
     <row r="30">
@@ -1242,13 +1242,13 @@
         <v>1</v>
       </c>
       <c r="E30" t="n">
-        <v>1882965</v>
+        <v>1889775</v>
       </c>
       <c r="F30" t="n">
-        <v>-88536</v>
+        <v>-81726</v>
       </c>
       <c r="G30" t="n">
-        <v>-4.490791533963209</v>
+        <v>-4.14536944186181</v>
       </c>
     </row>
     <row r="31">
@@ -1269,13 +1269,13 @@
         <v>1</v>
       </c>
       <c r="E31" t="n">
-        <v>1717500</v>
+        <v>1663500</v>
       </c>
       <c r="F31" t="n">
-        <v>35000</v>
+        <v>-19000</v>
       </c>
       <c r="G31" t="n">
-        <v>2.080237741456166</v>
+        <v>-1.12927191679049</v>
       </c>
     </row>
     <row r="32">
@@ -1350,13 +1350,13 @@
         <v>1</v>
       </c>
       <c r="E34" t="n">
-        <v>1640000</v>
+        <v>1600000</v>
       </c>
       <c r="F34" t="n">
-        <v>-9500.000000000698</v>
+        <v>-49500.0000000007</v>
       </c>
       <c r="G34" t="n">
-        <v>-0.5759321006365986</v>
+        <v>-3.00090936647473</v>
       </c>
     </row>
     <row r="35">
@@ -1377,13 +1377,13 @@
         <v>1</v>
       </c>
       <c r="E35" t="n">
-        <v>940000</v>
+        <v>922000</v>
       </c>
       <c r="F35" t="n">
-        <v>107000</v>
+        <v>89000</v>
       </c>
       <c r="G35" t="n">
-        <v>12.84513805522209</v>
+        <v>10.68427370948379</v>
       </c>
     </row>
     <row r="36">
@@ -1431,13 +1431,13 @@
         <v>1</v>
       </c>
       <c r="E37" t="n">
-        <v>844800</v>
+        <v>827200</v>
       </c>
       <c r="F37" t="n">
-        <v>179685</v>
+        <v>162085</v>
       </c>
       <c r="G37" t="n">
-        <v>27.01562887620938</v>
+        <v>24.36946994128835</v>
       </c>
     </row>
     <row r="38">
@@ -1549,7 +1549,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2026-03-19T00:08:49</t>
+          <t>2026-03-19T00:21:23</t>
         </is>
       </c>
       <c r="E2" t="n">
@@ -4462,7 +4462,7 @@
       </c>
       <c r="I78" t="inlineStr">
         <is>
-          <t>2026-03-19T00:08:49</t>
+          <t>2026-03-19T00:21:23</t>
         </is>
       </c>
     </row>
@@ -4499,7 +4499,7 @@
       </c>
       <c r="I79" t="inlineStr">
         <is>
-          <t>2026-03-19T00:08:49</t>
+          <t>2026-03-19T00:21:23</t>
         </is>
       </c>
     </row>
@@ -4526,17 +4526,17 @@
         <v>1</v>
       </c>
       <c r="F80" t="n">
-        <v>9570000</v>
+        <v>9530000</v>
       </c>
       <c r="G80" t="n">
-        <v>2357000</v>
+        <v>2317000</v>
       </c>
       <c r="H80" t="n">
-        <v>32.67711077221684</v>
+        <v>32.12255649521697</v>
       </c>
       <c r="I80" t="inlineStr">
         <is>
-          <t>2026-03-19T00:08:49</t>
+          <t>2026-03-19T00:21:23</t>
         </is>
       </c>
     </row>
@@ -4573,7 +4573,7 @@
       </c>
       <c r="I81" t="inlineStr">
         <is>
-          <t>2026-03-19T00:08:49</t>
+          <t>2026-03-19T00:21:23</t>
         </is>
       </c>
     </row>
@@ -4610,7 +4610,7 @@
       </c>
       <c r="I82" t="inlineStr">
         <is>
-          <t>2026-03-19T00:08:49</t>
+          <t>2026-03-19T00:21:23</t>
         </is>
       </c>
     </row>
@@ -4647,7 +4647,7 @@
       </c>
       <c r="I83" t="inlineStr">
         <is>
-          <t>2026-03-19T00:08:49</t>
+          <t>2026-03-19T00:21:23</t>
         </is>
       </c>
     </row>
@@ -4684,7 +4684,7 @@
       </c>
       <c r="I84" t="inlineStr">
         <is>
-          <t>2026-03-19T00:08:49</t>
+          <t>2026-03-19T00:21:23</t>
         </is>
       </c>
     </row>
@@ -4711,17 +4711,17 @@
         <v>1</v>
       </c>
       <c r="F85" t="n">
-        <v>6915000</v>
+        <v>6900000</v>
       </c>
       <c r="G85" t="n">
-        <v>605000</v>
+        <v>590000</v>
       </c>
       <c r="H85" t="n">
-        <v>9.587955625990491</v>
+        <v>9.350237717908081</v>
       </c>
       <c r="I85" t="inlineStr">
         <is>
-          <t>2026-03-19T00:08:49</t>
+          <t>2026-03-19T00:21:23</t>
         </is>
       </c>
     </row>
@@ -4758,7 +4758,7 @@
       </c>
       <c r="I86" t="inlineStr">
         <is>
-          <t>2026-03-19T00:08:49</t>
+          <t>2026-03-19T00:21:23</t>
         </is>
       </c>
     </row>
@@ -4795,7 +4795,7 @@
       </c>
       <c r="I87" t="inlineStr">
         <is>
-          <t>2026-03-19T00:08:49</t>
+          <t>2026-03-19T00:21:23</t>
         </is>
       </c>
     </row>
@@ -4832,7 +4832,7 @@
       </c>
       <c r="I88" t="inlineStr">
         <is>
-          <t>2026-03-19T00:08:49</t>
+          <t>2026-03-19T00:21:23</t>
         </is>
       </c>
     </row>
@@ -4859,17 +4859,17 @@
         <v>1</v>
       </c>
       <c r="F89" t="n">
-        <v>4904400</v>
+        <v>4756665</v>
       </c>
       <c r="G89" t="n">
-        <v>180603</v>
+        <v>32868</v>
       </c>
       <c r="H89" t="n">
-        <v>3.823259128197084</v>
+        <v>0.6957961995403275</v>
       </c>
       <c r="I89" t="inlineStr">
         <is>
-          <t>2026-03-19T00:08:49</t>
+          <t>2026-03-19T00:21:23</t>
         </is>
       </c>
     </row>
@@ -4906,7 +4906,7 @@
       </c>
       <c r="I90" t="inlineStr">
         <is>
-          <t>2026-03-19T00:08:49</t>
+          <t>2026-03-19T00:21:23</t>
         </is>
       </c>
     </row>
@@ -4933,17 +4933,17 @@
         <v>1</v>
       </c>
       <c r="F91" t="n">
-        <v>4446000</v>
+        <v>4356000</v>
       </c>
       <c r="G91" t="n">
-        <v>-185000</v>
+        <v>-275000</v>
       </c>
       <c r="H91" t="n">
-        <v>-3.994817534009933</v>
+        <v>-5.938242280285035</v>
       </c>
       <c r="I91" t="inlineStr">
         <is>
-          <t>2026-03-19T00:08:49</t>
+          <t>2026-03-19T00:21:23</t>
         </is>
       </c>
     </row>
@@ -4955,11 +4955,11 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>DL이앤씨</t>
+          <t>차코스 에너지 내비게이션</t>
         </is>
       </c>
       <c r="C92" t="n">
-        <v>80</v>
+        <v>75</v>
       </c>
       <c r="D92" t="inlineStr">
         <is>
@@ -4970,17 +4970,17 @@
         <v>1</v>
       </c>
       <c r="F92" t="n">
-        <v>4128000</v>
+        <v>4023266.715580446</v>
       </c>
       <c r="G92" t="n">
-        <v>717000</v>
+        <v>198618.7155804457</v>
       </c>
       <c r="H92" t="n">
-        <v>21.02022867194371</v>
+        <v>5.193124062147567</v>
       </c>
       <c r="I92" t="inlineStr">
         <is>
-          <t>2026-03-19T00:08:49</t>
+          <t>2026-03-19T00:21:23</t>
         </is>
       </c>
     </row>
@@ -4992,11 +4992,11 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>차코스 에너지 내비게이션</t>
+          <t>DL이앤씨</t>
         </is>
       </c>
       <c r="C93" t="n">
-        <v>75</v>
+        <v>80</v>
       </c>
       <c r="D93" t="inlineStr">
         <is>
@@ -5007,17 +5007,17 @@
         <v>1</v>
       </c>
       <c r="F93" t="n">
-        <v>4023266.715580446</v>
+        <v>4016000</v>
       </c>
       <c r="G93" t="n">
-        <v>198618.7155804457</v>
+        <v>605000</v>
       </c>
       <c r="H93" t="n">
-        <v>5.193124062147567</v>
+        <v>17.73673409557314</v>
       </c>
       <c r="I93" t="inlineStr">
         <is>
-          <t>2026-03-19T00:08:49</t>
+          <t>2026-03-19T00:21:23</t>
         </is>
       </c>
     </row>
@@ -5044,17 +5044,17 @@
         <v>1</v>
       </c>
       <c r="F94" t="n">
-        <v>3978000</v>
+        <v>3971200</v>
       </c>
       <c r="G94" t="n">
-        <v>240600</v>
+        <v>233800</v>
       </c>
       <c r="H94" t="n">
-        <v>6.437630438272596</v>
+        <v>6.255685770856745</v>
       </c>
       <c r="I94" t="inlineStr">
         <is>
-          <t>2026-03-19T00:08:49</t>
+          <t>2026-03-19T00:21:23</t>
         </is>
       </c>
     </row>
@@ -5081,17 +5081,17 @@
         <v>1</v>
       </c>
       <c r="F95" t="n">
-        <v>3955600</v>
+        <v>3865700</v>
       </c>
       <c r="G95" t="n">
-        <v>-79496</v>
+        <v>-169396</v>
       </c>
       <c r="H95" t="n">
-        <v>-1.970114217852561</v>
+        <v>-4.198066167446822</v>
       </c>
       <c r="I95" t="inlineStr">
         <is>
-          <t>2026-03-19T00:08:49</t>
+          <t>2026-03-19T00:21:23</t>
         </is>
       </c>
     </row>
@@ -5128,7 +5128,7 @@
       </c>
       <c r="I96" t="inlineStr">
         <is>
-          <t>2026-03-19T00:08:49</t>
+          <t>2026-03-19T00:21:23</t>
         </is>
       </c>
     </row>
@@ -5165,7 +5165,7 @@
       </c>
       <c r="I97" t="inlineStr">
         <is>
-          <t>2026-03-19T00:08:49</t>
+          <t>2026-03-19T00:21:23</t>
         </is>
       </c>
     </row>
@@ -5177,11 +5177,11 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>현대제철</t>
+          <t>휴스틸</t>
         </is>
       </c>
       <c r="C98" t="n">
-        <v>70</v>
+        <v>500</v>
       </c>
       <c r="D98" t="inlineStr">
         <is>
@@ -5192,17 +5192,17 @@
         <v>1</v>
       </c>
       <c r="F98" t="n">
-        <v>2607500</v>
+        <v>2547500</v>
       </c>
       <c r="G98" t="n">
-        <v>-200000</v>
+        <v>268890</v>
       </c>
       <c r="H98" t="n">
-        <v>-7.123775601068566</v>
+        <v>11.80061528739012</v>
       </c>
       <c r="I98" t="inlineStr">
         <is>
-          <t>2026-03-19T00:08:49</t>
+          <t>2026-03-19T00:21:23</t>
         </is>
       </c>
     </row>
@@ -5214,11 +5214,11 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>KoAct 코스닥액티브</t>
+          <t>현대제철</t>
         </is>
       </c>
       <c r="C99" t="n">
-        <v>200</v>
+        <v>70</v>
       </c>
       <c r="D99" t="inlineStr">
         <is>
@@ -5229,17 +5229,17 @@
         <v>1</v>
       </c>
       <c r="F99" t="n">
-        <v>2598000</v>
+        <v>2532250</v>
       </c>
       <c r="G99" t="n">
-        <v>-104000</v>
+        <v>-275250</v>
       </c>
       <c r="H99" t="n">
-        <v>-3.84900074019245</v>
+        <v>-9.804096170970615</v>
       </c>
       <c r="I99" t="inlineStr">
         <is>
-          <t>2026-03-19T00:08:49</t>
+          <t>2026-03-19T00:21:23</t>
         </is>
       </c>
     </row>
@@ -5251,11 +5251,11 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>휴스틸</t>
+          <t>KoAct 코스닥액티브</t>
         </is>
       </c>
       <c r="C100" t="n">
-        <v>500</v>
+        <v>200</v>
       </c>
       <c r="D100" t="inlineStr">
         <is>
@@ -5266,17 +5266,17 @@
         <v>1</v>
       </c>
       <c r="F100" t="n">
-        <v>2560000</v>
+        <v>2526000</v>
       </c>
       <c r="G100" t="n">
-        <v>281390</v>
+        <v>-176000</v>
       </c>
       <c r="H100" t="n">
-        <v>12.34919534277476</v>
+        <v>-6.513693560325684</v>
       </c>
       <c r="I100" t="inlineStr">
         <is>
-          <t>2026-03-19T00:08:49</t>
+          <t>2026-03-19T00:21:23</t>
         </is>
       </c>
     </row>
@@ -5303,17 +5303,17 @@
         <v>1</v>
       </c>
       <c r="F101" t="n">
-        <v>2400000</v>
+        <v>2360000</v>
       </c>
       <c r="G101" t="n">
-        <v>389000</v>
+        <v>349000</v>
       </c>
       <c r="H101" t="n">
-        <v>19.34361014420686</v>
+        <v>17.35454997513675</v>
       </c>
       <c r="I101" t="inlineStr">
         <is>
-          <t>2026-03-19T00:08:49</t>
+          <t>2026-03-19T00:21:23</t>
         </is>
       </c>
     </row>
@@ -5340,17 +5340,17 @@
         <v>1</v>
       </c>
       <c r="F102" t="n">
-        <v>2238500</v>
+        <v>2180750</v>
       </c>
       <c r="G102" t="n">
-        <v>528999</v>
+        <v>471249</v>
       </c>
       <c r="H102" t="n">
-        <v>30.94464408034859</v>
+        <v>27.56646530186294</v>
       </c>
       <c r="I102" t="inlineStr">
         <is>
-          <t>2026-03-19T00:08:49</t>
+          <t>2026-03-19T00:21:23</t>
         </is>
       </c>
     </row>
@@ -5387,7 +5387,7 @@
       </c>
       <c r="I103" t="inlineStr">
         <is>
-          <t>2026-03-19T00:08:49</t>
+          <t>2026-03-19T00:21:23</t>
         </is>
       </c>
     </row>
@@ -5414,17 +5414,17 @@
         <v>1</v>
       </c>
       <c r="F104" t="n">
-        <v>2032200</v>
+        <v>2044800</v>
       </c>
       <c r="G104" t="n">
-        <v>-360000</v>
+        <v>-347400</v>
       </c>
       <c r="H104" t="n">
-        <v>-15.04890895410083</v>
+        <v>-14.5221971407073</v>
       </c>
       <c r="I104" t="inlineStr">
         <is>
-          <t>2026-03-19T00:08:49</t>
+          <t>2026-03-19T00:21:23</t>
         </is>
       </c>
     </row>
@@ -5451,17 +5451,17 @@
         <v>1</v>
       </c>
       <c r="F105" t="n">
-        <v>1914000</v>
+        <v>1899000</v>
       </c>
       <c r="G105" t="n">
-        <v>-144000</v>
+        <v>-159000</v>
       </c>
       <c r="H105" t="n">
-        <v>-6.997084548104956</v>
+        <v>-7.725947521865889</v>
       </c>
       <c r="I105" t="inlineStr">
         <is>
-          <t>2026-03-19T00:08:49</t>
+          <t>2026-03-19T00:21:23</t>
         </is>
       </c>
     </row>
@@ -5488,17 +5488,17 @@
         <v>1</v>
       </c>
       <c r="F106" t="n">
-        <v>1882965</v>
+        <v>1889775</v>
       </c>
       <c r="G106" t="n">
-        <v>-88536</v>
+        <v>-81726</v>
       </c>
       <c r="H106" t="n">
-        <v>-4.490791533963209</v>
+        <v>-4.14536944186181</v>
       </c>
       <c r="I106" t="inlineStr">
         <is>
-          <t>2026-03-19T00:08:49</t>
+          <t>2026-03-19T00:21:23</t>
         </is>
       </c>
     </row>
@@ -5510,11 +5510,11 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>하나금융지주</t>
+          <t>스타 벌크 캐리어스</t>
         </is>
       </c>
       <c r="C107" t="n">
-        <v>15</v>
+        <v>50</v>
       </c>
       <c r="D107" t="inlineStr">
         <is>
@@ -5525,17 +5525,17 @@
         <v>1</v>
       </c>
       <c r="F107" t="n">
-        <v>1717500</v>
+        <v>1709635.204022215</v>
       </c>
       <c r="G107" t="n">
-        <v>35000</v>
+        <v>395282.2040222154</v>
       </c>
       <c r="H107" t="n">
-        <v>2.080237741456166</v>
+        <v>30.0742801988671</v>
       </c>
       <c r="I107" t="inlineStr">
         <is>
-          <t>2026-03-19T00:08:49</t>
+          <t>2026-03-19T00:21:23</t>
         </is>
       </c>
     </row>
@@ -5547,11 +5547,11 @@
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>스타 벌크 캐리어스</t>
+          <t>유나이티드헬스 그룹</t>
         </is>
       </c>
       <c r="C108" t="n">
-        <v>50</v>
+        <v>4</v>
       </c>
       <c r="D108" t="inlineStr">
         <is>
@@ -5562,17 +5562,17 @@
         <v>1</v>
       </c>
       <c r="F108" t="n">
-        <v>1709635.204022215</v>
+        <v>1705616.038137302</v>
       </c>
       <c r="G108" t="n">
-        <v>395282.2040222154</v>
+        <v>11160.03813730204</v>
       </c>
       <c r="H108" t="n">
-        <v>30.0742801988671</v>
+        <v>0.6586207099683933</v>
       </c>
       <c r="I108" t="inlineStr">
         <is>
-          <t>2026-03-19T00:08:49</t>
+          <t>2026-03-19T00:21:23</t>
         </is>
       </c>
     </row>
@@ -5584,11 +5584,11 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>유나이티드헬스 그룹</t>
+          <t>하나금융지주</t>
         </is>
       </c>
       <c r="C109" t="n">
-        <v>4</v>
+        <v>15</v>
       </c>
       <c r="D109" t="inlineStr">
         <is>
@@ -5599,17 +5599,17 @@
         <v>1</v>
       </c>
       <c r="F109" t="n">
-        <v>1705616.038137302</v>
+        <v>1663500</v>
       </c>
       <c r="G109" t="n">
-        <v>11160.03813730204</v>
+        <v>-19000</v>
       </c>
       <c r="H109" t="n">
-        <v>0.6586207099683933</v>
+        <v>-1.12927191679049</v>
       </c>
       <c r="I109" t="inlineStr">
         <is>
-          <t>2026-03-19T00:08:49</t>
+          <t>2026-03-19T00:21:23</t>
         </is>
       </c>
     </row>
@@ -5636,17 +5636,17 @@
         <v>1</v>
       </c>
       <c r="F110" t="n">
-        <v>1640000</v>
+        <v>1600000</v>
       </c>
       <c r="G110" t="n">
-        <v>-9500.000000000698</v>
+        <v>-49500.0000000007</v>
       </c>
       <c r="H110" t="n">
-        <v>-0.5759321006365986</v>
+        <v>-3.00090936647473</v>
       </c>
       <c r="I110" t="inlineStr">
         <is>
-          <t>2026-03-19T00:08:49</t>
+          <t>2026-03-19T00:21:23</t>
         </is>
       </c>
     </row>
@@ -5673,17 +5673,17 @@
         <v>1</v>
       </c>
       <c r="F111" t="n">
-        <v>940000</v>
+        <v>922000</v>
       </c>
       <c r="G111" t="n">
-        <v>107000</v>
+        <v>89000</v>
       </c>
       <c r="H111" t="n">
-        <v>12.84513805522209</v>
+        <v>10.68427370948379</v>
       </c>
       <c r="I111" t="inlineStr">
         <is>
-          <t>2026-03-19T00:08:49</t>
+          <t>2026-03-19T00:21:23</t>
         </is>
       </c>
     </row>
@@ -5720,7 +5720,7 @@
       </c>
       <c r="I112" t="inlineStr">
         <is>
-          <t>2026-03-19T00:08:49</t>
+          <t>2026-03-19T00:21:23</t>
         </is>
       </c>
     </row>
@@ -5732,11 +5732,11 @@
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>비에이치아이</t>
+          <t>하프니아</t>
         </is>
       </c>
       <c r="C113" t="n">
-        <v>8</v>
+        <v>80</v>
       </c>
       <c r="D113" t="inlineStr">
         <is>
@@ -5747,17 +5747,17 @@
         <v>1</v>
       </c>
       <c r="F113" t="n">
-        <v>844800</v>
+        <v>830222.8868876956</v>
       </c>
       <c r="G113" t="n">
-        <v>179685</v>
+        <v>204491.8868876956</v>
       </c>
       <c r="H113" t="n">
-        <v>27.01562887620938</v>
+        <v>32.68047881401044</v>
       </c>
       <c r="I113" t="inlineStr">
         <is>
-          <t>2026-03-19T00:08:49</t>
+          <t>2026-03-19T00:21:23</t>
         </is>
       </c>
     </row>
@@ -5769,11 +5769,11 @@
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>하프니아</t>
+          <t>비에이치아이</t>
         </is>
       </c>
       <c r="C114" t="n">
-        <v>80</v>
+        <v>8</v>
       </c>
       <c r="D114" t="inlineStr">
         <is>
@@ -5784,17 +5784,17 @@
         <v>1</v>
       </c>
       <c r="F114" t="n">
-        <v>830222.8868876956</v>
+        <v>827200</v>
       </c>
       <c r="G114" t="n">
-        <v>204491.8868876956</v>
+        <v>162085</v>
       </c>
       <c r="H114" t="n">
-        <v>32.68047881401044</v>
+        <v>24.36946994128835</v>
       </c>
       <c r="I114" t="inlineStr">
         <is>
-          <t>2026-03-19T00:08:49</t>
+          <t>2026-03-19T00:21:23</t>
         </is>
       </c>
     </row>
@@ -5831,7 +5831,7 @@
       </c>
       <c r="I115" t="inlineStr">
         <is>
-          <t>2026-03-19T00:08:49</t>
+          <t>2026-03-19T00:21:23</t>
         </is>
       </c>
     </row>
@@ -5941,7 +5941,7 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>2026-03-19T00:08:49</t>
+          <t>2026-03-19T00:21:23</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: portfolio snapshot 2026-03-19 (2026-03-19T13:27:46)
</commit_message>
<xml_diff>
--- a/portfolio_auto.xlsx
+++ b/portfolio_auto.xlsx
@@ -540,13 +540,13 @@
         <v>1</v>
       </c>
       <c r="E4" t="n">
-        <v>9530000</v>
+        <v>9490000</v>
       </c>
       <c r="F4" t="n">
-        <v>2317000</v>
+        <v>2277000</v>
       </c>
       <c r="G4" t="n">
-        <v>32.12255649521697</v>
+        <v>31.56800221821711</v>
       </c>
     </row>
     <row r="5">
@@ -675,13 +675,13 @@
         <v>1</v>
       </c>
       <c r="E9" t="n">
-        <v>6900000</v>
+        <v>6945000</v>
       </c>
       <c r="F9" t="n">
-        <v>590000</v>
+        <v>635000</v>
       </c>
       <c r="G9" t="n">
-        <v>9.350237717908081</v>
+        <v>10.06339144215531</v>
       </c>
     </row>
     <row r="10">
@@ -783,13 +783,13 @@
         <v>1</v>
       </c>
       <c r="E13" t="n">
-        <v>4756665</v>
+        <v>4763700</v>
       </c>
       <c r="F13" t="n">
-        <v>32868</v>
+        <v>39903</v>
       </c>
       <c r="G13" t="n">
-        <v>0.6957961995403275</v>
+        <v>0.8447230056668396</v>
       </c>
     </row>
     <row r="14">
@@ -837,23 +837,23 @@
         <v>1</v>
       </c>
       <c r="E15" t="n">
-        <v>4356000</v>
+        <v>4306500</v>
       </c>
       <c r="F15" t="n">
-        <v>-275000</v>
+        <v>-324500</v>
       </c>
       <c r="G15" t="n">
-        <v>-5.938242280285035</v>
+        <v>-7.007125890736342</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>DL이앤씨</t>
+          <t>차코스 에너지 내비게이션</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>80</v>
+        <v>75</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
@@ -864,23 +864,23 @@
         <v>1</v>
       </c>
       <c r="E16" t="n">
-        <v>4016000</v>
+        <v>4023266.715580446</v>
       </c>
       <c r="F16" t="n">
-        <v>605000</v>
+        <v>198618.7155804457</v>
       </c>
       <c r="G16" t="n">
-        <v>17.73673409557314</v>
+        <v>5.193124062147567</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>차코스 에너지 내비게이션</t>
+          <t>DL이앤씨</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>75</v>
+        <v>80</v>
       </c>
       <c r="C17" t="inlineStr">
         <is>
@@ -891,13 +891,13 @@
         <v>1</v>
       </c>
       <c r="E17" t="n">
-        <v>4023266.715580446</v>
+        <v>4152000</v>
       </c>
       <c r="F17" t="n">
-        <v>198618.7155804457</v>
+        <v>741000</v>
       </c>
       <c r="G17" t="n">
-        <v>5.193124062147567</v>
+        <v>21.72383465259455</v>
       </c>
     </row>
     <row r="18">
@@ -918,13 +918,13 @@
         <v>1</v>
       </c>
       <c r="E18" t="n">
-        <v>3971200</v>
+        <v>3957600</v>
       </c>
       <c r="F18" t="n">
-        <v>233800</v>
+        <v>220200</v>
       </c>
       <c r="G18" t="n">
-        <v>6.255685770856745</v>
+        <v>5.891796436025045</v>
       </c>
     </row>
     <row r="19">
@@ -945,13 +945,13 @@
         <v>1</v>
       </c>
       <c r="E19" t="n">
-        <v>3865700</v>
+        <v>4082700</v>
       </c>
       <c r="F19" t="n">
-        <v>-169396</v>
+        <v>47604</v>
       </c>
       <c r="G19" t="n">
-        <v>-4.198066167446822</v>
+        <v>1.179748883297944</v>
       </c>
     </row>
     <row r="20">
@@ -1011,11 +1011,11 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>현대제철</t>
+          <t>휴스틸</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>70</v>
+        <v>500</v>
       </c>
       <c r="C22" t="inlineStr">
         <is>
@@ -1026,23 +1026,23 @@
         <v>1</v>
       </c>
       <c r="E22" t="n">
-        <v>2532250</v>
+        <v>2620000</v>
       </c>
       <c r="F22" t="n">
-        <v>-275250</v>
+        <v>341390</v>
       </c>
       <c r="G22" t="n">
-        <v>-9.804096170970615</v>
+        <v>14.98237960862105</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>KoAct 코스닥액티브</t>
+          <t>현대제철</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>200</v>
+        <v>70</v>
       </c>
       <c r="C23" t="inlineStr">
         <is>
@@ -1053,23 +1053,23 @@
         <v>1</v>
       </c>
       <c r="E23" t="n">
-        <v>2526000</v>
+        <v>2509500</v>
       </c>
       <c r="F23" t="n">
-        <v>-176000</v>
+        <v>-298000</v>
       </c>
       <c r="G23" t="n">
-        <v>-6.513693560325684</v>
+        <v>-10.61442564559216</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>휴스틸</t>
+          <t>KoAct 코스닥액티브</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>500</v>
+        <v>200</v>
       </c>
       <c r="C24" t="inlineStr">
         <is>
@@ -1080,13 +1080,13 @@
         <v>1</v>
       </c>
       <c r="E24" t="n">
-        <v>2547500</v>
+        <v>2526000</v>
       </c>
       <c r="F24" t="n">
-        <v>268890</v>
+        <v>-176000</v>
       </c>
       <c r="G24" t="n">
-        <v>11.80061528739012</v>
+        <v>-6.513693560325684</v>
       </c>
     </row>
     <row r="25">
@@ -1107,13 +1107,13 @@
         <v>1</v>
       </c>
       <c r="E25" t="n">
-        <v>2360000</v>
+        <v>2406000</v>
       </c>
       <c r="F25" t="n">
-        <v>349000</v>
+        <v>395000</v>
       </c>
       <c r="G25" t="n">
-        <v>17.35454997513675</v>
+        <v>19.64196916956738</v>
       </c>
     </row>
     <row r="26">
@@ -1188,13 +1188,13 @@
         <v>1</v>
       </c>
       <c r="E28" t="n">
-        <v>2044800</v>
+        <v>2023200</v>
       </c>
       <c r="F28" t="n">
-        <v>-347400</v>
+        <v>-369000</v>
       </c>
       <c r="G28" t="n">
-        <v>-14.5221971407073</v>
+        <v>-15.42513167795335</v>
       </c>
     </row>
     <row r="29">
@@ -1215,13 +1215,13 @@
         <v>1</v>
       </c>
       <c r="E29" t="n">
-        <v>1899000</v>
+        <v>1938000</v>
       </c>
       <c r="F29" t="n">
-        <v>-159000</v>
+        <v>-120000</v>
       </c>
       <c r="G29" t="n">
-        <v>-7.725947521865889</v>
+        <v>-5.830903790087463</v>
       </c>
     </row>
     <row r="30">
@@ -1242,23 +1242,23 @@
         <v>1</v>
       </c>
       <c r="E30" t="n">
-        <v>1889775</v>
+        <v>1906800</v>
       </c>
       <c r="F30" t="n">
-        <v>-81726</v>
+        <v>-64701</v>
       </c>
       <c r="G30" t="n">
-        <v>-4.14536944186181</v>
+        <v>-3.281814211608312</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>하나금융지주</t>
+          <t>스타 벌크 캐리어스</t>
         </is>
       </c>
       <c r="B31" t="n">
-        <v>15</v>
+        <v>50</v>
       </c>
       <c r="C31" t="inlineStr">
         <is>
@@ -1269,23 +1269,23 @@
         <v>1</v>
       </c>
       <c r="E31" t="n">
-        <v>1663500</v>
+        <v>1709635.204022215</v>
       </c>
       <c r="F31" t="n">
-        <v>-19000</v>
+        <v>395282.2040222154</v>
       </c>
       <c r="G31" t="n">
-        <v>-1.12927191679049</v>
+        <v>30.0742801988671</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>스타 벌크 캐리어스</t>
+          <t>유나이티드헬스 그룹</t>
         </is>
       </c>
       <c r="B32" t="n">
-        <v>50</v>
+        <v>4</v>
       </c>
       <c r="C32" t="inlineStr">
         <is>
@@ -1296,23 +1296,23 @@
         <v>1</v>
       </c>
       <c r="E32" t="n">
-        <v>1709635.204022215</v>
+        <v>1705616.038137302</v>
       </c>
       <c r="F32" t="n">
-        <v>395282.2040222154</v>
+        <v>11160.03813730204</v>
       </c>
       <c r="G32" t="n">
-        <v>30.0742801988671</v>
+        <v>0.6586207099683933</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>유나이티드헬스 그룹</t>
+          <t>하나금융지주</t>
         </is>
       </c>
       <c r="B33" t="n">
-        <v>4</v>
+        <v>15</v>
       </c>
       <c r="C33" t="inlineStr">
         <is>
@@ -1323,13 +1323,13 @@
         <v>1</v>
       </c>
       <c r="E33" t="n">
-        <v>1705616.038137302</v>
+        <v>1698000</v>
       </c>
       <c r="F33" t="n">
-        <v>11160.03813730204</v>
+        <v>15500</v>
       </c>
       <c r="G33" t="n">
-        <v>0.6586207099683933</v>
+        <v>0.9212481426448738</v>
       </c>
     </row>
     <row r="34">
@@ -1350,13 +1350,13 @@
         <v>1</v>
       </c>
       <c r="E34" t="n">
-        <v>1600000</v>
+        <v>1627500</v>
       </c>
       <c r="F34" t="n">
-        <v>-49500.0000000007</v>
+        <v>-22000.0000000007</v>
       </c>
       <c r="G34" t="n">
-        <v>-3.00090936647473</v>
+        <v>-1.333737496211015</v>
       </c>
     </row>
     <row r="35">
@@ -1416,11 +1416,11 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>비에이치아이</t>
+          <t>하프니아</t>
         </is>
       </c>
       <c r="B37" t="n">
-        <v>8</v>
+        <v>80</v>
       </c>
       <c r="C37" t="inlineStr">
         <is>
@@ -1431,23 +1431,23 @@
         <v>1</v>
       </c>
       <c r="E37" t="n">
-        <v>827200</v>
+        <v>830222.8868876956</v>
       </c>
       <c r="F37" t="n">
-        <v>162085</v>
+        <v>204491.8868876956</v>
       </c>
       <c r="G37" t="n">
-        <v>24.36946994128835</v>
+        <v>32.68047881401044</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>하프니아</t>
+          <t>비에이치아이</t>
         </is>
       </c>
       <c r="B38" t="n">
-        <v>80</v>
+        <v>8</v>
       </c>
       <c r="C38" t="inlineStr">
         <is>
@@ -1458,13 +1458,13 @@
         <v>1</v>
       </c>
       <c r="E38" t="n">
-        <v>830222.8868876956</v>
+        <v>834400</v>
       </c>
       <c r="F38" t="n">
-        <v>204491.8868876956</v>
+        <v>169285</v>
       </c>
       <c r="G38" t="n">
-        <v>32.68047881401044</v>
+        <v>25.45198950557423</v>
       </c>
     </row>
     <row r="39">
@@ -1549,7 +1549,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2026-03-19T00:21:23</t>
+          <t>2026-03-19T13:27:46</t>
         </is>
       </c>
       <c r="E2" t="n">
@@ -4462,7 +4462,7 @@
       </c>
       <c r="I78" t="inlineStr">
         <is>
-          <t>2026-03-19T00:21:23</t>
+          <t>2026-03-19T13:27:46</t>
         </is>
       </c>
     </row>
@@ -4499,7 +4499,7 @@
       </c>
       <c r="I79" t="inlineStr">
         <is>
-          <t>2026-03-19T00:21:23</t>
+          <t>2026-03-19T13:27:46</t>
         </is>
       </c>
     </row>
@@ -4526,17 +4526,17 @@
         <v>1</v>
       </c>
       <c r="F80" t="n">
-        <v>9530000</v>
+        <v>9490000</v>
       </c>
       <c r="G80" t="n">
-        <v>2317000</v>
+        <v>2277000</v>
       </c>
       <c r="H80" t="n">
-        <v>32.12255649521697</v>
+        <v>31.56800221821711</v>
       </c>
       <c r="I80" t="inlineStr">
         <is>
-          <t>2026-03-19T00:21:23</t>
+          <t>2026-03-19T13:27:46</t>
         </is>
       </c>
     </row>
@@ -4573,7 +4573,7 @@
       </c>
       <c r="I81" t="inlineStr">
         <is>
-          <t>2026-03-19T00:21:23</t>
+          <t>2026-03-19T13:27:46</t>
         </is>
       </c>
     </row>
@@ -4610,7 +4610,7 @@
       </c>
       <c r="I82" t="inlineStr">
         <is>
-          <t>2026-03-19T00:21:23</t>
+          <t>2026-03-19T13:27:46</t>
         </is>
       </c>
     </row>
@@ -4647,7 +4647,7 @@
       </c>
       <c r="I83" t="inlineStr">
         <is>
-          <t>2026-03-19T00:21:23</t>
+          <t>2026-03-19T13:27:46</t>
         </is>
       </c>
     </row>
@@ -4659,11 +4659,11 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>노블</t>
+          <t>세아제강</t>
         </is>
       </c>
       <c r="C84" t="n">
-        <v>99</v>
+        <v>50</v>
       </c>
       <c r="D84" t="inlineStr">
         <is>
@@ -4674,17 +4674,17 @@
         <v>1</v>
       </c>
       <c r="F84" t="n">
-        <v>6926047.602600594</v>
+        <v>6945000</v>
       </c>
       <c r="G84" t="n">
-        <v>3018839.602600594</v>
+        <v>635000</v>
       </c>
       <c r="H84" t="n">
-        <v>77.2633451457049</v>
+        <v>10.06339144215531</v>
       </c>
       <c r="I84" t="inlineStr">
         <is>
-          <t>2026-03-19T00:21:23</t>
+          <t>2026-03-19T13:27:46</t>
         </is>
       </c>
     </row>
@@ -4696,11 +4696,11 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>세아제강</t>
+          <t>노블</t>
         </is>
       </c>
       <c r="C85" t="n">
-        <v>50</v>
+        <v>99</v>
       </c>
       <c r="D85" t="inlineStr">
         <is>
@@ -4711,17 +4711,17 @@
         <v>1</v>
       </c>
       <c r="F85" t="n">
-        <v>6900000</v>
+        <v>6926047.602600594</v>
       </c>
       <c r="G85" t="n">
-        <v>590000</v>
+        <v>3018839.602600594</v>
       </c>
       <c r="H85" t="n">
-        <v>9.350237717908081</v>
+        <v>77.2633451457049</v>
       </c>
       <c r="I85" t="inlineStr">
         <is>
-          <t>2026-03-19T00:21:23</t>
+          <t>2026-03-19T13:27:46</t>
         </is>
       </c>
     </row>
@@ -4758,7 +4758,7 @@
       </c>
       <c r="I86" t="inlineStr">
         <is>
-          <t>2026-03-19T00:21:23</t>
+          <t>2026-03-19T13:27:46</t>
         </is>
       </c>
     </row>
@@ -4795,7 +4795,7 @@
       </c>
       <c r="I87" t="inlineStr">
         <is>
-          <t>2026-03-19T00:21:23</t>
+          <t>2026-03-19T13:27:46</t>
         </is>
       </c>
     </row>
@@ -4832,7 +4832,7 @@
       </c>
       <c r="I88" t="inlineStr">
         <is>
-          <t>2026-03-19T00:21:23</t>
+          <t>2026-03-19T13:27:46</t>
         </is>
       </c>
     </row>
@@ -4859,17 +4859,17 @@
         <v>1</v>
       </c>
       <c r="F89" t="n">
-        <v>4756665</v>
+        <v>4763700</v>
       </c>
       <c r="G89" t="n">
-        <v>32868</v>
+        <v>39903</v>
       </c>
       <c r="H89" t="n">
-        <v>0.6957961995403275</v>
+        <v>0.8447230056668396</v>
       </c>
       <c r="I89" t="inlineStr">
         <is>
-          <t>2026-03-19T00:21:23</t>
+          <t>2026-03-19T13:27:46</t>
         </is>
       </c>
     </row>
@@ -4906,7 +4906,7 @@
       </c>
       <c r="I90" t="inlineStr">
         <is>
-          <t>2026-03-19T00:21:23</t>
+          <t>2026-03-19T13:27:46</t>
         </is>
       </c>
     </row>
@@ -4933,17 +4933,17 @@
         <v>1</v>
       </c>
       <c r="F91" t="n">
-        <v>4356000</v>
+        <v>4306500</v>
       </c>
       <c r="G91" t="n">
-        <v>-275000</v>
+        <v>-324500</v>
       </c>
       <c r="H91" t="n">
-        <v>-5.938242280285035</v>
+        <v>-7.007125890736342</v>
       </c>
       <c r="I91" t="inlineStr">
         <is>
-          <t>2026-03-19T00:21:23</t>
+          <t>2026-03-19T13:27:46</t>
         </is>
       </c>
     </row>
@@ -4955,11 +4955,11 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>차코스 에너지 내비게이션</t>
+          <t>DL이앤씨</t>
         </is>
       </c>
       <c r="C92" t="n">
-        <v>75</v>
+        <v>80</v>
       </c>
       <c r="D92" t="inlineStr">
         <is>
@@ -4970,17 +4970,17 @@
         <v>1</v>
       </c>
       <c r="F92" t="n">
-        <v>4023266.715580446</v>
+        <v>4152000</v>
       </c>
       <c r="G92" t="n">
-        <v>198618.7155804457</v>
+        <v>741000</v>
       </c>
       <c r="H92" t="n">
-        <v>5.193124062147567</v>
+        <v>21.72383465259455</v>
       </c>
       <c r="I92" t="inlineStr">
         <is>
-          <t>2026-03-19T00:21:23</t>
+          <t>2026-03-19T13:27:46</t>
         </is>
       </c>
     </row>
@@ -4992,11 +4992,11 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>DL이앤씨</t>
+          <t>HD건설기계</t>
         </is>
       </c>
       <c r="C93" t="n">
-        <v>80</v>
+        <v>31</v>
       </c>
       <c r="D93" t="inlineStr">
         <is>
@@ -5007,17 +5007,17 @@
         <v>1</v>
       </c>
       <c r="F93" t="n">
-        <v>4016000</v>
+        <v>4082700</v>
       </c>
       <c r="G93" t="n">
-        <v>605000</v>
+        <v>47604</v>
       </c>
       <c r="H93" t="n">
-        <v>17.73673409557314</v>
+        <v>1.179748883297944</v>
       </c>
       <c r="I93" t="inlineStr">
         <is>
-          <t>2026-03-19T00:21:23</t>
+          <t>2026-03-19T13:27:46</t>
         </is>
       </c>
     </row>
@@ -5029,11 +5029,11 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>동원개발</t>
+          <t>차코스 에너지 내비게이션</t>
         </is>
       </c>
       <c r="C94" t="n">
-        <v>1360</v>
+        <v>75</v>
       </c>
       <c r="D94" t="inlineStr">
         <is>
@@ -5044,17 +5044,17 @@
         <v>1</v>
       </c>
       <c r="F94" t="n">
-        <v>3971200</v>
+        <v>4023266.715580446</v>
       </c>
       <c r="G94" t="n">
-        <v>233800</v>
+        <v>198618.7155804457</v>
       </c>
       <c r="H94" t="n">
-        <v>6.255685770856745</v>
+        <v>5.193124062147567</v>
       </c>
       <c r="I94" t="inlineStr">
         <is>
-          <t>2026-03-19T00:21:23</t>
+          <t>2026-03-19T13:27:46</t>
         </is>
       </c>
     </row>
@@ -5066,11 +5066,11 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>HD건설기계</t>
+          <t>동원개발</t>
         </is>
       </c>
       <c r="C95" t="n">
-        <v>31</v>
+        <v>1360</v>
       </c>
       <c r="D95" t="inlineStr">
         <is>
@@ -5081,17 +5081,17 @@
         <v>1</v>
       </c>
       <c r="F95" t="n">
-        <v>3865700</v>
+        <v>3957600</v>
       </c>
       <c r="G95" t="n">
-        <v>-169396</v>
+        <v>220200</v>
       </c>
       <c r="H95" t="n">
-        <v>-4.198066167446822</v>
+        <v>5.891796436025045</v>
       </c>
       <c r="I95" t="inlineStr">
         <is>
-          <t>2026-03-19T00:21:23</t>
+          <t>2026-03-19T13:27:46</t>
         </is>
       </c>
     </row>
@@ -5128,7 +5128,7 @@
       </c>
       <c r="I96" t="inlineStr">
         <is>
-          <t>2026-03-19T00:21:23</t>
+          <t>2026-03-19T13:27:46</t>
         </is>
       </c>
     </row>
@@ -5165,7 +5165,7 @@
       </c>
       <c r="I97" t="inlineStr">
         <is>
-          <t>2026-03-19T00:21:23</t>
+          <t>2026-03-19T13:27:46</t>
         </is>
       </c>
     </row>
@@ -5192,17 +5192,17 @@
         <v>1</v>
       </c>
       <c r="F98" t="n">
-        <v>2547500</v>
+        <v>2620000</v>
       </c>
       <c r="G98" t="n">
-        <v>268890</v>
+        <v>341390</v>
       </c>
       <c r="H98" t="n">
-        <v>11.80061528739012</v>
+        <v>14.98237960862105</v>
       </c>
       <c r="I98" t="inlineStr">
         <is>
-          <t>2026-03-19T00:21:23</t>
+          <t>2026-03-19T13:27:46</t>
         </is>
       </c>
     </row>
@@ -5214,11 +5214,11 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>현대제철</t>
+          <t>KoAct 코스닥액티브</t>
         </is>
       </c>
       <c r="C99" t="n">
-        <v>70</v>
+        <v>200</v>
       </c>
       <c r="D99" t="inlineStr">
         <is>
@@ -5229,17 +5229,17 @@
         <v>1</v>
       </c>
       <c r="F99" t="n">
-        <v>2532250</v>
+        <v>2526000</v>
       </c>
       <c r="G99" t="n">
-        <v>-275250</v>
+        <v>-176000</v>
       </c>
       <c r="H99" t="n">
-        <v>-9.804096170970615</v>
+        <v>-6.513693560325684</v>
       </c>
       <c r="I99" t="inlineStr">
         <is>
-          <t>2026-03-19T00:21:23</t>
+          <t>2026-03-19T13:27:46</t>
         </is>
       </c>
     </row>
@@ -5251,11 +5251,11 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>KoAct 코스닥액티브</t>
+          <t>현대제철</t>
         </is>
       </c>
       <c r="C100" t="n">
-        <v>200</v>
+        <v>70</v>
       </c>
       <c r="D100" t="inlineStr">
         <is>
@@ -5266,17 +5266,17 @@
         <v>1</v>
       </c>
       <c r="F100" t="n">
-        <v>2526000</v>
+        <v>2509500</v>
       </c>
       <c r="G100" t="n">
-        <v>-176000</v>
+        <v>-298000</v>
       </c>
       <c r="H100" t="n">
-        <v>-6.513693560325684</v>
+        <v>-10.61442564559216</v>
       </c>
       <c r="I100" t="inlineStr">
         <is>
-          <t>2026-03-19T00:21:23</t>
+          <t>2026-03-19T13:27:46</t>
         </is>
       </c>
     </row>
@@ -5303,17 +5303,17 @@
         <v>1</v>
       </c>
       <c r="F101" t="n">
-        <v>2360000</v>
+        <v>2406000</v>
       </c>
       <c r="G101" t="n">
-        <v>349000</v>
+        <v>395000</v>
       </c>
       <c r="H101" t="n">
-        <v>17.35454997513675</v>
+        <v>19.64196916956738</v>
       </c>
       <c r="I101" t="inlineStr">
         <is>
-          <t>2026-03-19T00:21:23</t>
+          <t>2026-03-19T13:27:46</t>
         </is>
       </c>
     </row>
@@ -5350,7 +5350,7 @@
       </c>
       <c r="I102" t="inlineStr">
         <is>
-          <t>2026-03-19T00:21:23</t>
+          <t>2026-03-19T13:27:46</t>
         </is>
       </c>
     </row>
@@ -5387,7 +5387,7 @@
       </c>
       <c r="I103" t="inlineStr">
         <is>
-          <t>2026-03-19T00:21:23</t>
+          <t>2026-03-19T13:27:46</t>
         </is>
       </c>
     </row>
@@ -5414,17 +5414,17 @@
         <v>1</v>
       </c>
       <c r="F104" t="n">
-        <v>2044800</v>
+        <v>2023200</v>
       </c>
       <c r="G104" t="n">
-        <v>-347400</v>
+        <v>-369000</v>
       </c>
       <c r="H104" t="n">
-        <v>-14.5221971407073</v>
+        <v>-15.42513167795335</v>
       </c>
       <c r="I104" t="inlineStr">
         <is>
-          <t>2026-03-19T00:21:23</t>
+          <t>2026-03-19T13:27:46</t>
         </is>
       </c>
     </row>
@@ -5451,17 +5451,17 @@
         <v>1</v>
       </c>
       <c r="F105" t="n">
-        <v>1899000</v>
+        <v>1938000</v>
       </c>
       <c r="G105" t="n">
-        <v>-159000</v>
+        <v>-120000</v>
       </c>
       <c r="H105" t="n">
-        <v>-7.725947521865889</v>
+        <v>-5.830903790087463</v>
       </c>
       <c r="I105" t="inlineStr">
         <is>
-          <t>2026-03-19T00:21:23</t>
+          <t>2026-03-19T13:27:46</t>
         </is>
       </c>
     </row>
@@ -5488,17 +5488,17 @@
         <v>1</v>
       </c>
       <c r="F106" t="n">
-        <v>1889775</v>
+        <v>1906800</v>
       </c>
       <c r="G106" t="n">
-        <v>-81726</v>
+        <v>-64701</v>
       </c>
       <c r="H106" t="n">
-        <v>-4.14536944186181</v>
+        <v>-3.281814211608312</v>
       </c>
       <c r="I106" t="inlineStr">
         <is>
-          <t>2026-03-19T00:21:23</t>
+          <t>2026-03-19T13:27:46</t>
         </is>
       </c>
     </row>
@@ -5535,7 +5535,7 @@
       </c>
       <c r="I107" t="inlineStr">
         <is>
-          <t>2026-03-19T00:21:23</t>
+          <t>2026-03-19T13:27:46</t>
         </is>
       </c>
     </row>
@@ -5572,7 +5572,7 @@
       </c>
       <c r="I108" t="inlineStr">
         <is>
-          <t>2026-03-19T00:21:23</t>
+          <t>2026-03-19T13:27:46</t>
         </is>
       </c>
     </row>
@@ -5599,17 +5599,17 @@
         <v>1</v>
       </c>
       <c r="F109" t="n">
-        <v>1663500</v>
+        <v>1698000</v>
       </c>
       <c r="G109" t="n">
-        <v>-19000</v>
+        <v>15500</v>
       </c>
       <c r="H109" t="n">
-        <v>-1.12927191679049</v>
+        <v>0.9212481426448738</v>
       </c>
       <c r="I109" t="inlineStr">
         <is>
-          <t>2026-03-19T00:21:23</t>
+          <t>2026-03-19T13:27:46</t>
         </is>
       </c>
     </row>
@@ -5636,17 +5636,17 @@
         <v>1</v>
       </c>
       <c r="F110" t="n">
-        <v>1600000</v>
+        <v>1627500</v>
       </c>
       <c r="G110" t="n">
-        <v>-49500.0000000007</v>
+        <v>-22000.0000000007</v>
       </c>
       <c r="H110" t="n">
-        <v>-3.00090936647473</v>
+        <v>-1.333737496211015</v>
       </c>
       <c r="I110" t="inlineStr">
         <is>
-          <t>2026-03-19T00:21:23</t>
+          <t>2026-03-19T13:27:46</t>
         </is>
       </c>
     </row>
@@ -5683,7 +5683,7 @@
       </c>
       <c r="I111" t="inlineStr">
         <is>
-          <t>2026-03-19T00:21:23</t>
+          <t>2026-03-19T13:27:46</t>
         </is>
       </c>
     </row>
@@ -5720,7 +5720,7 @@
       </c>
       <c r="I112" t="inlineStr">
         <is>
-          <t>2026-03-19T00:21:23</t>
+          <t>2026-03-19T13:27:46</t>
         </is>
       </c>
     </row>
@@ -5732,11 +5732,11 @@
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>하프니아</t>
+          <t>비에이치아이</t>
         </is>
       </c>
       <c r="C113" t="n">
-        <v>80</v>
+        <v>8</v>
       </c>
       <c r="D113" t="inlineStr">
         <is>
@@ -5747,17 +5747,17 @@
         <v>1</v>
       </c>
       <c r="F113" t="n">
-        <v>830222.8868876956</v>
+        <v>834400</v>
       </c>
       <c r="G113" t="n">
-        <v>204491.8868876956</v>
+        <v>169285</v>
       </c>
       <c r="H113" t="n">
-        <v>32.68047881401044</v>
+        <v>25.45198950557423</v>
       </c>
       <c r="I113" t="inlineStr">
         <is>
-          <t>2026-03-19T00:21:23</t>
+          <t>2026-03-19T13:27:46</t>
         </is>
       </c>
     </row>
@@ -5769,11 +5769,11 @@
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>비에이치아이</t>
+          <t>하프니아</t>
         </is>
       </c>
       <c r="C114" t="n">
-        <v>8</v>
+        <v>80</v>
       </c>
       <c r="D114" t="inlineStr">
         <is>
@@ -5784,17 +5784,17 @@
         <v>1</v>
       </c>
       <c r="F114" t="n">
-        <v>827200</v>
+        <v>830222.8868876956</v>
       </c>
       <c r="G114" t="n">
-        <v>162085</v>
+        <v>204491.8868876956</v>
       </c>
       <c r="H114" t="n">
-        <v>24.36946994128835</v>
+        <v>32.68047881401044</v>
       </c>
       <c r="I114" t="inlineStr">
         <is>
-          <t>2026-03-19T00:21:23</t>
+          <t>2026-03-19T13:27:46</t>
         </is>
       </c>
     </row>
@@ -5831,7 +5831,7 @@
       </c>
       <c r="I115" t="inlineStr">
         <is>
-          <t>2026-03-19T00:21:23</t>
+          <t>2026-03-19T13:27:46</t>
         </is>
       </c>
     </row>
@@ -5941,7 +5941,7 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>2026-03-19T00:21:23</t>
+          <t>2026-03-19T13:27:46</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: portfolio snapshot 2026-03-19 (2026-03-19T21:54:06)
</commit_message>
<xml_diff>
--- a/portfolio_auto.xlsx
+++ b/portfolio_auto.xlsx
@@ -486,13 +486,13 @@
         <v>1</v>
       </c>
       <c r="E2" t="n">
-        <v>14231364.16721486</v>
+        <v>14238562.79623244</v>
       </c>
       <c r="F2" t="n">
-        <v>2124815.167214859</v>
+        <v>2132013.796232443</v>
       </c>
       <c r="G2" t="n">
-        <v>17.55095665341841</v>
+        <v>17.61041727277066</v>
       </c>
     </row>
     <row r="3">
@@ -513,13 +513,13 @@
         <v>1</v>
       </c>
       <c r="E3" t="n">
-        <v>10812693.38748475</v>
+        <v>10802195.38683411</v>
       </c>
       <c r="F3" t="n">
-        <v>-19321.61251525022</v>
+        <v>-29819.61316589266</v>
       </c>
       <c r="G3" t="n">
-        <v>-0.178375053166472</v>
+        <v>-0.2752914685392576</v>
       </c>
     </row>
     <row r="4">
@@ -567,13 +567,13 @@
         <v>1</v>
       </c>
       <c r="E5" t="n">
-        <v>8440199.302239379</v>
+        <v>8629159.309373179</v>
       </c>
       <c r="F5" t="n">
-        <v>4010335.302239379</v>
+        <v>4199295.309373179</v>
       </c>
       <c r="G5" t="n">
-        <v>90.52953549452938</v>
+        <v>94.79512936228244</v>
       </c>
     </row>
     <row r="6">
@@ -594,13 +594,13 @@
         <v>1</v>
       </c>
       <c r="E6" t="n">
-        <v>8149471.423365676</v>
+        <v>8280438.313577486</v>
       </c>
       <c r="F6" t="n">
-        <v>1699120.423365676</v>
+        <v>1830087.313577486</v>
       </c>
       <c r="G6" t="n">
-        <v>26.34151883154383</v>
+        <v>28.37190276277192</v>
       </c>
     </row>
     <row r="7">
@@ -621,23 +621,23 @@
         <v>1</v>
       </c>
       <c r="E7" t="n">
-        <v>7029750.25177002</v>
+        <v>7265949.903135682</v>
       </c>
       <c r="F7" t="n">
-        <v>2902516.25177002</v>
+        <v>3138715.903135683</v>
       </c>
       <c r="G7" t="n">
-        <v>70.32594351980092</v>
+        <v>76.04889626165328</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>노블</t>
+          <t>세아제강</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>99</v>
+        <v>50</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
@@ -648,23 +648,23 @@
         <v>1</v>
       </c>
       <c r="E8" t="n">
-        <v>6926047.602600594</v>
+        <v>6945000</v>
       </c>
       <c r="F8" t="n">
-        <v>3018839.602600594</v>
+        <v>635000</v>
       </c>
       <c r="G8" t="n">
-        <v>77.2633451457049</v>
+        <v>10.06339144215531</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>세아제강</t>
+          <t>노블</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>50</v>
+        <v>99</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
@@ -675,13 +675,13 @@
         <v>1</v>
       </c>
       <c r="E9" t="n">
-        <v>6945000</v>
+        <v>7089362.533905029</v>
       </c>
       <c r="F9" t="n">
-        <v>635000</v>
+        <v>3182154.533905029</v>
       </c>
       <c r="G9" t="n">
-        <v>10.06339144215531</v>
+        <v>81.4431822903984</v>
       </c>
     </row>
     <row r="10">
@@ -702,13 +702,13 @@
         <v>1</v>
       </c>
       <c r="E10" t="n">
-        <v>6565089.595369929</v>
+        <v>6458956.91119526</v>
       </c>
       <c r="F10" t="n">
-        <v>333870.5953699304</v>
+        <v>227737.9111952605</v>
       </c>
       <c r="G10" t="n">
-        <v>5.358030192325618</v>
+        <v>3.654789074100277</v>
       </c>
     </row>
     <row r="11">
@@ -729,13 +729,13 @@
         <v>1</v>
       </c>
       <c r="E11" t="n">
-        <v>5418283.805207804</v>
+        <v>5347019.162831247</v>
       </c>
       <c r="F11" t="n">
-        <v>1693738.805207804</v>
+        <v>1622474.162831247</v>
       </c>
       <c r="G11" t="n">
-        <v>45.47505279726259</v>
+        <v>43.56167432078944</v>
       </c>
     </row>
     <row r="12">
@@ -756,13 +756,13 @@
         <v>1</v>
       </c>
       <c r="E12" t="n">
-        <v>5063294.781341553</v>
+        <v>5157624.699054079</v>
       </c>
       <c r="F12" t="n">
-        <v>1753286.781341553</v>
+        <v>1847616.699054079</v>
       </c>
       <c r="G12" t="n">
-        <v>52.96926114201393</v>
+        <v>55.81910071075596</v>
       </c>
     </row>
     <row r="13">
@@ -810,13 +810,13 @@
         <v>1</v>
       </c>
       <c r="E14" t="n">
-        <v>4627337.908720952</v>
+        <v>4596144.593352056</v>
       </c>
       <c r="F14" t="n">
-        <v>2370977.908720952</v>
+        <v>2339784.593352056</v>
       </c>
       <c r="G14" t="n">
-        <v>105.0797704586569</v>
+        <v>103.6973086454314</v>
       </c>
     </row>
     <row r="15">
@@ -849,11 +849,11 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>차코스 에너지 내비게이션</t>
+          <t>DL이앤씨</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>75</v>
+        <v>80</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
@@ -864,23 +864,23 @@
         <v>1</v>
       </c>
       <c r="E16" t="n">
-        <v>4023266.715580446</v>
+        <v>4152000</v>
       </c>
       <c r="F16" t="n">
-        <v>198618.7155804457</v>
+        <v>741000</v>
       </c>
       <c r="G16" t="n">
-        <v>5.193124062147567</v>
+        <v>21.72383465259455</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>DL이앤씨</t>
+          <t>HD건설기계</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>80</v>
+        <v>31</v>
       </c>
       <c r="C17" t="inlineStr">
         <is>
@@ -891,23 +891,23 @@
         <v>1</v>
       </c>
       <c r="E17" t="n">
-        <v>4152000</v>
+        <v>4082700</v>
       </c>
       <c r="F17" t="n">
-        <v>741000</v>
+        <v>47604</v>
       </c>
       <c r="G17" t="n">
-        <v>21.72383465259455</v>
+        <v>1.179748883297944</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>동원개발</t>
+          <t>차코스 에너지 내비게이션</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>1360</v>
+        <v>75</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
@@ -918,23 +918,23 @@
         <v>1</v>
       </c>
       <c r="E18" t="n">
-        <v>3957600</v>
+        <v>4081754.289162601</v>
       </c>
       <c r="F18" t="n">
-        <v>220200</v>
+        <v>257106.2891626009</v>
       </c>
       <c r="G18" t="n">
-        <v>5.891796436025045</v>
+        <v>6.722351682105146</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>HD건설기계</t>
+          <t>동원개발</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>31</v>
+        <v>1360</v>
       </c>
       <c r="C19" t="inlineStr">
         <is>
@@ -945,13 +945,13 @@
         <v>1</v>
       </c>
       <c r="E19" t="n">
-        <v>4082700</v>
+        <v>3957600</v>
       </c>
       <c r="F19" t="n">
-        <v>47604</v>
+        <v>220200</v>
       </c>
       <c r="G19" t="n">
-        <v>1.179748883297944</v>
+        <v>5.891796436025045</v>
       </c>
     </row>
     <row r="20">
@@ -972,13 +972,13 @@
         <v>1</v>
       </c>
       <c r="E20" t="n">
-        <v>3534595.754975702</v>
+        <v>3650596.24511658</v>
       </c>
       <c r="F20" t="n">
-        <v>2063823.754975702</v>
+        <v>2179824.24511658</v>
       </c>
       <c r="G20" t="n">
-        <v>140.3224806411668</v>
+        <v>148.2095284052579</v>
       </c>
     </row>
     <row r="21">
@@ -999,13 +999,13 @@
         <v>1</v>
       </c>
       <c r="E21" t="n">
-        <v>2993391.398657081</v>
+        <v>2978769.518133399</v>
       </c>
       <c r="F21" t="n">
-        <v>-197252.6013429193</v>
+        <v>-211874.4818666009</v>
       </c>
       <c r="G21" t="n">
-        <v>-6.182219054928074</v>
+        <v>-6.640492698859569</v>
       </c>
     </row>
     <row r="22">
@@ -1038,11 +1038,11 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>현대제철</t>
+          <t>KoAct 코스닥액티브</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>70</v>
+        <v>200</v>
       </c>
       <c r="C23" t="inlineStr">
         <is>
@@ -1053,23 +1053,23 @@
         <v>1</v>
       </c>
       <c r="E23" t="n">
-        <v>2509500</v>
+        <v>2526000</v>
       </c>
       <c r="F23" t="n">
-        <v>-298000</v>
+        <v>-176000</v>
       </c>
       <c r="G23" t="n">
-        <v>-10.61442564559216</v>
+        <v>-6.513693560325684</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>KoAct 코스닥액티브</t>
+          <t>현대제철</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>200</v>
+        <v>70</v>
       </c>
       <c r="C24" t="inlineStr">
         <is>
@@ -1080,13 +1080,13 @@
         <v>1</v>
       </c>
       <c r="E24" t="n">
-        <v>2526000</v>
+        <v>2509500</v>
       </c>
       <c r="F24" t="n">
-        <v>-176000</v>
+        <v>-298000</v>
       </c>
       <c r="G24" t="n">
-        <v>-6.513693560325684</v>
+        <v>-10.61442564559216</v>
       </c>
     </row>
     <row r="25">
@@ -1161,13 +1161,13 @@
         <v>1</v>
       </c>
       <c r="E27" t="n">
-        <v>2145682.294059377</v>
+        <v>2178165.369514748</v>
       </c>
       <c r="F27" t="n">
-        <v>81692.29405937716</v>
+        <v>114175.3695147485</v>
       </c>
       <c r="G27" t="n">
-        <v>3.957979159752575</v>
+        <v>5.531779200226186</v>
       </c>
     </row>
     <row r="28">
@@ -1269,13 +1269,13 @@
         <v>1</v>
       </c>
       <c r="E31" t="n">
-        <v>1709635.204022215</v>
+        <v>1704386.346717528</v>
       </c>
       <c r="F31" t="n">
-        <v>395282.2040222154</v>
+        <v>390033.3467175288</v>
       </c>
       <c r="G31" t="n">
-        <v>30.0742801988671</v>
+        <v>29.67493106627588</v>
       </c>
     </row>
     <row r="32">
@@ -1296,13 +1296,13 @@
         <v>1</v>
       </c>
       <c r="E32" t="n">
-        <v>1705616.038137302</v>
+        <v>1682281.111696094</v>
       </c>
       <c r="F32" t="n">
-        <v>11160.03813730204</v>
+        <v>-12174.88830390549</v>
       </c>
       <c r="G32" t="n">
-        <v>0.6586207099683933</v>
+        <v>-0.7185130982395231</v>
       </c>
     </row>
     <row r="33">
@@ -1416,11 +1416,11 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>하프니아</t>
+          <t>비에이치아이</t>
         </is>
       </c>
       <c r="B37" t="n">
-        <v>80</v>
+        <v>8</v>
       </c>
       <c r="C37" t="inlineStr">
         <is>
@@ -1431,23 +1431,23 @@
         <v>1</v>
       </c>
       <c r="E37" t="n">
-        <v>830222.8868876956</v>
+        <v>834400</v>
       </c>
       <c r="F37" t="n">
-        <v>204491.8868876956</v>
+        <v>169285</v>
       </c>
       <c r="G37" t="n">
-        <v>32.68047881401044</v>
+        <v>25.45198950557423</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>비에이치아이</t>
+          <t>하프니아</t>
         </is>
       </c>
       <c r="B38" t="n">
-        <v>8</v>
+        <v>80</v>
       </c>
       <c r="C38" t="inlineStr">
         <is>
@@ -1458,13 +1458,13 @@
         <v>1</v>
       </c>
       <c r="E38" t="n">
-        <v>834400</v>
+        <v>855417.5163666997</v>
       </c>
       <c r="F38" t="n">
-        <v>169285</v>
+        <v>229686.5163666997</v>
       </c>
       <c r="G38" t="n">
-        <v>25.45198950557423</v>
+        <v>36.70691021648275</v>
       </c>
     </row>
     <row r="39">
@@ -1485,13 +1485,13 @@
         <v>1</v>
       </c>
       <c r="E39" t="n">
-        <v>794950.4285003915</v>
+        <v>798609.6514927745</v>
       </c>
       <c r="F39" t="n">
-        <v>16359.42850039154</v>
+        <v>20018.65149277449</v>
       </c>
       <c r="G39" t="n">
-        <v>2.101158181945533</v>
+        <v>2.571138311741914</v>
       </c>
     </row>
   </sheetData>
@@ -1549,7 +1549,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2026-03-19T13:27:46</t>
+          <t>2026-03-19T21:54:06</t>
         </is>
       </c>
       <c r="E2" t="n">
@@ -4452,17 +4452,17 @@
         <v>1</v>
       </c>
       <c r="F78" t="n">
-        <v>14231364.16721486</v>
+        <v>14238562.79623244</v>
       </c>
       <c r="G78" t="n">
-        <v>2124815.167214859</v>
+        <v>2132013.796232443</v>
       </c>
       <c r="H78" t="n">
-        <v>17.55095665341841</v>
+        <v>17.61041727277066</v>
       </c>
       <c r="I78" t="inlineStr">
         <is>
-          <t>2026-03-19T13:27:46</t>
+          <t>2026-03-19T21:54:06</t>
         </is>
       </c>
     </row>
@@ -4489,17 +4489,17 @@
         <v>1</v>
       </c>
       <c r="F79" t="n">
-        <v>10812693.38748475</v>
+        <v>10802195.38683411</v>
       </c>
       <c r="G79" t="n">
-        <v>-19321.61251525022</v>
+        <v>-29819.61316589266</v>
       </c>
       <c r="H79" t="n">
-        <v>-0.178375053166472</v>
+        <v>-0.2752914685392576</v>
       </c>
       <c r="I79" t="inlineStr">
         <is>
-          <t>2026-03-19T13:27:46</t>
+          <t>2026-03-19T21:54:06</t>
         </is>
       </c>
     </row>
@@ -4536,7 +4536,7 @@
       </c>
       <c r="I80" t="inlineStr">
         <is>
-          <t>2026-03-19T13:27:46</t>
+          <t>2026-03-19T21:54:06</t>
         </is>
       </c>
     </row>
@@ -4563,17 +4563,17 @@
         <v>1</v>
       </c>
       <c r="F81" t="n">
-        <v>8440199.302239379</v>
+        <v>8629159.309373179</v>
       </c>
       <c r="G81" t="n">
-        <v>4010335.302239379</v>
+        <v>4199295.309373179</v>
       </c>
       <c r="H81" t="n">
-        <v>90.52953549452938</v>
+        <v>94.79512936228244</v>
       </c>
       <c r="I81" t="inlineStr">
         <is>
-          <t>2026-03-19T13:27:46</t>
+          <t>2026-03-19T21:54:06</t>
         </is>
       </c>
     </row>
@@ -4600,17 +4600,17 @@
         <v>1</v>
       </c>
       <c r="F82" t="n">
-        <v>8149471.423365676</v>
+        <v>8280438.313577486</v>
       </c>
       <c r="G82" t="n">
-        <v>1699120.423365676</v>
+        <v>1830087.313577486</v>
       </c>
       <c r="H82" t="n">
-        <v>26.34151883154383</v>
+        <v>28.37190276277192</v>
       </c>
       <c r="I82" t="inlineStr">
         <is>
-          <t>2026-03-19T13:27:46</t>
+          <t>2026-03-19T21:54:06</t>
         </is>
       </c>
     </row>
@@ -4637,17 +4637,17 @@
         <v>1</v>
       </c>
       <c r="F83" t="n">
-        <v>7029750.25177002</v>
+        <v>7265949.903135682</v>
       </c>
       <c r="G83" t="n">
-        <v>2902516.25177002</v>
+        <v>3138715.903135683</v>
       </c>
       <c r="H83" t="n">
-        <v>70.32594351980092</v>
+        <v>76.04889626165328</v>
       </c>
       <c r="I83" t="inlineStr">
         <is>
-          <t>2026-03-19T13:27:46</t>
+          <t>2026-03-19T21:54:06</t>
         </is>
       </c>
     </row>
@@ -4659,11 +4659,11 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>세아제강</t>
+          <t>노블</t>
         </is>
       </c>
       <c r="C84" t="n">
-        <v>50</v>
+        <v>99</v>
       </c>
       <c r="D84" t="inlineStr">
         <is>
@@ -4674,17 +4674,17 @@
         <v>1</v>
       </c>
       <c r="F84" t="n">
-        <v>6945000</v>
+        <v>7089362.533905029</v>
       </c>
       <c r="G84" t="n">
-        <v>635000</v>
+        <v>3182154.533905029</v>
       </c>
       <c r="H84" t="n">
-        <v>10.06339144215531</v>
+        <v>81.4431822903984</v>
       </c>
       <c r="I84" t="inlineStr">
         <is>
-          <t>2026-03-19T13:27:46</t>
+          <t>2026-03-19T21:54:06</t>
         </is>
       </c>
     </row>
@@ -4696,11 +4696,11 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>노블</t>
+          <t>세아제강</t>
         </is>
       </c>
       <c r="C85" t="n">
-        <v>99</v>
+        <v>50</v>
       </c>
       <c r="D85" t="inlineStr">
         <is>
@@ -4711,17 +4711,17 @@
         <v>1</v>
       </c>
       <c r="F85" t="n">
-        <v>6926047.602600594</v>
+        <v>6945000</v>
       </c>
       <c r="G85" t="n">
-        <v>3018839.602600594</v>
+        <v>635000</v>
       </c>
       <c r="H85" t="n">
-        <v>77.2633451457049</v>
+        <v>10.06339144215531</v>
       </c>
       <c r="I85" t="inlineStr">
         <is>
-          <t>2026-03-19T13:27:46</t>
+          <t>2026-03-19T21:54:06</t>
         </is>
       </c>
     </row>
@@ -4748,17 +4748,17 @@
         <v>1</v>
       </c>
       <c r="F86" t="n">
-        <v>6565089.595369929</v>
+        <v>6458956.91119526</v>
       </c>
       <c r="G86" t="n">
-        <v>333870.5953699304</v>
+        <v>227737.9111952605</v>
       </c>
       <c r="H86" t="n">
-        <v>5.358030192325618</v>
+        <v>3.654789074100277</v>
       </c>
       <c r="I86" t="inlineStr">
         <is>
-          <t>2026-03-19T13:27:46</t>
+          <t>2026-03-19T21:54:06</t>
         </is>
       </c>
     </row>
@@ -4785,17 +4785,17 @@
         <v>1</v>
       </c>
       <c r="F87" t="n">
-        <v>5418283.805207804</v>
+        <v>5347019.162831247</v>
       </c>
       <c r="G87" t="n">
-        <v>1693738.805207804</v>
+        <v>1622474.162831247</v>
       </c>
       <c r="H87" t="n">
-        <v>45.47505279726259</v>
+        <v>43.56167432078944</v>
       </c>
       <c r="I87" t="inlineStr">
         <is>
-          <t>2026-03-19T13:27:46</t>
+          <t>2026-03-19T21:54:06</t>
         </is>
       </c>
     </row>
@@ -4822,17 +4822,17 @@
         <v>1</v>
       </c>
       <c r="F88" t="n">
-        <v>5063294.781341553</v>
+        <v>5157624.699054079</v>
       </c>
       <c r="G88" t="n">
-        <v>1753286.781341553</v>
+        <v>1847616.699054079</v>
       </c>
       <c r="H88" t="n">
-        <v>52.96926114201393</v>
+        <v>55.81910071075596</v>
       </c>
       <c r="I88" t="inlineStr">
         <is>
-          <t>2026-03-19T13:27:46</t>
+          <t>2026-03-19T21:54:06</t>
         </is>
       </c>
     </row>
@@ -4869,7 +4869,7 @@
       </c>
       <c r="I89" t="inlineStr">
         <is>
-          <t>2026-03-19T13:27:46</t>
+          <t>2026-03-19T21:54:06</t>
         </is>
       </c>
     </row>
@@ -4896,17 +4896,17 @@
         <v>1</v>
       </c>
       <c r="F90" t="n">
-        <v>4627337.908720952</v>
+        <v>4596144.593352056</v>
       </c>
       <c r="G90" t="n">
-        <v>2370977.908720952</v>
+        <v>2339784.593352056</v>
       </c>
       <c r="H90" t="n">
-        <v>105.0797704586569</v>
+        <v>103.6973086454314</v>
       </c>
       <c r="I90" t="inlineStr">
         <is>
-          <t>2026-03-19T13:27:46</t>
+          <t>2026-03-19T21:54:06</t>
         </is>
       </c>
     </row>
@@ -4943,7 +4943,7 @@
       </c>
       <c r="I91" t="inlineStr">
         <is>
-          <t>2026-03-19T13:27:46</t>
+          <t>2026-03-19T21:54:06</t>
         </is>
       </c>
     </row>
@@ -4980,7 +4980,7 @@
       </c>
       <c r="I92" t="inlineStr">
         <is>
-          <t>2026-03-19T13:27:46</t>
+          <t>2026-03-19T21:54:06</t>
         </is>
       </c>
     </row>
@@ -5017,7 +5017,7 @@
       </c>
       <c r="I93" t="inlineStr">
         <is>
-          <t>2026-03-19T13:27:46</t>
+          <t>2026-03-19T21:54:06</t>
         </is>
       </c>
     </row>
@@ -5044,17 +5044,17 @@
         <v>1</v>
       </c>
       <c r="F94" t="n">
-        <v>4023266.715580446</v>
+        <v>4081754.289162601</v>
       </c>
       <c r="G94" t="n">
-        <v>198618.7155804457</v>
+        <v>257106.2891626009</v>
       </c>
       <c r="H94" t="n">
-        <v>5.193124062147567</v>
+        <v>6.722351682105146</v>
       </c>
       <c r="I94" t="inlineStr">
         <is>
-          <t>2026-03-19T13:27:46</t>
+          <t>2026-03-19T21:54:06</t>
         </is>
       </c>
     </row>
@@ -5091,7 +5091,7 @@
       </c>
       <c r="I95" t="inlineStr">
         <is>
-          <t>2026-03-19T13:27:46</t>
+          <t>2026-03-19T21:54:06</t>
         </is>
       </c>
     </row>
@@ -5118,17 +5118,17 @@
         <v>1</v>
       </c>
       <c r="F96" t="n">
-        <v>3534595.754975702</v>
+        <v>3650596.24511658</v>
       </c>
       <c r="G96" t="n">
-        <v>2063823.754975702</v>
+        <v>2179824.24511658</v>
       </c>
       <c r="H96" t="n">
-        <v>140.3224806411668</v>
+        <v>148.2095284052579</v>
       </c>
       <c r="I96" t="inlineStr">
         <is>
-          <t>2026-03-19T13:27:46</t>
+          <t>2026-03-19T21:54:06</t>
         </is>
       </c>
     </row>
@@ -5155,17 +5155,17 @@
         <v>1</v>
       </c>
       <c r="F97" t="n">
-        <v>2993391.398657081</v>
+        <v>2978769.518133399</v>
       </c>
       <c r="G97" t="n">
-        <v>-197252.6013429193</v>
+        <v>-211874.4818666009</v>
       </c>
       <c r="H97" t="n">
-        <v>-6.182219054928074</v>
+        <v>-6.640492698859569</v>
       </c>
       <c r="I97" t="inlineStr">
         <is>
-          <t>2026-03-19T13:27:46</t>
+          <t>2026-03-19T21:54:06</t>
         </is>
       </c>
     </row>
@@ -5202,7 +5202,7 @@
       </c>
       <c r="I98" t="inlineStr">
         <is>
-          <t>2026-03-19T13:27:46</t>
+          <t>2026-03-19T21:54:06</t>
         </is>
       </c>
     </row>
@@ -5239,7 +5239,7 @@
       </c>
       <c r="I99" t="inlineStr">
         <is>
-          <t>2026-03-19T13:27:46</t>
+          <t>2026-03-19T21:54:06</t>
         </is>
       </c>
     </row>
@@ -5276,7 +5276,7 @@
       </c>
       <c r="I100" t="inlineStr">
         <is>
-          <t>2026-03-19T13:27:46</t>
+          <t>2026-03-19T21:54:06</t>
         </is>
       </c>
     </row>
@@ -5313,7 +5313,7 @@
       </c>
       <c r="I101" t="inlineStr">
         <is>
-          <t>2026-03-19T13:27:46</t>
+          <t>2026-03-19T21:54:06</t>
         </is>
       </c>
     </row>
@@ -5350,7 +5350,7 @@
       </c>
       <c r="I102" t="inlineStr">
         <is>
-          <t>2026-03-19T13:27:46</t>
+          <t>2026-03-19T21:54:06</t>
         </is>
       </c>
     </row>
@@ -5377,17 +5377,17 @@
         <v>1</v>
       </c>
       <c r="F103" t="n">
-        <v>2145682.294059377</v>
+        <v>2178165.369514748</v>
       </c>
       <c r="G103" t="n">
-        <v>81692.29405937716</v>
+        <v>114175.3695147485</v>
       </c>
       <c r="H103" t="n">
-        <v>3.957979159752575</v>
+        <v>5.531779200226186</v>
       </c>
       <c r="I103" t="inlineStr">
         <is>
-          <t>2026-03-19T13:27:46</t>
+          <t>2026-03-19T21:54:06</t>
         </is>
       </c>
     </row>
@@ -5424,7 +5424,7 @@
       </c>
       <c r="I104" t="inlineStr">
         <is>
-          <t>2026-03-19T13:27:46</t>
+          <t>2026-03-19T21:54:06</t>
         </is>
       </c>
     </row>
@@ -5461,7 +5461,7 @@
       </c>
       <c r="I105" t="inlineStr">
         <is>
-          <t>2026-03-19T13:27:46</t>
+          <t>2026-03-19T21:54:06</t>
         </is>
       </c>
     </row>
@@ -5498,7 +5498,7 @@
       </c>
       <c r="I106" t="inlineStr">
         <is>
-          <t>2026-03-19T13:27:46</t>
+          <t>2026-03-19T21:54:06</t>
         </is>
       </c>
     </row>
@@ -5525,17 +5525,17 @@
         <v>1</v>
       </c>
       <c r="F107" t="n">
-        <v>1709635.204022215</v>
+        <v>1704386.346717528</v>
       </c>
       <c r="G107" t="n">
-        <v>395282.2040222154</v>
+        <v>390033.3467175288</v>
       </c>
       <c r="H107" t="n">
-        <v>30.0742801988671</v>
+        <v>29.67493106627588</v>
       </c>
       <c r="I107" t="inlineStr">
         <is>
-          <t>2026-03-19T13:27:46</t>
+          <t>2026-03-19T21:54:06</t>
         </is>
       </c>
     </row>
@@ -5547,11 +5547,11 @@
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>유나이티드헬스 그룹</t>
+          <t>하나금융지주</t>
         </is>
       </c>
       <c r="C108" t="n">
-        <v>4</v>
+        <v>15</v>
       </c>
       <c r="D108" t="inlineStr">
         <is>
@@ -5562,17 +5562,17 @@
         <v>1</v>
       </c>
       <c r="F108" t="n">
-        <v>1705616.038137302</v>
+        <v>1698000</v>
       </c>
       <c r="G108" t="n">
-        <v>11160.03813730204</v>
+        <v>15500</v>
       </c>
       <c r="H108" t="n">
-        <v>0.6586207099683933</v>
+        <v>0.9212481426448738</v>
       </c>
       <c r="I108" t="inlineStr">
         <is>
-          <t>2026-03-19T13:27:46</t>
+          <t>2026-03-19T21:54:06</t>
         </is>
       </c>
     </row>
@@ -5584,11 +5584,11 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>하나금융지주</t>
+          <t>유나이티드헬스 그룹</t>
         </is>
       </c>
       <c r="C109" t="n">
-        <v>15</v>
+        <v>4</v>
       </c>
       <c r="D109" t="inlineStr">
         <is>
@@ -5599,17 +5599,17 @@
         <v>1</v>
       </c>
       <c r="F109" t="n">
-        <v>1698000</v>
+        <v>1682281.111696094</v>
       </c>
       <c r="G109" t="n">
-        <v>15500</v>
+        <v>-12174.88830390549</v>
       </c>
       <c r="H109" t="n">
-        <v>0.9212481426448738</v>
+        <v>-0.7185130982395231</v>
       </c>
       <c r="I109" t="inlineStr">
         <is>
-          <t>2026-03-19T13:27:46</t>
+          <t>2026-03-19T21:54:06</t>
         </is>
       </c>
     </row>
@@ -5646,7 +5646,7 @@
       </c>
       <c r="I110" t="inlineStr">
         <is>
-          <t>2026-03-19T13:27:46</t>
+          <t>2026-03-19T21:54:06</t>
         </is>
       </c>
     </row>
@@ -5683,7 +5683,7 @@
       </c>
       <c r="I111" t="inlineStr">
         <is>
-          <t>2026-03-19T13:27:46</t>
+          <t>2026-03-19T21:54:06</t>
         </is>
       </c>
     </row>
@@ -5720,7 +5720,7 @@
       </c>
       <c r="I112" t="inlineStr">
         <is>
-          <t>2026-03-19T13:27:46</t>
+          <t>2026-03-19T21:54:06</t>
         </is>
       </c>
     </row>
@@ -5732,11 +5732,11 @@
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>비에이치아이</t>
+          <t>하프니아</t>
         </is>
       </c>
       <c r="C113" t="n">
-        <v>8</v>
+        <v>80</v>
       </c>
       <c r="D113" t="inlineStr">
         <is>
@@ -5747,17 +5747,17 @@
         <v>1</v>
       </c>
       <c r="F113" t="n">
-        <v>834400</v>
+        <v>855417.5163666997</v>
       </c>
       <c r="G113" t="n">
-        <v>169285</v>
+        <v>229686.5163666997</v>
       </c>
       <c r="H113" t="n">
-        <v>25.45198950557423</v>
+        <v>36.70691021648275</v>
       </c>
       <c r="I113" t="inlineStr">
         <is>
-          <t>2026-03-19T13:27:46</t>
+          <t>2026-03-19T21:54:06</t>
         </is>
       </c>
     </row>
@@ -5769,11 +5769,11 @@
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>하프니아</t>
+          <t>비에이치아이</t>
         </is>
       </c>
       <c r="C114" t="n">
-        <v>80</v>
+        <v>8</v>
       </c>
       <c r="D114" t="inlineStr">
         <is>
@@ -5784,17 +5784,17 @@
         <v>1</v>
       </c>
       <c r="F114" t="n">
-        <v>830222.8868876956</v>
+        <v>834400</v>
       </c>
       <c r="G114" t="n">
-        <v>204491.8868876956</v>
+        <v>169285</v>
       </c>
       <c r="H114" t="n">
-        <v>32.68047881401044</v>
+        <v>25.45198950557423</v>
       </c>
       <c r="I114" t="inlineStr">
         <is>
-          <t>2026-03-19T13:27:46</t>
+          <t>2026-03-19T21:54:06</t>
         </is>
       </c>
     </row>
@@ -5821,17 +5821,17 @@
         <v>1</v>
       </c>
       <c r="F115" t="n">
-        <v>794950.4285003915</v>
+        <v>798609.6514927745</v>
       </c>
       <c r="G115" t="n">
-        <v>16359.42850039154</v>
+        <v>20018.65149277449</v>
       </c>
       <c r="H115" t="n">
-        <v>2.101158181945533</v>
+        <v>2.571138311741914</v>
       </c>
       <c r="I115" t="inlineStr">
         <is>
-          <t>2026-03-19T13:27:46</t>
+          <t>2026-03-19T21:54:06</t>
         </is>
       </c>
     </row>
@@ -5941,7 +5941,7 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>2026-03-19T13:27:46</t>
+          <t>2026-03-19T21:54:06</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: portfolio snapshot 2026-03-20 (2026-03-20T03:06:55)
</commit_message>
<xml_diff>
--- a/portfolio_auto.xlsx
+++ b/portfolio_auto.xlsx
@@ -486,13 +486,13 @@
         <v>1</v>
       </c>
       <c r="E2" t="n">
-        <v>14238562.79623244</v>
+        <v>14203432.81962231</v>
       </c>
       <c r="F2" t="n">
-        <v>2132013.796232443</v>
+        <v>2096883.819622312</v>
       </c>
       <c r="G2" t="n">
-        <v>17.61041727277066</v>
+        <v>17.32024394088119</v>
       </c>
     </row>
     <row r="3">
@@ -513,13 +513,13 @@
         <v>1</v>
       </c>
       <c r="E3" t="n">
-        <v>10802195.38683411</v>
+        <v>10775543.75936943</v>
       </c>
       <c r="F3" t="n">
-        <v>-29819.61316589266</v>
+        <v>-56471.2406305708</v>
       </c>
       <c r="G3" t="n">
-        <v>-0.2752914685392576</v>
+        <v>-0.5213364330696624</v>
       </c>
     </row>
     <row r="4">
@@ -540,13 +540,13 @@
         <v>1</v>
       </c>
       <c r="E4" t="n">
-        <v>9490000</v>
+        <v>9240000</v>
       </c>
       <c r="F4" t="n">
-        <v>2277000</v>
+        <v>2027000</v>
       </c>
       <c r="G4" t="n">
-        <v>31.56800221821711</v>
+        <v>28.10203798696798</v>
       </c>
     </row>
     <row r="5">
@@ -567,13 +567,13 @@
         <v>1</v>
       </c>
       <c r="E5" t="n">
-        <v>8629159.309373179</v>
+        <v>8607869.087246014</v>
       </c>
       <c r="F5" t="n">
-        <v>4199295.309373179</v>
+        <v>4178005.087246014</v>
       </c>
       <c r="G5" t="n">
-        <v>94.79512936228244</v>
+        <v>94.31452268615953</v>
       </c>
     </row>
     <row r="6">
@@ -594,13 +594,13 @@
         <v>1</v>
       </c>
       <c r="E6" t="n">
-        <v>8280438.313577486</v>
+        <v>8260008.470450722</v>
       </c>
       <c r="F6" t="n">
-        <v>1830087.313577486</v>
+        <v>1809657.470450722</v>
       </c>
       <c r="G6" t="n">
-        <v>28.37190276277192</v>
+        <v>28.05517824457494</v>
       </c>
     </row>
     <row r="7">
@@ -621,13 +621,13 @@
         <v>1</v>
       </c>
       <c r="E7" t="n">
-        <v>7265949.903135682</v>
+        <v>7248023.048171424</v>
       </c>
       <c r="F7" t="n">
-        <v>3138715.903135683</v>
+        <v>3120789.048171425</v>
       </c>
       <c r="G7" t="n">
-        <v>76.04889626165328</v>
+        <v>75.61454107451686</v>
       </c>
     </row>
     <row r="8">
@@ -648,13 +648,13 @@
         <v>1</v>
       </c>
       <c r="E8" t="n">
-        <v>6945000</v>
+        <v>7315000</v>
       </c>
       <c r="F8" t="n">
-        <v>635000</v>
+        <v>1005000</v>
       </c>
       <c r="G8" t="n">
-        <v>10.06339144215531</v>
+        <v>15.92709984152139</v>
       </c>
     </row>
     <row r="9">
@@ -675,13 +675,13 @@
         <v>1</v>
       </c>
       <c r="E9" t="n">
-        <v>7089362.533905029</v>
+        <v>7071871.362670898</v>
       </c>
       <c r="F9" t="n">
-        <v>3182154.533905029</v>
+        <v>3164663.362670898</v>
       </c>
       <c r="G9" t="n">
-        <v>81.4431822903984</v>
+        <v>80.99551809555309</v>
       </c>
     </row>
     <row r="10">
@@ -702,13 +702,13 @@
         <v>1</v>
       </c>
       <c r="E10" t="n">
-        <v>6458956.91119526</v>
+        <v>6443021.103033766</v>
       </c>
       <c r="F10" t="n">
-        <v>227737.9111952605</v>
+        <v>211802.1030337671</v>
       </c>
       <c r="G10" t="n">
-        <v>3.654789074100277</v>
+        <v>3.399047650768928</v>
       </c>
     </row>
     <row r="11">
@@ -729,13 +729,13 @@
         <v>1</v>
       </c>
       <c r="E11" t="n">
-        <v>5347019.162831247</v>
+        <v>5333826.773907423</v>
       </c>
       <c r="F11" t="n">
-        <v>1622474.162831247</v>
+        <v>1609281.773907423</v>
       </c>
       <c r="G11" t="n">
-        <v>43.56167432078944</v>
+        <v>43.20747296401098</v>
       </c>
     </row>
     <row r="12">
@@ -756,13 +756,13 @@
         <v>1</v>
       </c>
       <c r="E12" t="n">
-        <v>5157624.699054079</v>
+        <v>5144899.592058761</v>
       </c>
       <c r="F12" t="n">
-        <v>1847616.699054079</v>
+        <v>1834891.592058761</v>
       </c>
       <c r="G12" t="n">
-        <v>55.81910071075596</v>
+        <v>55.43465731982403</v>
       </c>
     </row>
     <row r="13">
@@ -783,13 +783,13 @@
         <v>1</v>
       </c>
       <c r="E13" t="n">
-        <v>4763700</v>
+        <v>4787820</v>
       </c>
       <c r="F13" t="n">
-        <v>39903</v>
+        <v>64023</v>
       </c>
       <c r="G13" t="n">
-        <v>0.8447230056668396</v>
+        <v>1.355329198100596</v>
       </c>
     </row>
     <row r="14">
@@ -810,13 +810,13 @@
         <v>1</v>
       </c>
       <c r="E14" t="n">
-        <v>4596144.593352056</v>
+        <v>4584804.793516081</v>
       </c>
       <c r="F14" t="n">
-        <v>2339784.593352056</v>
+        <v>2328444.793516081</v>
       </c>
       <c r="G14" t="n">
-        <v>103.6973086454314</v>
+        <v>103.1947381409031</v>
       </c>
     </row>
     <row r="15">
@@ -837,13 +837,13 @@
         <v>1</v>
       </c>
       <c r="E15" t="n">
-        <v>4306500</v>
+        <v>4293000</v>
       </c>
       <c r="F15" t="n">
-        <v>-324500</v>
+        <v>-338000</v>
       </c>
       <c r="G15" t="n">
-        <v>-7.007125890736342</v>
+        <v>-7.298639602677608</v>
       </c>
     </row>
     <row r="16">
@@ -864,13 +864,13 @@
         <v>1</v>
       </c>
       <c r="E16" t="n">
-        <v>4152000</v>
+        <v>5112000</v>
       </c>
       <c r="F16" t="n">
-        <v>741000</v>
+        <v>1701000</v>
       </c>
       <c r="G16" t="n">
-        <v>21.72383465259455</v>
+        <v>49.86807387862797</v>
       </c>
     </row>
     <row r="17">
@@ -891,13 +891,13 @@
         <v>1</v>
       </c>
       <c r="E17" t="n">
-        <v>4082700</v>
+        <v>4101300</v>
       </c>
       <c r="F17" t="n">
-        <v>47604</v>
+        <v>66204</v>
       </c>
       <c r="G17" t="n">
-        <v>1.179748883297944</v>
+        <v>1.640704459076066</v>
       </c>
     </row>
     <row r="18">
@@ -918,13 +918,13 @@
         <v>1</v>
       </c>
       <c r="E18" t="n">
-        <v>4081754.289162601</v>
+        <v>4071683.614561614</v>
       </c>
       <c r="F18" t="n">
-        <v>257106.2891626009</v>
+        <v>247035.6145616136</v>
       </c>
       <c r="G18" t="n">
-        <v>6.722351682105146</v>
+        <v>6.459041840232452</v>
       </c>
     </row>
     <row r="19">
@@ -945,13 +945,13 @@
         <v>1</v>
       </c>
       <c r="E19" t="n">
-        <v>3957600</v>
+        <v>4127600</v>
       </c>
       <c r="F19" t="n">
-        <v>220200</v>
+        <v>390200</v>
       </c>
       <c r="G19" t="n">
-        <v>5.891796436025045</v>
+        <v>10.44041312142131</v>
       </c>
     </row>
     <row r="20">
@@ -972,13 +972,13 @@
         <v>1</v>
       </c>
       <c r="E20" t="n">
-        <v>3650596.24511658</v>
+        <v>3641589.341643294</v>
       </c>
       <c r="F20" t="n">
-        <v>2179824.24511658</v>
+        <v>2170817.341643294</v>
       </c>
       <c r="G20" t="n">
-        <v>148.2095284052579</v>
+        <v>147.5971354936927</v>
       </c>
     </row>
     <row r="21">
@@ -999,13 +999,13 @@
         <v>1</v>
       </c>
       <c r="E21" t="n">
-        <v>2978769.518133399</v>
+        <v>2971420.173610602</v>
       </c>
       <c r="F21" t="n">
-        <v>-211874.4818666009</v>
+        <v>-219223.8263893984</v>
       </c>
       <c r="G21" t="n">
-        <v>-6.640492698859569</v>
+        <v>-6.870833173158723</v>
       </c>
     </row>
     <row r="22">
@@ -1026,13 +1026,13 @@
         <v>1</v>
       </c>
       <c r="E22" t="n">
-        <v>2620000</v>
+        <v>2735000</v>
       </c>
       <c r="F22" t="n">
-        <v>341390</v>
+        <v>456390</v>
       </c>
       <c r="G22" t="n">
-        <v>14.98237960862105</v>
+        <v>20.02931611815976</v>
       </c>
     </row>
     <row r="23">
@@ -1053,13 +1053,13 @@
         <v>1</v>
       </c>
       <c r="E23" t="n">
-        <v>2526000</v>
+        <v>2583000</v>
       </c>
       <c r="F23" t="n">
-        <v>-176000</v>
+        <v>-119000</v>
       </c>
       <c r="G23" t="n">
-        <v>-6.513693560325684</v>
+        <v>-4.404145077720207</v>
       </c>
     </row>
     <row r="24">
@@ -1080,13 +1080,13 @@
         <v>1</v>
       </c>
       <c r="E24" t="n">
-        <v>2509500</v>
+        <v>2593500</v>
       </c>
       <c r="F24" t="n">
-        <v>-298000</v>
+        <v>-214000</v>
       </c>
       <c r="G24" t="n">
-        <v>-10.61442564559216</v>
+        <v>-7.622439893143366</v>
       </c>
     </row>
     <row r="25">
@@ -1107,13 +1107,13 @@
         <v>1</v>
       </c>
       <c r="E25" t="n">
-        <v>2406000</v>
+        <v>2486000</v>
       </c>
       <c r="F25" t="n">
-        <v>395000</v>
+        <v>475000</v>
       </c>
       <c r="G25" t="n">
-        <v>19.64196916956738</v>
+        <v>23.62008950770761</v>
       </c>
     </row>
     <row r="26">
@@ -1134,13 +1134,13 @@
         <v>1</v>
       </c>
       <c r="E26" t="n">
-        <v>2180750</v>
+        <v>2216500</v>
       </c>
       <c r="F26" t="n">
-        <v>471249</v>
+        <v>506999</v>
       </c>
       <c r="G26" t="n">
-        <v>27.56646530186294</v>
+        <v>29.65771883140168</v>
       </c>
     </row>
     <row r="27">
@@ -1161,13 +1161,13 @@
         <v>1</v>
       </c>
       <c r="E27" t="n">
-        <v>2178165.369514748</v>
+        <v>2172791.30897373</v>
       </c>
       <c r="F27" t="n">
-        <v>114175.3695147485</v>
+        <v>108801.3089737301</v>
       </c>
       <c r="G27" t="n">
-        <v>5.531779200226186</v>
+        <v>5.271406788488806</v>
       </c>
     </row>
     <row r="28">
@@ -1188,13 +1188,13 @@
         <v>1</v>
       </c>
       <c r="E28" t="n">
-        <v>2023200</v>
+        <v>2071800</v>
       </c>
       <c r="F28" t="n">
-        <v>-369000</v>
+        <v>-320400</v>
       </c>
       <c r="G28" t="n">
-        <v>-15.42513167795335</v>
+        <v>-13.39352896914974</v>
       </c>
     </row>
     <row r="29">
@@ -1215,13 +1215,13 @@
         <v>1</v>
       </c>
       <c r="E29" t="n">
-        <v>1938000</v>
+        <v>1995000</v>
       </c>
       <c r="F29" t="n">
-        <v>-120000</v>
+        <v>-63000</v>
       </c>
       <c r="G29" t="n">
-        <v>-5.830903790087463</v>
+        <v>-3.061224489795918</v>
       </c>
     </row>
     <row r="30">
@@ -1242,13 +1242,13 @@
         <v>1</v>
       </c>
       <c r="E30" t="n">
-        <v>1906800</v>
+        <v>1961280</v>
       </c>
       <c r="F30" t="n">
-        <v>-64701</v>
+        <v>-10221</v>
       </c>
       <c r="G30" t="n">
-        <v>-3.281814211608312</v>
+        <v>-0.5184374747971215</v>
       </c>
     </row>
     <row r="31">
@@ -1269,13 +1269,13 @@
         <v>1</v>
       </c>
       <c r="E31" t="n">
-        <v>1704386.346717528</v>
+        <v>1700181.21356247</v>
       </c>
       <c r="F31" t="n">
-        <v>390033.3467175288</v>
+        <v>385828.2135624706</v>
       </c>
       <c r="G31" t="n">
-        <v>29.67493106627588</v>
+        <v>29.35499166224529</v>
       </c>
     </row>
     <row r="32">
@@ -1296,13 +1296,13 @@
         <v>1</v>
       </c>
       <c r="E32" t="n">
-        <v>1682281.111696094</v>
+        <v>1678130.517499804</v>
       </c>
       <c r="F32" t="n">
-        <v>-12174.88830390549</v>
+        <v>-16325.48250019504</v>
       </c>
       <c r="G32" t="n">
-        <v>-0.7185130982395231</v>
+        <v>-0.9634645278599764</v>
       </c>
     </row>
     <row r="33">
@@ -1323,13 +1323,13 @@
         <v>1</v>
       </c>
       <c r="E33" t="n">
-        <v>1698000</v>
+        <v>1713000</v>
       </c>
       <c r="F33" t="n">
-        <v>15500</v>
+        <v>30500</v>
       </c>
       <c r="G33" t="n">
-        <v>0.9212481426448738</v>
+        <v>1.812778603268945</v>
       </c>
     </row>
     <row r="34">
@@ -1350,13 +1350,13 @@
         <v>1</v>
       </c>
       <c r="E34" t="n">
-        <v>1627500</v>
+        <v>1647500</v>
       </c>
       <c r="F34" t="n">
-        <v>-22000.0000000007</v>
+        <v>-2000.000000000698</v>
       </c>
       <c r="G34" t="n">
-        <v>-1.333737496211015</v>
+        <v>-0.1212488632919489</v>
       </c>
     </row>
     <row r="35">
@@ -1377,13 +1377,13 @@
         <v>1</v>
       </c>
       <c r="E35" t="n">
-        <v>922000</v>
+        <v>900000</v>
       </c>
       <c r="F35" t="n">
-        <v>89000</v>
+        <v>67000</v>
       </c>
       <c r="G35" t="n">
-        <v>10.68427370948379</v>
+        <v>8.043217286914766</v>
       </c>
     </row>
     <row r="36">
@@ -1404,13 +1404,13 @@
         <v>1</v>
       </c>
       <c r="E36" t="n">
-        <v>858716.8307915051</v>
+        <v>856598.1687739864</v>
       </c>
       <c r="F36" t="n">
-        <v>-157338.1692084949</v>
+        <v>-159456.8312260136</v>
       </c>
       <c r="G36" t="n">
-        <v>-15.48520200269621</v>
+        <v>-15.69372044092235</v>
       </c>
     </row>
     <row r="37">
@@ -1431,13 +1431,13 @@
         <v>1</v>
       </c>
       <c r="E37" t="n">
-        <v>834400</v>
+        <v>887200</v>
       </c>
       <c r="F37" t="n">
-        <v>169285</v>
+        <v>222085</v>
       </c>
       <c r="G37" t="n">
-        <v>25.45198950557423</v>
+        <v>33.39046631033731</v>
       </c>
     </row>
     <row r="38">
@@ -1458,13 +1458,13 @@
         <v>1</v>
       </c>
       <c r="E38" t="n">
-        <v>855417.5163666997</v>
+        <v>853306.9945554808</v>
       </c>
       <c r="F38" t="n">
-        <v>229686.5163666997</v>
+        <v>227575.9945554808</v>
       </c>
       <c r="G38" t="n">
-        <v>36.70691021648275</v>
+        <v>36.36962121989813</v>
       </c>
     </row>
     <row r="39">
@@ -1485,13 +1485,13 @@
         <v>1</v>
       </c>
       <c r="E39" t="n">
-        <v>798609.6514927745</v>
+        <v>796639.2884175777</v>
       </c>
       <c r="F39" t="n">
-        <v>20018.65149277449</v>
+        <v>18048.28841757774</v>
       </c>
       <c r="G39" t="n">
-        <v>2.571138311741914</v>
+        <v>2.318070516815343</v>
       </c>
     </row>
   </sheetData>
@@ -1538,7 +1538,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-03-19</t>
+          <t>2026-03-20</t>
         </is>
       </c>
       <c r="B2" t="n">
@@ -1549,11 +1549,11 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2026-03-19T21:54:06</t>
+          <t>2026-03-20T03:06:55</t>
         </is>
       </c>
       <c r="E2" t="n">
-        <v>1499.680053710938</v>
+        <v>1495.97998046875</v>
       </c>
     </row>
   </sheetData>
@@ -1567,7 +1567,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I115"/>
+  <dimension ref="A1:I153"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5832,6 +5832,1412 @@
       <c r="I115" t="inlineStr">
         <is>
           <t>2026-03-19T21:54:06</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>2026-03-20</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>페트로브라스 (ADR)</t>
+        </is>
+      </c>
+      <c r="C116" t="n">
+        <v>480</v>
+      </c>
+      <c r="D116" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E116" t="n">
+        <v>1</v>
+      </c>
+      <c r="F116" t="n">
+        <v>14203432.81962231</v>
+      </c>
+      <c r="G116" t="n">
+        <v>2096883.819622312</v>
+      </c>
+      <c r="H116" t="n">
+        <v>17.32024394088119</v>
+      </c>
+      <c r="I116" t="inlineStr">
+        <is>
+          <t>2026-03-20T03:06:55</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>2026-03-20</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>AGNC 인베스트먼트</t>
+        </is>
+      </c>
+      <c r="C117" t="n">
+        <v>700</v>
+      </c>
+      <c r="D117" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E117" t="n">
+        <v>1</v>
+      </c>
+      <c r="F117" t="n">
+        <v>10775543.75936943</v>
+      </c>
+      <c r="G117" t="n">
+        <v>-56471.2406305708</v>
+      </c>
+      <c r="H117" t="n">
+        <v>-0.5213364330696624</v>
+      </c>
+      <c r="I117" t="inlineStr">
+        <is>
+          <t>2026-03-20T03:06:55</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>2026-03-20</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>대한조선</t>
+        </is>
+      </c>
+      <c r="C118" t="n">
+        <v>100</v>
+      </c>
+      <c r="D118" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E118" t="n">
+        <v>1</v>
+      </c>
+      <c r="F118" t="n">
+        <v>9240000</v>
+      </c>
+      <c r="G118" t="n">
+        <v>2027000</v>
+      </c>
+      <c r="H118" t="n">
+        <v>28.10203798696798</v>
+      </c>
+      <c r="I118" t="inlineStr">
+        <is>
+          <t>2026-03-20T03:06:55</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>2026-03-20</t>
+        </is>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>프론트라인</t>
+        </is>
+      </c>
+      <c r="C119" t="n">
+        <v>175</v>
+      </c>
+      <c r="D119" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E119" t="n">
+        <v>1</v>
+      </c>
+      <c r="F119" t="n">
+        <v>8607869.087246014</v>
+      </c>
+      <c r="G119" t="n">
+        <v>4178005.087246014</v>
+      </c>
+      <c r="H119" t="n">
+        <v>94.31452268615953</v>
+      </c>
+      <c r="I119" t="inlineStr">
+        <is>
+          <t>2026-03-20T03:06:55</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>2026-03-20</t>
+        </is>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>시드릴</t>
+        </is>
+      </c>
+      <c r="C120" t="n">
+        <v>123</v>
+      </c>
+      <c r="D120" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E120" t="n">
+        <v>1</v>
+      </c>
+      <c r="F120" t="n">
+        <v>8260008.470450722</v>
+      </c>
+      <c r="G120" t="n">
+        <v>1809657.470450722</v>
+      </c>
+      <c r="H120" t="n">
+        <v>28.05517824457494</v>
+      </c>
+      <c r="I120" t="inlineStr">
+        <is>
+          <t>2026-03-20T03:06:55</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>2026-03-20</t>
+        </is>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>세아제강</t>
+        </is>
+      </c>
+      <c r="C121" t="n">
+        <v>50</v>
+      </c>
+      <c r="D121" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E121" t="n">
+        <v>1</v>
+      </c>
+      <c r="F121" t="n">
+        <v>7315000</v>
+      </c>
+      <c r="G121" t="n">
+        <v>1005000</v>
+      </c>
+      <c r="H121" t="n">
+        <v>15.92709984152139</v>
+      </c>
+      <c r="I121" t="inlineStr">
+        <is>
+          <t>2026-03-20T03:06:55</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>2026-03-20</t>
+        </is>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>트랜스오션</t>
+        </is>
+      </c>
+      <c r="C122" t="n">
+        <v>750</v>
+      </c>
+      <c r="D122" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E122" t="n">
+        <v>1</v>
+      </c>
+      <c r="F122" t="n">
+        <v>7248023.048171424</v>
+      </c>
+      <c r="G122" t="n">
+        <v>3120789.048171425</v>
+      </c>
+      <c r="H122" t="n">
+        <v>75.61454107451686</v>
+      </c>
+      <c r="I122" t="inlineStr">
+        <is>
+          <t>2026-03-20T03:06:55</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>2026-03-20</t>
+        </is>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>노블</t>
+        </is>
+      </c>
+      <c r="C123" t="n">
+        <v>99</v>
+      </c>
+      <c r="D123" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E123" t="n">
+        <v>1</v>
+      </c>
+      <c r="F123" t="n">
+        <v>7071871.362670898</v>
+      </c>
+      <c r="G123" t="n">
+        <v>3164663.362670898</v>
+      </c>
+      <c r="H123" t="n">
+        <v>80.99551809555309</v>
+      </c>
+      <c r="I123" t="inlineStr">
+        <is>
+          <t>2026-03-20T03:06:55</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>2026-03-20</t>
+        </is>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>센트러스 에너지</t>
+        </is>
+      </c>
+      <c r="C124" t="n">
+        <v>21</v>
+      </c>
+      <c r="D124" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E124" t="n">
+        <v>1</v>
+      </c>
+      <c r="F124" t="n">
+        <v>6443021.103033766</v>
+      </c>
+      <c r="G124" t="n">
+        <v>211802.1030337671</v>
+      </c>
+      <c r="H124" t="n">
+        <v>3.399047650768928</v>
+      </c>
+      <c r="I124" t="inlineStr">
+        <is>
+          <t>2026-03-20T03:06:55</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>2026-03-20</t>
+        </is>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>타이드워터</t>
+        </is>
+      </c>
+      <c r="C125" t="n">
+        <v>48</v>
+      </c>
+      <c r="D125" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E125" t="n">
+        <v>1</v>
+      </c>
+      <c r="F125" t="n">
+        <v>5333826.773907423</v>
+      </c>
+      <c r="G125" t="n">
+        <v>1609281.773907423</v>
+      </c>
+      <c r="H125" t="n">
+        <v>43.20747296401098</v>
+      </c>
+      <c r="I125" t="inlineStr">
+        <is>
+          <t>2026-03-20T03:06:55</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>2026-03-20</t>
+        </is>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>노브</t>
+        </is>
+      </c>
+      <c r="C126" t="n">
+        <v>185</v>
+      </c>
+      <c r="D126" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E126" t="n">
+        <v>1</v>
+      </c>
+      <c r="F126" t="n">
+        <v>5144899.592058761</v>
+      </c>
+      <c r="G126" t="n">
+        <v>1834891.592058761</v>
+      </c>
+      <c r="H126" t="n">
+        <v>55.43465731982403</v>
+      </c>
+      <c r="I126" t="inlineStr">
+        <is>
+          <t>2026-03-20T03:06:55</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>2026-03-20</t>
+        </is>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>DL이앤씨</t>
+        </is>
+      </c>
+      <c r="C127" t="n">
+        <v>80</v>
+      </c>
+      <c r="D127" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E127" t="n">
+        <v>1</v>
+      </c>
+      <c r="F127" t="n">
+        <v>5112000</v>
+      </c>
+      <c r="G127" t="n">
+        <v>1701000</v>
+      </c>
+      <c r="H127" t="n">
+        <v>49.86807387862797</v>
+      </c>
+      <c r="I127" t="inlineStr">
+        <is>
+          <t>2026-03-20T03:06:55</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>2026-03-20</t>
+        </is>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>TIME 코리아밸류업액티브</t>
+        </is>
+      </c>
+      <c r="C128" t="n">
+        <v>201</v>
+      </c>
+      <c r="D128" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E128" t="n">
+        <v>1</v>
+      </c>
+      <c r="F128" t="n">
+        <v>4787820</v>
+      </c>
+      <c r="G128" t="n">
+        <v>64023</v>
+      </c>
+      <c r="H128" t="n">
+        <v>1.355329198100596</v>
+      </c>
+      <c r="I128" t="inlineStr">
+        <is>
+          <t>2026-03-20T03:06:55</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>2026-03-20</t>
+        </is>
+      </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>오케아니스 에코 탱커스</t>
+        </is>
+      </c>
+      <c r="C129" t="n">
+        <v>65</v>
+      </c>
+      <c r="D129" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E129" t="n">
+        <v>1</v>
+      </c>
+      <c r="F129" t="n">
+        <v>4584804.793516081</v>
+      </c>
+      <c r="G129" t="n">
+        <v>2328444.793516081</v>
+      </c>
+      <c r="H129" t="n">
+        <v>103.1947381409031</v>
+      </c>
+      <c r="I129" t="inlineStr">
+        <is>
+          <t>2026-03-20T03:06:55</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>2026-03-20</t>
+        </is>
+      </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>삼성화재</t>
+        </is>
+      </c>
+      <c r="C130" t="n">
+        <v>9</v>
+      </c>
+      <c r="D130" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E130" t="n">
+        <v>1</v>
+      </c>
+      <c r="F130" t="n">
+        <v>4293000</v>
+      </c>
+      <c r="G130" t="n">
+        <v>-338000</v>
+      </c>
+      <c r="H130" t="n">
+        <v>-7.298639602677608</v>
+      </c>
+      <c r="I130" t="inlineStr">
+        <is>
+          <t>2026-03-20T03:06:55</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>2026-03-20</t>
+        </is>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>동원개발</t>
+        </is>
+      </c>
+      <c r="C131" t="n">
+        <v>1360</v>
+      </c>
+      <c r="D131" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E131" t="n">
+        <v>1</v>
+      </c>
+      <c r="F131" t="n">
+        <v>4127600</v>
+      </c>
+      <c r="G131" t="n">
+        <v>390200</v>
+      </c>
+      <c r="H131" t="n">
+        <v>10.44041312142131</v>
+      </c>
+      <c r="I131" t="inlineStr">
+        <is>
+          <t>2026-03-20T03:06:55</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>2026-03-20</t>
+        </is>
+      </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>HD건설기계</t>
+        </is>
+      </c>
+      <c r="C132" t="n">
+        <v>31</v>
+      </c>
+      <c r="D132" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E132" t="n">
+        <v>1</v>
+      </c>
+      <c r="F132" t="n">
+        <v>4101300</v>
+      </c>
+      <c r="G132" t="n">
+        <v>66204</v>
+      </c>
+      <c r="H132" t="n">
+        <v>1.640704459076066</v>
+      </c>
+      <c r="I132" t="inlineStr">
+        <is>
+          <t>2026-03-20T03:06:55</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>2026-03-20</t>
+        </is>
+      </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>차코스 에너지 내비게이션</t>
+        </is>
+      </c>
+      <c r="C133" t="n">
+        <v>75</v>
+      </c>
+      <c r="D133" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E133" t="n">
+        <v>1</v>
+      </c>
+      <c r="F133" t="n">
+        <v>4071683.614561614</v>
+      </c>
+      <c r="G133" t="n">
+        <v>247035.6145616136</v>
+      </c>
+      <c r="H133" t="n">
+        <v>6.459041840232452</v>
+      </c>
+      <c r="I133" t="inlineStr">
+        <is>
+          <t>2026-03-20T03:06:55</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>2026-03-20</t>
+        </is>
+      </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>피바디 에너지</t>
+        </is>
+      </c>
+      <c r="C134" t="n">
+        <v>65</v>
+      </c>
+      <c r="D134" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E134" t="n">
+        <v>1</v>
+      </c>
+      <c r="F134" t="n">
+        <v>3641589.341643294</v>
+      </c>
+      <c r="G134" t="n">
+        <v>2170817.341643294</v>
+      </c>
+      <c r="H134" t="n">
+        <v>147.5971354936927</v>
+      </c>
+      <c r="I134" t="inlineStr">
+        <is>
+          <t>2026-03-20T03:06:55</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>2026-03-20</t>
+        </is>
+      </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>더치 브로스</t>
+        </is>
+      </c>
+      <c r="C135" t="n">
+        <v>39</v>
+      </c>
+      <c r="D135" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E135" t="n">
+        <v>1</v>
+      </c>
+      <c r="F135" t="n">
+        <v>2971420.173610602</v>
+      </c>
+      <c r="G135" t="n">
+        <v>-219223.8263893984</v>
+      </c>
+      <c r="H135" t="n">
+        <v>-6.870833173158723</v>
+      </c>
+      <c r="I135" t="inlineStr">
+        <is>
+          <t>2026-03-20T03:06:55</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="inlineStr">
+        <is>
+          <t>2026-03-20</t>
+        </is>
+      </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>휴스틸</t>
+        </is>
+      </c>
+      <c r="C136" t="n">
+        <v>500</v>
+      </c>
+      <c r="D136" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E136" t="n">
+        <v>1</v>
+      </c>
+      <c r="F136" t="n">
+        <v>2735000</v>
+      </c>
+      <c r="G136" t="n">
+        <v>456390</v>
+      </c>
+      <c r="H136" t="n">
+        <v>20.02931611815976</v>
+      </c>
+      <c r="I136" t="inlineStr">
+        <is>
+          <t>2026-03-20T03:06:55</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="inlineStr">
+        <is>
+          <t>2026-03-20</t>
+        </is>
+      </c>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>현대제철</t>
+        </is>
+      </c>
+      <c r="C137" t="n">
+        <v>70</v>
+      </c>
+      <c r="D137" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E137" t="n">
+        <v>1</v>
+      </c>
+      <c r="F137" t="n">
+        <v>2593500</v>
+      </c>
+      <c r="G137" t="n">
+        <v>-214000</v>
+      </c>
+      <c r="H137" t="n">
+        <v>-7.622439893143366</v>
+      </c>
+      <c r="I137" t="inlineStr">
+        <is>
+          <t>2026-03-20T03:06:55</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="inlineStr">
+        <is>
+          <t>2026-03-20</t>
+        </is>
+      </c>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>KoAct 코스닥액티브</t>
+        </is>
+      </c>
+      <c r="C138" t="n">
+        <v>200</v>
+      </c>
+      <c r="D138" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E138" t="n">
+        <v>1</v>
+      </c>
+      <c r="F138" t="n">
+        <v>2583000</v>
+      </c>
+      <c r="G138" t="n">
+        <v>-119000</v>
+      </c>
+      <c r="H138" t="n">
+        <v>-4.404145077720207</v>
+      </c>
+      <c r="I138" t="inlineStr">
+        <is>
+          <t>2026-03-20T03:06:55</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="inlineStr">
+        <is>
+          <t>2026-03-20</t>
+        </is>
+      </c>
+      <c r="B139" t="inlineStr">
+        <is>
+          <t>넥스틸</t>
+        </is>
+      </c>
+      <c r="C139" t="n">
+        <v>200</v>
+      </c>
+      <c r="D139" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E139" t="n">
+        <v>1</v>
+      </c>
+      <c r="F139" t="n">
+        <v>2486000</v>
+      </c>
+      <c r="G139" t="n">
+        <v>475000</v>
+      </c>
+      <c r="H139" t="n">
+        <v>23.62008950770761</v>
+      </c>
+      <c r="I139" t="inlineStr">
+        <is>
+          <t>2026-03-20T03:06:55</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="inlineStr">
+        <is>
+          <t>2026-03-20</t>
+        </is>
+      </c>
+      <c r="B140" t="inlineStr">
+        <is>
+          <t>대신증권</t>
+        </is>
+      </c>
+      <c r="C140" t="n">
+        <v>55</v>
+      </c>
+      <c r="D140" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E140" t="n">
+        <v>1</v>
+      </c>
+      <c r="F140" t="n">
+        <v>2216500</v>
+      </c>
+      <c r="G140" t="n">
+        <v>506999</v>
+      </c>
+      <c r="H140" t="n">
+        <v>29.65771883140168</v>
+      </c>
+      <c r="I140" t="inlineStr">
+        <is>
+          <t>2026-03-20T03:06:55</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="inlineStr">
+        <is>
+          <t>2026-03-20</t>
+        </is>
+      </c>
+      <c r="B141" t="inlineStr">
+        <is>
+          <t>발레로 에너지</t>
+        </is>
+      </c>
+      <c r="C141" t="n">
+        <v>6</v>
+      </c>
+      <c r="D141" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E141" t="n">
+        <v>1</v>
+      </c>
+      <c r="F141" t="n">
+        <v>2172791.30897373</v>
+      </c>
+      <c r="G141" t="n">
+        <v>108801.3089737301</v>
+      </c>
+      <c r="H141" t="n">
+        <v>5.271406788488806</v>
+      </c>
+      <c r="I141" t="inlineStr">
+        <is>
+          <t>2026-03-20T03:06:55</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="inlineStr">
+        <is>
+          <t>2026-03-20</t>
+        </is>
+      </c>
+      <c r="B142" t="inlineStr">
+        <is>
+          <t>미창석유</t>
+        </is>
+      </c>
+      <c r="C142" t="n">
+        <v>18</v>
+      </c>
+      <c r="D142" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E142" t="n">
+        <v>1</v>
+      </c>
+      <c r="F142" t="n">
+        <v>2071800</v>
+      </c>
+      <c r="G142" t="n">
+        <v>-320400</v>
+      </c>
+      <c r="H142" t="n">
+        <v>-13.39352896914974</v>
+      </c>
+      <c r="I142" t="inlineStr">
+        <is>
+          <t>2026-03-20T03:06:55</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="inlineStr">
+        <is>
+          <t>2026-03-20</t>
+        </is>
+      </c>
+      <c r="B143" t="inlineStr">
+        <is>
+          <t>대창단조</t>
+        </is>
+      </c>
+      <c r="C143" t="n">
+        <v>300</v>
+      </c>
+      <c r="D143" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E143" t="n">
+        <v>1</v>
+      </c>
+      <c r="F143" t="n">
+        <v>1995000</v>
+      </c>
+      <c r="G143" t="n">
+        <v>-63000</v>
+      </c>
+      <c r="H143" t="n">
+        <v>-3.061224489795918</v>
+      </c>
+      <c r="I143" t="inlineStr">
+        <is>
+          <t>2026-03-20T03:06:55</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" t="inlineStr">
+        <is>
+          <t>2026-03-20</t>
+        </is>
+      </c>
+      <c r="B144" t="inlineStr">
+        <is>
+          <t>동방</t>
+        </is>
+      </c>
+      <c r="C144" t="n">
+        <v>681</v>
+      </c>
+      <c r="D144" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E144" t="n">
+        <v>1</v>
+      </c>
+      <c r="F144" t="n">
+        <v>1961280</v>
+      </c>
+      <c r="G144" t="n">
+        <v>-10221</v>
+      </c>
+      <c r="H144" t="n">
+        <v>-0.5184374747971215</v>
+      </c>
+      <c r="I144" t="inlineStr">
+        <is>
+          <t>2026-03-20T03:06:55</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="inlineStr">
+        <is>
+          <t>2026-03-20</t>
+        </is>
+      </c>
+      <c r="B145" t="inlineStr">
+        <is>
+          <t>하나금융지주</t>
+        </is>
+      </c>
+      <c r="C145" t="n">
+        <v>15</v>
+      </c>
+      <c r="D145" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E145" t="n">
+        <v>1</v>
+      </c>
+      <c r="F145" t="n">
+        <v>1713000</v>
+      </c>
+      <c r="G145" t="n">
+        <v>30500</v>
+      </c>
+      <c r="H145" t="n">
+        <v>1.812778603268945</v>
+      </c>
+      <c r="I145" t="inlineStr">
+        <is>
+          <t>2026-03-20T03:06:55</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" t="inlineStr">
+        <is>
+          <t>2026-03-20</t>
+        </is>
+      </c>
+      <c r="B146" t="inlineStr">
+        <is>
+          <t>스타 벌크 캐리어스</t>
+        </is>
+      </c>
+      <c r="C146" t="n">
+        <v>50</v>
+      </c>
+      <c r="D146" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E146" t="n">
+        <v>1</v>
+      </c>
+      <c r="F146" t="n">
+        <v>1700181.21356247</v>
+      </c>
+      <c r="G146" t="n">
+        <v>385828.2135624706</v>
+      </c>
+      <c r="H146" t="n">
+        <v>29.35499166224529</v>
+      </c>
+      <c r="I146" t="inlineStr">
+        <is>
+          <t>2026-03-20T03:06:55</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" t="inlineStr">
+        <is>
+          <t>2026-03-20</t>
+        </is>
+      </c>
+      <c r="B147" t="inlineStr">
+        <is>
+          <t>유나이티드헬스 그룹</t>
+        </is>
+      </c>
+      <c r="C147" t="n">
+        <v>4</v>
+      </c>
+      <c r="D147" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E147" t="n">
+        <v>1</v>
+      </c>
+      <c r="F147" t="n">
+        <v>1678130.517499804</v>
+      </c>
+      <c r="G147" t="n">
+        <v>-16325.48250019504</v>
+      </c>
+      <c r="H147" t="n">
+        <v>-0.9634645278599764</v>
+      </c>
+      <c r="I147" t="inlineStr">
+        <is>
+          <t>2026-03-20T03:06:55</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" t="inlineStr">
+        <is>
+          <t>2026-03-20</t>
+        </is>
+      </c>
+      <c r="B148" t="inlineStr">
+        <is>
+          <t>케이씨</t>
+        </is>
+      </c>
+      <c r="C148" t="n">
+        <v>50</v>
+      </c>
+      <c r="D148" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E148" t="n">
+        <v>1</v>
+      </c>
+      <c r="F148" t="n">
+        <v>1647500</v>
+      </c>
+      <c r="G148" t="n">
+        <v>-2000.000000000698</v>
+      </c>
+      <c r="H148" t="n">
+        <v>-0.1212488632919489</v>
+      </c>
+      <c r="I148" t="inlineStr">
+        <is>
+          <t>2026-03-20T03:06:55</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="inlineStr">
+        <is>
+          <t>2026-03-20</t>
+        </is>
+      </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>삼성생명</t>
+        </is>
+      </c>
+      <c r="C149" t="n">
+        <v>4</v>
+      </c>
+      <c r="D149" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E149" t="n">
+        <v>1</v>
+      </c>
+      <c r="F149" t="n">
+        <v>900000</v>
+      </c>
+      <c r="G149" t="n">
+        <v>67000</v>
+      </c>
+      <c r="H149" t="n">
+        <v>8.043217286914766</v>
+      </c>
+      <c r="I149" t="inlineStr">
+        <is>
+          <t>2026-03-20T03:06:55</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="inlineStr">
+        <is>
+          <t>2026-03-20</t>
+        </is>
+      </c>
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>비에이치아이</t>
+        </is>
+      </c>
+      <c r="C150" t="n">
+        <v>8</v>
+      </c>
+      <c r="D150" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E150" t="n">
+        <v>1</v>
+      </c>
+      <c r="F150" t="n">
+        <v>887200</v>
+      </c>
+      <c r="G150" t="n">
+        <v>222085</v>
+      </c>
+      <c r="H150" t="n">
+        <v>33.39046631033731</v>
+      </c>
+      <c r="I150" t="inlineStr">
+        <is>
+          <t>2026-03-20T03:06:55</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="inlineStr">
+        <is>
+          <t>2026-03-20</t>
+        </is>
+      </c>
+      <c r="B151" t="inlineStr">
+        <is>
+          <t>클리블랜드 클리프스</t>
+        </is>
+      </c>
+      <c r="C151" t="n">
+        <v>70</v>
+      </c>
+      <c r="D151" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E151" t="n">
+        <v>1</v>
+      </c>
+      <c r="F151" t="n">
+        <v>856598.1687739864</v>
+      </c>
+      <c r="G151" t="n">
+        <v>-159456.8312260136</v>
+      </c>
+      <c r="H151" t="n">
+        <v>-15.69372044092235</v>
+      </c>
+      <c r="I151" t="inlineStr">
+        <is>
+          <t>2026-03-20T03:06:55</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="inlineStr">
+        <is>
+          <t>2026-03-20</t>
+        </is>
+      </c>
+      <c r="B152" t="inlineStr">
+        <is>
+          <t>하프니아</t>
+        </is>
+      </c>
+      <c r="C152" t="n">
+        <v>80</v>
+      </c>
+      <c r="D152" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E152" t="n">
+        <v>1</v>
+      </c>
+      <c r="F152" t="n">
+        <v>853306.9945554808</v>
+      </c>
+      <c r="G152" t="n">
+        <v>227575.9945554808</v>
+      </c>
+      <c r="H152" t="n">
+        <v>36.36962121989813</v>
+      </c>
+      <c r="I152" t="inlineStr">
+        <is>
+          <t>2026-03-20T03:06:55</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" t="inlineStr">
+        <is>
+          <t>2026-03-20</t>
+        </is>
+      </c>
+      <c r="B153" t="inlineStr">
+        <is>
+          <t>텍사스 퍼시픽 랜드</t>
+        </is>
+      </c>
+      <c r="C153" t="n">
+        <v>1</v>
+      </c>
+      <c r="D153" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E153" t="n">
+        <v>1</v>
+      </c>
+      <c r="F153" t="n">
+        <v>796639.2884175777</v>
+      </c>
+      <c r="G153" t="n">
+        <v>18048.28841757774</v>
+      </c>
+      <c r="H153" t="n">
+        <v>2.318070516815343</v>
+      </c>
+      <c r="I153" t="inlineStr">
+        <is>
+          <t>2026-03-20T03:06:55</t>
         </is>
       </c>
     </row>
@@ -5846,7 +7252,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E4"/>
+  <dimension ref="A1:E5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5945,6 +7351,29 @@
         </is>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2026-03-20</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>31505056</v>
+      </c>
+      <c r="C5" t="n">
+        <v>6016.63</v>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>2026-03-20T03:06:55</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>2026-03-20T03:06:55</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
auto: portfolio snapshot 2026-03-20 (2026-03-20T03:09:27)
</commit_message>
<xml_diff>
--- a/portfolio_auto.xlsx
+++ b/portfolio_auto.xlsx
@@ -540,13 +540,13 @@
         <v>1</v>
       </c>
       <c r="E4" t="n">
-        <v>9240000</v>
+        <v>9220000</v>
       </c>
       <c r="F4" t="n">
-        <v>2027000</v>
+        <v>2007000</v>
       </c>
       <c r="G4" t="n">
-        <v>28.10203798696798</v>
+        <v>27.82476084846805</v>
       </c>
     </row>
     <row r="5">
@@ -648,13 +648,13 @@
         <v>1</v>
       </c>
       <c r="E8" t="n">
-        <v>7315000</v>
+        <v>7325000</v>
       </c>
       <c r="F8" t="n">
-        <v>1005000</v>
+        <v>1015000</v>
       </c>
       <c r="G8" t="n">
-        <v>15.92709984152139</v>
+        <v>16.08557844690967</v>
       </c>
     </row>
     <row r="9">
@@ -864,13 +864,13 @@
         <v>1</v>
       </c>
       <c r="E16" t="n">
-        <v>5112000</v>
+        <v>5096000</v>
       </c>
       <c r="F16" t="n">
-        <v>1701000</v>
+        <v>1685000</v>
       </c>
       <c r="G16" t="n">
-        <v>49.86807387862797</v>
+        <v>49.39900322486074</v>
       </c>
     </row>
     <row r="17">
@@ -891,13 +891,13 @@
         <v>1</v>
       </c>
       <c r="E17" t="n">
-        <v>4101300</v>
+        <v>4088900</v>
       </c>
       <c r="F17" t="n">
-        <v>66204</v>
+        <v>53804</v>
       </c>
       <c r="G17" t="n">
-        <v>1.640704459076066</v>
+        <v>1.333400741890651</v>
       </c>
     </row>
     <row r="18">
@@ -945,13 +945,13 @@
         <v>1</v>
       </c>
       <c r="E19" t="n">
-        <v>4127600</v>
+        <v>4134400</v>
       </c>
       <c r="F19" t="n">
-        <v>390200</v>
+        <v>397000</v>
       </c>
       <c r="G19" t="n">
-        <v>10.44041312142131</v>
+        <v>10.62235778883716</v>
       </c>
     </row>
     <row r="20">
@@ -1026,13 +1026,13 @@
         <v>1</v>
       </c>
       <c r="E22" t="n">
-        <v>2735000</v>
+        <v>2725000</v>
       </c>
       <c r="F22" t="n">
-        <v>456390</v>
+        <v>446390</v>
       </c>
       <c r="G22" t="n">
-        <v>20.02931611815976</v>
+        <v>19.59045207385204</v>
       </c>
     </row>
     <row r="23">
@@ -1053,13 +1053,13 @@
         <v>1</v>
       </c>
       <c r="E23" t="n">
-        <v>2583000</v>
+        <v>2582400</v>
       </c>
       <c r="F23" t="n">
-        <v>-119000</v>
+        <v>-119600</v>
       </c>
       <c r="G23" t="n">
-        <v>-4.404145077720207</v>
+        <v>-4.426350851221318</v>
       </c>
     </row>
     <row r="24">
@@ -1080,13 +1080,13 @@
         <v>1</v>
       </c>
       <c r="E24" t="n">
-        <v>2593500</v>
+        <v>2590000</v>
       </c>
       <c r="F24" t="n">
-        <v>-214000</v>
+        <v>-217500</v>
       </c>
       <c r="G24" t="n">
-        <v>-7.622439893143366</v>
+        <v>-7.747105966162065</v>
       </c>
     </row>
     <row r="25">
@@ -1107,13 +1107,13 @@
         <v>1</v>
       </c>
       <c r="E25" t="n">
-        <v>2486000</v>
+        <v>2484000</v>
       </c>
       <c r="F25" t="n">
-        <v>475000</v>
+        <v>473000</v>
       </c>
       <c r="G25" t="n">
-        <v>23.62008950770761</v>
+        <v>23.5206364992541</v>
       </c>
     </row>
     <row r="26">
@@ -1134,13 +1134,13 @@
         <v>1</v>
       </c>
       <c r="E26" t="n">
-        <v>2216500</v>
+        <v>2213750</v>
       </c>
       <c r="F26" t="n">
-        <v>506999</v>
+        <v>504249</v>
       </c>
       <c r="G26" t="n">
-        <v>29.65771883140168</v>
+        <v>29.49685317528332</v>
       </c>
     </row>
     <row r="27">
@@ -1215,13 +1215,13 @@
         <v>1</v>
       </c>
       <c r="E29" t="n">
-        <v>1995000</v>
+        <v>1983000</v>
       </c>
       <c r="F29" t="n">
-        <v>-63000</v>
+        <v>-75000</v>
       </c>
       <c r="G29" t="n">
-        <v>-3.061224489795918</v>
+        <v>-3.644314868804665</v>
       </c>
     </row>
     <row r="30">
@@ -1242,13 +1242,13 @@
         <v>1</v>
       </c>
       <c r="E30" t="n">
-        <v>1961280</v>
+        <v>1971495</v>
       </c>
       <c r="F30" t="n">
-        <v>-10221</v>
+        <v>-6</v>
       </c>
       <c r="G30" t="n">
-        <v>-0.5184374747971215</v>
+        <v>-0.0003043366450232589</v>
       </c>
     </row>
     <row r="31">
@@ -1323,13 +1323,13 @@
         <v>1</v>
       </c>
       <c r="E33" t="n">
-        <v>1713000</v>
+        <v>1714500</v>
       </c>
       <c r="F33" t="n">
-        <v>30500</v>
+        <v>32000</v>
       </c>
       <c r="G33" t="n">
-        <v>1.812778603268945</v>
+        <v>1.901931649331352</v>
       </c>
     </row>
     <row r="34">
@@ -1350,13 +1350,13 @@
         <v>1</v>
       </c>
       <c r="E34" t="n">
-        <v>1647500</v>
+        <v>1650000</v>
       </c>
       <c r="F34" t="n">
-        <v>-2000.000000000698</v>
+        <v>499.9999999993015</v>
       </c>
       <c r="G34" t="n">
-        <v>-0.1212488632919489</v>
+        <v>0.0303122158229343</v>
       </c>
     </row>
     <row r="35">
@@ -1377,13 +1377,13 @@
         <v>1</v>
       </c>
       <c r="E35" t="n">
-        <v>900000</v>
+        <v>902000</v>
       </c>
       <c r="F35" t="n">
-        <v>67000</v>
+        <v>69000</v>
       </c>
       <c r="G35" t="n">
-        <v>8.043217286914766</v>
+        <v>8.283313325330131</v>
       </c>
     </row>
     <row r="36">
@@ -1431,13 +1431,13 @@
         <v>1</v>
       </c>
       <c r="E37" t="n">
-        <v>887200</v>
+        <v>886400</v>
       </c>
       <c r="F37" t="n">
-        <v>222085</v>
+        <v>221285</v>
       </c>
       <c r="G37" t="n">
-        <v>33.39046631033731</v>
+        <v>33.27018635875</v>
       </c>
     </row>
     <row r="38">
@@ -1549,7 +1549,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2026-03-20T03:06:55</t>
+          <t>2026-03-20T03:09:27</t>
         </is>
       </c>
       <c r="E2" t="n">
@@ -5868,7 +5868,7 @@
       </c>
       <c r="I116" t="inlineStr">
         <is>
-          <t>2026-03-20T03:06:55</t>
+          <t>2026-03-20T03:09:27</t>
         </is>
       </c>
     </row>
@@ -5905,7 +5905,7 @@
       </c>
       <c r="I117" t="inlineStr">
         <is>
-          <t>2026-03-20T03:06:55</t>
+          <t>2026-03-20T03:09:27</t>
         </is>
       </c>
     </row>
@@ -5932,17 +5932,17 @@
         <v>1</v>
       </c>
       <c r="F118" t="n">
-        <v>9240000</v>
+        <v>9220000</v>
       </c>
       <c r="G118" t="n">
-        <v>2027000</v>
+        <v>2007000</v>
       </c>
       <c r="H118" t="n">
-        <v>28.10203798696798</v>
+        <v>27.82476084846805</v>
       </c>
       <c r="I118" t="inlineStr">
         <is>
-          <t>2026-03-20T03:06:55</t>
+          <t>2026-03-20T03:09:27</t>
         </is>
       </c>
     </row>
@@ -5979,7 +5979,7 @@
       </c>
       <c r="I119" t="inlineStr">
         <is>
-          <t>2026-03-20T03:06:55</t>
+          <t>2026-03-20T03:09:27</t>
         </is>
       </c>
     </row>
@@ -6016,7 +6016,7 @@
       </c>
       <c r="I120" t="inlineStr">
         <is>
-          <t>2026-03-20T03:06:55</t>
+          <t>2026-03-20T03:09:27</t>
         </is>
       </c>
     </row>
@@ -6043,17 +6043,17 @@
         <v>1</v>
       </c>
       <c r="F121" t="n">
-        <v>7315000</v>
+        <v>7325000</v>
       </c>
       <c r="G121" t="n">
-        <v>1005000</v>
+        <v>1015000</v>
       </c>
       <c r="H121" t="n">
-        <v>15.92709984152139</v>
+        <v>16.08557844690967</v>
       </c>
       <c r="I121" t="inlineStr">
         <is>
-          <t>2026-03-20T03:06:55</t>
+          <t>2026-03-20T03:09:27</t>
         </is>
       </c>
     </row>
@@ -6090,7 +6090,7 @@
       </c>
       <c r="I122" t="inlineStr">
         <is>
-          <t>2026-03-20T03:06:55</t>
+          <t>2026-03-20T03:09:27</t>
         </is>
       </c>
     </row>
@@ -6127,7 +6127,7 @@
       </c>
       <c r="I123" t="inlineStr">
         <is>
-          <t>2026-03-20T03:06:55</t>
+          <t>2026-03-20T03:09:27</t>
         </is>
       </c>
     </row>
@@ -6164,7 +6164,7 @@
       </c>
       <c r="I124" t="inlineStr">
         <is>
-          <t>2026-03-20T03:06:55</t>
+          <t>2026-03-20T03:09:27</t>
         </is>
       </c>
     </row>
@@ -6201,7 +6201,7 @@
       </c>
       <c r="I125" t="inlineStr">
         <is>
-          <t>2026-03-20T03:06:55</t>
+          <t>2026-03-20T03:09:27</t>
         </is>
       </c>
     </row>
@@ -6238,7 +6238,7 @@
       </c>
       <c r="I126" t="inlineStr">
         <is>
-          <t>2026-03-20T03:06:55</t>
+          <t>2026-03-20T03:09:27</t>
         </is>
       </c>
     </row>
@@ -6265,17 +6265,17 @@
         <v>1</v>
       </c>
       <c r="F127" t="n">
-        <v>5112000</v>
+        <v>5096000</v>
       </c>
       <c r="G127" t="n">
-        <v>1701000</v>
+        <v>1685000</v>
       </c>
       <c r="H127" t="n">
-        <v>49.86807387862797</v>
+        <v>49.39900322486074</v>
       </c>
       <c r="I127" t="inlineStr">
         <is>
-          <t>2026-03-20T03:06:55</t>
+          <t>2026-03-20T03:09:27</t>
         </is>
       </c>
     </row>
@@ -6312,7 +6312,7 @@
       </c>
       <c r="I128" t="inlineStr">
         <is>
-          <t>2026-03-20T03:06:55</t>
+          <t>2026-03-20T03:09:27</t>
         </is>
       </c>
     </row>
@@ -6349,7 +6349,7 @@
       </c>
       <c r="I129" t="inlineStr">
         <is>
-          <t>2026-03-20T03:06:55</t>
+          <t>2026-03-20T03:09:27</t>
         </is>
       </c>
     </row>
@@ -6386,7 +6386,7 @@
       </c>
       <c r="I130" t="inlineStr">
         <is>
-          <t>2026-03-20T03:06:55</t>
+          <t>2026-03-20T03:09:27</t>
         </is>
       </c>
     </row>
@@ -6413,17 +6413,17 @@
         <v>1</v>
       </c>
       <c r="F131" t="n">
-        <v>4127600</v>
+        <v>4134400</v>
       </c>
       <c r="G131" t="n">
-        <v>390200</v>
+        <v>397000</v>
       </c>
       <c r="H131" t="n">
-        <v>10.44041312142131</v>
+        <v>10.62235778883716</v>
       </c>
       <c r="I131" t="inlineStr">
         <is>
-          <t>2026-03-20T03:06:55</t>
+          <t>2026-03-20T03:09:27</t>
         </is>
       </c>
     </row>
@@ -6450,17 +6450,17 @@
         <v>1</v>
       </c>
       <c r="F132" t="n">
-        <v>4101300</v>
+        <v>4088900</v>
       </c>
       <c r="G132" t="n">
-        <v>66204</v>
+        <v>53804</v>
       </c>
       <c r="H132" t="n">
-        <v>1.640704459076066</v>
+        <v>1.333400741890651</v>
       </c>
       <c r="I132" t="inlineStr">
         <is>
-          <t>2026-03-20T03:06:55</t>
+          <t>2026-03-20T03:09:27</t>
         </is>
       </c>
     </row>
@@ -6497,7 +6497,7 @@
       </c>
       <c r="I133" t="inlineStr">
         <is>
-          <t>2026-03-20T03:06:55</t>
+          <t>2026-03-20T03:09:27</t>
         </is>
       </c>
     </row>
@@ -6534,7 +6534,7 @@
       </c>
       <c r="I134" t="inlineStr">
         <is>
-          <t>2026-03-20T03:06:55</t>
+          <t>2026-03-20T03:09:27</t>
         </is>
       </c>
     </row>
@@ -6571,7 +6571,7 @@
       </c>
       <c r="I135" t="inlineStr">
         <is>
-          <t>2026-03-20T03:06:55</t>
+          <t>2026-03-20T03:09:27</t>
         </is>
       </c>
     </row>
@@ -6598,17 +6598,17 @@
         <v>1</v>
       </c>
       <c r="F136" t="n">
-        <v>2735000</v>
+        <v>2725000</v>
       </c>
       <c r="G136" t="n">
-        <v>456390</v>
+        <v>446390</v>
       </c>
       <c r="H136" t="n">
-        <v>20.02931611815976</v>
+        <v>19.59045207385204</v>
       </c>
       <c r="I136" t="inlineStr">
         <is>
-          <t>2026-03-20T03:06:55</t>
+          <t>2026-03-20T03:09:27</t>
         </is>
       </c>
     </row>
@@ -6635,17 +6635,17 @@
         <v>1</v>
       </c>
       <c r="F137" t="n">
-        <v>2593500</v>
+        <v>2590000</v>
       </c>
       <c r="G137" t="n">
-        <v>-214000</v>
+        <v>-217500</v>
       </c>
       <c r="H137" t="n">
-        <v>-7.622439893143366</v>
+        <v>-7.747105966162065</v>
       </c>
       <c r="I137" t="inlineStr">
         <is>
-          <t>2026-03-20T03:06:55</t>
+          <t>2026-03-20T03:09:27</t>
         </is>
       </c>
     </row>
@@ -6672,17 +6672,17 @@
         <v>1</v>
       </c>
       <c r="F138" t="n">
-        <v>2583000</v>
+        <v>2582400</v>
       </c>
       <c r="G138" t="n">
-        <v>-119000</v>
+        <v>-119600</v>
       </c>
       <c r="H138" t="n">
-        <v>-4.404145077720207</v>
+        <v>-4.426350851221318</v>
       </c>
       <c r="I138" t="inlineStr">
         <is>
-          <t>2026-03-20T03:06:55</t>
+          <t>2026-03-20T03:09:27</t>
         </is>
       </c>
     </row>
@@ -6709,17 +6709,17 @@
         <v>1</v>
       </c>
       <c r="F139" t="n">
-        <v>2486000</v>
+        <v>2484000</v>
       </c>
       <c r="G139" t="n">
-        <v>475000</v>
+        <v>473000</v>
       </c>
       <c r="H139" t="n">
-        <v>23.62008950770761</v>
+        <v>23.5206364992541</v>
       </c>
       <c r="I139" t="inlineStr">
         <is>
-          <t>2026-03-20T03:06:55</t>
+          <t>2026-03-20T03:09:27</t>
         </is>
       </c>
     </row>
@@ -6746,17 +6746,17 @@
         <v>1</v>
       </c>
       <c r="F140" t="n">
-        <v>2216500</v>
+        <v>2213750</v>
       </c>
       <c r="G140" t="n">
-        <v>506999</v>
+        <v>504249</v>
       </c>
       <c r="H140" t="n">
-        <v>29.65771883140168</v>
+        <v>29.49685317528332</v>
       </c>
       <c r="I140" t="inlineStr">
         <is>
-          <t>2026-03-20T03:06:55</t>
+          <t>2026-03-20T03:09:27</t>
         </is>
       </c>
     </row>
@@ -6793,7 +6793,7 @@
       </c>
       <c r="I141" t="inlineStr">
         <is>
-          <t>2026-03-20T03:06:55</t>
+          <t>2026-03-20T03:09:27</t>
         </is>
       </c>
     </row>
@@ -6830,7 +6830,7 @@
       </c>
       <c r="I142" t="inlineStr">
         <is>
-          <t>2026-03-20T03:06:55</t>
+          <t>2026-03-20T03:09:27</t>
         </is>
       </c>
     </row>
@@ -6857,17 +6857,17 @@
         <v>1</v>
       </c>
       <c r="F143" t="n">
-        <v>1995000</v>
+        <v>1983000</v>
       </c>
       <c r="G143" t="n">
-        <v>-63000</v>
+        <v>-75000</v>
       </c>
       <c r="H143" t="n">
-        <v>-3.061224489795918</v>
+        <v>-3.644314868804665</v>
       </c>
       <c r="I143" t="inlineStr">
         <is>
-          <t>2026-03-20T03:06:55</t>
+          <t>2026-03-20T03:09:27</t>
         </is>
       </c>
     </row>
@@ -6894,17 +6894,17 @@
         <v>1</v>
       </c>
       <c r="F144" t="n">
-        <v>1961280</v>
+        <v>1971495</v>
       </c>
       <c r="G144" t="n">
-        <v>-10221</v>
+        <v>-6</v>
       </c>
       <c r="H144" t="n">
-        <v>-0.5184374747971215</v>
+        <v>-0.0003043366450232589</v>
       </c>
       <c r="I144" t="inlineStr">
         <is>
-          <t>2026-03-20T03:06:55</t>
+          <t>2026-03-20T03:09:27</t>
         </is>
       </c>
     </row>
@@ -6931,17 +6931,17 @@
         <v>1</v>
       </c>
       <c r="F145" t="n">
-        <v>1713000</v>
+        <v>1714500</v>
       </c>
       <c r="G145" t="n">
-        <v>30500</v>
+        <v>32000</v>
       </c>
       <c r="H145" t="n">
-        <v>1.812778603268945</v>
+        <v>1.901931649331352</v>
       </c>
       <c r="I145" t="inlineStr">
         <is>
-          <t>2026-03-20T03:06:55</t>
+          <t>2026-03-20T03:09:27</t>
         </is>
       </c>
     </row>
@@ -6978,7 +6978,7 @@
       </c>
       <c r="I146" t="inlineStr">
         <is>
-          <t>2026-03-20T03:06:55</t>
+          <t>2026-03-20T03:09:27</t>
         </is>
       </c>
     </row>
@@ -7015,7 +7015,7 @@
       </c>
       <c r="I147" t="inlineStr">
         <is>
-          <t>2026-03-20T03:06:55</t>
+          <t>2026-03-20T03:09:27</t>
         </is>
       </c>
     </row>
@@ -7042,17 +7042,17 @@
         <v>1</v>
       </c>
       <c r="F148" t="n">
-        <v>1647500</v>
+        <v>1650000</v>
       </c>
       <c r="G148" t="n">
-        <v>-2000.000000000698</v>
+        <v>499.9999999993015</v>
       </c>
       <c r="H148" t="n">
-        <v>-0.1212488632919489</v>
+        <v>0.0303122158229343</v>
       </c>
       <c r="I148" t="inlineStr">
         <is>
-          <t>2026-03-20T03:06:55</t>
+          <t>2026-03-20T03:09:27</t>
         </is>
       </c>
     </row>
@@ -7079,17 +7079,17 @@
         <v>1</v>
       </c>
       <c r="F149" t="n">
-        <v>900000</v>
+        <v>902000</v>
       </c>
       <c r="G149" t="n">
-        <v>67000</v>
+        <v>69000</v>
       </c>
       <c r="H149" t="n">
-        <v>8.043217286914766</v>
+        <v>8.283313325330131</v>
       </c>
       <c r="I149" t="inlineStr">
         <is>
-          <t>2026-03-20T03:06:55</t>
+          <t>2026-03-20T03:09:27</t>
         </is>
       </c>
     </row>
@@ -7116,17 +7116,17 @@
         <v>1</v>
       </c>
       <c r="F150" t="n">
-        <v>887200</v>
+        <v>886400</v>
       </c>
       <c r="G150" t="n">
-        <v>222085</v>
+        <v>221285</v>
       </c>
       <c r="H150" t="n">
-        <v>33.39046631033731</v>
+        <v>33.27018635875</v>
       </c>
       <c r="I150" t="inlineStr">
         <is>
-          <t>2026-03-20T03:06:55</t>
+          <t>2026-03-20T03:09:27</t>
         </is>
       </c>
     </row>
@@ -7163,7 +7163,7 @@
       </c>
       <c r="I151" t="inlineStr">
         <is>
-          <t>2026-03-20T03:06:55</t>
+          <t>2026-03-20T03:09:27</t>
         </is>
       </c>
     </row>
@@ -7200,7 +7200,7 @@
       </c>
       <c r="I152" t="inlineStr">
         <is>
-          <t>2026-03-20T03:06:55</t>
+          <t>2026-03-20T03:09:27</t>
         </is>
       </c>
     </row>
@@ -7237,7 +7237,7 @@
       </c>
       <c r="I153" t="inlineStr">
         <is>
-          <t>2026-03-20T03:06:55</t>
+          <t>2026-03-20T03:09:27</t>
         </is>
       </c>
     </row>
@@ -7370,7 +7370,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>2026-03-20T03:06:55</t>
+          <t>2026-03-20T03:09:27</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: portfolio snapshot 2026-03-20 (2026-03-20T07:02:39)
</commit_message>
<xml_diff>
--- a/portfolio_auto.xlsx
+++ b/portfolio_auto.xlsx
@@ -540,13 +540,13 @@
         <v>1</v>
       </c>
       <c r="E4" t="n">
-        <v>9220000</v>
+        <v>9120000</v>
       </c>
       <c r="F4" t="n">
-        <v>2007000</v>
+        <v>1907000</v>
       </c>
       <c r="G4" t="n">
-        <v>27.82476084846805</v>
+        <v>26.43837515596839</v>
       </c>
     </row>
     <row r="5">
@@ -606,11 +606,11 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>트랜스오션</t>
+          <t>세아제강</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>750</v>
+        <v>50</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -621,23 +621,23 @@
         <v>1</v>
       </c>
       <c r="E7" t="n">
-        <v>7248023.048171424</v>
+        <v>7395000</v>
       </c>
       <c r="F7" t="n">
-        <v>3120789.048171425</v>
+        <v>1085000</v>
       </c>
       <c r="G7" t="n">
-        <v>75.61454107451686</v>
+        <v>17.19492868462758</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>세아제강</t>
+          <t>트랜스오션</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>50</v>
+        <v>750</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
@@ -648,13 +648,13 @@
         <v>1</v>
       </c>
       <c r="E8" t="n">
-        <v>7325000</v>
+        <v>7248023.048171424</v>
       </c>
       <c r="F8" t="n">
-        <v>1015000</v>
+        <v>3120789.048171425</v>
       </c>
       <c r="G8" t="n">
-        <v>16.08557844690967</v>
+        <v>75.61454107451686</v>
       </c>
     </row>
     <row r="9">
@@ -768,11 +768,11 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>TIME 코리아밸류업액티브</t>
+          <t>DL이앤씨</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>201</v>
+        <v>80</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
@@ -783,23 +783,23 @@
         <v>1</v>
       </c>
       <c r="E13" t="n">
-        <v>4787820</v>
+        <v>5392000</v>
       </c>
       <c r="F13" t="n">
-        <v>64023</v>
+        <v>1981000</v>
       </c>
       <c r="G13" t="n">
-        <v>1.355329198100596</v>
+        <v>58.07681031955438</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>오케아니스 에코 탱커스</t>
+          <t>TIME 코리아밸류업액티브</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>65</v>
+        <v>201</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
@@ -810,23 +810,23 @@
         <v>1</v>
       </c>
       <c r="E14" t="n">
-        <v>4584804.793516081</v>
+        <v>4797870</v>
       </c>
       <c r="F14" t="n">
-        <v>2328444.793516081</v>
+        <v>74073</v>
       </c>
       <c r="G14" t="n">
-        <v>103.1947381409031</v>
+        <v>1.568081778281328</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>삼성화재</t>
+          <t>오케아니스 에코 탱커스</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>9</v>
+        <v>65</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
@@ -837,23 +837,23 @@
         <v>1</v>
       </c>
       <c r="E15" t="n">
-        <v>4293000</v>
+        <v>4584804.793516081</v>
       </c>
       <c r="F15" t="n">
-        <v>-338000</v>
+        <v>2328444.793516081</v>
       </c>
       <c r="G15" t="n">
-        <v>-7.298639602677608</v>
+        <v>103.1947381409031</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>DL이앤씨</t>
+          <t>삼성화재</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>80</v>
+        <v>9</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
@@ -864,23 +864,23 @@
         <v>1</v>
       </c>
       <c r="E16" t="n">
-        <v>5096000</v>
+        <v>4270500</v>
       </c>
       <c r="F16" t="n">
-        <v>1685000</v>
+        <v>-360500</v>
       </c>
       <c r="G16" t="n">
-        <v>49.39900322486074</v>
+        <v>-7.784495789246384</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>HD건설기계</t>
+          <t>동원개발</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>31</v>
+        <v>1360</v>
       </c>
       <c r="C17" t="inlineStr">
         <is>
@@ -891,23 +891,23 @@
         <v>1</v>
       </c>
       <c r="E17" t="n">
-        <v>4088900</v>
+        <v>4202400</v>
       </c>
       <c r="F17" t="n">
-        <v>53804</v>
+        <v>465000</v>
       </c>
       <c r="G17" t="n">
-        <v>1.333400741890651</v>
+        <v>12.44180446299566</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>차코스 에너지 내비게이션</t>
+          <t>HD건설기계</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>75</v>
+        <v>31</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
@@ -918,23 +918,23 @@
         <v>1</v>
       </c>
       <c r="E18" t="n">
-        <v>4071683.614561614</v>
+        <v>4123000</v>
       </c>
       <c r="F18" t="n">
-        <v>247035.6145616136</v>
+        <v>87904</v>
       </c>
       <c r="G18" t="n">
-        <v>6.459041840232452</v>
+        <v>2.178485964150543</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>동원개발</t>
+          <t>차코스 에너지 내비게이션</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>1360</v>
+        <v>75</v>
       </c>
       <c r="C19" t="inlineStr">
         <is>
@@ -945,13 +945,13 @@
         <v>1</v>
       </c>
       <c r="E19" t="n">
-        <v>4134400</v>
+        <v>4071683.614561614</v>
       </c>
       <c r="F19" t="n">
-        <v>397000</v>
+        <v>247035.6145616136</v>
       </c>
       <c r="G19" t="n">
-        <v>10.62235778883716</v>
+        <v>6.459041840232452</v>
       </c>
     </row>
     <row r="20">
@@ -1026,23 +1026,23 @@
         <v>1</v>
       </c>
       <c r="E22" t="n">
-        <v>2725000</v>
+        <v>2750000</v>
       </c>
       <c r="F22" t="n">
-        <v>446390</v>
+        <v>471390</v>
       </c>
       <c r="G22" t="n">
-        <v>19.59045207385204</v>
+        <v>20.68761218462133</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>KoAct 코스닥액티브</t>
+          <t>현대제철</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>200</v>
+        <v>70</v>
       </c>
       <c r="C23" t="inlineStr">
         <is>
@@ -1053,23 +1053,23 @@
         <v>1</v>
       </c>
       <c r="E23" t="n">
-        <v>2582400</v>
+        <v>2621500</v>
       </c>
       <c r="F23" t="n">
-        <v>-119600</v>
+        <v>-186000</v>
       </c>
       <c r="G23" t="n">
-        <v>-4.426350851221318</v>
+        <v>-6.625111308993767</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>현대제철</t>
+          <t>KoAct 코스닥액티브</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>70</v>
+        <v>200</v>
       </c>
       <c r="C24" t="inlineStr">
         <is>
@@ -1080,13 +1080,13 @@
         <v>1</v>
       </c>
       <c r="E24" t="n">
-        <v>2590000</v>
+        <v>2582000</v>
       </c>
       <c r="F24" t="n">
-        <v>-217500</v>
+        <v>-120000</v>
       </c>
       <c r="G24" t="n">
-        <v>-7.747105966162065</v>
+        <v>-4.441154700222058</v>
       </c>
     </row>
     <row r="25">
@@ -1107,13 +1107,13 @@
         <v>1</v>
       </c>
       <c r="E25" t="n">
-        <v>2484000</v>
+        <v>2514000</v>
       </c>
       <c r="F25" t="n">
-        <v>473000</v>
+        <v>503000</v>
       </c>
       <c r="G25" t="n">
-        <v>23.5206364992541</v>
+        <v>25.01243162605669</v>
       </c>
     </row>
     <row r="26">
@@ -1134,13 +1134,13 @@
         <v>1</v>
       </c>
       <c r="E26" t="n">
-        <v>2213750</v>
+        <v>2219250</v>
       </c>
       <c r="F26" t="n">
-        <v>504249</v>
+        <v>509749</v>
       </c>
       <c r="G26" t="n">
-        <v>29.49685317528332</v>
+        <v>29.81858448752005</v>
       </c>
     </row>
     <row r="27">
@@ -1188,13 +1188,13 @@
         <v>1</v>
       </c>
       <c r="E28" t="n">
-        <v>2071800</v>
+        <v>2097000</v>
       </c>
       <c r="F28" t="n">
-        <v>-320400</v>
+        <v>-295200</v>
       </c>
       <c r="G28" t="n">
-        <v>-13.39352896914974</v>
+        <v>-12.34010534236268</v>
       </c>
     </row>
     <row r="29">
@@ -1215,13 +1215,13 @@
         <v>1</v>
       </c>
       <c r="E29" t="n">
-        <v>1983000</v>
+        <v>2004000</v>
       </c>
       <c r="F29" t="n">
-        <v>-75000</v>
+        <v>-54000</v>
       </c>
       <c r="G29" t="n">
-        <v>-3.644314868804665</v>
+        <v>-2.623906705539359</v>
       </c>
     </row>
     <row r="30">
@@ -1242,23 +1242,23 @@
         <v>1</v>
       </c>
       <c r="E30" t="n">
-        <v>1971495</v>
+        <v>1995330</v>
       </c>
       <c r="F30" t="n">
-        <v>-6</v>
+        <v>23829</v>
       </c>
       <c r="G30" t="n">
-        <v>-0.0003043366450232589</v>
+        <v>1.208672985709873</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>스타 벌크 캐리어스</t>
+          <t>하나금융지주</t>
         </is>
       </c>
       <c r="B31" t="n">
-        <v>50</v>
+        <v>15</v>
       </c>
       <c r="C31" t="inlineStr">
         <is>
@@ -1269,23 +1269,23 @@
         <v>1</v>
       </c>
       <c r="E31" t="n">
-        <v>1700181.21356247</v>
+        <v>1698000</v>
       </c>
       <c r="F31" t="n">
-        <v>385828.2135624706</v>
+        <v>15500</v>
       </c>
       <c r="G31" t="n">
-        <v>29.35499166224529</v>
+        <v>0.9212481426448738</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>유나이티드헬스 그룹</t>
+          <t>스타 벌크 캐리어스</t>
         </is>
       </c>
       <c r="B32" t="n">
-        <v>4</v>
+        <v>50</v>
       </c>
       <c r="C32" t="inlineStr">
         <is>
@@ -1296,23 +1296,23 @@
         <v>1</v>
       </c>
       <c r="E32" t="n">
-        <v>1678130.517499804</v>
+        <v>1700181.21356247</v>
       </c>
       <c r="F32" t="n">
-        <v>-16325.48250019504</v>
+        <v>385828.2135624706</v>
       </c>
       <c r="G32" t="n">
-        <v>-0.9634645278599764</v>
+        <v>29.35499166224529</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>하나금융지주</t>
+          <t>유나이티드헬스 그룹</t>
         </is>
       </c>
       <c r="B33" t="n">
-        <v>15</v>
+        <v>4</v>
       </c>
       <c r="C33" t="inlineStr">
         <is>
@@ -1323,13 +1323,13 @@
         <v>1</v>
       </c>
       <c r="E33" t="n">
-        <v>1714500</v>
+        <v>1678130.517499804</v>
       </c>
       <c r="F33" t="n">
-        <v>32000</v>
+        <v>-16325.48250019504</v>
       </c>
       <c r="G33" t="n">
-        <v>1.901931649331352</v>
+        <v>-0.9634645278599764</v>
       </c>
     </row>
     <row r="34">
@@ -1350,13 +1350,13 @@
         <v>1</v>
       </c>
       <c r="E34" t="n">
-        <v>1650000</v>
+        <v>1670000</v>
       </c>
       <c r="F34" t="n">
-        <v>499.9999999993015</v>
+        <v>20499.9999999993</v>
       </c>
       <c r="G34" t="n">
-        <v>0.0303122158229343</v>
+        <v>1.242800848742</v>
       </c>
     </row>
     <row r="35">
@@ -1377,23 +1377,23 @@
         <v>1</v>
       </c>
       <c r="E35" t="n">
-        <v>902000</v>
+        <v>926000</v>
       </c>
       <c r="F35" t="n">
-        <v>69000</v>
+        <v>93000</v>
       </c>
       <c r="G35" t="n">
-        <v>8.283313325330131</v>
+        <v>11.16446578631453</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>클리블랜드 클리프스</t>
+          <t>비에이치아이</t>
         </is>
       </c>
       <c r="B36" t="n">
-        <v>70</v>
+        <v>8</v>
       </c>
       <c r="C36" t="inlineStr">
         <is>
@@ -1404,23 +1404,23 @@
         <v>1</v>
       </c>
       <c r="E36" t="n">
-        <v>856598.1687739864</v>
+        <v>876000</v>
       </c>
       <c r="F36" t="n">
-        <v>-159456.8312260136</v>
+        <v>210885</v>
       </c>
       <c r="G36" t="n">
-        <v>-15.69372044092235</v>
+        <v>31.70654698811484</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>비에이치아이</t>
+          <t>클리블랜드 클리프스</t>
         </is>
       </c>
       <c r="B37" t="n">
-        <v>8</v>
+        <v>70</v>
       </c>
       <c r="C37" t="inlineStr">
         <is>
@@ -1431,13 +1431,13 @@
         <v>1</v>
       </c>
       <c r="E37" t="n">
-        <v>886400</v>
+        <v>856598.1687739864</v>
       </c>
       <c r="F37" t="n">
-        <v>221285</v>
+        <v>-159456.8312260136</v>
       </c>
       <c r="G37" t="n">
-        <v>33.27018635875</v>
+        <v>-15.69372044092235</v>
       </c>
     </row>
     <row r="38">
@@ -1549,7 +1549,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2026-03-20T03:09:27</t>
+          <t>2026-03-20T07:02:39</t>
         </is>
       </c>
       <c r="E2" t="n">
@@ -5868,7 +5868,7 @@
       </c>
       <c r="I116" t="inlineStr">
         <is>
-          <t>2026-03-20T03:09:27</t>
+          <t>2026-03-20T07:02:39</t>
         </is>
       </c>
     </row>
@@ -5905,7 +5905,7 @@
       </c>
       <c r="I117" t="inlineStr">
         <is>
-          <t>2026-03-20T03:09:27</t>
+          <t>2026-03-20T07:02:39</t>
         </is>
       </c>
     </row>
@@ -5932,17 +5932,17 @@
         <v>1</v>
       </c>
       <c r="F118" t="n">
-        <v>9220000</v>
+        <v>9120000</v>
       </c>
       <c r="G118" t="n">
-        <v>2007000</v>
+        <v>1907000</v>
       </c>
       <c r="H118" t="n">
-        <v>27.82476084846805</v>
+        <v>26.43837515596839</v>
       </c>
       <c r="I118" t="inlineStr">
         <is>
-          <t>2026-03-20T03:09:27</t>
+          <t>2026-03-20T07:02:39</t>
         </is>
       </c>
     </row>
@@ -5979,7 +5979,7 @@
       </c>
       <c r="I119" t="inlineStr">
         <is>
-          <t>2026-03-20T03:09:27</t>
+          <t>2026-03-20T07:02:39</t>
         </is>
       </c>
     </row>
@@ -6016,7 +6016,7 @@
       </c>
       <c r="I120" t="inlineStr">
         <is>
-          <t>2026-03-20T03:09:27</t>
+          <t>2026-03-20T07:02:39</t>
         </is>
       </c>
     </row>
@@ -6043,17 +6043,17 @@
         <v>1</v>
       </c>
       <c r="F121" t="n">
-        <v>7325000</v>
+        <v>7395000</v>
       </c>
       <c r="G121" t="n">
-        <v>1015000</v>
+        <v>1085000</v>
       </c>
       <c r="H121" t="n">
-        <v>16.08557844690967</v>
+        <v>17.19492868462758</v>
       </c>
       <c r="I121" t="inlineStr">
         <is>
-          <t>2026-03-20T03:09:27</t>
+          <t>2026-03-20T07:02:39</t>
         </is>
       </c>
     </row>
@@ -6090,7 +6090,7 @@
       </c>
       <c r="I122" t="inlineStr">
         <is>
-          <t>2026-03-20T03:09:27</t>
+          <t>2026-03-20T07:02:39</t>
         </is>
       </c>
     </row>
@@ -6127,7 +6127,7 @@
       </c>
       <c r="I123" t="inlineStr">
         <is>
-          <t>2026-03-20T03:09:27</t>
+          <t>2026-03-20T07:02:39</t>
         </is>
       </c>
     </row>
@@ -6164,7 +6164,7 @@
       </c>
       <c r="I124" t="inlineStr">
         <is>
-          <t>2026-03-20T03:09:27</t>
+          <t>2026-03-20T07:02:39</t>
         </is>
       </c>
     </row>
@@ -6176,11 +6176,11 @@
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>타이드워터</t>
+          <t>DL이앤씨</t>
         </is>
       </c>
       <c r="C125" t="n">
-        <v>48</v>
+        <v>80</v>
       </c>
       <c r="D125" t="inlineStr">
         <is>
@@ -6191,17 +6191,17 @@
         <v>1</v>
       </c>
       <c r="F125" t="n">
-        <v>5333826.773907423</v>
+        <v>5392000</v>
       </c>
       <c r="G125" t="n">
-        <v>1609281.773907423</v>
+        <v>1981000</v>
       </c>
       <c r="H125" t="n">
-        <v>43.20747296401098</v>
+        <v>58.07681031955438</v>
       </c>
       <c r="I125" t="inlineStr">
         <is>
-          <t>2026-03-20T03:09:27</t>
+          <t>2026-03-20T07:02:39</t>
         </is>
       </c>
     </row>
@@ -6213,11 +6213,11 @@
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>노브</t>
+          <t>타이드워터</t>
         </is>
       </c>
       <c r="C126" t="n">
-        <v>185</v>
+        <v>48</v>
       </c>
       <c r="D126" t="inlineStr">
         <is>
@@ -6228,17 +6228,17 @@
         <v>1</v>
       </c>
       <c r="F126" t="n">
-        <v>5144899.592058761</v>
+        <v>5333826.773907423</v>
       </c>
       <c r="G126" t="n">
-        <v>1834891.592058761</v>
+        <v>1609281.773907423</v>
       </c>
       <c r="H126" t="n">
-        <v>55.43465731982403</v>
+        <v>43.20747296401098</v>
       </c>
       <c r="I126" t="inlineStr">
         <is>
-          <t>2026-03-20T03:09:27</t>
+          <t>2026-03-20T07:02:39</t>
         </is>
       </c>
     </row>
@@ -6250,11 +6250,11 @@
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>DL이앤씨</t>
+          <t>노브</t>
         </is>
       </c>
       <c r="C127" t="n">
-        <v>80</v>
+        <v>185</v>
       </c>
       <c r="D127" t="inlineStr">
         <is>
@@ -6265,17 +6265,17 @@
         <v>1</v>
       </c>
       <c r="F127" t="n">
-        <v>5096000</v>
+        <v>5144899.592058761</v>
       </c>
       <c r="G127" t="n">
-        <v>1685000</v>
+        <v>1834891.592058761</v>
       </c>
       <c r="H127" t="n">
-        <v>49.39900322486074</v>
+        <v>55.43465731982403</v>
       </c>
       <c r="I127" t="inlineStr">
         <is>
-          <t>2026-03-20T03:09:27</t>
+          <t>2026-03-20T07:02:39</t>
         </is>
       </c>
     </row>
@@ -6302,17 +6302,17 @@
         <v>1</v>
       </c>
       <c r="F128" t="n">
-        <v>4787820</v>
+        <v>4797870</v>
       </c>
       <c r="G128" t="n">
-        <v>64023</v>
+        <v>74073</v>
       </c>
       <c r="H128" t="n">
-        <v>1.355329198100596</v>
+        <v>1.568081778281328</v>
       </c>
       <c r="I128" t="inlineStr">
         <is>
-          <t>2026-03-20T03:09:27</t>
+          <t>2026-03-20T07:02:39</t>
         </is>
       </c>
     </row>
@@ -6349,7 +6349,7 @@
       </c>
       <c r="I129" t="inlineStr">
         <is>
-          <t>2026-03-20T03:09:27</t>
+          <t>2026-03-20T07:02:39</t>
         </is>
       </c>
     </row>
@@ -6376,17 +6376,17 @@
         <v>1</v>
       </c>
       <c r="F130" t="n">
-        <v>4293000</v>
+        <v>4270500</v>
       </c>
       <c r="G130" t="n">
-        <v>-338000</v>
+        <v>-360500</v>
       </c>
       <c r="H130" t="n">
-        <v>-7.298639602677608</v>
+        <v>-7.784495789246384</v>
       </c>
       <c r="I130" t="inlineStr">
         <is>
-          <t>2026-03-20T03:09:27</t>
+          <t>2026-03-20T07:02:39</t>
         </is>
       </c>
     </row>
@@ -6413,17 +6413,17 @@
         <v>1</v>
       </c>
       <c r="F131" t="n">
-        <v>4134400</v>
+        <v>4202400</v>
       </c>
       <c r="G131" t="n">
-        <v>397000</v>
+        <v>465000</v>
       </c>
       <c r="H131" t="n">
-        <v>10.62235778883716</v>
+        <v>12.44180446299566</v>
       </c>
       <c r="I131" t="inlineStr">
         <is>
-          <t>2026-03-20T03:09:27</t>
+          <t>2026-03-20T07:02:39</t>
         </is>
       </c>
     </row>
@@ -6450,17 +6450,17 @@
         <v>1</v>
       </c>
       <c r="F132" t="n">
-        <v>4088900</v>
+        <v>4123000</v>
       </c>
       <c r="G132" t="n">
-        <v>53804</v>
+        <v>87904</v>
       </c>
       <c r="H132" t="n">
-        <v>1.333400741890651</v>
+        <v>2.178485964150543</v>
       </c>
       <c r="I132" t="inlineStr">
         <is>
-          <t>2026-03-20T03:09:27</t>
+          <t>2026-03-20T07:02:39</t>
         </is>
       </c>
     </row>
@@ -6497,7 +6497,7 @@
       </c>
       <c r="I133" t="inlineStr">
         <is>
-          <t>2026-03-20T03:09:27</t>
+          <t>2026-03-20T07:02:39</t>
         </is>
       </c>
     </row>
@@ -6534,7 +6534,7 @@
       </c>
       <c r="I134" t="inlineStr">
         <is>
-          <t>2026-03-20T03:09:27</t>
+          <t>2026-03-20T07:02:39</t>
         </is>
       </c>
     </row>
@@ -6571,7 +6571,7 @@
       </c>
       <c r="I135" t="inlineStr">
         <is>
-          <t>2026-03-20T03:09:27</t>
+          <t>2026-03-20T07:02:39</t>
         </is>
       </c>
     </row>
@@ -6598,17 +6598,17 @@
         <v>1</v>
       </c>
       <c r="F136" t="n">
-        <v>2725000</v>
+        <v>2750000</v>
       </c>
       <c r="G136" t="n">
-        <v>446390</v>
+        <v>471390</v>
       </c>
       <c r="H136" t="n">
-        <v>19.59045207385204</v>
+        <v>20.68761218462133</v>
       </c>
       <c r="I136" t="inlineStr">
         <is>
-          <t>2026-03-20T03:09:27</t>
+          <t>2026-03-20T07:02:39</t>
         </is>
       </c>
     </row>
@@ -6635,17 +6635,17 @@
         <v>1</v>
       </c>
       <c r="F137" t="n">
-        <v>2590000</v>
+        <v>2621500</v>
       </c>
       <c r="G137" t="n">
-        <v>-217500</v>
+        <v>-186000</v>
       </c>
       <c r="H137" t="n">
-        <v>-7.747105966162065</v>
+        <v>-6.625111308993767</v>
       </c>
       <c r="I137" t="inlineStr">
         <is>
-          <t>2026-03-20T03:09:27</t>
+          <t>2026-03-20T07:02:39</t>
         </is>
       </c>
     </row>
@@ -6672,17 +6672,17 @@
         <v>1</v>
       </c>
       <c r="F138" t="n">
-        <v>2582400</v>
+        <v>2582000</v>
       </c>
       <c r="G138" t="n">
-        <v>-119600</v>
+        <v>-120000</v>
       </c>
       <c r="H138" t="n">
-        <v>-4.426350851221318</v>
+        <v>-4.441154700222058</v>
       </c>
       <c r="I138" t="inlineStr">
         <is>
-          <t>2026-03-20T03:09:27</t>
+          <t>2026-03-20T07:02:39</t>
         </is>
       </c>
     </row>
@@ -6709,17 +6709,17 @@
         <v>1</v>
       </c>
       <c r="F139" t="n">
-        <v>2484000</v>
+        <v>2514000</v>
       </c>
       <c r="G139" t="n">
-        <v>473000</v>
+        <v>503000</v>
       </c>
       <c r="H139" t="n">
-        <v>23.5206364992541</v>
+        <v>25.01243162605669</v>
       </c>
       <c r="I139" t="inlineStr">
         <is>
-          <t>2026-03-20T03:09:27</t>
+          <t>2026-03-20T07:02:39</t>
         </is>
       </c>
     </row>
@@ -6746,17 +6746,17 @@
         <v>1</v>
       </c>
       <c r="F140" t="n">
-        <v>2213750</v>
+        <v>2219250</v>
       </c>
       <c r="G140" t="n">
-        <v>504249</v>
+        <v>509749</v>
       </c>
       <c r="H140" t="n">
-        <v>29.49685317528332</v>
+        <v>29.81858448752005</v>
       </c>
       <c r="I140" t="inlineStr">
         <is>
-          <t>2026-03-20T03:09:27</t>
+          <t>2026-03-20T07:02:39</t>
         </is>
       </c>
     </row>
@@ -6793,7 +6793,7 @@
       </c>
       <c r="I141" t="inlineStr">
         <is>
-          <t>2026-03-20T03:09:27</t>
+          <t>2026-03-20T07:02:39</t>
         </is>
       </c>
     </row>
@@ -6820,17 +6820,17 @@
         <v>1</v>
       </c>
       <c r="F142" t="n">
-        <v>2071800</v>
+        <v>2097000</v>
       </c>
       <c r="G142" t="n">
-        <v>-320400</v>
+        <v>-295200</v>
       </c>
       <c r="H142" t="n">
-        <v>-13.39352896914974</v>
+        <v>-12.34010534236268</v>
       </c>
       <c r="I142" t="inlineStr">
         <is>
-          <t>2026-03-20T03:09:27</t>
+          <t>2026-03-20T07:02:39</t>
         </is>
       </c>
     </row>
@@ -6857,17 +6857,17 @@
         <v>1</v>
       </c>
       <c r="F143" t="n">
-        <v>1983000</v>
+        <v>2004000</v>
       </c>
       <c r="G143" t="n">
-        <v>-75000</v>
+        <v>-54000</v>
       </c>
       <c r="H143" t="n">
-        <v>-3.644314868804665</v>
+        <v>-2.623906705539359</v>
       </c>
       <c r="I143" t="inlineStr">
         <is>
-          <t>2026-03-20T03:09:27</t>
+          <t>2026-03-20T07:02:39</t>
         </is>
       </c>
     </row>
@@ -6894,17 +6894,17 @@
         <v>1</v>
       </c>
       <c r="F144" t="n">
-        <v>1971495</v>
+        <v>1995330</v>
       </c>
       <c r="G144" t="n">
-        <v>-6</v>
+        <v>23829</v>
       </c>
       <c r="H144" t="n">
-        <v>-0.0003043366450232589</v>
+        <v>1.208672985709873</v>
       </c>
       <c r="I144" t="inlineStr">
         <is>
-          <t>2026-03-20T03:09:27</t>
+          <t>2026-03-20T07:02:39</t>
         </is>
       </c>
     </row>
@@ -6916,11 +6916,11 @@
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>하나금융지주</t>
+          <t>스타 벌크 캐리어스</t>
         </is>
       </c>
       <c r="C145" t="n">
-        <v>15</v>
+        <v>50</v>
       </c>
       <c r="D145" t="inlineStr">
         <is>
@@ -6931,17 +6931,17 @@
         <v>1</v>
       </c>
       <c r="F145" t="n">
-        <v>1714500</v>
+        <v>1700181.21356247</v>
       </c>
       <c r="G145" t="n">
-        <v>32000</v>
+        <v>385828.2135624706</v>
       </c>
       <c r="H145" t="n">
-        <v>1.901931649331352</v>
+        <v>29.35499166224529</v>
       </c>
       <c r="I145" t="inlineStr">
         <is>
-          <t>2026-03-20T03:09:27</t>
+          <t>2026-03-20T07:02:39</t>
         </is>
       </c>
     </row>
@@ -6953,11 +6953,11 @@
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>스타 벌크 캐리어스</t>
+          <t>하나금융지주</t>
         </is>
       </c>
       <c r="C146" t="n">
-        <v>50</v>
+        <v>15</v>
       </c>
       <c r="D146" t="inlineStr">
         <is>
@@ -6968,17 +6968,17 @@
         <v>1</v>
       </c>
       <c r="F146" t="n">
-        <v>1700181.21356247</v>
+        <v>1698000</v>
       </c>
       <c r="G146" t="n">
-        <v>385828.2135624706</v>
+        <v>15500</v>
       </c>
       <c r="H146" t="n">
-        <v>29.35499166224529</v>
+        <v>0.9212481426448738</v>
       </c>
       <c r="I146" t="inlineStr">
         <is>
-          <t>2026-03-20T03:09:27</t>
+          <t>2026-03-20T07:02:39</t>
         </is>
       </c>
     </row>
@@ -7015,7 +7015,7 @@
       </c>
       <c r="I147" t="inlineStr">
         <is>
-          <t>2026-03-20T03:09:27</t>
+          <t>2026-03-20T07:02:39</t>
         </is>
       </c>
     </row>
@@ -7042,17 +7042,17 @@
         <v>1</v>
       </c>
       <c r="F148" t="n">
-        <v>1650000</v>
+        <v>1670000</v>
       </c>
       <c r="G148" t="n">
-        <v>499.9999999993015</v>
+        <v>20499.9999999993</v>
       </c>
       <c r="H148" t="n">
-        <v>0.0303122158229343</v>
+        <v>1.242800848742</v>
       </c>
       <c r="I148" t="inlineStr">
         <is>
-          <t>2026-03-20T03:09:27</t>
+          <t>2026-03-20T07:02:39</t>
         </is>
       </c>
     </row>
@@ -7079,17 +7079,17 @@
         <v>1</v>
       </c>
       <c r="F149" t="n">
-        <v>902000</v>
+        <v>926000</v>
       </c>
       <c r="G149" t="n">
-        <v>69000</v>
+        <v>93000</v>
       </c>
       <c r="H149" t="n">
-        <v>8.283313325330131</v>
+        <v>11.16446578631453</v>
       </c>
       <c r="I149" t="inlineStr">
         <is>
-          <t>2026-03-20T03:09:27</t>
+          <t>2026-03-20T07:02:39</t>
         </is>
       </c>
     </row>
@@ -7116,17 +7116,17 @@
         <v>1</v>
       </c>
       <c r="F150" t="n">
-        <v>886400</v>
+        <v>876000</v>
       </c>
       <c r="G150" t="n">
-        <v>221285</v>
+        <v>210885</v>
       </c>
       <c r="H150" t="n">
-        <v>33.27018635875</v>
+        <v>31.70654698811484</v>
       </c>
       <c r="I150" t="inlineStr">
         <is>
-          <t>2026-03-20T03:09:27</t>
+          <t>2026-03-20T07:02:39</t>
         </is>
       </c>
     </row>
@@ -7163,7 +7163,7 @@
       </c>
       <c r="I151" t="inlineStr">
         <is>
-          <t>2026-03-20T03:09:27</t>
+          <t>2026-03-20T07:02:39</t>
         </is>
       </c>
     </row>
@@ -7200,7 +7200,7 @@
       </c>
       <c r="I152" t="inlineStr">
         <is>
-          <t>2026-03-20T03:09:27</t>
+          <t>2026-03-20T07:02:39</t>
         </is>
       </c>
     </row>
@@ -7237,7 +7237,7 @@
       </c>
       <c r="I153" t="inlineStr">
         <is>
-          <t>2026-03-20T03:09:27</t>
+          <t>2026-03-20T07:02:39</t>
         </is>
       </c>
     </row>
@@ -7370,7 +7370,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>2026-03-20T03:09:27</t>
+          <t>2026-03-20T07:02:39</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: portfolio snapshot 2026-03-20 (2026-03-20T13:46:30)
</commit_message>
<xml_diff>
--- a/portfolio_auto.xlsx
+++ b/portfolio_auto.xlsx
@@ -486,13 +486,13 @@
         <v>1</v>
       </c>
       <c r="E2" t="n">
-        <v>14203432.81962231</v>
+        <v>13768999.19239014</v>
       </c>
       <c r="F2" t="n">
-        <v>2096883.819622312</v>
+        <v>1662450.192390148</v>
       </c>
       <c r="G2" t="n">
-        <v>17.32024394088119</v>
+        <v>13.73182557961107</v>
       </c>
     </row>
     <row r="3">
@@ -513,13 +513,13 @@
         <v>1</v>
       </c>
       <c r="E3" t="n">
-        <v>10775543.75936943</v>
+        <v>10644645.51107842</v>
       </c>
       <c r="F3" t="n">
-        <v>-56471.2406305708</v>
+        <v>-187369.4889215864</v>
       </c>
       <c r="G3" t="n">
-        <v>-0.5213364330696624</v>
+        <v>-1.729775013435509</v>
       </c>
     </row>
     <row r="4">
@@ -567,13 +567,13 @@
         <v>1</v>
       </c>
       <c r="E5" t="n">
-        <v>8607869.087246014</v>
+        <v>8410212.452697754</v>
       </c>
       <c r="F5" t="n">
-        <v>4178005.087246014</v>
+        <v>3980348.452697754</v>
       </c>
       <c r="G5" t="n">
-        <v>94.31452268615953</v>
+        <v>89.85261066023142</v>
       </c>
     </row>
     <row r="6">
@@ -594,13 +594,13 @@
         <v>1</v>
       </c>
       <c r="E6" t="n">
-        <v>8260008.470450722</v>
+        <v>8156965.818628304</v>
       </c>
       <c r="F6" t="n">
-        <v>1809657.470450722</v>
+        <v>1706614.818628304</v>
       </c>
       <c r="G6" t="n">
-        <v>28.05517824457494</v>
+        <v>26.45770468348627</v>
       </c>
     </row>
     <row r="7">
@@ -648,13 +648,13 @@
         <v>1</v>
       </c>
       <c r="E8" t="n">
-        <v>7248023.048171424</v>
+        <v>7175093.959923077</v>
       </c>
       <c r="F8" t="n">
-        <v>3120789.048171425</v>
+        <v>3047859.959923078</v>
       </c>
       <c r="G8" t="n">
-        <v>75.61454107451686</v>
+        <v>73.84752015328131</v>
       </c>
     </row>
     <row r="9">
@@ -675,13 +675,13 @@
         <v>1</v>
       </c>
       <c r="E9" t="n">
-        <v>7071871.362670898</v>
+        <v>7014955.722778145</v>
       </c>
       <c r="F9" t="n">
-        <v>3164663.362670898</v>
+        <v>3107747.722778145</v>
       </c>
       <c r="G9" t="n">
-        <v>80.99551809555309</v>
+        <v>79.53883496292353</v>
       </c>
     </row>
     <row r="10">
@@ -702,23 +702,23 @@
         <v>1</v>
       </c>
       <c r="E10" t="n">
-        <v>6443021.103033766</v>
+        <v>6301685.50906603</v>
       </c>
       <c r="F10" t="n">
-        <v>211802.1030337671</v>
+        <v>70466.50906603131</v>
       </c>
       <c r="G10" t="n">
-        <v>3.399047650768928</v>
+        <v>1.130862341157185</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>타이드워터</t>
+          <t>DL이앤씨</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>48</v>
+        <v>80</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
@@ -729,23 +729,23 @@
         <v>1</v>
       </c>
       <c r="E11" t="n">
-        <v>5333826.773907423</v>
+        <v>5392000</v>
       </c>
       <c r="F11" t="n">
-        <v>1609281.773907423</v>
+        <v>1981000</v>
       </c>
       <c r="G11" t="n">
-        <v>43.20747296401098</v>
+        <v>58.07681031955438</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>노브</t>
+          <t>타이드워터</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>185</v>
+        <v>48</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
@@ -756,23 +756,23 @@
         <v>1</v>
       </c>
       <c r="E12" t="n">
-        <v>5144899.592058761</v>
+        <v>5264173.858361721</v>
       </c>
       <c r="F12" t="n">
-        <v>1834891.592058761</v>
+        <v>1539628.858361721</v>
       </c>
       <c r="G12" t="n">
-        <v>55.43465731982403</v>
+        <v>41.33736760763318</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>DL이앤씨</t>
+          <t>노브</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>80</v>
+        <v>185</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
@@ -783,13 +783,13 @@
         <v>1</v>
       </c>
       <c r="E13" t="n">
-        <v>5392000</v>
+        <v>5156523.305831412</v>
       </c>
       <c r="F13" t="n">
-        <v>1981000</v>
+        <v>1846515.305831412</v>
       </c>
       <c r="G13" t="n">
-        <v>58.07681031955438</v>
+        <v>55.78582607146001</v>
       </c>
     </row>
     <row r="14">
@@ -837,13 +837,13 @@
         <v>1</v>
       </c>
       <c r="E15" t="n">
-        <v>4584804.793516081</v>
+        <v>4511875.769468229</v>
       </c>
       <c r="F15" t="n">
-        <v>2328444.793516081</v>
+        <v>2255515.769468229</v>
       </c>
       <c r="G15" t="n">
-        <v>103.1947381409031</v>
+        <v>99.96258440444917</v>
       </c>
     </row>
     <row r="16">
@@ -945,13 +945,13 @@
         <v>1</v>
       </c>
       <c r="E19" t="n">
-        <v>4071683.614561614</v>
+        <v>4087391.335876007</v>
       </c>
       <c r="F19" t="n">
-        <v>247035.6145616136</v>
+        <v>262743.3358760066</v>
       </c>
       <c r="G19" t="n">
-        <v>6.459041840232452</v>
+        <v>6.869739015878236</v>
       </c>
     </row>
     <row r="20">
@@ -972,13 +972,13 @@
         <v>1</v>
       </c>
       <c r="E20" t="n">
-        <v>3641589.341643294</v>
+        <v>3711115.026073027</v>
       </c>
       <c r="F20" t="n">
-        <v>2170817.341643294</v>
+        <v>2240343.026073027</v>
       </c>
       <c r="G20" t="n">
-        <v>147.5971354936927</v>
+        <v>152.3242913295213</v>
       </c>
     </row>
     <row r="21">
@@ -999,13 +999,13 @@
         <v>1</v>
       </c>
       <c r="E21" t="n">
-        <v>2971420.173610602</v>
+        <v>2945895.015193854</v>
       </c>
       <c r="F21" t="n">
-        <v>-219223.8263893984</v>
+        <v>-244748.9848061465</v>
       </c>
       <c r="G21" t="n">
-        <v>-6.870833173158723</v>
+        <v>-7.6708333742701</v>
       </c>
     </row>
     <row r="22">
@@ -1161,13 +1161,13 @@
         <v>1</v>
       </c>
       <c r="E27" t="n">
-        <v>2172791.30897373</v>
+        <v>2162693.444105566</v>
       </c>
       <c r="F27" t="n">
-        <v>108801.3089737301</v>
+        <v>98703.44410556601</v>
       </c>
       <c r="G27" t="n">
-        <v>5.271406788488806</v>
+        <v>4.782166779178485</v>
       </c>
     </row>
     <row r="28">
@@ -1254,11 +1254,11 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>하나금융지주</t>
+          <t>스타 벌크 캐리어스</t>
         </is>
       </c>
       <c r="B31" t="n">
-        <v>15</v>
+        <v>50</v>
       </c>
       <c r="C31" t="inlineStr">
         <is>
@@ -1269,23 +1269,23 @@
         <v>1</v>
       </c>
       <c r="E31" t="n">
-        <v>1698000</v>
+        <v>1691579.345794907</v>
       </c>
       <c r="F31" t="n">
-        <v>15500</v>
+        <v>377226.3457949075</v>
       </c>
       <c r="G31" t="n">
-        <v>0.9212481426448738</v>
+        <v>28.7005352287329</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>스타 벌크 캐리어스</t>
+          <t>하나금융지주</t>
         </is>
       </c>
       <c r="B32" t="n">
-        <v>50</v>
+        <v>15</v>
       </c>
       <c r="C32" t="inlineStr">
         <is>
@@ -1296,13 +1296,13 @@
         <v>1</v>
       </c>
       <c r="E32" t="n">
-        <v>1700181.21356247</v>
+        <v>1698000</v>
       </c>
       <c r="F32" t="n">
-        <v>385828.2135624706</v>
+        <v>15500</v>
       </c>
       <c r="G32" t="n">
-        <v>29.35499166224529</v>
+        <v>0.9212481426448738</v>
       </c>
     </row>
     <row r="33">
@@ -1323,13 +1323,13 @@
         <v>1</v>
       </c>
       <c r="E33" t="n">
-        <v>1678130.517499804</v>
+        <v>1688243.356776953</v>
       </c>
       <c r="F33" t="n">
-        <v>-16325.48250019504</v>
+        <v>-6212.643223046791</v>
       </c>
       <c r="G33" t="n">
-        <v>-0.9634645278599764</v>
+        <v>-0.366645296369265</v>
       </c>
     </row>
     <row r="34">
@@ -1431,13 +1431,13 @@
         <v>1</v>
       </c>
       <c r="E37" t="n">
-        <v>856598.1687739864</v>
+        <v>846649.8739409866</v>
       </c>
       <c r="F37" t="n">
-        <v>-159456.8312260136</v>
+        <v>-169405.1260590134</v>
       </c>
       <c r="G37" t="n">
-        <v>-15.69372044092235</v>
+        <v>-16.67283031519095</v>
       </c>
     </row>
     <row r="38">
@@ -1458,13 +1458,13 @@
         <v>1</v>
       </c>
       <c r="E38" t="n">
-        <v>853306.9945554808</v>
+        <v>852110.1831788942</v>
       </c>
       <c r="F38" t="n">
-        <v>227575.9945554808</v>
+        <v>226379.1831788942</v>
       </c>
       <c r="G38" t="n">
-        <v>36.36962121989813</v>
+        <v>36.17835510449286</v>
       </c>
     </row>
     <row r="39">
@@ -1485,13 +1485,13 @@
         <v>1</v>
       </c>
       <c r="E39" t="n">
-        <v>796639.2884175777</v>
+        <v>796564.4163726568</v>
       </c>
       <c r="F39" t="n">
-        <v>18048.28841757774</v>
+        <v>17973.41637265682</v>
       </c>
       <c r="G39" t="n">
-        <v>2.318070516815343</v>
+        <v>2.308454165621851</v>
       </c>
     </row>
   </sheetData>
@@ -1549,7 +1549,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2026-03-20T07:02:39</t>
+          <t>2026-03-20T13:46:30</t>
         </is>
       </c>
       <c r="E2" t="n">
@@ -5858,17 +5858,17 @@
         <v>1</v>
       </c>
       <c r="F116" t="n">
-        <v>14203432.81962231</v>
+        <v>13768999.19239014</v>
       </c>
       <c r="G116" t="n">
-        <v>2096883.819622312</v>
+        <v>1662450.192390148</v>
       </c>
       <c r="H116" t="n">
-        <v>17.32024394088119</v>
+        <v>13.73182557961107</v>
       </c>
       <c r="I116" t="inlineStr">
         <is>
-          <t>2026-03-20T07:02:39</t>
+          <t>2026-03-20T13:46:30</t>
         </is>
       </c>
     </row>
@@ -5895,17 +5895,17 @@
         <v>1</v>
       </c>
       <c r="F117" t="n">
-        <v>10775543.75936943</v>
+        <v>10644645.51107842</v>
       </c>
       <c r="G117" t="n">
-        <v>-56471.2406305708</v>
+        <v>-187369.4889215864</v>
       </c>
       <c r="H117" t="n">
-        <v>-0.5213364330696624</v>
+        <v>-1.729775013435509</v>
       </c>
       <c r="I117" t="inlineStr">
         <is>
-          <t>2026-03-20T07:02:39</t>
+          <t>2026-03-20T13:46:30</t>
         </is>
       </c>
     </row>
@@ -5942,7 +5942,7 @@
       </c>
       <c r="I118" t="inlineStr">
         <is>
-          <t>2026-03-20T07:02:39</t>
+          <t>2026-03-20T13:46:30</t>
         </is>
       </c>
     </row>
@@ -5969,17 +5969,17 @@
         <v>1</v>
       </c>
       <c r="F119" t="n">
-        <v>8607869.087246014</v>
+        <v>8410212.452697754</v>
       </c>
       <c r="G119" t="n">
-        <v>4178005.087246014</v>
+        <v>3980348.452697754</v>
       </c>
       <c r="H119" t="n">
-        <v>94.31452268615953</v>
+        <v>89.85261066023142</v>
       </c>
       <c r="I119" t="inlineStr">
         <is>
-          <t>2026-03-20T07:02:39</t>
+          <t>2026-03-20T13:46:30</t>
         </is>
       </c>
     </row>
@@ -6006,17 +6006,17 @@
         <v>1</v>
       </c>
       <c r="F120" t="n">
-        <v>8260008.470450722</v>
+        <v>8156965.818628304</v>
       </c>
       <c r="G120" t="n">
-        <v>1809657.470450722</v>
+        <v>1706614.818628304</v>
       </c>
       <c r="H120" t="n">
-        <v>28.05517824457494</v>
+        <v>26.45770468348627</v>
       </c>
       <c r="I120" t="inlineStr">
         <is>
-          <t>2026-03-20T07:02:39</t>
+          <t>2026-03-20T13:46:30</t>
         </is>
       </c>
     </row>
@@ -6053,7 +6053,7 @@
       </c>
       <c r="I121" t="inlineStr">
         <is>
-          <t>2026-03-20T07:02:39</t>
+          <t>2026-03-20T13:46:30</t>
         </is>
       </c>
     </row>
@@ -6080,17 +6080,17 @@
         <v>1</v>
       </c>
       <c r="F122" t="n">
-        <v>7248023.048171424</v>
+        <v>7175093.959923077</v>
       </c>
       <c r="G122" t="n">
-        <v>3120789.048171425</v>
+        <v>3047859.959923078</v>
       </c>
       <c r="H122" t="n">
-        <v>75.61454107451686</v>
+        <v>73.84752015328131</v>
       </c>
       <c r="I122" t="inlineStr">
         <is>
-          <t>2026-03-20T07:02:39</t>
+          <t>2026-03-20T13:46:30</t>
         </is>
       </c>
     </row>
@@ -6117,17 +6117,17 @@
         <v>1</v>
       </c>
       <c r="F123" t="n">
-        <v>7071871.362670898</v>
+        <v>7014955.722778145</v>
       </c>
       <c r="G123" t="n">
-        <v>3164663.362670898</v>
+        <v>3107747.722778145</v>
       </c>
       <c r="H123" t="n">
-        <v>80.99551809555309</v>
+        <v>79.53883496292353</v>
       </c>
       <c r="I123" t="inlineStr">
         <is>
-          <t>2026-03-20T07:02:39</t>
+          <t>2026-03-20T13:46:30</t>
         </is>
       </c>
     </row>
@@ -6154,17 +6154,17 @@
         <v>1</v>
       </c>
       <c r="F124" t="n">
-        <v>6443021.103033766</v>
+        <v>6301685.50906603</v>
       </c>
       <c r="G124" t="n">
-        <v>211802.1030337671</v>
+        <v>70466.50906603131</v>
       </c>
       <c r="H124" t="n">
-        <v>3.399047650768928</v>
+        <v>1.130862341157185</v>
       </c>
       <c r="I124" t="inlineStr">
         <is>
-          <t>2026-03-20T07:02:39</t>
+          <t>2026-03-20T13:46:30</t>
         </is>
       </c>
     </row>
@@ -6201,7 +6201,7 @@
       </c>
       <c r="I125" t="inlineStr">
         <is>
-          <t>2026-03-20T07:02:39</t>
+          <t>2026-03-20T13:46:30</t>
         </is>
       </c>
     </row>
@@ -6228,17 +6228,17 @@
         <v>1</v>
       </c>
       <c r="F126" t="n">
-        <v>5333826.773907423</v>
+        <v>5264173.858361721</v>
       </c>
       <c r="G126" t="n">
-        <v>1609281.773907423</v>
+        <v>1539628.858361721</v>
       </c>
       <c r="H126" t="n">
-        <v>43.20747296401098</v>
+        <v>41.33736760763318</v>
       </c>
       <c r="I126" t="inlineStr">
         <is>
-          <t>2026-03-20T07:02:39</t>
+          <t>2026-03-20T13:46:30</t>
         </is>
       </c>
     </row>
@@ -6265,17 +6265,17 @@
         <v>1</v>
       </c>
       <c r="F127" t="n">
-        <v>5144899.592058761</v>
+        <v>5156523.305831412</v>
       </c>
       <c r="G127" t="n">
-        <v>1834891.592058761</v>
+        <v>1846515.305831412</v>
       </c>
       <c r="H127" t="n">
-        <v>55.43465731982403</v>
+        <v>55.78582607146001</v>
       </c>
       <c r="I127" t="inlineStr">
         <is>
-          <t>2026-03-20T07:02:39</t>
+          <t>2026-03-20T13:46:30</t>
         </is>
       </c>
     </row>
@@ -6312,7 +6312,7 @@
       </c>
       <c r="I128" t="inlineStr">
         <is>
-          <t>2026-03-20T07:02:39</t>
+          <t>2026-03-20T13:46:30</t>
         </is>
       </c>
     </row>
@@ -6339,17 +6339,17 @@
         <v>1</v>
       </c>
       <c r="F129" t="n">
-        <v>4584804.793516081</v>
+        <v>4511875.769468229</v>
       </c>
       <c r="G129" t="n">
-        <v>2328444.793516081</v>
+        <v>2255515.769468229</v>
       </c>
       <c r="H129" t="n">
-        <v>103.1947381409031</v>
+        <v>99.96258440444917</v>
       </c>
       <c r="I129" t="inlineStr">
         <is>
-          <t>2026-03-20T07:02:39</t>
+          <t>2026-03-20T13:46:30</t>
         </is>
       </c>
     </row>
@@ -6386,7 +6386,7 @@
       </c>
       <c r="I130" t="inlineStr">
         <is>
-          <t>2026-03-20T07:02:39</t>
+          <t>2026-03-20T13:46:30</t>
         </is>
       </c>
     </row>
@@ -6423,7 +6423,7 @@
       </c>
       <c r="I131" t="inlineStr">
         <is>
-          <t>2026-03-20T07:02:39</t>
+          <t>2026-03-20T13:46:30</t>
         </is>
       </c>
     </row>
@@ -6460,7 +6460,7 @@
       </c>
       <c r="I132" t="inlineStr">
         <is>
-          <t>2026-03-20T07:02:39</t>
+          <t>2026-03-20T13:46:30</t>
         </is>
       </c>
     </row>
@@ -6487,17 +6487,17 @@
         <v>1</v>
       </c>
       <c r="F133" t="n">
-        <v>4071683.614561614</v>
+        <v>4087391.335876007</v>
       </c>
       <c r="G133" t="n">
-        <v>247035.6145616136</v>
+        <v>262743.3358760066</v>
       </c>
       <c r="H133" t="n">
-        <v>6.459041840232452</v>
+        <v>6.869739015878236</v>
       </c>
       <c r="I133" t="inlineStr">
         <is>
-          <t>2026-03-20T07:02:39</t>
+          <t>2026-03-20T13:46:30</t>
         </is>
       </c>
     </row>
@@ -6524,17 +6524,17 @@
         <v>1</v>
       </c>
       <c r="F134" t="n">
-        <v>3641589.341643294</v>
+        <v>3711115.026073027</v>
       </c>
       <c r="G134" t="n">
-        <v>2170817.341643294</v>
+        <v>2240343.026073027</v>
       </c>
       <c r="H134" t="n">
-        <v>147.5971354936927</v>
+        <v>152.3242913295213</v>
       </c>
       <c r="I134" t="inlineStr">
         <is>
-          <t>2026-03-20T07:02:39</t>
+          <t>2026-03-20T13:46:30</t>
         </is>
       </c>
     </row>
@@ -6561,17 +6561,17 @@
         <v>1</v>
       </c>
       <c r="F135" t="n">
-        <v>2971420.173610602</v>
+        <v>2945895.015193854</v>
       </c>
       <c r="G135" t="n">
-        <v>-219223.8263893984</v>
+        <v>-244748.9848061465</v>
       </c>
       <c r="H135" t="n">
-        <v>-6.870833173158723</v>
+        <v>-7.6708333742701</v>
       </c>
       <c r="I135" t="inlineStr">
         <is>
-          <t>2026-03-20T07:02:39</t>
+          <t>2026-03-20T13:46:30</t>
         </is>
       </c>
     </row>
@@ -6608,7 +6608,7 @@
       </c>
       <c r="I136" t="inlineStr">
         <is>
-          <t>2026-03-20T07:02:39</t>
+          <t>2026-03-20T13:46:30</t>
         </is>
       </c>
     </row>
@@ -6645,7 +6645,7 @@
       </c>
       <c r="I137" t="inlineStr">
         <is>
-          <t>2026-03-20T07:02:39</t>
+          <t>2026-03-20T13:46:30</t>
         </is>
       </c>
     </row>
@@ -6682,7 +6682,7 @@
       </c>
       <c r="I138" t="inlineStr">
         <is>
-          <t>2026-03-20T07:02:39</t>
+          <t>2026-03-20T13:46:30</t>
         </is>
       </c>
     </row>
@@ -6719,7 +6719,7 @@
       </c>
       <c r="I139" t="inlineStr">
         <is>
-          <t>2026-03-20T07:02:39</t>
+          <t>2026-03-20T13:46:30</t>
         </is>
       </c>
     </row>
@@ -6756,7 +6756,7 @@
       </c>
       <c r="I140" t="inlineStr">
         <is>
-          <t>2026-03-20T07:02:39</t>
+          <t>2026-03-20T13:46:30</t>
         </is>
       </c>
     </row>
@@ -6783,17 +6783,17 @@
         <v>1</v>
       </c>
       <c r="F141" t="n">
-        <v>2172791.30897373</v>
+        <v>2162693.444105566</v>
       </c>
       <c r="G141" t="n">
-        <v>108801.3089737301</v>
+        <v>98703.44410556601</v>
       </c>
       <c r="H141" t="n">
-        <v>5.271406788488806</v>
+        <v>4.782166779178485</v>
       </c>
       <c r="I141" t="inlineStr">
         <is>
-          <t>2026-03-20T07:02:39</t>
+          <t>2026-03-20T13:46:30</t>
         </is>
       </c>
     </row>
@@ -6830,7 +6830,7 @@
       </c>
       <c r="I142" t="inlineStr">
         <is>
-          <t>2026-03-20T07:02:39</t>
+          <t>2026-03-20T13:46:30</t>
         </is>
       </c>
     </row>
@@ -6867,7 +6867,7 @@
       </c>
       <c r="I143" t="inlineStr">
         <is>
-          <t>2026-03-20T07:02:39</t>
+          <t>2026-03-20T13:46:30</t>
         </is>
       </c>
     </row>
@@ -6904,7 +6904,7 @@
       </c>
       <c r="I144" t="inlineStr">
         <is>
-          <t>2026-03-20T07:02:39</t>
+          <t>2026-03-20T13:46:30</t>
         </is>
       </c>
     </row>
@@ -6916,11 +6916,11 @@
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>스타 벌크 캐리어스</t>
+          <t>하나금융지주</t>
         </is>
       </c>
       <c r="C145" t="n">
-        <v>50</v>
+        <v>15</v>
       </c>
       <c r="D145" t="inlineStr">
         <is>
@@ -6931,17 +6931,17 @@
         <v>1</v>
       </c>
       <c r="F145" t="n">
-        <v>1700181.21356247</v>
+        <v>1698000</v>
       </c>
       <c r="G145" t="n">
-        <v>385828.2135624706</v>
+        <v>15500</v>
       </c>
       <c r="H145" t="n">
-        <v>29.35499166224529</v>
+        <v>0.9212481426448738</v>
       </c>
       <c r="I145" t="inlineStr">
         <is>
-          <t>2026-03-20T07:02:39</t>
+          <t>2026-03-20T13:46:30</t>
         </is>
       </c>
     </row>
@@ -6953,11 +6953,11 @@
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>하나금융지주</t>
+          <t>스타 벌크 캐리어스</t>
         </is>
       </c>
       <c r="C146" t="n">
-        <v>15</v>
+        <v>50</v>
       </c>
       <c r="D146" t="inlineStr">
         <is>
@@ -6968,17 +6968,17 @@
         <v>1</v>
       </c>
       <c r="F146" t="n">
-        <v>1698000</v>
+        <v>1691579.345794907</v>
       </c>
       <c r="G146" t="n">
-        <v>15500</v>
+        <v>377226.3457949075</v>
       </c>
       <c r="H146" t="n">
-        <v>0.9212481426448738</v>
+        <v>28.7005352287329</v>
       </c>
       <c r="I146" t="inlineStr">
         <is>
-          <t>2026-03-20T07:02:39</t>
+          <t>2026-03-20T13:46:30</t>
         </is>
       </c>
     </row>
@@ -7005,17 +7005,17 @@
         <v>1</v>
       </c>
       <c r="F147" t="n">
-        <v>1678130.517499804</v>
+        <v>1688243.356776953</v>
       </c>
       <c r="G147" t="n">
-        <v>-16325.48250019504</v>
+        <v>-6212.643223046791</v>
       </c>
       <c r="H147" t="n">
-        <v>-0.9634645278599764</v>
+        <v>-0.366645296369265</v>
       </c>
       <c r="I147" t="inlineStr">
         <is>
-          <t>2026-03-20T07:02:39</t>
+          <t>2026-03-20T13:46:30</t>
         </is>
       </c>
     </row>
@@ -7052,7 +7052,7 @@
       </c>
       <c r="I148" t="inlineStr">
         <is>
-          <t>2026-03-20T07:02:39</t>
+          <t>2026-03-20T13:46:30</t>
         </is>
       </c>
     </row>
@@ -7089,7 +7089,7 @@
       </c>
       <c r="I149" t="inlineStr">
         <is>
-          <t>2026-03-20T07:02:39</t>
+          <t>2026-03-20T13:46:30</t>
         </is>
       </c>
     </row>
@@ -7126,7 +7126,7 @@
       </c>
       <c r="I150" t="inlineStr">
         <is>
-          <t>2026-03-20T07:02:39</t>
+          <t>2026-03-20T13:46:30</t>
         </is>
       </c>
     </row>
@@ -7138,11 +7138,11 @@
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>클리블랜드 클리프스</t>
+          <t>하프니아</t>
         </is>
       </c>
       <c r="C151" t="n">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="D151" t="inlineStr">
         <is>
@@ -7153,17 +7153,17 @@
         <v>1</v>
       </c>
       <c r="F151" t="n">
-        <v>856598.1687739864</v>
+        <v>852110.1831788942</v>
       </c>
       <c r="G151" t="n">
-        <v>-159456.8312260136</v>
+        <v>226379.1831788942</v>
       </c>
       <c r="H151" t="n">
-        <v>-15.69372044092235</v>
+        <v>36.17835510449286</v>
       </c>
       <c r="I151" t="inlineStr">
         <is>
-          <t>2026-03-20T07:02:39</t>
+          <t>2026-03-20T13:46:30</t>
         </is>
       </c>
     </row>
@@ -7175,11 +7175,11 @@
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>하프니아</t>
+          <t>클리블랜드 클리프스</t>
         </is>
       </c>
       <c r="C152" t="n">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="D152" t="inlineStr">
         <is>
@@ -7190,17 +7190,17 @@
         <v>1</v>
       </c>
       <c r="F152" t="n">
-        <v>853306.9945554808</v>
+        <v>846649.8739409866</v>
       </c>
       <c r="G152" t="n">
-        <v>227575.9945554808</v>
+        <v>-169405.1260590134</v>
       </c>
       <c r="H152" t="n">
-        <v>36.36962121989813</v>
+        <v>-16.67283031519095</v>
       </c>
       <c r="I152" t="inlineStr">
         <is>
-          <t>2026-03-20T07:02:39</t>
+          <t>2026-03-20T13:46:30</t>
         </is>
       </c>
     </row>
@@ -7227,17 +7227,17 @@
         <v>1</v>
       </c>
       <c r="F153" t="n">
-        <v>796639.2884175777</v>
+        <v>796564.4163726568</v>
       </c>
       <c r="G153" t="n">
-        <v>18048.28841757774</v>
+        <v>17973.41637265682</v>
       </c>
       <c r="H153" t="n">
-        <v>2.318070516815343</v>
+        <v>2.308454165621851</v>
       </c>
       <c r="I153" t="inlineStr">
         <is>
-          <t>2026-03-20T07:02:39</t>
+          <t>2026-03-20T13:46:30</t>
         </is>
       </c>
     </row>
@@ -7370,7 +7370,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>2026-03-20T07:02:39</t>
+          <t>2026-03-20T13:46:30</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: portfolio snapshot 2026-03-20 (2026-03-20T15:46:48)
</commit_message>
<xml_diff>
--- a/portfolio_auto.xlsx
+++ b/portfolio_auto.xlsx
@@ -486,13 +486,13 @@
         <v>1</v>
       </c>
       <c r="E2" t="n">
-        <v>13768999.19239014</v>
+        <v>13553578.62304688</v>
       </c>
       <c r="F2" t="n">
-        <v>1662450.192390148</v>
+        <v>1447029.623046879</v>
       </c>
       <c r="G2" t="n">
-        <v>13.73182557961107</v>
+        <v>11.95245336261291</v>
       </c>
     </row>
     <row r="3">
@@ -513,13 +513,13 @@
         <v>1</v>
       </c>
       <c r="E3" t="n">
-        <v>10644645.51107842</v>
+        <v>10351433.71453537</v>
       </c>
       <c r="F3" t="n">
-        <v>-187369.4889215864</v>
+        <v>-480581.2854646351</v>
       </c>
       <c r="G3" t="n">
-        <v>-1.729775013435509</v>
+        <v>-4.436674851951692</v>
       </c>
     </row>
     <row r="4">
@@ -567,13 +567,13 @@
         <v>1</v>
       </c>
       <c r="E5" t="n">
-        <v>8410212.452697754</v>
+        <v>8453409.11431564</v>
       </c>
       <c r="F5" t="n">
-        <v>3980348.452697754</v>
+        <v>4023545.11431564</v>
       </c>
       <c r="G5" t="n">
-        <v>89.85261066023142</v>
+        <v>90.82773453802736</v>
       </c>
     </row>
     <row r="6">
@@ -594,13 +594,13 @@
         <v>1</v>
       </c>
       <c r="E6" t="n">
-        <v>8156965.818628304</v>
+        <v>8081063.113214018</v>
       </c>
       <c r="F6" t="n">
-        <v>1706614.818628304</v>
+        <v>1630712.113214018</v>
       </c>
       <c r="G6" t="n">
-        <v>26.45770468348627</v>
+        <v>25.28098258860669</v>
       </c>
     </row>
     <row r="7">
@@ -648,13 +648,13 @@
         <v>1</v>
       </c>
       <c r="E8" t="n">
-        <v>7175093.959923077</v>
+        <v>7074115.140040115</v>
       </c>
       <c r="F8" t="n">
-        <v>3047859.959923078</v>
+        <v>2946881.140040115</v>
       </c>
       <c r="G8" t="n">
-        <v>73.84752015328131</v>
+        <v>71.40087380652794</v>
       </c>
     </row>
     <row r="9">
@@ -675,13 +675,13 @@
         <v>1</v>
       </c>
       <c r="E9" t="n">
-        <v>7014955.722778145</v>
+        <v>6886743.840087891</v>
       </c>
       <c r="F9" t="n">
-        <v>3107747.722778145</v>
+        <v>2979535.840087891</v>
       </c>
       <c r="G9" t="n">
-        <v>79.53883496292353</v>
+        <v>76.25741552760668</v>
       </c>
     </row>
     <row r="10">
@@ -702,13 +702,13 @@
         <v>1</v>
       </c>
       <c r="E10" t="n">
-        <v>6301685.50906603</v>
+        <v>5996448.754211426</v>
       </c>
       <c r="F10" t="n">
-        <v>70466.50906603131</v>
+        <v>-234770.2457885733</v>
       </c>
       <c r="G10" t="n">
-        <v>1.130862341157185</v>
+        <v>-3.767645556809564</v>
       </c>
     </row>
     <row r="11">
@@ -756,13 +756,13 @@
         <v>1</v>
       </c>
       <c r="E12" t="n">
-        <v>5264173.858361721</v>
+        <v>5211036.802851856</v>
       </c>
       <c r="F12" t="n">
-        <v>1539628.858361721</v>
+        <v>1486491.802851856</v>
       </c>
       <c r="G12" t="n">
-        <v>41.33736760763318</v>
+        <v>39.91069520845783</v>
       </c>
     </row>
     <row r="13">
@@ -783,13 +783,13 @@
         <v>1</v>
       </c>
       <c r="E13" t="n">
-        <v>5156523.305831412</v>
+        <v>5179494.129107101</v>
       </c>
       <c r="F13" t="n">
-        <v>1846515.305831412</v>
+        <v>1869486.129107101</v>
       </c>
       <c r="G13" t="n">
-        <v>55.78582607146001</v>
+        <v>56.47980697046958</v>
       </c>
     </row>
     <row r="14">
@@ -837,13 +837,13 @@
         <v>1</v>
       </c>
       <c r="E15" t="n">
-        <v>4511875.769468229</v>
+        <v>4596307.895957222</v>
       </c>
       <c r="F15" t="n">
-        <v>2255515.769468229</v>
+        <v>2339947.895957222</v>
       </c>
       <c r="G15" t="n">
-        <v>99.96258440444917</v>
+        <v>103.704546081176</v>
       </c>
     </row>
     <row r="16">
@@ -945,13 +945,13 @@
         <v>1</v>
       </c>
       <c r="E19" t="n">
-        <v>4087391.335876007</v>
+        <v>4052048.962918622</v>
       </c>
       <c r="F19" t="n">
-        <v>262743.3358760066</v>
+        <v>227400.9629186224</v>
       </c>
       <c r="G19" t="n">
-        <v>6.869739015878236</v>
+        <v>5.94567037067522</v>
       </c>
     </row>
     <row r="20">
@@ -972,13 +972,13 @@
         <v>1</v>
       </c>
       <c r="E20" t="n">
-        <v>3711115.026073027</v>
+        <v>3596373.331896178</v>
       </c>
       <c r="F20" t="n">
-        <v>2240343.026073027</v>
+        <v>2125601.331896178</v>
       </c>
       <c r="G20" t="n">
-        <v>152.3242913295213</v>
+        <v>144.5228309959789</v>
       </c>
     </row>
     <row r="21">
@@ -999,13 +999,13 @@
         <v>1</v>
       </c>
       <c r="E21" t="n">
-        <v>2945895.015193854</v>
+        <v>2959763.281021703</v>
       </c>
       <c r="F21" t="n">
-        <v>-244748.9848061465</v>
+        <v>-230880.718978297</v>
       </c>
       <c r="G21" t="n">
-        <v>-7.6708333742701</v>
+        <v>-7.236179247145621</v>
       </c>
     </row>
     <row r="22">
@@ -1161,13 +1161,13 @@
         <v>1</v>
       </c>
       <c r="E27" t="n">
-        <v>2162693.444105566</v>
+        <v>2176561.162089184</v>
       </c>
       <c r="F27" t="n">
-        <v>98703.44410556601</v>
+        <v>112571.1620891844</v>
       </c>
       <c r="G27" t="n">
-        <v>4.782166779178485</v>
+        <v>5.45405559567558</v>
       </c>
     </row>
     <row r="28">
@@ -1254,11 +1254,11 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>스타 벌크 캐리어스</t>
+          <t>하나금융지주</t>
         </is>
       </c>
       <c r="B31" t="n">
-        <v>50</v>
+        <v>15</v>
       </c>
       <c r="C31" t="inlineStr">
         <is>
@@ -1269,23 +1269,23 @@
         <v>1</v>
       </c>
       <c r="E31" t="n">
-        <v>1691579.345794907</v>
+        <v>1698000</v>
       </c>
       <c r="F31" t="n">
-        <v>377226.3457949075</v>
+        <v>15500</v>
       </c>
       <c r="G31" t="n">
-        <v>28.7005352287329</v>
+        <v>0.9212481426448738</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>하나금융지주</t>
+          <t>스타 벌크 캐리어스</t>
         </is>
       </c>
       <c r="B32" t="n">
-        <v>15</v>
+        <v>50</v>
       </c>
       <c r="C32" t="inlineStr">
         <is>
@@ -1296,13 +1296,13 @@
         <v>1</v>
       </c>
       <c r="E32" t="n">
-        <v>1698000</v>
+        <v>1696441.320678405</v>
       </c>
       <c r="F32" t="n">
-        <v>15500</v>
+        <v>382088.3206784062</v>
       </c>
       <c r="G32" t="n">
-        <v>0.9212481426448738</v>
+        <v>29.07044916231837</v>
       </c>
     </row>
     <row r="33">
@@ -1323,13 +1323,13 @@
         <v>1</v>
       </c>
       <c r="E33" t="n">
-        <v>1688243.356776953</v>
+        <v>1683366.447431445</v>
       </c>
       <c r="F33" t="n">
-        <v>-6212.643223046791</v>
+        <v>-11089.55256855441</v>
       </c>
       <c r="G33" t="n">
-        <v>-0.366645296369265</v>
+        <v>-0.6544609342794628</v>
       </c>
     </row>
     <row r="34">
@@ -1416,11 +1416,11 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>클리블랜드 클리프스</t>
+          <t>하프니아</t>
         </is>
       </c>
       <c r="B37" t="n">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="C37" t="inlineStr">
         <is>
@@ -1431,23 +1431,23 @@
         <v>1</v>
       </c>
       <c r="E37" t="n">
-        <v>846649.8739409866</v>
+        <v>848519.8631833494</v>
       </c>
       <c r="F37" t="n">
-        <v>-169405.1260590134</v>
+        <v>222788.8631833494</v>
       </c>
       <c r="G37" t="n">
-        <v>-16.67283031519095</v>
+        <v>35.60457499841775</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>하프니아</t>
+          <t>클리블랜드 클리프스</t>
         </is>
       </c>
       <c r="B38" t="n">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="C38" t="inlineStr">
         <is>
@@ -1458,13 +1458,13 @@
         <v>1</v>
       </c>
       <c r="E38" t="n">
-        <v>852110.1831788942</v>
+        <v>833036.4441346284</v>
       </c>
       <c r="F38" t="n">
-        <v>226379.1831788942</v>
+        <v>-183018.5558653716</v>
       </c>
       <c r="G38" t="n">
-        <v>36.17835510449286</v>
+        <v>-18.01266229341636</v>
       </c>
     </row>
     <row r="39">
@@ -1485,13 +1485,13 @@
         <v>1</v>
       </c>
       <c r="E39" t="n">
-        <v>796564.4163726568</v>
+        <v>798210.0491355956</v>
       </c>
       <c r="F39" t="n">
-        <v>17973.41637265682</v>
+        <v>19619.04913559556</v>
       </c>
       <c r="G39" t="n">
-        <v>2.308454165621851</v>
+        <v>2.519814528500273</v>
       </c>
     </row>
   </sheetData>
@@ -1549,7 +1549,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2026-03-20T13:46:30</t>
+          <t>2026-03-20T15:46:48</t>
         </is>
       </c>
       <c r="E2" t="n">
@@ -5858,17 +5858,17 @@
         <v>1</v>
       </c>
       <c r="F116" t="n">
-        <v>13768999.19239014</v>
+        <v>13553578.62304688</v>
       </c>
       <c r="G116" t="n">
-        <v>1662450.192390148</v>
+        <v>1447029.623046879</v>
       </c>
       <c r="H116" t="n">
-        <v>13.73182557961107</v>
+        <v>11.95245336261291</v>
       </c>
       <c r="I116" t="inlineStr">
         <is>
-          <t>2026-03-20T13:46:30</t>
+          <t>2026-03-20T15:46:48</t>
         </is>
       </c>
     </row>
@@ -5895,17 +5895,17 @@
         <v>1</v>
       </c>
       <c r="F117" t="n">
-        <v>10644645.51107842</v>
+        <v>10351433.71453537</v>
       </c>
       <c r="G117" t="n">
-        <v>-187369.4889215864</v>
+        <v>-480581.2854646351</v>
       </c>
       <c r="H117" t="n">
-        <v>-1.729775013435509</v>
+        <v>-4.436674851951692</v>
       </c>
       <c r="I117" t="inlineStr">
         <is>
-          <t>2026-03-20T13:46:30</t>
+          <t>2026-03-20T15:46:48</t>
         </is>
       </c>
     </row>
@@ -5942,7 +5942,7 @@
       </c>
       <c r="I118" t="inlineStr">
         <is>
-          <t>2026-03-20T13:46:30</t>
+          <t>2026-03-20T15:46:48</t>
         </is>
       </c>
     </row>
@@ -5969,17 +5969,17 @@
         <v>1</v>
       </c>
       <c r="F119" t="n">
-        <v>8410212.452697754</v>
+        <v>8453409.11431564</v>
       </c>
       <c r="G119" t="n">
-        <v>3980348.452697754</v>
+        <v>4023545.11431564</v>
       </c>
       <c r="H119" t="n">
-        <v>89.85261066023142</v>
+        <v>90.82773453802736</v>
       </c>
       <c r="I119" t="inlineStr">
         <is>
-          <t>2026-03-20T13:46:30</t>
+          <t>2026-03-20T15:46:48</t>
         </is>
       </c>
     </row>
@@ -6006,17 +6006,17 @@
         <v>1</v>
       </c>
       <c r="F120" t="n">
-        <v>8156965.818628304</v>
+        <v>8081063.113214018</v>
       </c>
       <c r="G120" t="n">
-        <v>1706614.818628304</v>
+        <v>1630712.113214018</v>
       </c>
       <c r="H120" t="n">
-        <v>26.45770468348627</v>
+        <v>25.28098258860669</v>
       </c>
       <c r="I120" t="inlineStr">
         <is>
-          <t>2026-03-20T13:46:30</t>
+          <t>2026-03-20T15:46:48</t>
         </is>
       </c>
     </row>
@@ -6053,7 +6053,7 @@
       </c>
       <c r="I121" t="inlineStr">
         <is>
-          <t>2026-03-20T13:46:30</t>
+          <t>2026-03-20T15:46:48</t>
         </is>
       </c>
     </row>
@@ -6080,17 +6080,17 @@
         <v>1</v>
       </c>
       <c r="F122" t="n">
-        <v>7175093.959923077</v>
+        <v>7074115.140040115</v>
       </c>
       <c r="G122" t="n">
-        <v>3047859.959923078</v>
+        <v>2946881.140040115</v>
       </c>
       <c r="H122" t="n">
-        <v>73.84752015328131</v>
+        <v>71.40087380652794</v>
       </c>
       <c r="I122" t="inlineStr">
         <is>
-          <t>2026-03-20T13:46:30</t>
+          <t>2026-03-20T15:46:48</t>
         </is>
       </c>
     </row>
@@ -6117,17 +6117,17 @@
         <v>1</v>
       </c>
       <c r="F123" t="n">
-        <v>7014955.722778145</v>
+        <v>6886743.840087891</v>
       </c>
       <c r="G123" t="n">
-        <v>3107747.722778145</v>
+        <v>2979535.840087891</v>
       </c>
       <c r="H123" t="n">
-        <v>79.53883496292353</v>
+        <v>76.25741552760668</v>
       </c>
       <c r="I123" t="inlineStr">
         <is>
-          <t>2026-03-20T13:46:30</t>
+          <t>2026-03-20T15:46:48</t>
         </is>
       </c>
     </row>
@@ -6154,17 +6154,17 @@
         <v>1</v>
       </c>
       <c r="F124" t="n">
-        <v>6301685.50906603</v>
+        <v>5996448.754211426</v>
       </c>
       <c r="G124" t="n">
-        <v>70466.50906603131</v>
+        <v>-234770.2457885733</v>
       </c>
       <c r="H124" t="n">
-        <v>1.130862341157185</v>
+        <v>-3.767645556809564</v>
       </c>
       <c r="I124" t="inlineStr">
         <is>
-          <t>2026-03-20T13:46:30</t>
+          <t>2026-03-20T15:46:48</t>
         </is>
       </c>
     </row>
@@ -6201,7 +6201,7 @@
       </c>
       <c r="I125" t="inlineStr">
         <is>
-          <t>2026-03-20T13:46:30</t>
+          <t>2026-03-20T15:46:48</t>
         </is>
       </c>
     </row>
@@ -6228,17 +6228,17 @@
         <v>1</v>
       </c>
       <c r="F126" t="n">
-        <v>5264173.858361721</v>
+        <v>5211036.802851856</v>
       </c>
       <c r="G126" t="n">
-        <v>1539628.858361721</v>
+        <v>1486491.802851856</v>
       </c>
       <c r="H126" t="n">
-        <v>41.33736760763318</v>
+        <v>39.91069520845783</v>
       </c>
       <c r="I126" t="inlineStr">
         <is>
-          <t>2026-03-20T13:46:30</t>
+          <t>2026-03-20T15:46:48</t>
         </is>
       </c>
     </row>
@@ -6265,17 +6265,17 @@
         <v>1</v>
       </c>
       <c r="F127" t="n">
-        <v>5156523.305831412</v>
+        <v>5179494.129107101</v>
       </c>
       <c r="G127" t="n">
-        <v>1846515.305831412</v>
+        <v>1869486.129107101</v>
       </c>
       <c r="H127" t="n">
-        <v>55.78582607146001</v>
+        <v>56.47980697046958</v>
       </c>
       <c r="I127" t="inlineStr">
         <is>
-          <t>2026-03-20T13:46:30</t>
+          <t>2026-03-20T15:46:48</t>
         </is>
       </c>
     </row>
@@ -6312,7 +6312,7 @@
       </c>
       <c r="I128" t="inlineStr">
         <is>
-          <t>2026-03-20T13:46:30</t>
+          <t>2026-03-20T15:46:48</t>
         </is>
       </c>
     </row>
@@ -6339,17 +6339,17 @@
         <v>1</v>
       </c>
       <c r="F129" t="n">
-        <v>4511875.769468229</v>
+        <v>4596307.895957222</v>
       </c>
       <c r="G129" t="n">
-        <v>2255515.769468229</v>
+        <v>2339947.895957222</v>
       </c>
       <c r="H129" t="n">
-        <v>99.96258440444917</v>
+        <v>103.704546081176</v>
       </c>
       <c r="I129" t="inlineStr">
         <is>
-          <t>2026-03-20T13:46:30</t>
+          <t>2026-03-20T15:46:48</t>
         </is>
       </c>
     </row>
@@ -6386,7 +6386,7 @@
       </c>
       <c r="I130" t="inlineStr">
         <is>
-          <t>2026-03-20T13:46:30</t>
+          <t>2026-03-20T15:46:48</t>
         </is>
       </c>
     </row>
@@ -6423,7 +6423,7 @@
       </c>
       <c r="I131" t="inlineStr">
         <is>
-          <t>2026-03-20T13:46:30</t>
+          <t>2026-03-20T15:46:48</t>
         </is>
       </c>
     </row>
@@ -6460,7 +6460,7 @@
       </c>
       <c r="I132" t="inlineStr">
         <is>
-          <t>2026-03-20T13:46:30</t>
+          <t>2026-03-20T15:46:48</t>
         </is>
       </c>
     </row>
@@ -6487,17 +6487,17 @@
         <v>1</v>
       </c>
       <c r="F133" t="n">
-        <v>4087391.335876007</v>
+        <v>4052048.962918622</v>
       </c>
       <c r="G133" t="n">
-        <v>262743.3358760066</v>
+        <v>227400.9629186224</v>
       </c>
       <c r="H133" t="n">
-        <v>6.869739015878236</v>
+        <v>5.94567037067522</v>
       </c>
       <c r="I133" t="inlineStr">
         <is>
-          <t>2026-03-20T13:46:30</t>
+          <t>2026-03-20T15:46:48</t>
         </is>
       </c>
     </row>
@@ -6524,17 +6524,17 @@
         <v>1</v>
       </c>
       <c r="F134" t="n">
-        <v>3711115.026073027</v>
+        <v>3596373.331896178</v>
       </c>
       <c r="G134" t="n">
-        <v>2240343.026073027</v>
+        <v>2125601.331896178</v>
       </c>
       <c r="H134" t="n">
-        <v>152.3242913295213</v>
+        <v>144.5228309959789</v>
       </c>
       <c r="I134" t="inlineStr">
         <is>
-          <t>2026-03-20T13:46:30</t>
+          <t>2026-03-20T15:46:48</t>
         </is>
       </c>
     </row>
@@ -6561,17 +6561,17 @@
         <v>1</v>
       </c>
       <c r="F135" t="n">
-        <v>2945895.015193854</v>
+        <v>2959763.281021703</v>
       </c>
       <c r="G135" t="n">
-        <v>-244748.9848061465</v>
+        <v>-230880.718978297</v>
       </c>
       <c r="H135" t="n">
-        <v>-7.6708333742701</v>
+        <v>-7.236179247145621</v>
       </c>
       <c r="I135" t="inlineStr">
         <is>
-          <t>2026-03-20T13:46:30</t>
+          <t>2026-03-20T15:46:48</t>
         </is>
       </c>
     </row>
@@ -6608,7 +6608,7 @@
       </c>
       <c r="I136" t="inlineStr">
         <is>
-          <t>2026-03-20T13:46:30</t>
+          <t>2026-03-20T15:46:48</t>
         </is>
       </c>
     </row>
@@ -6645,7 +6645,7 @@
       </c>
       <c r="I137" t="inlineStr">
         <is>
-          <t>2026-03-20T13:46:30</t>
+          <t>2026-03-20T15:46:48</t>
         </is>
       </c>
     </row>
@@ -6682,7 +6682,7 @@
       </c>
       <c r="I138" t="inlineStr">
         <is>
-          <t>2026-03-20T13:46:30</t>
+          <t>2026-03-20T15:46:48</t>
         </is>
       </c>
     </row>
@@ -6719,7 +6719,7 @@
       </c>
       <c r="I139" t="inlineStr">
         <is>
-          <t>2026-03-20T13:46:30</t>
+          <t>2026-03-20T15:46:48</t>
         </is>
       </c>
     </row>
@@ -6756,7 +6756,7 @@
       </c>
       <c r="I140" t="inlineStr">
         <is>
-          <t>2026-03-20T13:46:30</t>
+          <t>2026-03-20T15:46:48</t>
         </is>
       </c>
     </row>
@@ -6783,17 +6783,17 @@
         <v>1</v>
       </c>
       <c r="F141" t="n">
-        <v>2162693.444105566</v>
+        <v>2176561.162089184</v>
       </c>
       <c r="G141" t="n">
-        <v>98703.44410556601</v>
+        <v>112571.1620891844</v>
       </c>
       <c r="H141" t="n">
-        <v>4.782166779178485</v>
+        <v>5.45405559567558</v>
       </c>
       <c r="I141" t="inlineStr">
         <is>
-          <t>2026-03-20T13:46:30</t>
+          <t>2026-03-20T15:46:48</t>
         </is>
       </c>
     </row>
@@ -6830,7 +6830,7 @@
       </c>
       <c r="I142" t="inlineStr">
         <is>
-          <t>2026-03-20T13:46:30</t>
+          <t>2026-03-20T15:46:48</t>
         </is>
       </c>
     </row>
@@ -6867,7 +6867,7 @@
       </c>
       <c r="I143" t="inlineStr">
         <is>
-          <t>2026-03-20T13:46:30</t>
+          <t>2026-03-20T15:46:48</t>
         </is>
       </c>
     </row>
@@ -6904,7 +6904,7 @@
       </c>
       <c r="I144" t="inlineStr">
         <is>
-          <t>2026-03-20T13:46:30</t>
+          <t>2026-03-20T15:46:48</t>
         </is>
       </c>
     </row>
@@ -6941,7 +6941,7 @@
       </c>
       <c r="I145" t="inlineStr">
         <is>
-          <t>2026-03-20T13:46:30</t>
+          <t>2026-03-20T15:46:48</t>
         </is>
       </c>
     </row>
@@ -6968,17 +6968,17 @@
         <v>1</v>
       </c>
       <c r="F146" t="n">
-        <v>1691579.345794907</v>
+        <v>1696441.320678405</v>
       </c>
       <c r="G146" t="n">
-        <v>377226.3457949075</v>
+        <v>382088.3206784062</v>
       </c>
       <c r="H146" t="n">
-        <v>28.7005352287329</v>
+        <v>29.07044916231837</v>
       </c>
       <c r="I146" t="inlineStr">
         <is>
-          <t>2026-03-20T13:46:30</t>
+          <t>2026-03-20T15:46:48</t>
         </is>
       </c>
     </row>
@@ -7005,17 +7005,17 @@
         <v>1</v>
       </c>
       <c r="F147" t="n">
-        <v>1688243.356776953</v>
+        <v>1683366.447431445</v>
       </c>
       <c r="G147" t="n">
-        <v>-6212.643223046791</v>
+        <v>-11089.55256855441</v>
       </c>
       <c r="H147" t="n">
-        <v>-0.366645296369265</v>
+        <v>-0.6544609342794628</v>
       </c>
       <c r="I147" t="inlineStr">
         <is>
-          <t>2026-03-20T13:46:30</t>
+          <t>2026-03-20T15:46:48</t>
         </is>
       </c>
     </row>
@@ -7052,7 +7052,7 @@
       </c>
       <c r="I148" t="inlineStr">
         <is>
-          <t>2026-03-20T13:46:30</t>
+          <t>2026-03-20T15:46:48</t>
         </is>
       </c>
     </row>
@@ -7089,7 +7089,7 @@
       </c>
       <c r="I149" t="inlineStr">
         <is>
-          <t>2026-03-20T13:46:30</t>
+          <t>2026-03-20T15:46:48</t>
         </is>
       </c>
     </row>
@@ -7126,7 +7126,7 @@
       </c>
       <c r="I150" t="inlineStr">
         <is>
-          <t>2026-03-20T13:46:30</t>
+          <t>2026-03-20T15:46:48</t>
         </is>
       </c>
     </row>
@@ -7153,17 +7153,17 @@
         <v>1</v>
       </c>
       <c r="F151" t="n">
-        <v>852110.1831788942</v>
+        <v>848519.8631833494</v>
       </c>
       <c r="G151" t="n">
-        <v>226379.1831788942</v>
+        <v>222788.8631833494</v>
       </c>
       <c r="H151" t="n">
-        <v>36.17835510449286</v>
+        <v>35.60457499841775</v>
       </c>
       <c r="I151" t="inlineStr">
         <is>
-          <t>2026-03-20T13:46:30</t>
+          <t>2026-03-20T15:46:48</t>
         </is>
       </c>
     </row>
@@ -7190,17 +7190,17 @@
         <v>1</v>
       </c>
       <c r="F152" t="n">
-        <v>846649.8739409866</v>
+        <v>833036.4441346284</v>
       </c>
       <c r="G152" t="n">
-        <v>-169405.1260590134</v>
+        <v>-183018.5558653716</v>
       </c>
       <c r="H152" t="n">
-        <v>-16.67283031519095</v>
+        <v>-18.01266229341636</v>
       </c>
       <c r="I152" t="inlineStr">
         <is>
-          <t>2026-03-20T13:46:30</t>
+          <t>2026-03-20T15:46:48</t>
         </is>
       </c>
     </row>
@@ -7227,17 +7227,17 @@
         <v>1</v>
       </c>
       <c r="F153" t="n">
-        <v>796564.4163726568</v>
+        <v>798210.0491355956</v>
       </c>
       <c r="G153" t="n">
-        <v>17973.41637265682</v>
+        <v>19619.04913559556</v>
       </c>
       <c r="H153" t="n">
-        <v>2.308454165621851</v>
+        <v>2.519814528500273</v>
       </c>
       <c r="I153" t="inlineStr">
         <is>
-          <t>2026-03-20T13:46:30</t>
+          <t>2026-03-20T15:46:48</t>
         </is>
       </c>
     </row>
@@ -7370,7 +7370,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>2026-03-20T13:46:30</t>
+          <t>2026-03-20T15:46:48</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: portfolio snapshot 2026-03-20 (2026-03-20T15:47:06)
</commit_message>
<xml_diff>
--- a/portfolio_auto.xlsx
+++ b/portfolio_auto.xlsx
@@ -1549,7 +1549,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2026-03-20T15:46:48</t>
+          <t>2026-03-20T15:47:06</t>
         </is>
       </c>
       <c r="E2" t="n">
@@ -5868,7 +5868,7 @@
       </c>
       <c r="I116" t="inlineStr">
         <is>
-          <t>2026-03-20T15:46:48</t>
+          <t>2026-03-20T15:47:06</t>
         </is>
       </c>
     </row>
@@ -5905,7 +5905,7 @@
       </c>
       <c r="I117" t="inlineStr">
         <is>
-          <t>2026-03-20T15:46:48</t>
+          <t>2026-03-20T15:47:06</t>
         </is>
       </c>
     </row>
@@ -5942,7 +5942,7 @@
       </c>
       <c r="I118" t="inlineStr">
         <is>
-          <t>2026-03-20T15:46:48</t>
+          <t>2026-03-20T15:47:06</t>
         </is>
       </c>
     </row>
@@ -5979,7 +5979,7 @@
       </c>
       <c r="I119" t="inlineStr">
         <is>
-          <t>2026-03-20T15:46:48</t>
+          <t>2026-03-20T15:47:06</t>
         </is>
       </c>
     </row>
@@ -6016,7 +6016,7 @@
       </c>
       <c r="I120" t="inlineStr">
         <is>
-          <t>2026-03-20T15:46:48</t>
+          <t>2026-03-20T15:47:06</t>
         </is>
       </c>
     </row>
@@ -6053,7 +6053,7 @@
       </c>
       <c r="I121" t="inlineStr">
         <is>
-          <t>2026-03-20T15:46:48</t>
+          <t>2026-03-20T15:47:06</t>
         </is>
       </c>
     </row>
@@ -6090,7 +6090,7 @@
       </c>
       <c r="I122" t="inlineStr">
         <is>
-          <t>2026-03-20T15:46:48</t>
+          <t>2026-03-20T15:47:06</t>
         </is>
       </c>
     </row>
@@ -6127,7 +6127,7 @@
       </c>
       <c r="I123" t="inlineStr">
         <is>
-          <t>2026-03-20T15:46:48</t>
+          <t>2026-03-20T15:47:06</t>
         </is>
       </c>
     </row>
@@ -6164,7 +6164,7 @@
       </c>
       <c r="I124" t="inlineStr">
         <is>
-          <t>2026-03-20T15:46:48</t>
+          <t>2026-03-20T15:47:06</t>
         </is>
       </c>
     </row>
@@ -6201,7 +6201,7 @@
       </c>
       <c r="I125" t="inlineStr">
         <is>
-          <t>2026-03-20T15:46:48</t>
+          <t>2026-03-20T15:47:06</t>
         </is>
       </c>
     </row>
@@ -6238,7 +6238,7 @@
       </c>
       <c r="I126" t="inlineStr">
         <is>
-          <t>2026-03-20T15:46:48</t>
+          <t>2026-03-20T15:47:06</t>
         </is>
       </c>
     </row>
@@ -6275,7 +6275,7 @@
       </c>
       <c r="I127" t="inlineStr">
         <is>
-          <t>2026-03-20T15:46:48</t>
+          <t>2026-03-20T15:47:06</t>
         </is>
       </c>
     </row>
@@ -6312,7 +6312,7 @@
       </c>
       <c r="I128" t="inlineStr">
         <is>
-          <t>2026-03-20T15:46:48</t>
+          <t>2026-03-20T15:47:06</t>
         </is>
       </c>
     </row>
@@ -6349,7 +6349,7 @@
       </c>
       <c r="I129" t="inlineStr">
         <is>
-          <t>2026-03-20T15:46:48</t>
+          <t>2026-03-20T15:47:06</t>
         </is>
       </c>
     </row>
@@ -6386,7 +6386,7 @@
       </c>
       <c r="I130" t="inlineStr">
         <is>
-          <t>2026-03-20T15:46:48</t>
+          <t>2026-03-20T15:47:06</t>
         </is>
       </c>
     </row>
@@ -6423,7 +6423,7 @@
       </c>
       <c r="I131" t="inlineStr">
         <is>
-          <t>2026-03-20T15:46:48</t>
+          <t>2026-03-20T15:47:06</t>
         </is>
       </c>
     </row>
@@ -6460,7 +6460,7 @@
       </c>
       <c r="I132" t="inlineStr">
         <is>
-          <t>2026-03-20T15:46:48</t>
+          <t>2026-03-20T15:47:06</t>
         </is>
       </c>
     </row>
@@ -6497,7 +6497,7 @@
       </c>
       <c r="I133" t="inlineStr">
         <is>
-          <t>2026-03-20T15:46:48</t>
+          <t>2026-03-20T15:47:06</t>
         </is>
       </c>
     </row>
@@ -6534,7 +6534,7 @@
       </c>
       <c r="I134" t="inlineStr">
         <is>
-          <t>2026-03-20T15:46:48</t>
+          <t>2026-03-20T15:47:06</t>
         </is>
       </c>
     </row>
@@ -6571,7 +6571,7 @@
       </c>
       <c r="I135" t="inlineStr">
         <is>
-          <t>2026-03-20T15:46:48</t>
+          <t>2026-03-20T15:47:06</t>
         </is>
       </c>
     </row>
@@ -6608,7 +6608,7 @@
       </c>
       <c r="I136" t="inlineStr">
         <is>
-          <t>2026-03-20T15:46:48</t>
+          <t>2026-03-20T15:47:06</t>
         </is>
       </c>
     </row>
@@ -6645,7 +6645,7 @@
       </c>
       <c r="I137" t="inlineStr">
         <is>
-          <t>2026-03-20T15:46:48</t>
+          <t>2026-03-20T15:47:06</t>
         </is>
       </c>
     </row>
@@ -6682,7 +6682,7 @@
       </c>
       <c r="I138" t="inlineStr">
         <is>
-          <t>2026-03-20T15:46:48</t>
+          <t>2026-03-20T15:47:06</t>
         </is>
       </c>
     </row>
@@ -6719,7 +6719,7 @@
       </c>
       <c r="I139" t="inlineStr">
         <is>
-          <t>2026-03-20T15:46:48</t>
+          <t>2026-03-20T15:47:06</t>
         </is>
       </c>
     </row>
@@ -6756,7 +6756,7 @@
       </c>
       <c r="I140" t="inlineStr">
         <is>
-          <t>2026-03-20T15:46:48</t>
+          <t>2026-03-20T15:47:06</t>
         </is>
       </c>
     </row>
@@ -6793,7 +6793,7 @@
       </c>
       <c r="I141" t="inlineStr">
         <is>
-          <t>2026-03-20T15:46:48</t>
+          <t>2026-03-20T15:47:06</t>
         </is>
       </c>
     </row>
@@ -6830,7 +6830,7 @@
       </c>
       <c r="I142" t="inlineStr">
         <is>
-          <t>2026-03-20T15:46:48</t>
+          <t>2026-03-20T15:47:06</t>
         </is>
       </c>
     </row>
@@ -6867,7 +6867,7 @@
       </c>
       <c r="I143" t="inlineStr">
         <is>
-          <t>2026-03-20T15:46:48</t>
+          <t>2026-03-20T15:47:06</t>
         </is>
       </c>
     </row>
@@ -6904,7 +6904,7 @@
       </c>
       <c r="I144" t="inlineStr">
         <is>
-          <t>2026-03-20T15:46:48</t>
+          <t>2026-03-20T15:47:06</t>
         </is>
       </c>
     </row>
@@ -6941,7 +6941,7 @@
       </c>
       <c r="I145" t="inlineStr">
         <is>
-          <t>2026-03-20T15:46:48</t>
+          <t>2026-03-20T15:47:06</t>
         </is>
       </c>
     </row>
@@ -6978,7 +6978,7 @@
       </c>
       <c r="I146" t="inlineStr">
         <is>
-          <t>2026-03-20T15:46:48</t>
+          <t>2026-03-20T15:47:06</t>
         </is>
       </c>
     </row>
@@ -7015,7 +7015,7 @@
       </c>
       <c r="I147" t="inlineStr">
         <is>
-          <t>2026-03-20T15:46:48</t>
+          <t>2026-03-20T15:47:06</t>
         </is>
       </c>
     </row>
@@ -7052,7 +7052,7 @@
       </c>
       <c r="I148" t="inlineStr">
         <is>
-          <t>2026-03-20T15:46:48</t>
+          <t>2026-03-20T15:47:06</t>
         </is>
       </c>
     </row>
@@ -7089,7 +7089,7 @@
       </c>
       <c r="I149" t="inlineStr">
         <is>
-          <t>2026-03-20T15:46:48</t>
+          <t>2026-03-20T15:47:06</t>
         </is>
       </c>
     </row>
@@ -7126,7 +7126,7 @@
       </c>
       <c r="I150" t="inlineStr">
         <is>
-          <t>2026-03-20T15:46:48</t>
+          <t>2026-03-20T15:47:06</t>
         </is>
       </c>
     </row>
@@ -7163,7 +7163,7 @@
       </c>
       <c r="I151" t="inlineStr">
         <is>
-          <t>2026-03-20T15:46:48</t>
+          <t>2026-03-20T15:47:06</t>
         </is>
       </c>
     </row>
@@ -7200,7 +7200,7 @@
       </c>
       <c r="I152" t="inlineStr">
         <is>
-          <t>2026-03-20T15:46:48</t>
+          <t>2026-03-20T15:47:06</t>
         </is>
       </c>
     </row>
@@ -7237,7 +7237,7 @@
       </c>
       <c r="I153" t="inlineStr">
         <is>
-          <t>2026-03-20T15:46:48</t>
+          <t>2026-03-20T15:47:06</t>
         </is>
       </c>
     </row>
@@ -7370,7 +7370,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>2026-03-20T15:46:48</t>
+          <t>2026-03-20T15:47:06</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: portfolio snapshot 2026-03-19 (2026-03-20T15:47:44)
</commit_message>
<xml_diff>
--- a/portfolio_auto.xlsx
+++ b/portfolio_auto.xlsx
@@ -486,13 +486,13 @@
         <v>1</v>
       </c>
       <c r="E2" t="n">
-        <v>13553578.62304688</v>
+        <v>14238562.79623244</v>
       </c>
       <c r="F2" t="n">
-        <v>1447029.623046879</v>
+        <v>2132013.796232443</v>
       </c>
       <c r="G2" t="n">
-        <v>11.95245336261291</v>
+        <v>17.61041727277066</v>
       </c>
     </row>
     <row r="3">
@@ -513,13 +513,13 @@
         <v>1</v>
       </c>
       <c r="E3" t="n">
-        <v>10351433.71453537</v>
+        <v>10802195.38683411</v>
       </c>
       <c r="F3" t="n">
-        <v>-480581.2854646351</v>
+        <v>-29819.61316589266</v>
       </c>
       <c r="G3" t="n">
-        <v>-4.436674851951692</v>
+        <v>-0.2752914685392576</v>
       </c>
     </row>
     <row r="4">
@@ -540,13 +540,13 @@
         <v>1</v>
       </c>
       <c r="E4" t="n">
-        <v>9120000</v>
+        <v>9490000</v>
       </c>
       <c r="F4" t="n">
-        <v>1907000</v>
+        <v>2277000</v>
       </c>
       <c r="G4" t="n">
-        <v>26.43837515596839</v>
+        <v>31.56800221821711</v>
       </c>
     </row>
     <row r="5">
@@ -567,13 +567,13 @@
         <v>1</v>
       </c>
       <c r="E5" t="n">
-        <v>8453409.11431564</v>
+        <v>8629159.309373179</v>
       </c>
       <c r="F5" t="n">
-        <v>4023545.11431564</v>
+        <v>4199295.309373179</v>
       </c>
       <c r="G5" t="n">
-        <v>90.82773453802736</v>
+        <v>94.79512936228244</v>
       </c>
     </row>
     <row r="6">
@@ -594,23 +594,23 @@
         <v>1</v>
       </c>
       <c r="E6" t="n">
-        <v>8081063.113214018</v>
+        <v>8280438.313577486</v>
       </c>
       <c r="F6" t="n">
-        <v>1630712.113214018</v>
+        <v>1830087.313577486</v>
       </c>
       <c r="G6" t="n">
-        <v>25.28098258860669</v>
+        <v>28.37190276277192</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>세아제강</t>
+          <t>트랜스오션</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>50</v>
+        <v>750</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -621,23 +621,23 @@
         <v>1</v>
       </c>
       <c r="E7" t="n">
-        <v>7395000</v>
+        <v>7265949.903135682</v>
       </c>
       <c r="F7" t="n">
-        <v>1085000</v>
+        <v>3138715.903135683</v>
       </c>
       <c r="G7" t="n">
-        <v>17.19492868462758</v>
+        <v>76.04889626165328</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>트랜스오션</t>
+          <t>노블</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>750</v>
+        <v>99</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
@@ -648,23 +648,23 @@
         <v>1</v>
       </c>
       <c r="E8" t="n">
-        <v>7074115.140040115</v>
+        <v>7089362.533905029</v>
       </c>
       <c r="F8" t="n">
-        <v>2946881.140040115</v>
+        <v>3182154.533905029</v>
       </c>
       <c r="G8" t="n">
-        <v>71.40087380652794</v>
+        <v>81.4431822903984</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>노블</t>
+          <t>세아제강</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>99</v>
+        <v>50</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
@@ -675,13 +675,13 @@
         <v>1</v>
       </c>
       <c r="E9" t="n">
-        <v>6886743.840087891</v>
+        <v>6945000</v>
       </c>
       <c r="F9" t="n">
-        <v>2979535.840087891</v>
+        <v>635000</v>
       </c>
       <c r="G9" t="n">
-        <v>76.25741552760668</v>
+        <v>10.06339144215531</v>
       </c>
     </row>
     <row r="10">
@@ -702,23 +702,23 @@
         <v>1</v>
       </c>
       <c r="E10" t="n">
-        <v>5996448.754211426</v>
+        <v>6458956.91119526</v>
       </c>
       <c r="F10" t="n">
-        <v>-234770.2457885733</v>
+        <v>227737.9111952605</v>
       </c>
       <c r="G10" t="n">
-        <v>-3.767645556809564</v>
+        <v>3.654789074100277</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>DL이앤씨</t>
+          <t>타이드워터</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>80</v>
+        <v>48</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
@@ -729,23 +729,23 @@
         <v>1</v>
       </c>
       <c r="E11" t="n">
-        <v>5392000</v>
+        <v>5347019.162831247</v>
       </c>
       <c r="F11" t="n">
-        <v>1981000</v>
+        <v>1622474.162831247</v>
       </c>
       <c r="G11" t="n">
-        <v>58.07681031955438</v>
+        <v>43.56167432078944</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>타이드워터</t>
+          <t>노브</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>48</v>
+        <v>185</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
@@ -756,23 +756,23 @@
         <v>1</v>
       </c>
       <c r="E12" t="n">
-        <v>5211036.802851856</v>
+        <v>5157624.699054079</v>
       </c>
       <c r="F12" t="n">
-        <v>1486491.802851856</v>
+        <v>1847616.699054079</v>
       </c>
       <c r="G12" t="n">
-        <v>39.91069520845783</v>
+        <v>55.81910071075596</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>노브</t>
+          <t>TIME 코리아밸류업액티브</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>185</v>
+        <v>201</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
@@ -783,23 +783,23 @@
         <v>1</v>
       </c>
       <c r="E13" t="n">
-        <v>5179494.129107101</v>
+        <v>4763700</v>
       </c>
       <c r="F13" t="n">
-        <v>1869486.129107101</v>
+        <v>39903</v>
       </c>
       <c r="G13" t="n">
-        <v>56.47980697046958</v>
+        <v>0.8447230056668396</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>TIME 코리아밸류업액티브</t>
+          <t>오케아니스 에코 탱커스</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>201</v>
+        <v>65</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
@@ -810,23 +810,23 @@
         <v>1</v>
       </c>
       <c r="E14" t="n">
-        <v>4797870</v>
+        <v>4596144.593352056</v>
       </c>
       <c r="F14" t="n">
-        <v>74073</v>
+        <v>2339784.593352056</v>
       </c>
       <c r="G14" t="n">
-        <v>1.568081778281328</v>
+        <v>103.6973086454314</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>오케아니스 에코 탱커스</t>
+          <t>삼성화재</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>65</v>
+        <v>9</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
@@ -837,23 +837,23 @@
         <v>1</v>
       </c>
       <c r="E15" t="n">
-        <v>4596307.895957222</v>
+        <v>4306500</v>
       </c>
       <c r="F15" t="n">
-        <v>2339947.895957222</v>
+        <v>-324500</v>
       </c>
       <c r="G15" t="n">
-        <v>103.704546081176</v>
+        <v>-7.007125890736342</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>삼성화재</t>
+          <t>DL이앤씨</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>9</v>
+        <v>80</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
@@ -864,23 +864,23 @@
         <v>1</v>
       </c>
       <c r="E16" t="n">
-        <v>4270500</v>
+        <v>4152000</v>
       </c>
       <c r="F16" t="n">
-        <v>-360500</v>
+        <v>741000</v>
       </c>
       <c r="G16" t="n">
-        <v>-7.784495789246384</v>
+        <v>21.72383465259455</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>동원개발</t>
+          <t>HD건설기계</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>1360</v>
+        <v>31</v>
       </c>
       <c r="C17" t="inlineStr">
         <is>
@@ -891,23 +891,23 @@
         <v>1</v>
       </c>
       <c r="E17" t="n">
-        <v>4202400</v>
+        <v>4082700</v>
       </c>
       <c r="F17" t="n">
-        <v>465000</v>
+        <v>47604</v>
       </c>
       <c r="G17" t="n">
-        <v>12.44180446299566</v>
+        <v>1.179748883297944</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>HD건설기계</t>
+          <t>차코스 에너지 내비게이션</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>31</v>
+        <v>75</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
@@ -918,23 +918,23 @@
         <v>1</v>
       </c>
       <c r="E18" t="n">
-        <v>4123000</v>
+        <v>4081754.289162601</v>
       </c>
       <c r="F18" t="n">
-        <v>87904</v>
+        <v>257106.2891626009</v>
       </c>
       <c r="G18" t="n">
-        <v>2.178485964150543</v>
+        <v>6.722351682105146</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>차코스 에너지 내비게이션</t>
+          <t>동원개발</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>75</v>
+        <v>1360</v>
       </c>
       <c r="C19" t="inlineStr">
         <is>
@@ -945,13 +945,13 @@
         <v>1</v>
       </c>
       <c r="E19" t="n">
-        <v>4052048.962918622</v>
+        <v>3957600</v>
       </c>
       <c r="F19" t="n">
-        <v>227400.9629186224</v>
+        <v>220200</v>
       </c>
       <c r="G19" t="n">
-        <v>5.94567037067522</v>
+        <v>5.891796436025045</v>
       </c>
     </row>
     <row r="20">
@@ -972,13 +972,13 @@
         <v>1</v>
       </c>
       <c r="E20" t="n">
-        <v>3596373.331896178</v>
+        <v>3650596.24511658</v>
       </c>
       <c r="F20" t="n">
-        <v>2125601.331896178</v>
+        <v>2179824.24511658</v>
       </c>
       <c r="G20" t="n">
-        <v>144.5228309959789</v>
+        <v>148.2095284052579</v>
       </c>
     </row>
     <row r="21">
@@ -999,13 +999,13 @@
         <v>1</v>
       </c>
       <c r="E21" t="n">
-        <v>2959763.281021703</v>
+        <v>2978769.518133399</v>
       </c>
       <c r="F21" t="n">
-        <v>-230880.718978297</v>
+        <v>-211874.4818666009</v>
       </c>
       <c r="G21" t="n">
-        <v>-7.236179247145621</v>
+        <v>-6.640492698859569</v>
       </c>
     </row>
     <row r="22">
@@ -1026,23 +1026,23 @@
         <v>1</v>
       </c>
       <c r="E22" t="n">
-        <v>2750000</v>
+        <v>2620000</v>
       </c>
       <c r="F22" t="n">
-        <v>471390</v>
+        <v>341390</v>
       </c>
       <c r="G22" t="n">
-        <v>20.68761218462133</v>
+        <v>14.98237960862105</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>현대제철</t>
+          <t>KoAct 코스닥액티브</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>70</v>
+        <v>200</v>
       </c>
       <c r="C23" t="inlineStr">
         <is>
@@ -1053,23 +1053,23 @@
         <v>1</v>
       </c>
       <c r="E23" t="n">
-        <v>2621500</v>
+        <v>2526000</v>
       </c>
       <c r="F23" t="n">
-        <v>-186000</v>
+        <v>-176000</v>
       </c>
       <c r="G23" t="n">
-        <v>-6.625111308993767</v>
+        <v>-6.513693560325684</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>KoAct 코스닥액티브</t>
+          <t>현대제철</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>200</v>
+        <v>70</v>
       </c>
       <c r="C24" t="inlineStr">
         <is>
@@ -1080,13 +1080,13 @@
         <v>1</v>
       </c>
       <c r="E24" t="n">
-        <v>2582000</v>
+        <v>2509500</v>
       </c>
       <c r="F24" t="n">
-        <v>-120000</v>
+        <v>-298000</v>
       </c>
       <c r="G24" t="n">
-        <v>-4.441154700222058</v>
+        <v>-10.61442564559216</v>
       </c>
     </row>
     <row r="25">
@@ -1107,13 +1107,13 @@
         <v>1</v>
       </c>
       <c r="E25" t="n">
-        <v>2514000</v>
+        <v>2406000</v>
       </c>
       <c r="F25" t="n">
-        <v>503000</v>
+        <v>395000</v>
       </c>
       <c r="G25" t="n">
-        <v>25.01243162605669</v>
+        <v>19.64196916956738</v>
       </c>
     </row>
     <row r="26">
@@ -1134,13 +1134,13 @@
         <v>1</v>
       </c>
       <c r="E26" t="n">
-        <v>2219250</v>
+        <v>2180750</v>
       </c>
       <c r="F26" t="n">
-        <v>509749</v>
+        <v>471249</v>
       </c>
       <c r="G26" t="n">
-        <v>29.81858448752005</v>
+        <v>27.56646530186294</v>
       </c>
     </row>
     <row r="27">
@@ -1161,13 +1161,13 @@
         <v>1</v>
       </c>
       <c r="E27" t="n">
-        <v>2176561.162089184</v>
+        <v>2178165.369514748</v>
       </c>
       <c r="F27" t="n">
-        <v>112571.1620891844</v>
+        <v>114175.3695147485</v>
       </c>
       <c r="G27" t="n">
-        <v>5.45405559567558</v>
+        <v>5.531779200226186</v>
       </c>
     </row>
     <row r="28">
@@ -1188,13 +1188,13 @@
         <v>1</v>
       </c>
       <c r="E28" t="n">
-        <v>2097000</v>
+        <v>2023200</v>
       </c>
       <c r="F28" t="n">
-        <v>-295200</v>
+        <v>-369000</v>
       </c>
       <c r="G28" t="n">
-        <v>-12.34010534236268</v>
+        <v>-15.42513167795335</v>
       </c>
     </row>
     <row r="29">
@@ -1215,13 +1215,13 @@
         <v>1</v>
       </c>
       <c r="E29" t="n">
-        <v>2004000</v>
+        <v>1938000</v>
       </c>
       <c r="F29" t="n">
-        <v>-54000</v>
+        <v>-120000</v>
       </c>
       <c r="G29" t="n">
-        <v>-2.623906705539359</v>
+        <v>-5.830903790087463</v>
       </c>
     </row>
     <row r="30">
@@ -1242,23 +1242,23 @@
         <v>1</v>
       </c>
       <c r="E30" t="n">
-        <v>1995330</v>
+        <v>1906800</v>
       </c>
       <c r="F30" t="n">
-        <v>23829</v>
+        <v>-64701</v>
       </c>
       <c r="G30" t="n">
-        <v>1.208672985709873</v>
+        <v>-3.281814211608312</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>하나금융지주</t>
+          <t>스타 벌크 캐리어스</t>
         </is>
       </c>
       <c r="B31" t="n">
-        <v>15</v>
+        <v>50</v>
       </c>
       <c r="C31" t="inlineStr">
         <is>
@@ -1269,23 +1269,23 @@
         <v>1</v>
       </c>
       <c r="E31" t="n">
-        <v>1698000</v>
+        <v>1704386.346717528</v>
       </c>
       <c r="F31" t="n">
-        <v>15500</v>
+        <v>390033.3467175288</v>
       </c>
       <c r="G31" t="n">
-        <v>0.9212481426448738</v>
+        <v>29.67493106627588</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>스타 벌크 캐리어스</t>
+          <t>하나금융지주</t>
         </is>
       </c>
       <c r="B32" t="n">
-        <v>50</v>
+        <v>15</v>
       </c>
       <c r="C32" t="inlineStr">
         <is>
@@ -1296,13 +1296,13 @@
         <v>1</v>
       </c>
       <c r="E32" t="n">
-        <v>1696441.320678405</v>
+        <v>1698000</v>
       </c>
       <c r="F32" t="n">
-        <v>382088.3206784062</v>
+        <v>15500</v>
       </c>
       <c r="G32" t="n">
-        <v>29.07044916231837</v>
+        <v>0.9212481426448738</v>
       </c>
     </row>
     <row r="33">
@@ -1323,13 +1323,13 @@
         <v>1</v>
       </c>
       <c r="E33" t="n">
-        <v>1683366.447431445</v>
+        <v>1682281.111696094</v>
       </c>
       <c r="F33" t="n">
-        <v>-11089.55256855441</v>
+        <v>-12174.88830390549</v>
       </c>
       <c r="G33" t="n">
-        <v>-0.6544609342794628</v>
+        <v>-0.7185130982395231</v>
       </c>
     </row>
     <row r="34">
@@ -1350,13 +1350,13 @@
         <v>1</v>
       </c>
       <c r="E34" t="n">
-        <v>1670000</v>
+        <v>1627500</v>
       </c>
       <c r="F34" t="n">
-        <v>20499.9999999993</v>
+        <v>-22000.0000000007</v>
       </c>
       <c r="G34" t="n">
-        <v>1.242800848742</v>
+        <v>-1.333737496211015</v>
       </c>
     </row>
     <row r="35">
@@ -1377,23 +1377,23 @@
         <v>1</v>
       </c>
       <c r="E35" t="n">
-        <v>926000</v>
+        <v>922000</v>
       </c>
       <c r="F35" t="n">
-        <v>93000</v>
+        <v>89000</v>
       </c>
       <c r="G35" t="n">
-        <v>11.16446578631453</v>
+        <v>10.68427370948379</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>비에이치아이</t>
+          <t>클리블랜드 클리프스</t>
         </is>
       </c>
       <c r="B36" t="n">
-        <v>8</v>
+        <v>70</v>
       </c>
       <c r="C36" t="inlineStr">
         <is>
@@ -1404,13 +1404,13 @@
         <v>1</v>
       </c>
       <c r="E36" t="n">
-        <v>876000</v>
+        <v>858716.8307915051</v>
       </c>
       <c r="F36" t="n">
-        <v>210885</v>
+        <v>-157338.1692084949</v>
       </c>
       <c r="G36" t="n">
-        <v>31.70654698811484</v>
+        <v>-15.48520200269621</v>
       </c>
     </row>
     <row r="37">
@@ -1431,23 +1431,23 @@
         <v>1</v>
       </c>
       <c r="E37" t="n">
-        <v>848519.8631833494</v>
+        <v>855417.5163666997</v>
       </c>
       <c r="F37" t="n">
-        <v>222788.8631833494</v>
+        <v>229686.5163666997</v>
       </c>
       <c r="G37" t="n">
-        <v>35.60457499841775</v>
+        <v>36.70691021648275</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>클리블랜드 클리프스</t>
+          <t>비에이치아이</t>
         </is>
       </c>
       <c r="B38" t="n">
-        <v>70</v>
+        <v>8</v>
       </c>
       <c r="C38" t="inlineStr">
         <is>
@@ -1458,13 +1458,13 @@
         <v>1</v>
       </c>
       <c r="E38" t="n">
-        <v>833036.4441346284</v>
+        <v>834400</v>
       </c>
       <c r="F38" t="n">
-        <v>-183018.5558653716</v>
+        <v>169285</v>
       </c>
       <c r="G38" t="n">
-        <v>-18.01266229341636</v>
+        <v>25.45198950557423</v>
       </c>
     </row>
     <row r="39">
@@ -1485,13 +1485,13 @@
         <v>1</v>
       </c>
       <c r="E39" t="n">
-        <v>798210.0491355956</v>
+        <v>798609.6514927745</v>
       </c>
       <c r="F39" t="n">
-        <v>19619.04913559556</v>
+        <v>20018.65149277449</v>
       </c>
       <c r="G39" t="n">
-        <v>2.519814528500273</v>
+        <v>2.571138311741914</v>
       </c>
     </row>
   </sheetData>
@@ -1538,7 +1538,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-03-20</t>
+          <t>2026-03-19</t>
         </is>
       </c>
       <c r="B2" t="n">
@@ -1549,11 +1549,11 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2026-03-20T15:47:06</t>
+          <t>2026-03-20T15:47:44</t>
         </is>
       </c>
       <c r="E2" t="n">
-        <v>1495.97998046875</v>
+        <v>1499.680053710938</v>
       </c>
     </row>
   </sheetData>
@@ -1567,7 +1567,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I153"/>
+  <dimension ref="A1:I115"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5832,1412 +5832,6 @@
       <c r="I115" t="inlineStr">
         <is>
           <t>2026-03-19T21:54:06</t>
-        </is>
-      </c>
-    </row>
-    <row r="116">
-      <c r="A116" t="inlineStr">
-        <is>
-          <t>2026-03-20</t>
-        </is>
-      </c>
-      <c r="B116" t="inlineStr">
-        <is>
-          <t>페트로브라스 (ADR)</t>
-        </is>
-      </c>
-      <c r="C116" t="n">
-        <v>480</v>
-      </c>
-      <c r="D116" t="inlineStr">
-        <is>
-          <t>KRW</t>
-        </is>
-      </c>
-      <c r="E116" t="n">
-        <v>1</v>
-      </c>
-      <c r="F116" t="n">
-        <v>13553578.62304688</v>
-      </c>
-      <c r="G116" t="n">
-        <v>1447029.623046879</v>
-      </c>
-      <c r="H116" t="n">
-        <v>11.95245336261291</v>
-      </c>
-      <c r="I116" t="inlineStr">
-        <is>
-          <t>2026-03-20T15:47:06</t>
-        </is>
-      </c>
-    </row>
-    <row r="117">
-      <c r="A117" t="inlineStr">
-        <is>
-          <t>2026-03-20</t>
-        </is>
-      </c>
-      <c r="B117" t="inlineStr">
-        <is>
-          <t>AGNC 인베스트먼트</t>
-        </is>
-      </c>
-      <c r="C117" t="n">
-        <v>700</v>
-      </c>
-      <c r="D117" t="inlineStr">
-        <is>
-          <t>KRW</t>
-        </is>
-      </c>
-      <c r="E117" t="n">
-        <v>1</v>
-      </c>
-      <c r="F117" t="n">
-        <v>10351433.71453537</v>
-      </c>
-      <c r="G117" t="n">
-        <v>-480581.2854646351</v>
-      </c>
-      <c r="H117" t="n">
-        <v>-4.436674851951692</v>
-      </c>
-      <c r="I117" t="inlineStr">
-        <is>
-          <t>2026-03-20T15:47:06</t>
-        </is>
-      </c>
-    </row>
-    <row r="118">
-      <c r="A118" t="inlineStr">
-        <is>
-          <t>2026-03-20</t>
-        </is>
-      </c>
-      <c r="B118" t="inlineStr">
-        <is>
-          <t>대한조선</t>
-        </is>
-      </c>
-      <c r="C118" t="n">
-        <v>100</v>
-      </c>
-      <c r="D118" t="inlineStr">
-        <is>
-          <t>KRW</t>
-        </is>
-      </c>
-      <c r="E118" t="n">
-        <v>1</v>
-      </c>
-      <c r="F118" t="n">
-        <v>9120000</v>
-      </c>
-      <c r="G118" t="n">
-        <v>1907000</v>
-      </c>
-      <c r="H118" t="n">
-        <v>26.43837515596839</v>
-      </c>
-      <c r="I118" t="inlineStr">
-        <is>
-          <t>2026-03-20T15:47:06</t>
-        </is>
-      </c>
-    </row>
-    <row r="119">
-      <c r="A119" t="inlineStr">
-        <is>
-          <t>2026-03-20</t>
-        </is>
-      </c>
-      <c r="B119" t="inlineStr">
-        <is>
-          <t>프론트라인</t>
-        </is>
-      </c>
-      <c r="C119" t="n">
-        <v>175</v>
-      </c>
-      <c r="D119" t="inlineStr">
-        <is>
-          <t>KRW</t>
-        </is>
-      </c>
-      <c r="E119" t="n">
-        <v>1</v>
-      </c>
-      <c r="F119" t="n">
-        <v>8453409.11431564</v>
-      </c>
-      <c r="G119" t="n">
-        <v>4023545.11431564</v>
-      </c>
-      <c r="H119" t="n">
-        <v>90.82773453802736</v>
-      </c>
-      <c r="I119" t="inlineStr">
-        <is>
-          <t>2026-03-20T15:47:06</t>
-        </is>
-      </c>
-    </row>
-    <row r="120">
-      <c r="A120" t="inlineStr">
-        <is>
-          <t>2026-03-20</t>
-        </is>
-      </c>
-      <c r="B120" t="inlineStr">
-        <is>
-          <t>시드릴</t>
-        </is>
-      </c>
-      <c r="C120" t="n">
-        <v>123</v>
-      </c>
-      <c r="D120" t="inlineStr">
-        <is>
-          <t>KRW</t>
-        </is>
-      </c>
-      <c r="E120" t="n">
-        <v>1</v>
-      </c>
-      <c r="F120" t="n">
-        <v>8081063.113214018</v>
-      </c>
-      <c r="G120" t="n">
-        <v>1630712.113214018</v>
-      </c>
-      <c r="H120" t="n">
-        <v>25.28098258860669</v>
-      </c>
-      <c r="I120" t="inlineStr">
-        <is>
-          <t>2026-03-20T15:47:06</t>
-        </is>
-      </c>
-    </row>
-    <row r="121">
-      <c r="A121" t="inlineStr">
-        <is>
-          <t>2026-03-20</t>
-        </is>
-      </c>
-      <c r="B121" t="inlineStr">
-        <is>
-          <t>세아제강</t>
-        </is>
-      </c>
-      <c r="C121" t="n">
-        <v>50</v>
-      </c>
-      <c r="D121" t="inlineStr">
-        <is>
-          <t>KRW</t>
-        </is>
-      </c>
-      <c r="E121" t="n">
-        <v>1</v>
-      </c>
-      <c r="F121" t="n">
-        <v>7395000</v>
-      </c>
-      <c r="G121" t="n">
-        <v>1085000</v>
-      </c>
-      <c r="H121" t="n">
-        <v>17.19492868462758</v>
-      </c>
-      <c r="I121" t="inlineStr">
-        <is>
-          <t>2026-03-20T15:47:06</t>
-        </is>
-      </c>
-    </row>
-    <row r="122">
-      <c r="A122" t="inlineStr">
-        <is>
-          <t>2026-03-20</t>
-        </is>
-      </c>
-      <c r="B122" t="inlineStr">
-        <is>
-          <t>트랜스오션</t>
-        </is>
-      </c>
-      <c r="C122" t="n">
-        <v>750</v>
-      </c>
-      <c r="D122" t="inlineStr">
-        <is>
-          <t>KRW</t>
-        </is>
-      </c>
-      <c r="E122" t="n">
-        <v>1</v>
-      </c>
-      <c r="F122" t="n">
-        <v>7074115.140040115</v>
-      </c>
-      <c r="G122" t="n">
-        <v>2946881.140040115</v>
-      </c>
-      <c r="H122" t="n">
-        <v>71.40087380652794</v>
-      </c>
-      <c r="I122" t="inlineStr">
-        <is>
-          <t>2026-03-20T15:47:06</t>
-        </is>
-      </c>
-    </row>
-    <row r="123">
-      <c r="A123" t="inlineStr">
-        <is>
-          <t>2026-03-20</t>
-        </is>
-      </c>
-      <c r="B123" t="inlineStr">
-        <is>
-          <t>노블</t>
-        </is>
-      </c>
-      <c r="C123" t="n">
-        <v>99</v>
-      </c>
-      <c r="D123" t="inlineStr">
-        <is>
-          <t>KRW</t>
-        </is>
-      </c>
-      <c r="E123" t="n">
-        <v>1</v>
-      </c>
-      <c r="F123" t="n">
-        <v>6886743.840087891</v>
-      </c>
-      <c r="G123" t="n">
-        <v>2979535.840087891</v>
-      </c>
-      <c r="H123" t="n">
-        <v>76.25741552760668</v>
-      </c>
-      <c r="I123" t="inlineStr">
-        <is>
-          <t>2026-03-20T15:47:06</t>
-        </is>
-      </c>
-    </row>
-    <row r="124">
-      <c r="A124" t="inlineStr">
-        <is>
-          <t>2026-03-20</t>
-        </is>
-      </c>
-      <c r="B124" t="inlineStr">
-        <is>
-          <t>센트러스 에너지</t>
-        </is>
-      </c>
-      <c r="C124" t="n">
-        <v>21</v>
-      </c>
-      <c r="D124" t="inlineStr">
-        <is>
-          <t>KRW</t>
-        </is>
-      </c>
-      <c r="E124" t="n">
-        <v>1</v>
-      </c>
-      <c r="F124" t="n">
-        <v>5996448.754211426</v>
-      </c>
-      <c r="G124" t="n">
-        <v>-234770.2457885733</v>
-      </c>
-      <c r="H124" t="n">
-        <v>-3.767645556809564</v>
-      </c>
-      <c r="I124" t="inlineStr">
-        <is>
-          <t>2026-03-20T15:47:06</t>
-        </is>
-      </c>
-    </row>
-    <row r="125">
-      <c r="A125" t="inlineStr">
-        <is>
-          <t>2026-03-20</t>
-        </is>
-      </c>
-      <c r="B125" t="inlineStr">
-        <is>
-          <t>DL이앤씨</t>
-        </is>
-      </c>
-      <c r="C125" t="n">
-        <v>80</v>
-      </c>
-      <c r="D125" t="inlineStr">
-        <is>
-          <t>KRW</t>
-        </is>
-      </c>
-      <c r="E125" t="n">
-        <v>1</v>
-      </c>
-      <c r="F125" t="n">
-        <v>5392000</v>
-      </c>
-      <c r="G125" t="n">
-        <v>1981000</v>
-      </c>
-      <c r="H125" t="n">
-        <v>58.07681031955438</v>
-      </c>
-      <c r="I125" t="inlineStr">
-        <is>
-          <t>2026-03-20T15:47:06</t>
-        </is>
-      </c>
-    </row>
-    <row r="126">
-      <c r="A126" t="inlineStr">
-        <is>
-          <t>2026-03-20</t>
-        </is>
-      </c>
-      <c r="B126" t="inlineStr">
-        <is>
-          <t>타이드워터</t>
-        </is>
-      </c>
-      <c r="C126" t="n">
-        <v>48</v>
-      </c>
-      <c r="D126" t="inlineStr">
-        <is>
-          <t>KRW</t>
-        </is>
-      </c>
-      <c r="E126" t="n">
-        <v>1</v>
-      </c>
-      <c r="F126" t="n">
-        <v>5211036.802851856</v>
-      </c>
-      <c r="G126" t="n">
-        <v>1486491.802851856</v>
-      </c>
-      <c r="H126" t="n">
-        <v>39.91069520845783</v>
-      </c>
-      <c r="I126" t="inlineStr">
-        <is>
-          <t>2026-03-20T15:47:06</t>
-        </is>
-      </c>
-    </row>
-    <row r="127">
-      <c r="A127" t="inlineStr">
-        <is>
-          <t>2026-03-20</t>
-        </is>
-      </c>
-      <c r="B127" t="inlineStr">
-        <is>
-          <t>노브</t>
-        </is>
-      </c>
-      <c r="C127" t="n">
-        <v>185</v>
-      </c>
-      <c r="D127" t="inlineStr">
-        <is>
-          <t>KRW</t>
-        </is>
-      </c>
-      <c r="E127" t="n">
-        <v>1</v>
-      </c>
-      <c r="F127" t="n">
-        <v>5179494.129107101</v>
-      </c>
-      <c r="G127" t="n">
-        <v>1869486.129107101</v>
-      </c>
-      <c r="H127" t="n">
-        <v>56.47980697046958</v>
-      </c>
-      <c r="I127" t="inlineStr">
-        <is>
-          <t>2026-03-20T15:47:06</t>
-        </is>
-      </c>
-    </row>
-    <row r="128">
-      <c r="A128" t="inlineStr">
-        <is>
-          <t>2026-03-20</t>
-        </is>
-      </c>
-      <c r="B128" t="inlineStr">
-        <is>
-          <t>TIME 코리아밸류업액티브</t>
-        </is>
-      </c>
-      <c r="C128" t="n">
-        <v>201</v>
-      </c>
-      <c r="D128" t="inlineStr">
-        <is>
-          <t>KRW</t>
-        </is>
-      </c>
-      <c r="E128" t="n">
-        <v>1</v>
-      </c>
-      <c r="F128" t="n">
-        <v>4797870</v>
-      </c>
-      <c r="G128" t="n">
-        <v>74073</v>
-      </c>
-      <c r="H128" t="n">
-        <v>1.568081778281328</v>
-      </c>
-      <c r="I128" t="inlineStr">
-        <is>
-          <t>2026-03-20T15:47:06</t>
-        </is>
-      </c>
-    </row>
-    <row r="129">
-      <c r="A129" t="inlineStr">
-        <is>
-          <t>2026-03-20</t>
-        </is>
-      </c>
-      <c r="B129" t="inlineStr">
-        <is>
-          <t>오케아니스 에코 탱커스</t>
-        </is>
-      </c>
-      <c r="C129" t="n">
-        <v>65</v>
-      </c>
-      <c r="D129" t="inlineStr">
-        <is>
-          <t>KRW</t>
-        </is>
-      </c>
-      <c r="E129" t="n">
-        <v>1</v>
-      </c>
-      <c r="F129" t="n">
-        <v>4596307.895957222</v>
-      </c>
-      <c r="G129" t="n">
-        <v>2339947.895957222</v>
-      </c>
-      <c r="H129" t="n">
-        <v>103.704546081176</v>
-      </c>
-      <c r="I129" t="inlineStr">
-        <is>
-          <t>2026-03-20T15:47:06</t>
-        </is>
-      </c>
-    </row>
-    <row r="130">
-      <c r="A130" t="inlineStr">
-        <is>
-          <t>2026-03-20</t>
-        </is>
-      </c>
-      <c r="B130" t="inlineStr">
-        <is>
-          <t>삼성화재</t>
-        </is>
-      </c>
-      <c r="C130" t="n">
-        <v>9</v>
-      </c>
-      <c r="D130" t="inlineStr">
-        <is>
-          <t>KRW</t>
-        </is>
-      </c>
-      <c r="E130" t="n">
-        <v>1</v>
-      </c>
-      <c r="F130" t="n">
-        <v>4270500</v>
-      </c>
-      <c r="G130" t="n">
-        <v>-360500</v>
-      </c>
-      <c r="H130" t="n">
-        <v>-7.784495789246384</v>
-      </c>
-      <c r="I130" t="inlineStr">
-        <is>
-          <t>2026-03-20T15:47:06</t>
-        </is>
-      </c>
-    </row>
-    <row r="131">
-      <c r="A131" t="inlineStr">
-        <is>
-          <t>2026-03-20</t>
-        </is>
-      </c>
-      <c r="B131" t="inlineStr">
-        <is>
-          <t>동원개발</t>
-        </is>
-      </c>
-      <c r="C131" t="n">
-        <v>1360</v>
-      </c>
-      <c r="D131" t="inlineStr">
-        <is>
-          <t>KRW</t>
-        </is>
-      </c>
-      <c r="E131" t="n">
-        <v>1</v>
-      </c>
-      <c r="F131" t="n">
-        <v>4202400</v>
-      </c>
-      <c r="G131" t="n">
-        <v>465000</v>
-      </c>
-      <c r="H131" t="n">
-        <v>12.44180446299566</v>
-      </c>
-      <c r="I131" t="inlineStr">
-        <is>
-          <t>2026-03-20T15:47:06</t>
-        </is>
-      </c>
-    </row>
-    <row r="132">
-      <c r="A132" t="inlineStr">
-        <is>
-          <t>2026-03-20</t>
-        </is>
-      </c>
-      <c r="B132" t="inlineStr">
-        <is>
-          <t>HD건설기계</t>
-        </is>
-      </c>
-      <c r="C132" t="n">
-        <v>31</v>
-      </c>
-      <c r="D132" t="inlineStr">
-        <is>
-          <t>KRW</t>
-        </is>
-      </c>
-      <c r="E132" t="n">
-        <v>1</v>
-      </c>
-      <c r="F132" t="n">
-        <v>4123000</v>
-      </c>
-      <c r="G132" t="n">
-        <v>87904</v>
-      </c>
-      <c r="H132" t="n">
-        <v>2.178485964150543</v>
-      </c>
-      <c r="I132" t="inlineStr">
-        <is>
-          <t>2026-03-20T15:47:06</t>
-        </is>
-      </c>
-    </row>
-    <row r="133">
-      <c r="A133" t="inlineStr">
-        <is>
-          <t>2026-03-20</t>
-        </is>
-      </c>
-      <c r="B133" t="inlineStr">
-        <is>
-          <t>차코스 에너지 내비게이션</t>
-        </is>
-      </c>
-      <c r="C133" t="n">
-        <v>75</v>
-      </c>
-      <c r="D133" t="inlineStr">
-        <is>
-          <t>KRW</t>
-        </is>
-      </c>
-      <c r="E133" t="n">
-        <v>1</v>
-      </c>
-      <c r="F133" t="n">
-        <v>4052048.962918622</v>
-      </c>
-      <c r="G133" t="n">
-        <v>227400.9629186224</v>
-      </c>
-      <c r="H133" t="n">
-        <v>5.94567037067522</v>
-      </c>
-      <c r="I133" t="inlineStr">
-        <is>
-          <t>2026-03-20T15:47:06</t>
-        </is>
-      </c>
-    </row>
-    <row r="134">
-      <c r="A134" t="inlineStr">
-        <is>
-          <t>2026-03-20</t>
-        </is>
-      </c>
-      <c r="B134" t="inlineStr">
-        <is>
-          <t>피바디 에너지</t>
-        </is>
-      </c>
-      <c r="C134" t="n">
-        <v>65</v>
-      </c>
-      <c r="D134" t="inlineStr">
-        <is>
-          <t>KRW</t>
-        </is>
-      </c>
-      <c r="E134" t="n">
-        <v>1</v>
-      </c>
-      <c r="F134" t="n">
-        <v>3596373.331896178</v>
-      </c>
-      <c r="G134" t="n">
-        <v>2125601.331896178</v>
-      </c>
-      <c r="H134" t="n">
-        <v>144.5228309959789</v>
-      </c>
-      <c r="I134" t="inlineStr">
-        <is>
-          <t>2026-03-20T15:47:06</t>
-        </is>
-      </c>
-    </row>
-    <row r="135">
-      <c r="A135" t="inlineStr">
-        <is>
-          <t>2026-03-20</t>
-        </is>
-      </c>
-      <c r="B135" t="inlineStr">
-        <is>
-          <t>더치 브로스</t>
-        </is>
-      </c>
-      <c r="C135" t="n">
-        <v>39</v>
-      </c>
-      <c r="D135" t="inlineStr">
-        <is>
-          <t>KRW</t>
-        </is>
-      </c>
-      <c r="E135" t="n">
-        <v>1</v>
-      </c>
-      <c r="F135" t="n">
-        <v>2959763.281021703</v>
-      </c>
-      <c r="G135" t="n">
-        <v>-230880.718978297</v>
-      </c>
-      <c r="H135" t="n">
-        <v>-7.236179247145621</v>
-      </c>
-      <c r="I135" t="inlineStr">
-        <is>
-          <t>2026-03-20T15:47:06</t>
-        </is>
-      </c>
-    </row>
-    <row r="136">
-      <c r="A136" t="inlineStr">
-        <is>
-          <t>2026-03-20</t>
-        </is>
-      </c>
-      <c r="B136" t="inlineStr">
-        <is>
-          <t>휴스틸</t>
-        </is>
-      </c>
-      <c r="C136" t="n">
-        <v>500</v>
-      </c>
-      <c r="D136" t="inlineStr">
-        <is>
-          <t>KRW</t>
-        </is>
-      </c>
-      <c r="E136" t="n">
-        <v>1</v>
-      </c>
-      <c r="F136" t="n">
-        <v>2750000</v>
-      </c>
-      <c r="G136" t="n">
-        <v>471390</v>
-      </c>
-      <c r="H136" t="n">
-        <v>20.68761218462133</v>
-      </c>
-      <c r="I136" t="inlineStr">
-        <is>
-          <t>2026-03-20T15:47:06</t>
-        </is>
-      </c>
-    </row>
-    <row r="137">
-      <c r="A137" t="inlineStr">
-        <is>
-          <t>2026-03-20</t>
-        </is>
-      </c>
-      <c r="B137" t="inlineStr">
-        <is>
-          <t>현대제철</t>
-        </is>
-      </c>
-      <c r="C137" t="n">
-        <v>70</v>
-      </c>
-      <c r="D137" t="inlineStr">
-        <is>
-          <t>KRW</t>
-        </is>
-      </c>
-      <c r="E137" t="n">
-        <v>1</v>
-      </c>
-      <c r="F137" t="n">
-        <v>2621500</v>
-      </c>
-      <c r="G137" t="n">
-        <v>-186000</v>
-      </c>
-      <c r="H137" t="n">
-        <v>-6.625111308993767</v>
-      </c>
-      <c r="I137" t="inlineStr">
-        <is>
-          <t>2026-03-20T15:47:06</t>
-        </is>
-      </c>
-    </row>
-    <row r="138">
-      <c r="A138" t="inlineStr">
-        <is>
-          <t>2026-03-20</t>
-        </is>
-      </c>
-      <c r="B138" t="inlineStr">
-        <is>
-          <t>KoAct 코스닥액티브</t>
-        </is>
-      </c>
-      <c r="C138" t="n">
-        <v>200</v>
-      </c>
-      <c r="D138" t="inlineStr">
-        <is>
-          <t>KRW</t>
-        </is>
-      </c>
-      <c r="E138" t="n">
-        <v>1</v>
-      </c>
-      <c r="F138" t="n">
-        <v>2582000</v>
-      </c>
-      <c r="G138" t="n">
-        <v>-120000</v>
-      </c>
-      <c r="H138" t="n">
-        <v>-4.441154700222058</v>
-      </c>
-      <c r="I138" t="inlineStr">
-        <is>
-          <t>2026-03-20T15:47:06</t>
-        </is>
-      </c>
-    </row>
-    <row r="139">
-      <c r="A139" t="inlineStr">
-        <is>
-          <t>2026-03-20</t>
-        </is>
-      </c>
-      <c r="B139" t="inlineStr">
-        <is>
-          <t>넥스틸</t>
-        </is>
-      </c>
-      <c r="C139" t="n">
-        <v>200</v>
-      </c>
-      <c r="D139" t="inlineStr">
-        <is>
-          <t>KRW</t>
-        </is>
-      </c>
-      <c r="E139" t="n">
-        <v>1</v>
-      </c>
-      <c r="F139" t="n">
-        <v>2514000</v>
-      </c>
-      <c r="G139" t="n">
-        <v>503000</v>
-      </c>
-      <c r="H139" t="n">
-        <v>25.01243162605669</v>
-      </c>
-      <c r="I139" t="inlineStr">
-        <is>
-          <t>2026-03-20T15:47:06</t>
-        </is>
-      </c>
-    </row>
-    <row r="140">
-      <c r="A140" t="inlineStr">
-        <is>
-          <t>2026-03-20</t>
-        </is>
-      </c>
-      <c r="B140" t="inlineStr">
-        <is>
-          <t>대신증권</t>
-        </is>
-      </c>
-      <c r="C140" t="n">
-        <v>55</v>
-      </c>
-      <c r="D140" t="inlineStr">
-        <is>
-          <t>KRW</t>
-        </is>
-      </c>
-      <c r="E140" t="n">
-        <v>1</v>
-      </c>
-      <c r="F140" t="n">
-        <v>2219250</v>
-      </c>
-      <c r="G140" t="n">
-        <v>509749</v>
-      </c>
-      <c r="H140" t="n">
-        <v>29.81858448752005</v>
-      </c>
-      <c r="I140" t="inlineStr">
-        <is>
-          <t>2026-03-20T15:47:06</t>
-        </is>
-      </c>
-    </row>
-    <row r="141">
-      <c r="A141" t="inlineStr">
-        <is>
-          <t>2026-03-20</t>
-        </is>
-      </c>
-      <c r="B141" t="inlineStr">
-        <is>
-          <t>발레로 에너지</t>
-        </is>
-      </c>
-      <c r="C141" t="n">
-        <v>6</v>
-      </c>
-      <c r="D141" t="inlineStr">
-        <is>
-          <t>KRW</t>
-        </is>
-      </c>
-      <c r="E141" t="n">
-        <v>1</v>
-      </c>
-      <c r="F141" t="n">
-        <v>2176561.162089184</v>
-      </c>
-      <c r="G141" t="n">
-        <v>112571.1620891844</v>
-      </c>
-      <c r="H141" t="n">
-        <v>5.45405559567558</v>
-      </c>
-      <c r="I141" t="inlineStr">
-        <is>
-          <t>2026-03-20T15:47:06</t>
-        </is>
-      </c>
-    </row>
-    <row r="142">
-      <c r="A142" t="inlineStr">
-        <is>
-          <t>2026-03-20</t>
-        </is>
-      </c>
-      <c r="B142" t="inlineStr">
-        <is>
-          <t>미창석유</t>
-        </is>
-      </c>
-      <c r="C142" t="n">
-        <v>18</v>
-      </c>
-      <c r="D142" t="inlineStr">
-        <is>
-          <t>KRW</t>
-        </is>
-      </c>
-      <c r="E142" t="n">
-        <v>1</v>
-      </c>
-      <c r="F142" t="n">
-        <v>2097000</v>
-      </c>
-      <c r="G142" t="n">
-        <v>-295200</v>
-      </c>
-      <c r="H142" t="n">
-        <v>-12.34010534236268</v>
-      </c>
-      <c r="I142" t="inlineStr">
-        <is>
-          <t>2026-03-20T15:47:06</t>
-        </is>
-      </c>
-    </row>
-    <row r="143">
-      <c r="A143" t="inlineStr">
-        <is>
-          <t>2026-03-20</t>
-        </is>
-      </c>
-      <c r="B143" t="inlineStr">
-        <is>
-          <t>대창단조</t>
-        </is>
-      </c>
-      <c r="C143" t="n">
-        <v>300</v>
-      </c>
-      <c r="D143" t="inlineStr">
-        <is>
-          <t>KRW</t>
-        </is>
-      </c>
-      <c r="E143" t="n">
-        <v>1</v>
-      </c>
-      <c r="F143" t="n">
-        <v>2004000</v>
-      </c>
-      <c r="G143" t="n">
-        <v>-54000</v>
-      </c>
-      <c r="H143" t="n">
-        <v>-2.623906705539359</v>
-      </c>
-      <c r="I143" t="inlineStr">
-        <is>
-          <t>2026-03-20T15:47:06</t>
-        </is>
-      </c>
-    </row>
-    <row r="144">
-      <c r="A144" t="inlineStr">
-        <is>
-          <t>2026-03-20</t>
-        </is>
-      </c>
-      <c r="B144" t="inlineStr">
-        <is>
-          <t>동방</t>
-        </is>
-      </c>
-      <c r="C144" t="n">
-        <v>681</v>
-      </c>
-      <c r="D144" t="inlineStr">
-        <is>
-          <t>KRW</t>
-        </is>
-      </c>
-      <c r="E144" t="n">
-        <v>1</v>
-      </c>
-      <c r="F144" t="n">
-        <v>1995330</v>
-      </c>
-      <c r="G144" t="n">
-        <v>23829</v>
-      </c>
-      <c r="H144" t="n">
-        <v>1.208672985709873</v>
-      </c>
-      <c r="I144" t="inlineStr">
-        <is>
-          <t>2026-03-20T15:47:06</t>
-        </is>
-      </c>
-    </row>
-    <row r="145">
-      <c r="A145" t="inlineStr">
-        <is>
-          <t>2026-03-20</t>
-        </is>
-      </c>
-      <c r="B145" t="inlineStr">
-        <is>
-          <t>하나금융지주</t>
-        </is>
-      </c>
-      <c r="C145" t="n">
-        <v>15</v>
-      </c>
-      <c r="D145" t="inlineStr">
-        <is>
-          <t>KRW</t>
-        </is>
-      </c>
-      <c r="E145" t="n">
-        <v>1</v>
-      </c>
-      <c r="F145" t="n">
-        <v>1698000</v>
-      </c>
-      <c r="G145" t="n">
-        <v>15500</v>
-      </c>
-      <c r="H145" t="n">
-        <v>0.9212481426448738</v>
-      </c>
-      <c r="I145" t="inlineStr">
-        <is>
-          <t>2026-03-20T15:47:06</t>
-        </is>
-      </c>
-    </row>
-    <row r="146">
-      <c r="A146" t="inlineStr">
-        <is>
-          <t>2026-03-20</t>
-        </is>
-      </c>
-      <c r="B146" t="inlineStr">
-        <is>
-          <t>스타 벌크 캐리어스</t>
-        </is>
-      </c>
-      <c r="C146" t="n">
-        <v>50</v>
-      </c>
-      <c r="D146" t="inlineStr">
-        <is>
-          <t>KRW</t>
-        </is>
-      </c>
-      <c r="E146" t="n">
-        <v>1</v>
-      </c>
-      <c r="F146" t="n">
-        <v>1696441.320678405</v>
-      </c>
-      <c r="G146" t="n">
-        <v>382088.3206784062</v>
-      </c>
-      <c r="H146" t="n">
-        <v>29.07044916231837</v>
-      </c>
-      <c r="I146" t="inlineStr">
-        <is>
-          <t>2026-03-20T15:47:06</t>
-        </is>
-      </c>
-    </row>
-    <row r="147">
-      <c r="A147" t="inlineStr">
-        <is>
-          <t>2026-03-20</t>
-        </is>
-      </c>
-      <c r="B147" t="inlineStr">
-        <is>
-          <t>유나이티드헬스 그룹</t>
-        </is>
-      </c>
-      <c r="C147" t="n">
-        <v>4</v>
-      </c>
-      <c r="D147" t="inlineStr">
-        <is>
-          <t>KRW</t>
-        </is>
-      </c>
-      <c r="E147" t="n">
-        <v>1</v>
-      </c>
-      <c r="F147" t="n">
-        <v>1683366.447431445</v>
-      </c>
-      <c r="G147" t="n">
-        <v>-11089.55256855441</v>
-      </c>
-      <c r="H147" t="n">
-        <v>-0.6544609342794628</v>
-      </c>
-      <c r="I147" t="inlineStr">
-        <is>
-          <t>2026-03-20T15:47:06</t>
-        </is>
-      </c>
-    </row>
-    <row r="148">
-      <c r="A148" t="inlineStr">
-        <is>
-          <t>2026-03-20</t>
-        </is>
-      </c>
-      <c r="B148" t="inlineStr">
-        <is>
-          <t>케이씨</t>
-        </is>
-      </c>
-      <c r="C148" t="n">
-        <v>50</v>
-      </c>
-      <c r="D148" t="inlineStr">
-        <is>
-          <t>KRW</t>
-        </is>
-      </c>
-      <c r="E148" t="n">
-        <v>1</v>
-      </c>
-      <c r="F148" t="n">
-        <v>1670000</v>
-      </c>
-      <c r="G148" t="n">
-        <v>20499.9999999993</v>
-      </c>
-      <c r="H148" t="n">
-        <v>1.242800848742</v>
-      </c>
-      <c r="I148" t="inlineStr">
-        <is>
-          <t>2026-03-20T15:47:06</t>
-        </is>
-      </c>
-    </row>
-    <row r="149">
-      <c r="A149" t="inlineStr">
-        <is>
-          <t>2026-03-20</t>
-        </is>
-      </c>
-      <c r="B149" t="inlineStr">
-        <is>
-          <t>삼성생명</t>
-        </is>
-      </c>
-      <c r="C149" t="n">
-        <v>4</v>
-      </c>
-      <c r="D149" t="inlineStr">
-        <is>
-          <t>KRW</t>
-        </is>
-      </c>
-      <c r="E149" t="n">
-        <v>1</v>
-      </c>
-      <c r="F149" t="n">
-        <v>926000</v>
-      </c>
-      <c r="G149" t="n">
-        <v>93000</v>
-      </c>
-      <c r="H149" t="n">
-        <v>11.16446578631453</v>
-      </c>
-      <c r="I149" t="inlineStr">
-        <is>
-          <t>2026-03-20T15:47:06</t>
-        </is>
-      </c>
-    </row>
-    <row r="150">
-      <c r="A150" t="inlineStr">
-        <is>
-          <t>2026-03-20</t>
-        </is>
-      </c>
-      <c r="B150" t="inlineStr">
-        <is>
-          <t>비에이치아이</t>
-        </is>
-      </c>
-      <c r="C150" t="n">
-        <v>8</v>
-      </c>
-      <c r="D150" t="inlineStr">
-        <is>
-          <t>KRW</t>
-        </is>
-      </c>
-      <c r="E150" t="n">
-        <v>1</v>
-      </c>
-      <c r="F150" t="n">
-        <v>876000</v>
-      </c>
-      <c r="G150" t="n">
-        <v>210885</v>
-      </c>
-      <c r="H150" t="n">
-        <v>31.70654698811484</v>
-      </c>
-      <c r="I150" t="inlineStr">
-        <is>
-          <t>2026-03-20T15:47:06</t>
-        </is>
-      </c>
-    </row>
-    <row r="151">
-      <c r="A151" t="inlineStr">
-        <is>
-          <t>2026-03-20</t>
-        </is>
-      </c>
-      <c r="B151" t="inlineStr">
-        <is>
-          <t>하프니아</t>
-        </is>
-      </c>
-      <c r="C151" t="n">
-        <v>80</v>
-      </c>
-      <c r="D151" t="inlineStr">
-        <is>
-          <t>KRW</t>
-        </is>
-      </c>
-      <c r="E151" t="n">
-        <v>1</v>
-      </c>
-      <c r="F151" t="n">
-        <v>848519.8631833494</v>
-      </c>
-      <c r="G151" t="n">
-        <v>222788.8631833494</v>
-      </c>
-      <c r="H151" t="n">
-        <v>35.60457499841775</v>
-      </c>
-      <c r="I151" t="inlineStr">
-        <is>
-          <t>2026-03-20T15:47:06</t>
-        </is>
-      </c>
-    </row>
-    <row r="152">
-      <c r="A152" t="inlineStr">
-        <is>
-          <t>2026-03-20</t>
-        </is>
-      </c>
-      <c r="B152" t="inlineStr">
-        <is>
-          <t>클리블랜드 클리프스</t>
-        </is>
-      </c>
-      <c r="C152" t="n">
-        <v>70</v>
-      </c>
-      <c r="D152" t="inlineStr">
-        <is>
-          <t>KRW</t>
-        </is>
-      </c>
-      <c r="E152" t="n">
-        <v>1</v>
-      </c>
-      <c r="F152" t="n">
-        <v>833036.4441346284</v>
-      </c>
-      <c r="G152" t="n">
-        <v>-183018.5558653716</v>
-      </c>
-      <c r="H152" t="n">
-        <v>-18.01266229341636</v>
-      </c>
-      <c r="I152" t="inlineStr">
-        <is>
-          <t>2026-03-20T15:47:06</t>
-        </is>
-      </c>
-    </row>
-    <row r="153">
-      <c r="A153" t="inlineStr">
-        <is>
-          <t>2026-03-20</t>
-        </is>
-      </c>
-      <c r="B153" t="inlineStr">
-        <is>
-          <t>텍사스 퍼시픽 랜드</t>
-        </is>
-      </c>
-      <c r="C153" t="n">
-        <v>1</v>
-      </c>
-      <c r="D153" t="inlineStr">
-        <is>
-          <t>KRW</t>
-        </is>
-      </c>
-      <c r="E153" t="n">
-        <v>1</v>
-      </c>
-      <c r="F153" t="n">
-        <v>798210.0491355956</v>
-      </c>
-      <c r="G153" t="n">
-        <v>19619.04913559556</v>
-      </c>
-      <c r="H153" t="n">
-        <v>2.519814528500273</v>
-      </c>
-      <c r="I153" t="inlineStr">
-        <is>
-          <t>2026-03-20T15:47:06</t>
         </is>
       </c>
     </row>
@@ -7252,7 +5846,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E5"/>
+  <dimension ref="A1:E4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7351,29 +5945,6 @@
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>2026-03-20</t>
-        </is>
-      </c>
-      <c r="B5" t="n">
-        <v>31505056</v>
-      </c>
-      <c r="C5" t="n">
-        <v>6016.63</v>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>2026-03-20T03:06:55</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>2026-03-20T15:47:06</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
auto: portfolio snapshot 2026-03-20 (2026-03-20T15:48:40)
</commit_message>
<xml_diff>
--- a/portfolio_auto.xlsx
+++ b/portfolio_auto.xlsx
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G39"/>
+  <dimension ref="A1:G41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -486,13 +486,13 @@
         <v>1</v>
       </c>
       <c r="E2" t="n">
-        <v>14238562.79623244</v>
+        <v>13553578.62304688</v>
       </c>
       <c r="F2" t="n">
-        <v>2132013.796232443</v>
+        <v>1447029.623046879</v>
       </c>
       <c r="G2" t="n">
-        <v>17.61041727277066</v>
+        <v>11.95245336261291</v>
       </c>
     </row>
     <row r="3">
@@ -513,13 +513,13 @@
         <v>1</v>
       </c>
       <c r="E3" t="n">
-        <v>10802195.38683411</v>
+        <v>10351433.71453537</v>
       </c>
       <c r="F3" t="n">
-        <v>-29819.61316589266</v>
+        <v>-480581.2854646351</v>
       </c>
       <c r="G3" t="n">
-        <v>-0.2752914685392576</v>
+        <v>-4.436674851951692</v>
       </c>
     </row>
     <row r="4">
@@ -540,13 +540,13 @@
         <v>1</v>
       </c>
       <c r="E4" t="n">
-        <v>9490000</v>
+        <v>9120000</v>
       </c>
       <c r="F4" t="n">
-        <v>2277000</v>
+        <v>1907000</v>
       </c>
       <c r="G4" t="n">
-        <v>31.56800221821711</v>
+        <v>26.43837515596839</v>
       </c>
     </row>
     <row r="5">
@@ -567,13 +567,13 @@
         <v>1</v>
       </c>
       <c r="E5" t="n">
-        <v>8629159.309373179</v>
+        <v>8453409.11431564</v>
       </c>
       <c r="F5" t="n">
-        <v>4199295.309373179</v>
+        <v>4023545.11431564</v>
       </c>
       <c r="G5" t="n">
-        <v>94.79512936228244</v>
+        <v>90.82773453802736</v>
       </c>
     </row>
     <row r="6">
@@ -594,13 +594,13 @@
         <v>1</v>
       </c>
       <c r="E6" t="n">
-        <v>8280438.313577486</v>
+        <v>8081063.113214018</v>
       </c>
       <c r="F6" t="n">
-        <v>1830087.313577486</v>
+        <v>1630712.113214018</v>
       </c>
       <c r="G6" t="n">
-        <v>28.37190276277192</v>
+        <v>25.28098258860669</v>
       </c>
     </row>
     <row r="7">
@@ -621,13 +621,13 @@
         <v>1</v>
       </c>
       <c r="E7" t="n">
-        <v>7265949.903135682</v>
+        <v>7074115.140040115</v>
       </c>
       <c r="F7" t="n">
-        <v>3138715.903135683</v>
+        <v>2946881.140040115</v>
       </c>
       <c r="G7" t="n">
-        <v>76.04889626165328</v>
+        <v>71.40087380652794</v>
       </c>
     </row>
     <row r="8">
@@ -648,13 +648,13 @@
         <v>1</v>
       </c>
       <c r="E8" t="n">
-        <v>7089362.533905029</v>
+        <v>6886743.840087891</v>
       </c>
       <c r="F8" t="n">
-        <v>3182154.533905029</v>
+        <v>2979535.840087891</v>
       </c>
       <c r="G8" t="n">
-        <v>81.4431822903984</v>
+        <v>76.25741552760668</v>
       </c>
     </row>
     <row r="9">
@@ -675,13 +675,13 @@
         <v>1</v>
       </c>
       <c r="E9" t="n">
-        <v>6945000</v>
+        <v>7395000</v>
       </c>
       <c r="F9" t="n">
-        <v>635000</v>
+        <v>1085000</v>
       </c>
       <c r="G9" t="n">
-        <v>10.06339144215531</v>
+        <v>17.19492868462758</v>
       </c>
     </row>
     <row r="10">
@@ -702,13 +702,13 @@
         <v>1</v>
       </c>
       <c r="E10" t="n">
-        <v>6458956.91119526</v>
+        <v>5996448.754211426</v>
       </c>
       <c r="F10" t="n">
-        <v>227737.9111952605</v>
+        <v>-234770.2457885733</v>
       </c>
       <c r="G10" t="n">
-        <v>3.654789074100277</v>
+        <v>-3.767645556809564</v>
       </c>
     </row>
     <row r="11">
@@ -729,13 +729,13 @@
         <v>1</v>
       </c>
       <c r="E11" t="n">
-        <v>5347019.162831247</v>
+        <v>5211036.802851856</v>
       </c>
       <c r="F11" t="n">
-        <v>1622474.162831247</v>
+        <v>1486491.802851856</v>
       </c>
       <c r="G11" t="n">
-        <v>43.56167432078944</v>
+        <v>39.91069520845783</v>
       </c>
     </row>
     <row r="12">
@@ -756,23 +756,23 @@
         <v>1</v>
       </c>
       <c r="E12" t="n">
-        <v>5157624.699054079</v>
+        <v>5179494.129107101</v>
       </c>
       <c r="F12" t="n">
-        <v>1847616.699054079</v>
+        <v>1869486.129107101</v>
       </c>
       <c r="G12" t="n">
-        <v>55.81910071075596</v>
+        <v>56.47980697046958</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>TIME 코리아밸류업액티브</t>
+          <t>오케아니스 에코 탱커스</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>201</v>
+        <v>65</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
@@ -783,23 +783,23 @@
         <v>1</v>
       </c>
       <c r="E13" t="n">
-        <v>4763700</v>
+        <v>4596307.895957222</v>
       </c>
       <c r="F13" t="n">
-        <v>39903</v>
+        <v>2339947.895957222</v>
       </c>
       <c r="G13" t="n">
-        <v>0.8447230056668396</v>
+        <v>103.704546081176</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>오케아니스 에코 탱커스</t>
+          <t>삼성화재</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>65</v>
+        <v>9</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
@@ -810,23 +810,23 @@
         <v>1</v>
       </c>
       <c r="E14" t="n">
-        <v>4596144.593352056</v>
+        <v>4270500</v>
       </c>
       <c r="F14" t="n">
-        <v>2339784.593352056</v>
+        <v>-360500</v>
       </c>
       <c r="G14" t="n">
-        <v>103.6973086454314</v>
+        <v>-7.784495789246384</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>삼성화재</t>
+          <t>차코스 에너지 내비게이션</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>9</v>
+        <v>75</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
@@ -837,23 +837,23 @@
         <v>1</v>
       </c>
       <c r="E15" t="n">
-        <v>4306500</v>
+        <v>4052048.962918622</v>
       </c>
       <c r="F15" t="n">
-        <v>-324500</v>
+        <v>227400.9629186224</v>
       </c>
       <c r="G15" t="n">
-        <v>-7.007125890736342</v>
+        <v>5.94567037067522</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>DL이앤씨</t>
+          <t>동원개발</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>80</v>
+        <v>1360</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
@@ -864,23 +864,23 @@
         <v>1</v>
       </c>
       <c r="E16" t="n">
-        <v>4152000</v>
+        <v>4202400</v>
       </c>
       <c r="F16" t="n">
-        <v>741000</v>
+        <v>465000</v>
       </c>
       <c r="G16" t="n">
-        <v>21.72383465259455</v>
+        <v>12.44180446299566</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>HD건설기계</t>
+          <t>피바디 에너지</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>31</v>
+        <v>65</v>
       </c>
       <c r="C17" t="inlineStr">
         <is>
@@ -891,23 +891,23 @@
         <v>1</v>
       </c>
       <c r="E17" t="n">
-        <v>4082700</v>
+        <v>3596373.331896178</v>
       </c>
       <c r="F17" t="n">
-        <v>47604</v>
+        <v>2125601.331896178</v>
       </c>
       <c r="G17" t="n">
-        <v>1.179748883297944</v>
+        <v>144.5228309959789</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>차코스 에너지 내비게이션</t>
+          <t>더치 브로스</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>75</v>
+        <v>39</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
@@ -918,23 +918,23 @@
         <v>1</v>
       </c>
       <c r="E18" t="n">
-        <v>4081754.289162601</v>
+        <v>2959763.281021703</v>
       </c>
       <c r="F18" t="n">
-        <v>257106.2891626009</v>
+        <v>-230880.718978297</v>
       </c>
       <c r="G18" t="n">
-        <v>6.722351682105146</v>
+        <v>-7.236179247145621</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>동원개발</t>
+          <t>넥스틸</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>1360</v>
+        <v>200</v>
       </c>
       <c r="C19" t="inlineStr">
         <is>
@@ -945,23 +945,23 @@
         <v>1</v>
       </c>
       <c r="E19" t="n">
-        <v>3957600</v>
+        <v>2514000</v>
       </c>
       <c r="F19" t="n">
-        <v>220200</v>
+        <v>503000</v>
       </c>
       <c r="G19" t="n">
-        <v>5.891796436025045</v>
+        <v>25.01243162605669</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>피바디 에너지</t>
+          <t>대신증권</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>65</v>
+        <v>55</v>
       </c>
       <c r="C20" t="inlineStr">
         <is>
@@ -972,23 +972,23 @@
         <v>1</v>
       </c>
       <c r="E20" t="n">
-        <v>3650596.24511658</v>
+        <v>2219250</v>
       </c>
       <c r="F20" t="n">
-        <v>2179824.24511658</v>
+        <v>509749</v>
       </c>
       <c r="G20" t="n">
-        <v>148.2095284052579</v>
+        <v>29.81858448752005</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>더치 브로스</t>
+          <t>발레로 에너지</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>39</v>
+        <v>6</v>
       </c>
       <c r="C21" t="inlineStr">
         <is>
@@ -999,23 +999,23 @@
         <v>1</v>
       </c>
       <c r="E21" t="n">
-        <v>2978769.518133399</v>
+        <v>2176561.162089184</v>
       </c>
       <c r="F21" t="n">
-        <v>-211874.4818666009</v>
+        <v>112571.1620891844</v>
       </c>
       <c r="G21" t="n">
-        <v>-6.640492698859569</v>
+        <v>5.45405559567558</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>휴스틸</t>
+          <t>미창석유</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>500</v>
+        <v>18</v>
       </c>
       <c r="C22" t="inlineStr">
         <is>
@@ -1026,23 +1026,23 @@
         <v>1</v>
       </c>
       <c r="E22" t="n">
-        <v>2620000</v>
+        <v>2097000</v>
       </c>
       <c r="F22" t="n">
-        <v>341390</v>
+        <v>-295200</v>
       </c>
       <c r="G22" t="n">
-        <v>14.98237960862105</v>
+        <v>-12.34010534236268</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>KoAct 코스닥액티브</t>
+          <t>대창단조</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>200</v>
+        <v>300</v>
       </c>
       <c r="C23" t="inlineStr">
         <is>
@@ -1053,23 +1053,23 @@
         <v>1</v>
       </c>
       <c r="E23" t="n">
-        <v>2526000</v>
+        <v>2004000</v>
       </c>
       <c r="F23" t="n">
-        <v>-176000</v>
+        <v>-54000</v>
       </c>
       <c r="G23" t="n">
-        <v>-6.513693560325684</v>
+        <v>-2.623906705539359</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>현대제철</t>
+          <t>동방</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>70</v>
+        <v>681</v>
       </c>
       <c r="C24" t="inlineStr">
         <is>
@@ -1080,23 +1080,23 @@
         <v>1</v>
       </c>
       <c r="E24" t="n">
-        <v>2509500</v>
+        <v>1995330</v>
       </c>
       <c r="F24" t="n">
-        <v>-298000</v>
+        <v>23829</v>
       </c>
       <c r="G24" t="n">
-        <v>-10.61442564559216</v>
+        <v>1.208672985709873</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>넥스틸</t>
+          <t>스타 벌크 캐리어스</t>
         </is>
       </c>
       <c r="B25" t="n">
-        <v>200</v>
+        <v>50</v>
       </c>
       <c r="C25" t="inlineStr">
         <is>
@@ -1107,23 +1107,23 @@
         <v>1</v>
       </c>
       <c r="E25" t="n">
-        <v>2406000</v>
+        <v>1696441.320678405</v>
       </c>
       <c r="F25" t="n">
-        <v>395000</v>
+        <v>382088.3206784062</v>
       </c>
       <c r="G25" t="n">
-        <v>19.64196916956738</v>
+        <v>29.07044916231837</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>대신증권</t>
+          <t>유나이티드헬스 그룹</t>
         </is>
       </c>
       <c r="B26" t="n">
-        <v>55</v>
+        <v>4</v>
       </c>
       <c r="C26" t="inlineStr">
         <is>
@@ -1134,23 +1134,23 @@
         <v>1</v>
       </c>
       <c r="E26" t="n">
-        <v>2180750</v>
+        <v>1683366.447431445</v>
       </c>
       <c r="F26" t="n">
-        <v>471249</v>
+        <v>-11089.55256855441</v>
       </c>
       <c r="G26" t="n">
-        <v>27.56646530186294</v>
+        <v>-0.6544609342794628</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>발레로 에너지</t>
+          <t>삼성생명</t>
         </is>
       </c>
       <c r="B27" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C27" t="inlineStr">
         <is>
@@ -1161,23 +1161,23 @@
         <v>1</v>
       </c>
       <c r="E27" t="n">
-        <v>2178165.369514748</v>
+        <v>926000</v>
       </c>
       <c r="F27" t="n">
-        <v>114175.3695147485</v>
+        <v>93000</v>
       </c>
       <c r="G27" t="n">
-        <v>5.531779200226186</v>
+        <v>11.16446578631453</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>미창석유</t>
+          <t>클리블랜드 클리프스</t>
         </is>
       </c>
       <c r="B28" t="n">
-        <v>18</v>
+        <v>70</v>
       </c>
       <c r="C28" t="inlineStr">
         <is>
@@ -1188,23 +1188,23 @@
         <v>1</v>
       </c>
       <c r="E28" t="n">
-        <v>2023200</v>
+        <v>833036.4441346284</v>
       </c>
       <c r="F28" t="n">
-        <v>-369000</v>
+        <v>-183018.5558653716</v>
       </c>
       <c r="G28" t="n">
-        <v>-15.42513167795335</v>
+        <v>-18.01266229341636</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>대창단조</t>
+          <t>하프니아</t>
         </is>
       </c>
       <c r="B29" t="n">
-        <v>300</v>
+        <v>80</v>
       </c>
       <c r="C29" t="inlineStr">
         <is>
@@ -1215,23 +1215,23 @@
         <v>1</v>
       </c>
       <c r="E29" t="n">
-        <v>1938000</v>
+        <v>848519.8631833494</v>
       </c>
       <c r="F29" t="n">
-        <v>-120000</v>
+        <v>222788.8631833494</v>
       </c>
       <c r="G29" t="n">
-        <v>-5.830903790087463</v>
+        <v>35.60457499841775</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>동방</t>
+          <t>비에이치아이</t>
         </is>
       </c>
       <c r="B30" t="n">
-        <v>681</v>
+        <v>8</v>
       </c>
       <c r="C30" t="inlineStr">
         <is>
@@ -1242,23 +1242,23 @@
         <v>1</v>
       </c>
       <c r="E30" t="n">
-        <v>1906800</v>
+        <v>876000</v>
       </c>
       <c r="F30" t="n">
-        <v>-64701</v>
+        <v>210885</v>
       </c>
       <c r="G30" t="n">
-        <v>-3.281814211608312</v>
+        <v>31.70654698811484</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>스타 벌크 캐리어스</t>
+          <t>텍사스 퍼시픽 랜드</t>
         </is>
       </c>
       <c r="B31" t="n">
-        <v>50</v>
+        <v>1</v>
       </c>
       <c r="C31" t="inlineStr">
         <is>
@@ -1269,23 +1269,23 @@
         <v>1</v>
       </c>
       <c r="E31" t="n">
-        <v>1704386.346717528</v>
+        <v>798210.0491355956</v>
       </c>
       <c r="F31" t="n">
-        <v>390033.3467175288</v>
+        <v>19619.04913559556</v>
       </c>
       <c r="G31" t="n">
-        <v>29.67493106627588</v>
+        <v>2.519814528500273</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>하나금융지주</t>
+          <t>케이씨</t>
         </is>
       </c>
       <c r="B32" t="n">
-        <v>15</v>
+        <v>50</v>
       </c>
       <c r="C32" t="inlineStr">
         <is>
@@ -1296,23 +1296,23 @@
         <v>1</v>
       </c>
       <c r="E32" t="n">
-        <v>1698000</v>
+        <v>1670000</v>
       </c>
       <c r="F32" t="n">
-        <v>15500</v>
+        <v>20500</v>
       </c>
       <c r="G32" t="n">
-        <v>0.9212481426448738</v>
+        <v>1.242800848742043</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>유나이티드헬스 그룹</t>
+          <t>하나금융지주</t>
         </is>
       </c>
       <c r="B33" t="n">
-        <v>4</v>
+        <v>18</v>
       </c>
       <c r="C33" t="inlineStr">
         <is>
@@ -1323,23 +1323,23 @@
         <v>1</v>
       </c>
       <c r="E33" t="n">
-        <v>1682281.111696094</v>
+        <v>2037600</v>
       </c>
       <c r="F33" t="n">
-        <v>-12174.88830390549</v>
+        <v>12200</v>
       </c>
       <c r="G33" t="n">
-        <v>-0.7185130982395231</v>
+        <v>0.6023501530561864</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>케이씨</t>
+          <t>현대제철</t>
         </is>
       </c>
       <c r="B34" t="n">
-        <v>50</v>
+        <v>80</v>
       </c>
       <c r="C34" t="inlineStr">
         <is>
@@ -1350,23 +1350,23 @@
         <v>1</v>
       </c>
       <c r="E34" t="n">
-        <v>1627500</v>
+        <v>2996000</v>
       </c>
       <c r="F34" t="n">
-        <v>-22000.0000000007</v>
+        <v>-182000</v>
       </c>
       <c r="G34" t="n">
-        <v>-1.333737496211015</v>
+        <v>-5.726872246696035</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>삼성생명</t>
+          <t>휴스틸</t>
         </is>
       </c>
       <c r="B35" t="n">
-        <v>4</v>
+        <v>500</v>
       </c>
       <c r="C35" t="inlineStr">
         <is>
@@ -1377,23 +1377,23 @@
         <v>1</v>
       </c>
       <c r="E35" t="n">
-        <v>922000</v>
+        <v>2750000</v>
       </c>
       <c r="F35" t="n">
-        <v>89000</v>
+        <v>471390</v>
       </c>
       <c r="G35" t="n">
-        <v>10.68427370948379</v>
+        <v>20.68761218462133</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>클리블랜드 클리프스</t>
+          <t>DL이앤씨</t>
         </is>
       </c>
       <c r="B36" t="n">
-        <v>70</v>
+        <v>40</v>
       </c>
       <c r="C36" t="inlineStr">
         <is>
@@ -1404,23 +1404,23 @@
         <v>1</v>
       </c>
       <c r="E36" t="n">
-        <v>858716.8307915051</v>
+        <v>2696000</v>
       </c>
       <c r="F36" t="n">
-        <v>-157338.1692084949</v>
+        <v>990500</v>
       </c>
       <c r="G36" t="n">
-        <v>-15.48520200269621</v>
+        <v>58.07681031955438</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>하프니아</t>
+          <t>HD건설기계</t>
         </is>
       </c>
       <c r="B37" t="n">
-        <v>80</v>
+        <v>31</v>
       </c>
       <c r="C37" t="inlineStr">
         <is>
@@ -1431,23 +1431,23 @@
         <v>1</v>
       </c>
       <c r="E37" t="n">
-        <v>855417.5163666997</v>
+        <v>4123000</v>
       </c>
       <c r="F37" t="n">
-        <v>229686.5163666997</v>
+        <v>87904</v>
       </c>
       <c r="G37" t="n">
-        <v>36.70691021648275</v>
+        <v>2.178485964150543</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>비에이치아이</t>
+          <t>KoAct 코스닥액티브</t>
         </is>
       </c>
       <c r="B38" t="n">
-        <v>8</v>
+        <v>200</v>
       </c>
       <c r="C38" t="inlineStr">
         <is>
@@ -1458,23 +1458,23 @@
         <v>1</v>
       </c>
       <c r="E38" t="n">
-        <v>834400</v>
+        <v>2582000</v>
       </c>
       <c r="F38" t="n">
-        <v>169285</v>
+        <v>-120000</v>
       </c>
       <c r="G38" t="n">
-        <v>25.45198950557423</v>
+        <v>-4.441154700222058</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>텍사스 퍼시픽 랜드</t>
+          <t>LX인터내셔널</t>
         </is>
       </c>
       <c r="B39" t="n">
-        <v>1</v>
+        <v>20</v>
       </c>
       <c r="C39" t="inlineStr">
         <is>
@@ -1485,13 +1485,67 @@
         <v>1</v>
       </c>
       <c r="E39" t="n">
-        <v>798609.6514927745</v>
+        <v>943000</v>
       </c>
       <c r="F39" t="n">
-        <v>20018.65149277449</v>
+        <v>4000</v>
       </c>
       <c r="G39" t="n">
-        <v>2.571138311741914</v>
+        <v>0.4259850905218318</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>NH투자증권우</t>
+        </is>
+      </c>
+      <c r="B40" t="n">
+        <v>2</v>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="D40" t="n">
+        <v>1</v>
+      </c>
+      <c r="E40" t="n">
+        <v>54591</v>
+      </c>
+      <c r="F40" t="n">
+        <v>-9</v>
+      </c>
+      <c r="G40" t="n">
+        <v>-0.01648351648351648</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>TIME 코리아밸류업액티브</t>
+        </is>
+      </c>
+      <c r="B41" t="n">
+        <v>201</v>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="D41" t="n">
+        <v>1</v>
+      </c>
+      <c r="E41" t="n">
+        <v>4797870</v>
+      </c>
+      <c r="F41" t="n">
+        <v>74073</v>
+      </c>
+      <c r="G41" t="n">
+        <v>1.568081778281328</v>
       </c>
     </row>
   </sheetData>
@@ -1538,7 +1592,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-03-19</t>
+          <t>2026-03-20</t>
         </is>
       </c>
       <c r="B2" t="n">
@@ -1549,11 +1603,11 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2026-03-20T15:47:44</t>
+          <t>2026-03-20T15:48:40</t>
         </is>
       </c>
       <c r="E2" t="n">
-        <v>1499.680053710938</v>
+        <v>1495.97998046875</v>
       </c>
     </row>
   </sheetData>
@@ -1567,7 +1621,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I115"/>
+  <dimension ref="A1:I155"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5832,6 +5886,1486 @@
       <c r="I115" t="inlineStr">
         <is>
           <t>2026-03-19T21:54:06</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>2026-03-20</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>페트로브라스 (ADR)</t>
+        </is>
+      </c>
+      <c r="C116" t="n">
+        <v>480</v>
+      </c>
+      <c r="D116" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E116" t="n">
+        <v>1</v>
+      </c>
+      <c r="F116" t="n">
+        <v>13553578.62304688</v>
+      </c>
+      <c r="G116" t="n">
+        <v>1447029.623046879</v>
+      </c>
+      <c r="H116" t="n">
+        <v>11.95245336261291</v>
+      </c>
+      <c r="I116" t="inlineStr">
+        <is>
+          <t>2026-03-20T15:48:40</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>2026-03-20</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>AGNC 인베스트먼트</t>
+        </is>
+      </c>
+      <c r="C117" t="n">
+        <v>700</v>
+      </c>
+      <c r="D117" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E117" t="n">
+        <v>1</v>
+      </c>
+      <c r="F117" t="n">
+        <v>10351433.71453537</v>
+      </c>
+      <c r="G117" t="n">
+        <v>-480581.2854646351</v>
+      </c>
+      <c r="H117" t="n">
+        <v>-4.436674851951692</v>
+      </c>
+      <c r="I117" t="inlineStr">
+        <is>
+          <t>2026-03-20T15:48:40</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>2026-03-20</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>대한조선</t>
+        </is>
+      </c>
+      <c r="C118" t="n">
+        <v>100</v>
+      </c>
+      <c r="D118" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E118" t="n">
+        <v>1</v>
+      </c>
+      <c r="F118" t="n">
+        <v>9120000</v>
+      </c>
+      <c r="G118" t="n">
+        <v>1907000</v>
+      </c>
+      <c r="H118" t="n">
+        <v>26.43837515596839</v>
+      </c>
+      <c r="I118" t="inlineStr">
+        <is>
+          <t>2026-03-20T15:48:40</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>2026-03-20</t>
+        </is>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>프론트라인</t>
+        </is>
+      </c>
+      <c r="C119" t="n">
+        <v>175</v>
+      </c>
+      <c r="D119" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E119" t="n">
+        <v>1</v>
+      </c>
+      <c r="F119" t="n">
+        <v>8453409.11431564</v>
+      </c>
+      <c r="G119" t="n">
+        <v>4023545.11431564</v>
+      </c>
+      <c r="H119" t="n">
+        <v>90.82773453802736</v>
+      </c>
+      <c r="I119" t="inlineStr">
+        <is>
+          <t>2026-03-20T15:48:40</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>2026-03-20</t>
+        </is>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>시드릴</t>
+        </is>
+      </c>
+      <c r="C120" t="n">
+        <v>123</v>
+      </c>
+      <c r="D120" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E120" t="n">
+        <v>1</v>
+      </c>
+      <c r="F120" t="n">
+        <v>8081063.113214018</v>
+      </c>
+      <c r="G120" t="n">
+        <v>1630712.113214018</v>
+      </c>
+      <c r="H120" t="n">
+        <v>25.28098258860669</v>
+      </c>
+      <c r="I120" t="inlineStr">
+        <is>
+          <t>2026-03-20T15:48:40</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>2026-03-20</t>
+        </is>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>세아제강</t>
+        </is>
+      </c>
+      <c r="C121" t="n">
+        <v>50</v>
+      </c>
+      <c r="D121" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E121" t="n">
+        <v>1</v>
+      </c>
+      <c r="F121" t="n">
+        <v>7395000</v>
+      </c>
+      <c r="G121" t="n">
+        <v>1085000</v>
+      </c>
+      <c r="H121" t="n">
+        <v>17.19492868462758</v>
+      </c>
+      <c r="I121" t="inlineStr">
+        <is>
+          <t>2026-03-20T15:48:40</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>2026-03-20</t>
+        </is>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>트랜스오션</t>
+        </is>
+      </c>
+      <c r="C122" t="n">
+        <v>750</v>
+      </c>
+      <c r="D122" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E122" t="n">
+        <v>1</v>
+      </c>
+      <c r="F122" t="n">
+        <v>7074115.140040115</v>
+      </c>
+      <c r="G122" t="n">
+        <v>2946881.140040115</v>
+      </c>
+      <c r="H122" t="n">
+        <v>71.40087380652794</v>
+      </c>
+      <c r="I122" t="inlineStr">
+        <is>
+          <t>2026-03-20T15:48:40</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>2026-03-20</t>
+        </is>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>노블</t>
+        </is>
+      </c>
+      <c r="C123" t="n">
+        <v>99</v>
+      </c>
+      <c r="D123" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E123" t="n">
+        <v>1</v>
+      </c>
+      <c r="F123" t="n">
+        <v>6886743.840087891</v>
+      </c>
+      <c r="G123" t="n">
+        <v>2979535.840087891</v>
+      </c>
+      <c r="H123" t="n">
+        <v>76.25741552760668</v>
+      </c>
+      <c r="I123" t="inlineStr">
+        <is>
+          <t>2026-03-20T15:48:40</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>2026-03-20</t>
+        </is>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>센트러스 에너지</t>
+        </is>
+      </c>
+      <c r="C124" t="n">
+        <v>21</v>
+      </c>
+      <c r="D124" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E124" t="n">
+        <v>1</v>
+      </c>
+      <c r="F124" t="n">
+        <v>5996448.754211426</v>
+      </c>
+      <c r="G124" t="n">
+        <v>-234770.2457885733</v>
+      </c>
+      <c r="H124" t="n">
+        <v>-3.767645556809564</v>
+      </c>
+      <c r="I124" t="inlineStr">
+        <is>
+          <t>2026-03-20T15:48:40</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>2026-03-20</t>
+        </is>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>타이드워터</t>
+        </is>
+      </c>
+      <c r="C125" t="n">
+        <v>48</v>
+      </c>
+      <c r="D125" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E125" t="n">
+        <v>1</v>
+      </c>
+      <c r="F125" t="n">
+        <v>5211036.802851856</v>
+      </c>
+      <c r="G125" t="n">
+        <v>1486491.802851856</v>
+      </c>
+      <c r="H125" t="n">
+        <v>39.91069520845783</v>
+      </c>
+      <c r="I125" t="inlineStr">
+        <is>
+          <t>2026-03-20T15:48:40</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>2026-03-20</t>
+        </is>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>노브</t>
+        </is>
+      </c>
+      <c r="C126" t="n">
+        <v>185</v>
+      </c>
+      <c r="D126" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E126" t="n">
+        <v>1</v>
+      </c>
+      <c r="F126" t="n">
+        <v>5179494.129107101</v>
+      </c>
+      <c r="G126" t="n">
+        <v>1869486.129107101</v>
+      </c>
+      <c r="H126" t="n">
+        <v>56.47980697046958</v>
+      </c>
+      <c r="I126" t="inlineStr">
+        <is>
+          <t>2026-03-20T15:48:40</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>2026-03-20</t>
+        </is>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>TIME 코리아밸류업액티브</t>
+        </is>
+      </c>
+      <c r="C127" t="n">
+        <v>201</v>
+      </c>
+      <c r="D127" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E127" t="n">
+        <v>1</v>
+      </c>
+      <c r="F127" t="n">
+        <v>4797870</v>
+      </c>
+      <c r="G127" t="n">
+        <v>74073</v>
+      </c>
+      <c r="H127" t="n">
+        <v>1.568081778281328</v>
+      </c>
+      <c r="I127" t="inlineStr">
+        <is>
+          <t>2026-03-20T15:48:40</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>2026-03-20</t>
+        </is>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>오케아니스 에코 탱커스</t>
+        </is>
+      </c>
+      <c r="C128" t="n">
+        <v>65</v>
+      </c>
+      <c r="D128" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E128" t="n">
+        <v>1</v>
+      </c>
+      <c r="F128" t="n">
+        <v>4596307.895957222</v>
+      </c>
+      <c r="G128" t="n">
+        <v>2339947.895957222</v>
+      </c>
+      <c r="H128" t="n">
+        <v>103.704546081176</v>
+      </c>
+      <c r="I128" t="inlineStr">
+        <is>
+          <t>2026-03-20T15:48:40</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>2026-03-20</t>
+        </is>
+      </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>삼성화재</t>
+        </is>
+      </c>
+      <c r="C129" t="n">
+        <v>9</v>
+      </c>
+      <c r="D129" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E129" t="n">
+        <v>1</v>
+      </c>
+      <c r="F129" t="n">
+        <v>4270500</v>
+      </c>
+      <c r="G129" t="n">
+        <v>-360500</v>
+      </c>
+      <c r="H129" t="n">
+        <v>-7.784495789246384</v>
+      </c>
+      <c r="I129" t="inlineStr">
+        <is>
+          <t>2026-03-20T15:48:40</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>2026-03-20</t>
+        </is>
+      </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>동원개발</t>
+        </is>
+      </c>
+      <c r="C130" t="n">
+        <v>1360</v>
+      </c>
+      <c r="D130" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E130" t="n">
+        <v>1</v>
+      </c>
+      <c r="F130" t="n">
+        <v>4202400</v>
+      </c>
+      <c r="G130" t="n">
+        <v>465000</v>
+      </c>
+      <c r="H130" t="n">
+        <v>12.44180446299566</v>
+      </c>
+      <c r="I130" t="inlineStr">
+        <is>
+          <t>2026-03-20T15:48:40</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>2026-03-20</t>
+        </is>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>HD건설기계</t>
+        </is>
+      </c>
+      <c r="C131" t="n">
+        <v>31</v>
+      </c>
+      <c r="D131" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E131" t="n">
+        <v>1</v>
+      </c>
+      <c r="F131" t="n">
+        <v>4123000</v>
+      </c>
+      <c r="G131" t="n">
+        <v>87904</v>
+      </c>
+      <c r="H131" t="n">
+        <v>2.178485964150543</v>
+      </c>
+      <c r="I131" t="inlineStr">
+        <is>
+          <t>2026-03-20T15:48:40</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>2026-03-20</t>
+        </is>
+      </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>차코스 에너지 내비게이션</t>
+        </is>
+      </c>
+      <c r="C132" t="n">
+        <v>75</v>
+      </c>
+      <c r="D132" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E132" t="n">
+        <v>1</v>
+      </c>
+      <c r="F132" t="n">
+        <v>4052048.962918622</v>
+      </c>
+      <c r="G132" t="n">
+        <v>227400.9629186224</v>
+      </c>
+      <c r="H132" t="n">
+        <v>5.94567037067522</v>
+      </c>
+      <c r="I132" t="inlineStr">
+        <is>
+          <t>2026-03-20T15:48:40</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>2026-03-20</t>
+        </is>
+      </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>피바디 에너지</t>
+        </is>
+      </c>
+      <c r="C133" t="n">
+        <v>65</v>
+      </c>
+      <c r="D133" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E133" t="n">
+        <v>1</v>
+      </c>
+      <c r="F133" t="n">
+        <v>3596373.331896178</v>
+      </c>
+      <c r="G133" t="n">
+        <v>2125601.331896178</v>
+      </c>
+      <c r="H133" t="n">
+        <v>144.5228309959789</v>
+      </c>
+      <c r="I133" t="inlineStr">
+        <is>
+          <t>2026-03-20T15:48:40</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>2026-03-20</t>
+        </is>
+      </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>현대제철</t>
+        </is>
+      </c>
+      <c r="C134" t="n">
+        <v>80</v>
+      </c>
+      <c r="D134" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E134" t="n">
+        <v>1</v>
+      </c>
+      <c r="F134" t="n">
+        <v>2996000</v>
+      </c>
+      <c r="G134" t="n">
+        <v>-182000</v>
+      </c>
+      <c r="H134" t="n">
+        <v>-5.726872246696035</v>
+      </c>
+      <c r="I134" t="inlineStr">
+        <is>
+          <t>2026-03-20T15:48:40</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>2026-03-20</t>
+        </is>
+      </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>더치 브로스</t>
+        </is>
+      </c>
+      <c r="C135" t="n">
+        <v>39</v>
+      </c>
+      <c r="D135" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E135" t="n">
+        <v>1</v>
+      </c>
+      <c r="F135" t="n">
+        <v>2959763.281021703</v>
+      </c>
+      <c r="G135" t="n">
+        <v>-230880.718978297</v>
+      </c>
+      <c r="H135" t="n">
+        <v>-7.236179247145621</v>
+      </c>
+      <c r="I135" t="inlineStr">
+        <is>
+          <t>2026-03-20T15:48:40</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="inlineStr">
+        <is>
+          <t>2026-03-20</t>
+        </is>
+      </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>휴스틸</t>
+        </is>
+      </c>
+      <c r="C136" t="n">
+        <v>500</v>
+      </c>
+      <c r="D136" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E136" t="n">
+        <v>1</v>
+      </c>
+      <c r="F136" t="n">
+        <v>2750000</v>
+      </c>
+      <c r="G136" t="n">
+        <v>471390</v>
+      </c>
+      <c r="H136" t="n">
+        <v>20.68761218462133</v>
+      </c>
+      <c r="I136" t="inlineStr">
+        <is>
+          <t>2026-03-20T15:48:40</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="inlineStr">
+        <is>
+          <t>2026-03-20</t>
+        </is>
+      </c>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>DL이앤씨</t>
+        </is>
+      </c>
+      <c r="C137" t="n">
+        <v>40</v>
+      </c>
+      <c r="D137" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E137" t="n">
+        <v>1</v>
+      </c>
+      <c r="F137" t="n">
+        <v>2696000</v>
+      </c>
+      <c r="G137" t="n">
+        <v>990500</v>
+      </c>
+      <c r="H137" t="n">
+        <v>58.07681031955438</v>
+      </c>
+      <c r="I137" t="inlineStr">
+        <is>
+          <t>2026-03-20T15:48:40</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="inlineStr">
+        <is>
+          <t>2026-03-20</t>
+        </is>
+      </c>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>KoAct 코스닥액티브</t>
+        </is>
+      </c>
+      <c r="C138" t="n">
+        <v>200</v>
+      </c>
+      <c r="D138" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E138" t="n">
+        <v>1</v>
+      </c>
+      <c r="F138" t="n">
+        <v>2582000</v>
+      </c>
+      <c r="G138" t="n">
+        <v>-120000</v>
+      </c>
+      <c r="H138" t="n">
+        <v>-4.441154700222058</v>
+      </c>
+      <c r="I138" t="inlineStr">
+        <is>
+          <t>2026-03-20T15:48:40</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="inlineStr">
+        <is>
+          <t>2026-03-20</t>
+        </is>
+      </c>
+      <c r="B139" t="inlineStr">
+        <is>
+          <t>넥스틸</t>
+        </is>
+      </c>
+      <c r="C139" t="n">
+        <v>200</v>
+      </c>
+      <c r="D139" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E139" t="n">
+        <v>1</v>
+      </c>
+      <c r="F139" t="n">
+        <v>2514000</v>
+      </c>
+      <c r="G139" t="n">
+        <v>503000</v>
+      </c>
+      <c r="H139" t="n">
+        <v>25.01243162605669</v>
+      </c>
+      <c r="I139" t="inlineStr">
+        <is>
+          <t>2026-03-20T15:48:40</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="inlineStr">
+        <is>
+          <t>2026-03-20</t>
+        </is>
+      </c>
+      <c r="B140" t="inlineStr">
+        <is>
+          <t>대신증권</t>
+        </is>
+      </c>
+      <c r="C140" t="n">
+        <v>55</v>
+      </c>
+      <c r="D140" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E140" t="n">
+        <v>1</v>
+      </c>
+      <c r="F140" t="n">
+        <v>2219250</v>
+      </c>
+      <c r="G140" t="n">
+        <v>509749</v>
+      </c>
+      <c r="H140" t="n">
+        <v>29.81858448752005</v>
+      </c>
+      <c r="I140" t="inlineStr">
+        <is>
+          <t>2026-03-20T15:48:40</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="inlineStr">
+        <is>
+          <t>2026-03-20</t>
+        </is>
+      </c>
+      <c r="B141" t="inlineStr">
+        <is>
+          <t>발레로 에너지</t>
+        </is>
+      </c>
+      <c r="C141" t="n">
+        <v>6</v>
+      </c>
+      <c r="D141" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E141" t="n">
+        <v>1</v>
+      </c>
+      <c r="F141" t="n">
+        <v>2176561.162089184</v>
+      </c>
+      <c r="G141" t="n">
+        <v>112571.1620891844</v>
+      </c>
+      <c r="H141" t="n">
+        <v>5.45405559567558</v>
+      </c>
+      <c r="I141" t="inlineStr">
+        <is>
+          <t>2026-03-20T15:48:40</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="inlineStr">
+        <is>
+          <t>2026-03-20</t>
+        </is>
+      </c>
+      <c r="B142" t="inlineStr">
+        <is>
+          <t>미창석유</t>
+        </is>
+      </c>
+      <c r="C142" t="n">
+        <v>18</v>
+      </c>
+      <c r="D142" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E142" t="n">
+        <v>1</v>
+      </c>
+      <c r="F142" t="n">
+        <v>2097000</v>
+      </c>
+      <c r="G142" t="n">
+        <v>-295200</v>
+      </c>
+      <c r="H142" t="n">
+        <v>-12.34010534236268</v>
+      </c>
+      <c r="I142" t="inlineStr">
+        <is>
+          <t>2026-03-20T15:48:40</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="inlineStr">
+        <is>
+          <t>2026-03-20</t>
+        </is>
+      </c>
+      <c r="B143" t="inlineStr">
+        <is>
+          <t>하나금융지주</t>
+        </is>
+      </c>
+      <c r="C143" t="n">
+        <v>18</v>
+      </c>
+      <c r="D143" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E143" t="n">
+        <v>1</v>
+      </c>
+      <c r="F143" t="n">
+        <v>2037600</v>
+      </c>
+      <c r="G143" t="n">
+        <v>12200</v>
+      </c>
+      <c r="H143" t="n">
+        <v>0.6023501530561864</v>
+      </c>
+      <c r="I143" t="inlineStr">
+        <is>
+          <t>2026-03-20T15:48:40</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" t="inlineStr">
+        <is>
+          <t>2026-03-20</t>
+        </is>
+      </c>
+      <c r="B144" t="inlineStr">
+        <is>
+          <t>대창단조</t>
+        </is>
+      </c>
+      <c r="C144" t="n">
+        <v>300</v>
+      </c>
+      <c r="D144" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E144" t="n">
+        <v>1</v>
+      </c>
+      <c r="F144" t="n">
+        <v>2004000</v>
+      </c>
+      <c r="G144" t="n">
+        <v>-54000</v>
+      </c>
+      <c r="H144" t="n">
+        <v>-2.623906705539359</v>
+      </c>
+      <c r="I144" t="inlineStr">
+        <is>
+          <t>2026-03-20T15:48:40</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="inlineStr">
+        <is>
+          <t>2026-03-20</t>
+        </is>
+      </c>
+      <c r="B145" t="inlineStr">
+        <is>
+          <t>동방</t>
+        </is>
+      </c>
+      <c r="C145" t="n">
+        <v>681</v>
+      </c>
+      <c r="D145" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E145" t="n">
+        <v>1</v>
+      </c>
+      <c r="F145" t="n">
+        <v>1995330</v>
+      </c>
+      <c r="G145" t="n">
+        <v>23829</v>
+      </c>
+      <c r="H145" t="n">
+        <v>1.208672985709873</v>
+      </c>
+      <c r="I145" t="inlineStr">
+        <is>
+          <t>2026-03-20T15:48:40</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" t="inlineStr">
+        <is>
+          <t>2026-03-20</t>
+        </is>
+      </c>
+      <c r="B146" t="inlineStr">
+        <is>
+          <t>스타 벌크 캐리어스</t>
+        </is>
+      </c>
+      <c r="C146" t="n">
+        <v>50</v>
+      </c>
+      <c r="D146" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E146" t="n">
+        <v>1</v>
+      </c>
+      <c r="F146" t="n">
+        <v>1696441.320678405</v>
+      </c>
+      <c r="G146" t="n">
+        <v>382088.3206784062</v>
+      </c>
+      <c r="H146" t="n">
+        <v>29.07044916231837</v>
+      </c>
+      <c r="I146" t="inlineStr">
+        <is>
+          <t>2026-03-20T15:48:40</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" t="inlineStr">
+        <is>
+          <t>2026-03-20</t>
+        </is>
+      </c>
+      <c r="B147" t="inlineStr">
+        <is>
+          <t>유나이티드헬스 그룹</t>
+        </is>
+      </c>
+      <c r="C147" t="n">
+        <v>4</v>
+      </c>
+      <c r="D147" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E147" t="n">
+        <v>1</v>
+      </c>
+      <c r="F147" t="n">
+        <v>1683366.447431445</v>
+      </c>
+      <c r="G147" t="n">
+        <v>-11089.55256855441</v>
+      </c>
+      <c r="H147" t="n">
+        <v>-0.6544609342794628</v>
+      </c>
+      <c r="I147" t="inlineStr">
+        <is>
+          <t>2026-03-20T15:48:40</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" t="inlineStr">
+        <is>
+          <t>2026-03-20</t>
+        </is>
+      </c>
+      <c r="B148" t="inlineStr">
+        <is>
+          <t>케이씨</t>
+        </is>
+      </c>
+      <c r="C148" t="n">
+        <v>50</v>
+      </c>
+      <c r="D148" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E148" t="n">
+        <v>1</v>
+      </c>
+      <c r="F148" t="n">
+        <v>1670000</v>
+      </c>
+      <c r="G148" t="n">
+        <v>20500</v>
+      </c>
+      <c r="H148" t="n">
+        <v>1.242800848742043</v>
+      </c>
+      <c r="I148" t="inlineStr">
+        <is>
+          <t>2026-03-20T15:48:40</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="inlineStr">
+        <is>
+          <t>2026-03-20</t>
+        </is>
+      </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>LX인터내셔널</t>
+        </is>
+      </c>
+      <c r="C149" t="n">
+        <v>20</v>
+      </c>
+      <c r="D149" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E149" t="n">
+        <v>1</v>
+      </c>
+      <c r="F149" t="n">
+        <v>943000</v>
+      </c>
+      <c r="G149" t="n">
+        <v>4000</v>
+      </c>
+      <c r="H149" t="n">
+        <v>0.4259850905218318</v>
+      </c>
+      <c r="I149" t="inlineStr">
+        <is>
+          <t>2026-03-20T15:48:40</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="inlineStr">
+        <is>
+          <t>2026-03-20</t>
+        </is>
+      </c>
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>삼성생명</t>
+        </is>
+      </c>
+      <c r="C150" t="n">
+        <v>4</v>
+      </c>
+      <c r="D150" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E150" t="n">
+        <v>1</v>
+      </c>
+      <c r="F150" t="n">
+        <v>926000</v>
+      </c>
+      <c r="G150" t="n">
+        <v>93000</v>
+      </c>
+      <c r="H150" t="n">
+        <v>11.16446578631453</v>
+      </c>
+      <c r="I150" t="inlineStr">
+        <is>
+          <t>2026-03-20T15:48:40</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="inlineStr">
+        <is>
+          <t>2026-03-20</t>
+        </is>
+      </c>
+      <c r="B151" t="inlineStr">
+        <is>
+          <t>비에이치아이</t>
+        </is>
+      </c>
+      <c r="C151" t="n">
+        <v>8</v>
+      </c>
+      <c r="D151" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E151" t="n">
+        <v>1</v>
+      </c>
+      <c r="F151" t="n">
+        <v>876000</v>
+      </c>
+      <c r="G151" t="n">
+        <v>210885</v>
+      </c>
+      <c r="H151" t="n">
+        <v>31.70654698811484</v>
+      </c>
+      <c r="I151" t="inlineStr">
+        <is>
+          <t>2026-03-20T15:48:40</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="inlineStr">
+        <is>
+          <t>2026-03-20</t>
+        </is>
+      </c>
+      <c r="B152" t="inlineStr">
+        <is>
+          <t>하프니아</t>
+        </is>
+      </c>
+      <c r="C152" t="n">
+        <v>80</v>
+      </c>
+      <c r="D152" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E152" t="n">
+        <v>1</v>
+      </c>
+      <c r="F152" t="n">
+        <v>848519.8631833494</v>
+      </c>
+      <c r="G152" t="n">
+        <v>222788.8631833494</v>
+      </c>
+      <c r="H152" t="n">
+        <v>35.60457499841775</v>
+      </c>
+      <c r="I152" t="inlineStr">
+        <is>
+          <t>2026-03-20T15:48:40</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" t="inlineStr">
+        <is>
+          <t>2026-03-20</t>
+        </is>
+      </c>
+      <c r="B153" t="inlineStr">
+        <is>
+          <t>클리블랜드 클리프스</t>
+        </is>
+      </c>
+      <c r="C153" t="n">
+        <v>70</v>
+      </c>
+      <c r="D153" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E153" t="n">
+        <v>1</v>
+      </c>
+      <c r="F153" t="n">
+        <v>833036.4441346284</v>
+      </c>
+      <c r="G153" t="n">
+        <v>-183018.5558653716</v>
+      </c>
+      <c r="H153" t="n">
+        <v>-18.01266229341636</v>
+      </c>
+      <c r="I153" t="inlineStr">
+        <is>
+          <t>2026-03-20T15:48:40</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" t="inlineStr">
+        <is>
+          <t>2026-03-20</t>
+        </is>
+      </c>
+      <c r="B154" t="inlineStr">
+        <is>
+          <t>텍사스 퍼시픽 랜드</t>
+        </is>
+      </c>
+      <c r="C154" t="n">
+        <v>1</v>
+      </c>
+      <c r="D154" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E154" t="n">
+        <v>1</v>
+      </c>
+      <c r="F154" t="n">
+        <v>798210.0491355956</v>
+      </c>
+      <c r="G154" t="n">
+        <v>19619.04913559556</v>
+      </c>
+      <c r="H154" t="n">
+        <v>2.519814528500273</v>
+      </c>
+      <c r="I154" t="inlineStr">
+        <is>
+          <t>2026-03-20T15:48:40</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" t="inlineStr">
+        <is>
+          <t>2026-03-20</t>
+        </is>
+      </c>
+      <c r="B155" t="inlineStr">
+        <is>
+          <t>NH투자증권우</t>
+        </is>
+      </c>
+      <c r="C155" t="n">
+        <v>2</v>
+      </c>
+      <c r="D155" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E155" t="n">
+        <v>1</v>
+      </c>
+      <c r="F155" t="n">
+        <v>54591</v>
+      </c>
+      <c r="G155" t="n">
+        <v>-9</v>
+      </c>
+      <c r="H155" t="n">
+        <v>-0.01648351648351648</v>
+      </c>
+      <c r="I155" t="inlineStr">
+        <is>
+          <t>2026-03-20T15:48:40</t>
         </is>
       </c>
     </row>
@@ -5846,7 +7380,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E4"/>
+  <dimension ref="A1:E5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5945,6 +7479,29 @@
         </is>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2026-03-20</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>31505056</v>
+      </c>
+      <c r="C5" t="n">
+        <v>6016.63</v>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>2026-03-20T15:48:40</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>2026-03-20T15:48:40</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
auto: portfolio snapshot 2026-03-20 (2026-03-20T15:48:41)
</commit_message>
<xml_diff>
--- a/portfolio_auto.xlsx
+++ b/portfolio_auto.xlsx
@@ -1603,7 +1603,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2026-03-20T15:48:40</t>
+          <t>2026-03-20T15:48:41</t>
         </is>
       </c>
       <c r="E2" t="n">
@@ -5922,7 +5922,7 @@
       </c>
       <c r="I116" t="inlineStr">
         <is>
-          <t>2026-03-20T15:48:40</t>
+          <t>2026-03-20T15:48:41</t>
         </is>
       </c>
     </row>
@@ -5959,7 +5959,7 @@
       </c>
       <c r="I117" t="inlineStr">
         <is>
-          <t>2026-03-20T15:48:40</t>
+          <t>2026-03-20T15:48:41</t>
         </is>
       </c>
     </row>
@@ -5996,7 +5996,7 @@
       </c>
       <c r="I118" t="inlineStr">
         <is>
-          <t>2026-03-20T15:48:40</t>
+          <t>2026-03-20T15:48:41</t>
         </is>
       </c>
     </row>
@@ -6033,7 +6033,7 @@
       </c>
       <c r="I119" t="inlineStr">
         <is>
-          <t>2026-03-20T15:48:40</t>
+          <t>2026-03-20T15:48:41</t>
         </is>
       </c>
     </row>
@@ -6070,7 +6070,7 @@
       </c>
       <c r="I120" t="inlineStr">
         <is>
-          <t>2026-03-20T15:48:40</t>
+          <t>2026-03-20T15:48:41</t>
         </is>
       </c>
     </row>
@@ -6107,7 +6107,7 @@
       </c>
       <c r="I121" t="inlineStr">
         <is>
-          <t>2026-03-20T15:48:40</t>
+          <t>2026-03-20T15:48:41</t>
         </is>
       </c>
     </row>
@@ -6144,7 +6144,7 @@
       </c>
       <c r="I122" t="inlineStr">
         <is>
-          <t>2026-03-20T15:48:40</t>
+          <t>2026-03-20T15:48:41</t>
         </is>
       </c>
     </row>
@@ -6181,7 +6181,7 @@
       </c>
       <c r="I123" t="inlineStr">
         <is>
-          <t>2026-03-20T15:48:40</t>
+          <t>2026-03-20T15:48:41</t>
         </is>
       </c>
     </row>
@@ -6218,7 +6218,7 @@
       </c>
       <c r="I124" t="inlineStr">
         <is>
-          <t>2026-03-20T15:48:40</t>
+          <t>2026-03-20T15:48:41</t>
         </is>
       </c>
     </row>
@@ -6255,7 +6255,7 @@
       </c>
       <c r="I125" t="inlineStr">
         <is>
-          <t>2026-03-20T15:48:40</t>
+          <t>2026-03-20T15:48:41</t>
         </is>
       </c>
     </row>
@@ -6292,7 +6292,7 @@
       </c>
       <c r="I126" t="inlineStr">
         <is>
-          <t>2026-03-20T15:48:40</t>
+          <t>2026-03-20T15:48:41</t>
         </is>
       </c>
     </row>
@@ -6329,7 +6329,7 @@
       </c>
       <c r="I127" t="inlineStr">
         <is>
-          <t>2026-03-20T15:48:40</t>
+          <t>2026-03-20T15:48:41</t>
         </is>
       </c>
     </row>
@@ -6366,7 +6366,7 @@
       </c>
       <c r="I128" t="inlineStr">
         <is>
-          <t>2026-03-20T15:48:40</t>
+          <t>2026-03-20T15:48:41</t>
         </is>
       </c>
     </row>
@@ -6403,7 +6403,7 @@
       </c>
       <c r="I129" t="inlineStr">
         <is>
-          <t>2026-03-20T15:48:40</t>
+          <t>2026-03-20T15:48:41</t>
         </is>
       </c>
     </row>
@@ -6440,7 +6440,7 @@
       </c>
       <c r="I130" t="inlineStr">
         <is>
-          <t>2026-03-20T15:48:40</t>
+          <t>2026-03-20T15:48:41</t>
         </is>
       </c>
     </row>
@@ -6477,7 +6477,7 @@
       </c>
       <c r="I131" t="inlineStr">
         <is>
-          <t>2026-03-20T15:48:40</t>
+          <t>2026-03-20T15:48:41</t>
         </is>
       </c>
     </row>
@@ -6514,7 +6514,7 @@
       </c>
       <c r="I132" t="inlineStr">
         <is>
-          <t>2026-03-20T15:48:40</t>
+          <t>2026-03-20T15:48:41</t>
         </is>
       </c>
     </row>
@@ -6551,7 +6551,7 @@
       </c>
       <c r="I133" t="inlineStr">
         <is>
-          <t>2026-03-20T15:48:40</t>
+          <t>2026-03-20T15:48:41</t>
         </is>
       </c>
     </row>
@@ -6588,7 +6588,7 @@
       </c>
       <c r="I134" t="inlineStr">
         <is>
-          <t>2026-03-20T15:48:40</t>
+          <t>2026-03-20T15:48:41</t>
         </is>
       </c>
     </row>
@@ -6625,7 +6625,7 @@
       </c>
       <c r="I135" t="inlineStr">
         <is>
-          <t>2026-03-20T15:48:40</t>
+          <t>2026-03-20T15:48:41</t>
         </is>
       </c>
     </row>
@@ -6662,7 +6662,7 @@
       </c>
       <c r="I136" t="inlineStr">
         <is>
-          <t>2026-03-20T15:48:40</t>
+          <t>2026-03-20T15:48:41</t>
         </is>
       </c>
     </row>
@@ -6699,7 +6699,7 @@
       </c>
       <c r="I137" t="inlineStr">
         <is>
-          <t>2026-03-20T15:48:40</t>
+          <t>2026-03-20T15:48:41</t>
         </is>
       </c>
     </row>
@@ -6736,7 +6736,7 @@
       </c>
       <c r="I138" t="inlineStr">
         <is>
-          <t>2026-03-20T15:48:40</t>
+          <t>2026-03-20T15:48:41</t>
         </is>
       </c>
     </row>
@@ -6773,7 +6773,7 @@
       </c>
       <c r="I139" t="inlineStr">
         <is>
-          <t>2026-03-20T15:48:40</t>
+          <t>2026-03-20T15:48:41</t>
         </is>
       </c>
     </row>
@@ -6810,7 +6810,7 @@
       </c>
       <c r="I140" t="inlineStr">
         <is>
-          <t>2026-03-20T15:48:40</t>
+          <t>2026-03-20T15:48:41</t>
         </is>
       </c>
     </row>
@@ -6847,7 +6847,7 @@
       </c>
       <c r="I141" t="inlineStr">
         <is>
-          <t>2026-03-20T15:48:40</t>
+          <t>2026-03-20T15:48:41</t>
         </is>
       </c>
     </row>
@@ -6884,7 +6884,7 @@
       </c>
       <c r="I142" t="inlineStr">
         <is>
-          <t>2026-03-20T15:48:40</t>
+          <t>2026-03-20T15:48:41</t>
         </is>
       </c>
     </row>
@@ -6921,7 +6921,7 @@
       </c>
       <c r="I143" t="inlineStr">
         <is>
-          <t>2026-03-20T15:48:40</t>
+          <t>2026-03-20T15:48:41</t>
         </is>
       </c>
     </row>
@@ -6958,7 +6958,7 @@
       </c>
       <c r="I144" t="inlineStr">
         <is>
-          <t>2026-03-20T15:48:40</t>
+          <t>2026-03-20T15:48:41</t>
         </is>
       </c>
     </row>
@@ -6995,7 +6995,7 @@
       </c>
       <c r="I145" t="inlineStr">
         <is>
-          <t>2026-03-20T15:48:40</t>
+          <t>2026-03-20T15:48:41</t>
         </is>
       </c>
     </row>
@@ -7032,7 +7032,7 @@
       </c>
       <c r="I146" t="inlineStr">
         <is>
-          <t>2026-03-20T15:48:40</t>
+          <t>2026-03-20T15:48:41</t>
         </is>
       </c>
     </row>
@@ -7069,7 +7069,7 @@
       </c>
       <c r="I147" t="inlineStr">
         <is>
-          <t>2026-03-20T15:48:40</t>
+          <t>2026-03-20T15:48:41</t>
         </is>
       </c>
     </row>
@@ -7106,7 +7106,7 @@
       </c>
       <c r="I148" t="inlineStr">
         <is>
-          <t>2026-03-20T15:48:40</t>
+          <t>2026-03-20T15:48:41</t>
         </is>
       </c>
     </row>
@@ -7143,7 +7143,7 @@
       </c>
       <c r="I149" t="inlineStr">
         <is>
-          <t>2026-03-20T15:48:40</t>
+          <t>2026-03-20T15:48:41</t>
         </is>
       </c>
     </row>
@@ -7180,7 +7180,7 @@
       </c>
       <c r="I150" t="inlineStr">
         <is>
-          <t>2026-03-20T15:48:40</t>
+          <t>2026-03-20T15:48:41</t>
         </is>
       </c>
     </row>
@@ -7217,7 +7217,7 @@
       </c>
       <c r="I151" t="inlineStr">
         <is>
-          <t>2026-03-20T15:48:40</t>
+          <t>2026-03-20T15:48:41</t>
         </is>
       </c>
     </row>
@@ -7254,7 +7254,7 @@
       </c>
       <c r="I152" t="inlineStr">
         <is>
-          <t>2026-03-20T15:48:40</t>
+          <t>2026-03-20T15:48:41</t>
         </is>
       </c>
     </row>
@@ -7291,7 +7291,7 @@
       </c>
       <c r="I153" t="inlineStr">
         <is>
-          <t>2026-03-20T15:48:40</t>
+          <t>2026-03-20T15:48:41</t>
         </is>
       </c>
     </row>
@@ -7328,7 +7328,7 @@
       </c>
       <c r="I154" t="inlineStr">
         <is>
-          <t>2026-03-20T15:48:40</t>
+          <t>2026-03-20T15:48:41</t>
         </is>
       </c>
     </row>
@@ -7365,7 +7365,7 @@
       </c>
       <c r="I155" t="inlineStr">
         <is>
-          <t>2026-03-20T15:48:40</t>
+          <t>2026-03-20T15:48:41</t>
         </is>
       </c>
     </row>
@@ -7498,7 +7498,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>2026-03-20T15:48:40</t>
+          <t>2026-03-20T15:48:41</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: portfolio snapshot 2026-03-20 (2026-03-20T15:49:08)
</commit_message>
<xml_diff>
--- a/portfolio_auto.xlsx
+++ b/portfolio_auto.xlsx
@@ -498,11 +498,11 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>AGNC 인베스트먼트</t>
+          <t>시드릴</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>700</v>
+        <v>123</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
@@ -513,23 +513,23 @@
         <v>1</v>
       </c>
       <c r="E3" t="n">
-        <v>10351433.71453537</v>
+        <v>8081063.113214018</v>
       </c>
       <c r="F3" t="n">
-        <v>-480581.2854646351</v>
+        <v>1630712.113214018</v>
       </c>
       <c r="G3" t="n">
-        <v>-4.436674851951692</v>
+        <v>25.28098258860669</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>대한조선</t>
+          <t>트랜스오션</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>100</v>
+        <v>750</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
@@ -540,23 +540,23 @@
         <v>1</v>
       </c>
       <c r="E4" t="n">
-        <v>9120000</v>
+        <v>7074115.140040115</v>
       </c>
       <c r="F4" t="n">
-        <v>1907000</v>
+        <v>2946881.140040115</v>
       </c>
       <c r="G4" t="n">
-        <v>26.43837515596839</v>
+        <v>71.40087380652794</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>프론트라인</t>
+          <t>노블</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>175</v>
+        <v>99</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -567,23 +567,23 @@
         <v>1</v>
       </c>
       <c r="E5" t="n">
-        <v>8453409.11431564</v>
+        <v>6886743.840087891</v>
       </c>
       <c r="F5" t="n">
-        <v>4023545.11431564</v>
+        <v>2979535.840087891</v>
       </c>
       <c r="G5" t="n">
-        <v>90.82773453802736</v>
+        <v>76.25741552760668</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>시드릴</t>
+          <t>센트러스 에너지</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>123</v>
+        <v>21</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
@@ -594,23 +594,23 @@
         <v>1</v>
       </c>
       <c r="E6" t="n">
-        <v>8081063.113214018</v>
+        <v>5996448.754211426</v>
       </c>
       <c r="F6" t="n">
-        <v>1630712.113214018</v>
+        <v>-234770.2457885733</v>
       </c>
       <c r="G6" t="n">
-        <v>25.28098258860669</v>
+        <v>-3.767645556809564</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>트랜스오션</t>
+          <t>타이드워터</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>750</v>
+        <v>48</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -621,23 +621,23 @@
         <v>1</v>
       </c>
       <c r="E7" t="n">
-        <v>7074115.140040115</v>
+        <v>5211036.802851856</v>
       </c>
       <c r="F7" t="n">
-        <v>2946881.140040115</v>
+        <v>1486491.802851856</v>
       </c>
       <c r="G7" t="n">
-        <v>71.40087380652794</v>
+        <v>39.91069520845783</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>노블</t>
+          <t>노브</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>99</v>
+        <v>185</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
@@ -648,23 +648,23 @@
         <v>1</v>
       </c>
       <c r="E8" t="n">
-        <v>6886743.840087891</v>
+        <v>5179494.129107101</v>
       </c>
       <c r="F8" t="n">
-        <v>2979535.840087891</v>
+        <v>1869486.129107101</v>
       </c>
       <c r="G8" t="n">
-        <v>76.25741552760668</v>
+        <v>56.47980697046958</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>세아제강</t>
+          <t>오케아니스 에코 탱커스</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>50</v>
+        <v>65</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
@@ -675,23 +675,23 @@
         <v>1</v>
       </c>
       <c r="E9" t="n">
-        <v>7395000</v>
+        <v>4596307.895957222</v>
       </c>
       <c r="F9" t="n">
-        <v>1085000</v>
+        <v>2339947.895957222</v>
       </c>
       <c r="G9" t="n">
-        <v>17.19492868462758</v>
+        <v>103.704546081176</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>센트러스 에너지</t>
+          <t>차코스 에너지 내비게이션</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>21</v>
+        <v>75</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
@@ -702,23 +702,23 @@
         <v>1</v>
       </c>
       <c r="E10" t="n">
-        <v>5996448.754211426</v>
+        <v>4052048.962918622</v>
       </c>
       <c r="F10" t="n">
-        <v>-234770.2457885733</v>
+        <v>227400.9629186224</v>
       </c>
       <c r="G10" t="n">
-        <v>-3.767645556809564</v>
+        <v>5.94567037067522</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>타이드워터</t>
+          <t>더치 브로스</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>48</v>
+        <v>39</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
@@ -729,23 +729,23 @@
         <v>1</v>
       </c>
       <c r="E11" t="n">
-        <v>5211036.802851856</v>
+        <v>2959763.281021703</v>
       </c>
       <c r="F11" t="n">
-        <v>1486491.802851856</v>
+        <v>-230880.718978297</v>
       </c>
       <c r="G11" t="n">
-        <v>39.91069520845783</v>
+        <v>-7.236179247145621</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>노브</t>
+          <t>발레로 에너지</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>185</v>
+        <v>6</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
@@ -756,23 +756,23 @@
         <v>1</v>
       </c>
       <c r="E12" t="n">
-        <v>5179494.129107101</v>
+        <v>2176561.162089184</v>
       </c>
       <c r="F12" t="n">
-        <v>1869486.129107101</v>
+        <v>112571.1620891844</v>
       </c>
       <c r="G12" t="n">
-        <v>56.47980697046958</v>
+        <v>5.45405559567558</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>오케아니스 에코 탱커스</t>
+          <t>스타 벌크 캐리어스</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>65</v>
+        <v>50</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
@@ -783,23 +783,23 @@
         <v>1</v>
       </c>
       <c r="E13" t="n">
-        <v>4596307.895957222</v>
+        <v>1696441.320678405</v>
       </c>
       <c r="F13" t="n">
-        <v>2339947.895957222</v>
+        <v>382088.3206784062</v>
       </c>
       <c r="G13" t="n">
-        <v>103.704546081176</v>
+        <v>29.07044916231837</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>삼성화재</t>
+          <t>유나이티드헬스 그룹</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
@@ -810,23 +810,23 @@
         <v>1</v>
       </c>
       <c r="E14" t="n">
-        <v>4270500</v>
+        <v>1683366.447431445</v>
       </c>
       <c r="F14" t="n">
-        <v>-360500</v>
+        <v>-11089.55256855441</v>
       </c>
       <c r="G14" t="n">
-        <v>-7.784495789246384</v>
+        <v>-0.6544609342794628</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>차코스 에너지 내비게이션</t>
+          <t>클리블랜드 클리프스</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>75</v>
+        <v>70</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
@@ -837,23 +837,23 @@
         <v>1</v>
       </c>
       <c r="E15" t="n">
-        <v>4052048.962918622</v>
+        <v>833036.4441346284</v>
       </c>
       <c r="F15" t="n">
-        <v>227400.9629186224</v>
+        <v>-183018.5558653716</v>
       </c>
       <c r="G15" t="n">
-        <v>5.94567037067522</v>
+        <v>-18.01266229341636</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>동원개발</t>
+          <t>텍사스 퍼시픽 랜드</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>1360</v>
+        <v>1</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
@@ -864,23 +864,23 @@
         <v>1</v>
       </c>
       <c r="E16" t="n">
-        <v>4202400</v>
+        <v>798210.0491355956</v>
       </c>
       <c r="F16" t="n">
-        <v>465000</v>
+        <v>19619.04913559556</v>
       </c>
       <c r="G16" t="n">
-        <v>12.44180446299566</v>
+        <v>2.519814528500273</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>피바디 에너지</t>
+          <t>케이씨</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>65</v>
+        <v>50</v>
       </c>
       <c r="C17" t="inlineStr">
         <is>
@@ -891,23 +891,23 @@
         <v>1</v>
       </c>
       <c r="E17" t="n">
-        <v>3596373.331896178</v>
+        <v>1670000</v>
       </c>
       <c r="F17" t="n">
-        <v>2125601.331896178</v>
+        <v>20500</v>
       </c>
       <c r="G17" t="n">
-        <v>144.5228309959789</v>
+        <v>1.242800848742043</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>더치 브로스</t>
+          <t>하나금융지주</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>39</v>
+        <v>18</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
@@ -918,23 +918,23 @@
         <v>1</v>
       </c>
       <c r="E18" t="n">
-        <v>2959763.281021703</v>
+        <v>2037600</v>
       </c>
       <c r="F18" t="n">
-        <v>-230880.718978297</v>
+        <v>12200</v>
       </c>
       <c r="G18" t="n">
-        <v>-7.236179247145621</v>
+        <v>0.6023501530561864</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>넥스틸</t>
+          <t>현대제철</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>200</v>
+        <v>80</v>
       </c>
       <c r="C19" t="inlineStr">
         <is>
@@ -945,23 +945,23 @@
         <v>1</v>
       </c>
       <c r="E19" t="n">
-        <v>2514000</v>
+        <v>2996000</v>
       </c>
       <c r="F19" t="n">
-        <v>503000</v>
+        <v>-182000</v>
       </c>
       <c r="G19" t="n">
-        <v>25.01243162605669</v>
+        <v>-5.726872246696035</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>대신증권</t>
+          <t>휴스틸</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>55</v>
+        <v>500</v>
       </c>
       <c r="C20" t="inlineStr">
         <is>
@@ -972,23 +972,23 @@
         <v>1</v>
       </c>
       <c r="E20" t="n">
-        <v>2219250</v>
+        <v>2750000</v>
       </c>
       <c r="F20" t="n">
-        <v>509749</v>
+        <v>471390</v>
       </c>
       <c r="G20" t="n">
-        <v>29.81858448752005</v>
+        <v>20.68761218462133</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>발레로 에너지</t>
+          <t>DL이앤씨</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>6</v>
+        <v>40</v>
       </c>
       <c r="C21" t="inlineStr">
         <is>
@@ -999,23 +999,23 @@
         <v>1</v>
       </c>
       <c r="E21" t="n">
-        <v>2176561.162089184</v>
+        <v>2696000</v>
       </c>
       <c r="F21" t="n">
-        <v>112571.1620891844</v>
+        <v>990500</v>
       </c>
       <c r="G21" t="n">
-        <v>5.45405559567558</v>
+        <v>58.07681031955438</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>미창석유</t>
+          <t>HD건설기계</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>18</v>
+        <v>31</v>
       </c>
       <c r="C22" t="inlineStr">
         <is>
@@ -1026,23 +1026,23 @@
         <v>1</v>
       </c>
       <c r="E22" t="n">
-        <v>2097000</v>
+        <v>4123000</v>
       </c>
       <c r="F22" t="n">
-        <v>-295200</v>
+        <v>87904</v>
       </c>
       <c r="G22" t="n">
-        <v>-12.34010534236268</v>
+        <v>2.178485964150543</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>대창단조</t>
+          <t>KoAct 코스닥액티브</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>300</v>
+        <v>200</v>
       </c>
       <c r="C23" t="inlineStr">
         <is>
@@ -1053,23 +1053,23 @@
         <v>1</v>
       </c>
       <c r="E23" t="n">
-        <v>2004000</v>
+        <v>2582000</v>
       </c>
       <c r="F23" t="n">
-        <v>-54000</v>
+        <v>-120000</v>
       </c>
       <c r="G23" t="n">
-        <v>-2.623906705539359</v>
+        <v>-4.441154700222058</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>동방</t>
+          <t>LX인터내셔널</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>681</v>
+        <v>20</v>
       </c>
       <c r="C24" t="inlineStr">
         <is>
@@ -1080,23 +1080,23 @@
         <v>1</v>
       </c>
       <c r="E24" t="n">
-        <v>1995330</v>
+        <v>943000</v>
       </c>
       <c r="F24" t="n">
-        <v>23829</v>
+        <v>4000</v>
       </c>
       <c r="G24" t="n">
-        <v>1.208672985709873</v>
+        <v>0.4259850905218318</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>스타 벌크 캐리어스</t>
+          <t>NH투자증권우</t>
         </is>
       </c>
       <c r="B25" t="n">
-        <v>50</v>
+        <v>2</v>
       </c>
       <c r="C25" t="inlineStr">
         <is>
@@ -1107,23 +1107,23 @@
         <v>1</v>
       </c>
       <c r="E25" t="n">
-        <v>1696441.320678405</v>
+        <v>54591</v>
       </c>
       <c r="F25" t="n">
-        <v>382088.3206784062</v>
+        <v>-9</v>
       </c>
       <c r="G25" t="n">
-        <v>29.07044916231837</v>
+        <v>-0.01648351648351648</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>유나이티드헬스 그룹</t>
+          <t>TIME 코리아밸류업액티브</t>
         </is>
       </c>
       <c r="B26" t="n">
-        <v>4</v>
+        <v>201</v>
       </c>
       <c r="C26" t="inlineStr">
         <is>
@@ -1134,23 +1134,23 @@
         <v>1</v>
       </c>
       <c r="E26" t="n">
-        <v>1683366.447431445</v>
+        <v>4797870</v>
       </c>
       <c r="F26" t="n">
-        <v>-11089.55256855441</v>
+        <v>74073</v>
       </c>
       <c r="G26" t="n">
-        <v>-0.6544609342794628</v>
+        <v>1.568081778281328</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>삼성생명</t>
+          <t>프론트라인</t>
         </is>
       </c>
       <c r="B27" t="n">
-        <v>4</v>
+        <v>175</v>
       </c>
       <c r="C27" t="inlineStr">
         <is>
@@ -1161,23 +1161,23 @@
         <v>1</v>
       </c>
       <c r="E27" t="n">
-        <v>926000</v>
+        <v>8453409.11431564</v>
       </c>
       <c r="F27" t="n">
-        <v>93000</v>
+        <v>4023545.11431564</v>
       </c>
       <c r="G27" t="n">
-        <v>11.16446578631453</v>
+        <v>90.82773453802736</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>클리블랜드 클리프스</t>
+          <t>피바디 에너지</t>
         </is>
       </c>
       <c r="B28" t="n">
-        <v>70</v>
+        <v>65</v>
       </c>
       <c r="C28" t="inlineStr">
         <is>
@@ -1188,13 +1188,13 @@
         <v>1</v>
       </c>
       <c r="E28" t="n">
-        <v>833036.4441346284</v>
+        <v>3596373.331896178</v>
       </c>
       <c r="F28" t="n">
-        <v>-183018.5558653716</v>
+        <v>2125601.331896178</v>
       </c>
       <c r="G28" t="n">
-        <v>-18.01266229341636</v>
+        <v>144.5228309959789</v>
       </c>
     </row>
     <row r="29">
@@ -1227,11 +1227,11 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>비에이치아이</t>
+          <t>AGNC 인베스트먼트</t>
         </is>
       </c>
       <c r="B30" t="n">
-        <v>8</v>
+        <v>700</v>
       </c>
       <c r="C30" t="inlineStr">
         <is>
@@ -1242,23 +1242,23 @@
         <v>1</v>
       </c>
       <c r="E30" t="n">
-        <v>876000</v>
+        <v>10351433.71453537</v>
       </c>
       <c r="F30" t="n">
-        <v>210885</v>
+        <v>-480580.2854646333</v>
       </c>
       <c r="G30" t="n">
-        <v>31.70654698811484</v>
+        <v>-4.43666602964724</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>텍사스 퍼시픽 랜드</t>
+          <t>넥스틸</t>
         </is>
       </c>
       <c r="B31" t="n">
-        <v>1</v>
+        <v>300</v>
       </c>
       <c r="C31" t="inlineStr">
         <is>
@@ -1269,23 +1269,23 @@
         <v>1</v>
       </c>
       <c r="E31" t="n">
-        <v>798210.0491355956</v>
+        <v>3771000</v>
       </c>
       <c r="F31" t="n">
-        <v>19619.04913559556</v>
+        <v>521000</v>
       </c>
       <c r="G31" t="n">
-        <v>2.519814528500273</v>
+        <v>16.03076923076923</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>케이씨</t>
+          <t>대신증권</t>
         </is>
       </c>
       <c r="B32" t="n">
-        <v>50</v>
+        <v>55</v>
       </c>
       <c r="C32" t="inlineStr">
         <is>
@@ -1296,23 +1296,23 @@
         <v>1</v>
       </c>
       <c r="E32" t="n">
-        <v>1670000</v>
+        <v>2219250</v>
       </c>
       <c r="F32" t="n">
-        <v>20500</v>
+        <v>509749</v>
       </c>
       <c r="G32" t="n">
-        <v>1.242800848742043</v>
+        <v>29.81858448752005</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>하나금융지주</t>
+          <t>대창단조</t>
         </is>
       </c>
       <c r="B33" t="n">
-        <v>18</v>
+        <v>300</v>
       </c>
       <c r="C33" t="inlineStr">
         <is>
@@ -1323,23 +1323,23 @@
         <v>1</v>
       </c>
       <c r="E33" t="n">
-        <v>2037600</v>
+        <v>2004000</v>
       </c>
       <c r="F33" t="n">
-        <v>12200</v>
+        <v>-54000</v>
       </c>
       <c r="G33" t="n">
-        <v>0.6023501530561864</v>
+        <v>-2.623906705539359</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>현대제철</t>
+          <t>대한조선</t>
         </is>
       </c>
       <c r="B34" t="n">
-        <v>80</v>
+        <v>100</v>
       </c>
       <c r="C34" t="inlineStr">
         <is>
@@ -1350,23 +1350,23 @@
         <v>1</v>
       </c>
       <c r="E34" t="n">
-        <v>2996000</v>
+        <v>9120000</v>
       </c>
       <c r="F34" t="n">
-        <v>-182000</v>
+        <v>1907000</v>
       </c>
       <c r="G34" t="n">
-        <v>-5.726872246696035</v>
+        <v>26.43837515596839</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>휴스틸</t>
+          <t>동방</t>
         </is>
       </c>
       <c r="B35" t="n">
-        <v>500</v>
+        <v>681</v>
       </c>
       <c r="C35" t="inlineStr">
         <is>
@@ -1377,23 +1377,23 @@
         <v>1</v>
       </c>
       <c r="E35" t="n">
-        <v>2750000</v>
+        <v>1995330</v>
       </c>
       <c r="F35" t="n">
-        <v>471390</v>
+        <v>23829</v>
       </c>
       <c r="G35" t="n">
-        <v>20.68761218462133</v>
+        <v>1.208672985709873</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>DL이앤씨</t>
+          <t>동원개발</t>
         </is>
       </c>
       <c r="B36" t="n">
-        <v>40</v>
+        <v>1360</v>
       </c>
       <c r="C36" t="inlineStr">
         <is>
@@ -1404,23 +1404,23 @@
         <v>1</v>
       </c>
       <c r="E36" t="n">
-        <v>2696000</v>
+        <v>4202400</v>
       </c>
       <c r="F36" t="n">
-        <v>990500</v>
+        <v>465000</v>
       </c>
       <c r="G36" t="n">
-        <v>58.07681031955438</v>
+        <v>12.44180446299566</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>HD건설기계</t>
+          <t>미창석유</t>
         </is>
       </c>
       <c r="B37" t="n">
-        <v>31</v>
+        <v>18</v>
       </c>
       <c r="C37" t="inlineStr">
         <is>
@@ -1431,23 +1431,23 @@
         <v>1</v>
       </c>
       <c r="E37" t="n">
-        <v>4123000</v>
+        <v>2097000</v>
       </c>
       <c r="F37" t="n">
-        <v>87904</v>
+        <v>-295200</v>
       </c>
       <c r="G37" t="n">
-        <v>2.178485964150543</v>
+        <v>-12.34010534236268</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>KoAct 코스닥액티브</t>
+          <t>비에이치아이</t>
         </is>
       </c>
       <c r="B38" t="n">
-        <v>200</v>
+        <v>8</v>
       </c>
       <c r="C38" t="inlineStr">
         <is>
@@ -1458,23 +1458,23 @@
         <v>1</v>
       </c>
       <c r="E38" t="n">
-        <v>2582000</v>
+        <v>876000</v>
       </c>
       <c r="F38" t="n">
-        <v>-120000</v>
+        <v>210885</v>
       </c>
       <c r="G38" t="n">
-        <v>-4.441154700222058</v>
+        <v>31.70654698811484</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>LX인터내셔널</t>
+          <t>삼성생명</t>
         </is>
       </c>
       <c r="B39" t="n">
-        <v>20</v>
+        <v>4</v>
       </c>
       <c r="C39" t="inlineStr">
         <is>
@@ -1485,23 +1485,23 @@
         <v>1</v>
       </c>
       <c r="E39" t="n">
-        <v>943000</v>
+        <v>926000</v>
       </c>
       <c r="F39" t="n">
-        <v>4000</v>
+        <v>93000</v>
       </c>
       <c r="G39" t="n">
-        <v>0.4259850905218318</v>
+        <v>11.16446578631453</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>NH투자증권우</t>
+          <t>삼성화재</t>
         </is>
       </c>
       <c r="B40" t="n">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="C40" t="inlineStr">
         <is>
@@ -1512,23 +1512,23 @@
         <v>1</v>
       </c>
       <c r="E40" t="n">
-        <v>54591</v>
+        <v>4270500</v>
       </c>
       <c r="F40" t="n">
-        <v>-9</v>
+        <v>-360500</v>
       </c>
       <c r="G40" t="n">
-        <v>-0.01648351648351648</v>
+        <v>-7.784495789246384</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>TIME 코리아밸류업액티브</t>
+          <t>세아제강</t>
         </is>
       </c>
       <c r="B41" t="n">
-        <v>201</v>
+        <v>50</v>
       </c>
       <c r="C41" t="inlineStr">
         <is>
@@ -1539,13 +1539,13 @@
         <v>1</v>
       </c>
       <c r="E41" t="n">
-        <v>4797870</v>
+        <v>7395000</v>
       </c>
       <c r="F41" t="n">
-        <v>74073</v>
+        <v>1085000</v>
       </c>
       <c r="G41" t="n">
-        <v>1.568081778281328</v>
+        <v>17.19492868462758</v>
       </c>
     </row>
   </sheetData>
@@ -1603,7 +1603,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2026-03-20T15:48:41</t>
+          <t>2026-03-20T15:49:08</t>
         </is>
       </c>
       <c r="E2" t="n">
@@ -5922,7 +5922,7 @@
       </c>
       <c r="I116" t="inlineStr">
         <is>
-          <t>2026-03-20T15:48:41</t>
+          <t>2026-03-20T15:49:08</t>
         </is>
       </c>
     </row>
@@ -5952,14 +5952,14 @@
         <v>10351433.71453537</v>
       </c>
       <c r="G117" t="n">
-        <v>-480581.2854646351</v>
+        <v>-480580.2854646333</v>
       </c>
       <c r="H117" t="n">
-        <v>-4.436674851951692</v>
+        <v>-4.43666602964724</v>
       </c>
       <c r="I117" t="inlineStr">
         <is>
-          <t>2026-03-20T15:48:41</t>
+          <t>2026-03-20T15:49:08</t>
         </is>
       </c>
     </row>
@@ -5996,7 +5996,7 @@
       </c>
       <c r="I118" t="inlineStr">
         <is>
-          <t>2026-03-20T15:48:41</t>
+          <t>2026-03-20T15:49:08</t>
         </is>
       </c>
     </row>
@@ -6033,7 +6033,7 @@
       </c>
       <c r="I119" t="inlineStr">
         <is>
-          <t>2026-03-20T15:48:41</t>
+          <t>2026-03-20T15:49:08</t>
         </is>
       </c>
     </row>
@@ -6070,7 +6070,7 @@
       </c>
       <c r="I120" t="inlineStr">
         <is>
-          <t>2026-03-20T15:48:41</t>
+          <t>2026-03-20T15:49:08</t>
         </is>
       </c>
     </row>
@@ -6107,7 +6107,7 @@
       </c>
       <c r="I121" t="inlineStr">
         <is>
-          <t>2026-03-20T15:48:41</t>
+          <t>2026-03-20T15:49:08</t>
         </is>
       </c>
     </row>
@@ -6144,7 +6144,7 @@
       </c>
       <c r="I122" t="inlineStr">
         <is>
-          <t>2026-03-20T15:48:41</t>
+          <t>2026-03-20T15:49:08</t>
         </is>
       </c>
     </row>
@@ -6181,7 +6181,7 @@
       </c>
       <c r="I123" t="inlineStr">
         <is>
-          <t>2026-03-20T15:48:41</t>
+          <t>2026-03-20T15:49:08</t>
         </is>
       </c>
     </row>
@@ -6218,7 +6218,7 @@
       </c>
       <c r="I124" t="inlineStr">
         <is>
-          <t>2026-03-20T15:48:41</t>
+          <t>2026-03-20T15:49:08</t>
         </is>
       </c>
     </row>
@@ -6255,7 +6255,7 @@
       </c>
       <c r="I125" t="inlineStr">
         <is>
-          <t>2026-03-20T15:48:41</t>
+          <t>2026-03-20T15:49:08</t>
         </is>
       </c>
     </row>
@@ -6292,7 +6292,7 @@
       </c>
       <c r="I126" t="inlineStr">
         <is>
-          <t>2026-03-20T15:48:41</t>
+          <t>2026-03-20T15:49:08</t>
         </is>
       </c>
     </row>
@@ -6329,7 +6329,7 @@
       </c>
       <c r="I127" t="inlineStr">
         <is>
-          <t>2026-03-20T15:48:41</t>
+          <t>2026-03-20T15:49:08</t>
         </is>
       </c>
     </row>
@@ -6366,7 +6366,7 @@
       </c>
       <c r="I128" t="inlineStr">
         <is>
-          <t>2026-03-20T15:48:41</t>
+          <t>2026-03-20T15:49:08</t>
         </is>
       </c>
     </row>
@@ -6403,7 +6403,7 @@
       </c>
       <c r="I129" t="inlineStr">
         <is>
-          <t>2026-03-20T15:48:41</t>
+          <t>2026-03-20T15:49:08</t>
         </is>
       </c>
     </row>
@@ -6440,7 +6440,7 @@
       </c>
       <c r="I130" t="inlineStr">
         <is>
-          <t>2026-03-20T15:48:41</t>
+          <t>2026-03-20T15:49:08</t>
         </is>
       </c>
     </row>
@@ -6477,7 +6477,7 @@
       </c>
       <c r="I131" t="inlineStr">
         <is>
-          <t>2026-03-20T15:48:41</t>
+          <t>2026-03-20T15:49:08</t>
         </is>
       </c>
     </row>
@@ -6514,7 +6514,7 @@
       </c>
       <c r="I132" t="inlineStr">
         <is>
-          <t>2026-03-20T15:48:41</t>
+          <t>2026-03-20T15:49:08</t>
         </is>
       </c>
     </row>
@@ -6526,11 +6526,11 @@
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>피바디 에너지</t>
+          <t>넥스틸</t>
         </is>
       </c>
       <c r="C133" t="n">
-        <v>65</v>
+        <v>300</v>
       </c>
       <c r="D133" t="inlineStr">
         <is>
@@ -6541,17 +6541,17 @@
         <v>1</v>
       </c>
       <c r="F133" t="n">
-        <v>3596373.331896178</v>
+        <v>3771000</v>
       </c>
       <c r="G133" t="n">
-        <v>2125601.331896178</v>
+        <v>521000</v>
       </c>
       <c r="H133" t="n">
-        <v>144.5228309959789</v>
+        <v>16.03076923076923</v>
       </c>
       <c r="I133" t="inlineStr">
         <is>
-          <t>2026-03-20T15:48:41</t>
+          <t>2026-03-20T15:49:08</t>
         </is>
       </c>
     </row>
@@ -6563,11 +6563,11 @@
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>현대제철</t>
+          <t>피바디 에너지</t>
         </is>
       </c>
       <c r="C134" t="n">
-        <v>80</v>
+        <v>65</v>
       </c>
       <c r="D134" t="inlineStr">
         <is>
@@ -6578,17 +6578,17 @@
         <v>1</v>
       </c>
       <c r="F134" t="n">
-        <v>2996000</v>
+        <v>3596373.331896178</v>
       </c>
       <c r="G134" t="n">
-        <v>-182000</v>
+        <v>2125601.331896178</v>
       </c>
       <c r="H134" t="n">
-        <v>-5.726872246696035</v>
+        <v>144.5228309959789</v>
       </c>
       <c r="I134" t="inlineStr">
         <is>
-          <t>2026-03-20T15:48:41</t>
+          <t>2026-03-20T15:49:08</t>
         </is>
       </c>
     </row>
@@ -6600,11 +6600,11 @@
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>더치 브로스</t>
+          <t>현대제철</t>
         </is>
       </c>
       <c r="C135" t="n">
-        <v>39</v>
+        <v>80</v>
       </c>
       <c r="D135" t="inlineStr">
         <is>
@@ -6615,17 +6615,17 @@
         <v>1</v>
       </c>
       <c r="F135" t="n">
-        <v>2959763.281021703</v>
+        <v>2996000</v>
       </c>
       <c r="G135" t="n">
-        <v>-230880.718978297</v>
+        <v>-182000</v>
       </c>
       <c r="H135" t="n">
-        <v>-7.236179247145621</v>
+        <v>-5.726872246696035</v>
       </c>
       <c r="I135" t="inlineStr">
         <is>
-          <t>2026-03-20T15:48:41</t>
+          <t>2026-03-20T15:49:08</t>
         </is>
       </c>
     </row>
@@ -6637,11 +6637,11 @@
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>휴스틸</t>
+          <t>더치 브로스</t>
         </is>
       </c>
       <c r="C136" t="n">
-        <v>500</v>
+        <v>39</v>
       </c>
       <c r="D136" t="inlineStr">
         <is>
@@ -6652,17 +6652,17 @@
         <v>1</v>
       </c>
       <c r="F136" t="n">
-        <v>2750000</v>
+        <v>2959763.281021703</v>
       </c>
       <c r="G136" t="n">
-        <v>471390</v>
+        <v>-230880.718978297</v>
       </c>
       <c r="H136" t="n">
-        <v>20.68761218462133</v>
+        <v>-7.236179247145621</v>
       </c>
       <c r="I136" t="inlineStr">
         <is>
-          <t>2026-03-20T15:48:41</t>
+          <t>2026-03-20T15:49:08</t>
         </is>
       </c>
     </row>
@@ -6674,11 +6674,11 @@
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>DL이앤씨</t>
+          <t>휴스틸</t>
         </is>
       </c>
       <c r="C137" t="n">
-        <v>40</v>
+        <v>500</v>
       </c>
       <c r="D137" t="inlineStr">
         <is>
@@ -6689,17 +6689,17 @@
         <v>1</v>
       </c>
       <c r="F137" t="n">
-        <v>2696000</v>
+        <v>2750000</v>
       </c>
       <c r="G137" t="n">
-        <v>990500</v>
+        <v>471390</v>
       </c>
       <c r="H137" t="n">
-        <v>58.07681031955438</v>
+        <v>20.68761218462133</v>
       </c>
       <c r="I137" t="inlineStr">
         <is>
-          <t>2026-03-20T15:48:41</t>
+          <t>2026-03-20T15:49:08</t>
         </is>
       </c>
     </row>
@@ -6711,11 +6711,11 @@
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>KoAct 코스닥액티브</t>
+          <t>DL이앤씨</t>
         </is>
       </c>
       <c r="C138" t="n">
-        <v>200</v>
+        <v>40</v>
       </c>
       <c r="D138" t="inlineStr">
         <is>
@@ -6726,17 +6726,17 @@
         <v>1</v>
       </c>
       <c r="F138" t="n">
-        <v>2582000</v>
+        <v>2696000</v>
       </c>
       <c r="G138" t="n">
-        <v>-120000</v>
+        <v>990500</v>
       </c>
       <c r="H138" t="n">
-        <v>-4.441154700222058</v>
+        <v>58.07681031955438</v>
       </c>
       <c r="I138" t="inlineStr">
         <is>
-          <t>2026-03-20T15:48:41</t>
+          <t>2026-03-20T15:49:08</t>
         </is>
       </c>
     </row>
@@ -6748,7 +6748,7 @@
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>넥스틸</t>
+          <t>KoAct 코스닥액티브</t>
         </is>
       </c>
       <c r="C139" t="n">
@@ -6763,17 +6763,17 @@
         <v>1</v>
       </c>
       <c r="F139" t="n">
-        <v>2514000</v>
+        <v>2582000</v>
       </c>
       <c r="G139" t="n">
-        <v>503000</v>
+        <v>-120000</v>
       </c>
       <c r="H139" t="n">
-        <v>25.01243162605669</v>
+        <v>-4.441154700222058</v>
       </c>
       <c r="I139" t="inlineStr">
         <is>
-          <t>2026-03-20T15:48:41</t>
+          <t>2026-03-20T15:49:08</t>
         </is>
       </c>
     </row>
@@ -6810,7 +6810,7 @@
       </c>
       <c r="I140" t="inlineStr">
         <is>
-          <t>2026-03-20T15:48:41</t>
+          <t>2026-03-20T15:49:08</t>
         </is>
       </c>
     </row>
@@ -6847,7 +6847,7 @@
       </c>
       <c r="I141" t="inlineStr">
         <is>
-          <t>2026-03-20T15:48:41</t>
+          <t>2026-03-20T15:49:08</t>
         </is>
       </c>
     </row>
@@ -6884,7 +6884,7 @@
       </c>
       <c r="I142" t="inlineStr">
         <is>
-          <t>2026-03-20T15:48:41</t>
+          <t>2026-03-20T15:49:08</t>
         </is>
       </c>
     </row>
@@ -6921,7 +6921,7 @@
       </c>
       <c r="I143" t="inlineStr">
         <is>
-          <t>2026-03-20T15:48:41</t>
+          <t>2026-03-20T15:49:08</t>
         </is>
       </c>
     </row>
@@ -6958,7 +6958,7 @@
       </c>
       <c r="I144" t="inlineStr">
         <is>
-          <t>2026-03-20T15:48:41</t>
+          <t>2026-03-20T15:49:08</t>
         </is>
       </c>
     </row>
@@ -6995,7 +6995,7 @@
       </c>
       <c r="I145" t="inlineStr">
         <is>
-          <t>2026-03-20T15:48:41</t>
+          <t>2026-03-20T15:49:08</t>
         </is>
       </c>
     </row>
@@ -7032,7 +7032,7 @@
       </c>
       <c r="I146" t="inlineStr">
         <is>
-          <t>2026-03-20T15:48:41</t>
+          <t>2026-03-20T15:49:08</t>
         </is>
       </c>
     </row>
@@ -7069,7 +7069,7 @@
       </c>
       <c r="I147" t="inlineStr">
         <is>
-          <t>2026-03-20T15:48:41</t>
+          <t>2026-03-20T15:49:08</t>
         </is>
       </c>
     </row>
@@ -7106,7 +7106,7 @@
       </c>
       <c r="I148" t="inlineStr">
         <is>
-          <t>2026-03-20T15:48:41</t>
+          <t>2026-03-20T15:49:08</t>
         </is>
       </c>
     </row>
@@ -7143,7 +7143,7 @@
       </c>
       <c r="I149" t="inlineStr">
         <is>
-          <t>2026-03-20T15:48:41</t>
+          <t>2026-03-20T15:49:08</t>
         </is>
       </c>
     </row>
@@ -7180,7 +7180,7 @@
       </c>
       <c r="I150" t="inlineStr">
         <is>
-          <t>2026-03-20T15:48:41</t>
+          <t>2026-03-20T15:49:08</t>
         </is>
       </c>
     </row>
@@ -7217,7 +7217,7 @@
       </c>
       <c r="I151" t="inlineStr">
         <is>
-          <t>2026-03-20T15:48:41</t>
+          <t>2026-03-20T15:49:08</t>
         </is>
       </c>
     </row>
@@ -7254,7 +7254,7 @@
       </c>
       <c r="I152" t="inlineStr">
         <is>
-          <t>2026-03-20T15:48:41</t>
+          <t>2026-03-20T15:49:08</t>
         </is>
       </c>
     </row>
@@ -7291,7 +7291,7 @@
       </c>
       <c r="I153" t="inlineStr">
         <is>
-          <t>2026-03-20T15:48:41</t>
+          <t>2026-03-20T15:49:08</t>
         </is>
       </c>
     </row>
@@ -7328,7 +7328,7 @@
       </c>
       <c r="I154" t="inlineStr">
         <is>
-          <t>2026-03-20T15:48:41</t>
+          <t>2026-03-20T15:49:08</t>
         </is>
       </c>
     </row>
@@ -7365,7 +7365,7 @@
       </c>
       <c r="I155" t="inlineStr">
         <is>
-          <t>2026-03-20T15:48:41</t>
+          <t>2026-03-20T15:49:08</t>
         </is>
       </c>
     </row>
@@ -7498,7 +7498,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>2026-03-20T15:48:41</t>
+          <t>2026-03-20T15:49:08</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: portfolio snapshot 2026-03-20 (2026-03-20T15:49:10)
</commit_message>
<xml_diff>
--- a/portfolio_auto.xlsx
+++ b/portfolio_auto.xlsx
@@ -1603,7 +1603,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2026-03-20T15:49:08</t>
+          <t>2026-03-20T15:49:10</t>
         </is>
       </c>
       <c r="E2" t="n">
@@ -5922,7 +5922,7 @@
       </c>
       <c r="I116" t="inlineStr">
         <is>
-          <t>2026-03-20T15:49:08</t>
+          <t>2026-03-20T15:49:10</t>
         </is>
       </c>
     </row>
@@ -5959,7 +5959,7 @@
       </c>
       <c r="I117" t="inlineStr">
         <is>
-          <t>2026-03-20T15:49:08</t>
+          <t>2026-03-20T15:49:10</t>
         </is>
       </c>
     </row>
@@ -5996,7 +5996,7 @@
       </c>
       <c r="I118" t="inlineStr">
         <is>
-          <t>2026-03-20T15:49:08</t>
+          <t>2026-03-20T15:49:10</t>
         </is>
       </c>
     </row>
@@ -6033,7 +6033,7 @@
       </c>
       <c r="I119" t="inlineStr">
         <is>
-          <t>2026-03-20T15:49:08</t>
+          <t>2026-03-20T15:49:10</t>
         </is>
       </c>
     </row>
@@ -6070,7 +6070,7 @@
       </c>
       <c r="I120" t="inlineStr">
         <is>
-          <t>2026-03-20T15:49:08</t>
+          <t>2026-03-20T15:49:10</t>
         </is>
       </c>
     </row>
@@ -6107,7 +6107,7 @@
       </c>
       <c r="I121" t="inlineStr">
         <is>
-          <t>2026-03-20T15:49:08</t>
+          <t>2026-03-20T15:49:10</t>
         </is>
       </c>
     </row>
@@ -6144,7 +6144,7 @@
       </c>
       <c r="I122" t="inlineStr">
         <is>
-          <t>2026-03-20T15:49:08</t>
+          <t>2026-03-20T15:49:10</t>
         </is>
       </c>
     </row>
@@ -6181,7 +6181,7 @@
       </c>
       <c r="I123" t="inlineStr">
         <is>
-          <t>2026-03-20T15:49:08</t>
+          <t>2026-03-20T15:49:10</t>
         </is>
       </c>
     </row>
@@ -6218,7 +6218,7 @@
       </c>
       <c r="I124" t="inlineStr">
         <is>
-          <t>2026-03-20T15:49:08</t>
+          <t>2026-03-20T15:49:10</t>
         </is>
       </c>
     </row>
@@ -6255,7 +6255,7 @@
       </c>
       <c r="I125" t="inlineStr">
         <is>
-          <t>2026-03-20T15:49:08</t>
+          <t>2026-03-20T15:49:10</t>
         </is>
       </c>
     </row>
@@ -6292,7 +6292,7 @@
       </c>
       <c r="I126" t="inlineStr">
         <is>
-          <t>2026-03-20T15:49:08</t>
+          <t>2026-03-20T15:49:10</t>
         </is>
       </c>
     </row>
@@ -6329,7 +6329,7 @@
       </c>
       <c r="I127" t="inlineStr">
         <is>
-          <t>2026-03-20T15:49:08</t>
+          <t>2026-03-20T15:49:10</t>
         </is>
       </c>
     </row>
@@ -6366,7 +6366,7 @@
       </c>
       <c r="I128" t="inlineStr">
         <is>
-          <t>2026-03-20T15:49:08</t>
+          <t>2026-03-20T15:49:10</t>
         </is>
       </c>
     </row>
@@ -6403,7 +6403,7 @@
       </c>
       <c r="I129" t="inlineStr">
         <is>
-          <t>2026-03-20T15:49:08</t>
+          <t>2026-03-20T15:49:10</t>
         </is>
       </c>
     </row>
@@ -6440,7 +6440,7 @@
       </c>
       <c r="I130" t="inlineStr">
         <is>
-          <t>2026-03-20T15:49:08</t>
+          <t>2026-03-20T15:49:10</t>
         </is>
       </c>
     </row>
@@ -6477,7 +6477,7 @@
       </c>
       <c r="I131" t="inlineStr">
         <is>
-          <t>2026-03-20T15:49:08</t>
+          <t>2026-03-20T15:49:10</t>
         </is>
       </c>
     </row>
@@ -6514,7 +6514,7 @@
       </c>
       <c r="I132" t="inlineStr">
         <is>
-          <t>2026-03-20T15:49:08</t>
+          <t>2026-03-20T15:49:10</t>
         </is>
       </c>
     </row>
@@ -6551,7 +6551,7 @@
       </c>
       <c r="I133" t="inlineStr">
         <is>
-          <t>2026-03-20T15:49:08</t>
+          <t>2026-03-20T15:49:10</t>
         </is>
       </c>
     </row>
@@ -6588,7 +6588,7 @@
       </c>
       <c r="I134" t="inlineStr">
         <is>
-          <t>2026-03-20T15:49:08</t>
+          <t>2026-03-20T15:49:10</t>
         </is>
       </c>
     </row>
@@ -6625,7 +6625,7 @@
       </c>
       <c r="I135" t="inlineStr">
         <is>
-          <t>2026-03-20T15:49:08</t>
+          <t>2026-03-20T15:49:10</t>
         </is>
       </c>
     </row>
@@ -6662,7 +6662,7 @@
       </c>
       <c r="I136" t="inlineStr">
         <is>
-          <t>2026-03-20T15:49:08</t>
+          <t>2026-03-20T15:49:10</t>
         </is>
       </c>
     </row>
@@ -6699,7 +6699,7 @@
       </c>
       <c r="I137" t="inlineStr">
         <is>
-          <t>2026-03-20T15:49:08</t>
+          <t>2026-03-20T15:49:10</t>
         </is>
       </c>
     </row>
@@ -6736,7 +6736,7 @@
       </c>
       <c r="I138" t="inlineStr">
         <is>
-          <t>2026-03-20T15:49:08</t>
+          <t>2026-03-20T15:49:10</t>
         </is>
       </c>
     </row>
@@ -6773,7 +6773,7 @@
       </c>
       <c r="I139" t="inlineStr">
         <is>
-          <t>2026-03-20T15:49:08</t>
+          <t>2026-03-20T15:49:10</t>
         </is>
       </c>
     </row>
@@ -6810,7 +6810,7 @@
       </c>
       <c r="I140" t="inlineStr">
         <is>
-          <t>2026-03-20T15:49:08</t>
+          <t>2026-03-20T15:49:10</t>
         </is>
       </c>
     </row>
@@ -6847,7 +6847,7 @@
       </c>
       <c r="I141" t="inlineStr">
         <is>
-          <t>2026-03-20T15:49:08</t>
+          <t>2026-03-20T15:49:10</t>
         </is>
       </c>
     </row>
@@ -6884,7 +6884,7 @@
       </c>
       <c r="I142" t="inlineStr">
         <is>
-          <t>2026-03-20T15:49:08</t>
+          <t>2026-03-20T15:49:10</t>
         </is>
       </c>
     </row>
@@ -6921,7 +6921,7 @@
       </c>
       <c r="I143" t="inlineStr">
         <is>
-          <t>2026-03-20T15:49:08</t>
+          <t>2026-03-20T15:49:10</t>
         </is>
       </c>
     </row>
@@ -6958,7 +6958,7 @@
       </c>
       <c r="I144" t="inlineStr">
         <is>
-          <t>2026-03-20T15:49:08</t>
+          <t>2026-03-20T15:49:10</t>
         </is>
       </c>
     </row>
@@ -6995,7 +6995,7 @@
       </c>
       <c r="I145" t="inlineStr">
         <is>
-          <t>2026-03-20T15:49:08</t>
+          <t>2026-03-20T15:49:10</t>
         </is>
       </c>
     </row>
@@ -7032,7 +7032,7 @@
       </c>
       <c r="I146" t="inlineStr">
         <is>
-          <t>2026-03-20T15:49:08</t>
+          <t>2026-03-20T15:49:10</t>
         </is>
       </c>
     </row>
@@ -7069,7 +7069,7 @@
       </c>
       <c r="I147" t="inlineStr">
         <is>
-          <t>2026-03-20T15:49:08</t>
+          <t>2026-03-20T15:49:10</t>
         </is>
       </c>
     </row>
@@ -7106,7 +7106,7 @@
       </c>
       <c r="I148" t="inlineStr">
         <is>
-          <t>2026-03-20T15:49:08</t>
+          <t>2026-03-20T15:49:10</t>
         </is>
       </c>
     </row>
@@ -7143,7 +7143,7 @@
       </c>
       <c r="I149" t="inlineStr">
         <is>
-          <t>2026-03-20T15:49:08</t>
+          <t>2026-03-20T15:49:10</t>
         </is>
       </c>
     </row>
@@ -7180,7 +7180,7 @@
       </c>
       <c r="I150" t="inlineStr">
         <is>
-          <t>2026-03-20T15:49:08</t>
+          <t>2026-03-20T15:49:10</t>
         </is>
       </c>
     </row>
@@ -7217,7 +7217,7 @@
       </c>
       <c r="I151" t="inlineStr">
         <is>
-          <t>2026-03-20T15:49:08</t>
+          <t>2026-03-20T15:49:10</t>
         </is>
       </c>
     </row>
@@ -7254,7 +7254,7 @@
       </c>
       <c r="I152" t="inlineStr">
         <is>
-          <t>2026-03-20T15:49:08</t>
+          <t>2026-03-20T15:49:10</t>
         </is>
       </c>
     </row>
@@ -7291,7 +7291,7 @@
       </c>
       <c r="I153" t="inlineStr">
         <is>
-          <t>2026-03-20T15:49:08</t>
+          <t>2026-03-20T15:49:10</t>
         </is>
       </c>
     </row>
@@ -7328,7 +7328,7 @@
       </c>
       <c r="I154" t="inlineStr">
         <is>
-          <t>2026-03-20T15:49:08</t>
+          <t>2026-03-20T15:49:10</t>
         </is>
       </c>
     </row>
@@ -7365,7 +7365,7 @@
       </c>
       <c r="I155" t="inlineStr">
         <is>
-          <t>2026-03-20T15:49:08</t>
+          <t>2026-03-20T15:49:10</t>
         </is>
       </c>
     </row>
@@ -7498,7 +7498,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>2026-03-20T15:49:08</t>
+          <t>2026-03-20T15:49:10</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: portfolio snapshot 2026-03-20 (2026-03-20T15:49:39)
</commit_message>
<xml_diff>
--- a/portfolio_auto.xlsx
+++ b/portfolio_auto.xlsx
@@ -471,11 +471,11 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>페트로브라스 (ADR)</t>
+          <t>유나이티드헬스 그룹</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>480</v>
+        <v>4</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
@@ -486,23 +486,23 @@
         <v>1</v>
       </c>
       <c r="E2" t="n">
-        <v>13553578.62304688</v>
+        <v>1683366.447431445</v>
       </c>
       <c r="F2" t="n">
-        <v>1447029.623046879</v>
+        <v>-11089.55256855441</v>
       </c>
       <c r="G2" t="n">
-        <v>11.95245336261291</v>
+        <v>-0.6544609342794628</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>시드릴</t>
+          <t>케이씨</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>123</v>
+        <v>50</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
@@ -513,23 +513,23 @@
         <v>1</v>
       </c>
       <c r="E3" t="n">
-        <v>8081063.113214018</v>
+        <v>1670000</v>
       </c>
       <c r="F3" t="n">
-        <v>1630712.113214018</v>
+        <v>20500</v>
       </c>
       <c r="G3" t="n">
-        <v>25.28098258860669</v>
+        <v>1.242800848742043</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>트랜스오션</t>
+          <t>하나금융지주</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>750</v>
+        <v>18</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
@@ -540,23 +540,23 @@
         <v>1</v>
       </c>
       <c r="E4" t="n">
-        <v>7074115.140040115</v>
+        <v>2037600</v>
       </c>
       <c r="F4" t="n">
-        <v>2946881.140040115</v>
+        <v>12200</v>
       </c>
       <c r="G4" t="n">
-        <v>71.40087380652794</v>
+        <v>0.6023501530561864</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>노블</t>
+          <t>현대제철</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>99</v>
+        <v>80</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -567,23 +567,23 @@
         <v>1</v>
       </c>
       <c r="E5" t="n">
-        <v>6886743.840087891</v>
+        <v>2996000</v>
       </c>
       <c r="F5" t="n">
-        <v>2979535.840087891</v>
+        <v>-182000</v>
       </c>
       <c r="G5" t="n">
-        <v>76.25741552760668</v>
+        <v>-5.726872246696035</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>센트러스 에너지</t>
+          <t>휴스틸</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>21</v>
+        <v>500</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
@@ -594,23 +594,23 @@
         <v>1</v>
       </c>
       <c r="E6" t="n">
-        <v>5996448.754211426</v>
+        <v>2750000</v>
       </c>
       <c r="F6" t="n">
-        <v>-234770.2457885733</v>
+        <v>471390</v>
       </c>
       <c r="G6" t="n">
-        <v>-3.767645556809564</v>
+        <v>20.68761218462133</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>타이드워터</t>
+          <t>DL이앤씨</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>48</v>
+        <v>40</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -621,23 +621,23 @@
         <v>1</v>
       </c>
       <c r="E7" t="n">
-        <v>5211036.802851856</v>
+        <v>2696000</v>
       </c>
       <c r="F7" t="n">
-        <v>1486491.802851856</v>
+        <v>990500</v>
       </c>
       <c r="G7" t="n">
-        <v>39.91069520845783</v>
+        <v>58.07681031955438</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>노브</t>
+          <t>HD건설기계</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>185</v>
+        <v>31</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
@@ -648,23 +648,23 @@
         <v>1</v>
       </c>
       <c r="E8" t="n">
-        <v>5179494.129107101</v>
+        <v>4123000</v>
       </c>
       <c r="F8" t="n">
-        <v>1869486.129107101</v>
+        <v>87904</v>
       </c>
       <c r="G8" t="n">
-        <v>56.47980697046958</v>
+        <v>2.178485964150543</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>오케아니스 에코 탱커스</t>
+          <t>KoAct 코스닥액티브</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>65</v>
+        <v>200</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
@@ -675,23 +675,23 @@
         <v>1</v>
       </c>
       <c r="E9" t="n">
-        <v>4596307.895957222</v>
+        <v>2582000</v>
       </c>
       <c r="F9" t="n">
-        <v>2339947.895957222</v>
+        <v>-120000</v>
       </c>
       <c r="G9" t="n">
-        <v>103.704546081176</v>
+        <v>-4.441154700222058</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>차코스 에너지 내비게이션</t>
+          <t>LX인터내셔널</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>75</v>
+        <v>20</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
@@ -702,23 +702,23 @@
         <v>1</v>
       </c>
       <c r="E10" t="n">
-        <v>4052048.962918622</v>
+        <v>943000</v>
       </c>
       <c r="F10" t="n">
-        <v>227400.9629186224</v>
+        <v>4000</v>
       </c>
       <c r="G10" t="n">
-        <v>5.94567037067522</v>
+        <v>0.4259850905218318</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>더치 브로스</t>
+          <t>NH투자증권우</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>39</v>
+        <v>2</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
@@ -729,23 +729,23 @@
         <v>1</v>
       </c>
       <c r="E11" t="n">
-        <v>2959763.281021703</v>
+        <v>54591</v>
       </c>
       <c r="F11" t="n">
-        <v>-230880.718978297</v>
+        <v>-9</v>
       </c>
       <c r="G11" t="n">
-        <v>-7.236179247145621</v>
+        <v>-0.01648351648351648</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>발레로 에너지</t>
+          <t>TIME 코리아밸류업액티브</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>6</v>
+        <v>201</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
@@ -756,23 +756,23 @@
         <v>1</v>
       </c>
       <c r="E12" t="n">
-        <v>2176561.162089184</v>
+        <v>4797870</v>
       </c>
       <c r="F12" t="n">
-        <v>112571.1620891844</v>
+        <v>74073</v>
       </c>
       <c r="G12" t="n">
-        <v>5.45405559567558</v>
+        <v>1.568081778281328</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>스타 벌크 캐리어스</t>
+          <t>프론트라인</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>50</v>
+        <v>175</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
@@ -783,23 +783,23 @@
         <v>1</v>
       </c>
       <c r="E13" t="n">
-        <v>1696441.320678405</v>
+        <v>8453409.11431564</v>
       </c>
       <c r="F13" t="n">
-        <v>382088.3206784062</v>
+        <v>4023545.11431564</v>
       </c>
       <c r="G13" t="n">
-        <v>29.07044916231837</v>
+        <v>90.82773453802736</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>유나이티드헬스 그룹</t>
+          <t>피바디 에너지</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>4</v>
+        <v>65</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
@@ -810,23 +810,23 @@
         <v>1</v>
       </c>
       <c r="E14" t="n">
-        <v>1683366.447431445</v>
+        <v>3596373.331896178</v>
       </c>
       <c r="F14" t="n">
-        <v>-11089.55256855441</v>
+        <v>2125601.331896178</v>
       </c>
       <c r="G14" t="n">
-        <v>-0.6544609342794628</v>
+        <v>144.5228309959789</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>클리블랜드 클리프스</t>
+          <t>하프니아</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
@@ -837,23 +837,23 @@
         <v>1</v>
       </c>
       <c r="E15" t="n">
-        <v>833036.4441346284</v>
+        <v>848519.8631833494</v>
       </c>
       <c r="F15" t="n">
-        <v>-183018.5558653716</v>
+        <v>222788.8631833494</v>
       </c>
       <c r="G15" t="n">
-        <v>-18.01266229341636</v>
+        <v>35.60457499841775</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>텍사스 퍼시픽 랜드</t>
+          <t>AGNC 인베스트먼트</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>1</v>
+        <v>700</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
@@ -864,23 +864,23 @@
         <v>1</v>
       </c>
       <c r="E16" t="n">
-        <v>798210.0491355956</v>
+        <v>10351433.71453537</v>
       </c>
       <c r="F16" t="n">
-        <v>19619.04913559556</v>
+        <v>-480580.2854646333</v>
       </c>
       <c r="G16" t="n">
-        <v>2.519814528500273</v>
+        <v>-4.43666602964724</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>케이씨</t>
+          <t>넥스틸</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>50</v>
+        <v>300</v>
       </c>
       <c r="C17" t="inlineStr">
         <is>
@@ -891,23 +891,23 @@
         <v>1</v>
       </c>
       <c r="E17" t="n">
-        <v>1670000</v>
+        <v>3771000</v>
       </c>
       <c r="F17" t="n">
-        <v>20500</v>
+        <v>521000</v>
       </c>
       <c r="G17" t="n">
-        <v>1.242800848742043</v>
+        <v>16.03076923076923</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>하나금융지주</t>
+          <t>대신증권</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>18</v>
+        <v>55</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
@@ -918,23 +918,23 @@
         <v>1</v>
       </c>
       <c r="E18" t="n">
-        <v>2037600</v>
+        <v>2219250</v>
       </c>
       <c r="F18" t="n">
-        <v>12200</v>
+        <v>509749</v>
       </c>
       <c r="G18" t="n">
-        <v>0.6023501530561864</v>
+        <v>29.81858448752005</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>현대제철</t>
+          <t>대창단조</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>80</v>
+        <v>300</v>
       </c>
       <c r="C19" t="inlineStr">
         <is>
@@ -945,23 +945,23 @@
         <v>1</v>
       </c>
       <c r="E19" t="n">
-        <v>2996000</v>
+        <v>2004000</v>
       </c>
       <c r="F19" t="n">
-        <v>-182000</v>
+        <v>-54000</v>
       </c>
       <c r="G19" t="n">
-        <v>-5.726872246696035</v>
+        <v>-2.623906705539359</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>휴스틸</t>
+          <t>대한조선</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>500</v>
+        <v>100</v>
       </c>
       <c r="C20" t="inlineStr">
         <is>
@@ -972,23 +972,23 @@
         <v>1</v>
       </c>
       <c r="E20" t="n">
-        <v>2750000</v>
+        <v>9120000</v>
       </c>
       <c r="F20" t="n">
-        <v>471390</v>
+        <v>1907000</v>
       </c>
       <c r="G20" t="n">
-        <v>20.68761218462133</v>
+        <v>26.43837515596839</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>DL이앤씨</t>
+          <t>동방</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>40</v>
+        <v>681</v>
       </c>
       <c r="C21" t="inlineStr">
         <is>
@@ -999,23 +999,23 @@
         <v>1</v>
       </c>
       <c r="E21" t="n">
-        <v>2696000</v>
+        <v>1995330</v>
       </c>
       <c r="F21" t="n">
-        <v>990500</v>
+        <v>23829</v>
       </c>
       <c r="G21" t="n">
-        <v>58.07681031955438</v>
+        <v>1.208672985709873</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>HD건설기계</t>
+          <t>동원개발</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>31</v>
+        <v>1360</v>
       </c>
       <c r="C22" t="inlineStr">
         <is>
@@ -1026,23 +1026,23 @@
         <v>1</v>
       </c>
       <c r="E22" t="n">
-        <v>4123000</v>
+        <v>4202400</v>
       </c>
       <c r="F22" t="n">
-        <v>87904</v>
+        <v>465000</v>
       </c>
       <c r="G22" t="n">
-        <v>2.178485964150543</v>
+        <v>12.44180446299566</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>KoAct 코스닥액티브</t>
+          <t>미창석유</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>200</v>
+        <v>18</v>
       </c>
       <c r="C23" t="inlineStr">
         <is>
@@ -1053,23 +1053,23 @@
         <v>1</v>
       </c>
       <c r="E23" t="n">
-        <v>2582000</v>
+        <v>2097000</v>
       </c>
       <c r="F23" t="n">
-        <v>-120000</v>
+        <v>-295200</v>
       </c>
       <c r="G23" t="n">
-        <v>-4.441154700222058</v>
+        <v>-12.34010534236268</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>LX인터내셔널</t>
+          <t>비에이치아이</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>20</v>
+        <v>8</v>
       </c>
       <c r="C24" t="inlineStr">
         <is>
@@ -1080,23 +1080,23 @@
         <v>1</v>
       </c>
       <c r="E24" t="n">
-        <v>943000</v>
+        <v>876000</v>
       </c>
       <c r="F24" t="n">
-        <v>4000</v>
+        <v>210885</v>
       </c>
       <c r="G24" t="n">
-        <v>0.4259850905218318</v>
+        <v>31.70654698811484</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>NH투자증권우</t>
+          <t>삼성생명</t>
         </is>
       </c>
       <c r="B25" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="C25" t="inlineStr">
         <is>
@@ -1107,23 +1107,23 @@
         <v>1</v>
       </c>
       <c r="E25" t="n">
-        <v>54591</v>
+        <v>926000</v>
       </c>
       <c r="F25" t="n">
-        <v>-9</v>
+        <v>93000</v>
       </c>
       <c r="G25" t="n">
-        <v>-0.01648351648351648</v>
+        <v>11.16446578631453</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>TIME 코리아밸류업액티브</t>
+          <t>삼성화재</t>
         </is>
       </c>
       <c r="B26" t="n">
-        <v>201</v>
+        <v>9</v>
       </c>
       <c r="C26" t="inlineStr">
         <is>
@@ -1134,23 +1134,23 @@
         <v>1</v>
       </c>
       <c r="E26" t="n">
-        <v>4797870</v>
+        <v>4270500</v>
       </c>
       <c r="F26" t="n">
-        <v>74073</v>
+        <v>-360500</v>
       </c>
       <c r="G26" t="n">
-        <v>1.568081778281328</v>
+        <v>-7.784495789246384</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>프론트라인</t>
+          <t>세아제강</t>
         </is>
       </c>
       <c r="B27" t="n">
-        <v>175</v>
+        <v>50</v>
       </c>
       <c r="C27" t="inlineStr">
         <is>
@@ -1161,23 +1161,23 @@
         <v>1</v>
       </c>
       <c r="E27" t="n">
-        <v>8453409.11431564</v>
+        <v>7395000</v>
       </c>
       <c r="F27" t="n">
-        <v>4023545.11431564</v>
+        <v>1085000</v>
       </c>
       <c r="G27" t="n">
-        <v>90.82773453802736</v>
+        <v>17.19492868462758</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>피바디 에너지</t>
+          <t>노브</t>
         </is>
       </c>
       <c r="B28" t="n">
-        <v>65</v>
+        <v>185</v>
       </c>
       <c r="C28" t="inlineStr">
         <is>
@@ -1188,23 +1188,23 @@
         <v>1</v>
       </c>
       <c r="E28" t="n">
-        <v>3596373.331896178</v>
+        <v>5179494.129107101</v>
       </c>
       <c r="F28" t="n">
-        <v>2125601.331896178</v>
+        <v>1869486.129107101</v>
       </c>
       <c r="G28" t="n">
-        <v>144.5228309959789</v>
+        <v>56.47980697046958</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>하프니아</t>
+          <t>노블</t>
         </is>
       </c>
       <c r="B29" t="n">
-        <v>80</v>
+        <v>99</v>
       </c>
       <c r="C29" t="inlineStr">
         <is>
@@ -1215,23 +1215,23 @@
         <v>1</v>
       </c>
       <c r="E29" t="n">
-        <v>848519.8631833494</v>
+        <v>6886743.840087891</v>
       </c>
       <c r="F29" t="n">
-        <v>222788.8631833494</v>
+        <v>2979535.840087891</v>
       </c>
       <c r="G29" t="n">
-        <v>35.60457499841775</v>
+        <v>76.25741552760668</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>AGNC 인베스트먼트</t>
+          <t>더치 브로스</t>
         </is>
       </c>
       <c r="B30" t="n">
-        <v>700</v>
+        <v>39</v>
       </c>
       <c r="C30" t="inlineStr">
         <is>
@@ -1242,23 +1242,23 @@
         <v>1</v>
       </c>
       <c r="E30" t="n">
-        <v>10351433.71453537</v>
+        <v>2959763.281021703</v>
       </c>
       <c r="F30" t="n">
-        <v>-480580.2854646333</v>
+        <v>-230880.718978297</v>
       </c>
       <c r="G30" t="n">
-        <v>-4.43666602964724</v>
+        <v>-7.236179247145621</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>넥스틸</t>
+          <t>발레로 에너지</t>
         </is>
       </c>
       <c r="B31" t="n">
-        <v>300</v>
+        <v>6</v>
       </c>
       <c r="C31" t="inlineStr">
         <is>
@@ -1269,23 +1269,23 @@
         <v>1</v>
       </c>
       <c r="E31" t="n">
-        <v>3771000</v>
+        <v>2176561.162089184</v>
       </c>
       <c r="F31" t="n">
-        <v>521000</v>
+        <v>112571.1620891839</v>
       </c>
       <c r="G31" t="n">
-        <v>16.03076923076923</v>
+        <v>5.454055595675557</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>대신증권</t>
+          <t>센트러스 에너지</t>
         </is>
       </c>
       <c r="B32" t="n">
-        <v>55</v>
+        <v>25</v>
       </c>
       <c r="C32" t="inlineStr">
         <is>
@@ -1296,23 +1296,23 @@
         <v>1</v>
       </c>
       <c r="E32" t="n">
-        <v>2219250</v>
+        <v>7138629.469299316</v>
       </c>
       <c r="F32" t="n">
-        <v>509749</v>
+        <v>-294226.5307006836</v>
       </c>
       <c r="G32" t="n">
-        <v>29.81858448752005</v>
+        <v>-3.958458642286136</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>대창단조</t>
+          <t>스타 벌크 캐리어스</t>
         </is>
       </c>
       <c r="B33" t="n">
-        <v>300</v>
+        <v>50</v>
       </c>
       <c r="C33" t="inlineStr">
         <is>
@@ -1323,23 +1323,23 @@
         <v>1</v>
       </c>
       <c r="E33" t="n">
-        <v>2004000</v>
+        <v>1696441.320678405</v>
       </c>
       <c r="F33" t="n">
-        <v>-54000</v>
+        <v>382088.3206784055</v>
       </c>
       <c r="G33" t="n">
-        <v>-2.623906705539359</v>
+        <v>29.0704491623183</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>대한조선</t>
+          <t>시드릴</t>
         </is>
       </c>
       <c r="B34" t="n">
-        <v>100</v>
+        <v>123</v>
       </c>
       <c r="C34" t="inlineStr">
         <is>
@@ -1350,23 +1350,23 @@
         <v>1</v>
       </c>
       <c r="E34" t="n">
-        <v>9120000</v>
+        <v>8081063.113214018</v>
       </c>
       <c r="F34" t="n">
-        <v>1907000</v>
+        <v>1630712.113214018</v>
       </c>
       <c r="G34" t="n">
-        <v>26.43837515596839</v>
+        <v>25.28098258860669</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>동방</t>
+          <t>오케아니스 에코 탱커스</t>
         </is>
       </c>
       <c r="B35" t="n">
-        <v>681</v>
+        <v>65</v>
       </c>
       <c r="C35" t="inlineStr">
         <is>
@@ -1377,23 +1377,23 @@
         <v>1</v>
       </c>
       <c r="E35" t="n">
-        <v>1995330</v>
+        <v>4596307.895957222</v>
       </c>
       <c r="F35" t="n">
-        <v>23829</v>
+        <v>2339947.895957222</v>
       </c>
       <c r="G35" t="n">
-        <v>1.208672985709873</v>
+        <v>103.704546081176</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>동원개발</t>
+          <t>차코스 에너지 내비게이션</t>
         </is>
       </c>
       <c r="B36" t="n">
-        <v>1360</v>
+        <v>75</v>
       </c>
       <c r="C36" t="inlineStr">
         <is>
@@ -1404,23 +1404,23 @@
         <v>1</v>
       </c>
       <c r="E36" t="n">
-        <v>4202400</v>
+        <v>4052048.962918622</v>
       </c>
       <c r="F36" t="n">
-        <v>465000</v>
+        <v>227400.9629186224</v>
       </c>
       <c r="G36" t="n">
-        <v>12.44180446299566</v>
+        <v>5.94567037067522</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>미창석유</t>
+          <t>클리블랜드 클리프스</t>
         </is>
       </c>
       <c r="B37" t="n">
-        <v>18</v>
+        <v>70</v>
       </c>
       <c r="C37" t="inlineStr">
         <is>
@@ -1431,23 +1431,23 @@
         <v>1</v>
       </c>
       <c r="E37" t="n">
-        <v>2097000</v>
+        <v>833036.4441346284</v>
       </c>
       <c r="F37" t="n">
-        <v>-295200</v>
+        <v>-183018.5558653716</v>
       </c>
       <c r="G37" t="n">
-        <v>-12.34010534236268</v>
+        <v>-18.01266229341636</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>비에이치아이</t>
+          <t>타이드워터</t>
         </is>
       </c>
       <c r="B38" t="n">
-        <v>8</v>
+        <v>48</v>
       </c>
       <c r="C38" t="inlineStr">
         <is>
@@ -1458,23 +1458,23 @@
         <v>1</v>
       </c>
       <c r="E38" t="n">
-        <v>876000</v>
+        <v>5211036.802851856</v>
       </c>
       <c r="F38" t="n">
-        <v>210885</v>
+        <v>1486491.802851856</v>
       </c>
       <c r="G38" t="n">
-        <v>31.70654698811484</v>
+        <v>39.91069520845783</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>삼성생명</t>
+          <t>텍사스 퍼시픽 랜드</t>
         </is>
       </c>
       <c r="B39" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="C39" t="inlineStr">
         <is>
@@ -1485,23 +1485,23 @@
         <v>1</v>
       </c>
       <c r="E39" t="n">
-        <v>926000</v>
+        <v>1596420.098271191</v>
       </c>
       <c r="F39" t="n">
-        <v>93000</v>
+        <v>18525.09827119112</v>
       </c>
       <c r="G39" t="n">
-        <v>11.16446578631453</v>
+        <v>1.174038720649417</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>삼성화재</t>
+          <t>트랜스오션</t>
         </is>
       </c>
       <c r="B40" t="n">
-        <v>9</v>
+        <v>750</v>
       </c>
       <c r="C40" t="inlineStr">
         <is>
@@ -1512,23 +1512,23 @@
         <v>1</v>
       </c>
       <c r="E40" t="n">
-        <v>4270500</v>
+        <v>7074115.140040115</v>
       </c>
       <c r="F40" t="n">
-        <v>-360500</v>
+        <v>2946881.140040115</v>
       </c>
       <c r="G40" t="n">
-        <v>-7.784495789246384</v>
+        <v>71.40087380652793</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>세아제강</t>
+          <t>페트로브라스 (ADR)</t>
         </is>
       </c>
       <c r="B41" t="n">
-        <v>50</v>
+        <v>480</v>
       </c>
       <c r="C41" t="inlineStr">
         <is>
@@ -1539,13 +1539,13 @@
         <v>1</v>
       </c>
       <c r="E41" t="n">
-        <v>7395000</v>
+        <v>13553578.62304688</v>
       </c>
       <c r="F41" t="n">
-        <v>1085000</v>
+        <v>1447029.623046875</v>
       </c>
       <c r="G41" t="n">
-        <v>17.19492868462758</v>
+        <v>11.95245336261287</v>
       </c>
     </row>
   </sheetData>
@@ -1603,7 +1603,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2026-03-20T15:49:10</t>
+          <t>2026-03-20T15:49:39</t>
         </is>
       </c>
       <c r="E2" t="n">
@@ -5915,14 +5915,14 @@
         <v>13553578.62304688</v>
       </c>
       <c r="G116" t="n">
-        <v>1447029.623046879</v>
+        <v>1447029.623046875</v>
       </c>
       <c r="H116" t="n">
-        <v>11.95245336261291</v>
+        <v>11.95245336261287</v>
       </c>
       <c r="I116" t="inlineStr">
         <is>
-          <t>2026-03-20T15:49:10</t>
+          <t>2026-03-20T15:49:39</t>
         </is>
       </c>
     </row>
@@ -5959,7 +5959,7 @@
       </c>
       <c r="I117" t="inlineStr">
         <is>
-          <t>2026-03-20T15:49:10</t>
+          <t>2026-03-20T15:49:39</t>
         </is>
       </c>
     </row>
@@ -5996,7 +5996,7 @@
       </c>
       <c r="I118" t="inlineStr">
         <is>
-          <t>2026-03-20T15:49:10</t>
+          <t>2026-03-20T15:49:39</t>
         </is>
       </c>
     </row>
@@ -6033,7 +6033,7 @@
       </c>
       <c r="I119" t="inlineStr">
         <is>
-          <t>2026-03-20T15:49:10</t>
+          <t>2026-03-20T15:49:39</t>
         </is>
       </c>
     </row>
@@ -6070,7 +6070,7 @@
       </c>
       <c r="I120" t="inlineStr">
         <is>
-          <t>2026-03-20T15:49:10</t>
+          <t>2026-03-20T15:49:39</t>
         </is>
       </c>
     </row>
@@ -6107,7 +6107,7 @@
       </c>
       <c r="I121" t="inlineStr">
         <is>
-          <t>2026-03-20T15:49:10</t>
+          <t>2026-03-20T15:49:39</t>
         </is>
       </c>
     </row>
@@ -6119,11 +6119,11 @@
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>트랜스오션</t>
+          <t>센트러스 에너지</t>
         </is>
       </c>
       <c r="C122" t="n">
-        <v>750</v>
+        <v>25</v>
       </c>
       <c r="D122" t="inlineStr">
         <is>
@@ -6134,17 +6134,17 @@
         <v>1</v>
       </c>
       <c r="F122" t="n">
-        <v>7074115.140040115</v>
+        <v>7138629.469299316</v>
       </c>
       <c r="G122" t="n">
-        <v>2946881.140040115</v>
+        <v>-294226.5307006836</v>
       </c>
       <c r="H122" t="n">
-        <v>71.40087380652794</v>
+        <v>-3.958458642286136</v>
       </c>
       <c r="I122" t="inlineStr">
         <is>
-          <t>2026-03-20T15:49:10</t>
+          <t>2026-03-20T15:49:39</t>
         </is>
       </c>
     </row>
@@ -6156,11 +6156,11 @@
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>노블</t>
+          <t>트랜스오션</t>
         </is>
       </c>
       <c r="C123" t="n">
-        <v>99</v>
+        <v>750</v>
       </c>
       <c r="D123" t="inlineStr">
         <is>
@@ -6171,17 +6171,17 @@
         <v>1</v>
       </c>
       <c r="F123" t="n">
-        <v>6886743.840087891</v>
+        <v>7074115.140040115</v>
       </c>
       <c r="G123" t="n">
-        <v>2979535.840087891</v>
+        <v>2946881.140040115</v>
       </c>
       <c r="H123" t="n">
-        <v>76.25741552760668</v>
+        <v>71.40087380652793</v>
       </c>
       <c r="I123" t="inlineStr">
         <is>
-          <t>2026-03-20T15:49:10</t>
+          <t>2026-03-20T15:49:39</t>
         </is>
       </c>
     </row>
@@ -6193,11 +6193,11 @@
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>센트러스 에너지</t>
+          <t>노블</t>
         </is>
       </c>
       <c r="C124" t="n">
-        <v>21</v>
+        <v>99</v>
       </c>
       <c r="D124" t="inlineStr">
         <is>
@@ -6208,17 +6208,17 @@
         <v>1</v>
       </c>
       <c r="F124" t="n">
-        <v>5996448.754211426</v>
+        <v>6886743.840087891</v>
       </c>
       <c r="G124" t="n">
-        <v>-234770.2457885733</v>
+        <v>2979535.840087891</v>
       </c>
       <c r="H124" t="n">
-        <v>-3.767645556809564</v>
+        <v>76.25741552760668</v>
       </c>
       <c r="I124" t="inlineStr">
         <is>
-          <t>2026-03-20T15:49:10</t>
+          <t>2026-03-20T15:49:39</t>
         </is>
       </c>
     </row>
@@ -6255,7 +6255,7 @@
       </c>
       <c r="I125" t="inlineStr">
         <is>
-          <t>2026-03-20T15:49:10</t>
+          <t>2026-03-20T15:49:39</t>
         </is>
       </c>
     </row>
@@ -6292,7 +6292,7 @@
       </c>
       <c r="I126" t="inlineStr">
         <is>
-          <t>2026-03-20T15:49:10</t>
+          <t>2026-03-20T15:49:39</t>
         </is>
       </c>
     </row>
@@ -6329,7 +6329,7 @@
       </c>
       <c r="I127" t="inlineStr">
         <is>
-          <t>2026-03-20T15:49:10</t>
+          <t>2026-03-20T15:49:39</t>
         </is>
       </c>
     </row>
@@ -6366,7 +6366,7 @@
       </c>
       <c r="I128" t="inlineStr">
         <is>
-          <t>2026-03-20T15:49:10</t>
+          <t>2026-03-20T15:49:39</t>
         </is>
       </c>
     </row>
@@ -6403,7 +6403,7 @@
       </c>
       <c r="I129" t="inlineStr">
         <is>
-          <t>2026-03-20T15:49:10</t>
+          <t>2026-03-20T15:49:39</t>
         </is>
       </c>
     </row>
@@ -6440,7 +6440,7 @@
       </c>
       <c r="I130" t="inlineStr">
         <is>
-          <t>2026-03-20T15:49:10</t>
+          <t>2026-03-20T15:49:39</t>
         </is>
       </c>
     </row>
@@ -6477,7 +6477,7 @@
       </c>
       <c r="I131" t="inlineStr">
         <is>
-          <t>2026-03-20T15:49:10</t>
+          <t>2026-03-20T15:49:39</t>
         </is>
       </c>
     </row>
@@ -6514,7 +6514,7 @@
       </c>
       <c r="I132" t="inlineStr">
         <is>
-          <t>2026-03-20T15:49:10</t>
+          <t>2026-03-20T15:49:39</t>
         </is>
       </c>
     </row>
@@ -6551,7 +6551,7 @@
       </c>
       <c r="I133" t="inlineStr">
         <is>
-          <t>2026-03-20T15:49:10</t>
+          <t>2026-03-20T15:49:39</t>
         </is>
       </c>
     </row>
@@ -6588,7 +6588,7 @@
       </c>
       <c r="I134" t="inlineStr">
         <is>
-          <t>2026-03-20T15:49:10</t>
+          <t>2026-03-20T15:49:39</t>
         </is>
       </c>
     </row>
@@ -6625,7 +6625,7 @@
       </c>
       <c r="I135" t="inlineStr">
         <is>
-          <t>2026-03-20T15:49:10</t>
+          <t>2026-03-20T15:49:39</t>
         </is>
       </c>
     </row>
@@ -6662,7 +6662,7 @@
       </c>
       <c r="I136" t="inlineStr">
         <is>
-          <t>2026-03-20T15:49:10</t>
+          <t>2026-03-20T15:49:39</t>
         </is>
       </c>
     </row>
@@ -6699,7 +6699,7 @@
       </c>
       <c r="I137" t="inlineStr">
         <is>
-          <t>2026-03-20T15:49:10</t>
+          <t>2026-03-20T15:49:39</t>
         </is>
       </c>
     </row>
@@ -6736,7 +6736,7 @@
       </c>
       <c r="I138" t="inlineStr">
         <is>
-          <t>2026-03-20T15:49:10</t>
+          <t>2026-03-20T15:49:39</t>
         </is>
       </c>
     </row>
@@ -6773,7 +6773,7 @@
       </c>
       <c r="I139" t="inlineStr">
         <is>
-          <t>2026-03-20T15:49:10</t>
+          <t>2026-03-20T15:49:39</t>
         </is>
       </c>
     </row>
@@ -6810,7 +6810,7 @@
       </c>
       <c r="I140" t="inlineStr">
         <is>
-          <t>2026-03-20T15:49:10</t>
+          <t>2026-03-20T15:49:39</t>
         </is>
       </c>
     </row>
@@ -6840,14 +6840,14 @@
         <v>2176561.162089184</v>
       </c>
       <c r="G141" t="n">
-        <v>112571.1620891844</v>
+        <v>112571.1620891839</v>
       </c>
       <c r="H141" t="n">
-        <v>5.45405559567558</v>
+        <v>5.454055595675557</v>
       </c>
       <c r="I141" t="inlineStr">
         <is>
-          <t>2026-03-20T15:49:10</t>
+          <t>2026-03-20T15:49:39</t>
         </is>
       </c>
     </row>
@@ -6884,7 +6884,7 @@
       </c>
       <c r="I142" t="inlineStr">
         <is>
-          <t>2026-03-20T15:49:10</t>
+          <t>2026-03-20T15:49:39</t>
         </is>
       </c>
     </row>
@@ -6921,7 +6921,7 @@
       </c>
       <c r="I143" t="inlineStr">
         <is>
-          <t>2026-03-20T15:49:10</t>
+          <t>2026-03-20T15:49:39</t>
         </is>
       </c>
     </row>
@@ -6958,7 +6958,7 @@
       </c>
       <c r="I144" t="inlineStr">
         <is>
-          <t>2026-03-20T15:49:10</t>
+          <t>2026-03-20T15:49:39</t>
         </is>
       </c>
     </row>
@@ -6995,7 +6995,7 @@
       </c>
       <c r="I145" t="inlineStr">
         <is>
-          <t>2026-03-20T15:49:10</t>
+          <t>2026-03-20T15:49:39</t>
         </is>
       </c>
     </row>
@@ -7025,14 +7025,14 @@
         <v>1696441.320678405</v>
       </c>
       <c r="G146" t="n">
-        <v>382088.3206784062</v>
+        <v>382088.3206784055</v>
       </c>
       <c r="H146" t="n">
-        <v>29.07044916231837</v>
+        <v>29.0704491623183</v>
       </c>
       <c r="I146" t="inlineStr">
         <is>
-          <t>2026-03-20T15:49:10</t>
+          <t>2026-03-20T15:49:39</t>
         </is>
       </c>
     </row>
@@ -7069,7 +7069,7 @@
       </c>
       <c r="I147" t="inlineStr">
         <is>
-          <t>2026-03-20T15:49:10</t>
+          <t>2026-03-20T15:49:39</t>
         </is>
       </c>
     </row>
@@ -7106,7 +7106,7 @@
       </c>
       <c r="I148" t="inlineStr">
         <is>
-          <t>2026-03-20T15:49:10</t>
+          <t>2026-03-20T15:49:39</t>
         </is>
       </c>
     </row>
@@ -7118,11 +7118,11 @@
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>LX인터내셔널</t>
+          <t>텍사스 퍼시픽 랜드</t>
         </is>
       </c>
       <c r="C149" t="n">
-        <v>20</v>
+        <v>2</v>
       </c>
       <c r="D149" t="inlineStr">
         <is>
@@ -7133,17 +7133,17 @@
         <v>1</v>
       </c>
       <c r="F149" t="n">
-        <v>943000</v>
+        <v>1596420.098271191</v>
       </c>
       <c r="G149" t="n">
-        <v>4000</v>
+        <v>18525.09827119112</v>
       </c>
       <c r="H149" t="n">
-        <v>0.4259850905218318</v>
+        <v>1.174038720649417</v>
       </c>
       <c r="I149" t="inlineStr">
         <is>
-          <t>2026-03-20T15:49:10</t>
+          <t>2026-03-20T15:49:39</t>
         </is>
       </c>
     </row>
@@ -7155,11 +7155,11 @@
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>삼성생명</t>
+          <t>LX인터내셔널</t>
         </is>
       </c>
       <c r="C150" t="n">
-        <v>4</v>
+        <v>20</v>
       </c>
       <c r="D150" t="inlineStr">
         <is>
@@ -7170,17 +7170,17 @@
         <v>1</v>
       </c>
       <c r="F150" t="n">
-        <v>926000</v>
+        <v>943000</v>
       </c>
       <c r="G150" t="n">
-        <v>93000</v>
+        <v>4000</v>
       </c>
       <c r="H150" t="n">
-        <v>11.16446578631453</v>
+        <v>0.4259850905218318</v>
       </c>
       <c r="I150" t="inlineStr">
         <is>
-          <t>2026-03-20T15:49:10</t>
+          <t>2026-03-20T15:49:39</t>
         </is>
       </c>
     </row>
@@ -7192,11 +7192,11 @@
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>비에이치아이</t>
+          <t>삼성생명</t>
         </is>
       </c>
       <c r="C151" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="D151" t="inlineStr">
         <is>
@@ -7207,17 +7207,17 @@
         <v>1</v>
       </c>
       <c r="F151" t="n">
-        <v>876000</v>
+        <v>926000</v>
       </c>
       <c r="G151" t="n">
-        <v>210885</v>
+        <v>93000</v>
       </c>
       <c r="H151" t="n">
-        <v>31.70654698811484</v>
+        <v>11.16446578631453</v>
       </c>
       <c r="I151" t="inlineStr">
         <is>
-          <t>2026-03-20T15:49:10</t>
+          <t>2026-03-20T15:49:39</t>
         </is>
       </c>
     </row>
@@ -7229,11 +7229,11 @@
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>하프니아</t>
+          <t>비에이치아이</t>
         </is>
       </c>
       <c r="C152" t="n">
-        <v>80</v>
+        <v>8</v>
       </c>
       <c r="D152" t="inlineStr">
         <is>
@@ -7244,17 +7244,17 @@
         <v>1</v>
       </c>
       <c r="F152" t="n">
-        <v>848519.8631833494</v>
+        <v>876000</v>
       </c>
       <c r="G152" t="n">
-        <v>222788.8631833494</v>
+        <v>210885</v>
       </c>
       <c r="H152" t="n">
-        <v>35.60457499841775</v>
+        <v>31.70654698811484</v>
       </c>
       <c r="I152" t="inlineStr">
         <is>
-          <t>2026-03-20T15:49:10</t>
+          <t>2026-03-20T15:49:39</t>
         </is>
       </c>
     </row>
@@ -7266,11 +7266,11 @@
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>클리블랜드 클리프스</t>
+          <t>하프니아</t>
         </is>
       </c>
       <c r="C153" t="n">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="D153" t="inlineStr">
         <is>
@@ -7281,17 +7281,17 @@
         <v>1</v>
       </c>
       <c r="F153" t="n">
-        <v>833036.4441346284</v>
+        <v>848519.8631833494</v>
       </c>
       <c r="G153" t="n">
-        <v>-183018.5558653716</v>
+        <v>222788.8631833494</v>
       </c>
       <c r="H153" t="n">
-        <v>-18.01266229341636</v>
+        <v>35.60457499841775</v>
       </c>
       <c r="I153" t="inlineStr">
         <is>
-          <t>2026-03-20T15:49:10</t>
+          <t>2026-03-20T15:49:39</t>
         </is>
       </c>
     </row>
@@ -7303,11 +7303,11 @@
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>텍사스 퍼시픽 랜드</t>
+          <t>클리블랜드 클리프스</t>
         </is>
       </c>
       <c r="C154" t="n">
-        <v>1</v>
+        <v>70</v>
       </c>
       <c r="D154" t="inlineStr">
         <is>
@@ -7318,17 +7318,17 @@
         <v>1</v>
       </c>
       <c r="F154" t="n">
-        <v>798210.0491355956</v>
+        <v>833036.4441346284</v>
       </c>
       <c r="G154" t="n">
-        <v>19619.04913559556</v>
+        <v>-183018.5558653716</v>
       </c>
       <c r="H154" t="n">
-        <v>2.519814528500273</v>
+        <v>-18.01266229341636</v>
       </c>
       <c r="I154" t="inlineStr">
         <is>
-          <t>2026-03-20T15:49:10</t>
+          <t>2026-03-20T15:49:39</t>
         </is>
       </c>
     </row>
@@ -7365,7 +7365,7 @@
       </c>
       <c r="I155" t="inlineStr">
         <is>
-          <t>2026-03-20T15:49:10</t>
+          <t>2026-03-20T15:49:39</t>
         </is>
       </c>
     </row>
@@ -7498,7 +7498,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>2026-03-20T15:49:10</t>
+          <t>2026-03-20T15:49:39</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: portfolio snapshot 2026-03-20 (2026-03-20T15:49:41)
</commit_message>
<xml_diff>
--- a/portfolio_auto.xlsx
+++ b/portfolio_auto.xlsx
@@ -1603,7 +1603,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2026-03-20T15:49:39</t>
+          <t>2026-03-20T15:49:40</t>
         </is>
       </c>
       <c r="E2" t="n">
@@ -5922,7 +5922,7 @@
       </c>
       <c r="I116" t="inlineStr">
         <is>
-          <t>2026-03-20T15:49:39</t>
+          <t>2026-03-20T15:49:40</t>
         </is>
       </c>
     </row>
@@ -5959,7 +5959,7 @@
       </c>
       <c r="I117" t="inlineStr">
         <is>
-          <t>2026-03-20T15:49:39</t>
+          <t>2026-03-20T15:49:40</t>
         </is>
       </c>
     </row>
@@ -5996,7 +5996,7 @@
       </c>
       <c r="I118" t="inlineStr">
         <is>
-          <t>2026-03-20T15:49:39</t>
+          <t>2026-03-20T15:49:40</t>
         </is>
       </c>
     </row>
@@ -6033,7 +6033,7 @@
       </c>
       <c r="I119" t="inlineStr">
         <is>
-          <t>2026-03-20T15:49:39</t>
+          <t>2026-03-20T15:49:40</t>
         </is>
       </c>
     </row>
@@ -6070,7 +6070,7 @@
       </c>
       <c r="I120" t="inlineStr">
         <is>
-          <t>2026-03-20T15:49:39</t>
+          <t>2026-03-20T15:49:40</t>
         </is>
       </c>
     </row>
@@ -6107,7 +6107,7 @@
       </c>
       <c r="I121" t="inlineStr">
         <is>
-          <t>2026-03-20T15:49:39</t>
+          <t>2026-03-20T15:49:40</t>
         </is>
       </c>
     </row>
@@ -6144,7 +6144,7 @@
       </c>
       <c r="I122" t="inlineStr">
         <is>
-          <t>2026-03-20T15:49:39</t>
+          <t>2026-03-20T15:49:40</t>
         </is>
       </c>
     </row>
@@ -6181,7 +6181,7 @@
       </c>
       <c r="I123" t="inlineStr">
         <is>
-          <t>2026-03-20T15:49:39</t>
+          <t>2026-03-20T15:49:40</t>
         </is>
       </c>
     </row>
@@ -6218,7 +6218,7 @@
       </c>
       <c r="I124" t="inlineStr">
         <is>
-          <t>2026-03-20T15:49:39</t>
+          <t>2026-03-20T15:49:40</t>
         </is>
       </c>
     </row>
@@ -6255,7 +6255,7 @@
       </c>
       <c r="I125" t="inlineStr">
         <is>
-          <t>2026-03-20T15:49:39</t>
+          <t>2026-03-20T15:49:40</t>
         </is>
       </c>
     </row>
@@ -6292,7 +6292,7 @@
       </c>
       <c r="I126" t="inlineStr">
         <is>
-          <t>2026-03-20T15:49:39</t>
+          <t>2026-03-20T15:49:40</t>
         </is>
       </c>
     </row>
@@ -6329,7 +6329,7 @@
       </c>
       <c r="I127" t="inlineStr">
         <is>
-          <t>2026-03-20T15:49:39</t>
+          <t>2026-03-20T15:49:40</t>
         </is>
       </c>
     </row>
@@ -6366,7 +6366,7 @@
       </c>
       <c r="I128" t="inlineStr">
         <is>
-          <t>2026-03-20T15:49:39</t>
+          <t>2026-03-20T15:49:40</t>
         </is>
       </c>
     </row>
@@ -6403,7 +6403,7 @@
       </c>
       <c r="I129" t="inlineStr">
         <is>
-          <t>2026-03-20T15:49:39</t>
+          <t>2026-03-20T15:49:40</t>
         </is>
       </c>
     </row>
@@ -6440,7 +6440,7 @@
       </c>
       <c r="I130" t="inlineStr">
         <is>
-          <t>2026-03-20T15:49:39</t>
+          <t>2026-03-20T15:49:40</t>
         </is>
       </c>
     </row>
@@ -6477,7 +6477,7 @@
       </c>
       <c r="I131" t="inlineStr">
         <is>
-          <t>2026-03-20T15:49:39</t>
+          <t>2026-03-20T15:49:40</t>
         </is>
       </c>
     </row>
@@ -6514,7 +6514,7 @@
       </c>
       <c r="I132" t="inlineStr">
         <is>
-          <t>2026-03-20T15:49:39</t>
+          <t>2026-03-20T15:49:40</t>
         </is>
       </c>
     </row>
@@ -6551,7 +6551,7 @@
       </c>
       <c r="I133" t="inlineStr">
         <is>
-          <t>2026-03-20T15:49:39</t>
+          <t>2026-03-20T15:49:40</t>
         </is>
       </c>
     </row>
@@ -6588,7 +6588,7 @@
       </c>
       <c r="I134" t="inlineStr">
         <is>
-          <t>2026-03-20T15:49:39</t>
+          <t>2026-03-20T15:49:40</t>
         </is>
       </c>
     </row>
@@ -6625,7 +6625,7 @@
       </c>
       <c r="I135" t="inlineStr">
         <is>
-          <t>2026-03-20T15:49:39</t>
+          <t>2026-03-20T15:49:40</t>
         </is>
       </c>
     </row>
@@ -6662,7 +6662,7 @@
       </c>
       <c r="I136" t="inlineStr">
         <is>
-          <t>2026-03-20T15:49:39</t>
+          <t>2026-03-20T15:49:40</t>
         </is>
       </c>
     </row>
@@ -6699,7 +6699,7 @@
       </c>
       <c r="I137" t="inlineStr">
         <is>
-          <t>2026-03-20T15:49:39</t>
+          <t>2026-03-20T15:49:40</t>
         </is>
       </c>
     </row>
@@ -6736,7 +6736,7 @@
       </c>
       <c r="I138" t="inlineStr">
         <is>
-          <t>2026-03-20T15:49:39</t>
+          <t>2026-03-20T15:49:40</t>
         </is>
       </c>
     </row>
@@ -6773,7 +6773,7 @@
       </c>
       <c r="I139" t="inlineStr">
         <is>
-          <t>2026-03-20T15:49:39</t>
+          <t>2026-03-20T15:49:40</t>
         </is>
       </c>
     </row>
@@ -6810,7 +6810,7 @@
       </c>
       <c r="I140" t="inlineStr">
         <is>
-          <t>2026-03-20T15:49:39</t>
+          <t>2026-03-20T15:49:40</t>
         </is>
       </c>
     </row>
@@ -6847,7 +6847,7 @@
       </c>
       <c r="I141" t="inlineStr">
         <is>
-          <t>2026-03-20T15:49:39</t>
+          <t>2026-03-20T15:49:40</t>
         </is>
       </c>
     </row>
@@ -6884,7 +6884,7 @@
       </c>
       <c r="I142" t="inlineStr">
         <is>
-          <t>2026-03-20T15:49:39</t>
+          <t>2026-03-20T15:49:40</t>
         </is>
       </c>
     </row>
@@ -6921,7 +6921,7 @@
       </c>
       <c r="I143" t="inlineStr">
         <is>
-          <t>2026-03-20T15:49:39</t>
+          <t>2026-03-20T15:49:40</t>
         </is>
       </c>
     </row>
@@ -6958,7 +6958,7 @@
       </c>
       <c r="I144" t="inlineStr">
         <is>
-          <t>2026-03-20T15:49:39</t>
+          <t>2026-03-20T15:49:40</t>
         </is>
       </c>
     </row>
@@ -6995,7 +6995,7 @@
       </c>
       <c r="I145" t="inlineStr">
         <is>
-          <t>2026-03-20T15:49:39</t>
+          <t>2026-03-20T15:49:40</t>
         </is>
       </c>
     </row>
@@ -7032,7 +7032,7 @@
       </c>
       <c r="I146" t="inlineStr">
         <is>
-          <t>2026-03-20T15:49:39</t>
+          <t>2026-03-20T15:49:40</t>
         </is>
       </c>
     </row>
@@ -7069,7 +7069,7 @@
       </c>
       <c r="I147" t="inlineStr">
         <is>
-          <t>2026-03-20T15:49:39</t>
+          <t>2026-03-20T15:49:40</t>
         </is>
       </c>
     </row>
@@ -7106,7 +7106,7 @@
       </c>
       <c r="I148" t="inlineStr">
         <is>
-          <t>2026-03-20T15:49:39</t>
+          <t>2026-03-20T15:49:40</t>
         </is>
       </c>
     </row>
@@ -7143,7 +7143,7 @@
       </c>
       <c r="I149" t="inlineStr">
         <is>
-          <t>2026-03-20T15:49:39</t>
+          <t>2026-03-20T15:49:40</t>
         </is>
       </c>
     </row>
@@ -7180,7 +7180,7 @@
       </c>
       <c r="I150" t="inlineStr">
         <is>
-          <t>2026-03-20T15:49:39</t>
+          <t>2026-03-20T15:49:40</t>
         </is>
       </c>
     </row>
@@ -7217,7 +7217,7 @@
       </c>
       <c r="I151" t="inlineStr">
         <is>
-          <t>2026-03-20T15:49:39</t>
+          <t>2026-03-20T15:49:40</t>
         </is>
       </c>
     </row>
@@ -7254,7 +7254,7 @@
       </c>
       <c r="I152" t="inlineStr">
         <is>
-          <t>2026-03-20T15:49:39</t>
+          <t>2026-03-20T15:49:40</t>
         </is>
       </c>
     </row>
@@ -7291,7 +7291,7 @@
       </c>
       <c r="I153" t="inlineStr">
         <is>
-          <t>2026-03-20T15:49:39</t>
+          <t>2026-03-20T15:49:40</t>
         </is>
       </c>
     </row>
@@ -7328,7 +7328,7 @@
       </c>
       <c r="I154" t="inlineStr">
         <is>
-          <t>2026-03-20T15:49:39</t>
+          <t>2026-03-20T15:49:40</t>
         </is>
       </c>
     </row>
@@ -7365,7 +7365,7 @@
       </c>
       <c r="I155" t="inlineStr">
         <is>
-          <t>2026-03-20T15:49:39</t>
+          <t>2026-03-20T15:49:40</t>
         </is>
       </c>
     </row>
@@ -7498,7 +7498,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>2026-03-20T15:49:39</t>
+          <t>2026-03-20T15:49:40</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: portfolio snapshot 2026-03-20 (2026-03-20T15:49:57)
</commit_message>
<xml_diff>
--- a/portfolio_auto.xlsx
+++ b/portfolio_auto.xlsx
@@ -471,11 +471,11 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>유나이티드헬스 그룹</t>
+          <t>페트로브라스 (ADR)</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>4</v>
+        <v>480</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
@@ -486,23 +486,23 @@
         <v>1</v>
       </c>
       <c r="E2" t="n">
-        <v>1683366.447431445</v>
+        <v>13553578.62304688</v>
       </c>
       <c r="F2" t="n">
-        <v>-11089.55256855441</v>
+        <v>1447029.623046875</v>
       </c>
       <c r="G2" t="n">
-        <v>-0.6544609342794628</v>
+        <v>11.95245336261287</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>케이씨</t>
+          <t>AGNC 인베스트먼트</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>50</v>
+        <v>700</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
@@ -513,23 +513,23 @@
         <v>1</v>
       </c>
       <c r="E3" t="n">
-        <v>1670000</v>
+        <v>10351433.71453537</v>
       </c>
       <c r="F3" t="n">
-        <v>20500</v>
+        <v>-480580.2854646333</v>
       </c>
       <c r="G3" t="n">
-        <v>1.242800848742043</v>
+        <v>-4.43666602964724</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>하나금융지주</t>
+          <t>대한조선</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>18</v>
+        <v>100</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
@@ -540,23 +540,23 @@
         <v>1</v>
       </c>
       <c r="E4" t="n">
-        <v>2037600</v>
+        <v>9120000</v>
       </c>
       <c r="F4" t="n">
-        <v>12200</v>
+        <v>1907000</v>
       </c>
       <c r="G4" t="n">
-        <v>0.6023501530561864</v>
+        <v>26.43837515596839</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>현대제철</t>
+          <t>프론트라인</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>80</v>
+        <v>175</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -567,23 +567,23 @@
         <v>1</v>
       </c>
       <c r="E5" t="n">
-        <v>2996000</v>
+        <v>8453409.11431564</v>
       </c>
       <c r="F5" t="n">
-        <v>-182000</v>
+        <v>4023545.11431564</v>
       </c>
       <c r="G5" t="n">
-        <v>-5.726872246696035</v>
+        <v>90.82773453802736</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>휴스틸</t>
+          <t>시드릴</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>500</v>
+        <v>123</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
@@ -594,23 +594,23 @@
         <v>1</v>
       </c>
       <c r="E6" t="n">
-        <v>2750000</v>
+        <v>8081063.113214018</v>
       </c>
       <c r="F6" t="n">
-        <v>471390</v>
+        <v>1630712.113214018</v>
       </c>
       <c r="G6" t="n">
-        <v>20.68761218462133</v>
+        <v>25.28098258860669</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>DL이앤씨</t>
+          <t>세아제강</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>40</v>
+        <v>50</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -621,23 +621,23 @@
         <v>1</v>
       </c>
       <c r="E7" t="n">
-        <v>2696000</v>
+        <v>7395000</v>
       </c>
       <c r="F7" t="n">
-        <v>990500</v>
+        <v>1085000</v>
       </c>
       <c r="G7" t="n">
-        <v>58.07681031955438</v>
+        <v>17.19492868462758</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>HD건설기계</t>
+          <t>센트러스 에너지</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>31</v>
+        <v>25</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
@@ -648,23 +648,23 @@
         <v>1</v>
       </c>
       <c r="E8" t="n">
-        <v>4123000</v>
+        <v>7138629.469299316</v>
       </c>
       <c r="F8" t="n">
-        <v>87904</v>
+        <v>-294226.5307006836</v>
       </c>
       <c r="G8" t="n">
-        <v>2.178485964150543</v>
+        <v>-3.958458642286136</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>KoAct 코스닥액티브</t>
+          <t>트랜스오션</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>200</v>
+        <v>750</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
@@ -675,23 +675,23 @@
         <v>1</v>
       </c>
       <c r="E9" t="n">
-        <v>2582000</v>
+        <v>7074115.140040115</v>
       </c>
       <c r="F9" t="n">
-        <v>-120000</v>
+        <v>2946881.140040115</v>
       </c>
       <c r="G9" t="n">
-        <v>-4.441154700222058</v>
+        <v>71.40087380652793</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>LX인터내셔널</t>
+          <t>노블</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>20</v>
+        <v>99</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
@@ -702,23 +702,23 @@
         <v>1</v>
       </c>
       <c r="E10" t="n">
-        <v>943000</v>
+        <v>6886743.840087891</v>
       </c>
       <c r="F10" t="n">
-        <v>4000</v>
+        <v>2979535.840087891</v>
       </c>
       <c r="G10" t="n">
-        <v>0.4259850905218318</v>
+        <v>76.25741552760668</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>NH투자증권우</t>
+          <t>타이드워터</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>2</v>
+        <v>48</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
@@ -729,23 +729,23 @@
         <v>1</v>
       </c>
       <c r="E11" t="n">
-        <v>54591</v>
+        <v>5211036.802851856</v>
       </c>
       <c r="F11" t="n">
-        <v>-9</v>
+        <v>1486491.802851856</v>
       </c>
       <c r="G11" t="n">
-        <v>-0.01648351648351648</v>
+        <v>39.91069520845783</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>TIME 코리아밸류업액티브</t>
+          <t>노브</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>201</v>
+        <v>185</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
@@ -756,23 +756,23 @@
         <v>1</v>
       </c>
       <c r="E12" t="n">
-        <v>4797870</v>
+        <v>5179494.129107101</v>
       </c>
       <c r="F12" t="n">
-        <v>74073</v>
+        <v>1869486.129107101</v>
       </c>
       <c r="G12" t="n">
-        <v>1.568081778281328</v>
+        <v>56.47980697046958</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>프론트라인</t>
+          <t>TIME 코리아밸류업액티브</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>175</v>
+        <v>201</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
@@ -783,19 +783,19 @@
         <v>1</v>
       </c>
       <c r="E13" t="n">
-        <v>8453409.11431564</v>
+        <v>4797870</v>
       </c>
       <c r="F13" t="n">
-        <v>4023545.11431564</v>
+        <v>74073</v>
       </c>
       <c r="G13" t="n">
-        <v>90.82773453802736</v>
+        <v>1.568081778281328</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>피바디 에너지</t>
+          <t>오케아니스 에코 탱커스</t>
         </is>
       </c>
       <c r="B14" t="n">
@@ -810,23 +810,23 @@
         <v>1</v>
       </c>
       <c r="E14" t="n">
-        <v>3596373.331896178</v>
+        <v>4596307.895957222</v>
       </c>
       <c r="F14" t="n">
-        <v>2125601.331896178</v>
+        <v>2339947.895957222</v>
       </c>
       <c r="G14" t="n">
-        <v>144.5228309959789</v>
+        <v>103.704546081176</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>하프니아</t>
+          <t>삼성화재</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>80</v>
+        <v>9</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
@@ -837,23 +837,23 @@
         <v>1</v>
       </c>
       <c r="E15" t="n">
-        <v>848519.8631833494</v>
+        <v>4270500</v>
       </c>
       <c r="F15" t="n">
-        <v>222788.8631833494</v>
+        <v>-360500</v>
       </c>
       <c r="G15" t="n">
-        <v>35.60457499841775</v>
+        <v>-7.784495789246384</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>AGNC 인베스트먼트</t>
+          <t>동원개발</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>700</v>
+        <v>1360</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
@@ -864,23 +864,23 @@
         <v>1</v>
       </c>
       <c r="E16" t="n">
-        <v>10351433.71453537</v>
+        <v>4202400</v>
       </c>
       <c r="F16" t="n">
-        <v>-480580.2854646333</v>
+        <v>465000</v>
       </c>
       <c r="G16" t="n">
-        <v>-4.43666602964724</v>
+        <v>12.44180446299566</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>넥스틸</t>
+          <t>HD건설기계</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>300</v>
+        <v>31</v>
       </c>
       <c r="C17" t="inlineStr">
         <is>
@@ -891,23 +891,23 @@
         <v>1</v>
       </c>
       <c r="E17" t="n">
-        <v>3771000</v>
+        <v>4123000</v>
       </c>
       <c r="F17" t="n">
-        <v>521000</v>
+        <v>87904</v>
       </c>
       <c r="G17" t="n">
-        <v>16.03076923076923</v>
+        <v>2.178485964150543</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>대신증권</t>
+          <t>차코스 에너지 내비게이션</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>55</v>
+        <v>75</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
@@ -918,19 +918,19 @@
         <v>1</v>
       </c>
       <c r="E18" t="n">
-        <v>2219250</v>
+        <v>4052048.962918622</v>
       </c>
       <c r="F18" t="n">
-        <v>509749</v>
+        <v>227400.9629186224</v>
       </c>
       <c r="G18" t="n">
-        <v>29.81858448752005</v>
+        <v>5.94567037067522</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>대창단조</t>
+          <t>넥스틸</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -945,23 +945,23 @@
         <v>1</v>
       </c>
       <c r="E19" t="n">
-        <v>2004000</v>
+        <v>3771000</v>
       </c>
       <c r="F19" t="n">
-        <v>-54000</v>
+        <v>521000</v>
       </c>
       <c r="G19" t="n">
-        <v>-2.623906705539359</v>
+        <v>16.03076923076923</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>대한조선</t>
+          <t>피바디 에너지</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>100</v>
+        <v>65</v>
       </c>
       <c r="C20" t="inlineStr">
         <is>
@@ -972,23 +972,23 @@
         <v>1</v>
       </c>
       <c r="E20" t="n">
-        <v>9120000</v>
+        <v>3596373.331896178</v>
       </c>
       <c r="F20" t="n">
-        <v>1907000</v>
+        <v>2125601.331896178</v>
       </c>
       <c r="G20" t="n">
-        <v>26.43837515596839</v>
+        <v>144.5228309959789</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>동방</t>
+          <t>현대제철</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>681</v>
+        <v>80</v>
       </c>
       <c r="C21" t="inlineStr">
         <is>
@@ -999,23 +999,23 @@
         <v>1</v>
       </c>
       <c r="E21" t="n">
-        <v>1995330</v>
+        <v>2996000</v>
       </c>
       <c r="F21" t="n">
-        <v>23829</v>
+        <v>-182000</v>
       </c>
       <c r="G21" t="n">
-        <v>1.208672985709873</v>
+        <v>-5.726872246696035</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>동원개발</t>
+          <t>더치 브로스</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>1360</v>
+        <v>39</v>
       </c>
       <c r="C22" t="inlineStr">
         <is>
@@ -1026,23 +1026,23 @@
         <v>1</v>
       </c>
       <c r="E22" t="n">
-        <v>4202400</v>
+        <v>2959763.281021703</v>
       </c>
       <c r="F22" t="n">
-        <v>465000</v>
+        <v>-230880.718978297</v>
       </c>
       <c r="G22" t="n">
-        <v>12.44180446299566</v>
+        <v>-7.236179247145621</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>미창석유</t>
+          <t>휴스틸</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>18</v>
+        <v>500</v>
       </c>
       <c r="C23" t="inlineStr">
         <is>
@@ -1053,23 +1053,23 @@
         <v>1</v>
       </c>
       <c r="E23" t="n">
-        <v>2097000</v>
+        <v>2750000</v>
       </c>
       <c r="F23" t="n">
-        <v>-295200</v>
+        <v>471390</v>
       </c>
       <c r="G23" t="n">
-        <v>-12.34010534236268</v>
+        <v>20.68761218462133</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>비에이치아이</t>
+          <t>DL이앤씨</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>8</v>
+        <v>40</v>
       </c>
       <c r="C24" t="inlineStr">
         <is>
@@ -1080,23 +1080,23 @@
         <v>1</v>
       </c>
       <c r="E24" t="n">
-        <v>876000</v>
+        <v>2696000</v>
       </c>
       <c r="F24" t="n">
-        <v>210885</v>
+        <v>990500</v>
       </c>
       <c r="G24" t="n">
-        <v>31.70654698811484</v>
+        <v>58.07681031955438</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>삼성생명</t>
+          <t>KoAct 코스닥액티브</t>
         </is>
       </c>
       <c r="B25" t="n">
-        <v>4</v>
+        <v>200</v>
       </c>
       <c r="C25" t="inlineStr">
         <is>
@@ -1107,23 +1107,23 @@
         <v>1</v>
       </c>
       <c r="E25" t="n">
-        <v>926000</v>
+        <v>2582000</v>
       </c>
       <c r="F25" t="n">
-        <v>93000</v>
+        <v>-120000</v>
       </c>
       <c r="G25" t="n">
-        <v>11.16446578631453</v>
+        <v>-4.441154700222058</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>삼성화재</t>
+          <t>대신증권</t>
         </is>
       </c>
       <c r="B26" t="n">
-        <v>9</v>
+        <v>55</v>
       </c>
       <c r="C26" t="inlineStr">
         <is>
@@ -1134,23 +1134,23 @@
         <v>1</v>
       </c>
       <c r="E26" t="n">
-        <v>4270500</v>
+        <v>2219250</v>
       </c>
       <c r="F26" t="n">
-        <v>-360500</v>
+        <v>509749</v>
       </c>
       <c r="G26" t="n">
-        <v>-7.784495789246384</v>
+        <v>29.81858448752005</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>세아제강</t>
+          <t>발레로 에너지</t>
         </is>
       </c>
       <c r="B27" t="n">
-        <v>50</v>
+        <v>6</v>
       </c>
       <c r="C27" t="inlineStr">
         <is>
@@ -1161,23 +1161,23 @@
         <v>1</v>
       </c>
       <c r="E27" t="n">
-        <v>7395000</v>
+        <v>2176561.162089184</v>
       </c>
       <c r="F27" t="n">
-        <v>1085000</v>
+        <v>112571.1620891839</v>
       </c>
       <c r="G27" t="n">
-        <v>17.19492868462758</v>
+        <v>5.454055595675557</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>노브</t>
+          <t>미창석유</t>
         </is>
       </c>
       <c r="B28" t="n">
-        <v>185</v>
+        <v>18</v>
       </c>
       <c r="C28" t="inlineStr">
         <is>
@@ -1188,23 +1188,23 @@
         <v>1</v>
       </c>
       <c r="E28" t="n">
-        <v>5179494.129107101</v>
+        <v>2097000</v>
       </c>
       <c r="F28" t="n">
-        <v>1869486.129107101</v>
+        <v>-295200</v>
       </c>
       <c r="G28" t="n">
-        <v>56.47980697046958</v>
+        <v>-12.34010534236268</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>노블</t>
+          <t>하나금융지주</t>
         </is>
       </c>
       <c r="B29" t="n">
-        <v>99</v>
+        <v>18</v>
       </c>
       <c r="C29" t="inlineStr">
         <is>
@@ -1215,23 +1215,23 @@
         <v>1</v>
       </c>
       <c r="E29" t="n">
-        <v>6886743.840087891</v>
+        <v>2037600</v>
       </c>
       <c r="F29" t="n">
-        <v>2979535.840087891</v>
+        <v>12200</v>
       </c>
       <c r="G29" t="n">
-        <v>76.25741552760668</v>
+        <v>0.6023501530561864</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>더치 브로스</t>
+          <t>대창단조</t>
         </is>
       </c>
       <c r="B30" t="n">
-        <v>39</v>
+        <v>300</v>
       </c>
       <c r="C30" t="inlineStr">
         <is>
@@ -1242,23 +1242,23 @@
         <v>1</v>
       </c>
       <c r="E30" t="n">
-        <v>2959763.281021703</v>
+        <v>2004000</v>
       </c>
       <c r="F30" t="n">
-        <v>-230880.718978297</v>
+        <v>-54000</v>
       </c>
       <c r="G30" t="n">
-        <v>-7.236179247145621</v>
+        <v>-2.623906705539359</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>발레로 에너지</t>
+          <t>동방</t>
         </is>
       </c>
       <c r="B31" t="n">
-        <v>6</v>
+        <v>681</v>
       </c>
       <c r="C31" t="inlineStr">
         <is>
@@ -1269,23 +1269,23 @@
         <v>1</v>
       </c>
       <c r="E31" t="n">
-        <v>2176561.162089184</v>
+        <v>1995330</v>
       </c>
       <c r="F31" t="n">
-        <v>112571.1620891839</v>
+        <v>23829</v>
       </c>
       <c r="G31" t="n">
-        <v>5.454055595675557</v>
+        <v>1.208672985709873</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>센트러스 에너지</t>
+          <t>스타 벌크 캐리어스</t>
         </is>
       </c>
       <c r="B32" t="n">
-        <v>25</v>
+        <v>50</v>
       </c>
       <c r="C32" t="inlineStr">
         <is>
@@ -1296,23 +1296,23 @@
         <v>1</v>
       </c>
       <c r="E32" t="n">
-        <v>7138629.469299316</v>
+        <v>1696441.320678405</v>
       </c>
       <c r="F32" t="n">
-        <v>-294226.5307006836</v>
+        <v>382088.3206784055</v>
       </c>
       <c r="G32" t="n">
-        <v>-3.958458642286136</v>
+        <v>29.0704491623183</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>스타 벌크 캐리어스</t>
+          <t>유나이티드헬스 그룹</t>
         </is>
       </c>
       <c r="B33" t="n">
-        <v>50</v>
+        <v>4</v>
       </c>
       <c r="C33" t="inlineStr">
         <is>
@@ -1323,23 +1323,23 @@
         <v>1</v>
       </c>
       <c r="E33" t="n">
-        <v>1696441.320678405</v>
+        <v>1683366.447431445</v>
       </c>
       <c r="F33" t="n">
-        <v>382088.3206784055</v>
+        <v>-11089.55256855441</v>
       </c>
       <c r="G33" t="n">
-        <v>29.0704491623183</v>
+        <v>-0.6544609342794628</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>시드릴</t>
+          <t>케이씨</t>
         </is>
       </c>
       <c r="B34" t="n">
-        <v>123</v>
+        <v>50</v>
       </c>
       <c r="C34" t="inlineStr">
         <is>
@@ -1350,23 +1350,23 @@
         <v>1</v>
       </c>
       <c r="E34" t="n">
-        <v>8081063.113214018</v>
+        <v>1670000</v>
       </c>
       <c r="F34" t="n">
-        <v>1630712.113214018</v>
+        <v>20500</v>
       </c>
       <c r="G34" t="n">
-        <v>25.28098258860669</v>
+        <v>1.242800848742043</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>오케아니스 에코 탱커스</t>
+          <t>텍사스 퍼시픽 랜드</t>
         </is>
       </c>
       <c r="B35" t="n">
-        <v>65</v>
+        <v>2</v>
       </c>
       <c r="C35" t="inlineStr">
         <is>
@@ -1377,23 +1377,23 @@
         <v>1</v>
       </c>
       <c r="E35" t="n">
-        <v>4596307.895957222</v>
+        <v>1596420.098271191</v>
       </c>
       <c r="F35" t="n">
-        <v>2339947.895957222</v>
+        <v>18525.09827119112</v>
       </c>
       <c r="G35" t="n">
-        <v>103.704546081176</v>
+        <v>1.174038720649417</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>차코스 에너지 내비게이션</t>
+          <t>LX인터내셔널</t>
         </is>
       </c>
       <c r="B36" t="n">
-        <v>75</v>
+        <v>20</v>
       </c>
       <c r="C36" t="inlineStr">
         <is>
@@ -1404,23 +1404,23 @@
         <v>1</v>
       </c>
       <c r="E36" t="n">
-        <v>4052048.962918622</v>
+        <v>943000</v>
       </c>
       <c r="F36" t="n">
-        <v>227400.9629186224</v>
+        <v>4000</v>
       </c>
       <c r="G36" t="n">
-        <v>5.94567037067522</v>
+        <v>0.4259850905218318</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>클리블랜드 클리프스</t>
+          <t>삼성생명</t>
         </is>
       </c>
       <c r="B37" t="n">
-        <v>70</v>
+        <v>4</v>
       </c>
       <c r="C37" t="inlineStr">
         <is>
@@ -1431,23 +1431,23 @@
         <v>1</v>
       </c>
       <c r="E37" t="n">
-        <v>833036.4441346284</v>
+        <v>926000</v>
       </c>
       <c r="F37" t="n">
-        <v>-183018.5558653716</v>
+        <v>93000</v>
       </c>
       <c r="G37" t="n">
-        <v>-18.01266229341636</v>
+        <v>11.16446578631453</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>타이드워터</t>
+          <t>비에이치아이</t>
         </is>
       </c>
       <c r="B38" t="n">
-        <v>48</v>
+        <v>8</v>
       </c>
       <c r="C38" t="inlineStr">
         <is>
@@ -1458,23 +1458,23 @@
         <v>1</v>
       </c>
       <c r="E38" t="n">
-        <v>5211036.802851856</v>
+        <v>876000</v>
       </c>
       <c r="F38" t="n">
-        <v>1486491.802851856</v>
+        <v>210885</v>
       </c>
       <c r="G38" t="n">
-        <v>39.91069520845783</v>
+        <v>31.70654698811484</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>텍사스 퍼시픽 랜드</t>
+          <t>하프니아</t>
         </is>
       </c>
       <c r="B39" t="n">
-        <v>2</v>
+        <v>80</v>
       </c>
       <c r="C39" t="inlineStr">
         <is>
@@ -1485,23 +1485,23 @@
         <v>1</v>
       </c>
       <c r="E39" t="n">
-        <v>1596420.098271191</v>
+        <v>848519.8631833494</v>
       </c>
       <c r="F39" t="n">
-        <v>18525.09827119112</v>
+        <v>222788.8631833494</v>
       </c>
       <c r="G39" t="n">
-        <v>1.174038720649417</v>
+        <v>35.60457499841775</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>트랜스오션</t>
+          <t>클리블랜드 클리프스</t>
         </is>
       </c>
       <c r="B40" t="n">
-        <v>750</v>
+        <v>70</v>
       </c>
       <c r="C40" t="inlineStr">
         <is>
@@ -1512,23 +1512,23 @@
         <v>1</v>
       </c>
       <c r="E40" t="n">
-        <v>7074115.140040115</v>
+        <v>833036.4441346284</v>
       </c>
       <c r="F40" t="n">
-        <v>2946881.140040115</v>
+        <v>-183018.5558653716</v>
       </c>
       <c r="G40" t="n">
-        <v>71.40087380652793</v>
+        <v>-18.01266229341636</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>페트로브라스 (ADR)</t>
+          <t>NH투자증권우</t>
         </is>
       </c>
       <c r="B41" t="n">
-        <v>480</v>
+        <v>2</v>
       </c>
       <c r="C41" t="inlineStr">
         <is>
@@ -1539,13 +1539,13 @@
         <v>1</v>
       </c>
       <c r="E41" t="n">
-        <v>13553578.62304688</v>
+        <v>54591</v>
       </c>
       <c r="F41" t="n">
-        <v>1447029.623046875</v>
+        <v>-9</v>
       </c>
       <c r="G41" t="n">
-        <v>11.95245336261287</v>
+        <v>-0.01648351648351648</v>
       </c>
     </row>
   </sheetData>
@@ -1596,14 +1596,14 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>31505056</v>
+        <v>31036676</v>
       </c>
       <c r="C2" t="n">
-        <v>6016.63</v>
+        <v>6052.96</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2026-03-20T15:49:40</t>
+          <t>2026-03-20T15:49:57</t>
         </is>
       </c>
       <c r="E2" t="n">
@@ -7486,10 +7486,10 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>31505056</v>
+        <v>31036676</v>
       </c>
       <c r="C5" t="n">
-        <v>6016.63</v>
+        <v>6052.96</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
@@ -7498,7 +7498,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>2026-03-20T15:49:40</t>
+          <t>2026-03-20T15:49:57</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: portfolio snapshot 2026-03-20 (2026-03-20T15:50:28)
</commit_message>
<xml_diff>
--- a/portfolio_auto.xlsx
+++ b/portfolio_auto.xlsx
@@ -471,11 +471,11 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>페트로브라스 (ADR)</t>
+          <t>유나이티드헬스 그룹</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>480</v>
+        <v>4</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
@@ -486,23 +486,23 @@
         <v>1</v>
       </c>
       <c r="E2" t="n">
-        <v>13553578.62304688</v>
+        <v>1681032.631006837</v>
       </c>
       <c r="F2" t="n">
-        <v>1447029.623046875</v>
+        <v>-13423.36899316264</v>
       </c>
       <c r="G2" t="n">
-        <v>11.95245336261287</v>
+        <v>-0.7921934233265808</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>AGNC 인베스트먼트</t>
+          <t>케이씨</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>700</v>
+        <v>50</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
@@ -513,23 +513,23 @@
         <v>1</v>
       </c>
       <c r="E3" t="n">
-        <v>10351433.71453537</v>
+        <v>1670000</v>
       </c>
       <c r="F3" t="n">
-        <v>-480580.2854646333</v>
+        <v>20500</v>
       </c>
       <c r="G3" t="n">
-        <v>-4.43666602964724</v>
+        <v>1.242800848742043</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>대한조선</t>
+          <t>하나금융지주</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>100</v>
+        <v>18</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
@@ -540,23 +540,23 @@
         <v>1</v>
       </c>
       <c r="E4" t="n">
-        <v>9120000</v>
+        <v>2037600</v>
       </c>
       <c r="F4" t="n">
-        <v>1907000</v>
+        <v>12200</v>
       </c>
       <c r="G4" t="n">
-        <v>26.43837515596839</v>
+        <v>0.6023501530561864</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>프론트라인</t>
+          <t>현대제철</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>175</v>
+        <v>80</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -567,23 +567,23 @@
         <v>1</v>
       </c>
       <c r="E5" t="n">
-        <v>8453409.11431564</v>
+        <v>2996000</v>
       </c>
       <c r="F5" t="n">
-        <v>4023545.11431564</v>
+        <v>-182000</v>
       </c>
       <c r="G5" t="n">
-        <v>90.82773453802736</v>
+        <v>-5.726872246696035</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>시드릴</t>
+          <t>휴스틸</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>123</v>
+        <v>500</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
@@ -594,23 +594,23 @@
         <v>1</v>
       </c>
       <c r="E6" t="n">
-        <v>8081063.113214018</v>
+        <v>2750000</v>
       </c>
       <c r="F6" t="n">
-        <v>1630712.113214018</v>
+        <v>471390</v>
       </c>
       <c r="G6" t="n">
-        <v>25.28098258860669</v>
+        <v>20.68761218462133</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>세아제강</t>
+          <t>DL이앤씨</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>50</v>
+        <v>40</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -621,23 +621,23 @@
         <v>1</v>
       </c>
       <c r="E7" t="n">
-        <v>7395000</v>
+        <v>2696000</v>
       </c>
       <c r="F7" t="n">
-        <v>1085000</v>
+        <v>990500</v>
       </c>
       <c r="G7" t="n">
-        <v>17.19492868462758</v>
+        <v>58.07681031955438</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>센트러스 에너지</t>
+          <t>HD건설기계</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>25</v>
+        <v>31</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
@@ -648,23 +648,23 @@
         <v>1</v>
       </c>
       <c r="E8" t="n">
-        <v>7138629.469299316</v>
+        <v>4123000</v>
       </c>
       <c r="F8" t="n">
-        <v>-294226.5307006836</v>
+        <v>87904</v>
       </c>
       <c r="G8" t="n">
-        <v>-3.958458642286136</v>
+        <v>2.178485964150543</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>트랜스오션</t>
+          <t>KoAct 코스닥액티브</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>750</v>
+        <v>200</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
@@ -675,23 +675,23 @@
         <v>1</v>
       </c>
       <c r="E9" t="n">
-        <v>7074115.140040115</v>
+        <v>2582000</v>
       </c>
       <c r="F9" t="n">
-        <v>2946881.140040115</v>
+        <v>-120000</v>
       </c>
       <c r="G9" t="n">
-        <v>71.40087380652793</v>
+        <v>-4.441154700222058</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>노블</t>
+          <t>LX인터내셔널</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>99</v>
+        <v>20</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
@@ -702,23 +702,23 @@
         <v>1</v>
       </c>
       <c r="E10" t="n">
-        <v>6886743.840087891</v>
+        <v>943000</v>
       </c>
       <c r="F10" t="n">
-        <v>2979535.840087891</v>
+        <v>4000</v>
       </c>
       <c r="G10" t="n">
-        <v>76.25741552760668</v>
+        <v>0.4259850905218318</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>타이드워터</t>
+          <t>NH투자증권우</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>48</v>
+        <v>2</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
@@ -729,23 +729,23 @@
         <v>1</v>
       </c>
       <c r="E11" t="n">
-        <v>5211036.802851856</v>
+        <v>54700</v>
       </c>
       <c r="F11" t="n">
-        <v>1486491.802851856</v>
+        <v>100</v>
       </c>
       <c r="G11" t="n">
-        <v>39.91069520845783</v>
+        <v>0.1831501831501831</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>노브</t>
+          <t>TIME 코리아밸류업액티브</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>185</v>
+        <v>201</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
@@ -756,23 +756,23 @@
         <v>1</v>
       </c>
       <c r="E12" t="n">
-        <v>5179494.129107101</v>
+        <v>4797870</v>
       </c>
       <c r="F12" t="n">
-        <v>1869486.129107101</v>
+        <v>74073</v>
       </c>
       <c r="G12" t="n">
-        <v>56.47980697046958</v>
+        <v>1.568081778281328</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>TIME 코리아밸류업액티브</t>
+          <t>프론트라인</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>201</v>
+        <v>175</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
@@ -783,19 +783,19 @@
         <v>1</v>
       </c>
       <c r="E13" t="n">
-        <v>4797870</v>
+        <v>8448173.064543074</v>
       </c>
       <c r="F13" t="n">
-        <v>74073</v>
+        <v>4018309.064543074</v>
       </c>
       <c r="G13" t="n">
-        <v>1.568081778281328</v>
+        <v>90.7095356548886</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>오케아니스 에코 탱커스</t>
+          <t>피바디 에너지</t>
         </is>
       </c>
       <c r="B14" t="n">
@@ -810,23 +810,23 @@
         <v>1</v>
       </c>
       <c r="E14" t="n">
-        <v>4596307.895957222</v>
+        <v>3605124.829619369</v>
       </c>
       <c r="F14" t="n">
-        <v>2339947.895957222</v>
+        <v>2134352.829619369</v>
       </c>
       <c r="G14" t="n">
-        <v>103.704546081176</v>
+        <v>145.1178584865206</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>삼성화재</t>
+          <t>하프니아</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>9</v>
+        <v>80</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
@@ -837,23 +837,23 @@
         <v>1</v>
       </c>
       <c r="E15" t="n">
-        <v>4270500</v>
+        <v>848519.8631833494</v>
       </c>
       <c r="F15" t="n">
-        <v>-360500</v>
+        <v>222788.8631833494</v>
       </c>
       <c r="G15" t="n">
-        <v>-7.784495789246384</v>
+        <v>35.60457499841775</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>동원개발</t>
+          <t>AGNC 인베스트먼트</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>1360</v>
+        <v>700</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
@@ -864,23 +864,23 @@
         <v>1</v>
       </c>
       <c r="E16" t="n">
-        <v>4202400</v>
+        <v>10346092.80395294</v>
       </c>
       <c r="F16" t="n">
-        <v>465000</v>
+        <v>-485921.1960470639</v>
       </c>
       <c r="G16" t="n">
-        <v>12.44180446299566</v>
+        <v>-4.485972747515503</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>HD건설기계</t>
+          <t>넥스틸</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>31</v>
+        <v>300</v>
       </c>
       <c r="C17" t="inlineStr">
         <is>
@@ -891,23 +891,23 @@
         <v>1</v>
       </c>
       <c r="E17" t="n">
-        <v>4123000</v>
+        <v>3771000</v>
       </c>
       <c r="F17" t="n">
-        <v>87904</v>
+        <v>521000</v>
       </c>
       <c r="G17" t="n">
-        <v>2.178485964150543</v>
+        <v>16.03076923076923</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>차코스 에너지 내비게이션</t>
+          <t>대신증권</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>75</v>
+        <v>55</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
@@ -918,19 +918,19 @@
         <v>1</v>
       </c>
       <c r="E18" t="n">
-        <v>4052048.962918622</v>
+        <v>2219250</v>
       </c>
       <c r="F18" t="n">
-        <v>227400.9629186224</v>
+        <v>509749</v>
       </c>
       <c r="G18" t="n">
-        <v>5.94567037067522</v>
+        <v>29.81858448752005</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>넥스틸</t>
+          <t>대창단조</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -945,23 +945,23 @@
         <v>1</v>
       </c>
       <c r="E19" t="n">
-        <v>3771000</v>
+        <v>2004000</v>
       </c>
       <c r="F19" t="n">
-        <v>521000</v>
+        <v>-54000</v>
       </c>
       <c r="G19" t="n">
-        <v>16.03076923076923</v>
+        <v>-2.623906705539359</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>피바디 에너지</t>
+          <t>대한조선</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>65</v>
+        <v>100</v>
       </c>
       <c r="C20" t="inlineStr">
         <is>
@@ -972,23 +972,23 @@
         <v>1</v>
       </c>
       <c r="E20" t="n">
-        <v>3596373.331896178</v>
+        <v>9120000</v>
       </c>
       <c r="F20" t="n">
-        <v>2125601.331896178</v>
+        <v>1907000</v>
       </c>
       <c r="G20" t="n">
-        <v>144.5228309959789</v>
+        <v>26.43837515596839</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>현대제철</t>
+          <t>동방</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>80</v>
+        <v>681</v>
       </c>
       <c r="C21" t="inlineStr">
         <is>
@@ -999,23 +999,23 @@
         <v>1</v>
       </c>
       <c r="E21" t="n">
-        <v>2996000</v>
+        <v>1995330</v>
       </c>
       <c r="F21" t="n">
-        <v>-182000</v>
+        <v>23829</v>
       </c>
       <c r="G21" t="n">
-        <v>-5.726872246696035</v>
+        <v>1.208672985709873</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>더치 브로스</t>
+          <t>동원개발</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>39</v>
+        <v>1360</v>
       </c>
       <c r="C22" t="inlineStr">
         <is>
@@ -1026,23 +1026,23 @@
         <v>1</v>
       </c>
       <c r="E22" t="n">
-        <v>2959763.281021703</v>
+        <v>4202400</v>
       </c>
       <c r="F22" t="n">
-        <v>-230880.718978297</v>
+        <v>465000</v>
       </c>
       <c r="G22" t="n">
-        <v>-7.236179247145621</v>
+        <v>12.44180446299566</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>휴스틸</t>
+          <t>미창석유</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>500</v>
+        <v>18</v>
       </c>
       <c r="C23" t="inlineStr">
         <is>
@@ -1053,23 +1053,23 @@
         <v>1</v>
       </c>
       <c r="E23" t="n">
-        <v>2750000</v>
+        <v>2097000</v>
       </c>
       <c r="F23" t="n">
-        <v>471390</v>
+        <v>-295200</v>
       </c>
       <c r="G23" t="n">
-        <v>20.68761218462133</v>
+        <v>-12.34010534236268</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>DL이앤씨</t>
+          <t>비에이치아이</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>40</v>
+        <v>8</v>
       </c>
       <c r="C24" t="inlineStr">
         <is>
@@ -1080,23 +1080,23 @@
         <v>1</v>
       </c>
       <c r="E24" t="n">
-        <v>2696000</v>
+        <v>876000</v>
       </c>
       <c r="F24" t="n">
-        <v>990500</v>
+        <v>210885</v>
       </c>
       <c r="G24" t="n">
-        <v>58.07681031955438</v>
+        <v>31.70654698811484</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>KoAct 코스닥액티브</t>
+          <t>삼성생명</t>
         </is>
       </c>
       <c r="B25" t="n">
-        <v>200</v>
+        <v>4</v>
       </c>
       <c r="C25" t="inlineStr">
         <is>
@@ -1107,23 +1107,23 @@
         <v>1</v>
       </c>
       <c r="E25" t="n">
-        <v>2582000</v>
+        <v>926000</v>
       </c>
       <c r="F25" t="n">
-        <v>-120000</v>
+        <v>93000</v>
       </c>
       <c r="G25" t="n">
-        <v>-4.441154700222058</v>
+        <v>11.16446578631453</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>대신증권</t>
+          <t>삼성화재</t>
         </is>
       </c>
       <c r="B26" t="n">
-        <v>55</v>
+        <v>9</v>
       </c>
       <c r="C26" t="inlineStr">
         <is>
@@ -1134,23 +1134,23 @@
         <v>1</v>
       </c>
       <c r="E26" t="n">
-        <v>2219250</v>
+        <v>4270500</v>
       </c>
       <c r="F26" t="n">
-        <v>509749</v>
+        <v>-360500</v>
       </c>
       <c r="G26" t="n">
-        <v>29.81858448752005</v>
+        <v>-7.784495789246384</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>발레로 에너지</t>
+          <t>세아제강</t>
         </is>
       </c>
       <c r="B27" t="n">
-        <v>6</v>
+        <v>50</v>
       </c>
       <c r="C27" t="inlineStr">
         <is>
@@ -1161,23 +1161,23 @@
         <v>1</v>
       </c>
       <c r="E27" t="n">
-        <v>2176561.162089184</v>
+        <v>7395000</v>
       </c>
       <c r="F27" t="n">
-        <v>112571.1620891839</v>
+        <v>1085000</v>
       </c>
       <c r="G27" t="n">
-        <v>5.454055595675557</v>
+        <v>17.19492868462758</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>미창석유</t>
+          <t>노브</t>
         </is>
       </c>
       <c r="B28" t="n">
-        <v>18</v>
+        <v>185</v>
       </c>
       <c r="C28" t="inlineStr">
         <is>
@@ -1188,23 +1188,23 @@
         <v>1</v>
       </c>
       <c r="E28" t="n">
-        <v>2097000</v>
+        <v>5179494.129107101</v>
       </c>
       <c r="F28" t="n">
-        <v>-295200</v>
+        <v>1869486.129107101</v>
       </c>
       <c r="G28" t="n">
-        <v>-12.34010534236268</v>
+        <v>56.47980697046958</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>하나금융지주</t>
+          <t>노블</t>
         </is>
       </c>
       <c r="B29" t="n">
-        <v>18</v>
+        <v>99</v>
       </c>
       <c r="C29" t="inlineStr">
         <is>
@@ -1215,23 +1215,23 @@
         <v>1</v>
       </c>
       <c r="E29" t="n">
-        <v>2037600</v>
+        <v>6891186.719841287</v>
       </c>
       <c r="F29" t="n">
-        <v>12200</v>
+        <v>2983978.719841287</v>
       </c>
       <c r="G29" t="n">
-        <v>0.6023501530561864</v>
+        <v>76.37112536218412</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>대창단조</t>
+          <t>더치 브로스</t>
         </is>
       </c>
       <c r="B30" t="n">
-        <v>300</v>
+        <v>39</v>
       </c>
       <c r="C30" t="inlineStr">
         <is>
@@ -1242,23 +1242,23 @@
         <v>1</v>
       </c>
       <c r="E30" t="n">
-        <v>2004000</v>
+        <v>2966169.274976688</v>
       </c>
       <c r="F30" t="n">
-        <v>-54000</v>
+        <v>-224474.7250233125</v>
       </c>
       <c r="G30" t="n">
-        <v>-2.623906705539359</v>
+        <v>-7.035404922119562</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>동방</t>
+          <t>발레로 에너지</t>
         </is>
       </c>
       <c r="B31" t="n">
-        <v>681</v>
+        <v>6</v>
       </c>
       <c r="C31" t="inlineStr">
         <is>
@@ -1269,23 +1269,23 @@
         <v>1</v>
       </c>
       <c r="E31" t="n">
-        <v>1995330</v>
+        <v>2176078.237399444</v>
       </c>
       <c r="F31" t="n">
-        <v>23829</v>
+        <v>112088.237399444</v>
       </c>
       <c r="G31" t="n">
-        <v>1.208672985709873</v>
+        <v>5.430657968277171</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>스타 벌크 캐리어스</t>
+          <t>센트러스 에너지</t>
         </is>
       </c>
       <c r="B32" t="n">
-        <v>50</v>
+        <v>25</v>
       </c>
       <c r="C32" t="inlineStr">
         <is>
@@ -1296,23 +1296,23 @@
         <v>1</v>
       </c>
       <c r="E32" t="n">
-        <v>1696441.320678405</v>
+        <v>7136946.560301818</v>
       </c>
       <c r="F32" t="n">
-        <v>382088.3206784055</v>
+        <v>-295909.439698182</v>
       </c>
       <c r="G32" t="n">
-        <v>29.0704491623183</v>
+        <v>-3.981100127571179</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>유나이티드헬스 그룹</t>
+          <t>스타 벌크 캐리어스</t>
         </is>
       </c>
       <c r="B33" t="n">
-        <v>4</v>
+        <v>50</v>
       </c>
       <c r="C33" t="inlineStr">
         <is>
@@ -1323,23 +1323,23 @@
         <v>1</v>
       </c>
       <c r="E33" t="n">
-        <v>1683366.447431445</v>
+        <v>1697189.327788772</v>
       </c>
       <c r="F33" t="n">
-        <v>-11089.55256855441</v>
+        <v>382836.3277887721</v>
       </c>
       <c r="G33" t="n">
-        <v>-0.6544609342794628</v>
+        <v>29.1273598332238</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>케이씨</t>
+          <t>시드릴</t>
         </is>
       </c>
       <c r="B34" t="n">
-        <v>50</v>
+        <v>123</v>
       </c>
       <c r="C34" t="inlineStr">
         <is>
@@ -1350,23 +1350,23 @@
         <v>1</v>
       </c>
       <c r="E34" t="n">
-        <v>1670000</v>
+        <v>8045641.850687351</v>
       </c>
       <c r="F34" t="n">
-        <v>20500</v>
+        <v>1595290.850687351</v>
       </c>
       <c r="G34" t="n">
-        <v>1.242800848742043</v>
+        <v>24.73184561099622</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>텍사스 퍼시픽 랜드</t>
+          <t>오케아니스 에코 탱커스</t>
         </is>
       </c>
       <c r="B35" t="n">
-        <v>2</v>
+        <v>65</v>
       </c>
       <c r="C35" t="inlineStr">
         <is>
@@ -1377,23 +1377,23 @@
         <v>1</v>
       </c>
       <c r="E35" t="n">
-        <v>1596420.098271191</v>
+        <v>4579942.561830599</v>
       </c>
       <c r="F35" t="n">
-        <v>18525.09827119112</v>
+        <v>2323582.561830599</v>
       </c>
       <c r="G35" t="n">
-        <v>1.174038720649417</v>
+        <v>102.9792480734723</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>LX인터내셔널</t>
+          <t>차코스 에너지 내비게이션</t>
         </is>
       </c>
       <c r="B36" t="n">
-        <v>20</v>
+        <v>75</v>
       </c>
       <c r="C36" t="inlineStr">
         <is>
@@ -1404,23 +1404,23 @@
         <v>1</v>
       </c>
       <c r="E36" t="n">
-        <v>943000</v>
+        <v>4054853.668580018</v>
       </c>
       <c r="F36" t="n">
-        <v>4000</v>
+        <v>230205.668580018</v>
       </c>
       <c r="G36" t="n">
-        <v>0.4259850905218318</v>
+        <v>6.019002757378404</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>삼성생명</t>
+          <t>클리블랜드 클리프스</t>
         </is>
       </c>
       <c r="B37" t="n">
-        <v>4</v>
+        <v>70</v>
       </c>
       <c r="C37" t="inlineStr">
         <is>
@@ -1431,23 +1431,23 @@
         <v>1</v>
       </c>
       <c r="E37" t="n">
-        <v>926000</v>
+        <v>832649.0084090387</v>
       </c>
       <c r="F37" t="n">
-        <v>93000</v>
+        <v>-183405.9915909613</v>
       </c>
       <c r="G37" t="n">
-        <v>11.16446578631453</v>
+        <v>-18.05079366677605</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>비에이치아이</t>
+          <t>타이드워터</t>
         </is>
       </c>
       <c r="B38" t="n">
-        <v>8</v>
+        <v>48</v>
       </c>
       <c r="C38" t="inlineStr">
         <is>
@@ -1458,23 +1458,23 @@
         <v>1</v>
       </c>
       <c r="E38" t="n">
-        <v>876000</v>
+        <v>5207446.231761038</v>
       </c>
       <c r="F38" t="n">
-        <v>210885</v>
+        <v>1482901.231761038</v>
       </c>
       <c r="G38" t="n">
-        <v>31.70654698811484</v>
+        <v>39.81429226284119</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>하프니아</t>
+          <t>텍사스 퍼시픽 랜드</t>
         </is>
       </c>
       <c r="B39" t="n">
-        <v>80</v>
+        <v>2</v>
       </c>
       <c r="C39" t="inlineStr">
         <is>
@@ -1485,23 +1485,23 @@
         <v>1</v>
       </c>
       <c r="E39" t="n">
-        <v>848519.8631833494</v>
+        <v>1600937.987030566</v>
       </c>
       <c r="F39" t="n">
-        <v>222788.8631833494</v>
+        <v>23042.98703056574</v>
       </c>
       <c r="G39" t="n">
-        <v>35.60457499841775</v>
+        <v>1.460362510215556</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>클리블랜드 클리프스</t>
+          <t>트랜스오션</t>
         </is>
       </c>
       <c r="B40" t="n">
-        <v>70</v>
+        <v>750</v>
       </c>
       <c r="C40" t="inlineStr">
         <is>
@@ -1512,23 +1512,23 @@
         <v>1</v>
       </c>
       <c r="E40" t="n">
-        <v>833036.4441346284</v>
+        <v>7074115.140040115</v>
       </c>
       <c r="F40" t="n">
-        <v>-183018.5558653716</v>
+        <v>2946881.140040115</v>
       </c>
       <c r="G40" t="n">
-        <v>-18.01266229341636</v>
+        <v>71.40087380652793</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>NH투자증권우</t>
+          <t>페트로브라스 (ADR)</t>
         </is>
       </c>
       <c r="B41" t="n">
-        <v>2</v>
+        <v>480</v>
       </c>
       <c r="C41" t="inlineStr">
         <is>
@@ -1539,13 +1539,13 @@
         <v>1</v>
       </c>
       <c r="E41" t="n">
-        <v>54591</v>
+        <v>13539216.88652784</v>
       </c>
       <c r="F41" t="n">
-        <v>-9</v>
+        <v>1432667.886527836</v>
       </c>
       <c r="G41" t="n">
-        <v>-0.01648351648351648</v>
+        <v>11.83382553135362</v>
       </c>
     </row>
   </sheetData>
@@ -1603,7 +1603,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2026-03-20T15:49:57</t>
+          <t>2026-03-20T15:50:28</t>
         </is>
       </c>
       <c r="E2" t="n">
@@ -5912,17 +5912,17 @@
         <v>1</v>
       </c>
       <c r="F116" t="n">
-        <v>13553578.62304688</v>
+        <v>13539216.88652784</v>
       </c>
       <c r="G116" t="n">
-        <v>1447029.623046875</v>
+        <v>1432667.886527836</v>
       </c>
       <c r="H116" t="n">
-        <v>11.95245336261287</v>
+        <v>11.83382553135362</v>
       </c>
       <c r="I116" t="inlineStr">
         <is>
-          <t>2026-03-20T15:49:40</t>
+          <t>2026-03-20T15:50:28</t>
         </is>
       </c>
     </row>
@@ -5949,17 +5949,17 @@
         <v>1</v>
       </c>
       <c r="F117" t="n">
-        <v>10351433.71453537</v>
+        <v>10346092.80395294</v>
       </c>
       <c r="G117" t="n">
-        <v>-480580.2854646333</v>
+        <v>-485921.1960470639</v>
       </c>
       <c r="H117" t="n">
-        <v>-4.43666602964724</v>
+        <v>-4.485972747515503</v>
       </c>
       <c r="I117" t="inlineStr">
         <is>
-          <t>2026-03-20T15:49:40</t>
+          <t>2026-03-20T15:50:28</t>
         </is>
       </c>
     </row>
@@ -5996,7 +5996,7 @@
       </c>
       <c r="I118" t="inlineStr">
         <is>
-          <t>2026-03-20T15:49:40</t>
+          <t>2026-03-20T15:50:28</t>
         </is>
       </c>
     </row>
@@ -6023,17 +6023,17 @@
         <v>1</v>
       </c>
       <c r="F119" t="n">
-        <v>8453409.11431564</v>
+        <v>8448173.064543074</v>
       </c>
       <c r="G119" t="n">
-        <v>4023545.11431564</v>
+        <v>4018309.064543074</v>
       </c>
       <c r="H119" t="n">
-        <v>90.82773453802736</v>
+        <v>90.7095356548886</v>
       </c>
       <c r="I119" t="inlineStr">
         <is>
-          <t>2026-03-20T15:49:40</t>
+          <t>2026-03-20T15:50:28</t>
         </is>
       </c>
     </row>
@@ -6060,17 +6060,17 @@
         <v>1</v>
       </c>
       <c r="F120" t="n">
-        <v>8081063.113214018</v>
+        <v>8045641.850687351</v>
       </c>
       <c r="G120" t="n">
-        <v>1630712.113214018</v>
+        <v>1595290.850687351</v>
       </c>
       <c r="H120" t="n">
-        <v>25.28098258860669</v>
+        <v>24.73184561099622</v>
       </c>
       <c r="I120" t="inlineStr">
         <is>
-          <t>2026-03-20T15:49:40</t>
+          <t>2026-03-20T15:50:28</t>
         </is>
       </c>
     </row>
@@ -6107,7 +6107,7 @@
       </c>
       <c r="I121" t="inlineStr">
         <is>
-          <t>2026-03-20T15:49:40</t>
+          <t>2026-03-20T15:50:28</t>
         </is>
       </c>
     </row>
@@ -6134,17 +6134,17 @@
         <v>1</v>
       </c>
       <c r="F122" t="n">
-        <v>7138629.469299316</v>
+        <v>7136946.560301818</v>
       </c>
       <c r="G122" t="n">
-        <v>-294226.5307006836</v>
+        <v>-295909.439698182</v>
       </c>
       <c r="H122" t="n">
-        <v>-3.958458642286136</v>
+        <v>-3.981100127571179</v>
       </c>
       <c r="I122" t="inlineStr">
         <is>
-          <t>2026-03-20T15:49:40</t>
+          <t>2026-03-20T15:50:28</t>
         </is>
       </c>
     </row>
@@ -6181,7 +6181,7 @@
       </c>
       <c r="I123" t="inlineStr">
         <is>
-          <t>2026-03-20T15:49:40</t>
+          <t>2026-03-20T15:50:28</t>
         </is>
       </c>
     </row>
@@ -6208,17 +6208,17 @@
         <v>1</v>
       </c>
       <c r="F124" t="n">
-        <v>6886743.840087891</v>
+        <v>6891186.719841287</v>
       </c>
       <c r="G124" t="n">
-        <v>2979535.840087891</v>
+        <v>2983978.719841287</v>
       </c>
       <c r="H124" t="n">
-        <v>76.25741552760668</v>
+        <v>76.37112536218412</v>
       </c>
       <c r="I124" t="inlineStr">
         <is>
-          <t>2026-03-20T15:49:40</t>
+          <t>2026-03-20T15:50:28</t>
         </is>
       </c>
     </row>
@@ -6245,17 +6245,17 @@
         <v>1</v>
       </c>
       <c r="F125" t="n">
-        <v>5211036.802851856</v>
+        <v>5207446.231761038</v>
       </c>
       <c r="G125" t="n">
-        <v>1486491.802851856</v>
+        <v>1482901.231761038</v>
       </c>
       <c r="H125" t="n">
-        <v>39.91069520845783</v>
+        <v>39.81429226284119</v>
       </c>
       <c r="I125" t="inlineStr">
         <is>
-          <t>2026-03-20T15:49:40</t>
+          <t>2026-03-20T15:50:28</t>
         </is>
       </c>
     </row>
@@ -6292,7 +6292,7 @@
       </c>
       <c r="I126" t="inlineStr">
         <is>
-          <t>2026-03-20T15:49:40</t>
+          <t>2026-03-20T15:50:28</t>
         </is>
       </c>
     </row>
@@ -6329,7 +6329,7 @@
       </c>
       <c r="I127" t="inlineStr">
         <is>
-          <t>2026-03-20T15:49:40</t>
+          <t>2026-03-20T15:50:28</t>
         </is>
       </c>
     </row>
@@ -6356,17 +6356,17 @@
         <v>1</v>
       </c>
       <c r="F128" t="n">
-        <v>4596307.895957222</v>
+        <v>4579942.561830599</v>
       </c>
       <c r="G128" t="n">
-        <v>2339947.895957222</v>
+        <v>2323582.561830599</v>
       </c>
       <c r="H128" t="n">
-        <v>103.704546081176</v>
+        <v>102.9792480734723</v>
       </c>
       <c r="I128" t="inlineStr">
         <is>
-          <t>2026-03-20T15:49:40</t>
+          <t>2026-03-20T15:50:28</t>
         </is>
       </c>
     </row>
@@ -6403,7 +6403,7 @@
       </c>
       <c r="I129" t="inlineStr">
         <is>
-          <t>2026-03-20T15:49:40</t>
+          <t>2026-03-20T15:50:28</t>
         </is>
       </c>
     </row>
@@ -6440,7 +6440,7 @@
       </c>
       <c r="I130" t="inlineStr">
         <is>
-          <t>2026-03-20T15:49:40</t>
+          <t>2026-03-20T15:50:28</t>
         </is>
       </c>
     </row>
@@ -6477,7 +6477,7 @@
       </c>
       <c r="I131" t="inlineStr">
         <is>
-          <t>2026-03-20T15:49:40</t>
+          <t>2026-03-20T15:50:28</t>
         </is>
       </c>
     </row>
@@ -6504,17 +6504,17 @@
         <v>1</v>
       </c>
       <c r="F132" t="n">
-        <v>4052048.962918622</v>
+        <v>4054853.668580018</v>
       </c>
       <c r="G132" t="n">
-        <v>227400.9629186224</v>
+        <v>230205.668580018</v>
       </c>
       <c r="H132" t="n">
-        <v>5.94567037067522</v>
+        <v>6.019002757378404</v>
       </c>
       <c r="I132" t="inlineStr">
         <is>
-          <t>2026-03-20T15:49:40</t>
+          <t>2026-03-20T15:50:28</t>
         </is>
       </c>
     </row>
@@ -6551,7 +6551,7 @@
       </c>
       <c r="I133" t="inlineStr">
         <is>
-          <t>2026-03-20T15:49:40</t>
+          <t>2026-03-20T15:50:28</t>
         </is>
       </c>
     </row>
@@ -6578,17 +6578,17 @@
         <v>1</v>
       </c>
       <c r="F134" t="n">
-        <v>3596373.331896178</v>
+        <v>3605124.829619369</v>
       </c>
       <c r="G134" t="n">
-        <v>2125601.331896178</v>
+        <v>2134352.829619369</v>
       </c>
       <c r="H134" t="n">
-        <v>144.5228309959789</v>
+        <v>145.1178584865206</v>
       </c>
       <c r="I134" t="inlineStr">
         <is>
-          <t>2026-03-20T15:49:40</t>
+          <t>2026-03-20T15:50:28</t>
         </is>
       </c>
     </row>
@@ -6625,7 +6625,7 @@
       </c>
       <c r="I135" t="inlineStr">
         <is>
-          <t>2026-03-20T15:49:40</t>
+          <t>2026-03-20T15:50:28</t>
         </is>
       </c>
     </row>
@@ -6652,17 +6652,17 @@
         <v>1</v>
       </c>
       <c r="F136" t="n">
-        <v>2959763.281021703</v>
+        <v>2966169.274976688</v>
       </c>
       <c r="G136" t="n">
-        <v>-230880.718978297</v>
+        <v>-224474.7250233125</v>
       </c>
       <c r="H136" t="n">
-        <v>-7.236179247145621</v>
+        <v>-7.035404922119562</v>
       </c>
       <c r="I136" t="inlineStr">
         <is>
-          <t>2026-03-20T15:49:40</t>
+          <t>2026-03-20T15:50:28</t>
         </is>
       </c>
     </row>
@@ -6699,7 +6699,7 @@
       </c>
       <c r="I137" t="inlineStr">
         <is>
-          <t>2026-03-20T15:49:40</t>
+          <t>2026-03-20T15:50:28</t>
         </is>
       </c>
     </row>
@@ -6736,7 +6736,7 @@
       </c>
       <c r="I138" t="inlineStr">
         <is>
-          <t>2026-03-20T15:49:40</t>
+          <t>2026-03-20T15:50:28</t>
         </is>
       </c>
     </row>
@@ -6773,7 +6773,7 @@
       </c>
       <c r="I139" t="inlineStr">
         <is>
-          <t>2026-03-20T15:49:40</t>
+          <t>2026-03-20T15:50:28</t>
         </is>
       </c>
     </row>
@@ -6810,7 +6810,7 @@
       </c>
       <c r="I140" t="inlineStr">
         <is>
-          <t>2026-03-20T15:49:40</t>
+          <t>2026-03-20T15:50:28</t>
         </is>
       </c>
     </row>
@@ -6837,17 +6837,17 @@
         <v>1</v>
       </c>
       <c r="F141" t="n">
-        <v>2176561.162089184</v>
+        <v>2176078.237399444</v>
       </c>
       <c r="G141" t="n">
-        <v>112571.1620891839</v>
+        <v>112088.237399444</v>
       </c>
       <c r="H141" t="n">
-        <v>5.454055595675557</v>
+        <v>5.430657968277171</v>
       </c>
       <c r="I141" t="inlineStr">
         <is>
-          <t>2026-03-20T15:49:40</t>
+          <t>2026-03-20T15:50:28</t>
         </is>
       </c>
     </row>
@@ -6884,7 +6884,7 @@
       </c>
       <c r="I142" t="inlineStr">
         <is>
-          <t>2026-03-20T15:49:40</t>
+          <t>2026-03-20T15:50:28</t>
         </is>
       </c>
     </row>
@@ -6921,7 +6921,7 @@
       </c>
       <c r="I143" t="inlineStr">
         <is>
-          <t>2026-03-20T15:49:40</t>
+          <t>2026-03-20T15:50:28</t>
         </is>
       </c>
     </row>
@@ -6958,7 +6958,7 @@
       </c>
       <c r="I144" t="inlineStr">
         <is>
-          <t>2026-03-20T15:49:40</t>
+          <t>2026-03-20T15:50:28</t>
         </is>
       </c>
     </row>
@@ -6995,7 +6995,7 @@
       </c>
       <c r="I145" t="inlineStr">
         <is>
-          <t>2026-03-20T15:49:40</t>
+          <t>2026-03-20T15:50:28</t>
         </is>
       </c>
     </row>
@@ -7022,17 +7022,17 @@
         <v>1</v>
       </c>
       <c r="F146" t="n">
-        <v>1696441.320678405</v>
+        <v>1697189.327788772</v>
       </c>
       <c r="G146" t="n">
-        <v>382088.3206784055</v>
+        <v>382836.3277887721</v>
       </c>
       <c r="H146" t="n">
-        <v>29.0704491623183</v>
+        <v>29.1273598332238</v>
       </c>
       <c r="I146" t="inlineStr">
         <is>
-          <t>2026-03-20T15:49:40</t>
+          <t>2026-03-20T15:50:28</t>
         </is>
       </c>
     </row>
@@ -7059,17 +7059,17 @@
         <v>1</v>
       </c>
       <c r="F147" t="n">
-        <v>1683366.447431445</v>
+        <v>1681032.631006837</v>
       </c>
       <c r="G147" t="n">
-        <v>-11089.55256855441</v>
+        <v>-13423.36899316264</v>
       </c>
       <c r="H147" t="n">
-        <v>-0.6544609342794628</v>
+        <v>-0.7921934233265808</v>
       </c>
       <c r="I147" t="inlineStr">
         <is>
-          <t>2026-03-20T15:49:40</t>
+          <t>2026-03-20T15:50:28</t>
         </is>
       </c>
     </row>
@@ -7106,7 +7106,7 @@
       </c>
       <c r="I148" t="inlineStr">
         <is>
-          <t>2026-03-20T15:49:40</t>
+          <t>2026-03-20T15:50:28</t>
         </is>
       </c>
     </row>
@@ -7133,17 +7133,17 @@
         <v>1</v>
       </c>
       <c r="F149" t="n">
-        <v>1596420.098271191</v>
+        <v>1600937.987030566</v>
       </c>
       <c r="G149" t="n">
-        <v>18525.09827119112</v>
+        <v>23042.98703056574</v>
       </c>
       <c r="H149" t="n">
-        <v>1.174038720649417</v>
+        <v>1.460362510215556</v>
       </c>
       <c r="I149" t="inlineStr">
         <is>
-          <t>2026-03-20T15:49:40</t>
+          <t>2026-03-20T15:50:28</t>
         </is>
       </c>
     </row>
@@ -7180,7 +7180,7 @@
       </c>
       <c r="I150" t="inlineStr">
         <is>
-          <t>2026-03-20T15:49:40</t>
+          <t>2026-03-20T15:50:28</t>
         </is>
       </c>
     </row>
@@ -7217,7 +7217,7 @@
       </c>
       <c r="I151" t="inlineStr">
         <is>
-          <t>2026-03-20T15:49:40</t>
+          <t>2026-03-20T15:50:28</t>
         </is>
       </c>
     </row>
@@ -7254,7 +7254,7 @@
       </c>
       <c r="I152" t="inlineStr">
         <is>
-          <t>2026-03-20T15:49:40</t>
+          <t>2026-03-20T15:50:28</t>
         </is>
       </c>
     </row>
@@ -7291,7 +7291,7 @@
       </c>
       <c r="I153" t="inlineStr">
         <is>
-          <t>2026-03-20T15:49:40</t>
+          <t>2026-03-20T15:50:28</t>
         </is>
       </c>
     </row>
@@ -7318,17 +7318,17 @@
         <v>1</v>
       </c>
       <c r="F154" t="n">
-        <v>833036.4441346284</v>
+        <v>832649.0084090387</v>
       </c>
       <c r="G154" t="n">
-        <v>-183018.5558653716</v>
+        <v>-183405.9915909613</v>
       </c>
       <c r="H154" t="n">
-        <v>-18.01266229341636</v>
+        <v>-18.05079366677605</v>
       </c>
       <c r="I154" t="inlineStr">
         <is>
-          <t>2026-03-20T15:49:40</t>
+          <t>2026-03-20T15:50:28</t>
         </is>
       </c>
     </row>
@@ -7355,17 +7355,17 @@
         <v>1</v>
       </c>
       <c r="F155" t="n">
-        <v>54591</v>
+        <v>54700</v>
       </c>
       <c r="G155" t="n">
-        <v>-9</v>
+        <v>100</v>
       </c>
       <c r="H155" t="n">
-        <v>-0.01648351648351648</v>
+        <v>0.1831501831501831</v>
       </c>
       <c r="I155" t="inlineStr">
         <is>
-          <t>2026-03-20T15:49:40</t>
+          <t>2026-03-20T15:50:28</t>
         </is>
       </c>
     </row>
@@ -7498,7 +7498,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>2026-03-20T15:49:57</t>
+          <t>2026-03-20T15:50:28</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: portfolio snapshot 2026-03-20 (2026-03-20T15:51:21)
</commit_message>
<xml_diff>
--- a/portfolio_auto.xlsx
+++ b/portfolio_auto.xlsx
@@ -486,13 +486,13 @@
         <v>1</v>
       </c>
       <c r="E2" t="n">
-        <v>1681032.631006837</v>
+        <v>1679626.497480273</v>
       </c>
       <c r="F2" t="n">
-        <v>-13423.36899316264</v>
+        <v>-14829.50251972629</v>
       </c>
       <c r="G2" t="n">
-        <v>-0.7921934233265808</v>
+        <v>-0.8751777868369726</v>
       </c>
     </row>
     <row r="3">
@@ -783,13 +783,13 @@
         <v>1</v>
       </c>
       <c r="E13" t="n">
-        <v>8448173.064543074</v>
+        <v>8445554.540319601</v>
       </c>
       <c r="F13" t="n">
-        <v>4018309.064543074</v>
+        <v>4015690.540319601</v>
       </c>
       <c r="G13" t="n">
-        <v>90.7095356548886</v>
+        <v>90.65042494125331</v>
       </c>
     </row>
     <row r="14">
@@ -810,13 +810,13 @@
         <v>1</v>
       </c>
       <c r="E14" t="n">
-        <v>3605124.829619369</v>
+        <v>3585190.718330247</v>
       </c>
       <c r="F14" t="n">
-        <v>2134352.829619369</v>
+        <v>2114418.718330247</v>
       </c>
       <c r="G14" t="n">
-        <v>145.1178584865206</v>
+        <v>143.7625082834217</v>
       </c>
     </row>
     <row r="15">
@@ -837,13 +837,13 @@
         <v>1</v>
       </c>
       <c r="E15" t="n">
-        <v>848519.8631833494</v>
+        <v>849118.2118045352</v>
       </c>
       <c r="F15" t="n">
-        <v>222788.8631833494</v>
+        <v>223387.2118045352</v>
       </c>
       <c r="G15" t="n">
-        <v>35.60457499841775</v>
+        <v>35.70019893605003</v>
       </c>
     </row>
     <row r="16">
@@ -864,13 +864,13 @@
         <v>1</v>
       </c>
       <c r="E16" t="n">
-        <v>10346092.80395294</v>
+        <v>10340961.61499023</v>
       </c>
       <c r="F16" t="n">
-        <v>-485921.1960470639</v>
+        <v>-491052.3850097656</v>
       </c>
       <c r="G16" t="n">
-        <v>-4.485972747515503</v>
+        <v>-4.53334333771878</v>
       </c>
     </row>
     <row r="17">
@@ -1188,13 +1188,13 @@
         <v>1</v>
       </c>
       <c r="E28" t="n">
-        <v>5179494.129107101</v>
+        <v>5172575.327271582</v>
       </c>
       <c r="F28" t="n">
-        <v>1869486.129107101</v>
+        <v>1862567.327271582</v>
       </c>
       <c r="G28" t="n">
-        <v>56.47980697046958</v>
+        <v>56.27078022988409</v>
       </c>
     </row>
     <row r="29">
@@ -1215,13 +1215,13 @@
         <v>1</v>
       </c>
       <c r="E29" t="n">
-        <v>6891186.719841287</v>
+        <v>6886743.840087891</v>
       </c>
       <c r="F29" t="n">
-        <v>2983978.719841287</v>
+        <v>2979535.840087891</v>
       </c>
       <c r="G29" t="n">
-        <v>76.37112536218412</v>
+        <v>76.25741552760668</v>
       </c>
     </row>
     <row r="30">
@@ -1242,13 +1242,13 @@
         <v>1</v>
       </c>
       <c r="E30" t="n">
-        <v>2966169.274976688</v>
+        <v>2966461.05339016</v>
       </c>
       <c r="F30" t="n">
-        <v>-224474.7250233125</v>
+        <v>-224182.9466098398</v>
       </c>
       <c r="G30" t="n">
-        <v>-7.035404922119562</v>
+        <v>-7.026260109552799</v>
       </c>
     </row>
     <row r="31">
@@ -1269,13 +1269,13 @@
         <v>1</v>
       </c>
       <c r="E31" t="n">
-        <v>2176078.237399444</v>
+        <v>2176695.794808984</v>
       </c>
       <c r="F31" t="n">
-        <v>112088.237399444</v>
+        <v>112705.7948089838</v>
       </c>
       <c r="G31" t="n">
-        <v>5.430657968277171</v>
+        <v>5.460578530370002</v>
       </c>
     </row>
     <row r="32">
@@ -1296,13 +1296,13 @@
         <v>1</v>
       </c>
       <c r="E32" t="n">
-        <v>7136946.560301818</v>
+        <v>7118620.600099489</v>
       </c>
       <c r="F32" t="n">
-        <v>-295909.439698182</v>
+        <v>-314235.3999005109</v>
       </c>
       <c r="G32" t="n">
-        <v>-3.981100127571179</v>
+        <v>-4.227653541256697</v>
       </c>
     </row>
     <row r="33">
@@ -1323,13 +1323,13 @@
         <v>1</v>
       </c>
       <c r="E33" t="n">
-        <v>1697189.327788772</v>
+        <v>1696441.320678405</v>
       </c>
       <c r="F33" t="n">
-        <v>382836.3277887721</v>
+        <v>382088.3206784055</v>
       </c>
       <c r="G33" t="n">
-        <v>29.1273598332238</v>
+        <v>29.0704491623183</v>
       </c>
     </row>
     <row r="34">
@@ -1350,13 +1350,13 @@
         <v>1</v>
       </c>
       <c r="E34" t="n">
-        <v>8045641.850687351</v>
+        <v>8054842.689107571</v>
       </c>
       <c r="F34" t="n">
-        <v>1595290.850687351</v>
+        <v>1604491.689107571</v>
       </c>
       <c r="G34" t="n">
-        <v>24.73184561099622</v>
+        <v>24.87448650635556</v>
       </c>
     </row>
     <row r="35">
@@ -1431,13 +1431,13 @@
         <v>1</v>
       </c>
       <c r="E37" t="n">
-        <v>832649.0084090387</v>
+        <v>832251.0866024625</v>
       </c>
       <c r="F37" t="n">
-        <v>-183405.9915909613</v>
+        <v>-183803.9133975375</v>
       </c>
       <c r="G37" t="n">
-        <v>-18.05079366677605</v>
+        <v>-18.08995707885277</v>
       </c>
     </row>
     <row r="38">
@@ -1458,13 +1458,13 @@
         <v>1</v>
       </c>
       <c r="E38" t="n">
-        <v>5207446.231761038</v>
+        <v>5216422.111643851</v>
       </c>
       <c r="F38" t="n">
-        <v>1482901.231761038</v>
+        <v>1491877.111643851</v>
       </c>
       <c r="G38" t="n">
-        <v>39.81429226284119</v>
+        <v>40.05528491785844</v>
       </c>
     </row>
     <row r="39">
@@ -1512,13 +1512,13 @@
         <v>1</v>
       </c>
       <c r="E40" t="n">
-        <v>7074115.140040115</v>
+        <v>7068505.621716497</v>
       </c>
       <c r="F40" t="n">
-        <v>2946881.140040115</v>
+        <v>2941271.621716497</v>
       </c>
       <c r="G40" t="n">
-        <v>71.40087380652793</v>
+        <v>71.26495909164579</v>
       </c>
     </row>
     <row r="41">
@@ -1539,13 +1539,13 @@
         <v>1</v>
       </c>
       <c r="E41" t="n">
-        <v>13539216.88652784</v>
+        <v>13542808.00546288</v>
       </c>
       <c r="F41" t="n">
-        <v>1432667.886527836</v>
+        <v>1436259.005462885</v>
       </c>
       <c r="G41" t="n">
-        <v>11.83382553135362</v>
+        <v>11.86348814565476</v>
       </c>
     </row>
   </sheetData>
@@ -1603,7 +1603,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2026-03-20T15:50:28</t>
+          <t>2026-03-20T15:51:21</t>
         </is>
       </c>
       <c r="E2" t="n">
@@ -5912,17 +5912,17 @@
         <v>1</v>
       </c>
       <c r="F116" t="n">
-        <v>13539216.88652784</v>
+        <v>13542808.00546288</v>
       </c>
       <c r="G116" t="n">
-        <v>1432667.886527836</v>
+        <v>1436259.005462885</v>
       </c>
       <c r="H116" t="n">
-        <v>11.83382553135362</v>
+        <v>11.86348814565476</v>
       </c>
       <c r="I116" t="inlineStr">
         <is>
-          <t>2026-03-20T15:50:28</t>
+          <t>2026-03-20T15:51:21</t>
         </is>
       </c>
     </row>
@@ -5949,17 +5949,17 @@
         <v>1</v>
       </c>
       <c r="F117" t="n">
-        <v>10346092.80395294</v>
+        <v>10340961.61499023</v>
       </c>
       <c r="G117" t="n">
-        <v>-485921.1960470639</v>
+        <v>-491052.3850097656</v>
       </c>
       <c r="H117" t="n">
-        <v>-4.485972747515503</v>
+        <v>-4.53334333771878</v>
       </c>
       <c r="I117" t="inlineStr">
         <is>
-          <t>2026-03-20T15:50:28</t>
+          <t>2026-03-20T15:51:21</t>
         </is>
       </c>
     </row>
@@ -5996,7 +5996,7 @@
       </c>
       <c r="I118" t="inlineStr">
         <is>
-          <t>2026-03-20T15:50:28</t>
+          <t>2026-03-20T15:51:21</t>
         </is>
       </c>
     </row>
@@ -6023,17 +6023,17 @@
         <v>1</v>
       </c>
       <c r="F119" t="n">
-        <v>8448173.064543074</v>
+        <v>8445554.540319601</v>
       </c>
       <c r="G119" t="n">
-        <v>4018309.064543074</v>
+        <v>4015690.540319601</v>
       </c>
       <c r="H119" t="n">
-        <v>90.7095356548886</v>
+        <v>90.65042494125331</v>
       </c>
       <c r="I119" t="inlineStr">
         <is>
-          <t>2026-03-20T15:50:28</t>
+          <t>2026-03-20T15:51:21</t>
         </is>
       </c>
     </row>
@@ -6060,17 +6060,17 @@
         <v>1</v>
       </c>
       <c r="F120" t="n">
-        <v>8045641.850687351</v>
+        <v>8054842.689107571</v>
       </c>
       <c r="G120" t="n">
-        <v>1595290.850687351</v>
+        <v>1604491.689107571</v>
       </c>
       <c r="H120" t="n">
-        <v>24.73184561099622</v>
+        <v>24.87448650635556</v>
       </c>
       <c r="I120" t="inlineStr">
         <is>
-          <t>2026-03-20T15:50:28</t>
+          <t>2026-03-20T15:51:21</t>
         </is>
       </c>
     </row>
@@ -6107,7 +6107,7 @@
       </c>
       <c r="I121" t="inlineStr">
         <is>
-          <t>2026-03-20T15:50:28</t>
+          <t>2026-03-20T15:51:21</t>
         </is>
       </c>
     </row>
@@ -6134,17 +6134,17 @@
         <v>1</v>
       </c>
       <c r="F122" t="n">
-        <v>7136946.560301818</v>
+        <v>7118620.600099489</v>
       </c>
       <c r="G122" t="n">
-        <v>-295909.439698182</v>
+        <v>-314235.3999005109</v>
       </c>
       <c r="H122" t="n">
-        <v>-3.981100127571179</v>
+        <v>-4.227653541256697</v>
       </c>
       <c r="I122" t="inlineStr">
         <is>
-          <t>2026-03-20T15:50:28</t>
+          <t>2026-03-20T15:51:21</t>
         </is>
       </c>
     </row>
@@ -6171,17 +6171,17 @@
         <v>1</v>
       </c>
       <c r="F123" t="n">
-        <v>7074115.140040115</v>
+        <v>7068505.621716497</v>
       </c>
       <c r="G123" t="n">
-        <v>2946881.140040115</v>
+        <v>2941271.621716497</v>
       </c>
       <c r="H123" t="n">
-        <v>71.40087380652793</v>
+        <v>71.26495909164579</v>
       </c>
       <c r="I123" t="inlineStr">
         <is>
-          <t>2026-03-20T15:50:28</t>
+          <t>2026-03-20T15:51:21</t>
         </is>
       </c>
     </row>
@@ -6208,17 +6208,17 @@
         <v>1</v>
       </c>
       <c r="F124" t="n">
-        <v>6891186.719841287</v>
+        <v>6886743.840087891</v>
       </c>
       <c r="G124" t="n">
-        <v>2983978.719841287</v>
+        <v>2979535.840087891</v>
       </c>
       <c r="H124" t="n">
-        <v>76.37112536218412</v>
+        <v>76.25741552760668</v>
       </c>
       <c r="I124" t="inlineStr">
         <is>
-          <t>2026-03-20T15:50:28</t>
+          <t>2026-03-20T15:51:21</t>
         </is>
       </c>
     </row>
@@ -6245,17 +6245,17 @@
         <v>1</v>
       </c>
       <c r="F125" t="n">
-        <v>5207446.231761038</v>
+        <v>5216422.111643851</v>
       </c>
       <c r="G125" t="n">
-        <v>1482901.231761038</v>
+        <v>1491877.111643851</v>
       </c>
       <c r="H125" t="n">
-        <v>39.81429226284119</v>
+        <v>40.05528491785844</v>
       </c>
       <c r="I125" t="inlineStr">
         <is>
-          <t>2026-03-20T15:50:28</t>
+          <t>2026-03-20T15:51:21</t>
         </is>
       </c>
     </row>
@@ -6282,17 +6282,17 @@
         <v>1</v>
       </c>
       <c r="F126" t="n">
-        <v>5179494.129107101</v>
+        <v>5172575.327271582</v>
       </c>
       <c r="G126" t="n">
-        <v>1869486.129107101</v>
+        <v>1862567.327271582</v>
       </c>
       <c r="H126" t="n">
-        <v>56.47980697046958</v>
+        <v>56.27078022988409</v>
       </c>
       <c r="I126" t="inlineStr">
         <is>
-          <t>2026-03-20T15:50:28</t>
+          <t>2026-03-20T15:51:21</t>
         </is>
       </c>
     </row>
@@ -6329,7 +6329,7 @@
       </c>
       <c r="I127" t="inlineStr">
         <is>
-          <t>2026-03-20T15:50:28</t>
+          <t>2026-03-20T15:51:21</t>
         </is>
       </c>
     </row>
@@ -6366,7 +6366,7 @@
       </c>
       <c r="I128" t="inlineStr">
         <is>
-          <t>2026-03-20T15:50:28</t>
+          <t>2026-03-20T15:51:21</t>
         </is>
       </c>
     </row>
@@ -6403,7 +6403,7 @@
       </c>
       <c r="I129" t="inlineStr">
         <is>
-          <t>2026-03-20T15:50:28</t>
+          <t>2026-03-20T15:51:21</t>
         </is>
       </c>
     </row>
@@ -6440,7 +6440,7 @@
       </c>
       <c r="I130" t="inlineStr">
         <is>
-          <t>2026-03-20T15:50:28</t>
+          <t>2026-03-20T15:51:21</t>
         </is>
       </c>
     </row>
@@ -6477,7 +6477,7 @@
       </c>
       <c r="I131" t="inlineStr">
         <is>
-          <t>2026-03-20T15:50:28</t>
+          <t>2026-03-20T15:51:21</t>
         </is>
       </c>
     </row>
@@ -6514,7 +6514,7 @@
       </c>
       <c r="I132" t="inlineStr">
         <is>
-          <t>2026-03-20T15:50:28</t>
+          <t>2026-03-20T15:51:21</t>
         </is>
       </c>
     </row>
@@ -6551,7 +6551,7 @@
       </c>
       <c r="I133" t="inlineStr">
         <is>
-          <t>2026-03-20T15:50:28</t>
+          <t>2026-03-20T15:51:21</t>
         </is>
       </c>
     </row>
@@ -6578,17 +6578,17 @@
         <v>1</v>
       </c>
       <c r="F134" t="n">
-        <v>3605124.829619369</v>
+        <v>3585190.718330247</v>
       </c>
       <c r="G134" t="n">
-        <v>2134352.829619369</v>
+        <v>2114418.718330247</v>
       </c>
       <c r="H134" t="n">
-        <v>145.1178584865206</v>
+        <v>143.7625082834217</v>
       </c>
       <c r="I134" t="inlineStr">
         <is>
-          <t>2026-03-20T15:50:28</t>
+          <t>2026-03-20T15:51:21</t>
         </is>
       </c>
     </row>
@@ -6625,7 +6625,7 @@
       </c>
       <c r="I135" t="inlineStr">
         <is>
-          <t>2026-03-20T15:50:28</t>
+          <t>2026-03-20T15:51:21</t>
         </is>
       </c>
     </row>
@@ -6652,17 +6652,17 @@
         <v>1</v>
       </c>
       <c r="F136" t="n">
-        <v>2966169.274976688</v>
+        <v>2966461.05339016</v>
       </c>
       <c r="G136" t="n">
-        <v>-224474.7250233125</v>
+        <v>-224182.9466098398</v>
       </c>
       <c r="H136" t="n">
-        <v>-7.035404922119562</v>
+        <v>-7.026260109552799</v>
       </c>
       <c r="I136" t="inlineStr">
         <is>
-          <t>2026-03-20T15:50:28</t>
+          <t>2026-03-20T15:51:21</t>
         </is>
       </c>
     </row>
@@ -6699,7 +6699,7 @@
       </c>
       <c r="I137" t="inlineStr">
         <is>
-          <t>2026-03-20T15:50:28</t>
+          <t>2026-03-20T15:51:21</t>
         </is>
       </c>
     </row>
@@ -6736,7 +6736,7 @@
       </c>
       <c r="I138" t="inlineStr">
         <is>
-          <t>2026-03-20T15:50:28</t>
+          <t>2026-03-20T15:51:21</t>
         </is>
       </c>
     </row>
@@ -6773,7 +6773,7 @@
       </c>
       <c r="I139" t="inlineStr">
         <is>
-          <t>2026-03-20T15:50:28</t>
+          <t>2026-03-20T15:51:21</t>
         </is>
       </c>
     </row>
@@ -6810,7 +6810,7 @@
       </c>
       <c r="I140" t="inlineStr">
         <is>
-          <t>2026-03-20T15:50:28</t>
+          <t>2026-03-20T15:51:21</t>
         </is>
       </c>
     </row>
@@ -6837,17 +6837,17 @@
         <v>1</v>
       </c>
       <c r="F141" t="n">
-        <v>2176078.237399444</v>
+        <v>2176695.794808984</v>
       </c>
       <c r="G141" t="n">
-        <v>112088.237399444</v>
+        <v>112705.7948089838</v>
       </c>
       <c r="H141" t="n">
-        <v>5.430657968277171</v>
+        <v>5.460578530370002</v>
       </c>
       <c r="I141" t="inlineStr">
         <is>
-          <t>2026-03-20T15:50:28</t>
+          <t>2026-03-20T15:51:21</t>
         </is>
       </c>
     </row>
@@ -6884,7 +6884,7 @@
       </c>
       <c r="I142" t="inlineStr">
         <is>
-          <t>2026-03-20T15:50:28</t>
+          <t>2026-03-20T15:51:21</t>
         </is>
       </c>
     </row>
@@ -6921,7 +6921,7 @@
       </c>
       <c r="I143" t="inlineStr">
         <is>
-          <t>2026-03-20T15:50:28</t>
+          <t>2026-03-20T15:51:21</t>
         </is>
       </c>
     </row>
@@ -6958,7 +6958,7 @@
       </c>
       <c r="I144" t="inlineStr">
         <is>
-          <t>2026-03-20T15:50:28</t>
+          <t>2026-03-20T15:51:21</t>
         </is>
       </c>
     </row>
@@ -6995,7 +6995,7 @@
       </c>
       <c r="I145" t="inlineStr">
         <is>
-          <t>2026-03-20T15:50:28</t>
+          <t>2026-03-20T15:51:21</t>
         </is>
       </c>
     </row>
@@ -7022,17 +7022,17 @@
         <v>1</v>
       </c>
       <c r="F146" t="n">
-        <v>1697189.327788772</v>
+        <v>1696441.320678405</v>
       </c>
       <c r="G146" t="n">
-        <v>382836.3277887721</v>
+        <v>382088.3206784055</v>
       </c>
       <c r="H146" t="n">
-        <v>29.1273598332238</v>
+        <v>29.0704491623183</v>
       </c>
       <c r="I146" t="inlineStr">
         <is>
-          <t>2026-03-20T15:50:28</t>
+          <t>2026-03-20T15:51:21</t>
         </is>
       </c>
     </row>
@@ -7059,17 +7059,17 @@
         <v>1</v>
       </c>
       <c r="F147" t="n">
-        <v>1681032.631006837</v>
+        <v>1679626.497480273</v>
       </c>
       <c r="G147" t="n">
-        <v>-13423.36899316264</v>
+        <v>-14829.50251972629</v>
       </c>
       <c r="H147" t="n">
-        <v>-0.7921934233265808</v>
+        <v>-0.8751777868369726</v>
       </c>
       <c r="I147" t="inlineStr">
         <is>
-          <t>2026-03-20T15:50:28</t>
+          <t>2026-03-20T15:51:21</t>
         </is>
       </c>
     </row>
@@ -7106,7 +7106,7 @@
       </c>
       <c r="I148" t="inlineStr">
         <is>
-          <t>2026-03-20T15:50:28</t>
+          <t>2026-03-20T15:51:21</t>
         </is>
       </c>
     </row>
@@ -7143,7 +7143,7 @@
       </c>
       <c r="I149" t="inlineStr">
         <is>
-          <t>2026-03-20T15:50:28</t>
+          <t>2026-03-20T15:51:21</t>
         </is>
       </c>
     </row>
@@ -7180,7 +7180,7 @@
       </c>
       <c r="I150" t="inlineStr">
         <is>
-          <t>2026-03-20T15:50:28</t>
+          <t>2026-03-20T15:51:21</t>
         </is>
       </c>
     </row>
@@ -7217,7 +7217,7 @@
       </c>
       <c r="I151" t="inlineStr">
         <is>
-          <t>2026-03-20T15:50:28</t>
+          <t>2026-03-20T15:51:21</t>
         </is>
       </c>
     </row>
@@ -7254,7 +7254,7 @@
       </c>
       <c r="I152" t="inlineStr">
         <is>
-          <t>2026-03-20T15:50:28</t>
+          <t>2026-03-20T15:51:21</t>
         </is>
       </c>
     </row>
@@ -7281,17 +7281,17 @@
         <v>1</v>
       </c>
       <c r="F153" t="n">
-        <v>848519.8631833494</v>
+        <v>849118.2118045352</v>
       </c>
       <c r="G153" t="n">
-        <v>222788.8631833494</v>
+        <v>223387.2118045352</v>
       </c>
       <c r="H153" t="n">
-        <v>35.60457499841775</v>
+        <v>35.70019893605003</v>
       </c>
       <c r="I153" t="inlineStr">
         <is>
-          <t>2026-03-20T15:50:28</t>
+          <t>2026-03-20T15:51:21</t>
         </is>
       </c>
     </row>
@@ -7318,17 +7318,17 @@
         <v>1</v>
       </c>
       <c r="F154" t="n">
-        <v>832649.0084090387</v>
+        <v>832251.0866024625</v>
       </c>
       <c r="G154" t="n">
-        <v>-183405.9915909613</v>
+        <v>-183803.9133975375</v>
       </c>
       <c r="H154" t="n">
-        <v>-18.05079366677605</v>
+        <v>-18.08995707885277</v>
       </c>
       <c r="I154" t="inlineStr">
         <is>
-          <t>2026-03-20T15:50:28</t>
+          <t>2026-03-20T15:51:21</t>
         </is>
       </c>
     </row>
@@ -7365,7 +7365,7 @@
       </c>
       <c r="I155" t="inlineStr">
         <is>
-          <t>2026-03-20T15:50:28</t>
+          <t>2026-03-20T15:51:21</t>
         </is>
       </c>
     </row>
@@ -7498,7 +7498,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>2026-03-20T15:50:28</t>
+          <t>2026-03-20T15:51:21</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: portfolio snapshot 2026-03-20 (2026-03-20T15:57:44)
</commit_message>
<xml_diff>
--- a/portfolio_auto.xlsx
+++ b/portfolio_auto.xlsx
@@ -1603,7 +1603,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2026-03-20T15:51:21</t>
+          <t>2026-03-20T15:57:44</t>
         </is>
       </c>
       <c r="E2" t="n">
@@ -5922,7 +5922,7 @@
       </c>
       <c r="I116" t="inlineStr">
         <is>
-          <t>2026-03-20T15:51:21</t>
+          <t>2026-03-20T15:57:44</t>
         </is>
       </c>
     </row>
@@ -5959,7 +5959,7 @@
       </c>
       <c r="I117" t="inlineStr">
         <is>
-          <t>2026-03-20T15:51:21</t>
+          <t>2026-03-20T15:57:44</t>
         </is>
       </c>
     </row>
@@ -5996,7 +5996,7 @@
       </c>
       <c r="I118" t="inlineStr">
         <is>
-          <t>2026-03-20T15:51:21</t>
+          <t>2026-03-20T15:57:44</t>
         </is>
       </c>
     </row>
@@ -6033,7 +6033,7 @@
       </c>
       <c r="I119" t="inlineStr">
         <is>
-          <t>2026-03-20T15:51:21</t>
+          <t>2026-03-20T15:57:44</t>
         </is>
       </c>
     </row>
@@ -6070,7 +6070,7 @@
       </c>
       <c r="I120" t="inlineStr">
         <is>
-          <t>2026-03-20T15:51:21</t>
+          <t>2026-03-20T15:57:44</t>
         </is>
       </c>
     </row>
@@ -6107,7 +6107,7 @@
       </c>
       <c r="I121" t="inlineStr">
         <is>
-          <t>2026-03-20T15:51:21</t>
+          <t>2026-03-20T15:57:44</t>
         </is>
       </c>
     </row>
@@ -6144,7 +6144,7 @@
       </c>
       <c r="I122" t="inlineStr">
         <is>
-          <t>2026-03-20T15:51:21</t>
+          <t>2026-03-20T15:57:44</t>
         </is>
       </c>
     </row>
@@ -6181,7 +6181,7 @@
       </c>
       <c r="I123" t="inlineStr">
         <is>
-          <t>2026-03-20T15:51:21</t>
+          <t>2026-03-20T15:57:44</t>
         </is>
       </c>
     </row>
@@ -6218,7 +6218,7 @@
       </c>
       <c r="I124" t="inlineStr">
         <is>
-          <t>2026-03-20T15:51:21</t>
+          <t>2026-03-20T15:57:44</t>
         </is>
       </c>
     </row>
@@ -6255,7 +6255,7 @@
       </c>
       <c r="I125" t="inlineStr">
         <is>
-          <t>2026-03-20T15:51:21</t>
+          <t>2026-03-20T15:57:44</t>
         </is>
       </c>
     </row>
@@ -6292,7 +6292,7 @@
       </c>
       <c r="I126" t="inlineStr">
         <is>
-          <t>2026-03-20T15:51:21</t>
+          <t>2026-03-20T15:57:44</t>
         </is>
       </c>
     </row>
@@ -6329,7 +6329,7 @@
       </c>
       <c r="I127" t="inlineStr">
         <is>
-          <t>2026-03-20T15:51:21</t>
+          <t>2026-03-20T15:57:44</t>
         </is>
       </c>
     </row>
@@ -6366,7 +6366,7 @@
       </c>
       <c r="I128" t="inlineStr">
         <is>
-          <t>2026-03-20T15:51:21</t>
+          <t>2026-03-20T15:57:44</t>
         </is>
       </c>
     </row>
@@ -6403,7 +6403,7 @@
       </c>
       <c r="I129" t="inlineStr">
         <is>
-          <t>2026-03-20T15:51:21</t>
+          <t>2026-03-20T15:57:44</t>
         </is>
       </c>
     </row>
@@ -6440,7 +6440,7 @@
       </c>
       <c r="I130" t="inlineStr">
         <is>
-          <t>2026-03-20T15:51:21</t>
+          <t>2026-03-20T15:57:44</t>
         </is>
       </c>
     </row>
@@ -6477,7 +6477,7 @@
       </c>
       <c r="I131" t="inlineStr">
         <is>
-          <t>2026-03-20T15:51:21</t>
+          <t>2026-03-20T15:57:44</t>
         </is>
       </c>
     </row>
@@ -6514,7 +6514,7 @@
       </c>
       <c r="I132" t="inlineStr">
         <is>
-          <t>2026-03-20T15:51:21</t>
+          <t>2026-03-20T15:57:44</t>
         </is>
       </c>
     </row>
@@ -6551,7 +6551,7 @@
       </c>
       <c r="I133" t="inlineStr">
         <is>
-          <t>2026-03-20T15:51:21</t>
+          <t>2026-03-20T15:57:44</t>
         </is>
       </c>
     </row>
@@ -6588,7 +6588,7 @@
       </c>
       <c r="I134" t="inlineStr">
         <is>
-          <t>2026-03-20T15:51:21</t>
+          <t>2026-03-20T15:57:44</t>
         </is>
       </c>
     </row>
@@ -6625,7 +6625,7 @@
       </c>
       <c r="I135" t="inlineStr">
         <is>
-          <t>2026-03-20T15:51:21</t>
+          <t>2026-03-20T15:57:44</t>
         </is>
       </c>
     </row>
@@ -6662,7 +6662,7 @@
       </c>
       <c r="I136" t="inlineStr">
         <is>
-          <t>2026-03-20T15:51:21</t>
+          <t>2026-03-20T15:57:44</t>
         </is>
       </c>
     </row>
@@ -6699,7 +6699,7 @@
       </c>
       <c r="I137" t="inlineStr">
         <is>
-          <t>2026-03-20T15:51:21</t>
+          <t>2026-03-20T15:57:44</t>
         </is>
       </c>
     </row>
@@ -6736,7 +6736,7 @@
       </c>
       <c r="I138" t="inlineStr">
         <is>
-          <t>2026-03-20T15:51:21</t>
+          <t>2026-03-20T15:57:44</t>
         </is>
       </c>
     </row>
@@ -6773,7 +6773,7 @@
       </c>
       <c r="I139" t="inlineStr">
         <is>
-          <t>2026-03-20T15:51:21</t>
+          <t>2026-03-20T15:57:44</t>
         </is>
       </c>
     </row>
@@ -6810,7 +6810,7 @@
       </c>
       <c r="I140" t="inlineStr">
         <is>
-          <t>2026-03-20T15:51:21</t>
+          <t>2026-03-20T15:57:44</t>
         </is>
       </c>
     </row>
@@ -6847,7 +6847,7 @@
       </c>
       <c r="I141" t="inlineStr">
         <is>
-          <t>2026-03-20T15:51:21</t>
+          <t>2026-03-20T15:57:44</t>
         </is>
       </c>
     </row>
@@ -6884,7 +6884,7 @@
       </c>
       <c r="I142" t="inlineStr">
         <is>
-          <t>2026-03-20T15:51:21</t>
+          <t>2026-03-20T15:57:44</t>
         </is>
       </c>
     </row>
@@ -6921,7 +6921,7 @@
       </c>
       <c r="I143" t="inlineStr">
         <is>
-          <t>2026-03-20T15:51:21</t>
+          <t>2026-03-20T15:57:44</t>
         </is>
       </c>
     </row>
@@ -6958,7 +6958,7 @@
       </c>
       <c r="I144" t="inlineStr">
         <is>
-          <t>2026-03-20T15:51:21</t>
+          <t>2026-03-20T15:57:44</t>
         </is>
       </c>
     </row>
@@ -6995,7 +6995,7 @@
       </c>
       <c r="I145" t="inlineStr">
         <is>
-          <t>2026-03-20T15:51:21</t>
+          <t>2026-03-20T15:57:44</t>
         </is>
       </c>
     </row>
@@ -7032,7 +7032,7 @@
       </c>
       <c r="I146" t="inlineStr">
         <is>
-          <t>2026-03-20T15:51:21</t>
+          <t>2026-03-20T15:57:44</t>
         </is>
       </c>
     </row>
@@ -7069,7 +7069,7 @@
       </c>
       <c r="I147" t="inlineStr">
         <is>
-          <t>2026-03-20T15:51:21</t>
+          <t>2026-03-20T15:57:44</t>
         </is>
       </c>
     </row>
@@ -7106,7 +7106,7 @@
       </c>
       <c r="I148" t="inlineStr">
         <is>
-          <t>2026-03-20T15:51:21</t>
+          <t>2026-03-20T15:57:44</t>
         </is>
       </c>
     </row>
@@ -7143,7 +7143,7 @@
       </c>
       <c r="I149" t="inlineStr">
         <is>
-          <t>2026-03-20T15:51:21</t>
+          <t>2026-03-20T15:57:44</t>
         </is>
       </c>
     </row>
@@ -7180,7 +7180,7 @@
       </c>
       <c r="I150" t="inlineStr">
         <is>
-          <t>2026-03-20T15:51:21</t>
+          <t>2026-03-20T15:57:44</t>
         </is>
       </c>
     </row>
@@ -7217,7 +7217,7 @@
       </c>
       <c r="I151" t="inlineStr">
         <is>
-          <t>2026-03-20T15:51:21</t>
+          <t>2026-03-20T15:57:44</t>
         </is>
       </c>
     </row>
@@ -7254,7 +7254,7 @@
       </c>
       <c r="I152" t="inlineStr">
         <is>
-          <t>2026-03-20T15:51:21</t>
+          <t>2026-03-20T15:57:44</t>
         </is>
       </c>
     </row>
@@ -7291,7 +7291,7 @@
       </c>
       <c r="I153" t="inlineStr">
         <is>
-          <t>2026-03-20T15:51:21</t>
+          <t>2026-03-20T15:57:44</t>
         </is>
       </c>
     </row>
@@ -7328,7 +7328,7 @@
       </c>
       <c r="I154" t="inlineStr">
         <is>
-          <t>2026-03-20T15:51:21</t>
+          <t>2026-03-20T15:57:44</t>
         </is>
       </c>
     </row>
@@ -7365,7 +7365,7 @@
       </c>
       <c r="I155" t="inlineStr">
         <is>
-          <t>2026-03-20T15:51:21</t>
+          <t>2026-03-20T15:57:44</t>
         </is>
       </c>
     </row>
@@ -7498,7 +7498,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>2026-03-20T15:51:21</t>
+          <t>2026-03-20T15:57:44</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: portfolio snapshot 2026-03-20 (2026-03-20T15:58:09)
</commit_message>
<xml_diff>
--- a/portfolio_auto.xlsx
+++ b/portfolio_auto.xlsx
@@ -1603,7 +1603,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2026-03-20T15:57:44</t>
+          <t>2026-03-20T15:58:09</t>
         </is>
       </c>
       <c r="E2" t="n">
@@ -5922,7 +5922,7 @@
       </c>
       <c r="I116" t="inlineStr">
         <is>
-          <t>2026-03-20T15:57:44</t>
+          <t>2026-03-20T15:58:09</t>
         </is>
       </c>
     </row>
@@ -5959,7 +5959,7 @@
       </c>
       <c r="I117" t="inlineStr">
         <is>
-          <t>2026-03-20T15:57:44</t>
+          <t>2026-03-20T15:58:09</t>
         </is>
       </c>
     </row>
@@ -5996,7 +5996,7 @@
       </c>
       <c r="I118" t="inlineStr">
         <is>
-          <t>2026-03-20T15:57:44</t>
+          <t>2026-03-20T15:58:09</t>
         </is>
       </c>
     </row>
@@ -6033,7 +6033,7 @@
       </c>
       <c r="I119" t="inlineStr">
         <is>
-          <t>2026-03-20T15:57:44</t>
+          <t>2026-03-20T15:58:09</t>
         </is>
       </c>
     </row>
@@ -6070,7 +6070,7 @@
       </c>
       <c r="I120" t="inlineStr">
         <is>
-          <t>2026-03-20T15:57:44</t>
+          <t>2026-03-20T15:58:09</t>
         </is>
       </c>
     </row>
@@ -6107,7 +6107,7 @@
       </c>
       <c r="I121" t="inlineStr">
         <is>
-          <t>2026-03-20T15:57:44</t>
+          <t>2026-03-20T15:58:09</t>
         </is>
       </c>
     </row>
@@ -6144,7 +6144,7 @@
       </c>
       <c r="I122" t="inlineStr">
         <is>
-          <t>2026-03-20T15:57:44</t>
+          <t>2026-03-20T15:58:09</t>
         </is>
       </c>
     </row>
@@ -6181,7 +6181,7 @@
       </c>
       <c r="I123" t="inlineStr">
         <is>
-          <t>2026-03-20T15:57:44</t>
+          <t>2026-03-20T15:58:09</t>
         </is>
       </c>
     </row>
@@ -6218,7 +6218,7 @@
       </c>
       <c r="I124" t="inlineStr">
         <is>
-          <t>2026-03-20T15:57:44</t>
+          <t>2026-03-20T15:58:09</t>
         </is>
       </c>
     </row>
@@ -6255,7 +6255,7 @@
       </c>
       <c r="I125" t="inlineStr">
         <is>
-          <t>2026-03-20T15:57:44</t>
+          <t>2026-03-20T15:58:09</t>
         </is>
       </c>
     </row>
@@ -6292,7 +6292,7 @@
       </c>
       <c r="I126" t="inlineStr">
         <is>
-          <t>2026-03-20T15:57:44</t>
+          <t>2026-03-20T15:58:09</t>
         </is>
       </c>
     </row>
@@ -6329,7 +6329,7 @@
       </c>
       <c r="I127" t="inlineStr">
         <is>
-          <t>2026-03-20T15:57:44</t>
+          <t>2026-03-20T15:58:09</t>
         </is>
       </c>
     </row>
@@ -6366,7 +6366,7 @@
       </c>
       <c r="I128" t="inlineStr">
         <is>
-          <t>2026-03-20T15:57:44</t>
+          <t>2026-03-20T15:58:09</t>
         </is>
       </c>
     </row>
@@ -6403,7 +6403,7 @@
       </c>
       <c r="I129" t="inlineStr">
         <is>
-          <t>2026-03-20T15:57:44</t>
+          <t>2026-03-20T15:58:09</t>
         </is>
       </c>
     </row>
@@ -6440,7 +6440,7 @@
       </c>
       <c r="I130" t="inlineStr">
         <is>
-          <t>2026-03-20T15:57:44</t>
+          <t>2026-03-20T15:58:09</t>
         </is>
       </c>
     </row>
@@ -6477,7 +6477,7 @@
       </c>
       <c r="I131" t="inlineStr">
         <is>
-          <t>2026-03-20T15:57:44</t>
+          <t>2026-03-20T15:58:09</t>
         </is>
       </c>
     </row>
@@ -6514,7 +6514,7 @@
       </c>
       <c r="I132" t="inlineStr">
         <is>
-          <t>2026-03-20T15:57:44</t>
+          <t>2026-03-20T15:58:09</t>
         </is>
       </c>
     </row>
@@ -6551,7 +6551,7 @@
       </c>
       <c r="I133" t="inlineStr">
         <is>
-          <t>2026-03-20T15:57:44</t>
+          <t>2026-03-20T15:58:09</t>
         </is>
       </c>
     </row>
@@ -6588,7 +6588,7 @@
       </c>
       <c r="I134" t="inlineStr">
         <is>
-          <t>2026-03-20T15:57:44</t>
+          <t>2026-03-20T15:58:09</t>
         </is>
       </c>
     </row>
@@ -6625,7 +6625,7 @@
       </c>
       <c r="I135" t="inlineStr">
         <is>
-          <t>2026-03-20T15:57:44</t>
+          <t>2026-03-20T15:58:09</t>
         </is>
       </c>
     </row>
@@ -6662,7 +6662,7 @@
       </c>
       <c r="I136" t="inlineStr">
         <is>
-          <t>2026-03-20T15:57:44</t>
+          <t>2026-03-20T15:58:09</t>
         </is>
       </c>
     </row>
@@ -6699,7 +6699,7 @@
       </c>
       <c r="I137" t="inlineStr">
         <is>
-          <t>2026-03-20T15:57:44</t>
+          <t>2026-03-20T15:58:09</t>
         </is>
       </c>
     </row>
@@ -6736,7 +6736,7 @@
       </c>
       <c r="I138" t="inlineStr">
         <is>
-          <t>2026-03-20T15:57:44</t>
+          <t>2026-03-20T15:58:09</t>
         </is>
       </c>
     </row>
@@ -6773,7 +6773,7 @@
       </c>
       <c r="I139" t="inlineStr">
         <is>
-          <t>2026-03-20T15:57:44</t>
+          <t>2026-03-20T15:58:09</t>
         </is>
       </c>
     </row>
@@ -6810,7 +6810,7 @@
       </c>
       <c r="I140" t="inlineStr">
         <is>
-          <t>2026-03-20T15:57:44</t>
+          <t>2026-03-20T15:58:09</t>
         </is>
       </c>
     </row>
@@ -6847,7 +6847,7 @@
       </c>
       <c r="I141" t="inlineStr">
         <is>
-          <t>2026-03-20T15:57:44</t>
+          <t>2026-03-20T15:58:09</t>
         </is>
       </c>
     </row>
@@ -6884,7 +6884,7 @@
       </c>
       <c r="I142" t="inlineStr">
         <is>
-          <t>2026-03-20T15:57:44</t>
+          <t>2026-03-20T15:58:09</t>
         </is>
       </c>
     </row>
@@ -6921,7 +6921,7 @@
       </c>
       <c r="I143" t="inlineStr">
         <is>
-          <t>2026-03-20T15:57:44</t>
+          <t>2026-03-20T15:58:09</t>
         </is>
       </c>
     </row>
@@ -6958,7 +6958,7 @@
       </c>
       <c r="I144" t="inlineStr">
         <is>
-          <t>2026-03-20T15:57:44</t>
+          <t>2026-03-20T15:58:09</t>
         </is>
       </c>
     </row>
@@ -6995,7 +6995,7 @@
       </c>
       <c r="I145" t="inlineStr">
         <is>
-          <t>2026-03-20T15:57:44</t>
+          <t>2026-03-20T15:58:09</t>
         </is>
       </c>
     </row>
@@ -7032,7 +7032,7 @@
       </c>
       <c r="I146" t="inlineStr">
         <is>
-          <t>2026-03-20T15:57:44</t>
+          <t>2026-03-20T15:58:09</t>
         </is>
       </c>
     </row>
@@ -7069,7 +7069,7 @@
       </c>
       <c r="I147" t="inlineStr">
         <is>
-          <t>2026-03-20T15:57:44</t>
+          <t>2026-03-20T15:58:09</t>
         </is>
       </c>
     </row>
@@ -7106,7 +7106,7 @@
       </c>
       <c r="I148" t="inlineStr">
         <is>
-          <t>2026-03-20T15:57:44</t>
+          <t>2026-03-20T15:58:09</t>
         </is>
       </c>
     </row>
@@ -7143,7 +7143,7 @@
       </c>
       <c r="I149" t="inlineStr">
         <is>
-          <t>2026-03-20T15:57:44</t>
+          <t>2026-03-20T15:58:09</t>
         </is>
       </c>
     </row>
@@ -7180,7 +7180,7 @@
       </c>
       <c r="I150" t="inlineStr">
         <is>
-          <t>2026-03-20T15:57:44</t>
+          <t>2026-03-20T15:58:09</t>
         </is>
       </c>
     </row>
@@ -7217,7 +7217,7 @@
       </c>
       <c r="I151" t="inlineStr">
         <is>
-          <t>2026-03-20T15:57:44</t>
+          <t>2026-03-20T15:58:09</t>
         </is>
       </c>
     </row>
@@ -7254,7 +7254,7 @@
       </c>
       <c r="I152" t="inlineStr">
         <is>
-          <t>2026-03-20T15:57:44</t>
+          <t>2026-03-20T15:58:09</t>
         </is>
       </c>
     </row>
@@ -7291,7 +7291,7 @@
       </c>
       <c r="I153" t="inlineStr">
         <is>
-          <t>2026-03-20T15:57:44</t>
+          <t>2026-03-20T15:58:09</t>
         </is>
       </c>
     </row>
@@ -7328,7 +7328,7 @@
       </c>
       <c r="I154" t="inlineStr">
         <is>
-          <t>2026-03-20T15:57:44</t>
+          <t>2026-03-20T15:58:09</t>
         </is>
       </c>
     </row>
@@ -7365,7 +7365,7 @@
       </c>
       <c r="I155" t="inlineStr">
         <is>
-          <t>2026-03-20T15:57:44</t>
+          <t>2026-03-20T15:58:09</t>
         </is>
       </c>
     </row>
@@ -7498,7 +7498,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>2026-03-20T15:57:44</t>
+          <t>2026-03-20T15:58:09</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: portfolio snapshot 2026-03-20 (2026-03-20T22:42:49)
</commit_message>
<xml_diff>
--- a/portfolio_auto.xlsx
+++ b/portfolio_auto.xlsx
@@ -471,11 +471,11 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>유나이티드헬스 그룹</t>
+          <t>페트로브라스 (ADR)</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>4</v>
+        <v>480</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
@@ -486,23 +486,23 @@
         <v>1</v>
       </c>
       <c r="E2" t="n">
-        <v>1679626.497480273</v>
+        <v>13499722.79590577</v>
       </c>
       <c r="F2" t="n">
-        <v>-14829.50251972629</v>
+        <v>1393173.795905769</v>
       </c>
       <c r="G2" t="n">
-        <v>-0.8751777868369726</v>
+        <v>11.507604651877</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>케이씨</t>
+          <t>AGNC 인베스트먼트</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>50</v>
+        <v>700</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
@@ -513,23 +513,23 @@
         <v>1</v>
       </c>
       <c r="E3" t="n">
-        <v>1670000</v>
+        <v>10210063.36669922</v>
       </c>
       <c r="F3" t="n">
-        <v>20500</v>
+        <v>-621950.6333007812</v>
       </c>
       <c r="G3" t="n">
-        <v>1.242800848742043</v>
+        <v>-5.741782029646391</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>하나금융지주</t>
+          <t>대한조선</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>18</v>
+        <v>100</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
@@ -540,23 +540,23 @@
         <v>1</v>
       </c>
       <c r="E4" t="n">
-        <v>2037600</v>
+        <v>9120000</v>
       </c>
       <c r="F4" t="n">
-        <v>12200</v>
+        <v>1907000</v>
       </c>
       <c r="G4" t="n">
-        <v>0.6023501530561864</v>
+        <v>26.43837515596839</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>현대제철</t>
+          <t>프론트라인</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>80</v>
+        <v>175</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -567,23 +567,23 @@
         <v>1</v>
       </c>
       <c r="E5" t="n">
-        <v>2996000</v>
+        <v>8421992.815680243</v>
       </c>
       <c r="F5" t="n">
-        <v>-182000</v>
+        <v>3992128.815680243</v>
       </c>
       <c r="G5" t="n">
-        <v>-5.726872246696035</v>
+        <v>90.11854123919477</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>휴스틸</t>
+          <t>시드릴</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>500</v>
+        <v>123</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
@@ -594,23 +594,23 @@
         <v>1</v>
       </c>
       <c r="E6" t="n">
-        <v>2750000</v>
+        <v>8022641.158487644</v>
       </c>
       <c r="F6" t="n">
-        <v>471390</v>
+        <v>1572290.158487644</v>
       </c>
       <c r="G6" t="n">
-        <v>20.68761218462133</v>
+        <v>24.37526513654286</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>DL이앤씨</t>
+          <t>세아제강</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>40</v>
+        <v>50</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -621,23 +621,23 @@
         <v>1</v>
       </c>
       <c r="E7" t="n">
-        <v>2696000</v>
+        <v>7395000</v>
       </c>
       <c r="F7" t="n">
-        <v>990500</v>
+        <v>1085000</v>
       </c>
       <c r="G7" t="n">
-        <v>58.07681031955438</v>
+        <v>17.19492868462758</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>HD건설기계</t>
+          <t>센트러스 에너지</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>31</v>
+        <v>25</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
@@ -648,23 +648,23 @@
         <v>1</v>
       </c>
       <c r="E8" t="n">
-        <v>4123000</v>
+        <v>6984730.323367007</v>
       </c>
       <c r="F8" t="n">
-        <v>87904</v>
+        <v>-448125.6766329929</v>
       </c>
       <c r="G8" t="n">
-        <v>2.178485964150543</v>
+        <v>-6.028983699307412</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>KoAct 코스닥액티브</t>
+          <t>트랜스오션</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>200</v>
+        <v>750</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
@@ -675,23 +675,23 @@
         <v>1</v>
       </c>
       <c r="E9" t="n">
-        <v>2582000</v>
+        <v>6978746.3734849</v>
       </c>
       <c r="F9" t="n">
-        <v>-120000</v>
+        <v>2851512.3734849</v>
       </c>
       <c r="G9" t="n">
-        <v>-4.441154700222058</v>
+        <v>69.09015513743346</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>LX인터내셔널</t>
+          <t>노블</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>20</v>
+        <v>99</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
@@ -702,23 +702,23 @@
         <v>1</v>
       </c>
       <c r="E10" t="n">
-        <v>943000</v>
+        <v>6917845.128290389</v>
       </c>
       <c r="F10" t="n">
-        <v>4000</v>
+        <v>3010637.128290389</v>
       </c>
       <c r="G10" t="n">
-        <v>0.4259850905218318</v>
+        <v>77.05341328873172</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>NH투자증권우</t>
+          <t>타이드워터</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>2</v>
+        <v>48</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
@@ -729,23 +729,23 @@
         <v>1</v>
       </c>
       <c r="E11" t="n">
-        <v>54700</v>
+        <v>5204574.432301462</v>
       </c>
       <c r="F11" t="n">
-        <v>100</v>
+        <v>1480029.432301462</v>
       </c>
       <c r="G11" t="n">
-        <v>0.1831501831501831</v>
+        <v>39.73718755717709</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>TIME 코리아밸류업액티브</t>
+          <t>노브</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>201</v>
+        <v>185</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
@@ -756,23 +756,23 @@
         <v>1</v>
       </c>
       <c r="E12" t="n">
-        <v>4797870</v>
+        <v>5169807.700963225</v>
       </c>
       <c r="F12" t="n">
-        <v>74073</v>
+        <v>1859799.700963225</v>
       </c>
       <c r="G12" t="n">
-        <v>1.568081778281328</v>
+        <v>56.18716634410627</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>프론트라인</t>
+          <t>TIME 코리아밸류업액티브</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>175</v>
+        <v>201</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
@@ -783,19 +783,19 @@
         <v>1</v>
       </c>
       <c r="E13" t="n">
-        <v>8445554.540319601</v>
+        <v>4797870</v>
       </c>
       <c r="F13" t="n">
-        <v>4015690.540319601</v>
+        <v>74073</v>
       </c>
       <c r="G13" t="n">
-        <v>90.65042494125331</v>
+        <v>1.568081778281328</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>피바디 에너지</t>
+          <t>오케아니스 에코 탱커스</t>
         </is>
       </c>
       <c r="B14" t="n">
@@ -810,23 +810,23 @@
         <v>1</v>
       </c>
       <c r="E14" t="n">
-        <v>3585190.718330247</v>
+        <v>4484648.681587083</v>
       </c>
       <c r="F14" t="n">
-        <v>2114418.718330247</v>
+        <v>2228288.681587083</v>
       </c>
       <c r="G14" t="n">
-        <v>143.7625082834217</v>
+        <v>98.7559024972559</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>하프니아</t>
+          <t>삼성화재</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>80</v>
+        <v>9</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
@@ -837,23 +837,23 @@
         <v>1</v>
       </c>
       <c r="E15" t="n">
-        <v>849118.2118045352</v>
+        <v>4270500</v>
       </c>
       <c r="F15" t="n">
-        <v>223387.2118045352</v>
+        <v>-360500</v>
       </c>
       <c r="G15" t="n">
-        <v>35.70019893605003</v>
+        <v>-7.784495789246384</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>AGNC 인베스트먼트</t>
+          <t>동원개발</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>700</v>
+        <v>1360</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
@@ -864,23 +864,23 @@
         <v>1</v>
       </c>
       <c r="E16" t="n">
-        <v>10340961.61499023</v>
+        <v>4202400</v>
       </c>
       <c r="F16" t="n">
-        <v>-491052.3850097656</v>
+        <v>465000</v>
       </c>
       <c r="G16" t="n">
-        <v>-4.53334333771878</v>
+        <v>12.44180446299566</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>넥스틸</t>
+          <t>HD건설기계</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>300</v>
+        <v>31</v>
       </c>
       <c r="C17" t="inlineStr">
         <is>
@@ -891,23 +891,23 @@
         <v>1</v>
       </c>
       <c r="E17" t="n">
-        <v>3771000</v>
+        <v>4123000</v>
       </c>
       <c r="F17" t="n">
-        <v>521000</v>
+        <v>87904</v>
       </c>
       <c r="G17" t="n">
-        <v>16.03076923076923</v>
+        <v>2.178485964150543</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>대신증권</t>
+          <t>차코스 에너지 내비게이션</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>55</v>
+        <v>75</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
@@ -918,19 +918,19 @@
         <v>1</v>
       </c>
       <c r="E18" t="n">
-        <v>2219250</v>
+        <v>4003242.461974639</v>
       </c>
       <c r="F18" t="n">
-        <v>509749</v>
+        <v>178594.4619746394</v>
       </c>
       <c r="G18" t="n">
-        <v>29.81858448752005</v>
+        <v>4.669565982925473</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>대창단조</t>
+          <t>넥스틸</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -945,23 +945,23 @@
         <v>1</v>
       </c>
       <c r="E19" t="n">
-        <v>2004000</v>
+        <v>3771000</v>
       </c>
       <c r="F19" t="n">
-        <v>-54000</v>
+        <v>521000</v>
       </c>
       <c r="G19" t="n">
-        <v>-2.623906705539359</v>
+        <v>16.03076923076923</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>대한조선</t>
+          <t>피바디 에너지</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>100</v>
+        <v>65</v>
       </c>
       <c r="C20" t="inlineStr">
         <is>
@@ -972,23 +972,23 @@
         <v>1</v>
       </c>
       <c r="E20" t="n">
-        <v>9120000</v>
+        <v>3627975.98317082</v>
       </c>
       <c r="F20" t="n">
-        <v>1907000</v>
+        <v>2157203.98317082</v>
       </c>
       <c r="G20" t="n">
-        <v>26.43837515596839</v>
+        <v>146.67154277963</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>동방</t>
+          <t>현대제철</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>681</v>
+        <v>80</v>
       </c>
       <c r="C21" t="inlineStr">
         <is>
@@ -999,23 +999,23 @@
         <v>1</v>
       </c>
       <c r="E21" t="n">
-        <v>1995330</v>
+        <v>2996000</v>
       </c>
       <c r="F21" t="n">
-        <v>23829</v>
+        <v>-182000</v>
       </c>
       <c r="G21" t="n">
-        <v>1.208672985709873</v>
+        <v>-5.726872246696035</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>동원개발</t>
+          <t>더치 브로스</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>1360</v>
+        <v>39</v>
       </c>
       <c r="C22" t="inlineStr">
         <is>
@@ -1026,23 +1026,23 @@
         <v>1</v>
       </c>
       <c r="E22" t="n">
-        <v>4202400</v>
+        <v>2917160.961914062</v>
       </c>
       <c r="F22" t="n">
-        <v>465000</v>
+        <v>-273483.0380859375</v>
       </c>
       <c r="G22" t="n">
-        <v>12.44180446299566</v>
+        <v>-8.571405587271332</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>미창석유</t>
+          <t>휴스틸</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>18</v>
+        <v>500</v>
       </c>
       <c r="C23" t="inlineStr">
         <is>
@@ -1053,23 +1053,23 @@
         <v>1</v>
       </c>
       <c r="E23" t="n">
-        <v>2097000</v>
+        <v>2750000</v>
       </c>
       <c r="F23" t="n">
-        <v>-295200</v>
+        <v>471390</v>
       </c>
       <c r="G23" t="n">
-        <v>-12.34010534236268</v>
+        <v>20.68761218462133</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>비에이치아이</t>
+          <t>DL이앤씨</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>8</v>
+        <v>40</v>
       </c>
       <c r="C24" t="inlineStr">
         <is>
@@ -1080,23 +1080,23 @@
         <v>1</v>
       </c>
       <c r="E24" t="n">
-        <v>876000</v>
+        <v>2696000</v>
       </c>
       <c r="F24" t="n">
-        <v>210885</v>
+        <v>990500</v>
       </c>
       <c r="G24" t="n">
-        <v>31.70654698811484</v>
+        <v>58.07681031955438</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>삼성생명</t>
+          <t>KoAct 코스닥액티브</t>
         </is>
       </c>
       <c r="B25" t="n">
-        <v>4</v>
+        <v>200</v>
       </c>
       <c r="C25" t="inlineStr">
         <is>
@@ -1107,23 +1107,23 @@
         <v>1</v>
       </c>
       <c r="E25" t="n">
-        <v>926000</v>
+        <v>2582000</v>
       </c>
       <c r="F25" t="n">
-        <v>93000</v>
+        <v>-120000</v>
       </c>
       <c r="G25" t="n">
-        <v>11.16446578631453</v>
+        <v>-4.441154700222058</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>삼성화재</t>
+          <t>대신증권</t>
         </is>
       </c>
       <c r="B26" t="n">
-        <v>9</v>
+        <v>55</v>
       </c>
       <c r="C26" t="inlineStr">
         <is>
@@ -1134,23 +1134,23 @@
         <v>1</v>
       </c>
       <c r="E26" t="n">
-        <v>4270500</v>
+        <v>2219250</v>
       </c>
       <c r="F26" t="n">
-        <v>-360500</v>
+        <v>509749</v>
       </c>
       <c r="G26" t="n">
-        <v>-7.784495789246384</v>
+        <v>29.81858448752005</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>세아제강</t>
+          <t>발레로 에너지</t>
         </is>
       </c>
       <c r="B27" t="n">
-        <v>50</v>
+        <v>6</v>
       </c>
       <c r="C27" t="inlineStr">
         <is>
@@ -1161,23 +1161,23 @@
         <v>1</v>
       </c>
       <c r="E27" t="n">
-        <v>7395000</v>
+        <v>2152954.554169849</v>
       </c>
       <c r="F27" t="n">
-        <v>1085000</v>
+        <v>88964.55416984856</v>
       </c>
       <c r="G27" t="n">
-        <v>17.19492868462758</v>
+        <v>4.310319050472558</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>노브</t>
+          <t>미창석유</t>
         </is>
       </c>
       <c r="B28" t="n">
-        <v>185</v>
+        <v>18</v>
       </c>
       <c r="C28" t="inlineStr">
         <is>
@@ -1188,23 +1188,23 @@
         <v>1</v>
       </c>
       <c r="E28" t="n">
-        <v>5172575.327271582</v>
+        <v>2097000</v>
       </c>
       <c r="F28" t="n">
-        <v>1862567.327271582</v>
+        <v>-295200</v>
       </c>
       <c r="G28" t="n">
-        <v>56.27078022988409</v>
+        <v>-12.34010534236268</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>노블</t>
+          <t>하나금융지주</t>
         </is>
       </c>
       <c r="B29" t="n">
-        <v>99</v>
+        <v>18</v>
       </c>
       <c r="C29" t="inlineStr">
         <is>
@@ -1215,23 +1215,23 @@
         <v>1</v>
       </c>
       <c r="E29" t="n">
-        <v>6886743.840087891</v>
+        <v>2037600</v>
       </c>
       <c r="F29" t="n">
-        <v>2979535.840087891</v>
+        <v>12200</v>
       </c>
       <c r="G29" t="n">
-        <v>76.25741552760668</v>
+        <v>0.6023501530561864</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>더치 브로스</t>
+          <t>대창단조</t>
         </is>
       </c>
       <c r="B30" t="n">
-        <v>39</v>
+        <v>300</v>
       </c>
       <c r="C30" t="inlineStr">
         <is>
@@ -1242,23 +1242,23 @@
         <v>1</v>
       </c>
       <c r="E30" t="n">
-        <v>2966461.05339016</v>
+        <v>2004000</v>
       </c>
       <c r="F30" t="n">
-        <v>-224182.9466098398</v>
+        <v>-54000</v>
       </c>
       <c r="G30" t="n">
-        <v>-7.026260109552799</v>
+        <v>-2.623906705539359</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>발레로 에너지</t>
+          <t>동방</t>
         </is>
       </c>
       <c r="B31" t="n">
-        <v>6</v>
+        <v>681</v>
       </c>
       <c r="C31" t="inlineStr">
         <is>
@@ -1269,23 +1269,23 @@
         <v>1</v>
       </c>
       <c r="E31" t="n">
-        <v>2176695.794808984</v>
+        <v>1995330</v>
       </c>
       <c r="F31" t="n">
-        <v>112705.7948089838</v>
+        <v>23829</v>
       </c>
       <c r="G31" t="n">
-        <v>5.460578530370002</v>
+        <v>1.208672985709873</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>센트러스 에너지</t>
+          <t>스타 벌크 캐리어스</t>
         </is>
       </c>
       <c r="B32" t="n">
-        <v>25</v>
+        <v>50</v>
       </c>
       <c r="C32" t="inlineStr">
         <is>
@@ -1296,23 +1296,23 @@
         <v>1</v>
       </c>
       <c r="E32" t="n">
-        <v>7118620.600099489</v>
+        <v>1670261.642486649</v>
       </c>
       <c r="F32" t="n">
-        <v>-314235.3999005109</v>
+        <v>355908.6424866486</v>
       </c>
       <c r="G32" t="n">
-        <v>-4.227653541256697</v>
+        <v>27.07861909902809</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>스타 벌크 캐리어스</t>
+          <t>유나이티드헬스 그룹</t>
         </is>
       </c>
       <c r="B33" t="n">
-        <v>50</v>
+        <v>4</v>
       </c>
       <c r="C33" t="inlineStr">
         <is>
@@ -1323,23 +1323,23 @@
         <v>1</v>
       </c>
       <c r="E33" t="n">
-        <v>1696441.320678405</v>
+        <v>1649108.469355762</v>
       </c>
       <c r="F33" t="n">
-        <v>382088.3206784055</v>
+        <v>-45347.53064423753</v>
       </c>
       <c r="G33" t="n">
-        <v>29.0704491623183</v>
+        <v>-2.676229459144265</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>시드릴</t>
+          <t>케이씨</t>
         </is>
       </c>
       <c r="B34" t="n">
-        <v>123</v>
+        <v>50</v>
       </c>
       <c r="C34" t="inlineStr">
         <is>
@@ -1350,23 +1350,23 @@
         <v>1</v>
       </c>
       <c r="E34" t="n">
-        <v>8054842.689107571</v>
+        <v>1670000</v>
       </c>
       <c r="F34" t="n">
-        <v>1604491.689107571</v>
+        <v>20500</v>
       </c>
       <c r="G34" t="n">
-        <v>24.87448650635556</v>
+        <v>1.242800848742043</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>오케아니스 에코 탱커스</t>
+          <t>텍사스 퍼시픽 랜드</t>
         </is>
       </c>
       <c r="B35" t="n">
-        <v>65</v>
+        <v>2</v>
       </c>
       <c r="C35" t="inlineStr">
         <is>
@@ -1377,23 +1377,23 @@
         <v>1</v>
       </c>
       <c r="E35" t="n">
-        <v>4579942.561830599</v>
+        <v>1554053.84296006</v>
       </c>
       <c r="F35" t="n">
-        <v>2323582.561830599</v>
+        <v>-23841.15703994036</v>
       </c>
       <c r="G35" t="n">
-        <v>102.9792480734723</v>
+        <v>-1.510946992033079</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>차코스 에너지 내비게이션</t>
+          <t>LX인터내셔널</t>
         </is>
       </c>
       <c r="B36" t="n">
-        <v>75</v>
+        <v>20</v>
       </c>
       <c r="C36" t="inlineStr">
         <is>
@@ -1404,23 +1404,23 @@
         <v>1</v>
       </c>
       <c r="E36" t="n">
-        <v>4054853.668580018</v>
+        <v>943000</v>
       </c>
       <c r="F36" t="n">
-        <v>230205.668580018</v>
+        <v>4000</v>
       </c>
       <c r="G36" t="n">
-        <v>6.019002757378404</v>
+        <v>0.4259850905218318</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>클리블랜드 클리프스</t>
+          <t>삼성생명</t>
         </is>
       </c>
       <c r="B37" t="n">
-        <v>70</v>
+        <v>4</v>
       </c>
       <c r="C37" t="inlineStr">
         <is>
@@ -1431,23 +1431,23 @@
         <v>1</v>
       </c>
       <c r="E37" t="n">
-        <v>832251.0866024625</v>
+        <v>926000</v>
       </c>
       <c r="F37" t="n">
-        <v>-183803.9133975375</v>
+        <v>93000</v>
       </c>
       <c r="G37" t="n">
-        <v>-18.08995707885277</v>
+        <v>11.16446578631453</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>타이드워터</t>
+          <t>비에이치아이</t>
         </is>
       </c>
       <c r="B38" t="n">
-        <v>48</v>
+        <v>8</v>
       </c>
       <c r="C38" t="inlineStr">
         <is>
@@ -1458,23 +1458,23 @@
         <v>1</v>
       </c>
       <c r="E38" t="n">
-        <v>5216422.111643851</v>
+        <v>876000</v>
       </c>
       <c r="F38" t="n">
-        <v>1491877.111643851</v>
+        <v>210885</v>
       </c>
       <c r="G38" t="n">
-        <v>40.05528491785844</v>
+        <v>31.70654698811484</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>텍사스 퍼시픽 랜드</t>
+          <t>하프니아</t>
         </is>
       </c>
       <c r="B39" t="n">
-        <v>2</v>
+        <v>80</v>
       </c>
       <c r="C39" t="inlineStr">
         <is>
@@ -1485,23 +1485,23 @@
         <v>1</v>
       </c>
       <c r="E39" t="n">
-        <v>1600937.987030566</v>
+        <v>837748.7890625</v>
       </c>
       <c r="F39" t="n">
-        <v>23042.98703056574</v>
+        <v>212017.7890625</v>
       </c>
       <c r="G39" t="n">
-        <v>1.460362510215556</v>
+        <v>33.88321644005172</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>트랜스오션</t>
+          <t>클리블랜드 클리프스</t>
         </is>
       </c>
       <c r="B40" t="n">
-        <v>750</v>
+        <v>70</v>
       </c>
       <c r="C40" t="inlineStr">
         <is>
@@ -1512,23 +1512,23 @@
         <v>1</v>
       </c>
       <c r="E40" t="n">
-        <v>7068505.621716497</v>
+        <v>818899.4592847326</v>
       </c>
       <c r="F40" t="n">
-        <v>2941271.621716497</v>
+        <v>-197155.5407152674</v>
       </c>
       <c r="G40" t="n">
-        <v>71.26495909164579</v>
+        <v>-19.40402249044269</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>페트로브라스 (ADR)</t>
+          <t>NH투자증권우</t>
         </is>
       </c>
       <c r="B41" t="n">
-        <v>480</v>
+        <v>2</v>
       </c>
       <c r="C41" t="inlineStr">
         <is>
@@ -1539,13 +1539,13 @@
         <v>1</v>
       </c>
       <c r="E41" t="n">
-        <v>13542808.00546288</v>
+        <v>54700</v>
       </c>
       <c r="F41" t="n">
-        <v>1436259.005462885</v>
+        <v>100</v>
       </c>
       <c r="G41" t="n">
-        <v>11.86348814565476</v>
+        <v>0.1831501831501831</v>
       </c>
     </row>
   </sheetData>
@@ -1603,7 +1603,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2026-03-20T15:58:09</t>
+          <t>2026-03-20T22:42:49</t>
         </is>
       </c>
       <c r="E2" t="n">
@@ -5912,17 +5912,17 @@
         <v>1</v>
       </c>
       <c r="F116" t="n">
-        <v>13542808.00546288</v>
+        <v>13499722.79590577</v>
       </c>
       <c r="G116" t="n">
-        <v>1436259.005462885</v>
+        <v>1393173.795905769</v>
       </c>
       <c r="H116" t="n">
-        <v>11.86348814565476</v>
+        <v>11.507604651877</v>
       </c>
       <c r="I116" t="inlineStr">
         <is>
-          <t>2026-03-20T15:58:09</t>
+          <t>2026-03-20T22:42:49</t>
         </is>
       </c>
     </row>
@@ -5949,17 +5949,17 @@
         <v>1</v>
       </c>
       <c r="F117" t="n">
-        <v>10340961.61499023</v>
+        <v>10210063.36669922</v>
       </c>
       <c r="G117" t="n">
-        <v>-491052.3850097656</v>
+        <v>-621950.6333007812</v>
       </c>
       <c r="H117" t="n">
-        <v>-4.53334333771878</v>
+        <v>-5.741782029646391</v>
       </c>
       <c r="I117" t="inlineStr">
         <is>
-          <t>2026-03-20T15:58:09</t>
+          <t>2026-03-20T22:42:49</t>
         </is>
       </c>
     </row>
@@ -5996,7 +5996,7 @@
       </c>
       <c r="I118" t="inlineStr">
         <is>
-          <t>2026-03-20T15:58:09</t>
+          <t>2026-03-20T22:42:49</t>
         </is>
       </c>
     </row>
@@ -6023,17 +6023,17 @@
         <v>1</v>
       </c>
       <c r="F119" t="n">
-        <v>8445554.540319601</v>
+        <v>8421992.815680243</v>
       </c>
       <c r="G119" t="n">
-        <v>4015690.540319601</v>
+        <v>3992128.815680243</v>
       </c>
       <c r="H119" t="n">
-        <v>90.65042494125331</v>
+        <v>90.11854123919477</v>
       </c>
       <c r="I119" t="inlineStr">
         <is>
-          <t>2026-03-20T15:58:09</t>
+          <t>2026-03-20T22:42:49</t>
         </is>
       </c>
     </row>
@@ -6060,17 +6060,17 @@
         <v>1</v>
       </c>
       <c r="F120" t="n">
-        <v>8054842.689107571</v>
+        <v>8022641.158487644</v>
       </c>
       <c r="G120" t="n">
-        <v>1604491.689107571</v>
+        <v>1572290.158487644</v>
       </c>
       <c r="H120" t="n">
-        <v>24.87448650635556</v>
+        <v>24.37526513654286</v>
       </c>
       <c r="I120" t="inlineStr">
         <is>
-          <t>2026-03-20T15:58:09</t>
+          <t>2026-03-20T22:42:49</t>
         </is>
       </c>
     </row>
@@ -6107,7 +6107,7 @@
       </c>
       <c r="I121" t="inlineStr">
         <is>
-          <t>2026-03-20T15:58:09</t>
+          <t>2026-03-20T22:42:49</t>
         </is>
       </c>
     </row>
@@ -6134,17 +6134,17 @@
         <v>1</v>
       </c>
       <c r="F122" t="n">
-        <v>7118620.600099489</v>
+        <v>6984730.323367007</v>
       </c>
       <c r="G122" t="n">
-        <v>-314235.3999005109</v>
+        <v>-448125.6766329929</v>
       </c>
       <c r="H122" t="n">
-        <v>-4.227653541256697</v>
+        <v>-6.028983699307412</v>
       </c>
       <c r="I122" t="inlineStr">
         <is>
-          <t>2026-03-20T15:58:09</t>
+          <t>2026-03-20T22:42:49</t>
         </is>
       </c>
     </row>
@@ -6171,17 +6171,17 @@
         <v>1</v>
       </c>
       <c r="F123" t="n">
-        <v>7068505.621716497</v>
+        <v>6978746.3734849</v>
       </c>
       <c r="G123" t="n">
-        <v>2941271.621716497</v>
+        <v>2851512.3734849</v>
       </c>
       <c r="H123" t="n">
-        <v>71.26495909164579</v>
+        <v>69.09015513743346</v>
       </c>
       <c r="I123" t="inlineStr">
         <is>
-          <t>2026-03-20T15:58:09</t>
+          <t>2026-03-20T22:42:49</t>
         </is>
       </c>
     </row>
@@ -6208,17 +6208,17 @@
         <v>1</v>
       </c>
       <c r="F124" t="n">
-        <v>6886743.840087891</v>
+        <v>6917845.128290389</v>
       </c>
       <c r="G124" t="n">
-        <v>2979535.840087891</v>
+        <v>3010637.128290389</v>
       </c>
       <c r="H124" t="n">
-        <v>76.25741552760668</v>
+        <v>77.05341328873172</v>
       </c>
       <c r="I124" t="inlineStr">
         <is>
-          <t>2026-03-20T15:58:09</t>
+          <t>2026-03-20T22:42:49</t>
         </is>
       </c>
     </row>
@@ -6245,17 +6245,17 @@
         <v>1</v>
       </c>
       <c r="F125" t="n">
-        <v>5216422.111643851</v>
+        <v>5204574.432301462</v>
       </c>
       <c r="G125" t="n">
-        <v>1491877.111643851</v>
+        <v>1480029.432301462</v>
       </c>
       <c r="H125" t="n">
-        <v>40.05528491785844</v>
+        <v>39.73718755717709</v>
       </c>
       <c r="I125" t="inlineStr">
         <is>
-          <t>2026-03-20T15:58:09</t>
+          <t>2026-03-20T22:42:49</t>
         </is>
       </c>
     </row>
@@ -6282,17 +6282,17 @@
         <v>1</v>
       </c>
       <c r="F126" t="n">
-        <v>5172575.327271582</v>
+        <v>5169807.700963225</v>
       </c>
       <c r="G126" t="n">
-        <v>1862567.327271582</v>
+        <v>1859799.700963225</v>
       </c>
       <c r="H126" t="n">
-        <v>56.27078022988409</v>
+        <v>56.18716634410627</v>
       </c>
       <c r="I126" t="inlineStr">
         <is>
-          <t>2026-03-20T15:58:09</t>
+          <t>2026-03-20T22:42:49</t>
         </is>
       </c>
     </row>
@@ -6329,7 +6329,7 @@
       </c>
       <c r="I127" t="inlineStr">
         <is>
-          <t>2026-03-20T15:58:09</t>
+          <t>2026-03-20T22:42:49</t>
         </is>
       </c>
     </row>
@@ -6356,17 +6356,17 @@
         <v>1</v>
       </c>
       <c r="F128" t="n">
-        <v>4579942.561830599</v>
+        <v>4484648.681587083</v>
       </c>
       <c r="G128" t="n">
-        <v>2323582.561830599</v>
+        <v>2228288.681587083</v>
       </c>
       <c r="H128" t="n">
-        <v>102.9792480734723</v>
+        <v>98.7559024972559</v>
       </c>
       <c r="I128" t="inlineStr">
         <is>
-          <t>2026-03-20T15:58:09</t>
+          <t>2026-03-20T22:42:49</t>
         </is>
       </c>
     </row>
@@ -6403,7 +6403,7 @@
       </c>
       <c r="I129" t="inlineStr">
         <is>
-          <t>2026-03-20T15:58:09</t>
+          <t>2026-03-20T22:42:49</t>
         </is>
       </c>
     </row>
@@ -6440,7 +6440,7 @@
       </c>
       <c r="I130" t="inlineStr">
         <is>
-          <t>2026-03-20T15:58:09</t>
+          <t>2026-03-20T22:42:49</t>
         </is>
       </c>
     </row>
@@ -6477,7 +6477,7 @@
       </c>
       <c r="I131" t="inlineStr">
         <is>
-          <t>2026-03-20T15:58:09</t>
+          <t>2026-03-20T22:42:49</t>
         </is>
       </c>
     </row>
@@ -6504,17 +6504,17 @@
         <v>1</v>
       </c>
       <c r="F132" t="n">
-        <v>4054853.668580018</v>
+        <v>4003242.461974639</v>
       </c>
       <c r="G132" t="n">
-        <v>230205.668580018</v>
+        <v>178594.4619746394</v>
       </c>
       <c r="H132" t="n">
-        <v>6.019002757378404</v>
+        <v>4.669565982925473</v>
       </c>
       <c r="I132" t="inlineStr">
         <is>
-          <t>2026-03-20T15:58:09</t>
+          <t>2026-03-20T22:42:49</t>
         </is>
       </c>
     </row>
@@ -6551,7 +6551,7 @@
       </c>
       <c r="I133" t="inlineStr">
         <is>
-          <t>2026-03-20T15:58:09</t>
+          <t>2026-03-20T22:42:49</t>
         </is>
       </c>
     </row>
@@ -6578,17 +6578,17 @@
         <v>1</v>
       </c>
       <c r="F134" t="n">
-        <v>3585190.718330247</v>
+        <v>3627975.98317082</v>
       </c>
       <c r="G134" t="n">
-        <v>2114418.718330247</v>
+        <v>2157203.98317082</v>
       </c>
       <c r="H134" t="n">
-        <v>143.7625082834217</v>
+        <v>146.67154277963</v>
       </c>
       <c r="I134" t="inlineStr">
         <is>
-          <t>2026-03-20T15:58:09</t>
+          <t>2026-03-20T22:42:49</t>
         </is>
       </c>
     </row>
@@ -6625,7 +6625,7 @@
       </c>
       <c r="I135" t="inlineStr">
         <is>
-          <t>2026-03-20T15:58:09</t>
+          <t>2026-03-20T22:42:49</t>
         </is>
       </c>
     </row>
@@ -6652,17 +6652,17 @@
         <v>1</v>
       </c>
       <c r="F136" t="n">
-        <v>2966461.05339016</v>
+        <v>2917160.961914062</v>
       </c>
       <c r="G136" t="n">
-        <v>-224182.9466098398</v>
+        <v>-273483.0380859375</v>
       </c>
       <c r="H136" t="n">
-        <v>-7.026260109552799</v>
+        <v>-8.571405587271332</v>
       </c>
       <c r="I136" t="inlineStr">
         <is>
-          <t>2026-03-20T15:58:09</t>
+          <t>2026-03-20T22:42:49</t>
         </is>
       </c>
     </row>
@@ -6699,7 +6699,7 @@
       </c>
       <c r="I137" t="inlineStr">
         <is>
-          <t>2026-03-20T15:58:09</t>
+          <t>2026-03-20T22:42:49</t>
         </is>
       </c>
     </row>
@@ -6736,7 +6736,7 @@
       </c>
       <c r="I138" t="inlineStr">
         <is>
-          <t>2026-03-20T15:58:09</t>
+          <t>2026-03-20T22:42:49</t>
         </is>
       </c>
     </row>
@@ -6773,7 +6773,7 @@
       </c>
       <c r="I139" t="inlineStr">
         <is>
-          <t>2026-03-20T15:58:09</t>
+          <t>2026-03-20T22:42:49</t>
         </is>
       </c>
     </row>
@@ -6810,7 +6810,7 @@
       </c>
       <c r="I140" t="inlineStr">
         <is>
-          <t>2026-03-20T15:58:09</t>
+          <t>2026-03-20T22:42:49</t>
         </is>
       </c>
     </row>
@@ -6837,17 +6837,17 @@
         <v>1</v>
       </c>
       <c r="F141" t="n">
-        <v>2176695.794808984</v>
+        <v>2152954.554169849</v>
       </c>
       <c r="G141" t="n">
-        <v>112705.7948089838</v>
+        <v>88964.55416984856</v>
       </c>
       <c r="H141" t="n">
-        <v>5.460578530370002</v>
+        <v>4.310319050472558</v>
       </c>
       <c r="I141" t="inlineStr">
         <is>
-          <t>2026-03-20T15:58:09</t>
+          <t>2026-03-20T22:42:49</t>
         </is>
       </c>
     </row>
@@ -6884,7 +6884,7 @@
       </c>
       <c r="I142" t="inlineStr">
         <is>
-          <t>2026-03-20T15:58:09</t>
+          <t>2026-03-20T22:42:49</t>
         </is>
       </c>
     </row>
@@ -6921,7 +6921,7 @@
       </c>
       <c r="I143" t="inlineStr">
         <is>
-          <t>2026-03-20T15:58:09</t>
+          <t>2026-03-20T22:42:49</t>
         </is>
       </c>
     </row>
@@ -6958,7 +6958,7 @@
       </c>
       <c r="I144" t="inlineStr">
         <is>
-          <t>2026-03-20T15:58:09</t>
+          <t>2026-03-20T22:42:49</t>
         </is>
       </c>
     </row>
@@ -6995,7 +6995,7 @@
       </c>
       <c r="I145" t="inlineStr">
         <is>
-          <t>2026-03-20T15:58:09</t>
+          <t>2026-03-20T22:42:49</t>
         </is>
       </c>
     </row>
@@ -7022,17 +7022,17 @@
         <v>1</v>
       </c>
       <c r="F146" t="n">
-        <v>1696441.320678405</v>
+        <v>1670261.642486649</v>
       </c>
       <c r="G146" t="n">
-        <v>382088.3206784055</v>
+        <v>355908.6424866486</v>
       </c>
       <c r="H146" t="n">
-        <v>29.0704491623183</v>
+        <v>27.07861909902809</v>
       </c>
       <c r="I146" t="inlineStr">
         <is>
-          <t>2026-03-20T15:58:09</t>
+          <t>2026-03-20T22:42:49</t>
         </is>
       </c>
     </row>
@@ -7044,11 +7044,11 @@
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>유나이티드헬스 그룹</t>
+          <t>케이씨</t>
         </is>
       </c>
       <c r="C147" t="n">
-        <v>4</v>
+        <v>50</v>
       </c>
       <c r="D147" t="inlineStr">
         <is>
@@ -7059,17 +7059,17 @@
         <v>1</v>
       </c>
       <c r="F147" t="n">
-        <v>1679626.497480273</v>
+        <v>1670000</v>
       </c>
       <c r="G147" t="n">
-        <v>-14829.50251972629</v>
+        <v>20500</v>
       </c>
       <c r="H147" t="n">
-        <v>-0.8751777868369726</v>
+        <v>1.242800848742043</v>
       </c>
       <c r="I147" t="inlineStr">
         <is>
-          <t>2026-03-20T15:58:09</t>
+          <t>2026-03-20T22:42:49</t>
         </is>
       </c>
     </row>
@@ -7081,11 +7081,11 @@
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>케이씨</t>
+          <t>유나이티드헬스 그룹</t>
         </is>
       </c>
       <c r="C148" t="n">
-        <v>50</v>
+        <v>4</v>
       </c>
       <c r="D148" t="inlineStr">
         <is>
@@ -7096,17 +7096,17 @@
         <v>1</v>
       </c>
       <c r="F148" t="n">
-        <v>1670000</v>
+        <v>1649108.469355762</v>
       </c>
       <c r="G148" t="n">
-        <v>20500</v>
+        <v>-45347.53064423753</v>
       </c>
       <c r="H148" t="n">
-        <v>1.242800848742043</v>
+        <v>-2.676229459144265</v>
       </c>
       <c r="I148" t="inlineStr">
         <is>
-          <t>2026-03-20T15:58:09</t>
+          <t>2026-03-20T22:42:49</t>
         </is>
       </c>
     </row>
@@ -7133,17 +7133,17 @@
         <v>1</v>
       </c>
       <c r="F149" t="n">
-        <v>1600937.987030566</v>
+        <v>1554053.84296006</v>
       </c>
       <c r="G149" t="n">
-        <v>23042.98703056574</v>
+        <v>-23841.15703994036</v>
       </c>
       <c r="H149" t="n">
-        <v>1.460362510215556</v>
+        <v>-1.510946992033079</v>
       </c>
       <c r="I149" t="inlineStr">
         <is>
-          <t>2026-03-20T15:58:09</t>
+          <t>2026-03-20T22:42:49</t>
         </is>
       </c>
     </row>
@@ -7180,7 +7180,7 @@
       </c>
       <c r="I150" t="inlineStr">
         <is>
-          <t>2026-03-20T15:58:09</t>
+          <t>2026-03-20T22:42:49</t>
         </is>
       </c>
     </row>
@@ -7217,7 +7217,7 @@
       </c>
       <c r="I151" t="inlineStr">
         <is>
-          <t>2026-03-20T15:58:09</t>
+          <t>2026-03-20T22:42:49</t>
         </is>
       </c>
     </row>
@@ -7254,7 +7254,7 @@
       </c>
       <c r="I152" t="inlineStr">
         <is>
-          <t>2026-03-20T15:58:09</t>
+          <t>2026-03-20T22:42:49</t>
         </is>
       </c>
     </row>
@@ -7281,17 +7281,17 @@
         <v>1</v>
       </c>
       <c r="F153" t="n">
-        <v>849118.2118045352</v>
+        <v>837748.7890625</v>
       </c>
       <c r="G153" t="n">
-        <v>223387.2118045352</v>
+        <v>212017.7890625</v>
       </c>
       <c r="H153" t="n">
-        <v>35.70019893605003</v>
+        <v>33.88321644005172</v>
       </c>
       <c r="I153" t="inlineStr">
         <is>
-          <t>2026-03-20T15:58:09</t>
+          <t>2026-03-20T22:42:49</t>
         </is>
       </c>
     </row>
@@ -7318,17 +7318,17 @@
         <v>1</v>
       </c>
       <c r="F154" t="n">
-        <v>832251.0866024625</v>
+        <v>818899.4592847326</v>
       </c>
       <c r="G154" t="n">
-        <v>-183803.9133975375</v>
+        <v>-197155.5407152674</v>
       </c>
       <c r="H154" t="n">
-        <v>-18.08995707885277</v>
+        <v>-19.40402249044269</v>
       </c>
       <c r="I154" t="inlineStr">
         <is>
-          <t>2026-03-20T15:58:09</t>
+          <t>2026-03-20T22:42:49</t>
         </is>
       </c>
     </row>
@@ -7365,7 +7365,7 @@
       </c>
       <c r="I155" t="inlineStr">
         <is>
-          <t>2026-03-20T15:58:09</t>
+          <t>2026-03-20T22:42:49</t>
         </is>
       </c>
     </row>
@@ -7498,7 +7498,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>2026-03-20T15:58:09</t>
+          <t>2026-03-20T22:42:49</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: portfolio snapshot 2026-03-17 (2026-03-21T03:44:38)
</commit_message>
<xml_diff>
--- a/portfolio_auto.xlsx
+++ b/portfolio_auto.xlsx
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G15"/>
+  <dimension ref="A1:G29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -844,6 +844,384 @@
       </c>
       <c r="G15" t="n">
         <v>68.28057241241955</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>페트로브라스 (ADR)</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>480</v>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>1</v>
+      </c>
+      <c r="E16" t="n">
+        <v>13847377</v>
+      </c>
+      <c r="F16" t="n">
+        <v>1740828</v>
+      </c>
+      <c r="G16" t="n">
+        <v>14.37922565712161</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>프론트라인</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>175</v>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>1</v>
+      </c>
+      <c r="E17" t="n">
+        <v>8304681.999999999</v>
+      </c>
+      <c r="F17" t="n">
+        <v>3874817.999999999</v>
+      </c>
+      <c r="G17" t="n">
+        <v>87.47036026388167</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>피바디 에너지</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>65</v>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>1</v>
+      </c>
+      <c r="E18" t="n">
+        <v>3427688</v>
+      </c>
+      <c r="F18" t="n">
+        <v>1956916</v>
+      </c>
+      <c r="G18" t="n">
+        <v>133.0536616144446</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>하프니아</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>80</v>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
+        <v>1</v>
+      </c>
+      <c r="E19" t="n">
+        <v>798051</v>
+      </c>
+      <c r="F19" t="n">
+        <v>172320</v>
+      </c>
+      <c r="G19" t="n">
+        <v>27.53899039683186</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>AGNC 인베스트먼트</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>700</v>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="D20" t="n">
+        <v>1</v>
+      </c>
+      <c r="E20" t="n">
+        <v>10848269</v>
+      </c>
+      <c r="F20" t="n">
+        <v>16254</v>
+      </c>
+      <c r="G20" t="n">
+        <v>0.1500551836385012</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>넥스틸</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>200</v>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
+        <v>1</v>
+      </c>
+      <c r="E21" t="n">
+        <v>2391208</v>
+      </c>
+      <c r="F21" t="n">
+        <v>380208</v>
+      </c>
+      <c r="G21" t="n">
+        <v>18.90641471904525</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>대신증권</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>55</v>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="D22" t="n">
+        <v>1</v>
+      </c>
+      <c r="E22" t="n">
+        <v>2190111</v>
+      </c>
+      <c r="F22" t="n">
+        <v>480610</v>
+      </c>
+      <c r="G22" t="n">
+        <v>28.11405199528985</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>대창단조</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>300</v>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="D23" t="n">
+        <v>1</v>
+      </c>
+      <c r="E23" t="n">
+        <v>1901190</v>
+      </c>
+      <c r="F23" t="n">
+        <v>-156810</v>
+      </c>
+      <c r="G23" t="n">
+        <v>-7.619533527696793</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>대한조선</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>100</v>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="D24" t="n">
+        <v>1</v>
+      </c>
+      <c r="E24" t="n">
+        <v>9740480</v>
+      </c>
+      <c r="F24" t="n">
+        <v>2527480</v>
+      </c>
+      <c r="G24" t="n">
+        <v>35.04062110079024</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>동방</t>
+        </is>
+      </c>
+      <c r="B25" t="n">
+        <v>681</v>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="D25" t="n">
+        <v>1</v>
+      </c>
+      <c r="E25" t="n">
+        <v>1841600</v>
+      </c>
+      <c r="F25" t="n">
+        <v>-129901</v>
+      </c>
+      <c r="G25" t="n">
+        <v>-6.588939087527726</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>동원개발</t>
+        </is>
+      </c>
+      <c r="B26" t="n">
+        <v>1360</v>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="D26" t="n">
+        <v>1</v>
+      </c>
+      <c r="E26" t="n">
+        <v>3881821</v>
+      </c>
+      <c r="F26" t="n">
+        <v>144420.9999999995</v>
+      </c>
+      <c r="G26" t="n">
+        <v>3.86421041365654</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>미창석유</t>
+        </is>
+      </c>
+      <c r="B27" t="n">
+        <v>18</v>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="D27" t="n">
+        <v>1</v>
+      </c>
+      <c r="E27" t="n">
+        <v>2049693</v>
+      </c>
+      <c r="F27" t="n">
+        <v>-342507</v>
+      </c>
+      <c r="G27" t="n">
+        <v>-14.31765738650614</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>비에이치아이</t>
+        </is>
+      </c>
+      <c r="B28" t="n">
+        <v>8</v>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="D28" t="n">
+        <v>1</v>
+      </c>
+      <c r="E28" t="n">
+        <v>850296</v>
+      </c>
+      <c r="F28" t="n">
+        <v>185181</v>
+      </c>
+      <c r="G28" t="n">
+        <v>27.84195214361426</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>삼성생명</t>
+        </is>
+      </c>
+      <c r="B29" t="n">
+        <v>4</v>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="D29" t="n">
+        <v>1</v>
+      </c>
+      <c r="E29" t="n">
+        <v>872252</v>
+      </c>
+      <c r="F29" t="n">
+        <v>39252</v>
+      </c>
+      <c r="G29" t="n">
+        <v>4.712124849939976</v>
       </c>
     </row>
   </sheetData>
@@ -901,7 +1279,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2026-03-21T03:44:05</t>
+          <t>2026-03-21T03:44:38</t>
         </is>
       </c>
       <c r="E2" t="n">
@@ -919,7 +1297,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I15"/>
+  <dimension ref="A1:I29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -977,11 +1355,11 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>시드릴</t>
+          <t>페트로브라스 (ADR)</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>123</v>
+        <v>480</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
@@ -992,17 +1370,17 @@
         <v>1</v>
       </c>
       <c r="F2" t="n">
-        <v>7927448</v>
+        <v>13847377</v>
       </c>
       <c r="G2" t="n">
-        <v>1477097</v>
+        <v>1740828</v>
       </c>
       <c r="H2" t="n">
-        <v>22.89948252428434</v>
+        <v>14.37922565712161</v>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>2026-03-21T03:44:05</t>
+          <t>2026-03-21T03:44:38</t>
         </is>
       </c>
     </row>
@@ -1014,11 +1392,11 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>트랜스오션</t>
+          <t>AGNC 인베스트먼트</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>750</v>
+        <v>700</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
@@ -1029,17 +1407,17 @@
         <v>1</v>
       </c>
       <c r="F3" t="n">
-        <v>6945333</v>
+        <v>10848269</v>
       </c>
       <c r="G3" t="n">
-        <v>2818099</v>
+        <v>16254</v>
       </c>
       <c r="H3" t="n">
-        <v>68.28057241241955</v>
+        <v>0.1500551836385012</v>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>2026-03-21T03:44:05</t>
+          <t>2026-03-21T03:44:38</t>
         </is>
       </c>
     </row>
@@ -1051,11 +1429,11 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>노블</t>
+          <t>대한조선</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
@@ -1066,17 +1444,17 @@
         <v>1</v>
       </c>
       <c r="F4" t="n">
-        <v>6882090</v>
+        <v>9740480</v>
       </c>
       <c r="G4" t="n">
-        <v>2974882</v>
+        <v>2527480</v>
       </c>
       <c r="H4" t="n">
-        <v>76.13830643262402</v>
+        <v>35.04062110079024</v>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>2026-03-21T03:44:05</t>
+          <t>2026-03-21T03:44:38</t>
         </is>
       </c>
     </row>
@@ -1088,11 +1466,11 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>센트러스 에너지</t>
+          <t>프론트라인</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>21</v>
+        <v>175</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
@@ -1103,17 +1481,17 @@
         <v>1</v>
       </c>
       <c r="F5" t="n">
-        <v>6691594</v>
+        <v>8304681.999999999</v>
       </c>
       <c r="G5" t="n">
-        <v>460375.0000000009</v>
+        <v>3874817.999999999</v>
       </c>
       <c r="H5" t="n">
-        <v>7.38820124922589</v>
+        <v>87.47036026388167</v>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>2026-03-21T03:44:05</t>
+          <t>2026-03-21T03:44:38</t>
         </is>
       </c>
     </row>
@@ -1125,11 +1503,11 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>타이드워터</t>
+          <t>시드릴</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>48</v>
+        <v>123</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
@@ -1140,17 +1518,17 @@
         <v>1</v>
       </c>
       <c r="F6" t="n">
-        <v>5429641</v>
+        <v>7927448</v>
       </c>
       <c r="G6" t="n">
-        <v>1705096</v>
+        <v>1477097</v>
       </c>
       <c r="H6" t="n">
-        <v>45.7799811789091</v>
+        <v>22.89948252428434</v>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>2026-03-21T03:44:05</t>
+          <t>2026-03-21T03:44:38</t>
         </is>
       </c>
     </row>
@@ -1162,11 +1540,11 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>노브</t>
+          <t>트랜스오션</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>185</v>
+        <v>750</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
@@ -1177,17 +1555,17 @@
         <v>1</v>
       </c>
       <c r="F7" t="n">
-        <v>5067449</v>
+        <v>6945333</v>
       </c>
       <c r="G7" t="n">
-        <v>1757441</v>
+        <v>2818099</v>
       </c>
       <c r="H7" t="n">
-        <v>53.09476593410047</v>
+        <v>68.28057241241955</v>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>2026-03-21T03:44:05</t>
+          <t>2026-03-21T03:44:38</t>
         </is>
       </c>
     </row>
@@ -1199,11 +1577,11 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>오케아니스 에코 탱커스</t>
+          <t>노블</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>65</v>
+        <v>99</v>
       </c>
       <c r="D8" t="inlineStr">
         <is>
@@ -1214,17 +1592,17 @@
         <v>1</v>
       </c>
       <c r="F8" t="n">
-        <v>4451759</v>
+        <v>6882090</v>
       </c>
       <c r="G8" t="n">
-        <v>2195399</v>
+        <v>2974882</v>
       </c>
       <c r="H8" t="n">
-        <v>97.29825914304455</v>
+        <v>76.13830643262402</v>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>2026-03-21T03:44:05</t>
+          <t>2026-03-21T03:44:38</t>
         </is>
       </c>
     </row>
@@ -1236,11 +1614,11 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>차코스 에너지 내비게이션</t>
+          <t>센트러스 에너지</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>75</v>
+        <v>21</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
@@ -1251,17 +1629,17 @@
         <v>1</v>
       </c>
       <c r="F9" t="n">
-        <v>3919272</v>
+        <v>6691594</v>
       </c>
       <c r="G9" t="n">
-        <v>94624</v>
+        <v>460375.0000000009</v>
       </c>
       <c r="H9" t="n">
-        <v>2.474057743353114</v>
+        <v>7.38820124922589</v>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>2026-03-21T03:44:05</t>
+          <t>2026-03-21T03:44:38</t>
         </is>
       </c>
     </row>
@@ -1273,11 +1651,11 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>더치 브로스</t>
+          <t>타이드워터</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>39</v>
+        <v>48</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
@@ -1288,17 +1666,17 @@
         <v>1</v>
       </c>
       <c r="F10" t="n">
-        <v>2926290</v>
+        <v>5429641</v>
       </c>
       <c r="G10" t="n">
-        <v>-264354</v>
+        <v>1705096</v>
       </c>
       <c r="H10" t="n">
-        <v>-8.285286606716387</v>
+        <v>45.7799811789091</v>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>2026-03-21T03:44:05</t>
+          <t>2026-03-21T03:44:38</t>
         </is>
       </c>
     </row>
@@ -1310,11 +1688,11 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>발레로 에너지</t>
+          <t>노브</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>6</v>
+        <v>185</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
@@ -1325,17 +1703,17 @@
         <v>1</v>
       </c>
       <c r="F11" t="n">
-        <v>2096946</v>
+        <v>5067449</v>
       </c>
       <c r="G11" t="n">
-        <v>32956</v>
+        <v>1757441</v>
       </c>
       <c r="H11" t="n">
-        <v>1.596713162369973</v>
+        <v>53.09476593410047</v>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>2026-03-21T03:44:05</t>
+          <t>2026-03-21T03:44:38</t>
         </is>
       </c>
     </row>
@@ -1347,11 +1725,11 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>유나이티드헬스 그룹</t>
+          <t>오케아니스 에코 탱커스</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>4</v>
+        <v>65</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
@@ -1362,17 +1740,17 @@
         <v>1</v>
       </c>
       <c r="F12" t="n">
-        <v>1710490</v>
+        <v>4451759</v>
       </c>
       <c r="G12" t="n">
-        <v>16034</v>
+        <v>2195399</v>
       </c>
       <c r="H12" t="n">
-        <v>0.9462623992597033</v>
+        <v>97.29825914304455</v>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>2026-03-21T03:44:05</t>
+          <t>2026-03-21T03:44:38</t>
         </is>
       </c>
     </row>
@@ -1384,11 +1762,11 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>스타 벌크 캐리어스</t>
+          <t>차코스 에너지 내비게이션</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>50</v>
+        <v>75</v>
       </c>
       <c r="D13" t="inlineStr">
         <is>
@@ -1399,17 +1777,17 @@
         <v>1</v>
       </c>
       <c r="F13" t="n">
-        <v>1661361</v>
+        <v>3919272</v>
       </c>
       <c r="G13" t="n">
-        <v>347008</v>
+        <v>94624</v>
       </c>
       <c r="H13" t="n">
-        <v>26.40143097021881</v>
+        <v>2.474057743353114</v>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>2026-03-21T03:44:05</t>
+          <t>2026-03-21T03:44:38</t>
         </is>
       </c>
     </row>
@@ -1421,11 +1799,11 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>클리블랜드 클리프스</t>
+          <t>동원개발</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>70</v>
+        <v>1360</v>
       </c>
       <c r="D14" t="inlineStr">
         <is>
@@ -1436,17 +1814,17 @@
         <v>1</v>
       </c>
       <c r="F14" t="n">
-        <v>908091</v>
+        <v>3881821</v>
       </c>
       <c r="G14" t="n">
-        <v>-107964</v>
+        <v>144420.9999999995</v>
       </c>
       <c r="H14" t="n">
-        <v>-10.62580273705656</v>
+        <v>3.86421041365654</v>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>2026-03-21T03:44:05</t>
+          <t>2026-03-21T03:44:38</t>
         </is>
       </c>
     </row>
@@ -1458,32 +1836,550 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
+          <t>피바디 에너지</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>65</v>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E15" t="n">
+        <v>1</v>
+      </c>
+      <c r="F15" t="n">
+        <v>3427688</v>
+      </c>
+      <c r="G15" t="n">
+        <v>1956916</v>
+      </c>
+      <c r="H15" t="n">
+        <v>133.0536616144446</v>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>2026-03-21T03:44:38</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-03-17</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>더치 브로스</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>39</v>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E16" t="n">
+        <v>1</v>
+      </c>
+      <c r="F16" t="n">
+        <v>2926290</v>
+      </c>
+      <c r="G16" t="n">
+        <v>-264354</v>
+      </c>
+      <c r="H16" t="n">
+        <v>-8.285286606716387</v>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>2026-03-21T03:44:38</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2026-03-17</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>넥스틸</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
+        <v>200</v>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E17" t="n">
+        <v>1</v>
+      </c>
+      <c r="F17" t="n">
+        <v>2391208</v>
+      </c>
+      <c r="G17" t="n">
+        <v>380208</v>
+      </c>
+      <c r="H17" t="n">
+        <v>18.90641471904525</v>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>2026-03-21T03:44:38</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>2026-03-17</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>대신증권</t>
+        </is>
+      </c>
+      <c r="C18" t="n">
+        <v>55</v>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E18" t="n">
+        <v>1</v>
+      </c>
+      <c r="F18" t="n">
+        <v>2190111</v>
+      </c>
+      <c r="G18" t="n">
+        <v>480610</v>
+      </c>
+      <c r="H18" t="n">
+        <v>28.11405199528985</v>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>2026-03-21T03:44:38</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>2026-03-17</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>발레로 에너지</t>
+        </is>
+      </c>
+      <c r="C19" t="n">
+        <v>6</v>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E19" t="n">
+        <v>1</v>
+      </c>
+      <c r="F19" t="n">
+        <v>2096946</v>
+      </c>
+      <c r="G19" t="n">
+        <v>32956</v>
+      </c>
+      <c r="H19" t="n">
+        <v>1.596713162369973</v>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>2026-03-21T03:44:38</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>2026-03-17</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>미창석유</t>
+        </is>
+      </c>
+      <c r="C20" t="n">
+        <v>18</v>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E20" t="n">
+        <v>1</v>
+      </c>
+      <c r="F20" t="n">
+        <v>2049693</v>
+      </c>
+      <c r="G20" t="n">
+        <v>-342507</v>
+      </c>
+      <c r="H20" t="n">
+        <v>-14.31765738650614</v>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>2026-03-21T03:44:38</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>2026-03-17</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>대창단조</t>
+        </is>
+      </c>
+      <c r="C21" t="n">
+        <v>300</v>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E21" t="n">
+        <v>1</v>
+      </c>
+      <c r="F21" t="n">
+        <v>1901190</v>
+      </c>
+      <c r="G21" t="n">
+        <v>-156810</v>
+      </c>
+      <c r="H21" t="n">
+        <v>-7.619533527696793</v>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>2026-03-21T03:44:38</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>2026-03-17</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>동방</t>
+        </is>
+      </c>
+      <c r="C22" t="n">
+        <v>681</v>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E22" t="n">
+        <v>1</v>
+      </c>
+      <c r="F22" t="n">
+        <v>1841600</v>
+      </c>
+      <c r="G22" t="n">
+        <v>-129901</v>
+      </c>
+      <c r="H22" t="n">
+        <v>-6.588939087527726</v>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>2026-03-21T03:44:38</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>2026-03-17</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>유나이티드헬스 그룹</t>
+        </is>
+      </c>
+      <c r="C23" t="n">
+        <v>4</v>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E23" t="n">
+        <v>1</v>
+      </c>
+      <c r="F23" t="n">
+        <v>1710490</v>
+      </c>
+      <c r="G23" t="n">
+        <v>16034</v>
+      </c>
+      <c r="H23" t="n">
+        <v>0.9462623992597033</v>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>2026-03-21T03:44:38</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>2026-03-17</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>스타 벌크 캐리어스</t>
+        </is>
+      </c>
+      <c r="C24" t="n">
+        <v>50</v>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E24" t="n">
+        <v>1</v>
+      </c>
+      <c r="F24" t="n">
+        <v>1661361</v>
+      </c>
+      <c r="G24" t="n">
+        <v>347008</v>
+      </c>
+      <c r="H24" t="n">
+        <v>26.40143097021881</v>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>2026-03-21T03:44:38</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>2026-03-17</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>클리블랜드 클리프스</t>
+        </is>
+      </c>
+      <c r="C25" t="n">
+        <v>70</v>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E25" t="n">
+        <v>1</v>
+      </c>
+      <c r="F25" t="n">
+        <v>908091</v>
+      </c>
+      <c r="G25" t="n">
+        <v>-107964</v>
+      </c>
+      <c r="H25" t="n">
+        <v>-10.62580273705656</v>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>2026-03-21T03:44:38</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>2026-03-17</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>삼성생명</t>
+        </is>
+      </c>
+      <c r="C26" t="n">
+        <v>4</v>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E26" t="n">
+        <v>1</v>
+      </c>
+      <c r="F26" t="n">
+        <v>872252</v>
+      </c>
+      <c r="G26" t="n">
+        <v>39252</v>
+      </c>
+      <c r="H26" t="n">
+        <v>4.712124849939976</v>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>2026-03-21T03:44:38</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>2026-03-17</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>비에이치아이</t>
+        </is>
+      </c>
+      <c r="C27" t="n">
+        <v>8</v>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E27" t="n">
+        <v>1</v>
+      </c>
+      <c r="F27" t="n">
+        <v>850296</v>
+      </c>
+      <c r="G27" t="n">
+        <v>185181</v>
+      </c>
+      <c r="H27" t="n">
+        <v>27.84195214361426</v>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>2026-03-21T03:44:38</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>2026-03-17</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>하프니아</t>
+        </is>
+      </c>
+      <c r="C28" t="n">
+        <v>80</v>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E28" t="n">
+        <v>1</v>
+      </c>
+      <c r="F28" t="n">
+        <v>798051</v>
+      </c>
+      <c r="G28" t="n">
+        <v>172320</v>
+      </c>
+      <c r="H28" t="n">
+        <v>27.53899039683186</v>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>2026-03-21T03:44:38</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>2026-03-17</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
           <t>텍사스 퍼시픽 랜드</t>
         </is>
       </c>
-      <c r="C15" t="n">
-        <v>1</v>
-      </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>KRW</t>
-        </is>
-      </c>
-      <c r="E15" t="n">
-        <v>1</v>
-      </c>
-      <c r="F15" t="n">
+      <c r="C29" t="n">
+        <v>1</v>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E29" t="n">
+        <v>1</v>
+      </c>
+      <c r="F29" t="n">
         <v>786665</v>
       </c>
-      <c r="G15" t="n">
+      <c r="G29" t="n">
         <v>8074</v>
       </c>
-      <c r="H15" t="n">
+      <c r="H29" t="n">
         <v>1.037001455192778</v>
       </c>
-      <c r="I15" t="inlineStr">
-        <is>
-          <t>2026-03-21T03:44:05</t>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>2026-03-21T03:44:38</t>
         </is>
       </c>
     </row>
@@ -1547,7 +2443,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>2026-03-21T03:44:05</t>
+          <t>2026-03-21T03:44:38</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: portfolio snapshot 2026-03-17 (2026-03-21T03:44:39)
</commit_message>
<xml_diff>
--- a/portfolio_auto.xlsx
+++ b/portfolio_auto.xlsx
@@ -1279,7 +1279,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2026-03-21T03:44:38</t>
+          <t>2026-03-21T03:44:39</t>
         </is>
       </c>
       <c r="E2" t="n">
@@ -1380,7 +1380,7 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>2026-03-21T03:44:38</t>
+          <t>2026-03-21T03:44:39</t>
         </is>
       </c>
     </row>
@@ -1417,7 +1417,7 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>2026-03-21T03:44:38</t>
+          <t>2026-03-21T03:44:39</t>
         </is>
       </c>
     </row>
@@ -1454,7 +1454,7 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>2026-03-21T03:44:38</t>
+          <t>2026-03-21T03:44:39</t>
         </is>
       </c>
     </row>
@@ -1491,7 +1491,7 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>2026-03-21T03:44:38</t>
+          <t>2026-03-21T03:44:39</t>
         </is>
       </c>
     </row>
@@ -1528,7 +1528,7 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>2026-03-21T03:44:38</t>
+          <t>2026-03-21T03:44:39</t>
         </is>
       </c>
     </row>
@@ -1565,7 +1565,7 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>2026-03-21T03:44:38</t>
+          <t>2026-03-21T03:44:39</t>
         </is>
       </c>
     </row>
@@ -1602,7 +1602,7 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>2026-03-21T03:44:38</t>
+          <t>2026-03-21T03:44:39</t>
         </is>
       </c>
     </row>
@@ -1639,7 +1639,7 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>2026-03-21T03:44:38</t>
+          <t>2026-03-21T03:44:39</t>
         </is>
       </c>
     </row>
@@ -1676,7 +1676,7 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>2026-03-21T03:44:38</t>
+          <t>2026-03-21T03:44:39</t>
         </is>
       </c>
     </row>
@@ -1713,7 +1713,7 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>2026-03-21T03:44:38</t>
+          <t>2026-03-21T03:44:39</t>
         </is>
       </c>
     </row>
@@ -1750,7 +1750,7 @@
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>2026-03-21T03:44:38</t>
+          <t>2026-03-21T03:44:39</t>
         </is>
       </c>
     </row>
@@ -1787,7 +1787,7 @@
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>2026-03-21T03:44:38</t>
+          <t>2026-03-21T03:44:39</t>
         </is>
       </c>
     </row>
@@ -1824,7 +1824,7 @@
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>2026-03-21T03:44:38</t>
+          <t>2026-03-21T03:44:39</t>
         </is>
       </c>
     </row>
@@ -1861,7 +1861,7 @@
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>2026-03-21T03:44:38</t>
+          <t>2026-03-21T03:44:39</t>
         </is>
       </c>
     </row>
@@ -1898,7 +1898,7 @@
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>2026-03-21T03:44:38</t>
+          <t>2026-03-21T03:44:39</t>
         </is>
       </c>
     </row>
@@ -1935,7 +1935,7 @@
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>2026-03-21T03:44:38</t>
+          <t>2026-03-21T03:44:39</t>
         </is>
       </c>
     </row>
@@ -1972,7 +1972,7 @@
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>2026-03-21T03:44:38</t>
+          <t>2026-03-21T03:44:39</t>
         </is>
       </c>
     </row>
@@ -2009,7 +2009,7 @@
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>2026-03-21T03:44:38</t>
+          <t>2026-03-21T03:44:39</t>
         </is>
       </c>
     </row>
@@ -2046,7 +2046,7 @@
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>2026-03-21T03:44:38</t>
+          <t>2026-03-21T03:44:39</t>
         </is>
       </c>
     </row>
@@ -2083,7 +2083,7 @@
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>2026-03-21T03:44:38</t>
+          <t>2026-03-21T03:44:39</t>
         </is>
       </c>
     </row>
@@ -2120,7 +2120,7 @@
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>2026-03-21T03:44:38</t>
+          <t>2026-03-21T03:44:39</t>
         </is>
       </c>
     </row>
@@ -2157,7 +2157,7 @@
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>2026-03-21T03:44:38</t>
+          <t>2026-03-21T03:44:39</t>
         </is>
       </c>
     </row>
@@ -2194,7 +2194,7 @@
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>2026-03-21T03:44:38</t>
+          <t>2026-03-21T03:44:39</t>
         </is>
       </c>
     </row>
@@ -2231,7 +2231,7 @@
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>2026-03-21T03:44:38</t>
+          <t>2026-03-21T03:44:39</t>
         </is>
       </c>
     </row>
@@ -2268,7 +2268,7 @@
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>2026-03-21T03:44:38</t>
+          <t>2026-03-21T03:44:39</t>
         </is>
       </c>
     </row>
@@ -2305,7 +2305,7 @@
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>2026-03-21T03:44:38</t>
+          <t>2026-03-21T03:44:39</t>
         </is>
       </c>
     </row>
@@ -2342,7 +2342,7 @@
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>2026-03-21T03:44:38</t>
+          <t>2026-03-21T03:44:39</t>
         </is>
       </c>
     </row>
@@ -2379,7 +2379,7 @@
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>2026-03-21T03:44:38</t>
+          <t>2026-03-21T03:44:39</t>
         </is>
       </c>
     </row>
@@ -2443,7 +2443,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>2026-03-21T03:44:38</t>
+          <t>2026-03-21T03:44:39</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: portfolio snapshot 2026-03-17 (2026-03-21T03:45:08)
</commit_message>
<xml_diff>
--- a/portfolio_auto.xlsx
+++ b/portfolio_auto.xlsx
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G29"/>
+  <dimension ref="A1:G39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1222,6 +1222,276 @@
       </c>
       <c r="G29" t="n">
         <v>4.712124849939976</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>삼성화재</t>
+        </is>
+      </c>
+      <c r="B30" t="n">
+        <v>7</v>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="D30" t="n">
+        <v>1</v>
+      </c>
+      <c r="E30" t="n">
+        <v>3335815</v>
+      </c>
+      <c r="F30" t="n">
+        <v>-295185</v>
+      </c>
+      <c r="G30" t="n">
+        <v>-8.129578628477004</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>세아제강</t>
+        </is>
+      </c>
+      <c r="B31" t="n">
+        <v>50</v>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="D31" t="n">
+        <v>1</v>
+      </c>
+      <c r="E31" t="n">
+        <v>6896180</v>
+      </c>
+      <c r="F31" t="n">
+        <v>586180</v>
+      </c>
+      <c r="G31" t="n">
+        <v>9.289698890649763</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>케이씨</t>
+        </is>
+      </c>
+      <c r="B32" t="n">
+        <v>50</v>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="D32" t="n">
+        <v>1</v>
+      </c>
+      <c r="E32" t="n">
+        <v>1576840</v>
+      </c>
+      <c r="F32" t="n">
+        <v>-72660</v>
+      </c>
+      <c r="G32" t="n">
+        <v>-4.404971203394968</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>하나금융지주</t>
+        </is>
+      </c>
+      <c r="B33" t="n">
+        <v>10</v>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="D33" t="n">
+        <v>1</v>
+      </c>
+      <c r="E33" t="n">
+        <v>1107780</v>
+      </c>
+      <c r="F33" t="n">
+        <v>-1220</v>
+      </c>
+      <c r="G33" t="n">
+        <v>-0.1100090171325518</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>현대제철</t>
+        </is>
+      </c>
+      <c r="B34" t="n">
+        <v>70</v>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="D34" t="n">
+        <v>1</v>
+      </c>
+      <c r="E34" t="n">
+        <v>2494002</v>
+      </c>
+      <c r="F34" t="n">
+        <v>-313498</v>
+      </c>
+      <c r="G34" t="n">
+        <v>-11.16644701691897</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>휴스틸</t>
+        </is>
+      </c>
+      <c r="B35" t="n">
+        <v>500</v>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="D35" t="n">
+        <v>1</v>
+      </c>
+      <c r="E35" t="n">
+        <v>2450090</v>
+      </c>
+      <c r="F35" t="n">
+        <v>171480</v>
+      </c>
+      <c r="G35" t="n">
+        <v>7.525640631788678</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>DL이앤씨</t>
+        </is>
+      </c>
+      <c r="B36" t="n">
+        <v>80</v>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="D36" t="n">
+        <v>1</v>
+      </c>
+      <c r="E36" t="n">
+        <v>3792400</v>
+      </c>
+      <c r="F36" t="n">
+        <v>381400</v>
+      </c>
+      <c r="G36" t="n">
+        <v>11.1814717091762</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>HD건설기계</t>
+        </is>
+      </c>
+      <c r="B37" t="n">
+        <v>31</v>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="D37" t="n">
+        <v>1</v>
+      </c>
+      <c r="E37" t="n">
+        <v>3885810</v>
+      </c>
+      <c r="F37" t="n">
+        <v>-149286</v>
+      </c>
+      <c r="G37" t="n">
+        <v>-3.699688929334023</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>KoAct 코스닥액티브</t>
+        </is>
+      </c>
+      <c r="B38" t="n">
+        <v>200</v>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="D38" t="n">
+        <v>1</v>
+      </c>
+      <c r="E38" t="n">
+        <v>2580000</v>
+      </c>
+      <c r="F38" t="n">
+        <v>-122000</v>
+      </c>
+      <c r="G38" t="n">
+        <v>-4.515173945225759</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>TIME 코리아밸류업액티브</t>
+        </is>
+      </c>
+      <c r="B39" t="n">
+        <v>201</v>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="D39" t="n">
+        <v>1</v>
+      </c>
+      <c r="E39" t="n">
+        <v>4656165</v>
+      </c>
+      <c r="F39" t="n">
+        <v>-67632</v>
+      </c>
+      <c r="G39" t="n">
+        <v>-1.43172960226699</v>
       </c>
     </row>
   </sheetData>
@@ -1279,7 +1549,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2026-03-21T03:44:39</t>
+          <t>2026-03-21T03:45:08</t>
         </is>
       </c>
       <c r="E2" t="n">
@@ -1297,7 +1567,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I29"/>
+  <dimension ref="A1:I39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1380,7 +1650,7 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>2026-03-21T03:44:39</t>
+          <t>2026-03-21T03:45:08</t>
         </is>
       </c>
     </row>
@@ -1417,7 +1687,7 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>2026-03-21T03:44:39</t>
+          <t>2026-03-21T03:45:08</t>
         </is>
       </c>
     </row>
@@ -1454,7 +1724,7 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>2026-03-21T03:44:39</t>
+          <t>2026-03-21T03:45:08</t>
         </is>
       </c>
     </row>
@@ -1491,7 +1761,7 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>2026-03-21T03:44:39</t>
+          <t>2026-03-21T03:45:08</t>
         </is>
       </c>
     </row>
@@ -1528,7 +1798,7 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>2026-03-21T03:44:39</t>
+          <t>2026-03-21T03:45:08</t>
         </is>
       </c>
     </row>
@@ -1565,7 +1835,7 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>2026-03-21T03:44:39</t>
+          <t>2026-03-21T03:45:08</t>
         </is>
       </c>
     </row>
@@ -1577,11 +1847,11 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>노블</t>
+          <t>세아제강</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>99</v>
+        <v>50</v>
       </c>
       <c r="D8" t="inlineStr">
         <is>
@@ -1592,17 +1862,17 @@
         <v>1</v>
       </c>
       <c r="F8" t="n">
-        <v>6882090</v>
+        <v>6896180</v>
       </c>
       <c r="G8" t="n">
-        <v>2974882</v>
+        <v>586180</v>
       </c>
       <c r="H8" t="n">
-        <v>76.13830643262402</v>
+        <v>9.289698890649763</v>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>2026-03-21T03:44:39</t>
+          <t>2026-03-21T03:45:08</t>
         </is>
       </c>
     </row>
@@ -1614,11 +1884,11 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>센트러스 에너지</t>
+          <t>노블</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>21</v>
+        <v>99</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
@@ -1629,17 +1899,17 @@
         <v>1</v>
       </c>
       <c r="F9" t="n">
-        <v>6691594</v>
+        <v>6882090</v>
       </c>
       <c r="G9" t="n">
-        <v>460375.0000000009</v>
+        <v>2974882</v>
       </c>
       <c r="H9" t="n">
-        <v>7.38820124922589</v>
+        <v>76.13830643262402</v>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>2026-03-21T03:44:39</t>
+          <t>2026-03-21T03:45:08</t>
         </is>
       </c>
     </row>
@@ -1651,11 +1921,11 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>타이드워터</t>
+          <t>센트러스 에너지</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>48</v>
+        <v>21</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
@@ -1666,17 +1936,17 @@
         <v>1</v>
       </c>
       <c r="F10" t="n">
-        <v>5429641</v>
+        <v>6691594</v>
       </c>
       <c r="G10" t="n">
-        <v>1705096</v>
+        <v>460375.0000000009</v>
       </c>
       <c r="H10" t="n">
-        <v>45.7799811789091</v>
+        <v>7.38820124922589</v>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>2026-03-21T03:44:39</t>
+          <t>2026-03-21T03:45:08</t>
         </is>
       </c>
     </row>
@@ -1688,11 +1958,11 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>노브</t>
+          <t>타이드워터</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>185</v>
+        <v>48</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
@@ -1703,17 +1973,17 @@
         <v>1</v>
       </c>
       <c r="F11" t="n">
-        <v>5067449</v>
+        <v>5429641</v>
       </c>
       <c r="G11" t="n">
-        <v>1757441</v>
+        <v>1705096</v>
       </c>
       <c r="H11" t="n">
-        <v>53.09476593410047</v>
+        <v>45.7799811789091</v>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>2026-03-21T03:44:39</t>
+          <t>2026-03-21T03:45:08</t>
         </is>
       </c>
     </row>
@@ -1725,11 +1995,11 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>오케아니스 에코 탱커스</t>
+          <t>노브</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>65</v>
+        <v>185</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
@@ -1740,17 +2010,17 @@
         <v>1</v>
       </c>
       <c r="F12" t="n">
-        <v>4451759</v>
+        <v>5067449</v>
       </c>
       <c r="G12" t="n">
-        <v>2195399</v>
+        <v>1757441</v>
       </c>
       <c r="H12" t="n">
-        <v>97.29825914304455</v>
+        <v>53.09476593410047</v>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>2026-03-21T03:44:39</t>
+          <t>2026-03-21T03:45:08</t>
         </is>
       </c>
     </row>
@@ -1762,11 +2032,11 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>차코스 에너지 내비게이션</t>
+          <t>TIME 코리아밸류업액티브</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>75</v>
+        <v>201</v>
       </c>
       <c r="D13" t="inlineStr">
         <is>
@@ -1777,17 +2047,17 @@
         <v>1</v>
       </c>
       <c r="F13" t="n">
-        <v>3919272</v>
+        <v>4656165</v>
       </c>
       <c r="G13" t="n">
-        <v>94624</v>
+        <v>-67632</v>
       </c>
       <c r="H13" t="n">
-        <v>2.474057743353114</v>
+        <v>-1.43172960226699</v>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>2026-03-21T03:44:39</t>
+          <t>2026-03-21T03:45:08</t>
         </is>
       </c>
     </row>
@@ -1799,11 +2069,11 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>동원개발</t>
+          <t>오케아니스 에코 탱커스</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>1360</v>
+        <v>65</v>
       </c>
       <c r="D14" t="inlineStr">
         <is>
@@ -1814,17 +2084,17 @@
         <v>1</v>
       </c>
       <c r="F14" t="n">
-        <v>3881821</v>
+        <v>4451759</v>
       </c>
       <c r="G14" t="n">
-        <v>144420.9999999995</v>
+        <v>2195399</v>
       </c>
       <c r="H14" t="n">
-        <v>3.86421041365654</v>
+        <v>97.29825914304455</v>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>2026-03-21T03:44:39</t>
+          <t>2026-03-21T03:45:08</t>
         </is>
       </c>
     </row>
@@ -1836,11 +2106,11 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>피바디 에너지</t>
+          <t>차코스 에너지 내비게이션</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>65</v>
+        <v>75</v>
       </c>
       <c r="D15" t="inlineStr">
         <is>
@@ -1851,17 +2121,17 @@
         <v>1</v>
       </c>
       <c r="F15" t="n">
-        <v>3427688</v>
+        <v>3919272</v>
       </c>
       <c r="G15" t="n">
-        <v>1956916</v>
+        <v>94624</v>
       </c>
       <c r="H15" t="n">
-        <v>133.0536616144446</v>
+        <v>2.474057743353114</v>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>2026-03-21T03:44:39</t>
+          <t>2026-03-21T03:45:08</t>
         </is>
       </c>
     </row>
@@ -1873,11 +2143,11 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>더치 브로스</t>
+          <t>HD건설기계</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>39</v>
+        <v>31</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
@@ -1888,17 +2158,17 @@
         <v>1</v>
       </c>
       <c r="F16" t="n">
-        <v>2926290</v>
+        <v>3885810</v>
       </c>
       <c r="G16" t="n">
-        <v>-264354</v>
+        <v>-149286</v>
       </c>
       <c r="H16" t="n">
-        <v>-8.285286606716387</v>
+        <v>-3.699688929334023</v>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>2026-03-21T03:44:39</t>
+          <t>2026-03-21T03:45:08</t>
         </is>
       </c>
     </row>
@@ -1910,11 +2180,11 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>넥스틸</t>
+          <t>동원개발</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>200</v>
+        <v>1360</v>
       </c>
       <c r="D17" t="inlineStr">
         <is>
@@ -1925,17 +2195,17 @@
         <v>1</v>
       </c>
       <c r="F17" t="n">
-        <v>2391208</v>
+        <v>3881821</v>
       </c>
       <c r="G17" t="n">
-        <v>380208</v>
+        <v>144420.9999999995</v>
       </c>
       <c r="H17" t="n">
-        <v>18.90641471904525</v>
+        <v>3.86421041365654</v>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>2026-03-21T03:44:39</t>
+          <t>2026-03-21T03:45:08</t>
         </is>
       </c>
     </row>
@@ -1947,11 +2217,11 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>대신증권</t>
+          <t>DL이앤씨</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>55</v>
+        <v>80</v>
       </c>
       <c r="D18" t="inlineStr">
         <is>
@@ -1962,17 +2232,17 @@
         <v>1</v>
       </c>
       <c r="F18" t="n">
-        <v>2190111</v>
+        <v>3792400</v>
       </c>
       <c r="G18" t="n">
-        <v>480610</v>
+        <v>381400</v>
       </c>
       <c r="H18" t="n">
-        <v>28.11405199528985</v>
+        <v>11.1814717091762</v>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>2026-03-21T03:44:39</t>
+          <t>2026-03-21T03:45:08</t>
         </is>
       </c>
     </row>
@@ -1984,11 +2254,11 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>발레로 에너지</t>
+          <t>피바디 에너지</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>6</v>
+        <v>65</v>
       </c>
       <c r="D19" t="inlineStr">
         <is>
@@ -1999,17 +2269,17 @@
         <v>1</v>
       </c>
       <c r="F19" t="n">
-        <v>2096946</v>
+        <v>3427688</v>
       </c>
       <c r="G19" t="n">
-        <v>32956</v>
+        <v>1956916</v>
       </c>
       <c r="H19" t="n">
-        <v>1.596713162369973</v>
+        <v>133.0536616144446</v>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>2026-03-21T03:44:39</t>
+          <t>2026-03-21T03:45:08</t>
         </is>
       </c>
     </row>
@@ -2021,11 +2291,11 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>미창석유</t>
+          <t>삼성화재</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>18</v>
+        <v>7</v>
       </c>
       <c r="D20" t="inlineStr">
         <is>
@@ -2036,17 +2306,17 @@
         <v>1</v>
       </c>
       <c r="F20" t="n">
-        <v>2049693</v>
+        <v>3335815</v>
       </c>
       <c r="G20" t="n">
-        <v>-342507</v>
+        <v>-295185</v>
       </c>
       <c r="H20" t="n">
-        <v>-14.31765738650614</v>
+        <v>-8.129578628477004</v>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>2026-03-21T03:44:39</t>
+          <t>2026-03-21T03:45:08</t>
         </is>
       </c>
     </row>
@@ -2058,11 +2328,11 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>대창단조</t>
+          <t>더치 브로스</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>300</v>
+        <v>39</v>
       </c>
       <c r="D21" t="inlineStr">
         <is>
@@ -2073,17 +2343,17 @@
         <v>1</v>
       </c>
       <c r="F21" t="n">
-        <v>1901190</v>
+        <v>2926290</v>
       </c>
       <c r="G21" t="n">
-        <v>-156810</v>
+        <v>-264354</v>
       </c>
       <c r="H21" t="n">
-        <v>-7.619533527696793</v>
+        <v>-8.285286606716387</v>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>2026-03-21T03:44:39</t>
+          <t>2026-03-21T03:45:08</t>
         </is>
       </c>
     </row>
@@ -2095,11 +2365,11 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>동방</t>
+          <t>KoAct 코스닥액티브</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>681</v>
+        <v>200</v>
       </c>
       <c r="D22" t="inlineStr">
         <is>
@@ -2110,17 +2380,17 @@
         <v>1</v>
       </c>
       <c r="F22" t="n">
-        <v>1841600</v>
+        <v>2580000</v>
       </c>
       <c r="G22" t="n">
-        <v>-129901</v>
+        <v>-122000</v>
       </c>
       <c r="H22" t="n">
-        <v>-6.588939087527726</v>
+        <v>-4.515173945225759</v>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>2026-03-21T03:44:39</t>
+          <t>2026-03-21T03:45:08</t>
         </is>
       </c>
     </row>
@@ -2132,11 +2402,11 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>유나이티드헬스 그룹</t>
+          <t>현대제철</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>4</v>
+        <v>70</v>
       </c>
       <c r="D23" t="inlineStr">
         <is>
@@ -2147,17 +2417,17 @@
         <v>1</v>
       </c>
       <c r="F23" t="n">
-        <v>1710490</v>
+        <v>2494002</v>
       </c>
       <c r="G23" t="n">
-        <v>16034</v>
+        <v>-313498</v>
       </c>
       <c r="H23" t="n">
-        <v>0.9462623992597033</v>
+        <v>-11.16644701691897</v>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>2026-03-21T03:44:39</t>
+          <t>2026-03-21T03:45:08</t>
         </is>
       </c>
     </row>
@@ -2169,11 +2439,11 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>스타 벌크 캐리어스</t>
+          <t>휴스틸</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>50</v>
+        <v>500</v>
       </c>
       <c r="D24" t="inlineStr">
         <is>
@@ -2184,17 +2454,17 @@
         <v>1</v>
       </c>
       <c r="F24" t="n">
-        <v>1661361</v>
+        <v>2450090</v>
       </c>
       <c r="G24" t="n">
-        <v>347008</v>
+        <v>171480</v>
       </c>
       <c r="H24" t="n">
-        <v>26.40143097021881</v>
+        <v>7.525640631788678</v>
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>2026-03-21T03:44:39</t>
+          <t>2026-03-21T03:45:08</t>
         </is>
       </c>
     </row>
@@ -2206,11 +2476,11 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>클리블랜드 클리프스</t>
+          <t>넥스틸</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>70</v>
+        <v>200</v>
       </c>
       <c r="D25" t="inlineStr">
         <is>
@@ -2221,17 +2491,17 @@
         <v>1</v>
       </c>
       <c r="F25" t="n">
-        <v>908091</v>
+        <v>2391208</v>
       </c>
       <c r="G25" t="n">
-        <v>-107964</v>
+        <v>380208</v>
       </c>
       <c r="H25" t="n">
-        <v>-10.62580273705656</v>
+        <v>18.90641471904525</v>
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>2026-03-21T03:44:39</t>
+          <t>2026-03-21T03:45:08</t>
         </is>
       </c>
     </row>
@@ -2243,11 +2513,11 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>삼성생명</t>
+          <t>대신증권</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>4</v>
+        <v>55</v>
       </c>
       <c r="D26" t="inlineStr">
         <is>
@@ -2258,17 +2528,17 @@
         <v>1</v>
       </c>
       <c r="F26" t="n">
-        <v>872252</v>
+        <v>2190111</v>
       </c>
       <c r="G26" t="n">
-        <v>39252</v>
+        <v>480610</v>
       </c>
       <c r="H26" t="n">
-        <v>4.712124849939976</v>
+        <v>28.11405199528985</v>
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>2026-03-21T03:44:39</t>
+          <t>2026-03-21T03:45:08</t>
         </is>
       </c>
     </row>
@@ -2280,11 +2550,11 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>비에이치아이</t>
+          <t>발레로 에너지</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="D27" t="inlineStr">
         <is>
@@ -2295,17 +2565,17 @@
         <v>1</v>
       </c>
       <c r="F27" t="n">
-        <v>850296</v>
+        <v>2096946</v>
       </c>
       <c r="G27" t="n">
-        <v>185181</v>
+        <v>32956</v>
       </c>
       <c r="H27" t="n">
-        <v>27.84195214361426</v>
+        <v>1.596713162369973</v>
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>2026-03-21T03:44:39</t>
+          <t>2026-03-21T03:45:08</t>
         </is>
       </c>
     </row>
@@ -2317,11 +2587,11 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>하프니아</t>
+          <t>미창석유</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>80</v>
+        <v>18</v>
       </c>
       <c r="D28" t="inlineStr">
         <is>
@@ -2332,17 +2602,17 @@
         <v>1</v>
       </c>
       <c r="F28" t="n">
-        <v>798051</v>
+        <v>2049693</v>
       </c>
       <c r="G28" t="n">
-        <v>172320</v>
+        <v>-342507</v>
       </c>
       <c r="H28" t="n">
-        <v>27.53899039683186</v>
+        <v>-14.31765738650614</v>
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>2026-03-21T03:44:39</t>
+          <t>2026-03-21T03:45:08</t>
         </is>
       </c>
     </row>
@@ -2354,32 +2624,402 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
+          <t>대창단조</t>
+        </is>
+      </c>
+      <c r="C29" t="n">
+        <v>300</v>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E29" t="n">
+        <v>1</v>
+      </c>
+      <c r="F29" t="n">
+        <v>1901190</v>
+      </c>
+      <c r="G29" t="n">
+        <v>-156810</v>
+      </c>
+      <c r="H29" t="n">
+        <v>-7.619533527696793</v>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>2026-03-21T03:45:08</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>2026-03-17</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>동방</t>
+        </is>
+      </c>
+      <c r="C30" t="n">
+        <v>681</v>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E30" t="n">
+        <v>1</v>
+      </c>
+      <c r="F30" t="n">
+        <v>1841600</v>
+      </c>
+      <c r="G30" t="n">
+        <v>-129901</v>
+      </c>
+      <c r="H30" t="n">
+        <v>-6.588939087527726</v>
+      </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>2026-03-21T03:45:08</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>2026-03-17</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>유나이티드헬스 그룹</t>
+        </is>
+      </c>
+      <c r="C31" t="n">
+        <v>4</v>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E31" t="n">
+        <v>1</v>
+      </c>
+      <c r="F31" t="n">
+        <v>1710490</v>
+      </c>
+      <c r="G31" t="n">
+        <v>16034</v>
+      </c>
+      <c r="H31" t="n">
+        <v>0.9462623992597033</v>
+      </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>2026-03-21T03:45:08</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>2026-03-17</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>스타 벌크 캐리어스</t>
+        </is>
+      </c>
+      <c r="C32" t="n">
+        <v>50</v>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E32" t="n">
+        <v>1</v>
+      </c>
+      <c r="F32" t="n">
+        <v>1661361</v>
+      </c>
+      <c r="G32" t="n">
+        <v>347008</v>
+      </c>
+      <c r="H32" t="n">
+        <v>26.40143097021881</v>
+      </c>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>2026-03-21T03:45:08</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>2026-03-17</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>케이씨</t>
+        </is>
+      </c>
+      <c r="C33" t="n">
+        <v>50</v>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E33" t="n">
+        <v>1</v>
+      </c>
+      <c r="F33" t="n">
+        <v>1576840</v>
+      </c>
+      <c r="G33" t="n">
+        <v>-72660</v>
+      </c>
+      <c r="H33" t="n">
+        <v>-4.404971203394968</v>
+      </c>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>2026-03-21T03:45:08</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>2026-03-17</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>하나금융지주</t>
+        </is>
+      </c>
+      <c r="C34" t="n">
+        <v>10</v>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E34" t="n">
+        <v>1</v>
+      </c>
+      <c r="F34" t="n">
+        <v>1107780</v>
+      </c>
+      <c r="G34" t="n">
+        <v>-1220</v>
+      </c>
+      <c r="H34" t="n">
+        <v>-0.1100090171325518</v>
+      </c>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>2026-03-21T03:45:08</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>2026-03-17</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>클리블랜드 클리프스</t>
+        </is>
+      </c>
+      <c r="C35" t="n">
+        <v>70</v>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E35" t="n">
+        <v>1</v>
+      </c>
+      <c r="F35" t="n">
+        <v>908091</v>
+      </c>
+      <c r="G35" t="n">
+        <v>-107964</v>
+      </c>
+      <c r="H35" t="n">
+        <v>-10.62580273705656</v>
+      </c>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>2026-03-21T03:45:08</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>2026-03-17</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>삼성생명</t>
+        </is>
+      </c>
+      <c r="C36" t="n">
+        <v>4</v>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E36" t="n">
+        <v>1</v>
+      </c>
+      <c r="F36" t="n">
+        <v>872252</v>
+      </c>
+      <c r="G36" t="n">
+        <v>39252</v>
+      </c>
+      <c r="H36" t="n">
+        <v>4.712124849939976</v>
+      </c>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>2026-03-21T03:45:08</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>2026-03-17</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>비에이치아이</t>
+        </is>
+      </c>
+      <c r="C37" t="n">
+        <v>8</v>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E37" t="n">
+        <v>1</v>
+      </c>
+      <c r="F37" t="n">
+        <v>850296</v>
+      </c>
+      <c r="G37" t="n">
+        <v>185181</v>
+      </c>
+      <c r="H37" t="n">
+        <v>27.84195214361426</v>
+      </c>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>2026-03-21T03:45:08</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>2026-03-17</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>하프니아</t>
+        </is>
+      </c>
+      <c r="C38" t="n">
+        <v>80</v>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E38" t="n">
+        <v>1</v>
+      </c>
+      <c r="F38" t="n">
+        <v>798051</v>
+      </c>
+      <c r="G38" t="n">
+        <v>172320</v>
+      </c>
+      <c r="H38" t="n">
+        <v>27.53899039683186</v>
+      </c>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>2026-03-21T03:45:08</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>2026-03-17</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
           <t>텍사스 퍼시픽 랜드</t>
         </is>
       </c>
-      <c r="C29" t="n">
-        <v>1</v>
-      </c>
-      <c r="D29" t="inlineStr">
-        <is>
-          <t>KRW</t>
-        </is>
-      </c>
-      <c r="E29" t="n">
-        <v>1</v>
-      </c>
-      <c r="F29" t="n">
+      <c r="C39" t="n">
+        <v>1</v>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E39" t="n">
+        <v>1</v>
+      </c>
+      <c r="F39" t="n">
         <v>786665</v>
       </c>
-      <c r="G29" t="n">
+      <c r="G39" t="n">
         <v>8074</v>
       </c>
-      <c r="H29" t="n">
+      <c r="H39" t="n">
         <v>1.037001455192778</v>
       </c>
-      <c r="I29" t="inlineStr">
-        <is>
-          <t>2026-03-21T03:44:39</t>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>2026-03-21T03:45:08</t>
         </is>
       </c>
     </row>
@@ -2443,7 +3083,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>2026-03-21T03:44:39</t>
+          <t>2026-03-21T03:45:08</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: portfolio snapshot 2026-03-17 (2026-03-21T03:45:09)
</commit_message>
<xml_diff>
--- a/portfolio_auto.xlsx
+++ b/portfolio_auto.xlsx
@@ -1549,7 +1549,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2026-03-21T03:45:08</t>
+          <t>2026-03-21T03:45:09</t>
         </is>
       </c>
       <c r="E2" t="n">
@@ -1650,7 +1650,7 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>2026-03-21T03:45:08</t>
+          <t>2026-03-21T03:45:09</t>
         </is>
       </c>
     </row>
@@ -1687,7 +1687,7 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>2026-03-21T03:45:08</t>
+          <t>2026-03-21T03:45:09</t>
         </is>
       </c>
     </row>
@@ -1724,7 +1724,7 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>2026-03-21T03:45:08</t>
+          <t>2026-03-21T03:45:09</t>
         </is>
       </c>
     </row>
@@ -1761,7 +1761,7 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>2026-03-21T03:45:08</t>
+          <t>2026-03-21T03:45:09</t>
         </is>
       </c>
     </row>
@@ -1798,7 +1798,7 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>2026-03-21T03:45:08</t>
+          <t>2026-03-21T03:45:09</t>
         </is>
       </c>
     </row>
@@ -1835,7 +1835,7 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>2026-03-21T03:45:08</t>
+          <t>2026-03-21T03:45:09</t>
         </is>
       </c>
     </row>
@@ -1872,7 +1872,7 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>2026-03-21T03:45:08</t>
+          <t>2026-03-21T03:45:09</t>
         </is>
       </c>
     </row>
@@ -1909,7 +1909,7 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>2026-03-21T03:45:08</t>
+          <t>2026-03-21T03:45:09</t>
         </is>
       </c>
     </row>
@@ -1946,7 +1946,7 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>2026-03-21T03:45:08</t>
+          <t>2026-03-21T03:45:09</t>
         </is>
       </c>
     </row>
@@ -1983,7 +1983,7 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>2026-03-21T03:45:08</t>
+          <t>2026-03-21T03:45:09</t>
         </is>
       </c>
     </row>
@@ -2020,7 +2020,7 @@
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>2026-03-21T03:45:08</t>
+          <t>2026-03-21T03:45:09</t>
         </is>
       </c>
     </row>
@@ -2057,7 +2057,7 @@
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>2026-03-21T03:45:08</t>
+          <t>2026-03-21T03:45:09</t>
         </is>
       </c>
     </row>
@@ -2094,7 +2094,7 @@
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>2026-03-21T03:45:08</t>
+          <t>2026-03-21T03:45:09</t>
         </is>
       </c>
     </row>
@@ -2131,7 +2131,7 @@
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>2026-03-21T03:45:08</t>
+          <t>2026-03-21T03:45:09</t>
         </is>
       </c>
     </row>
@@ -2168,7 +2168,7 @@
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>2026-03-21T03:45:08</t>
+          <t>2026-03-21T03:45:09</t>
         </is>
       </c>
     </row>
@@ -2205,7 +2205,7 @@
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>2026-03-21T03:45:08</t>
+          <t>2026-03-21T03:45:09</t>
         </is>
       </c>
     </row>
@@ -2242,7 +2242,7 @@
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>2026-03-21T03:45:08</t>
+          <t>2026-03-21T03:45:09</t>
         </is>
       </c>
     </row>
@@ -2279,7 +2279,7 @@
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>2026-03-21T03:45:08</t>
+          <t>2026-03-21T03:45:09</t>
         </is>
       </c>
     </row>
@@ -2316,7 +2316,7 @@
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>2026-03-21T03:45:08</t>
+          <t>2026-03-21T03:45:09</t>
         </is>
       </c>
     </row>
@@ -2353,7 +2353,7 @@
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>2026-03-21T03:45:08</t>
+          <t>2026-03-21T03:45:09</t>
         </is>
       </c>
     </row>
@@ -2390,7 +2390,7 @@
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>2026-03-21T03:45:08</t>
+          <t>2026-03-21T03:45:09</t>
         </is>
       </c>
     </row>
@@ -2427,7 +2427,7 @@
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>2026-03-21T03:45:08</t>
+          <t>2026-03-21T03:45:09</t>
         </is>
       </c>
     </row>
@@ -2464,7 +2464,7 @@
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>2026-03-21T03:45:08</t>
+          <t>2026-03-21T03:45:09</t>
         </is>
       </c>
     </row>
@@ -2501,7 +2501,7 @@
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>2026-03-21T03:45:08</t>
+          <t>2026-03-21T03:45:09</t>
         </is>
       </c>
     </row>
@@ -2538,7 +2538,7 @@
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>2026-03-21T03:45:08</t>
+          <t>2026-03-21T03:45:09</t>
         </is>
       </c>
     </row>
@@ -2575,7 +2575,7 @@
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>2026-03-21T03:45:08</t>
+          <t>2026-03-21T03:45:09</t>
         </is>
       </c>
     </row>
@@ -2612,7 +2612,7 @@
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>2026-03-21T03:45:08</t>
+          <t>2026-03-21T03:45:09</t>
         </is>
       </c>
     </row>
@@ -2649,7 +2649,7 @@
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>2026-03-21T03:45:08</t>
+          <t>2026-03-21T03:45:09</t>
         </is>
       </c>
     </row>
@@ -2686,7 +2686,7 @@
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>2026-03-21T03:45:08</t>
+          <t>2026-03-21T03:45:09</t>
         </is>
       </c>
     </row>
@@ -2723,7 +2723,7 @@
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>2026-03-21T03:45:08</t>
+          <t>2026-03-21T03:45:09</t>
         </is>
       </c>
     </row>
@@ -2760,7 +2760,7 @@
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>2026-03-21T03:45:08</t>
+          <t>2026-03-21T03:45:09</t>
         </is>
       </c>
     </row>
@@ -2797,7 +2797,7 @@
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>2026-03-21T03:45:08</t>
+          <t>2026-03-21T03:45:09</t>
         </is>
       </c>
     </row>
@@ -2834,7 +2834,7 @@
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>2026-03-21T03:45:08</t>
+          <t>2026-03-21T03:45:09</t>
         </is>
       </c>
     </row>
@@ -2871,7 +2871,7 @@
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>2026-03-21T03:45:08</t>
+          <t>2026-03-21T03:45:09</t>
         </is>
       </c>
     </row>
@@ -2908,7 +2908,7 @@
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>2026-03-21T03:45:08</t>
+          <t>2026-03-21T03:45:09</t>
         </is>
       </c>
     </row>
@@ -2945,7 +2945,7 @@
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>2026-03-21T03:45:08</t>
+          <t>2026-03-21T03:45:09</t>
         </is>
       </c>
     </row>
@@ -2982,7 +2982,7 @@
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>2026-03-21T03:45:08</t>
+          <t>2026-03-21T03:45:09</t>
         </is>
       </c>
     </row>
@@ -3019,7 +3019,7 @@
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>2026-03-21T03:45:08</t>
+          <t>2026-03-21T03:45:09</t>
         </is>
       </c>
     </row>
@@ -3083,7 +3083,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>2026-03-21T03:45:08</t>
+          <t>2026-03-21T03:45:09</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: portfolio snapshot 2026-03-17 (2026-03-21T03:45:29)
</commit_message>
<xml_diff>
--- a/portfolio_auto.xlsx
+++ b/portfolio_auto.xlsx
@@ -471,11 +471,11 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>노브</t>
+          <t>페트로브라스 (ADR)</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>185</v>
+        <v>480</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
@@ -486,23 +486,23 @@
         <v>1</v>
       </c>
       <c r="E2" t="n">
-        <v>5067449</v>
+        <v>13847377</v>
       </c>
       <c r="F2" t="n">
-        <v>1757441</v>
+        <v>1740828</v>
       </c>
       <c r="G2" t="n">
-        <v>53.09476593410047</v>
+        <v>14.37922565712161</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>노블</t>
+          <t>AGNC 인베스트먼트</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>99</v>
+        <v>700</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
@@ -513,23 +513,23 @@
         <v>1</v>
       </c>
       <c r="E3" t="n">
-        <v>6882090</v>
+        <v>10848269</v>
       </c>
       <c r="F3" t="n">
-        <v>2974882</v>
+        <v>16254</v>
       </c>
       <c r="G3" t="n">
-        <v>76.13830643262402</v>
+        <v>0.1500551836385012</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>더치 브로스</t>
+          <t>대한조선</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>39</v>
+        <v>100</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
@@ -540,23 +540,23 @@
         <v>1</v>
       </c>
       <c r="E4" t="n">
-        <v>2926290</v>
+        <v>9740480</v>
       </c>
       <c r="F4" t="n">
-        <v>-264354</v>
+        <v>2527480</v>
       </c>
       <c r="G4" t="n">
-        <v>-8.285286606716387</v>
+        <v>35.04062110079024</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>발레로 에너지</t>
+          <t>프론트라인</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>6</v>
+        <v>175</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -567,23 +567,23 @@
         <v>1</v>
       </c>
       <c r="E5" t="n">
-        <v>2096946</v>
+        <v>8304681.999999999</v>
       </c>
       <c r="F5" t="n">
-        <v>32956</v>
+        <v>3874817.999999999</v>
       </c>
       <c r="G5" t="n">
-        <v>1.596713162369973</v>
+        <v>87.47036026388167</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>센트러스 에너지</t>
+          <t>시드릴</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>21</v>
+        <v>123</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
@@ -594,23 +594,23 @@
         <v>1</v>
       </c>
       <c r="E6" t="n">
-        <v>6691594</v>
+        <v>7927448</v>
       </c>
       <c r="F6" t="n">
-        <v>460375.0000000009</v>
+        <v>1477097</v>
       </c>
       <c r="G6" t="n">
-        <v>7.38820124922589</v>
+        <v>22.89948252428434</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>스타 벌크 캐리어스</t>
+          <t>트랜스오션</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>50</v>
+        <v>750</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -621,23 +621,23 @@
         <v>1</v>
       </c>
       <c r="E7" t="n">
-        <v>1661361</v>
+        <v>6945333</v>
       </c>
       <c r="F7" t="n">
-        <v>347008</v>
+        <v>2818099</v>
       </c>
       <c r="G7" t="n">
-        <v>26.40143097021881</v>
+        <v>68.28057241241955</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>시드릴</t>
+          <t>세아제강</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>123</v>
+        <v>50</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
@@ -648,23 +648,23 @@
         <v>1</v>
       </c>
       <c r="E8" t="n">
-        <v>7927448</v>
+        <v>6896180</v>
       </c>
       <c r="F8" t="n">
-        <v>1477097</v>
+        <v>586180</v>
       </c>
       <c r="G8" t="n">
-        <v>22.89948252428434</v>
+        <v>9.289698890649763</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>오케아니스 에코 탱커스</t>
+          <t>노블</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>65</v>
+        <v>99</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
@@ -675,23 +675,23 @@
         <v>1</v>
       </c>
       <c r="E9" t="n">
-        <v>4451759</v>
+        <v>6882090</v>
       </c>
       <c r="F9" t="n">
-        <v>2195399</v>
+        <v>2974882</v>
       </c>
       <c r="G9" t="n">
-        <v>97.29825914304455</v>
+        <v>76.13830643262402</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>유나이티드헬스 그룹</t>
+          <t>센트러스 에너지</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>4</v>
+        <v>21</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
@@ -702,23 +702,23 @@
         <v>1</v>
       </c>
       <c r="E10" t="n">
-        <v>1710490</v>
+        <v>6691594</v>
       </c>
       <c r="F10" t="n">
-        <v>16034</v>
+        <v>460375.0000000009</v>
       </c>
       <c r="G10" t="n">
-        <v>0.9462623992597033</v>
+        <v>7.38820124922589</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>차코스 에너지 내비게이션</t>
+          <t>타이드워터</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>75</v>
+        <v>48</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
@@ -729,23 +729,23 @@
         <v>1</v>
       </c>
       <c r="E11" t="n">
-        <v>3919272</v>
+        <v>5429641</v>
       </c>
       <c r="F11" t="n">
-        <v>94624</v>
+        <v>1705096</v>
       </c>
       <c r="G11" t="n">
-        <v>2.474057743353114</v>
+        <v>45.7799811789091</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>클리블랜드 클리프스</t>
+          <t>노브</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>70</v>
+        <v>185</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
@@ -756,23 +756,23 @@
         <v>1</v>
       </c>
       <c r="E12" t="n">
-        <v>908091</v>
+        <v>5067449</v>
       </c>
       <c r="F12" t="n">
-        <v>-107964</v>
+        <v>1757441</v>
       </c>
       <c r="G12" t="n">
-        <v>-10.62580273705656</v>
+        <v>53.09476593410047</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>타이드워터</t>
+          <t>TIME 코리아밸류업액티브</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>48</v>
+        <v>201</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
@@ -783,23 +783,23 @@
         <v>1</v>
       </c>
       <c r="E13" t="n">
-        <v>5429641</v>
+        <v>4656165</v>
       </c>
       <c r="F13" t="n">
-        <v>1705096</v>
+        <v>-67632</v>
       </c>
       <c r="G13" t="n">
-        <v>45.7799811789091</v>
+        <v>-1.43172960226699</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>텍사스 퍼시픽 랜드</t>
+          <t>오케아니스 에코 탱커스</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>1</v>
+        <v>65</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
@@ -810,23 +810,23 @@
         <v>1</v>
       </c>
       <c r="E14" t="n">
-        <v>786665</v>
+        <v>4451759</v>
       </c>
       <c r="F14" t="n">
-        <v>8074</v>
+        <v>2195399</v>
       </c>
       <c r="G14" t="n">
-        <v>1.037001455192778</v>
+        <v>97.29825914304455</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>트랜스오션</t>
+          <t>차코스 에너지 내비게이션</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>750</v>
+        <v>75</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
@@ -837,23 +837,23 @@
         <v>1</v>
       </c>
       <c r="E15" t="n">
-        <v>6945333</v>
+        <v>3919272</v>
       </c>
       <c r="F15" t="n">
-        <v>2818099</v>
+        <v>94624</v>
       </c>
       <c r="G15" t="n">
-        <v>68.28057241241955</v>
+        <v>2.474057743353114</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>페트로브라스 (ADR)</t>
+          <t>HD건설기계</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>480</v>
+        <v>31</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
@@ -864,23 +864,23 @@
         <v>1</v>
       </c>
       <c r="E16" t="n">
-        <v>13847377</v>
+        <v>3885810</v>
       </c>
       <c r="F16" t="n">
-        <v>1740828</v>
+        <v>-149286</v>
       </c>
       <c r="G16" t="n">
-        <v>14.37922565712161</v>
+        <v>-3.699688929334023</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>프론트라인</t>
+          <t>동원개발</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>175</v>
+        <v>1360</v>
       </c>
       <c r="C17" t="inlineStr">
         <is>
@@ -891,23 +891,23 @@
         <v>1</v>
       </c>
       <c r="E17" t="n">
-        <v>8304681.999999999</v>
+        <v>3881821</v>
       </c>
       <c r="F17" t="n">
-        <v>3874817.999999999</v>
+        <v>144420.9999999995</v>
       </c>
       <c r="G17" t="n">
-        <v>87.47036026388167</v>
+        <v>3.86421041365654</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>피바디 에너지</t>
+          <t>DL이앤씨</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>65</v>
+        <v>80</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
@@ -918,23 +918,23 @@
         <v>1</v>
       </c>
       <c r="E18" t="n">
-        <v>3427688</v>
+        <v>3792400</v>
       </c>
       <c r="F18" t="n">
-        <v>1956916</v>
+        <v>381400</v>
       </c>
       <c r="G18" t="n">
-        <v>133.0536616144446</v>
+        <v>11.1814717091762</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>하프니아</t>
+          <t>피바디 에너지</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>80</v>
+        <v>65</v>
       </c>
       <c r="C19" t="inlineStr">
         <is>
@@ -945,23 +945,23 @@
         <v>1</v>
       </c>
       <c r="E19" t="n">
-        <v>798051</v>
+        <v>3427688</v>
       </c>
       <c r="F19" t="n">
-        <v>172320</v>
+        <v>1956916</v>
       </c>
       <c r="G19" t="n">
-        <v>27.53899039683186</v>
+        <v>133.0536616144446</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>AGNC 인베스트먼트</t>
+          <t>삼성화재</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>700</v>
+        <v>7</v>
       </c>
       <c r="C20" t="inlineStr">
         <is>
@@ -972,23 +972,23 @@
         <v>1</v>
       </c>
       <c r="E20" t="n">
-        <v>10848269</v>
+        <v>3335815</v>
       </c>
       <c r="F20" t="n">
-        <v>16254</v>
+        <v>-295185</v>
       </c>
       <c r="G20" t="n">
-        <v>0.1500551836385012</v>
+        <v>-8.129578628477004</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>넥스틸</t>
+          <t>더치 브로스</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>200</v>
+        <v>39</v>
       </c>
       <c r="C21" t="inlineStr">
         <is>
@@ -999,23 +999,23 @@
         <v>1</v>
       </c>
       <c r="E21" t="n">
-        <v>2391208</v>
+        <v>2926290</v>
       </c>
       <c r="F21" t="n">
-        <v>380208</v>
+        <v>-264354</v>
       </c>
       <c r="G21" t="n">
-        <v>18.90641471904525</v>
+        <v>-8.285286606716387</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>대신증권</t>
+          <t>KoAct 코스닥액티브</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>55</v>
+        <v>200</v>
       </c>
       <c r="C22" t="inlineStr">
         <is>
@@ -1026,23 +1026,23 @@
         <v>1</v>
       </c>
       <c r="E22" t="n">
-        <v>2190111</v>
+        <v>2580000</v>
       </c>
       <c r="F22" t="n">
-        <v>480610</v>
+        <v>-122000</v>
       </c>
       <c r="G22" t="n">
-        <v>28.11405199528985</v>
+        <v>-4.515173945225759</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>대창단조</t>
+          <t>현대제철</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>300</v>
+        <v>70</v>
       </c>
       <c r="C23" t="inlineStr">
         <is>
@@ -1053,23 +1053,23 @@
         <v>1</v>
       </c>
       <c r="E23" t="n">
-        <v>1901190</v>
+        <v>2494002</v>
       </c>
       <c r="F23" t="n">
-        <v>-156810</v>
+        <v>-313498</v>
       </c>
       <c r="G23" t="n">
-        <v>-7.619533527696793</v>
+        <v>-11.16644701691897</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>대한조선</t>
+          <t>휴스틸</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>100</v>
+        <v>500</v>
       </c>
       <c r="C24" t="inlineStr">
         <is>
@@ -1080,23 +1080,23 @@
         <v>1</v>
       </c>
       <c r="E24" t="n">
-        <v>9740480</v>
+        <v>2450090</v>
       </c>
       <c r="F24" t="n">
-        <v>2527480</v>
+        <v>171480</v>
       </c>
       <c r="G24" t="n">
-        <v>35.04062110079024</v>
+        <v>7.525640631788678</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>동방</t>
+          <t>넥스틸</t>
         </is>
       </c>
       <c r="B25" t="n">
-        <v>681</v>
+        <v>200</v>
       </c>
       <c r="C25" t="inlineStr">
         <is>
@@ -1107,23 +1107,23 @@
         <v>1</v>
       </c>
       <c r="E25" t="n">
-        <v>1841600</v>
+        <v>2391208</v>
       </c>
       <c r="F25" t="n">
-        <v>-129901</v>
+        <v>380208</v>
       </c>
       <c r="G25" t="n">
-        <v>-6.588939087527726</v>
+        <v>18.90641471904525</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>동원개발</t>
+          <t>대신증권</t>
         </is>
       </c>
       <c r="B26" t="n">
-        <v>1360</v>
+        <v>55</v>
       </c>
       <c r="C26" t="inlineStr">
         <is>
@@ -1134,23 +1134,23 @@
         <v>1</v>
       </c>
       <c r="E26" t="n">
-        <v>3881821</v>
+        <v>2190111</v>
       </c>
       <c r="F26" t="n">
-        <v>144420.9999999995</v>
+        <v>480610</v>
       </c>
       <c r="G26" t="n">
-        <v>3.86421041365654</v>
+        <v>28.11405199528985</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>미창석유</t>
+          <t>발레로 에너지</t>
         </is>
       </c>
       <c r="B27" t="n">
-        <v>18</v>
+        <v>6</v>
       </c>
       <c r="C27" t="inlineStr">
         <is>
@@ -1161,23 +1161,23 @@
         <v>1</v>
       </c>
       <c r="E27" t="n">
-        <v>2049693</v>
+        <v>2096946</v>
       </c>
       <c r="F27" t="n">
-        <v>-342507</v>
+        <v>32956</v>
       </c>
       <c r="G27" t="n">
-        <v>-14.31765738650614</v>
+        <v>1.596713162369973</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>비에이치아이</t>
+          <t>미창석유</t>
         </is>
       </c>
       <c r="B28" t="n">
-        <v>8</v>
+        <v>18</v>
       </c>
       <c r="C28" t="inlineStr">
         <is>
@@ -1188,23 +1188,23 @@
         <v>1</v>
       </c>
       <c r="E28" t="n">
-        <v>850296</v>
+        <v>2049693</v>
       </c>
       <c r="F28" t="n">
-        <v>185181</v>
+        <v>-342507</v>
       </c>
       <c r="G28" t="n">
-        <v>27.84195214361426</v>
+        <v>-14.31765738650614</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>삼성생명</t>
+          <t>대창단조</t>
         </is>
       </c>
       <c r="B29" t="n">
-        <v>4</v>
+        <v>300</v>
       </c>
       <c r="C29" t="inlineStr">
         <is>
@@ -1215,23 +1215,23 @@
         <v>1</v>
       </c>
       <c r="E29" t="n">
-        <v>872252</v>
+        <v>1901190</v>
       </c>
       <c r="F29" t="n">
-        <v>39252</v>
+        <v>-156810</v>
       </c>
       <c r="G29" t="n">
-        <v>4.712124849939976</v>
+        <v>-7.619533527696793</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>삼성화재</t>
+          <t>동방</t>
         </is>
       </c>
       <c r="B30" t="n">
-        <v>7</v>
+        <v>681</v>
       </c>
       <c r="C30" t="inlineStr">
         <is>
@@ -1242,23 +1242,23 @@
         <v>1</v>
       </c>
       <c r="E30" t="n">
-        <v>3335815</v>
+        <v>1841600</v>
       </c>
       <c r="F30" t="n">
-        <v>-295185</v>
+        <v>-129901</v>
       </c>
       <c r="G30" t="n">
-        <v>-8.129578628477004</v>
+        <v>-6.588939087527726</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>세아제강</t>
+          <t>유나이티드헬스 그룹</t>
         </is>
       </c>
       <c r="B31" t="n">
-        <v>50</v>
+        <v>4</v>
       </c>
       <c r="C31" t="inlineStr">
         <is>
@@ -1269,19 +1269,19 @@
         <v>1</v>
       </c>
       <c r="E31" t="n">
-        <v>6896180</v>
+        <v>1710490</v>
       </c>
       <c r="F31" t="n">
-        <v>586180</v>
+        <v>16034</v>
       </c>
       <c r="G31" t="n">
-        <v>9.289698890649763</v>
+        <v>0.9462623992597033</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>케이씨</t>
+          <t>스타 벌크 캐리어스</t>
         </is>
       </c>
       <c r="B32" t="n">
@@ -1296,23 +1296,23 @@
         <v>1</v>
       </c>
       <c r="E32" t="n">
-        <v>1576840</v>
+        <v>1661361</v>
       </c>
       <c r="F32" t="n">
-        <v>-72660</v>
+        <v>347008</v>
       </c>
       <c r="G32" t="n">
-        <v>-4.404971203394968</v>
+        <v>26.40143097021881</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>하나금융지주</t>
+          <t>케이씨</t>
         </is>
       </c>
       <c r="B33" t="n">
-        <v>10</v>
+        <v>50</v>
       </c>
       <c r="C33" t="inlineStr">
         <is>
@@ -1323,23 +1323,23 @@
         <v>1</v>
       </c>
       <c r="E33" t="n">
-        <v>1107780</v>
+        <v>1576840</v>
       </c>
       <c r="F33" t="n">
-        <v>-1220</v>
+        <v>-72660</v>
       </c>
       <c r="G33" t="n">
-        <v>-0.1100090171325518</v>
+        <v>-4.404971203394968</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>현대제철</t>
+          <t>하나금융지주</t>
         </is>
       </c>
       <c r="B34" t="n">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="C34" t="inlineStr">
         <is>
@@ -1350,23 +1350,23 @@
         <v>1</v>
       </c>
       <c r="E34" t="n">
-        <v>2494002</v>
+        <v>1107780</v>
       </c>
       <c r="F34" t="n">
-        <v>-313498</v>
+        <v>-1220</v>
       </c>
       <c r="G34" t="n">
-        <v>-11.16644701691897</v>
+        <v>-0.1100090171325518</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>휴스틸</t>
+          <t>클리블랜드 클리프스</t>
         </is>
       </c>
       <c r="B35" t="n">
-        <v>500</v>
+        <v>70</v>
       </c>
       <c r="C35" t="inlineStr">
         <is>
@@ -1377,23 +1377,23 @@
         <v>1</v>
       </c>
       <c r="E35" t="n">
-        <v>2450090</v>
+        <v>908091</v>
       </c>
       <c r="F35" t="n">
-        <v>171480</v>
+        <v>-107964</v>
       </c>
       <c r="G35" t="n">
-        <v>7.525640631788678</v>
+        <v>-10.62580273705656</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>DL이앤씨</t>
+          <t>삼성생명</t>
         </is>
       </c>
       <c r="B36" t="n">
-        <v>80</v>
+        <v>4</v>
       </c>
       <c r="C36" t="inlineStr">
         <is>
@@ -1404,23 +1404,23 @@
         <v>1</v>
       </c>
       <c r="E36" t="n">
-        <v>3792400</v>
+        <v>872252</v>
       </c>
       <c r="F36" t="n">
-        <v>381400</v>
+        <v>39252</v>
       </c>
       <c r="G36" t="n">
-        <v>11.1814717091762</v>
+        <v>4.712124849939976</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>HD건설기계</t>
+          <t>비에이치아이</t>
         </is>
       </c>
       <c r="B37" t="n">
-        <v>31</v>
+        <v>8</v>
       </c>
       <c r="C37" t="inlineStr">
         <is>
@@ -1431,23 +1431,23 @@
         <v>1</v>
       </c>
       <c r="E37" t="n">
-        <v>3885810</v>
+        <v>850296</v>
       </c>
       <c r="F37" t="n">
-        <v>-149286</v>
+        <v>185181</v>
       </c>
       <c r="G37" t="n">
-        <v>-3.699688929334023</v>
+        <v>27.84195214361426</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>KoAct 코스닥액티브</t>
+          <t>하프니아</t>
         </is>
       </c>
       <c r="B38" t="n">
-        <v>200</v>
+        <v>80</v>
       </c>
       <c r="C38" t="inlineStr">
         <is>
@@ -1458,23 +1458,23 @@
         <v>1</v>
       </c>
       <c r="E38" t="n">
-        <v>2580000</v>
+        <v>798051</v>
       </c>
       <c r="F38" t="n">
-        <v>-122000</v>
+        <v>172320</v>
       </c>
       <c r="G38" t="n">
-        <v>-4.515173945225759</v>
+        <v>27.53899039683186</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>TIME 코리아밸류업액티브</t>
+          <t>텍사스 퍼시픽 랜드</t>
         </is>
       </c>
       <c r="B39" t="n">
-        <v>201</v>
+        <v>1</v>
       </c>
       <c r="C39" t="inlineStr">
         <is>
@@ -1485,13 +1485,13 @@
         <v>1</v>
       </c>
       <c r="E39" t="n">
-        <v>4656165</v>
+        <v>786665</v>
       </c>
       <c r="F39" t="n">
-        <v>-67632</v>
+        <v>8074</v>
       </c>
       <c r="G39" t="n">
-        <v>-1.43172960226699</v>
+        <v>1.037001455192778</v>
       </c>
     </row>
   </sheetData>
@@ -1542,14 +1542,14 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0</v>
+        <v>33078556</v>
       </c>
       <c r="C2" t="n">
-        <v>0</v>
+        <v>6010.99</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2026-03-21T03:45:09</t>
+          <t>2026-03-21T03:45:29</t>
         </is>
       </c>
       <c r="E2" t="n">
@@ -3071,10 +3071,10 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0</v>
+        <v>33078556</v>
       </c>
       <c r="C2" t="n">
-        <v>0</v>
+        <v>6010.99</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
@@ -3083,7 +3083,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>2026-03-21T03:45:09</t>
+          <t>2026-03-21T03:45:29</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: portfolio snapshot 2026-03-17 (2026-03-21T03:46:22)
</commit_message>
<xml_diff>
--- a/portfolio_auto.xlsx
+++ b/portfolio_auto.xlsx
@@ -471,11 +471,11 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>페트로브라스 (ADR)</t>
+          <t>노브</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>480</v>
+        <v>185</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
@@ -486,23 +486,23 @@
         <v>1</v>
       </c>
       <c r="E2" t="n">
-        <v>13847377</v>
+        <v>5200391.447092756</v>
       </c>
       <c r="F2" t="n">
-        <v>1740828</v>
+        <v>1890383.447092756</v>
       </c>
       <c r="G2" t="n">
-        <v>14.37922565712161</v>
+        <v>57.11114435653194</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>AGNC 인베스트먼트</t>
+          <t>노블</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>700</v>
+        <v>99</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
@@ -513,23 +513,23 @@
         <v>1</v>
       </c>
       <c r="E3" t="n">
-        <v>10848269</v>
+        <v>40689</v>
       </c>
       <c r="F3" t="n">
-        <v>16254</v>
+        <v>-3866519</v>
       </c>
       <c r="G3" t="n">
-        <v>0.1500551836385012</v>
+        <v>-98.95861699709869</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>대한조선</t>
+          <t>더치 브로스</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>100</v>
+        <v>39</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
@@ -540,23 +540,23 @@
         <v>1</v>
       </c>
       <c r="E4" t="n">
-        <v>9740480</v>
+        <v>2934418.414306641</v>
       </c>
       <c r="F4" t="n">
-        <v>2527480</v>
+        <v>-256225.5856933594</v>
       </c>
       <c r="G4" t="n">
-        <v>35.04062110079024</v>
+        <v>-8.030528811530193</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>프론트라인</t>
+          <t>발레로 에너지</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>175</v>
+        <v>6</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -567,23 +567,23 @@
         <v>1</v>
       </c>
       <c r="E5" t="n">
-        <v>8304681.999999999</v>
+        <v>2165691.085066516</v>
       </c>
       <c r="F5" t="n">
-        <v>3874817.999999999</v>
+        <v>101701.085066516</v>
       </c>
       <c r="G5" t="n">
-        <v>87.47036026388167</v>
+        <v>4.927402025519307</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>시드릴</t>
+          <t>센트러스 에너지</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>123</v>
+        <v>21</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
@@ -594,23 +594,23 @@
         <v>1</v>
       </c>
       <c r="E6" t="n">
-        <v>7927448</v>
+        <v>5901882.720856408</v>
       </c>
       <c r="F6" t="n">
-        <v>1477097</v>
+        <v>-329336.2791435914</v>
       </c>
       <c r="G6" t="n">
-        <v>22.89948252428434</v>
+        <v>-5.285262468605123</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>트랜스오션</t>
+          <t>스타 벌크 캐리어스</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>750</v>
+        <v>50</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -621,23 +621,23 @@
         <v>1</v>
       </c>
       <c r="E7" t="n">
-        <v>6945333</v>
+        <v>1680142.640194588</v>
       </c>
       <c r="F7" t="n">
-        <v>2818099</v>
+        <v>365789.6401945879</v>
       </c>
       <c r="G7" t="n">
-        <v>68.28057241241955</v>
+        <v>27.83039565433242</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>세아제강</t>
+          <t>시드릴</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>50</v>
+        <v>123</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
@@ -648,23 +648,23 @@
         <v>1</v>
       </c>
       <c r="E8" t="n">
-        <v>6896180</v>
+        <v>8070101.805898919</v>
       </c>
       <c r="F8" t="n">
-        <v>586180</v>
+        <v>1619750.805898919</v>
       </c>
       <c r="G8" t="n">
-        <v>9.289698890649763</v>
+        <v>25.11104908707943</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>노블</t>
+          <t>오케아니스 에코 탱커스</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>99</v>
+        <v>65</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
@@ -675,23 +675,23 @@
         <v>1</v>
       </c>
       <c r="E9" t="n">
-        <v>6882090</v>
+        <v>4511179.137784176</v>
       </c>
       <c r="F9" t="n">
-        <v>2974882</v>
+        <v>2254819.137784176</v>
       </c>
       <c r="G9" t="n">
-        <v>76.13830643262402</v>
+        <v>99.93171026716374</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>센트러스 에너지</t>
+          <t>유나이티드헬스 그룹</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>21</v>
+        <v>4</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
@@ -702,23 +702,23 @@
         <v>1</v>
       </c>
       <c r="E10" t="n">
-        <v>6691594</v>
+        <v>1658864.328313038</v>
       </c>
       <c r="F10" t="n">
-        <v>460375.0000000009</v>
+        <v>-35591.67168696225</v>
       </c>
       <c r="G10" t="n">
-        <v>7.38820124922589</v>
+        <v>-2.100477774988684</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>타이드워터</t>
+          <t>차코스 에너지 내비게이션</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>48</v>
+        <v>75</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
@@ -729,23 +729,23 @@
         <v>1</v>
       </c>
       <c r="E11" t="n">
-        <v>5429641</v>
+        <v>4026924.996845168</v>
       </c>
       <c r="F11" t="n">
-        <v>1705096</v>
+        <v>202276.9968451681</v>
       </c>
       <c r="G11" t="n">
-        <v>45.7799811789091</v>
+        <v>5.28877420471552</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>노브</t>
+          <t>클리블랜드 클리프스</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>185</v>
+        <v>70</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
@@ -756,23 +756,23 @@
         <v>1</v>
       </c>
       <c r="E12" t="n">
-        <v>5067449</v>
+        <v>823743.9360268187</v>
       </c>
       <c r="F12" t="n">
-        <v>1757441</v>
+        <v>-192311.0639731813</v>
       </c>
       <c r="G12" t="n">
-        <v>53.09476593410047</v>
+        <v>-18.92722972409774</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>TIME 코리아밸류업액티브</t>
+          <t>타이드워터</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>201</v>
+        <v>48</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
@@ -783,23 +783,23 @@
         <v>1</v>
       </c>
       <c r="E13" t="n">
-        <v>4656165</v>
+        <v>5235363.852789983</v>
       </c>
       <c r="F13" t="n">
-        <v>-67632</v>
+        <v>1510818.852789983</v>
       </c>
       <c r="G13" t="n">
-        <v>-1.43172960226699</v>
+        <v>40.56385015592463</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>오케아니스 에코 탱커스</t>
+          <t>텍사스 퍼시픽 랜드</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>65</v>
+        <v>1</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
@@ -810,23 +810,23 @@
         <v>1</v>
       </c>
       <c r="E14" t="n">
-        <v>4451759</v>
+        <v>781623.6870614514</v>
       </c>
       <c r="F14" t="n">
-        <v>2195399</v>
+        <v>3032.687061451375</v>
       </c>
       <c r="G14" t="n">
-        <v>97.29825914304455</v>
+        <v>0.3895096477420591</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>차코스 에너지 내비게이션</t>
+          <t>트랜스오션</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>75</v>
+        <v>750</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
@@ -837,23 +837,23 @@
         <v>1</v>
       </c>
       <c r="E15" t="n">
-        <v>3919272</v>
+        <v>7020031.5082007</v>
       </c>
       <c r="F15" t="n">
-        <v>94624</v>
+        <v>2892797.5082007</v>
       </c>
       <c r="G15" t="n">
-        <v>2.474057743353114</v>
+        <v>70.09046514446965</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>HD건설기계</t>
+          <t>페트로브라스 (ADR)</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>31</v>
+        <v>480</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
@@ -864,23 +864,23 @@
         <v>1</v>
       </c>
       <c r="E16" t="n">
-        <v>3885810</v>
+        <v>13579584.97235231</v>
       </c>
       <c r="F16" t="n">
-        <v>-149286</v>
+        <v>1473035.972352311</v>
       </c>
       <c r="G16" t="n">
-        <v>-3.699688929334023</v>
+        <v>12.16726560436265</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>동원개발</t>
+          <t>프론트라인</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>1360</v>
+        <v>175</v>
       </c>
       <c r="C17" t="inlineStr">
         <is>
@@ -891,23 +891,23 @@
         <v>1</v>
       </c>
       <c r="E17" t="n">
-        <v>3881821</v>
+        <v>8471815.962899337</v>
       </c>
       <c r="F17" t="n">
-        <v>144420.9999999995</v>
+        <v>4041951.962899337</v>
       </c>
       <c r="G17" t="n">
-        <v>3.86421041365654</v>
+        <v>91.24325177701475</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>DL이앤씨</t>
+          <t>피바디 에너지</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>80</v>
+        <v>65</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
@@ -918,23 +918,23 @@
         <v>1</v>
       </c>
       <c r="E18" t="n">
-        <v>3792400</v>
+        <v>3649438.50225304</v>
       </c>
       <c r="F18" t="n">
-        <v>381400</v>
+        <v>2178666.50225304</v>
       </c>
       <c r="G18" t="n">
-        <v>11.1814717091762</v>
+        <v>148.1308117269733</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>피바디 에너지</t>
+          <t>하프니아</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>65</v>
+        <v>80</v>
       </c>
       <c r="C19" t="inlineStr">
         <is>
@@ -945,23 +945,23 @@
         <v>1</v>
       </c>
       <c r="E19" t="n">
-        <v>3427688</v>
+        <v>798051</v>
       </c>
       <c r="F19" t="n">
-        <v>1956916</v>
+        <v>172320</v>
       </c>
       <c r="G19" t="n">
-        <v>133.0536616144446</v>
+        <v>27.53899039683186</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>삼성화재</t>
+          <t>AGNC 인베스트먼트</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>7</v>
+        <v>700</v>
       </c>
       <c r="C20" t="inlineStr">
         <is>
@@ -972,23 +972,23 @@
         <v>1</v>
       </c>
       <c r="E20" t="n">
-        <v>3335815</v>
+        <v>10270464.45007324</v>
       </c>
       <c r="F20" t="n">
-        <v>-295185</v>
+        <v>-561550.5499267578</v>
       </c>
       <c r="G20" t="n">
-        <v>-8.129578628477004</v>
+        <v>-5.184174411933125</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>더치 브로스</t>
+          <t>넥스틸</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>39</v>
+        <v>200</v>
       </c>
       <c r="C21" t="inlineStr">
         <is>
@@ -999,23 +999,23 @@
         <v>1</v>
       </c>
       <c r="E21" t="n">
-        <v>2926290</v>
+        <v>2514000</v>
       </c>
       <c r="F21" t="n">
-        <v>-264354</v>
+        <v>503000</v>
       </c>
       <c r="G21" t="n">
-        <v>-8.285286606716387</v>
+        <v>25.01243162605669</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>KoAct 코스닥액티브</t>
+          <t>대신증권</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>200</v>
+        <v>55</v>
       </c>
       <c r="C22" t="inlineStr">
         <is>
@@ -1026,23 +1026,23 @@
         <v>1</v>
       </c>
       <c r="E22" t="n">
-        <v>2580000</v>
+        <v>2219250</v>
       </c>
       <c r="F22" t="n">
-        <v>-122000</v>
+        <v>509749</v>
       </c>
       <c r="G22" t="n">
-        <v>-4.515173945225759</v>
+        <v>29.81858448752005</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>현대제철</t>
+          <t>대창단조</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>70</v>
+        <v>300</v>
       </c>
       <c r="C23" t="inlineStr">
         <is>
@@ -1053,23 +1053,23 @@
         <v>1</v>
       </c>
       <c r="E23" t="n">
-        <v>2494002</v>
+        <v>2004000</v>
       </c>
       <c r="F23" t="n">
-        <v>-313498</v>
+        <v>-54000</v>
       </c>
       <c r="G23" t="n">
-        <v>-11.16644701691897</v>
+        <v>-2.623906705539359</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>휴스틸</t>
+          <t>대한조선</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>500</v>
+        <v>100</v>
       </c>
       <c r="C24" t="inlineStr">
         <is>
@@ -1080,23 +1080,23 @@
         <v>1</v>
       </c>
       <c r="E24" t="n">
-        <v>2450090</v>
+        <v>9120000</v>
       </c>
       <c r="F24" t="n">
-        <v>171480</v>
+        <v>1907000</v>
       </c>
       <c r="G24" t="n">
-        <v>7.525640631788678</v>
+        <v>26.43837515596839</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>넥스틸</t>
+          <t>동방</t>
         </is>
       </c>
       <c r="B25" t="n">
-        <v>200</v>
+        <v>681</v>
       </c>
       <c r="C25" t="inlineStr">
         <is>
@@ -1107,23 +1107,23 @@
         <v>1</v>
       </c>
       <c r="E25" t="n">
-        <v>2391208</v>
+        <v>1995330</v>
       </c>
       <c r="F25" t="n">
-        <v>380208</v>
+        <v>23829</v>
       </c>
       <c r="G25" t="n">
-        <v>18.90641471904525</v>
+        <v>1.208672985709873</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>대신증권</t>
+          <t>동원개발</t>
         </is>
       </c>
       <c r="B26" t="n">
-        <v>55</v>
+        <v>1360</v>
       </c>
       <c r="C26" t="inlineStr">
         <is>
@@ -1134,23 +1134,23 @@
         <v>1</v>
       </c>
       <c r="E26" t="n">
-        <v>2190111</v>
+        <v>4202400</v>
       </c>
       <c r="F26" t="n">
-        <v>480610</v>
+        <v>465000</v>
       </c>
       <c r="G26" t="n">
-        <v>28.11405199528985</v>
+        <v>12.44180446299566</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>발레로 에너지</t>
+          <t>미창석유</t>
         </is>
       </c>
       <c r="B27" t="n">
-        <v>6</v>
+        <v>18</v>
       </c>
       <c r="C27" t="inlineStr">
         <is>
@@ -1161,23 +1161,23 @@
         <v>1</v>
       </c>
       <c r="E27" t="n">
-        <v>2096946</v>
+        <v>2097000</v>
       </c>
       <c r="F27" t="n">
-        <v>32956</v>
+        <v>-295200</v>
       </c>
       <c r="G27" t="n">
-        <v>1.596713162369973</v>
+        <v>-12.34010534236268</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>미창석유</t>
+          <t>비에이치아이</t>
         </is>
       </c>
       <c r="B28" t="n">
-        <v>18</v>
+        <v>8</v>
       </c>
       <c r="C28" t="inlineStr">
         <is>
@@ -1188,23 +1188,23 @@
         <v>1</v>
       </c>
       <c r="E28" t="n">
-        <v>2049693</v>
+        <v>876000</v>
       </c>
       <c r="F28" t="n">
-        <v>-342507</v>
+        <v>210885</v>
       </c>
       <c r="G28" t="n">
-        <v>-14.31765738650614</v>
+        <v>31.70654698811484</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>대창단조</t>
+          <t>삼성생명</t>
         </is>
       </c>
       <c r="B29" t="n">
-        <v>300</v>
+        <v>4</v>
       </c>
       <c r="C29" t="inlineStr">
         <is>
@@ -1215,23 +1215,23 @@
         <v>1</v>
       </c>
       <c r="E29" t="n">
-        <v>1901190</v>
+        <v>926000</v>
       </c>
       <c r="F29" t="n">
-        <v>-156810</v>
+        <v>93000</v>
       </c>
       <c r="G29" t="n">
-        <v>-7.619533527696793</v>
+        <v>11.16446578631453</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>동방</t>
+          <t>삼성화재</t>
         </is>
       </c>
       <c r="B30" t="n">
-        <v>681</v>
+        <v>7</v>
       </c>
       <c r="C30" t="inlineStr">
         <is>
@@ -1242,23 +1242,23 @@
         <v>1</v>
       </c>
       <c r="E30" t="n">
-        <v>1841600</v>
+        <v>3321500</v>
       </c>
       <c r="F30" t="n">
-        <v>-129901</v>
+        <v>-309500</v>
       </c>
       <c r="G30" t="n">
-        <v>-6.588939087527726</v>
+        <v>-8.523822638391627</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>유나이티드헬스 그룹</t>
+          <t>세아제강</t>
         </is>
       </c>
       <c r="B31" t="n">
-        <v>4</v>
+        <v>50</v>
       </c>
       <c r="C31" t="inlineStr">
         <is>
@@ -1269,19 +1269,19 @@
         <v>1</v>
       </c>
       <c r="E31" t="n">
-        <v>1710490</v>
+        <v>7395000</v>
       </c>
       <c r="F31" t="n">
-        <v>16034</v>
+        <v>1085000</v>
       </c>
       <c r="G31" t="n">
-        <v>0.9462623992597033</v>
+        <v>17.19492868462758</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>스타 벌크 캐리어스</t>
+          <t>케이씨</t>
         </is>
       </c>
       <c r="B32" t="n">
@@ -1296,23 +1296,23 @@
         <v>1</v>
       </c>
       <c r="E32" t="n">
-        <v>1661361</v>
+        <v>1670000</v>
       </c>
       <c r="F32" t="n">
-        <v>347008</v>
+        <v>20500</v>
       </c>
       <c r="G32" t="n">
-        <v>26.40143097021881</v>
+        <v>1.242800848742043</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>케이씨</t>
+          <t>하나금융지주</t>
         </is>
       </c>
       <c r="B33" t="n">
-        <v>50</v>
+        <v>10</v>
       </c>
       <c r="C33" t="inlineStr">
         <is>
@@ -1323,23 +1323,23 @@
         <v>1</v>
       </c>
       <c r="E33" t="n">
-        <v>1576840</v>
+        <v>1132000</v>
       </c>
       <c r="F33" t="n">
-        <v>-72660</v>
+        <v>23000</v>
       </c>
       <c r="G33" t="n">
-        <v>-4.404971203394968</v>
+        <v>2.073940486925157</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>하나금융지주</t>
+          <t>현대제철</t>
         </is>
       </c>
       <c r="B34" t="n">
-        <v>10</v>
+        <v>70</v>
       </c>
       <c r="C34" t="inlineStr">
         <is>
@@ -1350,23 +1350,23 @@
         <v>1</v>
       </c>
       <c r="E34" t="n">
-        <v>1107780</v>
+        <v>2621500</v>
       </c>
       <c r="F34" t="n">
-        <v>-1220</v>
+        <v>-186000</v>
       </c>
       <c r="G34" t="n">
-        <v>-0.1100090171325518</v>
+        <v>-6.625111308993767</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>클리블랜드 클리프스</t>
+          <t>휴스틸</t>
         </is>
       </c>
       <c r="B35" t="n">
-        <v>70</v>
+        <v>500</v>
       </c>
       <c r="C35" t="inlineStr">
         <is>
@@ -1377,23 +1377,23 @@
         <v>1</v>
       </c>
       <c r="E35" t="n">
-        <v>908091</v>
+        <v>2750000</v>
       </c>
       <c r="F35" t="n">
-        <v>-107964</v>
+        <v>471390</v>
       </c>
       <c r="G35" t="n">
-        <v>-10.62580273705656</v>
+        <v>20.68761218462133</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>삼성생명</t>
+          <t>DL이앤씨</t>
         </is>
       </c>
       <c r="B36" t="n">
-        <v>4</v>
+        <v>80</v>
       </c>
       <c r="C36" t="inlineStr">
         <is>
@@ -1404,23 +1404,23 @@
         <v>1</v>
       </c>
       <c r="E36" t="n">
-        <v>872252</v>
+        <v>5392000</v>
       </c>
       <c r="F36" t="n">
-        <v>39252</v>
+        <v>1981000</v>
       </c>
       <c r="G36" t="n">
-        <v>4.712124849939976</v>
+        <v>58.07681031955438</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>비에이치아이</t>
+          <t>HD건설기계</t>
         </is>
       </c>
       <c r="B37" t="n">
-        <v>8</v>
+        <v>31</v>
       </c>
       <c r="C37" t="inlineStr">
         <is>
@@ -1431,23 +1431,23 @@
         <v>1</v>
       </c>
       <c r="E37" t="n">
-        <v>850296</v>
+        <v>4123000</v>
       </c>
       <c r="F37" t="n">
-        <v>185181</v>
+        <v>87904</v>
       </c>
       <c r="G37" t="n">
-        <v>27.84195214361426</v>
+        <v>2.178485964150543</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>하프니아</t>
+          <t>KoAct 코스닥액티브</t>
         </is>
       </c>
       <c r="B38" t="n">
-        <v>80</v>
+        <v>200</v>
       </c>
       <c r="C38" t="inlineStr">
         <is>
@@ -1458,23 +1458,23 @@
         <v>1</v>
       </c>
       <c r="E38" t="n">
-        <v>798051</v>
+        <v>2582000</v>
       </c>
       <c r="F38" t="n">
-        <v>172320</v>
+        <v>-120000</v>
       </c>
       <c r="G38" t="n">
-        <v>27.53899039683186</v>
+        <v>-4.441154700222058</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>텍사스 퍼시픽 랜드</t>
+          <t>TIME 코리아밸류업액티브</t>
         </is>
       </c>
       <c r="B39" t="n">
-        <v>1</v>
+        <v>201</v>
       </c>
       <c r="C39" t="inlineStr">
         <is>
@@ -1485,13 +1485,13 @@
         <v>1</v>
       </c>
       <c r="E39" t="n">
-        <v>786665</v>
+        <v>4797870</v>
       </c>
       <c r="F39" t="n">
-        <v>8074</v>
+        <v>74073</v>
       </c>
       <c r="G39" t="n">
-        <v>1.037001455192778</v>
+        <v>1.568081778281328</v>
       </c>
     </row>
   </sheetData>
@@ -1549,7 +1549,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2026-03-21T03:45:29</t>
+          <t>2026-03-21T03:46:22</t>
         </is>
       </c>
       <c r="E2" t="n">
@@ -1640,17 +1640,17 @@
         <v>1</v>
       </c>
       <c r="F2" t="n">
-        <v>13847377</v>
+        <v>13579584.97235231</v>
       </c>
       <c r="G2" t="n">
-        <v>1740828</v>
+        <v>1473035.972352311</v>
       </c>
       <c r="H2" t="n">
-        <v>14.37922565712161</v>
+        <v>12.16726560436265</v>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>2026-03-21T03:45:09</t>
+          <t>2026-03-21T03:46:22</t>
         </is>
       </c>
     </row>
@@ -1677,17 +1677,17 @@
         <v>1</v>
       </c>
       <c r="F3" t="n">
-        <v>10848269</v>
+        <v>10270464.45007324</v>
       </c>
       <c r="G3" t="n">
-        <v>16254</v>
+        <v>-561550.5499267578</v>
       </c>
       <c r="H3" t="n">
-        <v>0.1500551836385012</v>
+        <v>-5.184174411933125</v>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>2026-03-21T03:45:09</t>
+          <t>2026-03-21T03:46:22</t>
         </is>
       </c>
     </row>
@@ -1714,17 +1714,17 @@
         <v>1</v>
       </c>
       <c r="F4" t="n">
-        <v>9740480</v>
+        <v>9120000</v>
       </c>
       <c r="G4" t="n">
-        <v>2527480</v>
+        <v>1907000</v>
       </c>
       <c r="H4" t="n">
-        <v>35.04062110079024</v>
+        <v>26.43837515596839</v>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>2026-03-21T03:45:09</t>
+          <t>2026-03-21T03:46:22</t>
         </is>
       </c>
     </row>
@@ -1751,17 +1751,17 @@
         <v>1</v>
       </c>
       <c r="F5" t="n">
-        <v>8304681.999999999</v>
+        <v>8471815.962899337</v>
       </c>
       <c r="G5" t="n">
-        <v>3874817.999999999</v>
+        <v>4041951.962899337</v>
       </c>
       <c r="H5" t="n">
-        <v>87.47036026388167</v>
+        <v>91.24325177701475</v>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>2026-03-21T03:45:09</t>
+          <t>2026-03-21T03:46:22</t>
         </is>
       </c>
     </row>
@@ -1788,17 +1788,17 @@
         <v>1</v>
       </c>
       <c r="F6" t="n">
-        <v>7927448</v>
+        <v>8070101.805898919</v>
       </c>
       <c r="G6" t="n">
-        <v>1477097</v>
+        <v>1619750.805898919</v>
       </c>
       <c r="H6" t="n">
-        <v>22.89948252428434</v>
+        <v>25.11104908707943</v>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>2026-03-21T03:45:09</t>
+          <t>2026-03-21T03:46:22</t>
         </is>
       </c>
     </row>
@@ -1810,11 +1810,11 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>트랜스오션</t>
+          <t>세아제강</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>750</v>
+        <v>50</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
@@ -1825,17 +1825,17 @@
         <v>1</v>
       </c>
       <c r="F7" t="n">
-        <v>6945333</v>
+        <v>7395000</v>
       </c>
       <c r="G7" t="n">
-        <v>2818099</v>
+        <v>1085000</v>
       </c>
       <c r="H7" t="n">
-        <v>68.28057241241955</v>
+        <v>17.19492868462758</v>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>2026-03-21T03:45:09</t>
+          <t>2026-03-21T03:46:22</t>
         </is>
       </c>
     </row>
@@ -1847,11 +1847,11 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>세아제강</t>
+          <t>트랜스오션</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>50</v>
+        <v>750</v>
       </c>
       <c r="D8" t="inlineStr">
         <is>
@@ -1862,17 +1862,17 @@
         <v>1</v>
       </c>
       <c r="F8" t="n">
-        <v>6896180</v>
+        <v>7020031.5082007</v>
       </c>
       <c r="G8" t="n">
-        <v>586180</v>
+        <v>2892797.5082007</v>
       </c>
       <c r="H8" t="n">
-        <v>9.289698890649763</v>
+        <v>70.09046514446965</v>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>2026-03-21T03:45:09</t>
+          <t>2026-03-21T03:46:22</t>
         </is>
       </c>
     </row>
@@ -1884,11 +1884,11 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>노블</t>
+          <t>센트러스 에너지</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>99</v>
+        <v>21</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
@@ -1899,17 +1899,17 @@
         <v>1</v>
       </c>
       <c r="F9" t="n">
-        <v>6882090</v>
+        <v>5901882.720856408</v>
       </c>
       <c r="G9" t="n">
-        <v>2974882</v>
+        <v>-329336.2791435914</v>
       </c>
       <c r="H9" t="n">
-        <v>76.13830643262402</v>
+        <v>-5.285262468605123</v>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>2026-03-21T03:45:09</t>
+          <t>2026-03-21T03:46:22</t>
         </is>
       </c>
     </row>
@@ -1921,11 +1921,11 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>센트러스 에너지</t>
+          <t>DL이앤씨</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>21</v>
+        <v>80</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
@@ -1936,17 +1936,17 @@
         <v>1</v>
       </c>
       <c r="F10" t="n">
-        <v>6691594</v>
+        <v>5392000</v>
       </c>
       <c r="G10" t="n">
-        <v>460375.0000000009</v>
+        <v>1981000</v>
       </c>
       <c r="H10" t="n">
-        <v>7.38820124922589</v>
+        <v>58.07681031955438</v>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>2026-03-21T03:45:09</t>
+          <t>2026-03-21T03:46:22</t>
         </is>
       </c>
     </row>
@@ -1973,17 +1973,17 @@
         <v>1</v>
       </c>
       <c r="F11" t="n">
-        <v>5429641</v>
+        <v>5235363.852789983</v>
       </c>
       <c r="G11" t="n">
-        <v>1705096</v>
+        <v>1510818.852789983</v>
       </c>
       <c r="H11" t="n">
-        <v>45.7799811789091</v>
+        <v>40.56385015592463</v>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>2026-03-21T03:45:09</t>
+          <t>2026-03-21T03:46:22</t>
         </is>
       </c>
     </row>
@@ -2010,17 +2010,17 @@
         <v>1</v>
       </c>
       <c r="F12" t="n">
-        <v>5067449</v>
+        <v>5200391.447092756</v>
       </c>
       <c r="G12" t="n">
-        <v>1757441</v>
+        <v>1890383.447092756</v>
       </c>
       <c r="H12" t="n">
-        <v>53.09476593410047</v>
+        <v>57.11114435653194</v>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>2026-03-21T03:45:09</t>
+          <t>2026-03-21T03:46:22</t>
         </is>
       </c>
     </row>
@@ -2047,17 +2047,17 @@
         <v>1</v>
       </c>
       <c r="F13" t="n">
-        <v>4656165</v>
+        <v>4797870</v>
       </c>
       <c r="G13" t="n">
-        <v>-67632</v>
+        <v>74073</v>
       </c>
       <c r="H13" t="n">
-        <v>-1.43172960226699</v>
+        <v>1.568081778281328</v>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>2026-03-21T03:45:09</t>
+          <t>2026-03-21T03:46:22</t>
         </is>
       </c>
     </row>
@@ -2084,17 +2084,17 @@
         <v>1</v>
       </c>
       <c r="F14" t="n">
-        <v>4451759</v>
+        <v>4511179.137784176</v>
       </c>
       <c r="G14" t="n">
-        <v>2195399</v>
+        <v>2254819.137784176</v>
       </c>
       <c r="H14" t="n">
-        <v>97.29825914304455</v>
+        <v>99.93171026716374</v>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>2026-03-21T03:45:09</t>
+          <t>2026-03-21T03:46:22</t>
         </is>
       </c>
     </row>
@@ -2106,11 +2106,11 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>차코스 에너지 내비게이션</t>
+          <t>동원개발</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>75</v>
+        <v>1360</v>
       </c>
       <c r="D15" t="inlineStr">
         <is>
@@ -2121,17 +2121,17 @@
         <v>1</v>
       </c>
       <c r="F15" t="n">
-        <v>3919272</v>
+        <v>4202400</v>
       </c>
       <c r="G15" t="n">
-        <v>94624</v>
+        <v>465000</v>
       </c>
       <c r="H15" t="n">
-        <v>2.474057743353114</v>
+        <v>12.44180446299566</v>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>2026-03-21T03:45:09</t>
+          <t>2026-03-21T03:46:22</t>
         </is>
       </c>
     </row>
@@ -2158,17 +2158,17 @@
         <v>1</v>
       </c>
       <c r="F16" t="n">
-        <v>3885810</v>
+        <v>4123000</v>
       </c>
       <c r="G16" t="n">
-        <v>-149286</v>
+        <v>87904</v>
       </c>
       <c r="H16" t="n">
-        <v>-3.699688929334023</v>
+        <v>2.178485964150543</v>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>2026-03-21T03:45:09</t>
+          <t>2026-03-21T03:46:22</t>
         </is>
       </c>
     </row>
@@ -2180,11 +2180,11 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>동원개발</t>
+          <t>차코스 에너지 내비게이션</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>1360</v>
+        <v>75</v>
       </c>
       <c r="D17" t="inlineStr">
         <is>
@@ -2195,17 +2195,17 @@
         <v>1</v>
       </c>
       <c r="F17" t="n">
-        <v>3881821</v>
+        <v>4026924.996845168</v>
       </c>
       <c r="G17" t="n">
-        <v>144420.9999999995</v>
+        <v>202276.9968451681</v>
       </c>
       <c r="H17" t="n">
-        <v>3.86421041365654</v>
+        <v>5.28877420471552</v>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>2026-03-21T03:45:09</t>
+          <t>2026-03-21T03:46:22</t>
         </is>
       </c>
     </row>
@@ -2217,11 +2217,11 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>DL이앤씨</t>
+          <t>피바디 에너지</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>80</v>
+        <v>65</v>
       </c>
       <c r="D18" t="inlineStr">
         <is>
@@ -2232,17 +2232,17 @@
         <v>1</v>
       </c>
       <c r="F18" t="n">
-        <v>3792400</v>
+        <v>3649438.50225304</v>
       </c>
       <c r="G18" t="n">
-        <v>381400</v>
+        <v>2178666.50225304</v>
       </c>
       <c r="H18" t="n">
-        <v>11.1814717091762</v>
+        <v>148.1308117269733</v>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>2026-03-21T03:45:09</t>
+          <t>2026-03-21T03:46:22</t>
         </is>
       </c>
     </row>
@@ -2254,11 +2254,11 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>피바디 에너지</t>
+          <t>삼성화재</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>65</v>
+        <v>7</v>
       </c>
       <c r="D19" t="inlineStr">
         <is>
@@ -2269,17 +2269,17 @@
         <v>1</v>
       </c>
       <c r="F19" t="n">
-        <v>3427688</v>
+        <v>3321500</v>
       </c>
       <c r="G19" t="n">
-        <v>1956916</v>
+        <v>-309500</v>
       </c>
       <c r="H19" t="n">
-        <v>133.0536616144446</v>
+        <v>-8.523822638391627</v>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>2026-03-21T03:45:09</t>
+          <t>2026-03-21T03:46:22</t>
         </is>
       </c>
     </row>
@@ -2291,11 +2291,11 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>삼성화재</t>
+          <t>더치 브로스</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>7</v>
+        <v>39</v>
       </c>
       <c r="D20" t="inlineStr">
         <is>
@@ -2306,17 +2306,17 @@
         <v>1</v>
       </c>
       <c r="F20" t="n">
-        <v>3335815</v>
+        <v>2934418.414306641</v>
       </c>
       <c r="G20" t="n">
-        <v>-295185</v>
+        <v>-256225.5856933594</v>
       </c>
       <c r="H20" t="n">
-        <v>-8.129578628477004</v>
+        <v>-8.030528811530193</v>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>2026-03-21T03:45:09</t>
+          <t>2026-03-21T03:46:22</t>
         </is>
       </c>
     </row>
@@ -2328,11 +2328,11 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>더치 브로스</t>
+          <t>휴스틸</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>39</v>
+        <v>500</v>
       </c>
       <c r="D21" t="inlineStr">
         <is>
@@ -2343,17 +2343,17 @@
         <v>1</v>
       </c>
       <c r="F21" t="n">
-        <v>2926290</v>
+        <v>2750000</v>
       </c>
       <c r="G21" t="n">
-        <v>-264354</v>
+        <v>471390</v>
       </c>
       <c r="H21" t="n">
-        <v>-8.285286606716387</v>
+        <v>20.68761218462133</v>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>2026-03-21T03:45:09</t>
+          <t>2026-03-21T03:46:22</t>
         </is>
       </c>
     </row>
@@ -2365,11 +2365,11 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>KoAct 코스닥액티브</t>
+          <t>현대제철</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>200</v>
+        <v>70</v>
       </c>
       <c r="D22" t="inlineStr">
         <is>
@@ -2380,17 +2380,17 @@
         <v>1</v>
       </c>
       <c r="F22" t="n">
-        <v>2580000</v>
+        <v>2621500</v>
       </c>
       <c r="G22" t="n">
-        <v>-122000</v>
+        <v>-186000</v>
       </c>
       <c r="H22" t="n">
-        <v>-4.515173945225759</v>
+        <v>-6.625111308993767</v>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>2026-03-21T03:45:09</t>
+          <t>2026-03-21T03:46:22</t>
         </is>
       </c>
     </row>
@@ -2402,11 +2402,11 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>현대제철</t>
+          <t>KoAct 코스닥액티브</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>70</v>
+        <v>200</v>
       </c>
       <c r="D23" t="inlineStr">
         <is>
@@ -2417,17 +2417,17 @@
         <v>1</v>
       </c>
       <c r="F23" t="n">
-        <v>2494002</v>
+        <v>2582000</v>
       </c>
       <c r="G23" t="n">
-        <v>-313498</v>
+        <v>-120000</v>
       </c>
       <c r="H23" t="n">
-        <v>-11.16644701691897</v>
+        <v>-4.441154700222058</v>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>2026-03-21T03:45:09</t>
+          <t>2026-03-21T03:46:22</t>
         </is>
       </c>
     </row>
@@ -2439,11 +2439,11 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>휴스틸</t>
+          <t>넥스틸</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>500</v>
+        <v>200</v>
       </c>
       <c r="D24" t="inlineStr">
         <is>
@@ -2454,17 +2454,17 @@
         <v>1</v>
       </c>
       <c r="F24" t="n">
-        <v>2450090</v>
+        <v>2514000</v>
       </c>
       <c r="G24" t="n">
-        <v>171480</v>
+        <v>503000</v>
       </c>
       <c r="H24" t="n">
-        <v>7.525640631788678</v>
+        <v>25.01243162605669</v>
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>2026-03-21T03:45:09</t>
+          <t>2026-03-21T03:46:22</t>
         </is>
       </c>
     </row>
@@ -2476,11 +2476,11 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>넥스틸</t>
+          <t>대신증권</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>200</v>
+        <v>55</v>
       </c>
       <c r="D25" t="inlineStr">
         <is>
@@ -2491,17 +2491,17 @@
         <v>1</v>
       </c>
       <c r="F25" t="n">
-        <v>2391208</v>
+        <v>2219250</v>
       </c>
       <c r="G25" t="n">
-        <v>380208</v>
+        <v>509749</v>
       </c>
       <c r="H25" t="n">
-        <v>18.90641471904525</v>
+        <v>29.81858448752005</v>
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>2026-03-21T03:45:09</t>
+          <t>2026-03-21T03:46:22</t>
         </is>
       </c>
     </row>
@@ -2513,11 +2513,11 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>대신증권</t>
+          <t>발레로 에너지</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>55</v>
+        <v>6</v>
       </c>
       <c r="D26" t="inlineStr">
         <is>
@@ -2528,17 +2528,17 @@
         <v>1</v>
       </c>
       <c r="F26" t="n">
-        <v>2190111</v>
+        <v>2165691.085066516</v>
       </c>
       <c r="G26" t="n">
-        <v>480610</v>
+        <v>101701.085066516</v>
       </c>
       <c r="H26" t="n">
-        <v>28.11405199528985</v>
+        <v>4.927402025519307</v>
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>2026-03-21T03:45:09</t>
+          <t>2026-03-21T03:46:22</t>
         </is>
       </c>
     </row>
@@ -2550,11 +2550,11 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>발레로 에너지</t>
+          <t>미창석유</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>6</v>
+        <v>18</v>
       </c>
       <c r="D27" t="inlineStr">
         <is>
@@ -2565,17 +2565,17 @@
         <v>1</v>
       </c>
       <c r="F27" t="n">
-        <v>2096946</v>
+        <v>2097000</v>
       </c>
       <c r="G27" t="n">
-        <v>32956</v>
+        <v>-295200</v>
       </c>
       <c r="H27" t="n">
-        <v>1.596713162369973</v>
+        <v>-12.34010534236268</v>
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>2026-03-21T03:45:09</t>
+          <t>2026-03-21T03:46:22</t>
         </is>
       </c>
     </row>
@@ -2587,11 +2587,11 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>미창석유</t>
+          <t>대창단조</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>18</v>
+        <v>300</v>
       </c>
       <c r="D28" t="inlineStr">
         <is>
@@ -2602,17 +2602,17 @@
         <v>1</v>
       </c>
       <c r="F28" t="n">
-        <v>2049693</v>
+        <v>2004000</v>
       </c>
       <c r="G28" t="n">
-        <v>-342507</v>
+        <v>-54000</v>
       </c>
       <c r="H28" t="n">
-        <v>-14.31765738650614</v>
+        <v>-2.623906705539359</v>
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>2026-03-21T03:45:09</t>
+          <t>2026-03-21T03:46:22</t>
         </is>
       </c>
     </row>
@@ -2624,11 +2624,11 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>대창단조</t>
+          <t>동방</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>300</v>
+        <v>681</v>
       </c>
       <c r="D29" t="inlineStr">
         <is>
@@ -2639,17 +2639,17 @@
         <v>1</v>
       </c>
       <c r="F29" t="n">
-        <v>1901190</v>
+        <v>1995330</v>
       </c>
       <c r="G29" t="n">
-        <v>-156810</v>
+        <v>23829</v>
       </c>
       <c r="H29" t="n">
-        <v>-7.619533527696793</v>
+        <v>1.208672985709873</v>
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>2026-03-21T03:45:09</t>
+          <t>2026-03-21T03:46:22</t>
         </is>
       </c>
     </row>
@@ -2661,11 +2661,11 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>동방</t>
+          <t>스타 벌크 캐리어스</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>681</v>
+        <v>50</v>
       </c>
       <c r="D30" t="inlineStr">
         <is>
@@ -2676,17 +2676,17 @@
         <v>1</v>
       </c>
       <c r="F30" t="n">
-        <v>1841600</v>
+        <v>1680142.640194588</v>
       </c>
       <c r="G30" t="n">
-        <v>-129901</v>
+        <v>365789.6401945879</v>
       </c>
       <c r="H30" t="n">
-        <v>-6.588939087527726</v>
+        <v>27.83039565433242</v>
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>2026-03-21T03:45:09</t>
+          <t>2026-03-21T03:46:22</t>
         </is>
       </c>
     </row>
@@ -2698,11 +2698,11 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>유나이티드헬스 그룹</t>
+          <t>케이씨</t>
         </is>
       </c>
       <c r="C31" t="n">
-        <v>4</v>
+        <v>50</v>
       </c>
       <c r="D31" t="inlineStr">
         <is>
@@ -2713,17 +2713,17 @@
         <v>1</v>
       </c>
       <c r="F31" t="n">
-        <v>1710490</v>
+        <v>1670000</v>
       </c>
       <c r="G31" t="n">
-        <v>16034</v>
+        <v>20500</v>
       </c>
       <c r="H31" t="n">
-        <v>0.9462623992597033</v>
+        <v>1.242800848742043</v>
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>2026-03-21T03:45:09</t>
+          <t>2026-03-21T03:46:22</t>
         </is>
       </c>
     </row>
@@ -2735,11 +2735,11 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>스타 벌크 캐리어스</t>
+          <t>유나이티드헬스 그룹</t>
         </is>
       </c>
       <c r="C32" t="n">
-        <v>50</v>
+        <v>4</v>
       </c>
       <c r="D32" t="inlineStr">
         <is>
@@ -2750,17 +2750,17 @@
         <v>1</v>
       </c>
       <c r="F32" t="n">
-        <v>1661361</v>
+        <v>1658864.328313038</v>
       </c>
       <c r="G32" t="n">
-        <v>347008</v>
+        <v>-35591.67168696225</v>
       </c>
       <c r="H32" t="n">
-        <v>26.40143097021881</v>
+        <v>-2.100477774988684</v>
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>2026-03-21T03:45:09</t>
+          <t>2026-03-21T03:46:22</t>
         </is>
       </c>
     </row>
@@ -2772,11 +2772,11 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>케이씨</t>
+          <t>하나금융지주</t>
         </is>
       </c>
       <c r="C33" t="n">
-        <v>50</v>
+        <v>10</v>
       </c>
       <c r="D33" t="inlineStr">
         <is>
@@ -2787,17 +2787,17 @@
         <v>1</v>
       </c>
       <c r="F33" t="n">
-        <v>1576840</v>
+        <v>1132000</v>
       </c>
       <c r="G33" t="n">
-        <v>-72660</v>
+        <v>23000</v>
       </c>
       <c r="H33" t="n">
-        <v>-4.404971203394968</v>
+        <v>2.073940486925157</v>
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>2026-03-21T03:45:09</t>
+          <t>2026-03-21T03:46:22</t>
         </is>
       </c>
     </row>
@@ -2809,11 +2809,11 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>하나금융지주</t>
+          <t>삼성생명</t>
         </is>
       </c>
       <c r="C34" t="n">
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="D34" t="inlineStr">
         <is>
@@ -2824,17 +2824,17 @@
         <v>1</v>
       </c>
       <c r="F34" t="n">
-        <v>1107780</v>
+        <v>926000</v>
       </c>
       <c r="G34" t="n">
-        <v>-1220</v>
+        <v>93000</v>
       </c>
       <c r="H34" t="n">
-        <v>-0.1100090171325518</v>
+        <v>11.16446578631453</v>
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>2026-03-21T03:45:09</t>
+          <t>2026-03-21T03:46:22</t>
         </is>
       </c>
     </row>
@@ -2846,11 +2846,11 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>클리블랜드 클리프스</t>
+          <t>비에이치아이</t>
         </is>
       </c>
       <c r="C35" t="n">
-        <v>70</v>
+        <v>8</v>
       </c>
       <c r="D35" t="inlineStr">
         <is>
@@ -2861,17 +2861,17 @@
         <v>1</v>
       </c>
       <c r="F35" t="n">
-        <v>908091</v>
+        <v>876000</v>
       </c>
       <c r="G35" t="n">
-        <v>-107964</v>
+        <v>210885</v>
       </c>
       <c r="H35" t="n">
-        <v>-10.62580273705656</v>
+        <v>31.70654698811484</v>
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>2026-03-21T03:45:09</t>
+          <t>2026-03-21T03:46:22</t>
         </is>
       </c>
     </row>
@@ -2883,11 +2883,11 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>삼성생명</t>
+          <t>클리블랜드 클리프스</t>
         </is>
       </c>
       <c r="C36" t="n">
-        <v>4</v>
+        <v>70</v>
       </c>
       <c r="D36" t="inlineStr">
         <is>
@@ -2898,17 +2898,17 @@
         <v>1</v>
       </c>
       <c r="F36" t="n">
-        <v>872252</v>
+        <v>823743.9360268187</v>
       </c>
       <c r="G36" t="n">
-        <v>39252</v>
+        <v>-192311.0639731813</v>
       </c>
       <c r="H36" t="n">
-        <v>4.712124849939976</v>
+        <v>-18.92722972409774</v>
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>2026-03-21T03:45:09</t>
+          <t>2026-03-21T03:46:22</t>
         </is>
       </c>
     </row>
@@ -2920,11 +2920,11 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>비에이치아이</t>
+          <t>하프니아</t>
         </is>
       </c>
       <c r="C37" t="n">
-        <v>8</v>
+        <v>80</v>
       </c>
       <c r="D37" t="inlineStr">
         <is>
@@ -2935,17 +2935,17 @@
         <v>1</v>
       </c>
       <c r="F37" t="n">
-        <v>850296</v>
+        <v>798051</v>
       </c>
       <c r="G37" t="n">
-        <v>185181</v>
+        <v>172320</v>
       </c>
       <c r="H37" t="n">
-        <v>27.84195214361426</v>
+        <v>27.53899039683186</v>
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>2026-03-21T03:45:09</t>
+          <t>2026-03-21T03:46:22</t>
         </is>
       </c>
     </row>
@@ -2957,11 +2957,11 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>하프니아</t>
+          <t>텍사스 퍼시픽 랜드</t>
         </is>
       </c>
       <c r="C38" t="n">
-        <v>80</v>
+        <v>1</v>
       </c>
       <c r="D38" t="inlineStr">
         <is>
@@ -2972,17 +2972,17 @@
         <v>1</v>
       </c>
       <c r="F38" t="n">
-        <v>798051</v>
+        <v>781623.6870614514</v>
       </c>
       <c r="G38" t="n">
-        <v>172320</v>
+        <v>3032.687061451375</v>
       </c>
       <c r="H38" t="n">
-        <v>27.53899039683186</v>
+        <v>0.3895096477420591</v>
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>2026-03-21T03:45:09</t>
+          <t>2026-03-21T03:46:22</t>
         </is>
       </c>
     </row>
@@ -2994,11 +2994,11 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>텍사스 퍼시픽 랜드</t>
+          <t>노블</t>
         </is>
       </c>
       <c r="C39" t="n">
-        <v>1</v>
+        <v>99</v>
       </c>
       <c r="D39" t="inlineStr">
         <is>
@@ -3009,17 +3009,17 @@
         <v>1</v>
       </c>
       <c r="F39" t="n">
-        <v>786665</v>
+        <v>40689</v>
       </c>
       <c r="G39" t="n">
-        <v>8074</v>
+        <v>-3866519</v>
       </c>
       <c r="H39" t="n">
-        <v>1.037001455192778</v>
+        <v>-98.95861699709869</v>
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>2026-03-21T03:45:09</t>
+          <t>2026-03-21T03:46:22</t>
         </is>
       </c>
     </row>
@@ -3083,7 +3083,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>2026-03-21T03:45:29</t>
+          <t>2026-03-21T03:46:22</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: portfolio snapshot 2026-03-21 (2026-03-21T04:48:19)
</commit_message>
<xml_diff>
--- a/portfolio_auto.xlsx
+++ b/portfolio_auto.xlsx
@@ -543,10 +543,10 @@
         <v>2934418.414306641</v>
       </c>
       <c r="F4" t="n">
-        <v>-256225.5856933594</v>
+        <v>-256225.5856933598</v>
       </c>
       <c r="G4" t="n">
-        <v>-8.030528811530193</v>
+        <v>-8.030528811530205</v>
       </c>
     </row>
     <row r="5">
@@ -624,10 +624,10 @@
         <v>1680142.640194588</v>
       </c>
       <c r="F7" t="n">
-        <v>365789.6401945879</v>
+        <v>365789.6401945876</v>
       </c>
       <c r="G7" t="n">
-        <v>27.83039565433242</v>
+        <v>27.8303956543324</v>
       </c>
     </row>
     <row r="8">
@@ -681,7 +681,7 @@
         <v>2254819.137784176</v>
       </c>
       <c r="G9" t="n">
-        <v>99.93171026716374</v>
+        <v>99.93171026716378</v>
       </c>
     </row>
     <row r="10">
@@ -705,10 +705,10 @@
         <v>1658864.328313038</v>
       </c>
       <c r="F10" t="n">
-        <v>-35591.67168696225</v>
+        <v>-35591.67168696248</v>
       </c>
       <c r="G10" t="n">
-        <v>-2.100477774988684</v>
+        <v>-2.100477774988697</v>
       </c>
     </row>
     <row r="11">
@@ -867,10 +867,10 @@
         <v>13579584.97235231</v>
       </c>
       <c r="F16" t="n">
-        <v>1473035.972352311</v>
+        <v>1473035.972352313</v>
       </c>
       <c r="G16" t="n">
-        <v>12.16726560436265</v>
+        <v>12.16726560436267</v>
       </c>
     </row>
     <row r="17">
@@ -945,13 +945,13 @@
         <v>1</v>
       </c>
       <c r="E19" t="n">
-        <v>798051</v>
+        <v>842704.775390625</v>
       </c>
       <c r="F19" t="n">
-        <v>172320</v>
+        <v>216973.775390625</v>
       </c>
       <c r="G19" t="n">
-        <v>27.53899039683186</v>
+        <v>34.67524789256486</v>
       </c>
     </row>
     <row r="20">
@@ -975,10 +975,10 @@
         <v>10270464.45007324</v>
       </c>
       <c r="F20" t="n">
-        <v>-561550.5499267578</v>
+        <v>-561550.5499267559</v>
       </c>
       <c r="G20" t="n">
-        <v>-5.184174411933125</v>
+        <v>-5.184174411933109</v>
       </c>
     </row>
     <row r="21">
@@ -1538,22 +1538,22 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-03-17</t>
+          <t>2026-03-21</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>33078556</v>
+        <v>31036676</v>
       </c>
       <c r="C2" t="n">
-        <v>6010.99</v>
+        <v>6052.96</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2026-03-21T03:46:22</t>
+          <t>2026-03-21T04:48:19</t>
         </is>
       </c>
       <c r="E2" t="n">
-        <v>1488.910034179688</v>
+        <v>1504.829956054688</v>
       </c>
     </row>
   </sheetData>
@@ -1567,7 +1567,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I39"/>
+  <dimension ref="A1:I77"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3020,6 +3020,1412 @@
       <c r="I39" t="inlineStr">
         <is>
           <t>2026-03-21T03:46:22</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>2026-03-21</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>페트로브라스 (ADR)</t>
+        </is>
+      </c>
+      <c r="C40" t="n">
+        <v>480</v>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E40" t="n">
+        <v>1</v>
+      </c>
+      <c r="F40" t="n">
+        <v>13579584.97235231</v>
+      </c>
+      <c r="G40" t="n">
+        <v>1473035.972352313</v>
+      </c>
+      <c r="H40" t="n">
+        <v>12.16726560436267</v>
+      </c>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>2026-03-21T04:48:19</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>2026-03-21</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>AGNC 인베스트먼트</t>
+        </is>
+      </c>
+      <c r="C41" t="n">
+        <v>700</v>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E41" t="n">
+        <v>1</v>
+      </c>
+      <c r="F41" t="n">
+        <v>10270464.45007324</v>
+      </c>
+      <c r="G41" t="n">
+        <v>-561550.5499267559</v>
+      </c>
+      <c r="H41" t="n">
+        <v>-5.184174411933109</v>
+      </c>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>2026-03-21T04:48:19</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>2026-03-21</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>대한조선</t>
+        </is>
+      </c>
+      <c r="C42" t="n">
+        <v>100</v>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E42" t="n">
+        <v>1</v>
+      </c>
+      <c r="F42" t="n">
+        <v>9120000</v>
+      </c>
+      <c r="G42" t="n">
+        <v>1907000</v>
+      </c>
+      <c r="H42" t="n">
+        <v>26.43837515596839</v>
+      </c>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>2026-03-21T04:48:19</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>2026-03-21</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>프론트라인</t>
+        </is>
+      </c>
+      <c r="C43" t="n">
+        <v>175</v>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E43" t="n">
+        <v>1</v>
+      </c>
+      <c r="F43" t="n">
+        <v>8471815.962899337</v>
+      </c>
+      <c r="G43" t="n">
+        <v>4041951.962899337</v>
+      </c>
+      <c r="H43" t="n">
+        <v>91.24325177701475</v>
+      </c>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>2026-03-21T04:48:19</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>2026-03-21</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>시드릴</t>
+        </is>
+      </c>
+      <c r="C44" t="n">
+        <v>123</v>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E44" t="n">
+        <v>1</v>
+      </c>
+      <c r="F44" t="n">
+        <v>8070101.805898919</v>
+      </c>
+      <c r="G44" t="n">
+        <v>1619750.805898919</v>
+      </c>
+      <c r="H44" t="n">
+        <v>25.11104908707943</v>
+      </c>
+      <c r="I44" t="inlineStr">
+        <is>
+          <t>2026-03-21T04:48:19</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>2026-03-21</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>세아제강</t>
+        </is>
+      </c>
+      <c r="C45" t="n">
+        <v>50</v>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E45" t="n">
+        <v>1</v>
+      </c>
+      <c r="F45" t="n">
+        <v>7395000</v>
+      </c>
+      <c r="G45" t="n">
+        <v>1085000</v>
+      </c>
+      <c r="H45" t="n">
+        <v>17.19492868462758</v>
+      </c>
+      <c r="I45" t="inlineStr">
+        <is>
+          <t>2026-03-21T04:48:19</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>2026-03-21</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>트랜스오션</t>
+        </is>
+      </c>
+      <c r="C46" t="n">
+        <v>750</v>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E46" t="n">
+        <v>1</v>
+      </c>
+      <c r="F46" t="n">
+        <v>7020031.5082007</v>
+      </c>
+      <c r="G46" t="n">
+        <v>2892797.5082007</v>
+      </c>
+      <c r="H46" t="n">
+        <v>70.09046514446965</v>
+      </c>
+      <c r="I46" t="inlineStr">
+        <is>
+          <t>2026-03-21T04:48:19</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>2026-03-21</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>센트러스 에너지</t>
+        </is>
+      </c>
+      <c r="C47" t="n">
+        <v>21</v>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E47" t="n">
+        <v>1</v>
+      </c>
+      <c r="F47" t="n">
+        <v>5901882.720856408</v>
+      </c>
+      <c r="G47" t="n">
+        <v>-329336.2791435914</v>
+      </c>
+      <c r="H47" t="n">
+        <v>-5.285262468605123</v>
+      </c>
+      <c r="I47" t="inlineStr">
+        <is>
+          <t>2026-03-21T04:48:19</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>2026-03-21</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>DL이앤씨</t>
+        </is>
+      </c>
+      <c r="C48" t="n">
+        <v>80</v>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E48" t="n">
+        <v>1</v>
+      </c>
+      <c r="F48" t="n">
+        <v>5392000</v>
+      </c>
+      <c r="G48" t="n">
+        <v>1981000</v>
+      </c>
+      <c r="H48" t="n">
+        <v>58.07681031955438</v>
+      </c>
+      <c r="I48" t="inlineStr">
+        <is>
+          <t>2026-03-21T04:48:19</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>2026-03-21</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>타이드워터</t>
+        </is>
+      </c>
+      <c r="C49" t="n">
+        <v>48</v>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E49" t="n">
+        <v>1</v>
+      </c>
+      <c r="F49" t="n">
+        <v>5235363.852789983</v>
+      </c>
+      <c r="G49" t="n">
+        <v>1510818.852789983</v>
+      </c>
+      <c r="H49" t="n">
+        <v>40.56385015592463</v>
+      </c>
+      <c r="I49" t="inlineStr">
+        <is>
+          <t>2026-03-21T04:48:19</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>2026-03-21</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>노브</t>
+        </is>
+      </c>
+      <c r="C50" t="n">
+        <v>185</v>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E50" t="n">
+        <v>1</v>
+      </c>
+      <c r="F50" t="n">
+        <v>5200391.447092756</v>
+      </c>
+      <c r="G50" t="n">
+        <v>1890383.447092756</v>
+      </c>
+      <c r="H50" t="n">
+        <v>57.11114435653194</v>
+      </c>
+      <c r="I50" t="inlineStr">
+        <is>
+          <t>2026-03-21T04:48:19</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>2026-03-21</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>TIME 코리아밸류업액티브</t>
+        </is>
+      </c>
+      <c r="C51" t="n">
+        <v>201</v>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E51" t="n">
+        <v>1</v>
+      </c>
+      <c r="F51" t="n">
+        <v>4797870</v>
+      </c>
+      <c r="G51" t="n">
+        <v>74073</v>
+      </c>
+      <c r="H51" t="n">
+        <v>1.568081778281328</v>
+      </c>
+      <c r="I51" t="inlineStr">
+        <is>
+          <t>2026-03-21T04:48:19</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>2026-03-21</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>오케아니스 에코 탱커스</t>
+        </is>
+      </c>
+      <c r="C52" t="n">
+        <v>65</v>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E52" t="n">
+        <v>1</v>
+      </c>
+      <c r="F52" t="n">
+        <v>4511179.137784176</v>
+      </c>
+      <c r="G52" t="n">
+        <v>2254819.137784176</v>
+      </c>
+      <c r="H52" t="n">
+        <v>99.93171026716378</v>
+      </c>
+      <c r="I52" t="inlineStr">
+        <is>
+          <t>2026-03-21T04:48:19</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>2026-03-21</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>동원개발</t>
+        </is>
+      </c>
+      <c r="C53" t="n">
+        <v>1360</v>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E53" t="n">
+        <v>1</v>
+      </c>
+      <c r="F53" t="n">
+        <v>4202400</v>
+      </c>
+      <c r="G53" t="n">
+        <v>465000</v>
+      </c>
+      <c r="H53" t="n">
+        <v>12.44180446299566</v>
+      </c>
+      <c r="I53" t="inlineStr">
+        <is>
+          <t>2026-03-21T04:48:19</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>2026-03-21</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>HD건설기계</t>
+        </is>
+      </c>
+      <c r="C54" t="n">
+        <v>31</v>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E54" t="n">
+        <v>1</v>
+      </c>
+      <c r="F54" t="n">
+        <v>4123000</v>
+      </c>
+      <c r="G54" t="n">
+        <v>87904</v>
+      </c>
+      <c r="H54" t="n">
+        <v>2.178485964150543</v>
+      </c>
+      <c r="I54" t="inlineStr">
+        <is>
+          <t>2026-03-21T04:48:19</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>2026-03-21</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>차코스 에너지 내비게이션</t>
+        </is>
+      </c>
+      <c r="C55" t="n">
+        <v>75</v>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E55" t="n">
+        <v>1</v>
+      </c>
+      <c r="F55" t="n">
+        <v>4026924.996845168</v>
+      </c>
+      <c r="G55" t="n">
+        <v>202276.9968451681</v>
+      </c>
+      <c r="H55" t="n">
+        <v>5.28877420471552</v>
+      </c>
+      <c r="I55" t="inlineStr">
+        <is>
+          <t>2026-03-21T04:48:19</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>2026-03-21</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>피바디 에너지</t>
+        </is>
+      </c>
+      <c r="C56" t="n">
+        <v>65</v>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E56" t="n">
+        <v>1</v>
+      </c>
+      <c r="F56" t="n">
+        <v>3649438.50225304</v>
+      </c>
+      <c r="G56" t="n">
+        <v>2178666.50225304</v>
+      </c>
+      <c r="H56" t="n">
+        <v>148.1308117269733</v>
+      </c>
+      <c r="I56" t="inlineStr">
+        <is>
+          <t>2026-03-21T04:48:19</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>2026-03-21</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>삼성화재</t>
+        </is>
+      </c>
+      <c r="C57" t="n">
+        <v>7</v>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E57" t="n">
+        <v>1</v>
+      </c>
+      <c r="F57" t="n">
+        <v>3321500</v>
+      </c>
+      <c r="G57" t="n">
+        <v>-309500</v>
+      </c>
+      <c r="H57" t="n">
+        <v>-8.523822638391627</v>
+      </c>
+      <c r="I57" t="inlineStr">
+        <is>
+          <t>2026-03-21T04:48:19</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>2026-03-21</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>더치 브로스</t>
+        </is>
+      </c>
+      <c r="C58" t="n">
+        <v>39</v>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E58" t="n">
+        <v>1</v>
+      </c>
+      <c r="F58" t="n">
+        <v>2934418.414306641</v>
+      </c>
+      <c r="G58" t="n">
+        <v>-256225.5856933598</v>
+      </c>
+      <c r="H58" t="n">
+        <v>-8.030528811530205</v>
+      </c>
+      <c r="I58" t="inlineStr">
+        <is>
+          <t>2026-03-21T04:48:19</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>2026-03-21</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>휴스틸</t>
+        </is>
+      </c>
+      <c r="C59" t="n">
+        <v>500</v>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E59" t="n">
+        <v>1</v>
+      </c>
+      <c r="F59" t="n">
+        <v>2750000</v>
+      </c>
+      <c r="G59" t="n">
+        <v>471390</v>
+      </c>
+      <c r="H59" t="n">
+        <v>20.68761218462133</v>
+      </c>
+      <c r="I59" t="inlineStr">
+        <is>
+          <t>2026-03-21T04:48:19</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>2026-03-21</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>현대제철</t>
+        </is>
+      </c>
+      <c r="C60" t="n">
+        <v>70</v>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E60" t="n">
+        <v>1</v>
+      </c>
+      <c r="F60" t="n">
+        <v>2621500</v>
+      </c>
+      <c r="G60" t="n">
+        <v>-186000</v>
+      </c>
+      <c r="H60" t="n">
+        <v>-6.625111308993767</v>
+      </c>
+      <c r="I60" t="inlineStr">
+        <is>
+          <t>2026-03-21T04:48:19</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>2026-03-21</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>KoAct 코스닥액티브</t>
+        </is>
+      </c>
+      <c r="C61" t="n">
+        <v>200</v>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E61" t="n">
+        <v>1</v>
+      </c>
+      <c r="F61" t="n">
+        <v>2582000</v>
+      </c>
+      <c r="G61" t="n">
+        <v>-120000</v>
+      </c>
+      <c r="H61" t="n">
+        <v>-4.441154700222058</v>
+      </c>
+      <c r="I61" t="inlineStr">
+        <is>
+          <t>2026-03-21T04:48:19</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>2026-03-21</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>넥스틸</t>
+        </is>
+      </c>
+      <c r="C62" t="n">
+        <v>200</v>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E62" t="n">
+        <v>1</v>
+      </c>
+      <c r="F62" t="n">
+        <v>2514000</v>
+      </c>
+      <c r="G62" t="n">
+        <v>503000</v>
+      </c>
+      <c r="H62" t="n">
+        <v>25.01243162605669</v>
+      </c>
+      <c r="I62" t="inlineStr">
+        <is>
+          <t>2026-03-21T04:48:19</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>2026-03-21</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>대신증권</t>
+        </is>
+      </c>
+      <c r="C63" t="n">
+        <v>55</v>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E63" t="n">
+        <v>1</v>
+      </c>
+      <c r="F63" t="n">
+        <v>2219250</v>
+      </c>
+      <c r="G63" t="n">
+        <v>509749</v>
+      </c>
+      <c r="H63" t="n">
+        <v>29.81858448752005</v>
+      </c>
+      <c r="I63" t="inlineStr">
+        <is>
+          <t>2026-03-21T04:48:19</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>2026-03-21</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>발레로 에너지</t>
+        </is>
+      </c>
+      <c r="C64" t="n">
+        <v>6</v>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E64" t="n">
+        <v>1</v>
+      </c>
+      <c r="F64" t="n">
+        <v>2165691.085066516</v>
+      </c>
+      <c r="G64" t="n">
+        <v>101701.085066516</v>
+      </c>
+      <c r="H64" t="n">
+        <v>4.927402025519307</v>
+      </c>
+      <c r="I64" t="inlineStr">
+        <is>
+          <t>2026-03-21T04:48:19</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>2026-03-21</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>미창석유</t>
+        </is>
+      </c>
+      <c r="C65" t="n">
+        <v>18</v>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E65" t="n">
+        <v>1</v>
+      </c>
+      <c r="F65" t="n">
+        <v>2097000</v>
+      </c>
+      <c r="G65" t="n">
+        <v>-295200</v>
+      </c>
+      <c r="H65" t="n">
+        <v>-12.34010534236268</v>
+      </c>
+      <c r="I65" t="inlineStr">
+        <is>
+          <t>2026-03-21T04:48:19</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>2026-03-21</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>대창단조</t>
+        </is>
+      </c>
+      <c r="C66" t="n">
+        <v>300</v>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E66" t="n">
+        <v>1</v>
+      </c>
+      <c r="F66" t="n">
+        <v>2004000</v>
+      </c>
+      <c r="G66" t="n">
+        <v>-54000</v>
+      </c>
+      <c r="H66" t="n">
+        <v>-2.623906705539359</v>
+      </c>
+      <c r="I66" t="inlineStr">
+        <is>
+          <t>2026-03-21T04:48:19</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>2026-03-21</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>동방</t>
+        </is>
+      </c>
+      <c r="C67" t="n">
+        <v>681</v>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E67" t="n">
+        <v>1</v>
+      </c>
+      <c r="F67" t="n">
+        <v>1995330</v>
+      </c>
+      <c r="G67" t="n">
+        <v>23829</v>
+      </c>
+      <c r="H67" t="n">
+        <v>1.208672985709873</v>
+      </c>
+      <c r="I67" t="inlineStr">
+        <is>
+          <t>2026-03-21T04:48:19</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>2026-03-21</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>스타 벌크 캐리어스</t>
+        </is>
+      </c>
+      <c r="C68" t="n">
+        <v>50</v>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E68" t="n">
+        <v>1</v>
+      </c>
+      <c r="F68" t="n">
+        <v>1680142.640194588</v>
+      </c>
+      <c r="G68" t="n">
+        <v>365789.6401945876</v>
+      </c>
+      <c r="H68" t="n">
+        <v>27.8303956543324</v>
+      </c>
+      <c r="I68" t="inlineStr">
+        <is>
+          <t>2026-03-21T04:48:19</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>2026-03-21</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>케이씨</t>
+        </is>
+      </c>
+      <c r="C69" t="n">
+        <v>50</v>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E69" t="n">
+        <v>1</v>
+      </c>
+      <c r="F69" t="n">
+        <v>1670000</v>
+      </c>
+      <c r="G69" t="n">
+        <v>20500</v>
+      </c>
+      <c r="H69" t="n">
+        <v>1.242800848742043</v>
+      </c>
+      <c r="I69" t="inlineStr">
+        <is>
+          <t>2026-03-21T04:48:19</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>2026-03-21</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>유나이티드헬스 그룹</t>
+        </is>
+      </c>
+      <c r="C70" t="n">
+        <v>4</v>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E70" t="n">
+        <v>1</v>
+      </c>
+      <c r="F70" t="n">
+        <v>1658864.328313038</v>
+      </c>
+      <c r="G70" t="n">
+        <v>-35591.67168696248</v>
+      </c>
+      <c r="H70" t="n">
+        <v>-2.100477774988697</v>
+      </c>
+      <c r="I70" t="inlineStr">
+        <is>
+          <t>2026-03-21T04:48:19</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>2026-03-21</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>하나금융지주</t>
+        </is>
+      </c>
+      <c r="C71" t="n">
+        <v>10</v>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E71" t="n">
+        <v>1</v>
+      </c>
+      <c r="F71" t="n">
+        <v>1132000</v>
+      </c>
+      <c r="G71" t="n">
+        <v>23000</v>
+      </c>
+      <c r="H71" t="n">
+        <v>2.073940486925157</v>
+      </c>
+      <c r="I71" t="inlineStr">
+        <is>
+          <t>2026-03-21T04:48:19</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>2026-03-21</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>삼성생명</t>
+        </is>
+      </c>
+      <c r="C72" t="n">
+        <v>4</v>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E72" t="n">
+        <v>1</v>
+      </c>
+      <c r="F72" t="n">
+        <v>926000</v>
+      </c>
+      <c r="G72" t="n">
+        <v>93000</v>
+      </c>
+      <c r="H72" t="n">
+        <v>11.16446578631453</v>
+      </c>
+      <c r="I72" t="inlineStr">
+        <is>
+          <t>2026-03-21T04:48:19</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>2026-03-21</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>비에이치아이</t>
+        </is>
+      </c>
+      <c r="C73" t="n">
+        <v>8</v>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E73" t="n">
+        <v>1</v>
+      </c>
+      <c r="F73" t="n">
+        <v>876000</v>
+      </c>
+      <c r="G73" t="n">
+        <v>210885</v>
+      </c>
+      <c r="H73" t="n">
+        <v>31.70654698811484</v>
+      </c>
+      <c r="I73" t="inlineStr">
+        <is>
+          <t>2026-03-21T04:48:19</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>2026-03-21</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>하프니아</t>
+        </is>
+      </c>
+      <c r="C74" t="n">
+        <v>80</v>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E74" t="n">
+        <v>1</v>
+      </c>
+      <c r="F74" t="n">
+        <v>842704.775390625</v>
+      </c>
+      <c r="G74" t="n">
+        <v>216973.775390625</v>
+      </c>
+      <c r="H74" t="n">
+        <v>34.67524789256486</v>
+      </c>
+      <c r="I74" t="inlineStr">
+        <is>
+          <t>2026-03-21T04:48:19</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>2026-03-21</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>클리블랜드 클리프스</t>
+        </is>
+      </c>
+      <c r="C75" t="n">
+        <v>70</v>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E75" t="n">
+        <v>1</v>
+      </c>
+      <c r="F75" t="n">
+        <v>823743.9360268187</v>
+      </c>
+      <c r="G75" t="n">
+        <v>-192311.0639731813</v>
+      </c>
+      <c r="H75" t="n">
+        <v>-18.92722972409774</v>
+      </c>
+      <c r="I75" t="inlineStr">
+        <is>
+          <t>2026-03-21T04:48:19</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>2026-03-21</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>텍사스 퍼시픽 랜드</t>
+        </is>
+      </c>
+      <c r="C76" t="n">
+        <v>1</v>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E76" t="n">
+        <v>1</v>
+      </c>
+      <c r="F76" t="n">
+        <v>781623.6870614514</v>
+      </c>
+      <c r="G76" t="n">
+        <v>3032.687061451375</v>
+      </c>
+      <c r="H76" t="n">
+        <v>0.3895096477420591</v>
+      </c>
+      <c r="I76" t="inlineStr">
+        <is>
+          <t>2026-03-21T04:48:19</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>2026-03-21</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>노블</t>
+        </is>
+      </c>
+      <c r="C77" t="n">
+        <v>99</v>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E77" t="n">
+        <v>1</v>
+      </c>
+      <c r="F77" t="n">
+        <v>40689</v>
+      </c>
+      <c r="G77" t="n">
+        <v>-3866519</v>
+      </c>
+      <c r="H77" t="n">
+        <v>-98.95861699709869</v>
+      </c>
+      <c r="I77" t="inlineStr">
+        <is>
+          <t>2026-03-21T04:48:19</t>
         </is>
       </c>
     </row>
@@ -3106,7 +4512,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>2026-03-21T03:07:34</t>
+          <t>2026-03-21T04:48:19</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: portfolio snapshot 2026-03-21 (2026-03-21T04:48:29)
</commit_message>
<xml_diff>
--- a/portfolio_auto.xlsx
+++ b/portfolio_auto.xlsx
@@ -1549,7 +1549,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2026-03-21T04:48:19</t>
+          <t>2026-03-21T04:48:29</t>
         </is>
       </c>
       <c r="E2" t="n">
@@ -3056,7 +3056,7 @@
       </c>
       <c r="I40" t="inlineStr">
         <is>
-          <t>2026-03-21T04:48:19</t>
+          <t>2026-03-21T04:48:28</t>
         </is>
       </c>
     </row>
@@ -3093,7 +3093,7 @@
       </c>
       <c r="I41" t="inlineStr">
         <is>
-          <t>2026-03-21T04:48:19</t>
+          <t>2026-03-21T04:48:28</t>
         </is>
       </c>
     </row>
@@ -3130,7 +3130,7 @@
       </c>
       <c r="I42" t="inlineStr">
         <is>
-          <t>2026-03-21T04:48:19</t>
+          <t>2026-03-21T04:48:28</t>
         </is>
       </c>
     </row>
@@ -3167,7 +3167,7 @@
       </c>
       <c r="I43" t="inlineStr">
         <is>
-          <t>2026-03-21T04:48:19</t>
+          <t>2026-03-21T04:48:28</t>
         </is>
       </c>
     </row>
@@ -3204,7 +3204,7 @@
       </c>
       <c r="I44" t="inlineStr">
         <is>
-          <t>2026-03-21T04:48:19</t>
+          <t>2026-03-21T04:48:28</t>
         </is>
       </c>
     </row>
@@ -3241,7 +3241,7 @@
       </c>
       <c r="I45" t="inlineStr">
         <is>
-          <t>2026-03-21T04:48:19</t>
+          <t>2026-03-21T04:48:28</t>
         </is>
       </c>
     </row>
@@ -3278,7 +3278,7 @@
       </c>
       <c r="I46" t="inlineStr">
         <is>
-          <t>2026-03-21T04:48:19</t>
+          <t>2026-03-21T04:48:28</t>
         </is>
       </c>
     </row>
@@ -3315,7 +3315,7 @@
       </c>
       <c r="I47" t="inlineStr">
         <is>
-          <t>2026-03-21T04:48:19</t>
+          <t>2026-03-21T04:48:28</t>
         </is>
       </c>
     </row>
@@ -3352,7 +3352,7 @@
       </c>
       <c r="I48" t="inlineStr">
         <is>
-          <t>2026-03-21T04:48:19</t>
+          <t>2026-03-21T04:48:28</t>
         </is>
       </c>
     </row>
@@ -3389,7 +3389,7 @@
       </c>
       <c r="I49" t="inlineStr">
         <is>
-          <t>2026-03-21T04:48:19</t>
+          <t>2026-03-21T04:48:28</t>
         </is>
       </c>
     </row>
@@ -3426,7 +3426,7 @@
       </c>
       <c r="I50" t="inlineStr">
         <is>
-          <t>2026-03-21T04:48:19</t>
+          <t>2026-03-21T04:48:28</t>
         </is>
       </c>
     </row>
@@ -3463,7 +3463,7 @@
       </c>
       <c r="I51" t="inlineStr">
         <is>
-          <t>2026-03-21T04:48:19</t>
+          <t>2026-03-21T04:48:28</t>
         </is>
       </c>
     </row>
@@ -3500,7 +3500,7 @@
       </c>
       <c r="I52" t="inlineStr">
         <is>
-          <t>2026-03-21T04:48:19</t>
+          <t>2026-03-21T04:48:28</t>
         </is>
       </c>
     </row>
@@ -3537,7 +3537,7 @@
       </c>
       <c r="I53" t="inlineStr">
         <is>
-          <t>2026-03-21T04:48:19</t>
+          <t>2026-03-21T04:48:28</t>
         </is>
       </c>
     </row>
@@ -3574,7 +3574,7 @@
       </c>
       <c r="I54" t="inlineStr">
         <is>
-          <t>2026-03-21T04:48:19</t>
+          <t>2026-03-21T04:48:28</t>
         </is>
       </c>
     </row>
@@ -3611,7 +3611,7 @@
       </c>
       <c r="I55" t="inlineStr">
         <is>
-          <t>2026-03-21T04:48:19</t>
+          <t>2026-03-21T04:48:28</t>
         </is>
       </c>
     </row>
@@ -3648,7 +3648,7 @@
       </c>
       <c r="I56" t="inlineStr">
         <is>
-          <t>2026-03-21T04:48:19</t>
+          <t>2026-03-21T04:48:28</t>
         </is>
       </c>
     </row>
@@ -3685,7 +3685,7 @@
       </c>
       <c r="I57" t="inlineStr">
         <is>
-          <t>2026-03-21T04:48:19</t>
+          <t>2026-03-21T04:48:28</t>
         </is>
       </c>
     </row>
@@ -3722,7 +3722,7 @@
       </c>
       <c r="I58" t="inlineStr">
         <is>
-          <t>2026-03-21T04:48:19</t>
+          <t>2026-03-21T04:48:28</t>
         </is>
       </c>
     </row>
@@ -3759,7 +3759,7 @@
       </c>
       <c r="I59" t="inlineStr">
         <is>
-          <t>2026-03-21T04:48:19</t>
+          <t>2026-03-21T04:48:28</t>
         </is>
       </c>
     </row>
@@ -3796,7 +3796,7 @@
       </c>
       <c r="I60" t="inlineStr">
         <is>
-          <t>2026-03-21T04:48:19</t>
+          <t>2026-03-21T04:48:28</t>
         </is>
       </c>
     </row>
@@ -3833,7 +3833,7 @@
       </c>
       <c r="I61" t="inlineStr">
         <is>
-          <t>2026-03-21T04:48:19</t>
+          <t>2026-03-21T04:48:28</t>
         </is>
       </c>
     </row>
@@ -3870,7 +3870,7 @@
       </c>
       <c r="I62" t="inlineStr">
         <is>
-          <t>2026-03-21T04:48:19</t>
+          <t>2026-03-21T04:48:28</t>
         </is>
       </c>
     </row>
@@ -3907,7 +3907,7 @@
       </c>
       <c r="I63" t="inlineStr">
         <is>
-          <t>2026-03-21T04:48:19</t>
+          <t>2026-03-21T04:48:28</t>
         </is>
       </c>
     </row>
@@ -3944,7 +3944,7 @@
       </c>
       <c r="I64" t="inlineStr">
         <is>
-          <t>2026-03-21T04:48:19</t>
+          <t>2026-03-21T04:48:28</t>
         </is>
       </c>
     </row>
@@ -3981,7 +3981,7 @@
       </c>
       <c r="I65" t="inlineStr">
         <is>
-          <t>2026-03-21T04:48:19</t>
+          <t>2026-03-21T04:48:28</t>
         </is>
       </c>
     </row>
@@ -4018,7 +4018,7 @@
       </c>
       <c r="I66" t="inlineStr">
         <is>
-          <t>2026-03-21T04:48:19</t>
+          <t>2026-03-21T04:48:28</t>
         </is>
       </c>
     </row>
@@ -4055,7 +4055,7 @@
       </c>
       <c r="I67" t="inlineStr">
         <is>
-          <t>2026-03-21T04:48:19</t>
+          <t>2026-03-21T04:48:28</t>
         </is>
       </c>
     </row>
@@ -4092,7 +4092,7 @@
       </c>
       <c r="I68" t="inlineStr">
         <is>
-          <t>2026-03-21T04:48:19</t>
+          <t>2026-03-21T04:48:28</t>
         </is>
       </c>
     </row>
@@ -4129,7 +4129,7 @@
       </c>
       <c r="I69" t="inlineStr">
         <is>
-          <t>2026-03-21T04:48:19</t>
+          <t>2026-03-21T04:48:28</t>
         </is>
       </c>
     </row>
@@ -4166,7 +4166,7 @@
       </c>
       <c r="I70" t="inlineStr">
         <is>
-          <t>2026-03-21T04:48:19</t>
+          <t>2026-03-21T04:48:28</t>
         </is>
       </c>
     </row>
@@ -4203,7 +4203,7 @@
       </c>
       <c r="I71" t="inlineStr">
         <is>
-          <t>2026-03-21T04:48:19</t>
+          <t>2026-03-21T04:48:28</t>
         </is>
       </c>
     </row>
@@ -4240,7 +4240,7 @@
       </c>
       <c r="I72" t="inlineStr">
         <is>
-          <t>2026-03-21T04:48:19</t>
+          <t>2026-03-21T04:48:28</t>
         </is>
       </c>
     </row>
@@ -4277,7 +4277,7 @@
       </c>
       <c r="I73" t="inlineStr">
         <is>
-          <t>2026-03-21T04:48:19</t>
+          <t>2026-03-21T04:48:28</t>
         </is>
       </c>
     </row>
@@ -4314,7 +4314,7 @@
       </c>
       <c r="I74" t="inlineStr">
         <is>
-          <t>2026-03-21T04:48:19</t>
+          <t>2026-03-21T04:48:28</t>
         </is>
       </c>
     </row>
@@ -4351,7 +4351,7 @@
       </c>
       <c r="I75" t="inlineStr">
         <is>
-          <t>2026-03-21T04:48:19</t>
+          <t>2026-03-21T04:48:28</t>
         </is>
       </c>
     </row>
@@ -4388,7 +4388,7 @@
       </c>
       <c r="I76" t="inlineStr">
         <is>
-          <t>2026-03-21T04:48:19</t>
+          <t>2026-03-21T04:48:28</t>
         </is>
       </c>
     </row>
@@ -4425,7 +4425,7 @@
       </c>
       <c r="I77" t="inlineStr">
         <is>
-          <t>2026-03-21T04:48:19</t>
+          <t>2026-03-21T04:48:28</t>
         </is>
       </c>
     </row>
@@ -4512,7 +4512,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>2026-03-21T04:48:19</t>
+          <t>2026-03-21T04:48:28</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: portfolio snapshot 2026-03-21 (2026-03-21T04:51:19)
</commit_message>
<xml_diff>
--- a/portfolio_auto.xlsx
+++ b/portfolio_auto.xlsx
@@ -579,11 +579,11 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>센트러스 에너지</t>
+          <t>유나이티드헬스 그룹</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>21</v>
+        <v>4</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
@@ -594,23 +594,23 @@
         <v>1</v>
       </c>
       <c r="E6" t="n">
-        <v>5901882.720856408</v>
+        <v>1658864.328313038</v>
       </c>
       <c r="F6" t="n">
-        <v>-329336.2791435914</v>
+        <v>-35591.67168696248</v>
       </c>
       <c r="G6" t="n">
-        <v>-5.285262468605123</v>
+        <v>-2.100477774988697</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>스타 벌크 캐리어스</t>
+          <t>AGNC 인베스트먼트</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>50</v>
+        <v>700</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -621,23 +621,23 @@
         <v>1</v>
       </c>
       <c r="E7" t="n">
-        <v>1680142.640194588</v>
+        <v>10270464.45007324</v>
       </c>
       <c r="F7" t="n">
-        <v>365789.6401945876</v>
+        <v>-561550.5499267559</v>
       </c>
       <c r="G7" t="n">
-        <v>27.8303956543324</v>
+        <v>-5.184174411933109</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>시드릴</t>
+          <t>넥스틸</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>123</v>
+        <v>200</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
@@ -648,23 +648,23 @@
         <v>1</v>
       </c>
       <c r="E8" t="n">
-        <v>8070101.805898919</v>
+        <v>2514000</v>
       </c>
       <c r="F8" t="n">
-        <v>1619750.805898919</v>
+        <v>503000</v>
       </c>
       <c r="G8" t="n">
-        <v>25.11104908707943</v>
+        <v>25.01243162605669</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>오케아니스 에코 탱커스</t>
+          <t>대신증권</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>65</v>
+        <v>55</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
@@ -675,23 +675,23 @@
         <v>1</v>
       </c>
       <c r="E9" t="n">
-        <v>4511179.137784176</v>
+        <v>2219250</v>
       </c>
       <c r="F9" t="n">
-        <v>2254819.137784176</v>
+        <v>509749</v>
       </c>
       <c r="G9" t="n">
-        <v>99.93171026716378</v>
+        <v>29.81858448752005</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>유나이티드헬스 그룹</t>
+          <t>대창단조</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>4</v>
+        <v>300</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
@@ -702,23 +702,23 @@
         <v>1</v>
       </c>
       <c r="E10" t="n">
-        <v>1658864.328313038</v>
+        <v>2004000</v>
       </c>
       <c r="F10" t="n">
-        <v>-35591.67168696248</v>
+        <v>-54000</v>
       </c>
       <c r="G10" t="n">
-        <v>-2.100477774988697</v>
+        <v>-2.623906705539359</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>차코스 에너지 내비게이션</t>
+          <t>대한조선</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>75</v>
+        <v>100</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
@@ -729,23 +729,23 @@
         <v>1</v>
       </c>
       <c r="E11" t="n">
-        <v>4026924.996845168</v>
+        <v>9120000</v>
       </c>
       <c r="F11" t="n">
-        <v>202276.9968451681</v>
+        <v>1907000</v>
       </c>
       <c r="G11" t="n">
-        <v>5.28877420471552</v>
+        <v>26.43837515596839</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>클리블랜드 클리프스</t>
+          <t>동방</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>70</v>
+        <v>681</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
@@ -756,23 +756,23 @@
         <v>1</v>
       </c>
       <c r="E12" t="n">
-        <v>823743.9360268187</v>
+        <v>1995330</v>
       </c>
       <c r="F12" t="n">
-        <v>-192311.0639731813</v>
+        <v>23829</v>
       </c>
       <c r="G12" t="n">
-        <v>-18.92722972409774</v>
+        <v>1.208672985709873</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>타이드워터</t>
+          <t>동원개발</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>48</v>
+        <v>1360</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
@@ -783,23 +783,23 @@
         <v>1</v>
       </c>
       <c r="E13" t="n">
-        <v>5235363.852789983</v>
+        <v>4202400</v>
       </c>
       <c r="F13" t="n">
-        <v>1510818.852789983</v>
+        <v>465000</v>
       </c>
       <c r="G13" t="n">
-        <v>40.56385015592463</v>
+        <v>12.44180446299566</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>텍사스 퍼시픽 랜드</t>
+          <t>미창석유</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>1</v>
+        <v>18</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
@@ -810,23 +810,23 @@
         <v>1</v>
       </c>
       <c r="E14" t="n">
-        <v>781623.6870614514</v>
+        <v>2097000</v>
       </c>
       <c r="F14" t="n">
-        <v>3032.687061451375</v>
+        <v>-295200</v>
       </c>
       <c r="G14" t="n">
-        <v>0.3895096477420591</v>
+        <v>-12.34010534236268</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>트랜스오션</t>
+          <t>비에이치아이</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>750</v>
+        <v>8</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
@@ -837,23 +837,23 @@
         <v>1</v>
       </c>
       <c r="E15" t="n">
-        <v>7020031.5082007</v>
+        <v>876000</v>
       </c>
       <c r="F15" t="n">
-        <v>2892797.5082007</v>
+        <v>210885</v>
       </c>
       <c r="G15" t="n">
-        <v>70.09046514446965</v>
+        <v>31.70654698811484</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>페트로브라스 (ADR)</t>
+          <t>삼성생명</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>480</v>
+        <v>4</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
@@ -864,23 +864,23 @@
         <v>1</v>
       </c>
       <c r="E16" t="n">
-        <v>13579584.97235231</v>
+        <v>926000</v>
       </c>
       <c r="F16" t="n">
-        <v>1473035.972352313</v>
+        <v>93000</v>
       </c>
       <c r="G16" t="n">
-        <v>12.16726560436267</v>
+        <v>11.16446578631453</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>프론트라인</t>
+          <t>삼성화재</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>175</v>
+        <v>7</v>
       </c>
       <c r="C17" t="inlineStr">
         <is>
@@ -891,23 +891,23 @@
         <v>1</v>
       </c>
       <c r="E17" t="n">
-        <v>8471815.962899337</v>
+        <v>3321500</v>
       </c>
       <c r="F17" t="n">
-        <v>4041951.962899337</v>
+        <v>-309500</v>
       </c>
       <c r="G17" t="n">
-        <v>91.24325177701475</v>
+        <v>-8.523822638391627</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>피바디 에너지</t>
+          <t>세아제강</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>65</v>
+        <v>50</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
@@ -918,23 +918,23 @@
         <v>1</v>
       </c>
       <c r="E18" t="n">
-        <v>3649438.50225304</v>
+        <v>7395000</v>
       </c>
       <c r="F18" t="n">
-        <v>2178666.50225304</v>
+        <v>1085000</v>
       </c>
       <c r="G18" t="n">
-        <v>148.1308117269733</v>
+        <v>17.19492868462758</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>하프니아</t>
+          <t>케이씨</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>80</v>
+        <v>50</v>
       </c>
       <c r="C19" t="inlineStr">
         <is>
@@ -945,23 +945,23 @@
         <v>1</v>
       </c>
       <c r="E19" t="n">
-        <v>842704.775390625</v>
+        <v>1670000</v>
       </c>
       <c r="F19" t="n">
-        <v>216973.775390625</v>
+        <v>20500</v>
       </c>
       <c r="G19" t="n">
-        <v>34.67524789256486</v>
+        <v>1.242800848742043</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>AGNC 인베스트먼트</t>
+          <t>하나금융지주</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>700</v>
+        <v>10</v>
       </c>
       <c r="C20" t="inlineStr">
         <is>
@@ -972,23 +972,23 @@
         <v>1</v>
       </c>
       <c r="E20" t="n">
-        <v>10270464.45007324</v>
+        <v>1132000</v>
       </c>
       <c r="F20" t="n">
-        <v>-561550.5499267559</v>
+        <v>23000</v>
       </c>
       <c r="G20" t="n">
-        <v>-5.184174411933109</v>
+        <v>2.073940486925157</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>넥스틸</t>
+          <t>현대제철</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>200</v>
+        <v>70</v>
       </c>
       <c r="C21" t="inlineStr">
         <is>
@@ -999,23 +999,23 @@
         <v>1</v>
       </c>
       <c r="E21" t="n">
-        <v>2514000</v>
+        <v>2621500</v>
       </c>
       <c r="F21" t="n">
-        <v>503000</v>
+        <v>-186000</v>
       </c>
       <c r="G21" t="n">
-        <v>25.01243162605669</v>
+        <v>-6.625111308993767</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>대신증권</t>
+          <t>휴스틸</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>55</v>
+        <v>500</v>
       </c>
       <c r="C22" t="inlineStr">
         <is>
@@ -1026,23 +1026,23 @@
         <v>1</v>
       </c>
       <c r="E22" t="n">
-        <v>2219250</v>
+        <v>2750000</v>
       </c>
       <c r="F22" t="n">
-        <v>509749</v>
+        <v>471390</v>
       </c>
       <c r="G22" t="n">
-        <v>29.81858448752005</v>
+        <v>20.68761218462133</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>대창단조</t>
+          <t>DL이앤씨</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>300</v>
+        <v>80</v>
       </c>
       <c r="C23" t="inlineStr">
         <is>
@@ -1053,23 +1053,23 @@
         <v>1</v>
       </c>
       <c r="E23" t="n">
-        <v>2004000</v>
+        <v>5392000</v>
       </c>
       <c r="F23" t="n">
-        <v>-54000</v>
+        <v>1981000</v>
       </c>
       <c r="G23" t="n">
-        <v>-2.623906705539359</v>
+        <v>58.07681031955438</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>대한조선</t>
+          <t>HD건설기계</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>100</v>
+        <v>31</v>
       </c>
       <c r="C24" t="inlineStr">
         <is>
@@ -1080,23 +1080,23 @@
         <v>1</v>
       </c>
       <c r="E24" t="n">
-        <v>9120000</v>
+        <v>4123000</v>
       </c>
       <c r="F24" t="n">
-        <v>1907000</v>
+        <v>87904</v>
       </c>
       <c r="G24" t="n">
-        <v>26.43837515596839</v>
+        <v>2.178485964150543</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>동방</t>
+          <t>KoAct 코스닥액티브</t>
         </is>
       </c>
       <c r="B25" t="n">
-        <v>681</v>
+        <v>200</v>
       </c>
       <c r="C25" t="inlineStr">
         <is>
@@ -1107,23 +1107,23 @@
         <v>1</v>
       </c>
       <c r="E25" t="n">
-        <v>1995330</v>
+        <v>2582000</v>
       </c>
       <c r="F25" t="n">
-        <v>23829</v>
+        <v>-120000</v>
       </c>
       <c r="G25" t="n">
-        <v>1.208672985709873</v>
+        <v>-4.441154700222058</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>동원개발</t>
+          <t>TIME 코리아밸류업액티브</t>
         </is>
       </c>
       <c r="B26" t="n">
-        <v>1360</v>
+        <v>201</v>
       </c>
       <c r="C26" t="inlineStr">
         <is>
@@ -1134,23 +1134,23 @@
         <v>1</v>
       </c>
       <c r="E26" t="n">
-        <v>4202400</v>
+        <v>4797870</v>
       </c>
       <c r="F26" t="n">
-        <v>465000</v>
+        <v>74073</v>
       </c>
       <c r="G26" t="n">
-        <v>12.44180446299566</v>
+        <v>1.568081778281328</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>미창석유</t>
+          <t>센트러스 에너지</t>
         </is>
       </c>
       <c r="B27" t="n">
-        <v>18</v>
+        <v>25</v>
       </c>
       <c r="C27" t="inlineStr">
         <is>
@@ -1161,23 +1161,23 @@
         <v>1</v>
       </c>
       <c r="E27" t="n">
-        <v>2097000</v>
+        <v>7026050.85816239</v>
       </c>
       <c r="F27" t="n">
-        <v>-295200</v>
+        <v>-406805.1418376099</v>
       </c>
       <c r="G27" t="n">
-        <v>-12.34010534236268</v>
+        <v>-5.473066366920198</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>비에이치아이</t>
+          <t>스타 벌크 캐리어스</t>
         </is>
       </c>
       <c r="B28" t="n">
-        <v>8</v>
+        <v>50</v>
       </c>
       <c r="C28" t="inlineStr">
         <is>
@@ -1188,23 +1188,23 @@
         <v>1</v>
       </c>
       <c r="E28" t="n">
-        <v>876000</v>
+        <v>1680142.640194588</v>
       </c>
       <c r="F28" t="n">
-        <v>210885</v>
+        <v>365789.6401945879</v>
       </c>
       <c r="G28" t="n">
-        <v>31.70654698811484</v>
+        <v>27.83039565433242</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>삼성생명</t>
+          <t>시드릴</t>
         </is>
       </c>
       <c r="B29" t="n">
-        <v>4</v>
+        <v>123</v>
       </c>
       <c r="C29" t="inlineStr">
         <is>
@@ -1215,23 +1215,23 @@
         <v>1</v>
       </c>
       <c r="E29" t="n">
-        <v>926000</v>
+        <v>8070101.805898919</v>
       </c>
       <c r="F29" t="n">
-        <v>93000</v>
+        <v>1619750.805898919</v>
       </c>
       <c r="G29" t="n">
-        <v>11.16446578631453</v>
+        <v>25.11104908707943</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>삼성화재</t>
+          <t>오케아니스 에코 탱커스</t>
         </is>
       </c>
       <c r="B30" t="n">
-        <v>7</v>
+        <v>65</v>
       </c>
       <c r="C30" t="inlineStr">
         <is>
@@ -1242,23 +1242,23 @@
         <v>1</v>
       </c>
       <c r="E30" t="n">
-        <v>3321500</v>
+        <v>4511179.137784176</v>
       </c>
       <c r="F30" t="n">
-        <v>-309500</v>
+        <v>2254819.137784176</v>
       </c>
       <c r="G30" t="n">
-        <v>-8.523822638391627</v>
+        <v>99.93171026716374</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>세아제강</t>
+          <t>차코스 에너지 내비게이션</t>
         </is>
       </c>
       <c r="B31" t="n">
-        <v>50</v>
+        <v>75</v>
       </c>
       <c r="C31" t="inlineStr">
         <is>
@@ -1269,23 +1269,23 @@
         <v>1</v>
       </c>
       <c r="E31" t="n">
-        <v>7395000</v>
+        <v>4026924.996845168</v>
       </c>
       <c r="F31" t="n">
-        <v>1085000</v>
+        <v>202276.9968451681</v>
       </c>
       <c r="G31" t="n">
-        <v>17.19492868462758</v>
+        <v>5.28877420471552</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>케이씨</t>
+          <t>클리블랜드 클리프스</t>
         </is>
       </c>
       <c r="B32" t="n">
-        <v>50</v>
+        <v>70</v>
       </c>
       <c r="C32" t="inlineStr">
         <is>
@@ -1296,23 +1296,23 @@
         <v>1</v>
       </c>
       <c r="E32" t="n">
-        <v>1670000</v>
+        <v>823743.9360268187</v>
       </c>
       <c r="F32" t="n">
-        <v>20500</v>
+        <v>-192311.0639731813</v>
       </c>
       <c r="G32" t="n">
-        <v>1.242800848742043</v>
+        <v>-18.92722972409774</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>하나금융지주</t>
+          <t>타이드워터</t>
         </is>
       </c>
       <c r="B33" t="n">
-        <v>10</v>
+        <v>48</v>
       </c>
       <c r="C33" t="inlineStr">
         <is>
@@ -1323,23 +1323,23 @@
         <v>1</v>
       </c>
       <c r="E33" t="n">
-        <v>1132000</v>
+        <v>5235363.852789983</v>
       </c>
       <c r="F33" t="n">
-        <v>23000</v>
+        <v>1510818.852789983</v>
       </c>
       <c r="G33" t="n">
-        <v>2.073940486925157</v>
+        <v>40.56385015592463</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>현대제철</t>
+          <t>텍사스 퍼시픽 랜드</t>
         </is>
       </c>
       <c r="B34" t="n">
-        <v>70</v>
+        <v>2</v>
       </c>
       <c r="C34" t="inlineStr">
         <is>
@@ -1350,23 +1350,23 @@
         <v>1</v>
       </c>
       <c r="E34" t="n">
-        <v>2621500</v>
+        <v>1563247.374122903</v>
       </c>
       <c r="F34" t="n">
-        <v>-186000</v>
+        <v>-14646.62587709725</v>
       </c>
       <c r="G34" t="n">
-        <v>-6.625111308993767</v>
+        <v>-0.9282388979929735</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>휴스틸</t>
+          <t>트랜스오션</t>
         </is>
       </c>
       <c r="B35" t="n">
-        <v>500</v>
+        <v>750</v>
       </c>
       <c r="C35" t="inlineStr">
         <is>
@@ -1377,23 +1377,23 @@
         <v>1</v>
       </c>
       <c r="E35" t="n">
-        <v>2750000</v>
+        <v>7020031.5082007</v>
       </c>
       <c r="F35" t="n">
-        <v>471390</v>
+        <v>2892797.5082007</v>
       </c>
       <c r="G35" t="n">
-        <v>20.68761218462133</v>
+        <v>70.09046514446965</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>DL이앤씨</t>
+          <t>페트로브라스 (ADR)</t>
         </is>
       </c>
       <c r="B36" t="n">
-        <v>80</v>
+        <v>480</v>
       </c>
       <c r="C36" t="inlineStr">
         <is>
@@ -1404,23 +1404,23 @@
         <v>1</v>
       </c>
       <c r="E36" t="n">
-        <v>5392000</v>
+        <v>13579584.97235231</v>
       </c>
       <c r="F36" t="n">
-        <v>1981000</v>
+        <v>1473035.972352311</v>
       </c>
       <c r="G36" t="n">
-        <v>58.07681031955438</v>
+        <v>12.16726560436265</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>HD건설기계</t>
+          <t>프론트라인</t>
         </is>
       </c>
       <c r="B37" t="n">
-        <v>31</v>
+        <v>175</v>
       </c>
       <c r="C37" t="inlineStr">
         <is>
@@ -1431,23 +1431,23 @@
         <v>1</v>
       </c>
       <c r="E37" t="n">
-        <v>4123000</v>
+        <v>8471815.962899337</v>
       </c>
       <c r="F37" t="n">
-        <v>87904</v>
+        <v>4041951.962899337</v>
       </c>
       <c r="G37" t="n">
-        <v>2.178485964150543</v>
+        <v>91.24325177701475</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>KoAct 코스닥액티브</t>
+          <t>피바디 에너지</t>
         </is>
       </c>
       <c r="B38" t="n">
-        <v>200</v>
+        <v>65</v>
       </c>
       <c r="C38" t="inlineStr">
         <is>
@@ -1458,23 +1458,23 @@
         <v>1</v>
       </c>
       <c r="E38" t="n">
-        <v>2582000</v>
+        <v>3649438.50225304</v>
       </c>
       <c r="F38" t="n">
-        <v>-120000</v>
+        <v>2178666.50225304</v>
       </c>
       <c r="G38" t="n">
-        <v>-4.441154700222058</v>
+        <v>148.1308117269733</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>TIME 코리아밸류업액티브</t>
+          <t>하프니아</t>
         </is>
       </c>
       <c r="B39" t="n">
-        <v>201</v>
+        <v>80</v>
       </c>
       <c r="C39" t="inlineStr">
         <is>
@@ -1485,13 +1485,13 @@
         <v>1</v>
       </c>
       <c r="E39" t="n">
-        <v>4797870</v>
+        <v>842704.775390625</v>
       </c>
       <c r="F39" t="n">
-        <v>74073</v>
+        <v>216973.775390625</v>
       </c>
       <c r="G39" t="n">
-        <v>1.568081778281328</v>
+        <v>34.67524789256486</v>
       </c>
     </row>
   </sheetData>
@@ -1549,7 +1549,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2026-03-21T04:48:29</t>
+          <t>2026-03-21T04:51:19</t>
         </is>
       </c>
       <c r="E2" t="n">
@@ -3049,14 +3049,14 @@
         <v>13579584.97235231</v>
       </c>
       <c r="G40" t="n">
-        <v>1473035.972352313</v>
+        <v>1473035.972352311</v>
       </c>
       <c r="H40" t="n">
-        <v>12.16726560436267</v>
+        <v>12.16726560436265</v>
       </c>
       <c r="I40" t="inlineStr">
         <is>
-          <t>2026-03-21T04:48:28</t>
+          <t>2026-03-21T04:51:19</t>
         </is>
       </c>
     </row>
@@ -3093,7 +3093,7 @@
       </c>
       <c r="I41" t="inlineStr">
         <is>
-          <t>2026-03-21T04:48:28</t>
+          <t>2026-03-21T04:51:19</t>
         </is>
       </c>
     </row>
@@ -3130,7 +3130,7 @@
       </c>
       <c r="I42" t="inlineStr">
         <is>
-          <t>2026-03-21T04:48:28</t>
+          <t>2026-03-21T04:51:19</t>
         </is>
       </c>
     </row>
@@ -3167,7 +3167,7 @@
       </c>
       <c r="I43" t="inlineStr">
         <is>
-          <t>2026-03-21T04:48:28</t>
+          <t>2026-03-21T04:51:19</t>
         </is>
       </c>
     </row>
@@ -3204,7 +3204,7 @@
       </c>
       <c r="I44" t="inlineStr">
         <is>
-          <t>2026-03-21T04:48:28</t>
+          <t>2026-03-21T04:51:19</t>
         </is>
       </c>
     </row>
@@ -3241,7 +3241,7 @@
       </c>
       <c r="I45" t="inlineStr">
         <is>
-          <t>2026-03-21T04:48:28</t>
+          <t>2026-03-21T04:51:19</t>
         </is>
       </c>
     </row>
@@ -3253,11 +3253,11 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>트랜스오션</t>
+          <t>센트러스 에너지</t>
         </is>
       </c>
       <c r="C46" t="n">
-        <v>750</v>
+        <v>25</v>
       </c>
       <c r="D46" t="inlineStr">
         <is>
@@ -3268,17 +3268,17 @@
         <v>1</v>
       </c>
       <c r="F46" t="n">
-        <v>7020031.5082007</v>
+        <v>7026050.85816239</v>
       </c>
       <c r="G46" t="n">
-        <v>2892797.5082007</v>
+        <v>-406805.1418376099</v>
       </c>
       <c r="H46" t="n">
-        <v>70.09046514446965</v>
+        <v>-5.473066366920198</v>
       </c>
       <c r="I46" t="inlineStr">
         <is>
-          <t>2026-03-21T04:48:28</t>
+          <t>2026-03-21T04:51:19</t>
         </is>
       </c>
     </row>
@@ -3290,11 +3290,11 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>센트러스 에너지</t>
+          <t>트랜스오션</t>
         </is>
       </c>
       <c r="C47" t="n">
-        <v>21</v>
+        <v>750</v>
       </c>
       <c r="D47" t="inlineStr">
         <is>
@@ -3305,17 +3305,17 @@
         <v>1</v>
       </c>
       <c r="F47" t="n">
-        <v>5901882.720856408</v>
+        <v>7020031.5082007</v>
       </c>
       <c r="G47" t="n">
-        <v>-329336.2791435914</v>
+        <v>2892797.5082007</v>
       </c>
       <c r="H47" t="n">
-        <v>-5.285262468605123</v>
+        <v>70.09046514446965</v>
       </c>
       <c r="I47" t="inlineStr">
         <is>
-          <t>2026-03-21T04:48:28</t>
+          <t>2026-03-21T04:51:19</t>
         </is>
       </c>
     </row>
@@ -3352,7 +3352,7 @@
       </c>
       <c r="I48" t="inlineStr">
         <is>
-          <t>2026-03-21T04:48:28</t>
+          <t>2026-03-21T04:51:19</t>
         </is>
       </c>
     </row>
@@ -3389,7 +3389,7 @@
       </c>
       <c r="I49" t="inlineStr">
         <is>
-          <t>2026-03-21T04:48:28</t>
+          <t>2026-03-21T04:51:19</t>
         </is>
       </c>
     </row>
@@ -3426,7 +3426,7 @@
       </c>
       <c r="I50" t="inlineStr">
         <is>
-          <t>2026-03-21T04:48:28</t>
+          <t>2026-03-21T04:51:19</t>
         </is>
       </c>
     </row>
@@ -3463,7 +3463,7 @@
       </c>
       <c r="I51" t="inlineStr">
         <is>
-          <t>2026-03-21T04:48:28</t>
+          <t>2026-03-21T04:51:19</t>
         </is>
       </c>
     </row>
@@ -3496,11 +3496,11 @@
         <v>2254819.137784176</v>
       </c>
       <c r="H52" t="n">
-        <v>99.93171026716378</v>
+        <v>99.93171026716374</v>
       </c>
       <c r="I52" t="inlineStr">
         <is>
-          <t>2026-03-21T04:48:28</t>
+          <t>2026-03-21T04:51:19</t>
         </is>
       </c>
     </row>
@@ -3537,7 +3537,7 @@
       </c>
       <c r="I53" t="inlineStr">
         <is>
-          <t>2026-03-21T04:48:28</t>
+          <t>2026-03-21T04:51:19</t>
         </is>
       </c>
     </row>
@@ -3574,7 +3574,7 @@
       </c>
       <c r="I54" t="inlineStr">
         <is>
-          <t>2026-03-21T04:48:28</t>
+          <t>2026-03-21T04:51:19</t>
         </is>
       </c>
     </row>
@@ -3611,7 +3611,7 @@
       </c>
       <c r="I55" t="inlineStr">
         <is>
-          <t>2026-03-21T04:48:28</t>
+          <t>2026-03-21T04:51:19</t>
         </is>
       </c>
     </row>
@@ -3648,7 +3648,7 @@
       </c>
       <c r="I56" t="inlineStr">
         <is>
-          <t>2026-03-21T04:48:28</t>
+          <t>2026-03-21T04:51:19</t>
         </is>
       </c>
     </row>
@@ -3685,7 +3685,7 @@
       </c>
       <c r="I57" t="inlineStr">
         <is>
-          <t>2026-03-21T04:48:28</t>
+          <t>2026-03-21T04:51:19</t>
         </is>
       </c>
     </row>
@@ -3722,7 +3722,7 @@
       </c>
       <c r="I58" t="inlineStr">
         <is>
-          <t>2026-03-21T04:48:28</t>
+          <t>2026-03-21T04:51:19</t>
         </is>
       </c>
     </row>
@@ -3759,7 +3759,7 @@
       </c>
       <c r="I59" t="inlineStr">
         <is>
-          <t>2026-03-21T04:48:28</t>
+          <t>2026-03-21T04:51:19</t>
         </is>
       </c>
     </row>
@@ -3796,7 +3796,7 @@
       </c>
       <c r="I60" t="inlineStr">
         <is>
-          <t>2026-03-21T04:48:28</t>
+          <t>2026-03-21T04:51:19</t>
         </is>
       </c>
     </row>
@@ -3833,7 +3833,7 @@
       </c>
       <c r="I61" t="inlineStr">
         <is>
-          <t>2026-03-21T04:48:28</t>
+          <t>2026-03-21T04:51:19</t>
         </is>
       </c>
     </row>
@@ -3870,7 +3870,7 @@
       </c>
       <c r="I62" t="inlineStr">
         <is>
-          <t>2026-03-21T04:48:28</t>
+          <t>2026-03-21T04:51:19</t>
         </is>
       </c>
     </row>
@@ -3907,7 +3907,7 @@
       </c>
       <c r="I63" t="inlineStr">
         <is>
-          <t>2026-03-21T04:48:28</t>
+          <t>2026-03-21T04:51:19</t>
         </is>
       </c>
     </row>
@@ -3944,7 +3944,7 @@
       </c>
       <c r="I64" t="inlineStr">
         <is>
-          <t>2026-03-21T04:48:28</t>
+          <t>2026-03-21T04:51:19</t>
         </is>
       </c>
     </row>
@@ -3981,7 +3981,7 @@
       </c>
       <c r="I65" t="inlineStr">
         <is>
-          <t>2026-03-21T04:48:28</t>
+          <t>2026-03-21T04:51:19</t>
         </is>
       </c>
     </row>
@@ -4018,7 +4018,7 @@
       </c>
       <c r="I66" t="inlineStr">
         <is>
-          <t>2026-03-21T04:48:28</t>
+          <t>2026-03-21T04:51:19</t>
         </is>
       </c>
     </row>
@@ -4055,7 +4055,7 @@
       </c>
       <c r="I67" t="inlineStr">
         <is>
-          <t>2026-03-21T04:48:28</t>
+          <t>2026-03-21T04:51:19</t>
         </is>
       </c>
     </row>
@@ -4085,14 +4085,14 @@
         <v>1680142.640194588</v>
       </c>
       <c r="G68" t="n">
-        <v>365789.6401945876</v>
+        <v>365789.6401945879</v>
       </c>
       <c r="H68" t="n">
-        <v>27.8303956543324</v>
+        <v>27.83039565433242</v>
       </c>
       <c r="I68" t="inlineStr">
         <is>
-          <t>2026-03-21T04:48:28</t>
+          <t>2026-03-21T04:51:19</t>
         </is>
       </c>
     </row>
@@ -4129,7 +4129,7 @@
       </c>
       <c r="I69" t="inlineStr">
         <is>
-          <t>2026-03-21T04:48:28</t>
+          <t>2026-03-21T04:51:19</t>
         </is>
       </c>
     </row>
@@ -4166,7 +4166,7 @@
       </c>
       <c r="I70" t="inlineStr">
         <is>
-          <t>2026-03-21T04:48:28</t>
+          <t>2026-03-21T04:51:19</t>
         </is>
       </c>
     </row>
@@ -4178,11 +4178,11 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>하나금융지주</t>
+          <t>텍사스 퍼시픽 랜드</t>
         </is>
       </c>
       <c r="C71" t="n">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="D71" t="inlineStr">
         <is>
@@ -4193,17 +4193,17 @@
         <v>1</v>
       </c>
       <c r="F71" t="n">
-        <v>1132000</v>
+        <v>1563247.374122903</v>
       </c>
       <c r="G71" t="n">
-        <v>23000</v>
+        <v>-14646.62587709725</v>
       </c>
       <c r="H71" t="n">
-        <v>2.073940486925157</v>
+        <v>-0.9282388979929735</v>
       </c>
       <c r="I71" t="inlineStr">
         <is>
-          <t>2026-03-21T04:48:28</t>
+          <t>2026-03-21T04:51:19</t>
         </is>
       </c>
     </row>
@@ -4215,11 +4215,11 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>삼성생명</t>
+          <t>하나금융지주</t>
         </is>
       </c>
       <c r="C72" t="n">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="D72" t="inlineStr">
         <is>
@@ -4230,17 +4230,17 @@
         <v>1</v>
       </c>
       <c r="F72" t="n">
-        <v>926000</v>
+        <v>1132000</v>
       </c>
       <c r="G72" t="n">
-        <v>93000</v>
+        <v>23000</v>
       </c>
       <c r="H72" t="n">
-        <v>11.16446578631453</v>
+        <v>2.073940486925157</v>
       </c>
       <c r="I72" t="inlineStr">
         <is>
-          <t>2026-03-21T04:48:28</t>
+          <t>2026-03-21T04:51:19</t>
         </is>
       </c>
     </row>
@@ -4252,11 +4252,11 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>비에이치아이</t>
+          <t>삼성생명</t>
         </is>
       </c>
       <c r="C73" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="D73" t="inlineStr">
         <is>
@@ -4267,17 +4267,17 @@
         <v>1</v>
       </c>
       <c r="F73" t="n">
-        <v>876000</v>
+        <v>926000</v>
       </c>
       <c r="G73" t="n">
-        <v>210885</v>
+        <v>93000</v>
       </c>
       <c r="H73" t="n">
-        <v>31.70654698811484</v>
+        <v>11.16446578631453</v>
       </c>
       <c r="I73" t="inlineStr">
         <is>
-          <t>2026-03-21T04:48:28</t>
+          <t>2026-03-21T04:51:19</t>
         </is>
       </c>
     </row>
@@ -4289,11 +4289,11 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>하프니아</t>
+          <t>비에이치아이</t>
         </is>
       </c>
       <c r="C74" t="n">
-        <v>80</v>
+        <v>8</v>
       </c>
       <c r="D74" t="inlineStr">
         <is>
@@ -4304,17 +4304,17 @@
         <v>1</v>
       </c>
       <c r="F74" t="n">
-        <v>842704.775390625</v>
+        <v>876000</v>
       </c>
       <c r="G74" t="n">
-        <v>216973.775390625</v>
+        <v>210885</v>
       </c>
       <c r="H74" t="n">
-        <v>34.67524789256486</v>
+        <v>31.70654698811484</v>
       </c>
       <c r="I74" t="inlineStr">
         <is>
-          <t>2026-03-21T04:48:28</t>
+          <t>2026-03-21T04:51:19</t>
         </is>
       </c>
     </row>
@@ -4326,11 +4326,11 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>클리블랜드 클리프스</t>
+          <t>하프니아</t>
         </is>
       </c>
       <c r="C75" t="n">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="D75" t="inlineStr">
         <is>
@@ -4341,17 +4341,17 @@
         <v>1</v>
       </c>
       <c r="F75" t="n">
-        <v>823743.9360268187</v>
+        <v>842704.775390625</v>
       </c>
       <c r="G75" t="n">
-        <v>-192311.0639731813</v>
+        <v>216973.775390625</v>
       </c>
       <c r="H75" t="n">
-        <v>-18.92722972409774</v>
+        <v>34.67524789256486</v>
       </c>
       <c r="I75" t="inlineStr">
         <is>
-          <t>2026-03-21T04:48:28</t>
+          <t>2026-03-21T04:51:19</t>
         </is>
       </c>
     </row>
@@ -4363,11 +4363,11 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>텍사스 퍼시픽 랜드</t>
+          <t>클리블랜드 클리프스</t>
         </is>
       </c>
       <c r="C76" t="n">
-        <v>1</v>
+        <v>70</v>
       </c>
       <c r="D76" t="inlineStr">
         <is>
@@ -4378,17 +4378,17 @@
         <v>1</v>
       </c>
       <c r="F76" t="n">
-        <v>781623.6870614514</v>
+        <v>823743.9360268187</v>
       </c>
       <c r="G76" t="n">
-        <v>3032.687061451375</v>
+        <v>-192311.0639731813</v>
       </c>
       <c r="H76" t="n">
-        <v>0.3895096477420591</v>
+        <v>-18.92722972409774</v>
       </c>
       <c r="I76" t="inlineStr">
         <is>
-          <t>2026-03-21T04:48:28</t>
+          <t>2026-03-21T04:51:19</t>
         </is>
       </c>
     </row>
@@ -4425,7 +4425,7 @@
       </c>
       <c r="I77" t="inlineStr">
         <is>
-          <t>2026-03-21T04:48:28</t>
+          <t>2026-03-21T04:51:19</t>
         </is>
       </c>
     </row>
@@ -4512,7 +4512,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>2026-03-21T04:48:28</t>
+          <t>2026-03-21T04:51:19</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: portfolio snapshot 2026-03-21 (2026-03-21T04:51:20)
</commit_message>
<xml_diff>
--- a/portfolio_auto.xlsx
+++ b/portfolio_auto.xlsx
@@ -1549,7 +1549,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2026-03-21T04:51:19</t>
+          <t>2026-03-21T04:51:20</t>
         </is>
       </c>
       <c r="E2" t="n">
@@ -3056,7 +3056,7 @@
       </c>
       <c r="I40" t="inlineStr">
         <is>
-          <t>2026-03-21T04:51:19</t>
+          <t>2026-03-21T04:51:20</t>
         </is>
       </c>
     </row>
@@ -3093,7 +3093,7 @@
       </c>
       <c r="I41" t="inlineStr">
         <is>
-          <t>2026-03-21T04:51:19</t>
+          <t>2026-03-21T04:51:20</t>
         </is>
       </c>
     </row>
@@ -3130,7 +3130,7 @@
       </c>
       <c r="I42" t="inlineStr">
         <is>
-          <t>2026-03-21T04:51:19</t>
+          <t>2026-03-21T04:51:20</t>
         </is>
       </c>
     </row>
@@ -3167,7 +3167,7 @@
       </c>
       <c r="I43" t="inlineStr">
         <is>
-          <t>2026-03-21T04:51:19</t>
+          <t>2026-03-21T04:51:20</t>
         </is>
       </c>
     </row>
@@ -3204,7 +3204,7 @@
       </c>
       <c r="I44" t="inlineStr">
         <is>
-          <t>2026-03-21T04:51:19</t>
+          <t>2026-03-21T04:51:20</t>
         </is>
       </c>
     </row>
@@ -3241,7 +3241,7 @@
       </c>
       <c r="I45" t="inlineStr">
         <is>
-          <t>2026-03-21T04:51:19</t>
+          <t>2026-03-21T04:51:20</t>
         </is>
       </c>
     </row>
@@ -3278,7 +3278,7 @@
       </c>
       <c r="I46" t="inlineStr">
         <is>
-          <t>2026-03-21T04:51:19</t>
+          <t>2026-03-21T04:51:20</t>
         </is>
       </c>
     </row>
@@ -3315,7 +3315,7 @@
       </c>
       <c r="I47" t="inlineStr">
         <is>
-          <t>2026-03-21T04:51:19</t>
+          <t>2026-03-21T04:51:20</t>
         </is>
       </c>
     </row>
@@ -3352,7 +3352,7 @@
       </c>
       <c r="I48" t="inlineStr">
         <is>
-          <t>2026-03-21T04:51:19</t>
+          <t>2026-03-21T04:51:20</t>
         </is>
       </c>
     </row>
@@ -3389,7 +3389,7 @@
       </c>
       <c r="I49" t="inlineStr">
         <is>
-          <t>2026-03-21T04:51:19</t>
+          <t>2026-03-21T04:51:20</t>
         </is>
       </c>
     </row>
@@ -3426,7 +3426,7 @@
       </c>
       <c r="I50" t="inlineStr">
         <is>
-          <t>2026-03-21T04:51:19</t>
+          <t>2026-03-21T04:51:20</t>
         </is>
       </c>
     </row>
@@ -3463,7 +3463,7 @@
       </c>
       <c r="I51" t="inlineStr">
         <is>
-          <t>2026-03-21T04:51:19</t>
+          <t>2026-03-21T04:51:20</t>
         </is>
       </c>
     </row>
@@ -3500,7 +3500,7 @@
       </c>
       <c r="I52" t="inlineStr">
         <is>
-          <t>2026-03-21T04:51:19</t>
+          <t>2026-03-21T04:51:20</t>
         </is>
       </c>
     </row>
@@ -3537,7 +3537,7 @@
       </c>
       <c r="I53" t="inlineStr">
         <is>
-          <t>2026-03-21T04:51:19</t>
+          <t>2026-03-21T04:51:20</t>
         </is>
       </c>
     </row>
@@ -3574,7 +3574,7 @@
       </c>
       <c r="I54" t="inlineStr">
         <is>
-          <t>2026-03-21T04:51:19</t>
+          <t>2026-03-21T04:51:20</t>
         </is>
       </c>
     </row>
@@ -3611,7 +3611,7 @@
       </c>
       <c r="I55" t="inlineStr">
         <is>
-          <t>2026-03-21T04:51:19</t>
+          <t>2026-03-21T04:51:20</t>
         </is>
       </c>
     </row>
@@ -3648,7 +3648,7 @@
       </c>
       <c r="I56" t="inlineStr">
         <is>
-          <t>2026-03-21T04:51:19</t>
+          <t>2026-03-21T04:51:20</t>
         </is>
       </c>
     </row>
@@ -3685,7 +3685,7 @@
       </c>
       <c r="I57" t="inlineStr">
         <is>
-          <t>2026-03-21T04:51:19</t>
+          <t>2026-03-21T04:51:20</t>
         </is>
       </c>
     </row>
@@ -3722,7 +3722,7 @@
       </c>
       <c r="I58" t="inlineStr">
         <is>
-          <t>2026-03-21T04:51:19</t>
+          <t>2026-03-21T04:51:20</t>
         </is>
       </c>
     </row>
@@ -3759,7 +3759,7 @@
       </c>
       <c r="I59" t="inlineStr">
         <is>
-          <t>2026-03-21T04:51:19</t>
+          <t>2026-03-21T04:51:20</t>
         </is>
       </c>
     </row>
@@ -3796,7 +3796,7 @@
       </c>
       <c r="I60" t="inlineStr">
         <is>
-          <t>2026-03-21T04:51:19</t>
+          <t>2026-03-21T04:51:20</t>
         </is>
       </c>
     </row>
@@ -3833,7 +3833,7 @@
       </c>
       <c r="I61" t="inlineStr">
         <is>
-          <t>2026-03-21T04:51:19</t>
+          <t>2026-03-21T04:51:20</t>
         </is>
       </c>
     </row>
@@ -3870,7 +3870,7 @@
       </c>
       <c r="I62" t="inlineStr">
         <is>
-          <t>2026-03-21T04:51:19</t>
+          <t>2026-03-21T04:51:20</t>
         </is>
       </c>
     </row>
@@ -3907,7 +3907,7 @@
       </c>
       <c r="I63" t="inlineStr">
         <is>
-          <t>2026-03-21T04:51:19</t>
+          <t>2026-03-21T04:51:20</t>
         </is>
       </c>
     </row>
@@ -3944,7 +3944,7 @@
       </c>
       <c r="I64" t="inlineStr">
         <is>
-          <t>2026-03-21T04:51:19</t>
+          <t>2026-03-21T04:51:20</t>
         </is>
       </c>
     </row>
@@ -3981,7 +3981,7 @@
       </c>
       <c r="I65" t="inlineStr">
         <is>
-          <t>2026-03-21T04:51:19</t>
+          <t>2026-03-21T04:51:20</t>
         </is>
       </c>
     </row>
@@ -4018,7 +4018,7 @@
       </c>
       <c r="I66" t="inlineStr">
         <is>
-          <t>2026-03-21T04:51:19</t>
+          <t>2026-03-21T04:51:20</t>
         </is>
       </c>
     </row>
@@ -4055,7 +4055,7 @@
       </c>
       <c r="I67" t="inlineStr">
         <is>
-          <t>2026-03-21T04:51:19</t>
+          <t>2026-03-21T04:51:20</t>
         </is>
       </c>
     </row>
@@ -4092,7 +4092,7 @@
       </c>
       <c r="I68" t="inlineStr">
         <is>
-          <t>2026-03-21T04:51:19</t>
+          <t>2026-03-21T04:51:20</t>
         </is>
       </c>
     </row>
@@ -4129,7 +4129,7 @@
       </c>
       <c r="I69" t="inlineStr">
         <is>
-          <t>2026-03-21T04:51:19</t>
+          <t>2026-03-21T04:51:20</t>
         </is>
       </c>
     </row>
@@ -4166,7 +4166,7 @@
       </c>
       <c r="I70" t="inlineStr">
         <is>
-          <t>2026-03-21T04:51:19</t>
+          <t>2026-03-21T04:51:20</t>
         </is>
       </c>
     </row>
@@ -4203,7 +4203,7 @@
       </c>
       <c r="I71" t="inlineStr">
         <is>
-          <t>2026-03-21T04:51:19</t>
+          <t>2026-03-21T04:51:20</t>
         </is>
       </c>
     </row>
@@ -4240,7 +4240,7 @@
       </c>
       <c r="I72" t="inlineStr">
         <is>
-          <t>2026-03-21T04:51:19</t>
+          <t>2026-03-21T04:51:20</t>
         </is>
       </c>
     </row>
@@ -4277,7 +4277,7 @@
       </c>
       <c r="I73" t="inlineStr">
         <is>
-          <t>2026-03-21T04:51:19</t>
+          <t>2026-03-21T04:51:20</t>
         </is>
       </c>
     </row>
@@ -4314,7 +4314,7 @@
       </c>
       <c r="I74" t="inlineStr">
         <is>
-          <t>2026-03-21T04:51:19</t>
+          <t>2026-03-21T04:51:20</t>
         </is>
       </c>
     </row>
@@ -4351,7 +4351,7 @@
       </c>
       <c r="I75" t="inlineStr">
         <is>
-          <t>2026-03-21T04:51:19</t>
+          <t>2026-03-21T04:51:20</t>
         </is>
       </c>
     </row>
@@ -4388,7 +4388,7 @@
       </c>
       <c r="I76" t="inlineStr">
         <is>
-          <t>2026-03-21T04:51:19</t>
+          <t>2026-03-21T04:51:20</t>
         </is>
       </c>
     </row>
@@ -4425,7 +4425,7 @@
       </c>
       <c r="I77" t="inlineStr">
         <is>
-          <t>2026-03-21T04:51:19</t>
+          <t>2026-03-21T04:51:20</t>
         </is>
       </c>
     </row>
@@ -4512,7 +4512,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>2026-03-21T04:51:19</t>
+          <t>2026-03-21T04:51:20</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: portfolio snapshot 2026-03-17 (2026-03-21T04:51:36)
</commit_message>
<xml_diff>
--- a/portfolio_auto.xlsx
+++ b/portfolio_auto.xlsx
@@ -471,11 +471,11 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>노브</t>
+          <t>페트로브라스 (ADR)</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>185</v>
+        <v>480</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
@@ -486,23 +486,23 @@
         <v>1</v>
       </c>
       <c r="E2" t="n">
-        <v>5200391.447092756</v>
+        <v>13579584.97235231</v>
       </c>
       <c r="F2" t="n">
-        <v>1890383.447092756</v>
+        <v>1473035.972352311</v>
       </c>
       <c r="G2" t="n">
-        <v>57.11114435653194</v>
+        <v>12.16726560436265</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>노블</t>
+          <t>AGNC 인베스트먼트</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>99</v>
+        <v>700</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
@@ -513,23 +513,23 @@
         <v>1</v>
       </c>
       <c r="E3" t="n">
-        <v>40689</v>
+        <v>10270464.45007324</v>
       </c>
       <c r="F3" t="n">
-        <v>-3866519</v>
+        <v>-561550.5499267578</v>
       </c>
       <c r="G3" t="n">
-        <v>-98.95861699709869</v>
+        <v>-5.184174411933125</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>더치 브로스</t>
+          <t>대한조선</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>39</v>
+        <v>100</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
@@ -540,23 +540,23 @@
         <v>1</v>
       </c>
       <c r="E4" t="n">
-        <v>2934418.414306641</v>
+        <v>9120000</v>
       </c>
       <c r="F4" t="n">
-        <v>-256225.5856933598</v>
+        <v>1907000</v>
       </c>
       <c r="G4" t="n">
-        <v>-8.030528811530205</v>
+        <v>26.43837515596839</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>발레로 에너지</t>
+          <t>프론트라인</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>6</v>
+        <v>175</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -567,23 +567,23 @@
         <v>1</v>
       </c>
       <c r="E5" t="n">
-        <v>2165691.085066516</v>
+        <v>8471815.962899337</v>
       </c>
       <c r="F5" t="n">
-        <v>101701.085066516</v>
+        <v>4041951.962899337</v>
       </c>
       <c r="G5" t="n">
-        <v>4.927402025519307</v>
+        <v>91.24325177701475</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>유나이티드헬스 그룹</t>
+          <t>시드릴</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>4</v>
+        <v>123</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
@@ -594,23 +594,23 @@
         <v>1</v>
       </c>
       <c r="E6" t="n">
-        <v>1658864.328313038</v>
+        <v>8070101.805898919</v>
       </c>
       <c r="F6" t="n">
-        <v>-35591.67168696248</v>
+        <v>1619750.805898919</v>
       </c>
       <c r="G6" t="n">
-        <v>-2.100477774988697</v>
+        <v>25.11104908707943</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>AGNC 인베스트먼트</t>
+          <t>세아제강</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>700</v>
+        <v>50</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -621,23 +621,23 @@
         <v>1</v>
       </c>
       <c r="E7" t="n">
-        <v>10270464.45007324</v>
+        <v>7395000</v>
       </c>
       <c r="F7" t="n">
-        <v>-561550.5499267559</v>
+        <v>1085000</v>
       </c>
       <c r="G7" t="n">
-        <v>-5.184174411933109</v>
+        <v>17.19492868462758</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>넥스틸</t>
+          <t>트랜스오션</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>200</v>
+        <v>750</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
@@ -648,23 +648,23 @@
         <v>1</v>
       </c>
       <c r="E8" t="n">
-        <v>2514000</v>
+        <v>7020031.5082007</v>
       </c>
       <c r="F8" t="n">
-        <v>503000</v>
+        <v>2892797.5082007</v>
       </c>
       <c r="G8" t="n">
-        <v>25.01243162605669</v>
+        <v>70.09046514446965</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>대신증권</t>
+          <t>센트러스 에너지</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>55</v>
+        <v>21</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
@@ -675,23 +675,23 @@
         <v>1</v>
       </c>
       <c r="E9" t="n">
-        <v>2219250</v>
+        <v>5901882.720856408</v>
       </c>
       <c r="F9" t="n">
-        <v>509749</v>
+        <v>-329336.2791435914</v>
       </c>
       <c r="G9" t="n">
-        <v>29.81858448752005</v>
+        <v>-5.285262468605123</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>대창단조</t>
+          <t>DL이앤씨</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>300</v>
+        <v>80</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
@@ -702,23 +702,23 @@
         <v>1</v>
       </c>
       <c r="E10" t="n">
-        <v>2004000</v>
+        <v>5392000</v>
       </c>
       <c r="F10" t="n">
-        <v>-54000</v>
+        <v>1981000</v>
       </c>
       <c r="G10" t="n">
-        <v>-2.623906705539359</v>
+        <v>58.07681031955438</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>대한조선</t>
+          <t>타이드워터</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>100</v>
+        <v>48</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
@@ -729,23 +729,23 @@
         <v>1</v>
       </c>
       <c r="E11" t="n">
-        <v>9120000</v>
+        <v>5235363.852789983</v>
       </c>
       <c r="F11" t="n">
-        <v>1907000</v>
+        <v>1510818.852789983</v>
       </c>
       <c r="G11" t="n">
-        <v>26.43837515596839</v>
+        <v>40.56385015592463</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>동방</t>
+          <t>노브</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>681</v>
+        <v>185</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
@@ -756,23 +756,23 @@
         <v>1</v>
       </c>
       <c r="E12" t="n">
-        <v>1995330</v>
+        <v>5200391.447092756</v>
       </c>
       <c r="F12" t="n">
-        <v>23829</v>
+        <v>1890383.447092756</v>
       </c>
       <c r="G12" t="n">
-        <v>1.208672985709873</v>
+        <v>57.11114435653194</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>동원개발</t>
+          <t>TIME 코리아밸류업액티브</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>1360</v>
+        <v>201</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
@@ -783,23 +783,23 @@
         <v>1</v>
       </c>
       <c r="E13" t="n">
-        <v>4202400</v>
+        <v>4797870</v>
       </c>
       <c r="F13" t="n">
-        <v>465000</v>
+        <v>74073</v>
       </c>
       <c r="G13" t="n">
-        <v>12.44180446299566</v>
+        <v>1.568081778281328</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>미창석유</t>
+          <t>오케아니스 에코 탱커스</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>18</v>
+        <v>65</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
@@ -810,23 +810,23 @@
         <v>1</v>
       </c>
       <c r="E14" t="n">
-        <v>2097000</v>
+        <v>4511179.137784176</v>
       </c>
       <c r="F14" t="n">
-        <v>-295200</v>
+        <v>2254819.137784176</v>
       </c>
       <c r="G14" t="n">
-        <v>-12.34010534236268</v>
+        <v>99.93171026716374</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>비에이치아이</t>
+          <t>동원개발</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>8</v>
+        <v>1360</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
@@ -837,23 +837,23 @@
         <v>1</v>
       </c>
       <c r="E15" t="n">
-        <v>876000</v>
+        <v>4202400</v>
       </c>
       <c r="F15" t="n">
-        <v>210885</v>
+        <v>465000</v>
       </c>
       <c r="G15" t="n">
-        <v>31.70654698811484</v>
+        <v>12.44180446299566</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>삼성생명</t>
+          <t>HD건설기계</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>4</v>
+        <v>31</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
@@ -864,23 +864,23 @@
         <v>1</v>
       </c>
       <c r="E16" t="n">
-        <v>926000</v>
+        <v>4123000</v>
       </c>
       <c r="F16" t="n">
-        <v>93000</v>
+        <v>87904</v>
       </c>
       <c r="G16" t="n">
-        <v>11.16446578631453</v>
+        <v>2.178485964150543</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>삼성화재</t>
+          <t>차코스 에너지 내비게이션</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>7</v>
+        <v>75</v>
       </c>
       <c r="C17" t="inlineStr">
         <is>
@@ -891,23 +891,23 @@
         <v>1</v>
       </c>
       <c r="E17" t="n">
-        <v>3321500</v>
+        <v>4026924.996845168</v>
       </c>
       <c r="F17" t="n">
-        <v>-309500</v>
+        <v>202276.9968451681</v>
       </c>
       <c r="G17" t="n">
-        <v>-8.523822638391627</v>
+        <v>5.28877420471552</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>세아제강</t>
+          <t>피바디 에너지</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>50</v>
+        <v>65</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
@@ -918,23 +918,23 @@
         <v>1</v>
       </c>
       <c r="E18" t="n">
-        <v>7395000</v>
+        <v>3649438.50225304</v>
       </c>
       <c r="F18" t="n">
-        <v>1085000</v>
+        <v>2178666.50225304</v>
       </c>
       <c r="G18" t="n">
-        <v>17.19492868462758</v>
+        <v>148.1308117269733</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>케이씨</t>
+          <t>삼성화재</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>50</v>
+        <v>7</v>
       </c>
       <c r="C19" t="inlineStr">
         <is>
@@ -945,23 +945,23 @@
         <v>1</v>
       </c>
       <c r="E19" t="n">
-        <v>1670000</v>
+        <v>3321500</v>
       </c>
       <c r="F19" t="n">
-        <v>20500</v>
+        <v>-309500</v>
       </c>
       <c r="G19" t="n">
-        <v>1.242800848742043</v>
+        <v>-8.523822638391627</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>하나금융지주</t>
+          <t>더치 브로스</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>10</v>
+        <v>39</v>
       </c>
       <c r="C20" t="inlineStr">
         <is>
@@ -972,23 +972,23 @@
         <v>1</v>
       </c>
       <c r="E20" t="n">
-        <v>1132000</v>
+        <v>2934418.414306641</v>
       </c>
       <c r="F20" t="n">
-        <v>23000</v>
+        <v>-256225.5856933594</v>
       </c>
       <c r="G20" t="n">
-        <v>2.073940486925157</v>
+        <v>-8.030528811530193</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>현대제철</t>
+          <t>휴스틸</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>70</v>
+        <v>500</v>
       </c>
       <c r="C21" t="inlineStr">
         <is>
@@ -999,23 +999,23 @@
         <v>1</v>
       </c>
       <c r="E21" t="n">
-        <v>2621500</v>
+        <v>2750000</v>
       </c>
       <c r="F21" t="n">
-        <v>-186000</v>
+        <v>471390</v>
       </c>
       <c r="G21" t="n">
-        <v>-6.625111308993767</v>
+        <v>20.68761218462133</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>휴스틸</t>
+          <t>현대제철</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>500</v>
+        <v>70</v>
       </c>
       <c r="C22" t="inlineStr">
         <is>
@@ -1026,23 +1026,23 @@
         <v>1</v>
       </c>
       <c r="E22" t="n">
-        <v>2750000</v>
+        <v>2621500</v>
       </c>
       <c r="F22" t="n">
-        <v>471390</v>
+        <v>-186000</v>
       </c>
       <c r="G22" t="n">
-        <v>20.68761218462133</v>
+        <v>-6.625111308993767</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>DL이앤씨</t>
+          <t>KoAct 코스닥액티브</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>80</v>
+        <v>200</v>
       </c>
       <c r="C23" t="inlineStr">
         <is>
@@ -1053,23 +1053,23 @@
         <v>1</v>
       </c>
       <c r="E23" t="n">
-        <v>5392000</v>
+        <v>2582000</v>
       </c>
       <c r="F23" t="n">
-        <v>1981000</v>
+        <v>-120000</v>
       </c>
       <c r="G23" t="n">
-        <v>58.07681031955438</v>
+        <v>-4.441154700222058</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>HD건설기계</t>
+          <t>넥스틸</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>31</v>
+        <v>200</v>
       </c>
       <c r="C24" t="inlineStr">
         <is>
@@ -1080,23 +1080,23 @@
         <v>1</v>
       </c>
       <c r="E24" t="n">
-        <v>4123000</v>
+        <v>2514000</v>
       </c>
       <c r="F24" t="n">
-        <v>87904</v>
+        <v>503000</v>
       </c>
       <c r="G24" t="n">
-        <v>2.178485964150543</v>
+        <v>25.01243162605669</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>KoAct 코스닥액티브</t>
+          <t>대신증권</t>
         </is>
       </c>
       <c r="B25" t="n">
-        <v>200</v>
+        <v>55</v>
       </c>
       <c r="C25" t="inlineStr">
         <is>
@@ -1107,23 +1107,23 @@
         <v>1</v>
       </c>
       <c r="E25" t="n">
-        <v>2582000</v>
+        <v>2219250</v>
       </c>
       <c r="F25" t="n">
-        <v>-120000</v>
+        <v>509749</v>
       </c>
       <c r="G25" t="n">
-        <v>-4.441154700222058</v>
+        <v>29.81858448752005</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>TIME 코리아밸류업액티브</t>
+          <t>발레로 에너지</t>
         </is>
       </c>
       <c r="B26" t="n">
-        <v>201</v>
+        <v>6</v>
       </c>
       <c r="C26" t="inlineStr">
         <is>
@@ -1134,23 +1134,23 @@
         <v>1</v>
       </c>
       <c r="E26" t="n">
-        <v>4797870</v>
+        <v>2165691.085066516</v>
       </c>
       <c r="F26" t="n">
-        <v>74073</v>
+        <v>101701.085066516</v>
       </c>
       <c r="G26" t="n">
-        <v>1.568081778281328</v>
+        <v>4.927402025519307</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>센트러스 에너지</t>
+          <t>미창석유</t>
         </is>
       </c>
       <c r="B27" t="n">
-        <v>25</v>
+        <v>18</v>
       </c>
       <c r="C27" t="inlineStr">
         <is>
@@ -1161,23 +1161,23 @@
         <v>1</v>
       </c>
       <c r="E27" t="n">
-        <v>7026050.85816239</v>
+        <v>2097000</v>
       </c>
       <c r="F27" t="n">
-        <v>-406805.1418376099</v>
+        <v>-295200</v>
       </c>
       <c r="G27" t="n">
-        <v>-5.473066366920198</v>
+        <v>-12.34010534236268</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>스타 벌크 캐리어스</t>
+          <t>대창단조</t>
         </is>
       </c>
       <c r="B28" t="n">
-        <v>50</v>
+        <v>300</v>
       </c>
       <c r="C28" t="inlineStr">
         <is>
@@ -1188,23 +1188,23 @@
         <v>1</v>
       </c>
       <c r="E28" t="n">
-        <v>1680142.640194588</v>
+        <v>2004000</v>
       </c>
       <c r="F28" t="n">
-        <v>365789.6401945879</v>
+        <v>-54000</v>
       </c>
       <c r="G28" t="n">
-        <v>27.83039565433242</v>
+        <v>-2.623906705539359</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>시드릴</t>
+          <t>동방</t>
         </is>
       </c>
       <c r="B29" t="n">
-        <v>123</v>
+        <v>681</v>
       </c>
       <c r="C29" t="inlineStr">
         <is>
@@ -1215,23 +1215,23 @@
         <v>1</v>
       </c>
       <c r="E29" t="n">
-        <v>8070101.805898919</v>
+        <v>1995330</v>
       </c>
       <c r="F29" t="n">
-        <v>1619750.805898919</v>
+        <v>23829</v>
       </c>
       <c r="G29" t="n">
-        <v>25.11104908707943</v>
+        <v>1.208672985709873</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>오케아니스 에코 탱커스</t>
+          <t>스타 벌크 캐리어스</t>
         </is>
       </c>
       <c r="B30" t="n">
-        <v>65</v>
+        <v>50</v>
       </c>
       <c r="C30" t="inlineStr">
         <is>
@@ -1242,23 +1242,23 @@
         <v>1</v>
       </c>
       <c r="E30" t="n">
-        <v>4511179.137784176</v>
+        <v>1680142.640194588</v>
       </c>
       <c r="F30" t="n">
-        <v>2254819.137784176</v>
+        <v>365789.6401945879</v>
       </c>
       <c r="G30" t="n">
-        <v>99.93171026716374</v>
+        <v>27.83039565433242</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>차코스 에너지 내비게이션</t>
+          <t>케이씨</t>
         </is>
       </c>
       <c r="B31" t="n">
-        <v>75</v>
+        <v>50</v>
       </c>
       <c r="C31" t="inlineStr">
         <is>
@@ -1269,23 +1269,23 @@
         <v>1</v>
       </c>
       <c r="E31" t="n">
-        <v>4026924.996845168</v>
+        <v>1670000</v>
       </c>
       <c r="F31" t="n">
-        <v>202276.9968451681</v>
+        <v>20500</v>
       </c>
       <c r="G31" t="n">
-        <v>5.28877420471552</v>
+        <v>1.242800848742043</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>클리블랜드 클리프스</t>
+          <t>유나이티드헬스 그룹</t>
         </is>
       </c>
       <c r="B32" t="n">
-        <v>70</v>
+        <v>4</v>
       </c>
       <c r="C32" t="inlineStr">
         <is>
@@ -1296,23 +1296,23 @@
         <v>1</v>
       </c>
       <c r="E32" t="n">
-        <v>823743.9360268187</v>
+        <v>1658864.328313038</v>
       </c>
       <c r="F32" t="n">
-        <v>-192311.0639731813</v>
+        <v>-35591.67168696225</v>
       </c>
       <c r="G32" t="n">
-        <v>-18.92722972409774</v>
+        <v>-2.100477774988684</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>타이드워터</t>
+          <t>하나금융지주</t>
         </is>
       </c>
       <c r="B33" t="n">
-        <v>48</v>
+        <v>10</v>
       </c>
       <c r="C33" t="inlineStr">
         <is>
@@ -1323,23 +1323,23 @@
         <v>1</v>
       </c>
       <c r="E33" t="n">
-        <v>5235363.852789983</v>
+        <v>1132000</v>
       </c>
       <c r="F33" t="n">
-        <v>1510818.852789983</v>
+        <v>23000</v>
       </c>
       <c r="G33" t="n">
-        <v>40.56385015592463</v>
+        <v>2.073940486925157</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>텍사스 퍼시픽 랜드</t>
+          <t>삼성생명</t>
         </is>
       </c>
       <c r="B34" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="C34" t="inlineStr">
         <is>
@@ -1350,23 +1350,23 @@
         <v>1</v>
       </c>
       <c r="E34" t="n">
-        <v>1563247.374122903</v>
+        <v>926000</v>
       </c>
       <c r="F34" t="n">
-        <v>-14646.62587709725</v>
+        <v>93000</v>
       </c>
       <c r="G34" t="n">
-        <v>-0.9282388979929735</v>
+        <v>11.16446578631453</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>트랜스오션</t>
+          <t>비에이치아이</t>
         </is>
       </c>
       <c r="B35" t="n">
-        <v>750</v>
+        <v>8</v>
       </c>
       <c r="C35" t="inlineStr">
         <is>
@@ -1377,23 +1377,23 @@
         <v>1</v>
       </c>
       <c r="E35" t="n">
-        <v>7020031.5082007</v>
+        <v>876000</v>
       </c>
       <c r="F35" t="n">
-        <v>2892797.5082007</v>
+        <v>210885</v>
       </c>
       <c r="G35" t="n">
-        <v>70.09046514446965</v>
+        <v>31.70654698811484</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>페트로브라스 (ADR)</t>
+          <t>클리블랜드 클리프스</t>
         </is>
       </c>
       <c r="B36" t="n">
-        <v>480</v>
+        <v>70</v>
       </c>
       <c r="C36" t="inlineStr">
         <is>
@@ -1404,23 +1404,23 @@
         <v>1</v>
       </c>
       <c r="E36" t="n">
-        <v>13579584.97235231</v>
+        <v>823743.9360268187</v>
       </c>
       <c r="F36" t="n">
-        <v>1473035.972352311</v>
+        <v>-192311.0639731813</v>
       </c>
       <c r="G36" t="n">
-        <v>12.16726560436265</v>
+        <v>-18.92722972409774</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>프론트라인</t>
+          <t>하프니아</t>
         </is>
       </c>
       <c r="B37" t="n">
-        <v>175</v>
+        <v>80</v>
       </c>
       <c r="C37" t="inlineStr">
         <is>
@@ -1431,23 +1431,23 @@
         <v>1</v>
       </c>
       <c r="E37" t="n">
-        <v>8471815.962899337</v>
+        <v>798051</v>
       </c>
       <c r="F37" t="n">
-        <v>4041951.962899337</v>
+        <v>172320</v>
       </c>
       <c r="G37" t="n">
-        <v>91.24325177701475</v>
+        <v>27.53899039683186</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>피바디 에너지</t>
+          <t>텍사스 퍼시픽 랜드</t>
         </is>
       </c>
       <c r="B38" t="n">
-        <v>65</v>
+        <v>1</v>
       </c>
       <c r="C38" t="inlineStr">
         <is>
@@ -1458,23 +1458,23 @@
         <v>1</v>
       </c>
       <c r="E38" t="n">
-        <v>3649438.50225304</v>
+        <v>781623.6870614514</v>
       </c>
       <c r="F38" t="n">
-        <v>2178666.50225304</v>
+        <v>3032.687061451375</v>
       </c>
       <c r="G38" t="n">
-        <v>148.1308117269733</v>
+        <v>0.3895096477420591</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>하프니아</t>
+          <t>노블</t>
         </is>
       </c>
       <c r="B39" t="n">
-        <v>80</v>
+        <v>99</v>
       </c>
       <c r="C39" t="inlineStr">
         <is>
@@ -1485,13 +1485,13 @@
         <v>1</v>
       </c>
       <c r="E39" t="n">
-        <v>842704.775390625</v>
+        <v>40689</v>
       </c>
       <c r="F39" t="n">
-        <v>216973.775390625</v>
+        <v>-3866519</v>
       </c>
       <c r="G39" t="n">
-        <v>34.67524789256486</v>
+        <v>-98.95861699709869</v>
       </c>
     </row>
   </sheetData>
@@ -1538,22 +1538,22 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-03-21</t>
+          <t>2026-03-17</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>31036676</v>
+        <v>33078556</v>
       </c>
       <c r="C2" t="n">
-        <v>6052.96</v>
+        <v>6010.99</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2026-03-21T04:51:20</t>
+          <t>2026-03-21T04:51:36</t>
         </is>
       </c>
       <c r="E2" t="n">
-        <v>1504.829956054688</v>
+        <v>1488.910034179688</v>
       </c>
     </row>
   </sheetData>
@@ -1567,7 +1567,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I77"/>
+  <dimension ref="A1:I39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3020,1412 +3020,6 @@
       <c r="I39" t="inlineStr">
         <is>
           <t>2026-03-21T03:46:22</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" t="inlineStr">
-        <is>
-          <t>2026-03-21</t>
-        </is>
-      </c>
-      <c r="B40" t="inlineStr">
-        <is>
-          <t>페트로브라스 (ADR)</t>
-        </is>
-      </c>
-      <c r="C40" t="n">
-        <v>480</v>
-      </c>
-      <c r="D40" t="inlineStr">
-        <is>
-          <t>KRW</t>
-        </is>
-      </c>
-      <c r="E40" t="n">
-        <v>1</v>
-      </c>
-      <c r="F40" t="n">
-        <v>13579584.97235231</v>
-      </c>
-      <c r="G40" t="n">
-        <v>1473035.972352311</v>
-      </c>
-      <c r="H40" t="n">
-        <v>12.16726560436265</v>
-      </c>
-      <c r="I40" t="inlineStr">
-        <is>
-          <t>2026-03-21T04:51:20</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" t="inlineStr">
-        <is>
-          <t>2026-03-21</t>
-        </is>
-      </c>
-      <c r="B41" t="inlineStr">
-        <is>
-          <t>AGNC 인베스트먼트</t>
-        </is>
-      </c>
-      <c r="C41" t="n">
-        <v>700</v>
-      </c>
-      <c r="D41" t="inlineStr">
-        <is>
-          <t>KRW</t>
-        </is>
-      </c>
-      <c r="E41" t="n">
-        <v>1</v>
-      </c>
-      <c r="F41" t="n">
-        <v>10270464.45007324</v>
-      </c>
-      <c r="G41" t="n">
-        <v>-561550.5499267559</v>
-      </c>
-      <c r="H41" t="n">
-        <v>-5.184174411933109</v>
-      </c>
-      <c r="I41" t="inlineStr">
-        <is>
-          <t>2026-03-21T04:51:20</t>
-        </is>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" t="inlineStr">
-        <is>
-          <t>2026-03-21</t>
-        </is>
-      </c>
-      <c r="B42" t="inlineStr">
-        <is>
-          <t>대한조선</t>
-        </is>
-      </c>
-      <c r="C42" t="n">
-        <v>100</v>
-      </c>
-      <c r="D42" t="inlineStr">
-        <is>
-          <t>KRW</t>
-        </is>
-      </c>
-      <c r="E42" t="n">
-        <v>1</v>
-      </c>
-      <c r="F42" t="n">
-        <v>9120000</v>
-      </c>
-      <c r="G42" t="n">
-        <v>1907000</v>
-      </c>
-      <c r="H42" t="n">
-        <v>26.43837515596839</v>
-      </c>
-      <c r="I42" t="inlineStr">
-        <is>
-          <t>2026-03-21T04:51:20</t>
-        </is>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" t="inlineStr">
-        <is>
-          <t>2026-03-21</t>
-        </is>
-      </c>
-      <c r="B43" t="inlineStr">
-        <is>
-          <t>프론트라인</t>
-        </is>
-      </c>
-      <c r="C43" t="n">
-        <v>175</v>
-      </c>
-      <c r="D43" t="inlineStr">
-        <is>
-          <t>KRW</t>
-        </is>
-      </c>
-      <c r="E43" t="n">
-        <v>1</v>
-      </c>
-      <c r="F43" t="n">
-        <v>8471815.962899337</v>
-      </c>
-      <c r="G43" t="n">
-        <v>4041951.962899337</v>
-      </c>
-      <c r="H43" t="n">
-        <v>91.24325177701475</v>
-      </c>
-      <c r="I43" t="inlineStr">
-        <is>
-          <t>2026-03-21T04:51:20</t>
-        </is>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" t="inlineStr">
-        <is>
-          <t>2026-03-21</t>
-        </is>
-      </c>
-      <c r="B44" t="inlineStr">
-        <is>
-          <t>시드릴</t>
-        </is>
-      </c>
-      <c r="C44" t="n">
-        <v>123</v>
-      </c>
-      <c r="D44" t="inlineStr">
-        <is>
-          <t>KRW</t>
-        </is>
-      </c>
-      <c r="E44" t="n">
-        <v>1</v>
-      </c>
-      <c r="F44" t="n">
-        <v>8070101.805898919</v>
-      </c>
-      <c r="G44" t="n">
-        <v>1619750.805898919</v>
-      </c>
-      <c r="H44" t="n">
-        <v>25.11104908707943</v>
-      </c>
-      <c r="I44" t="inlineStr">
-        <is>
-          <t>2026-03-21T04:51:20</t>
-        </is>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" t="inlineStr">
-        <is>
-          <t>2026-03-21</t>
-        </is>
-      </c>
-      <c r="B45" t="inlineStr">
-        <is>
-          <t>세아제강</t>
-        </is>
-      </c>
-      <c r="C45" t="n">
-        <v>50</v>
-      </c>
-      <c r="D45" t="inlineStr">
-        <is>
-          <t>KRW</t>
-        </is>
-      </c>
-      <c r="E45" t="n">
-        <v>1</v>
-      </c>
-      <c r="F45" t="n">
-        <v>7395000</v>
-      </c>
-      <c r="G45" t="n">
-        <v>1085000</v>
-      </c>
-      <c r="H45" t="n">
-        <v>17.19492868462758</v>
-      </c>
-      <c r="I45" t="inlineStr">
-        <is>
-          <t>2026-03-21T04:51:20</t>
-        </is>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" t="inlineStr">
-        <is>
-          <t>2026-03-21</t>
-        </is>
-      </c>
-      <c r="B46" t="inlineStr">
-        <is>
-          <t>센트러스 에너지</t>
-        </is>
-      </c>
-      <c r="C46" t="n">
-        <v>25</v>
-      </c>
-      <c r="D46" t="inlineStr">
-        <is>
-          <t>KRW</t>
-        </is>
-      </c>
-      <c r="E46" t="n">
-        <v>1</v>
-      </c>
-      <c r="F46" t="n">
-        <v>7026050.85816239</v>
-      </c>
-      <c r="G46" t="n">
-        <v>-406805.1418376099</v>
-      </c>
-      <c r="H46" t="n">
-        <v>-5.473066366920198</v>
-      </c>
-      <c r="I46" t="inlineStr">
-        <is>
-          <t>2026-03-21T04:51:20</t>
-        </is>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" t="inlineStr">
-        <is>
-          <t>2026-03-21</t>
-        </is>
-      </c>
-      <c r="B47" t="inlineStr">
-        <is>
-          <t>트랜스오션</t>
-        </is>
-      </c>
-      <c r="C47" t="n">
-        <v>750</v>
-      </c>
-      <c r="D47" t="inlineStr">
-        <is>
-          <t>KRW</t>
-        </is>
-      </c>
-      <c r="E47" t="n">
-        <v>1</v>
-      </c>
-      <c r="F47" t="n">
-        <v>7020031.5082007</v>
-      </c>
-      <c r="G47" t="n">
-        <v>2892797.5082007</v>
-      </c>
-      <c r="H47" t="n">
-        <v>70.09046514446965</v>
-      </c>
-      <c r="I47" t="inlineStr">
-        <is>
-          <t>2026-03-21T04:51:20</t>
-        </is>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" t="inlineStr">
-        <is>
-          <t>2026-03-21</t>
-        </is>
-      </c>
-      <c r="B48" t="inlineStr">
-        <is>
-          <t>DL이앤씨</t>
-        </is>
-      </c>
-      <c r="C48" t="n">
-        <v>80</v>
-      </c>
-      <c r="D48" t="inlineStr">
-        <is>
-          <t>KRW</t>
-        </is>
-      </c>
-      <c r="E48" t="n">
-        <v>1</v>
-      </c>
-      <c r="F48" t="n">
-        <v>5392000</v>
-      </c>
-      <c r="G48" t="n">
-        <v>1981000</v>
-      </c>
-      <c r="H48" t="n">
-        <v>58.07681031955438</v>
-      </c>
-      <c r="I48" t="inlineStr">
-        <is>
-          <t>2026-03-21T04:51:20</t>
-        </is>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" t="inlineStr">
-        <is>
-          <t>2026-03-21</t>
-        </is>
-      </c>
-      <c r="B49" t="inlineStr">
-        <is>
-          <t>타이드워터</t>
-        </is>
-      </c>
-      <c r="C49" t="n">
-        <v>48</v>
-      </c>
-      <c r="D49" t="inlineStr">
-        <is>
-          <t>KRW</t>
-        </is>
-      </c>
-      <c r="E49" t="n">
-        <v>1</v>
-      </c>
-      <c r="F49" t="n">
-        <v>5235363.852789983</v>
-      </c>
-      <c r="G49" t="n">
-        <v>1510818.852789983</v>
-      </c>
-      <c r="H49" t="n">
-        <v>40.56385015592463</v>
-      </c>
-      <c r="I49" t="inlineStr">
-        <is>
-          <t>2026-03-21T04:51:20</t>
-        </is>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" t="inlineStr">
-        <is>
-          <t>2026-03-21</t>
-        </is>
-      </c>
-      <c r="B50" t="inlineStr">
-        <is>
-          <t>노브</t>
-        </is>
-      </c>
-      <c r="C50" t="n">
-        <v>185</v>
-      </c>
-      <c r="D50" t="inlineStr">
-        <is>
-          <t>KRW</t>
-        </is>
-      </c>
-      <c r="E50" t="n">
-        <v>1</v>
-      </c>
-      <c r="F50" t="n">
-        <v>5200391.447092756</v>
-      </c>
-      <c r="G50" t="n">
-        <v>1890383.447092756</v>
-      </c>
-      <c r="H50" t="n">
-        <v>57.11114435653194</v>
-      </c>
-      <c r="I50" t="inlineStr">
-        <is>
-          <t>2026-03-21T04:51:20</t>
-        </is>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" t="inlineStr">
-        <is>
-          <t>2026-03-21</t>
-        </is>
-      </c>
-      <c r="B51" t="inlineStr">
-        <is>
-          <t>TIME 코리아밸류업액티브</t>
-        </is>
-      </c>
-      <c r="C51" t="n">
-        <v>201</v>
-      </c>
-      <c r="D51" t="inlineStr">
-        <is>
-          <t>KRW</t>
-        </is>
-      </c>
-      <c r="E51" t="n">
-        <v>1</v>
-      </c>
-      <c r="F51" t="n">
-        <v>4797870</v>
-      </c>
-      <c r="G51" t="n">
-        <v>74073</v>
-      </c>
-      <c r="H51" t="n">
-        <v>1.568081778281328</v>
-      </c>
-      <c r="I51" t="inlineStr">
-        <is>
-          <t>2026-03-21T04:51:20</t>
-        </is>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" t="inlineStr">
-        <is>
-          <t>2026-03-21</t>
-        </is>
-      </c>
-      <c r="B52" t="inlineStr">
-        <is>
-          <t>오케아니스 에코 탱커스</t>
-        </is>
-      </c>
-      <c r="C52" t="n">
-        <v>65</v>
-      </c>
-      <c r="D52" t="inlineStr">
-        <is>
-          <t>KRW</t>
-        </is>
-      </c>
-      <c r="E52" t="n">
-        <v>1</v>
-      </c>
-      <c r="F52" t="n">
-        <v>4511179.137784176</v>
-      </c>
-      <c r="G52" t="n">
-        <v>2254819.137784176</v>
-      </c>
-      <c r="H52" t="n">
-        <v>99.93171026716374</v>
-      </c>
-      <c r="I52" t="inlineStr">
-        <is>
-          <t>2026-03-21T04:51:20</t>
-        </is>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" t="inlineStr">
-        <is>
-          <t>2026-03-21</t>
-        </is>
-      </c>
-      <c r="B53" t="inlineStr">
-        <is>
-          <t>동원개발</t>
-        </is>
-      </c>
-      <c r="C53" t="n">
-        <v>1360</v>
-      </c>
-      <c r="D53" t="inlineStr">
-        <is>
-          <t>KRW</t>
-        </is>
-      </c>
-      <c r="E53" t="n">
-        <v>1</v>
-      </c>
-      <c r="F53" t="n">
-        <v>4202400</v>
-      </c>
-      <c r="G53" t="n">
-        <v>465000</v>
-      </c>
-      <c r="H53" t="n">
-        <v>12.44180446299566</v>
-      </c>
-      <c r="I53" t="inlineStr">
-        <is>
-          <t>2026-03-21T04:51:20</t>
-        </is>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" t="inlineStr">
-        <is>
-          <t>2026-03-21</t>
-        </is>
-      </c>
-      <c r="B54" t="inlineStr">
-        <is>
-          <t>HD건설기계</t>
-        </is>
-      </c>
-      <c r="C54" t="n">
-        <v>31</v>
-      </c>
-      <c r="D54" t="inlineStr">
-        <is>
-          <t>KRW</t>
-        </is>
-      </c>
-      <c r="E54" t="n">
-        <v>1</v>
-      </c>
-      <c r="F54" t="n">
-        <v>4123000</v>
-      </c>
-      <c r="G54" t="n">
-        <v>87904</v>
-      </c>
-      <c r="H54" t="n">
-        <v>2.178485964150543</v>
-      </c>
-      <c r="I54" t="inlineStr">
-        <is>
-          <t>2026-03-21T04:51:20</t>
-        </is>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" t="inlineStr">
-        <is>
-          <t>2026-03-21</t>
-        </is>
-      </c>
-      <c r="B55" t="inlineStr">
-        <is>
-          <t>차코스 에너지 내비게이션</t>
-        </is>
-      </c>
-      <c r="C55" t="n">
-        <v>75</v>
-      </c>
-      <c r="D55" t="inlineStr">
-        <is>
-          <t>KRW</t>
-        </is>
-      </c>
-      <c r="E55" t="n">
-        <v>1</v>
-      </c>
-      <c r="F55" t="n">
-        <v>4026924.996845168</v>
-      </c>
-      <c r="G55" t="n">
-        <v>202276.9968451681</v>
-      </c>
-      <c r="H55" t="n">
-        <v>5.28877420471552</v>
-      </c>
-      <c r="I55" t="inlineStr">
-        <is>
-          <t>2026-03-21T04:51:20</t>
-        </is>
-      </c>
-    </row>
-    <row r="56">
-      <c r="A56" t="inlineStr">
-        <is>
-          <t>2026-03-21</t>
-        </is>
-      </c>
-      <c r="B56" t="inlineStr">
-        <is>
-          <t>피바디 에너지</t>
-        </is>
-      </c>
-      <c r="C56" t="n">
-        <v>65</v>
-      </c>
-      <c r="D56" t="inlineStr">
-        <is>
-          <t>KRW</t>
-        </is>
-      </c>
-      <c r="E56" t="n">
-        <v>1</v>
-      </c>
-      <c r="F56" t="n">
-        <v>3649438.50225304</v>
-      </c>
-      <c r="G56" t="n">
-        <v>2178666.50225304</v>
-      </c>
-      <c r="H56" t="n">
-        <v>148.1308117269733</v>
-      </c>
-      <c r="I56" t="inlineStr">
-        <is>
-          <t>2026-03-21T04:51:20</t>
-        </is>
-      </c>
-    </row>
-    <row r="57">
-      <c r="A57" t="inlineStr">
-        <is>
-          <t>2026-03-21</t>
-        </is>
-      </c>
-      <c r="B57" t="inlineStr">
-        <is>
-          <t>삼성화재</t>
-        </is>
-      </c>
-      <c r="C57" t="n">
-        <v>7</v>
-      </c>
-      <c r="D57" t="inlineStr">
-        <is>
-          <t>KRW</t>
-        </is>
-      </c>
-      <c r="E57" t="n">
-        <v>1</v>
-      </c>
-      <c r="F57" t="n">
-        <v>3321500</v>
-      </c>
-      <c r="G57" t="n">
-        <v>-309500</v>
-      </c>
-      <c r="H57" t="n">
-        <v>-8.523822638391627</v>
-      </c>
-      <c r="I57" t="inlineStr">
-        <is>
-          <t>2026-03-21T04:51:20</t>
-        </is>
-      </c>
-    </row>
-    <row r="58">
-      <c r="A58" t="inlineStr">
-        <is>
-          <t>2026-03-21</t>
-        </is>
-      </c>
-      <c r="B58" t="inlineStr">
-        <is>
-          <t>더치 브로스</t>
-        </is>
-      </c>
-      <c r="C58" t="n">
-        <v>39</v>
-      </c>
-      <c r="D58" t="inlineStr">
-        <is>
-          <t>KRW</t>
-        </is>
-      </c>
-      <c r="E58" t="n">
-        <v>1</v>
-      </c>
-      <c r="F58" t="n">
-        <v>2934418.414306641</v>
-      </c>
-      <c r="G58" t="n">
-        <v>-256225.5856933598</v>
-      </c>
-      <c r="H58" t="n">
-        <v>-8.030528811530205</v>
-      </c>
-      <c r="I58" t="inlineStr">
-        <is>
-          <t>2026-03-21T04:51:20</t>
-        </is>
-      </c>
-    </row>
-    <row r="59">
-      <c r="A59" t="inlineStr">
-        <is>
-          <t>2026-03-21</t>
-        </is>
-      </c>
-      <c r="B59" t="inlineStr">
-        <is>
-          <t>휴스틸</t>
-        </is>
-      </c>
-      <c r="C59" t="n">
-        <v>500</v>
-      </c>
-      <c r="D59" t="inlineStr">
-        <is>
-          <t>KRW</t>
-        </is>
-      </c>
-      <c r="E59" t="n">
-        <v>1</v>
-      </c>
-      <c r="F59" t="n">
-        <v>2750000</v>
-      </c>
-      <c r="G59" t="n">
-        <v>471390</v>
-      </c>
-      <c r="H59" t="n">
-        <v>20.68761218462133</v>
-      </c>
-      <c r="I59" t="inlineStr">
-        <is>
-          <t>2026-03-21T04:51:20</t>
-        </is>
-      </c>
-    </row>
-    <row r="60">
-      <c r="A60" t="inlineStr">
-        <is>
-          <t>2026-03-21</t>
-        </is>
-      </c>
-      <c r="B60" t="inlineStr">
-        <is>
-          <t>현대제철</t>
-        </is>
-      </c>
-      <c r="C60" t="n">
-        <v>70</v>
-      </c>
-      <c r="D60" t="inlineStr">
-        <is>
-          <t>KRW</t>
-        </is>
-      </c>
-      <c r="E60" t="n">
-        <v>1</v>
-      </c>
-      <c r="F60" t="n">
-        <v>2621500</v>
-      </c>
-      <c r="G60" t="n">
-        <v>-186000</v>
-      </c>
-      <c r="H60" t="n">
-        <v>-6.625111308993767</v>
-      </c>
-      <c r="I60" t="inlineStr">
-        <is>
-          <t>2026-03-21T04:51:20</t>
-        </is>
-      </c>
-    </row>
-    <row r="61">
-      <c r="A61" t="inlineStr">
-        <is>
-          <t>2026-03-21</t>
-        </is>
-      </c>
-      <c r="B61" t="inlineStr">
-        <is>
-          <t>KoAct 코스닥액티브</t>
-        </is>
-      </c>
-      <c r="C61" t="n">
-        <v>200</v>
-      </c>
-      <c r="D61" t="inlineStr">
-        <is>
-          <t>KRW</t>
-        </is>
-      </c>
-      <c r="E61" t="n">
-        <v>1</v>
-      </c>
-      <c r="F61" t="n">
-        <v>2582000</v>
-      </c>
-      <c r="G61" t="n">
-        <v>-120000</v>
-      </c>
-      <c r="H61" t="n">
-        <v>-4.441154700222058</v>
-      </c>
-      <c r="I61" t="inlineStr">
-        <is>
-          <t>2026-03-21T04:51:20</t>
-        </is>
-      </c>
-    </row>
-    <row r="62">
-      <c r="A62" t="inlineStr">
-        <is>
-          <t>2026-03-21</t>
-        </is>
-      </c>
-      <c r="B62" t="inlineStr">
-        <is>
-          <t>넥스틸</t>
-        </is>
-      </c>
-      <c r="C62" t="n">
-        <v>200</v>
-      </c>
-      <c r="D62" t="inlineStr">
-        <is>
-          <t>KRW</t>
-        </is>
-      </c>
-      <c r="E62" t="n">
-        <v>1</v>
-      </c>
-      <c r="F62" t="n">
-        <v>2514000</v>
-      </c>
-      <c r="G62" t="n">
-        <v>503000</v>
-      </c>
-      <c r="H62" t="n">
-        <v>25.01243162605669</v>
-      </c>
-      <c r="I62" t="inlineStr">
-        <is>
-          <t>2026-03-21T04:51:20</t>
-        </is>
-      </c>
-    </row>
-    <row r="63">
-      <c r="A63" t="inlineStr">
-        <is>
-          <t>2026-03-21</t>
-        </is>
-      </c>
-      <c r="B63" t="inlineStr">
-        <is>
-          <t>대신증권</t>
-        </is>
-      </c>
-      <c r="C63" t="n">
-        <v>55</v>
-      </c>
-      <c r="D63" t="inlineStr">
-        <is>
-          <t>KRW</t>
-        </is>
-      </c>
-      <c r="E63" t="n">
-        <v>1</v>
-      </c>
-      <c r="F63" t="n">
-        <v>2219250</v>
-      </c>
-      <c r="G63" t="n">
-        <v>509749</v>
-      </c>
-      <c r="H63" t="n">
-        <v>29.81858448752005</v>
-      </c>
-      <c r="I63" t="inlineStr">
-        <is>
-          <t>2026-03-21T04:51:20</t>
-        </is>
-      </c>
-    </row>
-    <row r="64">
-      <c r="A64" t="inlineStr">
-        <is>
-          <t>2026-03-21</t>
-        </is>
-      </c>
-      <c r="B64" t="inlineStr">
-        <is>
-          <t>발레로 에너지</t>
-        </is>
-      </c>
-      <c r="C64" t="n">
-        <v>6</v>
-      </c>
-      <c r="D64" t="inlineStr">
-        <is>
-          <t>KRW</t>
-        </is>
-      </c>
-      <c r="E64" t="n">
-        <v>1</v>
-      </c>
-      <c r="F64" t="n">
-        <v>2165691.085066516</v>
-      </c>
-      <c r="G64" t="n">
-        <v>101701.085066516</v>
-      </c>
-      <c r="H64" t="n">
-        <v>4.927402025519307</v>
-      </c>
-      <c r="I64" t="inlineStr">
-        <is>
-          <t>2026-03-21T04:51:20</t>
-        </is>
-      </c>
-    </row>
-    <row r="65">
-      <c r="A65" t="inlineStr">
-        <is>
-          <t>2026-03-21</t>
-        </is>
-      </c>
-      <c r="B65" t="inlineStr">
-        <is>
-          <t>미창석유</t>
-        </is>
-      </c>
-      <c r="C65" t="n">
-        <v>18</v>
-      </c>
-      <c r="D65" t="inlineStr">
-        <is>
-          <t>KRW</t>
-        </is>
-      </c>
-      <c r="E65" t="n">
-        <v>1</v>
-      </c>
-      <c r="F65" t="n">
-        <v>2097000</v>
-      </c>
-      <c r="G65" t="n">
-        <v>-295200</v>
-      </c>
-      <c r="H65" t="n">
-        <v>-12.34010534236268</v>
-      </c>
-      <c r="I65" t="inlineStr">
-        <is>
-          <t>2026-03-21T04:51:20</t>
-        </is>
-      </c>
-    </row>
-    <row r="66">
-      <c r="A66" t="inlineStr">
-        <is>
-          <t>2026-03-21</t>
-        </is>
-      </c>
-      <c r="B66" t="inlineStr">
-        <is>
-          <t>대창단조</t>
-        </is>
-      </c>
-      <c r="C66" t="n">
-        <v>300</v>
-      </c>
-      <c r="D66" t="inlineStr">
-        <is>
-          <t>KRW</t>
-        </is>
-      </c>
-      <c r="E66" t="n">
-        <v>1</v>
-      </c>
-      <c r="F66" t="n">
-        <v>2004000</v>
-      </c>
-      <c r="G66" t="n">
-        <v>-54000</v>
-      </c>
-      <c r="H66" t="n">
-        <v>-2.623906705539359</v>
-      </c>
-      <c r="I66" t="inlineStr">
-        <is>
-          <t>2026-03-21T04:51:20</t>
-        </is>
-      </c>
-    </row>
-    <row r="67">
-      <c r="A67" t="inlineStr">
-        <is>
-          <t>2026-03-21</t>
-        </is>
-      </c>
-      <c r="B67" t="inlineStr">
-        <is>
-          <t>동방</t>
-        </is>
-      </c>
-      <c r="C67" t="n">
-        <v>681</v>
-      </c>
-      <c r="D67" t="inlineStr">
-        <is>
-          <t>KRW</t>
-        </is>
-      </c>
-      <c r="E67" t="n">
-        <v>1</v>
-      </c>
-      <c r="F67" t="n">
-        <v>1995330</v>
-      </c>
-      <c r="G67" t="n">
-        <v>23829</v>
-      </c>
-      <c r="H67" t="n">
-        <v>1.208672985709873</v>
-      </c>
-      <c r="I67" t="inlineStr">
-        <is>
-          <t>2026-03-21T04:51:20</t>
-        </is>
-      </c>
-    </row>
-    <row r="68">
-      <c r="A68" t="inlineStr">
-        <is>
-          <t>2026-03-21</t>
-        </is>
-      </c>
-      <c r="B68" t="inlineStr">
-        <is>
-          <t>스타 벌크 캐리어스</t>
-        </is>
-      </c>
-      <c r="C68" t="n">
-        <v>50</v>
-      </c>
-      <c r="D68" t="inlineStr">
-        <is>
-          <t>KRW</t>
-        </is>
-      </c>
-      <c r="E68" t="n">
-        <v>1</v>
-      </c>
-      <c r="F68" t="n">
-        <v>1680142.640194588</v>
-      </c>
-      <c r="G68" t="n">
-        <v>365789.6401945879</v>
-      </c>
-      <c r="H68" t="n">
-        <v>27.83039565433242</v>
-      </c>
-      <c r="I68" t="inlineStr">
-        <is>
-          <t>2026-03-21T04:51:20</t>
-        </is>
-      </c>
-    </row>
-    <row r="69">
-      <c r="A69" t="inlineStr">
-        <is>
-          <t>2026-03-21</t>
-        </is>
-      </c>
-      <c r="B69" t="inlineStr">
-        <is>
-          <t>케이씨</t>
-        </is>
-      </c>
-      <c r="C69" t="n">
-        <v>50</v>
-      </c>
-      <c r="D69" t="inlineStr">
-        <is>
-          <t>KRW</t>
-        </is>
-      </c>
-      <c r="E69" t="n">
-        <v>1</v>
-      </c>
-      <c r="F69" t="n">
-        <v>1670000</v>
-      </c>
-      <c r="G69" t="n">
-        <v>20500</v>
-      </c>
-      <c r="H69" t="n">
-        <v>1.242800848742043</v>
-      </c>
-      <c r="I69" t="inlineStr">
-        <is>
-          <t>2026-03-21T04:51:20</t>
-        </is>
-      </c>
-    </row>
-    <row r="70">
-      <c r="A70" t="inlineStr">
-        <is>
-          <t>2026-03-21</t>
-        </is>
-      </c>
-      <c r="B70" t="inlineStr">
-        <is>
-          <t>유나이티드헬스 그룹</t>
-        </is>
-      </c>
-      <c r="C70" t="n">
-        <v>4</v>
-      </c>
-      <c r="D70" t="inlineStr">
-        <is>
-          <t>KRW</t>
-        </is>
-      </c>
-      <c r="E70" t="n">
-        <v>1</v>
-      </c>
-      <c r="F70" t="n">
-        <v>1658864.328313038</v>
-      </c>
-      <c r="G70" t="n">
-        <v>-35591.67168696248</v>
-      </c>
-      <c r="H70" t="n">
-        <v>-2.100477774988697</v>
-      </c>
-      <c r="I70" t="inlineStr">
-        <is>
-          <t>2026-03-21T04:51:20</t>
-        </is>
-      </c>
-    </row>
-    <row r="71">
-      <c r="A71" t="inlineStr">
-        <is>
-          <t>2026-03-21</t>
-        </is>
-      </c>
-      <c r="B71" t="inlineStr">
-        <is>
-          <t>텍사스 퍼시픽 랜드</t>
-        </is>
-      </c>
-      <c r="C71" t="n">
-        <v>2</v>
-      </c>
-      <c r="D71" t="inlineStr">
-        <is>
-          <t>KRW</t>
-        </is>
-      </c>
-      <c r="E71" t="n">
-        <v>1</v>
-      </c>
-      <c r="F71" t="n">
-        <v>1563247.374122903</v>
-      </c>
-      <c r="G71" t="n">
-        <v>-14646.62587709725</v>
-      </c>
-      <c r="H71" t="n">
-        <v>-0.9282388979929735</v>
-      </c>
-      <c r="I71" t="inlineStr">
-        <is>
-          <t>2026-03-21T04:51:20</t>
-        </is>
-      </c>
-    </row>
-    <row r="72">
-      <c r="A72" t="inlineStr">
-        <is>
-          <t>2026-03-21</t>
-        </is>
-      </c>
-      <c r="B72" t="inlineStr">
-        <is>
-          <t>하나금융지주</t>
-        </is>
-      </c>
-      <c r="C72" t="n">
-        <v>10</v>
-      </c>
-      <c r="D72" t="inlineStr">
-        <is>
-          <t>KRW</t>
-        </is>
-      </c>
-      <c r="E72" t="n">
-        <v>1</v>
-      </c>
-      <c r="F72" t="n">
-        <v>1132000</v>
-      </c>
-      <c r="G72" t="n">
-        <v>23000</v>
-      </c>
-      <c r="H72" t="n">
-        <v>2.073940486925157</v>
-      </c>
-      <c r="I72" t="inlineStr">
-        <is>
-          <t>2026-03-21T04:51:20</t>
-        </is>
-      </c>
-    </row>
-    <row r="73">
-      <c r="A73" t="inlineStr">
-        <is>
-          <t>2026-03-21</t>
-        </is>
-      </c>
-      <c r="B73" t="inlineStr">
-        <is>
-          <t>삼성생명</t>
-        </is>
-      </c>
-      <c r="C73" t="n">
-        <v>4</v>
-      </c>
-      <c r="D73" t="inlineStr">
-        <is>
-          <t>KRW</t>
-        </is>
-      </c>
-      <c r="E73" t="n">
-        <v>1</v>
-      </c>
-      <c r="F73" t="n">
-        <v>926000</v>
-      </c>
-      <c r="G73" t="n">
-        <v>93000</v>
-      </c>
-      <c r="H73" t="n">
-        <v>11.16446578631453</v>
-      </c>
-      <c r="I73" t="inlineStr">
-        <is>
-          <t>2026-03-21T04:51:20</t>
-        </is>
-      </c>
-    </row>
-    <row r="74">
-      <c r="A74" t="inlineStr">
-        <is>
-          <t>2026-03-21</t>
-        </is>
-      </c>
-      <c r="B74" t="inlineStr">
-        <is>
-          <t>비에이치아이</t>
-        </is>
-      </c>
-      <c r="C74" t="n">
-        <v>8</v>
-      </c>
-      <c r="D74" t="inlineStr">
-        <is>
-          <t>KRW</t>
-        </is>
-      </c>
-      <c r="E74" t="n">
-        <v>1</v>
-      </c>
-      <c r="F74" t="n">
-        <v>876000</v>
-      </c>
-      <c r="G74" t="n">
-        <v>210885</v>
-      </c>
-      <c r="H74" t="n">
-        <v>31.70654698811484</v>
-      </c>
-      <c r="I74" t="inlineStr">
-        <is>
-          <t>2026-03-21T04:51:20</t>
-        </is>
-      </c>
-    </row>
-    <row r="75">
-      <c r="A75" t="inlineStr">
-        <is>
-          <t>2026-03-21</t>
-        </is>
-      </c>
-      <c r="B75" t="inlineStr">
-        <is>
-          <t>하프니아</t>
-        </is>
-      </c>
-      <c r="C75" t="n">
-        <v>80</v>
-      </c>
-      <c r="D75" t="inlineStr">
-        <is>
-          <t>KRW</t>
-        </is>
-      </c>
-      <c r="E75" t="n">
-        <v>1</v>
-      </c>
-      <c r="F75" t="n">
-        <v>842704.775390625</v>
-      </c>
-      <c r="G75" t="n">
-        <v>216973.775390625</v>
-      </c>
-      <c r="H75" t="n">
-        <v>34.67524789256486</v>
-      </c>
-      <c r="I75" t="inlineStr">
-        <is>
-          <t>2026-03-21T04:51:20</t>
-        </is>
-      </c>
-    </row>
-    <row r="76">
-      <c r="A76" t="inlineStr">
-        <is>
-          <t>2026-03-21</t>
-        </is>
-      </c>
-      <c r="B76" t="inlineStr">
-        <is>
-          <t>클리블랜드 클리프스</t>
-        </is>
-      </c>
-      <c r="C76" t="n">
-        <v>70</v>
-      </c>
-      <c r="D76" t="inlineStr">
-        <is>
-          <t>KRW</t>
-        </is>
-      </c>
-      <c r="E76" t="n">
-        <v>1</v>
-      </c>
-      <c r="F76" t="n">
-        <v>823743.9360268187</v>
-      </c>
-      <c r="G76" t="n">
-        <v>-192311.0639731813</v>
-      </c>
-      <c r="H76" t="n">
-        <v>-18.92722972409774</v>
-      </c>
-      <c r="I76" t="inlineStr">
-        <is>
-          <t>2026-03-21T04:51:20</t>
-        </is>
-      </c>
-    </row>
-    <row r="77">
-      <c r="A77" t="inlineStr">
-        <is>
-          <t>2026-03-21</t>
-        </is>
-      </c>
-      <c r="B77" t="inlineStr">
-        <is>
-          <t>노블</t>
-        </is>
-      </c>
-      <c r="C77" t="n">
-        <v>99</v>
-      </c>
-      <c r="D77" t="inlineStr">
-        <is>
-          <t>KRW</t>
-        </is>
-      </c>
-      <c r="E77" t="n">
-        <v>1</v>
-      </c>
-      <c r="F77" t="n">
-        <v>40689</v>
-      </c>
-      <c r="G77" t="n">
-        <v>-3866519</v>
-      </c>
-      <c r="H77" t="n">
-        <v>-98.95861699709869</v>
-      </c>
-      <c r="I77" t="inlineStr">
-        <is>
-          <t>2026-03-21T04:51:20</t>
         </is>
       </c>
     </row>
@@ -4440,7 +3034,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E3"/>
+  <dimension ref="A1:E2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4493,29 +3087,6 @@
         </is>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>2026-03-21</t>
-        </is>
-      </c>
-      <c r="B3" t="n">
-        <v>31036676</v>
-      </c>
-      <c r="C3" t="n">
-        <v>6052.96</v>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>2026-03-21T03:07:34</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>2026-03-21T04:51:20</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
auto: portfolio snapshot 2026-03-21 (2026-03-21T04:52:57)
</commit_message>
<xml_diff>
--- a/portfolio_auto.xlsx
+++ b/portfolio_auto.xlsx
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G1"/>
+  <dimension ref="A1:G39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -466,6 +466,1032 @@
         <is>
           <t>수익률(%)</t>
         </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>노브</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>185</v>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E2" t="n">
+        <v>5200391.447092756</v>
+      </c>
+      <c r="F2" t="n">
+        <v>1890383.447092756</v>
+      </c>
+      <c r="G2" t="n">
+        <v>57.11114435653194</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>노블</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>99</v>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E3" t="n">
+        <v>40689</v>
+      </c>
+      <c r="F3" t="n">
+        <v>-3866519</v>
+      </c>
+      <c r="G3" t="n">
+        <v>-98.95861699709869</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>더치 브로스</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>39</v>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>1</v>
+      </c>
+      <c r="E4" t="n">
+        <v>2934418.414306641</v>
+      </c>
+      <c r="F4" t="n">
+        <v>-256225.5856933598</v>
+      </c>
+      <c r="G4" t="n">
+        <v>-8.030528811530205</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>발레로 에너지</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>6</v>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>1</v>
+      </c>
+      <c r="E5" t="n">
+        <v>2165691.085066516</v>
+      </c>
+      <c r="F5" t="n">
+        <v>101701.085066516</v>
+      </c>
+      <c r="G5" t="n">
+        <v>4.927402025519307</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>유나이티드헬스 그룹</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>4</v>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>1</v>
+      </c>
+      <c r="E6" t="n">
+        <v>1658864.328313038</v>
+      </c>
+      <c r="F6" t="n">
+        <v>-35591.67168696248</v>
+      </c>
+      <c r="G6" t="n">
+        <v>-2.100477774988697</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>AGNC 인베스트먼트</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>700</v>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>1</v>
+      </c>
+      <c r="E7" t="n">
+        <v>10270464.45007324</v>
+      </c>
+      <c r="F7" t="n">
+        <v>-561550.5499267559</v>
+      </c>
+      <c r="G7" t="n">
+        <v>-5.184174411933109</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>넥스틸</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>200</v>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>1</v>
+      </c>
+      <c r="E8" t="n">
+        <v>2514000</v>
+      </c>
+      <c r="F8" t="n">
+        <v>503000</v>
+      </c>
+      <c r="G8" t="n">
+        <v>25.01243162605669</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>대신증권</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>55</v>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>1</v>
+      </c>
+      <c r="E9" t="n">
+        <v>2219250</v>
+      </c>
+      <c r="F9" t="n">
+        <v>509749</v>
+      </c>
+      <c r="G9" t="n">
+        <v>29.81858448752005</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>대창단조</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>300</v>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>1</v>
+      </c>
+      <c r="E10" t="n">
+        <v>2004000</v>
+      </c>
+      <c r="F10" t="n">
+        <v>-54000</v>
+      </c>
+      <c r="G10" t="n">
+        <v>-2.623906705539359</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>대한조선</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>100</v>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>1</v>
+      </c>
+      <c r="E11" t="n">
+        <v>9120000</v>
+      </c>
+      <c r="F11" t="n">
+        <v>1907000</v>
+      </c>
+      <c r="G11" t="n">
+        <v>26.43837515596839</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>동방</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>681</v>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>1</v>
+      </c>
+      <c r="E12" t="n">
+        <v>1995330</v>
+      </c>
+      <c r="F12" t="n">
+        <v>23829</v>
+      </c>
+      <c r="G12" t="n">
+        <v>1.208672985709873</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>동원개발</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>1360</v>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>1</v>
+      </c>
+      <c r="E13" t="n">
+        <v>4202400</v>
+      </c>
+      <c r="F13" t="n">
+        <v>465000</v>
+      </c>
+      <c r="G13" t="n">
+        <v>12.44180446299566</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>미창석유</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>18</v>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>1</v>
+      </c>
+      <c r="E14" t="n">
+        <v>2097000</v>
+      </c>
+      <c r="F14" t="n">
+        <v>-295200</v>
+      </c>
+      <c r="G14" t="n">
+        <v>-12.34010534236268</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>비에이치아이</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>8</v>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>1</v>
+      </c>
+      <c r="E15" t="n">
+        <v>876000</v>
+      </c>
+      <c r="F15" t="n">
+        <v>210885</v>
+      </c>
+      <c r="G15" t="n">
+        <v>31.70654698811484</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>삼성생명</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>4</v>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>1</v>
+      </c>
+      <c r="E16" t="n">
+        <v>926000</v>
+      </c>
+      <c r="F16" t="n">
+        <v>93000</v>
+      </c>
+      <c r="G16" t="n">
+        <v>11.16446578631453</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>삼성화재</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>7</v>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>1</v>
+      </c>
+      <c r="E17" t="n">
+        <v>3321500</v>
+      </c>
+      <c r="F17" t="n">
+        <v>-309500</v>
+      </c>
+      <c r="G17" t="n">
+        <v>-8.523822638391627</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>세아제강</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>50</v>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>1</v>
+      </c>
+      <c r="E18" t="n">
+        <v>7395000</v>
+      </c>
+      <c r="F18" t="n">
+        <v>1085000</v>
+      </c>
+      <c r="G18" t="n">
+        <v>17.19492868462758</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>케이씨</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>50</v>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
+        <v>1</v>
+      </c>
+      <c r="E19" t="n">
+        <v>1670000</v>
+      </c>
+      <c r="F19" t="n">
+        <v>20500</v>
+      </c>
+      <c r="G19" t="n">
+        <v>1.242800848742043</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>하나금융지주</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>10</v>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="D20" t="n">
+        <v>1</v>
+      </c>
+      <c r="E20" t="n">
+        <v>1132000</v>
+      </c>
+      <c r="F20" t="n">
+        <v>23000</v>
+      </c>
+      <c r="G20" t="n">
+        <v>2.073940486925157</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>현대제철</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>70</v>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
+        <v>1</v>
+      </c>
+      <c r="E21" t="n">
+        <v>2621500</v>
+      </c>
+      <c r="F21" t="n">
+        <v>-186000</v>
+      </c>
+      <c r="G21" t="n">
+        <v>-6.625111308993767</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>휴스틸</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>500</v>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="D22" t="n">
+        <v>1</v>
+      </c>
+      <c r="E22" t="n">
+        <v>2750000</v>
+      </c>
+      <c r="F22" t="n">
+        <v>471390</v>
+      </c>
+      <c r="G22" t="n">
+        <v>20.68761218462133</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>DL이앤씨</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>80</v>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="D23" t="n">
+        <v>1</v>
+      </c>
+      <c r="E23" t="n">
+        <v>5392000</v>
+      </c>
+      <c r="F23" t="n">
+        <v>1981000</v>
+      </c>
+      <c r="G23" t="n">
+        <v>58.07681031955438</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>HD건설기계</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>31</v>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="D24" t="n">
+        <v>1</v>
+      </c>
+      <c r="E24" t="n">
+        <v>4123000</v>
+      </c>
+      <c r="F24" t="n">
+        <v>87904</v>
+      </c>
+      <c r="G24" t="n">
+        <v>2.178485964150543</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>KoAct 코스닥액티브</t>
+        </is>
+      </c>
+      <c r="B25" t="n">
+        <v>200</v>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="D25" t="n">
+        <v>1</v>
+      </c>
+      <c r="E25" t="n">
+        <v>2582000</v>
+      </c>
+      <c r="F25" t="n">
+        <v>-120000</v>
+      </c>
+      <c r="G25" t="n">
+        <v>-4.441154700222058</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>TIME 코리아밸류업액티브</t>
+        </is>
+      </c>
+      <c r="B26" t="n">
+        <v>201</v>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="D26" t="n">
+        <v>1</v>
+      </c>
+      <c r="E26" t="n">
+        <v>4797870</v>
+      </c>
+      <c r="F26" t="n">
+        <v>74073</v>
+      </c>
+      <c r="G26" t="n">
+        <v>1.568081778281328</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>센트러스 에너지</t>
+        </is>
+      </c>
+      <c r="B27" t="n">
+        <v>25</v>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="D27" t="n">
+        <v>1</v>
+      </c>
+      <c r="E27" t="n">
+        <v>7026050.85816239</v>
+      </c>
+      <c r="F27" t="n">
+        <v>-406805.1418376099</v>
+      </c>
+      <c r="G27" t="n">
+        <v>-5.473066366920198</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>스타 벌크 캐리어스</t>
+        </is>
+      </c>
+      <c r="B28" t="n">
+        <v>50</v>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="D28" t="n">
+        <v>1</v>
+      </c>
+      <c r="E28" t="n">
+        <v>1680142.640194588</v>
+      </c>
+      <c r="F28" t="n">
+        <v>365789.6401945879</v>
+      </c>
+      <c r="G28" t="n">
+        <v>27.83039565433242</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>시드릴</t>
+        </is>
+      </c>
+      <c r="B29" t="n">
+        <v>123</v>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="D29" t="n">
+        <v>1</v>
+      </c>
+      <c r="E29" t="n">
+        <v>8070101.805898919</v>
+      </c>
+      <c r="F29" t="n">
+        <v>1619750.805898919</v>
+      </c>
+      <c r="G29" t="n">
+        <v>25.11104908707943</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>오케아니스 에코 탱커스</t>
+        </is>
+      </c>
+      <c r="B30" t="n">
+        <v>65</v>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="D30" t="n">
+        <v>1</v>
+      </c>
+      <c r="E30" t="n">
+        <v>4511179.137784176</v>
+      </c>
+      <c r="F30" t="n">
+        <v>2254819.137784176</v>
+      </c>
+      <c r="G30" t="n">
+        <v>99.93171026716374</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>차코스 에너지 내비게이션</t>
+        </is>
+      </c>
+      <c r="B31" t="n">
+        <v>75</v>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="D31" t="n">
+        <v>1</v>
+      </c>
+      <c r="E31" t="n">
+        <v>4026924.996845168</v>
+      </c>
+      <c r="F31" t="n">
+        <v>202276.9968451681</v>
+      </c>
+      <c r="G31" t="n">
+        <v>5.28877420471552</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>클리블랜드 클리프스</t>
+        </is>
+      </c>
+      <c r="B32" t="n">
+        <v>70</v>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="D32" t="n">
+        <v>1</v>
+      </c>
+      <c r="E32" t="n">
+        <v>823743.9360268187</v>
+      </c>
+      <c r="F32" t="n">
+        <v>-192311.0639731813</v>
+      </c>
+      <c r="G32" t="n">
+        <v>-18.92722972409774</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>타이드워터</t>
+        </is>
+      </c>
+      <c r="B33" t="n">
+        <v>48</v>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="D33" t="n">
+        <v>1</v>
+      </c>
+      <c r="E33" t="n">
+        <v>5235363.852789983</v>
+      </c>
+      <c r="F33" t="n">
+        <v>1510818.852789983</v>
+      </c>
+      <c r="G33" t="n">
+        <v>40.56385015592463</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>텍사스 퍼시픽 랜드</t>
+        </is>
+      </c>
+      <c r="B34" t="n">
+        <v>2</v>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="D34" t="n">
+        <v>1</v>
+      </c>
+      <c r="E34" t="n">
+        <v>1563247.374122903</v>
+      </c>
+      <c r="F34" t="n">
+        <v>-14646.62587709725</v>
+      </c>
+      <c r="G34" t="n">
+        <v>-0.9282388979929735</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>트랜스오션</t>
+        </is>
+      </c>
+      <c r="B35" t="n">
+        <v>750</v>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="D35" t="n">
+        <v>1</v>
+      </c>
+      <c r="E35" t="n">
+        <v>7020031.5082007</v>
+      </c>
+      <c r="F35" t="n">
+        <v>2892797.5082007</v>
+      </c>
+      <c r="G35" t="n">
+        <v>70.09046514446965</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>페트로브라스 (ADR)</t>
+        </is>
+      </c>
+      <c r="B36" t="n">
+        <v>480</v>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="D36" t="n">
+        <v>1</v>
+      </c>
+      <c r="E36" t="n">
+        <v>13579584.97235231</v>
+      </c>
+      <c r="F36" t="n">
+        <v>1473035.972352311</v>
+      </c>
+      <c r="G36" t="n">
+        <v>12.16726560436265</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>프론트라인</t>
+        </is>
+      </c>
+      <c r="B37" t="n">
+        <v>175</v>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="D37" t="n">
+        <v>1</v>
+      </c>
+      <c r="E37" t="n">
+        <v>8471815.962899337</v>
+      </c>
+      <c r="F37" t="n">
+        <v>4041951.962899337</v>
+      </c>
+      <c r="G37" t="n">
+        <v>91.24325177701475</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>피바디 에너지</t>
+        </is>
+      </c>
+      <c r="B38" t="n">
+        <v>65</v>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="D38" t="n">
+        <v>1</v>
+      </c>
+      <c r="E38" t="n">
+        <v>3649438.50225304</v>
+      </c>
+      <c r="F38" t="n">
+        <v>2178666.50225304</v>
+      </c>
+      <c r="G38" t="n">
+        <v>148.1308117269733</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>하프니아</t>
+        </is>
+      </c>
+      <c r="B39" t="n">
+        <v>80</v>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="D39" t="n">
+        <v>1</v>
+      </c>
+      <c r="E39" t="n">
+        <v>842704.775390625</v>
+      </c>
+      <c r="F39" t="n">
+        <v>216973.775390625</v>
+      </c>
+      <c r="G39" t="n">
+        <v>34.67524789256486</v>
       </c>
     </row>
   </sheetData>
@@ -512,7 +1538,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-03-17</t>
+          <t>2026-03-21</t>
         </is>
       </c>
       <c r="B2" t="n">
@@ -523,11 +1549,11 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2026-03-21T04:52:16</t>
+          <t>2026-03-21T04:52:57</t>
         </is>
       </c>
       <c r="E2" t="n">
-        <v>1488.910034179688</v>
+        <v>1504.829956054688</v>
       </c>
     </row>
   </sheetData>
@@ -541,7 +1567,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I1"/>
+  <dimension ref="A1:I39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -588,6 +1614,1412 @@
       <c r="I1" s="1" t="inlineStr">
         <is>
           <t>created_at</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>2026-03-21</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>페트로브라스 (ADR)</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>480</v>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E2" t="n">
+        <v>1</v>
+      </c>
+      <c r="F2" t="n">
+        <v>13579584.97235231</v>
+      </c>
+      <c r="G2" t="n">
+        <v>1473035.972352311</v>
+      </c>
+      <c r="H2" t="n">
+        <v>12.16726560436265</v>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>2026-03-21T04:52:57</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-03-21</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>AGNC 인베스트먼트</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>700</v>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E3" t="n">
+        <v>1</v>
+      </c>
+      <c r="F3" t="n">
+        <v>10270464.45007324</v>
+      </c>
+      <c r="G3" t="n">
+        <v>-561550.5499267559</v>
+      </c>
+      <c r="H3" t="n">
+        <v>-5.184174411933109</v>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>2026-03-21T04:52:57</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2026-03-21</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>대한조선</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>100</v>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E4" t="n">
+        <v>1</v>
+      </c>
+      <c r="F4" t="n">
+        <v>9120000</v>
+      </c>
+      <c r="G4" t="n">
+        <v>1907000</v>
+      </c>
+      <c r="H4" t="n">
+        <v>26.43837515596839</v>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>2026-03-21T04:52:57</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2026-03-21</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>프론트라인</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>175</v>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E5" t="n">
+        <v>1</v>
+      </c>
+      <c r="F5" t="n">
+        <v>8471815.962899337</v>
+      </c>
+      <c r="G5" t="n">
+        <v>4041951.962899337</v>
+      </c>
+      <c r="H5" t="n">
+        <v>91.24325177701475</v>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>2026-03-21T04:52:57</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026-03-21</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>시드릴</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>123</v>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E6" t="n">
+        <v>1</v>
+      </c>
+      <c r="F6" t="n">
+        <v>8070101.805898919</v>
+      </c>
+      <c r="G6" t="n">
+        <v>1619750.805898919</v>
+      </c>
+      <c r="H6" t="n">
+        <v>25.11104908707943</v>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>2026-03-21T04:52:57</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2026-03-21</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>세아제강</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>50</v>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E7" t="n">
+        <v>1</v>
+      </c>
+      <c r="F7" t="n">
+        <v>7395000</v>
+      </c>
+      <c r="G7" t="n">
+        <v>1085000</v>
+      </c>
+      <c r="H7" t="n">
+        <v>17.19492868462758</v>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>2026-03-21T04:52:57</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2026-03-21</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>센트러스 에너지</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>25</v>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E8" t="n">
+        <v>1</v>
+      </c>
+      <c r="F8" t="n">
+        <v>7026050.85816239</v>
+      </c>
+      <c r="G8" t="n">
+        <v>-406805.1418376099</v>
+      </c>
+      <c r="H8" t="n">
+        <v>-5.473066366920198</v>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>2026-03-21T04:52:57</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-03-21</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>트랜스오션</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>750</v>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E9" t="n">
+        <v>1</v>
+      </c>
+      <c r="F9" t="n">
+        <v>7020031.5082007</v>
+      </c>
+      <c r="G9" t="n">
+        <v>2892797.5082007</v>
+      </c>
+      <c r="H9" t="n">
+        <v>70.09046514446965</v>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>2026-03-21T04:52:57</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-03-21</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>DL이앤씨</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>80</v>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E10" t="n">
+        <v>1</v>
+      </c>
+      <c r="F10" t="n">
+        <v>5392000</v>
+      </c>
+      <c r="G10" t="n">
+        <v>1981000</v>
+      </c>
+      <c r="H10" t="n">
+        <v>58.07681031955438</v>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>2026-03-21T04:52:57</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2026-03-21</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>타이드워터</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>48</v>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E11" t="n">
+        <v>1</v>
+      </c>
+      <c r="F11" t="n">
+        <v>5235363.852789983</v>
+      </c>
+      <c r="G11" t="n">
+        <v>1510818.852789983</v>
+      </c>
+      <c r="H11" t="n">
+        <v>40.56385015592463</v>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>2026-03-21T04:52:57</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2026-03-21</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>노브</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>185</v>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E12" t="n">
+        <v>1</v>
+      </c>
+      <c r="F12" t="n">
+        <v>5200391.447092756</v>
+      </c>
+      <c r="G12" t="n">
+        <v>1890383.447092756</v>
+      </c>
+      <c r="H12" t="n">
+        <v>57.11114435653194</v>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>2026-03-21T04:52:57</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2026-03-21</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>TIME 코리아밸류업액티브</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>201</v>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E13" t="n">
+        <v>1</v>
+      </c>
+      <c r="F13" t="n">
+        <v>4797870</v>
+      </c>
+      <c r="G13" t="n">
+        <v>74073</v>
+      </c>
+      <c r="H13" t="n">
+        <v>1.568081778281328</v>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>2026-03-21T04:52:57</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026-03-21</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>오케아니스 에코 탱커스</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>65</v>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E14" t="n">
+        <v>1</v>
+      </c>
+      <c r="F14" t="n">
+        <v>4511179.137784176</v>
+      </c>
+      <c r="G14" t="n">
+        <v>2254819.137784176</v>
+      </c>
+      <c r="H14" t="n">
+        <v>99.93171026716374</v>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>2026-03-21T04:52:57</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>2026-03-21</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>동원개발</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>1360</v>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E15" t="n">
+        <v>1</v>
+      </c>
+      <c r="F15" t="n">
+        <v>4202400</v>
+      </c>
+      <c r="G15" t="n">
+        <v>465000</v>
+      </c>
+      <c r="H15" t="n">
+        <v>12.44180446299566</v>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>2026-03-21T04:52:57</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-03-21</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>HD건설기계</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>31</v>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E16" t="n">
+        <v>1</v>
+      </c>
+      <c r="F16" t="n">
+        <v>4123000</v>
+      </c>
+      <c r="G16" t="n">
+        <v>87904</v>
+      </c>
+      <c r="H16" t="n">
+        <v>2.178485964150543</v>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>2026-03-21T04:52:57</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2026-03-21</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>차코스 에너지 내비게이션</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
+        <v>75</v>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E17" t="n">
+        <v>1</v>
+      </c>
+      <c r="F17" t="n">
+        <v>4026924.996845168</v>
+      </c>
+      <c r="G17" t="n">
+        <v>202276.9968451681</v>
+      </c>
+      <c r="H17" t="n">
+        <v>5.28877420471552</v>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>2026-03-21T04:52:57</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>2026-03-21</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>피바디 에너지</t>
+        </is>
+      </c>
+      <c r="C18" t="n">
+        <v>65</v>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E18" t="n">
+        <v>1</v>
+      </c>
+      <c r="F18" t="n">
+        <v>3649438.50225304</v>
+      </c>
+      <c r="G18" t="n">
+        <v>2178666.50225304</v>
+      </c>
+      <c r="H18" t="n">
+        <v>148.1308117269733</v>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>2026-03-21T04:52:57</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>2026-03-21</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>삼성화재</t>
+        </is>
+      </c>
+      <c r="C19" t="n">
+        <v>7</v>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E19" t="n">
+        <v>1</v>
+      </c>
+      <c r="F19" t="n">
+        <v>3321500</v>
+      </c>
+      <c r="G19" t="n">
+        <v>-309500</v>
+      </c>
+      <c r="H19" t="n">
+        <v>-8.523822638391627</v>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>2026-03-21T04:52:57</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>2026-03-21</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>더치 브로스</t>
+        </is>
+      </c>
+      <c r="C20" t="n">
+        <v>39</v>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E20" t="n">
+        <v>1</v>
+      </c>
+      <c r="F20" t="n">
+        <v>2934418.414306641</v>
+      </c>
+      <c r="G20" t="n">
+        <v>-256225.5856933598</v>
+      </c>
+      <c r="H20" t="n">
+        <v>-8.030528811530205</v>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>2026-03-21T04:52:57</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>2026-03-21</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>휴스틸</t>
+        </is>
+      </c>
+      <c r="C21" t="n">
+        <v>500</v>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E21" t="n">
+        <v>1</v>
+      </c>
+      <c r="F21" t="n">
+        <v>2750000</v>
+      </c>
+      <c r="G21" t="n">
+        <v>471390</v>
+      </c>
+      <c r="H21" t="n">
+        <v>20.68761218462133</v>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>2026-03-21T04:52:57</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>2026-03-21</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>현대제철</t>
+        </is>
+      </c>
+      <c r="C22" t="n">
+        <v>70</v>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E22" t="n">
+        <v>1</v>
+      </c>
+      <c r="F22" t="n">
+        <v>2621500</v>
+      </c>
+      <c r="G22" t="n">
+        <v>-186000</v>
+      </c>
+      <c r="H22" t="n">
+        <v>-6.625111308993767</v>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>2026-03-21T04:52:57</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>2026-03-21</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>KoAct 코스닥액티브</t>
+        </is>
+      </c>
+      <c r="C23" t="n">
+        <v>200</v>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E23" t="n">
+        <v>1</v>
+      </c>
+      <c r="F23" t="n">
+        <v>2582000</v>
+      </c>
+      <c r="G23" t="n">
+        <v>-120000</v>
+      </c>
+      <c r="H23" t="n">
+        <v>-4.441154700222058</v>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>2026-03-21T04:52:57</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>2026-03-21</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>넥스틸</t>
+        </is>
+      </c>
+      <c r="C24" t="n">
+        <v>200</v>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E24" t="n">
+        <v>1</v>
+      </c>
+      <c r="F24" t="n">
+        <v>2514000</v>
+      </c>
+      <c r="G24" t="n">
+        <v>503000</v>
+      </c>
+      <c r="H24" t="n">
+        <v>25.01243162605669</v>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>2026-03-21T04:52:57</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>2026-03-21</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>대신증권</t>
+        </is>
+      </c>
+      <c r="C25" t="n">
+        <v>55</v>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E25" t="n">
+        <v>1</v>
+      </c>
+      <c r="F25" t="n">
+        <v>2219250</v>
+      </c>
+      <c r="G25" t="n">
+        <v>509749</v>
+      </c>
+      <c r="H25" t="n">
+        <v>29.81858448752005</v>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>2026-03-21T04:52:57</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>2026-03-21</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>발레로 에너지</t>
+        </is>
+      </c>
+      <c r="C26" t="n">
+        <v>6</v>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E26" t="n">
+        <v>1</v>
+      </c>
+      <c r="F26" t="n">
+        <v>2165691.085066516</v>
+      </c>
+      <c r="G26" t="n">
+        <v>101701.085066516</v>
+      </c>
+      <c r="H26" t="n">
+        <v>4.927402025519307</v>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>2026-03-21T04:52:57</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>2026-03-21</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>미창석유</t>
+        </is>
+      </c>
+      <c r="C27" t="n">
+        <v>18</v>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E27" t="n">
+        <v>1</v>
+      </c>
+      <c r="F27" t="n">
+        <v>2097000</v>
+      </c>
+      <c r="G27" t="n">
+        <v>-295200</v>
+      </c>
+      <c r="H27" t="n">
+        <v>-12.34010534236268</v>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>2026-03-21T04:52:57</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>2026-03-21</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>대창단조</t>
+        </is>
+      </c>
+      <c r="C28" t="n">
+        <v>300</v>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E28" t="n">
+        <v>1</v>
+      </c>
+      <c r="F28" t="n">
+        <v>2004000</v>
+      </c>
+      <c r="G28" t="n">
+        <v>-54000</v>
+      </c>
+      <c r="H28" t="n">
+        <v>-2.623906705539359</v>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>2026-03-21T04:52:57</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>2026-03-21</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>동방</t>
+        </is>
+      </c>
+      <c r="C29" t="n">
+        <v>681</v>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E29" t="n">
+        <v>1</v>
+      </c>
+      <c r="F29" t="n">
+        <v>1995330</v>
+      </c>
+      <c r="G29" t="n">
+        <v>23829</v>
+      </c>
+      <c r="H29" t="n">
+        <v>1.208672985709873</v>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>2026-03-21T04:52:57</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>2026-03-21</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>스타 벌크 캐리어스</t>
+        </is>
+      </c>
+      <c r="C30" t="n">
+        <v>50</v>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E30" t="n">
+        <v>1</v>
+      </c>
+      <c r="F30" t="n">
+        <v>1680142.640194588</v>
+      </c>
+      <c r="G30" t="n">
+        <v>365789.6401945879</v>
+      </c>
+      <c r="H30" t="n">
+        <v>27.83039565433242</v>
+      </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>2026-03-21T04:52:57</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>2026-03-21</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>케이씨</t>
+        </is>
+      </c>
+      <c r="C31" t="n">
+        <v>50</v>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E31" t="n">
+        <v>1</v>
+      </c>
+      <c r="F31" t="n">
+        <v>1670000</v>
+      </c>
+      <c r="G31" t="n">
+        <v>20500</v>
+      </c>
+      <c r="H31" t="n">
+        <v>1.242800848742043</v>
+      </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>2026-03-21T04:52:57</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>2026-03-21</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>유나이티드헬스 그룹</t>
+        </is>
+      </c>
+      <c r="C32" t="n">
+        <v>4</v>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E32" t="n">
+        <v>1</v>
+      </c>
+      <c r="F32" t="n">
+        <v>1658864.328313038</v>
+      </c>
+      <c r="G32" t="n">
+        <v>-35591.67168696248</v>
+      </c>
+      <c r="H32" t="n">
+        <v>-2.100477774988697</v>
+      </c>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>2026-03-21T04:52:57</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>2026-03-21</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>텍사스 퍼시픽 랜드</t>
+        </is>
+      </c>
+      <c r="C33" t="n">
+        <v>2</v>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E33" t="n">
+        <v>1</v>
+      </c>
+      <c r="F33" t="n">
+        <v>1563247.374122903</v>
+      </c>
+      <c r="G33" t="n">
+        <v>-14646.62587709725</v>
+      </c>
+      <c r="H33" t="n">
+        <v>-0.9282388979929735</v>
+      </c>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>2026-03-21T04:52:57</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>2026-03-21</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>하나금융지주</t>
+        </is>
+      </c>
+      <c r="C34" t="n">
+        <v>10</v>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E34" t="n">
+        <v>1</v>
+      </c>
+      <c r="F34" t="n">
+        <v>1132000</v>
+      </c>
+      <c r="G34" t="n">
+        <v>23000</v>
+      </c>
+      <c r="H34" t="n">
+        <v>2.073940486925157</v>
+      </c>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>2026-03-21T04:52:57</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>2026-03-21</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>삼성생명</t>
+        </is>
+      </c>
+      <c r="C35" t="n">
+        <v>4</v>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E35" t="n">
+        <v>1</v>
+      </c>
+      <c r="F35" t="n">
+        <v>926000</v>
+      </c>
+      <c r="G35" t="n">
+        <v>93000</v>
+      </c>
+      <c r="H35" t="n">
+        <v>11.16446578631453</v>
+      </c>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>2026-03-21T04:52:57</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>2026-03-21</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>비에이치아이</t>
+        </is>
+      </c>
+      <c r="C36" t="n">
+        <v>8</v>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E36" t="n">
+        <v>1</v>
+      </c>
+      <c r="F36" t="n">
+        <v>876000</v>
+      </c>
+      <c r="G36" t="n">
+        <v>210885</v>
+      </c>
+      <c r="H36" t="n">
+        <v>31.70654698811484</v>
+      </c>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>2026-03-21T04:52:57</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>2026-03-21</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>하프니아</t>
+        </is>
+      </c>
+      <c r="C37" t="n">
+        <v>80</v>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E37" t="n">
+        <v>1</v>
+      </c>
+      <c r="F37" t="n">
+        <v>842704.775390625</v>
+      </c>
+      <c r="G37" t="n">
+        <v>216973.775390625</v>
+      </c>
+      <c r="H37" t="n">
+        <v>34.67524789256486</v>
+      </c>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>2026-03-21T04:52:57</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>2026-03-21</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>클리블랜드 클리프스</t>
+        </is>
+      </c>
+      <c r="C38" t="n">
+        <v>70</v>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E38" t="n">
+        <v>1</v>
+      </c>
+      <c r="F38" t="n">
+        <v>823743.9360268187</v>
+      </c>
+      <c r="G38" t="n">
+        <v>-192311.0639731813</v>
+      </c>
+      <c r="H38" t="n">
+        <v>-18.92722972409774</v>
+      </c>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>2026-03-21T04:52:57</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>2026-03-21</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>노블</t>
+        </is>
+      </c>
+      <c r="C39" t="n">
+        <v>99</v>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E39" t="n">
+        <v>1</v>
+      </c>
+      <c r="F39" t="n">
+        <v>40689</v>
+      </c>
+      <c r="G39" t="n">
+        <v>-3866519</v>
+      </c>
+      <c r="H39" t="n">
+        <v>-98.95861699709869</v>
+      </c>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>2026-03-21T04:52:57</t>
         </is>
       </c>
     </row>
@@ -602,7 +3034,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E1"/>
+  <dimension ref="A1:E2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -632,6 +3064,29 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>2026-03-21</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>0</v>
+      </c>
+      <c r="C2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>2026-03-21T04:52:57</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>2026-03-21T04:52:57</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
auto: portfolio snapshot 2026-03-21 (2026-03-21T04:54:09)
</commit_message>
<xml_diff>
--- a/portfolio_auto.xlsx
+++ b/portfolio_auto.xlsx
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G39"/>
+  <dimension ref="A1:G42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -471,11 +471,11 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>노브</t>
+          <t>유나이티드헬스 그룹</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>185</v>
+        <v>4</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
@@ -486,23 +486,23 @@
         <v>1</v>
       </c>
       <c r="E2" t="n">
-        <v>5200391.447092756</v>
+        <v>1658864.328313038</v>
       </c>
       <c r="F2" t="n">
-        <v>1890383.447092756</v>
+        <v>-35591.67168696248</v>
       </c>
       <c r="G2" t="n">
-        <v>57.11114435653194</v>
+        <v>-2.100477774988697</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>노블</t>
+          <t>AGNC 인베스트먼트</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>99</v>
+        <v>700</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
@@ -513,23 +513,23 @@
         <v>1</v>
       </c>
       <c r="E3" t="n">
-        <v>40689</v>
+        <v>10270464.45007324</v>
       </c>
       <c r="F3" t="n">
-        <v>-3866519</v>
+        <v>-561550.5499267559</v>
       </c>
       <c r="G3" t="n">
-        <v>-98.95861699709869</v>
+        <v>-5.184174411933109</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>더치 브로스</t>
+          <t>넥스틸</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>39</v>
+        <v>200</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
@@ -540,23 +540,23 @@
         <v>1</v>
       </c>
       <c r="E4" t="n">
-        <v>2934418.414306641</v>
+        <v>2514000</v>
       </c>
       <c r="F4" t="n">
-        <v>-256225.5856933598</v>
+        <v>503000</v>
       </c>
       <c r="G4" t="n">
-        <v>-8.030528811530205</v>
+        <v>25.01243162605669</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>발레로 에너지</t>
+          <t>대신증권</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>6</v>
+        <v>55</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -567,23 +567,23 @@
         <v>1</v>
       </c>
       <c r="E5" t="n">
-        <v>2165691.085066516</v>
+        <v>2219250</v>
       </c>
       <c r="F5" t="n">
-        <v>101701.085066516</v>
+        <v>509749</v>
       </c>
       <c r="G5" t="n">
-        <v>4.927402025519307</v>
+        <v>29.81858448752005</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>유나이티드헬스 그룹</t>
+          <t>대창단조</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>4</v>
+        <v>300</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
@@ -594,23 +594,23 @@
         <v>1</v>
       </c>
       <c r="E6" t="n">
-        <v>1658864.328313038</v>
+        <v>2004000</v>
       </c>
       <c r="F6" t="n">
-        <v>-35591.67168696248</v>
+        <v>-54000</v>
       </c>
       <c r="G6" t="n">
-        <v>-2.100477774988697</v>
+        <v>-2.623906705539359</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>AGNC 인베스트먼트</t>
+          <t>대한조선</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>700</v>
+        <v>100</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -621,23 +621,23 @@
         <v>1</v>
       </c>
       <c r="E7" t="n">
-        <v>10270464.45007324</v>
+        <v>9120000</v>
       </c>
       <c r="F7" t="n">
-        <v>-561550.5499267559</v>
+        <v>1907000</v>
       </c>
       <c r="G7" t="n">
-        <v>-5.184174411933109</v>
+        <v>26.43837515596839</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>넥스틸</t>
+          <t>동방</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>200</v>
+        <v>681</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
@@ -648,23 +648,23 @@
         <v>1</v>
       </c>
       <c r="E8" t="n">
-        <v>2514000</v>
+        <v>1995330</v>
       </c>
       <c r="F8" t="n">
-        <v>503000</v>
+        <v>23829</v>
       </c>
       <c r="G8" t="n">
-        <v>25.01243162605669</v>
+        <v>1.208672985709873</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>대신증권</t>
+          <t>동원개발</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>55</v>
+        <v>1360</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
@@ -675,23 +675,23 @@
         <v>1</v>
       </c>
       <c r="E9" t="n">
-        <v>2219250</v>
+        <v>4202400</v>
       </c>
       <c r="F9" t="n">
-        <v>509749</v>
+        <v>465000</v>
       </c>
       <c r="G9" t="n">
-        <v>29.81858448752005</v>
+        <v>12.44180446299566</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>대창단조</t>
+          <t>미창석유</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>300</v>
+        <v>18</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
@@ -702,23 +702,23 @@
         <v>1</v>
       </c>
       <c r="E10" t="n">
-        <v>2004000</v>
+        <v>2097000</v>
       </c>
       <c r="F10" t="n">
-        <v>-54000</v>
+        <v>-295200</v>
       </c>
       <c r="G10" t="n">
-        <v>-2.623906705539359</v>
+        <v>-12.34010534236268</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>대한조선</t>
+          <t>비에이치아이</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>100</v>
+        <v>8</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
@@ -729,23 +729,23 @@
         <v>1</v>
       </c>
       <c r="E11" t="n">
-        <v>9120000</v>
+        <v>876000</v>
       </c>
       <c r="F11" t="n">
-        <v>1907000</v>
+        <v>210885</v>
       </c>
       <c r="G11" t="n">
-        <v>26.43837515596839</v>
+        <v>31.70654698811484</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>동방</t>
+          <t>삼성생명</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>681</v>
+        <v>4</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
@@ -756,23 +756,23 @@
         <v>1</v>
       </c>
       <c r="E12" t="n">
-        <v>1995330</v>
+        <v>926000</v>
       </c>
       <c r="F12" t="n">
-        <v>23829</v>
+        <v>93000</v>
       </c>
       <c r="G12" t="n">
-        <v>1.208672985709873</v>
+        <v>11.16446578631453</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>동원개발</t>
+          <t>삼성화재</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>1360</v>
+        <v>7</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
@@ -783,23 +783,23 @@
         <v>1</v>
       </c>
       <c r="E13" t="n">
-        <v>4202400</v>
+        <v>3321500</v>
       </c>
       <c r="F13" t="n">
-        <v>465000</v>
+        <v>-309500</v>
       </c>
       <c r="G13" t="n">
-        <v>12.44180446299566</v>
+        <v>-8.523822638391627</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>미창석유</t>
+          <t>세아제강</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>18</v>
+        <v>50</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
@@ -810,23 +810,23 @@
         <v>1</v>
       </c>
       <c r="E14" t="n">
-        <v>2097000</v>
+        <v>7395000</v>
       </c>
       <c r="F14" t="n">
-        <v>-295200</v>
+        <v>1085000</v>
       </c>
       <c r="G14" t="n">
-        <v>-12.34010534236268</v>
+        <v>17.19492868462758</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>비에이치아이</t>
+          <t>케이씨</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>8</v>
+        <v>50</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
@@ -837,23 +837,23 @@
         <v>1</v>
       </c>
       <c r="E15" t="n">
-        <v>876000</v>
+        <v>1670000</v>
       </c>
       <c r="F15" t="n">
-        <v>210885</v>
+        <v>20500</v>
       </c>
       <c r="G15" t="n">
-        <v>31.70654698811484</v>
+        <v>1.242800848742043</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>삼성생명</t>
+          <t>하나금융지주</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
@@ -864,23 +864,23 @@
         <v>1</v>
       </c>
       <c r="E16" t="n">
-        <v>926000</v>
+        <v>1132000</v>
       </c>
       <c r="F16" t="n">
-        <v>93000</v>
+        <v>23000</v>
       </c>
       <c r="G16" t="n">
-        <v>11.16446578631453</v>
+        <v>2.073940486925157</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>삼성화재</t>
+          <t>현대제철</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>7</v>
+        <v>70</v>
       </c>
       <c r="C17" t="inlineStr">
         <is>
@@ -891,23 +891,23 @@
         <v>1</v>
       </c>
       <c r="E17" t="n">
-        <v>3321500</v>
+        <v>2621500</v>
       </c>
       <c r="F17" t="n">
-        <v>-309500</v>
+        <v>-186000</v>
       </c>
       <c r="G17" t="n">
-        <v>-8.523822638391627</v>
+        <v>-6.625111308993767</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>세아제강</t>
+          <t>휴스틸</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>50</v>
+        <v>500</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
@@ -918,23 +918,23 @@
         <v>1</v>
       </c>
       <c r="E18" t="n">
-        <v>7395000</v>
+        <v>2750000</v>
       </c>
       <c r="F18" t="n">
-        <v>1085000</v>
+        <v>471390</v>
       </c>
       <c r="G18" t="n">
-        <v>17.19492868462758</v>
+        <v>20.68761218462133</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>케이씨</t>
+          <t>센트러스 에너지</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>50</v>
+        <v>25</v>
       </c>
       <c r="C19" t="inlineStr">
         <is>
@@ -945,23 +945,23 @@
         <v>1</v>
       </c>
       <c r="E19" t="n">
-        <v>1670000</v>
+        <v>7026050.85816239</v>
       </c>
       <c r="F19" t="n">
-        <v>20500</v>
+        <v>-406805.1418376099</v>
       </c>
       <c r="G19" t="n">
-        <v>1.242800848742043</v>
+        <v>-5.473066366920198</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>하나금융지주</t>
+          <t>스타 벌크 캐리어스</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>10</v>
+        <v>50</v>
       </c>
       <c r="C20" t="inlineStr">
         <is>
@@ -972,23 +972,23 @@
         <v>1</v>
       </c>
       <c r="E20" t="n">
-        <v>1132000</v>
+        <v>1680142.640194588</v>
       </c>
       <c r="F20" t="n">
-        <v>23000</v>
+        <v>365789.6401945879</v>
       </c>
       <c r="G20" t="n">
-        <v>2.073940486925157</v>
+        <v>27.83039565433242</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>현대제철</t>
+          <t>시드릴</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>70</v>
+        <v>123</v>
       </c>
       <c r="C21" t="inlineStr">
         <is>
@@ -999,23 +999,23 @@
         <v>1</v>
       </c>
       <c r="E21" t="n">
-        <v>2621500</v>
+        <v>8070101.805898919</v>
       </c>
       <c r="F21" t="n">
-        <v>-186000</v>
+        <v>1619750.805898919</v>
       </c>
       <c r="G21" t="n">
-        <v>-6.625111308993767</v>
+        <v>25.11104908707943</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>휴스틸</t>
+          <t>오케아니스 에코 탱커스</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>500</v>
+        <v>65</v>
       </c>
       <c r="C22" t="inlineStr">
         <is>
@@ -1026,23 +1026,23 @@
         <v>1</v>
       </c>
       <c r="E22" t="n">
-        <v>2750000</v>
+        <v>4511179.137784176</v>
       </c>
       <c r="F22" t="n">
-        <v>471390</v>
+        <v>2254819.137784176</v>
       </c>
       <c r="G22" t="n">
-        <v>20.68761218462133</v>
+        <v>99.93171026716374</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>DL이앤씨</t>
+          <t>차코스 에너지 내비게이션</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>80</v>
+        <v>75</v>
       </c>
       <c r="C23" t="inlineStr">
         <is>
@@ -1053,23 +1053,23 @@
         <v>1</v>
       </c>
       <c r="E23" t="n">
-        <v>5392000</v>
+        <v>4026924.996845168</v>
       </c>
       <c r="F23" t="n">
-        <v>1981000</v>
+        <v>202276.9968451681</v>
       </c>
       <c r="G23" t="n">
-        <v>58.07681031955438</v>
+        <v>5.28877420471552</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>HD건설기계</t>
+          <t>클리블랜드 클리프스</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>31</v>
+        <v>70</v>
       </c>
       <c r="C24" t="inlineStr">
         <is>
@@ -1080,23 +1080,23 @@
         <v>1</v>
       </c>
       <c r="E24" t="n">
-        <v>4123000</v>
+        <v>823743.9360268187</v>
       </c>
       <c r="F24" t="n">
-        <v>87904</v>
+        <v>-192311.0639731813</v>
       </c>
       <c r="G24" t="n">
-        <v>2.178485964150543</v>
+        <v>-18.92722972409774</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>KoAct 코스닥액티브</t>
+          <t>타이드워터</t>
         </is>
       </c>
       <c r="B25" t="n">
-        <v>200</v>
+        <v>48</v>
       </c>
       <c r="C25" t="inlineStr">
         <is>
@@ -1107,23 +1107,23 @@
         <v>1</v>
       </c>
       <c r="E25" t="n">
-        <v>2582000</v>
+        <v>5235363.852789983</v>
       </c>
       <c r="F25" t="n">
-        <v>-120000</v>
+        <v>1510818.852789983</v>
       </c>
       <c r="G25" t="n">
-        <v>-4.441154700222058</v>
+        <v>40.56385015592463</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>TIME 코리아밸류업액티브</t>
+          <t>텍사스 퍼시픽 랜드</t>
         </is>
       </c>
       <c r="B26" t="n">
-        <v>201</v>
+        <v>2</v>
       </c>
       <c r="C26" t="inlineStr">
         <is>
@@ -1134,23 +1134,23 @@
         <v>1</v>
       </c>
       <c r="E26" t="n">
-        <v>4797870</v>
+        <v>1563247.374122903</v>
       </c>
       <c r="F26" t="n">
-        <v>74073</v>
+        <v>-14646.62587709725</v>
       </c>
       <c r="G26" t="n">
-        <v>1.568081778281328</v>
+        <v>-0.9282388979929735</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>센트러스 에너지</t>
+          <t>트랜스오션</t>
         </is>
       </c>
       <c r="B27" t="n">
-        <v>25</v>
+        <v>750</v>
       </c>
       <c r="C27" t="inlineStr">
         <is>
@@ -1161,23 +1161,23 @@
         <v>1</v>
       </c>
       <c r="E27" t="n">
-        <v>7026050.85816239</v>
+        <v>7020031.5082007</v>
       </c>
       <c r="F27" t="n">
-        <v>-406805.1418376099</v>
+        <v>2892797.5082007</v>
       </c>
       <c r="G27" t="n">
-        <v>-5.473066366920198</v>
+        <v>70.09046514446965</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>스타 벌크 캐리어스</t>
+          <t>페트로브라스 (ADR)</t>
         </is>
       </c>
       <c r="B28" t="n">
-        <v>50</v>
+        <v>480</v>
       </c>
       <c r="C28" t="inlineStr">
         <is>
@@ -1188,23 +1188,23 @@
         <v>1</v>
       </c>
       <c r="E28" t="n">
-        <v>1680142.640194588</v>
+        <v>13579584.97235231</v>
       </c>
       <c r="F28" t="n">
-        <v>365789.6401945879</v>
+        <v>1473035.972352311</v>
       </c>
       <c r="G28" t="n">
-        <v>27.83039565433242</v>
+        <v>12.16726560436265</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>시드릴</t>
+          <t>프론트라인</t>
         </is>
       </c>
       <c r="B29" t="n">
-        <v>123</v>
+        <v>175</v>
       </c>
       <c r="C29" t="inlineStr">
         <is>
@@ -1215,19 +1215,19 @@
         <v>1</v>
       </c>
       <c r="E29" t="n">
-        <v>8070101.805898919</v>
+        <v>8471815.962899337</v>
       </c>
       <c r="F29" t="n">
-        <v>1619750.805898919</v>
+        <v>4041951.962899337</v>
       </c>
       <c r="G29" t="n">
-        <v>25.11104908707943</v>
+        <v>91.24325177701475</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>오케아니스 에코 탱커스</t>
+          <t>피바디 에너지</t>
         </is>
       </c>
       <c r="B30" t="n">
@@ -1242,23 +1242,23 @@
         <v>1</v>
       </c>
       <c r="E30" t="n">
-        <v>4511179.137784176</v>
+        <v>3649438.50225304</v>
       </c>
       <c r="F30" t="n">
-        <v>2254819.137784176</v>
+        <v>2178666.50225304</v>
       </c>
       <c r="G30" t="n">
-        <v>99.93171026716374</v>
+        <v>148.1308117269733</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>차코스 에너지 내비게이션</t>
+          <t>하프니아</t>
         </is>
       </c>
       <c r="B31" t="n">
-        <v>75</v>
+        <v>80</v>
       </c>
       <c r="C31" t="inlineStr">
         <is>
@@ -1269,23 +1269,23 @@
         <v>1</v>
       </c>
       <c r="E31" t="n">
-        <v>4026924.996845168</v>
+        <v>842704.775390625</v>
       </c>
       <c r="F31" t="n">
-        <v>202276.9968451681</v>
+        <v>216973.775390625</v>
       </c>
       <c r="G31" t="n">
-        <v>5.28877420471552</v>
+        <v>34.67524789256486</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>클리블랜드 클리프스</t>
+          <t>DL이앤씨</t>
         </is>
       </c>
       <c r="B32" t="n">
-        <v>70</v>
+        <v>40</v>
       </c>
       <c r="C32" t="inlineStr">
         <is>
@@ -1296,23 +1296,23 @@
         <v>1</v>
       </c>
       <c r="E32" t="n">
-        <v>823743.9360268187</v>
+        <v>2696000</v>
       </c>
       <c r="F32" t="n">
-        <v>-192311.0639731813</v>
+        <v>990500</v>
       </c>
       <c r="G32" t="n">
-        <v>-18.92722972409774</v>
+        <v>58.07681031955438</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>타이드워터</t>
+          <t>HD건설기계</t>
         </is>
       </c>
       <c r="B33" t="n">
-        <v>48</v>
+        <v>31</v>
       </c>
       <c r="C33" t="inlineStr">
         <is>
@@ -1323,23 +1323,23 @@
         <v>1</v>
       </c>
       <c r="E33" t="n">
-        <v>5235363.852789983</v>
+        <v>4123000</v>
       </c>
       <c r="F33" t="n">
-        <v>1510818.852789983</v>
+        <v>87904</v>
       </c>
       <c r="G33" t="n">
-        <v>40.56385015592463</v>
+        <v>2.178485964150543</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>텍사스 퍼시픽 랜드</t>
+          <t>KoAct 코스닥액티브</t>
         </is>
       </c>
       <c r="B34" t="n">
-        <v>2</v>
+        <v>200</v>
       </c>
       <c r="C34" t="inlineStr">
         <is>
@@ -1350,23 +1350,23 @@
         <v>1</v>
       </c>
       <c r="E34" t="n">
-        <v>1563247.374122903</v>
+        <v>2582000</v>
       </c>
       <c r="F34" t="n">
-        <v>-14646.62587709725</v>
+        <v>-120000</v>
       </c>
       <c r="G34" t="n">
-        <v>-0.9282388979929735</v>
+        <v>-4.441154700222058</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>트랜스오션</t>
+          <t>LX인터내셔널</t>
         </is>
       </c>
       <c r="B35" t="n">
-        <v>750</v>
+        <v>20</v>
       </c>
       <c r="C35" t="inlineStr">
         <is>
@@ -1377,23 +1377,23 @@
         <v>1</v>
       </c>
       <c r="E35" t="n">
-        <v>7020031.5082007</v>
+        <v>944108</v>
       </c>
       <c r="F35" t="n">
-        <v>2892797.5082007</v>
+        <v>5108</v>
       </c>
       <c r="G35" t="n">
-        <v>70.09046514446965</v>
+        <v>0.5439829605963792</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>페트로브라스 (ADR)</t>
+          <t>NH투자증권우</t>
         </is>
       </c>
       <c r="B36" t="n">
-        <v>480</v>
+        <v>2</v>
       </c>
       <c r="C36" t="inlineStr">
         <is>
@@ -1404,23 +1404,23 @@
         <v>1</v>
       </c>
       <c r="E36" t="n">
-        <v>13579584.97235231</v>
+        <v>54591</v>
       </c>
       <c r="F36" t="n">
-        <v>1473035.972352311</v>
+        <v>-9</v>
       </c>
       <c r="G36" t="n">
-        <v>12.16726560436265</v>
+        <v>-0.01648351648351648</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>프론트라인</t>
+          <t>TIME 코리아밸류업액티브</t>
         </is>
       </c>
       <c r="B37" t="n">
-        <v>175</v>
+        <v>201</v>
       </c>
       <c r="C37" t="inlineStr">
         <is>
@@ -1431,23 +1431,23 @@
         <v>1</v>
       </c>
       <c r="E37" t="n">
-        <v>8471815.962899337</v>
+        <v>4797870</v>
       </c>
       <c r="F37" t="n">
-        <v>4041951.962899337</v>
+        <v>74073</v>
       </c>
       <c r="G37" t="n">
-        <v>91.24325177701475</v>
+        <v>1.568081778281328</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>피바디 에너지</t>
+          <t>노브</t>
         </is>
       </c>
       <c r="B38" t="n">
-        <v>65</v>
+        <v>185</v>
       </c>
       <c r="C38" t="inlineStr">
         <is>
@@ -1458,23 +1458,23 @@
         <v>1</v>
       </c>
       <c r="E38" t="n">
-        <v>3649438.50225304</v>
+        <v>5200391.447092756</v>
       </c>
       <c r="F38" t="n">
-        <v>2178666.50225304</v>
+        <v>1890383.447092756</v>
       </c>
       <c r="G38" t="n">
-        <v>148.1308117269733</v>
+        <v>57.11114435653194</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>하프니아</t>
+          <t>노블</t>
         </is>
       </c>
       <c r="B39" t="n">
-        <v>80</v>
+        <v>99</v>
       </c>
       <c r="C39" t="inlineStr">
         <is>
@@ -1485,13 +1485,94 @@
         <v>1</v>
       </c>
       <c r="E39" t="n">
-        <v>842704.775390625</v>
+        <v>40689</v>
       </c>
       <c r="F39" t="n">
-        <v>216973.775390625</v>
+        <v>-3866519</v>
       </c>
       <c r="G39" t="n">
-        <v>34.67524789256486</v>
+        <v>-98.95861699709869</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>낫 오프쇼어 파트너스</t>
+        </is>
+      </c>
+      <c r="B40" t="n">
+        <v>30</v>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="D40" t="n">
+        <v>1</v>
+      </c>
+      <c r="E40" t="n">
+        <v>410853</v>
+      </c>
+      <c r="F40" t="n">
+        <v>-6662</v>
+      </c>
+      <c r="G40" t="n">
+        <v>-1.595631294684023</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>더치 브로스</t>
+        </is>
+      </c>
+      <c r="B41" t="n">
+        <v>39</v>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="D41" t="n">
+        <v>1</v>
+      </c>
+      <c r="E41" t="n">
+        <v>2934418.414306641</v>
+      </c>
+      <c r="F41" t="n">
+        <v>-256226.5856933594</v>
+      </c>
+      <c r="G41" t="n">
+        <v>-8.030557636257226</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>발레로 에너지</t>
+        </is>
+      </c>
+      <c r="B42" t="n">
+        <v>6</v>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="D42" t="n">
+        <v>1</v>
+      </c>
+      <c r="E42" t="n">
+        <v>2165691.085066516</v>
+      </c>
+      <c r="F42" t="n">
+        <v>101701.085066516</v>
+      </c>
+      <c r="G42" t="n">
+        <v>4.927402025519307</v>
       </c>
     </row>
   </sheetData>
@@ -1549,7 +1630,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2026-03-21T04:52:57</t>
+          <t>2026-03-21T04:54:09</t>
         </is>
       </c>
       <c r="E2" t="n">
@@ -1567,7 +1648,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I39"/>
+  <dimension ref="A1:I42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1650,7 +1731,7 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>2026-03-21T04:52:57</t>
+          <t>2026-03-21T04:54:09</t>
         </is>
       </c>
     </row>
@@ -1687,7 +1768,7 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>2026-03-21T04:52:57</t>
+          <t>2026-03-21T04:54:09</t>
         </is>
       </c>
     </row>
@@ -1724,7 +1805,7 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>2026-03-21T04:52:57</t>
+          <t>2026-03-21T04:54:09</t>
         </is>
       </c>
     </row>
@@ -1761,7 +1842,7 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>2026-03-21T04:52:57</t>
+          <t>2026-03-21T04:54:09</t>
         </is>
       </c>
     </row>
@@ -1798,7 +1879,7 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>2026-03-21T04:52:57</t>
+          <t>2026-03-21T04:54:09</t>
         </is>
       </c>
     </row>
@@ -1835,7 +1916,7 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>2026-03-21T04:52:57</t>
+          <t>2026-03-21T04:54:09</t>
         </is>
       </c>
     </row>
@@ -1872,7 +1953,7 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>2026-03-21T04:52:57</t>
+          <t>2026-03-21T04:54:09</t>
         </is>
       </c>
     </row>
@@ -1909,7 +1990,7 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>2026-03-21T04:52:57</t>
+          <t>2026-03-21T04:54:09</t>
         </is>
       </c>
     </row>
@@ -1921,11 +2002,11 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>DL이앤씨</t>
+          <t>타이드워터</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>80</v>
+        <v>48</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
@@ -1936,17 +2017,17 @@
         <v>1</v>
       </c>
       <c r="F10" t="n">
-        <v>5392000</v>
+        <v>5235363.852789983</v>
       </c>
       <c r="G10" t="n">
-        <v>1981000</v>
+        <v>1510818.852789983</v>
       </c>
       <c r="H10" t="n">
-        <v>58.07681031955438</v>
+        <v>40.56385015592463</v>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>2026-03-21T04:52:57</t>
+          <t>2026-03-21T04:54:09</t>
         </is>
       </c>
     </row>
@@ -1958,11 +2039,11 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>타이드워터</t>
+          <t>노브</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>48</v>
+        <v>185</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
@@ -1973,17 +2054,17 @@
         <v>1</v>
       </c>
       <c r="F11" t="n">
-        <v>5235363.852789983</v>
+        <v>5200391.447092756</v>
       </c>
       <c r="G11" t="n">
-        <v>1510818.852789983</v>
+        <v>1890383.447092756</v>
       </c>
       <c r="H11" t="n">
-        <v>40.56385015592463</v>
+        <v>57.11114435653194</v>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>2026-03-21T04:52:57</t>
+          <t>2026-03-21T04:54:09</t>
         </is>
       </c>
     </row>
@@ -1995,11 +2076,11 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>노브</t>
+          <t>TIME 코리아밸류업액티브</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>185</v>
+        <v>201</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
@@ -2010,17 +2091,17 @@
         <v>1</v>
       </c>
       <c r="F12" t="n">
-        <v>5200391.447092756</v>
+        <v>4797870</v>
       </c>
       <c r="G12" t="n">
-        <v>1890383.447092756</v>
+        <v>74073</v>
       </c>
       <c r="H12" t="n">
-        <v>57.11114435653194</v>
+        <v>1.568081778281328</v>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>2026-03-21T04:52:57</t>
+          <t>2026-03-21T04:54:09</t>
         </is>
       </c>
     </row>
@@ -2032,11 +2113,11 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>TIME 코리아밸류업액티브</t>
+          <t>오케아니스 에코 탱커스</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>201</v>
+        <v>65</v>
       </c>
       <c r="D13" t="inlineStr">
         <is>
@@ -2047,17 +2128,17 @@
         <v>1</v>
       </c>
       <c r="F13" t="n">
-        <v>4797870</v>
+        <v>4511179.137784176</v>
       </c>
       <c r="G13" t="n">
-        <v>74073</v>
+        <v>2254819.137784176</v>
       </c>
       <c r="H13" t="n">
-        <v>1.568081778281328</v>
+        <v>99.93171026716374</v>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>2026-03-21T04:52:57</t>
+          <t>2026-03-21T04:54:09</t>
         </is>
       </c>
     </row>
@@ -2069,11 +2150,11 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>오케아니스 에코 탱커스</t>
+          <t>동원개발</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>65</v>
+        <v>1360</v>
       </c>
       <c r="D14" t="inlineStr">
         <is>
@@ -2084,17 +2165,17 @@
         <v>1</v>
       </c>
       <c r="F14" t="n">
-        <v>4511179.137784176</v>
+        <v>4202400</v>
       </c>
       <c r="G14" t="n">
-        <v>2254819.137784176</v>
+        <v>465000</v>
       </c>
       <c r="H14" t="n">
-        <v>99.93171026716374</v>
+        <v>12.44180446299566</v>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>2026-03-21T04:52:57</t>
+          <t>2026-03-21T04:54:09</t>
         </is>
       </c>
     </row>
@@ -2106,11 +2187,11 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>동원개발</t>
+          <t>HD건설기계</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>1360</v>
+        <v>31</v>
       </c>
       <c r="D15" t="inlineStr">
         <is>
@@ -2121,17 +2202,17 @@
         <v>1</v>
       </c>
       <c r="F15" t="n">
-        <v>4202400</v>
+        <v>4123000</v>
       </c>
       <c r="G15" t="n">
-        <v>465000</v>
+        <v>87904</v>
       </c>
       <c r="H15" t="n">
-        <v>12.44180446299566</v>
+        <v>2.178485964150543</v>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>2026-03-21T04:52:57</t>
+          <t>2026-03-21T04:54:09</t>
         </is>
       </c>
     </row>
@@ -2143,11 +2224,11 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>HD건설기계</t>
+          <t>차코스 에너지 내비게이션</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>31</v>
+        <v>75</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
@@ -2158,17 +2239,17 @@
         <v>1</v>
       </c>
       <c r="F16" t="n">
-        <v>4123000</v>
+        <v>4026924.996845168</v>
       </c>
       <c r="G16" t="n">
-        <v>87904</v>
+        <v>202276.9968451681</v>
       </c>
       <c r="H16" t="n">
-        <v>2.178485964150543</v>
+        <v>5.28877420471552</v>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>2026-03-21T04:52:57</t>
+          <t>2026-03-21T04:54:09</t>
         </is>
       </c>
     </row>
@@ -2180,11 +2261,11 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>차코스 에너지 내비게이션</t>
+          <t>피바디 에너지</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>75</v>
+        <v>65</v>
       </c>
       <c r="D17" t="inlineStr">
         <is>
@@ -2195,17 +2276,17 @@
         <v>1</v>
       </c>
       <c r="F17" t="n">
-        <v>4026924.996845168</v>
+        <v>3649438.50225304</v>
       </c>
       <c r="G17" t="n">
-        <v>202276.9968451681</v>
+        <v>2178666.50225304</v>
       </c>
       <c r="H17" t="n">
-        <v>5.28877420471552</v>
+        <v>148.1308117269733</v>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>2026-03-21T04:52:57</t>
+          <t>2026-03-21T04:54:09</t>
         </is>
       </c>
     </row>
@@ -2217,11 +2298,11 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>피바디 에너지</t>
+          <t>삼성화재</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>65</v>
+        <v>7</v>
       </c>
       <c r="D18" t="inlineStr">
         <is>
@@ -2232,17 +2313,17 @@
         <v>1</v>
       </c>
       <c r="F18" t="n">
-        <v>3649438.50225304</v>
+        <v>3321500</v>
       </c>
       <c r="G18" t="n">
-        <v>2178666.50225304</v>
+        <v>-309500</v>
       </c>
       <c r="H18" t="n">
-        <v>148.1308117269733</v>
+        <v>-8.523822638391627</v>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>2026-03-21T04:52:57</t>
+          <t>2026-03-21T04:54:09</t>
         </is>
       </c>
     </row>
@@ -2254,11 +2335,11 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>삼성화재</t>
+          <t>더치 브로스</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>7</v>
+        <v>39</v>
       </c>
       <c r="D19" t="inlineStr">
         <is>
@@ -2269,17 +2350,17 @@
         <v>1</v>
       </c>
       <c r="F19" t="n">
-        <v>3321500</v>
+        <v>2934418.414306641</v>
       </c>
       <c r="G19" t="n">
-        <v>-309500</v>
+        <v>-256226.5856933594</v>
       </c>
       <c r="H19" t="n">
-        <v>-8.523822638391627</v>
+        <v>-8.030557636257226</v>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>2026-03-21T04:52:57</t>
+          <t>2026-03-21T04:54:09</t>
         </is>
       </c>
     </row>
@@ -2291,11 +2372,11 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>더치 브로스</t>
+          <t>휴스틸</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>39</v>
+        <v>500</v>
       </c>
       <c r="D20" t="inlineStr">
         <is>
@@ -2306,17 +2387,17 @@
         <v>1</v>
       </c>
       <c r="F20" t="n">
-        <v>2934418.414306641</v>
+        <v>2750000</v>
       </c>
       <c r="G20" t="n">
-        <v>-256225.5856933598</v>
+        <v>471390</v>
       </c>
       <c r="H20" t="n">
-        <v>-8.030528811530205</v>
+        <v>20.68761218462133</v>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>2026-03-21T04:52:57</t>
+          <t>2026-03-21T04:54:09</t>
         </is>
       </c>
     </row>
@@ -2328,11 +2409,11 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>휴스틸</t>
+          <t>DL이앤씨</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>500</v>
+        <v>40</v>
       </c>
       <c r="D21" t="inlineStr">
         <is>
@@ -2343,17 +2424,17 @@
         <v>1</v>
       </c>
       <c r="F21" t="n">
-        <v>2750000</v>
+        <v>2696000</v>
       </c>
       <c r="G21" t="n">
-        <v>471390</v>
+        <v>990500</v>
       </c>
       <c r="H21" t="n">
-        <v>20.68761218462133</v>
+        <v>58.07681031955438</v>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>2026-03-21T04:52:57</t>
+          <t>2026-03-21T04:54:09</t>
         </is>
       </c>
     </row>
@@ -2390,7 +2471,7 @@
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>2026-03-21T04:52:57</t>
+          <t>2026-03-21T04:54:09</t>
         </is>
       </c>
     </row>
@@ -2427,7 +2508,7 @@
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>2026-03-21T04:52:57</t>
+          <t>2026-03-21T04:54:09</t>
         </is>
       </c>
     </row>
@@ -2464,7 +2545,7 @@
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>2026-03-21T04:52:57</t>
+          <t>2026-03-21T04:54:09</t>
         </is>
       </c>
     </row>
@@ -2501,7 +2582,7 @@
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>2026-03-21T04:52:57</t>
+          <t>2026-03-21T04:54:09</t>
         </is>
       </c>
     </row>
@@ -2538,7 +2619,7 @@
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>2026-03-21T04:52:57</t>
+          <t>2026-03-21T04:54:09</t>
         </is>
       </c>
     </row>
@@ -2575,7 +2656,7 @@
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>2026-03-21T04:52:57</t>
+          <t>2026-03-21T04:54:09</t>
         </is>
       </c>
     </row>
@@ -2612,7 +2693,7 @@
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>2026-03-21T04:52:57</t>
+          <t>2026-03-21T04:54:09</t>
         </is>
       </c>
     </row>
@@ -2649,7 +2730,7 @@
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>2026-03-21T04:52:57</t>
+          <t>2026-03-21T04:54:09</t>
         </is>
       </c>
     </row>
@@ -2686,7 +2767,7 @@
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>2026-03-21T04:52:57</t>
+          <t>2026-03-21T04:54:09</t>
         </is>
       </c>
     </row>
@@ -2723,7 +2804,7 @@
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>2026-03-21T04:52:57</t>
+          <t>2026-03-21T04:54:09</t>
         </is>
       </c>
     </row>
@@ -2760,7 +2841,7 @@
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>2026-03-21T04:52:57</t>
+          <t>2026-03-21T04:54:09</t>
         </is>
       </c>
     </row>
@@ -2797,7 +2878,7 @@
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>2026-03-21T04:52:57</t>
+          <t>2026-03-21T04:54:09</t>
         </is>
       </c>
     </row>
@@ -2834,7 +2915,7 @@
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>2026-03-21T04:52:57</t>
+          <t>2026-03-21T04:54:09</t>
         </is>
       </c>
     </row>
@@ -2846,11 +2927,11 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>삼성생명</t>
+          <t>LX인터내셔널</t>
         </is>
       </c>
       <c r="C35" t="n">
-        <v>4</v>
+        <v>20</v>
       </c>
       <c r="D35" t="inlineStr">
         <is>
@@ -2861,17 +2942,17 @@
         <v>1</v>
       </c>
       <c r="F35" t="n">
-        <v>926000</v>
+        <v>944108</v>
       </c>
       <c r="G35" t="n">
-        <v>93000</v>
+        <v>5108</v>
       </c>
       <c r="H35" t="n">
-        <v>11.16446578631453</v>
+        <v>0.5439829605963792</v>
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>2026-03-21T04:52:57</t>
+          <t>2026-03-21T04:54:09</t>
         </is>
       </c>
     </row>
@@ -2883,11 +2964,11 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>비에이치아이</t>
+          <t>삼성생명</t>
         </is>
       </c>
       <c r="C36" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="D36" t="inlineStr">
         <is>
@@ -2898,17 +2979,17 @@
         <v>1</v>
       </c>
       <c r="F36" t="n">
-        <v>876000</v>
+        <v>926000</v>
       </c>
       <c r="G36" t="n">
-        <v>210885</v>
+        <v>93000</v>
       </c>
       <c r="H36" t="n">
-        <v>31.70654698811484</v>
+        <v>11.16446578631453</v>
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>2026-03-21T04:52:57</t>
+          <t>2026-03-21T04:54:09</t>
         </is>
       </c>
     </row>
@@ -2920,11 +3001,11 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>하프니아</t>
+          <t>비에이치아이</t>
         </is>
       </c>
       <c r="C37" t="n">
-        <v>80</v>
+        <v>8</v>
       </c>
       <c r="D37" t="inlineStr">
         <is>
@@ -2935,17 +3016,17 @@
         <v>1</v>
       </c>
       <c r="F37" t="n">
-        <v>842704.775390625</v>
+        <v>876000</v>
       </c>
       <c r="G37" t="n">
-        <v>216973.775390625</v>
+        <v>210885</v>
       </c>
       <c r="H37" t="n">
-        <v>34.67524789256486</v>
+        <v>31.70654698811484</v>
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>2026-03-21T04:52:57</t>
+          <t>2026-03-21T04:54:09</t>
         </is>
       </c>
     </row>
@@ -2957,11 +3038,11 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>클리블랜드 클리프스</t>
+          <t>하프니아</t>
         </is>
       </c>
       <c r="C38" t="n">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="D38" t="inlineStr">
         <is>
@@ -2972,17 +3053,17 @@
         <v>1</v>
       </c>
       <c r="F38" t="n">
-        <v>823743.9360268187</v>
+        <v>842704.775390625</v>
       </c>
       <c r="G38" t="n">
-        <v>-192311.0639731813</v>
+        <v>216973.775390625</v>
       </c>
       <c r="H38" t="n">
-        <v>-18.92722972409774</v>
+        <v>34.67524789256486</v>
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>2026-03-21T04:52:57</t>
+          <t>2026-03-21T04:54:09</t>
         </is>
       </c>
     </row>
@@ -2994,32 +3075,143 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
+          <t>클리블랜드 클리프스</t>
+        </is>
+      </c>
+      <c r="C39" t="n">
+        <v>70</v>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E39" t="n">
+        <v>1</v>
+      </c>
+      <c r="F39" t="n">
+        <v>823743.9360268187</v>
+      </c>
+      <c r="G39" t="n">
+        <v>-192311.0639731813</v>
+      </c>
+      <c r="H39" t="n">
+        <v>-18.92722972409774</v>
+      </c>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>2026-03-21T04:54:09</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>2026-03-21</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>낫 오프쇼어 파트너스</t>
+        </is>
+      </c>
+      <c r="C40" t="n">
+        <v>30</v>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E40" t="n">
+        <v>1</v>
+      </c>
+      <c r="F40" t="n">
+        <v>410853</v>
+      </c>
+      <c r="G40" t="n">
+        <v>-6662</v>
+      </c>
+      <c r="H40" t="n">
+        <v>-1.595631294684023</v>
+      </c>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>2026-03-21T04:54:09</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>2026-03-21</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>NH투자증권우</t>
+        </is>
+      </c>
+      <c r="C41" t="n">
+        <v>2</v>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E41" t="n">
+        <v>1</v>
+      </c>
+      <c r="F41" t="n">
+        <v>54591</v>
+      </c>
+      <c r="G41" t="n">
+        <v>-9</v>
+      </c>
+      <c r="H41" t="n">
+        <v>-0.01648351648351648</v>
+      </c>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>2026-03-21T04:54:09</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>2026-03-21</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
           <t>노블</t>
         </is>
       </c>
-      <c r="C39" t="n">
+      <c r="C42" t="n">
         <v>99</v>
       </c>
-      <c r="D39" t="inlineStr">
-        <is>
-          <t>KRW</t>
-        </is>
-      </c>
-      <c r="E39" t="n">
-        <v>1</v>
-      </c>
-      <c r="F39" t="n">
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E42" t="n">
+        <v>1</v>
+      </c>
+      <c r="F42" t="n">
         <v>40689</v>
       </c>
-      <c r="G39" t="n">
+      <c r="G42" t="n">
         <v>-3866519</v>
       </c>
-      <c r="H39" t="n">
+      <c r="H42" t="n">
         <v>-98.95861699709869</v>
       </c>
-      <c r="I39" t="inlineStr">
-        <is>
-          <t>2026-03-21T04:52:57</t>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>2026-03-21T04:54:09</t>
         </is>
       </c>
     </row>
@@ -3083,7 +3275,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>2026-03-21T04:52:57</t>
+          <t>2026-03-21T04:54:09</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: portfolio snapshot 2026-03-21 (2026-03-21T04:54:11)
</commit_message>
<xml_diff>
--- a/portfolio_auto.xlsx
+++ b/portfolio_auto.xlsx
@@ -1630,7 +1630,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2026-03-21T04:54:09</t>
+          <t>2026-03-21T04:54:11</t>
         </is>
       </c>
       <c r="E2" t="n">
@@ -1731,7 +1731,7 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>2026-03-21T04:54:09</t>
+          <t>2026-03-21T04:54:11</t>
         </is>
       </c>
     </row>
@@ -1768,7 +1768,7 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>2026-03-21T04:54:09</t>
+          <t>2026-03-21T04:54:11</t>
         </is>
       </c>
     </row>
@@ -1805,7 +1805,7 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>2026-03-21T04:54:09</t>
+          <t>2026-03-21T04:54:11</t>
         </is>
       </c>
     </row>
@@ -1842,7 +1842,7 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>2026-03-21T04:54:09</t>
+          <t>2026-03-21T04:54:11</t>
         </is>
       </c>
     </row>
@@ -1879,7 +1879,7 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>2026-03-21T04:54:09</t>
+          <t>2026-03-21T04:54:11</t>
         </is>
       </c>
     </row>
@@ -1916,7 +1916,7 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>2026-03-21T04:54:09</t>
+          <t>2026-03-21T04:54:11</t>
         </is>
       </c>
     </row>
@@ -1953,7 +1953,7 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>2026-03-21T04:54:09</t>
+          <t>2026-03-21T04:54:11</t>
         </is>
       </c>
     </row>
@@ -1990,7 +1990,7 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>2026-03-21T04:54:09</t>
+          <t>2026-03-21T04:54:11</t>
         </is>
       </c>
     </row>
@@ -2027,7 +2027,7 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>2026-03-21T04:54:09</t>
+          <t>2026-03-21T04:54:11</t>
         </is>
       </c>
     </row>
@@ -2064,7 +2064,7 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>2026-03-21T04:54:09</t>
+          <t>2026-03-21T04:54:11</t>
         </is>
       </c>
     </row>
@@ -2101,7 +2101,7 @@
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>2026-03-21T04:54:09</t>
+          <t>2026-03-21T04:54:11</t>
         </is>
       </c>
     </row>
@@ -2138,7 +2138,7 @@
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>2026-03-21T04:54:09</t>
+          <t>2026-03-21T04:54:11</t>
         </is>
       </c>
     </row>
@@ -2175,7 +2175,7 @@
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>2026-03-21T04:54:09</t>
+          <t>2026-03-21T04:54:11</t>
         </is>
       </c>
     </row>
@@ -2212,7 +2212,7 @@
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>2026-03-21T04:54:09</t>
+          <t>2026-03-21T04:54:11</t>
         </is>
       </c>
     </row>
@@ -2249,7 +2249,7 @@
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>2026-03-21T04:54:09</t>
+          <t>2026-03-21T04:54:11</t>
         </is>
       </c>
     </row>
@@ -2286,7 +2286,7 @@
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>2026-03-21T04:54:09</t>
+          <t>2026-03-21T04:54:11</t>
         </is>
       </c>
     </row>
@@ -2323,7 +2323,7 @@
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>2026-03-21T04:54:09</t>
+          <t>2026-03-21T04:54:11</t>
         </is>
       </c>
     </row>
@@ -2360,7 +2360,7 @@
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>2026-03-21T04:54:09</t>
+          <t>2026-03-21T04:54:11</t>
         </is>
       </c>
     </row>
@@ -2397,7 +2397,7 @@
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>2026-03-21T04:54:09</t>
+          <t>2026-03-21T04:54:11</t>
         </is>
       </c>
     </row>
@@ -2434,7 +2434,7 @@
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>2026-03-21T04:54:09</t>
+          <t>2026-03-21T04:54:11</t>
         </is>
       </c>
     </row>
@@ -2471,7 +2471,7 @@
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>2026-03-21T04:54:09</t>
+          <t>2026-03-21T04:54:11</t>
         </is>
       </c>
     </row>
@@ -2508,7 +2508,7 @@
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>2026-03-21T04:54:09</t>
+          <t>2026-03-21T04:54:11</t>
         </is>
       </c>
     </row>
@@ -2545,7 +2545,7 @@
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>2026-03-21T04:54:09</t>
+          <t>2026-03-21T04:54:11</t>
         </is>
       </c>
     </row>
@@ -2582,7 +2582,7 @@
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>2026-03-21T04:54:09</t>
+          <t>2026-03-21T04:54:11</t>
         </is>
       </c>
     </row>
@@ -2619,7 +2619,7 @@
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>2026-03-21T04:54:09</t>
+          <t>2026-03-21T04:54:11</t>
         </is>
       </c>
     </row>
@@ -2656,7 +2656,7 @@
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>2026-03-21T04:54:09</t>
+          <t>2026-03-21T04:54:11</t>
         </is>
       </c>
     </row>
@@ -2693,7 +2693,7 @@
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>2026-03-21T04:54:09</t>
+          <t>2026-03-21T04:54:11</t>
         </is>
       </c>
     </row>
@@ -2730,7 +2730,7 @@
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>2026-03-21T04:54:09</t>
+          <t>2026-03-21T04:54:11</t>
         </is>
       </c>
     </row>
@@ -2767,7 +2767,7 @@
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>2026-03-21T04:54:09</t>
+          <t>2026-03-21T04:54:11</t>
         </is>
       </c>
     </row>
@@ -2804,7 +2804,7 @@
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>2026-03-21T04:54:09</t>
+          <t>2026-03-21T04:54:11</t>
         </is>
       </c>
     </row>
@@ -2841,7 +2841,7 @@
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>2026-03-21T04:54:09</t>
+          <t>2026-03-21T04:54:11</t>
         </is>
       </c>
     </row>
@@ -2878,7 +2878,7 @@
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>2026-03-21T04:54:09</t>
+          <t>2026-03-21T04:54:11</t>
         </is>
       </c>
     </row>
@@ -2915,7 +2915,7 @@
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>2026-03-21T04:54:09</t>
+          <t>2026-03-21T04:54:11</t>
         </is>
       </c>
     </row>
@@ -2952,7 +2952,7 @@
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>2026-03-21T04:54:09</t>
+          <t>2026-03-21T04:54:11</t>
         </is>
       </c>
     </row>
@@ -2989,7 +2989,7 @@
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>2026-03-21T04:54:09</t>
+          <t>2026-03-21T04:54:11</t>
         </is>
       </c>
     </row>
@@ -3026,7 +3026,7 @@
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>2026-03-21T04:54:09</t>
+          <t>2026-03-21T04:54:11</t>
         </is>
       </c>
     </row>
@@ -3063,7 +3063,7 @@
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>2026-03-21T04:54:09</t>
+          <t>2026-03-21T04:54:11</t>
         </is>
       </c>
     </row>
@@ -3100,7 +3100,7 @@
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>2026-03-21T04:54:09</t>
+          <t>2026-03-21T04:54:11</t>
         </is>
       </c>
     </row>
@@ -3137,7 +3137,7 @@
       </c>
       <c r="I40" t="inlineStr">
         <is>
-          <t>2026-03-21T04:54:09</t>
+          <t>2026-03-21T04:54:11</t>
         </is>
       </c>
     </row>
@@ -3174,7 +3174,7 @@
       </c>
       <c r="I41" t="inlineStr">
         <is>
-          <t>2026-03-21T04:54:09</t>
+          <t>2026-03-21T04:54:11</t>
         </is>
       </c>
     </row>
@@ -3211,7 +3211,7 @@
       </c>
       <c r="I42" t="inlineStr">
         <is>
-          <t>2026-03-21T04:54:09</t>
+          <t>2026-03-21T04:54:11</t>
         </is>
       </c>
     </row>
@@ -3275,7 +3275,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>2026-03-21T04:54:09</t>
+          <t>2026-03-21T04:54:11</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: portfolio snapshot 2026-03-21 (2026-03-21T04:54:36)
</commit_message>
<xml_diff>
--- a/portfolio_auto.xlsx
+++ b/portfolio_auto.xlsx
@@ -525,11 +525,11 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>넥스틸</t>
+          <t>센트러스 에너지</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>200</v>
+        <v>25</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
@@ -540,23 +540,23 @@
         <v>1</v>
       </c>
       <c r="E4" t="n">
-        <v>2514000</v>
+        <v>7026050.85816239</v>
       </c>
       <c r="F4" t="n">
-        <v>503000</v>
+        <v>-406805.1418376099</v>
       </c>
       <c r="G4" t="n">
-        <v>25.01243162605669</v>
+        <v>-5.473066366920198</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>대신증권</t>
+          <t>스타 벌크 캐리어스</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>55</v>
+        <v>50</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -567,23 +567,23 @@
         <v>1</v>
       </c>
       <c r="E5" t="n">
-        <v>2219250</v>
+        <v>1680142.640194588</v>
       </c>
       <c r="F5" t="n">
-        <v>509749</v>
+        <v>365789.6401945879</v>
       </c>
       <c r="G5" t="n">
-        <v>29.81858448752005</v>
+        <v>27.83039565433242</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>대창단조</t>
+          <t>시드릴</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>300</v>
+        <v>123</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
@@ -594,23 +594,23 @@
         <v>1</v>
       </c>
       <c r="E6" t="n">
-        <v>2004000</v>
+        <v>8070101.805898919</v>
       </c>
       <c r="F6" t="n">
-        <v>-54000</v>
+        <v>1619750.805898919</v>
       </c>
       <c r="G6" t="n">
-        <v>-2.623906705539359</v>
+        <v>25.11104908707943</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>대한조선</t>
+          <t>오케아니스 에코 탱커스</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>100</v>
+        <v>65</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -621,23 +621,23 @@
         <v>1</v>
       </c>
       <c r="E7" t="n">
-        <v>9120000</v>
+        <v>4511179.137784176</v>
       </c>
       <c r="F7" t="n">
-        <v>1907000</v>
+        <v>2254819.137784176</v>
       </c>
       <c r="G7" t="n">
-        <v>26.43837515596839</v>
+        <v>99.93171026716374</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>동방</t>
+          <t>차코스 에너지 내비게이션</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>681</v>
+        <v>75</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
@@ -648,23 +648,23 @@
         <v>1</v>
       </c>
       <c r="E8" t="n">
-        <v>1995330</v>
+        <v>4026924.996845168</v>
       </c>
       <c r="F8" t="n">
-        <v>23829</v>
+        <v>202276.9968451681</v>
       </c>
       <c r="G8" t="n">
-        <v>1.208672985709873</v>
+        <v>5.28877420471552</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>동원개발</t>
+          <t>클리블랜드 클리프스</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>1360</v>
+        <v>70</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
@@ -675,23 +675,23 @@
         <v>1</v>
       </c>
       <c r="E9" t="n">
-        <v>4202400</v>
+        <v>823743.9360268187</v>
       </c>
       <c r="F9" t="n">
-        <v>465000</v>
+        <v>-192311.0639731813</v>
       </c>
       <c r="G9" t="n">
-        <v>12.44180446299566</v>
+        <v>-18.92722972409774</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>미창석유</t>
+          <t>타이드워터</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>18</v>
+        <v>48</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
@@ -702,23 +702,23 @@
         <v>1</v>
       </c>
       <c r="E10" t="n">
-        <v>2097000</v>
+        <v>5235363.852789983</v>
       </c>
       <c r="F10" t="n">
-        <v>-295200</v>
+        <v>1510818.852789983</v>
       </c>
       <c r="G10" t="n">
-        <v>-12.34010534236268</v>
+        <v>40.56385015592463</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>비에이치아이</t>
+          <t>텍사스 퍼시픽 랜드</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
@@ -729,23 +729,23 @@
         <v>1</v>
       </c>
       <c r="E11" t="n">
-        <v>876000</v>
+        <v>1563247.374122903</v>
       </c>
       <c r="F11" t="n">
-        <v>210885</v>
+        <v>-14646.62587709725</v>
       </c>
       <c r="G11" t="n">
-        <v>31.70654698811484</v>
+        <v>-0.9282388979929735</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>삼성생명</t>
+          <t>트랜스오션</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>4</v>
+        <v>750</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
@@ -756,23 +756,23 @@
         <v>1</v>
       </c>
       <c r="E12" t="n">
-        <v>926000</v>
+        <v>7020031.5082007</v>
       </c>
       <c r="F12" t="n">
-        <v>93000</v>
+        <v>2892797.5082007</v>
       </c>
       <c r="G12" t="n">
-        <v>11.16446578631453</v>
+        <v>70.09046514446965</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>삼성화재</t>
+          <t>페트로브라스 (ADR)</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>7</v>
+        <v>480</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
@@ -783,23 +783,23 @@
         <v>1</v>
       </c>
       <c r="E13" t="n">
-        <v>3321500</v>
+        <v>13579584.97235231</v>
       </c>
       <c r="F13" t="n">
-        <v>-309500</v>
+        <v>1473035.972352311</v>
       </c>
       <c r="G13" t="n">
-        <v>-8.523822638391627</v>
+        <v>12.16726560436265</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>세아제강</t>
+          <t>프론트라인</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>50</v>
+        <v>175</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
@@ -810,23 +810,23 @@
         <v>1</v>
       </c>
       <c r="E14" t="n">
-        <v>7395000</v>
+        <v>8471815.962899337</v>
       </c>
       <c r="F14" t="n">
-        <v>1085000</v>
+        <v>4041951.962899337</v>
       </c>
       <c r="G14" t="n">
-        <v>17.19492868462758</v>
+        <v>91.24325177701475</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>케이씨</t>
+          <t>피바디 에너지</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>50</v>
+        <v>65</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
@@ -837,23 +837,23 @@
         <v>1</v>
       </c>
       <c r="E15" t="n">
-        <v>1670000</v>
+        <v>3649438.50225304</v>
       </c>
       <c r="F15" t="n">
-        <v>20500</v>
+        <v>2178666.50225304</v>
       </c>
       <c r="G15" t="n">
-        <v>1.242800848742043</v>
+        <v>148.1308117269733</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>하나금융지주</t>
+          <t>하프니아</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>10</v>
+        <v>80</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
@@ -864,23 +864,23 @@
         <v>1</v>
       </c>
       <c r="E16" t="n">
-        <v>1132000</v>
+        <v>842704.775390625</v>
       </c>
       <c r="F16" t="n">
-        <v>23000</v>
+        <v>216973.775390625</v>
       </c>
       <c r="G16" t="n">
-        <v>2.073940486925157</v>
+        <v>34.67524789256486</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>현대제철</t>
+          <t>DL이앤씨</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>70</v>
+        <v>40</v>
       </c>
       <c r="C17" t="inlineStr">
         <is>
@@ -891,23 +891,23 @@
         <v>1</v>
       </c>
       <c r="E17" t="n">
-        <v>2621500</v>
+        <v>2696000</v>
       </c>
       <c r="F17" t="n">
-        <v>-186000</v>
+        <v>990500</v>
       </c>
       <c r="G17" t="n">
-        <v>-6.625111308993767</v>
+        <v>58.07681031955438</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>휴스틸</t>
+          <t>HD건설기계</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>500</v>
+        <v>31</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
@@ -918,23 +918,23 @@
         <v>1</v>
       </c>
       <c r="E18" t="n">
-        <v>2750000</v>
+        <v>4123000</v>
       </c>
       <c r="F18" t="n">
-        <v>471390</v>
+        <v>87904</v>
       </c>
       <c r="G18" t="n">
-        <v>20.68761218462133</v>
+        <v>2.178485964150543</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>센트러스 에너지</t>
+          <t>KoAct 코스닥액티브</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>25</v>
+        <v>200</v>
       </c>
       <c r="C19" t="inlineStr">
         <is>
@@ -945,23 +945,23 @@
         <v>1</v>
       </c>
       <c r="E19" t="n">
-        <v>7026050.85816239</v>
+        <v>2582000</v>
       </c>
       <c r="F19" t="n">
-        <v>-406805.1418376099</v>
+        <v>-120000</v>
       </c>
       <c r="G19" t="n">
-        <v>-5.473066366920198</v>
+        <v>-4.441154700222058</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>스타 벌크 캐리어스</t>
+          <t>LX인터내셔널</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>50</v>
+        <v>20</v>
       </c>
       <c r="C20" t="inlineStr">
         <is>
@@ -972,23 +972,23 @@
         <v>1</v>
       </c>
       <c r="E20" t="n">
-        <v>1680142.640194588</v>
+        <v>944108</v>
       </c>
       <c r="F20" t="n">
-        <v>365789.6401945879</v>
+        <v>5108</v>
       </c>
       <c r="G20" t="n">
-        <v>27.83039565433242</v>
+        <v>0.5439829605963792</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>시드릴</t>
+          <t>NH투자증권우</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>123</v>
+        <v>2</v>
       </c>
       <c r="C21" t="inlineStr">
         <is>
@@ -999,23 +999,23 @@
         <v>1</v>
       </c>
       <c r="E21" t="n">
-        <v>8070101.805898919</v>
+        <v>54591</v>
       </c>
       <c r="F21" t="n">
-        <v>1619750.805898919</v>
+        <v>-9</v>
       </c>
       <c r="G21" t="n">
-        <v>25.11104908707943</v>
+        <v>-0.01648351648351648</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>오케아니스 에코 탱커스</t>
+          <t>TIME 코리아밸류업액티브</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>65</v>
+        <v>201</v>
       </c>
       <c r="C22" t="inlineStr">
         <is>
@@ -1026,23 +1026,23 @@
         <v>1</v>
       </c>
       <c r="E22" t="n">
-        <v>4511179.137784176</v>
+        <v>4797870</v>
       </c>
       <c r="F22" t="n">
-        <v>2254819.137784176</v>
+        <v>74073</v>
       </c>
       <c r="G22" t="n">
-        <v>99.93171026716374</v>
+        <v>1.568081778281328</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>차코스 에너지 내비게이션</t>
+          <t>노브</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>75</v>
+        <v>185</v>
       </c>
       <c r="C23" t="inlineStr">
         <is>
@@ -1053,23 +1053,23 @@
         <v>1</v>
       </c>
       <c r="E23" t="n">
-        <v>4026924.996845168</v>
+        <v>5200391.447092756</v>
       </c>
       <c r="F23" t="n">
-        <v>202276.9968451681</v>
+        <v>1890383.447092756</v>
       </c>
       <c r="G23" t="n">
-        <v>5.28877420471552</v>
+        <v>57.11114435653194</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>클리블랜드 클리프스</t>
+          <t>노블</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>70</v>
+        <v>99</v>
       </c>
       <c r="C24" t="inlineStr">
         <is>
@@ -1080,23 +1080,23 @@
         <v>1</v>
       </c>
       <c r="E24" t="n">
-        <v>823743.9360268187</v>
+        <v>40689</v>
       </c>
       <c r="F24" t="n">
-        <v>-192311.0639731813</v>
+        <v>-3866519</v>
       </c>
       <c r="G24" t="n">
-        <v>-18.92722972409774</v>
+        <v>-98.95861699709869</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>타이드워터</t>
+          <t>낫 오프쇼어 파트너스</t>
         </is>
       </c>
       <c r="B25" t="n">
-        <v>48</v>
+        <v>30</v>
       </c>
       <c r="C25" t="inlineStr">
         <is>
@@ -1107,23 +1107,23 @@
         <v>1</v>
       </c>
       <c r="E25" t="n">
-        <v>5235363.852789983</v>
+        <v>410853</v>
       </c>
       <c r="F25" t="n">
-        <v>1510818.852789983</v>
+        <v>-6662</v>
       </c>
       <c r="G25" t="n">
-        <v>40.56385015592463</v>
+        <v>-1.595631294684023</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>텍사스 퍼시픽 랜드</t>
+          <t>더치 브로스</t>
         </is>
       </c>
       <c r="B26" t="n">
-        <v>2</v>
+        <v>39</v>
       </c>
       <c r="C26" t="inlineStr">
         <is>
@@ -1134,23 +1134,23 @@
         <v>1</v>
       </c>
       <c r="E26" t="n">
-        <v>1563247.374122903</v>
+        <v>2934418.414306641</v>
       </c>
       <c r="F26" t="n">
-        <v>-14646.62587709725</v>
+        <v>-256226.5856933594</v>
       </c>
       <c r="G26" t="n">
-        <v>-0.9282388979929735</v>
+        <v>-8.030557636257226</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>트랜스오션</t>
+          <t>발레로 에너지</t>
         </is>
       </c>
       <c r="B27" t="n">
-        <v>750</v>
+        <v>6</v>
       </c>
       <c r="C27" t="inlineStr">
         <is>
@@ -1161,23 +1161,23 @@
         <v>1</v>
       </c>
       <c r="E27" t="n">
-        <v>7020031.5082007</v>
+        <v>2165691.085066516</v>
       </c>
       <c r="F27" t="n">
-        <v>2892797.5082007</v>
+        <v>101701.085066516</v>
       </c>
       <c r="G27" t="n">
-        <v>70.09046514446965</v>
+        <v>4.927402025519307</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>페트로브라스 (ADR)</t>
+          <t>넥스틸</t>
         </is>
       </c>
       <c r="B28" t="n">
-        <v>480</v>
+        <v>300</v>
       </c>
       <c r="C28" t="inlineStr">
         <is>
@@ -1188,23 +1188,23 @@
         <v>1</v>
       </c>
       <c r="E28" t="n">
-        <v>13579584.97235231</v>
+        <v>3771000</v>
       </c>
       <c r="F28" t="n">
-        <v>1473035.972352311</v>
+        <v>521000</v>
       </c>
       <c r="G28" t="n">
-        <v>12.16726560436265</v>
+        <v>16.03076923076923</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>프론트라인</t>
+          <t>대신증권</t>
         </is>
       </c>
       <c r="B29" t="n">
-        <v>175</v>
+        <v>55</v>
       </c>
       <c r="C29" t="inlineStr">
         <is>
@@ -1215,23 +1215,23 @@
         <v>1</v>
       </c>
       <c r="E29" t="n">
-        <v>8471815.962899337</v>
+        <v>2219250</v>
       </c>
       <c r="F29" t="n">
-        <v>4041951.962899337</v>
+        <v>509749</v>
       </c>
       <c r="G29" t="n">
-        <v>91.24325177701475</v>
+        <v>29.81858448752005</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>피바디 에너지</t>
+          <t>대창단조</t>
         </is>
       </c>
       <c r="B30" t="n">
-        <v>65</v>
+        <v>300</v>
       </c>
       <c r="C30" t="inlineStr">
         <is>
@@ -1242,23 +1242,23 @@
         <v>1</v>
       </c>
       <c r="E30" t="n">
-        <v>3649438.50225304</v>
+        <v>2004000</v>
       </c>
       <c r="F30" t="n">
-        <v>2178666.50225304</v>
+        <v>-54000</v>
       </c>
       <c r="G30" t="n">
-        <v>148.1308117269733</v>
+        <v>-2.623906705539359</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>하프니아</t>
+          <t>대한조선</t>
         </is>
       </c>
       <c r="B31" t="n">
-        <v>80</v>
+        <v>100</v>
       </c>
       <c r="C31" t="inlineStr">
         <is>
@@ -1269,23 +1269,23 @@
         <v>1</v>
       </c>
       <c r="E31" t="n">
-        <v>842704.775390625</v>
+        <v>9120000</v>
       </c>
       <c r="F31" t="n">
-        <v>216973.775390625</v>
+        <v>1907000</v>
       </c>
       <c r="G31" t="n">
-        <v>34.67524789256486</v>
+        <v>26.43837515596839</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>DL이앤씨</t>
+          <t>동방</t>
         </is>
       </c>
       <c r="B32" t="n">
-        <v>40</v>
+        <v>681</v>
       </c>
       <c r="C32" t="inlineStr">
         <is>
@@ -1296,23 +1296,23 @@
         <v>1</v>
       </c>
       <c r="E32" t="n">
-        <v>2696000</v>
+        <v>1995330</v>
       </c>
       <c r="F32" t="n">
-        <v>990500</v>
+        <v>23829</v>
       </c>
       <c r="G32" t="n">
-        <v>58.07681031955438</v>
+        <v>1.208672985709873</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>HD건설기계</t>
+          <t>동원개발</t>
         </is>
       </c>
       <c r="B33" t="n">
-        <v>31</v>
+        <v>1360</v>
       </c>
       <c r="C33" t="inlineStr">
         <is>
@@ -1323,23 +1323,23 @@
         <v>1</v>
       </c>
       <c r="E33" t="n">
-        <v>4123000</v>
+        <v>4202400</v>
       </c>
       <c r="F33" t="n">
-        <v>87904</v>
+        <v>465000</v>
       </c>
       <c r="G33" t="n">
-        <v>2.178485964150543</v>
+        <v>12.44180446299566</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>KoAct 코스닥액티브</t>
+          <t>미창석유</t>
         </is>
       </c>
       <c r="B34" t="n">
-        <v>200</v>
+        <v>18</v>
       </c>
       <c r="C34" t="inlineStr">
         <is>
@@ -1350,23 +1350,23 @@
         <v>1</v>
       </c>
       <c r="E34" t="n">
-        <v>2582000</v>
+        <v>2097000</v>
       </c>
       <c r="F34" t="n">
-        <v>-120000</v>
+        <v>-295200</v>
       </c>
       <c r="G34" t="n">
-        <v>-4.441154700222058</v>
+        <v>-12.34010534236268</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>LX인터내셔널</t>
+          <t>비에이치아이</t>
         </is>
       </c>
       <c r="B35" t="n">
-        <v>20</v>
+        <v>8</v>
       </c>
       <c r="C35" t="inlineStr">
         <is>
@@ -1377,23 +1377,23 @@
         <v>1</v>
       </c>
       <c r="E35" t="n">
-        <v>944108</v>
+        <v>876000</v>
       </c>
       <c r="F35" t="n">
-        <v>5108</v>
+        <v>210885</v>
       </c>
       <c r="G35" t="n">
-        <v>0.5439829605963792</v>
+        <v>31.70654698811484</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>NH투자증권우</t>
+          <t>삼성생명</t>
         </is>
       </c>
       <c r="B36" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="C36" t="inlineStr">
         <is>
@@ -1404,23 +1404,23 @@
         <v>1</v>
       </c>
       <c r="E36" t="n">
-        <v>54591</v>
+        <v>926000</v>
       </c>
       <c r="F36" t="n">
-        <v>-9</v>
+        <v>93000</v>
       </c>
       <c r="G36" t="n">
-        <v>-0.01648351648351648</v>
+        <v>11.16446578631453</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>TIME 코리아밸류업액티브</t>
+          <t>삼성화재</t>
         </is>
       </c>
       <c r="B37" t="n">
-        <v>201</v>
+        <v>9</v>
       </c>
       <c r="C37" t="inlineStr">
         <is>
@@ -1431,23 +1431,23 @@
         <v>1</v>
       </c>
       <c r="E37" t="n">
-        <v>4797870</v>
+        <v>4270500</v>
       </c>
       <c r="F37" t="n">
-        <v>74073</v>
+        <v>-360500</v>
       </c>
       <c r="G37" t="n">
-        <v>1.568081778281328</v>
+        <v>-7.784495789246384</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>노브</t>
+          <t>세아제강</t>
         </is>
       </c>
       <c r="B38" t="n">
-        <v>185</v>
+        <v>50</v>
       </c>
       <c r="C38" t="inlineStr">
         <is>
@@ -1458,23 +1458,23 @@
         <v>1</v>
       </c>
       <c r="E38" t="n">
-        <v>5200391.447092756</v>
+        <v>7395000</v>
       </c>
       <c r="F38" t="n">
-        <v>1890383.447092756</v>
+        <v>1085000</v>
       </c>
       <c r="G38" t="n">
-        <v>57.11114435653194</v>
+        <v>17.19492868462758</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>노블</t>
+          <t>케이씨</t>
         </is>
       </c>
       <c r="B39" t="n">
-        <v>99</v>
+        <v>50</v>
       </c>
       <c r="C39" t="inlineStr">
         <is>
@@ -1485,23 +1485,23 @@
         <v>1</v>
       </c>
       <c r="E39" t="n">
-        <v>40689</v>
+        <v>1670000</v>
       </c>
       <c r="F39" t="n">
-        <v>-3866519</v>
+        <v>20500</v>
       </c>
       <c r="G39" t="n">
-        <v>-98.95861699709869</v>
+        <v>1.242800848742043</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>낫 오프쇼어 파트너스</t>
+          <t>하나금융지주</t>
         </is>
       </c>
       <c r="B40" t="n">
-        <v>30</v>
+        <v>18</v>
       </c>
       <c r="C40" t="inlineStr">
         <is>
@@ -1512,23 +1512,23 @@
         <v>1</v>
       </c>
       <c r="E40" t="n">
-        <v>410853</v>
+        <v>2037600</v>
       </c>
       <c r="F40" t="n">
-        <v>-6662</v>
+        <v>12200</v>
       </c>
       <c r="G40" t="n">
-        <v>-1.595631294684023</v>
+        <v>0.6023501530561864</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>더치 브로스</t>
+          <t>현대제철</t>
         </is>
       </c>
       <c r="B41" t="n">
-        <v>39</v>
+        <v>80</v>
       </c>
       <c r="C41" t="inlineStr">
         <is>
@@ -1539,23 +1539,23 @@
         <v>1</v>
       </c>
       <c r="E41" t="n">
-        <v>2934418.414306641</v>
+        <v>2996000</v>
       </c>
       <c r="F41" t="n">
-        <v>-256226.5856933594</v>
+        <v>-182000</v>
       </c>
       <c r="G41" t="n">
-        <v>-8.030557636257226</v>
+        <v>-5.726872246696035</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>발레로 에너지</t>
+          <t>휴스틸</t>
         </is>
       </c>
       <c r="B42" t="n">
-        <v>6</v>
+        <v>500</v>
       </c>
       <c r="C42" t="inlineStr">
         <is>
@@ -1566,13 +1566,13 @@
         <v>1</v>
       </c>
       <c r="E42" t="n">
-        <v>2165691.085066516</v>
+        <v>2750000</v>
       </c>
       <c r="F42" t="n">
-        <v>101701.085066516</v>
+        <v>471390</v>
       </c>
       <c r="G42" t="n">
-        <v>4.927402025519307</v>
+        <v>20.68761218462133</v>
       </c>
     </row>
   </sheetData>
@@ -1630,7 +1630,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2026-03-21T04:54:11</t>
+          <t>2026-03-21T04:54:36</t>
         </is>
       </c>
       <c r="E2" t="n">
@@ -1731,7 +1731,7 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>2026-03-21T04:54:11</t>
+          <t>2026-03-21T04:54:36</t>
         </is>
       </c>
     </row>
@@ -1768,7 +1768,7 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>2026-03-21T04:54:11</t>
+          <t>2026-03-21T04:54:36</t>
         </is>
       </c>
     </row>
@@ -1805,7 +1805,7 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>2026-03-21T04:54:11</t>
+          <t>2026-03-21T04:54:36</t>
         </is>
       </c>
     </row>
@@ -1842,7 +1842,7 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>2026-03-21T04:54:11</t>
+          <t>2026-03-21T04:54:36</t>
         </is>
       </c>
     </row>
@@ -1879,7 +1879,7 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>2026-03-21T04:54:11</t>
+          <t>2026-03-21T04:54:36</t>
         </is>
       </c>
     </row>
@@ -1916,7 +1916,7 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>2026-03-21T04:54:11</t>
+          <t>2026-03-21T04:54:36</t>
         </is>
       </c>
     </row>
@@ -1953,7 +1953,7 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>2026-03-21T04:54:11</t>
+          <t>2026-03-21T04:54:36</t>
         </is>
       </c>
     </row>
@@ -1990,7 +1990,7 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>2026-03-21T04:54:11</t>
+          <t>2026-03-21T04:54:36</t>
         </is>
       </c>
     </row>
@@ -2027,7 +2027,7 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>2026-03-21T04:54:11</t>
+          <t>2026-03-21T04:54:36</t>
         </is>
       </c>
     </row>
@@ -2064,7 +2064,7 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>2026-03-21T04:54:11</t>
+          <t>2026-03-21T04:54:36</t>
         </is>
       </c>
     </row>
@@ -2101,7 +2101,7 @@
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>2026-03-21T04:54:11</t>
+          <t>2026-03-21T04:54:36</t>
         </is>
       </c>
     </row>
@@ -2138,7 +2138,7 @@
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>2026-03-21T04:54:11</t>
+          <t>2026-03-21T04:54:36</t>
         </is>
       </c>
     </row>
@@ -2150,11 +2150,11 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>동원개발</t>
+          <t>삼성화재</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>1360</v>
+        <v>9</v>
       </c>
       <c r="D14" t="inlineStr">
         <is>
@@ -2165,17 +2165,17 @@
         <v>1</v>
       </c>
       <c r="F14" t="n">
-        <v>4202400</v>
+        <v>4270500</v>
       </c>
       <c r="G14" t="n">
-        <v>465000</v>
+        <v>-360500</v>
       </c>
       <c r="H14" t="n">
-        <v>12.44180446299566</v>
+        <v>-7.784495789246384</v>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>2026-03-21T04:54:11</t>
+          <t>2026-03-21T04:54:36</t>
         </is>
       </c>
     </row>
@@ -2187,11 +2187,11 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>HD건설기계</t>
+          <t>동원개발</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>31</v>
+        <v>1360</v>
       </c>
       <c r="D15" t="inlineStr">
         <is>
@@ -2202,17 +2202,17 @@
         <v>1</v>
       </c>
       <c r="F15" t="n">
-        <v>4123000</v>
+        <v>4202400</v>
       </c>
       <c r="G15" t="n">
-        <v>87904</v>
+        <v>465000</v>
       </c>
       <c r="H15" t="n">
-        <v>2.178485964150543</v>
+        <v>12.44180446299566</v>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>2026-03-21T04:54:11</t>
+          <t>2026-03-21T04:54:36</t>
         </is>
       </c>
     </row>
@@ -2224,11 +2224,11 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>차코스 에너지 내비게이션</t>
+          <t>HD건설기계</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>75</v>
+        <v>31</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
@@ -2239,17 +2239,17 @@
         <v>1</v>
       </c>
       <c r="F16" t="n">
-        <v>4026924.996845168</v>
+        <v>4123000</v>
       </c>
       <c r="G16" t="n">
-        <v>202276.9968451681</v>
+        <v>87904</v>
       </c>
       <c r="H16" t="n">
-        <v>5.28877420471552</v>
+        <v>2.178485964150543</v>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>2026-03-21T04:54:11</t>
+          <t>2026-03-21T04:54:36</t>
         </is>
       </c>
     </row>
@@ -2261,11 +2261,11 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>피바디 에너지</t>
+          <t>차코스 에너지 내비게이션</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>65</v>
+        <v>75</v>
       </c>
       <c r="D17" t="inlineStr">
         <is>
@@ -2276,17 +2276,17 @@
         <v>1</v>
       </c>
       <c r="F17" t="n">
-        <v>3649438.50225304</v>
+        <v>4026924.996845168</v>
       </c>
       <c r="G17" t="n">
-        <v>2178666.50225304</v>
+        <v>202276.9968451681</v>
       </c>
       <c r="H17" t="n">
-        <v>148.1308117269733</v>
+        <v>5.28877420471552</v>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>2026-03-21T04:54:11</t>
+          <t>2026-03-21T04:54:36</t>
         </is>
       </c>
     </row>
@@ -2298,11 +2298,11 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>삼성화재</t>
+          <t>넥스틸</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>7</v>
+        <v>300</v>
       </c>
       <c r="D18" t="inlineStr">
         <is>
@@ -2313,17 +2313,17 @@
         <v>1</v>
       </c>
       <c r="F18" t="n">
-        <v>3321500</v>
+        <v>3771000</v>
       </c>
       <c r="G18" t="n">
-        <v>-309500</v>
+        <v>521000</v>
       </c>
       <c r="H18" t="n">
-        <v>-8.523822638391627</v>
+        <v>16.03076923076923</v>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>2026-03-21T04:54:11</t>
+          <t>2026-03-21T04:54:36</t>
         </is>
       </c>
     </row>
@@ -2335,11 +2335,11 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>더치 브로스</t>
+          <t>피바디 에너지</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>39</v>
+        <v>65</v>
       </c>
       <c r="D19" t="inlineStr">
         <is>
@@ -2350,17 +2350,17 @@
         <v>1</v>
       </c>
       <c r="F19" t="n">
-        <v>2934418.414306641</v>
+        <v>3649438.50225304</v>
       </c>
       <c r="G19" t="n">
-        <v>-256226.5856933594</v>
+        <v>2178666.50225304</v>
       </c>
       <c r="H19" t="n">
-        <v>-8.030557636257226</v>
+        <v>148.1308117269733</v>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>2026-03-21T04:54:11</t>
+          <t>2026-03-21T04:54:36</t>
         </is>
       </c>
     </row>
@@ -2372,11 +2372,11 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>휴스틸</t>
+          <t>현대제철</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>500</v>
+        <v>80</v>
       </c>
       <c r="D20" t="inlineStr">
         <is>
@@ -2387,17 +2387,17 @@
         <v>1</v>
       </c>
       <c r="F20" t="n">
-        <v>2750000</v>
+        <v>2996000</v>
       </c>
       <c r="G20" t="n">
-        <v>471390</v>
+        <v>-182000</v>
       </c>
       <c r="H20" t="n">
-        <v>20.68761218462133</v>
+        <v>-5.726872246696035</v>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>2026-03-21T04:54:11</t>
+          <t>2026-03-21T04:54:36</t>
         </is>
       </c>
     </row>
@@ -2409,11 +2409,11 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>DL이앤씨</t>
+          <t>더치 브로스</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D21" t="inlineStr">
         <is>
@@ -2424,17 +2424,17 @@
         <v>1</v>
       </c>
       <c r="F21" t="n">
-        <v>2696000</v>
+        <v>2934418.414306641</v>
       </c>
       <c r="G21" t="n">
-        <v>990500</v>
+        <v>-256226.5856933594</v>
       </c>
       <c r="H21" t="n">
-        <v>58.07681031955438</v>
+        <v>-8.030557636257226</v>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>2026-03-21T04:54:11</t>
+          <t>2026-03-21T04:54:36</t>
         </is>
       </c>
     </row>
@@ -2446,11 +2446,11 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>현대제철</t>
+          <t>휴스틸</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>70</v>
+        <v>500</v>
       </c>
       <c r="D22" t="inlineStr">
         <is>
@@ -2461,17 +2461,17 @@
         <v>1</v>
       </c>
       <c r="F22" t="n">
-        <v>2621500</v>
+        <v>2750000</v>
       </c>
       <c r="G22" t="n">
-        <v>-186000</v>
+        <v>471390</v>
       </c>
       <c r="H22" t="n">
-        <v>-6.625111308993767</v>
+        <v>20.68761218462133</v>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>2026-03-21T04:54:11</t>
+          <t>2026-03-21T04:54:36</t>
         </is>
       </c>
     </row>
@@ -2483,11 +2483,11 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>KoAct 코스닥액티브</t>
+          <t>DL이앤씨</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>200</v>
+        <v>40</v>
       </c>
       <c r="D23" t="inlineStr">
         <is>
@@ -2498,17 +2498,17 @@
         <v>1</v>
       </c>
       <c r="F23" t="n">
-        <v>2582000</v>
+        <v>2696000</v>
       </c>
       <c r="G23" t="n">
-        <v>-120000</v>
+        <v>990500</v>
       </c>
       <c r="H23" t="n">
-        <v>-4.441154700222058</v>
+        <v>58.07681031955438</v>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>2026-03-21T04:54:11</t>
+          <t>2026-03-21T04:54:36</t>
         </is>
       </c>
     </row>
@@ -2520,7 +2520,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>넥스틸</t>
+          <t>KoAct 코스닥액티브</t>
         </is>
       </c>
       <c r="C24" t="n">
@@ -2535,17 +2535,17 @@
         <v>1</v>
       </c>
       <c r="F24" t="n">
-        <v>2514000</v>
+        <v>2582000</v>
       </c>
       <c r="G24" t="n">
-        <v>503000</v>
+        <v>-120000</v>
       </c>
       <c r="H24" t="n">
-        <v>25.01243162605669</v>
+        <v>-4.441154700222058</v>
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>2026-03-21T04:54:11</t>
+          <t>2026-03-21T04:54:36</t>
         </is>
       </c>
     </row>
@@ -2582,7 +2582,7 @@
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>2026-03-21T04:54:11</t>
+          <t>2026-03-21T04:54:36</t>
         </is>
       </c>
     </row>
@@ -2619,7 +2619,7 @@
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>2026-03-21T04:54:11</t>
+          <t>2026-03-21T04:54:36</t>
         </is>
       </c>
     </row>
@@ -2656,7 +2656,7 @@
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>2026-03-21T04:54:11</t>
+          <t>2026-03-21T04:54:36</t>
         </is>
       </c>
     </row>
@@ -2668,11 +2668,11 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>대창단조</t>
+          <t>하나금융지주</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>300</v>
+        <v>18</v>
       </c>
       <c r="D28" t="inlineStr">
         <is>
@@ -2683,17 +2683,17 @@
         <v>1</v>
       </c>
       <c r="F28" t="n">
-        <v>2004000</v>
+        <v>2037600</v>
       </c>
       <c r="G28" t="n">
-        <v>-54000</v>
+        <v>12200</v>
       </c>
       <c r="H28" t="n">
-        <v>-2.623906705539359</v>
+        <v>0.6023501530561864</v>
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>2026-03-21T04:54:11</t>
+          <t>2026-03-21T04:54:36</t>
         </is>
       </c>
     </row>
@@ -2705,11 +2705,11 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>동방</t>
+          <t>대창단조</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>681</v>
+        <v>300</v>
       </c>
       <c r="D29" t="inlineStr">
         <is>
@@ -2720,17 +2720,17 @@
         <v>1</v>
       </c>
       <c r="F29" t="n">
-        <v>1995330</v>
+        <v>2004000</v>
       </c>
       <c r="G29" t="n">
-        <v>23829</v>
+        <v>-54000</v>
       </c>
       <c r="H29" t="n">
-        <v>1.208672985709873</v>
+        <v>-2.623906705539359</v>
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>2026-03-21T04:54:11</t>
+          <t>2026-03-21T04:54:36</t>
         </is>
       </c>
     </row>
@@ -2742,11 +2742,11 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>스타 벌크 캐리어스</t>
+          <t>동방</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>50</v>
+        <v>681</v>
       </c>
       <c r="D30" t="inlineStr">
         <is>
@@ -2757,17 +2757,17 @@
         <v>1</v>
       </c>
       <c r="F30" t="n">
-        <v>1680142.640194588</v>
+        <v>1995330</v>
       </c>
       <c r="G30" t="n">
-        <v>365789.6401945879</v>
+        <v>23829</v>
       </c>
       <c r="H30" t="n">
-        <v>27.83039565433242</v>
+        <v>1.208672985709873</v>
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>2026-03-21T04:54:11</t>
+          <t>2026-03-21T04:54:36</t>
         </is>
       </c>
     </row>
@@ -2779,7 +2779,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>케이씨</t>
+          <t>스타 벌크 캐리어스</t>
         </is>
       </c>
       <c r="C31" t="n">
@@ -2794,17 +2794,17 @@
         <v>1</v>
       </c>
       <c r="F31" t="n">
-        <v>1670000</v>
+        <v>1680142.640194588</v>
       </c>
       <c r="G31" t="n">
-        <v>20500</v>
+        <v>365789.6401945879</v>
       </c>
       <c r="H31" t="n">
-        <v>1.242800848742043</v>
+        <v>27.83039565433242</v>
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>2026-03-21T04:54:11</t>
+          <t>2026-03-21T04:54:36</t>
         </is>
       </c>
     </row>
@@ -2816,11 +2816,11 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>유나이티드헬스 그룹</t>
+          <t>케이씨</t>
         </is>
       </c>
       <c r="C32" t="n">
-        <v>4</v>
+        <v>50</v>
       </c>
       <c r="D32" t="inlineStr">
         <is>
@@ -2831,17 +2831,17 @@
         <v>1</v>
       </c>
       <c r="F32" t="n">
-        <v>1658864.328313038</v>
+        <v>1670000</v>
       </c>
       <c r="G32" t="n">
-        <v>-35591.67168696248</v>
+        <v>20500</v>
       </c>
       <c r="H32" t="n">
-        <v>-2.100477774988697</v>
+        <v>1.242800848742043</v>
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>2026-03-21T04:54:11</t>
+          <t>2026-03-21T04:54:36</t>
         </is>
       </c>
     </row>
@@ -2853,11 +2853,11 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>텍사스 퍼시픽 랜드</t>
+          <t>유나이티드헬스 그룹</t>
         </is>
       </c>
       <c r="C33" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D33" t="inlineStr">
         <is>
@@ -2868,17 +2868,17 @@
         <v>1</v>
       </c>
       <c r="F33" t="n">
-        <v>1563247.374122903</v>
+        <v>1658864.328313038</v>
       </c>
       <c r="G33" t="n">
-        <v>-14646.62587709725</v>
+        <v>-35591.67168696248</v>
       </c>
       <c r="H33" t="n">
-        <v>-0.9282388979929735</v>
+        <v>-2.100477774988697</v>
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>2026-03-21T04:54:11</t>
+          <t>2026-03-21T04:54:36</t>
         </is>
       </c>
     </row>
@@ -2890,11 +2890,11 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>하나금융지주</t>
+          <t>텍사스 퍼시픽 랜드</t>
         </is>
       </c>
       <c r="C34" t="n">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="D34" t="inlineStr">
         <is>
@@ -2905,17 +2905,17 @@
         <v>1</v>
       </c>
       <c r="F34" t="n">
-        <v>1132000</v>
+        <v>1563247.374122903</v>
       </c>
       <c r="G34" t="n">
-        <v>23000</v>
+        <v>-14646.62587709725</v>
       </c>
       <c r="H34" t="n">
-        <v>2.073940486925157</v>
+        <v>-0.9282388979929735</v>
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>2026-03-21T04:54:11</t>
+          <t>2026-03-21T04:54:36</t>
         </is>
       </c>
     </row>
@@ -2952,7 +2952,7 @@
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>2026-03-21T04:54:11</t>
+          <t>2026-03-21T04:54:36</t>
         </is>
       </c>
     </row>
@@ -2989,7 +2989,7 @@
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>2026-03-21T04:54:11</t>
+          <t>2026-03-21T04:54:36</t>
         </is>
       </c>
     </row>
@@ -3026,7 +3026,7 @@
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>2026-03-21T04:54:11</t>
+          <t>2026-03-21T04:54:36</t>
         </is>
       </c>
     </row>
@@ -3063,7 +3063,7 @@
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>2026-03-21T04:54:11</t>
+          <t>2026-03-21T04:54:36</t>
         </is>
       </c>
     </row>
@@ -3100,7 +3100,7 @@
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>2026-03-21T04:54:11</t>
+          <t>2026-03-21T04:54:36</t>
         </is>
       </c>
     </row>
@@ -3137,7 +3137,7 @@
       </c>
       <c r="I40" t="inlineStr">
         <is>
-          <t>2026-03-21T04:54:11</t>
+          <t>2026-03-21T04:54:36</t>
         </is>
       </c>
     </row>
@@ -3174,7 +3174,7 @@
       </c>
       <c r="I41" t="inlineStr">
         <is>
-          <t>2026-03-21T04:54:11</t>
+          <t>2026-03-21T04:54:36</t>
         </is>
       </c>
     </row>
@@ -3211,7 +3211,7 @@
       </c>
       <c r="I42" t="inlineStr">
         <is>
-          <t>2026-03-21T04:54:11</t>
+          <t>2026-03-21T04:54:36</t>
         </is>
       </c>
     </row>
@@ -3275,7 +3275,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>2026-03-21T04:54:11</t>
+          <t>2026-03-21T04:54:36</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: portfolio snapshot 2026-03-21 (2026-03-21T04:54:38)
</commit_message>
<xml_diff>
--- a/portfolio_auto.xlsx
+++ b/portfolio_auto.xlsx
@@ -1630,7 +1630,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2026-03-21T04:54:36</t>
+          <t>2026-03-21T04:54:38</t>
         </is>
       </c>
       <c r="E2" t="n">
@@ -1731,7 +1731,7 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>2026-03-21T04:54:36</t>
+          <t>2026-03-21T04:54:38</t>
         </is>
       </c>
     </row>
@@ -1768,7 +1768,7 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>2026-03-21T04:54:36</t>
+          <t>2026-03-21T04:54:38</t>
         </is>
       </c>
     </row>
@@ -1805,7 +1805,7 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>2026-03-21T04:54:36</t>
+          <t>2026-03-21T04:54:38</t>
         </is>
       </c>
     </row>
@@ -1842,7 +1842,7 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>2026-03-21T04:54:36</t>
+          <t>2026-03-21T04:54:38</t>
         </is>
       </c>
     </row>
@@ -1879,7 +1879,7 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>2026-03-21T04:54:36</t>
+          <t>2026-03-21T04:54:38</t>
         </is>
       </c>
     </row>
@@ -1916,7 +1916,7 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>2026-03-21T04:54:36</t>
+          <t>2026-03-21T04:54:38</t>
         </is>
       </c>
     </row>
@@ -1953,7 +1953,7 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>2026-03-21T04:54:36</t>
+          <t>2026-03-21T04:54:38</t>
         </is>
       </c>
     </row>
@@ -1990,7 +1990,7 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>2026-03-21T04:54:36</t>
+          <t>2026-03-21T04:54:38</t>
         </is>
       </c>
     </row>
@@ -2027,7 +2027,7 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>2026-03-21T04:54:36</t>
+          <t>2026-03-21T04:54:38</t>
         </is>
       </c>
     </row>
@@ -2064,7 +2064,7 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>2026-03-21T04:54:36</t>
+          <t>2026-03-21T04:54:38</t>
         </is>
       </c>
     </row>
@@ -2101,7 +2101,7 @@
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>2026-03-21T04:54:36</t>
+          <t>2026-03-21T04:54:38</t>
         </is>
       </c>
     </row>
@@ -2138,7 +2138,7 @@
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>2026-03-21T04:54:36</t>
+          <t>2026-03-21T04:54:38</t>
         </is>
       </c>
     </row>
@@ -2175,7 +2175,7 @@
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>2026-03-21T04:54:36</t>
+          <t>2026-03-21T04:54:38</t>
         </is>
       </c>
     </row>
@@ -2212,7 +2212,7 @@
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>2026-03-21T04:54:36</t>
+          <t>2026-03-21T04:54:38</t>
         </is>
       </c>
     </row>
@@ -2249,7 +2249,7 @@
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>2026-03-21T04:54:36</t>
+          <t>2026-03-21T04:54:38</t>
         </is>
       </c>
     </row>
@@ -2286,7 +2286,7 @@
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>2026-03-21T04:54:36</t>
+          <t>2026-03-21T04:54:38</t>
         </is>
       </c>
     </row>
@@ -2323,7 +2323,7 @@
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>2026-03-21T04:54:36</t>
+          <t>2026-03-21T04:54:38</t>
         </is>
       </c>
     </row>
@@ -2360,7 +2360,7 @@
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>2026-03-21T04:54:36</t>
+          <t>2026-03-21T04:54:38</t>
         </is>
       </c>
     </row>
@@ -2397,7 +2397,7 @@
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>2026-03-21T04:54:36</t>
+          <t>2026-03-21T04:54:38</t>
         </is>
       </c>
     </row>
@@ -2434,7 +2434,7 @@
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>2026-03-21T04:54:36</t>
+          <t>2026-03-21T04:54:38</t>
         </is>
       </c>
     </row>
@@ -2471,7 +2471,7 @@
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>2026-03-21T04:54:36</t>
+          <t>2026-03-21T04:54:38</t>
         </is>
       </c>
     </row>
@@ -2508,7 +2508,7 @@
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>2026-03-21T04:54:36</t>
+          <t>2026-03-21T04:54:38</t>
         </is>
       </c>
     </row>
@@ -2545,7 +2545,7 @@
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>2026-03-21T04:54:36</t>
+          <t>2026-03-21T04:54:38</t>
         </is>
       </c>
     </row>
@@ -2582,7 +2582,7 @@
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>2026-03-21T04:54:36</t>
+          <t>2026-03-21T04:54:38</t>
         </is>
       </c>
     </row>
@@ -2619,7 +2619,7 @@
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>2026-03-21T04:54:36</t>
+          <t>2026-03-21T04:54:38</t>
         </is>
       </c>
     </row>
@@ -2656,7 +2656,7 @@
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>2026-03-21T04:54:36</t>
+          <t>2026-03-21T04:54:38</t>
         </is>
       </c>
     </row>
@@ -2693,7 +2693,7 @@
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>2026-03-21T04:54:36</t>
+          <t>2026-03-21T04:54:38</t>
         </is>
       </c>
     </row>
@@ -2730,7 +2730,7 @@
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>2026-03-21T04:54:36</t>
+          <t>2026-03-21T04:54:38</t>
         </is>
       </c>
     </row>
@@ -2767,7 +2767,7 @@
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>2026-03-21T04:54:36</t>
+          <t>2026-03-21T04:54:38</t>
         </is>
       </c>
     </row>
@@ -2804,7 +2804,7 @@
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>2026-03-21T04:54:36</t>
+          <t>2026-03-21T04:54:38</t>
         </is>
       </c>
     </row>
@@ -2841,7 +2841,7 @@
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>2026-03-21T04:54:36</t>
+          <t>2026-03-21T04:54:38</t>
         </is>
       </c>
     </row>
@@ -2878,7 +2878,7 @@
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>2026-03-21T04:54:36</t>
+          <t>2026-03-21T04:54:38</t>
         </is>
       </c>
     </row>
@@ -2915,7 +2915,7 @@
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>2026-03-21T04:54:36</t>
+          <t>2026-03-21T04:54:38</t>
         </is>
       </c>
     </row>
@@ -2952,7 +2952,7 @@
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>2026-03-21T04:54:36</t>
+          <t>2026-03-21T04:54:38</t>
         </is>
       </c>
     </row>
@@ -2989,7 +2989,7 @@
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>2026-03-21T04:54:36</t>
+          <t>2026-03-21T04:54:38</t>
         </is>
       </c>
     </row>
@@ -3026,7 +3026,7 @@
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>2026-03-21T04:54:36</t>
+          <t>2026-03-21T04:54:38</t>
         </is>
       </c>
     </row>
@@ -3063,7 +3063,7 @@
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>2026-03-21T04:54:36</t>
+          <t>2026-03-21T04:54:38</t>
         </is>
       </c>
     </row>
@@ -3100,7 +3100,7 @@
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>2026-03-21T04:54:36</t>
+          <t>2026-03-21T04:54:38</t>
         </is>
       </c>
     </row>
@@ -3137,7 +3137,7 @@
       </c>
       <c r="I40" t="inlineStr">
         <is>
-          <t>2026-03-21T04:54:36</t>
+          <t>2026-03-21T04:54:38</t>
         </is>
       </c>
     </row>
@@ -3174,7 +3174,7 @@
       </c>
       <c r="I41" t="inlineStr">
         <is>
-          <t>2026-03-21T04:54:36</t>
+          <t>2026-03-21T04:54:38</t>
         </is>
       </c>
     </row>
@@ -3211,7 +3211,7 @@
       </c>
       <c r="I42" t="inlineStr">
         <is>
-          <t>2026-03-21T04:54:36</t>
+          <t>2026-03-21T04:54:38</t>
         </is>
       </c>
     </row>
@@ -3275,7 +3275,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>2026-03-21T04:54:36</t>
+          <t>2026-03-21T04:54:38</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: portfolio snapshot 2026-03-21 (2026-03-21T04:54:51)
</commit_message>
<xml_diff>
--- a/portfolio_auto.xlsx
+++ b/portfolio_auto.xlsx
@@ -471,11 +471,11 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>유나이티드헬스 그룹</t>
+          <t>페트로브라스 (ADR)</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>4</v>
+        <v>480</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
@@ -486,13 +486,13 @@
         <v>1</v>
       </c>
       <c r="E2" t="n">
-        <v>1658864.328313038</v>
+        <v>13579584.97235231</v>
       </c>
       <c r="F2" t="n">
-        <v>-35591.67168696248</v>
+        <v>1473035.972352311</v>
       </c>
       <c r="G2" t="n">
-        <v>-2.100477774988697</v>
+        <v>12.16726560436265</v>
       </c>
     </row>
     <row r="3">
@@ -525,11 +525,11 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>센트러스 에너지</t>
+          <t>대한조선</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>25</v>
+        <v>100</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
@@ -540,23 +540,23 @@
         <v>1</v>
       </c>
       <c r="E4" t="n">
-        <v>7026050.85816239</v>
+        <v>9120000</v>
       </c>
       <c r="F4" t="n">
-        <v>-406805.1418376099</v>
+        <v>1907000</v>
       </c>
       <c r="G4" t="n">
-        <v>-5.473066366920198</v>
+        <v>26.43837515596839</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>스타 벌크 캐리어스</t>
+          <t>프론트라인</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>50</v>
+        <v>175</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -567,13 +567,13 @@
         <v>1</v>
       </c>
       <c r="E5" t="n">
-        <v>1680142.640194588</v>
+        <v>8471815.962899337</v>
       </c>
       <c r="F5" t="n">
-        <v>365789.6401945879</v>
+        <v>4041951.962899337</v>
       </c>
       <c r="G5" t="n">
-        <v>27.83039565433242</v>
+        <v>91.24325177701475</v>
       </c>
     </row>
     <row r="6">
@@ -606,11 +606,11 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>오케아니스 에코 탱커스</t>
+          <t>세아제강</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>65</v>
+        <v>50</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -621,23 +621,23 @@
         <v>1</v>
       </c>
       <c r="E7" t="n">
-        <v>4511179.137784176</v>
+        <v>7395000</v>
       </c>
       <c r="F7" t="n">
-        <v>2254819.137784176</v>
+        <v>1085000</v>
       </c>
       <c r="G7" t="n">
-        <v>99.93171026716374</v>
+        <v>17.19492868462758</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>차코스 에너지 내비게이션</t>
+          <t>센트러스 에너지</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>75</v>
+        <v>25</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
@@ -648,23 +648,23 @@
         <v>1</v>
       </c>
       <c r="E8" t="n">
-        <v>4026924.996845168</v>
+        <v>7026050.85816239</v>
       </c>
       <c r="F8" t="n">
-        <v>202276.9968451681</v>
+        <v>-406805.1418376099</v>
       </c>
       <c r="G8" t="n">
-        <v>5.28877420471552</v>
+        <v>-5.473066366920198</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>클리블랜드 클리프스</t>
+          <t>트랜스오션</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>70</v>
+        <v>750</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
@@ -675,13 +675,13 @@
         <v>1</v>
       </c>
       <c r="E9" t="n">
-        <v>823743.9360268187</v>
+        <v>7020031.5082007</v>
       </c>
       <c r="F9" t="n">
-        <v>-192311.0639731813</v>
+        <v>2892797.5082007</v>
       </c>
       <c r="G9" t="n">
-        <v>-18.92722972409774</v>
+        <v>70.09046514446965</v>
       </c>
     </row>
     <row r="10">
@@ -714,11 +714,11 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>텍사스 퍼시픽 랜드</t>
+          <t>노브</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>2</v>
+        <v>185</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
@@ -729,23 +729,23 @@
         <v>1</v>
       </c>
       <c r="E11" t="n">
-        <v>1563247.374122903</v>
+        <v>5200391.447092756</v>
       </c>
       <c r="F11" t="n">
-        <v>-14646.62587709725</v>
+        <v>1890383.447092756</v>
       </c>
       <c r="G11" t="n">
-        <v>-0.9282388979929735</v>
+        <v>57.11114435653194</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>트랜스오션</t>
+          <t>TIME 코리아밸류업액티브</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>750</v>
+        <v>201</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
@@ -756,23 +756,23 @@
         <v>1</v>
       </c>
       <c r="E12" t="n">
-        <v>7020031.5082007</v>
+        <v>4797870</v>
       </c>
       <c r="F12" t="n">
-        <v>2892797.5082007</v>
+        <v>74073</v>
       </c>
       <c r="G12" t="n">
-        <v>70.09046514446965</v>
+        <v>1.568081778281328</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>페트로브라스 (ADR)</t>
+          <t>오케아니스 에코 탱커스</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>480</v>
+        <v>65</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
@@ -783,23 +783,23 @@
         <v>1</v>
       </c>
       <c r="E13" t="n">
-        <v>13579584.97235231</v>
+        <v>4511179.137784176</v>
       </c>
       <c r="F13" t="n">
-        <v>1473035.972352311</v>
+        <v>2254819.137784176</v>
       </c>
       <c r="G13" t="n">
-        <v>12.16726560436265</v>
+        <v>99.93171026716374</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>프론트라인</t>
+          <t>삼성화재</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>175</v>
+        <v>9</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
@@ -810,23 +810,23 @@
         <v>1</v>
       </c>
       <c r="E14" t="n">
-        <v>8471815.962899337</v>
+        <v>4270500</v>
       </c>
       <c r="F14" t="n">
-        <v>4041951.962899337</v>
+        <v>-360500</v>
       </c>
       <c r="G14" t="n">
-        <v>91.24325177701475</v>
+        <v>-7.784495789246384</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>피바디 에너지</t>
+          <t>동원개발</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>65</v>
+        <v>1360</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
@@ -837,23 +837,23 @@
         <v>1</v>
       </c>
       <c r="E15" t="n">
-        <v>3649438.50225304</v>
+        <v>4202400</v>
       </c>
       <c r="F15" t="n">
-        <v>2178666.50225304</v>
+        <v>465000</v>
       </c>
       <c r="G15" t="n">
-        <v>148.1308117269733</v>
+        <v>12.44180446299566</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>하프니아</t>
+          <t>HD건설기계</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>80</v>
+        <v>31</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
@@ -864,23 +864,23 @@
         <v>1</v>
       </c>
       <c r="E16" t="n">
-        <v>842704.775390625</v>
+        <v>4123000</v>
       </c>
       <c r="F16" t="n">
-        <v>216973.775390625</v>
+        <v>87904</v>
       </c>
       <c r="G16" t="n">
-        <v>34.67524789256486</v>
+        <v>2.178485964150543</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>DL이앤씨</t>
+          <t>차코스 에너지 내비게이션</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>40</v>
+        <v>75</v>
       </c>
       <c r="C17" t="inlineStr">
         <is>
@@ -891,23 +891,23 @@
         <v>1</v>
       </c>
       <c r="E17" t="n">
-        <v>2696000</v>
+        <v>4026924.996845168</v>
       </c>
       <c r="F17" t="n">
-        <v>990500</v>
+        <v>202276.9968451681</v>
       </c>
       <c r="G17" t="n">
-        <v>58.07681031955438</v>
+        <v>5.28877420471552</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>HD건설기계</t>
+          <t>넥스틸</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>31</v>
+        <v>300</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
@@ -918,23 +918,23 @@
         <v>1</v>
       </c>
       <c r="E18" t="n">
-        <v>4123000</v>
+        <v>3771000</v>
       </c>
       <c r="F18" t="n">
-        <v>87904</v>
+        <v>521000</v>
       </c>
       <c r="G18" t="n">
-        <v>2.178485964150543</v>
+        <v>16.03076923076923</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>KoAct 코스닥액티브</t>
+          <t>피바디 에너지</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>200</v>
+        <v>65</v>
       </c>
       <c r="C19" t="inlineStr">
         <is>
@@ -945,23 +945,23 @@
         <v>1</v>
       </c>
       <c r="E19" t="n">
-        <v>2582000</v>
+        <v>3649438.50225304</v>
       </c>
       <c r="F19" t="n">
-        <v>-120000</v>
+        <v>2178666.50225304</v>
       </c>
       <c r="G19" t="n">
-        <v>-4.441154700222058</v>
+        <v>148.1308117269733</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>LX인터내셔널</t>
+          <t>현대제철</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>20</v>
+        <v>80</v>
       </c>
       <c r="C20" t="inlineStr">
         <is>
@@ -972,23 +972,23 @@
         <v>1</v>
       </c>
       <c r="E20" t="n">
-        <v>944108</v>
+        <v>2996000</v>
       </c>
       <c r="F20" t="n">
-        <v>5108</v>
+        <v>-182000</v>
       </c>
       <c r="G20" t="n">
-        <v>0.5439829605963792</v>
+        <v>-5.726872246696035</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>NH투자증권우</t>
+          <t>더치 브로스</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>2</v>
+        <v>39</v>
       </c>
       <c r="C21" t="inlineStr">
         <is>
@@ -999,23 +999,23 @@
         <v>1</v>
       </c>
       <c r="E21" t="n">
-        <v>54591</v>
+        <v>2934418.414306641</v>
       </c>
       <c r="F21" t="n">
-        <v>-9</v>
+        <v>-256226.5856933594</v>
       </c>
       <c r="G21" t="n">
-        <v>-0.01648351648351648</v>
+        <v>-8.030557636257226</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>TIME 코리아밸류업액티브</t>
+          <t>휴스틸</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>201</v>
+        <v>500</v>
       </c>
       <c r="C22" t="inlineStr">
         <is>
@@ -1026,23 +1026,23 @@
         <v>1</v>
       </c>
       <c r="E22" t="n">
-        <v>4797870</v>
+        <v>2750000</v>
       </c>
       <c r="F22" t="n">
-        <v>74073</v>
+        <v>471390</v>
       </c>
       <c r="G22" t="n">
-        <v>1.568081778281328</v>
+        <v>20.68761218462133</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>노브</t>
+          <t>DL이앤씨</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>185</v>
+        <v>40</v>
       </c>
       <c r="C23" t="inlineStr">
         <is>
@@ -1053,23 +1053,23 @@
         <v>1</v>
       </c>
       <c r="E23" t="n">
-        <v>5200391.447092756</v>
+        <v>2696000</v>
       </c>
       <c r="F23" t="n">
-        <v>1890383.447092756</v>
+        <v>990500</v>
       </c>
       <c r="G23" t="n">
-        <v>57.11114435653194</v>
+        <v>58.07681031955438</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>노블</t>
+          <t>KoAct 코스닥액티브</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>99</v>
+        <v>200</v>
       </c>
       <c r="C24" t="inlineStr">
         <is>
@@ -1080,23 +1080,23 @@
         <v>1</v>
       </c>
       <c r="E24" t="n">
-        <v>40689</v>
+        <v>2582000</v>
       </c>
       <c r="F24" t="n">
-        <v>-3866519</v>
+        <v>-120000</v>
       </c>
       <c r="G24" t="n">
-        <v>-98.95861699709869</v>
+        <v>-4.441154700222058</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>낫 오프쇼어 파트너스</t>
+          <t>대신증권</t>
         </is>
       </c>
       <c r="B25" t="n">
-        <v>30</v>
+        <v>55</v>
       </c>
       <c r="C25" t="inlineStr">
         <is>
@@ -1107,23 +1107,23 @@
         <v>1</v>
       </c>
       <c r="E25" t="n">
-        <v>410853</v>
+        <v>2219250</v>
       </c>
       <c r="F25" t="n">
-        <v>-6662</v>
+        <v>509749</v>
       </c>
       <c r="G25" t="n">
-        <v>-1.595631294684023</v>
+        <v>29.81858448752005</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>더치 브로스</t>
+          <t>발레로 에너지</t>
         </is>
       </c>
       <c r="B26" t="n">
-        <v>39</v>
+        <v>6</v>
       </c>
       <c r="C26" t="inlineStr">
         <is>
@@ -1134,23 +1134,23 @@
         <v>1</v>
       </c>
       <c r="E26" t="n">
-        <v>2934418.414306641</v>
+        <v>2165691.085066516</v>
       </c>
       <c r="F26" t="n">
-        <v>-256226.5856933594</v>
+        <v>101701.085066516</v>
       </c>
       <c r="G26" t="n">
-        <v>-8.030557636257226</v>
+        <v>4.927402025519307</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>발레로 에너지</t>
+          <t>미창석유</t>
         </is>
       </c>
       <c r="B27" t="n">
-        <v>6</v>
+        <v>18</v>
       </c>
       <c r="C27" t="inlineStr">
         <is>
@@ -1161,23 +1161,23 @@
         <v>1</v>
       </c>
       <c r="E27" t="n">
-        <v>2165691.085066516</v>
+        <v>2097000</v>
       </c>
       <c r="F27" t="n">
-        <v>101701.085066516</v>
+        <v>-295200</v>
       </c>
       <c r="G27" t="n">
-        <v>4.927402025519307</v>
+        <v>-12.34010534236268</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>넥스틸</t>
+          <t>하나금융지주</t>
         </is>
       </c>
       <c r="B28" t="n">
-        <v>300</v>
+        <v>18</v>
       </c>
       <c r="C28" t="inlineStr">
         <is>
@@ -1188,23 +1188,23 @@
         <v>1</v>
       </c>
       <c r="E28" t="n">
-        <v>3771000</v>
+        <v>2037600</v>
       </c>
       <c r="F28" t="n">
-        <v>521000</v>
+        <v>12200</v>
       </c>
       <c r="G28" t="n">
-        <v>16.03076923076923</v>
+        <v>0.6023501530561864</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>대신증권</t>
+          <t>대창단조</t>
         </is>
       </c>
       <c r="B29" t="n">
-        <v>55</v>
+        <v>300</v>
       </c>
       <c r="C29" t="inlineStr">
         <is>
@@ -1215,23 +1215,23 @@
         <v>1</v>
       </c>
       <c r="E29" t="n">
-        <v>2219250</v>
+        <v>2004000</v>
       </c>
       <c r="F29" t="n">
-        <v>509749</v>
+        <v>-54000</v>
       </c>
       <c r="G29" t="n">
-        <v>29.81858448752005</v>
+        <v>-2.623906705539359</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>대창단조</t>
+          <t>동방</t>
         </is>
       </c>
       <c r="B30" t="n">
-        <v>300</v>
+        <v>681</v>
       </c>
       <c r="C30" t="inlineStr">
         <is>
@@ -1242,23 +1242,23 @@
         <v>1</v>
       </c>
       <c r="E30" t="n">
-        <v>2004000</v>
+        <v>1995330</v>
       </c>
       <c r="F30" t="n">
-        <v>-54000</v>
+        <v>23829</v>
       </c>
       <c r="G30" t="n">
-        <v>-2.623906705539359</v>
+        <v>1.208672985709873</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>대한조선</t>
+          <t>스타 벌크 캐리어스</t>
         </is>
       </c>
       <c r="B31" t="n">
-        <v>100</v>
+        <v>50</v>
       </c>
       <c r="C31" t="inlineStr">
         <is>
@@ -1269,23 +1269,23 @@
         <v>1</v>
       </c>
       <c r="E31" t="n">
-        <v>9120000</v>
+        <v>1680142.640194588</v>
       </c>
       <c r="F31" t="n">
-        <v>1907000</v>
+        <v>365789.6401945879</v>
       </c>
       <c r="G31" t="n">
-        <v>26.43837515596839</v>
+        <v>27.83039565433242</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>동방</t>
+          <t>케이씨</t>
         </is>
       </c>
       <c r="B32" t="n">
-        <v>681</v>
+        <v>50</v>
       </c>
       <c r="C32" t="inlineStr">
         <is>
@@ -1296,23 +1296,23 @@
         <v>1</v>
       </c>
       <c r="E32" t="n">
-        <v>1995330</v>
+        <v>1670000</v>
       </c>
       <c r="F32" t="n">
-        <v>23829</v>
+        <v>20500</v>
       </c>
       <c r="G32" t="n">
-        <v>1.208672985709873</v>
+        <v>1.242800848742043</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>동원개발</t>
+          <t>유나이티드헬스 그룹</t>
         </is>
       </c>
       <c r="B33" t="n">
-        <v>1360</v>
+        <v>4</v>
       </c>
       <c r="C33" t="inlineStr">
         <is>
@@ -1323,23 +1323,23 @@
         <v>1</v>
       </c>
       <c r="E33" t="n">
-        <v>4202400</v>
+        <v>1658864.328313038</v>
       </c>
       <c r="F33" t="n">
-        <v>465000</v>
+        <v>-35591.67168696248</v>
       </c>
       <c r="G33" t="n">
-        <v>12.44180446299566</v>
+        <v>-2.100477774988697</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>미창석유</t>
+          <t>텍사스 퍼시픽 랜드</t>
         </is>
       </c>
       <c r="B34" t="n">
-        <v>18</v>
+        <v>2</v>
       </c>
       <c r="C34" t="inlineStr">
         <is>
@@ -1350,23 +1350,23 @@
         <v>1</v>
       </c>
       <c r="E34" t="n">
-        <v>2097000</v>
+        <v>1563247.374122903</v>
       </c>
       <c r="F34" t="n">
-        <v>-295200</v>
+        <v>-14646.62587709725</v>
       </c>
       <c r="G34" t="n">
-        <v>-12.34010534236268</v>
+        <v>-0.9282388979929735</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>비에이치아이</t>
+          <t>LX인터내셔널</t>
         </is>
       </c>
       <c r="B35" t="n">
-        <v>8</v>
+        <v>20</v>
       </c>
       <c r="C35" t="inlineStr">
         <is>
@@ -1377,13 +1377,13 @@
         <v>1</v>
       </c>
       <c r="E35" t="n">
-        <v>876000</v>
+        <v>944108</v>
       </c>
       <c r="F35" t="n">
-        <v>210885</v>
+        <v>5108</v>
       </c>
       <c r="G35" t="n">
-        <v>31.70654698811484</v>
+        <v>0.5439829605963792</v>
       </c>
     </row>
     <row r="36">
@@ -1416,11 +1416,11 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>삼성화재</t>
+          <t>비에이치아이</t>
         </is>
       </c>
       <c r="B37" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C37" t="inlineStr">
         <is>
@@ -1431,23 +1431,23 @@
         <v>1</v>
       </c>
       <c r="E37" t="n">
-        <v>4270500</v>
+        <v>876000</v>
       </c>
       <c r="F37" t="n">
-        <v>-360500</v>
+        <v>210885</v>
       </c>
       <c r="G37" t="n">
-        <v>-7.784495789246384</v>
+        <v>31.70654698811484</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>세아제강</t>
+          <t>하프니아</t>
         </is>
       </c>
       <c r="B38" t="n">
-        <v>50</v>
+        <v>80</v>
       </c>
       <c r="C38" t="inlineStr">
         <is>
@@ -1458,23 +1458,23 @@
         <v>1</v>
       </c>
       <c r="E38" t="n">
-        <v>7395000</v>
+        <v>842704.775390625</v>
       </c>
       <c r="F38" t="n">
-        <v>1085000</v>
+        <v>216973.775390625</v>
       </c>
       <c r="G38" t="n">
-        <v>17.19492868462758</v>
+        <v>34.67524789256486</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>케이씨</t>
+          <t>클리블랜드 클리프스</t>
         </is>
       </c>
       <c r="B39" t="n">
-        <v>50</v>
+        <v>70</v>
       </c>
       <c r="C39" t="inlineStr">
         <is>
@@ -1485,23 +1485,23 @@
         <v>1</v>
       </c>
       <c r="E39" t="n">
-        <v>1670000</v>
+        <v>823743.9360268187</v>
       </c>
       <c r="F39" t="n">
-        <v>20500</v>
+        <v>-192311.0639731813</v>
       </c>
       <c r="G39" t="n">
-        <v>1.242800848742043</v>
+        <v>-18.92722972409774</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>하나금융지주</t>
+          <t>낫 오프쇼어 파트너스</t>
         </is>
       </c>
       <c r="B40" t="n">
-        <v>18</v>
+        <v>30</v>
       </c>
       <c r="C40" t="inlineStr">
         <is>
@@ -1512,23 +1512,23 @@
         <v>1</v>
       </c>
       <c r="E40" t="n">
-        <v>2037600</v>
+        <v>410853</v>
       </c>
       <c r="F40" t="n">
-        <v>12200</v>
+        <v>-6662</v>
       </c>
       <c r="G40" t="n">
-        <v>0.6023501530561864</v>
+        <v>-1.595631294684023</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>현대제철</t>
+          <t>NH투자증권우</t>
         </is>
       </c>
       <c r="B41" t="n">
-        <v>80</v>
+        <v>2</v>
       </c>
       <c r="C41" t="inlineStr">
         <is>
@@ -1539,23 +1539,23 @@
         <v>1</v>
       </c>
       <c r="E41" t="n">
-        <v>2996000</v>
+        <v>54591</v>
       </c>
       <c r="F41" t="n">
-        <v>-182000</v>
+        <v>-9</v>
       </c>
       <c r="G41" t="n">
-        <v>-5.726872246696035</v>
+        <v>-0.01648351648351648</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>휴스틸</t>
+          <t>노블</t>
         </is>
       </c>
       <c r="B42" t="n">
-        <v>500</v>
+        <v>99</v>
       </c>
       <c r="C42" t="inlineStr">
         <is>
@@ -1566,13 +1566,13 @@
         <v>1</v>
       </c>
       <c r="E42" t="n">
-        <v>2750000</v>
+        <v>40689</v>
       </c>
       <c r="F42" t="n">
-        <v>471390</v>
+        <v>-3866519</v>
       </c>
       <c r="G42" t="n">
-        <v>20.68761218462133</v>
+        <v>-98.95861699709869</v>
       </c>
     </row>
   </sheetData>
@@ -1623,14 +1623,14 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0</v>
+        <v>31036676</v>
       </c>
       <c r="C2" t="n">
-        <v>0</v>
+        <v>12663.38</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2026-03-21T04:54:38</t>
+          <t>2026-03-21T04:54:51</t>
         </is>
       </c>
       <c r="E2" t="n">
@@ -3263,10 +3263,10 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0</v>
+        <v>31036676</v>
       </c>
       <c r="C2" t="n">
-        <v>0</v>
+        <v>12663.38</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
@@ -3275,7 +3275,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>2026-03-21T04:54:38</t>
+          <t>2026-03-21T04:54:51</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: portfolio snapshot 2026-03-21 (2026-03-21T04:57:02)
</commit_message>
<xml_diff>
--- a/portfolio_auto.xlsx
+++ b/portfolio_auto.xlsx
@@ -471,11 +471,11 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>페트로브라스 (ADR)</t>
+          <t>유나이티드헬스 그룹</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>480</v>
+        <v>4</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
@@ -486,13 +486,13 @@
         <v>1</v>
       </c>
       <c r="E2" t="n">
-        <v>13579584.97235231</v>
+        <v>1658864.328313038</v>
       </c>
       <c r="F2" t="n">
-        <v>1473035.972352311</v>
+        <v>-35591.67168696248</v>
       </c>
       <c r="G2" t="n">
-        <v>12.16726560436265</v>
+        <v>-2.100477774988697</v>
       </c>
     </row>
     <row r="3">
@@ -525,11 +525,11 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>대한조선</t>
+          <t>센트러스 에너지</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>100</v>
+        <v>25</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
@@ -540,23 +540,23 @@
         <v>1</v>
       </c>
       <c r="E4" t="n">
-        <v>9120000</v>
+        <v>7026050.85816239</v>
       </c>
       <c r="F4" t="n">
-        <v>1907000</v>
+        <v>-406805.1418376099</v>
       </c>
       <c r="G4" t="n">
-        <v>26.43837515596839</v>
+        <v>-5.473066366920198</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>프론트라인</t>
+          <t>스타 벌크 캐리어스</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>175</v>
+        <v>50</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -567,13 +567,13 @@
         <v>1</v>
       </c>
       <c r="E5" t="n">
-        <v>8471815.962899337</v>
+        <v>1680142.640194588</v>
       </c>
       <c r="F5" t="n">
-        <v>4041951.962899337</v>
+        <v>365789.6401945879</v>
       </c>
       <c r="G5" t="n">
-        <v>91.24325177701475</v>
+        <v>27.83039565433242</v>
       </c>
     </row>
     <row r="6">
@@ -606,11 +606,11 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>세아제강</t>
+          <t>오케아니스 에코 탱커스</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>50</v>
+        <v>65</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -621,23 +621,23 @@
         <v>1</v>
       </c>
       <c r="E7" t="n">
-        <v>7395000</v>
+        <v>4511179.137784176</v>
       </c>
       <c r="F7" t="n">
-        <v>1085000</v>
+        <v>2254819.137784176</v>
       </c>
       <c r="G7" t="n">
-        <v>17.19492868462758</v>
+        <v>99.93171026716374</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>센트러스 에너지</t>
+          <t>차코스 에너지 내비게이션</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>25</v>
+        <v>75</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
@@ -648,23 +648,23 @@
         <v>1</v>
       </c>
       <c r="E8" t="n">
-        <v>7026050.85816239</v>
+        <v>4026924.996845168</v>
       </c>
       <c r="F8" t="n">
-        <v>-406805.1418376099</v>
+        <v>202276.9968451681</v>
       </c>
       <c r="G8" t="n">
-        <v>-5.473066366920198</v>
+        <v>5.28877420471552</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>트랜스오션</t>
+          <t>클리블랜드 클리프스</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>750</v>
+        <v>70</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
@@ -675,13 +675,13 @@
         <v>1</v>
       </c>
       <c r="E9" t="n">
-        <v>7020031.5082007</v>
+        <v>823743.9360268187</v>
       </c>
       <c r="F9" t="n">
-        <v>2892797.5082007</v>
+        <v>-192311.0639731813</v>
       </c>
       <c r="G9" t="n">
-        <v>70.09046514446965</v>
+        <v>-18.92722972409774</v>
       </c>
     </row>
     <row r="10">
@@ -714,11 +714,11 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>노브</t>
+          <t>텍사스 퍼시픽 랜드</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>185</v>
+        <v>2</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
@@ -729,23 +729,23 @@
         <v>1</v>
       </c>
       <c r="E11" t="n">
-        <v>5200391.447092756</v>
+        <v>1563247.374122903</v>
       </c>
       <c r="F11" t="n">
-        <v>1890383.447092756</v>
+        <v>-14646.62587709725</v>
       </c>
       <c r="G11" t="n">
-        <v>57.11114435653194</v>
+        <v>-0.9282388979929735</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>TIME 코리아밸류업액티브</t>
+          <t>트랜스오션</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>201</v>
+        <v>750</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
@@ -756,23 +756,23 @@
         <v>1</v>
       </c>
       <c r="E12" t="n">
-        <v>4797870</v>
+        <v>7020031.5082007</v>
       </c>
       <c r="F12" t="n">
-        <v>74073</v>
+        <v>2892797.5082007</v>
       </c>
       <c r="G12" t="n">
-        <v>1.568081778281328</v>
+        <v>70.09046514446965</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>오케아니스 에코 탱커스</t>
+          <t>페트로브라스 (ADR)</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>65</v>
+        <v>480</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
@@ -783,23 +783,23 @@
         <v>1</v>
       </c>
       <c r="E13" t="n">
-        <v>4511179.137784176</v>
+        <v>13579584.97235231</v>
       </c>
       <c r="F13" t="n">
-        <v>2254819.137784176</v>
+        <v>1473035.972352311</v>
       </c>
       <c r="G13" t="n">
-        <v>99.93171026716374</v>
+        <v>12.16726560436265</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>삼성화재</t>
+          <t>프론트라인</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>9</v>
+        <v>175</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
@@ -810,23 +810,23 @@
         <v>1</v>
       </c>
       <c r="E14" t="n">
-        <v>4270500</v>
+        <v>8471815.962899337</v>
       </c>
       <c r="F14" t="n">
-        <v>-360500</v>
+        <v>4041951.962899337</v>
       </c>
       <c r="G14" t="n">
-        <v>-7.784495789246384</v>
+        <v>91.24325177701475</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>동원개발</t>
+          <t>피바디 에너지</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>1360</v>
+        <v>65</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
@@ -837,23 +837,23 @@
         <v>1</v>
       </c>
       <c r="E15" t="n">
-        <v>4202400</v>
+        <v>3649438.50225304</v>
       </c>
       <c r="F15" t="n">
-        <v>465000</v>
+        <v>2178666.50225304</v>
       </c>
       <c r="G15" t="n">
-        <v>12.44180446299566</v>
+        <v>148.1308117269733</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>HD건설기계</t>
+          <t>하프니아</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>31</v>
+        <v>80</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
@@ -864,23 +864,23 @@
         <v>1</v>
       </c>
       <c r="E16" t="n">
-        <v>4123000</v>
+        <v>842704.775390625</v>
       </c>
       <c r="F16" t="n">
-        <v>87904</v>
+        <v>216973.775390625</v>
       </c>
       <c r="G16" t="n">
-        <v>2.178485964150543</v>
+        <v>34.67524789256486</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>차코스 에너지 내비게이션</t>
+          <t>DL이앤씨</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>75</v>
+        <v>40</v>
       </c>
       <c r="C17" t="inlineStr">
         <is>
@@ -891,23 +891,23 @@
         <v>1</v>
       </c>
       <c r="E17" t="n">
-        <v>4026924.996845168</v>
+        <v>2696000</v>
       </c>
       <c r="F17" t="n">
-        <v>202276.9968451681</v>
+        <v>990500</v>
       </c>
       <c r="G17" t="n">
-        <v>5.28877420471552</v>
+        <v>58.07681031955438</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>넥스틸</t>
+          <t>HD건설기계</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>300</v>
+        <v>31</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
@@ -918,23 +918,23 @@
         <v>1</v>
       </c>
       <c r="E18" t="n">
-        <v>3771000</v>
+        <v>4123000</v>
       </c>
       <c r="F18" t="n">
-        <v>521000</v>
+        <v>87904</v>
       </c>
       <c r="G18" t="n">
-        <v>16.03076923076923</v>
+        <v>2.178485964150543</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>피바디 에너지</t>
+          <t>KoAct 코스닥액티브</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>65</v>
+        <v>200</v>
       </c>
       <c r="C19" t="inlineStr">
         <is>
@@ -945,23 +945,23 @@
         <v>1</v>
       </c>
       <c r="E19" t="n">
-        <v>3649438.50225304</v>
+        <v>2582000</v>
       </c>
       <c r="F19" t="n">
-        <v>2178666.50225304</v>
+        <v>-120000</v>
       </c>
       <c r="G19" t="n">
-        <v>148.1308117269733</v>
+        <v>-4.441154700222058</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>현대제철</t>
+          <t>LX인터내셔널</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>80</v>
+        <v>20</v>
       </c>
       <c r="C20" t="inlineStr">
         <is>
@@ -972,23 +972,23 @@
         <v>1</v>
       </c>
       <c r="E20" t="n">
-        <v>2996000</v>
+        <v>943000</v>
       </c>
       <c r="F20" t="n">
-        <v>-182000</v>
+        <v>4000</v>
       </c>
       <c r="G20" t="n">
-        <v>-5.726872246696035</v>
+        <v>0.4259850905218318</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>더치 브로스</t>
+          <t>NH투자증권우</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>39</v>
+        <v>2</v>
       </c>
       <c r="C21" t="inlineStr">
         <is>
@@ -999,23 +999,23 @@
         <v>1</v>
       </c>
       <c r="E21" t="n">
-        <v>2934418.414306641</v>
+        <v>54700</v>
       </c>
       <c r="F21" t="n">
-        <v>-256226.5856933594</v>
+        <v>100</v>
       </c>
       <c r="G21" t="n">
-        <v>-8.030557636257226</v>
+        <v>0.1831501831501831</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>휴스틸</t>
+          <t>TIME 코리아밸류업액티브</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>500</v>
+        <v>201</v>
       </c>
       <c r="C22" t="inlineStr">
         <is>
@@ -1026,23 +1026,23 @@
         <v>1</v>
       </c>
       <c r="E22" t="n">
-        <v>2750000</v>
+        <v>4797870</v>
       </c>
       <c r="F22" t="n">
-        <v>471390</v>
+        <v>74073</v>
       </c>
       <c r="G22" t="n">
-        <v>20.68761218462133</v>
+        <v>1.568081778281328</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>DL이앤씨</t>
+          <t>노브</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>40</v>
+        <v>185</v>
       </c>
       <c r="C23" t="inlineStr">
         <is>
@@ -1053,23 +1053,23 @@
         <v>1</v>
       </c>
       <c r="E23" t="n">
-        <v>2696000</v>
+        <v>5200391.447092756</v>
       </c>
       <c r="F23" t="n">
-        <v>990500</v>
+        <v>1890383.447092756</v>
       </c>
       <c r="G23" t="n">
-        <v>58.07681031955438</v>
+        <v>57.11114435653194</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>KoAct 코스닥액티브</t>
+          <t>노블</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>200</v>
+        <v>99</v>
       </c>
       <c r="C24" t="inlineStr">
         <is>
@@ -1080,23 +1080,23 @@
         <v>1</v>
       </c>
       <c r="E24" t="n">
-        <v>2582000</v>
+        <v>6958769.981090547</v>
       </c>
       <c r="F24" t="n">
-        <v>-120000</v>
+        <v>3051561.981090547</v>
       </c>
       <c r="G24" t="n">
-        <v>-4.441154700222058</v>
+        <v>78.10083264291399</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>대신증권</t>
+          <t>낫 오프쇼어 파트너스</t>
         </is>
       </c>
       <c r="B25" t="n">
-        <v>55</v>
+        <v>30</v>
       </c>
       <c r="C25" t="inlineStr">
         <is>
@@ -1107,23 +1107,23 @@
         <v>1</v>
       </c>
       <c r="E25" t="n">
-        <v>2219250</v>
+        <v>413075.8057155996</v>
       </c>
       <c r="F25" t="n">
-        <v>509749</v>
+        <v>-4439.194284400437</v>
       </c>
       <c r="G25" t="n">
-        <v>29.81858448752005</v>
+        <v>-1.063241867813237</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>발레로 에너지</t>
+          <t>더치 브로스</t>
         </is>
       </c>
       <c r="B26" t="n">
-        <v>6</v>
+        <v>39</v>
       </c>
       <c r="C26" t="inlineStr">
         <is>
@@ -1134,23 +1134,23 @@
         <v>1</v>
       </c>
       <c r="E26" t="n">
-        <v>2165691.085066516</v>
+        <v>2934418.414306641</v>
       </c>
       <c r="F26" t="n">
-        <v>101701.085066516</v>
+        <v>-256226.5856933594</v>
       </c>
       <c r="G26" t="n">
-        <v>4.927402025519307</v>
+        <v>-8.030557636257226</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>미창석유</t>
+          <t>발레로 에너지</t>
         </is>
       </c>
       <c r="B27" t="n">
-        <v>18</v>
+        <v>6</v>
       </c>
       <c r="C27" t="inlineStr">
         <is>
@@ -1161,23 +1161,23 @@
         <v>1</v>
       </c>
       <c r="E27" t="n">
-        <v>2097000</v>
+        <v>2165691.085066516</v>
       </c>
       <c r="F27" t="n">
-        <v>-295200</v>
+        <v>101701.085066516</v>
       </c>
       <c r="G27" t="n">
-        <v>-12.34010534236268</v>
+        <v>4.927402025519307</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>하나금융지주</t>
+          <t>넥스틸</t>
         </is>
       </c>
       <c r="B28" t="n">
-        <v>18</v>
+        <v>300</v>
       </c>
       <c r="C28" t="inlineStr">
         <is>
@@ -1188,23 +1188,23 @@
         <v>1</v>
       </c>
       <c r="E28" t="n">
-        <v>2037600</v>
+        <v>3771000</v>
       </c>
       <c r="F28" t="n">
-        <v>12200</v>
+        <v>521000</v>
       </c>
       <c r="G28" t="n">
-        <v>0.6023501530561864</v>
+        <v>16.03076923076923</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>대창단조</t>
+          <t>대신증권</t>
         </is>
       </c>
       <c r="B29" t="n">
-        <v>300</v>
+        <v>55</v>
       </c>
       <c r="C29" t="inlineStr">
         <is>
@@ -1215,23 +1215,23 @@
         <v>1</v>
       </c>
       <c r="E29" t="n">
-        <v>2004000</v>
+        <v>2219250</v>
       </c>
       <c r="F29" t="n">
-        <v>-54000</v>
+        <v>509749</v>
       </c>
       <c r="G29" t="n">
-        <v>-2.623906705539359</v>
+        <v>29.81858448752005</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>동방</t>
+          <t>대창단조</t>
         </is>
       </c>
       <c r="B30" t="n">
-        <v>681</v>
+        <v>300</v>
       </c>
       <c r="C30" t="inlineStr">
         <is>
@@ -1242,23 +1242,23 @@
         <v>1</v>
       </c>
       <c r="E30" t="n">
-        <v>1995330</v>
+        <v>2004000</v>
       </c>
       <c r="F30" t="n">
-        <v>23829</v>
+        <v>-54000</v>
       </c>
       <c r="G30" t="n">
-        <v>1.208672985709873</v>
+        <v>-2.623906705539359</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>스타 벌크 캐리어스</t>
+          <t>대한조선</t>
         </is>
       </c>
       <c r="B31" t="n">
-        <v>50</v>
+        <v>100</v>
       </c>
       <c r="C31" t="inlineStr">
         <is>
@@ -1269,23 +1269,23 @@
         <v>1</v>
       </c>
       <c r="E31" t="n">
-        <v>1680142.640194588</v>
+        <v>9120000</v>
       </c>
       <c r="F31" t="n">
-        <v>365789.6401945879</v>
+        <v>1907000</v>
       </c>
       <c r="G31" t="n">
-        <v>27.83039565433242</v>
+        <v>26.43837515596839</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>케이씨</t>
+          <t>동방</t>
         </is>
       </c>
       <c r="B32" t="n">
-        <v>50</v>
+        <v>681</v>
       </c>
       <c r="C32" t="inlineStr">
         <is>
@@ -1296,23 +1296,23 @@
         <v>1</v>
       </c>
       <c r="E32" t="n">
-        <v>1670000</v>
+        <v>1995330</v>
       </c>
       <c r="F32" t="n">
-        <v>20500</v>
+        <v>23829</v>
       </c>
       <c r="G32" t="n">
-        <v>1.242800848742043</v>
+        <v>1.208672985709873</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>유나이티드헬스 그룹</t>
+          <t>동원개발</t>
         </is>
       </c>
       <c r="B33" t="n">
-        <v>4</v>
+        <v>1360</v>
       </c>
       <c r="C33" t="inlineStr">
         <is>
@@ -1323,23 +1323,23 @@
         <v>1</v>
       </c>
       <c r="E33" t="n">
-        <v>1658864.328313038</v>
+        <v>4202400</v>
       </c>
       <c r="F33" t="n">
-        <v>-35591.67168696248</v>
+        <v>465000</v>
       </c>
       <c r="G33" t="n">
-        <v>-2.100477774988697</v>
+        <v>12.44180446299566</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>텍사스 퍼시픽 랜드</t>
+          <t>미창석유</t>
         </is>
       </c>
       <c r="B34" t="n">
-        <v>2</v>
+        <v>18</v>
       </c>
       <c r="C34" t="inlineStr">
         <is>
@@ -1350,23 +1350,23 @@
         <v>1</v>
       </c>
       <c r="E34" t="n">
-        <v>1563247.374122903</v>
+        <v>2097000</v>
       </c>
       <c r="F34" t="n">
-        <v>-14646.62587709725</v>
+        <v>-295200</v>
       </c>
       <c r="G34" t="n">
-        <v>-0.9282388979929735</v>
+        <v>-12.34010534236268</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>LX인터내셔널</t>
+          <t>비에이치아이</t>
         </is>
       </c>
       <c r="B35" t="n">
-        <v>20</v>
+        <v>8</v>
       </c>
       <c r="C35" t="inlineStr">
         <is>
@@ -1377,13 +1377,13 @@
         <v>1</v>
       </c>
       <c r="E35" t="n">
-        <v>944108</v>
+        <v>876000</v>
       </c>
       <c r="F35" t="n">
-        <v>5108</v>
+        <v>210885</v>
       </c>
       <c r="G35" t="n">
-        <v>0.5439829605963792</v>
+        <v>31.70654698811484</v>
       </c>
     </row>
     <row r="36">
@@ -1416,11 +1416,11 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>비에이치아이</t>
+          <t>삼성화재</t>
         </is>
       </c>
       <c r="B37" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C37" t="inlineStr">
         <is>
@@ -1431,23 +1431,23 @@
         <v>1</v>
       </c>
       <c r="E37" t="n">
-        <v>876000</v>
+        <v>4270500</v>
       </c>
       <c r="F37" t="n">
-        <v>210885</v>
+        <v>-360500</v>
       </c>
       <c r="G37" t="n">
-        <v>31.70654698811484</v>
+        <v>-7.784495789246384</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>하프니아</t>
+          <t>세아제강</t>
         </is>
       </c>
       <c r="B38" t="n">
-        <v>80</v>
+        <v>50</v>
       </c>
       <c r="C38" t="inlineStr">
         <is>
@@ -1458,23 +1458,23 @@
         <v>1</v>
       </c>
       <c r="E38" t="n">
-        <v>842704.775390625</v>
+        <v>7395000</v>
       </c>
       <c r="F38" t="n">
-        <v>216973.775390625</v>
+        <v>1085000</v>
       </c>
       <c r="G38" t="n">
-        <v>34.67524789256486</v>
+        <v>17.19492868462758</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>클리블랜드 클리프스</t>
+          <t>케이씨</t>
         </is>
       </c>
       <c r="B39" t="n">
-        <v>70</v>
+        <v>50</v>
       </c>
       <c r="C39" t="inlineStr">
         <is>
@@ -1485,23 +1485,23 @@
         <v>1</v>
       </c>
       <c r="E39" t="n">
-        <v>823743.9360268187</v>
+        <v>1670000</v>
       </c>
       <c r="F39" t="n">
-        <v>-192311.0639731813</v>
+        <v>20500</v>
       </c>
       <c r="G39" t="n">
-        <v>-18.92722972409774</v>
+        <v>1.242800848742043</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>낫 오프쇼어 파트너스</t>
+          <t>하나금융지주</t>
         </is>
       </c>
       <c r="B40" t="n">
-        <v>30</v>
+        <v>18</v>
       </c>
       <c r="C40" t="inlineStr">
         <is>
@@ -1512,23 +1512,23 @@
         <v>1</v>
       </c>
       <c r="E40" t="n">
-        <v>410853</v>
+        <v>2037600</v>
       </c>
       <c r="F40" t="n">
-        <v>-6662</v>
+        <v>12200</v>
       </c>
       <c r="G40" t="n">
-        <v>-1.595631294684023</v>
+        <v>0.6023501530561864</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>NH투자증권우</t>
+          <t>현대제철</t>
         </is>
       </c>
       <c r="B41" t="n">
-        <v>2</v>
+        <v>80</v>
       </c>
       <c r="C41" t="inlineStr">
         <is>
@@ -1539,23 +1539,23 @@
         <v>1</v>
       </c>
       <c r="E41" t="n">
-        <v>54591</v>
+        <v>2996000</v>
       </c>
       <c r="F41" t="n">
-        <v>-9</v>
+        <v>-182000</v>
       </c>
       <c r="G41" t="n">
-        <v>-0.01648351648351648</v>
+        <v>-5.726872246696035</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>노블</t>
+          <t>휴스틸</t>
         </is>
       </c>
       <c r="B42" t="n">
-        <v>99</v>
+        <v>500</v>
       </c>
       <c r="C42" t="inlineStr">
         <is>
@@ -1566,13 +1566,13 @@
         <v>1</v>
       </c>
       <c r="E42" t="n">
-        <v>40689</v>
+        <v>2750000</v>
       </c>
       <c r="F42" t="n">
-        <v>-3866519</v>
+        <v>471390</v>
       </c>
       <c r="G42" t="n">
-        <v>-98.95861699709869</v>
+        <v>20.68761218462133</v>
       </c>
     </row>
   </sheetData>
@@ -1630,7 +1630,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2026-03-21T04:54:51</t>
+          <t>2026-03-21T04:57:02</t>
         </is>
       </c>
       <c r="E2" t="n">
@@ -1731,7 +1731,7 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>2026-03-21T04:54:38</t>
+          <t>2026-03-21T04:57:02</t>
         </is>
       </c>
     </row>
@@ -1768,7 +1768,7 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>2026-03-21T04:54:38</t>
+          <t>2026-03-21T04:57:02</t>
         </is>
       </c>
     </row>
@@ -1805,7 +1805,7 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>2026-03-21T04:54:38</t>
+          <t>2026-03-21T04:57:02</t>
         </is>
       </c>
     </row>
@@ -1842,7 +1842,7 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>2026-03-21T04:54:38</t>
+          <t>2026-03-21T04:57:02</t>
         </is>
       </c>
     </row>
@@ -1879,7 +1879,7 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>2026-03-21T04:54:38</t>
+          <t>2026-03-21T04:57:02</t>
         </is>
       </c>
     </row>
@@ -1916,7 +1916,7 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>2026-03-21T04:54:38</t>
+          <t>2026-03-21T04:57:02</t>
         </is>
       </c>
     </row>
@@ -1953,7 +1953,7 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>2026-03-21T04:54:38</t>
+          <t>2026-03-21T04:57:02</t>
         </is>
       </c>
     </row>
@@ -1990,7 +1990,7 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>2026-03-21T04:54:38</t>
+          <t>2026-03-21T04:57:02</t>
         </is>
       </c>
     </row>
@@ -2002,11 +2002,11 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>타이드워터</t>
+          <t>노블</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>48</v>
+        <v>99</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
@@ -2017,17 +2017,17 @@
         <v>1</v>
       </c>
       <c r="F10" t="n">
-        <v>5235363.852789983</v>
+        <v>6958769.981090547</v>
       </c>
       <c r="G10" t="n">
-        <v>1510818.852789983</v>
+        <v>3051561.981090547</v>
       </c>
       <c r="H10" t="n">
-        <v>40.56385015592463</v>
+        <v>78.10083264291399</v>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>2026-03-21T04:54:38</t>
+          <t>2026-03-21T04:57:02</t>
         </is>
       </c>
     </row>
@@ -2039,11 +2039,11 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>노브</t>
+          <t>타이드워터</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>185</v>
+        <v>48</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
@@ -2054,17 +2054,17 @@
         <v>1</v>
       </c>
       <c r="F11" t="n">
-        <v>5200391.447092756</v>
+        <v>5235363.852789983</v>
       </c>
       <c r="G11" t="n">
-        <v>1890383.447092756</v>
+        <v>1510818.852789983</v>
       </c>
       <c r="H11" t="n">
-        <v>57.11114435653194</v>
+        <v>40.56385015592463</v>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>2026-03-21T04:54:38</t>
+          <t>2026-03-21T04:57:02</t>
         </is>
       </c>
     </row>
@@ -2076,11 +2076,11 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>TIME 코리아밸류업액티브</t>
+          <t>노브</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>201</v>
+        <v>185</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
@@ -2091,17 +2091,17 @@
         <v>1</v>
       </c>
       <c r="F12" t="n">
-        <v>4797870</v>
+        <v>5200391.447092756</v>
       </c>
       <c r="G12" t="n">
-        <v>74073</v>
+        <v>1890383.447092756</v>
       </c>
       <c r="H12" t="n">
-        <v>1.568081778281328</v>
+        <v>57.11114435653194</v>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>2026-03-21T04:54:38</t>
+          <t>2026-03-21T04:57:02</t>
         </is>
       </c>
     </row>
@@ -2113,11 +2113,11 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>오케아니스 에코 탱커스</t>
+          <t>TIME 코리아밸류업액티브</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>65</v>
+        <v>201</v>
       </c>
       <c r="D13" t="inlineStr">
         <is>
@@ -2128,17 +2128,17 @@
         <v>1</v>
       </c>
       <c r="F13" t="n">
-        <v>4511179.137784176</v>
+        <v>4797870</v>
       </c>
       <c r="G13" t="n">
-        <v>2254819.137784176</v>
+        <v>74073</v>
       </c>
       <c r="H13" t="n">
-        <v>99.93171026716374</v>
+        <v>1.568081778281328</v>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>2026-03-21T04:54:38</t>
+          <t>2026-03-21T04:57:02</t>
         </is>
       </c>
     </row>
@@ -2150,11 +2150,11 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>삼성화재</t>
+          <t>오케아니스 에코 탱커스</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>9</v>
+        <v>65</v>
       </c>
       <c r="D14" t="inlineStr">
         <is>
@@ -2165,17 +2165,17 @@
         <v>1</v>
       </c>
       <c r="F14" t="n">
-        <v>4270500</v>
+        <v>4511179.137784176</v>
       </c>
       <c r="G14" t="n">
-        <v>-360500</v>
+        <v>2254819.137784176</v>
       </c>
       <c r="H14" t="n">
-        <v>-7.784495789246384</v>
+        <v>99.93171026716374</v>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>2026-03-21T04:54:38</t>
+          <t>2026-03-21T04:57:02</t>
         </is>
       </c>
     </row>
@@ -2187,11 +2187,11 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>동원개발</t>
+          <t>삼성화재</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>1360</v>
+        <v>9</v>
       </c>
       <c r="D15" t="inlineStr">
         <is>
@@ -2202,17 +2202,17 @@
         <v>1</v>
       </c>
       <c r="F15" t="n">
-        <v>4202400</v>
+        <v>4270500</v>
       </c>
       <c r="G15" t="n">
-        <v>465000</v>
+        <v>-360500</v>
       </c>
       <c r="H15" t="n">
-        <v>12.44180446299566</v>
+        <v>-7.784495789246384</v>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>2026-03-21T04:54:38</t>
+          <t>2026-03-21T04:57:02</t>
         </is>
       </c>
     </row>
@@ -2224,11 +2224,11 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>HD건설기계</t>
+          <t>동원개발</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>31</v>
+        <v>1360</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
@@ -2239,17 +2239,17 @@
         <v>1</v>
       </c>
       <c r="F16" t="n">
-        <v>4123000</v>
+        <v>4202400</v>
       </c>
       <c r="G16" t="n">
-        <v>87904</v>
+        <v>465000</v>
       </c>
       <c r="H16" t="n">
-        <v>2.178485964150543</v>
+        <v>12.44180446299566</v>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>2026-03-21T04:54:38</t>
+          <t>2026-03-21T04:57:02</t>
         </is>
       </c>
     </row>
@@ -2261,11 +2261,11 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>차코스 에너지 내비게이션</t>
+          <t>HD건설기계</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>75</v>
+        <v>31</v>
       </c>
       <c r="D17" t="inlineStr">
         <is>
@@ -2276,17 +2276,17 @@
         <v>1</v>
       </c>
       <c r="F17" t="n">
-        <v>4026924.996845168</v>
+        <v>4123000</v>
       </c>
       <c r="G17" t="n">
-        <v>202276.9968451681</v>
+        <v>87904</v>
       </c>
       <c r="H17" t="n">
-        <v>5.28877420471552</v>
+        <v>2.178485964150543</v>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>2026-03-21T04:54:38</t>
+          <t>2026-03-21T04:57:02</t>
         </is>
       </c>
     </row>
@@ -2298,11 +2298,11 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>넥스틸</t>
+          <t>차코스 에너지 내비게이션</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>300</v>
+        <v>75</v>
       </c>
       <c r="D18" t="inlineStr">
         <is>
@@ -2313,17 +2313,17 @@
         <v>1</v>
       </c>
       <c r="F18" t="n">
-        <v>3771000</v>
+        <v>4026924.996845168</v>
       </c>
       <c r="G18" t="n">
-        <v>521000</v>
+        <v>202276.9968451681</v>
       </c>
       <c r="H18" t="n">
-        <v>16.03076923076923</v>
+        <v>5.28877420471552</v>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>2026-03-21T04:54:38</t>
+          <t>2026-03-21T04:57:02</t>
         </is>
       </c>
     </row>
@@ -2335,11 +2335,11 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>피바디 에너지</t>
+          <t>넥스틸</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>65</v>
+        <v>300</v>
       </c>
       <c r="D19" t="inlineStr">
         <is>
@@ -2350,17 +2350,17 @@
         <v>1</v>
       </c>
       <c r="F19" t="n">
-        <v>3649438.50225304</v>
+        <v>3771000</v>
       </c>
       <c r="G19" t="n">
-        <v>2178666.50225304</v>
+        <v>521000</v>
       </c>
       <c r="H19" t="n">
-        <v>148.1308117269733</v>
+        <v>16.03076923076923</v>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>2026-03-21T04:54:38</t>
+          <t>2026-03-21T04:57:02</t>
         </is>
       </c>
     </row>
@@ -2372,11 +2372,11 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>현대제철</t>
+          <t>피바디 에너지</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>80</v>
+        <v>65</v>
       </c>
       <c r="D20" t="inlineStr">
         <is>
@@ -2387,17 +2387,17 @@
         <v>1</v>
       </c>
       <c r="F20" t="n">
-        <v>2996000</v>
+        <v>3649438.50225304</v>
       </c>
       <c r="G20" t="n">
-        <v>-182000</v>
+        <v>2178666.50225304</v>
       </c>
       <c r="H20" t="n">
-        <v>-5.726872246696035</v>
+        <v>148.1308117269733</v>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>2026-03-21T04:54:38</t>
+          <t>2026-03-21T04:57:02</t>
         </is>
       </c>
     </row>
@@ -2409,11 +2409,11 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>더치 브로스</t>
+          <t>현대제철</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>39</v>
+        <v>80</v>
       </c>
       <c r="D21" t="inlineStr">
         <is>
@@ -2424,17 +2424,17 @@
         <v>1</v>
       </c>
       <c r="F21" t="n">
-        <v>2934418.414306641</v>
+        <v>2996000</v>
       </c>
       <c r="G21" t="n">
-        <v>-256226.5856933594</v>
+        <v>-182000</v>
       </c>
       <c r="H21" t="n">
-        <v>-8.030557636257226</v>
+        <v>-5.726872246696035</v>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>2026-03-21T04:54:38</t>
+          <t>2026-03-21T04:57:02</t>
         </is>
       </c>
     </row>
@@ -2446,11 +2446,11 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>휴스틸</t>
+          <t>더치 브로스</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>500</v>
+        <v>39</v>
       </c>
       <c r="D22" t="inlineStr">
         <is>
@@ -2461,17 +2461,17 @@
         <v>1</v>
       </c>
       <c r="F22" t="n">
-        <v>2750000</v>
+        <v>2934418.414306641</v>
       </c>
       <c r="G22" t="n">
-        <v>471390</v>
+        <v>-256226.5856933594</v>
       </c>
       <c r="H22" t="n">
-        <v>20.68761218462133</v>
+        <v>-8.030557636257226</v>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>2026-03-21T04:54:38</t>
+          <t>2026-03-21T04:57:02</t>
         </is>
       </c>
     </row>
@@ -2483,11 +2483,11 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>DL이앤씨</t>
+          <t>휴스틸</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>40</v>
+        <v>500</v>
       </c>
       <c r="D23" t="inlineStr">
         <is>
@@ -2498,17 +2498,17 @@
         <v>1</v>
       </c>
       <c r="F23" t="n">
-        <v>2696000</v>
+        <v>2750000</v>
       </c>
       <c r="G23" t="n">
-        <v>990500</v>
+        <v>471390</v>
       </c>
       <c r="H23" t="n">
-        <v>58.07681031955438</v>
+        <v>20.68761218462133</v>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>2026-03-21T04:54:38</t>
+          <t>2026-03-21T04:57:02</t>
         </is>
       </c>
     </row>
@@ -2520,11 +2520,11 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>KoAct 코스닥액티브</t>
+          <t>DL이앤씨</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>200</v>
+        <v>40</v>
       </c>
       <c r="D24" t="inlineStr">
         <is>
@@ -2535,17 +2535,17 @@
         <v>1</v>
       </c>
       <c r="F24" t="n">
-        <v>2582000</v>
+        <v>2696000</v>
       </c>
       <c r="G24" t="n">
-        <v>-120000</v>
+        <v>990500</v>
       </c>
       <c r="H24" t="n">
-        <v>-4.441154700222058</v>
+        <v>58.07681031955438</v>
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>2026-03-21T04:54:38</t>
+          <t>2026-03-21T04:57:02</t>
         </is>
       </c>
     </row>
@@ -2557,11 +2557,11 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>대신증권</t>
+          <t>KoAct 코스닥액티브</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>55</v>
+        <v>200</v>
       </c>
       <c r="D25" t="inlineStr">
         <is>
@@ -2572,17 +2572,17 @@
         <v>1</v>
       </c>
       <c r="F25" t="n">
-        <v>2219250</v>
+        <v>2582000</v>
       </c>
       <c r="G25" t="n">
-        <v>509749</v>
+        <v>-120000</v>
       </c>
       <c r="H25" t="n">
-        <v>29.81858448752005</v>
+        <v>-4.441154700222058</v>
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>2026-03-21T04:54:38</t>
+          <t>2026-03-21T04:57:02</t>
         </is>
       </c>
     </row>
@@ -2594,11 +2594,11 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>발레로 에너지</t>
+          <t>대신증권</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>6</v>
+        <v>55</v>
       </c>
       <c r="D26" t="inlineStr">
         <is>
@@ -2609,17 +2609,17 @@
         <v>1</v>
       </c>
       <c r="F26" t="n">
-        <v>2165691.085066516</v>
+        <v>2219250</v>
       </c>
       <c r="G26" t="n">
-        <v>101701.085066516</v>
+        <v>509749</v>
       </c>
       <c r="H26" t="n">
-        <v>4.927402025519307</v>
+        <v>29.81858448752005</v>
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>2026-03-21T04:54:38</t>
+          <t>2026-03-21T04:57:02</t>
         </is>
       </c>
     </row>
@@ -2631,11 +2631,11 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>미창석유</t>
+          <t>발레로 에너지</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>18</v>
+        <v>6</v>
       </c>
       <c r="D27" t="inlineStr">
         <is>
@@ -2646,17 +2646,17 @@
         <v>1</v>
       </c>
       <c r="F27" t="n">
-        <v>2097000</v>
+        <v>2165691.085066516</v>
       </c>
       <c r="G27" t="n">
-        <v>-295200</v>
+        <v>101701.085066516</v>
       </c>
       <c r="H27" t="n">
-        <v>-12.34010534236268</v>
+        <v>4.927402025519307</v>
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>2026-03-21T04:54:38</t>
+          <t>2026-03-21T04:57:02</t>
         </is>
       </c>
     </row>
@@ -2668,7 +2668,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>하나금융지주</t>
+          <t>미창석유</t>
         </is>
       </c>
       <c r="C28" t="n">
@@ -2683,17 +2683,17 @@
         <v>1</v>
       </c>
       <c r="F28" t="n">
-        <v>2037600</v>
+        <v>2097000</v>
       </c>
       <c r="G28" t="n">
-        <v>12200</v>
+        <v>-295200</v>
       </c>
       <c r="H28" t="n">
-        <v>0.6023501530561864</v>
+        <v>-12.34010534236268</v>
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>2026-03-21T04:54:38</t>
+          <t>2026-03-21T04:57:02</t>
         </is>
       </c>
     </row>
@@ -2705,11 +2705,11 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>대창단조</t>
+          <t>하나금융지주</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>300</v>
+        <v>18</v>
       </c>
       <c r="D29" t="inlineStr">
         <is>
@@ -2720,17 +2720,17 @@
         <v>1</v>
       </c>
       <c r="F29" t="n">
-        <v>2004000</v>
+        <v>2037600</v>
       </c>
       <c r="G29" t="n">
-        <v>-54000</v>
+        <v>12200</v>
       </c>
       <c r="H29" t="n">
-        <v>-2.623906705539359</v>
+        <v>0.6023501530561864</v>
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>2026-03-21T04:54:38</t>
+          <t>2026-03-21T04:57:02</t>
         </is>
       </c>
     </row>
@@ -2742,11 +2742,11 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>동방</t>
+          <t>대창단조</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>681</v>
+        <v>300</v>
       </c>
       <c r="D30" t="inlineStr">
         <is>
@@ -2757,17 +2757,17 @@
         <v>1</v>
       </c>
       <c r="F30" t="n">
-        <v>1995330</v>
+        <v>2004000</v>
       </c>
       <c r="G30" t="n">
-        <v>23829</v>
+        <v>-54000</v>
       </c>
       <c r="H30" t="n">
-        <v>1.208672985709873</v>
+        <v>-2.623906705539359</v>
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>2026-03-21T04:54:38</t>
+          <t>2026-03-21T04:57:02</t>
         </is>
       </c>
     </row>
@@ -2779,11 +2779,11 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>스타 벌크 캐리어스</t>
+          <t>동방</t>
         </is>
       </c>
       <c r="C31" t="n">
-        <v>50</v>
+        <v>681</v>
       </c>
       <c r="D31" t="inlineStr">
         <is>
@@ -2794,17 +2794,17 @@
         <v>1</v>
       </c>
       <c r="F31" t="n">
-        <v>1680142.640194588</v>
+        <v>1995330</v>
       </c>
       <c r="G31" t="n">
-        <v>365789.6401945879</v>
+        <v>23829</v>
       </c>
       <c r="H31" t="n">
-        <v>27.83039565433242</v>
+        <v>1.208672985709873</v>
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>2026-03-21T04:54:38</t>
+          <t>2026-03-21T04:57:02</t>
         </is>
       </c>
     </row>
@@ -2816,7 +2816,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>케이씨</t>
+          <t>스타 벌크 캐리어스</t>
         </is>
       </c>
       <c r="C32" t="n">
@@ -2831,17 +2831,17 @@
         <v>1</v>
       </c>
       <c r="F32" t="n">
-        <v>1670000</v>
+        <v>1680142.640194588</v>
       </c>
       <c r="G32" t="n">
-        <v>20500</v>
+        <v>365789.6401945879</v>
       </c>
       <c r="H32" t="n">
-        <v>1.242800848742043</v>
+        <v>27.83039565433242</v>
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>2026-03-21T04:54:38</t>
+          <t>2026-03-21T04:57:02</t>
         </is>
       </c>
     </row>
@@ -2853,11 +2853,11 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>유나이티드헬스 그룹</t>
+          <t>케이씨</t>
         </is>
       </c>
       <c r="C33" t="n">
-        <v>4</v>
+        <v>50</v>
       </c>
       <c r="D33" t="inlineStr">
         <is>
@@ -2868,17 +2868,17 @@
         <v>1</v>
       </c>
       <c r="F33" t="n">
-        <v>1658864.328313038</v>
+        <v>1670000</v>
       </c>
       <c r="G33" t="n">
-        <v>-35591.67168696248</v>
+        <v>20500</v>
       </c>
       <c r="H33" t="n">
-        <v>-2.100477774988697</v>
+        <v>1.242800848742043</v>
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>2026-03-21T04:54:38</t>
+          <t>2026-03-21T04:57:02</t>
         </is>
       </c>
     </row>
@@ -2890,11 +2890,11 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>텍사스 퍼시픽 랜드</t>
+          <t>유나이티드헬스 그룹</t>
         </is>
       </c>
       <c r="C34" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D34" t="inlineStr">
         <is>
@@ -2905,17 +2905,17 @@
         <v>1</v>
       </c>
       <c r="F34" t="n">
-        <v>1563247.374122903</v>
+        <v>1658864.328313038</v>
       </c>
       <c r="G34" t="n">
-        <v>-14646.62587709725</v>
+        <v>-35591.67168696248</v>
       </c>
       <c r="H34" t="n">
-        <v>-0.9282388979929735</v>
+        <v>-2.100477774988697</v>
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>2026-03-21T04:54:38</t>
+          <t>2026-03-21T04:57:02</t>
         </is>
       </c>
     </row>
@@ -2927,11 +2927,11 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>LX인터내셔널</t>
+          <t>텍사스 퍼시픽 랜드</t>
         </is>
       </c>
       <c r="C35" t="n">
-        <v>20</v>
+        <v>2</v>
       </c>
       <c r="D35" t="inlineStr">
         <is>
@@ -2942,17 +2942,17 @@
         <v>1</v>
       </c>
       <c r="F35" t="n">
-        <v>944108</v>
+        <v>1563247.374122903</v>
       </c>
       <c r="G35" t="n">
-        <v>5108</v>
+        <v>-14646.62587709725</v>
       </c>
       <c r="H35" t="n">
-        <v>0.5439829605963792</v>
+        <v>-0.9282388979929735</v>
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>2026-03-21T04:54:38</t>
+          <t>2026-03-21T04:57:02</t>
         </is>
       </c>
     </row>
@@ -2964,11 +2964,11 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>삼성생명</t>
+          <t>LX인터내셔널</t>
         </is>
       </c>
       <c r="C36" t="n">
-        <v>4</v>
+        <v>20</v>
       </c>
       <c r="D36" t="inlineStr">
         <is>
@@ -2979,17 +2979,17 @@
         <v>1</v>
       </c>
       <c r="F36" t="n">
-        <v>926000</v>
+        <v>943000</v>
       </c>
       <c r="G36" t="n">
-        <v>93000</v>
+        <v>4000</v>
       </c>
       <c r="H36" t="n">
-        <v>11.16446578631453</v>
+        <v>0.4259850905218318</v>
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>2026-03-21T04:54:38</t>
+          <t>2026-03-21T04:57:02</t>
         </is>
       </c>
     </row>
@@ -3001,11 +3001,11 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>비에이치아이</t>
+          <t>삼성생명</t>
         </is>
       </c>
       <c r="C37" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="D37" t="inlineStr">
         <is>
@@ -3016,17 +3016,17 @@
         <v>1</v>
       </c>
       <c r="F37" t="n">
-        <v>876000</v>
+        <v>926000</v>
       </c>
       <c r="G37" t="n">
-        <v>210885</v>
+        <v>93000</v>
       </c>
       <c r="H37" t="n">
-        <v>31.70654698811484</v>
+        <v>11.16446578631453</v>
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>2026-03-21T04:54:38</t>
+          <t>2026-03-21T04:57:02</t>
         </is>
       </c>
     </row>
@@ -3038,11 +3038,11 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>하프니아</t>
+          <t>비에이치아이</t>
         </is>
       </c>
       <c r="C38" t="n">
-        <v>80</v>
+        <v>8</v>
       </c>
       <c r="D38" t="inlineStr">
         <is>
@@ -3053,17 +3053,17 @@
         <v>1</v>
       </c>
       <c r="F38" t="n">
-        <v>842704.775390625</v>
+        <v>876000</v>
       </c>
       <c r="G38" t="n">
-        <v>216973.775390625</v>
+        <v>210885</v>
       </c>
       <c r="H38" t="n">
-        <v>34.67524789256486</v>
+        <v>31.70654698811484</v>
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>2026-03-21T04:54:38</t>
+          <t>2026-03-21T04:57:02</t>
         </is>
       </c>
     </row>
@@ -3075,11 +3075,11 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>클리블랜드 클리프스</t>
+          <t>하프니아</t>
         </is>
       </c>
       <c r="C39" t="n">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="D39" t="inlineStr">
         <is>
@@ -3090,17 +3090,17 @@
         <v>1</v>
       </c>
       <c r="F39" t="n">
-        <v>823743.9360268187</v>
+        <v>842704.775390625</v>
       </c>
       <c r="G39" t="n">
-        <v>-192311.0639731813</v>
+        <v>216973.775390625</v>
       </c>
       <c r="H39" t="n">
-        <v>-18.92722972409774</v>
+        <v>34.67524789256486</v>
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>2026-03-21T04:54:38</t>
+          <t>2026-03-21T04:57:02</t>
         </is>
       </c>
     </row>
@@ -3112,11 +3112,11 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>낫 오프쇼어 파트너스</t>
+          <t>클리블랜드 클리프스</t>
         </is>
       </c>
       <c r="C40" t="n">
-        <v>30</v>
+        <v>70</v>
       </c>
       <c r="D40" t="inlineStr">
         <is>
@@ -3127,17 +3127,17 @@
         <v>1</v>
       </c>
       <c r="F40" t="n">
-        <v>410853</v>
+        <v>823743.9360268187</v>
       </c>
       <c r="G40" t="n">
-        <v>-6662</v>
+        <v>-192311.0639731813</v>
       </c>
       <c r="H40" t="n">
-        <v>-1.595631294684023</v>
+        <v>-18.92722972409774</v>
       </c>
       <c r="I40" t="inlineStr">
         <is>
-          <t>2026-03-21T04:54:38</t>
+          <t>2026-03-21T04:57:02</t>
         </is>
       </c>
     </row>
@@ -3149,11 +3149,11 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>NH투자증권우</t>
+          <t>낫 오프쇼어 파트너스</t>
         </is>
       </c>
       <c r="C41" t="n">
-        <v>2</v>
+        <v>30</v>
       </c>
       <c r="D41" t="inlineStr">
         <is>
@@ -3164,17 +3164,17 @@
         <v>1</v>
       </c>
       <c r="F41" t="n">
-        <v>54591</v>
+        <v>413075.8057155996</v>
       </c>
       <c r="G41" t="n">
-        <v>-9</v>
+        <v>-4439.194284400437</v>
       </c>
       <c r="H41" t="n">
-        <v>-0.01648351648351648</v>
+        <v>-1.063241867813237</v>
       </c>
       <c r="I41" t="inlineStr">
         <is>
-          <t>2026-03-21T04:54:38</t>
+          <t>2026-03-21T04:57:02</t>
         </is>
       </c>
     </row>
@@ -3186,11 +3186,11 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>노블</t>
+          <t>NH투자증권우</t>
         </is>
       </c>
       <c r="C42" t="n">
-        <v>99</v>
+        <v>2</v>
       </c>
       <c r="D42" t="inlineStr">
         <is>
@@ -3201,17 +3201,17 @@
         <v>1</v>
       </c>
       <c r="F42" t="n">
-        <v>40689</v>
+        <v>54700</v>
       </c>
       <c r="G42" t="n">
-        <v>-3866519</v>
+        <v>100</v>
       </c>
       <c r="H42" t="n">
-        <v>-98.95861699709869</v>
+        <v>0.1831501831501831</v>
       </c>
       <c r="I42" t="inlineStr">
         <is>
-          <t>2026-03-21T04:54:38</t>
+          <t>2026-03-21T04:57:02</t>
         </is>
       </c>
     </row>
@@ -3275,7 +3275,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>2026-03-21T04:54:51</t>
+          <t>2026-03-21T04:57:02</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: portfolio snapshot 2026-03-21 (2026-03-21T04:57:12)
</commit_message>
<xml_diff>
--- a/portfolio_auto.xlsx
+++ b/portfolio_auto.xlsx
@@ -1630,7 +1630,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2026-03-21T04:57:02</t>
+          <t>2026-03-21T04:57:12</t>
         </is>
       </c>
       <c r="E2" t="n">
@@ -1731,7 +1731,7 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>2026-03-21T04:57:02</t>
+          <t>2026-03-21T04:57:12</t>
         </is>
       </c>
     </row>
@@ -1768,7 +1768,7 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>2026-03-21T04:57:02</t>
+          <t>2026-03-21T04:57:12</t>
         </is>
       </c>
     </row>
@@ -1805,7 +1805,7 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>2026-03-21T04:57:02</t>
+          <t>2026-03-21T04:57:12</t>
         </is>
       </c>
     </row>
@@ -1842,7 +1842,7 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>2026-03-21T04:57:02</t>
+          <t>2026-03-21T04:57:12</t>
         </is>
       </c>
     </row>
@@ -1879,7 +1879,7 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>2026-03-21T04:57:02</t>
+          <t>2026-03-21T04:57:12</t>
         </is>
       </c>
     </row>
@@ -1916,7 +1916,7 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>2026-03-21T04:57:02</t>
+          <t>2026-03-21T04:57:12</t>
         </is>
       </c>
     </row>
@@ -1953,7 +1953,7 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>2026-03-21T04:57:02</t>
+          <t>2026-03-21T04:57:12</t>
         </is>
       </c>
     </row>
@@ -1990,7 +1990,7 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>2026-03-21T04:57:02</t>
+          <t>2026-03-21T04:57:12</t>
         </is>
       </c>
     </row>
@@ -2027,7 +2027,7 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>2026-03-21T04:57:02</t>
+          <t>2026-03-21T04:57:12</t>
         </is>
       </c>
     </row>
@@ -2064,7 +2064,7 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>2026-03-21T04:57:02</t>
+          <t>2026-03-21T04:57:12</t>
         </is>
       </c>
     </row>
@@ -2101,7 +2101,7 @@
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>2026-03-21T04:57:02</t>
+          <t>2026-03-21T04:57:12</t>
         </is>
       </c>
     </row>
@@ -2138,7 +2138,7 @@
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>2026-03-21T04:57:02</t>
+          <t>2026-03-21T04:57:12</t>
         </is>
       </c>
     </row>
@@ -2175,7 +2175,7 @@
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>2026-03-21T04:57:02</t>
+          <t>2026-03-21T04:57:12</t>
         </is>
       </c>
     </row>
@@ -2212,7 +2212,7 @@
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>2026-03-21T04:57:02</t>
+          <t>2026-03-21T04:57:12</t>
         </is>
       </c>
     </row>
@@ -2249,7 +2249,7 @@
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>2026-03-21T04:57:02</t>
+          <t>2026-03-21T04:57:12</t>
         </is>
       </c>
     </row>
@@ -2286,7 +2286,7 @@
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>2026-03-21T04:57:02</t>
+          <t>2026-03-21T04:57:12</t>
         </is>
       </c>
     </row>
@@ -2323,7 +2323,7 @@
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>2026-03-21T04:57:02</t>
+          <t>2026-03-21T04:57:12</t>
         </is>
       </c>
     </row>
@@ -2360,7 +2360,7 @@
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>2026-03-21T04:57:02</t>
+          <t>2026-03-21T04:57:12</t>
         </is>
       </c>
     </row>
@@ -2397,7 +2397,7 @@
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>2026-03-21T04:57:02</t>
+          <t>2026-03-21T04:57:12</t>
         </is>
       </c>
     </row>
@@ -2434,7 +2434,7 @@
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>2026-03-21T04:57:02</t>
+          <t>2026-03-21T04:57:12</t>
         </is>
       </c>
     </row>
@@ -2471,7 +2471,7 @@
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>2026-03-21T04:57:02</t>
+          <t>2026-03-21T04:57:12</t>
         </is>
       </c>
     </row>
@@ -2508,7 +2508,7 @@
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>2026-03-21T04:57:02</t>
+          <t>2026-03-21T04:57:12</t>
         </is>
       </c>
     </row>
@@ -2545,7 +2545,7 @@
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>2026-03-21T04:57:02</t>
+          <t>2026-03-21T04:57:12</t>
         </is>
       </c>
     </row>
@@ -2582,7 +2582,7 @@
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>2026-03-21T04:57:02</t>
+          <t>2026-03-21T04:57:12</t>
         </is>
       </c>
     </row>
@@ -2619,7 +2619,7 @@
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>2026-03-21T04:57:02</t>
+          <t>2026-03-21T04:57:12</t>
         </is>
       </c>
     </row>
@@ -2656,7 +2656,7 @@
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>2026-03-21T04:57:02</t>
+          <t>2026-03-21T04:57:12</t>
         </is>
       </c>
     </row>
@@ -2693,7 +2693,7 @@
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>2026-03-21T04:57:02</t>
+          <t>2026-03-21T04:57:12</t>
         </is>
       </c>
     </row>
@@ -2730,7 +2730,7 @@
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>2026-03-21T04:57:02</t>
+          <t>2026-03-21T04:57:12</t>
         </is>
       </c>
     </row>
@@ -2767,7 +2767,7 @@
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>2026-03-21T04:57:02</t>
+          <t>2026-03-21T04:57:12</t>
         </is>
       </c>
     </row>
@@ -2804,7 +2804,7 @@
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>2026-03-21T04:57:02</t>
+          <t>2026-03-21T04:57:12</t>
         </is>
       </c>
     </row>
@@ -2841,7 +2841,7 @@
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>2026-03-21T04:57:02</t>
+          <t>2026-03-21T04:57:12</t>
         </is>
       </c>
     </row>
@@ -2878,7 +2878,7 @@
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>2026-03-21T04:57:02</t>
+          <t>2026-03-21T04:57:12</t>
         </is>
       </c>
     </row>
@@ -2915,7 +2915,7 @@
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>2026-03-21T04:57:02</t>
+          <t>2026-03-21T04:57:12</t>
         </is>
       </c>
     </row>
@@ -2952,7 +2952,7 @@
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>2026-03-21T04:57:02</t>
+          <t>2026-03-21T04:57:12</t>
         </is>
       </c>
     </row>
@@ -2989,7 +2989,7 @@
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>2026-03-21T04:57:02</t>
+          <t>2026-03-21T04:57:12</t>
         </is>
       </c>
     </row>
@@ -3026,7 +3026,7 @@
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>2026-03-21T04:57:02</t>
+          <t>2026-03-21T04:57:12</t>
         </is>
       </c>
     </row>
@@ -3063,7 +3063,7 @@
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>2026-03-21T04:57:02</t>
+          <t>2026-03-21T04:57:12</t>
         </is>
       </c>
     </row>
@@ -3100,7 +3100,7 @@
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>2026-03-21T04:57:02</t>
+          <t>2026-03-21T04:57:12</t>
         </is>
       </c>
     </row>
@@ -3137,7 +3137,7 @@
       </c>
       <c r="I40" t="inlineStr">
         <is>
-          <t>2026-03-21T04:57:02</t>
+          <t>2026-03-21T04:57:12</t>
         </is>
       </c>
     </row>
@@ -3174,7 +3174,7 @@
       </c>
       <c r="I41" t="inlineStr">
         <is>
-          <t>2026-03-21T04:57:02</t>
+          <t>2026-03-21T04:57:12</t>
         </is>
       </c>
     </row>
@@ -3211,7 +3211,7 @@
       </c>
       <c r="I42" t="inlineStr">
         <is>
-          <t>2026-03-21T04:57:02</t>
+          <t>2026-03-21T04:57:12</t>
         </is>
       </c>
     </row>
@@ -3275,7 +3275,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>2026-03-21T04:57:02</t>
+          <t>2026-03-21T04:57:12</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: portfolio snapshot 2026-03-17 (2026-03-21T04:59:43)
</commit_message>
<xml_diff>
--- a/portfolio_auto.xlsx
+++ b/portfolio_auto.xlsx
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G42"/>
+  <dimension ref="A1:G11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -471,11 +471,11 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>유나이티드헬스 그룹</t>
+          <t>삼성화재</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
@@ -486,23 +486,23 @@
         <v>1</v>
       </c>
       <c r="E2" t="n">
-        <v>1658864.328313038</v>
+        <v>3321500</v>
       </c>
       <c r="F2" t="n">
-        <v>-35591.67168696248</v>
+        <v>-309500</v>
       </c>
       <c r="G2" t="n">
-        <v>-2.100477774988697</v>
+        <v>-8.523822638391627</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>AGNC 인베스트먼트</t>
+          <t>세아제강</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>700</v>
+        <v>50</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
@@ -513,23 +513,23 @@
         <v>1</v>
       </c>
       <c r="E3" t="n">
-        <v>10270464.45007324</v>
+        <v>7395000</v>
       </c>
       <c r="F3" t="n">
-        <v>-561550.5499267559</v>
+        <v>1085000</v>
       </c>
       <c r="G3" t="n">
-        <v>-5.184174411933109</v>
+        <v>17.19492868462758</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>센트러스 에너지</t>
+          <t>케이씨</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>25</v>
+        <v>50</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
@@ -540,23 +540,23 @@
         <v>1</v>
       </c>
       <c r="E4" t="n">
-        <v>7026050.85816239</v>
+        <v>1670000</v>
       </c>
       <c r="F4" t="n">
-        <v>-406805.1418376099</v>
+        <v>20500</v>
       </c>
       <c r="G4" t="n">
-        <v>-5.473066366920198</v>
+        <v>1.242800848742043</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>스타 벌크 캐리어스</t>
+          <t>하나금융지주</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>50</v>
+        <v>10</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -567,23 +567,23 @@
         <v>1</v>
       </c>
       <c r="E5" t="n">
-        <v>1680142.640194588</v>
+        <v>1132000</v>
       </c>
       <c r="F5" t="n">
-        <v>365789.6401945879</v>
+        <v>23000</v>
       </c>
       <c r="G5" t="n">
-        <v>27.83039565433242</v>
+        <v>2.073940486925157</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>시드릴</t>
+          <t>현대제철</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>123</v>
+        <v>70</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
@@ -594,23 +594,23 @@
         <v>1</v>
       </c>
       <c r="E6" t="n">
-        <v>8070101.805898919</v>
+        <v>2621500</v>
       </c>
       <c r="F6" t="n">
-        <v>1619750.805898919</v>
+        <v>-186000</v>
       </c>
       <c r="G6" t="n">
-        <v>25.11104908707943</v>
+        <v>-6.625111308993767</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>오케아니스 에코 탱커스</t>
+          <t>휴스틸</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>65</v>
+        <v>500</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -621,23 +621,23 @@
         <v>1</v>
       </c>
       <c r="E7" t="n">
-        <v>4511179.137784176</v>
+        <v>2750000</v>
       </c>
       <c r="F7" t="n">
-        <v>2254819.137784176</v>
+        <v>471390</v>
       </c>
       <c r="G7" t="n">
-        <v>99.93171026716374</v>
+        <v>20.68761218462133</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>차코스 에너지 내비게이션</t>
+          <t>DL이앤씨</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>75</v>
+        <v>80</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
@@ -648,23 +648,23 @@
         <v>1</v>
       </c>
       <c r="E8" t="n">
-        <v>4026924.996845168</v>
+        <v>5392000</v>
       </c>
       <c r="F8" t="n">
-        <v>202276.9968451681</v>
+        <v>1981000</v>
       </c>
       <c r="G8" t="n">
-        <v>5.28877420471552</v>
+        <v>58.07681031955438</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>클리블랜드 클리프스</t>
+          <t>HD건설기계</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>70</v>
+        <v>31</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
@@ -675,23 +675,23 @@
         <v>1</v>
       </c>
       <c r="E9" t="n">
-        <v>823743.9360268187</v>
+        <v>4123000</v>
       </c>
       <c r="F9" t="n">
-        <v>-192311.0639731813</v>
+        <v>87904</v>
       </c>
       <c r="G9" t="n">
-        <v>-18.92722972409774</v>
+        <v>2.178485964150543</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>타이드워터</t>
+          <t>KoAct 코스닥액티브</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>48</v>
+        <v>200</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
@@ -702,23 +702,23 @@
         <v>1</v>
       </c>
       <c r="E10" t="n">
-        <v>5235363.852789983</v>
+        <v>2582000</v>
       </c>
       <c r="F10" t="n">
-        <v>1510818.852789983</v>
+        <v>-120000</v>
       </c>
       <c r="G10" t="n">
-        <v>40.56385015592463</v>
+        <v>-4.441154700222058</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>텍사스 퍼시픽 랜드</t>
+          <t>TIME 코리아밸류업액티브</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>2</v>
+        <v>201</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
@@ -729,850 +729,13 @@
         <v>1</v>
       </c>
       <c r="E11" t="n">
-        <v>1563247.374122903</v>
+        <v>4797870</v>
       </c>
       <c r="F11" t="n">
-        <v>-14646.62587709725</v>
+        <v>74073</v>
       </c>
       <c r="G11" t="n">
-        <v>-0.9282388979929735</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>트랜스오션</t>
-        </is>
-      </c>
-      <c r="B12" t="n">
-        <v>750</v>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>KRW</t>
-        </is>
-      </c>
-      <c r="D12" t="n">
-        <v>1</v>
-      </c>
-      <c r="E12" t="n">
-        <v>7020031.5082007</v>
-      </c>
-      <c r="F12" t="n">
-        <v>2892797.5082007</v>
-      </c>
-      <c r="G12" t="n">
-        <v>70.09046514446965</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>페트로브라스 (ADR)</t>
-        </is>
-      </c>
-      <c r="B13" t="n">
-        <v>480</v>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>KRW</t>
-        </is>
-      </c>
-      <c r="D13" t="n">
-        <v>1</v>
-      </c>
-      <c r="E13" t="n">
-        <v>13579584.97235231</v>
-      </c>
-      <c r="F13" t="n">
-        <v>1473035.972352311</v>
-      </c>
-      <c r="G13" t="n">
-        <v>12.16726560436265</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>프론트라인</t>
-        </is>
-      </c>
-      <c r="B14" t="n">
-        <v>175</v>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>KRW</t>
-        </is>
-      </c>
-      <c r="D14" t="n">
-        <v>1</v>
-      </c>
-      <c r="E14" t="n">
-        <v>8471815.962899337</v>
-      </c>
-      <c r="F14" t="n">
-        <v>4041951.962899337</v>
-      </c>
-      <c r="G14" t="n">
-        <v>91.24325177701475</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>피바디 에너지</t>
-        </is>
-      </c>
-      <c r="B15" t="n">
-        <v>65</v>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>KRW</t>
-        </is>
-      </c>
-      <c r="D15" t="n">
-        <v>1</v>
-      </c>
-      <c r="E15" t="n">
-        <v>3649438.50225304</v>
-      </c>
-      <c r="F15" t="n">
-        <v>2178666.50225304</v>
-      </c>
-      <c r="G15" t="n">
-        <v>148.1308117269733</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>하프니아</t>
-        </is>
-      </c>
-      <c r="B16" t="n">
-        <v>80</v>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>KRW</t>
-        </is>
-      </c>
-      <c r="D16" t="n">
-        <v>1</v>
-      </c>
-      <c r="E16" t="n">
-        <v>842704.775390625</v>
-      </c>
-      <c r="F16" t="n">
-        <v>216973.775390625</v>
-      </c>
-      <c r="G16" t="n">
-        <v>34.67524789256486</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>DL이앤씨</t>
-        </is>
-      </c>
-      <c r="B17" t="n">
-        <v>40</v>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>KRW</t>
-        </is>
-      </c>
-      <c r="D17" t="n">
-        <v>1</v>
-      </c>
-      <c r="E17" t="n">
-        <v>2696000</v>
-      </c>
-      <c r="F17" t="n">
-        <v>990500</v>
-      </c>
-      <c r="G17" t="n">
-        <v>58.07681031955438</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>HD건설기계</t>
-        </is>
-      </c>
-      <c r="B18" t="n">
-        <v>31</v>
-      </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>KRW</t>
-        </is>
-      </c>
-      <c r="D18" t="n">
-        <v>1</v>
-      </c>
-      <c r="E18" t="n">
-        <v>4123000</v>
-      </c>
-      <c r="F18" t="n">
-        <v>87904</v>
-      </c>
-      <c r="G18" t="n">
-        <v>2.178485964150543</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>KoAct 코스닥액티브</t>
-        </is>
-      </c>
-      <c r="B19" t="n">
-        <v>200</v>
-      </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>KRW</t>
-        </is>
-      </c>
-      <c r="D19" t="n">
-        <v>1</v>
-      </c>
-      <c r="E19" t="n">
-        <v>2582000</v>
-      </c>
-      <c r="F19" t="n">
-        <v>-120000</v>
-      </c>
-      <c r="G19" t="n">
-        <v>-4.441154700222058</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>LX인터내셔널</t>
-        </is>
-      </c>
-      <c r="B20" t="n">
-        <v>20</v>
-      </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>KRW</t>
-        </is>
-      </c>
-      <c r="D20" t="n">
-        <v>1</v>
-      </c>
-      <c r="E20" t="n">
-        <v>943000</v>
-      </c>
-      <c r="F20" t="n">
-        <v>4000</v>
-      </c>
-      <c r="G20" t="n">
-        <v>0.4259850905218318</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>NH투자증권우</t>
-        </is>
-      </c>
-      <c r="B21" t="n">
-        <v>2</v>
-      </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>KRW</t>
-        </is>
-      </c>
-      <c r="D21" t="n">
-        <v>1</v>
-      </c>
-      <c r="E21" t="n">
-        <v>54700</v>
-      </c>
-      <c r="F21" t="n">
-        <v>100</v>
-      </c>
-      <c r="G21" t="n">
-        <v>0.1831501831501831</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>TIME 코리아밸류업액티브</t>
-        </is>
-      </c>
-      <c r="B22" t="n">
-        <v>201</v>
-      </c>
-      <c r="C22" t="inlineStr">
-        <is>
-          <t>KRW</t>
-        </is>
-      </c>
-      <c r="D22" t="n">
-        <v>1</v>
-      </c>
-      <c r="E22" t="n">
-        <v>4797870</v>
-      </c>
-      <c r="F22" t="n">
-        <v>74073</v>
-      </c>
-      <c r="G22" t="n">
         <v>1.568081778281328</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>노브</t>
-        </is>
-      </c>
-      <c r="B23" t="n">
-        <v>185</v>
-      </c>
-      <c r="C23" t="inlineStr">
-        <is>
-          <t>KRW</t>
-        </is>
-      </c>
-      <c r="D23" t="n">
-        <v>1</v>
-      </c>
-      <c r="E23" t="n">
-        <v>5200391.447092756</v>
-      </c>
-      <c r="F23" t="n">
-        <v>1890383.447092756</v>
-      </c>
-      <c r="G23" t="n">
-        <v>57.11114435653194</v>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>노블</t>
-        </is>
-      </c>
-      <c r="B24" t="n">
-        <v>99</v>
-      </c>
-      <c r="C24" t="inlineStr">
-        <is>
-          <t>KRW</t>
-        </is>
-      </c>
-      <c r="D24" t="n">
-        <v>1</v>
-      </c>
-      <c r="E24" t="n">
-        <v>6958769.981090547</v>
-      </c>
-      <c r="F24" t="n">
-        <v>3051561.981090547</v>
-      </c>
-      <c r="G24" t="n">
-        <v>78.10083264291399</v>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>낫 오프쇼어 파트너스</t>
-        </is>
-      </c>
-      <c r="B25" t="n">
-        <v>30</v>
-      </c>
-      <c r="C25" t="inlineStr">
-        <is>
-          <t>KRW</t>
-        </is>
-      </c>
-      <c r="D25" t="n">
-        <v>1</v>
-      </c>
-      <c r="E25" t="n">
-        <v>413075.8057155996</v>
-      </c>
-      <c r="F25" t="n">
-        <v>-4439.194284400437</v>
-      </c>
-      <c r="G25" t="n">
-        <v>-1.063241867813237</v>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>더치 브로스</t>
-        </is>
-      </c>
-      <c r="B26" t="n">
-        <v>39</v>
-      </c>
-      <c r="C26" t="inlineStr">
-        <is>
-          <t>KRW</t>
-        </is>
-      </c>
-      <c r="D26" t="n">
-        <v>1</v>
-      </c>
-      <c r="E26" t="n">
-        <v>2934418.414306641</v>
-      </c>
-      <c r="F26" t="n">
-        <v>-256226.5856933594</v>
-      </c>
-      <c r="G26" t="n">
-        <v>-8.030557636257226</v>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>발레로 에너지</t>
-        </is>
-      </c>
-      <c r="B27" t="n">
-        <v>6</v>
-      </c>
-      <c r="C27" t="inlineStr">
-        <is>
-          <t>KRW</t>
-        </is>
-      </c>
-      <c r="D27" t="n">
-        <v>1</v>
-      </c>
-      <c r="E27" t="n">
-        <v>2165691.085066516</v>
-      </c>
-      <c r="F27" t="n">
-        <v>101701.085066516</v>
-      </c>
-      <c r="G27" t="n">
-        <v>4.927402025519307</v>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>넥스틸</t>
-        </is>
-      </c>
-      <c r="B28" t="n">
-        <v>300</v>
-      </c>
-      <c r="C28" t="inlineStr">
-        <is>
-          <t>KRW</t>
-        </is>
-      </c>
-      <c r="D28" t="n">
-        <v>1</v>
-      </c>
-      <c r="E28" t="n">
-        <v>3771000</v>
-      </c>
-      <c r="F28" t="n">
-        <v>521000</v>
-      </c>
-      <c r="G28" t="n">
-        <v>16.03076923076923</v>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>대신증권</t>
-        </is>
-      </c>
-      <c r="B29" t="n">
-        <v>55</v>
-      </c>
-      <c r="C29" t="inlineStr">
-        <is>
-          <t>KRW</t>
-        </is>
-      </c>
-      <c r="D29" t="n">
-        <v>1</v>
-      </c>
-      <c r="E29" t="n">
-        <v>2219250</v>
-      </c>
-      <c r="F29" t="n">
-        <v>509749</v>
-      </c>
-      <c r="G29" t="n">
-        <v>29.81858448752005</v>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t>대창단조</t>
-        </is>
-      </c>
-      <c r="B30" t="n">
-        <v>300</v>
-      </c>
-      <c r="C30" t="inlineStr">
-        <is>
-          <t>KRW</t>
-        </is>
-      </c>
-      <c r="D30" t="n">
-        <v>1</v>
-      </c>
-      <c r="E30" t="n">
-        <v>2004000</v>
-      </c>
-      <c r="F30" t="n">
-        <v>-54000</v>
-      </c>
-      <c r="G30" t="n">
-        <v>-2.623906705539359</v>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="inlineStr">
-        <is>
-          <t>대한조선</t>
-        </is>
-      </c>
-      <c r="B31" t="n">
-        <v>100</v>
-      </c>
-      <c r="C31" t="inlineStr">
-        <is>
-          <t>KRW</t>
-        </is>
-      </c>
-      <c r="D31" t="n">
-        <v>1</v>
-      </c>
-      <c r="E31" t="n">
-        <v>9120000</v>
-      </c>
-      <c r="F31" t="n">
-        <v>1907000</v>
-      </c>
-      <c r="G31" t="n">
-        <v>26.43837515596839</v>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="inlineStr">
-        <is>
-          <t>동방</t>
-        </is>
-      </c>
-      <c r="B32" t="n">
-        <v>681</v>
-      </c>
-      <c r="C32" t="inlineStr">
-        <is>
-          <t>KRW</t>
-        </is>
-      </c>
-      <c r="D32" t="n">
-        <v>1</v>
-      </c>
-      <c r="E32" t="n">
-        <v>1995330</v>
-      </c>
-      <c r="F32" t="n">
-        <v>23829</v>
-      </c>
-      <c r="G32" t="n">
-        <v>1.208672985709873</v>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" t="inlineStr">
-        <is>
-          <t>동원개발</t>
-        </is>
-      </c>
-      <c r="B33" t="n">
-        <v>1360</v>
-      </c>
-      <c r="C33" t="inlineStr">
-        <is>
-          <t>KRW</t>
-        </is>
-      </c>
-      <c r="D33" t="n">
-        <v>1</v>
-      </c>
-      <c r="E33" t="n">
-        <v>4202400</v>
-      </c>
-      <c r="F33" t="n">
-        <v>465000</v>
-      </c>
-      <c r="G33" t="n">
-        <v>12.44180446299566</v>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" t="inlineStr">
-        <is>
-          <t>미창석유</t>
-        </is>
-      </c>
-      <c r="B34" t="n">
-        <v>18</v>
-      </c>
-      <c r="C34" t="inlineStr">
-        <is>
-          <t>KRW</t>
-        </is>
-      </c>
-      <c r="D34" t="n">
-        <v>1</v>
-      </c>
-      <c r="E34" t="n">
-        <v>2097000</v>
-      </c>
-      <c r="F34" t="n">
-        <v>-295200</v>
-      </c>
-      <c r="G34" t="n">
-        <v>-12.34010534236268</v>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" t="inlineStr">
-        <is>
-          <t>비에이치아이</t>
-        </is>
-      </c>
-      <c r="B35" t="n">
-        <v>8</v>
-      </c>
-      <c r="C35" t="inlineStr">
-        <is>
-          <t>KRW</t>
-        </is>
-      </c>
-      <c r="D35" t="n">
-        <v>1</v>
-      </c>
-      <c r="E35" t="n">
-        <v>876000</v>
-      </c>
-      <c r="F35" t="n">
-        <v>210885</v>
-      </c>
-      <c r="G35" t="n">
-        <v>31.70654698811484</v>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" t="inlineStr">
-        <is>
-          <t>삼성생명</t>
-        </is>
-      </c>
-      <c r="B36" t="n">
-        <v>4</v>
-      </c>
-      <c r="C36" t="inlineStr">
-        <is>
-          <t>KRW</t>
-        </is>
-      </c>
-      <c r="D36" t="n">
-        <v>1</v>
-      </c>
-      <c r="E36" t="n">
-        <v>926000</v>
-      </c>
-      <c r="F36" t="n">
-        <v>93000</v>
-      </c>
-      <c r="G36" t="n">
-        <v>11.16446578631453</v>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" t="inlineStr">
-        <is>
-          <t>삼성화재</t>
-        </is>
-      </c>
-      <c r="B37" t="n">
-        <v>9</v>
-      </c>
-      <c r="C37" t="inlineStr">
-        <is>
-          <t>KRW</t>
-        </is>
-      </c>
-      <c r="D37" t="n">
-        <v>1</v>
-      </c>
-      <c r="E37" t="n">
-        <v>4270500</v>
-      </c>
-      <c r="F37" t="n">
-        <v>-360500</v>
-      </c>
-      <c r="G37" t="n">
-        <v>-7.784495789246384</v>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" t="inlineStr">
-        <is>
-          <t>세아제강</t>
-        </is>
-      </c>
-      <c r="B38" t="n">
-        <v>50</v>
-      </c>
-      <c r="C38" t="inlineStr">
-        <is>
-          <t>KRW</t>
-        </is>
-      </c>
-      <c r="D38" t="n">
-        <v>1</v>
-      </c>
-      <c r="E38" t="n">
-        <v>7395000</v>
-      </c>
-      <c r="F38" t="n">
-        <v>1085000</v>
-      </c>
-      <c r="G38" t="n">
-        <v>17.19492868462758</v>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" t="inlineStr">
-        <is>
-          <t>케이씨</t>
-        </is>
-      </c>
-      <c r="B39" t="n">
-        <v>50</v>
-      </c>
-      <c r="C39" t="inlineStr">
-        <is>
-          <t>KRW</t>
-        </is>
-      </c>
-      <c r="D39" t="n">
-        <v>1</v>
-      </c>
-      <c r="E39" t="n">
-        <v>1670000</v>
-      </c>
-      <c r="F39" t="n">
-        <v>20500</v>
-      </c>
-      <c r="G39" t="n">
-        <v>1.242800848742043</v>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" t="inlineStr">
-        <is>
-          <t>하나금융지주</t>
-        </is>
-      </c>
-      <c r="B40" t="n">
-        <v>18</v>
-      </c>
-      <c r="C40" t="inlineStr">
-        <is>
-          <t>KRW</t>
-        </is>
-      </c>
-      <c r="D40" t="n">
-        <v>1</v>
-      </c>
-      <c r="E40" t="n">
-        <v>2037600</v>
-      </c>
-      <c r="F40" t="n">
-        <v>12200</v>
-      </c>
-      <c r="G40" t="n">
-        <v>0.6023501530561864</v>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" t="inlineStr">
-        <is>
-          <t>현대제철</t>
-        </is>
-      </c>
-      <c r="B41" t="n">
-        <v>80</v>
-      </c>
-      <c r="C41" t="inlineStr">
-        <is>
-          <t>KRW</t>
-        </is>
-      </c>
-      <c r="D41" t="n">
-        <v>1</v>
-      </c>
-      <c r="E41" t="n">
-        <v>2996000</v>
-      </c>
-      <c r="F41" t="n">
-        <v>-182000</v>
-      </c>
-      <c r="G41" t="n">
-        <v>-5.726872246696035</v>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" t="inlineStr">
-        <is>
-          <t>휴스틸</t>
-        </is>
-      </c>
-      <c r="B42" t="n">
-        <v>500</v>
-      </c>
-      <c r="C42" t="inlineStr">
-        <is>
-          <t>KRW</t>
-        </is>
-      </c>
-      <c r="D42" t="n">
-        <v>1</v>
-      </c>
-      <c r="E42" t="n">
-        <v>2750000</v>
-      </c>
-      <c r="F42" t="n">
-        <v>471390</v>
-      </c>
-      <c r="G42" t="n">
-        <v>20.68761218462133</v>
       </c>
     </row>
   </sheetData>
@@ -1619,22 +782,22 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-03-21</t>
+          <t>2026-03-17</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>31036676</v>
+        <v>0</v>
       </c>
       <c r="C2" t="n">
-        <v>12663.38</v>
+        <v>0</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2026-03-21T04:57:12</t>
+          <t>2026-03-21T04:59:43</t>
         </is>
       </c>
       <c r="E2" t="n">
-        <v>1504.829956054688</v>
+        <v>1488.910034179688</v>
       </c>
     </row>
   </sheetData>
@@ -1648,7 +811,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I42"/>
+  <dimension ref="A1:I52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1701,16 +864,16 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-03-21</t>
+          <t>2026-03-17</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>페트로브라스 (ADR)</t>
+          <t>세아제강</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>480</v>
+        <v>50</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
@@ -1721,33 +884,33 @@
         <v>1</v>
       </c>
       <c r="F2" t="n">
-        <v>13579584.97235231</v>
+        <v>7395000</v>
       </c>
       <c r="G2" t="n">
-        <v>1473035.972352311</v>
+        <v>1085000</v>
       </c>
       <c r="H2" t="n">
-        <v>12.16726560436265</v>
+        <v>17.19492868462758</v>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>2026-03-21T04:57:12</t>
+          <t>2026-03-21T04:59:43</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-03-21</t>
+          <t>2026-03-17</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>AGNC 인베스트먼트</t>
+          <t>DL이앤씨</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>700</v>
+        <v>80</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
@@ -1758,33 +921,33 @@
         <v>1</v>
       </c>
       <c r="F3" t="n">
-        <v>10270464.45007324</v>
+        <v>5392000</v>
       </c>
       <c r="G3" t="n">
-        <v>-561550.5499267559</v>
+        <v>1981000</v>
       </c>
       <c r="H3" t="n">
-        <v>-5.184174411933109</v>
+        <v>58.07681031955438</v>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>2026-03-21T04:57:12</t>
+          <t>2026-03-21T04:59:43</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-03-21</t>
+          <t>2026-03-17</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>대한조선</t>
+          <t>TIME 코리아밸류업액티브</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>100</v>
+        <v>201</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
@@ -1795,33 +958,33 @@
         <v>1</v>
       </c>
       <c r="F4" t="n">
-        <v>9120000</v>
+        <v>4797870</v>
       </c>
       <c r="G4" t="n">
-        <v>1907000</v>
+        <v>74073</v>
       </c>
       <c r="H4" t="n">
-        <v>26.43837515596839</v>
+        <v>1.568081778281328</v>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>2026-03-21T04:57:12</t>
+          <t>2026-03-21T04:59:43</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-03-21</t>
+          <t>2026-03-17</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>프론트라인</t>
+          <t>HD건설기계</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>175</v>
+        <v>31</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
@@ -1832,33 +995,33 @@
         <v>1</v>
       </c>
       <c r="F5" t="n">
-        <v>8471815.962899337</v>
+        <v>4123000</v>
       </c>
       <c r="G5" t="n">
-        <v>4041951.962899337</v>
+        <v>87904</v>
       </c>
       <c r="H5" t="n">
-        <v>91.24325177701475</v>
+        <v>2.178485964150543</v>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>2026-03-21T04:57:12</t>
+          <t>2026-03-21T04:59:43</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-03-21</t>
+          <t>2026-03-17</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>시드릴</t>
+          <t>삼성화재</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>123</v>
+        <v>7</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
@@ -1869,33 +1032,33 @@
         <v>1</v>
       </c>
       <c r="F6" t="n">
-        <v>8070101.805898919</v>
+        <v>3321500</v>
       </c>
       <c r="G6" t="n">
-        <v>1619750.805898919</v>
+        <v>-309500</v>
       </c>
       <c r="H6" t="n">
-        <v>25.11104908707943</v>
+        <v>-8.523822638391627</v>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>2026-03-21T04:57:12</t>
+          <t>2026-03-21T04:59:43</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-03-21</t>
+          <t>2026-03-17</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>세아제강</t>
+          <t>휴스틸</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>50</v>
+        <v>500</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
@@ -1906,33 +1069,33 @@
         <v>1</v>
       </c>
       <c r="F7" t="n">
-        <v>7395000</v>
+        <v>2750000</v>
       </c>
       <c r="G7" t="n">
-        <v>1085000</v>
+        <v>471390</v>
       </c>
       <c r="H7" t="n">
-        <v>17.19492868462758</v>
+        <v>20.68761218462133</v>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>2026-03-21T04:57:12</t>
+          <t>2026-03-21T04:59:43</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-03-21</t>
+          <t>2026-03-17</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>센트러스 에너지</t>
+          <t>현대제철</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>25</v>
+        <v>70</v>
       </c>
       <c r="D8" t="inlineStr">
         <is>
@@ -1943,33 +1106,33 @@
         <v>1</v>
       </c>
       <c r="F8" t="n">
-        <v>7026050.85816239</v>
+        <v>2621500</v>
       </c>
       <c r="G8" t="n">
-        <v>-406805.1418376099</v>
+        <v>-186000</v>
       </c>
       <c r="H8" t="n">
-        <v>-5.473066366920198</v>
+        <v>-6.625111308993767</v>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>2026-03-21T04:57:12</t>
+          <t>2026-03-21T04:59:43</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-03-21</t>
+          <t>2026-03-17</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>트랜스오션</t>
+          <t>KoAct 코스닥액티브</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>750</v>
+        <v>200</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
@@ -1980,33 +1143,33 @@
         <v>1</v>
       </c>
       <c r="F9" t="n">
-        <v>7020031.5082007</v>
+        <v>2582000</v>
       </c>
       <c r="G9" t="n">
-        <v>2892797.5082007</v>
+        <v>-120000</v>
       </c>
       <c r="H9" t="n">
-        <v>70.09046514446965</v>
+        <v>-4.441154700222058</v>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>2026-03-21T04:57:12</t>
+          <t>2026-03-21T04:59:43</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-03-21</t>
+          <t>2026-03-17</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>노블</t>
+          <t>케이씨</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>99</v>
+        <v>50</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
@@ -2017,33 +1180,33 @@
         <v>1</v>
       </c>
       <c r="F10" t="n">
-        <v>6958769.981090547</v>
+        <v>1670000</v>
       </c>
       <c r="G10" t="n">
-        <v>3051561.981090547</v>
+        <v>20500</v>
       </c>
       <c r="H10" t="n">
-        <v>78.10083264291399</v>
+        <v>1.242800848742043</v>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>2026-03-21T04:57:12</t>
+          <t>2026-03-21T04:59:43</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-03-21</t>
+          <t>2026-03-17</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>타이드워터</t>
+          <t>하나금융지주</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>48</v>
+        <v>10</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
@@ -2054,17 +1217,17 @@
         <v>1</v>
       </c>
       <c r="F11" t="n">
-        <v>5235363.852789983</v>
+        <v>1132000</v>
       </c>
       <c r="G11" t="n">
-        <v>1510818.852789983</v>
+        <v>23000</v>
       </c>
       <c r="H11" t="n">
-        <v>40.56385015592463</v>
+        <v>2.073940486925157</v>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>2026-03-21T04:57:12</t>
+          <t>2026-03-21T04:59:43</t>
         </is>
       </c>
     </row>
@@ -2076,11 +1239,11 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>노브</t>
+          <t>페트로브라스 (ADR)</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>185</v>
+        <v>480</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
@@ -2091,13 +1254,13 @@
         <v>1</v>
       </c>
       <c r="F12" t="n">
-        <v>5200391.447092756</v>
+        <v>13579584.97235231</v>
       </c>
       <c r="G12" t="n">
-        <v>1890383.447092756</v>
+        <v>1473035.972352311</v>
       </c>
       <c r="H12" t="n">
-        <v>57.11114435653194</v>
+        <v>12.16726560436265</v>
       </c>
       <c r="I12" t="inlineStr">
         <is>
@@ -2113,11 +1276,11 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>TIME 코리아밸류업액티브</t>
+          <t>AGNC 인베스트먼트</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>201</v>
+        <v>700</v>
       </c>
       <c r="D13" t="inlineStr">
         <is>
@@ -2128,13 +1291,13 @@
         <v>1</v>
       </c>
       <c r="F13" t="n">
-        <v>4797870</v>
+        <v>10270464.45007324</v>
       </c>
       <c r="G13" t="n">
-        <v>74073</v>
+        <v>-561550.5499267559</v>
       </c>
       <c r="H13" t="n">
-        <v>1.568081778281328</v>
+        <v>-5.184174411933109</v>
       </c>
       <c r="I13" t="inlineStr">
         <is>
@@ -2150,11 +1313,11 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>오케아니스 에코 탱커스</t>
+          <t>대한조선</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>65</v>
+        <v>100</v>
       </c>
       <c r="D14" t="inlineStr">
         <is>
@@ -2165,13 +1328,13 @@
         <v>1</v>
       </c>
       <c r="F14" t="n">
-        <v>4511179.137784176</v>
+        <v>9120000</v>
       </c>
       <c r="G14" t="n">
-        <v>2254819.137784176</v>
+        <v>1907000</v>
       </c>
       <c r="H14" t="n">
-        <v>99.93171026716374</v>
+        <v>26.43837515596839</v>
       </c>
       <c r="I14" t="inlineStr">
         <is>
@@ -2187,11 +1350,11 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>삼성화재</t>
+          <t>프론트라인</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>9</v>
+        <v>175</v>
       </c>
       <c r="D15" t="inlineStr">
         <is>
@@ -2202,13 +1365,13 @@
         <v>1</v>
       </c>
       <c r="F15" t="n">
-        <v>4270500</v>
+        <v>8471815.962899337</v>
       </c>
       <c r="G15" t="n">
-        <v>-360500</v>
+        <v>4041951.962899337</v>
       </c>
       <c r="H15" t="n">
-        <v>-7.784495789246384</v>
+        <v>91.24325177701475</v>
       </c>
       <c r="I15" t="inlineStr">
         <is>
@@ -2224,11 +1387,11 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>동원개발</t>
+          <t>시드릴</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>1360</v>
+        <v>123</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
@@ -2239,13 +1402,13 @@
         <v>1</v>
       </c>
       <c r="F16" t="n">
-        <v>4202400</v>
+        <v>8070101.805898919</v>
       </c>
       <c r="G16" t="n">
-        <v>465000</v>
+        <v>1619750.805898919</v>
       </c>
       <c r="H16" t="n">
-        <v>12.44180446299566</v>
+        <v>25.11104908707943</v>
       </c>
       <c r="I16" t="inlineStr">
         <is>
@@ -2261,11 +1424,11 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>HD건설기계</t>
+          <t>세아제강</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>31</v>
+        <v>50</v>
       </c>
       <c r="D17" t="inlineStr">
         <is>
@@ -2276,13 +1439,13 @@
         <v>1</v>
       </c>
       <c r="F17" t="n">
-        <v>4123000</v>
+        <v>7395000</v>
       </c>
       <c r="G17" t="n">
-        <v>87904</v>
+        <v>1085000</v>
       </c>
       <c r="H17" t="n">
-        <v>2.178485964150543</v>
+        <v>17.19492868462758</v>
       </c>
       <c r="I17" t="inlineStr">
         <is>
@@ -2298,11 +1461,11 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>차코스 에너지 내비게이션</t>
+          <t>센트러스 에너지</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>75</v>
+        <v>25</v>
       </c>
       <c r="D18" t="inlineStr">
         <is>
@@ -2313,13 +1476,13 @@
         <v>1</v>
       </c>
       <c r="F18" t="n">
-        <v>4026924.996845168</v>
+        <v>7026050.85816239</v>
       </c>
       <c r="G18" t="n">
-        <v>202276.9968451681</v>
+        <v>-406805.1418376099</v>
       </c>
       <c r="H18" t="n">
-        <v>5.28877420471552</v>
+        <v>-5.473066366920198</v>
       </c>
       <c r="I18" t="inlineStr">
         <is>
@@ -2335,11 +1498,11 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>넥스틸</t>
+          <t>트랜스오션</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>300</v>
+        <v>750</v>
       </c>
       <c r="D19" t="inlineStr">
         <is>
@@ -2350,13 +1513,13 @@
         <v>1</v>
       </c>
       <c r="F19" t="n">
-        <v>3771000</v>
+        <v>7020031.5082007</v>
       </c>
       <c r="G19" t="n">
-        <v>521000</v>
+        <v>2892797.5082007</v>
       </c>
       <c r="H19" t="n">
-        <v>16.03076923076923</v>
+        <v>70.09046514446965</v>
       </c>
       <c r="I19" t="inlineStr">
         <is>
@@ -2372,11 +1535,11 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>피바디 에너지</t>
+          <t>노블</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>65</v>
+        <v>99</v>
       </c>
       <c r="D20" t="inlineStr">
         <is>
@@ -2387,13 +1550,13 @@
         <v>1</v>
       </c>
       <c r="F20" t="n">
-        <v>3649438.50225304</v>
+        <v>6958769.981090547</v>
       </c>
       <c r="G20" t="n">
-        <v>2178666.50225304</v>
+        <v>3051561.981090547</v>
       </c>
       <c r="H20" t="n">
-        <v>148.1308117269733</v>
+        <v>78.10083264291399</v>
       </c>
       <c r="I20" t="inlineStr">
         <is>
@@ -2409,11 +1572,11 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>현대제철</t>
+          <t>타이드워터</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>80</v>
+        <v>48</v>
       </c>
       <c r="D21" t="inlineStr">
         <is>
@@ -2424,13 +1587,13 @@
         <v>1</v>
       </c>
       <c r="F21" t="n">
-        <v>2996000</v>
+        <v>5235363.852789983</v>
       </c>
       <c r="G21" t="n">
-        <v>-182000</v>
+        <v>1510818.852789983</v>
       </c>
       <c r="H21" t="n">
-        <v>-5.726872246696035</v>
+        <v>40.56385015592463</v>
       </c>
       <c r="I21" t="inlineStr">
         <is>
@@ -2446,11 +1609,11 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>더치 브로스</t>
+          <t>노브</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>39</v>
+        <v>185</v>
       </c>
       <c r="D22" t="inlineStr">
         <is>
@@ -2461,13 +1624,13 @@
         <v>1</v>
       </c>
       <c r="F22" t="n">
-        <v>2934418.414306641</v>
+        <v>5200391.447092756</v>
       </c>
       <c r="G22" t="n">
-        <v>-256226.5856933594</v>
+        <v>1890383.447092756</v>
       </c>
       <c r="H22" t="n">
-        <v>-8.030557636257226</v>
+        <v>57.11114435653194</v>
       </c>
       <c r="I22" t="inlineStr">
         <is>
@@ -2483,11 +1646,11 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>휴스틸</t>
+          <t>TIME 코리아밸류업액티브</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>500</v>
+        <v>201</v>
       </c>
       <c r="D23" t="inlineStr">
         <is>
@@ -2498,13 +1661,13 @@
         <v>1</v>
       </c>
       <c r="F23" t="n">
-        <v>2750000</v>
+        <v>4797870</v>
       </c>
       <c r="G23" t="n">
-        <v>471390</v>
+        <v>74073</v>
       </c>
       <c r="H23" t="n">
-        <v>20.68761218462133</v>
+        <v>1.568081778281328</v>
       </c>
       <c r="I23" t="inlineStr">
         <is>
@@ -2520,11 +1683,11 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>DL이앤씨</t>
+          <t>오케아니스 에코 탱커스</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>40</v>
+        <v>65</v>
       </c>
       <c r="D24" t="inlineStr">
         <is>
@@ -2535,13 +1698,13 @@
         <v>1</v>
       </c>
       <c r="F24" t="n">
-        <v>2696000</v>
+        <v>4511179.137784176</v>
       </c>
       <c r="G24" t="n">
-        <v>990500</v>
+        <v>2254819.137784176</v>
       </c>
       <c r="H24" t="n">
-        <v>58.07681031955438</v>
+        <v>99.93171026716374</v>
       </c>
       <c r="I24" t="inlineStr">
         <is>
@@ -2557,11 +1720,11 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>KoAct 코스닥액티브</t>
+          <t>삼성화재</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>200</v>
+        <v>9</v>
       </c>
       <c r="D25" t="inlineStr">
         <is>
@@ -2572,13 +1735,13 @@
         <v>1</v>
       </c>
       <c r="F25" t="n">
-        <v>2582000</v>
+        <v>4270500</v>
       </c>
       <c r="G25" t="n">
-        <v>-120000</v>
+        <v>-360500</v>
       </c>
       <c r="H25" t="n">
-        <v>-4.441154700222058</v>
+        <v>-7.784495789246384</v>
       </c>
       <c r="I25" t="inlineStr">
         <is>
@@ -2594,11 +1757,11 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>대신증권</t>
+          <t>동원개발</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>55</v>
+        <v>1360</v>
       </c>
       <c r="D26" t="inlineStr">
         <is>
@@ -2609,13 +1772,13 @@
         <v>1</v>
       </c>
       <c r="F26" t="n">
-        <v>2219250</v>
+        <v>4202400</v>
       </c>
       <c r="G26" t="n">
-        <v>509749</v>
+        <v>465000</v>
       </c>
       <c r="H26" t="n">
-        <v>29.81858448752005</v>
+        <v>12.44180446299566</v>
       </c>
       <c r="I26" t="inlineStr">
         <is>
@@ -2631,11 +1794,11 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>발레로 에너지</t>
+          <t>HD건설기계</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>6</v>
+        <v>31</v>
       </c>
       <c r="D27" t="inlineStr">
         <is>
@@ -2646,13 +1809,13 @@
         <v>1</v>
       </c>
       <c r="F27" t="n">
-        <v>2165691.085066516</v>
+        <v>4123000</v>
       </c>
       <c r="G27" t="n">
-        <v>101701.085066516</v>
+        <v>87904</v>
       </c>
       <c r="H27" t="n">
-        <v>4.927402025519307</v>
+        <v>2.178485964150543</v>
       </c>
       <c r="I27" t="inlineStr">
         <is>
@@ -2668,11 +1831,11 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>미창석유</t>
+          <t>차코스 에너지 내비게이션</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>18</v>
+        <v>75</v>
       </c>
       <c r="D28" t="inlineStr">
         <is>
@@ -2683,13 +1846,13 @@
         <v>1</v>
       </c>
       <c r="F28" t="n">
-        <v>2097000</v>
+        <v>4026924.996845168</v>
       </c>
       <c r="G28" t="n">
-        <v>-295200</v>
+        <v>202276.9968451681</v>
       </c>
       <c r="H28" t="n">
-        <v>-12.34010534236268</v>
+        <v>5.28877420471552</v>
       </c>
       <c r="I28" t="inlineStr">
         <is>
@@ -2705,11 +1868,11 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>하나금융지주</t>
+          <t>넥스틸</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>18</v>
+        <v>300</v>
       </c>
       <c r="D29" t="inlineStr">
         <is>
@@ -2720,13 +1883,13 @@
         <v>1</v>
       </c>
       <c r="F29" t="n">
-        <v>2037600</v>
+        <v>3771000</v>
       </c>
       <c r="G29" t="n">
-        <v>12200</v>
+        <v>521000</v>
       </c>
       <c r="H29" t="n">
-        <v>0.6023501530561864</v>
+        <v>16.03076923076923</v>
       </c>
       <c r="I29" t="inlineStr">
         <is>
@@ -2742,11 +1905,11 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>대창단조</t>
+          <t>피바디 에너지</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>300</v>
+        <v>65</v>
       </c>
       <c r="D30" t="inlineStr">
         <is>
@@ -2757,13 +1920,13 @@
         <v>1</v>
       </c>
       <c r="F30" t="n">
-        <v>2004000</v>
+        <v>3649438.50225304</v>
       </c>
       <c r="G30" t="n">
-        <v>-54000</v>
+        <v>2178666.50225304</v>
       </c>
       <c r="H30" t="n">
-        <v>-2.623906705539359</v>
+        <v>148.1308117269733</v>
       </c>
       <c r="I30" t="inlineStr">
         <is>
@@ -2779,11 +1942,11 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>동방</t>
+          <t>현대제철</t>
         </is>
       </c>
       <c r="C31" t="n">
-        <v>681</v>
+        <v>80</v>
       </c>
       <c r="D31" t="inlineStr">
         <is>
@@ -2794,13 +1957,13 @@
         <v>1</v>
       </c>
       <c r="F31" t="n">
-        <v>1995330</v>
+        <v>2996000</v>
       </c>
       <c r="G31" t="n">
-        <v>23829</v>
+        <v>-182000</v>
       </c>
       <c r="H31" t="n">
-        <v>1.208672985709873</v>
+        <v>-5.726872246696035</v>
       </c>
       <c r="I31" t="inlineStr">
         <is>
@@ -2816,11 +1979,11 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>스타 벌크 캐리어스</t>
+          <t>더치 브로스</t>
         </is>
       </c>
       <c r="C32" t="n">
-        <v>50</v>
+        <v>39</v>
       </c>
       <c r="D32" t="inlineStr">
         <is>
@@ -2831,13 +1994,13 @@
         <v>1</v>
       </c>
       <c r="F32" t="n">
-        <v>1680142.640194588</v>
+        <v>2934418.414306641</v>
       </c>
       <c r="G32" t="n">
-        <v>365789.6401945879</v>
+        <v>-256226.5856933594</v>
       </c>
       <c r="H32" t="n">
-        <v>27.83039565433242</v>
+        <v>-8.030557636257226</v>
       </c>
       <c r="I32" t="inlineStr">
         <is>
@@ -2853,11 +2016,11 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>케이씨</t>
+          <t>휴스틸</t>
         </is>
       </c>
       <c r="C33" t="n">
-        <v>50</v>
+        <v>500</v>
       </c>
       <c r="D33" t="inlineStr">
         <is>
@@ -2868,13 +2031,13 @@
         <v>1</v>
       </c>
       <c r="F33" t="n">
-        <v>1670000</v>
+        <v>2750000</v>
       </c>
       <c r="G33" t="n">
-        <v>20500</v>
+        <v>471390</v>
       </c>
       <c r="H33" t="n">
-        <v>1.242800848742043</v>
+        <v>20.68761218462133</v>
       </c>
       <c r="I33" t="inlineStr">
         <is>
@@ -2890,11 +2053,11 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>유나이티드헬스 그룹</t>
+          <t>DL이앤씨</t>
         </is>
       </c>
       <c r="C34" t="n">
-        <v>4</v>
+        <v>40</v>
       </c>
       <c r="D34" t="inlineStr">
         <is>
@@ -2905,13 +2068,13 @@
         <v>1</v>
       </c>
       <c r="F34" t="n">
-        <v>1658864.328313038</v>
+        <v>2696000</v>
       </c>
       <c r="G34" t="n">
-        <v>-35591.67168696248</v>
+        <v>990500</v>
       </c>
       <c r="H34" t="n">
-        <v>-2.100477774988697</v>
+        <v>58.07681031955438</v>
       </c>
       <c r="I34" t="inlineStr">
         <is>
@@ -2927,11 +2090,11 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>텍사스 퍼시픽 랜드</t>
+          <t>KoAct 코스닥액티브</t>
         </is>
       </c>
       <c r="C35" t="n">
-        <v>2</v>
+        <v>200</v>
       </c>
       <c r="D35" t="inlineStr">
         <is>
@@ -2942,13 +2105,13 @@
         <v>1</v>
       </c>
       <c r="F35" t="n">
-        <v>1563247.374122903</v>
+        <v>2582000</v>
       </c>
       <c r="G35" t="n">
-        <v>-14646.62587709725</v>
+        <v>-120000</v>
       </c>
       <c r="H35" t="n">
-        <v>-0.9282388979929735</v>
+        <v>-4.441154700222058</v>
       </c>
       <c r="I35" t="inlineStr">
         <is>
@@ -2964,11 +2127,11 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>LX인터내셔널</t>
+          <t>대신증권</t>
         </is>
       </c>
       <c r="C36" t="n">
-        <v>20</v>
+        <v>55</v>
       </c>
       <c r="D36" t="inlineStr">
         <is>
@@ -2979,13 +2142,13 @@
         <v>1</v>
       </c>
       <c r="F36" t="n">
-        <v>943000</v>
+        <v>2219250</v>
       </c>
       <c r="G36" t="n">
-        <v>4000</v>
+        <v>509749</v>
       </c>
       <c r="H36" t="n">
-        <v>0.4259850905218318</v>
+        <v>29.81858448752005</v>
       </c>
       <c r="I36" t="inlineStr">
         <is>
@@ -3001,11 +2164,11 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>삼성생명</t>
+          <t>발레로 에너지</t>
         </is>
       </c>
       <c r="C37" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="D37" t="inlineStr">
         <is>
@@ -3016,13 +2179,13 @@
         <v>1</v>
       </c>
       <c r="F37" t="n">
-        <v>926000</v>
+        <v>2165691.085066516</v>
       </c>
       <c r="G37" t="n">
-        <v>93000</v>
+        <v>101701.085066516</v>
       </c>
       <c r="H37" t="n">
-        <v>11.16446578631453</v>
+        <v>4.927402025519307</v>
       </c>
       <c r="I37" t="inlineStr">
         <is>
@@ -3038,11 +2201,11 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>비에이치아이</t>
+          <t>미창석유</t>
         </is>
       </c>
       <c r="C38" t="n">
-        <v>8</v>
+        <v>18</v>
       </c>
       <c r="D38" t="inlineStr">
         <is>
@@ -3053,13 +2216,13 @@
         <v>1</v>
       </c>
       <c r="F38" t="n">
-        <v>876000</v>
+        <v>2097000</v>
       </c>
       <c r="G38" t="n">
-        <v>210885</v>
+        <v>-295200</v>
       </c>
       <c r="H38" t="n">
-        <v>31.70654698811484</v>
+        <v>-12.34010534236268</v>
       </c>
       <c r="I38" t="inlineStr">
         <is>
@@ -3075,11 +2238,11 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>하프니아</t>
+          <t>하나금융지주</t>
         </is>
       </c>
       <c r="C39" t="n">
-        <v>80</v>
+        <v>18</v>
       </c>
       <c r="D39" t="inlineStr">
         <is>
@@ -3090,13 +2253,13 @@
         <v>1</v>
       </c>
       <c r="F39" t="n">
-        <v>842704.775390625</v>
+        <v>2037600</v>
       </c>
       <c r="G39" t="n">
-        <v>216973.775390625</v>
+        <v>12200</v>
       </c>
       <c r="H39" t="n">
-        <v>34.67524789256486</v>
+        <v>0.6023501530561864</v>
       </c>
       <c r="I39" t="inlineStr">
         <is>
@@ -3112,11 +2275,11 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>클리블랜드 클리프스</t>
+          <t>대창단조</t>
         </is>
       </c>
       <c r="C40" t="n">
-        <v>70</v>
+        <v>300</v>
       </c>
       <c r="D40" t="inlineStr">
         <is>
@@ -3127,13 +2290,13 @@
         <v>1</v>
       </c>
       <c r="F40" t="n">
-        <v>823743.9360268187</v>
+        <v>2004000</v>
       </c>
       <c r="G40" t="n">
-        <v>-192311.0639731813</v>
+        <v>-54000</v>
       </c>
       <c r="H40" t="n">
-        <v>-18.92722972409774</v>
+        <v>-2.623906705539359</v>
       </c>
       <c r="I40" t="inlineStr">
         <is>
@@ -3149,11 +2312,11 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>낫 오프쇼어 파트너스</t>
+          <t>동방</t>
         </is>
       </c>
       <c r="C41" t="n">
-        <v>30</v>
+        <v>681</v>
       </c>
       <c r="D41" t="inlineStr">
         <is>
@@ -3164,13 +2327,13 @@
         <v>1</v>
       </c>
       <c r="F41" t="n">
-        <v>413075.8057155996</v>
+        <v>1995330</v>
       </c>
       <c r="G41" t="n">
-        <v>-4439.194284400437</v>
+        <v>23829</v>
       </c>
       <c r="H41" t="n">
-        <v>-1.063241867813237</v>
+        <v>1.208672985709873</v>
       </c>
       <c r="I41" t="inlineStr">
         <is>
@@ -3186,30 +2349,400 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
+          <t>스타 벌크 캐리어스</t>
+        </is>
+      </c>
+      <c r="C42" t="n">
+        <v>50</v>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E42" t="n">
+        <v>1</v>
+      </c>
+      <c r="F42" t="n">
+        <v>1680142.640194588</v>
+      </c>
+      <c r="G42" t="n">
+        <v>365789.6401945879</v>
+      </c>
+      <c r="H42" t="n">
+        <v>27.83039565433242</v>
+      </c>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>2026-03-21T04:57:12</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>2026-03-21</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>케이씨</t>
+        </is>
+      </c>
+      <c r="C43" t="n">
+        <v>50</v>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E43" t="n">
+        <v>1</v>
+      </c>
+      <c r="F43" t="n">
+        <v>1670000</v>
+      </c>
+      <c r="G43" t="n">
+        <v>20500</v>
+      </c>
+      <c r="H43" t="n">
+        <v>1.242800848742043</v>
+      </c>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>2026-03-21T04:57:12</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>2026-03-21</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>유나이티드헬스 그룹</t>
+        </is>
+      </c>
+      <c r="C44" t="n">
+        <v>4</v>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E44" t="n">
+        <v>1</v>
+      </c>
+      <c r="F44" t="n">
+        <v>1658864.328313038</v>
+      </c>
+      <c r="G44" t="n">
+        <v>-35591.67168696248</v>
+      </c>
+      <c r="H44" t="n">
+        <v>-2.100477774988697</v>
+      </c>
+      <c r="I44" t="inlineStr">
+        <is>
+          <t>2026-03-21T04:57:12</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>2026-03-21</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>텍사스 퍼시픽 랜드</t>
+        </is>
+      </c>
+      <c r="C45" t="n">
+        <v>2</v>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E45" t="n">
+        <v>1</v>
+      </c>
+      <c r="F45" t="n">
+        <v>1563247.374122903</v>
+      </c>
+      <c r="G45" t="n">
+        <v>-14646.62587709725</v>
+      </c>
+      <c r="H45" t="n">
+        <v>-0.9282388979929735</v>
+      </c>
+      <c r="I45" t="inlineStr">
+        <is>
+          <t>2026-03-21T04:57:12</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>2026-03-21</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>LX인터내셔널</t>
+        </is>
+      </c>
+      <c r="C46" t="n">
+        <v>20</v>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E46" t="n">
+        <v>1</v>
+      </c>
+      <c r="F46" t="n">
+        <v>943000</v>
+      </c>
+      <c r="G46" t="n">
+        <v>4000</v>
+      </c>
+      <c r="H46" t="n">
+        <v>0.4259850905218318</v>
+      </c>
+      <c r="I46" t="inlineStr">
+        <is>
+          <t>2026-03-21T04:57:12</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>2026-03-21</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>삼성생명</t>
+        </is>
+      </c>
+      <c r="C47" t="n">
+        <v>4</v>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E47" t="n">
+        <v>1</v>
+      </c>
+      <c r="F47" t="n">
+        <v>926000</v>
+      </c>
+      <c r="G47" t="n">
+        <v>93000</v>
+      </c>
+      <c r="H47" t="n">
+        <v>11.16446578631453</v>
+      </c>
+      <c r="I47" t="inlineStr">
+        <is>
+          <t>2026-03-21T04:57:12</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>2026-03-21</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>비에이치아이</t>
+        </is>
+      </c>
+      <c r="C48" t="n">
+        <v>8</v>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E48" t="n">
+        <v>1</v>
+      </c>
+      <c r="F48" t="n">
+        <v>876000</v>
+      </c>
+      <c r="G48" t="n">
+        <v>210885</v>
+      </c>
+      <c r="H48" t="n">
+        <v>31.70654698811484</v>
+      </c>
+      <c r="I48" t="inlineStr">
+        <is>
+          <t>2026-03-21T04:57:12</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>2026-03-21</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>하프니아</t>
+        </is>
+      </c>
+      <c r="C49" t="n">
+        <v>80</v>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E49" t="n">
+        <v>1</v>
+      </c>
+      <c r="F49" t="n">
+        <v>842704.775390625</v>
+      </c>
+      <c r="G49" t="n">
+        <v>216973.775390625</v>
+      </c>
+      <c r="H49" t="n">
+        <v>34.67524789256486</v>
+      </c>
+      <c r="I49" t="inlineStr">
+        <is>
+          <t>2026-03-21T04:57:12</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>2026-03-21</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>클리블랜드 클리프스</t>
+        </is>
+      </c>
+      <c r="C50" t="n">
+        <v>70</v>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E50" t="n">
+        <v>1</v>
+      </c>
+      <c r="F50" t="n">
+        <v>823743.9360268187</v>
+      </c>
+      <c r="G50" t="n">
+        <v>-192311.0639731813</v>
+      </c>
+      <c r="H50" t="n">
+        <v>-18.92722972409774</v>
+      </c>
+      <c r="I50" t="inlineStr">
+        <is>
+          <t>2026-03-21T04:57:12</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>2026-03-21</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>낫 오프쇼어 파트너스</t>
+        </is>
+      </c>
+      <c r="C51" t="n">
+        <v>30</v>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E51" t="n">
+        <v>1</v>
+      </c>
+      <c r="F51" t="n">
+        <v>413075.8057155996</v>
+      </c>
+      <c r="G51" t="n">
+        <v>-4439.194284400437</v>
+      </c>
+      <c r="H51" t="n">
+        <v>-1.063241867813237</v>
+      </c>
+      <c r="I51" t="inlineStr">
+        <is>
+          <t>2026-03-21T04:57:12</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>2026-03-21</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
           <t>NH투자증권우</t>
         </is>
       </c>
-      <c r="C42" t="n">
+      <c r="C52" t="n">
         <v>2</v>
       </c>
-      <c r="D42" t="inlineStr">
-        <is>
-          <t>KRW</t>
-        </is>
-      </c>
-      <c r="E42" t="n">
-        <v>1</v>
-      </c>
-      <c r="F42" t="n">
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E52" t="n">
+        <v>1</v>
+      </c>
+      <c r="F52" t="n">
         <v>54700</v>
       </c>
-      <c r="G42" t="n">
+      <c r="G52" t="n">
         <v>100</v>
       </c>
-      <c r="H42" t="n">
+      <c r="H52" t="n">
         <v>0.1831501831501831</v>
       </c>
-      <c r="I42" t="inlineStr">
+      <c r="I52" t="inlineStr">
         <is>
           <t>2026-03-21T04:57:12</t>
         </is>
@@ -3226,7 +2759,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E2"/>
+  <dimension ref="A1:E3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3259,21 +2792,44 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-03-21</t>
+          <t>2026-03-17</t>
         </is>
       </c>
       <c r="B2" t="n">
+        <v>0</v>
+      </c>
+      <c r="C2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>2026-03-21T04:59:43</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>2026-03-21T04:59:43</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-03-21</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
         <v>31036676</v>
       </c>
-      <c r="C2" t="n">
+      <c r="C3" t="n">
         <v>12663.38</v>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="D3" t="inlineStr">
         <is>
           <t>2026-03-21T04:52:57</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="E3" t="inlineStr">
         <is>
           <t>2026-03-21T04:57:12</t>
         </is>

</xml_diff>

<commit_message>
auto: portfolio snapshot 2026-03-17 (2026-03-21T05:00:11)
</commit_message>
<xml_diff>
--- a/portfolio_auto.xlsx
+++ b/portfolio_auto.xlsx
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G11"/>
+  <dimension ref="A1:G25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -736,6 +736,384 @@
       </c>
       <c r="G11" t="n">
         <v>1.568081778281328</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>페트로브라스 (ADR)</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>480</v>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>1</v>
+      </c>
+      <c r="E12" t="n">
+        <v>13579584.97235231</v>
+      </c>
+      <c r="F12" t="n">
+        <v>1473035.972352311</v>
+      </c>
+      <c r="G12" t="n">
+        <v>12.16726560436265</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>프론트라인</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>175</v>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>1</v>
+      </c>
+      <c r="E13" t="n">
+        <v>8471815.962899337</v>
+      </c>
+      <c r="F13" t="n">
+        <v>4041951.962899337</v>
+      </c>
+      <c r="G13" t="n">
+        <v>91.24325177701475</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>피바디 에너지</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>65</v>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>1</v>
+      </c>
+      <c r="E14" t="n">
+        <v>3649438.50225304</v>
+      </c>
+      <c r="F14" t="n">
+        <v>2178666.50225304</v>
+      </c>
+      <c r="G14" t="n">
+        <v>148.1308117269733</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>하프니아</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>80</v>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>1</v>
+      </c>
+      <c r="E15" t="n">
+        <v>842704.775390625</v>
+      </c>
+      <c r="F15" t="n">
+        <v>216973.775390625</v>
+      </c>
+      <c r="G15" t="n">
+        <v>34.67524789256486</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>AGNC 인베스트먼트</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>700</v>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>1</v>
+      </c>
+      <c r="E16" t="n">
+        <v>10270464.45007324</v>
+      </c>
+      <c r="F16" t="n">
+        <v>-561550.5499267578</v>
+      </c>
+      <c r="G16" t="n">
+        <v>-5.184174411933125</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>넥스틸</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>200</v>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>1</v>
+      </c>
+      <c r="E17" t="n">
+        <v>2514000</v>
+      </c>
+      <c r="F17" t="n">
+        <v>503000</v>
+      </c>
+      <c r="G17" t="n">
+        <v>25.01243162605669</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>대신증권</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>55</v>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>1</v>
+      </c>
+      <c r="E18" t="n">
+        <v>2219250</v>
+      </c>
+      <c r="F18" t="n">
+        <v>509749</v>
+      </c>
+      <c r="G18" t="n">
+        <v>29.81858448752005</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>대창단조</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>300</v>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
+        <v>1</v>
+      </c>
+      <c r="E19" t="n">
+        <v>2004000</v>
+      </c>
+      <c r="F19" t="n">
+        <v>-54000</v>
+      </c>
+      <c r="G19" t="n">
+        <v>-2.623906705539359</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>대한조선</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>100</v>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="D20" t="n">
+        <v>1</v>
+      </c>
+      <c r="E20" t="n">
+        <v>9120000</v>
+      </c>
+      <c r="F20" t="n">
+        <v>1907000</v>
+      </c>
+      <c r="G20" t="n">
+        <v>26.43837515596839</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>동방</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>681</v>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
+        <v>1</v>
+      </c>
+      <c r="E21" t="n">
+        <v>1995330</v>
+      </c>
+      <c r="F21" t="n">
+        <v>23829</v>
+      </c>
+      <c r="G21" t="n">
+        <v>1.208672985709873</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>동원개발</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>1360</v>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="D22" t="n">
+        <v>1</v>
+      </c>
+      <c r="E22" t="n">
+        <v>4202400</v>
+      </c>
+      <c r="F22" t="n">
+        <v>465000</v>
+      </c>
+      <c r="G22" t="n">
+        <v>12.44180446299566</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>미창석유</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>18</v>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="D23" t="n">
+        <v>1</v>
+      </c>
+      <c r="E23" t="n">
+        <v>2097000</v>
+      </c>
+      <c r="F23" t="n">
+        <v>-295200</v>
+      </c>
+      <c r="G23" t="n">
+        <v>-12.34010534236268</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>비에이치아이</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>8</v>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="D24" t="n">
+        <v>1</v>
+      </c>
+      <c r="E24" t="n">
+        <v>876000</v>
+      </c>
+      <c r="F24" t="n">
+        <v>210885</v>
+      </c>
+      <c r="G24" t="n">
+        <v>31.70654698811484</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>삼성생명</t>
+        </is>
+      </c>
+      <c r="B25" t="n">
+        <v>4</v>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="D25" t="n">
+        <v>1</v>
+      </c>
+      <c r="E25" t="n">
+        <v>926000</v>
+      </c>
+      <c r="F25" t="n">
+        <v>93000</v>
+      </c>
+      <c r="G25" t="n">
+        <v>11.16446578631453</v>
       </c>
     </row>
   </sheetData>
@@ -793,7 +1171,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2026-03-21T04:59:43</t>
+          <t>2026-03-21T05:00:11</t>
         </is>
       </c>
       <c r="E2" t="n">
@@ -811,7 +1189,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I52"/>
+  <dimension ref="A1:I66"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -869,11 +1247,11 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>세아제강</t>
+          <t>페트로브라스 (ADR)</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>50</v>
+        <v>480</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
@@ -884,17 +1262,17 @@
         <v>1</v>
       </c>
       <c r="F2" t="n">
-        <v>7395000</v>
+        <v>13579584.97235231</v>
       </c>
       <c r="G2" t="n">
-        <v>1085000</v>
+        <v>1473035.972352311</v>
       </c>
       <c r="H2" t="n">
-        <v>17.19492868462758</v>
+        <v>12.16726560436265</v>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>2026-03-21T04:59:43</t>
+          <t>2026-03-21T05:00:11</t>
         </is>
       </c>
     </row>
@@ -906,11 +1284,11 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>DL이앤씨</t>
+          <t>AGNC 인베스트먼트</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>80</v>
+        <v>700</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
@@ -921,17 +1299,17 @@
         <v>1</v>
       </c>
       <c r="F3" t="n">
-        <v>5392000</v>
+        <v>10270464.45007324</v>
       </c>
       <c r="G3" t="n">
-        <v>1981000</v>
+        <v>-561550.5499267578</v>
       </c>
       <c r="H3" t="n">
-        <v>58.07681031955438</v>
+        <v>-5.184174411933125</v>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>2026-03-21T04:59:43</t>
+          <t>2026-03-21T05:00:11</t>
         </is>
       </c>
     </row>
@@ -943,11 +1321,11 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>TIME 코리아밸류업액티브</t>
+          <t>대한조선</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>201</v>
+        <v>100</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
@@ -958,17 +1336,17 @@
         <v>1</v>
       </c>
       <c r="F4" t="n">
-        <v>4797870</v>
+        <v>9120000</v>
       </c>
       <c r="G4" t="n">
-        <v>74073</v>
+        <v>1907000</v>
       </c>
       <c r="H4" t="n">
-        <v>1.568081778281328</v>
+        <v>26.43837515596839</v>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>2026-03-21T04:59:43</t>
+          <t>2026-03-21T05:00:11</t>
         </is>
       </c>
     </row>
@@ -980,11 +1358,11 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>HD건설기계</t>
+          <t>프론트라인</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>31</v>
+        <v>175</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
@@ -995,17 +1373,17 @@
         <v>1</v>
       </c>
       <c r="F5" t="n">
-        <v>4123000</v>
+        <v>8471815.962899337</v>
       </c>
       <c r="G5" t="n">
-        <v>87904</v>
+        <v>4041951.962899337</v>
       </c>
       <c r="H5" t="n">
-        <v>2.178485964150543</v>
+        <v>91.24325177701475</v>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>2026-03-21T04:59:43</t>
+          <t>2026-03-21T05:00:11</t>
         </is>
       </c>
     </row>
@@ -1017,11 +1395,11 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>삼성화재</t>
+          <t>세아제강</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>7</v>
+        <v>50</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
@@ -1032,17 +1410,17 @@
         <v>1</v>
       </c>
       <c r="F6" t="n">
-        <v>3321500</v>
+        <v>7395000</v>
       </c>
       <c r="G6" t="n">
-        <v>-309500</v>
+        <v>1085000</v>
       </c>
       <c r="H6" t="n">
-        <v>-8.523822638391627</v>
+        <v>17.19492868462758</v>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>2026-03-21T04:59:43</t>
+          <t>2026-03-21T05:00:11</t>
         </is>
       </c>
     </row>
@@ -1054,11 +1432,11 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>휴스틸</t>
+          <t>DL이앤씨</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>500</v>
+        <v>80</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
@@ -1069,17 +1447,17 @@
         <v>1</v>
       </c>
       <c r="F7" t="n">
-        <v>2750000</v>
+        <v>5392000</v>
       </c>
       <c r="G7" t="n">
-        <v>471390</v>
+        <v>1981000</v>
       </c>
       <c r="H7" t="n">
-        <v>20.68761218462133</v>
+        <v>58.07681031955438</v>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>2026-03-21T04:59:43</t>
+          <t>2026-03-21T05:00:11</t>
         </is>
       </c>
     </row>
@@ -1091,11 +1469,11 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>현대제철</t>
+          <t>TIME 코리아밸류업액티브</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>70</v>
+        <v>201</v>
       </c>
       <c r="D8" t="inlineStr">
         <is>
@@ -1106,17 +1484,17 @@
         <v>1</v>
       </c>
       <c r="F8" t="n">
-        <v>2621500</v>
+        <v>4797870</v>
       </c>
       <c r="G8" t="n">
-        <v>-186000</v>
+        <v>74073</v>
       </c>
       <c r="H8" t="n">
-        <v>-6.625111308993767</v>
+        <v>1.568081778281328</v>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>2026-03-21T04:59:43</t>
+          <t>2026-03-21T05:00:11</t>
         </is>
       </c>
     </row>
@@ -1128,11 +1506,11 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>KoAct 코스닥액티브</t>
+          <t>동원개발</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>200</v>
+        <v>1360</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
@@ -1143,17 +1521,17 @@
         <v>1</v>
       </c>
       <c r="F9" t="n">
-        <v>2582000</v>
+        <v>4202400</v>
       </c>
       <c r="G9" t="n">
-        <v>-120000</v>
+        <v>465000</v>
       </c>
       <c r="H9" t="n">
-        <v>-4.441154700222058</v>
+        <v>12.44180446299566</v>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>2026-03-21T04:59:43</t>
+          <t>2026-03-21T05:00:11</t>
         </is>
       </c>
     </row>
@@ -1165,11 +1543,11 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>케이씨</t>
+          <t>HD건설기계</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>50</v>
+        <v>31</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
@@ -1180,17 +1558,17 @@
         <v>1</v>
       </c>
       <c r="F10" t="n">
-        <v>1670000</v>
+        <v>4123000</v>
       </c>
       <c r="G10" t="n">
-        <v>20500</v>
+        <v>87904</v>
       </c>
       <c r="H10" t="n">
-        <v>1.242800848742043</v>
+        <v>2.178485964150543</v>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>2026-03-21T04:59:43</t>
+          <t>2026-03-21T05:00:11</t>
         </is>
       </c>
     </row>
@@ -1202,11 +1580,11 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>하나금융지주</t>
+          <t>피바디 에너지</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>10</v>
+        <v>65</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
@@ -1217,33 +1595,33 @@
         <v>1</v>
       </c>
       <c r="F11" t="n">
-        <v>1132000</v>
+        <v>3649438.50225304</v>
       </c>
       <c r="G11" t="n">
-        <v>23000</v>
+        <v>2178666.50225304</v>
       </c>
       <c r="H11" t="n">
-        <v>2.073940486925157</v>
+        <v>148.1308117269733</v>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>2026-03-21T04:59:43</t>
+          <t>2026-03-21T05:00:11</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-03-21</t>
+          <t>2026-03-17</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>페트로브라스 (ADR)</t>
+          <t>삼성화재</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>480</v>
+        <v>7</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
@@ -1254,33 +1632,33 @@
         <v>1</v>
       </c>
       <c r="F12" t="n">
-        <v>13579584.97235231</v>
+        <v>3321500</v>
       </c>
       <c r="G12" t="n">
-        <v>1473035.972352311</v>
+        <v>-309500</v>
       </c>
       <c r="H12" t="n">
-        <v>12.16726560436265</v>
+        <v>-8.523822638391627</v>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>2026-03-21T04:57:12</t>
+          <t>2026-03-21T05:00:11</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-03-21</t>
+          <t>2026-03-17</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>AGNC 인베스트먼트</t>
+          <t>휴스틸</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>700</v>
+        <v>500</v>
       </c>
       <c r="D13" t="inlineStr">
         <is>
@@ -1291,33 +1669,33 @@
         <v>1</v>
       </c>
       <c r="F13" t="n">
-        <v>10270464.45007324</v>
+        <v>2750000</v>
       </c>
       <c r="G13" t="n">
-        <v>-561550.5499267559</v>
+        <v>471390</v>
       </c>
       <c r="H13" t="n">
-        <v>-5.184174411933109</v>
+        <v>20.68761218462133</v>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>2026-03-21T04:57:12</t>
+          <t>2026-03-21T05:00:11</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-03-21</t>
+          <t>2026-03-17</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>대한조선</t>
+          <t>현대제철</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>100</v>
+        <v>70</v>
       </c>
       <c r="D14" t="inlineStr">
         <is>
@@ -1328,33 +1706,33 @@
         <v>1</v>
       </c>
       <c r="F14" t="n">
-        <v>9120000</v>
+        <v>2621500</v>
       </c>
       <c r="G14" t="n">
-        <v>1907000</v>
+        <v>-186000</v>
       </c>
       <c r="H14" t="n">
-        <v>26.43837515596839</v>
+        <v>-6.625111308993767</v>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>2026-03-21T04:57:12</t>
+          <t>2026-03-21T05:00:11</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-03-21</t>
+          <t>2026-03-17</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>프론트라인</t>
+          <t>KoAct 코스닥액티브</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>175</v>
+        <v>200</v>
       </c>
       <c r="D15" t="inlineStr">
         <is>
@@ -1365,33 +1743,33 @@
         <v>1</v>
       </c>
       <c r="F15" t="n">
-        <v>8471815.962899337</v>
+        <v>2582000</v>
       </c>
       <c r="G15" t="n">
-        <v>4041951.962899337</v>
+        <v>-120000</v>
       </c>
       <c r="H15" t="n">
-        <v>91.24325177701475</v>
+        <v>-4.441154700222058</v>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>2026-03-21T04:57:12</t>
+          <t>2026-03-21T05:00:11</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-03-21</t>
+          <t>2026-03-17</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>시드릴</t>
+          <t>넥스틸</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>123</v>
+        <v>200</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
@@ -1402,33 +1780,33 @@
         <v>1</v>
       </c>
       <c r="F16" t="n">
-        <v>8070101.805898919</v>
+        <v>2514000</v>
       </c>
       <c r="G16" t="n">
-        <v>1619750.805898919</v>
+        <v>503000</v>
       </c>
       <c r="H16" t="n">
-        <v>25.11104908707943</v>
+        <v>25.01243162605669</v>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>2026-03-21T04:57:12</t>
+          <t>2026-03-21T05:00:11</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-03-21</t>
+          <t>2026-03-17</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>세아제강</t>
+          <t>대신증권</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>50</v>
+        <v>55</v>
       </c>
       <c r="D17" t="inlineStr">
         <is>
@@ -1439,33 +1817,33 @@
         <v>1</v>
       </c>
       <c r="F17" t="n">
-        <v>7395000</v>
+        <v>2219250</v>
       </c>
       <c r="G17" t="n">
-        <v>1085000</v>
+        <v>509749</v>
       </c>
       <c r="H17" t="n">
-        <v>17.19492868462758</v>
+        <v>29.81858448752005</v>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>2026-03-21T04:57:12</t>
+          <t>2026-03-21T05:00:11</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-03-21</t>
+          <t>2026-03-17</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>센트러스 에너지</t>
+          <t>미창석유</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>25</v>
+        <v>18</v>
       </c>
       <c r="D18" t="inlineStr">
         <is>
@@ -1476,33 +1854,33 @@
         <v>1</v>
       </c>
       <c r="F18" t="n">
-        <v>7026050.85816239</v>
+        <v>2097000</v>
       </c>
       <c r="G18" t="n">
-        <v>-406805.1418376099</v>
+        <v>-295200</v>
       </c>
       <c r="H18" t="n">
-        <v>-5.473066366920198</v>
+        <v>-12.34010534236268</v>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>2026-03-21T04:57:12</t>
+          <t>2026-03-21T05:00:11</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-03-21</t>
+          <t>2026-03-17</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>트랜스오션</t>
+          <t>대창단조</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>750</v>
+        <v>300</v>
       </c>
       <c r="D19" t="inlineStr">
         <is>
@@ -1513,33 +1891,33 @@
         <v>1</v>
       </c>
       <c r="F19" t="n">
-        <v>7020031.5082007</v>
+        <v>2004000</v>
       </c>
       <c r="G19" t="n">
-        <v>2892797.5082007</v>
+        <v>-54000</v>
       </c>
       <c r="H19" t="n">
-        <v>70.09046514446965</v>
+        <v>-2.623906705539359</v>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>2026-03-21T04:57:12</t>
+          <t>2026-03-21T05:00:11</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-03-21</t>
+          <t>2026-03-17</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>노블</t>
+          <t>동방</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>99</v>
+        <v>681</v>
       </c>
       <c r="D20" t="inlineStr">
         <is>
@@ -1550,33 +1928,33 @@
         <v>1</v>
       </c>
       <c r="F20" t="n">
-        <v>6958769.981090547</v>
+        <v>1995330</v>
       </c>
       <c r="G20" t="n">
-        <v>3051561.981090547</v>
+        <v>23829</v>
       </c>
       <c r="H20" t="n">
-        <v>78.10083264291399</v>
+        <v>1.208672985709873</v>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>2026-03-21T04:57:12</t>
+          <t>2026-03-21T05:00:11</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-03-21</t>
+          <t>2026-03-17</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>타이드워터</t>
+          <t>케이씨</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="D21" t="inlineStr">
         <is>
@@ -1587,33 +1965,33 @@
         <v>1</v>
       </c>
       <c r="F21" t="n">
-        <v>5235363.852789983</v>
+        <v>1670000</v>
       </c>
       <c r="G21" t="n">
-        <v>1510818.852789983</v>
+        <v>20500</v>
       </c>
       <c r="H21" t="n">
-        <v>40.56385015592463</v>
+        <v>1.242800848742043</v>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>2026-03-21T04:57:12</t>
+          <t>2026-03-21T05:00:11</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2026-03-21</t>
+          <t>2026-03-17</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>노브</t>
+          <t>하나금융지주</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>185</v>
+        <v>10</v>
       </c>
       <c r="D22" t="inlineStr">
         <is>
@@ -1624,33 +2002,33 @@
         <v>1</v>
       </c>
       <c r="F22" t="n">
-        <v>5200391.447092756</v>
+        <v>1132000</v>
       </c>
       <c r="G22" t="n">
-        <v>1890383.447092756</v>
+        <v>23000</v>
       </c>
       <c r="H22" t="n">
-        <v>57.11114435653194</v>
+        <v>2.073940486925157</v>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>2026-03-21T04:57:12</t>
+          <t>2026-03-21T05:00:11</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-03-21</t>
+          <t>2026-03-17</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>TIME 코리아밸류업액티브</t>
+          <t>삼성생명</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>201</v>
+        <v>4</v>
       </c>
       <c r="D23" t="inlineStr">
         <is>
@@ -1661,33 +2039,33 @@
         <v>1</v>
       </c>
       <c r="F23" t="n">
-        <v>4797870</v>
+        <v>926000</v>
       </c>
       <c r="G23" t="n">
-        <v>74073</v>
+        <v>93000</v>
       </c>
       <c r="H23" t="n">
-        <v>1.568081778281328</v>
+        <v>11.16446578631453</v>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>2026-03-21T04:57:12</t>
+          <t>2026-03-21T05:00:11</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>2026-03-21</t>
+          <t>2026-03-17</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>오케아니스 에코 탱커스</t>
+          <t>비에이치아이</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>65</v>
+        <v>8</v>
       </c>
       <c r="D24" t="inlineStr">
         <is>
@@ -1698,33 +2076,33 @@
         <v>1</v>
       </c>
       <c r="F24" t="n">
-        <v>4511179.137784176</v>
+        <v>876000</v>
       </c>
       <c r="G24" t="n">
-        <v>2254819.137784176</v>
+        <v>210885</v>
       </c>
       <c r="H24" t="n">
-        <v>99.93171026716374</v>
+        <v>31.70654698811484</v>
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>2026-03-21T04:57:12</t>
+          <t>2026-03-21T05:00:11</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-03-21</t>
+          <t>2026-03-17</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>삼성화재</t>
+          <t>하프니아</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>9</v>
+        <v>80</v>
       </c>
       <c r="D25" t="inlineStr">
         <is>
@@ -1735,17 +2113,17 @@
         <v>1</v>
       </c>
       <c r="F25" t="n">
-        <v>4270500</v>
+        <v>842704.775390625</v>
       </c>
       <c r="G25" t="n">
-        <v>-360500</v>
+        <v>216973.775390625</v>
       </c>
       <c r="H25" t="n">
-        <v>-7.784495789246384</v>
+        <v>34.67524789256486</v>
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>2026-03-21T04:57:12</t>
+          <t>2026-03-21T05:00:11</t>
         </is>
       </c>
     </row>
@@ -1757,11 +2135,11 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>동원개발</t>
+          <t>페트로브라스 (ADR)</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>1360</v>
+        <v>480</v>
       </c>
       <c r="D26" t="inlineStr">
         <is>
@@ -1772,13 +2150,13 @@
         <v>1</v>
       </c>
       <c r="F26" t="n">
-        <v>4202400</v>
+        <v>13579584.97235231</v>
       </c>
       <c r="G26" t="n">
-        <v>465000</v>
+        <v>1473035.972352311</v>
       </c>
       <c r="H26" t="n">
-        <v>12.44180446299566</v>
+        <v>12.16726560436265</v>
       </c>
       <c r="I26" t="inlineStr">
         <is>
@@ -1794,11 +2172,11 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>HD건설기계</t>
+          <t>AGNC 인베스트먼트</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>31</v>
+        <v>700</v>
       </c>
       <c r="D27" t="inlineStr">
         <is>
@@ -1809,13 +2187,13 @@
         <v>1</v>
       </c>
       <c r="F27" t="n">
-        <v>4123000</v>
+        <v>10270464.45007324</v>
       </c>
       <c r="G27" t="n">
-        <v>87904</v>
+        <v>-561550.5499267559</v>
       </c>
       <c r="H27" t="n">
-        <v>2.178485964150543</v>
+        <v>-5.184174411933109</v>
       </c>
       <c r="I27" t="inlineStr">
         <is>
@@ -1831,11 +2209,11 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>차코스 에너지 내비게이션</t>
+          <t>대한조선</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>75</v>
+        <v>100</v>
       </c>
       <c r="D28" t="inlineStr">
         <is>
@@ -1846,13 +2224,13 @@
         <v>1</v>
       </c>
       <c r="F28" t="n">
-        <v>4026924.996845168</v>
+        <v>9120000</v>
       </c>
       <c r="G28" t="n">
-        <v>202276.9968451681</v>
+        <v>1907000</v>
       </c>
       <c r="H28" t="n">
-        <v>5.28877420471552</v>
+        <v>26.43837515596839</v>
       </c>
       <c r="I28" t="inlineStr">
         <is>
@@ -1868,11 +2246,11 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>넥스틸</t>
+          <t>프론트라인</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>300</v>
+        <v>175</v>
       </c>
       <c r="D29" t="inlineStr">
         <is>
@@ -1883,13 +2261,13 @@
         <v>1</v>
       </c>
       <c r="F29" t="n">
-        <v>3771000</v>
+        <v>8471815.962899337</v>
       </c>
       <c r="G29" t="n">
-        <v>521000</v>
+        <v>4041951.962899337</v>
       </c>
       <c r="H29" t="n">
-        <v>16.03076923076923</v>
+        <v>91.24325177701475</v>
       </c>
       <c r="I29" t="inlineStr">
         <is>
@@ -1905,11 +2283,11 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>피바디 에너지</t>
+          <t>시드릴</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>65</v>
+        <v>123</v>
       </c>
       <c r="D30" t="inlineStr">
         <is>
@@ -1920,13 +2298,13 @@
         <v>1</v>
       </c>
       <c r="F30" t="n">
-        <v>3649438.50225304</v>
+        <v>8070101.805898919</v>
       </c>
       <c r="G30" t="n">
-        <v>2178666.50225304</v>
+        <v>1619750.805898919</v>
       </c>
       <c r="H30" t="n">
-        <v>148.1308117269733</v>
+        <v>25.11104908707943</v>
       </c>
       <c r="I30" t="inlineStr">
         <is>
@@ -1942,11 +2320,11 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>현대제철</t>
+          <t>세아제강</t>
         </is>
       </c>
       <c r="C31" t="n">
-        <v>80</v>
+        <v>50</v>
       </c>
       <c r="D31" t="inlineStr">
         <is>
@@ -1957,13 +2335,13 @@
         <v>1</v>
       </c>
       <c r="F31" t="n">
-        <v>2996000</v>
+        <v>7395000</v>
       </c>
       <c r="G31" t="n">
-        <v>-182000</v>
+        <v>1085000</v>
       </c>
       <c r="H31" t="n">
-        <v>-5.726872246696035</v>
+        <v>17.19492868462758</v>
       </c>
       <c r="I31" t="inlineStr">
         <is>
@@ -1979,11 +2357,11 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>더치 브로스</t>
+          <t>센트러스 에너지</t>
         </is>
       </c>
       <c r="C32" t="n">
-        <v>39</v>
+        <v>25</v>
       </c>
       <c r="D32" t="inlineStr">
         <is>
@@ -1994,13 +2372,13 @@
         <v>1</v>
       </c>
       <c r="F32" t="n">
-        <v>2934418.414306641</v>
+        <v>7026050.85816239</v>
       </c>
       <c r="G32" t="n">
-        <v>-256226.5856933594</v>
+        <v>-406805.1418376099</v>
       </c>
       <c r="H32" t="n">
-        <v>-8.030557636257226</v>
+        <v>-5.473066366920198</v>
       </c>
       <c r="I32" t="inlineStr">
         <is>
@@ -2016,11 +2394,11 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>휴스틸</t>
+          <t>트랜스오션</t>
         </is>
       </c>
       <c r="C33" t="n">
-        <v>500</v>
+        <v>750</v>
       </c>
       <c r="D33" t="inlineStr">
         <is>
@@ -2031,13 +2409,13 @@
         <v>1</v>
       </c>
       <c r="F33" t="n">
-        <v>2750000</v>
+        <v>7020031.5082007</v>
       </c>
       <c r="G33" t="n">
-        <v>471390</v>
+        <v>2892797.5082007</v>
       </c>
       <c r="H33" t="n">
-        <v>20.68761218462133</v>
+        <v>70.09046514446965</v>
       </c>
       <c r="I33" t="inlineStr">
         <is>
@@ -2053,11 +2431,11 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>DL이앤씨</t>
+          <t>노블</t>
         </is>
       </c>
       <c r="C34" t="n">
-        <v>40</v>
+        <v>99</v>
       </c>
       <c r="D34" t="inlineStr">
         <is>
@@ -2068,13 +2446,13 @@
         <v>1</v>
       </c>
       <c r="F34" t="n">
-        <v>2696000</v>
+        <v>6958769.981090547</v>
       </c>
       <c r="G34" t="n">
-        <v>990500</v>
+        <v>3051561.981090547</v>
       </c>
       <c r="H34" t="n">
-        <v>58.07681031955438</v>
+        <v>78.10083264291399</v>
       </c>
       <c r="I34" t="inlineStr">
         <is>
@@ -2090,11 +2468,11 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>KoAct 코스닥액티브</t>
+          <t>타이드워터</t>
         </is>
       </c>
       <c r="C35" t="n">
-        <v>200</v>
+        <v>48</v>
       </c>
       <c r="D35" t="inlineStr">
         <is>
@@ -2105,13 +2483,13 @@
         <v>1</v>
       </c>
       <c r="F35" t="n">
-        <v>2582000</v>
+        <v>5235363.852789983</v>
       </c>
       <c r="G35" t="n">
-        <v>-120000</v>
+        <v>1510818.852789983</v>
       </c>
       <c r="H35" t="n">
-        <v>-4.441154700222058</v>
+        <v>40.56385015592463</v>
       </c>
       <c r="I35" t="inlineStr">
         <is>
@@ -2127,11 +2505,11 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>대신증권</t>
+          <t>노브</t>
         </is>
       </c>
       <c r="C36" t="n">
-        <v>55</v>
+        <v>185</v>
       </c>
       <c r="D36" t="inlineStr">
         <is>
@@ -2142,13 +2520,13 @@
         <v>1</v>
       </c>
       <c r="F36" t="n">
-        <v>2219250</v>
+        <v>5200391.447092756</v>
       </c>
       <c r="G36" t="n">
-        <v>509749</v>
+        <v>1890383.447092756</v>
       </c>
       <c r="H36" t="n">
-        <v>29.81858448752005</v>
+        <v>57.11114435653194</v>
       </c>
       <c r="I36" t="inlineStr">
         <is>
@@ -2164,11 +2542,11 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>발레로 에너지</t>
+          <t>TIME 코리아밸류업액티브</t>
         </is>
       </c>
       <c r="C37" t="n">
-        <v>6</v>
+        <v>201</v>
       </c>
       <c r="D37" t="inlineStr">
         <is>
@@ -2179,13 +2557,13 @@
         <v>1</v>
       </c>
       <c r="F37" t="n">
-        <v>2165691.085066516</v>
+        <v>4797870</v>
       </c>
       <c r="G37" t="n">
-        <v>101701.085066516</v>
+        <v>74073</v>
       </c>
       <c r="H37" t="n">
-        <v>4.927402025519307</v>
+        <v>1.568081778281328</v>
       </c>
       <c r="I37" t="inlineStr">
         <is>
@@ -2201,11 +2579,11 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>미창석유</t>
+          <t>오케아니스 에코 탱커스</t>
         </is>
       </c>
       <c r="C38" t="n">
-        <v>18</v>
+        <v>65</v>
       </c>
       <c r="D38" t="inlineStr">
         <is>
@@ -2216,13 +2594,13 @@
         <v>1</v>
       </c>
       <c r="F38" t="n">
-        <v>2097000</v>
+        <v>4511179.137784176</v>
       </c>
       <c r="G38" t="n">
-        <v>-295200</v>
+        <v>2254819.137784176</v>
       </c>
       <c r="H38" t="n">
-        <v>-12.34010534236268</v>
+        <v>99.93171026716374</v>
       </c>
       <c r="I38" t="inlineStr">
         <is>
@@ -2238,11 +2616,11 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>하나금융지주</t>
+          <t>삼성화재</t>
         </is>
       </c>
       <c r="C39" t="n">
-        <v>18</v>
+        <v>9</v>
       </c>
       <c r="D39" t="inlineStr">
         <is>
@@ -2253,13 +2631,13 @@
         <v>1</v>
       </c>
       <c r="F39" t="n">
-        <v>2037600</v>
+        <v>4270500</v>
       </c>
       <c r="G39" t="n">
-        <v>12200</v>
+        <v>-360500</v>
       </c>
       <c r="H39" t="n">
-        <v>0.6023501530561864</v>
+        <v>-7.784495789246384</v>
       </c>
       <c r="I39" t="inlineStr">
         <is>
@@ -2275,11 +2653,11 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>대창단조</t>
+          <t>동원개발</t>
         </is>
       </c>
       <c r="C40" t="n">
-        <v>300</v>
+        <v>1360</v>
       </c>
       <c r="D40" t="inlineStr">
         <is>
@@ -2290,13 +2668,13 @@
         <v>1</v>
       </c>
       <c r="F40" t="n">
-        <v>2004000</v>
+        <v>4202400</v>
       </c>
       <c r="G40" t="n">
-        <v>-54000</v>
+        <v>465000</v>
       </c>
       <c r="H40" t="n">
-        <v>-2.623906705539359</v>
+        <v>12.44180446299566</v>
       </c>
       <c r="I40" t="inlineStr">
         <is>
@@ -2312,11 +2690,11 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>동방</t>
+          <t>HD건설기계</t>
         </is>
       </c>
       <c r="C41" t="n">
-        <v>681</v>
+        <v>31</v>
       </c>
       <c r="D41" t="inlineStr">
         <is>
@@ -2327,13 +2705,13 @@
         <v>1</v>
       </c>
       <c r="F41" t="n">
-        <v>1995330</v>
+        <v>4123000</v>
       </c>
       <c r="G41" t="n">
-        <v>23829</v>
+        <v>87904</v>
       </c>
       <c r="H41" t="n">
-        <v>1.208672985709873</v>
+        <v>2.178485964150543</v>
       </c>
       <c r="I41" t="inlineStr">
         <is>
@@ -2349,11 +2727,11 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>스타 벌크 캐리어스</t>
+          <t>차코스 에너지 내비게이션</t>
         </is>
       </c>
       <c r="C42" t="n">
-        <v>50</v>
+        <v>75</v>
       </c>
       <c r="D42" t="inlineStr">
         <is>
@@ -2364,13 +2742,13 @@
         <v>1</v>
       </c>
       <c r="F42" t="n">
-        <v>1680142.640194588</v>
+        <v>4026924.996845168</v>
       </c>
       <c r="G42" t="n">
-        <v>365789.6401945879</v>
+        <v>202276.9968451681</v>
       </c>
       <c r="H42" t="n">
-        <v>27.83039565433242</v>
+        <v>5.28877420471552</v>
       </c>
       <c r="I42" t="inlineStr">
         <is>
@@ -2386,11 +2764,11 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>케이씨</t>
+          <t>넥스틸</t>
         </is>
       </c>
       <c r="C43" t="n">
-        <v>50</v>
+        <v>300</v>
       </c>
       <c r="D43" t="inlineStr">
         <is>
@@ -2401,13 +2779,13 @@
         <v>1</v>
       </c>
       <c r="F43" t="n">
-        <v>1670000</v>
+        <v>3771000</v>
       </c>
       <c r="G43" t="n">
-        <v>20500</v>
+        <v>521000</v>
       </c>
       <c r="H43" t="n">
-        <v>1.242800848742043</v>
+        <v>16.03076923076923</v>
       </c>
       <c r="I43" t="inlineStr">
         <is>
@@ -2423,11 +2801,11 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>유나이티드헬스 그룹</t>
+          <t>피바디 에너지</t>
         </is>
       </c>
       <c r="C44" t="n">
-        <v>4</v>
+        <v>65</v>
       </c>
       <c r="D44" t="inlineStr">
         <is>
@@ -2438,13 +2816,13 @@
         <v>1</v>
       </c>
       <c r="F44" t="n">
-        <v>1658864.328313038</v>
+        <v>3649438.50225304</v>
       </c>
       <c r="G44" t="n">
-        <v>-35591.67168696248</v>
+        <v>2178666.50225304</v>
       </c>
       <c r="H44" t="n">
-        <v>-2.100477774988697</v>
+        <v>148.1308117269733</v>
       </c>
       <c r="I44" t="inlineStr">
         <is>
@@ -2460,11 +2838,11 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>텍사스 퍼시픽 랜드</t>
+          <t>현대제철</t>
         </is>
       </c>
       <c r="C45" t="n">
-        <v>2</v>
+        <v>80</v>
       </c>
       <c r="D45" t="inlineStr">
         <is>
@@ -2475,13 +2853,13 @@
         <v>1</v>
       </c>
       <c r="F45" t="n">
-        <v>1563247.374122903</v>
+        <v>2996000</v>
       </c>
       <c r="G45" t="n">
-        <v>-14646.62587709725</v>
+        <v>-182000</v>
       </c>
       <c r="H45" t="n">
-        <v>-0.9282388979929735</v>
+        <v>-5.726872246696035</v>
       </c>
       <c r="I45" t="inlineStr">
         <is>
@@ -2497,11 +2875,11 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>LX인터내셔널</t>
+          <t>더치 브로스</t>
         </is>
       </c>
       <c r="C46" t="n">
-        <v>20</v>
+        <v>39</v>
       </c>
       <c r="D46" t="inlineStr">
         <is>
@@ -2512,13 +2890,13 @@
         <v>1</v>
       </c>
       <c r="F46" t="n">
-        <v>943000</v>
+        <v>2934418.414306641</v>
       </c>
       <c r="G46" t="n">
-        <v>4000</v>
+        <v>-256226.5856933594</v>
       </c>
       <c r="H46" t="n">
-        <v>0.4259850905218318</v>
+        <v>-8.030557636257226</v>
       </c>
       <c r="I46" t="inlineStr">
         <is>
@@ -2534,11 +2912,11 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>삼성생명</t>
+          <t>휴스틸</t>
         </is>
       </c>
       <c r="C47" t="n">
-        <v>4</v>
+        <v>500</v>
       </c>
       <c r="D47" t="inlineStr">
         <is>
@@ -2549,13 +2927,13 @@
         <v>1</v>
       </c>
       <c r="F47" t="n">
-        <v>926000</v>
+        <v>2750000</v>
       </c>
       <c r="G47" t="n">
-        <v>93000</v>
+        <v>471390</v>
       </c>
       <c r="H47" t="n">
-        <v>11.16446578631453</v>
+        <v>20.68761218462133</v>
       </c>
       <c r="I47" t="inlineStr">
         <is>
@@ -2571,11 +2949,11 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>비에이치아이</t>
+          <t>DL이앤씨</t>
         </is>
       </c>
       <c r="C48" t="n">
-        <v>8</v>
+        <v>40</v>
       </c>
       <c r="D48" t="inlineStr">
         <is>
@@ -2586,13 +2964,13 @@
         <v>1</v>
       </c>
       <c r="F48" t="n">
-        <v>876000</v>
+        <v>2696000</v>
       </c>
       <c r="G48" t="n">
-        <v>210885</v>
+        <v>990500</v>
       </c>
       <c r="H48" t="n">
-        <v>31.70654698811484</v>
+        <v>58.07681031955438</v>
       </c>
       <c r="I48" t="inlineStr">
         <is>
@@ -2608,11 +2986,11 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>하프니아</t>
+          <t>KoAct 코스닥액티브</t>
         </is>
       </c>
       <c r="C49" t="n">
-        <v>80</v>
+        <v>200</v>
       </c>
       <c r="D49" t="inlineStr">
         <is>
@@ -2623,13 +3001,13 @@
         <v>1</v>
       </c>
       <c r="F49" t="n">
-        <v>842704.775390625</v>
+        <v>2582000</v>
       </c>
       <c r="G49" t="n">
-        <v>216973.775390625</v>
+        <v>-120000</v>
       </c>
       <c r="H49" t="n">
-        <v>34.67524789256486</v>
+        <v>-4.441154700222058</v>
       </c>
       <c r="I49" t="inlineStr">
         <is>
@@ -2645,11 +3023,11 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>클리블랜드 클리프스</t>
+          <t>대신증권</t>
         </is>
       </c>
       <c r="C50" t="n">
-        <v>70</v>
+        <v>55</v>
       </c>
       <c r="D50" t="inlineStr">
         <is>
@@ -2660,13 +3038,13 @@
         <v>1</v>
       </c>
       <c r="F50" t="n">
-        <v>823743.9360268187</v>
+        <v>2219250</v>
       </c>
       <c r="G50" t="n">
-        <v>-192311.0639731813</v>
+        <v>509749</v>
       </c>
       <c r="H50" t="n">
-        <v>-18.92722972409774</v>
+        <v>29.81858448752005</v>
       </c>
       <c r="I50" t="inlineStr">
         <is>
@@ -2682,11 +3060,11 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>낫 오프쇼어 파트너스</t>
+          <t>발레로 에너지</t>
         </is>
       </c>
       <c r="C51" t="n">
-        <v>30</v>
+        <v>6</v>
       </c>
       <c r="D51" t="inlineStr">
         <is>
@@ -2697,13 +3075,13 @@
         <v>1</v>
       </c>
       <c r="F51" t="n">
-        <v>413075.8057155996</v>
+        <v>2165691.085066516</v>
       </c>
       <c r="G51" t="n">
-        <v>-4439.194284400437</v>
+        <v>101701.085066516</v>
       </c>
       <c r="H51" t="n">
-        <v>-1.063241867813237</v>
+        <v>4.927402025519307</v>
       </c>
       <c r="I51" t="inlineStr">
         <is>
@@ -2719,30 +3097,548 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
+          <t>미창석유</t>
+        </is>
+      </c>
+      <c r="C52" t="n">
+        <v>18</v>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E52" t="n">
+        <v>1</v>
+      </c>
+      <c r="F52" t="n">
+        <v>2097000</v>
+      </c>
+      <c r="G52" t="n">
+        <v>-295200</v>
+      </c>
+      <c r="H52" t="n">
+        <v>-12.34010534236268</v>
+      </c>
+      <c r="I52" t="inlineStr">
+        <is>
+          <t>2026-03-21T04:57:12</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>2026-03-21</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>하나금융지주</t>
+        </is>
+      </c>
+      <c r="C53" t="n">
+        <v>18</v>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E53" t="n">
+        <v>1</v>
+      </c>
+      <c r="F53" t="n">
+        <v>2037600</v>
+      </c>
+      <c r="G53" t="n">
+        <v>12200</v>
+      </c>
+      <c r="H53" t="n">
+        <v>0.6023501530561864</v>
+      </c>
+      <c r="I53" t="inlineStr">
+        <is>
+          <t>2026-03-21T04:57:12</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>2026-03-21</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>대창단조</t>
+        </is>
+      </c>
+      <c r="C54" t="n">
+        <v>300</v>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E54" t="n">
+        <v>1</v>
+      </c>
+      <c r="F54" t="n">
+        <v>2004000</v>
+      </c>
+      <c r="G54" t="n">
+        <v>-54000</v>
+      </c>
+      <c r="H54" t="n">
+        <v>-2.623906705539359</v>
+      </c>
+      <c r="I54" t="inlineStr">
+        <is>
+          <t>2026-03-21T04:57:12</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>2026-03-21</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>동방</t>
+        </is>
+      </c>
+      <c r="C55" t="n">
+        <v>681</v>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E55" t="n">
+        <v>1</v>
+      </c>
+      <c r="F55" t="n">
+        <v>1995330</v>
+      </c>
+      <c r="G55" t="n">
+        <v>23829</v>
+      </c>
+      <c r="H55" t="n">
+        <v>1.208672985709873</v>
+      </c>
+      <c r="I55" t="inlineStr">
+        <is>
+          <t>2026-03-21T04:57:12</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>2026-03-21</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>스타 벌크 캐리어스</t>
+        </is>
+      </c>
+      <c r="C56" t="n">
+        <v>50</v>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E56" t="n">
+        <v>1</v>
+      </c>
+      <c r="F56" t="n">
+        <v>1680142.640194588</v>
+      </c>
+      <c r="G56" t="n">
+        <v>365789.6401945879</v>
+      </c>
+      <c r="H56" t="n">
+        <v>27.83039565433242</v>
+      </c>
+      <c r="I56" t="inlineStr">
+        <is>
+          <t>2026-03-21T04:57:12</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>2026-03-21</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>케이씨</t>
+        </is>
+      </c>
+      <c r="C57" t="n">
+        <v>50</v>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E57" t="n">
+        <v>1</v>
+      </c>
+      <c r="F57" t="n">
+        <v>1670000</v>
+      </c>
+      <c r="G57" t="n">
+        <v>20500</v>
+      </c>
+      <c r="H57" t="n">
+        <v>1.242800848742043</v>
+      </c>
+      <c r="I57" t="inlineStr">
+        <is>
+          <t>2026-03-21T04:57:12</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>2026-03-21</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>유나이티드헬스 그룹</t>
+        </is>
+      </c>
+      <c r="C58" t="n">
+        <v>4</v>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E58" t="n">
+        <v>1</v>
+      </c>
+      <c r="F58" t="n">
+        <v>1658864.328313038</v>
+      </c>
+      <c r="G58" t="n">
+        <v>-35591.67168696248</v>
+      </c>
+      <c r="H58" t="n">
+        <v>-2.100477774988697</v>
+      </c>
+      <c r="I58" t="inlineStr">
+        <is>
+          <t>2026-03-21T04:57:12</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>2026-03-21</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>텍사스 퍼시픽 랜드</t>
+        </is>
+      </c>
+      <c r="C59" t="n">
+        <v>2</v>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E59" t="n">
+        <v>1</v>
+      </c>
+      <c r="F59" t="n">
+        <v>1563247.374122903</v>
+      </c>
+      <c r="G59" t="n">
+        <v>-14646.62587709725</v>
+      </c>
+      <c r="H59" t="n">
+        <v>-0.9282388979929735</v>
+      </c>
+      <c r="I59" t="inlineStr">
+        <is>
+          <t>2026-03-21T04:57:12</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>2026-03-21</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>LX인터내셔널</t>
+        </is>
+      </c>
+      <c r="C60" t="n">
+        <v>20</v>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E60" t="n">
+        <v>1</v>
+      </c>
+      <c r="F60" t="n">
+        <v>943000</v>
+      </c>
+      <c r="G60" t="n">
+        <v>4000</v>
+      </c>
+      <c r="H60" t="n">
+        <v>0.4259850905218318</v>
+      </c>
+      <c r="I60" t="inlineStr">
+        <is>
+          <t>2026-03-21T04:57:12</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>2026-03-21</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>삼성생명</t>
+        </is>
+      </c>
+      <c r="C61" t="n">
+        <v>4</v>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E61" t="n">
+        <v>1</v>
+      </c>
+      <c r="F61" t="n">
+        <v>926000</v>
+      </c>
+      <c r="G61" t="n">
+        <v>93000</v>
+      </c>
+      <c r="H61" t="n">
+        <v>11.16446578631453</v>
+      </c>
+      <c r="I61" t="inlineStr">
+        <is>
+          <t>2026-03-21T04:57:12</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>2026-03-21</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>비에이치아이</t>
+        </is>
+      </c>
+      <c r="C62" t="n">
+        <v>8</v>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E62" t="n">
+        <v>1</v>
+      </c>
+      <c r="F62" t="n">
+        <v>876000</v>
+      </c>
+      <c r="G62" t="n">
+        <v>210885</v>
+      </c>
+      <c r="H62" t="n">
+        <v>31.70654698811484</v>
+      </c>
+      <c r="I62" t="inlineStr">
+        <is>
+          <t>2026-03-21T04:57:12</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>2026-03-21</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>하프니아</t>
+        </is>
+      </c>
+      <c r="C63" t="n">
+        <v>80</v>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E63" t="n">
+        <v>1</v>
+      </c>
+      <c r="F63" t="n">
+        <v>842704.775390625</v>
+      </c>
+      <c r="G63" t="n">
+        <v>216973.775390625</v>
+      </c>
+      <c r="H63" t="n">
+        <v>34.67524789256486</v>
+      </c>
+      <c r="I63" t="inlineStr">
+        <is>
+          <t>2026-03-21T04:57:12</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>2026-03-21</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>클리블랜드 클리프스</t>
+        </is>
+      </c>
+      <c r="C64" t="n">
+        <v>70</v>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E64" t="n">
+        <v>1</v>
+      </c>
+      <c r="F64" t="n">
+        <v>823743.9360268187</v>
+      </c>
+      <c r="G64" t="n">
+        <v>-192311.0639731813</v>
+      </c>
+      <c r="H64" t="n">
+        <v>-18.92722972409774</v>
+      </c>
+      <c r="I64" t="inlineStr">
+        <is>
+          <t>2026-03-21T04:57:12</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>2026-03-21</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>낫 오프쇼어 파트너스</t>
+        </is>
+      </c>
+      <c r="C65" t="n">
+        <v>30</v>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E65" t="n">
+        <v>1</v>
+      </c>
+      <c r="F65" t="n">
+        <v>413075.8057155996</v>
+      </c>
+      <c r="G65" t="n">
+        <v>-4439.194284400437</v>
+      </c>
+      <c r="H65" t="n">
+        <v>-1.063241867813237</v>
+      </c>
+      <c r="I65" t="inlineStr">
+        <is>
+          <t>2026-03-21T04:57:12</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>2026-03-21</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
           <t>NH투자증권우</t>
         </is>
       </c>
-      <c r="C52" t="n">
+      <c r="C66" t="n">
         <v>2</v>
       </c>
-      <c r="D52" t="inlineStr">
-        <is>
-          <t>KRW</t>
-        </is>
-      </c>
-      <c r="E52" t="n">
-        <v>1</v>
-      </c>
-      <c r="F52" t="n">
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E66" t="n">
+        <v>1</v>
+      </c>
+      <c r="F66" t="n">
         <v>54700</v>
       </c>
-      <c r="G52" t="n">
+      <c r="G66" t="n">
         <v>100</v>
       </c>
-      <c r="H52" t="n">
+      <c r="H66" t="n">
         <v>0.1831501831501831</v>
       </c>
-      <c r="I52" t="inlineStr">
+      <c r="I66" t="inlineStr">
         <is>
           <t>2026-03-21T04:57:12</t>
         </is>
@@ -2808,7 +3704,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>2026-03-21T04:59:43</t>
+          <t>2026-03-21T05:00:11</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: portfolio snapshot 2026-03-17 (2026-03-21T05:00:13)
</commit_message>
<xml_diff>
--- a/portfolio_auto.xlsx
+++ b/portfolio_auto.xlsx
@@ -1171,7 +1171,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2026-03-21T05:00:11</t>
+          <t>2026-03-21T05:00:12</t>
         </is>
       </c>
       <c r="E2" t="n">
@@ -1272,7 +1272,7 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>2026-03-21T05:00:11</t>
+          <t>2026-03-21T05:00:12</t>
         </is>
       </c>
     </row>
@@ -1309,7 +1309,7 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>2026-03-21T05:00:11</t>
+          <t>2026-03-21T05:00:12</t>
         </is>
       </c>
     </row>
@@ -1346,7 +1346,7 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>2026-03-21T05:00:11</t>
+          <t>2026-03-21T05:00:12</t>
         </is>
       </c>
     </row>
@@ -1383,7 +1383,7 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>2026-03-21T05:00:11</t>
+          <t>2026-03-21T05:00:12</t>
         </is>
       </c>
     </row>
@@ -1420,7 +1420,7 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>2026-03-21T05:00:11</t>
+          <t>2026-03-21T05:00:12</t>
         </is>
       </c>
     </row>
@@ -1457,7 +1457,7 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>2026-03-21T05:00:11</t>
+          <t>2026-03-21T05:00:12</t>
         </is>
       </c>
     </row>
@@ -1494,7 +1494,7 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>2026-03-21T05:00:11</t>
+          <t>2026-03-21T05:00:12</t>
         </is>
       </c>
     </row>
@@ -1531,7 +1531,7 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>2026-03-21T05:00:11</t>
+          <t>2026-03-21T05:00:12</t>
         </is>
       </c>
     </row>
@@ -1568,7 +1568,7 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>2026-03-21T05:00:11</t>
+          <t>2026-03-21T05:00:12</t>
         </is>
       </c>
     </row>
@@ -1605,7 +1605,7 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>2026-03-21T05:00:11</t>
+          <t>2026-03-21T05:00:12</t>
         </is>
       </c>
     </row>
@@ -1642,7 +1642,7 @@
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>2026-03-21T05:00:11</t>
+          <t>2026-03-21T05:00:12</t>
         </is>
       </c>
     </row>
@@ -1679,7 +1679,7 @@
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>2026-03-21T05:00:11</t>
+          <t>2026-03-21T05:00:12</t>
         </is>
       </c>
     </row>
@@ -1716,7 +1716,7 @@
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>2026-03-21T05:00:11</t>
+          <t>2026-03-21T05:00:12</t>
         </is>
       </c>
     </row>
@@ -1753,7 +1753,7 @@
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>2026-03-21T05:00:11</t>
+          <t>2026-03-21T05:00:12</t>
         </is>
       </c>
     </row>
@@ -1790,7 +1790,7 @@
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>2026-03-21T05:00:11</t>
+          <t>2026-03-21T05:00:12</t>
         </is>
       </c>
     </row>
@@ -1827,7 +1827,7 @@
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>2026-03-21T05:00:11</t>
+          <t>2026-03-21T05:00:12</t>
         </is>
       </c>
     </row>
@@ -1864,7 +1864,7 @@
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>2026-03-21T05:00:11</t>
+          <t>2026-03-21T05:00:12</t>
         </is>
       </c>
     </row>
@@ -1901,7 +1901,7 @@
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>2026-03-21T05:00:11</t>
+          <t>2026-03-21T05:00:12</t>
         </is>
       </c>
     </row>
@@ -1938,7 +1938,7 @@
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>2026-03-21T05:00:11</t>
+          <t>2026-03-21T05:00:12</t>
         </is>
       </c>
     </row>
@@ -1975,7 +1975,7 @@
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>2026-03-21T05:00:11</t>
+          <t>2026-03-21T05:00:12</t>
         </is>
       </c>
     </row>
@@ -2012,7 +2012,7 @@
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>2026-03-21T05:00:11</t>
+          <t>2026-03-21T05:00:12</t>
         </is>
       </c>
     </row>
@@ -2049,7 +2049,7 @@
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>2026-03-21T05:00:11</t>
+          <t>2026-03-21T05:00:12</t>
         </is>
       </c>
     </row>
@@ -2086,7 +2086,7 @@
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>2026-03-21T05:00:11</t>
+          <t>2026-03-21T05:00:12</t>
         </is>
       </c>
     </row>
@@ -2123,7 +2123,7 @@
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>2026-03-21T05:00:11</t>
+          <t>2026-03-21T05:00:12</t>
         </is>
       </c>
     </row>
@@ -3704,7 +3704,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>2026-03-21T05:00:11</t>
+          <t>2026-03-21T05:00:12</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: portfolio snapshot 2026-03-17 (2026-03-21T05:00:47)
</commit_message>
<xml_diff>
--- a/portfolio_auto.xlsx
+++ b/portfolio_auto.xlsx
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G25"/>
+  <dimension ref="A1:G39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1114,6 +1114,384 @@
       </c>
       <c r="G25" t="n">
         <v>11.16446578631453</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>노브</t>
+        </is>
+      </c>
+      <c r="B26" t="n">
+        <v>185</v>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="D26" t="n">
+        <v>1</v>
+      </c>
+      <c r="E26" t="n">
+        <v>5200391.447092756</v>
+      </c>
+      <c r="F26" t="n">
+        <v>1890383.447092756</v>
+      </c>
+      <c r="G26" t="n">
+        <v>57.11114435653194</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>노블</t>
+        </is>
+      </c>
+      <c r="B27" t="n">
+        <v>99</v>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="D27" t="n">
+        <v>1</v>
+      </c>
+      <c r="E27" t="n">
+        <v>6958769.981090547</v>
+      </c>
+      <c r="F27" t="n">
+        <v>3051561.981090547</v>
+      </c>
+      <c r="G27" t="n">
+        <v>78.10083264291399</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>더치 브로스</t>
+        </is>
+      </c>
+      <c r="B28" t="n">
+        <v>39</v>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="D28" t="n">
+        <v>1</v>
+      </c>
+      <c r="E28" t="n">
+        <v>2934418.414306641</v>
+      </c>
+      <c r="F28" t="n">
+        <v>-256225.5856933594</v>
+      </c>
+      <c r="G28" t="n">
+        <v>-8.030528811530193</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>발레로 에너지</t>
+        </is>
+      </c>
+      <c r="B29" t="n">
+        <v>6</v>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="D29" t="n">
+        <v>1</v>
+      </c>
+      <c r="E29" t="n">
+        <v>2165691.085066516</v>
+      </c>
+      <c r="F29" t="n">
+        <v>101701.085066516</v>
+      </c>
+      <c r="G29" t="n">
+        <v>4.927402025519307</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>센트러스 에너지</t>
+        </is>
+      </c>
+      <c r="B30" t="n">
+        <v>21</v>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="D30" t="n">
+        <v>1</v>
+      </c>
+      <c r="E30" t="n">
+        <v>5901882.720856408</v>
+      </c>
+      <c r="F30" t="n">
+        <v>-329336.2791435914</v>
+      </c>
+      <c r="G30" t="n">
+        <v>-5.285262468605123</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>스타 벌크 캐리어스</t>
+        </is>
+      </c>
+      <c r="B31" t="n">
+        <v>50</v>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="D31" t="n">
+        <v>1</v>
+      </c>
+      <c r="E31" t="n">
+        <v>1680142.640194588</v>
+      </c>
+      <c r="F31" t="n">
+        <v>365789.6401945879</v>
+      </c>
+      <c r="G31" t="n">
+        <v>27.83039565433242</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>시드릴</t>
+        </is>
+      </c>
+      <c r="B32" t="n">
+        <v>123</v>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="D32" t="n">
+        <v>1</v>
+      </c>
+      <c r="E32" t="n">
+        <v>8070101.805898919</v>
+      </c>
+      <c r="F32" t="n">
+        <v>1619750.805898919</v>
+      </c>
+      <c r="G32" t="n">
+        <v>25.11104908707943</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>오케아니스 에코 탱커스</t>
+        </is>
+      </c>
+      <c r="B33" t="n">
+        <v>65</v>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="D33" t="n">
+        <v>1</v>
+      </c>
+      <c r="E33" t="n">
+        <v>4511179.137784176</v>
+      </c>
+      <c r="F33" t="n">
+        <v>2254819.137784176</v>
+      </c>
+      <c r="G33" t="n">
+        <v>99.93171026716374</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>유나이티드헬스 그룹</t>
+        </is>
+      </c>
+      <c r="B34" t="n">
+        <v>4</v>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="D34" t="n">
+        <v>1</v>
+      </c>
+      <c r="E34" t="n">
+        <v>1658864.328313038</v>
+      </c>
+      <c r="F34" t="n">
+        <v>-35591.67168696225</v>
+      </c>
+      <c r="G34" t="n">
+        <v>-2.100477774988684</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>차코스 에너지 내비게이션</t>
+        </is>
+      </c>
+      <c r="B35" t="n">
+        <v>75</v>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="D35" t="n">
+        <v>1</v>
+      </c>
+      <c r="E35" t="n">
+        <v>4026924.996845168</v>
+      </c>
+      <c r="F35" t="n">
+        <v>202276.9968451681</v>
+      </c>
+      <c r="G35" t="n">
+        <v>5.28877420471552</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>클리블랜드 클리프스</t>
+        </is>
+      </c>
+      <c r="B36" t="n">
+        <v>70</v>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="D36" t="n">
+        <v>1</v>
+      </c>
+      <c r="E36" t="n">
+        <v>823743.9360268187</v>
+      </c>
+      <c r="F36" t="n">
+        <v>-192311.0639731813</v>
+      </c>
+      <c r="G36" t="n">
+        <v>-18.92722972409774</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>타이드워터</t>
+        </is>
+      </c>
+      <c r="B37" t="n">
+        <v>48</v>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="D37" t="n">
+        <v>1</v>
+      </c>
+      <c r="E37" t="n">
+        <v>5235363.852789983</v>
+      </c>
+      <c r="F37" t="n">
+        <v>1510818.852789983</v>
+      </c>
+      <c r="G37" t="n">
+        <v>40.56385015592463</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>텍사스 퍼시픽 랜드</t>
+        </is>
+      </c>
+      <c r="B38" t="n">
+        <v>1</v>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="D38" t="n">
+        <v>1</v>
+      </c>
+      <c r="E38" t="n">
+        <v>781623.6870614514</v>
+      </c>
+      <c r="F38" t="n">
+        <v>3032.687061451375</v>
+      </c>
+      <c r="G38" t="n">
+        <v>0.3895096477420591</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>트랜스오션</t>
+        </is>
+      </c>
+      <c r="B39" t="n">
+        <v>750</v>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="D39" t="n">
+        <v>1</v>
+      </c>
+      <c r="E39" t="n">
+        <v>7020031.5082007</v>
+      </c>
+      <c r="F39" t="n">
+        <v>2892797.5082007</v>
+      </c>
+      <c r="G39" t="n">
+        <v>70.09046514446965</v>
       </c>
     </row>
   </sheetData>
@@ -1171,7 +1549,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2026-03-21T05:00:12</t>
+          <t>2026-03-21T05:00:47</t>
         </is>
       </c>
       <c r="E2" t="n">
@@ -1189,7 +1567,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I66"/>
+  <dimension ref="A1:I80"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1272,7 +1650,7 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>2026-03-21T05:00:12</t>
+          <t>2026-03-21T05:00:47</t>
         </is>
       </c>
     </row>
@@ -1309,7 +1687,7 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>2026-03-21T05:00:12</t>
+          <t>2026-03-21T05:00:47</t>
         </is>
       </c>
     </row>
@@ -1346,7 +1724,7 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>2026-03-21T05:00:12</t>
+          <t>2026-03-21T05:00:47</t>
         </is>
       </c>
     </row>
@@ -1383,7 +1761,7 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>2026-03-21T05:00:12</t>
+          <t>2026-03-21T05:00:47</t>
         </is>
       </c>
     </row>
@@ -1395,11 +1773,11 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>세아제강</t>
+          <t>시드릴</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>50</v>
+        <v>123</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
@@ -1410,17 +1788,17 @@
         <v>1</v>
       </c>
       <c r="F6" t="n">
-        <v>7395000</v>
+        <v>8070101.805898919</v>
       </c>
       <c r="G6" t="n">
-        <v>1085000</v>
+        <v>1619750.805898919</v>
       </c>
       <c r="H6" t="n">
-        <v>17.19492868462758</v>
+        <v>25.11104908707943</v>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>2026-03-21T05:00:12</t>
+          <t>2026-03-21T05:00:47</t>
         </is>
       </c>
     </row>
@@ -1432,11 +1810,11 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>DL이앤씨</t>
+          <t>세아제강</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>80</v>
+        <v>50</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
@@ -1447,17 +1825,17 @@
         <v>1</v>
       </c>
       <c r="F7" t="n">
-        <v>5392000</v>
+        <v>7395000</v>
       </c>
       <c r="G7" t="n">
-        <v>1981000</v>
+        <v>1085000</v>
       </c>
       <c r="H7" t="n">
-        <v>58.07681031955438</v>
+        <v>17.19492868462758</v>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>2026-03-21T05:00:12</t>
+          <t>2026-03-21T05:00:47</t>
         </is>
       </c>
     </row>
@@ -1469,11 +1847,11 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>TIME 코리아밸류업액티브</t>
+          <t>트랜스오션</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>201</v>
+        <v>750</v>
       </c>
       <c r="D8" t="inlineStr">
         <is>
@@ -1484,17 +1862,17 @@
         <v>1</v>
       </c>
       <c r="F8" t="n">
-        <v>4797870</v>
+        <v>7020031.5082007</v>
       </c>
       <c r="G8" t="n">
-        <v>74073</v>
+        <v>2892797.5082007</v>
       </c>
       <c r="H8" t="n">
-        <v>1.568081778281328</v>
+        <v>70.09046514446965</v>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>2026-03-21T05:00:12</t>
+          <t>2026-03-21T05:00:47</t>
         </is>
       </c>
     </row>
@@ -1506,11 +1884,11 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>동원개발</t>
+          <t>노블</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>1360</v>
+        <v>99</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
@@ -1521,17 +1899,17 @@
         <v>1</v>
       </c>
       <c r="F9" t="n">
-        <v>4202400</v>
+        <v>6958769.981090547</v>
       </c>
       <c r="G9" t="n">
-        <v>465000</v>
+        <v>3051561.981090547</v>
       </c>
       <c r="H9" t="n">
-        <v>12.44180446299566</v>
+        <v>78.10083264291399</v>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>2026-03-21T05:00:12</t>
+          <t>2026-03-21T05:00:47</t>
         </is>
       </c>
     </row>
@@ -1543,11 +1921,11 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>HD건설기계</t>
+          <t>센트러스 에너지</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>31</v>
+        <v>21</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
@@ -1558,17 +1936,17 @@
         <v>1</v>
       </c>
       <c r="F10" t="n">
-        <v>4123000</v>
+        <v>5901882.720856408</v>
       </c>
       <c r="G10" t="n">
-        <v>87904</v>
+        <v>-329336.2791435914</v>
       </c>
       <c r="H10" t="n">
-        <v>2.178485964150543</v>
+        <v>-5.285262468605123</v>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>2026-03-21T05:00:12</t>
+          <t>2026-03-21T05:00:47</t>
         </is>
       </c>
     </row>
@@ -1580,11 +1958,11 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>피바디 에너지</t>
+          <t>DL이앤씨</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>65</v>
+        <v>80</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
@@ -1595,17 +1973,17 @@
         <v>1</v>
       </c>
       <c r="F11" t="n">
-        <v>3649438.50225304</v>
+        <v>5392000</v>
       </c>
       <c r="G11" t="n">
-        <v>2178666.50225304</v>
+        <v>1981000</v>
       </c>
       <c r="H11" t="n">
-        <v>148.1308117269733</v>
+        <v>58.07681031955438</v>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>2026-03-21T05:00:12</t>
+          <t>2026-03-21T05:00:47</t>
         </is>
       </c>
     </row>
@@ -1617,11 +1995,11 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>삼성화재</t>
+          <t>타이드워터</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>7</v>
+        <v>48</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
@@ -1632,17 +2010,17 @@
         <v>1</v>
       </c>
       <c r="F12" t="n">
-        <v>3321500</v>
+        <v>5235363.852789983</v>
       </c>
       <c r="G12" t="n">
-        <v>-309500</v>
+        <v>1510818.852789983</v>
       </c>
       <c r="H12" t="n">
-        <v>-8.523822638391627</v>
+        <v>40.56385015592463</v>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>2026-03-21T05:00:12</t>
+          <t>2026-03-21T05:00:47</t>
         </is>
       </c>
     </row>
@@ -1654,11 +2032,11 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>휴스틸</t>
+          <t>노브</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>500</v>
+        <v>185</v>
       </c>
       <c r="D13" t="inlineStr">
         <is>
@@ -1669,17 +2047,17 @@
         <v>1</v>
       </c>
       <c r="F13" t="n">
-        <v>2750000</v>
+        <v>5200391.447092756</v>
       </c>
       <c r="G13" t="n">
-        <v>471390</v>
+        <v>1890383.447092756</v>
       </c>
       <c r="H13" t="n">
-        <v>20.68761218462133</v>
+        <v>57.11114435653194</v>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>2026-03-21T05:00:12</t>
+          <t>2026-03-21T05:00:47</t>
         </is>
       </c>
     </row>
@@ -1691,11 +2069,11 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>현대제철</t>
+          <t>TIME 코리아밸류업액티브</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>70</v>
+        <v>201</v>
       </c>
       <c r="D14" t="inlineStr">
         <is>
@@ -1706,17 +2084,17 @@
         <v>1</v>
       </c>
       <c r="F14" t="n">
-        <v>2621500</v>
+        <v>4797870</v>
       </c>
       <c r="G14" t="n">
-        <v>-186000</v>
+        <v>74073</v>
       </c>
       <c r="H14" t="n">
-        <v>-6.625111308993767</v>
+        <v>1.568081778281328</v>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>2026-03-21T05:00:12</t>
+          <t>2026-03-21T05:00:47</t>
         </is>
       </c>
     </row>
@@ -1728,11 +2106,11 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>KoAct 코스닥액티브</t>
+          <t>오케아니스 에코 탱커스</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>200</v>
+        <v>65</v>
       </c>
       <c r="D15" t="inlineStr">
         <is>
@@ -1743,17 +2121,17 @@
         <v>1</v>
       </c>
       <c r="F15" t="n">
-        <v>2582000</v>
+        <v>4511179.137784176</v>
       </c>
       <c r="G15" t="n">
-        <v>-120000</v>
+        <v>2254819.137784176</v>
       </c>
       <c r="H15" t="n">
-        <v>-4.441154700222058</v>
+        <v>99.93171026716374</v>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>2026-03-21T05:00:12</t>
+          <t>2026-03-21T05:00:47</t>
         </is>
       </c>
     </row>
@@ -1765,11 +2143,11 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>넥스틸</t>
+          <t>동원개발</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>200</v>
+        <v>1360</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
@@ -1780,17 +2158,17 @@
         <v>1</v>
       </c>
       <c r="F16" t="n">
-        <v>2514000</v>
+        <v>4202400</v>
       </c>
       <c r="G16" t="n">
-        <v>503000</v>
+        <v>465000</v>
       </c>
       <c r="H16" t="n">
-        <v>25.01243162605669</v>
+        <v>12.44180446299566</v>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>2026-03-21T05:00:12</t>
+          <t>2026-03-21T05:00:47</t>
         </is>
       </c>
     </row>
@@ -1802,11 +2180,11 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>대신증권</t>
+          <t>HD건설기계</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>55</v>
+        <v>31</v>
       </c>
       <c r="D17" t="inlineStr">
         <is>
@@ -1817,17 +2195,17 @@
         <v>1</v>
       </c>
       <c r="F17" t="n">
-        <v>2219250</v>
+        <v>4123000</v>
       </c>
       <c r="G17" t="n">
-        <v>509749</v>
+        <v>87904</v>
       </c>
       <c r="H17" t="n">
-        <v>29.81858448752005</v>
+        <v>2.178485964150543</v>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>2026-03-21T05:00:12</t>
+          <t>2026-03-21T05:00:47</t>
         </is>
       </c>
     </row>
@@ -1839,11 +2217,11 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>미창석유</t>
+          <t>차코스 에너지 내비게이션</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>18</v>
+        <v>75</v>
       </c>
       <c r="D18" t="inlineStr">
         <is>
@@ -1854,17 +2232,17 @@
         <v>1</v>
       </c>
       <c r="F18" t="n">
-        <v>2097000</v>
+        <v>4026924.996845168</v>
       </c>
       <c r="G18" t="n">
-        <v>-295200</v>
+        <v>202276.9968451681</v>
       </c>
       <c r="H18" t="n">
-        <v>-12.34010534236268</v>
+        <v>5.28877420471552</v>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>2026-03-21T05:00:12</t>
+          <t>2026-03-21T05:00:47</t>
         </is>
       </c>
     </row>
@@ -1876,11 +2254,11 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>대창단조</t>
+          <t>피바디 에너지</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>300</v>
+        <v>65</v>
       </c>
       <c r="D19" t="inlineStr">
         <is>
@@ -1891,17 +2269,17 @@
         <v>1</v>
       </c>
       <c r="F19" t="n">
-        <v>2004000</v>
+        <v>3649438.50225304</v>
       </c>
       <c r="G19" t="n">
-        <v>-54000</v>
+        <v>2178666.50225304</v>
       </c>
       <c r="H19" t="n">
-        <v>-2.623906705539359</v>
+        <v>148.1308117269733</v>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>2026-03-21T05:00:12</t>
+          <t>2026-03-21T05:00:47</t>
         </is>
       </c>
     </row>
@@ -1913,11 +2291,11 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>동방</t>
+          <t>삼성화재</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>681</v>
+        <v>7</v>
       </c>
       <c r="D20" t="inlineStr">
         <is>
@@ -1928,17 +2306,17 @@
         <v>1</v>
       </c>
       <c r="F20" t="n">
-        <v>1995330</v>
+        <v>3321500</v>
       </c>
       <c r="G20" t="n">
-        <v>23829</v>
+        <v>-309500</v>
       </c>
       <c r="H20" t="n">
-        <v>1.208672985709873</v>
+        <v>-8.523822638391627</v>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>2026-03-21T05:00:12</t>
+          <t>2026-03-21T05:00:47</t>
         </is>
       </c>
     </row>
@@ -1950,11 +2328,11 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>케이씨</t>
+          <t>더치 브로스</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>50</v>
+        <v>39</v>
       </c>
       <c r="D21" t="inlineStr">
         <is>
@@ -1965,17 +2343,17 @@
         <v>1</v>
       </c>
       <c r="F21" t="n">
-        <v>1670000</v>
+        <v>2934418.414306641</v>
       </c>
       <c r="G21" t="n">
-        <v>20500</v>
+        <v>-256225.5856933594</v>
       </c>
       <c r="H21" t="n">
-        <v>1.242800848742043</v>
+        <v>-8.030528811530193</v>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>2026-03-21T05:00:12</t>
+          <t>2026-03-21T05:00:47</t>
         </is>
       </c>
     </row>
@@ -1987,11 +2365,11 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>하나금융지주</t>
+          <t>휴스틸</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>10</v>
+        <v>500</v>
       </c>
       <c r="D22" t="inlineStr">
         <is>
@@ -2002,17 +2380,17 @@
         <v>1</v>
       </c>
       <c r="F22" t="n">
-        <v>1132000</v>
+        <v>2750000</v>
       </c>
       <c r="G22" t="n">
-        <v>23000</v>
+        <v>471390</v>
       </c>
       <c r="H22" t="n">
-        <v>2.073940486925157</v>
+        <v>20.68761218462133</v>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>2026-03-21T05:00:12</t>
+          <t>2026-03-21T05:00:47</t>
         </is>
       </c>
     </row>
@@ -2024,11 +2402,11 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>삼성생명</t>
+          <t>현대제철</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>4</v>
+        <v>70</v>
       </c>
       <c r="D23" t="inlineStr">
         <is>
@@ -2039,17 +2417,17 @@
         <v>1</v>
       </c>
       <c r="F23" t="n">
-        <v>926000</v>
+        <v>2621500</v>
       </c>
       <c r="G23" t="n">
-        <v>93000</v>
+        <v>-186000</v>
       </c>
       <c r="H23" t="n">
-        <v>11.16446578631453</v>
+        <v>-6.625111308993767</v>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>2026-03-21T05:00:12</t>
+          <t>2026-03-21T05:00:47</t>
         </is>
       </c>
     </row>
@@ -2061,11 +2439,11 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>비에이치아이</t>
+          <t>KoAct 코스닥액티브</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>8</v>
+        <v>200</v>
       </c>
       <c r="D24" t="inlineStr">
         <is>
@@ -2076,17 +2454,17 @@
         <v>1</v>
       </c>
       <c r="F24" t="n">
-        <v>876000</v>
+        <v>2582000</v>
       </c>
       <c r="G24" t="n">
-        <v>210885</v>
+        <v>-120000</v>
       </c>
       <c r="H24" t="n">
-        <v>31.70654698811484</v>
+        <v>-4.441154700222058</v>
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>2026-03-21T05:00:12</t>
+          <t>2026-03-21T05:00:47</t>
         </is>
       </c>
     </row>
@@ -2098,11 +2476,11 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>하프니아</t>
+          <t>넥스틸</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>80</v>
+        <v>200</v>
       </c>
       <c r="D25" t="inlineStr">
         <is>
@@ -2113,33 +2491,33 @@
         <v>1</v>
       </c>
       <c r="F25" t="n">
-        <v>842704.775390625</v>
+        <v>2514000</v>
       </c>
       <c r="G25" t="n">
-        <v>216973.775390625</v>
+        <v>503000</v>
       </c>
       <c r="H25" t="n">
-        <v>34.67524789256486</v>
+        <v>25.01243162605669</v>
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>2026-03-21T05:00:12</t>
+          <t>2026-03-21T05:00:47</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>2026-03-21</t>
+          <t>2026-03-17</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>페트로브라스 (ADR)</t>
+          <t>대신증권</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>480</v>
+        <v>55</v>
       </c>
       <c r="D26" t="inlineStr">
         <is>
@@ -2150,33 +2528,33 @@
         <v>1</v>
       </c>
       <c r="F26" t="n">
-        <v>13579584.97235231</v>
+        <v>2219250</v>
       </c>
       <c r="G26" t="n">
-        <v>1473035.972352311</v>
+        <v>509749</v>
       </c>
       <c r="H26" t="n">
-        <v>12.16726560436265</v>
+        <v>29.81858448752005</v>
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>2026-03-21T04:57:12</t>
+          <t>2026-03-21T05:00:47</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-03-21</t>
+          <t>2026-03-17</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>AGNC 인베스트먼트</t>
+          <t>발레로 에너지</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>700</v>
+        <v>6</v>
       </c>
       <c r="D27" t="inlineStr">
         <is>
@@ -2187,33 +2565,33 @@
         <v>1</v>
       </c>
       <c r="F27" t="n">
-        <v>10270464.45007324</v>
+        <v>2165691.085066516</v>
       </c>
       <c r="G27" t="n">
-        <v>-561550.5499267559</v>
+        <v>101701.085066516</v>
       </c>
       <c r="H27" t="n">
-        <v>-5.184174411933109</v>
+        <v>4.927402025519307</v>
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>2026-03-21T04:57:12</t>
+          <t>2026-03-21T05:00:47</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>2026-03-21</t>
+          <t>2026-03-17</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>대한조선</t>
+          <t>미창석유</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>100</v>
+        <v>18</v>
       </c>
       <c r="D28" t="inlineStr">
         <is>
@@ -2224,33 +2602,33 @@
         <v>1</v>
       </c>
       <c r="F28" t="n">
-        <v>9120000</v>
+        <v>2097000</v>
       </c>
       <c r="G28" t="n">
-        <v>1907000</v>
+        <v>-295200</v>
       </c>
       <c r="H28" t="n">
-        <v>26.43837515596839</v>
+        <v>-12.34010534236268</v>
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>2026-03-21T04:57:12</t>
+          <t>2026-03-21T05:00:47</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-03-21</t>
+          <t>2026-03-17</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>프론트라인</t>
+          <t>대창단조</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>175</v>
+        <v>300</v>
       </c>
       <c r="D29" t="inlineStr">
         <is>
@@ -2261,33 +2639,33 @@
         <v>1</v>
       </c>
       <c r="F29" t="n">
-        <v>8471815.962899337</v>
+        <v>2004000</v>
       </c>
       <c r="G29" t="n">
-        <v>4041951.962899337</v>
+        <v>-54000</v>
       </c>
       <c r="H29" t="n">
-        <v>91.24325177701475</v>
+        <v>-2.623906705539359</v>
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>2026-03-21T04:57:12</t>
+          <t>2026-03-21T05:00:47</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>2026-03-21</t>
+          <t>2026-03-17</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>시드릴</t>
+          <t>동방</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>123</v>
+        <v>681</v>
       </c>
       <c r="D30" t="inlineStr">
         <is>
@@ -2298,29 +2676,29 @@
         <v>1</v>
       </c>
       <c r="F30" t="n">
-        <v>8070101.805898919</v>
+        <v>1995330</v>
       </c>
       <c r="G30" t="n">
-        <v>1619750.805898919</v>
+        <v>23829</v>
       </c>
       <c r="H30" t="n">
-        <v>25.11104908707943</v>
+        <v>1.208672985709873</v>
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>2026-03-21T04:57:12</t>
+          <t>2026-03-21T05:00:47</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-03-21</t>
+          <t>2026-03-17</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>세아제강</t>
+          <t>스타 벌크 캐리어스</t>
         </is>
       </c>
       <c r="C31" t="n">
@@ -2335,33 +2713,33 @@
         <v>1</v>
       </c>
       <c r="F31" t="n">
-        <v>7395000</v>
+        <v>1680142.640194588</v>
       </c>
       <c r="G31" t="n">
-        <v>1085000</v>
+        <v>365789.6401945879</v>
       </c>
       <c r="H31" t="n">
-        <v>17.19492868462758</v>
+        <v>27.83039565433242</v>
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>2026-03-21T04:57:12</t>
+          <t>2026-03-21T05:00:47</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>2026-03-21</t>
+          <t>2026-03-17</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>센트러스 에너지</t>
+          <t>케이씨</t>
         </is>
       </c>
       <c r="C32" t="n">
-        <v>25</v>
+        <v>50</v>
       </c>
       <c r="D32" t="inlineStr">
         <is>
@@ -2372,33 +2750,33 @@
         <v>1</v>
       </c>
       <c r="F32" t="n">
-        <v>7026050.85816239</v>
+        <v>1670000</v>
       </c>
       <c r="G32" t="n">
-        <v>-406805.1418376099</v>
+        <v>20500</v>
       </c>
       <c r="H32" t="n">
-        <v>-5.473066366920198</v>
+        <v>1.242800848742043</v>
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>2026-03-21T04:57:12</t>
+          <t>2026-03-21T05:00:47</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-03-21</t>
+          <t>2026-03-17</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>트랜스오션</t>
+          <t>유나이티드헬스 그룹</t>
         </is>
       </c>
       <c r="C33" t="n">
-        <v>750</v>
+        <v>4</v>
       </c>
       <c r="D33" t="inlineStr">
         <is>
@@ -2409,33 +2787,33 @@
         <v>1</v>
       </c>
       <c r="F33" t="n">
-        <v>7020031.5082007</v>
+        <v>1658864.328313038</v>
       </c>
       <c r="G33" t="n">
-        <v>2892797.5082007</v>
+        <v>-35591.67168696225</v>
       </c>
       <c r="H33" t="n">
-        <v>70.09046514446965</v>
+        <v>-2.100477774988684</v>
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>2026-03-21T04:57:12</t>
+          <t>2026-03-21T05:00:47</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>2026-03-21</t>
+          <t>2026-03-17</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>노블</t>
+          <t>하나금융지주</t>
         </is>
       </c>
       <c r="C34" t="n">
-        <v>99</v>
+        <v>10</v>
       </c>
       <c r="D34" t="inlineStr">
         <is>
@@ -2446,33 +2824,33 @@
         <v>1</v>
       </c>
       <c r="F34" t="n">
-        <v>6958769.981090547</v>
+        <v>1132000</v>
       </c>
       <c r="G34" t="n">
-        <v>3051561.981090547</v>
+        <v>23000</v>
       </c>
       <c r="H34" t="n">
-        <v>78.10083264291399</v>
+        <v>2.073940486925157</v>
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>2026-03-21T04:57:12</t>
+          <t>2026-03-21T05:00:47</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-03-21</t>
+          <t>2026-03-17</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>타이드워터</t>
+          <t>삼성생명</t>
         </is>
       </c>
       <c r="C35" t="n">
-        <v>48</v>
+        <v>4</v>
       </c>
       <c r="D35" t="inlineStr">
         <is>
@@ -2483,33 +2861,33 @@
         <v>1</v>
       </c>
       <c r="F35" t="n">
-        <v>5235363.852789983</v>
+        <v>926000</v>
       </c>
       <c r="G35" t="n">
-        <v>1510818.852789983</v>
+        <v>93000</v>
       </c>
       <c r="H35" t="n">
-        <v>40.56385015592463</v>
+        <v>11.16446578631453</v>
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>2026-03-21T04:57:12</t>
+          <t>2026-03-21T05:00:47</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>2026-03-21</t>
+          <t>2026-03-17</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>노브</t>
+          <t>비에이치아이</t>
         </is>
       </c>
       <c r="C36" t="n">
-        <v>185</v>
+        <v>8</v>
       </c>
       <c r="D36" t="inlineStr">
         <is>
@@ -2520,33 +2898,33 @@
         <v>1</v>
       </c>
       <c r="F36" t="n">
-        <v>5200391.447092756</v>
+        <v>876000</v>
       </c>
       <c r="G36" t="n">
-        <v>1890383.447092756</v>
+        <v>210885</v>
       </c>
       <c r="H36" t="n">
-        <v>57.11114435653194</v>
+        <v>31.70654698811484</v>
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>2026-03-21T04:57:12</t>
+          <t>2026-03-21T05:00:47</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2026-03-21</t>
+          <t>2026-03-17</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>TIME 코리아밸류업액티브</t>
+          <t>하프니아</t>
         </is>
       </c>
       <c r="C37" t="n">
-        <v>201</v>
+        <v>80</v>
       </c>
       <c r="D37" t="inlineStr">
         <is>
@@ -2557,33 +2935,33 @@
         <v>1</v>
       </c>
       <c r="F37" t="n">
-        <v>4797870</v>
+        <v>842704.775390625</v>
       </c>
       <c r="G37" t="n">
-        <v>74073</v>
+        <v>216973.775390625</v>
       </c>
       <c r="H37" t="n">
-        <v>1.568081778281328</v>
+        <v>34.67524789256486</v>
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>2026-03-21T04:57:12</t>
+          <t>2026-03-21T05:00:47</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>2026-03-21</t>
+          <t>2026-03-17</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>오케아니스 에코 탱커스</t>
+          <t>클리블랜드 클리프스</t>
         </is>
       </c>
       <c r="C38" t="n">
-        <v>65</v>
+        <v>70</v>
       </c>
       <c r="D38" t="inlineStr">
         <is>
@@ -2594,33 +2972,33 @@
         <v>1</v>
       </c>
       <c r="F38" t="n">
-        <v>4511179.137784176</v>
+        <v>823743.9360268187</v>
       </c>
       <c r="G38" t="n">
-        <v>2254819.137784176</v>
+        <v>-192311.0639731813</v>
       </c>
       <c r="H38" t="n">
-        <v>99.93171026716374</v>
+        <v>-18.92722972409774</v>
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>2026-03-21T04:57:12</t>
+          <t>2026-03-21T05:00:47</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2026-03-21</t>
+          <t>2026-03-17</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>삼성화재</t>
+          <t>텍사스 퍼시픽 랜드</t>
         </is>
       </c>
       <c r="C39" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="D39" t="inlineStr">
         <is>
@@ -2631,17 +3009,17 @@
         <v>1</v>
       </c>
       <c r="F39" t="n">
-        <v>4270500</v>
+        <v>781623.6870614514</v>
       </c>
       <c r="G39" t="n">
-        <v>-360500</v>
+        <v>3032.687061451375</v>
       </c>
       <c r="H39" t="n">
-        <v>-7.784495789246384</v>
+        <v>0.3895096477420591</v>
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>2026-03-21T04:57:12</t>
+          <t>2026-03-21T05:00:47</t>
         </is>
       </c>
     </row>
@@ -2653,11 +3031,11 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>동원개발</t>
+          <t>페트로브라스 (ADR)</t>
         </is>
       </c>
       <c r="C40" t="n">
-        <v>1360</v>
+        <v>480</v>
       </c>
       <c r="D40" t="inlineStr">
         <is>
@@ -2668,13 +3046,13 @@
         <v>1</v>
       </c>
       <c r="F40" t="n">
-        <v>4202400</v>
+        <v>13579584.97235231</v>
       </c>
       <c r="G40" t="n">
-        <v>465000</v>
+        <v>1473035.972352311</v>
       </c>
       <c r="H40" t="n">
-        <v>12.44180446299566</v>
+        <v>12.16726560436265</v>
       </c>
       <c r="I40" t="inlineStr">
         <is>
@@ -2690,11 +3068,11 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>HD건설기계</t>
+          <t>AGNC 인베스트먼트</t>
         </is>
       </c>
       <c r="C41" t="n">
-        <v>31</v>
+        <v>700</v>
       </c>
       <c r="D41" t="inlineStr">
         <is>
@@ -2705,13 +3083,13 @@
         <v>1</v>
       </c>
       <c r="F41" t="n">
-        <v>4123000</v>
+        <v>10270464.45007324</v>
       </c>
       <c r="G41" t="n">
-        <v>87904</v>
+        <v>-561550.5499267559</v>
       </c>
       <c r="H41" t="n">
-        <v>2.178485964150543</v>
+        <v>-5.184174411933109</v>
       </c>
       <c r="I41" t="inlineStr">
         <is>
@@ -2727,11 +3105,11 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>차코스 에너지 내비게이션</t>
+          <t>대한조선</t>
         </is>
       </c>
       <c r="C42" t="n">
-        <v>75</v>
+        <v>100</v>
       </c>
       <c r="D42" t="inlineStr">
         <is>
@@ -2742,13 +3120,13 @@
         <v>1</v>
       </c>
       <c r="F42" t="n">
-        <v>4026924.996845168</v>
+        <v>9120000</v>
       </c>
       <c r="G42" t="n">
-        <v>202276.9968451681</v>
+        <v>1907000</v>
       </c>
       <c r="H42" t="n">
-        <v>5.28877420471552</v>
+        <v>26.43837515596839</v>
       </c>
       <c r="I42" t="inlineStr">
         <is>
@@ -2764,11 +3142,11 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>넥스틸</t>
+          <t>프론트라인</t>
         </is>
       </c>
       <c r="C43" t="n">
-        <v>300</v>
+        <v>175</v>
       </c>
       <c r="D43" t="inlineStr">
         <is>
@@ -2779,13 +3157,13 @@
         <v>1</v>
       </c>
       <c r="F43" t="n">
-        <v>3771000</v>
+        <v>8471815.962899337</v>
       </c>
       <c r="G43" t="n">
-        <v>521000</v>
+        <v>4041951.962899337</v>
       </c>
       <c r="H43" t="n">
-        <v>16.03076923076923</v>
+        <v>91.24325177701475</v>
       </c>
       <c r="I43" t="inlineStr">
         <is>
@@ -2801,11 +3179,11 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>피바디 에너지</t>
+          <t>시드릴</t>
         </is>
       </c>
       <c r="C44" t="n">
-        <v>65</v>
+        <v>123</v>
       </c>
       <c r="D44" t="inlineStr">
         <is>
@@ -2816,13 +3194,13 @@
         <v>1</v>
       </c>
       <c r="F44" t="n">
-        <v>3649438.50225304</v>
+        <v>8070101.805898919</v>
       </c>
       <c r="G44" t="n">
-        <v>2178666.50225304</v>
+        <v>1619750.805898919</v>
       </c>
       <c r="H44" t="n">
-        <v>148.1308117269733</v>
+        <v>25.11104908707943</v>
       </c>
       <c r="I44" t="inlineStr">
         <is>
@@ -2838,11 +3216,11 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>현대제철</t>
+          <t>세아제강</t>
         </is>
       </c>
       <c r="C45" t="n">
-        <v>80</v>
+        <v>50</v>
       </c>
       <c r="D45" t="inlineStr">
         <is>
@@ -2853,13 +3231,13 @@
         <v>1</v>
       </c>
       <c r="F45" t="n">
-        <v>2996000</v>
+        <v>7395000</v>
       </c>
       <c r="G45" t="n">
-        <v>-182000</v>
+        <v>1085000</v>
       </c>
       <c r="H45" t="n">
-        <v>-5.726872246696035</v>
+        <v>17.19492868462758</v>
       </c>
       <c r="I45" t="inlineStr">
         <is>
@@ -2875,11 +3253,11 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>더치 브로스</t>
+          <t>센트러스 에너지</t>
         </is>
       </c>
       <c r="C46" t="n">
-        <v>39</v>
+        <v>25</v>
       </c>
       <c r="D46" t="inlineStr">
         <is>
@@ -2890,13 +3268,13 @@
         <v>1</v>
       </c>
       <c r="F46" t="n">
-        <v>2934418.414306641</v>
+        <v>7026050.85816239</v>
       </c>
       <c r="G46" t="n">
-        <v>-256226.5856933594</v>
+        <v>-406805.1418376099</v>
       </c>
       <c r="H46" t="n">
-        <v>-8.030557636257226</v>
+        <v>-5.473066366920198</v>
       </c>
       <c r="I46" t="inlineStr">
         <is>
@@ -2912,11 +3290,11 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>휴스틸</t>
+          <t>트랜스오션</t>
         </is>
       </c>
       <c r="C47" t="n">
-        <v>500</v>
+        <v>750</v>
       </c>
       <c r="D47" t="inlineStr">
         <is>
@@ -2927,13 +3305,13 @@
         <v>1</v>
       </c>
       <c r="F47" t="n">
-        <v>2750000</v>
+        <v>7020031.5082007</v>
       </c>
       <c r="G47" t="n">
-        <v>471390</v>
+        <v>2892797.5082007</v>
       </c>
       <c r="H47" t="n">
-        <v>20.68761218462133</v>
+        <v>70.09046514446965</v>
       </c>
       <c r="I47" t="inlineStr">
         <is>
@@ -2949,11 +3327,11 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>DL이앤씨</t>
+          <t>노블</t>
         </is>
       </c>
       <c r="C48" t="n">
-        <v>40</v>
+        <v>99</v>
       </c>
       <c r="D48" t="inlineStr">
         <is>
@@ -2964,13 +3342,13 @@
         <v>1</v>
       </c>
       <c r="F48" t="n">
-        <v>2696000</v>
+        <v>6958769.981090547</v>
       </c>
       <c r="G48" t="n">
-        <v>990500</v>
+        <v>3051561.981090547</v>
       </c>
       <c r="H48" t="n">
-        <v>58.07681031955438</v>
+        <v>78.10083264291399</v>
       </c>
       <c r="I48" t="inlineStr">
         <is>
@@ -2986,11 +3364,11 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>KoAct 코스닥액티브</t>
+          <t>타이드워터</t>
         </is>
       </c>
       <c r="C49" t="n">
-        <v>200</v>
+        <v>48</v>
       </c>
       <c r="D49" t="inlineStr">
         <is>
@@ -3001,13 +3379,13 @@
         <v>1</v>
       </c>
       <c r="F49" t="n">
-        <v>2582000</v>
+        <v>5235363.852789983</v>
       </c>
       <c r="G49" t="n">
-        <v>-120000</v>
+        <v>1510818.852789983</v>
       </c>
       <c r="H49" t="n">
-        <v>-4.441154700222058</v>
+        <v>40.56385015592463</v>
       </c>
       <c r="I49" t="inlineStr">
         <is>
@@ -3023,11 +3401,11 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>대신증권</t>
+          <t>노브</t>
         </is>
       </c>
       <c r="C50" t="n">
-        <v>55</v>
+        <v>185</v>
       </c>
       <c r="D50" t="inlineStr">
         <is>
@@ -3038,13 +3416,13 @@
         <v>1</v>
       </c>
       <c r="F50" t="n">
-        <v>2219250</v>
+        <v>5200391.447092756</v>
       </c>
       <c r="G50" t="n">
-        <v>509749</v>
+        <v>1890383.447092756</v>
       </c>
       <c r="H50" t="n">
-        <v>29.81858448752005</v>
+        <v>57.11114435653194</v>
       </c>
       <c r="I50" t="inlineStr">
         <is>
@@ -3060,11 +3438,11 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>발레로 에너지</t>
+          <t>TIME 코리아밸류업액티브</t>
         </is>
       </c>
       <c r="C51" t="n">
-        <v>6</v>
+        <v>201</v>
       </c>
       <c r="D51" t="inlineStr">
         <is>
@@ -3075,13 +3453,13 @@
         <v>1</v>
       </c>
       <c r="F51" t="n">
-        <v>2165691.085066516</v>
+        <v>4797870</v>
       </c>
       <c r="G51" t="n">
-        <v>101701.085066516</v>
+        <v>74073</v>
       </c>
       <c r="H51" t="n">
-        <v>4.927402025519307</v>
+        <v>1.568081778281328</v>
       </c>
       <c r="I51" t="inlineStr">
         <is>
@@ -3097,11 +3475,11 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>미창석유</t>
+          <t>오케아니스 에코 탱커스</t>
         </is>
       </c>
       <c r="C52" t="n">
-        <v>18</v>
+        <v>65</v>
       </c>
       <c r="D52" t="inlineStr">
         <is>
@@ -3112,13 +3490,13 @@
         <v>1</v>
       </c>
       <c r="F52" t="n">
-        <v>2097000</v>
+        <v>4511179.137784176</v>
       </c>
       <c r="G52" t="n">
-        <v>-295200</v>
+        <v>2254819.137784176</v>
       </c>
       <c r="H52" t="n">
-        <v>-12.34010534236268</v>
+        <v>99.93171026716374</v>
       </c>
       <c r="I52" t="inlineStr">
         <is>
@@ -3134,11 +3512,11 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>하나금융지주</t>
+          <t>삼성화재</t>
         </is>
       </c>
       <c r="C53" t="n">
-        <v>18</v>
+        <v>9</v>
       </c>
       <c r="D53" t="inlineStr">
         <is>
@@ -3149,13 +3527,13 @@
         <v>1</v>
       </c>
       <c r="F53" t="n">
-        <v>2037600</v>
+        <v>4270500</v>
       </c>
       <c r="G53" t="n">
-        <v>12200</v>
+        <v>-360500</v>
       </c>
       <c r="H53" t="n">
-        <v>0.6023501530561864</v>
+        <v>-7.784495789246384</v>
       </c>
       <c r="I53" t="inlineStr">
         <is>
@@ -3171,11 +3549,11 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>대창단조</t>
+          <t>동원개발</t>
         </is>
       </c>
       <c r="C54" t="n">
-        <v>300</v>
+        <v>1360</v>
       </c>
       <c r="D54" t="inlineStr">
         <is>
@@ -3186,13 +3564,13 @@
         <v>1</v>
       </c>
       <c r="F54" t="n">
-        <v>2004000</v>
+        <v>4202400</v>
       </c>
       <c r="G54" t="n">
-        <v>-54000</v>
+        <v>465000</v>
       </c>
       <c r="H54" t="n">
-        <v>-2.623906705539359</v>
+        <v>12.44180446299566</v>
       </c>
       <c r="I54" t="inlineStr">
         <is>
@@ -3208,11 +3586,11 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>동방</t>
+          <t>HD건설기계</t>
         </is>
       </c>
       <c r="C55" t="n">
-        <v>681</v>
+        <v>31</v>
       </c>
       <c r="D55" t="inlineStr">
         <is>
@@ -3223,13 +3601,13 @@
         <v>1</v>
       </c>
       <c r="F55" t="n">
-        <v>1995330</v>
+        <v>4123000</v>
       </c>
       <c r="G55" t="n">
-        <v>23829</v>
+        <v>87904</v>
       </c>
       <c r="H55" t="n">
-        <v>1.208672985709873</v>
+        <v>2.178485964150543</v>
       </c>
       <c r="I55" t="inlineStr">
         <is>
@@ -3245,11 +3623,11 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>스타 벌크 캐리어스</t>
+          <t>차코스 에너지 내비게이션</t>
         </is>
       </c>
       <c r="C56" t="n">
-        <v>50</v>
+        <v>75</v>
       </c>
       <c r="D56" t="inlineStr">
         <is>
@@ -3260,13 +3638,13 @@
         <v>1</v>
       </c>
       <c r="F56" t="n">
-        <v>1680142.640194588</v>
+        <v>4026924.996845168</v>
       </c>
       <c r="G56" t="n">
-        <v>365789.6401945879</v>
+        <v>202276.9968451681</v>
       </c>
       <c r="H56" t="n">
-        <v>27.83039565433242</v>
+        <v>5.28877420471552</v>
       </c>
       <c r="I56" t="inlineStr">
         <is>
@@ -3282,11 +3660,11 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>케이씨</t>
+          <t>넥스틸</t>
         </is>
       </c>
       <c r="C57" t="n">
-        <v>50</v>
+        <v>300</v>
       </c>
       <c r="D57" t="inlineStr">
         <is>
@@ -3297,13 +3675,13 @@
         <v>1</v>
       </c>
       <c r="F57" t="n">
-        <v>1670000</v>
+        <v>3771000</v>
       </c>
       <c r="G57" t="n">
-        <v>20500</v>
+        <v>521000</v>
       </c>
       <c r="H57" t="n">
-        <v>1.242800848742043</v>
+        <v>16.03076923076923</v>
       </c>
       <c r="I57" t="inlineStr">
         <is>
@@ -3319,11 +3697,11 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>유나이티드헬스 그룹</t>
+          <t>피바디 에너지</t>
         </is>
       </c>
       <c r="C58" t="n">
-        <v>4</v>
+        <v>65</v>
       </c>
       <c r="D58" t="inlineStr">
         <is>
@@ -3334,13 +3712,13 @@
         <v>1</v>
       </c>
       <c r="F58" t="n">
-        <v>1658864.328313038</v>
+        <v>3649438.50225304</v>
       </c>
       <c r="G58" t="n">
-        <v>-35591.67168696248</v>
+        <v>2178666.50225304</v>
       </c>
       <c r="H58" t="n">
-        <v>-2.100477774988697</v>
+        <v>148.1308117269733</v>
       </c>
       <c r="I58" t="inlineStr">
         <is>
@@ -3356,11 +3734,11 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>텍사스 퍼시픽 랜드</t>
+          <t>현대제철</t>
         </is>
       </c>
       <c r="C59" t="n">
-        <v>2</v>
+        <v>80</v>
       </c>
       <c r="D59" t="inlineStr">
         <is>
@@ -3371,13 +3749,13 @@
         <v>1</v>
       </c>
       <c r="F59" t="n">
-        <v>1563247.374122903</v>
+        <v>2996000</v>
       </c>
       <c r="G59" t="n">
-        <v>-14646.62587709725</v>
+        <v>-182000</v>
       </c>
       <c r="H59" t="n">
-        <v>-0.9282388979929735</v>
+        <v>-5.726872246696035</v>
       </c>
       <c r="I59" t="inlineStr">
         <is>
@@ -3393,11 +3771,11 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>LX인터내셔널</t>
+          <t>더치 브로스</t>
         </is>
       </c>
       <c r="C60" t="n">
-        <v>20</v>
+        <v>39</v>
       </c>
       <c r="D60" t="inlineStr">
         <is>
@@ -3408,13 +3786,13 @@
         <v>1</v>
       </c>
       <c r="F60" t="n">
-        <v>943000</v>
+        <v>2934418.414306641</v>
       </c>
       <c r="G60" t="n">
-        <v>4000</v>
+        <v>-256226.5856933594</v>
       </c>
       <c r="H60" t="n">
-        <v>0.4259850905218318</v>
+        <v>-8.030557636257226</v>
       </c>
       <c r="I60" t="inlineStr">
         <is>
@@ -3430,11 +3808,11 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>삼성생명</t>
+          <t>휴스틸</t>
         </is>
       </c>
       <c r="C61" t="n">
-        <v>4</v>
+        <v>500</v>
       </c>
       <c r="D61" t="inlineStr">
         <is>
@@ -3445,13 +3823,13 @@
         <v>1</v>
       </c>
       <c r="F61" t="n">
-        <v>926000</v>
+        <v>2750000</v>
       </c>
       <c r="G61" t="n">
-        <v>93000</v>
+        <v>471390</v>
       </c>
       <c r="H61" t="n">
-        <v>11.16446578631453</v>
+        <v>20.68761218462133</v>
       </c>
       <c r="I61" t="inlineStr">
         <is>
@@ -3467,11 +3845,11 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>비에이치아이</t>
+          <t>DL이앤씨</t>
         </is>
       </c>
       <c r="C62" t="n">
-        <v>8</v>
+        <v>40</v>
       </c>
       <c r="D62" t="inlineStr">
         <is>
@@ -3482,13 +3860,13 @@
         <v>1</v>
       </c>
       <c r="F62" t="n">
-        <v>876000</v>
+        <v>2696000</v>
       </c>
       <c r="G62" t="n">
-        <v>210885</v>
+        <v>990500</v>
       </c>
       <c r="H62" t="n">
-        <v>31.70654698811484</v>
+        <v>58.07681031955438</v>
       </c>
       <c r="I62" t="inlineStr">
         <is>
@@ -3504,11 +3882,11 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>하프니아</t>
+          <t>KoAct 코스닥액티브</t>
         </is>
       </c>
       <c r="C63" t="n">
-        <v>80</v>
+        <v>200</v>
       </c>
       <c r="D63" t="inlineStr">
         <is>
@@ -3519,13 +3897,13 @@
         <v>1</v>
       </c>
       <c r="F63" t="n">
-        <v>842704.775390625</v>
+        <v>2582000</v>
       </c>
       <c r="G63" t="n">
-        <v>216973.775390625</v>
+        <v>-120000</v>
       </c>
       <c r="H63" t="n">
-        <v>34.67524789256486</v>
+        <v>-4.441154700222058</v>
       </c>
       <c r="I63" t="inlineStr">
         <is>
@@ -3541,11 +3919,11 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>클리블랜드 클리프스</t>
+          <t>대신증권</t>
         </is>
       </c>
       <c r="C64" t="n">
-        <v>70</v>
+        <v>55</v>
       </c>
       <c r="D64" t="inlineStr">
         <is>
@@ -3556,13 +3934,13 @@
         <v>1</v>
       </c>
       <c r="F64" t="n">
-        <v>823743.9360268187</v>
+        <v>2219250</v>
       </c>
       <c r="G64" t="n">
-        <v>-192311.0639731813</v>
+        <v>509749</v>
       </c>
       <c r="H64" t="n">
-        <v>-18.92722972409774</v>
+        <v>29.81858448752005</v>
       </c>
       <c r="I64" t="inlineStr">
         <is>
@@ -3578,11 +3956,11 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>낫 오프쇼어 파트너스</t>
+          <t>발레로 에너지</t>
         </is>
       </c>
       <c r="C65" t="n">
-        <v>30</v>
+        <v>6</v>
       </c>
       <c r="D65" t="inlineStr">
         <is>
@@ -3593,13 +3971,13 @@
         <v>1</v>
       </c>
       <c r="F65" t="n">
-        <v>413075.8057155996</v>
+        <v>2165691.085066516</v>
       </c>
       <c r="G65" t="n">
-        <v>-4439.194284400437</v>
+        <v>101701.085066516</v>
       </c>
       <c r="H65" t="n">
-        <v>-1.063241867813237</v>
+        <v>4.927402025519307</v>
       </c>
       <c r="I65" t="inlineStr">
         <is>
@@ -3615,30 +3993,548 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
+          <t>미창석유</t>
+        </is>
+      </c>
+      <c r="C66" t="n">
+        <v>18</v>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E66" t="n">
+        <v>1</v>
+      </c>
+      <c r="F66" t="n">
+        <v>2097000</v>
+      </c>
+      <c r="G66" t="n">
+        <v>-295200</v>
+      </c>
+      <c r="H66" t="n">
+        <v>-12.34010534236268</v>
+      </c>
+      <c r="I66" t="inlineStr">
+        <is>
+          <t>2026-03-21T04:57:12</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>2026-03-21</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>하나금융지주</t>
+        </is>
+      </c>
+      <c r="C67" t="n">
+        <v>18</v>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E67" t="n">
+        <v>1</v>
+      </c>
+      <c r="F67" t="n">
+        <v>2037600</v>
+      </c>
+      <c r="G67" t="n">
+        <v>12200</v>
+      </c>
+      <c r="H67" t="n">
+        <v>0.6023501530561864</v>
+      </c>
+      <c r="I67" t="inlineStr">
+        <is>
+          <t>2026-03-21T04:57:12</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>2026-03-21</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>대창단조</t>
+        </is>
+      </c>
+      <c r="C68" t="n">
+        <v>300</v>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E68" t="n">
+        <v>1</v>
+      </c>
+      <c r="F68" t="n">
+        <v>2004000</v>
+      </c>
+      <c r="G68" t="n">
+        <v>-54000</v>
+      </c>
+      <c r="H68" t="n">
+        <v>-2.623906705539359</v>
+      </c>
+      <c r="I68" t="inlineStr">
+        <is>
+          <t>2026-03-21T04:57:12</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>2026-03-21</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>동방</t>
+        </is>
+      </c>
+      <c r="C69" t="n">
+        <v>681</v>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E69" t="n">
+        <v>1</v>
+      </c>
+      <c r="F69" t="n">
+        <v>1995330</v>
+      </c>
+      <c r="G69" t="n">
+        <v>23829</v>
+      </c>
+      <c r="H69" t="n">
+        <v>1.208672985709873</v>
+      </c>
+      <c r="I69" t="inlineStr">
+        <is>
+          <t>2026-03-21T04:57:12</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>2026-03-21</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>스타 벌크 캐리어스</t>
+        </is>
+      </c>
+      <c r="C70" t="n">
+        <v>50</v>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E70" t="n">
+        <v>1</v>
+      </c>
+      <c r="F70" t="n">
+        <v>1680142.640194588</v>
+      </c>
+      <c r="G70" t="n">
+        <v>365789.6401945879</v>
+      </c>
+      <c r="H70" t="n">
+        <v>27.83039565433242</v>
+      </c>
+      <c r="I70" t="inlineStr">
+        <is>
+          <t>2026-03-21T04:57:12</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>2026-03-21</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>케이씨</t>
+        </is>
+      </c>
+      <c r="C71" t="n">
+        <v>50</v>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E71" t="n">
+        <v>1</v>
+      </c>
+      <c r="F71" t="n">
+        <v>1670000</v>
+      </c>
+      <c r="G71" t="n">
+        <v>20500</v>
+      </c>
+      <c r="H71" t="n">
+        <v>1.242800848742043</v>
+      </c>
+      <c r="I71" t="inlineStr">
+        <is>
+          <t>2026-03-21T04:57:12</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>2026-03-21</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>유나이티드헬스 그룹</t>
+        </is>
+      </c>
+      <c r="C72" t="n">
+        <v>4</v>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E72" t="n">
+        <v>1</v>
+      </c>
+      <c r="F72" t="n">
+        <v>1658864.328313038</v>
+      </c>
+      <c r="G72" t="n">
+        <v>-35591.67168696248</v>
+      </c>
+      <c r="H72" t="n">
+        <v>-2.100477774988697</v>
+      </c>
+      <c r="I72" t="inlineStr">
+        <is>
+          <t>2026-03-21T04:57:12</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>2026-03-21</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>텍사스 퍼시픽 랜드</t>
+        </is>
+      </c>
+      <c r="C73" t="n">
+        <v>2</v>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E73" t="n">
+        <v>1</v>
+      </c>
+      <c r="F73" t="n">
+        <v>1563247.374122903</v>
+      </c>
+      <c r="G73" t="n">
+        <v>-14646.62587709725</v>
+      </c>
+      <c r="H73" t="n">
+        <v>-0.9282388979929735</v>
+      </c>
+      <c r="I73" t="inlineStr">
+        <is>
+          <t>2026-03-21T04:57:12</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>2026-03-21</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>LX인터내셔널</t>
+        </is>
+      </c>
+      <c r="C74" t="n">
+        <v>20</v>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E74" t="n">
+        <v>1</v>
+      </c>
+      <c r="F74" t="n">
+        <v>943000</v>
+      </c>
+      <c r="G74" t="n">
+        <v>4000</v>
+      </c>
+      <c r="H74" t="n">
+        <v>0.4259850905218318</v>
+      </c>
+      <c r="I74" t="inlineStr">
+        <is>
+          <t>2026-03-21T04:57:12</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>2026-03-21</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>삼성생명</t>
+        </is>
+      </c>
+      <c r="C75" t="n">
+        <v>4</v>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E75" t="n">
+        <v>1</v>
+      </c>
+      <c r="F75" t="n">
+        <v>926000</v>
+      </c>
+      <c r="G75" t="n">
+        <v>93000</v>
+      </c>
+      <c r="H75" t="n">
+        <v>11.16446578631453</v>
+      </c>
+      <c r="I75" t="inlineStr">
+        <is>
+          <t>2026-03-21T04:57:12</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>2026-03-21</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>비에이치아이</t>
+        </is>
+      </c>
+      <c r="C76" t="n">
+        <v>8</v>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E76" t="n">
+        <v>1</v>
+      </c>
+      <c r="F76" t="n">
+        <v>876000</v>
+      </c>
+      <c r="G76" t="n">
+        <v>210885</v>
+      </c>
+      <c r="H76" t="n">
+        <v>31.70654698811484</v>
+      </c>
+      <c r="I76" t="inlineStr">
+        <is>
+          <t>2026-03-21T04:57:12</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>2026-03-21</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>하프니아</t>
+        </is>
+      </c>
+      <c r="C77" t="n">
+        <v>80</v>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E77" t="n">
+        <v>1</v>
+      </c>
+      <c r="F77" t="n">
+        <v>842704.775390625</v>
+      </c>
+      <c r="G77" t="n">
+        <v>216973.775390625</v>
+      </c>
+      <c r="H77" t="n">
+        <v>34.67524789256486</v>
+      </c>
+      <c r="I77" t="inlineStr">
+        <is>
+          <t>2026-03-21T04:57:12</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>2026-03-21</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>클리블랜드 클리프스</t>
+        </is>
+      </c>
+      <c r="C78" t="n">
+        <v>70</v>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E78" t="n">
+        <v>1</v>
+      </c>
+      <c r="F78" t="n">
+        <v>823743.9360268187</v>
+      </c>
+      <c r="G78" t="n">
+        <v>-192311.0639731813</v>
+      </c>
+      <c r="H78" t="n">
+        <v>-18.92722972409774</v>
+      </c>
+      <c r="I78" t="inlineStr">
+        <is>
+          <t>2026-03-21T04:57:12</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>2026-03-21</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>낫 오프쇼어 파트너스</t>
+        </is>
+      </c>
+      <c r="C79" t="n">
+        <v>30</v>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E79" t="n">
+        <v>1</v>
+      </c>
+      <c r="F79" t="n">
+        <v>413075.8057155996</v>
+      </c>
+      <c r="G79" t="n">
+        <v>-4439.194284400437</v>
+      </c>
+      <c r="H79" t="n">
+        <v>-1.063241867813237</v>
+      </c>
+      <c r="I79" t="inlineStr">
+        <is>
+          <t>2026-03-21T04:57:12</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>2026-03-21</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
           <t>NH투자증권우</t>
         </is>
       </c>
-      <c r="C66" t="n">
+      <c r="C80" t="n">
         <v>2</v>
       </c>
-      <c r="D66" t="inlineStr">
-        <is>
-          <t>KRW</t>
-        </is>
-      </c>
-      <c r="E66" t="n">
-        <v>1</v>
-      </c>
-      <c r="F66" t="n">
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E80" t="n">
+        <v>1</v>
+      </c>
+      <c r="F80" t="n">
         <v>54700</v>
       </c>
-      <c r="G66" t="n">
+      <c r="G80" t="n">
         <v>100</v>
       </c>
-      <c r="H66" t="n">
+      <c r="H80" t="n">
         <v>0.1831501831501831</v>
       </c>
-      <c r="I66" t="inlineStr">
+      <c r="I80" t="inlineStr">
         <is>
           <t>2026-03-21T04:57:12</t>
         </is>
@@ -3704,7 +4600,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>2026-03-21T05:00:12</t>
+          <t>2026-03-21T05:00:47</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: portfolio snapshot 2026-03-17 (2026-03-21T05:00:49)
</commit_message>
<xml_diff>
--- a/portfolio_auto.xlsx
+++ b/portfolio_auto.xlsx
@@ -1549,7 +1549,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2026-03-21T05:00:47</t>
+          <t>2026-03-21T05:00:49</t>
         </is>
       </c>
       <c r="E2" t="n">
@@ -1650,7 +1650,7 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>2026-03-21T05:00:47</t>
+          <t>2026-03-21T05:00:49</t>
         </is>
       </c>
     </row>
@@ -1687,7 +1687,7 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>2026-03-21T05:00:47</t>
+          <t>2026-03-21T05:00:49</t>
         </is>
       </c>
     </row>
@@ -1724,7 +1724,7 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>2026-03-21T05:00:47</t>
+          <t>2026-03-21T05:00:49</t>
         </is>
       </c>
     </row>
@@ -1761,7 +1761,7 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>2026-03-21T05:00:47</t>
+          <t>2026-03-21T05:00:49</t>
         </is>
       </c>
     </row>
@@ -1798,7 +1798,7 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>2026-03-21T05:00:47</t>
+          <t>2026-03-21T05:00:49</t>
         </is>
       </c>
     </row>
@@ -1835,7 +1835,7 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>2026-03-21T05:00:47</t>
+          <t>2026-03-21T05:00:49</t>
         </is>
       </c>
     </row>
@@ -1872,7 +1872,7 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>2026-03-21T05:00:47</t>
+          <t>2026-03-21T05:00:49</t>
         </is>
       </c>
     </row>
@@ -1909,7 +1909,7 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>2026-03-21T05:00:47</t>
+          <t>2026-03-21T05:00:49</t>
         </is>
       </c>
     </row>
@@ -1946,7 +1946,7 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>2026-03-21T05:00:47</t>
+          <t>2026-03-21T05:00:49</t>
         </is>
       </c>
     </row>
@@ -1983,7 +1983,7 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>2026-03-21T05:00:47</t>
+          <t>2026-03-21T05:00:49</t>
         </is>
       </c>
     </row>
@@ -2020,7 +2020,7 @@
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>2026-03-21T05:00:47</t>
+          <t>2026-03-21T05:00:49</t>
         </is>
       </c>
     </row>
@@ -2057,7 +2057,7 @@
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>2026-03-21T05:00:47</t>
+          <t>2026-03-21T05:00:49</t>
         </is>
       </c>
     </row>
@@ -2094,7 +2094,7 @@
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>2026-03-21T05:00:47</t>
+          <t>2026-03-21T05:00:49</t>
         </is>
       </c>
     </row>
@@ -2131,7 +2131,7 @@
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>2026-03-21T05:00:47</t>
+          <t>2026-03-21T05:00:49</t>
         </is>
       </c>
     </row>
@@ -2168,7 +2168,7 @@
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>2026-03-21T05:00:47</t>
+          <t>2026-03-21T05:00:49</t>
         </is>
       </c>
     </row>
@@ -2205,7 +2205,7 @@
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>2026-03-21T05:00:47</t>
+          <t>2026-03-21T05:00:49</t>
         </is>
       </c>
     </row>
@@ -2242,7 +2242,7 @@
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>2026-03-21T05:00:47</t>
+          <t>2026-03-21T05:00:49</t>
         </is>
       </c>
     </row>
@@ -2279,7 +2279,7 @@
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>2026-03-21T05:00:47</t>
+          <t>2026-03-21T05:00:49</t>
         </is>
       </c>
     </row>
@@ -2316,7 +2316,7 @@
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>2026-03-21T05:00:47</t>
+          <t>2026-03-21T05:00:49</t>
         </is>
       </c>
     </row>
@@ -2353,7 +2353,7 @@
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>2026-03-21T05:00:47</t>
+          <t>2026-03-21T05:00:49</t>
         </is>
       </c>
     </row>
@@ -2390,7 +2390,7 @@
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>2026-03-21T05:00:47</t>
+          <t>2026-03-21T05:00:49</t>
         </is>
       </c>
     </row>
@@ -2427,7 +2427,7 @@
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>2026-03-21T05:00:47</t>
+          <t>2026-03-21T05:00:49</t>
         </is>
       </c>
     </row>
@@ -2464,7 +2464,7 @@
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>2026-03-21T05:00:47</t>
+          <t>2026-03-21T05:00:49</t>
         </is>
       </c>
     </row>
@@ -2501,7 +2501,7 @@
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>2026-03-21T05:00:47</t>
+          <t>2026-03-21T05:00:49</t>
         </is>
       </c>
     </row>
@@ -2538,7 +2538,7 @@
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>2026-03-21T05:00:47</t>
+          <t>2026-03-21T05:00:49</t>
         </is>
       </c>
     </row>
@@ -2575,7 +2575,7 @@
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>2026-03-21T05:00:47</t>
+          <t>2026-03-21T05:00:49</t>
         </is>
       </c>
     </row>
@@ -2612,7 +2612,7 @@
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>2026-03-21T05:00:47</t>
+          <t>2026-03-21T05:00:49</t>
         </is>
       </c>
     </row>
@@ -2649,7 +2649,7 @@
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>2026-03-21T05:00:47</t>
+          <t>2026-03-21T05:00:49</t>
         </is>
       </c>
     </row>
@@ -2686,7 +2686,7 @@
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>2026-03-21T05:00:47</t>
+          <t>2026-03-21T05:00:49</t>
         </is>
       </c>
     </row>
@@ -2723,7 +2723,7 @@
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>2026-03-21T05:00:47</t>
+          <t>2026-03-21T05:00:49</t>
         </is>
       </c>
     </row>
@@ -2760,7 +2760,7 @@
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>2026-03-21T05:00:47</t>
+          <t>2026-03-21T05:00:49</t>
         </is>
       </c>
     </row>
@@ -2797,7 +2797,7 @@
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>2026-03-21T05:00:47</t>
+          <t>2026-03-21T05:00:49</t>
         </is>
       </c>
     </row>
@@ -2834,7 +2834,7 @@
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>2026-03-21T05:00:47</t>
+          <t>2026-03-21T05:00:49</t>
         </is>
       </c>
     </row>
@@ -2871,7 +2871,7 @@
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>2026-03-21T05:00:47</t>
+          <t>2026-03-21T05:00:49</t>
         </is>
       </c>
     </row>
@@ -2908,7 +2908,7 @@
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>2026-03-21T05:00:47</t>
+          <t>2026-03-21T05:00:49</t>
         </is>
       </c>
     </row>
@@ -2945,7 +2945,7 @@
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>2026-03-21T05:00:47</t>
+          <t>2026-03-21T05:00:49</t>
         </is>
       </c>
     </row>
@@ -2982,7 +2982,7 @@
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>2026-03-21T05:00:47</t>
+          <t>2026-03-21T05:00:49</t>
         </is>
       </c>
     </row>
@@ -3019,7 +3019,7 @@
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>2026-03-21T05:00:47</t>
+          <t>2026-03-21T05:00:49</t>
         </is>
       </c>
     </row>
@@ -4600,7 +4600,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>2026-03-21T05:00:47</t>
+          <t>2026-03-21T05:00:49</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: portfolio snapshot 2026-03-17 (2026-03-21T05:01:03)
</commit_message>
<xml_diff>
--- a/portfolio_auto.xlsx
+++ b/portfolio_auto.xlsx
@@ -471,11 +471,11 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>삼성화재</t>
+          <t>페트로브라스 (ADR)</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>7</v>
+        <v>480</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
@@ -486,23 +486,23 @@
         <v>1</v>
       </c>
       <c r="E2" t="n">
-        <v>3321500</v>
+        <v>13579584.97235231</v>
       </c>
       <c r="F2" t="n">
-        <v>-309500</v>
+        <v>1473035.972352311</v>
       </c>
       <c r="G2" t="n">
-        <v>-8.523822638391627</v>
+        <v>12.16726560436265</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>세아제강</t>
+          <t>AGNC 인베스트먼트</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>50</v>
+        <v>700</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
@@ -513,23 +513,23 @@
         <v>1</v>
       </c>
       <c r="E3" t="n">
-        <v>7395000</v>
+        <v>10270464.45007324</v>
       </c>
       <c r="F3" t="n">
-        <v>1085000</v>
+        <v>-561550.5499267578</v>
       </c>
       <c r="G3" t="n">
-        <v>17.19492868462758</v>
+        <v>-5.184174411933125</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>케이씨</t>
+          <t>대한조선</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>50</v>
+        <v>100</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
@@ -540,23 +540,23 @@
         <v>1</v>
       </c>
       <c r="E4" t="n">
-        <v>1670000</v>
+        <v>9120000</v>
       </c>
       <c r="F4" t="n">
-        <v>20500</v>
+        <v>1907000</v>
       </c>
       <c r="G4" t="n">
-        <v>1.242800848742043</v>
+        <v>26.43837515596839</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>하나금융지주</t>
+          <t>프론트라인</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>10</v>
+        <v>175</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -567,23 +567,23 @@
         <v>1</v>
       </c>
       <c r="E5" t="n">
-        <v>1132000</v>
+        <v>8471815.962899337</v>
       </c>
       <c r="F5" t="n">
-        <v>23000</v>
+        <v>4041951.962899337</v>
       </c>
       <c r="G5" t="n">
-        <v>2.073940486925157</v>
+        <v>91.24325177701475</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>현대제철</t>
+          <t>시드릴</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>70</v>
+        <v>123</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
@@ -594,23 +594,23 @@
         <v>1</v>
       </c>
       <c r="E6" t="n">
-        <v>2621500</v>
+        <v>8070101.805898919</v>
       </c>
       <c r="F6" t="n">
-        <v>-186000</v>
+        <v>1619750.805898919</v>
       </c>
       <c r="G6" t="n">
-        <v>-6.625111308993767</v>
+        <v>25.11104908707943</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>휴스틸</t>
+          <t>세아제강</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>500</v>
+        <v>50</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -621,23 +621,23 @@
         <v>1</v>
       </c>
       <c r="E7" t="n">
-        <v>2750000</v>
+        <v>7395000</v>
       </c>
       <c r="F7" t="n">
-        <v>471390</v>
+        <v>1085000</v>
       </c>
       <c r="G7" t="n">
-        <v>20.68761218462133</v>
+        <v>17.19492868462758</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>DL이앤씨</t>
+          <t>트랜스오션</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>80</v>
+        <v>750</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
@@ -648,23 +648,23 @@
         <v>1</v>
       </c>
       <c r="E8" t="n">
-        <v>5392000</v>
+        <v>7020031.5082007</v>
       </c>
       <c r="F8" t="n">
-        <v>1981000</v>
+        <v>2892797.5082007</v>
       </c>
       <c r="G8" t="n">
-        <v>58.07681031955438</v>
+        <v>70.09046514446965</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>HD건설기계</t>
+          <t>노블</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>31</v>
+        <v>99</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
@@ -675,23 +675,23 @@
         <v>1</v>
       </c>
       <c r="E9" t="n">
-        <v>4123000</v>
+        <v>6958769.981090547</v>
       </c>
       <c r="F9" t="n">
-        <v>87904</v>
+        <v>3051561.981090547</v>
       </c>
       <c r="G9" t="n">
-        <v>2.178485964150543</v>
+        <v>78.10083264291399</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>KoAct 코스닥액티브</t>
+          <t>센트러스 에너지</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>200</v>
+        <v>21</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
@@ -702,23 +702,23 @@
         <v>1</v>
       </c>
       <c r="E10" t="n">
-        <v>2582000</v>
+        <v>5901882.720856408</v>
       </c>
       <c r="F10" t="n">
-        <v>-120000</v>
+        <v>-329336.2791435914</v>
       </c>
       <c r="G10" t="n">
-        <v>-4.441154700222058</v>
+        <v>-5.285262468605123</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>TIME 코리아밸류업액티브</t>
+          <t>DL이앤씨</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>201</v>
+        <v>80</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
@@ -729,23 +729,23 @@
         <v>1</v>
       </c>
       <c r="E11" t="n">
-        <v>4797870</v>
+        <v>5392000</v>
       </c>
       <c r="F11" t="n">
-        <v>74073</v>
+        <v>1981000</v>
       </c>
       <c r="G11" t="n">
-        <v>1.568081778281328</v>
+        <v>58.07681031955438</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>페트로브라스 (ADR)</t>
+          <t>타이드워터</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>480</v>
+        <v>48</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
@@ -756,23 +756,23 @@
         <v>1</v>
       </c>
       <c r="E12" t="n">
-        <v>13579584.97235231</v>
+        <v>5235363.852789983</v>
       </c>
       <c r="F12" t="n">
-        <v>1473035.972352311</v>
+        <v>1510818.852789983</v>
       </c>
       <c r="G12" t="n">
-        <v>12.16726560436265</v>
+        <v>40.56385015592463</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>프론트라인</t>
+          <t>노브</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>175</v>
+        <v>185</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
@@ -783,23 +783,23 @@
         <v>1</v>
       </c>
       <c r="E13" t="n">
-        <v>8471815.962899337</v>
+        <v>5200391.447092756</v>
       </c>
       <c r="F13" t="n">
-        <v>4041951.962899337</v>
+        <v>1890383.447092756</v>
       </c>
       <c r="G13" t="n">
-        <v>91.24325177701475</v>
+        <v>57.11114435653194</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>피바디 에너지</t>
+          <t>TIME 코리아밸류업액티브</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>65</v>
+        <v>201</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
@@ -810,23 +810,23 @@
         <v>1</v>
       </c>
       <c r="E14" t="n">
-        <v>3649438.50225304</v>
+        <v>4797870</v>
       </c>
       <c r="F14" t="n">
-        <v>2178666.50225304</v>
+        <v>74073</v>
       </c>
       <c r="G14" t="n">
-        <v>148.1308117269733</v>
+        <v>1.568081778281328</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>하프니아</t>
+          <t>오케아니스 에코 탱커스</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>80</v>
+        <v>65</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
@@ -837,23 +837,23 @@
         <v>1</v>
       </c>
       <c r="E15" t="n">
-        <v>842704.775390625</v>
+        <v>4511179.137784176</v>
       </c>
       <c r="F15" t="n">
-        <v>216973.775390625</v>
+        <v>2254819.137784176</v>
       </c>
       <c r="G15" t="n">
-        <v>34.67524789256486</v>
+        <v>99.93171026716374</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>AGNC 인베스트먼트</t>
+          <t>동원개발</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>700</v>
+        <v>1360</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
@@ -864,23 +864,23 @@
         <v>1</v>
       </c>
       <c r="E16" t="n">
-        <v>10270464.45007324</v>
+        <v>4202400</v>
       </c>
       <c r="F16" t="n">
-        <v>-561550.5499267578</v>
+        <v>465000</v>
       </c>
       <c r="G16" t="n">
-        <v>-5.184174411933125</v>
+        <v>12.44180446299566</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>넥스틸</t>
+          <t>HD건설기계</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>200</v>
+        <v>31</v>
       </c>
       <c r="C17" t="inlineStr">
         <is>
@@ -891,23 +891,23 @@
         <v>1</v>
       </c>
       <c r="E17" t="n">
-        <v>2514000</v>
+        <v>4123000</v>
       </c>
       <c r="F17" t="n">
-        <v>503000</v>
+        <v>87904</v>
       </c>
       <c r="G17" t="n">
-        <v>25.01243162605669</v>
+        <v>2.178485964150543</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>대신증권</t>
+          <t>차코스 에너지 내비게이션</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>55</v>
+        <v>75</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
@@ -918,23 +918,23 @@
         <v>1</v>
       </c>
       <c r="E18" t="n">
-        <v>2219250</v>
+        <v>4026924.996845168</v>
       </c>
       <c r="F18" t="n">
-        <v>509749</v>
+        <v>202276.9968451681</v>
       </c>
       <c r="G18" t="n">
-        <v>29.81858448752005</v>
+        <v>5.28877420471552</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>대창단조</t>
+          <t>피바디 에너지</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>300</v>
+        <v>65</v>
       </c>
       <c r="C19" t="inlineStr">
         <is>
@@ -945,23 +945,23 @@
         <v>1</v>
       </c>
       <c r="E19" t="n">
-        <v>2004000</v>
+        <v>3649438.50225304</v>
       </c>
       <c r="F19" t="n">
-        <v>-54000</v>
+        <v>2178666.50225304</v>
       </c>
       <c r="G19" t="n">
-        <v>-2.623906705539359</v>
+        <v>148.1308117269733</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>대한조선</t>
+          <t>삼성화재</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>100</v>
+        <v>7</v>
       </c>
       <c r="C20" t="inlineStr">
         <is>
@@ -972,23 +972,23 @@
         <v>1</v>
       </c>
       <c r="E20" t="n">
-        <v>9120000</v>
+        <v>3321500</v>
       </c>
       <c r="F20" t="n">
-        <v>1907000</v>
+        <v>-309500</v>
       </c>
       <c r="G20" t="n">
-        <v>26.43837515596839</v>
+        <v>-8.523822638391627</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>동방</t>
+          <t>더치 브로스</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>681</v>
+        <v>39</v>
       </c>
       <c r="C21" t="inlineStr">
         <is>
@@ -999,23 +999,23 @@
         <v>1</v>
       </c>
       <c r="E21" t="n">
-        <v>1995330</v>
+        <v>2934418.414306641</v>
       </c>
       <c r="F21" t="n">
-        <v>23829</v>
+        <v>-256225.5856933594</v>
       </c>
       <c r="G21" t="n">
-        <v>1.208672985709873</v>
+        <v>-8.030528811530193</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>동원개발</t>
+          <t>휴스틸</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>1360</v>
+        <v>500</v>
       </c>
       <c r="C22" t="inlineStr">
         <is>
@@ -1026,23 +1026,23 @@
         <v>1</v>
       </c>
       <c r="E22" t="n">
-        <v>4202400</v>
+        <v>2750000</v>
       </c>
       <c r="F22" t="n">
-        <v>465000</v>
+        <v>471390</v>
       </c>
       <c r="G22" t="n">
-        <v>12.44180446299566</v>
+        <v>20.68761218462133</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>미창석유</t>
+          <t>현대제철</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>18</v>
+        <v>70</v>
       </c>
       <c r="C23" t="inlineStr">
         <is>
@@ -1053,23 +1053,23 @@
         <v>1</v>
       </c>
       <c r="E23" t="n">
-        <v>2097000</v>
+        <v>2621500</v>
       </c>
       <c r="F23" t="n">
-        <v>-295200</v>
+        <v>-186000</v>
       </c>
       <c r="G23" t="n">
-        <v>-12.34010534236268</v>
+        <v>-6.625111308993767</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>비에이치아이</t>
+          <t>KoAct 코스닥액티브</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>8</v>
+        <v>200</v>
       </c>
       <c r="C24" t="inlineStr">
         <is>
@@ -1080,23 +1080,23 @@
         <v>1</v>
       </c>
       <c r="E24" t="n">
-        <v>876000</v>
+        <v>2582000</v>
       </c>
       <c r="F24" t="n">
-        <v>210885</v>
+        <v>-120000</v>
       </c>
       <c r="G24" t="n">
-        <v>31.70654698811484</v>
+        <v>-4.441154700222058</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>삼성생명</t>
+          <t>넥스틸</t>
         </is>
       </c>
       <c r="B25" t="n">
-        <v>4</v>
+        <v>200</v>
       </c>
       <c r="C25" t="inlineStr">
         <is>
@@ -1107,23 +1107,23 @@
         <v>1</v>
       </c>
       <c r="E25" t="n">
-        <v>926000</v>
+        <v>2514000</v>
       </c>
       <c r="F25" t="n">
-        <v>93000</v>
+        <v>503000</v>
       </c>
       <c r="G25" t="n">
-        <v>11.16446578631453</v>
+        <v>25.01243162605669</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>노브</t>
+          <t>대신증권</t>
         </is>
       </c>
       <c r="B26" t="n">
-        <v>185</v>
+        <v>55</v>
       </c>
       <c r="C26" t="inlineStr">
         <is>
@@ -1134,23 +1134,23 @@
         <v>1</v>
       </c>
       <c r="E26" t="n">
-        <v>5200391.447092756</v>
+        <v>2219250</v>
       </c>
       <c r="F26" t="n">
-        <v>1890383.447092756</v>
+        <v>509749</v>
       </c>
       <c r="G26" t="n">
-        <v>57.11114435653194</v>
+        <v>29.81858448752005</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>노블</t>
+          <t>발레로 에너지</t>
         </is>
       </c>
       <c r="B27" t="n">
-        <v>99</v>
+        <v>6</v>
       </c>
       <c r="C27" t="inlineStr">
         <is>
@@ -1161,23 +1161,23 @@
         <v>1</v>
       </c>
       <c r="E27" t="n">
-        <v>6958769.981090547</v>
+        <v>2165691.085066516</v>
       </c>
       <c r="F27" t="n">
-        <v>3051561.981090547</v>
+        <v>101701.085066516</v>
       </c>
       <c r="G27" t="n">
-        <v>78.10083264291399</v>
+        <v>4.927402025519307</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>더치 브로스</t>
+          <t>미창석유</t>
         </is>
       </c>
       <c r="B28" t="n">
-        <v>39</v>
+        <v>18</v>
       </c>
       <c r="C28" t="inlineStr">
         <is>
@@ -1188,23 +1188,23 @@
         <v>1</v>
       </c>
       <c r="E28" t="n">
-        <v>2934418.414306641</v>
+        <v>2097000</v>
       </c>
       <c r="F28" t="n">
-        <v>-256225.5856933594</v>
+        <v>-295200</v>
       </c>
       <c r="G28" t="n">
-        <v>-8.030528811530193</v>
+        <v>-12.34010534236268</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>발레로 에너지</t>
+          <t>대창단조</t>
         </is>
       </c>
       <c r="B29" t="n">
-        <v>6</v>
+        <v>300</v>
       </c>
       <c r="C29" t="inlineStr">
         <is>
@@ -1215,23 +1215,23 @@
         <v>1</v>
       </c>
       <c r="E29" t="n">
-        <v>2165691.085066516</v>
+        <v>2004000</v>
       </c>
       <c r="F29" t="n">
-        <v>101701.085066516</v>
+        <v>-54000</v>
       </c>
       <c r="G29" t="n">
-        <v>4.927402025519307</v>
+        <v>-2.623906705539359</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>센트러스 에너지</t>
+          <t>동방</t>
         </is>
       </c>
       <c r="B30" t="n">
-        <v>21</v>
+        <v>681</v>
       </c>
       <c r="C30" t="inlineStr">
         <is>
@@ -1242,13 +1242,13 @@
         <v>1</v>
       </c>
       <c r="E30" t="n">
-        <v>5901882.720856408</v>
+        <v>1995330</v>
       </c>
       <c r="F30" t="n">
-        <v>-329336.2791435914</v>
+        <v>23829</v>
       </c>
       <c r="G30" t="n">
-        <v>-5.285262468605123</v>
+        <v>1.208672985709873</v>
       </c>
     </row>
     <row r="31">
@@ -1281,11 +1281,11 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>시드릴</t>
+          <t>케이씨</t>
         </is>
       </c>
       <c r="B32" t="n">
-        <v>123</v>
+        <v>50</v>
       </c>
       <c r="C32" t="inlineStr">
         <is>
@@ -1296,23 +1296,23 @@
         <v>1</v>
       </c>
       <c r="E32" t="n">
-        <v>8070101.805898919</v>
+        <v>1670000</v>
       </c>
       <c r="F32" t="n">
-        <v>1619750.805898919</v>
+        <v>20500</v>
       </c>
       <c r="G32" t="n">
-        <v>25.11104908707943</v>
+        <v>1.242800848742043</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>오케아니스 에코 탱커스</t>
+          <t>유나이티드헬스 그룹</t>
         </is>
       </c>
       <c r="B33" t="n">
-        <v>65</v>
+        <v>4</v>
       </c>
       <c r="C33" t="inlineStr">
         <is>
@@ -1323,23 +1323,23 @@
         <v>1</v>
       </c>
       <c r="E33" t="n">
-        <v>4511179.137784176</v>
+        <v>1658864.328313038</v>
       </c>
       <c r="F33" t="n">
-        <v>2254819.137784176</v>
+        <v>-35591.67168696225</v>
       </c>
       <c r="G33" t="n">
-        <v>99.93171026716374</v>
+        <v>-2.100477774988684</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>유나이티드헬스 그룹</t>
+          <t>하나금융지주</t>
         </is>
       </c>
       <c r="B34" t="n">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="C34" t="inlineStr">
         <is>
@@ -1350,23 +1350,23 @@
         <v>1</v>
       </c>
       <c r="E34" t="n">
-        <v>1658864.328313038</v>
+        <v>1132000</v>
       </c>
       <c r="F34" t="n">
-        <v>-35591.67168696225</v>
+        <v>23000</v>
       </c>
       <c r="G34" t="n">
-        <v>-2.100477774988684</v>
+        <v>2.073940486925157</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>차코스 에너지 내비게이션</t>
+          <t>삼성생명</t>
         </is>
       </c>
       <c r="B35" t="n">
-        <v>75</v>
+        <v>4</v>
       </c>
       <c r="C35" t="inlineStr">
         <is>
@@ -1377,23 +1377,23 @@
         <v>1</v>
       </c>
       <c r="E35" t="n">
-        <v>4026924.996845168</v>
+        <v>926000</v>
       </c>
       <c r="F35" t="n">
-        <v>202276.9968451681</v>
+        <v>93000</v>
       </c>
       <c r="G35" t="n">
-        <v>5.28877420471552</v>
+        <v>11.16446578631453</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>클리블랜드 클리프스</t>
+          <t>비에이치아이</t>
         </is>
       </c>
       <c r="B36" t="n">
-        <v>70</v>
+        <v>8</v>
       </c>
       <c r="C36" t="inlineStr">
         <is>
@@ -1404,23 +1404,23 @@
         <v>1</v>
       </c>
       <c r="E36" t="n">
-        <v>823743.9360268187</v>
+        <v>876000</v>
       </c>
       <c r="F36" t="n">
-        <v>-192311.0639731813</v>
+        <v>210885</v>
       </c>
       <c r="G36" t="n">
-        <v>-18.92722972409774</v>
+        <v>31.70654698811484</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>타이드워터</t>
+          <t>하프니아</t>
         </is>
       </c>
       <c r="B37" t="n">
-        <v>48</v>
+        <v>80</v>
       </c>
       <c r="C37" t="inlineStr">
         <is>
@@ -1431,23 +1431,23 @@
         <v>1</v>
       </c>
       <c r="E37" t="n">
-        <v>5235363.852789983</v>
+        <v>842704.775390625</v>
       </c>
       <c r="F37" t="n">
-        <v>1510818.852789983</v>
+        <v>216973.775390625</v>
       </c>
       <c r="G37" t="n">
-        <v>40.56385015592463</v>
+        <v>34.67524789256486</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>텍사스 퍼시픽 랜드</t>
+          <t>클리블랜드 클리프스</t>
         </is>
       </c>
       <c r="B38" t="n">
-        <v>1</v>
+        <v>70</v>
       </c>
       <c r="C38" t="inlineStr">
         <is>
@@ -1458,23 +1458,23 @@
         <v>1</v>
       </c>
       <c r="E38" t="n">
-        <v>781623.6870614514</v>
+        <v>823743.9360268187</v>
       </c>
       <c r="F38" t="n">
-        <v>3032.687061451375</v>
+        <v>-192311.0639731813</v>
       </c>
       <c r="G38" t="n">
-        <v>0.3895096477420591</v>
+        <v>-18.92722972409774</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>트랜스오션</t>
+          <t>텍사스 퍼시픽 랜드</t>
         </is>
       </c>
       <c r="B39" t="n">
-        <v>750</v>
+        <v>1</v>
       </c>
       <c r="C39" t="inlineStr">
         <is>
@@ -1485,13 +1485,13 @@
         <v>1</v>
       </c>
       <c r="E39" t="n">
-        <v>7020031.5082007</v>
+        <v>781623.6870614514</v>
       </c>
       <c r="F39" t="n">
-        <v>2892797.5082007</v>
+        <v>3032.687061451375</v>
       </c>
       <c r="G39" t="n">
-        <v>70.09046514446965</v>
+        <v>0.3895096477420591</v>
       </c>
     </row>
   </sheetData>
@@ -1542,14 +1542,14 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0</v>
+        <v>33078556</v>
       </c>
       <c r="C2" t="n">
-        <v>0</v>
+        <v>6010.99</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2026-03-21T05:00:49</t>
+          <t>2026-03-21T05:01:03</t>
         </is>
       </c>
       <c r="E2" t="n">
@@ -4588,10 +4588,10 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0</v>
+        <v>33078556</v>
       </c>
       <c r="C2" t="n">
-        <v>0</v>
+        <v>6010.99</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
@@ -4600,7 +4600,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>2026-03-21T05:00:49</t>
+          <t>2026-03-21T05:01:03</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: portfolio snapshot 2026-03-21 (2026-03-21T22:46:15)
</commit_message>
<xml_diff>
--- a/portfolio_auto.xlsx
+++ b/portfolio_auto.xlsx
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G39"/>
+  <dimension ref="A1:G41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -498,11 +498,11 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>AGNC 인베스트먼트</t>
+          <t>대한조선</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>700</v>
+        <v>100</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
@@ -513,23 +513,23 @@
         <v>1</v>
       </c>
       <c r="E3" t="n">
-        <v>10270464.45007324</v>
+        <v>9120000</v>
       </c>
       <c r="F3" t="n">
-        <v>-561550.5499267578</v>
+        <v>1907000</v>
       </c>
       <c r="G3" t="n">
-        <v>-5.184174411933125</v>
+        <v>26.43837515596839</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>대한조선</t>
+          <t>프론트라인</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>100</v>
+        <v>175</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
@@ -540,23 +540,23 @@
         <v>1</v>
       </c>
       <c r="E4" t="n">
-        <v>9120000</v>
+        <v>8471815.962899337</v>
       </c>
       <c r="F4" t="n">
-        <v>1907000</v>
+        <v>4041951.962899337</v>
       </c>
       <c r="G4" t="n">
-        <v>26.43837515596839</v>
+        <v>91.24325177701475</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>프론트라인</t>
+          <t>시드릴</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>175</v>
+        <v>123</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -567,23 +567,23 @@
         <v>1</v>
       </c>
       <c r="E5" t="n">
-        <v>8471815.962899337</v>
+        <v>8070101.805898919</v>
       </c>
       <c r="F5" t="n">
-        <v>4041951.962899337</v>
+        <v>1619750.805898919</v>
       </c>
       <c r="G5" t="n">
-        <v>91.24325177701475</v>
+        <v>25.11104908707943</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>시드릴</t>
+          <t>세아제강</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>123</v>
+        <v>50</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
@@ -594,23 +594,23 @@
         <v>1</v>
       </c>
       <c r="E6" t="n">
-        <v>8070101.805898919</v>
+        <v>7395000</v>
       </c>
       <c r="F6" t="n">
-        <v>1619750.805898919</v>
+        <v>1085000</v>
       </c>
       <c r="G6" t="n">
-        <v>25.11104908707943</v>
+        <v>17.19492868462758</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>세아제강</t>
+          <t>센트러스 에너지</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>50</v>
+        <v>25</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -621,13 +621,13 @@
         <v>1</v>
       </c>
       <c r="E7" t="n">
-        <v>7395000</v>
+        <v>7026050.85816239</v>
       </c>
       <c r="F7" t="n">
-        <v>1085000</v>
+        <v>-406805.1418376099</v>
       </c>
       <c r="G7" t="n">
-        <v>17.19492868462758</v>
+        <v>-5.473066366920198</v>
       </c>
     </row>
     <row r="8">
@@ -687,11 +687,11 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>센트러스 에너지</t>
+          <t>타이드워터</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>21</v>
+        <v>48</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
@@ -702,23 +702,23 @@
         <v>1</v>
       </c>
       <c r="E10" t="n">
-        <v>5901882.720856408</v>
+        <v>5235363.852789983</v>
       </c>
       <c r="F10" t="n">
-        <v>-329336.2791435914</v>
+        <v>1510818.852789983</v>
       </c>
       <c r="G10" t="n">
-        <v>-5.285262468605123</v>
+        <v>40.56385015592463</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>DL이앤씨</t>
+          <t>노브</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>80</v>
+        <v>185</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
@@ -729,23 +729,23 @@
         <v>1</v>
       </c>
       <c r="E11" t="n">
-        <v>5392000</v>
+        <v>5200391.447092756</v>
       </c>
       <c r="F11" t="n">
-        <v>1981000</v>
+        <v>1890383.447092756</v>
       </c>
       <c r="G11" t="n">
-        <v>58.07681031955438</v>
+        <v>57.11114435653194</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>타이드워터</t>
+          <t>TIME 코리아밸류업액티브</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>48</v>
+        <v>201</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
@@ -756,23 +756,23 @@
         <v>1</v>
       </c>
       <c r="E12" t="n">
-        <v>5235363.852789983</v>
+        <v>4797870</v>
       </c>
       <c r="F12" t="n">
-        <v>1510818.852789983</v>
+        <v>74073</v>
       </c>
       <c r="G12" t="n">
-        <v>40.56385015592463</v>
+        <v>1.568081778281328</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>노브</t>
+          <t>오케아니스 에코 탱커스</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>185</v>
+        <v>65</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
@@ -783,23 +783,23 @@
         <v>1</v>
       </c>
       <c r="E13" t="n">
-        <v>5200391.447092756</v>
+        <v>4511179.137784176</v>
       </c>
       <c r="F13" t="n">
-        <v>1890383.447092756</v>
+        <v>2254819.137784176</v>
       </c>
       <c r="G13" t="n">
-        <v>57.11114435653194</v>
+        <v>99.93171026716374</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>TIME 코리아밸류업액티브</t>
+          <t>삼성화재</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>201</v>
+        <v>9</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
@@ -810,23 +810,23 @@
         <v>1</v>
       </c>
       <c r="E14" t="n">
-        <v>4797870</v>
+        <v>4270500</v>
       </c>
       <c r="F14" t="n">
-        <v>74073</v>
+        <v>-360500</v>
       </c>
       <c r="G14" t="n">
-        <v>1.568081778281328</v>
+        <v>-7.784495789246384</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>오케아니스 에코 탱커스</t>
+          <t>동원개발</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>65</v>
+        <v>1360</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
@@ -837,23 +837,23 @@
         <v>1</v>
       </c>
       <c r="E15" t="n">
-        <v>4511179.137784176</v>
+        <v>4202400</v>
       </c>
       <c r="F15" t="n">
-        <v>2254819.137784176</v>
+        <v>465000</v>
       </c>
       <c r="G15" t="n">
-        <v>99.93171026716374</v>
+        <v>12.44180446299566</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>동원개발</t>
+          <t>HD건설기계</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>1360</v>
+        <v>31</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
@@ -864,23 +864,23 @@
         <v>1</v>
       </c>
       <c r="E16" t="n">
-        <v>4202400</v>
+        <v>4123000</v>
       </c>
       <c r="F16" t="n">
-        <v>465000</v>
+        <v>87904</v>
       </c>
       <c r="G16" t="n">
-        <v>12.44180446299566</v>
+        <v>2.178485964150543</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>HD건설기계</t>
+          <t>차코스 에너지 내비게이션</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>31</v>
+        <v>75</v>
       </c>
       <c r="C17" t="inlineStr">
         <is>
@@ -891,23 +891,23 @@
         <v>1</v>
       </c>
       <c r="E17" t="n">
-        <v>4123000</v>
+        <v>4026924.996845168</v>
       </c>
       <c r="F17" t="n">
-        <v>87904</v>
+        <v>202276.9968451681</v>
       </c>
       <c r="G17" t="n">
-        <v>2.178485964150543</v>
+        <v>5.28877420471552</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>차코스 에너지 내비게이션</t>
+          <t>넥스틸</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>75</v>
+        <v>300</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
@@ -918,13 +918,13 @@
         <v>1</v>
       </c>
       <c r="E18" t="n">
-        <v>4026924.996845168</v>
+        <v>3771000</v>
       </c>
       <c r="F18" t="n">
-        <v>202276.9968451681</v>
+        <v>521000</v>
       </c>
       <c r="G18" t="n">
-        <v>5.28877420471552</v>
+        <v>16.03076923076923</v>
       </c>
     </row>
     <row r="19">
@@ -957,11 +957,11 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>삼성화재</t>
+          <t>현대제철</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>7</v>
+        <v>80</v>
       </c>
       <c r="C20" t="inlineStr">
         <is>
@@ -972,13 +972,13 @@
         <v>1</v>
       </c>
       <c r="E20" t="n">
-        <v>3321500</v>
+        <v>2996000</v>
       </c>
       <c r="F20" t="n">
-        <v>-309500</v>
+        <v>-182000</v>
       </c>
       <c r="G20" t="n">
-        <v>-8.523822638391627</v>
+        <v>-5.726872246696035</v>
       </c>
     </row>
     <row r="21">
@@ -1002,10 +1002,10 @@
         <v>2934418.414306641</v>
       </c>
       <c r="F21" t="n">
-        <v>-256225.5856933594</v>
+        <v>-256226.5856933594</v>
       </c>
       <c r="G21" t="n">
-        <v>-8.030528811530193</v>
+        <v>-8.030557636257226</v>
       </c>
     </row>
     <row r="22">
@@ -1038,11 +1038,11 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>현대제철</t>
+          <t>DL이앤씨</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>70</v>
+        <v>40</v>
       </c>
       <c r="C23" t="inlineStr">
         <is>
@@ -1053,13 +1053,13 @@
         <v>1</v>
       </c>
       <c r="E23" t="n">
-        <v>2621500</v>
+        <v>2696000</v>
       </c>
       <c r="F23" t="n">
-        <v>-186000</v>
+        <v>990500</v>
       </c>
       <c r="G23" t="n">
-        <v>-6.625111308993767</v>
+        <v>58.07681031955438</v>
       </c>
     </row>
     <row r="24">
@@ -1092,11 +1092,11 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>넥스틸</t>
+          <t>대신증권</t>
         </is>
       </c>
       <c r="B25" t="n">
-        <v>200</v>
+        <v>55</v>
       </c>
       <c r="C25" t="inlineStr">
         <is>
@@ -1107,23 +1107,23 @@
         <v>1</v>
       </c>
       <c r="E25" t="n">
-        <v>2514000</v>
+        <v>2219250</v>
       </c>
       <c r="F25" t="n">
-        <v>503000</v>
+        <v>509749</v>
       </c>
       <c r="G25" t="n">
-        <v>25.01243162605669</v>
+        <v>29.81858448752005</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>대신증권</t>
+          <t>발레로 에너지</t>
         </is>
       </c>
       <c r="B26" t="n">
-        <v>55</v>
+        <v>6</v>
       </c>
       <c r="C26" t="inlineStr">
         <is>
@@ -1134,23 +1134,23 @@
         <v>1</v>
       </c>
       <c r="E26" t="n">
-        <v>2219250</v>
+        <v>2165691.085066516</v>
       </c>
       <c r="F26" t="n">
-        <v>509749</v>
+        <v>101701.085066516</v>
       </c>
       <c r="G26" t="n">
-        <v>29.81858448752005</v>
+        <v>4.927402025519307</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>발레로 에너지</t>
+          <t>미창석유</t>
         </is>
       </c>
       <c r="B27" t="n">
-        <v>6</v>
+        <v>18</v>
       </c>
       <c r="C27" t="inlineStr">
         <is>
@@ -1161,19 +1161,19 @@
         <v>1</v>
       </c>
       <c r="E27" t="n">
-        <v>2165691.085066516</v>
+        <v>2097000</v>
       </c>
       <c r="F27" t="n">
-        <v>101701.085066516</v>
+        <v>-295200</v>
       </c>
       <c r="G27" t="n">
-        <v>4.927402025519307</v>
+        <v>-12.34010534236268</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>미창석유</t>
+          <t>하나금융지주</t>
         </is>
       </c>
       <c r="B28" t="n">
@@ -1188,13 +1188,13 @@
         <v>1</v>
       </c>
       <c r="E28" t="n">
-        <v>2097000</v>
+        <v>2037600</v>
       </c>
       <c r="F28" t="n">
-        <v>-295200</v>
+        <v>12200</v>
       </c>
       <c r="G28" t="n">
-        <v>-12.34010534236268</v>
+        <v>0.6023501530561864</v>
       </c>
     </row>
     <row r="29">
@@ -1326,20 +1326,20 @@
         <v>1658864.328313038</v>
       </c>
       <c r="F33" t="n">
-        <v>-35591.67168696225</v>
+        <v>-35591.67168696248</v>
       </c>
       <c r="G33" t="n">
-        <v>-2.100477774988684</v>
+        <v>-2.100477774988697</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>하나금융지주</t>
+          <t>텍사스 퍼시픽 랜드</t>
         </is>
       </c>
       <c r="B34" t="n">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="C34" t="inlineStr">
         <is>
@@ -1350,23 +1350,23 @@
         <v>1</v>
       </c>
       <c r="E34" t="n">
-        <v>1132000</v>
+        <v>1563247.374122903</v>
       </c>
       <c r="F34" t="n">
-        <v>23000</v>
+        <v>-14646.62587709725</v>
       </c>
       <c r="G34" t="n">
-        <v>2.073940486925157</v>
+        <v>-0.9282388979929735</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>삼성생명</t>
+          <t>LX인터내셔널</t>
         </is>
       </c>
       <c r="B35" t="n">
-        <v>4</v>
+        <v>20</v>
       </c>
       <c r="C35" t="inlineStr">
         <is>
@@ -1377,23 +1377,23 @@
         <v>1</v>
       </c>
       <c r="E35" t="n">
-        <v>926000</v>
+        <v>943000</v>
       </c>
       <c r="F35" t="n">
-        <v>93000</v>
+        <v>4000</v>
       </c>
       <c r="G35" t="n">
-        <v>11.16446578631453</v>
+        <v>0.4259850905218318</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>비에이치아이</t>
+          <t>삼성생명</t>
         </is>
       </c>
       <c r="B36" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="C36" t="inlineStr">
         <is>
@@ -1404,23 +1404,23 @@
         <v>1</v>
       </c>
       <c r="E36" t="n">
-        <v>876000</v>
+        <v>926000</v>
       </c>
       <c r="F36" t="n">
-        <v>210885</v>
+        <v>93000</v>
       </c>
       <c r="G36" t="n">
-        <v>31.70654698811484</v>
+        <v>11.16446578631453</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>하프니아</t>
+          <t>비에이치아이</t>
         </is>
       </c>
       <c r="B37" t="n">
-        <v>80</v>
+        <v>8</v>
       </c>
       <c r="C37" t="inlineStr">
         <is>
@@ -1431,23 +1431,23 @@
         <v>1</v>
       </c>
       <c r="E37" t="n">
-        <v>842704.775390625</v>
+        <v>876000</v>
       </c>
       <c r="F37" t="n">
-        <v>216973.775390625</v>
+        <v>210885</v>
       </c>
       <c r="G37" t="n">
-        <v>34.67524789256486</v>
+        <v>31.70654698811484</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>클리블랜드 클리프스</t>
+          <t>하프니아</t>
         </is>
       </c>
       <c r="B38" t="n">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="C38" t="inlineStr">
         <is>
@@ -1458,23 +1458,23 @@
         <v>1</v>
       </c>
       <c r="E38" t="n">
-        <v>823743.9360268187</v>
+        <v>842704.775390625</v>
       </c>
       <c r="F38" t="n">
-        <v>-192311.0639731813</v>
+        <v>216973.775390625</v>
       </c>
       <c r="G38" t="n">
-        <v>-18.92722972409774</v>
+        <v>34.67524789256486</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>텍사스 퍼시픽 랜드</t>
+          <t>클리블랜드 클리프스</t>
         </is>
       </c>
       <c r="B39" t="n">
-        <v>1</v>
+        <v>70</v>
       </c>
       <c r="C39" t="inlineStr">
         <is>
@@ -1485,13 +1485,67 @@
         <v>1</v>
       </c>
       <c r="E39" t="n">
-        <v>781623.6870614514</v>
+        <v>823743.9360268187</v>
       </c>
       <c r="F39" t="n">
-        <v>3032.687061451375</v>
+        <v>-192311.0639731813</v>
       </c>
       <c r="G39" t="n">
-        <v>0.3895096477420591</v>
+        <v>-18.92722972409774</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>낫 오프쇼어 파트너스</t>
+        </is>
+      </c>
+      <c r="B40" t="n">
+        <v>30</v>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="D40" t="n">
+        <v>1</v>
+      </c>
+      <c r="E40" t="n">
+        <v>413075.8057155996</v>
+      </c>
+      <c r="F40" t="n">
+        <v>-4439.194284400437</v>
+      </c>
+      <c r="G40" t="n">
+        <v>-1.063241867813237</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>NH투자증권우</t>
+        </is>
+      </c>
+      <c r="B41" t="n">
+        <v>2</v>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="D41" t="n">
+        <v>1</v>
+      </c>
+      <c r="E41" t="n">
+        <v>54700</v>
+      </c>
+      <c r="F41" t="n">
+        <v>100</v>
+      </c>
+      <c r="G41" t="n">
+        <v>0.1831501831501831</v>
       </c>
     </row>
   </sheetData>
@@ -1538,22 +1592,22 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-03-17</t>
+          <t>2026-03-21</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>33078556</v>
+        <v>31036676</v>
       </c>
       <c r="C2" t="n">
-        <v>6010.99</v>
+        <v>12663.38</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2026-03-21T05:01:03</t>
+          <t>2026-03-21T22:46:15</t>
         </is>
       </c>
       <c r="E2" t="n">
-        <v>1488.910034179688</v>
+        <v>1504.829956054688</v>
       </c>
     </row>
   </sheetData>
@@ -1567,7 +1621,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I80"/>
+  <dimension ref="A1:I79"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3056,7 +3110,7 @@
       </c>
       <c r="I40" t="inlineStr">
         <is>
-          <t>2026-03-21T04:57:12</t>
+          <t>2026-03-21T22:46:15</t>
         </is>
       </c>
     </row>
@@ -3068,11 +3122,11 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>AGNC 인베스트먼트</t>
+          <t>대한조선</t>
         </is>
       </c>
       <c r="C41" t="n">
-        <v>700</v>
+        <v>100</v>
       </c>
       <c r="D41" t="inlineStr">
         <is>
@@ -3083,17 +3137,17 @@
         <v>1</v>
       </c>
       <c r="F41" t="n">
-        <v>10270464.45007324</v>
+        <v>9120000</v>
       </c>
       <c r="G41" t="n">
-        <v>-561550.5499267559</v>
+        <v>1907000</v>
       </c>
       <c r="H41" t="n">
-        <v>-5.184174411933109</v>
+        <v>26.43837515596839</v>
       </c>
       <c r="I41" t="inlineStr">
         <is>
-          <t>2026-03-21T04:57:12</t>
+          <t>2026-03-21T22:46:15</t>
         </is>
       </c>
     </row>
@@ -3105,11 +3159,11 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>대한조선</t>
+          <t>프론트라인</t>
         </is>
       </c>
       <c r="C42" t="n">
-        <v>100</v>
+        <v>175</v>
       </c>
       <c r="D42" t="inlineStr">
         <is>
@@ -3120,17 +3174,17 @@
         <v>1</v>
       </c>
       <c r="F42" t="n">
-        <v>9120000</v>
+        <v>8471815.962899337</v>
       </c>
       <c r="G42" t="n">
-        <v>1907000</v>
+        <v>4041951.962899337</v>
       </c>
       <c r="H42" t="n">
-        <v>26.43837515596839</v>
+        <v>91.24325177701475</v>
       </c>
       <c r="I42" t="inlineStr">
         <is>
-          <t>2026-03-21T04:57:12</t>
+          <t>2026-03-21T22:46:15</t>
         </is>
       </c>
     </row>
@@ -3142,11 +3196,11 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>프론트라인</t>
+          <t>시드릴</t>
         </is>
       </c>
       <c r="C43" t="n">
-        <v>175</v>
+        <v>123</v>
       </c>
       <c r="D43" t="inlineStr">
         <is>
@@ -3157,17 +3211,17 @@
         <v>1</v>
       </c>
       <c r="F43" t="n">
-        <v>8471815.962899337</v>
+        <v>8070101.805898919</v>
       </c>
       <c r="G43" t="n">
-        <v>4041951.962899337</v>
+        <v>1619750.805898919</v>
       </c>
       <c r="H43" t="n">
-        <v>91.24325177701475</v>
+        <v>25.11104908707943</v>
       </c>
       <c r="I43" t="inlineStr">
         <is>
-          <t>2026-03-21T04:57:12</t>
+          <t>2026-03-21T22:46:15</t>
         </is>
       </c>
     </row>
@@ -3179,11 +3233,11 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>시드릴</t>
+          <t>세아제강</t>
         </is>
       </c>
       <c r="C44" t="n">
-        <v>123</v>
+        <v>50</v>
       </c>
       <c r="D44" t="inlineStr">
         <is>
@@ -3194,17 +3248,17 @@
         <v>1</v>
       </c>
       <c r="F44" t="n">
-        <v>8070101.805898919</v>
+        <v>7395000</v>
       </c>
       <c r="G44" t="n">
-        <v>1619750.805898919</v>
+        <v>1085000</v>
       </c>
       <c r="H44" t="n">
-        <v>25.11104908707943</v>
+        <v>17.19492868462758</v>
       </c>
       <c r="I44" t="inlineStr">
         <is>
-          <t>2026-03-21T04:57:12</t>
+          <t>2026-03-21T22:46:15</t>
         </is>
       </c>
     </row>
@@ -3216,11 +3270,11 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>세아제강</t>
+          <t>센트러스 에너지</t>
         </is>
       </c>
       <c r="C45" t="n">
-        <v>50</v>
+        <v>25</v>
       </c>
       <c r="D45" t="inlineStr">
         <is>
@@ -3231,17 +3285,17 @@
         <v>1</v>
       </c>
       <c r="F45" t="n">
-        <v>7395000</v>
+        <v>7026050.85816239</v>
       </c>
       <c r="G45" t="n">
-        <v>1085000</v>
+        <v>-406805.1418376099</v>
       </c>
       <c r="H45" t="n">
-        <v>17.19492868462758</v>
+        <v>-5.473066366920198</v>
       </c>
       <c r="I45" t="inlineStr">
         <is>
-          <t>2026-03-21T04:57:12</t>
+          <t>2026-03-21T22:46:15</t>
         </is>
       </c>
     </row>
@@ -3253,11 +3307,11 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>센트러스 에너지</t>
+          <t>트랜스오션</t>
         </is>
       </c>
       <c r="C46" t="n">
-        <v>25</v>
+        <v>750</v>
       </c>
       <c r="D46" t="inlineStr">
         <is>
@@ -3268,17 +3322,17 @@
         <v>1</v>
       </c>
       <c r="F46" t="n">
-        <v>7026050.85816239</v>
+        <v>7020031.5082007</v>
       </c>
       <c r="G46" t="n">
-        <v>-406805.1418376099</v>
+        <v>2892797.5082007</v>
       </c>
       <c r="H46" t="n">
-        <v>-5.473066366920198</v>
+        <v>70.09046514446965</v>
       </c>
       <c r="I46" t="inlineStr">
         <is>
-          <t>2026-03-21T04:57:12</t>
+          <t>2026-03-21T22:46:15</t>
         </is>
       </c>
     </row>
@@ -3290,11 +3344,11 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>트랜스오션</t>
+          <t>노블</t>
         </is>
       </c>
       <c r="C47" t="n">
-        <v>750</v>
+        <v>99</v>
       </c>
       <c r="D47" t="inlineStr">
         <is>
@@ -3305,17 +3359,17 @@
         <v>1</v>
       </c>
       <c r="F47" t="n">
-        <v>7020031.5082007</v>
+        <v>6958769.981090547</v>
       </c>
       <c r="G47" t="n">
-        <v>2892797.5082007</v>
+        <v>3051561.981090547</v>
       </c>
       <c r="H47" t="n">
-        <v>70.09046514446965</v>
+        <v>78.10083264291399</v>
       </c>
       <c r="I47" t="inlineStr">
         <is>
-          <t>2026-03-21T04:57:12</t>
+          <t>2026-03-21T22:46:15</t>
         </is>
       </c>
     </row>
@@ -3327,11 +3381,11 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>노블</t>
+          <t>타이드워터</t>
         </is>
       </c>
       <c r="C48" t="n">
-        <v>99</v>
+        <v>48</v>
       </c>
       <c r="D48" t="inlineStr">
         <is>
@@ -3342,17 +3396,17 @@
         <v>1</v>
       </c>
       <c r="F48" t="n">
-        <v>6958769.981090547</v>
+        <v>5235363.852789983</v>
       </c>
       <c r="G48" t="n">
-        <v>3051561.981090547</v>
+        <v>1510818.852789983</v>
       </c>
       <c r="H48" t="n">
-        <v>78.10083264291399</v>
+        <v>40.56385015592463</v>
       </c>
       <c r="I48" t="inlineStr">
         <is>
-          <t>2026-03-21T04:57:12</t>
+          <t>2026-03-21T22:46:15</t>
         </is>
       </c>
     </row>
@@ -3364,11 +3418,11 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>타이드워터</t>
+          <t>노브</t>
         </is>
       </c>
       <c r="C49" t="n">
-        <v>48</v>
+        <v>185</v>
       </c>
       <c r="D49" t="inlineStr">
         <is>
@@ -3379,17 +3433,17 @@
         <v>1</v>
       </c>
       <c r="F49" t="n">
-        <v>5235363.852789983</v>
+        <v>5200391.447092756</v>
       </c>
       <c r="G49" t="n">
-        <v>1510818.852789983</v>
+        <v>1890383.447092756</v>
       </c>
       <c r="H49" t="n">
-        <v>40.56385015592463</v>
+        <v>57.11114435653194</v>
       </c>
       <c r="I49" t="inlineStr">
         <is>
-          <t>2026-03-21T04:57:12</t>
+          <t>2026-03-21T22:46:15</t>
         </is>
       </c>
     </row>
@@ -3401,11 +3455,11 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>노브</t>
+          <t>TIME 코리아밸류업액티브</t>
         </is>
       </c>
       <c r="C50" t="n">
-        <v>185</v>
+        <v>201</v>
       </c>
       <c r="D50" t="inlineStr">
         <is>
@@ -3416,17 +3470,17 @@
         <v>1</v>
       </c>
       <c r="F50" t="n">
-        <v>5200391.447092756</v>
+        <v>4797870</v>
       </c>
       <c r="G50" t="n">
-        <v>1890383.447092756</v>
+        <v>74073</v>
       </c>
       <c r="H50" t="n">
-        <v>57.11114435653194</v>
+        <v>1.568081778281328</v>
       </c>
       <c r="I50" t="inlineStr">
         <is>
-          <t>2026-03-21T04:57:12</t>
+          <t>2026-03-21T22:46:15</t>
         </is>
       </c>
     </row>
@@ -3438,11 +3492,11 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>TIME 코리아밸류업액티브</t>
+          <t>오케아니스 에코 탱커스</t>
         </is>
       </c>
       <c r="C51" t="n">
-        <v>201</v>
+        <v>65</v>
       </c>
       <c r="D51" t="inlineStr">
         <is>
@@ -3453,17 +3507,17 @@
         <v>1</v>
       </c>
       <c r="F51" t="n">
-        <v>4797870</v>
+        <v>4511179.137784176</v>
       </c>
       <c r="G51" t="n">
-        <v>74073</v>
+        <v>2254819.137784176</v>
       </c>
       <c r="H51" t="n">
-        <v>1.568081778281328</v>
+        <v>99.93171026716374</v>
       </c>
       <c r="I51" t="inlineStr">
         <is>
-          <t>2026-03-21T04:57:12</t>
+          <t>2026-03-21T22:46:15</t>
         </is>
       </c>
     </row>
@@ -3475,11 +3529,11 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>오케아니스 에코 탱커스</t>
+          <t>삼성화재</t>
         </is>
       </c>
       <c r="C52" t="n">
-        <v>65</v>
+        <v>9</v>
       </c>
       <c r="D52" t="inlineStr">
         <is>
@@ -3490,17 +3544,17 @@
         <v>1</v>
       </c>
       <c r="F52" t="n">
-        <v>4511179.137784176</v>
+        <v>4270500</v>
       </c>
       <c r="G52" t="n">
-        <v>2254819.137784176</v>
+        <v>-360500</v>
       </c>
       <c r="H52" t="n">
-        <v>99.93171026716374</v>
+        <v>-7.784495789246384</v>
       </c>
       <c r="I52" t="inlineStr">
         <is>
-          <t>2026-03-21T04:57:12</t>
+          <t>2026-03-21T22:46:15</t>
         </is>
       </c>
     </row>
@@ -3512,11 +3566,11 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>삼성화재</t>
+          <t>동원개발</t>
         </is>
       </c>
       <c r="C53" t="n">
-        <v>9</v>
+        <v>1360</v>
       </c>
       <c r="D53" t="inlineStr">
         <is>
@@ -3527,17 +3581,17 @@
         <v>1</v>
       </c>
       <c r="F53" t="n">
-        <v>4270500</v>
+        <v>4202400</v>
       </c>
       <c r="G53" t="n">
-        <v>-360500</v>
+        <v>465000</v>
       </c>
       <c r="H53" t="n">
-        <v>-7.784495789246384</v>
+        <v>12.44180446299566</v>
       </c>
       <c r="I53" t="inlineStr">
         <is>
-          <t>2026-03-21T04:57:12</t>
+          <t>2026-03-21T22:46:15</t>
         </is>
       </c>
     </row>
@@ -3549,11 +3603,11 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>동원개발</t>
+          <t>HD건설기계</t>
         </is>
       </c>
       <c r="C54" t="n">
-        <v>1360</v>
+        <v>31</v>
       </c>
       <c r="D54" t="inlineStr">
         <is>
@@ -3564,17 +3618,17 @@
         <v>1</v>
       </c>
       <c r="F54" t="n">
-        <v>4202400</v>
+        <v>4123000</v>
       </c>
       <c r="G54" t="n">
-        <v>465000</v>
+        <v>87904</v>
       </c>
       <c r="H54" t="n">
-        <v>12.44180446299566</v>
+        <v>2.178485964150543</v>
       </c>
       <c r="I54" t="inlineStr">
         <is>
-          <t>2026-03-21T04:57:12</t>
+          <t>2026-03-21T22:46:15</t>
         </is>
       </c>
     </row>
@@ -3586,11 +3640,11 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>HD건설기계</t>
+          <t>차코스 에너지 내비게이션</t>
         </is>
       </c>
       <c r="C55" t="n">
-        <v>31</v>
+        <v>75</v>
       </c>
       <c r="D55" t="inlineStr">
         <is>
@@ -3601,17 +3655,17 @@
         <v>1</v>
       </c>
       <c r="F55" t="n">
-        <v>4123000</v>
+        <v>4026924.996845168</v>
       </c>
       <c r="G55" t="n">
-        <v>87904</v>
+        <v>202276.9968451681</v>
       </c>
       <c r="H55" t="n">
-        <v>2.178485964150543</v>
+        <v>5.28877420471552</v>
       </c>
       <c r="I55" t="inlineStr">
         <is>
-          <t>2026-03-21T04:57:12</t>
+          <t>2026-03-21T22:46:15</t>
         </is>
       </c>
     </row>
@@ -3623,11 +3677,11 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>차코스 에너지 내비게이션</t>
+          <t>넥스틸</t>
         </is>
       </c>
       <c r="C56" t="n">
-        <v>75</v>
+        <v>300</v>
       </c>
       <c r="D56" t="inlineStr">
         <is>
@@ -3638,17 +3692,17 @@
         <v>1</v>
       </c>
       <c r="F56" t="n">
-        <v>4026924.996845168</v>
+        <v>3771000</v>
       </c>
       <c r="G56" t="n">
-        <v>202276.9968451681</v>
+        <v>521000</v>
       </c>
       <c r="H56" t="n">
-        <v>5.28877420471552</v>
+        <v>16.03076923076923</v>
       </c>
       <c r="I56" t="inlineStr">
         <is>
-          <t>2026-03-21T04:57:12</t>
+          <t>2026-03-21T22:46:15</t>
         </is>
       </c>
     </row>
@@ -3660,11 +3714,11 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>넥스틸</t>
+          <t>피바디 에너지</t>
         </is>
       </c>
       <c r="C57" t="n">
-        <v>300</v>
+        <v>65</v>
       </c>
       <c r="D57" t="inlineStr">
         <is>
@@ -3675,17 +3729,17 @@
         <v>1</v>
       </c>
       <c r="F57" t="n">
-        <v>3771000</v>
+        <v>3649438.50225304</v>
       </c>
       <c r="G57" t="n">
-        <v>521000</v>
+        <v>2178666.50225304</v>
       </c>
       <c r="H57" t="n">
-        <v>16.03076923076923</v>
+        <v>148.1308117269733</v>
       </c>
       <c r="I57" t="inlineStr">
         <is>
-          <t>2026-03-21T04:57:12</t>
+          <t>2026-03-21T22:46:15</t>
         </is>
       </c>
     </row>
@@ -3697,11 +3751,11 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>피바디 에너지</t>
+          <t>현대제철</t>
         </is>
       </c>
       <c r="C58" t="n">
-        <v>65</v>
+        <v>80</v>
       </c>
       <c r="D58" t="inlineStr">
         <is>
@@ -3712,17 +3766,17 @@
         <v>1</v>
       </c>
       <c r="F58" t="n">
-        <v>3649438.50225304</v>
+        <v>2996000</v>
       </c>
       <c r="G58" t="n">
-        <v>2178666.50225304</v>
+        <v>-182000</v>
       </c>
       <c r="H58" t="n">
-        <v>148.1308117269733</v>
+        <v>-5.726872246696035</v>
       </c>
       <c r="I58" t="inlineStr">
         <is>
-          <t>2026-03-21T04:57:12</t>
+          <t>2026-03-21T22:46:15</t>
         </is>
       </c>
     </row>
@@ -3734,11 +3788,11 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>현대제철</t>
+          <t>더치 브로스</t>
         </is>
       </c>
       <c r="C59" t="n">
-        <v>80</v>
+        <v>39</v>
       </c>
       <c r="D59" t="inlineStr">
         <is>
@@ -3749,17 +3803,17 @@
         <v>1</v>
       </c>
       <c r="F59" t="n">
-        <v>2996000</v>
+        <v>2934418.414306641</v>
       </c>
       <c r="G59" t="n">
-        <v>-182000</v>
+        <v>-256226.5856933594</v>
       </c>
       <c r="H59" t="n">
-        <v>-5.726872246696035</v>
+        <v>-8.030557636257226</v>
       </c>
       <c r="I59" t="inlineStr">
         <is>
-          <t>2026-03-21T04:57:12</t>
+          <t>2026-03-21T22:46:15</t>
         </is>
       </c>
     </row>
@@ -3771,11 +3825,11 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>더치 브로스</t>
+          <t>휴스틸</t>
         </is>
       </c>
       <c r="C60" t="n">
-        <v>39</v>
+        <v>500</v>
       </c>
       <c r="D60" t="inlineStr">
         <is>
@@ -3786,17 +3840,17 @@
         <v>1</v>
       </c>
       <c r="F60" t="n">
-        <v>2934418.414306641</v>
+        <v>2750000</v>
       </c>
       <c r="G60" t="n">
-        <v>-256226.5856933594</v>
+        <v>471390</v>
       </c>
       <c r="H60" t="n">
-        <v>-8.030557636257226</v>
+        <v>20.68761218462133</v>
       </c>
       <c r="I60" t="inlineStr">
         <is>
-          <t>2026-03-21T04:57:12</t>
+          <t>2026-03-21T22:46:15</t>
         </is>
       </c>
     </row>
@@ -3808,11 +3862,11 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>휴스틸</t>
+          <t>DL이앤씨</t>
         </is>
       </c>
       <c r="C61" t="n">
-        <v>500</v>
+        <v>40</v>
       </c>
       <c r="D61" t="inlineStr">
         <is>
@@ -3823,17 +3877,17 @@
         <v>1</v>
       </c>
       <c r="F61" t="n">
-        <v>2750000</v>
+        <v>2696000</v>
       </c>
       <c r="G61" t="n">
-        <v>471390</v>
+        <v>990500</v>
       </c>
       <c r="H61" t="n">
-        <v>20.68761218462133</v>
+        <v>58.07681031955438</v>
       </c>
       <c r="I61" t="inlineStr">
         <is>
-          <t>2026-03-21T04:57:12</t>
+          <t>2026-03-21T22:46:15</t>
         </is>
       </c>
     </row>
@@ -3845,11 +3899,11 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>DL이앤씨</t>
+          <t>KoAct 코스닥액티브</t>
         </is>
       </c>
       <c r="C62" t="n">
-        <v>40</v>
+        <v>200</v>
       </c>
       <c r="D62" t="inlineStr">
         <is>
@@ -3860,17 +3914,17 @@
         <v>1</v>
       </c>
       <c r="F62" t="n">
-        <v>2696000</v>
+        <v>2582000</v>
       </c>
       <c r="G62" t="n">
-        <v>990500</v>
+        <v>-120000</v>
       </c>
       <c r="H62" t="n">
-        <v>58.07681031955438</v>
+        <v>-4.441154700222058</v>
       </c>
       <c r="I62" t="inlineStr">
         <is>
-          <t>2026-03-21T04:57:12</t>
+          <t>2026-03-21T22:46:15</t>
         </is>
       </c>
     </row>
@@ -3882,11 +3936,11 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>KoAct 코스닥액티브</t>
+          <t>대신증권</t>
         </is>
       </c>
       <c r="C63" t="n">
-        <v>200</v>
+        <v>55</v>
       </c>
       <c r="D63" t="inlineStr">
         <is>
@@ -3897,17 +3951,17 @@
         <v>1</v>
       </c>
       <c r="F63" t="n">
-        <v>2582000</v>
+        <v>2219250</v>
       </c>
       <c r="G63" t="n">
-        <v>-120000</v>
+        <v>509749</v>
       </c>
       <c r="H63" t="n">
-        <v>-4.441154700222058</v>
+        <v>29.81858448752005</v>
       </c>
       <c r="I63" t="inlineStr">
         <is>
-          <t>2026-03-21T04:57:12</t>
+          <t>2026-03-21T22:46:15</t>
         </is>
       </c>
     </row>
@@ -3919,11 +3973,11 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>대신증권</t>
+          <t>발레로 에너지</t>
         </is>
       </c>
       <c r="C64" t="n">
-        <v>55</v>
+        <v>6</v>
       </c>
       <c r="D64" t="inlineStr">
         <is>
@@ -3934,17 +3988,17 @@
         <v>1</v>
       </c>
       <c r="F64" t="n">
-        <v>2219250</v>
+        <v>2165691.085066516</v>
       </c>
       <c r="G64" t="n">
-        <v>509749</v>
+        <v>101701.085066516</v>
       </c>
       <c r="H64" t="n">
-        <v>29.81858448752005</v>
+        <v>4.927402025519307</v>
       </c>
       <c r="I64" t="inlineStr">
         <is>
-          <t>2026-03-21T04:57:12</t>
+          <t>2026-03-21T22:46:15</t>
         </is>
       </c>
     </row>
@@ -3956,11 +4010,11 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>발레로 에너지</t>
+          <t>미창석유</t>
         </is>
       </c>
       <c r="C65" t="n">
-        <v>6</v>
+        <v>18</v>
       </c>
       <c r="D65" t="inlineStr">
         <is>
@@ -3971,17 +4025,17 @@
         <v>1</v>
       </c>
       <c r="F65" t="n">
-        <v>2165691.085066516</v>
+        <v>2097000</v>
       </c>
       <c r="G65" t="n">
-        <v>101701.085066516</v>
+        <v>-295200</v>
       </c>
       <c r="H65" t="n">
-        <v>4.927402025519307</v>
+        <v>-12.34010534236268</v>
       </c>
       <c r="I65" t="inlineStr">
         <is>
-          <t>2026-03-21T04:57:12</t>
+          <t>2026-03-21T22:46:15</t>
         </is>
       </c>
     </row>
@@ -3993,7 +4047,7 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>미창석유</t>
+          <t>하나금융지주</t>
         </is>
       </c>
       <c r="C66" t="n">
@@ -4008,17 +4062,17 @@
         <v>1</v>
       </c>
       <c r="F66" t="n">
-        <v>2097000</v>
+        <v>2037600</v>
       </c>
       <c r="G66" t="n">
-        <v>-295200</v>
+        <v>12200</v>
       </c>
       <c r="H66" t="n">
-        <v>-12.34010534236268</v>
+        <v>0.6023501530561864</v>
       </c>
       <c r="I66" t="inlineStr">
         <is>
-          <t>2026-03-21T04:57:12</t>
+          <t>2026-03-21T22:46:15</t>
         </is>
       </c>
     </row>
@@ -4030,11 +4084,11 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>하나금융지주</t>
+          <t>대창단조</t>
         </is>
       </c>
       <c r="C67" t="n">
-        <v>18</v>
+        <v>300</v>
       </c>
       <c r="D67" t="inlineStr">
         <is>
@@ -4045,17 +4099,17 @@
         <v>1</v>
       </c>
       <c r="F67" t="n">
-        <v>2037600</v>
+        <v>2004000</v>
       </c>
       <c r="G67" t="n">
-        <v>12200</v>
+        <v>-54000</v>
       </c>
       <c r="H67" t="n">
-        <v>0.6023501530561864</v>
+        <v>-2.623906705539359</v>
       </c>
       <c r="I67" t="inlineStr">
         <is>
-          <t>2026-03-21T04:57:12</t>
+          <t>2026-03-21T22:46:15</t>
         </is>
       </c>
     </row>
@@ -4067,11 +4121,11 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>대창단조</t>
+          <t>동방</t>
         </is>
       </c>
       <c r="C68" t="n">
-        <v>300</v>
+        <v>681</v>
       </c>
       <c r="D68" t="inlineStr">
         <is>
@@ -4082,17 +4136,17 @@
         <v>1</v>
       </c>
       <c r="F68" t="n">
-        <v>2004000</v>
+        <v>1995330</v>
       </c>
       <c r="G68" t="n">
-        <v>-54000</v>
+        <v>23829</v>
       </c>
       <c r="H68" t="n">
-        <v>-2.623906705539359</v>
+        <v>1.208672985709873</v>
       </c>
       <c r="I68" t="inlineStr">
         <is>
-          <t>2026-03-21T04:57:12</t>
+          <t>2026-03-21T22:46:15</t>
         </is>
       </c>
     </row>
@@ -4104,11 +4158,11 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>동방</t>
+          <t>스타 벌크 캐리어스</t>
         </is>
       </c>
       <c r="C69" t="n">
-        <v>681</v>
+        <v>50</v>
       </c>
       <c r="D69" t="inlineStr">
         <is>
@@ -4119,17 +4173,17 @@
         <v>1</v>
       </c>
       <c r="F69" t="n">
-        <v>1995330</v>
+        <v>1680142.640194588</v>
       </c>
       <c r="G69" t="n">
-        <v>23829</v>
+        <v>365789.6401945879</v>
       </c>
       <c r="H69" t="n">
-        <v>1.208672985709873</v>
+        <v>27.83039565433242</v>
       </c>
       <c r="I69" t="inlineStr">
         <is>
-          <t>2026-03-21T04:57:12</t>
+          <t>2026-03-21T22:46:15</t>
         </is>
       </c>
     </row>
@@ -4141,7 +4195,7 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>스타 벌크 캐리어스</t>
+          <t>케이씨</t>
         </is>
       </c>
       <c r="C70" t="n">
@@ -4156,17 +4210,17 @@
         <v>1</v>
       </c>
       <c r="F70" t="n">
-        <v>1680142.640194588</v>
+        <v>1670000</v>
       </c>
       <c r="G70" t="n">
-        <v>365789.6401945879</v>
+        <v>20500</v>
       </c>
       <c r="H70" t="n">
-        <v>27.83039565433242</v>
+        <v>1.242800848742043</v>
       </c>
       <c r="I70" t="inlineStr">
         <is>
-          <t>2026-03-21T04:57:12</t>
+          <t>2026-03-21T22:46:15</t>
         </is>
       </c>
     </row>
@@ -4178,11 +4232,11 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>케이씨</t>
+          <t>유나이티드헬스 그룹</t>
         </is>
       </c>
       <c r="C71" t="n">
-        <v>50</v>
+        <v>4</v>
       </c>
       <c r="D71" t="inlineStr">
         <is>
@@ -4193,17 +4247,17 @@
         <v>1</v>
       </c>
       <c r="F71" t="n">
-        <v>1670000</v>
+        <v>1658864.328313038</v>
       </c>
       <c r="G71" t="n">
-        <v>20500</v>
+        <v>-35591.67168696248</v>
       </c>
       <c r="H71" t="n">
-        <v>1.242800848742043</v>
+        <v>-2.100477774988697</v>
       </c>
       <c r="I71" t="inlineStr">
         <is>
-          <t>2026-03-21T04:57:12</t>
+          <t>2026-03-21T22:46:15</t>
         </is>
       </c>
     </row>
@@ -4215,11 +4269,11 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>유나이티드헬스 그룹</t>
+          <t>텍사스 퍼시픽 랜드</t>
         </is>
       </c>
       <c r="C72" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D72" t="inlineStr">
         <is>
@@ -4230,17 +4284,17 @@
         <v>1</v>
       </c>
       <c r="F72" t="n">
-        <v>1658864.328313038</v>
+        <v>1563247.374122903</v>
       </c>
       <c r="G72" t="n">
-        <v>-35591.67168696248</v>
+        <v>-14646.62587709725</v>
       </c>
       <c r="H72" t="n">
-        <v>-2.100477774988697</v>
+        <v>-0.9282388979929735</v>
       </c>
       <c r="I72" t="inlineStr">
         <is>
-          <t>2026-03-21T04:57:12</t>
+          <t>2026-03-21T22:46:15</t>
         </is>
       </c>
     </row>
@@ -4252,11 +4306,11 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>텍사스 퍼시픽 랜드</t>
+          <t>LX인터내셔널</t>
         </is>
       </c>
       <c r="C73" t="n">
-        <v>2</v>
+        <v>20</v>
       </c>
       <c r="D73" t="inlineStr">
         <is>
@@ -4267,17 +4321,17 @@
         <v>1</v>
       </c>
       <c r="F73" t="n">
-        <v>1563247.374122903</v>
+        <v>943000</v>
       </c>
       <c r="G73" t="n">
-        <v>-14646.62587709725</v>
+        <v>4000</v>
       </c>
       <c r="H73" t="n">
-        <v>-0.9282388979929735</v>
+        <v>0.4259850905218318</v>
       </c>
       <c r="I73" t="inlineStr">
         <is>
-          <t>2026-03-21T04:57:12</t>
+          <t>2026-03-21T22:46:15</t>
         </is>
       </c>
     </row>
@@ -4289,11 +4343,11 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>LX인터내셔널</t>
+          <t>삼성생명</t>
         </is>
       </c>
       <c r="C74" t="n">
-        <v>20</v>
+        <v>4</v>
       </c>
       <c r="D74" t="inlineStr">
         <is>
@@ -4304,17 +4358,17 @@
         <v>1</v>
       </c>
       <c r="F74" t="n">
-        <v>943000</v>
+        <v>926000</v>
       </c>
       <c r="G74" t="n">
-        <v>4000</v>
+        <v>93000</v>
       </c>
       <c r="H74" t="n">
-        <v>0.4259850905218318</v>
+        <v>11.16446578631453</v>
       </c>
       <c r="I74" t="inlineStr">
         <is>
-          <t>2026-03-21T04:57:12</t>
+          <t>2026-03-21T22:46:15</t>
         </is>
       </c>
     </row>
@@ -4326,11 +4380,11 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>삼성생명</t>
+          <t>비에이치아이</t>
         </is>
       </c>
       <c r="C75" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="D75" t="inlineStr">
         <is>
@@ -4341,17 +4395,17 @@
         <v>1</v>
       </c>
       <c r="F75" t="n">
-        <v>926000</v>
+        <v>876000</v>
       </c>
       <c r="G75" t="n">
-        <v>93000</v>
+        <v>210885</v>
       </c>
       <c r="H75" t="n">
-        <v>11.16446578631453</v>
+        <v>31.70654698811484</v>
       </c>
       <c r="I75" t="inlineStr">
         <is>
-          <t>2026-03-21T04:57:12</t>
+          <t>2026-03-21T22:46:15</t>
         </is>
       </c>
     </row>
@@ -4363,11 +4417,11 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>비에이치아이</t>
+          <t>하프니아</t>
         </is>
       </c>
       <c r="C76" t="n">
-        <v>8</v>
+        <v>80</v>
       </c>
       <c r="D76" t="inlineStr">
         <is>
@@ -4378,17 +4432,17 @@
         <v>1</v>
       </c>
       <c r="F76" t="n">
-        <v>876000</v>
+        <v>842704.775390625</v>
       </c>
       <c r="G76" t="n">
-        <v>210885</v>
+        <v>216973.775390625</v>
       </c>
       <c r="H76" t="n">
-        <v>31.70654698811484</v>
+        <v>34.67524789256486</v>
       </c>
       <c r="I76" t="inlineStr">
         <is>
-          <t>2026-03-21T04:57:12</t>
+          <t>2026-03-21T22:46:15</t>
         </is>
       </c>
     </row>
@@ -4400,11 +4454,11 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>하프니아</t>
+          <t>클리블랜드 클리프스</t>
         </is>
       </c>
       <c r="C77" t="n">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="D77" t="inlineStr">
         <is>
@@ -4415,17 +4469,17 @@
         <v>1</v>
       </c>
       <c r="F77" t="n">
-        <v>842704.775390625</v>
+        <v>823743.9360268187</v>
       </c>
       <c r="G77" t="n">
-        <v>216973.775390625</v>
+        <v>-192311.0639731813</v>
       </c>
       <c r="H77" t="n">
-        <v>34.67524789256486</v>
+        <v>-18.92722972409774</v>
       </c>
       <c r="I77" t="inlineStr">
         <is>
-          <t>2026-03-21T04:57:12</t>
+          <t>2026-03-21T22:46:15</t>
         </is>
       </c>
     </row>
@@ -4437,11 +4491,11 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>클리블랜드 클리프스</t>
+          <t>낫 오프쇼어 파트너스</t>
         </is>
       </c>
       <c r="C78" t="n">
-        <v>70</v>
+        <v>30</v>
       </c>
       <c r="D78" t="inlineStr">
         <is>
@@ -4452,17 +4506,17 @@
         <v>1</v>
       </c>
       <c r="F78" t="n">
-        <v>823743.9360268187</v>
+        <v>413075.8057155996</v>
       </c>
       <c r="G78" t="n">
-        <v>-192311.0639731813</v>
+        <v>-4439.194284400437</v>
       </c>
       <c r="H78" t="n">
-        <v>-18.92722972409774</v>
+        <v>-1.063241867813237</v>
       </c>
       <c r="I78" t="inlineStr">
         <is>
-          <t>2026-03-21T04:57:12</t>
+          <t>2026-03-21T22:46:15</t>
         </is>
       </c>
     </row>
@@ -4474,11 +4528,11 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>낫 오프쇼어 파트너스</t>
+          <t>NH투자증권우</t>
         </is>
       </c>
       <c r="C79" t="n">
-        <v>30</v>
+        <v>2</v>
       </c>
       <c r="D79" t="inlineStr">
         <is>
@@ -4489,54 +4543,17 @@
         <v>1</v>
       </c>
       <c r="F79" t="n">
-        <v>413075.8057155996</v>
+        <v>54700</v>
       </c>
       <c r="G79" t="n">
-        <v>-4439.194284400437</v>
+        <v>100</v>
       </c>
       <c r="H79" t="n">
-        <v>-1.063241867813237</v>
+        <v>0.1831501831501831</v>
       </c>
       <c r="I79" t="inlineStr">
         <is>
-          <t>2026-03-21T04:57:12</t>
-        </is>
-      </c>
-    </row>
-    <row r="80">
-      <c r="A80" t="inlineStr">
-        <is>
-          <t>2026-03-21</t>
-        </is>
-      </c>
-      <c r="B80" t="inlineStr">
-        <is>
-          <t>NH투자증권우</t>
-        </is>
-      </c>
-      <c r="C80" t="n">
-        <v>2</v>
-      </c>
-      <c r="D80" t="inlineStr">
-        <is>
-          <t>KRW</t>
-        </is>
-      </c>
-      <c r="E80" t="n">
-        <v>1</v>
-      </c>
-      <c r="F80" t="n">
-        <v>54700</v>
-      </c>
-      <c r="G80" t="n">
-        <v>100</v>
-      </c>
-      <c r="H80" t="n">
-        <v>0.1831501831501831</v>
-      </c>
-      <c r="I80" t="inlineStr">
-        <is>
-          <t>2026-03-21T04:57:12</t>
+          <t>2026-03-21T22:46:15</t>
         </is>
       </c>
     </row>
@@ -4623,7 +4640,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>2026-03-21T04:57:12</t>
+          <t>2026-03-21T22:46:15</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: portfolio snapshot 2026-03-21 (2026-03-21T22:46:54)
</commit_message>
<xml_diff>
--- a/portfolio_auto.xlsx
+++ b/portfolio_auto.xlsx
@@ -1603,7 +1603,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2026-03-21T22:46:15</t>
+          <t>2026-03-21T22:46:54</t>
         </is>
       </c>
       <c r="E2" t="n">
@@ -3110,7 +3110,7 @@
       </c>
       <c r="I40" t="inlineStr">
         <is>
-          <t>2026-03-21T22:46:15</t>
+          <t>2026-03-21T22:46:54</t>
         </is>
       </c>
     </row>
@@ -3147,7 +3147,7 @@
       </c>
       <c r="I41" t="inlineStr">
         <is>
-          <t>2026-03-21T22:46:15</t>
+          <t>2026-03-21T22:46:54</t>
         </is>
       </c>
     </row>
@@ -3184,7 +3184,7 @@
       </c>
       <c r="I42" t="inlineStr">
         <is>
-          <t>2026-03-21T22:46:15</t>
+          <t>2026-03-21T22:46:54</t>
         </is>
       </c>
     </row>
@@ -3221,7 +3221,7 @@
       </c>
       <c r="I43" t="inlineStr">
         <is>
-          <t>2026-03-21T22:46:15</t>
+          <t>2026-03-21T22:46:54</t>
         </is>
       </c>
     </row>
@@ -3258,7 +3258,7 @@
       </c>
       <c r="I44" t="inlineStr">
         <is>
-          <t>2026-03-21T22:46:15</t>
+          <t>2026-03-21T22:46:54</t>
         </is>
       </c>
     </row>
@@ -3295,7 +3295,7 @@
       </c>
       <c r="I45" t="inlineStr">
         <is>
-          <t>2026-03-21T22:46:15</t>
+          <t>2026-03-21T22:46:54</t>
         </is>
       </c>
     </row>
@@ -3332,7 +3332,7 @@
       </c>
       <c r="I46" t="inlineStr">
         <is>
-          <t>2026-03-21T22:46:15</t>
+          <t>2026-03-21T22:46:54</t>
         </is>
       </c>
     </row>
@@ -3369,7 +3369,7 @@
       </c>
       <c r="I47" t="inlineStr">
         <is>
-          <t>2026-03-21T22:46:15</t>
+          <t>2026-03-21T22:46:54</t>
         </is>
       </c>
     </row>
@@ -3406,7 +3406,7 @@
       </c>
       <c r="I48" t="inlineStr">
         <is>
-          <t>2026-03-21T22:46:15</t>
+          <t>2026-03-21T22:46:54</t>
         </is>
       </c>
     </row>
@@ -3443,7 +3443,7 @@
       </c>
       <c r="I49" t="inlineStr">
         <is>
-          <t>2026-03-21T22:46:15</t>
+          <t>2026-03-21T22:46:54</t>
         </is>
       </c>
     </row>
@@ -3480,7 +3480,7 @@
       </c>
       <c r="I50" t="inlineStr">
         <is>
-          <t>2026-03-21T22:46:15</t>
+          <t>2026-03-21T22:46:54</t>
         </is>
       </c>
     </row>
@@ -3517,7 +3517,7 @@
       </c>
       <c r="I51" t="inlineStr">
         <is>
-          <t>2026-03-21T22:46:15</t>
+          <t>2026-03-21T22:46:54</t>
         </is>
       </c>
     </row>
@@ -3554,7 +3554,7 @@
       </c>
       <c r="I52" t="inlineStr">
         <is>
-          <t>2026-03-21T22:46:15</t>
+          <t>2026-03-21T22:46:54</t>
         </is>
       </c>
     </row>
@@ -3591,7 +3591,7 @@
       </c>
       <c r="I53" t="inlineStr">
         <is>
-          <t>2026-03-21T22:46:15</t>
+          <t>2026-03-21T22:46:54</t>
         </is>
       </c>
     </row>
@@ -3628,7 +3628,7 @@
       </c>
       <c r="I54" t="inlineStr">
         <is>
-          <t>2026-03-21T22:46:15</t>
+          <t>2026-03-21T22:46:54</t>
         </is>
       </c>
     </row>
@@ -3665,7 +3665,7 @@
       </c>
       <c r="I55" t="inlineStr">
         <is>
-          <t>2026-03-21T22:46:15</t>
+          <t>2026-03-21T22:46:54</t>
         </is>
       </c>
     </row>
@@ -3702,7 +3702,7 @@
       </c>
       <c r="I56" t="inlineStr">
         <is>
-          <t>2026-03-21T22:46:15</t>
+          <t>2026-03-21T22:46:54</t>
         </is>
       </c>
     </row>
@@ -3739,7 +3739,7 @@
       </c>
       <c r="I57" t="inlineStr">
         <is>
-          <t>2026-03-21T22:46:15</t>
+          <t>2026-03-21T22:46:54</t>
         </is>
       </c>
     </row>
@@ -3776,7 +3776,7 @@
       </c>
       <c r="I58" t="inlineStr">
         <is>
-          <t>2026-03-21T22:46:15</t>
+          <t>2026-03-21T22:46:54</t>
         </is>
       </c>
     </row>
@@ -3813,7 +3813,7 @@
       </c>
       <c r="I59" t="inlineStr">
         <is>
-          <t>2026-03-21T22:46:15</t>
+          <t>2026-03-21T22:46:54</t>
         </is>
       </c>
     </row>
@@ -3850,7 +3850,7 @@
       </c>
       <c r="I60" t="inlineStr">
         <is>
-          <t>2026-03-21T22:46:15</t>
+          <t>2026-03-21T22:46:54</t>
         </is>
       </c>
     </row>
@@ -3887,7 +3887,7 @@
       </c>
       <c r="I61" t="inlineStr">
         <is>
-          <t>2026-03-21T22:46:15</t>
+          <t>2026-03-21T22:46:54</t>
         </is>
       </c>
     </row>
@@ -3924,7 +3924,7 @@
       </c>
       <c r="I62" t="inlineStr">
         <is>
-          <t>2026-03-21T22:46:15</t>
+          <t>2026-03-21T22:46:54</t>
         </is>
       </c>
     </row>
@@ -3961,7 +3961,7 @@
       </c>
       <c r="I63" t="inlineStr">
         <is>
-          <t>2026-03-21T22:46:15</t>
+          <t>2026-03-21T22:46:54</t>
         </is>
       </c>
     </row>
@@ -3998,7 +3998,7 @@
       </c>
       <c r="I64" t="inlineStr">
         <is>
-          <t>2026-03-21T22:46:15</t>
+          <t>2026-03-21T22:46:54</t>
         </is>
       </c>
     </row>
@@ -4035,7 +4035,7 @@
       </c>
       <c r="I65" t="inlineStr">
         <is>
-          <t>2026-03-21T22:46:15</t>
+          <t>2026-03-21T22:46:54</t>
         </is>
       </c>
     </row>
@@ -4072,7 +4072,7 @@
       </c>
       <c r="I66" t="inlineStr">
         <is>
-          <t>2026-03-21T22:46:15</t>
+          <t>2026-03-21T22:46:54</t>
         </is>
       </c>
     </row>
@@ -4109,7 +4109,7 @@
       </c>
       <c r="I67" t="inlineStr">
         <is>
-          <t>2026-03-21T22:46:15</t>
+          <t>2026-03-21T22:46:54</t>
         </is>
       </c>
     </row>
@@ -4146,7 +4146,7 @@
       </c>
       <c r="I68" t="inlineStr">
         <is>
-          <t>2026-03-21T22:46:15</t>
+          <t>2026-03-21T22:46:54</t>
         </is>
       </c>
     </row>
@@ -4183,7 +4183,7 @@
       </c>
       <c r="I69" t="inlineStr">
         <is>
-          <t>2026-03-21T22:46:15</t>
+          <t>2026-03-21T22:46:54</t>
         </is>
       </c>
     </row>
@@ -4220,7 +4220,7 @@
       </c>
       <c r="I70" t="inlineStr">
         <is>
-          <t>2026-03-21T22:46:15</t>
+          <t>2026-03-21T22:46:54</t>
         </is>
       </c>
     </row>
@@ -4257,7 +4257,7 @@
       </c>
       <c r="I71" t="inlineStr">
         <is>
-          <t>2026-03-21T22:46:15</t>
+          <t>2026-03-21T22:46:54</t>
         </is>
       </c>
     </row>
@@ -4294,7 +4294,7 @@
       </c>
       <c r="I72" t="inlineStr">
         <is>
-          <t>2026-03-21T22:46:15</t>
+          <t>2026-03-21T22:46:54</t>
         </is>
       </c>
     </row>
@@ -4331,7 +4331,7 @@
       </c>
       <c r="I73" t="inlineStr">
         <is>
-          <t>2026-03-21T22:46:15</t>
+          <t>2026-03-21T22:46:54</t>
         </is>
       </c>
     </row>
@@ -4368,7 +4368,7 @@
       </c>
       <c r="I74" t="inlineStr">
         <is>
-          <t>2026-03-21T22:46:15</t>
+          <t>2026-03-21T22:46:54</t>
         </is>
       </c>
     </row>
@@ -4405,7 +4405,7 @@
       </c>
       <c r="I75" t="inlineStr">
         <is>
-          <t>2026-03-21T22:46:15</t>
+          <t>2026-03-21T22:46:54</t>
         </is>
       </c>
     </row>
@@ -4442,7 +4442,7 @@
       </c>
       <c r="I76" t="inlineStr">
         <is>
-          <t>2026-03-21T22:46:15</t>
+          <t>2026-03-21T22:46:54</t>
         </is>
       </c>
     </row>
@@ -4479,7 +4479,7 @@
       </c>
       <c r="I77" t="inlineStr">
         <is>
-          <t>2026-03-21T22:46:15</t>
+          <t>2026-03-21T22:46:54</t>
         </is>
       </c>
     </row>
@@ -4516,7 +4516,7 @@
       </c>
       <c r="I78" t="inlineStr">
         <is>
-          <t>2026-03-21T22:46:15</t>
+          <t>2026-03-21T22:46:54</t>
         </is>
       </c>
     </row>
@@ -4553,7 +4553,7 @@
       </c>
       <c r="I79" t="inlineStr">
         <is>
-          <t>2026-03-21T22:46:15</t>
+          <t>2026-03-21T22:46:54</t>
         </is>
       </c>
     </row>
@@ -4640,7 +4640,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>2026-03-21T22:46:15</t>
+          <t>2026-03-21T22:46:54</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: portfolio snapshot 2026-03-22 (2026-03-21T22:47:58)
</commit_message>
<xml_diff>
--- a/portfolio_auto.xlsx
+++ b/portfolio_auto.xlsx
@@ -489,10 +489,10 @@
         <v>13579584.97235231</v>
       </c>
       <c r="F2" t="n">
-        <v>1473035.972352311</v>
+        <v>1473035.972352313</v>
       </c>
       <c r="G2" t="n">
-        <v>12.16726560436265</v>
+        <v>12.16726560436267</v>
       </c>
     </row>
     <row r="3">
@@ -681,7 +681,7 @@
         <v>3051561.981090547</v>
       </c>
       <c r="G9" t="n">
-        <v>78.10083264291399</v>
+        <v>78.10083264291401</v>
       </c>
     </row>
     <row r="10">
@@ -789,7 +789,7 @@
         <v>2254819.137784176</v>
       </c>
       <c r="G13" t="n">
-        <v>99.93171026716374</v>
+        <v>99.93171026716378</v>
       </c>
     </row>
     <row r="14">
@@ -1002,10 +1002,10 @@
         <v>2934418.414306641</v>
       </c>
       <c r="F21" t="n">
-        <v>-256226.5856933594</v>
+        <v>-256226.5856933598</v>
       </c>
       <c r="G21" t="n">
-        <v>-8.030557636257226</v>
+        <v>-8.030557636257239</v>
       </c>
     </row>
     <row r="22">
@@ -1272,10 +1272,10 @@
         <v>1680142.640194588</v>
       </c>
       <c r="F31" t="n">
-        <v>365789.6401945879</v>
+        <v>365789.6401945876</v>
       </c>
       <c r="G31" t="n">
-        <v>27.83039565433242</v>
+        <v>27.8303956543324</v>
       </c>
     </row>
     <row r="32">
@@ -1326,10 +1326,10 @@
         <v>1658864.328313038</v>
       </c>
       <c r="F33" t="n">
-        <v>-35591.67168696248</v>
+        <v>-35591.67168696271</v>
       </c>
       <c r="G33" t="n">
-        <v>-2.100477774988697</v>
+        <v>-2.10047777498871</v>
       </c>
     </row>
     <row r="34">
@@ -1353,10 +1353,10 @@
         <v>1563247.374122903</v>
       </c>
       <c r="F34" t="n">
-        <v>-14646.62587709725</v>
+        <v>-14646.62587709748</v>
       </c>
       <c r="G34" t="n">
-        <v>-0.9282388979929735</v>
+        <v>-0.9282388979929881</v>
       </c>
     </row>
     <row r="35">
@@ -1515,10 +1515,10 @@
         <v>413075.8057155996</v>
       </c>
       <c r="F40" t="n">
-        <v>-4439.194284400437</v>
+        <v>-4439.194284400495</v>
       </c>
       <c r="G40" t="n">
-        <v>-1.063241867813237</v>
+        <v>-1.063241867813251</v>
       </c>
     </row>
     <row r="41">
@@ -1592,7 +1592,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-03-21</t>
+          <t>2026-03-22</t>
         </is>
       </c>
       <c r="B2" t="n">
@@ -1603,7 +1603,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2026-03-21T22:46:54</t>
+          <t>2026-03-21T22:47:57</t>
         </is>
       </c>
       <c r="E2" t="n">
@@ -1621,7 +1621,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I79"/>
+  <dimension ref="A1:I119"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4554,6 +4554,1486 @@
       <c r="I79" t="inlineStr">
         <is>
           <t>2026-03-21T22:46:54</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>2026-03-22</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>페트로브라스 (ADR)</t>
+        </is>
+      </c>
+      <c r="C80" t="n">
+        <v>480</v>
+      </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E80" t="n">
+        <v>1</v>
+      </c>
+      <c r="F80" t="n">
+        <v>13579584.97235231</v>
+      </c>
+      <c r="G80" t="n">
+        <v>1473035.972352313</v>
+      </c>
+      <c r="H80" t="n">
+        <v>12.16726560436267</v>
+      </c>
+      <c r="I80" t="inlineStr">
+        <is>
+          <t>2026-03-21T22:47:57</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>2026-03-22</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>대한조선</t>
+        </is>
+      </c>
+      <c r="C81" t="n">
+        <v>100</v>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E81" t="n">
+        <v>1</v>
+      </c>
+      <c r="F81" t="n">
+        <v>9120000</v>
+      </c>
+      <c r="G81" t="n">
+        <v>1907000</v>
+      </c>
+      <c r="H81" t="n">
+        <v>26.43837515596839</v>
+      </c>
+      <c r="I81" t="inlineStr">
+        <is>
+          <t>2026-03-21T22:47:57</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>2026-03-22</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>프론트라인</t>
+        </is>
+      </c>
+      <c r="C82" t="n">
+        <v>175</v>
+      </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E82" t="n">
+        <v>1</v>
+      </c>
+      <c r="F82" t="n">
+        <v>8471815.962899337</v>
+      </c>
+      <c r="G82" t="n">
+        <v>4041951.962899337</v>
+      </c>
+      <c r="H82" t="n">
+        <v>91.24325177701475</v>
+      </c>
+      <c r="I82" t="inlineStr">
+        <is>
+          <t>2026-03-21T22:47:57</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>2026-03-22</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>시드릴</t>
+        </is>
+      </c>
+      <c r="C83" t="n">
+        <v>123</v>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E83" t="n">
+        <v>1</v>
+      </c>
+      <c r="F83" t="n">
+        <v>8070101.805898919</v>
+      </c>
+      <c r="G83" t="n">
+        <v>1619750.805898919</v>
+      </c>
+      <c r="H83" t="n">
+        <v>25.11104908707943</v>
+      </c>
+      <c r="I83" t="inlineStr">
+        <is>
+          <t>2026-03-21T22:47:57</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>2026-03-22</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>세아제강</t>
+        </is>
+      </c>
+      <c r="C84" t="n">
+        <v>50</v>
+      </c>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E84" t="n">
+        <v>1</v>
+      </c>
+      <c r="F84" t="n">
+        <v>7395000</v>
+      </c>
+      <c r="G84" t="n">
+        <v>1085000</v>
+      </c>
+      <c r="H84" t="n">
+        <v>17.19492868462758</v>
+      </c>
+      <c r="I84" t="inlineStr">
+        <is>
+          <t>2026-03-21T22:47:57</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>2026-03-22</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>센트러스 에너지</t>
+        </is>
+      </c>
+      <c r="C85" t="n">
+        <v>25</v>
+      </c>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E85" t="n">
+        <v>1</v>
+      </c>
+      <c r="F85" t="n">
+        <v>7026050.85816239</v>
+      </c>
+      <c r="G85" t="n">
+        <v>-406805.1418376099</v>
+      </c>
+      <c r="H85" t="n">
+        <v>-5.473066366920198</v>
+      </c>
+      <c r="I85" t="inlineStr">
+        <is>
+          <t>2026-03-21T22:47:57</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>2026-03-22</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>트랜스오션</t>
+        </is>
+      </c>
+      <c r="C86" t="n">
+        <v>750</v>
+      </c>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E86" t="n">
+        <v>1</v>
+      </c>
+      <c r="F86" t="n">
+        <v>7020031.5082007</v>
+      </c>
+      <c r="G86" t="n">
+        <v>2892797.5082007</v>
+      </c>
+      <c r="H86" t="n">
+        <v>70.09046514446965</v>
+      </c>
+      <c r="I86" t="inlineStr">
+        <is>
+          <t>2026-03-21T22:47:57</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>2026-03-22</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>노블</t>
+        </is>
+      </c>
+      <c r="C87" t="n">
+        <v>99</v>
+      </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E87" t="n">
+        <v>1</v>
+      </c>
+      <c r="F87" t="n">
+        <v>6958769.981090547</v>
+      </c>
+      <c r="G87" t="n">
+        <v>3051561.981090547</v>
+      </c>
+      <c r="H87" t="n">
+        <v>78.10083264291401</v>
+      </c>
+      <c r="I87" t="inlineStr">
+        <is>
+          <t>2026-03-21T22:47:57</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>2026-03-22</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>타이드워터</t>
+        </is>
+      </c>
+      <c r="C88" t="n">
+        <v>48</v>
+      </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E88" t="n">
+        <v>1</v>
+      </c>
+      <c r="F88" t="n">
+        <v>5235363.852789983</v>
+      </c>
+      <c r="G88" t="n">
+        <v>1510818.852789983</v>
+      </c>
+      <c r="H88" t="n">
+        <v>40.56385015592463</v>
+      </c>
+      <c r="I88" t="inlineStr">
+        <is>
+          <t>2026-03-21T22:47:57</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>2026-03-22</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>노브</t>
+        </is>
+      </c>
+      <c r="C89" t="n">
+        <v>185</v>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E89" t="n">
+        <v>1</v>
+      </c>
+      <c r="F89" t="n">
+        <v>5200391.447092756</v>
+      </c>
+      <c r="G89" t="n">
+        <v>1890383.447092756</v>
+      </c>
+      <c r="H89" t="n">
+        <v>57.11114435653194</v>
+      </c>
+      <c r="I89" t="inlineStr">
+        <is>
+          <t>2026-03-21T22:47:57</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>2026-03-22</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>TIME 코리아밸류업액티브</t>
+        </is>
+      </c>
+      <c r="C90" t="n">
+        <v>201</v>
+      </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E90" t="n">
+        <v>1</v>
+      </c>
+      <c r="F90" t="n">
+        <v>4797870</v>
+      </c>
+      <c r="G90" t="n">
+        <v>74073</v>
+      </c>
+      <c r="H90" t="n">
+        <v>1.568081778281328</v>
+      </c>
+      <c r="I90" t="inlineStr">
+        <is>
+          <t>2026-03-21T22:47:57</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>2026-03-22</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>오케아니스 에코 탱커스</t>
+        </is>
+      </c>
+      <c r="C91" t="n">
+        <v>65</v>
+      </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E91" t="n">
+        <v>1</v>
+      </c>
+      <c r="F91" t="n">
+        <v>4511179.137784176</v>
+      </c>
+      <c r="G91" t="n">
+        <v>2254819.137784176</v>
+      </c>
+      <c r="H91" t="n">
+        <v>99.93171026716378</v>
+      </c>
+      <c r="I91" t="inlineStr">
+        <is>
+          <t>2026-03-21T22:47:57</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>2026-03-22</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>삼성화재</t>
+        </is>
+      </c>
+      <c r="C92" t="n">
+        <v>9</v>
+      </c>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E92" t="n">
+        <v>1</v>
+      </c>
+      <c r="F92" t="n">
+        <v>4270500</v>
+      </c>
+      <c r="G92" t="n">
+        <v>-360500</v>
+      </c>
+      <c r="H92" t="n">
+        <v>-7.784495789246384</v>
+      </c>
+      <c r="I92" t="inlineStr">
+        <is>
+          <t>2026-03-21T22:47:57</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>2026-03-22</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>동원개발</t>
+        </is>
+      </c>
+      <c r="C93" t="n">
+        <v>1360</v>
+      </c>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E93" t="n">
+        <v>1</v>
+      </c>
+      <c r="F93" t="n">
+        <v>4202400</v>
+      </c>
+      <c r="G93" t="n">
+        <v>465000</v>
+      </c>
+      <c r="H93" t="n">
+        <v>12.44180446299566</v>
+      </c>
+      <c r="I93" t="inlineStr">
+        <is>
+          <t>2026-03-21T22:47:57</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>2026-03-22</t>
+        </is>
+      </c>
+      <c r="B9